<commit_message>
update: 2026-04-07 ~ 2026-04-07
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.26</v>
+        <v>3.255</v>
       </c>
       <c r="G2" t="n">
-        <v>3.484</v>
+        <v>3.479</v>
       </c>
       <c r="H2" t="n">
-        <v>3.631</v>
+        <v>3.63</v>
       </c>
       <c r="I2" t="n">
-        <v>3.847</v>
+        <v>3.856</v>
       </c>
       <c r="J2" t="n">
-        <v>4.073</v>
+        <v>4.078</v>
       </c>
       <c r="K2" t="n">
-        <v>4.47</v>
+        <v>4.475</v>
       </c>
       <c r="L2" t="n">
-        <v>4.637</v>
+        <v>4.644</v>
       </c>
       <c r="M2" t="n">
-        <v>4.925</v>
+        <v>4.942</v>
       </c>
       <c r="N2" t="n">
-        <v>5.17</v>
+        <v>5.194</v>
       </c>
       <c r="O2" t="n">
-        <v>5.384</v>
+        <v>5.41</v>
       </c>
       <c r="P2" t="n">
-        <v>5.558</v>
+        <v>5.585</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.195</v>
+        <v>6.225</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.284</v>
+        <v>4.279</v>
       </c>
       <c r="G3" t="n">
-        <v>4.689</v>
+        <v>4.684</v>
       </c>
       <c r="H3" t="n">
-        <v>4.869</v>
+        <v>4.867</v>
       </c>
       <c r="I3" t="n">
-        <v>5.087</v>
+        <v>5.093</v>
       </c>
       <c r="J3" t="n">
-        <v>5.322</v>
+        <v>5.325</v>
       </c>
       <c r="K3" t="n">
-        <v>5.786</v>
+        <v>5.79</v>
       </c>
       <c r="L3" t="n">
-        <v>6.024</v>
+        <v>6.029</v>
       </c>
       <c r="M3" t="n">
-        <v>6.342</v>
+        <v>6.359</v>
       </c>
       <c r="N3" t="n">
-        <v>6.53</v>
+        <v>6.554</v>
       </c>
       <c r="O3" t="n">
-        <v>6.693</v>
+        <v>6.72</v>
       </c>
       <c r="P3" t="n">
-        <v>6.736</v>
+        <v>6.764</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.263</v>
+        <v>7.293</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.775</v>
+        <v>3.77</v>
       </c>
       <c r="G4" t="n">
-        <v>4.069</v>
+        <v>4.064</v>
       </c>
       <c r="H4" t="n">
-        <v>4.278</v>
+        <v>4.276</v>
       </c>
       <c r="I4" t="n">
-        <v>4.525</v>
+        <v>4.534</v>
       </c>
       <c r="J4" t="n">
-        <v>4.767</v>
+        <v>4.772</v>
       </c>
       <c r="K4" t="n">
-        <v>5.225</v>
+        <v>5.231</v>
       </c>
       <c r="L4" t="n">
-        <v>5.393</v>
+        <v>5.4</v>
       </c>
       <c r="M4" t="n">
-        <v>5.699</v>
+        <v>5.717</v>
       </c>
       <c r="N4" t="n">
-        <v>5.858</v>
+        <v>5.882</v>
       </c>
       <c r="O4" t="n">
-        <v>6.046</v>
+        <v>6.072</v>
       </c>
       <c r="P4" t="n">
-        <v>6.086</v>
+        <v>6.113</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.616</v>
+        <v>6.646</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.97</v>
+        <v>2.965</v>
       </c>
       <c r="G5" t="n">
-        <v>3.034</v>
+        <v>3.03</v>
       </c>
       <c r="H5" t="n">
-        <v>3.134</v>
+        <v>3.133</v>
       </c>
       <c r="I5" t="n">
-        <v>3.419</v>
+        <v>3.428</v>
       </c>
       <c r="J5" t="n">
-        <v>3.642</v>
+        <v>3.648</v>
       </c>
       <c r="K5" t="n">
-        <v>3.897</v>
+        <v>3.904</v>
       </c>
       <c r="L5" t="n">
-        <v>3.909</v>
+        <v>3.915</v>
       </c>
       <c r="M5" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3.998</v>
+      </c>
+      <c r="O5" t="n">
         <v>4.003</v>
       </c>
-      <c r="N5" t="n">
-        <v>3.973</v>
-      </c>
-      <c r="O5" t="n">
-        <v>3.976</v>
-      </c>
       <c r="P5" t="n">
-        <v>4.228</v>
+        <v>4.255</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.107</v>
+        <v>5.137</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.01</v>
+        <v>3.005</v>
       </c>
       <c r="G6" t="n">
-        <v>3.087</v>
+        <v>3.083</v>
       </c>
       <c r="H6" t="n">
-        <v>3.203</v>
+        <v>3.202</v>
       </c>
       <c r="I6" t="n">
-        <v>3.493</v>
+        <v>3.502</v>
       </c>
       <c r="J6" t="n">
-        <v>3.727</v>
+        <v>3.733</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>4.007</v>
       </c>
       <c r="L6" t="n">
-        <v>4.023</v>
+        <v>4.029</v>
       </c>
       <c r="M6" t="n">
-        <v>4.15</v>
+        <v>4.168</v>
       </c>
       <c r="N6" t="n">
-        <v>4.143</v>
+        <v>4.168</v>
       </c>
       <c r="O6" t="n">
-        <v>4.252</v>
+        <v>4.278</v>
       </c>
       <c r="P6" t="n">
-        <v>4.66</v>
+        <v>4.687</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.503</v>
+        <v>5.533</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.99</v>
+        <v>2.985</v>
       </c>
       <c r="G7" t="n">
-        <v>3.053</v>
+        <v>3.049</v>
       </c>
       <c r="H7" t="n">
-        <v>3.15</v>
+        <v>3.149</v>
       </c>
       <c r="I7" t="n">
-        <v>3.435</v>
+        <v>3.443</v>
       </c>
       <c r="J7" t="n">
-        <v>3.668</v>
+        <v>3.674</v>
       </c>
       <c r="K7" t="n">
-        <v>3.923</v>
+        <v>3.929</v>
       </c>
       <c r="L7" t="n">
-        <v>3.934</v>
+        <v>3.941</v>
       </c>
       <c r="M7" t="n">
-        <v>4.061</v>
+        <v>4.078</v>
       </c>
       <c r="N7" t="n">
-        <v>4.034</v>
+        <v>4.058</v>
       </c>
       <c r="O7" t="n">
-        <v>4.152</v>
+        <v>4.178</v>
       </c>
       <c r="P7" t="n">
-        <v>4.444</v>
+        <v>4.471</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.271</v>
+        <v>5.301</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.393</v>
+        <v>5.388</v>
       </c>
       <c r="G8" t="n">
-        <v>5.986</v>
+        <v>5.982</v>
       </c>
       <c r="H8" t="n">
-        <v>6.318</v>
+        <v>6.317</v>
       </c>
       <c r="I8" t="n">
-        <v>6.606</v>
+        <v>6.614</v>
       </c>
       <c r="J8" t="n">
-        <v>6.905</v>
+        <v>6.91</v>
       </c>
       <c r="K8" t="n">
-        <v>7.651</v>
+        <v>7.656</v>
       </c>
       <c r="L8" t="n">
-        <v>7.978</v>
+        <v>7.984</v>
       </c>
       <c r="M8" t="n">
-        <v>8.324999999999999</v>
+        <v>8.342000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.451000000000001</v>
+        <v>8.475</v>
       </c>
       <c r="O8" t="n">
-        <v>8.699999999999999</v>
+        <v>8.727</v>
       </c>
       <c r="P8" t="n">
-        <v>8.842000000000001</v>
+        <v>8.869</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.571999999999999</v>
+        <v>9.602</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1072,48 +1072,48 @@
         <v>2.827</v>
       </c>
       <c r="I9" t="n">
-        <v>2.997</v>
+        <v>2.994</v>
       </c>
       <c r="J9" t="n">
-        <v>3.14</v>
+        <v>3.139</v>
       </c>
       <c r="K9" t="n">
-        <v>3.337</v>
+        <v>3.332</v>
       </c>
       <c r="L9" t="n">
         <v>3.38</v>
       </c>
       <c r="M9" t="n">
-        <v>3.43</v>
+        <v>3.445</v>
       </c>
       <c r="N9" t="n">
-        <v>3.569</v>
+        <v>3.59</v>
       </c>
       <c r="O9" t="n">
-        <v>3.592</v>
+        <v>3.617</v>
       </c>
       <c r="P9" t="n">
-        <v>3.656</v>
+        <v>3.682</v>
       </c>
       <c r="Q9" t="n">
+        <v>3.755</v>
+      </c>
+      <c r="R9" t="n">
+        <v>3.766</v>
+      </c>
+      <c r="S9" t="n">
         <v>3.725</v>
       </c>
-      <c r="R9" t="n">
-        <v>3.732</v>
-      </c>
-      <c r="S9" t="n">
-        <v>3.687</v>
-      </c>
       <c r="T9" t="n">
-        <v>3.611</v>
+        <v>3.637</v>
       </c>
       <c r="U9" t="n">
-        <v>3.515</v>
+        <v>3.542</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1145,25 +1145,25 @@
         <v>2.838</v>
       </c>
       <c r="I10" t="n">
-        <v>3.006</v>
+        <v>3.004</v>
       </c>
       <c r="J10" t="n">
-        <v>3.166</v>
+        <v>3.167</v>
       </c>
       <c r="K10" t="n">
-        <v>3.361</v>
+        <v>3.358</v>
       </c>
       <c r="L10" t="n">
-        <v>3.421</v>
+        <v>3.422</v>
       </c>
       <c r="M10" t="n">
-        <v>3.529</v>
+        <v>3.545</v>
       </c>
       <c r="N10" t="n">
-        <v>3.576</v>
+        <v>3.596</v>
       </c>
       <c r="O10" t="n">
-        <v>3.775</v>
+        <v>3.791</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.445</v>
+        <v>2.446</v>
       </c>
       <c r="G11" t="n">
-        <v>2.56</v>
+        <v>2.561</v>
       </c>
       <c r="H11" t="n">
-        <v>2.66</v>
+        <v>2.661</v>
       </c>
       <c r="I11" t="n">
-        <v>2.808</v>
+        <v>2.806</v>
       </c>
       <c r="J11" t="n">
-        <v>2.96</v>
+        <v>2.961</v>
       </c>
       <c r="K11" t="n">
-        <v>3.149</v>
+        <v>3.145</v>
       </c>
       <c r="L11" t="n">
-        <v>3.215</v>
+        <v>3.216</v>
       </c>
       <c r="M11" t="n">
-        <v>3.334</v>
+        <v>3.35</v>
       </c>
       <c r="N11" t="n">
-        <v>3.386</v>
+        <v>3.407</v>
       </c>
       <c r="O11" t="n">
-        <v>3.542</v>
+        <v>3.558</v>
       </c>
       <c r="P11" t="n">
-        <v>3.593</v>
+        <v>3.619</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.928</v>
+        <v>3.958</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1285,43 +1285,43 @@
         <v>3.228</v>
       </c>
       <c r="G12" t="n">
-        <v>3.388</v>
+        <v>3.387</v>
       </c>
       <c r="H12" t="n">
-        <v>3.502</v>
+        <v>3.503</v>
       </c>
       <c r="I12" t="n">
-        <v>3.737</v>
+        <v>3.742</v>
       </c>
       <c r="J12" t="n">
-        <v>4.064</v>
+        <v>4.066</v>
       </c>
       <c r="K12" t="n">
-        <v>4.273</v>
+        <v>4.275</v>
       </c>
       <c r="L12" t="n">
         <v>4.322</v>
       </c>
       <c r="M12" t="n">
-        <v>4.443</v>
+        <v>4.458</v>
       </c>
       <c r="N12" t="n">
-        <v>4.446</v>
+        <v>4.47</v>
       </c>
       <c r="O12" t="n">
-        <v>4.596</v>
+        <v>4.622</v>
       </c>
       <c r="P12" t="n">
-        <v>4.686</v>
+        <v>4.717</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.055</v>
+        <v>5.085</v>
       </c>
       <c r="R12" t="n">
-        <v>5.229</v>
+        <v>5.263</v>
       </c>
       <c r="S12" t="n">
-        <v>5.398</v>
+        <v>5.436</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1361,40 +1361,40 @@
         <v>3.078</v>
       </c>
       <c r="H13" t="n">
-        <v>3.17</v>
+        <v>3.171</v>
       </c>
       <c r="I13" t="n">
-        <v>3.385</v>
+        <v>3.389</v>
       </c>
       <c r="J13" t="n">
-        <v>3.701</v>
+        <v>3.703</v>
       </c>
       <c r="K13" t="n">
-        <v>3.907</v>
+        <v>3.908</v>
       </c>
       <c r="L13" t="n">
-        <v>3.961</v>
+        <v>3.962</v>
       </c>
       <c r="M13" t="n">
-        <v>4.07</v>
+        <v>4.086</v>
       </c>
       <c r="N13" t="n">
-        <v>4.074</v>
+        <v>4.098</v>
       </c>
       <c r="O13" t="n">
-        <v>4.223</v>
+        <v>4.248</v>
       </c>
       <c r="P13" t="n">
-        <v>4.277</v>
+        <v>4.309</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.576</v>
+        <v>4.606</v>
       </c>
       <c r="R13" t="n">
-        <v>4.778</v>
+        <v>4.811</v>
       </c>
       <c r="S13" t="n">
-        <v>4.96</v>
+        <v>4.998</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1431,43 +1431,43 @@
         <v>2.8</v>
       </c>
       <c r="G14" t="n">
-        <v>2.885</v>
+        <v>2.884</v>
       </c>
       <c r="H14" t="n">
-        <v>2.973</v>
+        <v>2.974</v>
       </c>
       <c r="I14" t="n">
-        <v>3.168</v>
+        <v>3.173</v>
       </c>
       <c r="J14" t="n">
-        <v>3.441</v>
+        <v>3.442</v>
       </c>
       <c r="K14" t="n">
-        <v>3.595</v>
+        <v>3.596</v>
       </c>
       <c r="L14" t="n">
-        <v>3.633</v>
+        <v>3.634</v>
       </c>
       <c r="M14" t="n">
-        <v>3.755</v>
+        <v>3.771</v>
       </c>
       <c r="N14" t="n">
-        <v>3.755</v>
+        <v>3.78</v>
       </c>
       <c r="O14" t="n">
-        <v>3.878</v>
+        <v>3.903</v>
       </c>
       <c r="P14" t="n">
-        <v>3.912</v>
+        <v>3.944</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.165</v>
+        <v>4.195</v>
       </c>
       <c r="R14" t="n">
-        <v>4.293</v>
+        <v>4.326</v>
       </c>
       <c r="S14" t="n">
-        <v>4.412</v>
+        <v>4.451</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1504,43 +1504,43 @@
         <v>2.778</v>
       </c>
       <c r="G15" t="n">
-        <v>2.859</v>
+        <v>2.858</v>
       </c>
       <c r="H15" t="n">
-        <v>2.942</v>
+        <v>2.943</v>
       </c>
       <c r="I15" t="n">
-        <v>3.119</v>
+        <v>3.123</v>
       </c>
       <c r="J15" t="n">
-        <v>3.377</v>
+        <v>3.379</v>
       </c>
       <c r="K15" t="n">
-        <v>3.549</v>
+        <v>3.55</v>
       </c>
       <c r="L15" t="n">
-        <v>3.567</v>
+        <v>3.568</v>
       </c>
       <c r="M15" t="n">
-        <v>3.667</v>
+        <v>3.683</v>
       </c>
       <c r="N15" t="n">
-        <v>3.659</v>
+        <v>3.683</v>
       </c>
       <c r="O15" t="n">
-        <v>3.801</v>
+        <v>3.826</v>
       </c>
       <c r="P15" t="n">
-        <v>3.808</v>
+        <v>3.84</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.07</v>
+        <v>4.1</v>
       </c>
       <c r="R15" t="n">
-        <v>4.189</v>
+        <v>4.222</v>
       </c>
       <c r="S15" t="n">
-        <v>4.308</v>
+        <v>4.346</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1577,43 +1577,43 @@
         <v>2.778</v>
       </c>
       <c r="G16" t="n">
-        <v>2.859</v>
+        <v>2.858</v>
       </c>
       <c r="H16" t="n">
-        <v>2.942</v>
+        <v>2.943</v>
       </c>
       <c r="I16" t="n">
-        <v>3.119</v>
+        <v>3.123</v>
       </c>
       <c r="J16" t="n">
-        <v>3.377</v>
+        <v>3.379</v>
       </c>
       <c r="K16" t="n">
-        <v>3.549</v>
+        <v>3.55</v>
       </c>
       <c r="L16" t="n">
-        <v>3.567</v>
+        <v>3.568</v>
       </c>
       <c r="M16" t="n">
-        <v>3.667</v>
+        <v>3.683</v>
       </c>
       <c r="N16" t="n">
-        <v>3.662</v>
+        <v>3.686</v>
       </c>
       <c r="O16" t="n">
-        <v>3.807</v>
+        <v>3.832</v>
       </c>
       <c r="P16" t="n">
-        <v>3.832</v>
+        <v>3.863</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.097</v>
+        <v>4.127</v>
       </c>
       <c r="R16" t="n">
-        <v>4.217</v>
+        <v>4.25</v>
       </c>
       <c r="S16" t="n">
-        <v>4.337</v>
+        <v>4.375</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1653,31 +1653,31 @@
         <v>2.844</v>
       </c>
       <c r="H17" t="n">
-        <v>2.931</v>
+        <v>2.932</v>
       </c>
       <c r="I17" t="n">
-        <v>3.09</v>
+        <v>3.087</v>
       </c>
       <c r="J17" t="n">
         <v>3.235</v>
       </c>
       <c r="K17" t="n">
-        <v>3.436</v>
+        <v>3.431</v>
       </c>
       <c r="L17" t="n">
-        <v>3.498</v>
+        <v>3.499</v>
       </c>
       <c r="M17" t="n">
-        <v>3.65</v>
+        <v>3.665</v>
       </c>
       <c r="N17" t="n">
-        <v>3.678</v>
+        <v>3.698</v>
       </c>
       <c r="O17" t="n">
-        <v>3.81</v>
+        <v>3.826</v>
       </c>
       <c r="P17" t="n">
-        <v>3.875</v>
+        <v>3.9</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.693</v>
       </c>
       <c r="G18" t="n">
-        <v>2.844</v>
+        <v>2.846</v>
       </c>
       <c r="H18" t="n">
-        <v>2.932</v>
+        <v>2.933</v>
       </c>
       <c r="I18" t="n">
-        <v>3.089</v>
+        <v>3.087</v>
       </c>
       <c r="J18" t="n">
         <v>3.235</v>
       </c>
       <c r="K18" t="n">
-        <v>3.437</v>
+        <v>3.433</v>
       </c>
       <c r="L18" t="n">
-        <v>3.497</v>
+        <v>3.498</v>
       </c>
       <c r="M18" t="n">
-        <v>3.65</v>
+        <v>3.665</v>
       </c>
       <c r="N18" t="n">
-        <v>3.677</v>
+        <v>3.697</v>
       </c>
       <c r="O18" t="n">
-        <v>3.809</v>
+        <v>3.825</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1796,43 +1796,43 @@
         <v>2.789</v>
       </c>
       <c r="G19" t="n">
-        <v>2.876</v>
+        <v>2.875</v>
       </c>
       <c r="H19" t="n">
-        <v>2.963</v>
+        <v>2.964</v>
       </c>
       <c r="I19" t="n">
-        <v>3.153</v>
+        <v>3.157</v>
       </c>
       <c r="J19" t="n">
-        <v>3.424</v>
+        <v>3.425</v>
       </c>
       <c r="K19" t="n">
-        <v>3.592</v>
+        <v>3.594</v>
       </c>
       <c r="L19" t="n">
-        <v>3.63</v>
+        <v>3.631</v>
       </c>
       <c r="M19" t="n">
-        <v>3.743</v>
+        <v>3.758</v>
       </c>
       <c r="N19" t="n">
-        <v>3.743</v>
+        <v>3.767</v>
       </c>
       <c r="O19" t="n">
-        <v>3.856</v>
+        <v>3.88</v>
       </c>
       <c r="P19" t="n">
-        <v>3.875</v>
+        <v>3.906</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.116</v>
+        <v>4.146</v>
       </c>
       <c r="R19" t="n">
-        <v>4.243</v>
+        <v>4.276</v>
       </c>
       <c r="S19" t="n">
-        <v>4.352</v>
+        <v>4.39</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.657</v>
+        <v>2.658</v>
       </c>
       <c r="H20" t="n">
-        <v>2.736</v>
+        <v>2.737</v>
       </c>
       <c r="I20" t="n">
-        <v>2.94</v>
+        <v>2.939</v>
       </c>
       <c r="J20" t="n">
-        <v>3.211</v>
+        <v>3.206</v>
       </c>
       <c r="K20" t="n">
         <v>3.368</v>
       </c>
       <c r="L20" t="n">
-        <v>3.385</v>
+        <v>3.397</v>
       </c>
       <c r="M20" t="n">
-        <v>3.475</v>
+        <v>3.49</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.882</v>
+        <v>2.878</v>
       </c>
       <c r="G21" t="n">
         <v>2.975</v>
       </c>
       <c r="H21" t="n">
-        <v>3.109</v>
+        <v>3.11</v>
       </c>
       <c r="I21" t="n">
-        <v>3.3</v>
+        <v>3.301</v>
       </c>
       <c r="J21" t="n">
         <v>3.554</v>
       </c>
       <c r="K21" t="n">
-        <v>3.829</v>
+        <v>3.827</v>
       </c>
       <c r="L21" t="n">
-        <v>3.899</v>
+        <v>3.898</v>
       </c>
       <c r="M21" t="n">
-        <v>3.997</v>
+        <v>4.013</v>
       </c>
       <c r="N21" t="n">
-        <v>4.003</v>
+        <v>4.026</v>
       </c>
       <c r="O21" t="n">
-        <v>4.091</v>
+        <v>4.116</v>
       </c>
       <c r="P21" t="n">
-        <v>4.144</v>
+        <v>4.172</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.272</v>
+        <v>4.303</v>
       </c>
       <c r="R21" t="n">
-        <v>4.291</v>
+        <v>4.325</v>
       </c>
       <c r="S21" t="n">
-        <v>4.314</v>
+        <v>4.351</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.83</v>
+        <v>2.825</v>
       </c>
       <c r="G22" t="n">
         <v>2.922</v>
       </c>
       <c r="H22" t="n">
-        <v>3.044</v>
+        <v>3.045</v>
       </c>
       <c r="I22" t="n">
-        <v>3.218</v>
+        <v>3.219</v>
       </c>
       <c r="J22" t="n">
         <v>3.439</v>
       </c>
       <c r="K22" t="n">
-        <v>3.71</v>
+        <v>3.707</v>
       </c>
       <c r="L22" t="n">
-        <v>3.768</v>
+        <v>3.767</v>
       </c>
       <c r="M22" t="n">
-        <v>3.869</v>
+        <v>3.885</v>
       </c>
       <c r="N22" t="n">
-        <v>3.876</v>
+        <v>3.899</v>
       </c>
       <c r="O22" t="n">
-        <v>3.96</v>
+        <v>3.985</v>
       </c>
       <c r="P22" t="n">
-        <v>4.006</v>
+        <v>4.035</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.131</v>
+        <v>4.161</v>
       </c>
       <c r="R22" t="n">
-        <v>4.136</v>
+        <v>4.169</v>
       </c>
       <c r="S22" t="n">
-        <v>4.156</v>
+        <v>4.194</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.782</v>
+        <v>2.778</v>
       </c>
       <c r="G23" t="n">
         <v>2.876</v>
       </c>
       <c r="H23" t="n">
-        <v>2.982</v>
+        <v>2.983</v>
       </c>
       <c r="I23" t="n">
-        <v>3.171</v>
+        <v>3.172</v>
       </c>
       <c r="J23" t="n">
         <v>3.385</v>
       </c>
       <c r="K23" t="n">
-        <v>3.629</v>
+        <v>3.627</v>
       </c>
       <c r="L23" t="n">
-        <v>3.679</v>
+        <v>3.678</v>
       </c>
       <c r="M23" t="n">
-        <v>3.772</v>
+        <v>3.789</v>
       </c>
       <c r="N23" t="n">
-        <v>3.771</v>
+        <v>3.794</v>
       </c>
       <c r="O23" t="n">
-        <v>3.834</v>
+        <v>3.859</v>
       </c>
       <c r="P23" t="n">
-        <v>3.866</v>
+        <v>3.895</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.941</v>
+        <v>3.971</v>
       </c>
       <c r="R23" t="n">
-        <v>3.918</v>
+        <v>3.952</v>
       </c>
       <c r="S23" t="n">
-        <v>3.91</v>
+        <v>3.948</v>
       </c>
       <c r="T23" t="n">
-        <v>3.823</v>
+        <v>3.849</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.713</v>
+        <v>2.707</v>
       </c>
       <c r="G24" t="n">
-        <v>2.791</v>
+        <v>2.79</v>
       </c>
       <c r="H24" t="n">
-        <v>2.883</v>
+        <v>2.885</v>
       </c>
       <c r="I24" t="n">
-        <v>3.081</v>
+        <v>3.082</v>
       </c>
       <c r="J24" t="n">
         <v>3.286</v>
       </c>
       <c r="K24" t="n">
-        <v>3.517</v>
+        <v>3.512</v>
       </c>
       <c r="L24" t="n">
-        <v>3.552</v>
+        <v>3.551</v>
       </c>
       <c r="M24" t="n">
-        <v>3.629</v>
+        <v>3.645</v>
       </c>
       <c r="N24" t="n">
-        <v>3.642</v>
+        <v>3.666</v>
       </c>
       <c r="O24" t="n">
-        <v>3.785</v>
+        <v>3.811</v>
       </c>
       <c r="P24" t="n">
-        <v>3.804</v>
+        <v>3.834</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.861</v>
+        <v>3.892</v>
       </c>
       <c r="R24" t="n">
-        <v>3.838</v>
+        <v>3.872</v>
       </c>
       <c r="S24" t="n">
-        <v>3.826</v>
+        <v>3.864</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.775</v>
+        <v>2.771</v>
       </c>
       <c r="G25" t="n">
         <v>2.875</v>
       </c>
       <c r="H25" t="n">
-        <v>2.985</v>
+        <v>2.987</v>
       </c>
       <c r="I25" t="n">
-        <v>3.179</v>
+        <v>3.18</v>
       </c>
       <c r="J25" t="n">
         <v>3.401</v>
       </c>
       <c r="K25" t="n">
-        <v>3.658</v>
+        <v>3.656</v>
       </c>
       <c r="L25" t="n">
         <v>3.707</v>
       </c>
       <c r="M25" t="n">
-        <v>3.8</v>
+        <v>3.816</v>
       </c>
       <c r="N25" t="n">
-        <v>3.798</v>
+        <v>3.821</v>
       </c>
       <c r="O25" t="n">
-        <v>3.863</v>
+        <v>3.888</v>
       </c>
       <c r="P25" t="n">
-        <v>3.889</v>
+        <v>3.918</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.973</v>
+        <v>4.003</v>
       </c>
       <c r="R25" t="n">
-        <v>3.942</v>
+        <v>3.976</v>
       </c>
       <c r="S25" t="n">
-        <v>3.933</v>
+        <v>3.971</v>
       </c>
       <c r="T25" t="n">
-        <v>3.841</v>
+        <v>3.867</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2310,28 +2310,28 @@
         <v>3.235</v>
       </c>
       <c r="H26" t="n">
-        <v>3.424</v>
+        <v>3.43</v>
       </c>
       <c r="I26" t="n">
-        <v>3.7</v>
+        <v>3.707</v>
       </c>
       <c r="J26" t="n">
-        <v>4.042</v>
+        <v>4.046</v>
       </c>
       <c r="K26" t="n">
-        <v>4.429</v>
+        <v>4.433</v>
       </c>
       <c r="L26" t="n">
-        <v>4.52</v>
+        <v>4.527</v>
       </c>
       <c r="M26" t="n">
-        <v>4.7</v>
+        <v>4.718</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.922</v>
+        <v>4.947</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.887</v>
+        <v>2.886</v>
       </c>
       <c r="G27" t="n">
         <v>2.969</v>
       </c>
       <c r="H27" t="n">
-        <v>3.068</v>
+        <v>3.071</v>
       </c>
       <c r="I27" t="n">
-        <v>3.286</v>
+        <v>3.292</v>
       </c>
       <c r="J27" t="n">
-        <v>3.55</v>
+        <v>3.553</v>
       </c>
       <c r="K27" t="n">
-        <v>3.76</v>
+        <v>3.762</v>
       </c>
       <c r="L27" t="n">
-        <v>3.803</v>
+        <v>3.808</v>
       </c>
       <c r="M27" t="n">
-        <v>3.918</v>
+        <v>3.933</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.021</v>
+        <v>4.046</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.986</v>
+        <v>2.985</v>
       </c>
       <c r="G28" t="n">
-        <v>3.074</v>
+        <v>3.073</v>
       </c>
       <c r="H28" t="n">
-        <v>3.191</v>
+        <v>3.194</v>
       </c>
       <c r="I28" t="n">
-        <v>3.422</v>
+        <v>3.428</v>
       </c>
       <c r="J28" t="n">
-        <v>3.724</v>
+        <v>3.727</v>
       </c>
       <c r="K28" t="n">
-        <v>3.952</v>
+        <v>3.954</v>
       </c>
       <c r="L28" t="n">
-        <v>4.007</v>
+        <v>4.011</v>
       </c>
       <c r="M28" t="n">
-        <v>4.131</v>
+        <v>4.146</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.317</v>
+        <v>4.34</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.846</v>
+        <v>2.845</v>
       </c>
       <c r="G29" t="n">
-        <v>2.93</v>
+        <v>2.929</v>
       </c>
       <c r="H29" t="n">
-        <v>3.013</v>
+        <v>3.017</v>
       </c>
       <c r="I29" t="n">
-        <v>3.219</v>
+        <v>3.224</v>
       </c>
       <c r="J29" t="n">
-        <v>3.463</v>
+        <v>3.466</v>
       </c>
       <c r="K29" t="n">
-        <v>3.657</v>
+        <v>3.659</v>
       </c>
       <c r="L29" t="n">
-        <v>3.688</v>
+        <v>3.692</v>
       </c>
       <c r="M29" t="n">
-        <v>3.78</v>
+        <v>3.795</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.879</v>
+        <v>3.904</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2602,34 +2602,34 @@
         <v>3.191</v>
       </c>
       <c r="H30" t="n">
-        <v>3.345</v>
+        <v>3.351</v>
       </c>
       <c r="I30" t="n">
-        <v>3.619</v>
+        <v>3.625</v>
       </c>
       <c r="J30" t="n">
-        <v>3.904</v>
+        <v>3.907</v>
       </c>
       <c r="K30" t="n">
-        <v>4.223</v>
+        <v>4.227</v>
       </c>
       <c r="L30" t="n">
-        <v>4.291</v>
+        <v>4.297</v>
       </c>
       <c r="M30" t="n">
-        <v>4.458</v>
+        <v>4.477</v>
       </c>
       <c r="N30" t="n">
-        <v>4.597</v>
+        <v>4.62</v>
       </c>
       <c r="O30" t="n">
-        <v>4.883</v>
+        <v>4.906</v>
       </c>
       <c r="P30" t="n">
-        <v>5.042</v>
+        <v>5.068</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.798</v>
+        <v>5.829</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2675,34 +2675,34 @@
         <v>3.551</v>
       </c>
       <c r="H31" t="n">
-        <v>3.758</v>
+        <v>3.764</v>
       </c>
       <c r="I31" t="n">
-        <v>4.047</v>
+        <v>4.053</v>
       </c>
       <c r="J31" t="n">
-        <v>4.392</v>
+        <v>4.395</v>
       </c>
       <c r="K31" t="n">
-        <v>4.755</v>
+        <v>4.76</v>
       </c>
       <c r="L31" t="n">
-        <v>4.901</v>
+        <v>4.907</v>
       </c>
       <c r="M31" t="n">
-        <v>5.187</v>
+        <v>5.206</v>
       </c>
       <c r="N31" t="n">
-        <v>5.454</v>
+        <v>5.476</v>
       </c>
       <c r="O31" t="n">
-        <v>5.911</v>
+        <v>5.936</v>
       </c>
       <c r="P31" t="n">
-        <v>6.026</v>
+        <v>6.054</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.772</v>
+        <v>6.803</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.206</v>
+        <v>3.207</v>
       </c>
       <c r="G32" t="n">
         <v>3.307</v>
       </c>
       <c r="H32" t="n">
-        <v>3.488</v>
+        <v>3.494</v>
       </c>
       <c r="I32" t="n">
-        <v>3.778</v>
+        <v>3.784</v>
       </c>
       <c r="J32" t="n">
-        <v>4.081</v>
+        <v>4.084</v>
       </c>
       <c r="K32" t="n">
-        <v>4.408</v>
+        <v>4.413</v>
       </c>
       <c r="L32" t="n">
-        <v>4.493</v>
+        <v>4.5</v>
       </c>
       <c r="M32" t="n">
-        <v>4.73</v>
+        <v>4.749</v>
       </c>
       <c r="N32" t="n">
-        <v>4.957</v>
+        <v>4.98</v>
       </c>
       <c r="O32" t="n">
-        <v>5.323</v>
+        <v>5.348</v>
       </c>
       <c r="P32" t="n">
-        <v>5.497</v>
+        <v>5.525</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.26</v>
+        <v>6.29</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.996</v>
+        <v>2.998</v>
       </c>
       <c r="G33" t="n">
-        <v>3.075</v>
+        <v>3.077</v>
       </c>
       <c r="H33" t="n">
-        <v>3.171</v>
+        <v>3.178</v>
       </c>
       <c r="I33" t="n">
-        <v>3.408</v>
+        <v>3.415</v>
       </c>
       <c r="J33" t="n">
-        <v>3.615</v>
+        <v>3.618</v>
       </c>
       <c r="K33" t="n">
-        <v>3.864</v>
+        <v>3.869</v>
       </c>
       <c r="L33" t="n">
-        <v>3.894</v>
+        <v>3.902</v>
       </c>
       <c r="M33" t="n">
-        <v>3.988</v>
+        <v>4.008</v>
       </c>
       <c r="N33" t="n">
-        <v>3.975</v>
+        <v>4</v>
       </c>
       <c r="O33" t="n">
-        <v>4.032</v>
+        <v>4.057</v>
       </c>
       <c r="P33" t="n">
-        <v>4.067</v>
+        <v>4.096</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.515</v>
+        <v>4.546</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.055</v>
+        <v>3.057</v>
       </c>
       <c r="G34" t="n">
-        <v>3.128</v>
+        <v>3.129</v>
       </c>
       <c r="H34" t="n">
-        <v>3.231</v>
+        <v>3.238</v>
       </c>
       <c r="I34" t="n">
-        <v>3.476</v>
+        <v>3.483</v>
       </c>
       <c r="J34" t="n">
-        <v>3.687</v>
+        <v>3.69</v>
       </c>
       <c r="K34" t="n">
-        <v>3.941</v>
+        <v>3.946</v>
       </c>
       <c r="L34" t="n">
-        <v>3.974</v>
+        <v>3.981</v>
       </c>
       <c r="M34" t="n">
-        <v>4.078</v>
+        <v>4.098</v>
       </c>
       <c r="N34" t="n">
-        <v>4.081</v>
+        <v>4.105</v>
       </c>
       <c r="O34" t="n">
-        <v>4.201</v>
+        <v>4.225</v>
       </c>
       <c r="P34" t="n">
-        <v>4.361</v>
+        <v>4.391</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.216</v>
+        <v>5.247</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.03</v>
+        <v>3.031</v>
       </c>
       <c r="G35" t="n">
-        <v>3.101</v>
+        <v>3.103</v>
       </c>
       <c r="H35" t="n">
-        <v>3.198</v>
+        <v>3.206</v>
       </c>
       <c r="I35" t="n">
-        <v>3.443</v>
+        <v>3.45</v>
       </c>
       <c r="J35" t="n">
-        <v>3.654</v>
+        <v>3.657</v>
       </c>
       <c r="K35" t="n">
-        <v>3.896</v>
+        <v>3.9</v>
       </c>
       <c r="L35" t="n">
-        <v>3.928</v>
+        <v>3.936</v>
       </c>
       <c r="M35" t="n">
-        <v>4.025</v>
+        <v>4.045</v>
       </c>
       <c r="N35" t="n">
-        <v>4.017</v>
+        <v>4.041</v>
       </c>
       <c r="O35" t="n">
-        <v>4.099</v>
+        <v>4.123</v>
       </c>
       <c r="P35" t="n">
-        <v>4.164</v>
+        <v>4.193</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.852</v>
+        <v>4.883</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.94</v>
+        <v>2.942</v>
       </c>
       <c r="G36" t="n">
-        <v>3.02</v>
+        <v>3.021</v>
       </c>
       <c r="H36" t="n">
-        <v>3.1</v>
+        <v>3.108</v>
       </c>
       <c r="I36" t="n">
-        <v>3.338</v>
+        <v>3.344</v>
       </c>
       <c r="J36" t="n">
-        <v>3.552</v>
+        <v>3.555</v>
       </c>
       <c r="K36" t="n">
-        <v>3.786</v>
+        <v>3.79</v>
       </c>
       <c r="L36" t="n">
-        <v>3.817</v>
+        <v>3.824</v>
       </c>
       <c r="M36" t="n">
-        <v>3.889</v>
+        <v>3.907</v>
       </c>
       <c r="N36" t="n">
-        <v>3.882</v>
+        <v>3.905</v>
       </c>
       <c r="O36" t="n">
-        <v>3.943</v>
+        <v>3.967</v>
       </c>
       <c r="P36" t="n">
-        <v>3.966</v>
+        <v>3.995</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.232</v>
+        <v>4.263</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3110,37 +3110,37 @@
         <v>3.78</v>
       </c>
       <c r="G37" t="n">
-        <v>4.246</v>
+        <v>4.247</v>
       </c>
       <c r="H37" t="n">
-        <v>4.735</v>
+        <v>4.741</v>
       </c>
       <c r="I37" t="n">
-        <v>5.119</v>
+        <v>5.125</v>
       </c>
       <c r="J37" t="n">
-        <v>5.883</v>
+        <v>5.886</v>
       </c>
       <c r="K37" t="n">
-        <v>6.791</v>
+        <v>6.795</v>
       </c>
       <c r="L37" t="n">
-        <v>7.098</v>
+        <v>7.104</v>
       </c>
       <c r="M37" t="n">
-        <v>7.46</v>
+        <v>7.479</v>
       </c>
       <c r="N37" t="n">
-        <v>7.606</v>
+        <v>7.629</v>
       </c>
       <c r="O37" t="n">
-        <v>7.794</v>
+        <v>7.816</v>
       </c>
       <c r="P37" t="n">
-        <v>7.825</v>
+        <v>7.851</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.263</v>
+        <v>8.294</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.835</v>
+        <v>4.836</v>
       </c>
       <c r="G38" t="n">
-        <v>5.556</v>
+        <v>5.557</v>
       </c>
       <c r="H38" t="n">
-        <v>6.259</v>
+        <v>6.265</v>
       </c>
       <c r="I38" t="n">
-        <v>6.799</v>
+        <v>6.805</v>
       </c>
       <c r="J38" t="n">
-        <v>7.823</v>
+        <v>7.826</v>
       </c>
       <c r="K38" t="n">
-        <v>8.906000000000001</v>
+        <v>8.91</v>
       </c>
       <c r="L38" t="n">
-        <v>9.372999999999999</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>9.867000000000001</v>
+        <v>9.885999999999999</v>
       </c>
       <c r="N38" t="n">
-        <v>10.024</v>
+        <v>10.046</v>
       </c>
       <c r="O38" t="n">
-        <v>10.193</v>
+        <v>10.215</v>
       </c>
       <c r="P38" t="n">
-        <v>10.223</v>
+        <v>10.25</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.715</v>
+        <v>10.746</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.156</v>
+        <v>4.157</v>
       </c>
       <c r="G39" t="n">
-        <v>4.754</v>
+        <v>4.755</v>
       </c>
       <c r="H39" t="n">
-        <v>5.324</v>
+        <v>5.33</v>
       </c>
       <c r="I39" t="n">
-        <v>5.803</v>
+        <v>5.809</v>
       </c>
       <c r="J39" t="n">
-        <v>6.695</v>
+        <v>6.698</v>
       </c>
       <c r="K39" t="n">
-        <v>7.739</v>
+        <v>7.744</v>
       </c>
       <c r="L39" t="n">
-        <v>8.132</v>
+        <v>8.138999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.505000000000001</v>
+        <v>8.523999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.651</v>
+        <v>8.673999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.843999999999999</v>
+        <v>8.866</v>
       </c>
       <c r="P39" t="n">
-        <v>8.879</v>
+        <v>8.904999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.359</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3329,37 +3329,37 @@
         <v>3.301</v>
       </c>
       <c r="G40" t="n">
-        <v>3.429</v>
+        <v>3.43</v>
       </c>
       <c r="H40" t="n">
-        <v>3.605</v>
+        <v>3.611</v>
       </c>
       <c r="I40" t="n">
-        <v>3.894</v>
+        <v>3.9</v>
       </c>
       <c r="J40" t="n">
-        <v>4.197</v>
+        <v>4.2</v>
       </c>
       <c r="K40" t="n">
-        <v>4.528</v>
+        <v>4.532</v>
       </c>
       <c r="L40" t="n">
-        <v>4.615</v>
+        <v>4.621</v>
       </c>
       <c r="M40" t="n">
-        <v>4.799</v>
+        <v>4.818</v>
       </c>
       <c r="N40" t="n">
-        <v>4.955</v>
+        <v>4.978</v>
       </c>
       <c r="O40" t="n">
-        <v>5.262</v>
+        <v>5.284</v>
       </c>
       <c r="P40" t="n">
-        <v>5.462</v>
+        <v>5.489</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.25</v>
+        <v>6.281</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3405,34 +3405,34 @@
         <v>3.854</v>
       </c>
       <c r="H41" t="n">
-        <v>4.088</v>
+        <v>4.094</v>
       </c>
       <c r="I41" t="n">
-        <v>4.396</v>
+        <v>4.402</v>
       </c>
       <c r="J41" t="n">
-        <v>4.748</v>
+        <v>4.751</v>
       </c>
       <c r="K41" t="n">
-        <v>5.127</v>
+        <v>5.132</v>
       </c>
       <c r="L41" t="n">
-        <v>5.29</v>
+        <v>5.297</v>
       </c>
       <c r="M41" t="n">
-        <v>5.601</v>
+        <v>5.619</v>
       </c>
       <c r="N41" t="n">
-        <v>5.883</v>
+        <v>5.906</v>
       </c>
       <c r="O41" t="n">
-        <v>6.368</v>
+        <v>6.393</v>
       </c>
       <c r="P41" t="n">
-        <v>6.518</v>
+        <v>6.546</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.297</v>
+        <v>7.328</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.421</v>
+        <v>3.422</v>
       </c>
       <c r="G42" t="n">
         <v>3.578</v>
       </c>
       <c r="H42" t="n">
-        <v>3.78</v>
+        <v>3.786</v>
       </c>
       <c r="I42" t="n">
-        <v>4.083</v>
+        <v>4.089</v>
       </c>
       <c r="J42" t="n">
-        <v>4.398</v>
+        <v>4.401</v>
       </c>
       <c r="K42" t="n">
-        <v>4.749</v>
+        <v>4.753</v>
       </c>
       <c r="L42" t="n">
-        <v>4.849</v>
+        <v>4.856</v>
       </c>
       <c r="M42" t="n">
-        <v>5.106</v>
+        <v>5.125</v>
       </c>
       <c r="N42" t="n">
-        <v>5.368</v>
+        <v>5.392</v>
       </c>
       <c r="O42" t="n">
-        <v>5.747</v>
+        <v>5.772</v>
       </c>
       <c r="P42" t="n">
-        <v>5.961</v>
+        <v>5.989</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.762</v>
+        <v>6.793</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.144</v>
+        <v>3.146</v>
       </c>
       <c r="G43" t="n">
-        <v>3.257</v>
+        <v>3.258</v>
       </c>
       <c r="H43" t="n">
-        <v>3.37</v>
+        <v>3.378</v>
       </c>
       <c r="I43" t="n">
-        <v>3.618</v>
+        <v>3.625</v>
       </c>
       <c r="J43" t="n">
-        <v>3.842</v>
+        <v>3.845</v>
       </c>
       <c r="K43" t="n">
-        <v>4.096</v>
+        <v>4.101</v>
       </c>
       <c r="L43" t="n">
-        <v>4.136</v>
+        <v>4.143</v>
       </c>
       <c r="M43" t="n">
-        <v>4.241</v>
+        <v>4.261</v>
       </c>
       <c r="N43" t="n">
-        <v>4.245</v>
+        <v>4.269</v>
       </c>
       <c r="O43" t="n">
-        <v>4.345</v>
+        <v>4.369</v>
       </c>
       <c r="P43" t="n">
-        <v>4.433</v>
+        <v>4.462</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.125</v>
+        <v>5.156</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.018</v>
+        <v>3.02</v>
       </c>
       <c r="G44" t="n">
         <v>3.13</v>
       </c>
       <c r="H44" t="n">
-        <v>3.225</v>
+        <v>3.232</v>
       </c>
       <c r="I44" t="n">
-        <v>3.466</v>
+        <v>3.472</v>
       </c>
       <c r="J44" t="n">
-        <v>3.694</v>
+        <v>3.697</v>
       </c>
       <c r="K44" t="n">
-        <v>3.936</v>
+        <v>3.941</v>
       </c>
       <c r="L44" t="n">
-        <v>3.977</v>
+        <v>3.984</v>
       </c>
       <c r="M44" t="n">
-        <v>4.057</v>
+        <v>4.076</v>
       </c>
       <c r="N44" t="n">
-        <v>4.064</v>
+        <v>4.087</v>
       </c>
       <c r="O44" t="n">
-        <v>4.141</v>
+        <v>4.167</v>
       </c>
       <c r="P44" t="n">
-        <v>4.197</v>
+        <v>4.225</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.496</v>
+        <v>4.527</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-08 ~ 2026-04-08
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.255</v>
+        <v>3.251</v>
       </c>
       <c r="G2" t="n">
-        <v>3.479</v>
+        <v>3.462</v>
       </c>
       <c r="H2" t="n">
-        <v>3.63</v>
+        <v>3.582</v>
       </c>
       <c r="I2" t="n">
-        <v>3.856</v>
+        <v>3.776</v>
       </c>
       <c r="J2" t="n">
-        <v>4.078</v>
+        <v>3.964</v>
       </c>
       <c r="K2" t="n">
-        <v>4.475</v>
+        <v>4.356</v>
       </c>
       <c r="L2" t="n">
-        <v>4.644</v>
+        <v>4.526</v>
       </c>
       <c r="M2" t="n">
-        <v>4.942</v>
+        <v>4.826</v>
       </c>
       <c r="N2" t="n">
-        <v>5.194</v>
+        <v>5.063</v>
       </c>
       <c r="O2" t="n">
-        <v>5.41</v>
+        <v>5.279</v>
       </c>
       <c r="P2" t="n">
-        <v>5.585</v>
+        <v>5.464</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.225</v>
+        <v>6.102</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.279</v>
+        <v>4.275</v>
       </c>
       <c r="G3" t="n">
-        <v>4.684</v>
+        <v>4.667</v>
       </c>
       <c r="H3" t="n">
-        <v>4.867</v>
+        <v>4.82</v>
       </c>
       <c r="I3" t="n">
-        <v>5.093</v>
+        <v>5.014</v>
       </c>
       <c r="J3" t="n">
-        <v>5.325</v>
+        <v>5.211</v>
       </c>
       <c r="K3" t="n">
-        <v>5.79</v>
+        <v>5.671</v>
       </c>
       <c r="L3" t="n">
-        <v>6.029</v>
+        <v>5.911</v>
       </c>
       <c r="M3" t="n">
-        <v>6.359</v>
+        <v>6.242</v>
       </c>
       <c r="N3" t="n">
-        <v>6.554</v>
+        <v>6.423</v>
       </c>
       <c r="O3" t="n">
-        <v>6.72</v>
+        <v>6.588</v>
       </c>
       <c r="P3" t="n">
-        <v>6.764</v>
+        <v>6.643</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.293</v>
+        <v>7.17</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.77</v>
+        <v>3.765</v>
       </c>
       <c r="G4" t="n">
-        <v>4.064</v>
+        <v>4.047</v>
       </c>
       <c r="H4" t="n">
-        <v>4.276</v>
+        <v>4.229</v>
       </c>
       <c r="I4" t="n">
-        <v>4.534</v>
+        <v>4.454</v>
       </c>
       <c r="J4" t="n">
-        <v>4.772</v>
+        <v>4.658</v>
       </c>
       <c r="K4" t="n">
-        <v>5.231</v>
+        <v>5.111</v>
       </c>
       <c r="L4" t="n">
-        <v>5.4</v>
+        <v>5.282</v>
       </c>
       <c r="M4" t="n">
-        <v>5.717</v>
+        <v>5.6</v>
       </c>
       <c r="N4" t="n">
-        <v>5.882</v>
+        <v>5.751</v>
       </c>
       <c r="O4" t="n">
-        <v>6.072</v>
+        <v>5.94</v>
       </c>
       <c r="P4" t="n">
-        <v>6.113</v>
+        <v>5.992</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.646</v>
+        <v>6.523</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.965</v>
+        <v>2.961</v>
       </c>
       <c r="G5" t="n">
-        <v>3.03</v>
+        <v>3.013</v>
       </c>
       <c r="H5" t="n">
-        <v>3.133</v>
+        <v>3.085</v>
       </c>
       <c r="I5" t="n">
-        <v>3.428</v>
+        <v>3.348</v>
       </c>
       <c r="J5" t="n">
-        <v>3.648</v>
+        <v>3.535</v>
       </c>
       <c r="K5" t="n">
+        <v>3.785</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3.797</v>
+      </c>
+      <c r="M5" t="n">
         <v>3.904</v>
       </c>
-      <c r="L5" t="n">
-        <v>3.915</v>
-      </c>
-      <c r="M5" t="n">
-        <v>4.02</v>
-      </c>
       <c r="N5" t="n">
-        <v>3.998</v>
+        <v>3.868</v>
       </c>
       <c r="O5" t="n">
-        <v>4.003</v>
+        <v>3.871</v>
       </c>
       <c r="P5" t="n">
-        <v>4.255</v>
+        <v>4.134</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.137</v>
+        <v>5.014</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.005</v>
+        <v>3.001</v>
       </c>
       <c r="G6" t="n">
-        <v>3.083</v>
+        <v>3.065</v>
       </c>
       <c r="H6" t="n">
-        <v>3.202</v>
+        <v>3.154</v>
       </c>
       <c r="I6" t="n">
-        <v>3.502</v>
+        <v>3.422</v>
       </c>
       <c r="J6" t="n">
-        <v>3.733</v>
+        <v>3.62</v>
       </c>
       <c r="K6" t="n">
-        <v>4.007</v>
+        <v>3.887</v>
       </c>
       <c r="L6" t="n">
-        <v>4.029</v>
+        <v>3.912</v>
       </c>
       <c r="M6" t="n">
-        <v>4.168</v>
+        <v>4.051</v>
       </c>
       <c r="N6" t="n">
-        <v>4.168</v>
+        <v>4.038</v>
       </c>
       <c r="O6" t="n">
-        <v>4.278</v>
+        <v>4.147</v>
       </c>
       <c r="P6" t="n">
-        <v>4.687</v>
+        <v>4.566</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.533</v>
+        <v>5.41</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.985</v>
+        <v>2.981</v>
       </c>
       <c r="G7" t="n">
-        <v>3.049</v>
+        <v>3.031</v>
       </c>
       <c r="H7" t="n">
-        <v>3.149</v>
+        <v>3.101</v>
       </c>
       <c r="I7" t="n">
-        <v>3.443</v>
+        <v>3.363</v>
       </c>
       <c r="J7" t="n">
-        <v>3.674</v>
+        <v>3.56</v>
       </c>
       <c r="K7" t="n">
-        <v>3.929</v>
+        <v>3.81</v>
       </c>
       <c r="L7" t="n">
-        <v>3.941</v>
+        <v>3.823</v>
       </c>
       <c r="M7" t="n">
-        <v>4.078</v>
+        <v>3.961</v>
       </c>
       <c r="N7" t="n">
-        <v>4.058</v>
+        <v>3.928</v>
       </c>
       <c r="O7" t="n">
-        <v>4.178</v>
+        <v>4.046</v>
       </c>
       <c r="P7" t="n">
-        <v>4.471</v>
+        <v>4.35</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.301</v>
+        <v>5.178</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.388</v>
+        <v>5.384</v>
       </c>
       <c r="G8" t="n">
-        <v>5.982</v>
+        <v>5.965</v>
       </c>
       <c r="H8" t="n">
-        <v>6.317</v>
+        <v>6.269</v>
       </c>
       <c r="I8" t="n">
-        <v>6.614</v>
+        <v>6.534</v>
       </c>
       <c r="J8" t="n">
-        <v>6.91</v>
+        <v>6.796</v>
       </c>
       <c r="K8" t="n">
-        <v>7.656</v>
+        <v>7.537</v>
       </c>
       <c r="L8" t="n">
-        <v>7.984</v>
+        <v>7.867</v>
       </c>
       <c r="M8" t="n">
-        <v>8.342000000000001</v>
+        <v>8.226000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.475</v>
+        <v>8.343999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>8.727</v>
+        <v>8.595000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>8.869</v>
+        <v>8.749000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.602</v>
+        <v>9.478999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.618</v>
+        <v>2.614</v>
       </c>
       <c r="G9" t="n">
-        <v>2.721</v>
+        <v>2.701</v>
       </c>
       <c r="H9" t="n">
-        <v>2.827</v>
+        <v>2.775</v>
       </c>
       <c r="I9" t="n">
-        <v>2.994</v>
+        <v>2.907</v>
       </c>
       <c r="J9" t="n">
-        <v>3.139</v>
+        <v>3.072</v>
       </c>
       <c r="K9" t="n">
-        <v>3.332</v>
+        <v>3.201</v>
       </c>
       <c r="L9" t="n">
-        <v>3.38</v>
+        <v>3.25</v>
       </c>
       <c r="M9" t="n">
-        <v>3.445</v>
+        <v>3.319</v>
       </c>
       <c r="N9" t="n">
-        <v>3.59</v>
+        <v>3.451</v>
       </c>
       <c r="O9" t="n">
-        <v>3.617</v>
+        <v>3.479</v>
       </c>
       <c r="P9" t="n">
-        <v>3.682</v>
+        <v>3.555</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.755</v>
+        <v>3.632</v>
       </c>
       <c r="R9" t="n">
-        <v>3.766</v>
+        <v>3.649</v>
       </c>
       <c r="S9" t="n">
-        <v>3.725</v>
+        <v>3.612</v>
       </c>
       <c r="T9" t="n">
-        <v>3.637</v>
+        <v>3.53</v>
       </c>
       <c r="U9" t="n">
-        <v>3.542</v>
+        <v>3.434</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.63</v>
+        <v>2.626</v>
       </c>
       <c r="G10" t="n">
-        <v>2.752</v>
+        <v>2.732</v>
       </c>
       <c r="H10" t="n">
-        <v>2.838</v>
+        <v>2.786</v>
       </c>
       <c r="I10" t="n">
-        <v>3.004</v>
+        <v>2.919</v>
       </c>
       <c r="J10" t="n">
-        <v>3.167</v>
+        <v>3.1</v>
       </c>
       <c r="K10" t="n">
-        <v>3.358</v>
+        <v>3.228</v>
       </c>
       <c r="L10" t="n">
-        <v>3.422</v>
+        <v>3.292</v>
       </c>
       <c r="M10" t="n">
-        <v>3.545</v>
+        <v>3.42</v>
       </c>
       <c r="N10" t="n">
-        <v>3.596</v>
+        <v>3.458</v>
       </c>
       <c r="O10" t="n">
-        <v>3.791</v>
+        <v>3.652</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.446</v>
+        <v>2.442</v>
       </c>
       <c r="G11" t="n">
-        <v>2.561</v>
+        <v>2.542</v>
       </c>
       <c r="H11" t="n">
-        <v>2.661</v>
+        <v>2.61</v>
       </c>
       <c r="I11" t="n">
-        <v>2.806</v>
+        <v>2.721</v>
       </c>
       <c r="J11" t="n">
-        <v>2.961</v>
+        <v>2.894</v>
       </c>
       <c r="K11" t="n">
-        <v>3.145</v>
+        <v>3.016</v>
       </c>
       <c r="L11" t="n">
-        <v>3.216</v>
+        <v>3.086</v>
       </c>
       <c r="M11" t="n">
-        <v>3.35</v>
+        <v>3.224</v>
       </c>
       <c r="N11" t="n">
-        <v>3.407</v>
+        <v>3.269</v>
       </c>
       <c r="O11" t="n">
-        <v>3.558</v>
+        <v>3.419</v>
       </c>
       <c r="P11" t="n">
-        <v>3.619</v>
+        <v>3.492</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.958</v>
+        <v>3.835</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.228</v>
+        <v>3.218</v>
       </c>
       <c r="G12" t="n">
-        <v>3.387</v>
+        <v>3.367</v>
       </c>
       <c r="H12" t="n">
-        <v>3.503</v>
+        <v>3.458</v>
       </c>
       <c r="I12" t="n">
-        <v>3.742</v>
+        <v>3.664</v>
       </c>
       <c r="J12" t="n">
-        <v>4.066</v>
+        <v>3.949</v>
       </c>
       <c r="K12" t="n">
-        <v>4.275</v>
+        <v>4.15</v>
       </c>
       <c r="L12" t="n">
-        <v>4.322</v>
+        <v>4.199</v>
       </c>
       <c r="M12" t="n">
-        <v>4.458</v>
+        <v>4.335</v>
       </c>
       <c r="N12" t="n">
-        <v>4.47</v>
+        <v>4.338</v>
       </c>
       <c r="O12" t="n">
-        <v>4.622</v>
+        <v>4.488</v>
       </c>
       <c r="P12" t="n">
-        <v>4.717</v>
+        <v>4.598</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.085</v>
+        <v>4.962</v>
       </c>
       <c r="R12" t="n">
-        <v>5.263</v>
+        <v>5.146</v>
       </c>
       <c r="S12" t="n">
-        <v>5.436</v>
+        <v>5.322</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.982</v>
+        <v>2.972</v>
       </c>
       <c r="G13" t="n">
-        <v>3.078</v>
+        <v>3.057</v>
       </c>
       <c r="H13" t="n">
-        <v>3.171</v>
+        <v>3.125</v>
       </c>
       <c r="I13" t="n">
-        <v>3.389</v>
+        <v>3.312</v>
       </c>
       <c r="J13" t="n">
-        <v>3.703</v>
+        <v>3.586</v>
       </c>
       <c r="K13" t="n">
-        <v>3.908</v>
+        <v>3.784</v>
       </c>
       <c r="L13" t="n">
+        <v>3.839</v>
+      </c>
+      <c r="M13" t="n">
         <v>3.962</v>
       </c>
-      <c r="M13" t="n">
-        <v>4.086</v>
-      </c>
       <c r="N13" t="n">
-        <v>4.098</v>
+        <v>3.966</v>
       </c>
       <c r="O13" t="n">
-        <v>4.248</v>
+        <v>4.114</v>
       </c>
       <c r="P13" t="n">
-        <v>4.309</v>
+        <v>4.19</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.606</v>
+        <v>4.483</v>
       </c>
       <c r="R13" t="n">
-        <v>4.811</v>
+        <v>4.694</v>
       </c>
       <c r="S13" t="n">
-        <v>4.998</v>
+        <v>4.885</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.8</v>
+        <v>2.79</v>
       </c>
       <c r="G14" t="n">
-        <v>2.884</v>
+        <v>2.864</v>
       </c>
       <c r="H14" t="n">
-        <v>2.974</v>
+        <v>2.928</v>
       </c>
       <c r="I14" t="n">
-        <v>3.173</v>
+        <v>3.095</v>
       </c>
       <c r="J14" t="n">
-        <v>3.442</v>
+        <v>3.325</v>
       </c>
       <c r="K14" t="n">
-        <v>3.596</v>
+        <v>3.472</v>
       </c>
       <c r="L14" t="n">
-        <v>3.634</v>
+        <v>3.511</v>
       </c>
       <c r="M14" t="n">
-        <v>3.771</v>
+        <v>3.647</v>
       </c>
       <c r="N14" t="n">
-        <v>3.78</v>
+        <v>3.646</v>
       </c>
       <c r="O14" t="n">
-        <v>3.903</v>
+        <v>3.769</v>
       </c>
       <c r="P14" t="n">
-        <v>3.944</v>
+        <v>3.825</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.195</v>
+        <v>4.072</v>
       </c>
       <c r="R14" t="n">
-        <v>4.326</v>
+        <v>4.209</v>
       </c>
       <c r="S14" t="n">
-        <v>4.451</v>
+        <v>4.338</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.778</v>
+        <v>2.768</v>
       </c>
       <c r="G15" t="n">
-        <v>2.858</v>
+        <v>2.838</v>
       </c>
       <c r="H15" t="n">
-        <v>2.943</v>
+        <v>2.897</v>
       </c>
       <c r="I15" t="n">
-        <v>3.123</v>
+        <v>3.046</v>
       </c>
       <c r="J15" t="n">
-        <v>3.379</v>
+        <v>3.262</v>
       </c>
       <c r="K15" t="n">
+        <v>3.426</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3.445</v>
+      </c>
+      <c r="M15" t="n">
+        <v>3.559</v>
+      </c>
+      <c r="N15" t="n">
         <v>3.55</v>
       </c>
-      <c r="L15" t="n">
-        <v>3.568</v>
-      </c>
-      <c r="M15" t="n">
-        <v>3.683</v>
-      </c>
-      <c r="N15" t="n">
-        <v>3.683</v>
-      </c>
       <c r="O15" t="n">
-        <v>3.826</v>
+        <v>3.692</v>
       </c>
       <c r="P15" t="n">
-        <v>3.84</v>
+        <v>3.722</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.1</v>
+        <v>3.977</v>
       </c>
       <c r="R15" t="n">
-        <v>4.222</v>
+        <v>4.106</v>
       </c>
       <c r="S15" t="n">
-        <v>4.346</v>
+        <v>4.233</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.778</v>
+        <v>2.768</v>
       </c>
       <c r="G16" t="n">
-        <v>2.858</v>
+        <v>2.838</v>
       </c>
       <c r="H16" t="n">
-        <v>2.943</v>
+        <v>2.897</v>
       </c>
       <c r="I16" t="n">
-        <v>3.123</v>
+        <v>3.046</v>
       </c>
       <c r="J16" t="n">
-        <v>3.379</v>
+        <v>3.262</v>
       </c>
       <c r="K16" t="n">
-        <v>3.55</v>
+        <v>3.426</v>
       </c>
       <c r="L16" t="n">
-        <v>3.568</v>
+        <v>3.445</v>
       </c>
       <c r="M16" t="n">
-        <v>3.683</v>
+        <v>3.559</v>
       </c>
       <c r="N16" t="n">
-        <v>3.686</v>
+        <v>3.553</v>
       </c>
       <c r="O16" t="n">
-        <v>3.832</v>
+        <v>3.698</v>
       </c>
       <c r="P16" t="n">
-        <v>3.863</v>
+        <v>3.745</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.127</v>
+        <v>4.004</v>
       </c>
       <c r="R16" t="n">
-        <v>4.25</v>
+        <v>4.133</v>
       </c>
       <c r="S16" t="n">
-        <v>4.375</v>
+        <v>4.262</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.692</v>
+        <v>2.688</v>
       </c>
       <c r="G17" t="n">
-        <v>2.844</v>
+        <v>2.824</v>
       </c>
       <c r="H17" t="n">
-        <v>2.932</v>
+        <v>2.88</v>
       </c>
       <c r="I17" t="n">
-        <v>3.087</v>
+        <v>3.001</v>
       </c>
       <c r="J17" t="n">
-        <v>3.235</v>
+        <v>3.169</v>
       </c>
       <c r="K17" t="n">
-        <v>3.431</v>
+        <v>3.301</v>
       </c>
       <c r="L17" t="n">
-        <v>3.499</v>
+        <v>3.369</v>
       </c>
       <c r="M17" t="n">
-        <v>3.665</v>
+        <v>3.54</v>
       </c>
       <c r="N17" t="n">
-        <v>3.698</v>
+        <v>3.56</v>
       </c>
       <c r="O17" t="n">
-        <v>3.826</v>
+        <v>3.687</v>
       </c>
       <c r="P17" t="n">
-        <v>3.9</v>
+        <v>3.772</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.693</v>
+        <v>2.689</v>
       </c>
       <c r="G18" t="n">
-        <v>2.846</v>
+        <v>2.825</v>
       </c>
       <c r="H18" t="n">
-        <v>2.933</v>
+        <v>2.881</v>
       </c>
       <c r="I18" t="n">
-        <v>3.087</v>
+        <v>3</v>
       </c>
       <c r="J18" t="n">
-        <v>3.235</v>
+        <v>3.169</v>
       </c>
       <c r="K18" t="n">
-        <v>3.433</v>
+        <v>3.303</v>
       </c>
       <c r="L18" t="n">
-        <v>3.498</v>
+        <v>3.369</v>
       </c>
       <c r="M18" t="n">
-        <v>3.665</v>
+        <v>3.54</v>
       </c>
       <c r="N18" t="n">
-        <v>3.697</v>
+        <v>3.559</v>
       </c>
       <c r="O18" t="n">
-        <v>3.825</v>
+        <v>3.685</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.789</v>
+        <v>2.779</v>
       </c>
       <c r="G19" t="n">
-        <v>2.875</v>
+        <v>2.855</v>
       </c>
       <c r="H19" t="n">
-        <v>2.964</v>
+        <v>2.918</v>
       </c>
       <c r="I19" t="n">
-        <v>3.157</v>
+        <v>3.08</v>
       </c>
       <c r="J19" t="n">
-        <v>3.425</v>
+        <v>3.309</v>
       </c>
       <c r="K19" t="n">
-        <v>3.594</v>
+        <v>3.469</v>
       </c>
       <c r="L19" t="n">
-        <v>3.631</v>
+        <v>3.508</v>
       </c>
       <c r="M19" t="n">
-        <v>3.758</v>
+        <v>3.634</v>
       </c>
       <c r="N19" t="n">
-        <v>3.767</v>
+        <v>3.634</v>
       </c>
       <c r="O19" t="n">
-        <v>3.88</v>
+        <v>3.746</v>
       </c>
       <c r="P19" t="n">
-        <v>3.906</v>
+        <v>3.788</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.146</v>
+        <v>4.023</v>
       </c>
       <c r="R19" t="n">
-        <v>4.276</v>
+        <v>4.159</v>
       </c>
       <c r="S19" t="n">
-        <v>4.39</v>
+        <v>4.277</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.573</v>
+        <v>2.569</v>
       </c>
       <c r="G20" t="n">
-        <v>2.658</v>
+        <v>2.639</v>
       </c>
       <c r="H20" t="n">
-        <v>2.737</v>
+        <v>2.687</v>
       </c>
       <c r="I20" t="n">
-        <v>2.939</v>
+        <v>2.849</v>
       </c>
       <c r="J20" t="n">
-        <v>3.206</v>
+        <v>3.08</v>
       </c>
       <c r="K20" t="n">
-        <v>3.368</v>
+        <v>3.235</v>
       </c>
       <c r="L20" t="n">
-        <v>3.397</v>
+        <v>3.268</v>
       </c>
       <c r="M20" t="n">
-        <v>3.49</v>
+        <v>3.363</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.878</v>
+        <v>2.874</v>
       </c>
       <c r="G21" t="n">
-        <v>2.975</v>
+        <v>2.956</v>
       </c>
       <c r="H21" t="n">
-        <v>3.11</v>
+        <v>3.067</v>
       </c>
       <c r="I21" t="n">
-        <v>3.301</v>
+        <v>3.224</v>
       </c>
       <c r="J21" t="n">
-        <v>3.554</v>
+        <v>3.44</v>
       </c>
       <c r="K21" t="n">
-        <v>3.827</v>
+        <v>3.704</v>
       </c>
       <c r="L21" t="n">
-        <v>3.898</v>
+        <v>3.774</v>
       </c>
       <c r="M21" t="n">
-        <v>4.013</v>
+        <v>3.891</v>
       </c>
       <c r="N21" t="n">
-        <v>4.026</v>
+        <v>3.899</v>
       </c>
       <c r="O21" t="n">
-        <v>4.116</v>
+        <v>3.984</v>
       </c>
       <c r="P21" t="n">
-        <v>4.172</v>
+        <v>4.053</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.303</v>
+        <v>4.182</v>
       </c>
       <c r="R21" t="n">
-        <v>4.325</v>
+        <v>4.206</v>
       </c>
       <c r="S21" t="n">
-        <v>4.351</v>
+        <v>4.237</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.825</v>
+        <v>2.822</v>
       </c>
       <c r="G22" t="n">
-        <v>2.922</v>
+        <v>2.903</v>
       </c>
       <c r="H22" t="n">
-        <v>3.045</v>
+        <v>3.001</v>
       </c>
       <c r="I22" t="n">
-        <v>3.219</v>
+        <v>3.142</v>
       </c>
       <c r="J22" t="n">
-        <v>3.439</v>
+        <v>3.324</v>
       </c>
       <c r="K22" t="n">
-        <v>3.707</v>
+        <v>3.585</v>
       </c>
       <c r="L22" t="n">
-        <v>3.767</v>
+        <v>3.643</v>
       </c>
       <c r="M22" t="n">
-        <v>3.885</v>
+        <v>3.763</v>
       </c>
       <c r="N22" t="n">
-        <v>3.899</v>
+        <v>3.771</v>
       </c>
       <c r="O22" t="n">
-        <v>3.985</v>
+        <v>3.853</v>
       </c>
       <c r="P22" t="n">
-        <v>4.035</v>
+        <v>3.915</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.161</v>
+        <v>4.041</v>
       </c>
       <c r="R22" t="n">
-        <v>4.169</v>
+        <v>4.052</v>
       </c>
       <c r="S22" t="n">
-        <v>4.194</v>
+        <v>4.081</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.778</v>
+        <v>2.774</v>
       </c>
       <c r="G23" t="n">
-        <v>2.876</v>
+        <v>2.856</v>
       </c>
       <c r="H23" t="n">
-        <v>2.983</v>
+        <v>2.94</v>
       </c>
       <c r="I23" t="n">
-        <v>3.172</v>
+        <v>3.095</v>
       </c>
       <c r="J23" t="n">
-        <v>3.385</v>
+        <v>3.27</v>
       </c>
       <c r="K23" t="n">
-        <v>3.627</v>
+        <v>3.504</v>
       </c>
       <c r="L23" t="n">
-        <v>3.678</v>
+        <v>3.554</v>
       </c>
       <c r="M23" t="n">
-        <v>3.789</v>
+        <v>3.667</v>
       </c>
       <c r="N23" t="n">
-        <v>3.794</v>
+        <v>3.667</v>
       </c>
       <c r="O23" t="n">
-        <v>3.859</v>
+        <v>3.727</v>
       </c>
       <c r="P23" t="n">
-        <v>3.895</v>
+        <v>3.777</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.971</v>
+        <v>3.851</v>
       </c>
       <c r="R23" t="n">
-        <v>3.952</v>
+        <v>3.835</v>
       </c>
       <c r="S23" t="n">
-        <v>3.948</v>
+        <v>3.835</v>
       </c>
       <c r="T23" t="n">
-        <v>3.849</v>
+        <v>3.742</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.707</v>
+        <v>2.706</v>
       </c>
       <c r="G24" t="n">
-        <v>2.79</v>
+        <v>2.771</v>
       </c>
       <c r="H24" t="n">
-        <v>2.885</v>
+        <v>2.842</v>
       </c>
       <c r="I24" t="n">
-        <v>3.082</v>
+        <v>3.005</v>
       </c>
       <c r="J24" t="n">
-        <v>3.286</v>
+        <v>3.171</v>
       </c>
       <c r="K24" t="n">
-        <v>3.512</v>
+        <v>3.389</v>
       </c>
       <c r="L24" t="n">
-        <v>3.551</v>
+        <v>3.427</v>
       </c>
       <c r="M24" t="n">
-        <v>3.645</v>
+        <v>3.523</v>
       </c>
       <c r="N24" t="n">
-        <v>3.666</v>
+        <v>3.538</v>
       </c>
       <c r="O24" t="n">
-        <v>3.811</v>
+        <v>3.678</v>
       </c>
       <c r="P24" t="n">
-        <v>3.834</v>
+        <v>3.716</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.892</v>
+        <v>3.771</v>
       </c>
       <c r="R24" t="n">
-        <v>3.872</v>
+        <v>3.755</v>
       </c>
       <c r="S24" t="n">
-        <v>3.864</v>
+        <v>3.751</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.771</v>
+        <v>2.767</v>
       </c>
       <c r="G25" t="n">
-        <v>2.875</v>
+        <v>2.855</v>
       </c>
       <c r="H25" t="n">
-        <v>2.987</v>
+        <v>2.943</v>
       </c>
       <c r="I25" t="n">
-        <v>3.18</v>
+        <v>3.103</v>
       </c>
       <c r="J25" t="n">
-        <v>3.401</v>
+        <v>3.286</v>
       </c>
       <c r="K25" t="n">
-        <v>3.656</v>
+        <v>3.533</v>
       </c>
       <c r="L25" t="n">
-        <v>3.707</v>
+        <v>3.583</v>
       </c>
       <c r="M25" t="n">
-        <v>3.816</v>
+        <v>3.695</v>
       </c>
       <c r="N25" t="n">
-        <v>3.821</v>
+        <v>3.694</v>
       </c>
       <c r="O25" t="n">
-        <v>3.888</v>
+        <v>3.756</v>
       </c>
       <c r="P25" t="n">
-        <v>3.918</v>
+        <v>3.799</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.003</v>
+        <v>3.883</v>
       </c>
       <c r="R25" t="n">
-        <v>3.976</v>
+        <v>3.859</v>
       </c>
       <c r="S25" t="n">
-        <v>3.971</v>
+        <v>3.858</v>
       </c>
       <c r="T25" t="n">
-        <v>3.867</v>
+        <v>3.76</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.09</v>
+        <v>3.085</v>
       </c>
       <c r="G26" t="n">
-        <v>3.235</v>
+        <v>3.213</v>
       </c>
       <c r="H26" t="n">
-        <v>3.43</v>
+        <v>3.386</v>
       </c>
       <c r="I26" t="n">
-        <v>3.707</v>
+        <v>3.627</v>
       </c>
       <c r="J26" t="n">
-        <v>4.046</v>
+        <v>3.93</v>
       </c>
       <c r="K26" t="n">
-        <v>4.433</v>
+        <v>4.31</v>
       </c>
       <c r="L26" t="n">
-        <v>4.527</v>
+        <v>4.41</v>
       </c>
       <c r="M26" t="n">
-        <v>4.718</v>
+        <v>4.6</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.947</v>
+        <v>4.814</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.886</v>
+        <v>2.879</v>
       </c>
       <c r="G27" t="n">
-        <v>2.969</v>
+        <v>2.945</v>
       </c>
       <c r="H27" t="n">
-        <v>3.071</v>
+        <v>3.027</v>
       </c>
       <c r="I27" t="n">
-        <v>3.292</v>
+        <v>3.213</v>
       </c>
       <c r="J27" t="n">
-        <v>3.553</v>
+        <v>3.438</v>
       </c>
       <c r="K27" t="n">
-        <v>3.762</v>
+        <v>3.638</v>
       </c>
       <c r="L27" t="n">
-        <v>3.808</v>
+        <v>3.686</v>
       </c>
       <c r="M27" t="n">
-        <v>3.933</v>
+        <v>3.814</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.046</v>
+        <v>3.911</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.985</v>
+        <v>2.978</v>
       </c>
       <c r="G28" t="n">
-        <v>3.073</v>
+        <v>3.05</v>
       </c>
       <c r="H28" t="n">
-        <v>3.194</v>
+        <v>3.15</v>
       </c>
       <c r="I28" t="n">
-        <v>3.428</v>
+        <v>3.349</v>
       </c>
       <c r="J28" t="n">
-        <v>3.727</v>
+        <v>3.611</v>
       </c>
       <c r="K28" t="n">
-        <v>3.954</v>
+        <v>3.831</v>
       </c>
       <c r="L28" t="n">
-        <v>4.011</v>
+        <v>3.889</v>
       </c>
       <c r="M28" t="n">
-        <v>4.146</v>
+        <v>4.026</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.34</v>
+        <v>4.205</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.845</v>
+        <v>2.838</v>
       </c>
       <c r="G29" t="n">
-        <v>2.929</v>
+        <v>2.906</v>
       </c>
       <c r="H29" t="n">
-        <v>3.017</v>
+        <v>2.972</v>
       </c>
       <c r="I29" t="n">
-        <v>3.224</v>
+        <v>3.145</v>
       </c>
       <c r="J29" t="n">
-        <v>3.466</v>
+        <v>3.35</v>
       </c>
       <c r="K29" t="n">
-        <v>3.659</v>
+        <v>3.536</v>
       </c>
       <c r="L29" t="n">
-        <v>3.692</v>
+        <v>3.57</v>
       </c>
       <c r="M29" t="n">
-        <v>3.795</v>
+        <v>3.675</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.904</v>
+        <v>3.77</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.109</v>
+        <v>3.103</v>
       </c>
       <c r="G30" t="n">
-        <v>3.191</v>
+        <v>3.17</v>
       </c>
       <c r="H30" t="n">
-        <v>3.351</v>
+        <v>3.309</v>
       </c>
       <c r="I30" t="n">
-        <v>3.625</v>
+        <v>3.545</v>
       </c>
       <c r="J30" t="n">
-        <v>3.907</v>
+        <v>3.791</v>
       </c>
       <c r="K30" t="n">
-        <v>4.227</v>
+        <v>4.102</v>
       </c>
       <c r="L30" t="n">
-        <v>4.297</v>
+        <v>4.178</v>
       </c>
       <c r="M30" t="n">
-        <v>4.477</v>
+        <v>4.359</v>
       </c>
       <c r="N30" t="n">
-        <v>4.62</v>
+        <v>4.489</v>
       </c>
       <c r="O30" t="n">
-        <v>4.906</v>
+        <v>4.773</v>
       </c>
       <c r="P30" t="n">
-        <v>5.068</v>
+        <v>4.944</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.829</v>
+        <v>5.706</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.435</v>
+        <v>3.429</v>
       </c>
       <c r="G31" t="n">
-        <v>3.551</v>
+        <v>3.53</v>
       </c>
       <c r="H31" t="n">
-        <v>3.764</v>
+        <v>3.721</v>
       </c>
       <c r="I31" t="n">
-        <v>4.053</v>
+        <v>3.973</v>
       </c>
       <c r="J31" t="n">
-        <v>4.395</v>
+        <v>4.279</v>
       </c>
       <c r="K31" t="n">
-        <v>4.76</v>
+        <v>4.634</v>
       </c>
       <c r="L31" t="n">
-        <v>4.907</v>
+        <v>4.788</v>
       </c>
       <c r="M31" t="n">
-        <v>5.206</v>
+        <v>5.088</v>
       </c>
       <c r="N31" t="n">
-        <v>5.476</v>
+        <v>5.345</v>
       </c>
       <c r="O31" t="n">
-        <v>5.936</v>
+        <v>5.804</v>
       </c>
       <c r="P31" t="n">
-        <v>6.054</v>
+        <v>5.93</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.803</v>
+        <v>6.68</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.207</v>
+        <v>3.2</v>
       </c>
       <c r="G32" t="n">
-        <v>3.307</v>
+        <v>3.286</v>
       </c>
       <c r="H32" t="n">
-        <v>3.494</v>
+        <v>3.452</v>
       </c>
       <c r="I32" t="n">
-        <v>3.784</v>
+        <v>3.704</v>
       </c>
       <c r="J32" t="n">
-        <v>4.084</v>
+        <v>3.968</v>
       </c>
       <c r="K32" t="n">
-        <v>4.413</v>
+        <v>4.287</v>
       </c>
       <c r="L32" t="n">
-        <v>4.5</v>
+        <v>4.381</v>
       </c>
       <c r="M32" t="n">
-        <v>4.749</v>
+        <v>4.631</v>
       </c>
       <c r="N32" t="n">
-        <v>4.98</v>
+        <v>4.849</v>
       </c>
       <c r="O32" t="n">
-        <v>5.348</v>
+        <v>5.216</v>
       </c>
       <c r="P32" t="n">
-        <v>5.525</v>
+        <v>5.401</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.29</v>
+        <v>6.168</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.998</v>
+        <v>2.992</v>
       </c>
       <c r="G33" t="n">
-        <v>3.077</v>
+        <v>3.055</v>
       </c>
       <c r="H33" t="n">
-        <v>3.178</v>
+        <v>3.135</v>
       </c>
       <c r="I33" t="n">
-        <v>3.415</v>
+        <v>3.335</v>
       </c>
       <c r="J33" t="n">
-        <v>3.618</v>
+        <v>3.502</v>
       </c>
       <c r="K33" t="n">
-        <v>3.869</v>
+        <v>3.744</v>
       </c>
       <c r="L33" t="n">
-        <v>3.902</v>
+        <v>3.784</v>
       </c>
       <c r="M33" t="n">
-        <v>4.008</v>
+        <v>3.89</v>
       </c>
       <c r="N33" t="n">
-        <v>4</v>
+        <v>3.87</v>
       </c>
       <c r="O33" t="n">
-        <v>4.057</v>
+        <v>3.925</v>
       </c>
       <c r="P33" t="n">
-        <v>4.096</v>
+        <v>3.972</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.546</v>
+        <v>4.423</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.057</v>
+        <v>3.051</v>
       </c>
       <c r="G34" t="n">
-        <v>3.129</v>
+        <v>3.107</v>
       </c>
       <c r="H34" t="n">
-        <v>3.238</v>
+        <v>3.195</v>
       </c>
       <c r="I34" t="n">
-        <v>3.483</v>
+        <v>3.403</v>
       </c>
       <c r="J34" t="n">
-        <v>3.69</v>
+        <v>3.574</v>
       </c>
       <c r="K34" t="n">
-        <v>3.946</v>
+        <v>3.821</v>
       </c>
       <c r="L34" t="n">
-        <v>3.981</v>
+        <v>3.863</v>
       </c>
       <c r="M34" t="n">
-        <v>4.098</v>
+        <v>3.98</v>
       </c>
       <c r="N34" t="n">
-        <v>4.105</v>
+        <v>3.975</v>
       </c>
       <c r="O34" t="n">
-        <v>4.225</v>
+        <v>4.093</v>
       </c>
       <c r="P34" t="n">
-        <v>4.391</v>
+        <v>4.267</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.247</v>
+        <v>5.124</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.031</v>
+        <v>3.025</v>
       </c>
       <c r="G35" t="n">
-        <v>3.103</v>
+        <v>3.081</v>
       </c>
       <c r="H35" t="n">
-        <v>3.206</v>
+        <v>3.162</v>
       </c>
       <c r="I35" t="n">
-        <v>3.45</v>
+        <v>3.37</v>
       </c>
       <c r="J35" t="n">
-        <v>3.657</v>
+        <v>3.541</v>
       </c>
       <c r="K35" t="n">
-        <v>3.9</v>
+        <v>3.775</v>
       </c>
       <c r="L35" t="n">
-        <v>3.936</v>
+        <v>3.818</v>
       </c>
       <c r="M35" t="n">
-        <v>4.045</v>
+        <v>3.927</v>
       </c>
       <c r="N35" t="n">
-        <v>4.041</v>
+        <v>3.911</v>
       </c>
       <c r="O35" t="n">
-        <v>4.123</v>
+        <v>3.991</v>
       </c>
       <c r="P35" t="n">
-        <v>4.193</v>
+        <v>4.069</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.883</v>
+        <v>4.76</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.942</v>
+        <v>2.936</v>
       </c>
       <c r="G36" t="n">
-        <v>3.021</v>
+        <v>2.999</v>
       </c>
       <c r="H36" t="n">
-        <v>3.108</v>
+        <v>3.064</v>
       </c>
       <c r="I36" t="n">
-        <v>3.344</v>
+        <v>3.264</v>
       </c>
       <c r="J36" t="n">
-        <v>3.555</v>
+        <v>3.439</v>
       </c>
       <c r="K36" t="n">
+        <v>3.667</v>
+      </c>
+      <c r="L36" t="n">
+        <v>3.708</v>
+      </c>
+      <c r="M36" t="n">
         <v>3.79</v>
       </c>
-      <c r="L36" t="n">
-        <v>3.824</v>
-      </c>
-      <c r="M36" t="n">
-        <v>3.907</v>
-      </c>
       <c r="N36" t="n">
-        <v>3.905</v>
+        <v>3.775</v>
       </c>
       <c r="O36" t="n">
-        <v>3.967</v>
+        <v>3.835</v>
       </c>
       <c r="P36" t="n">
-        <v>3.995</v>
+        <v>3.871</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.263</v>
+        <v>4.14</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.78</v>
+        <v>3.774</v>
       </c>
       <c r="G37" t="n">
-        <v>4.247</v>
+        <v>4.225</v>
       </c>
       <c r="H37" t="n">
-        <v>4.741</v>
+        <v>4.699</v>
       </c>
       <c r="I37" t="n">
-        <v>5.125</v>
+        <v>5.045</v>
       </c>
       <c r="J37" t="n">
-        <v>5.886</v>
+        <v>5.77</v>
       </c>
       <c r="K37" t="n">
-        <v>6.795</v>
+        <v>6.672</v>
       </c>
       <c r="L37" t="n">
-        <v>7.104</v>
+        <v>6.987</v>
       </c>
       <c r="M37" t="n">
-        <v>7.479</v>
+        <v>7.361</v>
       </c>
       <c r="N37" t="n">
-        <v>7.629</v>
+        <v>7.498</v>
       </c>
       <c r="O37" t="n">
-        <v>7.816</v>
+        <v>7.684</v>
       </c>
       <c r="P37" t="n">
-        <v>7.851</v>
+        <v>7.727</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.294</v>
+        <v>8.170999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.836</v>
+        <v>4.83</v>
       </c>
       <c r="G38" t="n">
-        <v>5.557</v>
+        <v>5.535</v>
       </c>
       <c r="H38" t="n">
-        <v>6.265</v>
+        <v>6.223</v>
       </c>
       <c r="I38" t="n">
-        <v>6.805</v>
+        <v>6.725</v>
       </c>
       <c r="J38" t="n">
-        <v>7.826</v>
+        <v>7.71</v>
       </c>
       <c r="K38" t="n">
-        <v>8.91</v>
+        <v>8.787000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.380000000000001</v>
+        <v>9.263</v>
       </c>
       <c r="M38" t="n">
-        <v>9.885999999999999</v>
+        <v>9.768000000000001</v>
       </c>
       <c r="N38" t="n">
-        <v>10.046</v>
+        <v>9.914999999999999</v>
       </c>
       <c r="O38" t="n">
-        <v>10.215</v>
+        <v>10.083</v>
       </c>
       <c r="P38" t="n">
-        <v>10.25</v>
+        <v>10.126</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.746</v>
+        <v>10.623</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.157</v>
+        <v>4.151</v>
       </c>
       <c r="G39" t="n">
-        <v>4.755</v>
+        <v>4.733</v>
       </c>
       <c r="H39" t="n">
-        <v>5.33</v>
+        <v>5.287</v>
       </c>
       <c r="I39" t="n">
-        <v>5.809</v>
+        <v>5.729</v>
       </c>
       <c r="J39" t="n">
-        <v>6.698</v>
+        <v>6.583</v>
       </c>
       <c r="K39" t="n">
-        <v>7.744</v>
+        <v>7.62</v>
       </c>
       <c r="L39" t="n">
-        <v>8.138999999999999</v>
+        <v>8.022</v>
       </c>
       <c r="M39" t="n">
-        <v>8.523999999999999</v>
+        <v>8.406000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.673999999999999</v>
+        <v>8.542999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.866</v>
+        <v>8.733000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>8.904999999999999</v>
+        <v>8.781000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.390000000000001</v>
+        <v>9.266999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.301</v>
+        <v>3.296</v>
       </c>
       <c r="G40" t="n">
-        <v>3.43</v>
+        <v>3.409</v>
       </c>
       <c r="H40" t="n">
-        <v>3.611</v>
+        <v>3.569</v>
       </c>
       <c r="I40" t="n">
-        <v>3.9</v>
+        <v>3.82</v>
       </c>
       <c r="J40" t="n">
-        <v>4.2</v>
+        <v>4.084</v>
       </c>
       <c r="K40" t="n">
-        <v>4.532</v>
+        <v>4.407</v>
       </c>
       <c r="L40" t="n">
-        <v>4.621</v>
+        <v>4.502</v>
       </c>
       <c r="M40" t="n">
-        <v>4.818</v>
+        <v>4.7</v>
       </c>
       <c r="N40" t="n">
-        <v>4.978</v>
+        <v>4.847</v>
       </c>
       <c r="O40" t="n">
-        <v>5.284</v>
+        <v>5.151</v>
       </c>
       <c r="P40" t="n">
-        <v>5.489</v>
+        <v>5.365</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.281</v>
+        <v>6.157</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.685</v>
+        <v>3.679</v>
       </c>
       <c r="G41" t="n">
-        <v>3.854</v>
+        <v>3.833</v>
       </c>
       <c r="H41" t="n">
-        <v>4.094</v>
+        <v>4.052</v>
       </c>
       <c r="I41" t="n">
-        <v>4.402</v>
+        <v>4.322</v>
       </c>
       <c r="J41" t="n">
-        <v>4.751</v>
+        <v>4.636</v>
       </c>
       <c r="K41" t="n">
-        <v>5.132</v>
+        <v>5.006</v>
       </c>
       <c r="L41" t="n">
-        <v>5.297</v>
+        <v>5.178</v>
       </c>
       <c r="M41" t="n">
-        <v>5.619</v>
+        <v>5.502</v>
       </c>
       <c r="N41" t="n">
-        <v>5.906</v>
+        <v>5.775</v>
       </c>
       <c r="O41" t="n">
-        <v>6.393</v>
+        <v>6.261</v>
       </c>
       <c r="P41" t="n">
-        <v>6.546</v>
+        <v>6.422</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.328</v>
+        <v>7.205</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.422</v>
+        <v>3.416</v>
       </c>
       <c r="G42" t="n">
-        <v>3.578</v>
+        <v>3.557</v>
       </c>
       <c r="H42" t="n">
-        <v>3.786</v>
+        <v>3.744</v>
       </c>
       <c r="I42" t="n">
-        <v>4.089</v>
+        <v>4.009</v>
       </c>
       <c r="J42" t="n">
-        <v>4.401</v>
+        <v>4.285</v>
       </c>
       <c r="K42" t="n">
-        <v>4.753</v>
+        <v>4.628</v>
       </c>
       <c r="L42" t="n">
-        <v>4.856</v>
+        <v>4.737</v>
       </c>
       <c r="M42" t="n">
-        <v>5.125</v>
+        <v>5.007</v>
       </c>
       <c r="N42" t="n">
-        <v>5.392</v>
+        <v>5.261</v>
       </c>
       <c r="O42" t="n">
-        <v>5.772</v>
+        <v>5.64</v>
       </c>
       <c r="P42" t="n">
-        <v>5.989</v>
+        <v>5.865</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.793</v>
+        <v>6.67</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.146</v>
+        <v>3.14</v>
       </c>
       <c r="G43" t="n">
-        <v>3.258</v>
+        <v>3.237</v>
       </c>
       <c r="H43" t="n">
-        <v>3.378</v>
+        <v>3.334</v>
       </c>
       <c r="I43" t="n">
-        <v>3.625</v>
+        <v>3.545</v>
       </c>
       <c r="J43" t="n">
-        <v>3.845</v>
+        <v>3.729</v>
       </c>
       <c r="K43" t="n">
-        <v>4.101</v>
+        <v>3.975</v>
       </c>
       <c r="L43" t="n">
+        <v>4.025</v>
+      </c>
+      <c r="M43" t="n">
         <v>4.143</v>
       </c>
-      <c r="M43" t="n">
-        <v>4.261</v>
-      </c>
       <c r="N43" t="n">
-        <v>4.269</v>
+        <v>4.139</v>
       </c>
       <c r="O43" t="n">
-        <v>4.369</v>
+        <v>4.237</v>
       </c>
       <c r="P43" t="n">
-        <v>4.462</v>
+        <v>4.338</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.156</v>
+        <v>5.033</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46119</v>
+        <v>46120</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.02</v>
+        <v>3.014</v>
       </c>
       <c r="G44" t="n">
-        <v>3.13</v>
+        <v>3.109</v>
       </c>
       <c r="H44" t="n">
-        <v>3.232</v>
+        <v>3.189</v>
       </c>
       <c r="I44" t="n">
-        <v>3.472</v>
+        <v>3.392</v>
       </c>
       <c r="J44" t="n">
-        <v>3.697</v>
+        <v>3.581</v>
       </c>
       <c r="K44" t="n">
-        <v>3.941</v>
+        <v>3.818</v>
       </c>
       <c r="L44" t="n">
-        <v>3.984</v>
+        <v>3.868</v>
       </c>
       <c r="M44" t="n">
-        <v>4.076</v>
+        <v>3.958</v>
       </c>
       <c r="N44" t="n">
-        <v>4.087</v>
+        <v>3.957</v>
       </c>
       <c r="O44" t="n">
-        <v>4.167</v>
+        <v>4.034</v>
       </c>
       <c r="P44" t="n">
-        <v>4.225</v>
+        <v>4.101</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.527</v>
+        <v>4.404</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-15 ~ 2026-04-15
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.239</v>
+        <v>3.234</v>
       </c>
       <c r="G2" t="n">
-        <v>3.449</v>
+        <v>3.444</v>
       </c>
       <c r="H2" t="n">
-        <v>3.586</v>
+        <v>3.582</v>
       </c>
       <c r="I2" t="n">
-        <v>3.809</v>
+        <v>3.804</v>
       </c>
       <c r="J2" t="n">
-        <v>4.001</v>
+        <v>4.004</v>
       </c>
       <c r="K2" t="n">
-        <v>4.379</v>
+        <v>4.376</v>
       </c>
       <c r="L2" t="n">
-        <v>4.545</v>
+        <v>4.543</v>
       </c>
       <c r="M2" t="n">
-        <v>4.851</v>
+        <v>4.847</v>
       </c>
       <c r="N2" t="n">
-        <v>5.108</v>
+        <v>5.107</v>
       </c>
       <c r="O2" t="n">
-        <v>5.323</v>
+        <v>5.327</v>
       </c>
       <c r="P2" t="n">
         <v>5.491</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.122</v>
+        <v>6.125</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.262</v>
+        <v>4.257</v>
       </c>
       <c r="G3" t="n">
-        <v>4.653</v>
+        <v>4.648</v>
       </c>
       <c r="H3" t="n">
-        <v>4.824</v>
+        <v>4.82</v>
       </c>
       <c r="I3" t="n">
-        <v>5.047</v>
+        <v>5.041</v>
       </c>
       <c r="J3" t="n">
-        <v>5.248</v>
+        <v>5.25</v>
       </c>
       <c r="K3" t="n">
-        <v>5.694</v>
+        <v>5.691</v>
       </c>
       <c r="L3" t="n">
-        <v>5.93</v>
+        <v>5.928</v>
       </c>
       <c r="M3" t="n">
-        <v>6.267</v>
+        <v>6.264</v>
       </c>
       <c r="N3" t="n">
-        <v>6.468</v>
+        <v>6.467</v>
       </c>
       <c r="O3" t="n">
-        <v>6.633</v>
+        <v>6.637</v>
       </c>
       <c r="P3" t="n">
-        <v>6.671</v>
+        <v>6.672</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.19</v>
+        <v>7.193</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.753</v>
+        <v>3.749</v>
       </c>
       <c r="G4" t="n">
-        <v>4.033</v>
+        <v>4.029</v>
       </c>
       <c r="H4" t="n">
-        <v>4.233</v>
+        <v>4.229</v>
       </c>
       <c r="I4" t="n">
-        <v>4.486</v>
+        <v>4.482</v>
       </c>
       <c r="J4" t="n">
-        <v>4.694</v>
+        <v>4.697</v>
       </c>
       <c r="K4" t="n">
-        <v>5.134</v>
+        <v>5.131</v>
       </c>
       <c r="L4" t="n">
-        <v>5.3</v>
+        <v>5.298</v>
       </c>
       <c r="M4" t="n">
-        <v>5.625</v>
+        <v>5.622</v>
       </c>
       <c r="N4" t="n">
-        <v>5.797</v>
+        <v>5.795</v>
       </c>
       <c r="O4" t="n">
-        <v>5.985</v>
+        <v>5.989</v>
       </c>
       <c r="P4" t="n">
         <v>6.021</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.543</v>
+        <v>6.546</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.946</v>
+        <v>2.939</v>
       </c>
       <c r="G5" t="n">
-        <v>2.997</v>
+        <v>2.991</v>
       </c>
       <c r="H5" t="n">
-        <v>3.089</v>
+        <v>3.083</v>
       </c>
       <c r="I5" t="n">
-        <v>3.383</v>
+        <v>3.375</v>
       </c>
       <c r="J5" t="n">
-        <v>3.571</v>
+        <v>3.57</v>
       </c>
       <c r="K5" t="n">
-        <v>3.806</v>
+        <v>3.8</v>
       </c>
       <c r="L5" t="n">
-        <v>3.816</v>
+        <v>3.812</v>
       </c>
       <c r="M5" t="n">
-        <v>3.927</v>
+        <v>3.922</v>
       </c>
       <c r="N5" t="n">
         <v>3.923</v>
       </c>
       <c r="O5" t="n">
-        <v>3.925</v>
+        <v>3.928</v>
       </c>
       <c r="P5" t="n">
-        <v>4.159</v>
+        <v>4.16</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.034</v>
+        <v>5.037</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.987</v>
+        <v>2.98</v>
       </c>
       <c r="G6" t="n">
-        <v>3.053</v>
+        <v>3.046</v>
       </c>
       <c r="H6" t="n">
-        <v>3.159</v>
+        <v>3.153</v>
       </c>
       <c r="I6" t="n">
-        <v>3.46</v>
+        <v>3.454</v>
       </c>
       <c r="J6" t="n">
-        <v>3.657</v>
+        <v>3.659</v>
       </c>
       <c r="K6" t="n">
-        <v>3.91</v>
+        <v>3.907</v>
       </c>
       <c r="L6" t="n">
-        <v>3.931</v>
+        <v>3.929</v>
       </c>
       <c r="M6" t="n">
-        <v>4.076</v>
+        <v>4.073</v>
       </c>
       <c r="N6" t="n">
-        <v>4.091</v>
+        <v>4.089</v>
       </c>
       <c r="O6" t="n">
-        <v>4.191</v>
+        <v>4.195</v>
       </c>
       <c r="P6" t="n">
         <v>4.592</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.43</v>
+        <v>5.433</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.967</v>
+        <v>2.96</v>
       </c>
       <c r="G7" t="n">
-        <v>3.016</v>
+        <v>3.009</v>
       </c>
       <c r="H7" t="n">
-        <v>3.105</v>
+        <v>3.099</v>
       </c>
       <c r="I7" t="n">
-        <v>3.398</v>
+        <v>3.39</v>
       </c>
       <c r="J7" t="n">
         <v>3.596</v>
       </c>
       <c r="K7" t="n">
-        <v>3.832</v>
+        <v>3.827</v>
       </c>
       <c r="L7" t="n">
-        <v>3.841</v>
+        <v>3.837</v>
       </c>
       <c r="M7" t="n">
-        <v>3.985</v>
+        <v>3.98</v>
       </c>
       <c r="N7" t="n">
         <v>3.983</v>
       </c>
       <c r="O7" t="n">
-        <v>4.089</v>
+        <v>4.093</v>
       </c>
       <c r="P7" t="n">
-        <v>4.375</v>
+        <v>4.376</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.198</v>
+        <v>5.201</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.372</v>
+        <v>5.367</v>
       </c>
       <c r="G8" t="n">
-        <v>5.951</v>
+        <v>5.946</v>
       </c>
       <c r="H8" t="n">
-        <v>6.274</v>
+        <v>6.269</v>
       </c>
       <c r="I8" t="n">
-        <v>6.567</v>
+        <v>6.561</v>
       </c>
       <c r="J8" t="n">
-        <v>6.832</v>
+        <v>6.835</v>
       </c>
       <c r="K8" t="n">
-        <v>7.56</v>
+        <v>7.557</v>
       </c>
       <c r="L8" t="n">
-        <v>7.885</v>
+        <v>7.883</v>
       </c>
       <c r="M8" t="n">
-        <v>8.250999999999999</v>
+        <v>8.247</v>
       </c>
       <c r="N8" t="n">
-        <v>8.388999999999999</v>
+        <v>8.388</v>
       </c>
       <c r="O8" t="n">
-        <v>8.640000000000001</v>
+        <v>8.644</v>
       </c>
       <c r="P8" t="n">
-        <v>8.779</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.499000000000001</v>
+        <v>9.502000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.616</v>
+        <v>2.621</v>
       </c>
       <c r="G9" t="n">
         <v>2.678</v>
@@ -1072,48 +1072,48 @@
         <v>2.774</v>
       </c>
       <c r="I9" t="n">
-        <v>2.916</v>
+        <v>2.924</v>
       </c>
       <c r="J9" t="n">
-        <v>3.098</v>
+        <v>3.099</v>
       </c>
       <c r="K9" t="n">
-        <v>3.203</v>
+        <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>3.25</v>
+        <v>3.247</v>
       </c>
       <c r="M9" t="n">
-        <v>3.337</v>
+        <v>3.332</v>
       </c>
       <c r="N9" t="n">
-        <v>3.491</v>
+        <v>3.49</v>
       </c>
       <c r="O9" t="n">
-        <v>3.516</v>
+        <v>3.52</v>
       </c>
       <c r="P9" t="n">
-        <v>3.579</v>
+        <v>3.58</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.652</v>
+        <v>3.655</v>
       </c>
       <c r="R9" t="n">
-        <v>3.665</v>
+        <v>3.66</v>
       </c>
       <c r="S9" t="n">
-        <v>3.63</v>
+        <v>3.622</v>
       </c>
       <c r="T9" t="n">
-        <v>3.537</v>
+        <v>3.532</v>
       </c>
       <c r="U9" t="n">
-        <v>3.41</v>
+        <v>3.405</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.628</v>
+        <v>2.634</v>
       </c>
       <c r="G10" t="n">
-        <v>2.71</v>
+        <v>2.714</v>
       </c>
       <c r="H10" t="n">
         <v>2.786</v>
       </c>
       <c r="I10" t="n">
-        <v>2.927</v>
+        <v>2.935</v>
       </c>
       <c r="J10" t="n">
-        <v>3.123</v>
+        <v>3.126</v>
       </c>
       <c r="K10" t="n">
-        <v>3.232</v>
+        <v>3.228</v>
       </c>
       <c r="L10" t="n">
-        <v>3.293</v>
+        <v>3.292</v>
       </c>
       <c r="M10" t="n">
-        <v>3.436</v>
+        <v>3.43</v>
       </c>
       <c r="N10" t="n">
         <v>3.501</v>
       </c>
       <c r="O10" t="n">
-        <v>3.686</v>
+        <v>3.688</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.444</v>
+        <v>2.449</v>
       </c>
       <c r="G11" t="n">
-        <v>2.52</v>
+        <v>2.524</v>
       </c>
       <c r="H11" t="n">
-        <v>2.61</v>
+        <v>2.611</v>
       </c>
       <c r="I11" t="n">
-        <v>2.729</v>
+        <v>2.738</v>
       </c>
       <c r="J11" t="n">
-        <v>2.917</v>
+        <v>2.92</v>
       </c>
       <c r="K11" t="n">
-        <v>3.019</v>
+        <v>3.016</v>
       </c>
       <c r="L11" t="n">
-        <v>3.086</v>
+        <v>3.085</v>
       </c>
       <c r="M11" t="n">
-        <v>3.24</v>
+        <v>3.235</v>
       </c>
       <c r="N11" t="n">
-        <v>3.311</v>
+        <v>3.31</v>
       </c>
       <c r="O11" t="n">
-        <v>3.452</v>
+        <v>3.455</v>
       </c>
       <c r="P11" t="n">
-        <v>3.516</v>
+        <v>3.517</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.855</v>
+        <v>3.858</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.207</v>
+        <v>3.202</v>
       </c>
       <c r="G12" t="n">
-        <v>3.358</v>
+        <v>3.353</v>
       </c>
       <c r="H12" t="n">
-        <v>3.459</v>
+        <v>3.457</v>
       </c>
       <c r="I12" t="n">
-        <v>3.682</v>
+        <v>3.674</v>
       </c>
       <c r="J12" t="n">
-        <v>3.971</v>
+        <v>3.968</v>
       </c>
       <c r="K12" t="n">
-        <v>4.155</v>
+        <v>4.15</v>
       </c>
       <c r="L12" t="n">
-        <v>4.207</v>
+        <v>4.204</v>
       </c>
       <c r="M12" t="n">
-        <v>4.352</v>
+        <v>4.347</v>
       </c>
       <c r="N12" t="n">
-        <v>4.384</v>
+        <v>4.382</v>
       </c>
       <c r="O12" t="n">
-        <v>4.522</v>
+        <v>4.525</v>
       </c>
       <c r="P12" t="n">
         <v>4.627</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.983</v>
+        <v>4.985</v>
       </c>
       <c r="R12" t="n">
-        <v>5.162</v>
+        <v>5.157</v>
       </c>
       <c r="S12" t="n">
-        <v>5.34</v>
+        <v>5.333</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.96</v>
+        <v>2.956</v>
       </c>
       <c r="G13" t="n">
-        <v>3.048</v>
+        <v>3.043</v>
       </c>
       <c r="H13" t="n">
-        <v>3.127</v>
+        <v>3.124</v>
       </c>
       <c r="I13" t="n">
-        <v>3.329</v>
+        <v>3.322</v>
       </c>
       <c r="J13" t="n">
-        <v>3.607</v>
+        <v>3.605</v>
       </c>
       <c r="K13" t="n">
-        <v>3.788</v>
+        <v>3.784</v>
       </c>
       <c r="L13" t="n">
-        <v>3.846</v>
+        <v>3.843</v>
       </c>
       <c r="M13" t="n">
-        <v>3.979</v>
+        <v>3.975</v>
       </c>
       <c r="N13" t="n">
-        <v>4.012</v>
+        <v>4.01</v>
       </c>
       <c r="O13" t="n">
-        <v>4.151</v>
+        <v>4.154</v>
       </c>
       <c r="P13" t="n">
-        <v>4.218</v>
+        <v>4.219</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.503</v>
+        <v>4.506</v>
       </c>
       <c r="R13" t="n">
-        <v>4.71</v>
+        <v>4.705</v>
       </c>
       <c r="S13" t="n">
-        <v>4.903</v>
+        <v>4.895</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.778</v>
+        <v>2.774</v>
       </c>
       <c r="G14" t="n">
-        <v>2.855</v>
+        <v>2.85</v>
       </c>
       <c r="H14" t="n">
-        <v>2.93</v>
+        <v>2.927</v>
       </c>
       <c r="I14" t="n">
-        <v>3.112</v>
+        <v>3.105</v>
       </c>
       <c r="J14" t="n">
-        <v>3.347</v>
+        <v>3.344</v>
       </c>
       <c r="K14" t="n">
-        <v>3.476</v>
+        <v>3.472</v>
       </c>
       <c r="L14" t="n">
-        <v>3.518</v>
+        <v>3.515</v>
       </c>
       <c r="M14" t="n">
-        <v>3.664</v>
+        <v>3.659</v>
       </c>
       <c r="N14" t="n">
-        <v>3.691</v>
+        <v>3.69</v>
       </c>
       <c r="O14" t="n">
-        <v>3.806</v>
+        <v>3.809</v>
       </c>
       <c r="P14" t="n">
-        <v>3.853</v>
+        <v>3.854</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.093</v>
+        <v>4.095</v>
       </c>
       <c r="R14" t="n">
-        <v>4.225</v>
+        <v>4.22</v>
       </c>
       <c r="S14" t="n">
-        <v>4.356</v>
+        <v>4.348</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.757</v>
+        <v>2.752</v>
       </c>
       <c r="G15" t="n">
-        <v>2.829</v>
+        <v>2.824</v>
       </c>
       <c r="H15" t="n">
-        <v>2.898</v>
+        <v>2.896</v>
       </c>
       <c r="I15" t="n">
-        <v>3.063</v>
+        <v>3.056</v>
       </c>
       <c r="J15" t="n">
-        <v>3.284</v>
+        <v>3.281</v>
       </c>
       <c r="K15" t="n">
-        <v>3.429</v>
+        <v>3.425</v>
       </c>
       <c r="L15" t="n">
-        <v>3.453</v>
+        <v>3.45</v>
       </c>
       <c r="M15" t="n">
-        <v>3.577</v>
+        <v>3.572</v>
       </c>
       <c r="N15" t="n">
-        <v>3.595</v>
+        <v>3.593</v>
       </c>
       <c r="O15" t="n">
-        <v>3.73</v>
+        <v>3.734</v>
       </c>
       <c r="P15" t="n">
-        <v>3.751</v>
+        <v>3.752</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.997</v>
+        <v>4</v>
       </c>
       <c r="R15" t="n">
-        <v>4.122</v>
+        <v>4.117</v>
       </c>
       <c r="S15" t="n">
-        <v>4.251</v>
+        <v>4.243</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.757</v>
+        <v>2.752</v>
       </c>
       <c r="G16" t="n">
-        <v>2.829</v>
+        <v>2.824</v>
       </c>
       <c r="H16" t="n">
-        <v>2.898</v>
+        <v>2.896</v>
       </c>
       <c r="I16" t="n">
-        <v>3.063</v>
+        <v>3.056</v>
       </c>
       <c r="J16" t="n">
-        <v>3.284</v>
+        <v>3.281</v>
       </c>
       <c r="K16" t="n">
-        <v>3.429</v>
+        <v>3.425</v>
       </c>
       <c r="L16" t="n">
-        <v>3.453</v>
+        <v>3.45</v>
       </c>
       <c r="M16" t="n">
-        <v>3.577</v>
+        <v>3.572</v>
       </c>
       <c r="N16" t="n">
-        <v>3.598</v>
+        <v>3.596</v>
       </c>
       <c r="O16" t="n">
-        <v>3.737</v>
+        <v>3.741</v>
       </c>
       <c r="P16" t="n">
         <v>3.775</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.024</v>
+        <v>4.027</v>
       </c>
       <c r="R16" t="n">
-        <v>4.15</v>
+        <v>4.145</v>
       </c>
       <c r="S16" t="n">
-        <v>4.28</v>
+        <v>4.272</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.693</v>
+        <v>2.699</v>
       </c>
       <c r="G17" t="n">
-        <v>2.801</v>
+        <v>2.805</v>
       </c>
       <c r="H17" t="n">
         <v>2.881</v>
       </c>
       <c r="I17" t="n">
-        <v>3.009</v>
+        <v>3.018</v>
       </c>
       <c r="J17" t="n">
-        <v>3.194</v>
+        <v>3.196</v>
       </c>
       <c r="K17" t="n">
-        <v>3.306</v>
+        <v>3.303</v>
       </c>
       <c r="L17" t="n">
-        <v>3.371</v>
+        <v>3.369</v>
       </c>
       <c r="M17" t="n">
-        <v>3.556</v>
+        <v>3.549</v>
       </c>
       <c r="N17" t="n">
-        <v>3.603</v>
+        <v>3.602</v>
       </c>
       <c r="O17" t="n">
-        <v>3.721</v>
+        <v>3.723</v>
       </c>
       <c r="P17" t="n">
-        <v>3.794</v>
+        <v>3.795</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.694</v>
+        <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.802</v>
+        <v>2.806</v>
       </c>
       <c r="H18" t="n">
         <v>2.881</v>
       </c>
       <c r="I18" t="n">
-        <v>3.01</v>
+        <v>3.019</v>
       </c>
       <c r="J18" t="n">
-        <v>3.194</v>
+        <v>3.196</v>
       </c>
       <c r="K18" t="n">
-        <v>3.307</v>
+        <v>3.303</v>
       </c>
       <c r="L18" t="n">
-        <v>3.371</v>
+        <v>3.369</v>
       </c>
       <c r="M18" t="n">
-        <v>3.556</v>
+        <v>3.549</v>
       </c>
       <c r="N18" t="n">
-        <v>3.603</v>
+        <v>3.602</v>
       </c>
       <c r="O18" t="n">
-        <v>3.72</v>
+        <v>3.722</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.767</v>
+        <v>2.764</v>
       </c>
       <c r="G19" t="n">
-        <v>2.845</v>
+        <v>2.841</v>
       </c>
       <c r="H19" t="n">
-        <v>2.919</v>
+        <v>2.917</v>
       </c>
       <c r="I19" t="n">
-        <v>3.097</v>
+        <v>3.09</v>
       </c>
       <c r="J19" t="n">
-        <v>3.33</v>
+        <v>3.328</v>
       </c>
       <c r="K19" t="n">
-        <v>3.472</v>
+        <v>3.468</v>
       </c>
       <c r="L19" t="n">
-        <v>3.515</v>
+        <v>3.512</v>
       </c>
       <c r="M19" t="n">
-        <v>3.654</v>
+        <v>3.651</v>
       </c>
       <c r="N19" t="n">
-        <v>3.679</v>
+        <v>3.678</v>
       </c>
       <c r="O19" t="n">
-        <v>3.784</v>
+        <v>3.788</v>
       </c>
       <c r="P19" t="n">
-        <v>3.816</v>
+        <v>3.817</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.041</v>
+        <v>4.044</v>
       </c>
       <c r="R19" t="n">
-        <v>4.174</v>
+        <v>4.169</v>
       </c>
       <c r="S19" t="n">
-        <v>4.294</v>
+        <v>4.286</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1875,19 +1875,19 @@
         <v>2.692</v>
       </c>
       <c r="I20" t="n">
-        <v>2.851</v>
+        <v>2.846</v>
       </c>
       <c r="J20" t="n">
-        <v>3.09</v>
+        <v>3.092</v>
       </c>
       <c r="K20" t="n">
-        <v>3.238</v>
+        <v>3.235</v>
       </c>
       <c r="L20" t="n">
-        <v>3.285</v>
+        <v>3.281</v>
       </c>
       <c r="M20" t="n">
-        <v>3.382</v>
+        <v>3.38</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.871</v>
+        <v>2.867</v>
       </c>
       <c r="G21" t="n">
-        <v>2.949</v>
+        <v>2.946</v>
       </c>
       <c r="H21" t="n">
-        <v>3.061</v>
+        <v>3.058</v>
       </c>
       <c r="I21" t="n">
-        <v>3.235</v>
+        <v>3.229</v>
       </c>
       <c r="J21" t="n">
         <v>3.46</v>
       </c>
       <c r="K21" t="n">
-        <v>3.711</v>
+        <v>3.707</v>
       </c>
       <c r="L21" t="n">
-        <v>3.776</v>
+        <v>3.772</v>
       </c>
       <c r="M21" t="n">
-        <v>3.911</v>
+        <v>3.904</v>
       </c>
       <c r="N21" t="n">
         <v>3.945</v>
       </c>
       <c r="O21" t="n">
-        <v>4.024</v>
+        <v>4.028</v>
       </c>
       <c r="P21" t="n">
         <v>4.08</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.204</v>
+        <v>4.207</v>
       </c>
       <c r="R21" t="n">
-        <v>4.222</v>
+        <v>4.217</v>
       </c>
       <c r="S21" t="n">
-        <v>4.255</v>
+        <v>4.247</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.819</v>
+        <v>2.815</v>
       </c>
       <c r="G22" t="n">
-        <v>2.896</v>
+        <v>2.893</v>
       </c>
       <c r="H22" t="n">
-        <v>2.996</v>
+        <v>2.992</v>
       </c>
       <c r="I22" t="n">
-        <v>3.154</v>
+        <v>3.147</v>
       </c>
       <c r="J22" t="n">
         <v>3.343</v>
       </c>
       <c r="K22" t="n">
-        <v>3.591</v>
+        <v>3.588</v>
       </c>
       <c r="L22" t="n">
-        <v>3.645</v>
+        <v>3.641</v>
       </c>
       <c r="M22" t="n">
-        <v>3.782</v>
+        <v>3.775</v>
       </c>
       <c r="N22" t="n">
-        <v>3.818</v>
+        <v>3.817</v>
       </c>
       <c r="O22" t="n">
-        <v>3.892</v>
+        <v>3.896</v>
       </c>
       <c r="P22" t="n">
         <v>3.942</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.062</v>
+        <v>4.065</v>
       </c>
       <c r="R22" t="n">
-        <v>4.07</v>
+        <v>4.065</v>
       </c>
       <c r="S22" t="n">
-        <v>4.1</v>
+        <v>4.092</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.771</v>
+        <v>2.767</v>
       </c>
       <c r="G23" t="n">
-        <v>2.851</v>
+        <v>2.848</v>
       </c>
       <c r="H23" t="n">
-        <v>2.934</v>
+        <v>2.931</v>
       </c>
       <c r="I23" t="n">
-        <v>3.107</v>
+        <v>3.1</v>
       </c>
       <c r="J23" t="n">
         <v>3.289</v>
       </c>
       <c r="K23" t="n">
-        <v>3.511</v>
+        <v>3.507</v>
       </c>
       <c r="L23" t="n">
-        <v>3.556</v>
+        <v>3.552</v>
       </c>
       <c r="M23" t="n">
-        <v>3.686</v>
+        <v>3.679</v>
       </c>
       <c r="N23" t="n">
         <v>3.714</v>
       </c>
       <c r="O23" t="n">
-        <v>3.767</v>
+        <v>3.771</v>
       </c>
       <c r="P23" t="n">
-        <v>3.803</v>
+        <v>3.804</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.87</v>
+        <v>3.873</v>
       </c>
       <c r="R23" t="n">
-        <v>3.854</v>
+        <v>3.849</v>
       </c>
       <c r="S23" t="n">
-        <v>3.854</v>
+        <v>3.846</v>
       </c>
       <c r="T23" t="n">
-        <v>3.75</v>
+        <v>3.745</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.703</v>
+        <v>2.699</v>
       </c>
       <c r="G24" t="n">
-        <v>2.764</v>
+        <v>2.761</v>
       </c>
       <c r="H24" t="n">
-        <v>2.835</v>
+        <v>2.832</v>
       </c>
       <c r="I24" t="n">
-        <v>3.017</v>
+        <v>3.01</v>
       </c>
       <c r="J24" t="n">
-        <v>3.19</v>
+        <v>3.189</v>
       </c>
       <c r="K24" t="n">
-        <v>3.395</v>
+        <v>3.39</v>
       </c>
       <c r="L24" t="n">
-        <v>3.428</v>
+        <v>3.424</v>
       </c>
       <c r="M24" t="n">
-        <v>3.542</v>
+        <v>3.536</v>
       </c>
       <c r="N24" t="n">
-        <v>3.585</v>
+        <v>3.584</v>
       </c>
       <c r="O24" t="n">
-        <v>3.715</v>
+        <v>3.719</v>
       </c>
       <c r="P24" t="n">
-        <v>3.742</v>
+        <v>3.743</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.793</v>
+        <v>3.795</v>
       </c>
       <c r="R24" t="n">
-        <v>3.774</v>
+        <v>3.769</v>
       </c>
       <c r="S24" t="n">
-        <v>3.769</v>
+        <v>3.761</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.764</v>
+        <v>2.761</v>
       </c>
       <c r="G25" t="n">
-        <v>2.85</v>
+        <v>2.847</v>
       </c>
       <c r="H25" t="n">
-        <v>2.938</v>
+        <v>2.934</v>
       </c>
       <c r="I25" t="n">
-        <v>3.114</v>
+        <v>3.107</v>
       </c>
       <c r="J25" t="n">
         <v>3.305</v>
       </c>
       <c r="K25" t="n">
-        <v>3.54</v>
+        <v>3.536</v>
       </c>
       <c r="L25" t="n">
-        <v>3.585</v>
+        <v>3.581</v>
       </c>
       <c r="M25" t="n">
-        <v>3.715</v>
+        <v>3.708</v>
       </c>
       <c r="N25" t="n">
-        <v>3.741</v>
+        <v>3.74</v>
       </c>
       <c r="O25" t="n">
-        <v>3.796</v>
+        <v>3.8</v>
       </c>
       <c r="P25" t="n">
-        <v>3.825</v>
+        <v>3.826</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.903</v>
+        <v>3.906</v>
       </c>
       <c r="R25" t="n">
-        <v>3.877</v>
+        <v>3.872</v>
       </c>
       <c r="S25" t="n">
-        <v>3.877</v>
+        <v>3.869</v>
       </c>
       <c r="T25" t="n">
-        <v>3.768</v>
+        <v>3.763</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2313,25 +2313,25 @@
         <v>3.396</v>
       </c>
       <c r="I26" t="n">
-        <v>3.648</v>
+        <v>3.643</v>
       </c>
       <c r="J26" t="n">
-        <v>3.959</v>
+        <v>3.962</v>
       </c>
       <c r="K26" t="n">
-        <v>4.328</v>
+        <v>4.326</v>
       </c>
       <c r="L26" t="n">
-        <v>4.425</v>
+        <v>4.424</v>
       </c>
       <c r="M26" t="n">
-        <v>4.622</v>
+        <v>4.617</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.856</v>
+        <v>4.86</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.869</v>
+        <v>2.868</v>
       </c>
       <c r="G27" t="n">
-        <v>2.936</v>
+        <v>2.934</v>
       </c>
       <c r="H27" t="n">
-        <v>3.032</v>
+        <v>3.031</v>
       </c>
       <c r="I27" t="n">
-        <v>3.23</v>
+        <v>3.223</v>
       </c>
       <c r="J27" t="n">
         <v>3.461</v>
       </c>
       <c r="K27" t="n">
-        <v>3.648</v>
+        <v>3.644</v>
       </c>
       <c r="L27" t="n">
-        <v>3.695</v>
+        <v>3.693</v>
       </c>
       <c r="M27" t="n">
-        <v>3.832</v>
+        <v>3.827</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.948</v>
+        <v>3.951</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.97</v>
+        <v>2.968</v>
       </c>
       <c r="G28" t="n">
-        <v>3.042</v>
+        <v>3.04</v>
       </c>
       <c r="H28" t="n">
-        <v>3.155</v>
+        <v>3.154</v>
       </c>
       <c r="I28" t="n">
-        <v>3.366</v>
+        <v>3.36</v>
       </c>
       <c r="J28" t="n">
-        <v>3.634</v>
+        <v>3.635</v>
       </c>
       <c r="K28" t="n">
-        <v>3.84</v>
+        <v>3.837</v>
       </c>
       <c r="L28" t="n">
-        <v>3.898</v>
+        <v>3.896</v>
       </c>
       <c r="M28" t="n">
-        <v>4.045</v>
+        <v>4.04</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.242</v>
+        <v>4.245</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.828</v>
+        <v>2.825</v>
       </c>
       <c r="G29" t="n">
-        <v>2.896</v>
+        <v>2.893</v>
       </c>
       <c r="H29" t="n">
-        <v>2.977</v>
+        <v>2.975</v>
       </c>
       <c r="I29" t="n">
-        <v>3.164</v>
+        <v>3.157</v>
       </c>
       <c r="J29" t="n">
-        <v>3.373</v>
+        <v>3.374</v>
       </c>
       <c r="K29" t="n">
-        <v>3.544</v>
+        <v>3.54</v>
       </c>
       <c r="L29" t="n">
-        <v>3.579</v>
+        <v>3.577</v>
       </c>
       <c r="M29" t="n">
-        <v>3.694</v>
+        <v>3.689</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.808</v>
+        <v>3.811</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.101</v>
+        <v>3.102</v>
       </c>
       <c r="G30" t="n">
-        <v>3.167</v>
+        <v>3.168</v>
       </c>
       <c r="H30" t="n">
-        <v>3.321</v>
+        <v>3.322</v>
       </c>
       <c r="I30" t="n">
-        <v>3.565</v>
+        <v>3.561</v>
       </c>
       <c r="J30" t="n">
-        <v>3.817</v>
+        <v>3.821</v>
       </c>
       <c r="K30" t="n">
-        <v>4.119</v>
+        <v>4.118</v>
       </c>
       <c r="L30" t="n">
         <v>4.193</v>
       </c>
       <c r="M30" t="n">
-        <v>4.38</v>
+        <v>4.377</v>
       </c>
       <c r="N30" t="n">
-        <v>4.537</v>
+        <v>4.536</v>
       </c>
       <c r="O30" t="n">
-        <v>4.809</v>
+        <v>4.813</v>
       </c>
       <c r="P30" t="n">
-        <v>4.967</v>
+        <v>4.969</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.727</v>
+        <v>5.73</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.427</v>
+        <v>3.428</v>
       </c>
       <c r="G31" t="n">
-        <v>3.527</v>
+        <v>3.528</v>
       </c>
       <c r="H31" t="n">
-        <v>3.733</v>
+        <v>3.735</v>
       </c>
       <c r="I31" t="n">
-        <v>3.993</v>
+        <v>3.989</v>
       </c>
       <c r="J31" t="n">
-        <v>4.307</v>
+        <v>4.311</v>
       </c>
       <c r="K31" t="n">
-        <v>4.651</v>
+        <v>4.65</v>
       </c>
       <c r="L31" t="n">
         <v>4.803</v>
       </c>
       <c r="M31" t="n">
-        <v>5.109</v>
+        <v>5.106</v>
       </c>
       <c r="N31" t="n">
-        <v>5.394</v>
+        <v>5.392</v>
       </c>
       <c r="O31" t="n">
-        <v>5.841</v>
+        <v>5.845</v>
       </c>
       <c r="P31" t="n">
-        <v>5.954</v>
+        <v>5.957</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.7</v>
+        <v>6.703</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.199</v>
+        <v>3.2</v>
       </c>
       <c r="G32" t="n">
-        <v>3.283</v>
+        <v>3.284</v>
       </c>
       <c r="H32" t="n">
-        <v>3.463</v>
+        <v>3.465</v>
       </c>
       <c r="I32" t="n">
-        <v>3.724</v>
+        <v>3.72</v>
       </c>
       <c r="J32" t="n">
-        <v>3.996</v>
+        <v>4</v>
       </c>
       <c r="K32" t="n">
-        <v>4.305</v>
+        <v>4.303</v>
       </c>
       <c r="L32" t="n">
         <v>4.396</v>
       </c>
       <c r="M32" t="n">
-        <v>4.652</v>
+        <v>4.649</v>
       </c>
       <c r="N32" t="n">
-        <v>4.897</v>
+        <v>4.896</v>
       </c>
       <c r="O32" t="n">
-        <v>5.253</v>
+        <v>5.257</v>
       </c>
       <c r="P32" t="n">
-        <v>5.426</v>
+        <v>5.428</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.188</v>
+        <v>6.191</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2821,13 +2821,13 @@
         <v>3.041</v>
       </c>
       <c r="H33" t="n">
-        <v>3.145</v>
+        <v>3.148</v>
       </c>
       <c r="I33" t="n">
-        <v>3.355</v>
+        <v>3.349</v>
       </c>
       <c r="J33" t="n">
-        <v>3.529</v>
+        <v>3.533</v>
       </c>
       <c r="K33" t="n">
         <v>3.761</v>
@@ -2836,19 +2836,19 @@
         <v>3.799</v>
       </c>
       <c r="M33" t="n">
-        <v>3.913</v>
+        <v>3.909</v>
       </c>
       <c r="N33" t="n">
-        <v>3.926</v>
+        <v>3.925</v>
       </c>
       <c r="O33" t="n">
-        <v>3.963</v>
+        <v>3.967</v>
       </c>
       <c r="P33" t="n">
-        <v>3.997</v>
+        <v>3.999</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.444</v>
+        <v>4.447</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2894,13 +2894,13 @@
         <v>3.094</v>
       </c>
       <c r="H34" t="n">
-        <v>3.204</v>
+        <v>3.207</v>
       </c>
       <c r="I34" t="n">
-        <v>3.423</v>
+        <v>3.417</v>
       </c>
       <c r="J34" t="n">
-        <v>3.601</v>
+        <v>3.605</v>
       </c>
       <c r="K34" t="n">
         <v>3.838</v>
@@ -2909,19 +2909,19 @@
         <v>3.878</v>
       </c>
       <c r="M34" t="n">
-        <v>4.003</v>
+        <v>4</v>
       </c>
       <c r="N34" t="n">
-        <v>4.03</v>
+        <v>4.029</v>
       </c>
       <c r="O34" t="n">
-        <v>4.131</v>
+        <v>4.135</v>
       </c>
       <c r="P34" t="n">
-        <v>4.291</v>
+        <v>4.294</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.145</v>
+        <v>5.148</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.016</v>
+        <v>3.017</v>
       </c>
       <c r="G35" t="n">
         <v>3.067</v>
       </c>
       <c r="H35" t="n">
-        <v>3.172</v>
+        <v>3.175</v>
       </c>
       <c r="I35" t="n">
-        <v>3.39</v>
+        <v>3.384</v>
       </c>
       <c r="J35" t="n">
-        <v>3.569</v>
+        <v>3.573</v>
       </c>
       <c r="K35" t="n">
-        <v>3.793</v>
+        <v>3.792</v>
       </c>
       <c r="L35" t="n">
         <v>3.833</v>
       </c>
       <c r="M35" t="n">
-        <v>3.95</v>
+        <v>3.947</v>
       </c>
       <c r="N35" t="n">
-        <v>3.967</v>
+        <v>3.966</v>
       </c>
       <c r="O35" t="n">
-        <v>4.029</v>
+        <v>4.033</v>
       </c>
       <c r="P35" t="n">
-        <v>4.094</v>
+        <v>4.096</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.78</v>
+        <v>4.783</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.928</v>
+        <v>2.927</v>
       </c>
       <c r="G36" t="n">
         <v>2.986</v>
       </c>
       <c r="H36" t="n">
-        <v>3.075</v>
+        <v>3.076</v>
       </c>
       <c r="I36" t="n">
-        <v>3.286</v>
+        <v>3.28</v>
       </c>
       <c r="J36" t="n">
-        <v>3.467</v>
+        <v>3.471</v>
       </c>
       <c r="K36" t="n">
-        <v>3.684</v>
+        <v>3.683</v>
       </c>
       <c r="L36" t="n">
         <v>3.722</v>
       </c>
       <c r="M36" t="n">
-        <v>3.812</v>
+        <v>3.808</v>
       </c>
       <c r="N36" t="n">
-        <v>3.829</v>
+        <v>3.828</v>
       </c>
       <c r="O36" t="n">
-        <v>3.873</v>
+        <v>3.877</v>
       </c>
       <c r="P36" t="n">
-        <v>3.896</v>
+        <v>3.898</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.161</v>
+        <v>4.164</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,19 +3107,19 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.771</v>
+        <v>3.772</v>
       </c>
       <c r="G37" t="n">
-        <v>4.221</v>
+        <v>4.222</v>
       </c>
       <c r="H37" t="n">
-        <v>4.71</v>
+        <v>4.712</v>
       </c>
       <c r="I37" t="n">
-        <v>5.065</v>
+        <v>5.06</v>
       </c>
       <c r="J37" t="n">
-        <v>5.798</v>
+        <v>5.802</v>
       </c>
       <c r="K37" t="n">
         <v>6.689</v>
@@ -3128,19 +3128,19 @@
         <v>7.003</v>
       </c>
       <c r="M37" t="n">
-        <v>7.382</v>
+        <v>7.379</v>
       </c>
       <c r="N37" t="n">
-        <v>7.546</v>
+        <v>7.544</v>
       </c>
       <c r="O37" t="n">
-        <v>7.721</v>
+        <v>7.725</v>
       </c>
       <c r="P37" t="n">
-        <v>7.752</v>
+        <v>7.754</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.192</v>
+        <v>8.195</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.827</v>
+        <v>4.828</v>
       </c>
       <c r="G38" t="n">
-        <v>5.531</v>
+        <v>5.532</v>
       </c>
       <c r="H38" t="n">
-        <v>6.234</v>
+        <v>6.236</v>
       </c>
       <c r="I38" t="n">
-        <v>6.745</v>
+        <v>6.74</v>
       </c>
       <c r="J38" t="n">
-        <v>7.738</v>
+        <v>7.742</v>
       </c>
       <c r="K38" t="n">
-        <v>8.804</v>
+        <v>8.803000000000001</v>
       </c>
       <c r="L38" t="n">
         <v>9.278</v>
       </c>
       <c r="M38" t="n">
-        <v>9.789999999999999</v>
+        <v>9.786</v>
       </c>
       <c r="N38" t="n">
-        <v>9.964</v>
+        <v>9.962</v>
       </c>
       <c r="O38" t="n">
-        <v>10.12</v>
+        <v>10.124</v>
       </c>
       <c r="P38" t="n">
-        <v>10.15</v>
+        <v>10.153</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.643</v>
+        <v>10.646</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.148</v>
+        <v>4.149</v>
       </c>
       <c r="G39" t="n">
-        <v>4.729</v>
+        <v>4.73</v>
       </c>
       <c r="H39" t="n">
-        <v>5.299</v>
+        <v>5.301</v>
       </c>
       <c r="I39" t="n">
-        <v>5.749</v>
+        <v>5.744</v>
       </c>
       <c r="J39" t="n">
-        <v>6.611</v>
+        <v>6.615</v>
       </c>
       <c r="K39" t="n">
-        <v>7.638</v>
+        <v>7.637</v>
       </c>
       <c r="L39" t="n">
         <v>8.037000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.427</v>
+        <v>8.423999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.590999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="O39" t="n">
-        <v>8.771000000000001</v>
+        <v>8.773999999999999</v>
       </c>
       <c r="P39" t="n">
-        <v>8.805</v>
+        <v>8.808</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.288</v>
+        <v>9.291</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.293</v>
+        <v>3.295</v>
       </c>
       <c r="G40" t="n">
-        <v>3.406</v>
+        <v>3.407</v>
       </c>
       <c r="H40" t="n">
-        <v>3.581</v>
+        <v>3.582</v>
       </c>
       <c r="I40" t="n">
-        <v>3.84</v>
+        <v>3.836</v>
       </c>
       <c r="J40" t="n">
-        <v>4.11</v>
+        <v>4.114</v>
       </c>
       <c r="K40" t="n">
-        <v>4.424</v>
+        <v>4.422</v>
       </c>
       <c r="L40" t="n">
         <v>4.517</v>
       </c>
       <c r="M40" t="n">
-        <v>4.721</v>
+        <v>4.718</v>
       </c>
       <c r="N40" t="n">
-        <v>4.895</v>
+        <v>4.893</v>
       </c>
       <c r="O40" t="n">
-        <v>5.188</v>
+        <v>5.191</v>
       </c>
       <c r="P40" t="n">
-        <v>5.388</v>
+        <v>5.391</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.178</v>
+        <v>6.181</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.677</v>
+        <v>3.678</v>
       </c>
       <c r="G41" t="n">
-        <v>3.83</v>
+        <v>3.831</v>
       </c>
       <c r="H41" t="n">
-        <v>4.063</v>
+        <v>4.065</v>
       </c>
       <c r="I41" t="n">
-        <v>4.342</v>
+        <v>4.338</v>
       </c>
       <c r="J41" t="n">
-        <v>4.664</v>
+        <v>4.668</v>
       </c>
       <c r="K41" t="n">
-        <v>5.024</v>
+        <v>5.022</v>
       </c>
       <c r="L41" t="n">
         <v>5.193</v>
       </c>
       <c r="M41" t="n">
-        <v>5.523</v>
+        <v>5.519</v>
       </c>
       <c r="N41" t="n">
-        <v>5.823</v>
+        <v>5.822</v>
       </c>
       <c r="O41" t="n">
-        <v>6.298</v>
+        <v>6.302</v>
       </c>
       <c r="P41" t="n">
-        <v>6.447</v>
+        <v>6.449</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.225</v>
+        <v>7.228</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.414</v>
+        <v>3.415</v>
       </c>
       <c r="G42" t="n">
         <v>3.554</v>
       </c>
       <c r="H42" t="n">
-        <v>3.755</v>
+        <v>3.757</v>
       </c>
       <c r="I42" t="n">
-        <v>4.028</v>
+        <v>4.025</v>
       </c>
       <c r="J42" t="n">
-        <v>4.313</v>
+        <v>4.317</v>
       </c>
       <c r="K42" t="n">
-        <v>4.645</v>
+        <v>4.643</v>
       </c>
       <c r="L42" t="n">
         <v>4.752</v>
       </c>
       <c r="M42" t="n">
-        <v>5.028</v>
+        <v>5.025</v>
       </c>
       <c r="N42" t="n">
-        <v>5.309</v>
+        <v>5.307</v>
       </c>
       <c r="O42" t="n">
-        <v>5.677</v>
+        <v>5.681</v>
       </c>
       <c r="P42" t="n">
-        <v>5.889</v>
+        <v>5.892</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.69</v>
+        <v>6.693</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3551,34 +3551,34 @@
         <v>3.223</v>
       </c>
       <c r="H43" t="n">
-        <v>3.344</v>
+        <v>3.347</v>
       </c>
       <c r="I43" t="n">
-        <v>3.565</v>
+        <v>3.559</v>
       </c>
       <c r="J43" t="n">
-        <v>3.758</v>
+        <v>3.761</v>
       </c>
       <c r="K43" t="n">
-        <v>3.993</v>
+        <v>3.992</v>
       </c>
       <c r="L43" t="n">
         <v>4.04</v>
       </c>
       <c r="M43" t="n">
-        <v>4.166</v>
+        <v>4.163</v>
       </c>
       <c r="N43" t="n">
-        <v>4.196</v>
+        <v>4.195</v>
       </c>
       <c r="O43" t="n">
-        <v>4.275</v>
+        <v>4.279</v>
       </c>
       <c r="P43" t="n">
-        <v>4.362</v>
+        <v>4.365</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.054</v>
+        <v>5.057</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.006</v>
+        <v>3.005</v>
       </c>
       <c r="G44" t="n">
         <v>3.096</v>
       </c>
       <c r="H44" t="n">
-        <v>3.199</v>
+        <v>3.2</v>
       </c>
       <c r="I44" t="n">
-        <v>3.414</v>
+        <v>3.408</v>
       </c>
       <c r="J44" t="n">
-        <v>3.608</v>
+        <v>3.613</v>
       </c>
       <c r="K44" t="n">
-        <v>3.835</v>
+        <v>3.834</v>
       </c>
       <c r="L44" t="n">
         <v>3.882</v>
       </c>
       <c r="M44" t="n">
-        <v>3.981</v>
+        <v>3.977</v>
       </c>
       <c r="N44" t="n">
-        <v>4.011</v>
+        <v>4.01</v>
       </c>
       <c r="O44" t="n">
-        <v>4.072</v>
+        <v>4.076</v>
       </c>
       <c r="P44" t="n">
-        <v>4.126</v>
+        <v>4.128</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.424</v>
+        <v>4.427</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-16 ~ 2026-04-16
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.234</v>
+        <v>3.232</v>
       </c>
       <c r="G2" t="n">
-        <v>3.444</v>
+        <v>3.442</v>
       </c>
       <c r="H2" t="n">
         <v>3.582</v>
       </c>
       <c r="I2" t="n">
-        <v>3.804</v>
+        <v>3.799</v>
       </c>
       <c r="J2" t="n">
-        <v>4.004</v>
+        <v>4.006</v>
       </c>
       <c r="K2" t="n">
-        <v>4.376</v>
+        <v>4.378</v>
       </c>
       <c r="L2" t="n">
-        <v>4.543</v>
+        <v>4.545</v>
       </c>
       <c r="M2" t="n">
-        <v>4.847</v>
+        <v>4.853</v>
       </c>
       <c r="N2" t="n">
-        <v>5.107</v>
+        <v>5.117</v>
       </c>
       <c r="O2" t="n">
-        <v>5.327</v>
+        <v>5.347</v>
       </c>
       <c r="P2" t="n">
-        <v>5.491</v>
+        <v>5.511</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.125</v>
+        <v>6.142</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.257</v>
+        <v>4.256</v>
       </c>
       <c r="G3" t="n">
-        <v>4.648</v>
+        <v>4.647</v>
       </c>
       <c r="H3" t="n">
         <v>4.82</v>
       </c>
       <c r="I3" t="n">
-        <v>5.041</v>
+        <v>5.037</v>
       </c>
       <c r="J3" t="n">
-        <v>5.25</v>
+        <v>5.253</v>
       </c>
       <c r="K3" t="n">
-        <v>5.691</v>
+        <v>5.693</v>
       </c>
       <c r="L3" t="n">
-        <v>5.928</v>
+        <v>5.931</v>
       </c>
       <c r="M3" t="n">
-        <v>6.264</v>
+        <v>6.27</v>
       </c>
       <c r="N3" t="n">
-        <v>6.467</v>
+        <v>6.477</v>
       </c>
       <c r="O3" t="n">
-        <v>6.637</v>
+        <v>6.657</v>
       </c>
       <c r="P3" t="n">
-        <v>6.672</v>
+        <v>6.692</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.193</v>
+        <v>7.21</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.749</v>
+        <v>3.747</v>
       </c>
       <c r="G4" t="n">
-        <v>4.029</v>
+        <v>4.028</v>
       </c>
       <c r="H4" t="n">
-        <v>4.229</v>
+        <v>4.23</v>
       </c>
       <c r="I4" t="n">
-        <v>4.482</v>
+        <v>4.477</v>
       </c>
       <c r="J4" t="n">
-        <v>4.697</v>
+        <v>4.7</v>
       </c>
       <c r="K4" t="n">
-        <v>5.131</v>
+        <v>5.133</v>
       </c>
       <c r="L4" t="n">
-        <v>5.298</v>
+        <v>5.301</v>
       </c>
       <c r="M4" t="n">
-        <v>5.622</v>
+        <v>5.627</v>
       </c>
       <c r="N4" t="n">
-        <v>5.795</v>
+        <v>5.805</v>
       </c>
       <c r="O4" t="n">
-        <v>5.989</v>
+        <v>6.009</v>
       </c>
       <c r="P4" t="n">
-        <v>6.021</v>
+        <v>6.041</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.546</v>
+        <v>6.563</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.939</v>
+        <v>2.934</v>
       </c>
       <c r="G5" t="n">
-        <v>2.991</v>
+        <v>2.986</v>
       </c>
       <c r="H5" t="n">
-        <v>3.083</v>
+        <v>3.082</v>
       </c>
       <c r="I5" t="n">
-        <v>3.375</v>
+        <v>3.37</v>
       </c>
       <c r="J5" t="n">
-        <v>3.57</v>
+        <v>3.573</v>
       </c>
       <c r="K5" t="n">
         <v>3.8</v>
       </c>
       <c r="L5" t="n">
-        <v>3.812</v>
+        <v>3.814</v>
       </c>
       <c r="M5" t="n">
-        <v>3.922</v>
+        <v>3.928</v>
       </c>
       <c r="N5" t="n">
-        <v>3.923</v>
+        <v>3.934</v>
       </c>
       <c r="O5" t="n">
-        <v>3.928</v>
+        <v>3.948</v>
       </c>
       <c r="P5" t="n">
-        <v>4.16</v>
+        <v>4.18</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.037</v>
+        <v>5.054</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.98</v>
+        <v>2.974</v>
       </c>
       <c r="G6" t="n">
-        <v>3.046</v>
+        <v>3.041</v>
       </c>
       <c r="H6" t="n">
-        <v>3.153</v>
+        <v>3.152</v>
       </c>
       <c r="I6" t="n">
-        <v>3.454</v>
+        <v>3.45</v>
       </c>
       <c r="J6" t="n">
-        <v>3.659</v>
+        <v>3.66</v>
       </c>
       <c r="K6" t="n">
         <v>3.907</v>
       </c>
       <c r="L6" t="n">
-        <v>3.929</v>
+        <v>3.93</v>
       </c>
       <c r="M6" t="n">
-        <v>4.073</v>
+        <v>4.077</v>
       </c>
       <c r="N6" t="n">
-        <v>4.089</v>
+        <v>4.1</v>
       </c>
       <c r="O6" t="n">
-        <v>4.195</v>
+        <v>4.215</v>
       </c>
       <c r="P6" t="n">
-        <v>4.592</v>
+        <v>4.612</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.433</v>
+        <v>5.45</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.96</v>
+        <v>2.954</v>
       </c>
       <c r="G7" t="n">
-        <v>3.009</v>
+        <v>3.004</v>
       </c>
       <c r="H7" t="n">
-        <v>3.099</v>
+        <v>3.098</v>
       </c>
       <c r="I7" t="n">
-        <v>3.39</v>
+        <v>3.385</v>
       </c>
       <c r="J7" t="n">
-        <v>3.596</v>
+        <v>3.598</v>
       </c>
       <c r="K7" t="n">
         <v>3.827</v>
       </c>
       <c r="L7" t="n">
-        <v>3.837</v>
+        <v>3.839</v>
       </c>
       <c r="M7" t="n">
-        <v>3.98</v>
+        <v>3.985</v>
       </c>
       <c r="N7" t="n">
-        <v>3.983</v>
+        <v>3.994</v>
       </c>
       <c r="O7" t="n">
-        <v>4.093</v>
+        <v>4.113</v>
       </c>
       <c r="P7" t="n">
-        <v>4.376</v>
+        <v>4.396</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.201</v>
+        <v>5.218</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.367</v>
+        <v>5.365</v>
       </c>
       <c r="G8" t="n">
-        <v>5.946</v>
+        <v>5.944</v>
       </c>
       <c r="H8" t="n">
-        <v>6.269</v>
+        <v>6.27</v>
       </c>
       <c r="I8" t="n">
-        <v>6.561</v>
+        <v>6.556</v>
       </c>
       <c r="J8" t="n">
-        <v>6.835</v>
+        <v>6.837</v>
       </c>
       <c r="K8" t="n">
-        <v>7.557</v>
+        <v>7.559</v>
       </c>
       <c r="L8" t="n">
-        <v>7.883</v>
+        <v>7.886</v>
       </c>
       <c r="M8" t="n">
-        <v>8.247</v>
+        <v>8.253</v>
       </c>
       <c r="N8" t="n">
-        <v>8.388</v>
+        <v>8.398</v>
       </c>
       <c r="O8" t="n">
-        <v>8.644</v>
+        <v>8.664</v>
       </c>
       <c r="P8" t="n">
-        <v>8.779999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.502000000000001</v>
+        <v>9.519</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1069,51 +1069,51 @@
         <v>2.678</v>
       </c>
       <c r="H9" t="n">
-        <v>2.774</v>
+        <v>2.776</v>
       </c>
       <c r="I9" t="n">
-        <v>2.924</v>
+        <v>2.925</v>
       </c>
       <c r="J9" t="n">
-        <v>3.099</v>
+        <v>3.101</v>
       </c>
       <c r="K9" t="n">
         <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>3.247</v>
+        <v>3.248</v>
       </c>
       <c r="M9" t="n">
-        <v>3.332</v>
+        <v>3.337</v>
       </c>
       <c r="N9" t="n">
-        <v>3.49</v>
+        <v>3.5</v>
       </c>
       <c r="O9" t="n">
-        <v>3.52</v>
+        <v>3.54</v>
       </c>
       <c r="P9" t="n">
-        <v>3.58</v>
+        <v>3.6</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.655</v>
+        <v>3.671</v>
       </c>
       <c r="R9" t="n">
-        <v>3.66</v>
+        <v>3.673</v>
       </c>
       <c r="S9" t="n">
-        <v>3.622</v>
+        <v>3.632</v>
       </c>
       <c r="T9" t="n">
-        <v>3.532</v>
+        <v>3.54</v>
       </c>
       <c r="U9" t="n">
-        <v>3.405</v>
+        <v>3.412</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,31 +1139,31 @@
         <v>2.634</v>
       </c>
       <c r="G10" t="n">
-        <v>2.714</v>
+        <v>2.715</v>
       </c>
       <c r="H10" t="n">
-        <v>2.786</v>
+        <v>2.789</v>
       </c>
       <c r="I10" t="n">
-        <v>2.935</v>
+        <v>2.937</v>
       </c>
       <c r="J10" t="n">
-        <v>3.126</v>
+        <v>3.127</v>
       </c>
       <c r="K10" t="n">
-        <v>3.228</v>
+        <v>3.231</v>
       </c>
       <c r="L10" t="n">
-        <v>3.292</v>
+        <v>3.293</v>
       </c>
       <c r="M10" t="n">
-        <v>3.43</v>
+        <v>3.435</v>
       </c>
       <c r="N10" t="n">
-        <v>3.501</v>
+        <v>3.511</v>
       </c>
       <c r="O10" t="n">
-        <v>3.688</v>
+        <v>3.697</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.449</v>
       </c>
       <c r="G11" t="n">
-        <v>2.524</v>
+        <v>2.525</v>
       </c>
       <c r="H11" t="n">
-        <v>2.611</v>
+        <v>2.614</v>
       </c>
       <c r="I11" t="n">
-        <v>2.738</v>
+        <v>2.74</v>
       </c>
       <c r="J11" t="n">
-        <v>2.92</v>
+        <v>2.921</v>
       </c>
       <c r="K11" t="n">
-        <v>3.016</v>
+        <v>3.018</v>
       </c>
       <c r="L11" t="n">
-        <v>3.085</v>
+        <v>3.087</v>
       </c>
       <c r="M11" t="n">
-        <v>3.235</v>
+        <v>3.239</v>
       </c>
       <c r="N11" t="n">
-        <v>3.31</v>
+        <v>3.32</v>
       </c>
       <c r="O11" t="n">
-        <v>3.455</v>
+        <v>3.463</v>
       </c>
       <c r="P11" t="n">
-        <v>3.517</v>
+        <v>3.537</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.858</v>
+        <v>3.875</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1285,43 +1285,43 @@
         <v>3.202</v>
       </c>
       <c r="G12" t="n">
-        <v>3.353</v>
+        <v>3.354</v>
       </c>
       <c r="H12" t="n">
-        <v>3.457</v>
+        <v>3.46</v>
       </c>
       <c r="I12" t="n">
         <v>3.674</v>
       </c>
       <c r="J12" t="n">
-        <v>3.968</v>
+        <v>3.97</v>
       </c>
       <c r="K12" t="n">
-        <v>4.15</v>
+        <v>4.152</v>
       </c>
       <c r="L12" t="n">
-        <v>4.204</v>
+        <v>4.206</v>
       </c>
       <c r="M12" t="n">
-        <v>4.347</v>
+        <v>4.352</v>
       </c>
       <c r="N12" t="n">
-        <v>4.382</v>
+        <v>4.393</v>
       </c>
       <c r="O12" t="n">
-        <v>4.525</v>
+        <v>4.545</v>
       </c>
       <c r="P12" t="n">
-        <v>4.627</v>
+        <v>4.647</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.985</v>
+        <v>5.002</v>
       </c>
       <c r="R12" t="n">
-        <v>5.157</v>
+        <v>5.171</v>
       </c>
       <c r="S12" t="n">
-        <v>5.333</v>
+        <v>5.343</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1358,43 +1358,43 @@
         <v>2.956</v>
       </c>
       <c r="G13" t="n">
-        <v>3.043</v>
+        <v>3.045</v>
       </c>
       <c r="H13" t="n">
-        <v>3.124</v>
+        <v>3.127</v>
       </c>
       <c r="I13" t="n">
         <v>3.322</v>
       </c>
       <c r="J13" t="n">
-        <v>3.605</v>
+        <v>3.607</v>
       </c>
       <c r="K13" t="n">
-        <v>3.784</v>
+        <v>3.786</v>
       </c>
       <c r="L13" t="n">
-        <v>3.843</v>
+        <v>3.845</v>
       </c>
       <c r="M13" t="n">
-        <v>3.975</v>
+        <v>3.979</v>
       </c>
       <c r="N13" t="n">
-        <v>4.01</v>
+        <v>4.021</v>
       </c>
       <c r="O13" t="n">
-        <v>4.154</v>
+        <v>4.174</v>
       </c>
       <c r="P13" t="n">
-        <v>4.219</v>
+        <v>4.239</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.506</v>
+        <v>4.523</v>
       </c>
       <c r="R13" t="n">
-        <v>4.705</v>
+        <v>4.719</v>
       </c>
       <c r="S13" t="n">
-        <v>4.895</v>
+        <v>4.905</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1431,43 +1431,43 @@
         <v>2.774</v>
       </c>
       <c r="G14" t="n">
-        <v>2.85</v>
+        <v>2.851</v>
       </c>
       <c r="H14" t="n">
-        <v>2.927</v>
+        <v>2.93</v>
       </c>
       <c r="I14" t="n">
         <v>3.105</v>
       </c>
       <c r="J14" t="n">
-        <v>3.344</v>
+        <v>3.346</v>
       </c>
       <c r="K14" t="n">
-        <v>3.472</v>
+        <v>3.474</v>
       </c>
       <c r="L14" t="n">
-        <v>3.515</v>
+        <v>3.517</v>
       </c>
       <c r="M14" t="n">
-        <v>3.659</v>
+        <v>3.664</v>
       </c>
       <c r="N14" t="n">
-        <v>3.69</v>
+        <v>3.7</v>
       </c>
       <c r="O14" t="n">
-        <v>3.809</v>
+        <v>3.829</v>
       </c>
       <c r="P14" t="n">
-        <v>3.854</v>
+        <v>3.874</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.095</v>
+        <v>4.112</v>
       </c>
       <c r="R14" t="n">
-        <v>4.22</v>
+        <v>4.234</v>
       </c>
       <c r="S14" t="n">
-        <v>4.348</v>
+        <v>4.358</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1504,43 +1504,43 @@
         <v>2.752</v>
       </c>
       <c r="G15" t="n">
-        <v>2.824</v>
+        <v>2.825</v>
       </c>
       <c r="H15" t="n">
-        <v>2.896</v>
+        <v>2.899</v>
       </c>
       <c r="I15" t="n">
         <v>3.056</v>
       </c>
       <c r="J15" t="n">
-        <v>3.281</v>
+        <v>3.283</v>
       </c>
       <c r="K15" t="n">
-        <v>3.425</v>
+        <v>3.426</v>
       </c>
       <c r="L15" t="n">
-        <v>3.45</v>
+        <v>3.452</v>
       </c>
       <c r="M15" t="n">
-        <v>3.572</v>
+        <v>3.578</v>
       </c>
       <c r="N15" t="n">
-        <v>3.593</v>
+        <v>3.604</v>
       </c>
       <c r="O15" t="n">
-        <v>3.734</v>
+        <v>3.754</v>
       </c>
       <c r="P15" t="n">
-        <v>3.752</v>
+        <v>3.772</v>
       </c>
       <c r="Q15" t="n">
-        <v>4</v>
+        <v>4.017</v>
       </c>
       <c r="R15" t="n">
-        <v>4.117</v>
+        <v>4.13</v>
       </c>
       <c r="S15" t="n">
-        <v>4.243</v>
+        <v>4.253</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1577,43 +1577,43 @@
         <v>2.752</v>
       </c>
       <c r="G16" t="n">
-        <v>2.824</v>
+        <v>2.825</v>
       </c>
       <c r="H16" t="n">
-        <v>2.896</v>
+        <v>2.899</v>
       </c>
       <c r="I16" t="n">
         <v>3.056</v>
       </c>
       <c r="J16" t="n">
-        <v>3.281</v>
+        <v>3.283</v>
       </c>
       <c r="K16" t="n">
-        <v>3.425</v>
+        <v>3.426</v>
       </c>
       <c r="L16" t="n">
-        <v>3.45</v>
+        <v>3.452</v>
       </c>
       <c r="M16" t="n">
-        <v>3.572</v>
+        <v>3.578</v>
       </c>
       <c r="N16" t="n">
-        <v>3.596</v>
+        <v>3.607</v>
       </c>
       <c r="O16" t="n">
-        <v>3.741</v>
+        <v>3.761</v>
       </c>
       <c r="P16" t="n">
-        <v>3.775</v>
+        <v>3.795</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.027</v>
+        <v>4.044</v>
       </c>
       <c r="R16" t="n">
-        <v>4.145</v>
+        <v>4.158</v>
       </c>
       <c r="S16" t="n">
-        <v>4.272</v>
+        <v>4.282</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.699</v>
       </c>
       <c r="G17" t="n">
-        <v>2.805</v>
+        <v>2.806</v>
       </c>
       <c r="H17" t="n">
-        <v>2.881</v>
+        <v>2.884</v>
       </c>
       <c r="I17" t="n">
-        <v>3.018</v>
+        <v>3.02</v>
       </c>
       <c r="J17" t="n">
-        <v>3.196</v>
+        <v>3.197</v>
       </c>
       <c r="K17" t="n">
-        <v>3.303</v>
+        <v>3.305</v>
       </c>
       <c r="L17" t="n">
-        <v>3.369</v>
+        <v>3.372</v>
       </c>
       <c r="M17" t="n">
-        <v>3.549</v>
+        <v>3.554</v>
       </c>
       <c r="N17" t="n">
-        <v>3.602</v>
+        <v>3.612</v>
       </c>
       <c r="O17" t="n">
-        <v>3.723</v>
+        <v>3.732</v>
       </c>
       <c r="P17" t="n">
-        <v>3.795</v>
+        <v>3.813</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.806</v>
+        <v>2.807</v>
       </c>
       <c r="H18" t="n">
-        <v>2.881</v>
+        <v>2.884</v>
       </c>
       <c r="I18" t="n">
-        <v>3.019</v>
+        <v>3.021</v>
       </c>
       <c r="J18" t="n">
-        <v>3.196</v>
+        <v>3.197</v>
       </c>
       <c r="K18" t="n">
-        <v>3.303</v>
+        <v>3.306</v>
       </c>
       <c r="L18" t="n">
-        <v>3.369</v>
+        <v>3.372</v>
       </c>
       <c r="M18" t="n">
-        <v>3.549</v>
+        <v>3.554</v>
       </c>
       <c r="N18" t="n">
-        <v>3.602</v>
+        <v>3.612</v>
       </c>
       <c r="O18" t="n">
-        <v>3.722</v>
+        <v>3.731</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1796,43 +1796,43 @@
         <v>2.764</v>
       </c>
       <c r="G19" t="n">
-        <v>2.841</v>
+        <v>2.842</v>
       </c>
       <c r="H19" t="n">
-        <v>2.917</v>
+        <v>2.92</v>
       </c>
       <c r="I19" t="n">
         <v>3.09</v>
       </c>
       <c r="J19" t="n">
-        <v>3.328</v>
+        <v>3.33</v>
       </c>
       <c r="K19" t="n">
-        <v>3.468</v>
+        <v>3.47</v>
       </c>
       <c r="L19" t="n">
-        <v>3.512</v>
+        <v>3.514</v>
       </c>
       <c r="M19" t="n">
-        <v>3.651</v>
+        <v>3.656</v>
       </c>
       <c r="N19" t="n">
-        <v>3.678</v>
+        <v>3.689</v>
       </c>
       <c r="O19" t="n">
-        <v>3.788</v>
+        <v>3.808</v>
       </c>
       <c r="P19" t="n">
-        <v>3.817</v>
+        <v>3.836</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.044</v>
+        <v>4.06</v>
       </c>
       <c r="R19" t="n">
-        <v>4.169</v>
+        <v>4.181</v>
       </c>
       <c r="S19" t="n">
-        <v>4.286</v>
+        <v>4.296</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1875,19 +1875,19 @@
         <v>2.692</v>
       </c>
       <c r="I20" t="n">
-        <v>2.846</v>
+        <v>2.841</v>
       </c>
       <c r="J20" t="n">
-        <v>3.092</v>
+        <v>3.093</v>
       </c>
       <c r="K20" t="n">
         <v>3.235</v>
       </c>
       <c r="L20" t="n">
-        <v>3.281</v>
+        <v>3.284</v>
       </c>
       <c r="M20" t="n">
-        <v>3.38</v>
+        <v>3.384</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1942,43 +1942,43 @@
         <v>2.867</v>
       </c>
       <c r="G21" t="n">
-        <v>2.946</v>
+        <v>2.945</v>
       </c>
       <c r="H21" t="n">
         <v>3.058</v>
       </c>
       <c r="I21" t="n">
-        <v>3.229</v>
+        <v>3.223</v>
       </c>
       <c r="J21" t="n">
-        <v>3.46</v>
+        <v>3.461</v>
       </c>
       <c r="K21" t="n">
-        <v>3.707</v>
+        <v>3.709</v>
       </c>
       <c r="L21" t="n">
-        <v>3.772</v>
+        <v>3.771</v>
       </c>
       <c r="M21" t="n">
-        <v>3.904</v>
+        <v>3.908</v>
       </c>
       <c r="N21" t="n">
-        <v>3.945</v>
+        <v>3.953</v>
       </c>
       <c r="O21" t="n">
-        <v>4.028</v>
+        <v>4.043</v>
       </c>
       <c r="P21" t="n">
-        <v>4.08</v>
+        <v>4.099</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.207</v>
+        <v>4.224</v>
       </c>
       <c r="R21" t="n">
-        <v>4.217</v>
+        <v>4.231</v>
       </c>
       <c r="S21" t="n">
-        <v>4.247</v>
+        <v>4.257</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.815</v>
+        <v>2.814</v>
       </c>
       <c r="G22" t="n">
-        <v>2.893</v>
+        <v>2.892</v>
       </c>
       <c r="H22" t="n">
-        <v>2.992</v>
+        <v>2.991</v>
       </c>
       <c r="I22" t="n">
-        <v>3.147</v>
+        <v>3.143</v>
       </c>
       <c r="J22" t="n">
-        <v>3.343</v>
+        <v>3.344</v>
       </c>
       <c r="K22" t="n">
-        <v>3.588</v>
+        <v>3.59</v>
       </c>
       <c r="L22" t="n">
-        <v>3.641</v>
+        <v>3.64</v>
       </c>
       <c r="M22" t="n">
-        <v>3.775</v>
+        <v>3.779</v>
       </c>
       <c r="N22" t="n">
-        <v>3.817</v>
+        <v>3.825</v>
       </c>
       <c r="O22" t="n">
-        <v>3.896</v>
+        <v>3.911</v>
       </c>
       <c r="P22" t="n">
-        <v>3.942</v>
+        <v>3.961</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.065</v>
+        <v>4.082</v>
       </c>
       <c r="R22" t="n">
-        <v>4.065</v>
+        <v>4.078</v>
       </c>
       <c r="S22" t="n">
-        <v>4.092</v>
+        <v>4.102</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2088,46 +2088,46 @@
         <v>2.767</v>
       </c>
       <c r="G23" t="n">
-        <v>2.848</v>
+        <v>2.847</v>
       </c>
       <c r="H23" t="n">
-        <v>2.931</v>
+        <v>2.93</v>
       </c>
       <c r="I23" t="n">
-        <v>3.1</v>
+        <v>3.096</v>
       </c>
       <c r="J23" t="n">
-        <v>3.289</v>
+        <v>3.29</v>
       </c>
       <c r="K23" t="n">
-        <v>3.507</v>
+        <v>3.509</v>
       </c>
       <c r="L23" t="n">
-        <v>3.552</v>
+        <v>3.551</v>
       </c>
       <c r="M23" t="n">
-        <v>3.679</v>
+        <v>3.683</v>
       </c>
       <c r="N23" t="n">
-        <v>3.714</v>
+        <v>3.722</v>
       </c>
       <c r="O23" t="n">
-        <v>3.771</v>
+        <v>3.786</v>
       </c>
       <c r="P23" t="n">
-        <v>3.804</v>
+        <v>3.823</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.873</v>
+        <v>3.89</v>
       </c>
       <c r="R23" t="n">
-        <v>3.849</v>
+        <v>3.862</v>
       </c>
       <c r="S23" t="n">
-        <v>3.846</v>
+        <v>3.857</v>
       </c>
       <c r="T23" t="n">
-        <v>3.745</v>
+        <v>3.754</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.699</v>
+        <v>2.7</v>
       </c>
       <c r="G24" t="n">
         <v>2.761</v>
       </c>
       <c r="H24" t="n">
-        <v>2.832</v>
+        <v>2.831</v>
       </c>
       <c r="I24" t="n">
-        <v>3.01</v>
+        <v>3.006</v>
       </c>
       <c r="J24" t="n">
-        <v>3.189</v>
+        <v>3.19</v>
       </c>
       <c r="K24" t="n">
-        <v>3.39</v>
+        <v>3.392</v>
       </c>
       <c r="L24" t="n">
-        <v>3.424</v>
+        <v>3.422</v>
       </c>
       <c r="M24" t="n">
-        <v>3.536</v>
+        <v>3.539</v>
       </c>
       <c r="N24" t="n">
-        <v>3.584</v>
+        <v>3.592</v>
       </c>
       <c r="O24" t="n">
-        <v>3.719</v>
+        <v>3.735</v>
       </c>
       <c r="P24" t="n">
-        <v>3.743</v>
+        <v>3.762</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.795</v>
+        <v>3.812</v>
       </c>
       <c r="R24" t="n">
-        <v>3.769</v>
+        <v>3.783</v>
       </c>
       <c r="S24" t="n">
-        <v>3.761</v>
+        <v>3.772</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.761</v>
+        <v>2.76</v>
       </c>
       <c r="G25" t="n">
-        <v>2.847</v>
+        <v>2.846</v>
       </c>
       <c r="H25" t="n">
-        <v>2.934</v>
+        <v>2.933</v>
       </c>
       <c r="I25" t="n">
-        <v>3.107</v>
+        <v>3.104</v>
       </c>
       <c r="J25" t="n">
-        <v>3.305</v>
+        <v>3.306</v>
       </c>
       <c r="K25" t="n">
-        <v>3.536</v>
+        <v>3.538</v>
       </c>
       <c r="L25" t="n">
-        <v>3.581</v>
+        <v>3.579</v>
       </c>
       <c r="M25" t="n">
-        <v>3.708</v>
+        <v>3.712</v>
       </c>
       <c r="N25" t="n">
-        <v>3.74</v>
+        <v>3.749</v>
       </c>
       <c r="O25" t="n">
-        <v>3.8</v>
+        <v>3.815</v>
       </c>
       <c r="P25" t="n">
-        <v>3.826</v>
+        <v>3.845</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.906</v>
+        <v>3.922</v>
       </c>
       <c r="R25" t="n">
-        <v>3.872</v>
+        <v>3.886</v>
       </c>
       <c r="S25" t="n">
-        <v>3.869</v>
+        <v>3.88</v>
       </c>
       <c r="T25" t="n">
-        <v>3.763</v>
+        <v>3.772</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.077</v>
+        <v>3.074</v>
       </c>
       <c r="G26" t="n">
-        <v>3.204</v>
+        <v>3.202</v>
       </c>
       <c r="H26" t="n">
-        <v>3.396</v>
+        <v>3.398</v>
       </c>
       <c r="I26" t="n">
-        <v>3.643</v>
+        <v>3.64</v>
       </c>
       <c r="J26" t="n">
-        <v>3.962</v>
+        <v>3.966</v>
       </c>
       <c r="K26" t="n">
-        <v>4.326</v>
+        <v>4.327</v>
       </c>
       <c r="L26" t="n">
-        <v>4.424</v>
+        <v>4.427</v>
       </c>
       <c r="M26" t="n">
-        <v>4.617</v>
+        <v>4.623</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.86</v>
+        <v>4.88</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.868</v>
+        <v>2.867</v>
       </c>
       <c r="G27" t="n">
-        <v>2.934</v>
+        <v>2.933</v>
       </c>
       <c r="H27" t="n">
-        <v>3.031</v>
+        <v>3.033</v>
       </c>
       <c r="I27" t="n">
-        <v>3.223</v>
+        <v>3.222</v>
       </c>
       <c r="J27" t="n">
-        <v>3.461</v>
+        <v>3.464</v>
       </c>
       <c r="K27" t="n">
-        <v>3.644</v>
+        <v>3.645</v>
       </c>
       <c r="L27" t="n">
-        <v>3.693</v>
+        <v>3.694</v>
       </c>
       <c r="M27" t="n">
-        <v>3.827</v>
+        <v>3.832</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.951</v>
+        <v>3.971</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2453,31 +2453,31 @@
         <v>2.968</v>
       </c>
       <c r="G28" t="n">
-        <v>3.04</v>
+        <v>3.041</v>
       </c>
       <c r="H28" t="n">
-        <v>3.154</v>
+        <v>3.157</v>
       </c>
       <c r="I28" t="n">
-        <v>3.36</v>
+        <v>3.359</v>
       </c>
       <c r="J28" t="n">
-        <v>3.635</v>
+        <v>3.637</v>
       </c>
       <c r="K28" t="n">
         <v>3.837</v>
       </c>
       <c r="L28" t="n">
-        <v>3.896</v>
+        <v>3.898</v>
       </c>
       <c r="M28" t="n">
-        <v>4.04</v>
+        <v>4.044</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.245</v>
+        <v>4.265</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2529,28 +2529,28 @@
         <v>2.893</v>
       </c>
       <c r="H29" t="n">
-        <v>2.975</v>
+        <v>2.977</v>
       </c>
       <c r="I29" t="n">
-        <v>3.157</v>
+        <v>3.155</v>
       </c>
       <c r="J29" t="n">
-        <v>3.374</v>
+        <v>3.376</v>
       </c>
       <c r="K29" t="n">
-        <v>3.54</v>
+        <v>3.541</v>
       </c>
       <c r="L29" t="n">
-        <v>3.577</v>
+        <v>3.579</v>
       </c>
       <c r="M29" t="n">
-        <v>3.689</v>
+        <v>3.694</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.811</v>
+        <v>3.831</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.102</v>
+        <v>3.101</v>
       </c>
       <c r="G30" t="n">
-        <v>3.168</v>
+        <v>3.166</v>
       </c>
       <c r="H30" t="n">
-        <v>3.322</v>
+        <v>3.326</v>
       </c>
       <c r="I30" t="n">
         <v>3.561</v>
       </c>
       <c r="J30" t="n">
-        <v>3.821</v>
+        <v>3.825</v>
       </c>
       <c r="K30" t="n">
-        <v>4.118</v>
+        <v>4.119</v>
       </c>
       <c r="L30" t="n">
-        <v>4.193</v>
+        <v>4.194</v>
       </c>
       <c r="M30" t="n">
-        <v>4.377</v>
+        <v>4.381</v>
       </c>
       <c r="N30" t="n">
-        <v>4.536</v>
+        <v>4.546</v>
       </c>
       <c r="O30" t="n">
-        <v>4.813</v>
+        <v>4.833</v>
       </c>
       <c r="P30" t="n">
-        <v>4.969</v>
+        <v>4.989</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.73</v>
+        <v>5.747</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.428</v>
+        <v>3.427</v>
       </c>
       <c r="G31" t="n">
-        <v>3.528</v>
+        <v>3.526</v>
       </c>
       <c r="H31" t="n">
-        <v>3.735</v>
+        <v>3.738</v>
       </c>
       <c r="I31" t="n">
-        <v>3.989</v>
+        <v>3.988</v>
       </c>
       <c r="J31" t="n">
-        <v>4.311</v>
+        <v>4.315</v>
       </c>
       <c r="K31" t="n">
-        <v>4.65</v>
+        <v>4.651</v>
       </c>
       <c r="L31" t="n">
-        <v>4.803</v>
+        <v>4.806</v>
       </c>
       <c r="M31" t="n">
-        <v>5.106</v>
+        <v>5.11</v>
       </c>
       <c r="N31" t="n">
-        <v>5.392</v>
+        <v>5.402</v>
       </c>
       <c r="O31" t="n">
-        <v>5.845</v>
+        <v>5.865</v>
       </c>
       <c r="P31" t="n">
-        <v>5.957</v>
+        <v>5.977</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.703</v>
+        <v>6.72</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.2</v>
+        <v>3.199</v>
       </c>
       <c r="G32" t="n">
-        <v>3.284</v>
+        <v>3.282</v>
       </c>
       <c r="H32" t="n">
-        <v>3.465</v>
+        <v>3.469</v>
       </c>
       <c r="I32" t="n">
         <v>3.72</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>4.004</v>
       </c>
       <c r="K32" t="n">
-        <v>4.303</v>
+        <v>4.304</v>
       </c>
       <c r="L32" t="n">
-        <v>4.396</v>
+        <v>4.399</v>
       </c>
       <c r="M32" t="n">
-        <v>4.649</v>
+        <v>4.653</v>
       </c>
       <c r="N32" t="n">
-        <v>4.896</v>
+        <v>4.906</v>
       </c>
       <c r="O32" t="n">
-        <v>5.257</v>
+        <v>5.277</v>
       </c>
       <c r="P32" t="n">
-        <v>5.428</v>
+        <v>5.448</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.191</v>
+        <v>6.208</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.983</v>
+        <v>2.981</v>
       </c>
       <c r="G33" t="n">
-        <v>3.041</v>
+        <v>3.04</v>
       </c>
       <c r="H33" t="n">
-        <v>3.148</v>
+        <v>3.149</v>
       </c>
       <c r="I33" t="n">
         <v>3.349</v>
       </c>
       <c r="J33" t="n">
-        <v>3.533</v>
+        <v>3.537</v>
       </c>
       <c r="K33" t="n">
         <v>3.761</v>
       </c>
       <c r="L33" t="n">
-        <v>3.799</v>
+        <v>3.8</v>
       </c>
       <c r="M33" t="n">
-        <v>3.909</v>
+        <v>3.914</v>
       </c>
       <c r="N33" t="n">
-        <v>3.925</v>
+        <v>3.935</v>
       </c>
       <c r="O33" t="n">
-        <v>3.967</v>
+        <v>3.986</v>
       </c>
       <c r="P33" t="n">
-        <v>3.999</v>
+        <v>4.02</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.447</v>
+        <v>4.464</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.042</v>
+        <v>3.04</v>
       </c>
       <c r="G34" t="n">
-        <v>3.094</v>
+        <v>3.093</v>
       </c>
       <c r="H34" t="n">
-        <v>3.207</v>
+        <v>3.209</v>
       </c>
       <c r="I34" t="n">
         <v>3.417</v>
       </c>
       <c r="J34" t="n">
-        <v>3.605</v>
+        <v>3.609</v>
       </c>
       <c r="K34" t="n">
         <v>3.838</v>
       </c>
       <c r="L34" t="n">
-        <v>3.878</v>
+        <v>3.88</v>
       </c>
       <c r="M34" t="n">
-        <v>4</v>
+        <v>4.005</v>
       </c>
       <c r="N34" t="n">
-        <v>4.029</v>
+        <v>4.039</v>
       </c>
       <c r="O34" t="n">
-        <v>4.135</v>
+        <v>4.155</v>
       </c>
       <c r="P34" t="n">
-        <v>4.294</v>
+        <v>4.314</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.148</v>
+        <v>5.165</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.017</v>
+        <v>3.015</v>
       </c>
       <c r="G35" t="n">
-        <v>3.067</v>
+        <v>3.066</v>
       </c>
       <c r="H35" t="n">
-        <v>3.175</v>
+        <v>3.176</v>
       </c>
       <c r="I35" t="n">
-        <v>3.384</v>
+        <v>3.383</v>
       </c>
       <c r="J35" t="n">
-        <v>3.573</v>
+        <v>3.577</v>
       </c>
       <c r="K35" t="n">
         <v>3.792</v>
       </c>
       <c r="L35" t="n">
-        <v>3.833</v>
+        <v>3.834</v>
       </c>
       <c r="M35" t="n">
-        <v>3.947</v>
+        <v>3.951</v>
       </c>
       <c r="N35" t="n">
-        <v>3.966</v>
+        <v>3.976</v>
       </c>
       <c r="O35" t="n">
-        <v>4.033</v>
+        <v>4.053</v>
       </c>
       <c r="P35" t="n">
-        <v>4.096</v>
+        <v>4.117</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.783</v>
+        <v>4.8</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.927</v>
+        <v>2.925</v>
       </c>
       <c r="G36" t="n">
-        <v>2.986</v>
+        <v>2.984</v>
       </c>
       <c r="H36" t="n">
-        <v>3.076</v>
+        <v>3.077</v>
       </c>
       <c r="I36" t="n">
-        <v>3.28</v>
+        <v>3.278</v>
       </c>
       <c r="J36" t="n">
-        <v>3.471</v>
+        <v>3.475</v>
       </c>
       <c r="K36" t="n">
-        <v>3.683</v>
+        <v>3.685</v>
       </c>
       <c r="L36" t="n">
-        <v>3.722</v>
+        <v>3.724</v>
       </c>
       <c r="M36" t="n">
-        <v>3.808</v>
+        <v>3.813</v>
       </c>
       <c r="N36" t="n">
-        <v>3.828</v>
+        <v>3.838</v>
       </c>
       <c r="O36" t="n">
-        <v>3.877</v>
+        <v>3.897</v>
       </c>
       <c r="P36" t="n">
-        <v>3.898</v>
+        <v>3.919</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.164</v>
+        <v>4.181</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.772</v>
+        <v>3.771</v>
       </c>
       <c r="G37" t="n">
-        <v>4.222</v>
+        <v>4.221</v>
       </c>
       <c r="H37" t="n">
-        <v>4.712</v>
+        <v>4.715</v>
       </c>
       <c r="I37" t="n">
-        <v>5.06</v>
+        <v>5.059</v>
       </c>
       <c r="J37" t="n">
-        <v>5.802</v>
+        <v>5.806</v>
       </c>
       <c r="K37" t="n">
-        <v>6.689</v>
+        <v>6.69</v>
       </c>
       <c r="L37" t="n">
-        <v>7.003</v>
+        <v>7.005</v>
       </c>
       <c r="M37" t="n">
-        <v>7.379</v>
+        <v>7.384</v>
       </c>
       <c r="N37" t="n">
-        <v>7.544</v>
+        <v>7.554</v>
       </c>
       <c r="O37" t="n">
-        <v>7.725</v>
+        <v>7.745</v>
       </c>
       <c r="P37" t="n">
-        <v>7.754</v>
+        <v>7.774</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.195</v>
+        <v>8.212</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.828</v>
+        <v>4.827</v>
       </c>
       <c r="G38" t="n">
-        <v>5.532</v>
+        <v>5.531</v>
       </c>
       <c r="H38" t="n">
-        <v>6.236</v>
+        <v>6.239</v>
       </c>
       <c r="I38" t="n">
-        <v>6.74</v>
+        <v>6.739</v>
       </c>
       <c r="J38" t="n">
-        <v>7.742</v>
+        <v>7.746</v>
       </c>
       <c r="K38" t="n">
-        <v>8.803000000000001</v>
+        <v>8.805</v>
       </c>
       <c r="L38" t="n">
-        <v>9.278</v>
+        <v>9.281000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>9.786</v>
+        <v>9.792</v>
       </c>
       <c r="N38" t="n">
-        <v>9.962</v>
+        <v>9.972</v>
       </c>
       <c r="O38" t="n">
-        <v>10.124</v>
+        <v>10.144</v>
       </c>
       <c r="P38" t="n">
-        <v>10.153</v>
+        <v>10.173</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.646</v>
+        <v>10.663</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.149</v>
+        <v>4.148</v>
       </c>
       <c r="G39" t="n">
-        <v>4.73</v>
+        <v>4.729</v>
       </c>
       <c r="H39" t="n">
-        <v>5.301</v>
+        <v>5.303</v>
       </c>
       <c r="I39" t="n">
-        <v>5.744</v>
+        <v>5.743</v>
       </c>
       <c r="J39" t="n">
-        <v>6.615</v>
+        <v>6.619</v>
       </c>
       <c r="K39" t="n">
-        <v>7.637</v>
+        <v>7.638</v>
       </c>
       <c r="L39" t="n">
-        <v>8.037000000000001</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.423999999999999</v>
+        <v>8.429</v>
       </c>
       <c r="N39" t="n">
-        <v>8.59</v>
+        <v>8.6</v>
       </c>
       <c r="O39" t="n">
-        <v>8.773999999999999</v>
+        <v>8.794</v>
       </c>
       <c r="P39" t="n">
-        <v>8.808</v>
+        <v>8.827999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.291</v>
+        <v>9.308</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.295</v>
+        <v>3.293</v>
       </c>
       <c r="G40" t="n">
-        <v>3.407</v>
+        <v>3.405</v>
       </c>
       <c r="H40" t="n">
-        <v>3.582</v>
+        <v>3.586</v>
       </c>
       <c r="I40" t="n">
         <v>3.836</v>
       </c>
       <c r="J40" t="n">
-        <v>4.114</v>
+        <v>4.118</v>
       </c>
       <c r="K40" t="n">
-        <v>4.422</v>
+        <v>4.424</v>
       </c>
       <c r="L40" t="n">
-        <v>4.517</v>
+        <v>4.518</v>
       </c>
       <c r="M40" t="n">
-        <v>4.718</v>
+        <v>4.722</v>
       </c>
       <c r="N40" t="n">
-        <v>4.893</v>
+        <v>4.903</v>
       </c>
       <c r="O40" t="n">
-        <v>5.191</v>
+        <v>5.211</v>
       </c>
       <c r="P40" t="n">
-        <v>5.391</v>
+        <v>5.411</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.181</v>
+        <v>6.198</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.678</v>
+        <v>3.677</v>
       </c>
       <c r="G41" t="n">
-        <v>3.831</v>
+        <v>3.829</v>
       </c>
       <c r="H41" t="n">
-        <v>4.065</v>
+        <v>4.069</v>
       </c>
       <c r="I41" t="n">
-        <v>4.338</v>
+        <v>4.337</v>
       </c>
       <c r="J41" t="n">
-        <v>4.668</v>
+        <v>4.672</v>
       </c>
       <c r="K41" t="n">
-        <v>5.022</v>
+        <v>5.023</v>
       </c>
       <c r="L41" t="n">
-        <v>5.193</v>
+        <v>5.196</v>
       </c>
       <c r="M41" t="n">
-        <v>5.519</v>
+        <v>5.524</v>
       </c>
       <c r="N41" t="n">
-        <v>5.822</v>
+        <v>5.832</v>
       </c>
       <c r="O41" t="n">
-        <v>6.302</v>
+        <v>6.322</v>
       </c>
       <c r="P41" t="n">
-        <v>6.449</v>
+        <v>6.469</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.228</v>
+        <v>7.245</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.415</v>
+        <v>3.414</v>
       </c>
       <c r="G42" t="n">
-        <v>3.554</v>
+        <v>3.553</v>
       </c>
       <c r="H42" t="n">
-        <v>3.757</v>
+        <v>3.761</v>
       </c>
       <c r="I42" t="n">
-        <v>4.025</v>
+        <v>4.024</v>
       </c>
       <c r="J42" t="n">
-        <v>4.317</v>
+        <v>4.321</v>
       </c>
       <c r="K42" t="n">
-        <v>4.643</v>
+        <v>4.645</v>
       </c>
       <c r="L42" t="n">
-        <v>4.752</v>
+        <v>4.755</v>
       </c>
       <c r="M42" t="n">
-        <v>5.025</v>
+        <v>5.029</v>
       </c>
       <c r="N42" t="n">
-        <v>5.307</v>
+        <v>5.317</v>
       </c>
       <c r="O42" t="n">
-        <v>5.681</v>
+        <v>5.701</v>
       </c>
       <c r="P42" t="n">
-        <v>5.892</v>
+        <v>5.912</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.693</v>
+        <v>6.71</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.131</v>
+        <v>3.129</v>
       </c>
       <c r="G43" t="n">
-        <v>3.223</v>
+        <v>3.222</v>
       </c>
       <c r="H43" t="n">
-        <v>3.347</v>
+        <v>3.348</v>
       </c>
       <c r="I43" t="n">
-        <v>3.559</v>
+        <v>3.558</v>
       </c>
       <c r="J43" t="n">
-        <v>3.761</v>
+        <v>3.765</v>
       </c>
       <c r="K43" t="n">
-        <v>3.992</v>
+        <v>3.993</v>
       </c>
       <c r="L43" t="n">
-        <v>4.04</v>
+        <v>4.042</v>
       </c>
       <c r="M43" t="n">
-        <v>4.163</v>
+        <v>4.168</v>
       </c>
       <c r="N43" t="n">
-        <v>4.195</v>
+        <v>4.205</v>
       </c>
       <c r="O43" t="n">
-        <v>4.279</v>
+        <v>4.299</v>
       </c>
       <c r="P43" t="n">
-        <v>4.365</v>
+        <v>4.386</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.057</v>
+        <v>5.074</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.005</v>
+        <v>3.003</v>
       </c>
       <c r="G44" t="n">
-        <v>3.096</v>
+        <v>3.094</v>
       </c>
       <c r="H44" t="n">
-        <v>3.2</v>
+        <v>3.202</v>
       </c>
       <c r="I44" t="n">
-        <v>3.408</v>
+        <v>3.406</v>
       </c>
       <c r="J44" t="n">
-        <v>3.613</v>
+        <v>3.617</v>
       </c>
       <c r="K44" t="n">
-        <v>3.834</v>
+        <v>3.835</v>
       </c>
       <c r="L44" t="n">
-        <v>3.882</v>
+        <v>3.884</v>
       </c>
       <c r="M44" t="n">
-        <v>3.977</v>
+        <v>3.982</v>
       </c>
       <c r="N44" t="n">
-        <v>4.01</v>
+        <v>4.02</v>
       </c>
       <c r="O44" t="n">
-        <v>4.076</v>
+        <v>4.096</v>
       </c>
       <c r="P44" t="n">
-        <v>4.128</v>
+        <v>4.149</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.427</v>
+        <v>4.444</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-17 ~ 2026-04-17
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.232</v>
+        <v>3.229</v>
       </c>
       <c r="G2" t="n">
-        <v>3.442</v>
+        <v>3.44</v>
       </c>
       <c r="H2" t="n">
         <v>3.582</v>
       </c>
       <c r="I2" t="n">
-        <v>3.799</v>
+        <v>3.8</v>
       </c>
       <c r="J2" t="n">
-        <v>4.006</v>
+        <v>4.028</v>
       </c>
       <c r="K2" t="n">
-        <v>4.378</v>
+        <v>4.4</v>
       </c>
       <c r="L2" t="n">
-        <v>4.545</v>
+        <v>4.574</v>
       </c>
       <c r="M2" t="n">
-        <v>4.853</v>
+        <v>4.885</v>
       </c>
       <c r="N2" t="n">
-        <v>5.117</v>
+        <v>5.153</v>
       </c>
       <c r="O2" t="n">
-        <v>5.347</v>
+        <v>5.385</v>
       </c>
       <c r="P2" t="n">
-        <v>5.511</v>
+        <v>5.551</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.142</v>
+        <v>6.185</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,10 +625,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.256</v>
+        <v>4.253</v>
       </c>
       <c r="G3" t="n">
-        <v>4.647</v>
+        <v>4.645</v>
       </c>
       <c r="H3" t="n">
         <v>4.82</v>
@@ -637,28 +637,28 @@
         <v>5.037</v>
       </c>
       <c r="J3" t="n">
-        <v>5.253</v>
+        <v>5.274</v>
       </c>
       <c r="K3" t="n">
-        <v>5.693</v>
+        <v>5.715</v>
       </c>
       <c r="L3" t="n">
-        <v>5.931</v>
+        <v>5.959</v>
       </c>
       <c r="M3" t="n">
-        <v>6.27</v>
+        <v>6.302</v>
       </c>
       <c r="N3" t="n">
-        <v>6.477</v>
+        <v>6.513</v>
       </c>
       <c r="O3" t="n">
-        <v>6.657</v>
+        <v>6.694</v>
       </c>
       <c r="P3" t="n">
-        <v>6.692</v>
+        <v>6.731</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.21</v>
+        <v>7.253</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.747</v>
+        <v>3.744</v>
       </c>
       <c r="G4" t="n">
-        <v>4.028</v>
+        <v>4.026</v>
       </c>
       <c r="H4" t="n">
-        <v>4.23</v>
+        <v>4.229</v>
       </c>
       <c r="I4" t="n">
-        <v>4.477</v>
+        <v>4.478</v>
       </c>
       <c r="J4" t="n">
-        <v>4.7</v>
+        <v>4.721</v>
       </c>
       <c r="K4" t="n">
-        <v>5.133</v>
+        <v>5.155</v>
       </c>
       <c r="L4" t="n">
-        <v>5.301</v>
+        <v>5.329</v>
       </c>
       <c r="M4" t="n">
-        <v>5.627</v>
+        <v>5.66</v>
       </c>
       <c r="N4" t="n">
-        <v>5.805</v>
+        <v>5.841</v>
       </c>
       <c r="O4" t="n">
-        <v>6.009</v>
+        <v>6.047</v>
       </c>
       <c r="P4" t="n">
-        <v>6.041</v>
+        <v>6.081</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.563</v>
+        <v>6.606</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,10 +771,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.934</v>
+        <v>2.931</v>
       </c>
       <c r="G5" t="n">
-        <v>2.986</v>
+        <v>2.985</v>
       </c>
       <c r="H5" t="n">
         <v>3.082</v>
@@ -783,28 +783,28 @@
         <v>3.37</v>
       </c>
       <c r="J5" t="n">
-        <v>3.573</v>
+        <v>3.593</v>
       </c>
       <c r="K5" t="n">
-        <v>3.8</v>
+        <v>3.824</v>
       </c>
       <c r="L5" t="n">
-        <v>3.814</v>
+        <v>3.844</v>
       </c>
       <c r="M5" t="n">
-        <v>3.928</v>
+        <v>3.96</v>
       </c>
       <c r="N5" t="n">
-        <v>3.934</v>
+        <v>3.97</v>
       </c>
       <c r="O5" t="n">
-        <v>3.948</v>
+        <v>3.985</v>
       </c>
       <c r="P5" t="n">
-        <v>4.18</v>
+        <v>4.22</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.054</v>
+        <v>5.097</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.974</v>
+        <v>2.97</v>
       </c>
       <c r="G6" t="n">
-        <v>3.041</v>
+        <v>3.038</v>
       </c>
       <c r="H6" t="n">
-        <v>3.152</v>
+        <v>3.151</v>
       </c>
       <c r="I6" t="n">
         <v>3.45</v>
       </c>
       <c r="J6" t="n">
-        <v>3.66</v>
+        <v>3.681</v>
       </c>
       <c r="K6" t="n">
-        <v>3.907</v>
+        <v>3.93</v>
       </c>
       <c r="L6" t="n">
-        <v>3.93</v>
+        <v>3.959</v>
       </c>
       <c r="M6" t="n">
-        <v>4.077</v>
+        <v>4.109</v>
       </c>
       <c r="N6" t="n">
-        <v>4.1</v>
+        <v>4.136</v>
       </c>
       <c r="O6" t="n">
-        <v>4.215</v>
+        <v>4.253</v>
       </c>
       <c r="P6" t="n">
-        <v>4.612</v>
+        <v>4.652</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.45</v>
+        <v>5.493</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.954</v>
+        <v>2.951</v>
       </c>
       <c r="G7" t="n">
-        <v>3.004</v>
+        <v>3.002</v>
       </c>
       <c r="H7" t="n">
-        <v>3.098</v>
+        <v>3.097</v>
       </c>
       <c r="I7" t="n">
         <v>3.385</v>
       </c>
       <c r="J7" t="n">
-        <v>3.598</v>
+        <v>3.619</v>
       </c>
       <c r="K7" t="n">
-        <v>3.827</v>
+        <v>3.85</v>
       </c>
       <c r="L7" t="n">
-        <v>3.839</v>
+        <v>3.869</v>
       </c>
       <c r="M7" t="n">
-        <v>3.985</v>
+        <v>4.018</v>
       </c>
       <c r="N7" t="n">
-        <v>3.994</v>
+        <v>4.03</v>
       </c>
       <c r="O7" t="n">
-        <v>4.113</v>
+        <v>4.151</v>
       </c>
       <c r="P7" t="n">
-        <v>4.396</v>
+        <v>4.436</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.218</v>
+        <v>5.261</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.365</v>
+        <v>5.362</v>
       </c>
       <c r="G8" t="n">
-        <v>5.944</v>
+        <v>5.942</v>
       </c>
       <c r="H8" t="n">
-        <v>6.27</v>
+        <v>6.269</v>
       </c>
       <c r="I8" t="n">
-        <v>6.556</v>
+        <v>6.557</v>
       </c>
       <c r="J8" t="n">
-        <v>6.837</v>
+        <v>6.859</v>
       </c>
       <c r="K8" t="n">
-        <v>7.559</v>
+        <v>7.581</v>
       </c>
       <c r="L8" t="n">
-        <v>7.886</v>
+        <v>7.914</v>
       </c>
       <c r="M8" t="n">
-        <v>8.253</v>
+        <v>8.285</v>
       </c>
       <c r="N8" t="n">
-        <v>8.398</v>
+        <v>8.433999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>8.664</v>
+        <v>8.701000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>8.800000000000001</v>
+        <v>8.84</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.519</v>
+        <v>9.561999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1066,54 +1066,54 @@
         <v>2.621</v>
       </c>
       <c r="G9" t="n">
-        <v>2.678</v>
+        <v>2.679</v>
       </c>
       <c r="H9" t="n">
         <v>2.776</v>
       </c>
       <c r="I9" t="n">
-        <v>2.925</v>
+        <v>2.93</v>
       </c>
       <c r="J9" t="n">
-        <v>3.101</v>
+        <v>3.118</v>
       </c>
       <c r="K9" t="n">
-        <v>3.2</v>
+        <v>3.229</v>
       </c>
       <c r="L9" t="n">
-        <v>3.248</v>
+        <v>3.275</v>
       </c>
       <c r="M9" t="n">
-        <v>3.337</v>
+        <v>3.37</v>
       </c>
       <c r="N9" t="n">
-        <v>3.5</v>
+        <v>3.537</v>
       </c>
       <c r="O9" t="n">
-        <v>3.54</v>
+        <v>3.577</v>
       </c>
       <c r="P9" t="n">
-        <v>3.6</v>
+        <v>3.64</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.671</v>
+        <v>3.715</v>
       </c>
       <c r="R9" t="n">
-        <v>3.673</v>
+        <v>3.717</v>
       </c>
       <c r="S9" t="n">
-        <v>3.632</v>
+        <v>3.677</v>
       </c>
       <c r="T9" t="n">
-        <v>3.54</v>
+        <v>3.579</v>
       </c>
       <c r="U9" t="n">
-        <v>3.412</v>
+        <v>3.451</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,31 +1139,31 @@
         <v>2.634</v>
       </c>
       <c r="G10" t="n">
-        <v>2.715</v>
+        <v>2.718</v>
       </c>
       <c r="H10" t="n">
-        <v>2.789</v>
+        <v>2.79</v>
       </c>
       <c r="I10" t="n">
-        <v>2.937</v>
+        <v>2.942</v>
       </c>
       <c r="J10" t="n">
-        <v>3.127</v>
+        <v>3.145</v>
       </c>
       <c r="K10" t="n">
-        <v>3.231</v>
+        <v>3.261</v>
       </c>
       <c r="L10" t="n">
-        <v>3.293</v>
+        <v>3.321</v>
       </c>
       <c r="M10" t="n">
-        <v>3.435</v>
+        <v>3.468</v>
       </c>
       <c r="N10" t="n">
-        <v>3.511</v>
+        <v>3.55</v>
       </c>
       <c r="O10" t="n">
-        <v>3.697</v>
+        <v>3.743</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.449</v>
       </c>
       <c r="G11" t="n">
-        <v>2.525</v>
+        <v>2.528</v>
       </c>
       <c r="H11" t="n">
-        <v>2.614</v>
+        <v>2.615</v>
       </c>
       <c r="I11" t="n">
-        <v>2.74</v>
+        <v>2.746</v>
       </c>
       <c r="J11" t="n">
-        <v>2.921</v>
+        <v>2.939</v>
       </c>
       <c r="K11" t="n">
-        <v>3.018</v>
+        <v>3.048</v>
       </c>
       <c r="L11" t="n">
-        <v>3.087</v>
+        <v>3.115</v>
       </c>
       <c r="M11" t="n">
-        <v>3.239</v>
+        <v>3.272</v>
       </c>
       <c r="N11" t="n">
-        <v>3.32</v>
+        <v>3.358</v>
       </c>
       <c r="O11" t="n">
-        <v>3.463</v>
+        <v>3.51</v>
       </c>
       <c r="P11" t="n">
-        <v>3.537</v>
+        <v>3.58</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.875</v>
+        <v>3.918</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.202</v>
+        <v>3.201</v>
       </c>
       <c r="G12" t="n">
-        <v>3.354</v>
+        <v>3.355</v>
       </c>
       <c r="H12" t="n">
         <v>3.46</v>
       </c>
       <c r="I12" t="n">
-        <v>3.674</v>
+        <v>3.675</v>
       </c>
       <c r="J12" t="n">
-        <v>3.97</v>
+        <v>3.988</v>
       </c>
       <c r="K12" t="n">
-        <v>4.152</v>
+        <v>4.167</v>
       </c>
       <c r="L12" t="n">
-        <v>4.206</v>
+        <v>4.232</v>
       </c>
       <c r="M12" t="n">
-        <v>4.352</v>
+        <v>4.385</v>
       </c>
       <c r="N12" t="n">
-        <v>4.393</v>
+        <v>4.43</v>
       </c>
       <c r="O12" t="n">
-        <v>4.545</v>
+        <v>4.582</v>
       </c>
       <c r="P12" t="n">
-        <v>4.647</v>
+        <v>4.687</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.002</v>
+        <v>5.045</v>
       </c>
       <c r="R12" t="n">
-        <v>5.171</v>
+        <v>5.215</v>
       </c>
       <c r="S12" t="n">
-        <v>5.343</v>
+        <v>5.388</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.956</v>
+        <v>2.955</v>
       </c>
       <c r="G13" t="n">
         <v>3.045</v>
       </c>
       <c r="H13" t="n">
-        <v>3.127</v>
+        <v>3.128</v>
       </c>
       <c r="I13" t="n">
-        <v>3.322</v>
+        <v>3.323</v>
       </c>
       <c r="J13" t="n">
-        <v>3.607</v>
+        <v>3.625</v>
       </c>
       <c r="K13" t="n">
-        <v>3.786</v>
+        <v>3.801</v>
       </c>
       <c r="L13" t="n">
-        <v>3.845</v>
+        <v>3.871</v>
       </c>
       <c r="M13" t="n">
-        <v>3.979</v>
+        <v>4.012</v>
       </c>
       <c r="N13" t="n">
-        <v>4.021</v>
+        <v>4.058</v>
       </c>
       <c r="O13" t="n">
-        <v>4.174</v>
+        <v>4.21</v>
       </c>
       <c r="P13" t="n">
-        <v>4.239</v>
+        <v>4.279</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.523</v>
+        <v>4.566</v>
       </c>
       <c r="R13" t="n">
-        <v>4.719</v>
+        <v>4.763</v>
       </c>
       <c r="S13" t="n">
-        <v>4.905</v>
+        <v>4.95</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.774</v>
+        <v>2.773</v>
       </c>
       <c r="G14" t="n">
-        <v>2.851</v>
+        <v>2.852</v>
       </c>
       <c r="H14" t="n">
-        <v>2.93</v>
+        <v>2.931</v>
       </c>
       <c r="I14" t="n">
-        <v>3.105</v>
+        <v>3.106</v>
       </c>
       <c r="J14" t="n">
-        <v>3.346</v>
+        <v>3.364</v>
       </c>
       <c r="K14" t="n">
-        <v>3.474</v>
+        <v>3.489</v>
       </c>
       <c r="L14" t="n">
-        <v>3.517</v>
+        <v>3.543</v>
       </c>
       <c r="M14" t="n">
-        <v>3.664</v>
+        <v>3.697</v>
       </c>
       <c r="N14" t="n">
-        <v>3.7</v>
+        <v>3.738</v>
       </c>
       <c r="O14" t="n">
-        <v>3.829</v>
+        <v>3.865</v>
       </c>
       <c r="P14" t="n">
-        <v>3.874</v>
+        <v>3.914</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.112</v>
+        <v>4.155</v>
       </c>
       <c r="R14" t="n">
-        <v>4.234</v>
+        <v>4.278</v>
       </c>
       <c r="S14" t="n">
-        <v>4.358</v>
+        <v>4.403</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.752</v>
+        <v>2.751</v>
       </c>
       <c r="G15" t="n">
-        <v>2.825</v>
+        <v>2.826</v>
       </c>
       <c r="H15" t="n">
-        <v>2.899</v>
+        <v>2.9</v>
       </c>
       <c r="I15" t="n">
-        <v>3.056</v>
+        <v>3.058</v>
       </c>
       <c r="J15" t="n">
-        <v>3.283</v>
+        <v>3.301</v>
       </c>
       <c r="K15" t="n">
-        <v>3.426</v>
+        <v>3.442</v>
       </c>
       <c r="L15" t="n">
-        <v>3.452</v>
+        <v>3.478</v>
       </c>
       <c r="M15" t="n">
-        <v>3.578</v>
+        <v>3.61</v>
       </c>
       <c r="N15" t="n">
-        <v>3.604</v>
+        <v>3.641</v>
       </c>
       <c r="O15" t="n">
-        <v>3.754</v>
+        <v>3.791</v>
       </c>
       <c r="P15" t="n">
-        <v>3.772</v>
+        <v>3.812</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.017</v>
+        <v>4.06</v>
       </c>
       <c r="R15" t="n">
-        <v>4.13</v>
+        <v>4.174</v>
       </c>
       <c r="S15" t="n">
-        <v>4.253</v>
+        <v>4.298</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.752</v>
+        <v>2.751</v>
       </c>
       <c r="G16" t="n">
-        <v>2.825</v>
+        <v>2.826</v>
       </c>
       <c r="H16" t="n">
-        <v>2.899</v>
+        <v>2.9</v>
       </c>
       <c r="I16" t="n">
-        <v>3.056</v>
+        <v>3.058</v>
       </c>
       <c r="J16" t="n">
-        <v>3.283</v>
+        <v>3.301</v>
       </c>
       <c r="K16" t="n">
-        <v>3.426</v>
+        <v>3.442</v>
       </c>
       <c r="L16" t="n">
-        <v>3.452</v>
+        <v>3.478</v>
       </c>
       <c r="M16" t="n">
-        <v>3.578</v>
+        <v>3.61</v>
       </c>
       <c r="N16" t="n">
-        <v>3.607</v>
+        <v>3.644</v>
       </c>
       <c r="O16" t="n">
-        <v>3.761</v>
+        <v>3.797</v>
       </c>
       <c r="P16" t="n">
-        <v>3.795</v>
+        <v>3.835</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.044</v>
+        <v>4.087</v>
       </c>
       <c r="R16" t="n">
-        <v>4.158</v>
+        <v>4.202</v>
       </c>
       <c r="S16" t="n">
-        <v>4.282</v>
+        <v>4.327</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.699</v>
       </c>
       <c r="G17" t="n">
-        <v>2.806</v>
+        <v>2.807</v>
       </c>
       <c r="H17" t="n">
-        <v>2.884</v>
+        <v>2.885</v>
       </c>
       <c r="I17" t="n">
-        <v>3.02</v>
+        <v>3.024</v>
       </c>
       <c r="J17" t="n">
-        <v>3.197</v>
+        <v>3.215</v>
       </c>
       <c r="K17" t="n">
-        <v>3.305</v>
+        <v>3.336</v>
       </c>
       <c r="L17" t="n">
-        <v>3.372</v>
+        <v>3.4</v>
       </c>
       <c r="M17" t="n">
-        <v>3.554</v>
+        <v>3.586</v>
       </c>
       <c r="N17" t="n">
-        <v>3.612</v>
+        <v>3.651</v>
       </c>
       <c r="O17" t="n">
-        <v>3.732</v>
+        <v>3.778</v>
       </c>
       <c r="P17" t="n">
-        <v>3.813</v>
+        <v>3.853</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.807</v>
+        <v>2.808</v>
       </c>
       <c r="H18" t="n">
-        <v>2.884</v>
+        <v>2.885</v>
       </c>
       <c r="I18" t="n">
-        <v>3.021</v>
+        <v>3.025</v>
       </c>
       <c r="J18" t="n">
-        <v>3.197</v>
+        <v>3.215</v>
       </c>
       <c r="K18" t="n">
-        <v>3.306</v>
+        <v>3.337</v>
       </c>
       <c r="L18" t="n">
-        <v>3.372</v>
+        <v>3.4</v>
       </c>
       <c r="M18" t="n">
-        <v>3.554</v>
+        <v>3.586</v>
       </c>
       <c r="N18" t="n">
-        <v>3.612</v>
+        <v>3.651</v>
       </c>
       <c r="O18" t="n">
-        <v>3.731</v>
+        <v>3.777</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.764</v>
+        <v>2.763</v>
       </c>
       <c r="G19" t="n">
         <v>2.842</v>
       </c>
       <c r="H19" t="n">
-        <v>2.92</v>
+        <v>2.921</v>
       </c>
       <c r="I19" t="n">
-        <v>3.09</v>
+        <v>3.092</v>
       </c>
       <c r="J19" t="n">
-        <v>3.33</v>
+        <v>3.347</v>
       </c>
       <c r="K19" t="n">
-        <v>3.47</v>
+        <v>3.485</v>
       </c>
       <c r="L19" t="n">
-        <v>3.514</v>
+        <v>3.54</v>
       </c>
       <c r="M19" t="n">
-        <v>3.656</v>
+        <v>3.688</v>
       </c>
       <c r="N19" t="n">
-        <v>3.689</v>
+        <v>3.725</v>
       </c>
       <c r="O19" t="n">
-        <v>3.808</v>
+        <v>3.844</v>
       </c>
       <c r="P19" t="n">
-        <v>3.836</v>
+        <v>3.875</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.06</v>
+        <v>4.102</v>
       </c>
       <c r="R19" t="n">
-        <v>4.181</v>
+        <v>4.224</v>
       </c>
       <c r="S19" t="n">
-        <v>4.296</v>
+        <v>4.341</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,7 +1869,7 @@
         <v>2.574</v>
       </c>
       <c r="G20" t="n">
-        <v>2.644</v>
+        <v>2.645</v>
       </c>
       <c r="H20" t="n">
         <v>2.692</v>
@@ -1878,16 +1878,16 @@
         <v>2.841</v>
       </c>
       <c r="J20" t="n">
-        <v>3.093</v>
+        <v>3.115</v>
       </c>
       <c r="K20" t="n">
-        <v>3.235</v>
+        <v>3.257</v>
       </c>
       <c r="L20" t="n">
-        <v>3.284</v>
+        <v>3.31</v>
       </c>
       <c r="M20" t="n">
-        <v>3.384</v>
+        <v>3.416</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.867</v>
+        <v>2.87</v>
       </c>
       <c r="G21" t="n">
-        <v>2.945</v>
+        <v>2.949</v>
       </c>
       <c r="H21" t="n">
-        <v>3.058</v>
+        <v>3.062</v>
       </c>
       <c r="I21" t="n">
-        <v>3.223</v>
+        <v>3.226</v>
       </c>
       <c r="J21" t="n">
-        <v>3.461</v>
+        <v>3.48</v>
       </c>
       <c r="K21" t="n">
-        <v>3.709</v>
+        <v>3.727</v>
       </c>
       <c r="L21" t="n">
-        <v>3.771</v>
+        <v>3.792</v>
       </c>
       <c r="M21" t="n">
-        <v>3.908</v>
+        <v>3.937</v>
       </c>
       <c r="N21" t="n">
-        <v>3.953</v>
+        <v>3.987</v>
       </c>
       <c r="O21" t="n">
-        <v>4.043</v>
+        <v>4.075</v>
       </c>
       <c r="P21" t="n">
-        <v>4.099</v>
+        <v>4.139</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.224</v>
+        <v>4.267</v>
       </c>
       <c r="R21" t="n">
-        <v>4.231</v>
+        <v>4.274</v>
       </c>
       <c r="S21" t="n">
-        <v>4.257</v>
+        <v>4.302</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.814</v>
+        <v>2.818</v>
       </c>
       <c r="G22" t="n">
-        <v>2.892</v>
+        <v>2.896</v>
       </c>
       <c r="H22" t="n">
-        <v>2.991</v>
+        <v>2.995</v>
       </c>
       <c r="I22" t="n">
-        <v>3.143</v>
+        <v>3.146</v>
       </c>
       <c r="J22" t="n">
-        <v>3.344</v>
+        <v>3.364</v>
       </c>
       <c r="K22" t="n">
-        <v>3.59</v>
+        <v>3.608</v>
       </c>
       <c r="L22" t="n">
-        <v>3.64</v>
+        <v>3.661</v>
       </c>
       <c r="M22" t="n">
-        <v>3.779</v>
+        <v>3.808</v>
       </c>
       <c r="N22" t="n">
-        <v>3.825</v>
+        <v>3.86</v>
       </c>
       <c r="O22" t="n">
-        <v>3.911</v>
+        <v>3.943</v>
       </c>
       <c r="P22" t="n">
-        <v>3.961</v>
+        <v>4.002</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.082</v>
+        <v>4.125</v>
       </c>
       <c r="R22" t="n">
-        <v>4.078</v>
+        <v>4.122</v>
       </c>
       <c r="S22" t="n">
-        <v>4.102</v>
+        <v>4.147</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.767</v>
+        <v>2.77</v>
       </c>
       <c r="G23" t="n">
-        <v>2.847</v>
+        <v>2.851</v>
       </c>
       <c r="H23" t="n">
-        <v>2.93</v>
+        <v>2.934</v>
       </c>
       <c r="I23" t="n">
-        <v>3.096</v>
+        <v>3.099</v>
       </c>
       <c r="J23" t="n">
-        <v>3.29</v>
+        <v>3.31</v>
       </c>
       <c r="K23" t="n">
-        <v>3.509</v>
+        <v>3.527</v>
       </c>
       <c r="L23" t="n">
-        <v>3.551</v>
+        <v>3.572</v>
       </c>
       <c r="M23" t="n">
-        <v>3.683</v>
+        <v>3.713</v>
       </c>
       <c r="N23" t="n">
-        <v>3.722</v>
+        <v>3.756</v>
       </c>
       <c r="O23" t="n">
-        <v>3.786</v>
+        <v>3.818</v>
       </c>
       <c r="P23" t="n">
-        <v>3.823</v>
+        <v>3.863</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.89</v>
+        <v>3.933</v>
       </c>
       <c r="R23" t="n">
-        <v>3.862</v>
+        <v>3.906</v>
       </c>
       <c r="S23" t="n">
-        <v>3.857</v>
+        <v>3.901</v>
       </c>
       <c r="T23" t="n">
-        <v>3.754</v>
+        <v>3.795</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.7</v>
+        <v>2.704</v>
       </c>
       <c r="G24" t="n">
-        <v>2.761</v>
+        <v>2.764</v>
       </c>
       <c r="H24" t="n">
-        <v>2.831</v>
+        <v>2.835</v>
       </c>
       <c r="I24" t="n">
-        <v>3.006</v>
+        <v>3.009</v>
       </c>
       <c r="J24" t="n">
-        <v>3.19</v>
+        <v>3.209</v>
       </c>
       <c r="K24" t="n">
-        <v>3.392</v>
+        <v>3.41</v>
       </c>
       <c r="L24" t="n">
-        <v>3.422</v>
+        <v>3.443</v>
       </c>
       <c r="M24" t="n">
-        <v>3.539</v>
+        <v>3.569</v>
       </c>
       <c r="N24" t="n">
-        <v>3.592</v>
+        <v>3.626</v>
       </c>
       <c r="O24" t="n">
-        <v>3.735</v>
+        <v>3.768</v>
       </c>
       <c r="P24" t="n">
-        <v>3.762</v>
+        <v>3.802</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.812</v>
+        <v>3.855</v>
       </c>
       <c r="R24" t="n">
-        <v>3.783</v>
+        <v>3.827</v>
       </c>
       <c r="S24" t="n">
-        <v>3.772</v>
+        <v>3.817</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.76</v>
+        <v>2.764</v>
       </c>
       <c r="G25" t="n">
-        <v>2.846</v>
+        <v>2.85</v>
       </c>
       <c r="H25" t="n">
-        <v>2.933</v>
+        <v>2.937</v>
       </c>
       <c r="I25" t="n">
-        <v>3.104</v>
+        <v>3.107</v>
       </c>
       <c r="J25" t="n">
-        <v>3.306</v>
+        <v>3.325</v>
       </c>
       <c r="K25" t="n">
-        <v>3.538</v>
+        <v>3.556</v>
       </c>
       <c r="L25" t="n">
-        <v>3.579</v>
+        <v>3.6</v>
       </c>
       <c r="M25" t="n">
-        <v>3.712</v>
+        <v>3.741</v>
       </c>
       <c r="N25" t="n">
-        <v>3.749</v>
+        <v>3.783</v>
       </c>
       <c r="O25" t="n">
-        <v>3.815</v>
+        <v>3.847</v>
       </c>
       <c r="P25" t="n">
-        <v>3.845</v>
+        <v>3.885</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.922</v>
+        <v>3.965</v>
       </c>
       <c r="R25" t="n">
-        <v>3.886</v>
+        <v>3.929</v>
       </c>
       <c r="S25" t="n">
-        <v>3.88</v>
+        <v>3.925</v>
       </c>
       <c r="T25" t="n">
-        <v>3.772</v>
+        <v>3.813</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2307,31 +2307,31 @@
         <v>3.074</v>
       </c>
       <c r="G26" t="n">
-        <v>3.202</v>
+        <v>3.204</v>
       </c>
       <c r="H26" t="n">
-        <v>3.398</v>
+        <v>3.4</v>
       </c>
       <c r="I26" t="n">
-        <v>3.64</v>
+        <v>3.641</v>
       </c>
       <c r="J26" t="n">
-        <v>3.966</v>
+        <v>3.986</v>
       </c>
       <c r="K26" t="n">
-        <v>4.327</v>
+        <v>4.348</v>
       </c>
       <c r="L26" t="n">
-        <v>4.427</v>
+        <v>4.454</v>
       </c>
       <c r="M26" t="n">
-        <v>4.623</v>
+        <v>4.654</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.88</v>
+        <v>4.918</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.867</v>
+        <v>2.866</v>
       </c>
       <c r="G27" t="n">
-        <v>2.933</v>
+        <v>2.936</v>
       </c>
       <c r="H27" t="n">
-        <v>3.033</v>
+        <v>3.035</v>
       </c>
       <c r="I27" t="n">
-        <v>3.222</v>
+        <v>3.224</v>
       </c>
       <c r="J27" t="n">
-        <v>3.464</v>
+        <v>3.483</v>
       </c>
       <c r="K27" t="n">
-        <v>3.645</v>
+        <v>3.662</v>
       </c>
       <c r="L27" t="n">
-        <v>3.694</v>
+        <v>3.721</v>
       </c>
       <c r="M27" t="n">
-        <v>3.832</v>
+        <v>3.864</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.971</v>
+        <v>4.008</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.968</v>
+        <v>2.967</v>
       </c>
       <c r="G28" t="n">
-        <v>3.041</v>
+        <v>3.043</v>
       </c>
       <c r="H28" t="n">
-        <v>3.157</v>
+        <v>3.158</v>
       </c>
       <c r="I28" t="n">
-        <v>3.359</v>
+        <v>3.36</v>
       </c>
       <c r="J28" t="n">
-        <v>3.637</v>
+        <v>3.657</v>
       </c>
       <c r="K28" t="n">
-        <v>3.837</v>
+        <v>3.855</v>
       </c>
       <c r="L28" t="n">
-        <v>3.898</v>
+        <v>3.925</v>
       </c>
       <c r="M28" t="n">
-        <v>4.044</v>
+        <v>4.076</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.265</v>
+        <v>4.301</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.825</v>
+        <v>2.824</v>
       </c>
       <c r="G29" t="n">
-        <v>2.893</v>
+        <v>2.895</v>
       </c>
       <c r="H29" t="n">
-        <v>2.977</v>
+        <v>2.978</v>
       </c>
       <c r="I29" t="n">
-        <v>3.155</v>
+        <v>3.156</v>
       </c>
       <c r="J29" t="n">
-        <v>3.376</v>
+        <v>3.396</v>
       </c>
       <c r="K29" t="n">
-        <v>3.541</v>
+        <v>3.559</v>
       </c>
       <c r="L29" t="n">
-        <v>3.579</v>
+        <v>3.606</v>
       </c>
       <c r="M29" t="n">
-        <v>3.694</v>
+        <v>3.726</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.831</v>
+        <v>3.868</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2599,37 +2599,37 @@
         <v>3.101</v>
       </c>
       <c r="G30" t="n">
-        <v>3.166</v>
+        <v>3.168</v>
       </c>
       <c r="H30" t="n">
-        <v>3.326</v>
+        <v>3.329</v>
       </c>
       <c r="I30" t="n">
-        <v>3.561</v>
+        <v>3.563</v>
       </c>
       <c r="J30" t="n">
-        <v>3.825</v>
+        <v>3.847</v>
       </c>
       <c r="K30" t="n">
-        <v>4.119</v>
+        <v>4.139</v>
       </c>
       <c r="L30" t="n">
-        <v>4.194</v>
+        <v>4.221</v>
       </c>
       <c r="M30" t="n">
-        <v>4.381</v>
+        <v>4.413</v>
       </c>
       <c r="N30" t="n">
-        <v>4.546</v>
+        <v>4.583</v>
       </c>
       <c r="O30" t="n">
-        <v>4.833</v>
+        <v>4.87</v>
       </c>
       <c r="P30" t="n">
-        <v>4.989</v>
+        <v>5.028</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.747</v>
+        <v>5.789</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2672,37 +2672,37 @@
         <v>3.427</v>
       </c>
       <c r="G31" t="n">
-        <v>3.526</v>
+        <v>3.529</v>
       </c>
       <c r="H31" t="n">
-        <v>3.738</v>
+        <v>3.741</v>
       </c>
       <c r="I31" t="n">
-        <v>3.988</v>
+        <v>3.99</v>
       </c>
       <c r="J31" t="n">
-        <v>4.315</v>
+        <v>4.337</v>
       </c>
       <c r="K31" t="n">
-        <v>4.651</v>
+        <v>4.671</v>
       </c>
       <c r="L31" t="n">
-        <v>4.806</v>
+        <v>4.833</v>
       </c>
       <c r="M31" t="n">
-        <v>5.11</v>
+        <v>5.142</v>
       </c>
       <c r="N31" t="n">
-        <v>5.402</v>
+        <v>5.439</v>
       </c>
       <c r="O31" t="n">
-        <v>5.865</v>
+        <v>5.902</v>
       </c>
       <c r="P31" t="n">
-        <v>5.977</v>
+        <v>6.016</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.72</v>
+        <v>6.763</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2745,37 +2745,37 @@
         <v>3.199</v>
       </c>
       <c r="G32" t="n">
-        <v>3.282</v>
+        <v>3.285</v>
       </c>
       <c r="H32" t="n">
-        <v>3.469</v>
+        <v>3.472</v>
       </c>
       <c r="I32" t="n">
-        <v>3.72</v>
+        <v>3.722</v>
       </c>
       <c r="J32" t="n">
-        <v>4.004</v>
+        <v>4.026</v>
       </c>
       <c r="K32" t="n">
-        <v>4.304</v>
+        <v>4.324</v>
       </c>
       <c r="L32" t="n">
-        <v>4.399</v>
+        <v>4.425</v>
       </c>
       <c r="M32" t="n">
-        <v>4.653</v>
+        <v>4.685</v>
       </c>
       <c r="N32" t="n">
-        <v>4.906</v>
+        <v>4.943</v>
       </c>
       <c r="O32" t="n">
-        <v>5.277</v>
+        <v>5.314</v>
       </c>
       <c r="P32" t="n">
-        <v>5.448</v>
+        <v>5.487</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.208</v>
+        <v>6.25</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2818,37 +2818,37 @@
         <v>2.981</v>
       </c>
       <c r="G33" t="n">
-        <v>3.04</v>
+        <v>3.043</v>
       </c>
       <c r="H33" t="n">
-        <v>3.149</v>
+        <v>3.152</v>
       </c>
       <c r="I33" t="n">
-        <v>3.349</v>
+        <v>3.351</v>
       </c>
       <c r="J33" t="n">
-        <v>3.537</v>
+        <v>3.56</v>
       </c>
       <c r="K33" t="n">
-        <v>3.761</v>
+        <v>3.781</v>
       </c>
       <c r="L33" t="n">
-        <v>3.8</v>
+        <v>3.827</v>
       </c>
       <c r="M33" t="n">
-        <v>3.914</v>
+        <v>3.946</v>
       </c>
       <c r="N33" t="n">
-        <v>3.935</v>
+        <v>3.973</v>
       </c>
       <c r="O33" t="n">
-        <v>3.986</v>
+        <v>4.024</v>
       </c>
       <c r="P33" t="n">
-        <v>4.02</v>
+        <v>4.059</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.464</v>
+        <v>4.506</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2891,37 +2891,37 @@
         <v>3.04</v>
       </c>
       <c r="G34" t="n">
-        <v>3.093</v>
+        <v>3.096</v>
       </c>
       <c r="H34" t="n">
-        <v>3.209</v>
+        <v>3.212</v>
       </c>
       <c r="I34" t="n">
-        <v>3.417</v>
+        <v>3.419</v>
       </c>
       <c r="J34" t="n">
-        <v>3.609</v>
+        <v>3.632</v>
       </c>
       <c r="K34" t="n">
-        <v>3.838</v>
+        <v>3.858</v>
       </c>
       <c r="L34" t="n">
-        <v>3.88</v>
+        <v>3.906</v>
       </c>
       <c r="M34" t="n">
-        <v>4.005</v>
+        <v>4.037</v>
       </c>
       <c r="N34" t="n">
-        <v>4.039</v>
+        <v>4.077</v>
       </c>
       <c r="O34" t="n">
-        <v>4.155</v>
+        <v>4.192</v>
       </c>
       <c r="P34" t="n">
-        <v>4.314</v>
+        <v>4.354</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.165</v>
+        <v>5.207</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2964,37 +2964,37 @@
         <v>3.015</v>
       </c>
       <c r="G35" t="n">
-        <v>3.066</v>
+        <v>3.069</v>
       </c>
       <c r="H35" t="n">
-        <v>3.176</v>
+        <v>3.179</v>
       </c>
       <c r="I35" t="n">
-        <v>3.383</v>
+        <v>3.385</v>
       </c>
       <c r="J35" t="n">
-        <v>3.577</v>
+        <v>3.6</v>
       </c>
       <c r="K35" t="n">
-        <v>3.792</v>
+        <v>3.813</v>
       </c>
       <c r="L35" t="n">
-        <v>3.834</v>
+        <v>3.861</v>
       </c>
       <c r="M35" t="n">
-        <v>3.951</v>
+        <v>3.984</v>
       </c>
       <c r="N35" t="n">
-        <v>3.976</v>
+        <v>4.014</v>
       </c>
       <c r="O35" t="n">
-        <v>4.053</v>
+        <v>4.09</v>
       </c>
       <c r="P35" t="n">
-        <v>4.117</v>
+        <v>4.156</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.8</v>
+        <v>4.843</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3037,37 +3037,37 @@
         <v>2.925</v>
       </c>
       <c r="G36" t="n">
-        <v>2.984</v>
+        <v>2.987</v>
       </c>
       <c r="H36" t="n">
-        <v>3.077</v>
+        <v>3.079</v>
       </c>
       <c r="I36" t="n">
-        <v>3.278</v>
+        <v>3.279</v>
       </c>
       <c r="J36" t="n">
-        <v>3.475</v>
+        <v>3.497</v>
       </c>
       <c r="K36" t="n">
-        <v>3.685</v>
+        <v>3.705</v>
       </c>
       <c r="L36" t="n">
-        <v>3.724</v>
+        <v>3.75</v>
       </c>
       <c r="M36" t="n">
-        <v>3.813</v>
+        <v>3.844</v>
       </c>
       <c r="N36" t="n">
-        <v>3.838</v>
+        <v>3.875</v>
       </c>
       <c r="O36" t="n">
-        <v>3.897</v>
+        <v>3.934</v>
       </c>
       <c r="P36" t="n">
-        <v>3.919</v>
+        <v>3.959</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.181</v>
+        <v>4.223</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3110,37 +3110,37 @@
         <v>3.771</v>
       </c>
       <c r="G37" t="n">
-        <v>4.221</v>
+        <v>4.224</v>
       </c>
       <c r="H37" t="n">
-        <v>4.715</v>
+        <v>4.718</v>
       </c>
       <c r="I37" t="n">
-        <v>5.059</v>
+        <v>5.061</v>
       </c>
       <c r="J37" t="n">
-        <v>5.806</v>
+        <v>5.828</v>
       </c>
       <c r="K37" t="n">
-        <v>6.69</v>
+        <v>6.71</v>
       </c>
       <c r="L37" t="n">
-        <v>7.005</v>
+        <v>7.032</v>
       </c>
       <c r="M37" t="n">
-        <v>7.384</v>
+        <v>7.416</v>
       </c>
       <c r="N37" t="n">
-        <v>7.554</v>
+        <v>7.591</v>
       </c>
       <c r="O37" t="n">
-        <v>7.745</v>
+        <v>7.782</v>
       </c>
       <c r="P37" t="n">
-        <v>7.774</v>
+        <v>7.813</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.212</v>
+        <v>8.254</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3183,37 +3183,37 @@
         <v>4.827</v>
       </c>
       <c r="G38" t="n">
-        <v>5.531</v>
+        <v>5.534</v>
       </c>
       <c r="H38" t="n">
-        <v>6.239</v>
+        <v>6.242</v>
       </c>
       <c r="I38" t="n">
-        <v>6.739</v>
+        <v>6.741</v>
       </c>
       <c r="J38" t="n">
-        <v>7.746</v>
+        <v>7.768</v>
       </c>
       <c r="K38" t="n">
-        <v>8.805</v>
+        <v>8.824999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.281000000000001</v>
+        <v>9.308</v>
       </c>
       <c r="M38" t="n">
-        <v>9.792</v>
+        <v>9.824</v>
       </c>
       <c r="N38" t="n">
-        <v>9.972</v>
+        <v>10.009</v>
       </c>
       <c r="O38" t="n">
-        <v>10.144</v>
+        <v>10.181</v>
       </c>
       <c r="P38" t="n">
-        <v>10.173</v>
+        <v>10.212</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.663</v>
+        <v>10.706</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3256,37 +3256,37 @@
         <v>4.148</v>
       </c>
       <c r="G39" t="n">
-        <v>4.729</v>
+        <v>4.732</v>
       </c>
       <c r="H39" t="n">
-        <v>5.303</v>
+        <v>5.306</v>
       </c>
       <c r="I39" t="n">
-        <v>5.743</v>
+        <v>5.745</v>
       </c>
       <c r="J39" t="n">
-        <v>6.619</v>
+        <v>6.64</v>
       </c>
       <c r="K39" t="n">
-        <v>7.638</v>
+        <v>7.659</v>
       </c>
       <c r="L39" t="n">
-        <v>8.039999999999999</v>
+        <v>8.066000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.429</v>
+        <v>8.461</v>
       </c>
       <c r="N39" t="n">
-        <v>8.6</v>
+        <v>8.637</v>
       </c>
       <c r="O39" t="n">
-        <v>8.794</v>
+        <v>8.832000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>8.827999999999999</v>
+        <v>8.867000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.308</v>
+        <v>9.35</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3329,37 +3329,37 @@
         <v>3.293</v>
       </c>
       <c r="G40" t="n">
-        <v>3.405</v>
+        <v>3.408</v>
       </c>
       <c r="H40" t="n">
-        <v>3.586</v>
+        <v>3.589</v>
       </c>
       <c r="I40" t="n">
-        <v>3.836</v>
+        <v>3.838</v>
       </c>
       <c r="J40" t="n">
-        <v>4.118</v>
+        <v>4.139</v>
       </c>
       <c r="K40" t="n">
-        <v>4.424</v>
+        <v>4.444</v>
       </c>
       <c r="L40" t="n">
-        <v>4.518</v>
+        <v>4.545</v>
       </c>
       <c r="M40" t="n">
-        <v>4.722</v>
+        <v>4.754</v>
       </c>
       <c r="N40" t="n">
-        <v>4.903</v>
+        <v>4.94</v>
       </c>
       <c r="O40" t="n">
-        <v>5.211</v>
+        <v>5.249</v>
       </c>
       <c r="P40" t="n">
-        <v>5.411</v>
+        <v>5.45</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.198</v>
+        <v>6.24</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3402,37 +3402,37 @@
         <v>3.677</v>
       </c>
       <c r="G41" t="n">
-        <v>3.829</v>
+        <v>3.832</v>
       </c>
       <c r="H41" t="n">
-        <v>4.069</v>
+        <v>4.072</v>
       </c>
       <c r="I41" t="n">
-        <v>4.337</v>
+        <v>4.339</v>
       </c>
       <c r="J41" t="n">
-        <v>4.672</v>
+        <v>4.693</v>
       </c>
       <c r="K41" t="n">
-        <v>5.023</v>
+        <v>5.044</v>
       </c>
       <c r="L41" t="n">
-        <v>5.196</v>
+        <v>5.223</v>
       </c>
       <c r="M41" t="n">
-        <v>5.524</v>
+        <v>5.556</v>
       </c>
       <c r="N41" t="n">
-        <v>5.832</v>
+        <v>5.869</v>
       </c>
       <c r="O41" t="n">
-        <v>6.322</v>
+        <v>6.359</v>
       </c>
       <c r="P41" t="n">
-        <v>6.469</v>
+        <v>6.508</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.245</v>
+        <v>7.287</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3475,37 +3475,37 @@
         <v>3.414</v>
       </c>
       <c r="G42" t="n">
-        <v>3.553</v>
+        <v>3.556</v>
       </c>
       <c r="H42" t="n">
-        <v>3.761</v>
+        <v>3.764</v>
       </c>
       <c r="I42" t="n">
-        <v>4.024</v>
+        <v>4.026</v>
       </c>
       <c r="J42" t="n">
-        <v>4.321</v>
+        <v>4.343</v>
       </c>
       <c r="K42" t="n">
-        <v>4.645</v>
+        <v>4.665</v>
       </c>
       <c r="L42" t="n">
-        <v>4.755</v>
+        <v>4.781</v>
       </c>
       <c r="M42" t="n">
-        <v>5.029</v>
+        <v>5.061</v>
       </c>
       <c r="N42" t="n">
-        <v>5.317</v>
+        <v>5.354</v>
       </c>
       <c r="O42" t="n">
-        <v>5.701</v>
+        <v>5.738</v>
       </c>
       <c r="P42" t="n">
-        <v>5.912</v>
+        <v>5.951</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.71</v>
+        <v>6.753</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3548,37 +3548,37 @@
         <v>3.129</v>
       </c>
       <c r="G43" t="n">
-        <v>3.222</v>
+        <v>3.225</v>
       </c>
       <c r="H43" t="n">
-        <v>3.348</v>
+        <v>3.351</v>
       </c>
       <c r="I43" t="n">
-        <v>3.558</v>
+        <v>3.56</v>
       </c>
       <c r="J43" t="n">
-        <v>3.765</v>
+        <v>3.788</v>
       </c>
       <c r="K43" t="n">
-        <v>3.993</v>
+        <v>4.013</v>
       </c>
       <c r="L43" t="n">
-        <v>4.042</v>
+        <v>4.068</v>
       </c>
       <c r="M43" t="n">
-        <v>4.168</v>
+        <v>4.2</v>
       </c>
       <c r="N43" t="n">
-        <v>4.205</v>
+        <v>4.242</v>
       </c>
       <c r="O43" t="n">
-        <v>4.299</v>
+        <v>4.336</v>
       </c>
       <c r="P43" t="n">
-        <v>4.386</v>
+        <v>4.425</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.074</v>
+        <v>5.116</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3621,37 +3621,37 @@
         <v>3.003</v>
       </c>
       <c r="G44" t="n">
-        <v>3.094</v>
+        <v>3.097</v>
       </c>
       <c r="H44" t="n">
-        <v>3.202</v>
+        <v>3.204</v>
       </c>
       <c r="I44" t="n">
-        <v>3.406</v>
+        <v>3.407</v>
       </c>
       <c r="J44" t="n">
-        <v>3.617</v>
+        <v>3.638</v>
       </c>
       <c r="K44" t="n">
-        <v>3.835</v>
+        <v>3.855</v>
       </c>
       <c r="L44" t="n">
-        <v>3.884</v>
+        <v>3.91</v>
       </c>
       <c r="M44" t="n">
-        <v>3.982</v>
+        <v>4.013</v>
       </c>
       <c r="N44" t="n">
-        <v>4.02</v>
+        <v>4.057</v>
       </c>
       <c r="O44" t="n">
-        <v>4.096</v>
+        <v>4.133</v>
       </c>
       <c r="P44" t="n">
-        <v>4.149</v>
+        <v>4.189</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.444</v>
+        <v>4.487</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-20 ~ 2026-04-20
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.229</v>
+        <v>3.219</v>
       </c>
       <c r="G2" t="n">
-        <v>3.44</v>
+        <v>3.429</v>
       </c>
       <c r="H2" t="n">
-        <v>3.582</v>
+        <v>3.579</v>
       </c>
       <c r="I2" t="n">
-        <v>3.8</v>
+        <v>3.792</v>
       </c>
       <c r="J2" t="n">
-        <v>4.028</v>
+        <v>4.011</v>
       </c>
       <c r="K2" t="n">
-        <v>4.4</v>
+        <v>4.381</v>
       </c>
       <c r="L2" t="n">
-        <v>4.574</v>
+        <v>4.559</v>
       </c>
       <c r="M2" t="n">
-        <v>4.885</v>
+        <v>4.863</v>
       </c>
       <c r="N2" t="n">
-        <v>5.153</v>
+        <v>5.125</v>
       </c>
       <c r="O2" t="n">
-        <v>5.385</v>
+        <v>5.374</v>
       </c>
       <c r="P2" t="n">
-        <v>5.551</v>
+        <v>5.531</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.185</v>
+        <v>6.155</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.253</v>
+        <v>4.242</v>
       </c>
       <c r="G3" t="n">
-        <v>4.645</v>
+        <v>4.634</v>
       </c>
       <c r="H3" t="n">
-        <v>4.82</v>
+        <v>4.817</v>
       </c>
       <c r="I3" t="n">
-        <v>5.037</v>
+        <v>5.029</v>
       </c>
       <c r="J3" t="n">
-        <v>5.274</v>
+        <v>5.258</v>
       </c>
       <c r="K3" t="n">
-        <v>5.715</v>
+        <v>5.697</v>
       </c>
       <c r="L3" t="n">
-        <v>5.959</v>
+        <v>5.945</v>
       </c>
       <c r="M3" t="n">
-        <v>6.302</v>
+        <v>6.28</v>
       </c>
       <c r="N3" t="n">
-        <v>6.513</v>
+        <v>6.486</v>
       </c>
       <c r="O3" t="n">
-        <v>6.694</v>
+        <v>6.684</v>
       </c>
       <c r="P3" t="n">
-        <v>6.731</v>
+        <v>6.711</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.253</v>
+        <v>7.223</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.744</v>
+        <v>3.734</v>
       </c>
       <c r="G4" t="n">
-        <v>4.026</v>
+        <v>4.015</v>
       </c>
       <c r="H4" t="n">
-        <v>4.229</v>
+        <v>4.227</v>
       </c>
       <c r="I4" t="n">
-        <v>4.478</v>
+        <v>4.47</v>
       </c>
       <c r="J4" t="n">
-        <v>4.721</v>
+        <v>4.704</v>
       </c>
       <c r="K4" t="n">
-        <v>5.155</v>
+        <v>5.137</v>
       </c>
       <c r="L4" t="n">
-        <v>5.329</v>
+        <v>5.314</v>
       </c>
       <c r="M4" t="n">
-        <v>5.66</v>
+        <v>5.638</v>
       </c>
       <c r="N4" t="n">
-        <v>5.841</v>
+        <v>5.814</v>
       </c>
       <c r="O4" t="n">
-        <v>6.047</v>
+        <v>6.036</v>
       </c>
       <c r="P4" t="n">
-        <v>6.081</v>
+        <v>6.061</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.606</v>
+        <v>6.576</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.931</v>
+        <v>2.92</v>
       </c>
       <c r="G5" t="n">
-        <v>2.985</v>
+        <v>2.975</v>
       </c>
       <c r="H5" t="n">
-        <v>3.082</v>
+        <v>3.078</v>
       </c>
       <c r="I5" t="n">
-        <v>3.37</v>
+        <v>3.36</v>
       </c>
       <c r="J5" t="n">
-        <v>3.593</v>
+        <v>3.575</v>
       </c>
       <c r="K5" t="n">
+        <v>3.802</v>
+      </c>
+      <c r="L5" t="n">
         <v>3.824</v>
       </c>
-      <c r="L5" t="n">
-        <v>3.844</v>
-      </c>
       <c r="M5" t="n">
-        <v>3.96</v>
+        <v>3.935</v>
       </c>
       <c r="N5" t="n">
-        <v>3.97</v>
+        <v>3.943</v>
       </c>
       <c r="O5" t="n">
-        <v>3.985</v>
+        <v>3.975</v>
       </c>
       <c r="P5" t="n">
-        <v>4.22</v>
+        <v>4.199</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.097</v>
+        <v>5.067</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.97</v>
+        <v>2.959</v>
       </c>
       <c r="G6" t="n">
-        <v>3.038</v>
+        <v>3.028</v>
       </c>
       <c r="H6" t="n">
-        <v>3.151</v>
+        <v>3.149</v>
       </c>
       <c r="I6" t="n">
-        <v>3.45</v>
+        <v>3.44</v>
       </c>
       <c r="J6" t="n">
-        <v>3.681</v>
+        <v>3.663</v>
       </c>
       <c r="K6" t="n">
-        <v>3.93</v>
+        <v>3.91</v>
       </c>
       <c r="L6" t="n">
-        <v>3.959</v>
+        <v>3.942</v>
       </c>
       <c r="M6" t="n">
-        <v>4.109</v>
+        <v>4.087</v>
       </c>
       <c r="N6" t="n">
-        <v>4.136</v>
+        <v>4.11</v>
       </c>
       <c r="O6" t="n">
-        <v>4.253</v>
+        <v>4.242</v>
       </c>
       <c r="P6" t="n">
-        <v>4.652</v>
+        <v>4.632</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.493</v>
+        <v>5.463</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.951</v>
+        <v>2.94</v>
       </c>
       <c r="G7" t="n">
-        <v>3.002</v>
+        <v>2.992</v>
       </c>
       <c r="H7" t="n">
-        <v>3.097</v>
+        <v>3.093</v>
       </c>
       <c r="I7" t="n">
-        <v>3.385</v>
+        <v>3.375</v>
       </c>
       <c r="J7" t="n">
-        <v>3.619</v>
+        <v>3.601</v>
       </c>
       <c r="K7" t="n">
-        <v>3.85</v>
+        <v>3.829</v>
       </c>
       <c r="L7" t="n">
-        <v>3.869</v>
+        <v>3.849</v>
       </c>
       <c r="M7" t="n">
-        <v>4.018</v>
+        <v>3.993</v>
       </c>
       <c r="N7" t="n">
-        <v>4.03</v>
+        <v>4.003</v>
       </c>
       <c r="O7" t="n">
-        <v>4.151</v>
+        <v>4.14</v>
       </c>
       <c r="P7" t="n">
-        <v>4.436</v>
+        <v>4.415</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.261</v>
+        <v>5.231</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.362</v>
+        <v>5.352</v>
       </c>
       <c r="G8" t="n">
-        <v>5.942</v>
+        <v>5.932</v>
       </c>
       <c r="H8" t="n">
-        <v>6.269</v>
+        <v>6.267</v>
       </c>
       <c r="I8" t="n">
-        <v>6.557</v>
+        <v>6.55</v>
       </c>
       <c r="J8" t="n">
-        <v>6.859</v>
+        <v>6.842</v>
       </c>
       <c r="K8" t="n">
-        <v>7.581</v>
+        <v>7.562</v>
       </c>
       <c r="L8" t="n">
-        <v>7.914</v>
+        <v>7.9</v>
       </c>
       <c r="M8" t="n">
-        <v>8.285</v>
+        <v>8.263</v>
       </c>
       <c r="N8" t="n">
-        <v>8.433999999999999</v>
+        <v>8.407</v>
       </c>
       <c r="O8" t="n">
-        <v>8.701000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="P8" t="n">
-        <v>8.84</v>
+        <v>8.819000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.561999999999999</v>
+        <v>9.532</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.621</v>
+        <v>2.62</v>
       </c>
       <c r="G9" t="n">
         <v>2.679</v>
       </c>
       <c r="H9" t="n">
-        <v>2.776</v>
+        <v>2.764</v>
       </c>
       <c r="I9" t="n">
-        <v>2.93</v>
+        <v>2.925</v>
       </c>
       <c r="J9" t="n">
-        <v>3.118</v>
+        <v>3.113</v>
       </c>
       <c r="K9" t="n">
-        <v>3.229</v>
+        <v>3.215</v>
       </c>
       <c r="L9" t="n">
-        <v>3.275</v>
+        <v>3.259</v>
       </c>
       <c r="M9" t="n">
-        <v>3.37</v>
+        <v>3.347</v>
       </c>
       <c r="N9" t="n">
-        <v>3.537</v>
+        <v>3.509</v>
       </c>
       <c r="O9" t="n">
-        <v>3.577</v>
+        <v>3.567</v>
       </c>
       <c r="P9" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.715</v>
+        <v>3.685</v>
       </c>
       <c r="R9" t="n">
-        <v>3.717</v>
+        <v>3.687</v>
       </c>
       <c r="S9" t="n">
-        <v>3.677</v>
+        <v>3.65</v>
       </c>
       <c r="T9" t="n">
-        <v>3.579</v>
+        <v>3.567</v>
       </c>
       <c r="U9" t="n">
-        <v>3.451</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.634</v>
+        <v>2.633</v>
       </c>
       <c r="G10" t="n">
-        <v>2.718</v>
+        <v>2.717</v>
       </c>
       <c r="H10" t="n">
-        <v>2.79</v>
+        <v>2.779</v>
       </c>
       <c r="I10" t="n">
-        <v>2.942</v>
+        <v>2.938</v>
       </c>
       <c r="J10" t="n">
-        <v>3.145</v>
+        <v>3.139</v>
       </c>
       <c r="K10" t="n">
-        <v>3.261</v>
+        <v>3.247</v>
       </c>
       <c r="L10" t="n">
-        <v>3.321</v>
+        <v>3.306</v>
       </c>
       <c r="M10" t="n">
-        <v>3.468</v>
+        <v>3.445</v>
       </c>
       <c r="N10" t="n">
-        <v>3.55</v>
+        <v>3.522</v>
       </c>
       <c r="O10" t="n">
-        <v>3.743</v>
+        <v>3.732</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.449</v>
+        <v>2.448</v>
       </c>
       <c r="G11" t="n">
-        <v>2.528</v>
+        <v>2.527</v>
       </c>
       <c r="H11" t="n">
-        <v>2.615</v>
+        <v>2.604</v>
       </c>
       <c r="I11" t="n">
-        <v>2.746</v>
+        <v>2.741</v>
       </c>
       <c r="J11" t="n">
-        <v>2.939</v>
+        <v>2.934</v>
       </c>
       <c r="K11" t="n">
-        <v>3.048</v>
+        <v>3.034</v>
       </c>
       <c r="L11" t="n">
-        <v>3.115</v>
+        <v>3.1</v>
       </c>
       <c r="M11" t="n">
-        <v>3.272</v>
+        <v>3.25</v>
       </c>
       <c r="N11" t="n">
-        <v>3.358</v>
+        <v>3.331</v>
       </c>
       <c r="O11" t="n">
-        <v>3.51</v>
+        <v>3.499</v>
       </c>
       <c r="P11" t="n">
-        <v>3.58</v>
+        <v>3.56</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.918</v>
+        <v>3.888</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.201</v>
+        <v>3.198</v>
       </c>
       <c r="G12" t="n">
-        <v>3.355</v>
+        <v>3.351</v>
       </c>
       <c r="H12" t="n">
-        <v>3.46</v>
+        <v>3.457</v>
       </c>
       <c r="I12" t="n">
-        <v>3.675</v>
+        <v>3.673</v>
       </c>
       <c r="J12" t="n">
-        <v>3.988</v>
+        <v>3.977</v>
       </c>
       <c r="K12" t="n">
-        <v>4.167</v>
+        <v>4.152</v>
       </c>
       <c r="L12" t="n">
-        <v>4.232</v>
+        <v>4.215</v>
       </c>
       <c r="M12" t="n">
-        <v>4.385</v>
+        <v>4.362</v>
       </c>
       <c r="N12" t="n">
-        <v>4.43</v>
+        <v>4.403</v>
       </c>
       <c r="O12" t="n">
-        <v>4.582</v>
+        <v>4.571</v>
       </c>
       <c r="P12" t="n">
-        <v>4.687</v>
+        <v>4.667</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.045</v>
+        <v>5.015</v>
       </c>
       <c r="R12" t="n">
-        <v>5.215</v>
+        <v>5.186</v>
       </c>
       <c r="S12" t="n">
-        <v>5.388</v>
+        <v>5.361</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.955</v>
+        <v>2.951</v>
       </c>
       <c r="G13" t="n">
-        <v>3.045</v>
+        <v>3.041</v>
       </c>
       <c r="H13" t="n">
-        <v>3.128</v>
+        <v>3.125</v>
       </c>
       <c r="I13" t="n">
-        <v>3.323</v>
+        <v>3.321</v>
       </c>
       <c r="J13" t="n">
-        <v>3.625</v>
+        <v>3.614</v>
       </c>
       <c r="K13" t="n">
-        <v>3.801</v>
+        <v>3.786</v>
       </c>
       <c r="L13" t="n">
-        <v>3.871</v>
+        <v>3.855</v>
       </c>
       <c r="M13" t="n">
-        <v>4.012</v>
+        <v>3.989</v>
       </c>
       <c r="N13" t="n">
-        <v>4.058</v>
+        <v>4.031</v>
       </c>
       <c r="O13" t="n">
-        <v>4.21</v>
+        <v>4.2</v>
       </c>
       <c r="P13" t="n">
-        <v>4.279</v>
+        <v>4.258</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.566</v>
+        <v>4.536</v>
       </c>
       <c r="R13" t="n">
-        <v>4.763</v>
+        <v>4.734</v>
       </c>
       <c r="S13" t="n">
-        <v>4.95</v>
+        <v>4.923</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.773</v>
+        <v>2.77</v>
       </c>
       <c r="G14" t="n">
-        <v>2.852</v>
+        <v>2.847</v>
       </c>
       <c r="H14" t="n">
-        <v>2.931</v>
+        <v>2.928</v>
       </c>
       <c r="I14" t="n">
-        <v>3.106</v>
+        <v>3.104</v>
       </c>
       <c r="J14" t="n">
-        <v>3.364</v>
+        <v>3.354</v>
       </c>
       <c r="K14" t="n">
-        <v>3.489</v>
+        <v>3.474</v>
       </c>
       <c r="L14" t="n">
-        <v>3.543</v>
+        <v>3.527</v>
       </c>
       <c r="M14" t="n">
-        <v>3.697</v>
+        <v>3.674</v>
       </c>
       <c r="N14" t="n">
-        <v>3.738</v>
+        <v>3.711</v>
       </c>
       <c r="O14" t="n">
-        <v>3.865</v>
+        <v>3.855</v>
       </c>
       <c r="P14" t="n">
-        <v>3.914</v>
+        <v>3.893</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.155</v>
+        <v>4.125</v>
       </c>
       <c r="R14" t="n">
-        <v>4.278</v>
+        <v>4.249</v>
       </c>
       <c r="S14" t="n">
-        <v>4.403</v>
+        <v>4.375</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.751</v>
+        <v>2.749</v>
       </c>
       <c r="G15" t="n">
-        <v>2.826</v>
+        <v>2.821</v>
       </c>
       <c r="H15" t="n">
-        <v>2.9</v>
+        <v>2.897</v>
       </c>
       <c r="I15" t="n">
-        <v>3.058</v>
+        <v>3.057</v>
       </c>
       <c r="J15" t="n">
-        <v>3.301</v>
+        <v>3.293</v>
       </c>
       <c r="K15" t="n">
-        <v>3.442</v>
+        <v>3.426</v>
       </c>
       <c r="L15" t="n">
-        <v>3.478</v>
+        <v>3.462</v>
       </c>
       <c r="M15" t="n">
-        <v>3.61</v>
+        <v>3.588</v>
       </c>
       <c r="N15" t="n">
-        <v>3.641</v>
+        <v>3.614</v>
       </c>
       <c r="O15" t="n">
-        <v>3.791</v>
+        <v>3.78</v>
       </c>
       <c r="P15" t="n">
-        <v>3.812</v>
+        <v>3.792</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.06</v>
+        <v>4.029</v>
       </c>
       <c r="R15" t="n">
-        <v>4.174</v>
+        <v>4.145</v>
       </c>
       <c r="S15" t="n">
-        <v>4.298</v>
+        <v>4.271</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.751</v>
+        <v>2.749</v>
       </c>
       <c r="G16" t="n">
-        <v>2.826</v>
+        <v>2.821</v>
       </c>
       <c r="H16" t="n">
-        <v>2.9</v>
+        <v>2.897</v>
       </c>
       <c r="I16" t="n">
-        <v>3.058</v>
+        <v>3.057</v>
       </c>
       <c r="J16" t="n">
-        <v>3.301</v>
+        <v>3.293</v>
       </c>
       <c r="K16" t="n">
-        <v>3.442</v>
+        <v>3.426</v>
       </c>
       <c r="L16" t="n">
-        <v>3.478</v>
+        <v>3.462</v>
       </c>
       <c r="M16" t="n">
-        <v>3.61</v>
+        <v>3.588</v>
       </c>
       <c r="N16" t="n">
-        <v>3.644</v>
+        <v>3.617</v>
       </c>
       <c r="O16" t="n">
-        <v>3.797</v>
+        <v>3.787</v>
       </c>
       <c r="P16" t="n">
-        <v>3.835</v>
+        <v>3.815</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.087</v>
+        <v>4.057</v>
       </c>
       <c r="R16" t="n">
-        <v>4.202</v>
+        <v>4.173</v>
       </c>
       <c r="S16" t="n">
-        <v>4.327</v>
+        <v>4.3</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.699</v>
+        <v>2.698</v>
       </c>
       <c r="G17" t="n">
         <v>2.807</v>
       </c>
       <c r="H17" t="n">
-        <v>2.885</v>
+        <v>2.874</v>
       </c>
       <c r="I17" t="n">
-        <v>3.024</v>
+        <v>3.02</v>
       </c>
       <c r="J17" t="n">
-        <v>3.215</v>
+        <v>3.21</v>
       </c>
       <c r="K17" t="n">
-        <v>3.336</v>
+        <v>3.322</v>
       </c>
       <c r="L17" t="n">
-        <v>3.4</v>
+        <v>3.385</v>
       </c>
       <c r="M17" t="n">
-        <v>3.586</v>
+        <v>3.563</v>
       </c>
       <c r="N17" t="n">
-        <v>3.651</v>
+        <v>3.624</v>
       </c>
       <c r="O17" t="n">
-        <v>3.778</v>
+        <v>3.767</v>
       </c>
       <c r="P17" t="n">
-        <v>3.853</v>
+        <v>3.832</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.7</v>
+        <v>2.699</v>
       </c>
       <c r="G18" t="n">
         <v>2.808</v>
       </c>
       <c r="H18" t="n">
-        <v>2.885</v>
+        <v>2.874</v>
       </c>
       <c r="I18" t="n">
-        <v>3.025</v>
+        <v>3.02</v>
       </c>
       <c r="J18" t="n">
-        <v>3.215</v>
+        <v>3.21</v>
       </c>
       <c r="K18" t="n">
-        <v>3.337</v>
+        <v>3.323</v>
       </c>
       <c r="L18" t="n">
-        <v>3.4</v>
+        <v>3.385</v>
       </c>
       <c r="M18" t="n">
-        <v>3.586</v>
+        <v>3.563</v>
       </c>
       <c r="N18" t="n">
-        <v>3.651</v>
+        <v>3.624</v>
       </c>
       <c r="O18" t="n">
-        <v>3.777</v>
+        <v>3.765</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.763</v>
+        <v>2.761</v>
       </c>
       <c r="G19" t="n">
-        <v>2.842</v>
+        <v>2.838</v>
       </c>
       <c r="H19" t="n">
-        <v>2.921</v>
+        <v>2.918</v>
       </c>
       <c r="I19" t="n">
-        <v>3.092</v>
+        <v>3.091</v>
       </c>
       <c r="J19" t="n">
-        <v>3.347</v>
+        <v>3.338</v>
       </c>
       <c r="K19" t="n">
-        <v>3.485</v>
+        <v>3.47</v>
       </c>
       <c r="L19" t="n">
-        <v>3.54</v>
+        <v>3.524</v>
       </c>
       <c r="M19" t="n">
-        <v>3.688</v>
+        <v>3.665</v>
       </c>
       <c r="N19" t="n">
-        <v>3.725</v>
+        <v>3.698</v>
       </c>
       <c r="O19" t="n">
-        <v>3.844</v>
+        <v>3.834</v>
       </c>
       <c r="P19" t="n">
-        <v>3.875</v>
+        <v>3.854</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.102</v>
+        <v>4.072</v>
       </c>
       <c r="R19" t="n">
-        <v>4.224</v>
+        <v>4.195</v>
       </c>
       <c r="S19" t="n">
-        <v>4.341</v>
+        <v>4.314</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.574</v>
+        <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.645</v>
+        <v>2.644</v>
       </c>
       <c r="H20" t="n">
-        <v>2.692</v>
+        <v>2.691</v>
       </c>
       <c r="I20" t="n">
-        <v>2.841</v>
+        <v>2.84</v>
       </c>
       <c r="J20" t="n">
-        <v>3.115</v>
+        <v>3.103</v>
       </c>
       <c r="K20" t="n">
-        <v>3.257</v>
+        <v>3.242</v>
       </c>
       <c r="L20" t="n">
-        <v>3.31</v>
+        <v>3.291</v>
       </c>
       <c r="M20" t="n">
-        <v>3.416</v>
+        <v>3.394</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.87</v>
+        <v>2.869</v>
       </c>
       <c r="G21" t="n">
-        <v>2.949</v>
+        <v>2.947</v>
       </c>
       <c r="H21" t="n">
-        <v>3.062</v>
+        <v>3.061</v>
       </c>
       <c r="I21" t="n">
-        <v>3.226</v>
+        <v>3.225</v>
       </c>
       <c r="J21" t="n">
-        <v>3.48</v>
+        <v>3.47</v>
       </c>
       <c r="K21" t="n">
-        <v>3.727</v>
+        <v>3.712</v>
       </c>
       <c r="L21" t="n">
-        <v>3.792</v>
+        <v>3.775</v>
       </c>
       <c r="M21" t="n">
-        <v>3.937</v>
+        <v>3.913</v>
       </c>
       <c r="N21" t="n">
-        <v>3.987</v>
+        <v>3.96</v>
       </c>
       <c r="O21" t="n">
-        <v>4.075</v>
+        <v>4.064</v>
       </c>
       <c r="P21" t="n">
-        <v>4.139</v>
+        <v>4.119</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.267</v>
+        <v>4.237</v>
       </c>
       <c r="R21" t="n">
-        <v>4.274</v>
+        <v>4.245</v>
       </c>
       <c r="S21" t="n">
-        <v>4.302</v>
+        <v>4.275</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.818</v>
+        <v>2.817</v>
       </c>
       <c r="G22" t="n">
-        <v>2.896</v>
+        <v>2.894</v>
       </c>
       <c r="H22" t="n">
-        <v>2.995</v>
+        <v>2.993</v>
       </c>
       <c r="I22" t="n">
-        <v>3.146</v>
+        <v>3.145</v>
       </c>
       <c r="J22" t="n">
-        <v>3.364</v>
+        <v>3.353</v>
       </c>
       <c r="K22" t="n">
-        <v>3.608</v>
+        <v>3.592</v>
       </c>
       <c r="L22" t="n">
-        <v>3.661</v>
+        <v>3.643</v>
       </c>
       <c r="M22" t="n">
-        <v>3.808</v>
+        <v>3.783</v>
       </c>
       <c r="N22" t="n">
-        <v>3.86</v>
+        <v>3.833</v>
       </c>
       <c r="O22" t="n">
-        <v>3.943</v>
+        <v>3.932</v>
       </c>
       <c r="P22" t="n">
-        <v>4.002</v>
+        <v>3.981</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.125</v>
+        <v>4.095</v>
       </c>
       <c r="R22" t="n">
-        <v>4.122</v>
+        <v>4.093</v>
       </c>
       <c r="S22" t="n">
-        <v>4.147</v>
+        <v>4.12</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.77</v>
+        <v>2.769</v>
       </c>
       <c r="G23" t="n">
-        <v>2.851</v>
+        <v>2.849</v>
       </c>
       <c r="H23" t="n">
-        <v>2.934</v>
+        <v>2.933</v>
       </c>
       <c r="I23" t="n">
-        <v>3.099</v>
+        <v>3.098</v>
       </c>
       <c r="J23" t="n">
-        <v>3.31</v>
+        <v>3.299</v>
       </c>
       <c r="K23" t="n">
-        <v>3.527</v>
+        <v>3.511</v>
       </c>
       <c r="L23" t="n">
-        <v>3.572</v>
+        <v>3.554</v>
       </c>
       <c r="M23" t="n">
-        <v>3.713</v>
+        <v>3.687</v>
       </c>
       <c r="N23" t="n">
-        <v>3.756</v>
+        <v>3.729</v>
       </c>
       <c r="O23" t="n">
-        <v>3.818</v>
+        <v>3.806</v>
       </c>
       <c r="P23" t="n">
-        <v>3.863</v>
+        <v>3.842</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.933</v>
+        <v>3.903</v>
       </c>
       <c r="R23" t="n">
-        <v>3.906</v>
+        <v>3.877</v>
       </c>
       <c r="S23" t="n">
-        <v>3.901</v>
+        <v>3.875</v>
       </c>
       <c r="T23" t="n">
-        <v>3.795</v>
+        <v>3.782</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.704</v>
+        <v>2.703</v>
       </c>
       <c r="G24" t="n">
-        <v>2.764</v>
+        <v>2.763</v>
       </c>
       <c r="H24" t="n">
-        <v>2.835</v>
+        <v>2.834</v>
       </c>
       <c r="I24" t="n">
-        <v>3.009</v>
+        <v>3.008</v>
       </c>
       <c r="J24" t="n">
-        <v>3.209</v>
+        <v>3.198</v>
       </c>
       <c r="K24" t="n">
-        <v>3.41</v>
+        <v>3.395</v>
       </c>
       <c r="L24" t="n">
-        <v>3.443</v>
+        <v>3.426</v>
       </c>
       <c r="M24" t="n">
-        <v>3.569</v>
+        <v>3.545</v>
       </c>
       <c r="N24" t="n">
-        <v>3.626</v>
+        <v>3.599</v>
       </c>
       <c r="O24" t="n">
-        <v>3.768</v>
+        <v>3.757</v>
       </c>
       <c r="P24" t="n">
-        <v>3.802</v>
+        <v>3.781</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.855</v>
+        <v>3.825</v>
       </c>
       <c r="R24" t="n">
-        <v>3.827</v>
+        <v>3.798</v>
       </c>
       <c r="S24" t="n">
-        <v>3.817</v>
+        <v>3.79</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.764</v>
+        <v>2.763</v>
       </c>
       <c r="G25" t="n">
-        <v>2.85</v>
+        <v>2.848</v>
       </c>
       <c r="H25" t="n">
-        <v>2.937</v>
+        <v>2.936</v>
       </c>
       <c r="I25" t="n">
-        <v>3.107</v>
+        <v>3.106</v>
       </c>
       <c r="J25" t="n">
-        <v>3.325</v>
+        <v>3.315</v>
       </c>
       <c r="K25" t="n">
-        <v>3.556</v>
+        <v>3.541</v>
       </c>
       <c r="L25" t="n">
-        <v>3.6</v>
+        <v>3.583</v>
       </c>
       <c r="M25" t="n">
-        <v>3.741</v>
+        <v>3.717</v>
       </c>
       <c r="N25" t="n">
-        <v>3.783</v>
+        <v>3.756</v>
       </c>
       <c r="O25" t="n">
-        <v>3.847</v>
+        <v>3.835</v>
       </c>
       <c r="P25" t="n">
-        <v>3.885</v>
+        <v>3.864</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.965</v>
+        <v>3.936</v>
       </c>
       <c r="R25" t="n">
-        <v>3.929</v>
+        <v>3.9</v>
       </c>
       <c r="S25" t="n">
-        <v>3.925</v>
+        <v>3.898</v>
       </c>
       <c r="T25" t="n">
-        <v>3.813</v>
+        <v>3.8</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.074</v>
+        <v>3.067</v>
       </c>
       <c r="G26" t="n">
-        <v>3.204</v>
+        <v>3.199</v>
       </c>
       <c r="H26" t="n">
-        <v>3.4</v>
+        <v>3.397</v>
       </c>
       <c r="I26" t="n">
-        <v>3.641</v>
+        <v>3.636</v>
       </c>
       <c r="J26" t="n">
-        <v>3.986</v>
+        <v>3.974</v>
       </c>
       <c r="K26" t="n">
-        <v>4.348</v>
+        <v>4.332</v>
       </c>
       <c r="L26" t="n">
-        <v>4.454</v>
+        <v>4.438</v>
       </c>
       <c r="M26" t="n">
-        <v>4.654</v>
+        <v>4.631</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.918</v>
+        <v>4.907</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.866</v>
+        <v>2.86</v>
       </c>
       <c r="G27" t="n">
-        <v>2.936</v>
+        <v>2.929</v>
       </c>
       <c r="H27" t="n">
-        <v>3.035</v>
+        <v>3.032</v>
       </c>
       <c r="I27" t="n">
-        <v>3.224</v>
+        <v>3.219</v>
       </c>
       <c r="J27" t="n">
-        <v>3.483</v>
+        <v>3.473</v>
       </c>
       <c r="K27" t="n">
-        <v>3.662</v>
+        <v>3.647</v>
       </c>
       <c r="L27" t="n">
-        <v>3.721</v>
+        <v>3.706</v>
       </c>
       <c r="M27" t="n">
-        <v>3.864</v>
+        <v>3.841</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.008</v>
+        <v>3.997</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.967</v>
+        <v>2.964</v>
       </c>
       <c r="G28" t="n">
-        <v>3.043</v>
+        <v>3.039</v>
       </c>
       <c r="H28" t="n">
-        <v>3.158</v>
+        <v>3.156</v>
       </c>
       <c r="I28" t="n">
-        <v>3.36</v>
+        <v>3.357</v>
       </c>
       <c r="J28" t="n">
-        <v>3.657</v>
+        <v>3.646</v>
       </c>
       <c r="K28" t="n">
-        <v>3.855</v>
+        <v>3.84</v>
       </c>
       <c r="L28" t="n">
-        <v>3.925</v>
+        <v>3.909</v>
       </c>
       <c r="M28" t="n">
-        <v>4.076</v>
+        <v>4.053</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.301</v>
+        <v>4.291</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.824</v>
+        <v>2.819</v>
       </c>
       <c r="G29" t="n">
-        <v>2.895</v>
+        <v>2.886</v>
       </c>
       <c r="H29" t="n">
-        <v>2.978</v>
+        <v>2.975</v>
       </c>
       <c r="I29" t="n">
-        <v>3.156</v>
+        <v>3.153</v>
       </c>
       <c r="J29" t="n">
-        <v>3.396</v>
+        <v>3.385</v>
       </c>
       <c r="K29" t="n">
-        <v>3.559</v>
+        <v>3.543</v>
       </c>
       <c r="L29" t="n">
-        <v>3.606</v>
+        <v>3.59</v>
       </c>
       <c r="M29" t="n">
-        <v>3.726</v>
+        <v>3.703</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.868</v>
+        <v>3.857</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.101</v>
+        <v>3.097</v>
       </c>
       <c r="G30" t="n">
-        <v>3.168</v>
+        <v>3.166</v>
       </c>
       <c r="H30" t="n">
-        <v>3.329</v>
+        <v>3.328</v>
       </c>
       <c r="I30" t="n">
-        <v>3.563</v>
+        <v>3.561</v>
       </c>
       <c r="J30" t="n">
-        <v>3.847</v>
+        <v>3.835</v>
       </c>
       <c r="K30" t="n">
-        <v>4.139</v>
+        <v>4.123</v>
       </c>
       <c r="L30" t="n">
-        <v>4.221</v>
+        <v>4.206</v>
       </c>
       <c r="M30" t="n">
-        <v>4.413</v>
+        <v>4.39</v>
       </c>
       <c r="N30" t="n">
-        <v>4.583</v>
+        <v>4.555</v>
       </c>
       <c r="O30" t="n">
-        <v>4.87</v>
+        <v>4.858</v>
       </c>
       <c r="P30" t="n">
-        <v>5.028</v>
+        <v>5.008</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.789</v>
+        <v>5.759</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.427</v>
+        <v>3.423</v>
       </c>
       <c r="G31" t="n">
-        <v>3.529</v>
+        <v>3.526</v>
       </c>
       <c r="H31" t="n">
-        <v>3.741</v>
+        <v>3.74</v>
       </c>
       <c r="I31" t="n">
-        <v>3.99</v>
+        <v>3.988</v>
       </c>
       <c r="J31" t="n">
-        <v>4.337</v>
+        <v>4.325</v>
       </c>
       <c r="K31" t="n">
-        <v>4.671</v>
+        <v>4.655</v>
       </c>
       <c r="L31" t="n">
-        <v>4.833</v>
+        <v>4.818</v>
       </c>
       <c r="M31" t="n">
-        <v>5.142</v>
+        <v>5.119</v>
       </c>
       <c r="N31" t="n">
-        <v>5.439</v>
+        <v>5.412</v>
       </c>
       <c r="O31" t="n">
-        <v>5.902</v>
+        <v>5.89</v>
       </c>
       <c r="P31" t="n">
-        <v>6.016</v>
+        <v>5.995</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.763</v>
+        <v>6.733</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.199</v>
+        <v>3.195</v>
       </c>
       <c r="G32" t="n">
-        <v>3.285</v>
+        <v>3.282</v>
       </c>
       <c r="H32" t="n">
-        <v>3.472</v>
+        <v>3.471</v>
       </c>
       <c r="I32" t="n">
-        <v>3.722</v>
+        <v>3.72</v>
       </c>
       <c r="J32" t="n">
-        <v>4.026</v>
+        <v>4.014</v>
       </c>
       <c r="K32" t="n">
-        <v>4.324</v>
+        <v>4.308</v>
       </c>
       <c r="L32" t="n">
-        <v>4.425</v>
+        <v>4.41</v>
       </c>
       <c r="M32" t="n">
-        <v>4.685</v>
+        <v>4.662</v>
       </c>
       <c r="N32" t="n">
-        <v>4.943</v>
+        <v>4.916</v>
       </c>
       <c r="O32" t="n">
-        <v>5.314</v>
+        <v>5.302</v>
       </c>
       <c r="P32" t="n">
-        <v>5.487</v>
+        <v>5.467</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.25</v>
+        <v>6.22</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.981</v>
+        <v>2.973</v>
       </c>
       <c r="G33" t="n">
-        <v>3.043</v>
+        <v>3.036</v>
       </c>
       <c r="H33" t="n">
-        <v>3.152</v>
+        <v>3.15</v>
       </c>
       <c r="I33" t="n">
-        <v>3.351</v>
+        <v>3.347</v>
       </c>
       <c r="J33" t="n">
-        <v>3.56</v>
+        <v>3.549</v>
       </c>
       <c r="K33" t="n">
-        <v>3.781</v>
+        <v>3.766</v>
       </c>
       <c r="L33" t="n">
-        <v>3.827</v>
+        <v>3.812</v>
       </c>
       <c r="M33" t="n">
+        <v>3.923</v>
+      </c>
+      <c r="N33" t="n">
         <v>3.946</v>
       </c>
-      <c r="N33" t="n">
-        <v>3.973</v>
-      </c>
       <c r="O33" t="n">
-        <v>4.024</v>
+        <v>4.012</v>
       </c>
       <c r="P33" t="n">
-        <v>4.059</v>
+        <v>4.039</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.506</v>
+        <v>4.476</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.04</v>
+        <v>3.032</v>
       </c>
       <c r="G34" t="n">
-        <v>3.096</v>
+        <v>3.089</v>
       </c>
       <c r="H34" t="n">
-        <v>3.212</v>
+        <v>3.21</v>
       </c>
       <c r="I34" t="n">
-        <v>3.419</v>
+        <v>3.415</v>
       </c>
       <c r="J34" t="n">
-        <v>3.632</v>
+        <v>3.621</v>
       </c>
       <c r="K34" t="n">
-        <v>3.858</v>
+        <v>3.843</v>
       </c>
       <c r="L34" t="n">
-        <v>3.906</v>
+        <v>3.891</v>
       </c>
       <c r="M34" t="n">
-        <v>4.037</v>
+        <v>4.014</v>
       </c>
       <c r="N34" t="n">
-        <v>4.077</v>
+        <v>4.05</v>
       </c>
       <c r="O34" t="n">
-        <v>4.192</v>
+        <v>4.18</v>
       </c>
       <c r="P34" t="n">
-        <v>4.354</v>
+        <v>4.334</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.207</v>
+        <v>5.177</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.015</v>
+        <v>3.007</v>
       </c>
       <c r="G35" t="n">
-        <v>3.069</v>
+        <v>3.062</v>
       </c>
       <c r="H35" t="n">
-        <v>3.179</v>
+        <v>3.177</v>
       </c>
       <c r="I35" t="n">
-        <v>3.385</v>
+        <v>3.382</v>
       </c>
       <c r="J35" t="n">
-        <v>3.6</v>
+        <v>3.589</v>
       </c>
       <c r="K35" t="n">
-        <v>3.813</v>
+        <v>3.797</v>
       </c>
       <c r="L35" t="n">
-        <v>3.861</v>
+        <v>3.846</v>
       </c>
       <c r="M35" t="n">
-        <v>3.984</v>
+        <v>3.961</v>
       </c>
       <c r="N35" t="n">
-        <v>4.014</v>
+        <v>3.987</v>
       </c>
       <c r="O35" t="n">
-        <v>4.09</v>
+        <v>4.078</v>
       </c>
       <c r="P35" t="n">
-        <v>4.156</v>
+        <v>4.136</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.843</v>
+        <v>4.813</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.925</v>
+        <v>2.917</v>
       </c>
       <c r="G36" t="n">
-        <v>2.987</v>
+        <v>2.978</v>
       </c>
       <c r="H36" t="n">
-        <v>3.079</v>
+        <v>3.076</v>
       </c>
       <c r="I36" t="n">
-        <v>3.279</v>
+        <v>3.275</v>
       </c>
       <c r="J36" t="n">
-        <v>3.497</v>
+        <v>3.485</v>
       </c>
       <c r="K36" t="n">
-        <v>3.705</v>
+        <v>3.689</v>
       </c>
       <c r="L36" t="n">
-        <v>3.75</v>
+        <v>3.735</v>
       </c>
       <c r="M36" t="n">
-        <v>3.844</v>
+        <v>3.821</v>
       </c>
       <c r="N36" t="n">
-        <v>3.875</v>
+        <v>3.848</v>
       </c>
       <c r="O36" t="n">
-        <v>3.934</v>
+        <v>3.923</v>
       </c>
       <c r="P36" t="n">
-        <v>3.959</v>
+        <v>3.938</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.223</v>
+        <v>4.193</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.771</v>
+        <v>3.767</v>
       </c>
       <c r="G37" t="n">
-        <v>4.224</v>
+        <v>4.221</v>
       </c>
       <c r="H37" t="n">
-        <v>4.718</v>
+        <v>4.717</v>
       </c>
       <c r="I37" t="n">
-        <v>5.061</v>
+        <v>5.059</v>
       </c>
       <c r="J37" t="n">
-        <v>5.828</v>
+        <v>5.816</v>
       </c>
       <c r="K37" t="n">
-        <v>6.71</v>
+        <v>6.694</v>
       </c>
       <c r="L37" t="n">
-        <v>7.032</v>
+        <v>7.017</v>
       </c>
       <c r="M37" t="n">
-        <v>7.416</v>
+        <v>7.393</v>
       </c>
       <c r="N37" t="n">
-        <v>7.591</v>
+        <v>7.564</v>
       </c>
       <c r="O37" t="n">
-        <v>7.782</v>
+        <v>7.77</v>
       </c>
       <c r="P37" t="n">
-        <v>7.813</v>
+        <v>7.794</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.254</v>
+        <v>8.224</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.827</v>
+        <v>4.823</v>
       </c>
       <c r="G38" t="n">
-        <v>5.534</v>
+        <v>5.531</v>
       </c>
       <c r="H38" t="n">
-        <v>6.242</v>
+        <v>6.241</v>
       </c>
       <c r="I38" t="n">
-        <v>6.741</v>
+        <v>6.739</v>
       </c>
       <c r="J38" t="n">
-        <v>7.768</v>
+        <v>7.756</v>
       </c>
       <c r="K38" t="n">
-        <v>8.824999999999999</v>
+        <v>8.808999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.308</v>
+        <v>9.292999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>9.824</v>
+        <v>9.801</v>
       </c>
       <c r="N38" t="n">
-        <v>10.009</v>
+        <v>9.981999999999999</v>
       </c>
       <c r="O38" t="n">
-        <v>10.181</v>
+        <v>10.17</v>
       </c>
       <c r="P38" t="n">
-        <v>10.212</v>
+        <v>10.192</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.706</v>
+        <v>10.675</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.148</v>
+        <v>4.144</v>
       </c>
       <c r="G39" t="n">
-        <v>4.732</v>
+        <v>4.729</v>
       </c>
       <c r="H39" t="n">
-        <v>5.306</v>
+        <v>5.305</v>
       </c>
       <c r="I39" t="n">
-        <v>5.745</v>
+        <v>5.743</v>
       </c>
       <c r="J39" t="n">
-        <v>6.64</v>
+        <v>6.629</v>
       </c>
       <c r="K39" t="n">
-        <v>7.659</v>
+        <v>7.643</v>
       </c>
       <c r="L39" t="n">
-        <v>8.066000000000001</v>
+        <v>8.051</v>
       </c>
       <c r="M39" t="n">
-        <v>8.461</v>
+        <v>8.438000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.637</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.832000000000001</v>
+        <v>8.82</v>
       </c>
       <c r="P39" t="n">
-        <v>8.867000000000001</v>
+        <v>8.846</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.35</v>
+        <v>9.32</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.293</v>
+        <v>3.29</v>
       </c>
       <c r="G40" t="n">
-        <v>3.408</v>
+        <v>3.405</v>
       </c>
       <c r="H40" t="n">
-        <v>3.589</v>
+        <v>3.588</v>
       </c>
       <c r="I40" t="n">
-        <v>3.838</v>
+        <v>3.836</v>
       </c>
       <c r="J40" t="n">
-        <v>4.139</v>
+        <v>4.128</v>
       </c>
       <c r="K40" t="n">
-        <v>4.444</v>
+        <v>4.428</v>
       </c>
       <c r="L40" t="n">
-        <v>4.545</v>
+        <v>4.53</v>
       </c>
       <c r="M40" t="n">
-        <v>4.754</v>
+        <v>4.731</v>
       </c>
       <c r="N40" t="n">
-        <v>4.94</v>
+        <v>4.913</v>
       </c>
       <c r="O40" t="n">
-        <v>5.249</v>
+        <v>5.236</v>
       </c>
       <c r="P40" t="n">
-        <v>5.45</v>
+        <v>5.429</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.24</v>
+        <v>6.21</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.677</v>
+        <v>3.673</v>
       </c>
       <c r="G41" t="n">
-        <v>3.832</v>
+        <v>3.829</v>
       </c>
       <c r="H41" t="n">
-        <v>4.072</v>
+        <v>4.071</v>
       </c>
       <c r="I41" t="n">
-        <v>4.339</v>
+        <v>4.337</v>
       </c>
       <c r="J41" t="n">
-        <v>4.693</v>
+        <v>4.682</v>
       </c>
       <c r="K41" t="n">
-        <v>5.044</v>
+        <v>5.028</v>
       </c>
       <c r="L41" t="n">
-        <v>5.223</v>
+        <v>5.208</v>
       </c>
       <c r="M41" t="n">
-        <v>5.556</v>
+        <v>5.533</v>
       </c>
       <c r="N41" t="n">
-        <v>5.869</v>
+        <v>5.842</v>
       </c>
       <c r="O41" t="n">
-        <v>6.359</v>
+        <v>6.348</v>
       </c>
       <c r="P41" t="n">
-        <v>6.508</v>
+        <v>6.487</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.287</v>
+        <v>7.257</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.414</v>
+        <v>3.41</v>
       </c>
       <c r="G42" t="n">
-        <v>3.556</v>
+        <v>3.553</v>
       </c>
       <c r="H42" t="n">
-        <v>3.764</v>
+        <v>3.763</v>
       </c>
       <c r="I42" t="n">
-        <v>4.026</v>
+        <v>4.024</v>
       </c>
       <c r="J42" t="n">
-        <v>4.343</v>
+        <v>4.331</v>
       </c>
       <c r="K42" t="n">
-        <v>4.665</v>
+        <v>4.649</v>
       </c>
       <c r="L42" t="n">
-        <v>4.781</v>
+        <v>4.766</v>
       </c>
       <c r="M42" t="n">
-        <v>5.061</v>
+        <v>5.038</v>
       </c>
       <c r="N42" t="n">
-        <v>5.354</v>
+        <v>5.327</v>
       </c>
       <c r="O42" t="n">
-        <v>5.738</v>
+        <v>5.727</v>
       </c>
       <c r="P42" t="n">
-        <v>5.951</v>
+        <v>5.93</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.753</v>
+        <v>6.723</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.129</v>
+        <v>3.121</v>
       </c>
       <c r="G43" t="n">
-        <v>3.225</v>
+        <v>3.218</v>
       </c>
       <c r="H43" t="n">
-        <v>3.351</v>
+        <v>3.349</v>
       </c>
       <c r="I43" t="n">
-        <v>3.56</v>
+        <v>3.557</v>
       </c>
       <c r="J43" t="n">
-        <v>3.788</v>
+        <v>3.778</v>
       </c>
       <c r="K43" t="n">
-        <v>4.013</v>
+        <v>3.998</v>
       </c>
       <c r="L43" t="n">
-        <v>4.068</v>
+        <v>4.053</v>
       </c>
       <c r="M43" t="n">
-        <v>4.2</v>
+        <v>4.177</v>
       </c>
       <c r="N43" t="n">
-        <v>4.242</v>
+        <v>4.215</v>
       </c>
       <c r="O43" t="n">
-        <v>4.336</v>
+        <v>4.325</v>
       </c>
       <c r="P43" t="n">
-        <v>4.425</v>
+        <v>4.405</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.116</v>
+        <v>5.086</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46129</v>
+        <v>46132</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.003</v>
+        <v>2.995</v>
       </c>
       <c r="G44" t="n">
-        <v>3.097</v>
+        <v>3.088</v>
       </c>
       <c r="H44" t="n">
-        <v>3.204</v>
+        <v>3.201</v>
       </c>
       <c r="I44" t="n">
-        <v>3.407</v>
+        <v>3.403</v>
       </c>
       <c r="J44" t="n">
-        <v>3.638</v>
+        <v>3.627</v>
       </c>
       <c r="K44" t="n">
-        <v>3.855</v>
+        <v>3.839</v>
       </c>
       <c r="L44" t="n">
-        <v>3.91</v>
+        <v>3.895</v>
       </c>
       <c r="M44" t="n">
-        <v>4.013</v>
+        <v>3.99</v>
       </c>
       <c r="N44" t="n">
-        <v>4.057</v>
+        <v>4.029</v>
       </c>
       <c r="O44" t="n">
-        <v>4.133</v>
+        <v>4.122</v>
       </c>
       <c r="P44" t="n">
-        <v>4.189</v>
+        <v>4.168</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.487</v>
+        <v>4.457</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-22 ~ 2026-04-22
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.218</v>
+        <v>3.212</v>
       </c>
       <c r="G2" t="n">
-        <v>3.426</v>
+        <v>3.418</v>
       </c>
       <c r="H2" t="n">
-        <v>3.582</v>
+        <v>3.575</v>
       </c>
       <c r="I2" t="n">
-        <v>3.786</v>
+        <v>3.777</v>
       </c>
       <c r="J2" t="n">
-        <v>4.005</v>
+        <v>4.027</v>
       </c>
       <c r="K2" t="n">
-        <v>4.375</v>
+        <v>4.401</v>
       </c>
       <c r="L2" t="n">
-        <v>4.549</v>
+        <v>4.572</v>
       </c>
       <c r="M2" t="n">
-        <v>4.851</v>
+        <v>4.877</v>
       </c>
       <c r="N2" t="n">
-        <v>5.108</v>
+        <v>5.133</v>
       </c>
       <c r="O2" t="n">
-        <v>5.347</v>
+        <v>5.369</v>
       </c>
       <c r="P2" t="n">
-        <v>5.504</v>
+        <v>5.534</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.126</v>
+        <v>6.167</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.241</v>
+        <v>4.235</v>
       </c>
       <c r="G3" t="n">
-        <v>4.631</v>
+        <v>4.623</v>
       </c>
       <c r="H3" t="n">
-        <v>4.82</v>
+        <v>4.813</v>
       </c>
       <c r="I3" t="n">
-        <v>5.024</v>
+        <v>5.015</v>
       </c>
       <c r="J3" t="n">
-        <v>5.252</v>
+        <v>5.274</v>
       </c>
       <c r="K3" t="n">
-        <v>5.691</v>
+        <v>5.716</v>
       </c>
       <c r="L3" t="n">
-        <v>5.934</v>
+        <v>5.958</v>
       </c>
       <c r="M3" t="n">
-        <v>6.268</v>
+        <v>6.294</v>
       </c>
       <c r="N3" t="n">
-        <v>6.468</v>
+        <v>6.493</v>
       </c>
       <c r="O3" t="n">
-        <v>6.657</v>
+        <v>6.679</v>
       </c>
       <c r="P3" t="n">
-        <v>6.684</v>
+        <v>6.714</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.195</v>
+        <v>7.235</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.732</v>
+        <v>3.727</v>
       </c>
       <c r="G4" t="n">
-        <v>4.012</v>
+        <v>4.004</v>
       </c>
       <c r="H4" t="n">
-        <v>4.229</v>
+        <v>4.223</v>
       </c>
       <c r="I4" t="n">
-        <v>4.465</v>
+        <v>4.456</v>
       </c>
       <c r="J4" t="n">
-        <v>4.698</v>
+        <v>4.721</v>
       </c>
       <c r="K4" t="n">
-        <v>5.131</v>
+        <v>5.156</v>
       </c>
       <c r="L4" t="n">
-        <v>5.304</v>
+        <v>5.327</v>
       </c>
       <c r="M4" t="n">
-        <v>5.626</v>
+        <v>5.652</v>
       </c>
       <c r="N4" t="n">
-        <v>5.796</v>
+        <v>5.821</v>
       </c>
       <c r="O4" t="n">
-        <v>6.009</v>
+        <v>6.031</v>
       </c>
       <c r="P4" t="n">
-        <v>6.034</v>
+        <v>6.064</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.547</v>
+        <v>6.588</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.915</v>
+        <v>2.907</v>
       </c>
       <c r="G5" t="n">
-        <v>2.969</v>
+        <v>2.959</v>
       </c>
       <c r="H5" t="n">
-        <v>3.081</v>
+        <v>3.073</v>
       </c>
       <c r="I5" t="n">
-        <v>3.355</v>
+        <v>3.345</v>
       </c>
       <c r="J5" t="n">
-        <v>3.568</v>
+        <v>3.589</v>
       </c>
       <c r="K5" t="n">
-        <v>3.796</v>
+        <v>3.821</v>
       </c>
       <c r="L5" t="n">
-        <v>3.813</v>
+        <v>3.835</v>
       </c>
       <c r="M5" t="n">
-        <v>3.918</v>
+        <v>3.943</v>
       </c>
       <c r="N5" t="n">
-        <v>3.925</v>
+        <v>3.949</v>
       </c>
       <c r="O5" t="n">
-        <v>3.948</v>
+        <v>3.968</v>
       </c>
       <c r="P5" t="n">
-        <v>4.173</v>
+        <v>4.203</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.038</v>
+        <v>5.079</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.954</v>
+        <v>2.946</v>
       </c>
       <c r="G6" t="n">
-        <v>3.022</v>
+        <v>3.012</v>
       </c>
       <c r="H6" t="n">
-        <v>3.151</v>
+        <v>3.143</v>
       </c>
       <c r="I6" t="n">
-        <v>3.436</v>
+        <v>3.427</v>
       </c>
       <c r="J6" t="n">
-        <v>3.656</v>
+        <v>3.678</v>
       </c>
       <c r="K6" t="n">
-        <v>3.904</v>
+        <v>3.93</v>
       </c>
       <c r="L6" t="n">
-        <v>3.931</v>
+        <v>3.953</v>
       </c>
       <c r="M6" t="n">
-        <v>4.075</v>
+        <v>4.1</v>
       </c>
       <c r="N6" t="n">
-        <v>4.092</v>
+        <v>4.117</v>
       </c>
       <c r="O6" t="n">
-        <v>4.215</v>
+        <v>4.236</v>
       </c>
       <c r="P6" t="n">
-        <v>4.605</v>
+        <v>4.635</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.434</v>
+        <v>5.475</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.935</v>
+        <v>2.927</v>
       </c>
       <c r="G7" t="n">
-        <v>2.986</v>
+        <v>2.976</v>
       </c>
       <c r="H7" t="n">
-        <v>3.096</v>
+        <v>3.088</v>
       </c>
       <c r="I7" t="n">
-        <v>3.37</v>
+        <v>3.36</v>
       </c>
       <c r="J7" t="n">
-        <v>3.593</v>
+        <v>3.614</v>
       </c>
       <c r="K7" t="n">
-        <v>3.823</v>
+        <v>3.848</v>
       </c>
       <c r="L7" t="n">
-        <v>3.838</v>
+        <v>3.86</v>
       </c>
       <c r="M7" t="n">
-        <v>3.979</v>
+        <v>4.003</v>
       </c>
       <c r="N7" t="n">
-        <v>3.985</v>
+        <v>4.01</v>
       </c>
       <c r="O7" t="n">
-        <v>4.113</v>
+        <v>4.134</v>
       </c>
       <c r="P7" t="n">
-        <v>4.389</v>
+        <v>4.419</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.202</v>
+        <v>5.243</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.35</v>
+        <v>5.345</v>
       </c>
       <c r="G8" t="n">
-        <v>5.929</v>
+        <v>5.921</v>
       </c>
       <c r="H8" t="n">
-        <v>6.269</v>
+        <v>6.262</v>
       </c>
       <c r="I8" t="n">
-        <v>6.544</v>
+        <v>6.535</v>
       </c>
       <c r="J8" t="n">
-        <v>6.836</v>
+        <v>6.859</v>
       </c>
       <c r="K8" t="n">
-        <v>7.556</v>
+        <v>7.583</v>
       </c>
       <c r="L8" t="n">
-        <v>7.889</v>
+        <v>7.913</v>
       </c>
       <c r="M8" t="n">
-        <v>8.250999999999999</v>
+        <v>8.278</v>
       </c>
       <c r="N8" t="n">
-        <v>8.388999999999999</v>
+        <v>8.414</v>
       </c>
       <c r="O8" t="n">
-        <v>8.664</v>
+        <v>8.686</v>
       </c>
       <c r="P8" t="n">
-        <v>8.792</v>
+        <v>8.823</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.503</v>
+        <v>9.544</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1066,54 +1066,54 @@
         <v>2.619</v>
       </c>
       <c r="G9" t="n">
-        <v>2.677</v>
+        <v>2.682</v>
       </c>
       <c r="H9" t="n">
-        <v>2.767</v>
+        <v>2.774</v>
       </c>
       <c r="I9" t="n">
-        <v>2.925</v>
+        <v>2.936</v>
       </c>
       <c r="J9" t="n">
-        <v>3.107</v>
+        <v>3.125</v>
       </c>
       <c r="K9" t="n">
-        <v>3.206</v>
+        <v>3.24</v>
       </c>
       <c r="L9" t="n">
-        <v>3.25</v>
+        <v>3.276</v>
       </c>
       <c r="M9" t="n">
-        <v>3.335</v>
+        <v>3.364</v>
       </c>
       <c r="N9" t="n">
-        <v>3.492</v>
+        <v>3.517</v>
       </c>
       <c r="O9" t="n">
-        <v>3.54</v>
+        <v>3.562</v>
       </c>
       <c r="P9" t="n">
-        <v>3.593</v>
+        <v>3.623</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.656</v>
+        <v>3.697</v>
       </c>
       <c r="R9" t="n">
-        <v>3.657</v>
+        <v>3.691</v>
       </c>
       <c r="S9" t="n">
-        <v>3.62</v>
+        <v>3.645</v>
       </c>
       <c r="T9" t="n">
-        <v>3.535</v>
+        <v>3.569</v>
       </c>
       <c r="U9" t="n">
-        <v>3.406</v>
+        <v>3.441</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,31 +1139,31 @@
         <v>2.633</v>
       </c>
       <c r="G10" t="n">
-        <v>2.715</v>
+        <v>2.72</v>
       </c>
       <c r="H10" t="n">
-        <v>2.782</v>
+        <v>2.789</v>
       </c>
       <c r="I10" t="n">
-        <v>2.938</v>
+        <v>2.949</v>
       </c>
       <c r="J10" t="n">
-        <v>3.133</v>
+        <v>3.151</v>
       </c>
       <c r="K10" t="n">
-        <v>3.238</v>
+        <v>3.273</v>
       </c>
       <c r="L10" t="n">
-        <v>3.297</v>
+        <v>3.324</v>
       </c>
       <c r="M10" t="n">
-        <v>3.433</v>
+        <v>3.463</v>
       </c>
       <c r="N10" t="n">
-        <v>3.505</v>
+        <v>3.531</v>
       </c>
       <c r="O10" t="n">
-        <v>3.732</v>
+        <v>3.774</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.448</v>
       </c>
       <c r="G11" t="n">
-        <v>2.525</v>
+        <v>2.53</v>
       </c>
       <c r="H11" t="n">
-        <v>2.606</v>
+        <v>2.613</v>
       </c>
       <c r="I11" t="n">
-        <v>2.741</v>
+        <v>2.752</v>
       </c>
       <c r="J11" t="n">
-        <v>2.928</v>
+        <v>2.946</v>
       </c>
       <c r="K11" t="n">
-        <v>3.025</v>
+        <v>3.06</v>
       </c>
       <c r="L11" t="n">
-        <v>3.091</v>
+        <v>3.118</v>
       </c>
       <c r="M11" t="n">
-        <v>3.238</v>
+        <v>3.267</v>
       </c>
       <c r="N11" t="n">
-        <v>3.314</v>
+        <v>3.339</v>
       </c>
       <c r="O11" t="n">
-        <v>3.499</v>
+        <v>3.54</v>
       </c>
       <c r="P11" t="n">
-        <v>3.535</v>
+        <v>3.567</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.859</v>
+        <v>3.899</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.195</v>
+        <v>3.193</v>
       </c>
       <c r="G12" t="n">
-        <v>3.347</v>
+        <v>3.341</v>
       </c>
       <c r="H12" t="n">
-        <v>3.458</v>
+        <v>3.45</v>
       </c>
       <c r="I12" t="n">
-        <v>3.67</v>
+        <v>3.668</v>
       </c>
       <c r="J12" t="n">
-        <v>3.973</v>
+        <v>3.995</v>
       </c>
       <c r="K12" t="n">
-        <v>4.145</v>
+        <v>4.169</v>
       </c>
       <c r="L12" t="n">
-        <v>4.204</v>
+        <v>4.229</v>
       </c>
       <c r="M12" t="n">
-        <v>4.347</v>
+        <v>4.375</v>
       </c>
       <c r="N12" t="n">
-        <v>4.385</v>
+        <v>4.411</v>
       </c>
       <c r="O12" t="n">
-        <v>4.544</v>
+        <v>4.566</v>
       </c>
       <c r="P12" t="n">
-        <v>4.64</v>
+        <v>4.67</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.986</v>
+        <v>5.027</v>
       </c>
       <c r="R12" t="n">
-        <v>5.156</v>
+        <v>5.189</v>
       </c>
       <c r="S12" t="n">
-        <v>5.331</v>
+        <v>5.356</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.949</v>
+        <v>2.946</v>
       </c>
       <c r="G13" t="n">
-        <v>3.038</v>
+        <v>3.031</v>
       </c>
       <c r="H13" t="n">
-        <v>3.125</v>
+        <v>3.117</v>
       </c>
       <c r="I13" t="n">
-        <v>3.318</v>
+        <v>3.316</v>
       </c>
       <c r="J13" t="n">
-        <v>3.61</v>
+        <v>3.632</v>
       </c>
       <c r="K13" t="n">
-        <v>3.778</v>
+        <v>3.802</v>
       </c>
       <c r="L13" t="n">
-        <v>3.843</v>
+        <v>3.869</v>
       </c>
       <c r="M13" t="n">
-        <v>3.975</v>
+        <v>4.002</v>
       </c>
       <c r="N13" t="n">
-        <v>4.013</v>
+        <v>4.039</v>
       </c>
       <c r="O13" t="n">
-        <v>4.172</v>
+        <v>4.195</v>
       </c>
       <c r="P13" t="n">
-        <v>4.231</v>
+        <v>4.261</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.507</v>
+        <v>4.548</v>
       </c>
       <c r="R13" t="n">
-        <v>4.704</v>
+        <v>4.738</v>
       </c>
       <c r="S13" t="n">
-        <v>4.893</v>
+        <v>4.919</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.767</v>
+        <v>2.765</v>
       </c>
       <c r="G14" t="n">
-        <v>2.843</v>
+        <v>2.837</v>
       </c>
       <c r="H14" t="n">
-        <v>2.929</v>
+        <v>2.921</v>
       </c>
       <c r="I14" t="n">
-        <v>3.102</v>
+        <v>3.1</v>
       </c>
       <c r="J14" t="n">
-        <v>3.35</v>
+        <v>3.372</v>
       </c>
       <c r="K14" t="n">
-        <v>3.466</v>
+        <v>3.49</v>
       </c>
       <c r="L14" t="n">
-        <v>3.515</v>
+        <v>3.541</v>
       </c>
       <c r="M14" t="n">
-        <v>3.66</v>
+        <v>3.687</v>
       </c>
       <c r="N14" t="n">
-        <v>3.693</v>
+        <v>3.718</v>
       </c>
       <c r="O14" t="n">
-        <v>3.827</v>
+        <v>3.85</v>
       </c>
       <c r="P14" t="n">
-        <v>3.866</v>
+        <v>3.896</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.096</v>
+        <v>4.137</v>
       </c>
       <c r="R14" t="n">
-        <v>4.219</v>
+        <v>4.253</v>
       </c>
       <c r="S14" t="n">
-        <v>4.346</v>
+        <v>4.371</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.746</v>
+        <v>2.744</v>
       </c>
       <c r="G15" t="n">
-        <v>2.817</v>
+        <v>2.811</v>
       </c>
       <c r="H15" t="n">
-        <v>2.897</v>
+        <v>2.889</v>
       </c>
       <c r="I15" t="n">
-        <v>3.054</v>
+        <v>3.052</v>
       </c>
       <c r="J15" t="n">
-        <v>3.289</v>
+        <v>3.311</v>
       </c>
       <c r="K15" t="n">
-        <v>3.419</v>
+        <v>3.443</v>
       </c>
       <c r="L15" t="n">
-        <v>3.451</v>
+        <v>3.476</v>
       </c>
       <c r="M15" t="n">
-        <v>3.573</v>
+        <v>3.601</v>
       </c>
       <c r="N15" t="n">
-        <v>3.596</v>
+        <v>3.622</v>
       </c>
       <c r="O15" t="n">
-        <v>3.753</v>
+        <v>3.776</v>
       </c>
       <c r="P15" t="n">
-        <v>3.765</v>
+        <v>3.795</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.001</v>
+        <v>4.042</v>
       </c>
       <c r="R15" t="n">
-        <v>4.115</v>
+        <v>4.149</v>
       </c>
       <c r="S15" t="n">
-        <v>4.241</v>
+        <v>4.267</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.746</v>
+        <v>2.744</v>
       </c>
       <c r="G16" t="n">
-        <v>2.817</v>
+        <v>2.811</v>
       </c>
       <c r="H16" t="n">
-        <v>2.897</v>
+        <v>2.889</v>
       </c>
       <c r="I16" t="n">
-        <v>3.054</v>
+        <v>3.052</v>
       </c>
       <c r="J16" t="n">
-        <v>3.289</v>
+        <v>3.311</v>
       </c>
       <c r="K16" t="n">
-        <v>3.419</v>
+        <v>3.443</v>
       </c>
       <c r="L16" t="n">
-        <v>3.451</v>
+        <v>3.476</v>
       </c>
       <c r="M16" t="n">
-        <v>3.573</v>
+        <v>3.601</v>
       </c>
       <c r="N16" t="n">
-        <v>3.599</v>
+        <v>3.625</v>
       </c>
       <c r="O16" t="n">
-        <v>3.76</v>
+        <v>3.783</v>
       </c>
       <c r="P16" t="n">
-        <v>3.789</v>
+        <v>3.819</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.028</v>
+        <v>4.069</v>
       </c>
       <c r="R16" t="n">
-        <v>4.143</v>
+        <v>4.177</v>
       </c>
       <c r="S16" t="n">
-        <v>4.27</v>
+        <v>4.296</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.697</v>
+        <v>2.696</v>
       </c>
       <c r="G17" t="n">
-        <v>2.805</v>
+        <v>2.809</v>
       </c>
       <c r="H17" t="n">
-        <v>2.876</v>
+        <v>2.883</v>
       </c>
       <c r="I17" t="n">
-        <v>3.02</v>
+        <v>3.031</v>
       </c>
       <c r="J17" t="n">
-        <v>3.204</v>
+        <v>3.222</v>
       </c>
       <c r="K17" t="n">
-        <v>3.314</v>
+        <v>3.348</v>
       </c>
       <c r="L17" t="n">
-        <v>3.376</v>
+        <v>3.403</v>
       </c>
       <c r="M17" t="n">
-        <v>3.551</v>
+        <v>3.58</v>
       </c>
       <c r="N17" t="n">
-        <v>3.606</v>
+        <v>3.631</v>
       </c>
       <c r="O17" t="n">
-        <v>3.763</v>
+        <v>3.8</v>
       </c>
       <c r="P17" t="n">
-        <v>3.807</v>
+        <v>3.839</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.698</v>
+        <v>2.697</v>
       </c>
       <c r="G18" t="n">
-        <v>2.806</v>
+        <v>2.81</v>
       </c>
       <c r="H18" t="n">
-        <v>2.876</v>
+        <v>2.883</v>
       </c>
       <c r="I18" t="n">
-        <v>3.02</v>
+        <v>3.031</v>
       </c>
       <c r="J18" t="n">
-        <v>3.204</v>
+        <v>3.222</v>
       </c>
       <c r="K18" t="n">
-        <v>3.314</v>
+        <v>3.349</v>
       </c>
       <c r="L18" t="n">
-        <v>3.376</v>
+        <v>3.403</v>
       </c>
       <c r="M18" t="n">
-        <v>3.551</v>
+        <v>3.58</v>
       </c>
       <c r="N18" t="n">
-        <v>3.607</v>
+        <v>3.632</v>
       </c>
       <c r="O18" t="n">
-        <v>3.761</v>
+        <v>3.8</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.759</v>
+        <v>2.756</v>
       </c>
       <c r="G19" t="n">
-        <v>2.834</v>
+        <v>2.828</v>
       </c>
       <c r="H19" t="n">
-        <v>2.918</v>
+        <v>2.91</v>
       </c>
       <c r="I19" t="n">
-        <v>3.088</v>
+        <v>3.087</v>
       </c>
       <c r="J19" t="n">
-        <v>3.334</v>
+        <v>3.356</v>
       </c>
       <c r="K19" t="n">
-        <v>3.462</v>
+        <v>3.486</v>
       </c>
       <c r="L19" t="n">
-        <v>3.512</v>
+        <v>3.538</v>
       </c>
       <c r="M19" t="n">
-        <v>3.651</v>
+        <v>3.679</v>
       </c>
       <c r="N19" t="n">
-        <v>3.68</v>
+        <v>3.705</v>
       </c>
       <c r="O19" t="n">
-        <v>3.806</v>
+        <v>3.828</v>
       </c>
       <c r="P19" t="n">
-        <v>3.828</v>
+        <v>3.857</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.043</v>
+        <v>4.084</v>
       </c>
       <c r="R19" t="n">
-        <v>4.165</v>
+        <v>4.199</v>
       </c>
       <c r="S19" t="n">
-        <v>4.284</v>
+        <v>4.31</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.643</v>
+        <v>2.64</v>
       </c>
       <c r="H20" t="n">
-        <v>2.69</v>
+        <v>2.685</v>
       </c>
       <c r="I20" t="n">
-        <v>2.832</v>
+        <v>2.821</v>
       </c>
       <c r="J20" t="n">
-        <v>3.099</v>
+        <v>3.125</v>
       </c>
       <c r="K20" t="n">
-        <v>3.237</v>
+        <v>3.266</v>
       </c>
       <c r="L20" t="n">
-        <v>3.28</v>
+        <v>3.309</v>
       </c>
       <c r="M20" t="n">
-        <v>3.381</v>
+        <v>3.409</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.867</v>
+        <v>2.863</v>
       </c>
       <c r="G21" t="n">
-        <v>2.946</v>
+        <v>2.939</v>
       </c>
       <c r="H21" t="n">
-        <v>3.06</v>
+        <v>3.056</v>
       </c>
       <c r="I21" t="n">
-        <v>3.22</v>
+        <v>3.213</v>
       </c>
       <c r="J21" t="n">
-        <v>3.464</v>
+        <v>3.488</v>
       </c>
       <c r="K21" t="n">
-        <v>3.705</v>
+        <v>3.727</v>
       </c>
       <c r="L21" t="n">
-        <v>3.761</v>
+        <v>3.786</v>
       </c>
       <c r="M21" t="n">
-        <v>3.898</v>
+        <v>3.925</v>
       </c>
       <c r="N21" t="n">
-        <v>3.943</v>
+        <v>3.968</v>
       </c>
       <c r="O21" t="n">
-        <v>4.036</v>
+        <v>4.058</v>
       </c>
       <c r="P21" t="n">
-        <v>4.092</v>
+        <v>4.122</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.208</v>
+        <v>4.249</v>
       </c>
       <c r="R21" t="n">
-        <v>4.215</v>
+        <v>4.249</v>
       </c>
       <c r="S21" t="n">
-        <v>4.245</v>
+        <v>4.271</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.814</v>
+        <v>2.81</v>
       </c>
       <c r="G22" t="n">
-        <v>2.892</v>
+        <v>2.886</v>
       </c>
       <c r="H22" t="n">
-        <v>2.992</v>
+        <v>2.988</v>
       </c>
       <c r="I22" t="n">
-        <v>3.14</v>
+        <v>3.133</v>
       </c>
       <c r="J22" t="n">
-        <v>3.348</v>
+        <v>3.372</v>
       </c>
       <c r="K22" t="n">
-        <v>3.584</v>
+        <v>3.607</v>
       </c>
       <c r="L22" t="n">
-        <v>3.63</v>
+        <v>3.654</v>
       </c>
       <c r="M22" t="n">
-        <v>3.768</v>
+        <v>3.795</v>
       </c>
       <c r="N22" t="n">
-        <v>3.815</v>
+        <v>3.84</v>
       </c>
       <c r="O22" t="n">
-        <v>3.904</v>
+        <v>3.926</v>
       </c>
       <c r="P22" t="n">
-        <v>3.954</v>
+        <v>3.985</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.067</v>
+        <v>4.107</v>
       </c>
       <c r="R22" t="n">
-        <v>4.063</v>
+        <v>4.096</v>
       </c>
       <c r="S22" t="n">
-        <v>4.09</v>
+        <v>4.116</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.766</v>
+        <v>2.763</v>
       </c>
       <c r="G23" t="n">
-        <v>2.847</v>
+        <v>2.841</v>
       </c>
       <c r="H23" t="n">
-        <v>2.932</v>
+        <v>2.928</v>
       </c>
       <c r="I23" t="n">
-        <v>3.093</v>
+        <v>3.086</v>
       </c>
       <c r="J23" t="n">
-        <v>3.294</v>
+        <v>3.318</v>
       </c>
       <c r="K23" t="n">
-        <v>3.503</v>
+        <v>3.524</v>
       </c>
       <c r="L23" t="n">
-        <v>3.541</v>
+        <v>3.565</v>
       </c>
       <c r="M23" t="n">
-        <v>3.672</v>
+        <v>3.699</v>
       </c>
       <c r="N23" t="n">
-        <v>3.712</v>
+        <v>3.737</v>
       </c>
       <c r="O23" t="n">
-        <v>3.779</v>
+        <v>3.8</v>
       </c>
       <c r="P23" t="n">
-        <v>3.816</v>
+        <v>3.846</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.874</v>
+        <v>3.915</v>
       </c>
       <c r="R23" t="n">
-        <v>3.847</v>
+        <v>3.88</v>
       </c>
       <c r="S23" t="n">
-        <v>3.845</v>
+        <v>3.87</v>
       </c>
       <c r="T23" t="n">
-        <v>3.75</v>
+        <v>3.785</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.701</v>
+        <v>2.698</v>
       </c>
       <c r="G24" t="n">
-        <v>2.761</v>
+        <v>2.755</v>
       </c>
       <c r="H24" t="n">
-        <v>2.833</v>
+        <v>2.829</v>
       </c>
       <c r="I24" t="n">
-        <v>3.003</v>
+        <v>2.996</v>
       </c>
       <c r="J24" t="n">
-        <v>3.193</v>
+        <v>3.217</v>
       </c>
       <c r="K24" t="n">
-        <v>3.386</v>
+        <v>3.409</v>
       </c>
       <c r="L24" t="n">
-        <v>3.413</v>
+        <v>3.438</v>
       </c>
       <c r="M24" t="n">
-        <v>3.53</v>
+        <v>3.556</v>
       </c>
       <c r="N24" t="n">
-        <v>3.582</v>
+        <v>3.608</v>
       </c>
       <c r="O24" t="n">
-        <v>3.731</v>
+        <v>3.766</v>
       </c>
       <c r="P24" t="n">
-        <v>3.755</v>
+        <v>3.787</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.796</v>
+        <v>3.837</v>
       </c>
       <c r="R24" t="n">
-        <v>3.768</v>
+        <v>3.802</v>
       </c>
       <c r="S24" t="n">
-        <v>3.76</v>
+        <v>3.785</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.76</v>
+        <v>2.756</v>
       </c>
       <c r="G25" t="n">
-        <v>2.846</v>
+        <v>2.84</v>
       </c>
       <c r="H25" t="n">
-        <v>2.935</v>
+        <v>2.931</v>
       </c>
       <c r="I25" t="n">
-        <v>3.101</v>
+        <v>3.093</v>
       </c>
       <c r="J25" t="n">
-        <v>3.309</v>
+        <v>3.333</v>
       </c>
       <c r="K25" t="n">
-        <v>3.533</v>
+        <v>3.556</v>
       </c>
       <c r="L25" t="n">
-        <v>3.57</v>
+        <v>3.594</v>
       </c>
       <c r="M25" t="n">
-        <v>3.702</v>
+        <v>3.729</v>
       </c>
       <c r="N25" t="n">
-        <v>3.739</v>
+        <v>3.764</v>
       </c>
       <c r="O25" t="n">
-        <v>3.808</v>
+        <v>3.83</v>
       </c>
       <c r="P25" t="n">
-        <v>3.838</v>
+        <v>3.868</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.907</v>
+        <v>3.948</v>
       </c>
       <c r="R25" t="n">
-        <v>3.87</v>
+        <v>3.904</v>
       </c>
       <c r="S25" t="n">
-        <v>3.868</v>
+        <v>3.893</v>
       </c>
       <c r="T25" t="n">
-        <v>3.768</v>
+        <v>3.803</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.066</v>
+        <v>3.062</v>
       </c>
       <c r="G26" t="n">
-        <v>3.198</v>
+        <v>3.19</v>
       </c>
       <c r="H26" t="n">
-        <v>3.399</v>
+        <v>3.394</v>
       </c>
       <c r="I26" t="n">
-        <v>3.631</v>
+        <v>3.627</v>
       </c>
       <c r="J26" t="n">
-        <v>3.969</v>
+        <v>3.993</v>
       </c>
       <c r="K26" t="n">
-        <v>4.327</v>
+        <v>4.354</v>
       </c>
       <c r="L26" t="n">
-        <v>4.428</v>
+        <v>4.454</v>
       </c>
       <c r="M26" t="n">
-        <v>4.618</v>
+        <v>4.646</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.88</v>
+        <v>4.901</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.859</v>
+        <v>2.856</v>
       </c>
       <c r="G27" t="n">
-        <v>2.926</v>
+        <v>2.919</v>
       </c>
       <c r="H27" t="n">
-        <v>3.033</v>
+        <v>3.026</v>
       </c>
       <c r="I27" t="n">
-        <v>3.215</v>
+        <v>3.213</v>
       </c>
       <c r="J27" t="n">
-        <v>3.468</v>
+        <v>3.493</v>
       </c>
       <c r="K27" t="n">
-        <v>3.642</v>
+        <v>3.667</v>
       </c>
       <c r="L27" t="n">
-        <v>3.695</v>
+        <v>3.721</v>
       </c>
       <c r="M27" t="n">
-        <v>3.828</v>
+        <v>3.855</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.969</v>
+        <v>3.992</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.962</v>
+        <v>2.96</v>
       </c>
       <c r="G28" t="n">
-        <v>3.036</v>
+        <v>3.029</v>
       </c>
       <c r="H28" t="n">
-        <v>3.157</v>
+        <v>3.15</v>
       </c>
       <c r="I28" t="n">
-        <v>3.353</v>
+        <v>3.351</v>
       </c>
       <c r="J28" t="n">
-        <v>3.641</v>
+        <v>3.666</v>
       </c>
       <c r="K28" t="n">
-        <v>3.834</v>
+        <v>3.859</v>
       </c>
       <c r="L28" t="n">
-        <v>3.899</v>
+        <v>3.925</v>
       </c>
       <c r="M28" t="n">
-        <v>4.04</v>
+        <v>4.067</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.263</v>
+        <v>4.286</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.817</v>
+        <v>2.812</v>
       </c>
       <c r="G29" t="n">
-        <v>2.884</v>
+        <v>2.876</v>
       </c>
       <c r="H29" t="n">
-        <v>2.976</v>
+        <v>2.969</v>
       </c>
       <c r="I29" t="n">
-        <v>3.149</v>
+        <v>3.147</v>
       </c>
       <c r="J29" t="n">
-        <v>3.381</v>
+        <v>3.405</v>
       </c>
       <c r="K29" t="n">
-        <v>3.538</v>
+        <v>3.563</v>
       </c>
       <c r="L29" t="n">
-        <v>3.58</v>
+        <v>3.606</v>
       </c>
       <c r="M29" t="n">
-        <v>3.69</v>
+        <v>3.717</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.83</v>
+        <v>3.853</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.097</v>
+        <v>3.095</v>
       </c>
       <c r="G30" t="n">
-        <v>3.166</v>
+        <v>3.16</v>
       </c>
       <c r="H30" t="n">
-        <v>3.329</v>
+        <v>3.325</v>
       </c>
       <c r="I30" t="n">
-        <v>3.553</v>
+        <v>3.552</v>
       </c>
       <c r="J30" t="n">
-        <v>3.831</v>
+        <v>3.859</v>
       </c>
       <c r="K30" t="n">
-        <v>4.118</v>
+        <v>4.147</v>
       </c>
       <c r="L30" t="n">
-        <v>4.196</v>
+        <v>4.223</v>
       </c>
       <c r="M30" t="n">
-        <v>4.377</v>
+        <v>4.407</v>
       </c>
       <c r="N30" t="n">
-        <v>4.537</v>
+        <v>4.562</v>
       </c>
       <c r="O30" t="n">
-        <v>4.831</v>
+        <v>4.853</v>
       </c>
       <c r="P30" t="n">
-        <v>4.981</v>
+        <v>5.011</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.73</v>
+        <v>5.771</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.423</v>
+        <v>3.421</v>
       </c>
       <c r="G31" t="n">
-        <v>3.526</v>
+        <v>3.52</v>
       </c>
       <c r="H31" t="n">
-        <v>3.742</v>
+        <v>3.738</v>
       </c>
       <c r="I31" t="n">
-        <v>3.981</v>
+        <v>3.98</v>
       </c>
       <c r="J31" t="n">
-        <v>4.321</v>
+        <v>4.349</v>
       </c>
       <c r="K31" t="n">
-        <v>4.65</v>
+        <v>4.679</v>
       </c>
       <c r="L31" t="n">
-        <v>4.808</v>
+        <v>4.835</v>
       </c>
       <c r="M31" t="n">
-        <v>5.107</v>
+        <v>5.136</v>
       </c>
       <c r="N31" t="n">
-        <v>5.394</v>
+        <v>5.419</v>
       </c>
       <c r="O31" t="n">
-        <v>5.863</v>
+        <v>5.885</v>
       </c>
       <c r="P31" t="n">
-        <v>5.968</v>
+        <v>5.998</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.704</v>
+        <v>6.745</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.195</v>
+        <v>3.193</v>
       </c>
       <c r="G32" t="n">
-        <v>3.282</v>
+        <v>3.276</v>
       </c>
       <c r="H32" t="n">
-        <v>3.472</v>
+        <v>3.468</v>
       </c>
       <c r="I32" t="n">
-        <v>3.712</v>
+        <v>3.711</v>
       </c>
       <c r="J32" t="n">
-        <v>4.01</v>
+        <v>4.038</v>
       </c>
       <c r="K32" t="n">
-        <v>4.303</v>
+        <v>4.332</v>
       </c>
       <c r="L32" t="n">
-        <v>4.4</v>
+        <v>4.427</v>
       </c>
       <c r="M32" t="n">
-        <v>4.65</v>
+        <v>4.679</v>
       </c>
       <c r="N32" t="n">
-        <v>4.898</v>
+        <v>4.923</v>
       </c>
       <c r="O32" t="n">
-        <v>5.275</v>
+        <v>5.297</v>
       </c>
       <c r="P32" t="n">
-        <v>5.44</v>
+        <v>5.47</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.192</v>
+        <v>6.232</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.973</v>
+        <v>2.97</v>
       </c>
       <c r="G33" t="n">
-        <v>3.036</v>
+        <v>3.03</v>
       </c>
       <c r="H33" t="n">
-        <v>3.152</v>
+        <v>3.148</v>
       </c>
       <c r="I33" t="n">
-        <v>3.34</v>
+        <v>3.336</v>
       </c>
       <c r="J33" t="n">
-        <v>3.545</v>
+        <v>3.57</v>
       </c>
       <c r="K33" t="n">
-        <v>3.761</v>
+        <v>3.789</v>
       </c>
       <c r="L33" t="n">
-        <v>3.802</v>
+        <v>3.829</v>
       </c>
       <c r="M33" t="n">
-        <v>3.911</v>
+        <v>3.94</v>
       </c>
       <c r="N33" t="n">
-        <v>3.928</v>
+        <v>3.953</v>
       </c>
       <c r="O33" t="n">
-        <v>3.985</v>
+        <v>4.007</v>
       </c>
       <c r="P33" t="n">
-        <v>4.013</v>
+        <v>4.043</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.447</v>
+        <v>4.488</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.032</v>
+        <v>3.029</v>
       </c>
       <c r="G34" t="n">
-        <v>3.089</v>
+        <v>3.082</v>
       </c>
       <c r="H34" t="n">
-        <v>3.211</v>
+        <v>3.207</v>
       </c>
       <c r="I34" t="n">
-        <v>3.409</v>
+        <v>3.405</v>
       </c>
       <c r="J34" t="n">
-        <v>3.617</v>
+        <v>3.642</v>
       </c>
       <c r="K34" t="n">
-        <v>3.838</v>
+        <v>3.866</v>
       </c>
       <c r="L34" t="n">
-        <v>3.881</v>
+        <v>3.908</v>
       </c>
       <c r="M34" t="n">
-        <v>4.001</v>
+        <v>4.031</v>
       </c>
       <c r="N34" t="n">
-        <v>4.032</v>
+        <v>4.058</v>
       </c>
       <c r="O34" t="n">
-        <v>4.153</v>
+        <v>4.175</v>
       </c>
       <c r="P34" t="n">
-        <v>4.307</v>
+        <v>4.337</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.148</v>
+        <v>5.189</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.007</v>
+        <v>3.004</v>
       </c>
       <c r="G35" t="n">
-        <v>3.062</v>
+        <v>3.056</v>
       </c>
       <c r="H35" t="n">
-        <v>3.179</v>
+        <v>3.175</v>
       </c>
       <c r="I35" t="n">
-        <v>3.375</v>
+        <v>3.371</v>
       </c>
       <c r="J35" t="n">
-        <v>3.585</v>
+        <v>3.61</v>
       </c>
       <c r="K35" t="n">
-        <v>3.793</v>
+        <v>3.82</v>
       </c>
       <c r="L35" t="n">
-        <v>3.836</v>
+        <v>3.863</v>
       </c>
       <c r="M35" t="n">
-        <v>3.948</v>
+        <v>3.978</v>
       </c>
       <c r="N35" t="n">
-        <v>3.969</v>
+        <v>3.994</v>
       </c>
       <c r="O35" t="n">
-        <v>4.051</v>
+        <v>4.073</v>
       </c>
       <c r="P35" t="n">
-        <v>4.11</v>
+        <v>4.14</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.784</v>
+        <v>4.825</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.917</v>
+        <v>2.912</v>
       </c>
       <c r="G36" t="n">
-        <v>2.978</v>
+        <v>2.97</v>
       </c>
       <c r="H36" t="n">
-        <v>3.078</v>
+        <v>3.074</v>
       </c>
       <c r="I36" t="n">
-        <v>3.268</v>
+        <v>3.264</v>
       </c>
       <c r="J36" t="n">
-        <v>3.481</v>
+        <v>3.506</v>
       </c>
       <c r="K36" t="n">
-        <v>3.685</v>
+        <v>3.713</v>
       </c>
       <c r="L36" t="n">
-        <v>3.726</v>
+        <v>3.753</v>
       </c>
       <c r="M36" t="n">
-        <v>3.81</v>
+        <v>3.839</v>
       </c>
       <c r="N36" t="n">
-        <v>3.831</v>
+        <v>3.855</v>
       </c>
       <c r="O36" t="n">
-        <v>3.896</v>
+        <v>3.917</v>
       </c>
       <c r="P36" t="n">
-        <v>3.911</v>
+        <v>3.941</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.164</v>
+        <v>4.205</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.767</v>
+        <v>3.765</v>
       </c>
       <c r="G37" t="n">
-        <v>4.221</v>
+        <v>4.215</v>
       </c>
       <c r="H37" t="n">
-        <v>4.718</v>
+        <v>4.714</v>
       </c>
       <c r="I37" t="n">
-        <v>5.052</v>
+        <v>5.051</v>
       </c>
       <c r="J37" t="n">
-        <v>5.812</v>
+        <v>5.84</v>
       </c>
       <c r="K37" t="n">
-        <v>6.689</v>
+        <v>6.718</v>
       </c>
       <c r="L37" t="n">
-        <v>7.007</v>
+        <v>7.034</v>
       </c>
       <c r="M37" t="n">
-        <v>7.381</v>
+        <v>7.41</v>
       </c>
       <c r="N37" t="n">
-        <v>7.546</v>
+        <v>7.571</v>
       </c>
       <c r="O37" t="n">
-        <v>7.742</v>
+        <v>7.764</v>
       </c>
       <c r="P37" t="n">
-        <v>7.768</v>
+        <v>7.798</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.195</v>
+        <v>8.236000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.823</v>
+        <v>4.822</v>
       </c>
       <c r="G38" t="n">
-        <v>5.531</v>
+        <v>5.526</v>
       </c>
       <c r="H38" t="n">
-        <v>6.242</v>
+        <v>6.238</v>
       </c>
       <c r="I38" t="n">
-        <v>6.732</v>
+        <v>6.731</v>
       </c>
       <c r="J38" t="n">
-        <v>7.752</v>
+        <v>7.78</v>
       </c>
       <c r="K38" t="n">
-        <v>8.804</v>
+        <v>8.834</v>
       </c>
       <c r="L38" t="n">
-        <v>9.282999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="M38" t="n">
-        <v>9.788</v>
+        <v>9.818</v>
       </c>
       <c r="N38" t="n">
-        <v>9.964</v>
+        <v>9.989000000000001</v>
       </c>
       <c r="O38" t="n">
-        <v>10.142</v>
+        <v>10.164</v>
       </c>
       <c r="P38" t="n">
-        <v>10.166</v>
+        <v>10.196</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.647</v>
+        <v>10.687</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.144</v>
+        <v>4.143</v>
       </c>
       <c r="G39" t="n">
-        <v>4.729</v>
+        <v>4.724</v>
       </c>
       <c r="H39" t="n">
-        <v>5.307</v>
+        <v>5.303</v>
       </c>
       <c r="I39" t="n">
-        <v>5.736</v>
+        <v>5.735</v>
       </c>
       <c r="J39" t="n">
-        <v>6.624</v>
+        <v>6.653</v>
       </c>
       <c r="K39" t="n">
-        <v>7.638</v>
+        <v>7.667</v>
       </c>
       <c r="L39" t="n">
-        <v>8.041</v>
+        <v>8.068</v>
       </c>
       <c r="M39" t="n">
-        <v>8.425000000000001</v>
+        <v>8.456</v>
       </c>
       <c r="N39" t="n">
-        <v>8.592000000000001</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="O39" t="n">
-        <v>8.792</v>
+        <v>8.814</v>
       </c>
       <c r="P39" t="n">
-        <v>8.82</v>
+        <v>8.85</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.291</v>
+        <v>9.332000000000001</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.29</v>
+        <v>3.288</v>
       </c>
       <c r="G40" t="n">
-        <v>3.405</v>
+        <v>3.398</v>
       </c>
       <c r="H40" t="n">
-        <v>3.59</v>
+        <v>3.586</v>
       </c>
       <c r="I40" t="n">
-        <v>3.828</v>
+        <v>3.827</v>
       </c>
       <c r="J40" t="n">
-        <v>4.123</v>
+        <v>4.152</v>
       </c>
       <c r="K40" t="n">
-        <v>4.423</v>
+        <v>4.452</v>
       </c>
       <c r="L40" t="n">
-        <v>4.52</v>
+        <v>4.547</v>
       </c>
       <c r="M40" t="n">
-        <v>4.718</v>
+        <v>4.748</v>
       </c>
       <c r="N40" t="n">
-        <v>4.895</v>
+        <v>4.92</v>
       </c>
       <c r="O40" t="n">
-        <v>5.209</v>
+        <v>5.231</v>
       </c>
       <c r="P40" t="n">
-        <v>5.402</v>
+        <v>5.432</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.182</v>
+        <v>6.222</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.673</v>
+        <v>3.671</v>
       </c>
       <c r="G41" t="n">
-        <v>3.829</v>
+        <v>3.823</v>
       </c>
       <c r="H41" t="n">
-        <v>4.072</v>
+        <v>4.068</v>
       </c>
       <c r="I41" t="n">
-        <v>4.33</v>
+        <v>4.329</v>
       </c>
       <c r="J41" t="n">
-        <v>4.677</v>
+        <v>4.706</v>
       </c>
       <c r="K41" t="n">
-        <v>5.023</v>
+        <v>5.051</v>
       </c>
       <c r="L41" t="n">
-        <v>5.198</v>
+        <v>5.225</v>
       </c>
       <c r="M41" t="n">
-        <v>5.52</v>
+        <v>5.55</v>
       </c>
       <c r="N41" t="n">
-        <v>5.824</v>
+        <v>5.849</v>
       </c>
       <c r="O41" t="n">
-        <v>6.321</v>
+        <v>6.343</v>
       </c>
       <c r="P41" t="n">
-        <v>6.461</v>
+        <v>6.491</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.228</v>
+        <v>7.269</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.41</v>
+        <v>3.408</v>
       </c>
       <c r="G42" t="n">
-        <v>3.553</v>
+        <v>3.546</v>
       </c>
       <c r="H42" t="n">
-        <v>3.764</v>
+        <v>3.76</v>
       </c>
       <c r="I42" t="n">
-        <v>4.017</v>
+        <v>4.016</v>
       </c>
       <c r="J42" t="n">
-        <v>4.327</v>
+        <v>4.355</v>
       </c>
       <c r="K42" t="n">
-        <v>4.644</v>
+        <v>4.673</v>
       </c>
       <c r="L42" t="n">
-        <v>4.756</v>
+        <v>4.783</v>
       </c>
       <c r="M42" t="n">
-        <v>5.026</v>
+        <v>5.055</v>
       </c>
       <c r="N42" t="n">
-        <v>5.309</v>
+        <v>5.334</v>
       </c>
       <c r="O42" t="n">
-        <v>5.7</v>
+        <v>5.722</v>
       </c>
       <c r="P42" t="n">
-        <v>5.903</v>
+        <v>5.933</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.694</v>
+        <v>6.735</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.121</v>
+        <v>3.118</v>
       </c>
       <c r="G43" t="n">
-        <v>3.218</v>
+        <v>3.212</v>
       </c>
       <c r="H43" t="n">
-        <v>3.351</v>
+        <v>3.347</v>
       </c>
       <c r="I43" t="n">
-        <v>3.55</v>
+        <v>3.546</v>
       </c>
       <c r="J43" t="n">
-        <v>3.773</v>
+        <v>3.799</v>
       </c>
       <c r="K43" t="n">
-        <v>3.993</v>
+        <v>4.02</v>
       </c>
       <c r="L43" t="n">
-        <v>4.043</v>
+        <v>4.07</v>
       </c>
       <c r="M43" t="n">
-        <v>4.164</v>
+        <v>4.194</v>
       </c>
       <c r="N43" t="n">
-        <v>4.197</v>
+        <v>4.222</v>
       </c>
       <c r="O43" t="n">
-        <v>4.298</v>
+        <v>4.32</v>
       </c>
       <c r="P43" t="n">
-        <v>4.378</v>
+        <v>4.408</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.057</v>
+        <v>5.098</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.995</v>
+        <v>2.99</v>
       </c>
       <c r="G44" t="n">
-        <v>3.088</v>
+        <v>3.08</v>
       </c>
       <c r="H44" t="n">
-        <v>3.202</v>
+        <v>3.198</v>
       </c>
       <c r="I44" t="n">
-        <v>3.396</v>
+        <v>3.392</v>
       </c>
       <c r="J44" t="n">
-        <v>3.622</v>
+        <v>3.647</v>
       </c>
       <c r="K44" t="n">
-        <v>3.835</v>
+        <v>3.863</v>
       </c>
       <c r="L44" t="n">
-        <v>3.886</v>
+        <v>3.913</v>
       </c>
       <c r="M44" t="n">
-        <v>3.979</v>
+        <v>4.008</v>
       </c>
       <c r="N44" t="n">
-        <v>4.013</v>
+        <v>4.037</v>
       </c>
       <c r="O44" t="n">
-        <v>4.096</v>
+        <v>4.117</v>
       </c>
       <c r="P44" t="n">
-        <v>4.141</v>
+        <v>4.171</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.428</v>
+        <v>4.469</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-27 ~ 2026-04-27
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.209</v>
+        <v>3.201</v>
       </c>
       <c r="G2" t="n">
-        <v>3.417</v>
+        <v>3.411</v>
       </c>
       <c r="H2" t="n">
-        <v>3.584</v>
+        <v>3.581</v>
       </c>
       <c r="I2" t="n">
-        <v>3.785</v>
+        <v>3.779</v>
       </c>
       <c r="J2" t="n">
-        <v>4.108</v>
+        <v>4.098</v>
       </c>
       <c r="K2" t="n">
-        <v>4.516</v>
+        <v>4.509</v>
       </c>
       <c r="L2" t="n">
-        <v>4.7</v>
+        <v>4.697</v>
       </c>
       <c r="M2" t="n">
-        <v>4.993</v>
+        <v>4.991</v>
       </c>
       <c r="N2" t="n">
-        <v>5.259</v>
+        <v>5.256</v>
       </c>
       <c r="O2" t="n">
-        <v>5.483</v>
+        <v>5.478</v>
       </c>
       <c r="P2" t="n">
-        <v>5.657</v>
+        <v>5.661</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.285</v>
+        <v>6.29</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.232</v>
+        <v>4.224</v>
       </c>
       <c r="G3" t="n">
-        <v>4.621</v>
+        <v>4.615</v>
       </c>
       <c r="H3" t="n">
-        <v>4.822</v>
+        <v>4.819</v>
       </c>
       <c r="I3" t="n">
-        <v>5.019</v>
+        <v>5.012</v>
       </c>
       <c r="J3" t="n">
-        <v>5.353</v>
+        <v>5.344</v>
       </c>
       <c r="K3" t="n">
-        <v>5.831</v>
+        <v>5.824</v>
       </c>
       <c r="L3" t="n">
-        <v>6.085</v>
+        <v>6.082</v>
       </c>
       <c r="M3" t="n">
-        <v>6.411</v>
+        <v>6.409</v>
       </c>
       <c r="N3" t="n">
-        <v>6.619</v>
+        <v>6.616</v>
       </c>
       <c r="O3" t="n">
-        <v>6.792</v>
+        <v>6.788</v>
       </c>
       <c r="P3" t="n">
-        <v>6.837</v>
+        <v>6.841</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.353</v>
+        <v>7.358</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.725</v>
+        <v>3.717</v>
       </c>
       <c r="G4" t="n">
-        <v>4.002</v>
+        <v>3.996</v>
       </c>
       <c r="H4" t="n">
-        <v>4.232</v>
+        <v>4.229</v>
       </c>
       <c r="I4" t="n">
-        <v>4.462</v>
+        <v>4.455</v>
       </c>
       <c r="J4" t="n">
-        <v>4.801</v>
+        <v>4.79</v>
       </c>
       <c r="K4" t="n">
-        <v>5.271</v>
+        <v>5.263</v>
       </c>
       <c r="L4" t="n">
-        <v>5.455</v>
+        <v>5.451</v>
       </c>
       <c r="M4" t="n">
-        <v>5.768</v>
+        <v>5.766</v>
       </c>
       <c r="N4" t="n">
-        <v>5.947</v>
+        <v>5.944</v>
       </c>
       <c r="O4" t="n">
-        <v>6.145</v>
+        <v>6.14</v>
       </c>
       <c r="P4" t="n">
-        <v>6.187</v>
+        <v>6.191</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.706</v>
+        <v>6.711</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.903</v>
+        <v>2.898</v>
       </c>
       <c r="G5" t="n">
-        <v>2.956</v>
+        <v>2.953</v>
       </c>
       <c r="H5" t="n">
         <v>3.081</v>
       </c>
       <c r="I5" t="n">
-        <v>3.354</v>
+        <v>3.349</v>
       </c>
       <c r="J5" t="n">
-        <v>3.668</v>
+        <v>3.66</v>
       </c>
       <c r="K5" t="n">
-        <v>3.934</v>
+        <v>3.928</v>
       </c>
       <c r="L5" t="n">
-        <v>3.961</v>
+        <v>3.958</v>
       </c>
       <c r="M5" t="n">
-        <v>4.057</v>
+        <v>4.054</v>
       </c>
       <c r="N5" t="n">
-        <v>4.075</v>
+        <v>4.072</v>
       </c>
       <c r="O5" t="n">
-        <v>4.081</v>
+        <v>4.077</v>
       </c>
       <c r="P5" t="n">
-        <v>4.326</v>
+        <v>4.329</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.197</v>
+        <v>5.202</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.943</v>
+        <v>2.938</v>
       </c>
       <c r="G6" t="n">
-        <v>3.01</v>
+        <v>3.007</v>
       </c>
       <c r="H6" t="n">
         <v>3.152</v>
       </c>
       <c r="I6" t="n">
-        <v>3.436</v>
+        <v>3.431</v>
       </c>
       <c r="J6" t="n">
-        <v>3.756</v>
+        <v>3.749</v>
       </c>
       <c r="K6" t="n">
-        <v>4.046</v>
+        <v>4.04</v>
       </c>
       <c r="L6" t="n">
-        <v>4.08</v>
+        <v>4.077</v>
       </c>
       <c r="M6" t="n">
-        <v>4.215</v>
+        <v>4.213</v>
       </c>
       <c r="N6" t="n">
-        <v>4.243</v>
+        <v>4.24</v>
       </c>
       <c r="O6" t="n">
-        <v>4.35</v>
+        <v>4.345</v>
       </c>
       <c r="P6" t="n">
-        <v>4.758</v>
+        <v>4.762</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.593</v>
+        <v>5.598</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.924</v>
+        <v>2.919</v>
       </c>
       <c r="G7" t="n">
-        <v>2.974</v>
+        <v>2.971</v>
       </c>
       <c r="H7" t="n">
         <v>3.097</v>
       </c>
       <c r="I7" t="n">
-        <v>3.369</v>
+        <v>3.364</v>
       </c>
       <c r="J7" t="n">
-        <v>3.693</v>
+        <v>3.686</v>
       </c>
       <c r="K7" t="n">
-        <v>3.961</v>
+        <v>3.955</v>
       </c>
       <c r="L7" t="n">
-        <v>3.986</v>
+        <v>3.983</v>
       </c>
       <c r="M7" t="n">
-        <v>4.119</v>
+        <v>4.117</v>
       </c>
       <c r="N7" t="n">
-        <v>4.136</v>
+        <v>4.132</v>
       </c>
       <c r="O7" t="n">
-        <v>4.247</v>
+        <v>4.242</v>
       </c>
       <c r="P7" t="n">
-        <v>4.542</v>
+        <v>4.545</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.361</v>
+        <v>5.366</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.342</v>
+        <v>5.334</v>
       </c>
       <c r="G8" t="n">
-        <v>5.919</v>
+        <v>5.913</v>
       </c>
       <c r="H8" t="n">
-        <v>6.271</v>
+        <v>6.268</v>
       </c>
       <c r="I8" t="n">
-        <v>6.546</v>
+        <v>6.539</v>
       </c>
       <c r="J8" t="n">
-        <v>6.944</v>
+        <v>6.935</v>
       </c>
       <c r="K8" t="n">
-        <v>7.702</v>
+        <v>7.695</v>
       </c>
       <c r="L8" t="n">
-        <v>8.042999999999999</v>
+        <v>8.041</v>
       </c>
       <c r="M8" t="n">
-        <v>8.398999999999999</v>
+        <v>8.397</v>
       </c>
       <c r="N8" t="n">
-        <v>8.542</v>
+        <v>8.539</v>
       </c>
       <c r="O8" t="n">
-        <v>8.801</v>
+        <v>8.797000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>8.948</v>
+        <v>8.952</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.662000000000001</v>
+        <v>9.667</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.623</v>
+        <v>2.618</v>
       </c>
       <c r="G9" t="n">
-        <v>2.703</v>
+        <v>2.699</v>
       </c>
       <c r="H9" t="n">
-        <v>2.809</v>
+        <v>2.797</v>
       </c>
       <c r="I9" t="n">
-        <v>2.985</v>
+        <v>2.987</v>
       </c>
       <c r="J9" t="n">
-        <v>3.227</v>
+        <v>3.223</v>
       </c>
       <c r="K9" t="n">
-        <v>3.383</v>
+        <v>3.38</v>
       </c>
       <c r="L9" t="n">
-        <v>3.418</v>
+        <v>3.42</v>
       </c>
       <c r="M9" t="n">
-        <v>3.495</v>
+        <v>3.497</v>
       </c>
       <c r="N9" t="n">
         <v>3.652</v>
       </c>
       <c r="O9" t="n">
-        <v>3.681</v>
+        <v>3.677</v>
       </c>
       <c r="P9" t="n">
-        <v>3.748</v>
+        <v>3.752</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.815</v>
+        <v>3.819</v>
       </c>
       <c r="R9" t="n">
-        <v>3.786</v>
+        <v>3.791</v>
       </c>
       <c r="S9" t="n">
-        <v>3.755</v>
+        <v>3.759</v>
       </c>
       <c r="T9" t="n">
-        <v>3.671</v>
+        <v>3.677</v>
       </c>
       <c r="U9" t="n">
-        <v>3.543</v>
+        <v>3.548</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.636</v>
+        <v>2.632</v>
       </c>
       <c r="G10" t="n">
-        <v>2.738</v>
+        <v>2.732</v>
       </c>
       <c r="H10" t="n">
-        <v>2.825</v>
+        <v>2.812</v>
       </c>
       <c r="I10" t="n">
-        <v>2.996</v>
+        <v>2.997</v>
       </c>
       <c r="J10" t="n">
-        <v>3.253</v>
+        <v>3.249</v>
       </c>
       <c r="K10" t="n">
-        <v>3.417</v>
+        <v>3.413</v>
       </c>
       <c r="L10" t="n">
-        <v>3.47</v>
+        <v>3.471</v>
       </c>
       <c r="M10" t="n">
-        <v>3.591</v>
+        <v>3.594</v>
       </c>
       <c r="N10" t="n">
         <v>3.668</v>
       </c>
       <c r="O10" t="n">
-        <v>3.908</v>
+        <v>3.899</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.452</v>
+        <v>2.447</v>
       </c>
       <c r="G11" t="n">
-        <v>2.548</v>
+        <v>2.542</v>
       </c>
       <c r="H11" t="n">
-        <v>2.649</v>
+        <v>2.636</v>
       </c>
       <c r="I11" t="n">
-        <v>2.799</v>
+        <v>2.8</v>
       </c>
       <c r="J11" t="n">
-        <v>3.047</v>
+        <v>3.043</v>
       </c>
       <c r="K11" t="n">
-        <v>3.204</v>
+        <v>3.2</v>
       </c>
       <c r="L11" t="n">
-        <v>3.264</v>
+        <v>3.265</v>
       </c>
       <c r="M11" t="n">
-        <v>3.397</v>
+        <v>3.399</v>
       </c>
       <c r="N11" t="n">
         <v>3.476</v>
       </c>
       <c r="O11" t="n">
-        <v>3.674</v>
+        <v>3.665</v>
       </c>
       <c r="P11" t="n">
-        <v>3.695</v>
+        <v>3.698</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.016</v>
+        <v>4.021</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.193</v>
+        <v>3.185</v>
       </c>
       <c r="G12" t="n">
-        <v>3.348</v>
+        <v>3.34</v>
       </c>
       <c r="H12" t="n">
-        <v>3.461</v>
+        <v>3.458</v>
       </c>
       <c r="I12" t="n">
-        <v>3.704</v>
+        <v>3.696</v>
       </c>
       <c r="J12" t="n">
-        <v>4.079</v>
+        <v>4.072</v>
       </c>
       <c r="K12" t="n">
-        <v>4.286</v>
+        <v>4.282</v>
       </c>
       <c r="L12" t="n">
-        <v>4.357</v>
+        <v>4.354</v>
       </c>
       <c r="M12" t="n">
-        <v>4.493</v>
+        <v>4.492</v>
       </c>
       <c r="N12" t="n">
         <v>4.538</v>
       </c>
       <c r="O12" t="n">
-        <v>4.683</v>
+        <v>4.678</v>
       </c>
       <c r="P12" t="n">
-        <v>4.793</v>
+        <v>4.797</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.144</v>
+        <v>5.149</v>
       </c>
       <c r="R12" t="n">
-        <v>5.286</v>
+        <v>5.291</v>
       </c>
       <c r="S12" t="n">
-        <v>5.465</v>
+        <v>5.471</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.947</v>
+        <v>2.939</v>
       </c>
       <c r="G13" t="n">
-        <v>3.038</v>
+        <v>3.03</v>
       </c>
       <c r="H13" t="n">
-        <v>3.129</v>
+        <v>3.126</v>
       </c>
       <c r="I13" t="n">
-        <v>3.352</v>
+        <v>3.344</v>
       </c>
       <c r="J13" t="n">
-        <v>3.716</v>
+        <v>3.709</v>
       </c>
       <c r="K13" t="n">
-        <v>3.919</v>
+        <v>3.916</v>
       </c>
       <c r="L13" t="n">
-        <v>3.997</v>
+        <v>3.994</v>
       </c>
       <c r="M13" t="n">
-        <v>4.12</v>
+        <v>4.119</v>
       </c>
       <c r="N13" t="n">
         <v>4.166</v>
       </c>
       <c r="O13" t="n">
-        <v>4.311</v>
+        <v>4.307</v>
       </c>
       <c r="P13" t="n">
-        <v>4.385</v>
+        <v>4.388</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.664</v>
+        <v>4.669</v>
       </c>
       <c r="R13" t="n">
-        <v>4.834</v>
+        <v>4.84</v>
       </c>
       <c r="S13" t="n">
-        <v>5.028</v>
+        <v>5.033</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.766</v>
+        <v>2.758</v>
       </c>
       <c r="G14" t="n">
-        <v>2.844</v>
+        <v>2.836</v>
       </c>
       <c r="H14" t="n">
-        <v>2.932</v>
+        <v>2.929</v>
       </c>
       <c r="I14" t="n">
-        <v>3.136</v>
+        <v>3.128</v>
       </c>
       <c r="J14" t="n">
-        <v>3.457</v>
+        <v>3.449</v>
       </c>
       <c r="K14" t="n">
-        <v>3.607</v>
+        <v>3.604</v>
       </c>
       <c r="L14" t="n">
-        <v>3.668</v>
+        <v>3.666</v>
       </c>
       <c r="M14" t="n">
-        <v>3.805</v>
+        <v>3.804</v>
       </c>
       <c r="N14" t="n">
         <v>3.845</v>
       </c>
       <c r="O14" t="n">
-        <v>3.966</v>
+        <v>3.961</v>
       </c>
       <c r="P14" t="n">
-        <v>4.02</v>
+        <v>4.023</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.253</v>
+        <v>4.258</v>
       </c>
       <c r="R14" t="n">
-        <v>4.35</v>
+        <v>4.354</v>
       </c>
       <c r="S14" t="n">
-        <v>4.481</v>
+        <v>4.486</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.744</v>
+        <v>2.736</v>
       </c>
       <c r="G15" t="n">
-        <v>2.818</v>
+        <v>2.81</v>
       </c>
       <c r="H15" t="n">
-        <v>2.901</v>
+        <v>2.9</v>
       </c>
       <c r="I15" t="n">
-        <v>3.088</v>
+        <v>3.079</v>
       </c>
       <c r="J15" t="n">
-        <v>3.396</v>
+        <v>3.388</v>
       </c>
       <c r="K15" t="n">
-        <v>3.56</v>
+        <v>3.557</v>
       </c>
       <c r="L15" t="n">
-        <v>3.604</v>
+        <v>3.601</v>
       </c>
       <c r="M15" t="n">
-        <v>3.719</v>
+        <v>3.718</v>
       </c>
       <c r="N15" t="n">
         <v>3.749</v>
       </c>
       <c r="O15" t="n">
-        <v>3.905</v>
+        <v>3.901</v>
       </c>
       <c r="P15" t="n">
-        <v>3.92</v>
+        <v>3.923</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.158</v>
+        <v>4.163</v>
       </c>
       <c r="R15" t="n">
-        <v>4.246</v>
+        <v>4.251</v>
       </c>
       <c r="S15" t="n">
-        <v>4.376</v>
+        <v>4.381</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.744</v>
+        <v>2.736</v>
       </c>
       <c r="G16" t="n">
-        <v>2.818</v>
+        <v>2.81</v>
       </c>
       <c r="H16" t="n">
-        <v>2.901</v>
+        <v>2.9</v>
       </c>
       <c r="I16" t="n">
-        <v>3.088</v>
+        <v>3.079</v>
       </c>
       <c r="J16" t="n">
-        <v>3.396</v>
+        <v>3.388</v>
       </c>
       <c r="K16" t="n">
-        <v>3.56</v>
+        <v>3.557</v>
       </c>
       <c r="L16" t="n">
-        <v>3.604</v>
+        <v>3.601</v>
       </c>
       <c r="M16" t="n">
-        <v>3.719</v>
+        <v>3.718</v>
       </c>
       <c r="N16" t="n">
         <v>3.752</v>
       </c>
       <c r="O16" t="n">
-        <v>3.911</v>
+        <v>3.908</v>
       </c>
       <c r="P16" t="n">
-        <v>3.943</v>
+        <v>3.947</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.185</v>
+        <v>4.19</v>
       </c>
       <c r="R16" t="n">
-        <v>4.274</v>
+        <v>4.279</v>
       </c>
       <c r="S16" t="n">
-        <v>4.405</v>
+        <v>4.41</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.699</v>
+        <v>2.693</v>
       </c>
       <c r="G17" t="n">
-        <v>2.828</v>
+        <v>2.823</v>
       </c>
       <c r="H17" t="n">
-        <v>2.918</v>
+        <v>2.905</v>
       </c>
       <c r="I17" t="n">
-        <v>3.078</v>
+        <v>3.079</v>
       </c>
       <c r="J17" t="n">
-        <v>3.324</v>
+        <v>3.319</v>
       </c>
       <c r="K17" t="n">
-        <v>3.493</v>
+        <v>3.488</v>
       </c>
       <c r="L17" t="n">
-        <v>3.549</v>
+        <v>3.551</v>
       </c>
       <c r="M17" t="n">
-        <v>3.711</v>
+        <v>3.713</v>
       </c>
       <c r="N17" t="n">
-        <v>3.769</v>
+        <v>3.771</v>
       </c>
       <c r="O17" t="n">
-        <v>3.935</v>
+        <v>3.925</v>
       </c>
       <c r="P17" t="n">
-        <v>3.969</v>
+        <v>3.974</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.7</v>
+        <v>2.694</v>
       </c>
       <c r="G18" t="n">
-        <v>2.829</v>
+        <v>2.824</v>
       </c>
       <c r="H18" t="n">
-        <v>2.918</v>
+        <v>2.905</v>
       </c>
       <c r="I18" t="n">
-        <v>3.078</v>
+        <v>3.079</v>
       </c>
       <c r="J18" t="n">
-        <v>3.324</v>
+        <v>3.319</v>
       </c>
       <c r="K18" t="n">
-        <v>3.494</v>
+        <v>3.489</v>
       </c>
       <c r="L18" t="n">
-        <v>3.549</v>
+        <v>3.551</v>
       </c>
       <c r="M18" t="n">
-        <v>3.711</v>
+        <v>3.713</v>
       </c>
       <c r="N18" t="n">
-        <v>3.77</v>
+        <v>3.772</v>
       </c>
       <c r="O18" t="n">
-        <v>3.934</v>
+        <v>3.925</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.757</v>
+        <v>2.749</v>
       </c>
       <c r="G19" t="n">
-        <v>2.835</v>
+        <v>2.827</v>
       </c>
       <c r="H19" t="n">
-        <v>2.921</v>
+        <v>2.918</v>
       </c>
       <c r="I19" t="n">
-        <v>3.123</v>
+        <v>3.115</v>
       </c>
       <c r="J19" t="n">
-        <v>3.44</v>
+        <v>3.432</v>
       </c>
       <c r="K19" t="n">
-        <v>3.604</v>
+        <v>3.6</v>
       </c>
       <c r="L19" t="n">
-        <v>3.665</v>
+        <v>3.663</v>
       </c>
       <c r="M19" t="n">
-        <v>3.797</v>
+        <v>3.796</v>
       </c>
       <c r="N19" t="n">
         <v>3.833</v>
       </c>
       <c r="O19" t="n">
-        <v>3.95</v>
+        <v>3.945</v>
       </c>
       <c r="P19" t="n">
-        <v>3.98</v>
+        <v>3.983</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.2</v>
+        <v>4.205</v>
       </c>
       <c r="R19" t="n">
-        <v>4.297</v>
+        <v>4.301</v>
       </c>
       <c r="S19" t="n">
-        <v>4.419</v>
+        <v>4.424</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.578</v>
+        <v>2.574</v>
       </c>
       <c r="G20" t="n">
-        <v>2.648</v>
+        <v>2.645</v>
       </c>
       <c r="H20" t="n">
-        <v>2.693</v>
+        <v>2.69</v>
       </c>
       <c r="I20" t="n">
-        <v>2.834</v>
+        <v>2.828</v>
       </c>
       <c r="J20" t="n">
-        <v>3.22</v>
+        <v>3.215</v>
       </c>
       <c r="K20" t="n">
         <v>3.397</v>
       </c>
       <c r="L20" t="n">
-        <v>3.439</v>
+        <v>3.435</v>
       </c>
       <c r="M20" t="n">
-        <v>3.54</v>
+        <v>3.53</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,25 +1939,25 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.866</v>
+        <v>2.861</v>
       </c>
       <c r="G21" t="n">
-        <v>2.942</v>
+        <v>2.937</v>
       </c>
       <c r="H21" t="n">
-        <v>3.071</v>
+        <v>3.067</v>
       </c>
       <c r="I21" t="n">
-        <v>3.245</v>
+        <v>3.238</v>
       </c>
       <c r="J21" t="n">
-        <v>3.578</v>
+        <v>3.57</v>
       </c>
       <c r="K21" t="n">
-        <v>3.841</v>
+        <v>3.835</v>
       </c>
       <c r="L21" t="n">
-        <v>3.907</v>
+        <v>3.908</v>
       </c>
       <c r="M21" t="n">
         <v>4.036</v>
@@ -1966,19 +1966,19 @@
         <v>4.088</v>
       </c>
       <c r="O21" t="n">
-        <v>4.166</v>
+        <v>4.161</v>
       </c>
       <c r="P21" t="n">
-        <v>4.246</v>
+        <v>4.25</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.366</v>
+        <v>4.368</v>
       </c>
       <c r="R21" t="n">
-        <v>4.349</v>
+        <v>4.354</v>
       </c>
       <c r="S21" t="n">
-        <v>4.38</v>
+        <v>4.385</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.813</v>
+        <v>2.808</v>
       </c>
       <c r="G22" t="n">
-        <v>2.888</v>
+        <v>2.883</v>
       </c>
       <c r="H22" t="n">
-        <v>3.003</v>
+        <v>2.999</v>
       </c>
       <c r="I22" t="n">
-        <v>3.165</v>
+        <v>3.158</v>
       </c>
       <c r="J22" t="n">
-        <v>3.462</v>
+        <v>3.453</v>
       </c>
       <c r="K22" t="n">
-        <v>3.72</v>
+        <v>3.714</v>
       </c>
       <c r="L22" t="n">
-        <v>3.775</v>
+        <v>3.776</v>
       </c>
       <c r="M22" t="n">
         <v>3.906</v>
       </c>
       <c r="N22" t="n">
-        <v>3.961</v>
+        <v>3.96</v>
       </c>
       <c r="O22" t="n">
-        <v>4.034</v>
+        <v>4.029</v>
       </c>
       <c r="P22" t="n">
-        <v>4.108</v>
+        <v>4.112</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.224</v>
+        <v>4.227</v>
       </c>
       <c r="R22" t="n">
-        <v>4.197</v>
+        <v>4.202</v>
       </c>
       <c r="S22" t="n">
-        <v>4.225</v>
+        <v>4.23</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.766</v>
+        <v>2.761</v>
       </c>
       <c r="G23" t="n">
-        <v>2.843</v>
+        <v>2.838</v>
       </c>
       <c r="H23" t="n">
-        <v>2.942</v>
+        <v>2.938</v>
       </c>
       <c r="I23" t="n">
-        <v>3.118</v>
+        <v>3.111</v>
       </c>
       <c r="J23" t="n">
-        <v>3.407</v>
+        <v>3.399</v>
       </c>
       <c r="K23" t="n">
-        <v>3.633</v>
+        <v>3.625</v>
       </c>
       <c r="L23" t="n">
-        <v>3.686</v>
+        <v>3.685</v>
       </c>
       <c r="M23" t="n">
-        <v>3.81</v>
+        <v>3.808</v>
       </c>
       <c r="N23" t="n">
         <v>3.857</v>
       </c>
       <c r="O23" t="n">
-        <v>3.91</v>
+        <v>3.905</v>
       </c>
       <c r="P23" t="n">
-        <v>3.969</v>
+        <v>3.973</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.031</v>
+        <v>4.034</v>
       </c>
       <c r="R23" t="n">
-        <v>3.98</v>
+        <v>3.985</v>
       </c>
       <c r="S23" t="n">
-        <v>3.979</v>
+        <v>3.985</v>
       </c>
       <c r="T23" t="n">
-        <v>3.887</v>
+        <v>3.892</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.701</v>
+        <v>2.696</v>
       </c>
       <c r="G24" t="n">
-        <v>2.757</v>
+        <v>2.752</v>
       </c>
       <c r="H24" t="n">
-        <v>2.843</v>
+        <v>2.839</v>
       </c>
       <c r="I24" t="n">
-        <v>3.028</v>
+        <v>3.021</v>
       </c>
       <c r="J24" t="n">
-        <v>3.306</v>
+        <v>3.297</v>
       </c>
       <c r="K24" t="n">
-        <v>3.517</v>
+        <v>3.511</v>
       </c>
       <c r="L24" t="n">
-        <v>3.56</v>
+        <v>3.559</v>
       </c>
       <c r="M24" t="n">
-        <v>3.669</v>
+        <v>3.667</v>
       </c>
       <c r="N24" t="n">
         <v>3.734</v>
       </c>
       <c r="O24" t="n">
-        <v>3.902</v>
+        <v>3.899</v>
       </c>
       <c r="P24" t="n">
-        <v>3.913</v>
+        <v>3.917</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.954</v>
+        <v>3.957</v>
       </c>
       <c r="R24" t="n">
-        <v>3.901</v>
+        <v>3.906</v>
       </c>
       <c r="S24" t="n">
-        <v>3.895</v>
+        <v>3.9</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.759</v>
+        <v>2.754</v>
       </c>
       <c r="G25" t="n">
-        <v>2.842</v>
+        <v>2.837</v>
       </c>
       <c r="H25" t="n">
-        <v>2.945</v>
+        <v>2.941</v>
       </c>
       <c r="I25" t="n">
-        <v>3.126</v>
+        <v>3.119</v>
       </c>
       <c r="J25" t="n">
-        <v>3.422</v>
+        <v>3.414</v>
       </c>
       <c r="K25" t="n">
-        <v>3.665</v>
+        <v>3.657</v>
       </c>
       <c r="L25" t="n">
-        <v>3.716</v>
+        <v>3.714</v>
       </c>
       <c r="M25" t="n">
-        <v>3.84</v>
+        <v>3.838</v>
       </c>
       <c r="N25" t="n">
         <v>3.884</v>
       </c>
       <c r="O25" t="n">
-        <v>3.939</v>
+        <v>3.935</v>
       </c>
       <c r="P25" t="n">
-        <v>3.991</v>
+        <v>3.995</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.064</v>
+        <v>4.066</v>
       </c>
       <c r="R25" t="n">
-        <v>4.004</v>
+        <v>4.009</v>
       </c>
       <c r="S25" t="n">
-        <v>4.003</v>
+        <v>4.008</v>
       </c>
       <c r="T25" t="n">
-        <v>3.905</v>
+        <v>3.91</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.062</v>
+        <v>3.054</v>
       </c>
       <c r="G26" t="n">
-        <v>3.194</v>
+        <v>3.189</v>
       </c>
       <c r="H26" t="n">
-        <v>3.41</v>
+        <v>3.408</v>
       </c>
       <c r="I26" t="n">
-        <v>3.65</v>
+        <v>3.643</v>
       </c>
       <c r="J26" t="n">
-        <v>4.083</v>
+        <v>4.074</v>
       </c>
       <c r="K26" t="n">
-        <v>4.476</v>
+        <v>4.47</v>
       </c>
       <c r="L26" t="n">
-        <v>4.588</v>
+        <v>4.586</v>
       </c>
       <c r="M26" t="n">
-        <v>4.77</v>
+        <v>4.769</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.018</v>
+        <v>5.014</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,25 +2377,25 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.857</v>
+        <v>2.848</v>
       </c>
       <c r="G27" t="n">
-        <v>2.925</v>
+        <v>2.918</v>
       </c>
       <c r="H27" t="n">
-        <v>3.041</v>
+        <v>3.038</v>
       </c>
       <c r="I27" t="n">
-        <v>3.246</v>
+        <v>3.238</v>
       </c>
       <c r="J27" t="n">
-        <v>3.581</v>
+        <v>3.572</v>
       </c>
       <c r="K27" t="n">
-        <v>3.786</v>
+        <v>3.783</v>
       </c>
       <c r="L27" t="n">
-        <v>3.851</v>
+        <v>3.849</v>
       </c>
       <c r="M27" t="n">
         <v>3.976</v>
@@ -2404,7 +2404,7 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.11</v>
+        <v>4.105</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,25 +2450,25 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.96</v>
+        <v>2.951</v>
       </c>
       <c r="G28" t="n">
-        <v>3.036</v>
+        <v>3.029</v>
       </c>
       <c r="H28" t="n">
-        <v>3.167</v>
+        <v>3.164</v>
       </c>
       <c r="I28" t="n">
-        <v>3.384</v>
+        <v>3.376</v>
       </c>
       <c r="J28" t="n">
-        <v>3.754</v>
+        <v>3.745</v>
       </c>
       <c r="K28" t="n">
-        <v>3.979</v>
+        <v>3.976</v>
       </c>
       <c r="L28" t="n">
-        <v>4.055</v>
+        <v>4.053</v>
       </c>
       <c r="M28" t="n">
         <v>4.188</v>
@@ -2477,7 +2477,7 @@
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.404</v>
+        <v>4.399</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,25 +2523,25 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.813</v>
+        <v>2.804</v>
       </c>
       <c r="G29" t="n">
-        <v>2.882</v>
+        <v>2.874</v>
       </c>
       <c r="H29" t="n">
-        <v>2.982</v>
+        <v>2.979</v>
       </c>
       <c r="I29" t="n">
-        <v>3.18</v>
+        <v>3.171</v>
       </c>
       <c r="J29" t="n">
-        <v>3.493</v>
+        <v>3.484</v>
       </c>
       <c r="K29" t="n">
-        <v>3.682</v>
+        <v>3.679</v>
       </c>
       <c r="L29" t="n">
-        <v>3.736</v>
+        <v>3.734</v>
       </c>
       <c r="M29" t="n">
         <v>3.838</v>
@@ -2550,7 +2550,7 @@
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.976</v>
+        <v>3.972</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.097</v>
+        <v>3.089</v>
       </c>
       <c r="G30" t="n">
-        <v>3.165</v>
+        <v>3.161</v>
       </c>
       <c r="H30" t="n">
-        <v>3.348</v>
+        <v>3.345</v>
       </c>
       <c r="I30" t="n">
-        <v>3.58</v>
+        <v>3.573</v>
       </c>
       <c r="J30" t="n">
-        <v>3.953</v>
+        <v>3.944</v>
       </c>
       <c r="K30" t="n">
-        <v>4.269</v>
+        <v>4.265</v>
       </c>
       <c r="L30" t="n">
-        <v>4.357</v>
+        <v>4.356</v>
       </c>
       <c r="M30" t="n">
         <v>4.532</v>
       </c>
       <c r="N30" t="n">
-        <v>4.696</v>
+        <v>4.695</v>
       </c>
       <c r="O30" t="n">
-        <v>4.969</v>
+        <v>4.965</v>
       </c>
       <c r="P30" t="n">
-        <v>5.133</v>
+        <v>5.137</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.889</v>
+        <v>5.894</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.423</v>
+        <v>3.415</v>
       </c>
       <c r="G31" t="n">
-        <v>3.525</v>
+        <v>3.521</v>
       </c>
       <c r="H31" t="n">
-        <v>3.759</v>
+        <v>3.756</v>
       </c>
       <c r="I31" t="n">
-        <v>4.008</v>
+        <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>4.443</v>
+        <v>4.434</v>
       </c>
       <c r="K31" t="n">
-        <v>4.801</v>
+        <v>4.797</v>
       </c>
       <c r="L31" t="n">
-        <v>4.968</v>
+        <v>4.967</v>
       </c>
       <c r="M31" t="n">
         <v>5.262</v>
       </c>
       <c r="N31" t="n">
-        <v>5.553</v>
+        <v>5.552</v>
       </c>
       <c r="O31" t="n">
-        <v>6.003</v>
+        <v>5.998</v>
       </c>
       <c r="P31" t="n">
-        <v>6.12</v>
+        <v>6.124</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.863</v>
+        <v>6.868</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,25 +2742,25 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.195</v>
+        <v>3.187</v>
       </c>
       <c r="G32" t="n">
-        <v>3.281</v>
+        <v>3.277</v>
       </c>
       <c r="H32" t="n">
-        <v>3.49</v>
+        <v>3.487</v>
       </c>
       <c r="I32" t="n">
-        <v>3.739</v>
+        <v>3.732</v>
       </c>
       <c r="J32" t="n">
-        <v>4.132</v>
+        <v>4.123</v>
       </c>
       <c r="K32" t="n">
-        <v>4.454</v>
+        <v>4.45</v>
       </c>
       <c r="L32" t="n">
-        <v>4.561</v>
+        <v>4.56</v>
       </c>
       <c r="M32" t="n">
         <v>4.805</v>
@@ -2769,13 +2769,13 @@
         <v>5.056</v>
       </c>
       <c r="O32" t="n">
-        <v>5.414</v>
+        <v>5.409</v>
       </c>
       <c r="P32" t="n">
-        <v>5.592</v>
+        <v>5.596</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.35</v>
+        <v>6.355</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.972</v>
+        <v>2.962</v>
       </c>
       <c r="G33" t="n">
-        <v>3.034</v>
+        <v>3.03</v>
       </c>
       <c r="H33" t="n">
-        <v>3.166</v>
+        <v>3.163</v>
       </c>
       <c r="I33" t="n">
-        <v>3.362</v>
+        <v>3.354</v>
       </c>
       <c r="J33" t="n">
-        <v>3.661</v>
+        <v>3.651</v>
       </c>
       <c r="K33" t="n">
-        <v>3.911</v>
+        <v>3.906</v>
       </c>
       <c r="L33" t="n">
-        <v>3.964</v>
+        <v>3.962</v>
       </c>
       <c r="M33" t="n">
         <v>4.066</v>
       </c>
       <c r="N33" t="n">
-        <v>4.087</v>
+        <v>4.086</v>
       </c>
       <c r="O33" t="n">
-        <v>4.125</v>
+        <v>4.121</v>
       </c>
       <c r="P33" t="n">
-        <v>4.165</v>
+        <v>4.169</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.606</v>
+        <v>4.611</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.031</v>
+        <v>3.021</v>
       </c>
       <c r="G34" t="n">
-        <v>3.088</v>
+        <v>3.084</v>
       </c>
       <c r="H34" t="n">
-        <v>3.227</v>
+        <v>3.224</v>
       </c>
       <c r="I34" t="n">
-        <v>3.43</v>
+        <v>3.422</v>
       </c>
       <c r="J34" t="n">
-        <v>3.733</v>
+        <v>3.723</v>
       </c>
       <c r="K34" t="n">
-        <v>3.988</v>
+        <v>3.982</v>
       </c>
       <c r="L34" t="n">
-        <v>4.043</v>
+        <v>4.041</v>
       </c>
       <c r="M34" t="n">
-        <v>4.157</v>
+        <v>4.156</v>
       </c>
       <c r="N34" t="n">
-        <v>4.192</v>
+        <v>4.191</v>
       </c>
       <c r="O34" t="n">
-        <v>4.294</v>
+        <v>4.289</v>
       </c>
       <c r="P34" t="n">
-        <v>4.46</v>
+        <v>4.463</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.307</v>
+        <v>5.312</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.006</v>
+        <v>2.996</v>
       </c>
       <c r="G35" t="n">
-        <v>3.061</v>
+        <v>3.057</v>
       </c>
       <c r="H35" t="n">
-        <v>3.195</v>
+        <v>3.192</v>
       </c>
       <c r="I35" t="n">
-        <v>3.396</v>
+        <v>3.389</v>
       </c>
       <c r="J35" t="n">
-        <v>3.701</v>
+        <v>3.691</v>
       </c>
       <c r="K35" t="n">
-        <v>3.942</v>
+        <v>3.937</v>
       </c>
       <c r="L35" t="n">
-        <v>3.998</v>
+        <v>3.996</v>
       </c>
       <c r="M35" t="n">
-        <v>4.104</v>
+        <v>4.103</v>
       </c>
       <c r="N35" t="n">
         <v>4.128</v>
       </c>
       <c r="O35" t="n">
-        <v>4.192</v>
+        <v>4.187</v>
       </c>
       <c r="P35" t="n">
-        <v>4.262</v>
+        <v>4.266</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.943</v>
+        <v>4.947</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,25 +3034,25 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.914</v>
+        <v>2.904</v>
       </c>
       <c r="G36" t="n">
-        <v>2.974</v>
+        <v>2.968</v>
       </c>
       <c r="H36" t="n">
-        <v>3.088</v>
+        <v>3.084</v>
       </c>
       <c r="I36" t="n">
-        <v>3.289</v>
+        <v>3.281</v>
       </c>
       <c r="J36" t="n">
-        <v>3.597</v>
+        <v>3.587</v>
       </c>
       <c r="K36" t="n">
-        <v>3.834</v>
+        <v>3.829</v>
       </c>
       <c r="L36" t="n">
-        <v>3.887</v>
+        <v>3.886</v>
       </c>
       <c r="M36" t="n">
         <v>3.965</v>
@@ -3061,13 +3061,13 @@
         <v>3.989</v>
       </c>
       <c r="O36" t="n">
-        <v>4.035</v>
+        <v>4.031</v>
       </c>
       <c r="P36" t="n">
-        <v>4.064</v>
+        <v>4.068</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.323</v>
+        <v>4.328</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.767</v>
+        <v>3.759</v>
       </c>
       <c r="G37" t="n">
-        <v>4.22</v>
+        <v>4.216</v>
       </c>
       <c r="H37" t="n">
-        <v>4.734</v>
+        <v>4.731</v>
       </c>
       <c r="I37" t="n">
-        <v>5.073</v>
+        <v>5.066</v>
       </c>
       <c r="J37" t="n">
-        <v>5.934</v>
+        <v>5.925</v>
       </c>
       <c r="K37" t="n">
-        <v>6.841</v>
+        <v>6.837</v>
       </c>
       <c r="L37" t="n">
         <v>7.168</v>
       </c>
       <c r="M37" t="n">
-        <v>7.535</v>
+        <v>7.534</v>
       </c>
       <c r="N37" t="n">
-        <v>7.703</v>
+        <v>7.702</v>
       </c>
       <c r="O37" t="n">
-        <v>7.882</v>
+        <v>7.877</v>
       </c>
       <c r="P37" t="n">
-        <v>7.92</v>
+        <v>7.923</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.352</v>
+        <v>8.356</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.824</v>
+        <v>4.818</v>
       </c>
       <c r="G38" t="n">
-        <v>5.531</v>
+        <v>5.528</v>
       </c>
       <c r="H38" t="n">
-        <v>6.258</v>
+        <v>6.255</v>
       </c>
       <c r="I38" t="n">
-        <v>6.753</v>
+        <v>6.747</v>
       </c>
       <c r="J38" t="n">
-        <v>7.874</v>
+        <v>7.867</v>
       </c>
       <c r="K38" t="n">
-        <v>8.959</v>
+        <v>8.956</v>
       </c>
       <c r="L38" t="n">
-        <v>9.446999999999999</v>
+        <v>9.446</v>
       </c>
       <c r="M38" t="n">
-        <v>9.945</v>
+        <v>9.944000000000001</v>
       </c>
       <c r="N38" t="n">
-        <v>10.121</v>
+        <v>10.12</v>
       </c>
       <c r="O38" t="n">
-        <v>10.281</v>
+        <v>10.277</v>
       </c>
       <c r="P38" t="n">
-        <v>10.318</v>
+        <v>10.321</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.803</v>
+        <v>10.806</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,25 +3253,25 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.145</v>
+        <v>4.139</v>
       </c>
       <c r="G39" t="n">
-        <v>4.729</v>
+        <v>4.726</v>
       </c>
       <c r="H39" t="n">
-        <v>5.323</v>
+        <v>5.32</v>
       </c>
       <c r="I39" t="n">
-        <v>5.757</v>
+        <v>5.75</v>
       </c>
       <c r="J39" t="n">
-        <v>6.747</v>
+        <v>6.739</v>
       </c>
       <c r="K39" t="n">
-        <v>7.792</v>
+        <v>7.789</v>
       </c>
       <c r="L39" t="n">
-        <v>8.204000000000001</v>
+        <v>8.202999999999999</v>
       </c>
       <c r="M39" t="n">
         <v>8.581</v>
@@ -3280,13 +3280,13 @@
         <v>8.747999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.930999999999999</v>
+        <v>8.927</v>
       </c>
       <c r="P39" t="n">
-        <v>8.972</v>
+        <v>8.976000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.448</v>
+        <v>9.452</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.29</v>
+        <v>3.282</v>
       </c>
       <c r="G40" t="n">
-        <v>3.404</v>
+        <v>3.4</v>
       </c>
       <c r="H40" t="n">
-        <v>3.607</v>
+        <v>3.604</v>
       </c>
       <c r="I40" t="n">
-        <v>3.855</v>
+        <v>3.848</v>
       </c>
       <c r="J40" t="n">
-        <v>4.246</v>
+        <v>4.236</v>
       </c>
       <c r="K40" t="n">
-        <v>4.574</v>
+        <v>4.57</v>
       </c>
       <c r="L40" t="n">
-        <v>4.681</v>
+        <v>4.68</v>
       </c>
       <c r="M40" t="n">
-        <v>4.874</v>
+        <v>4.873</v>
       </c>
       <c r="N40" t="n">
         <v>5.053</v>
       </c>
       <c r="O40" t="n">
-        <v>5.348</v>
+        <v>5.343</v>
       </c>
       <c r="P40" t="n">
-        <v>5.554</v>
+        <v>5.558</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.34</v>
+        <v>6.345</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,25 +3399,25 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.673</v>
+        <v>3.665</v>
       </c>
       <c r="G41" t="n">
-        <v>3.828</v>
+        <v>3.824</v>
       </c>
       <c r="H41" t="n">
-        <v>4.089</v>
+        <v>4.086</v>
       </c>
       <c r="I41" t="n">
-        <v>4.357</v>
+        <v>4.349</v>
       </c>
       <c r="J41" t="n">
-        <v>4.8</v>
+        <v>4.79</v>
       </c>
       <c r="K41" t="n">
-        <v>5.174</v>
+        <v>5.17</v>
       </c>
       <c r="L41" t="n">
-        <v>5.358</v>
+        <v>5.357</v>
       </c>
       <c r="M41" t="n">
         <v>5.675</v>
@@ -3426,13 +3426,13 @@
         <v>5.982</v>
       </c>
       <c r="O41" t="n">
-        <v>6.46</v>
+        <v>6.456</v>
       </c>
       <c r="P41" t="n">
-        <v>6.613</v>
+        <v>6.616</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.387</v>
+        <v>7.392</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.41</v>
+        <v>3.402</v>
       </c>
       <c r="G42" t="n">
-        <v>3.552</v>
+        <v>3.548</v>
       </c>
       <c r="H42" t="n">
-        <v>3.782</v>
+        <v>3.779</v>
       </c>
       <c r="I42" t="n">
-        <v>4.043</v>
+        <v>4.036</v>
       </c>
       <c r="J42" t="n">
-        <v>4.449</v>
+        <v>4.439</v>
       </c>
       <c r="K42" t="n">
-        <v>4.795</v>
+        <v>4.791</v>
       </c>
       <c r="L42" t="n">
-        <v>4.917</v>
+        <v>4.916</v>
       </c>
       <c r="M42" t="n">
-        <v>5.181</v>
+        <v>5.18</v>
       </c>
       <c r="N42" t="n">
-        <v>5.468</v>
+        <v>5.467</v>
       </c>
       <c r="O42" t="n">
-        <v>5.838</v>
+        <v>5.834</v>
       </c>
       <c r="P42" t="n">
-        <v>6.055</v>
+        <v>6.059</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.853</v>
+        <v>6.858</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.12</v>
+        <v>3.11</v>
       </c>
       <c r="G43" t="n">
-        <v>3.217</v>
+        <v>3.213</v>
       </c>
       <c r="H43" t="n">
-        <v>3.367</v>
+        <v>3.364</v>
       </c>
       <c r="I43" t="n">
-        <v>3.571</v>
+        <v>3.564</v>
       </c>
       <c r="J43" t="n">
-        <v>3.889</v>
+        <v>3.879</v>
       </c>
       <c r="K43" t="n">
-        <v>4.142</v>
+        <v>4.137</v>
       </c>
       <c r="L43" t="n">
-        <v>4.205</v>
+        <v>4.203</v>
       </c>
       <c r="M43" t="n">
-        <v>4.32</v>
+        <v>4.319</v>
       </c>
       <c r="N43" t="n">
         <v>4.356</v>
       </c>
       <c r="O43" t="n">
-        <v>4.438</v>
+        <v>4.433</v>
       </c>
       <c r="P43" t="n">
-        <v>4.531</v>
+        <v>4.535</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.216</v>
+        <v>5.221</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46136</v>
+        <v>46139</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,25 +3618,25 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.992</v>
+        <v>2.982</v>
       </c>
       <c r="G44" t="n">
-        <v>3.084</v>
+        <v>3.078</v>
       </c>
       <c r="H44" t="n">
-        <v>3.212</v>
+        <v>3.208</v>
       </c>
       <c r="I44" t="n">
-        <v>3.417</v>
+        <v>3.409</v>
       </c>
       <c r="J44" t="n">
-        <v>3.739</v>
+        <v>3.728</v>
       </c>
       <c r="K44" t="n">
-        <v>3.985</v>
+        <v>3.98</v>
       </c>
       <c r="L44" t="n">
-        <v>4.048</v>
+        <v>4.046</v>
       </c>
       <c r="M44" t="n">
         <v>4.134</v>
@@ -3645,13 +3645,13 @@
         <v>4.171</v>
       </c>
       <c r="O44" t="n">
-        <v>4.234</v>
+        <v>4.23</v>
       </c>
       <c r="P44" t="n">
-        <v>4.295</v>
+        <v>4.298</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.587</v>
+        <v>4.592</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-07 ~ 2026-05-07
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.184</v>
+        <v>3.175</v>
       </c>
       <c r="G2" t="n">
-        <v>3.403</v>
+        <v>3.395</v>
       </c>
       <c r="H2" t="n">
-        <v>3.612</v>
+        <v>3.613</v>
       </c>
       <c r="I2" t="n">
-        <v>3.806</v>
+        <v>3.798</v>
       </c>
       <c r="J2" t="n">
-        <v>4.144</v>
+        <v>4.111</v>
       </c>
       <c r="K2" t="n">
-        <v>4.597</v>
+        <v>4.537</v>
       </c>
       <c r="L2" t="n">
-        <v>4.779</v>
+        <v>4.7</v>
       </c>
       <c r="M2" t="n">
-        <v>5.074</v>
+        <v>5.013</v>
       </c>
       <c r="N2" t="n">
-        <v>5.352</v>
+        <v>5.282</v>
       </c>
       <c r="O2" t="n">
-        <v>5.587</v>
+        <v>5.518</v>
       </c>
       <c r="P2" t="n">
-        <v>5.775</v>
+        <v>5.711</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.405</v>
+        <v>6.346</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.208</v>
+        <v>4.199</v>
       </c>
       <c r="G3" t="n">
-        <v>4.608</v>
+        <v>4.6</v>
       </c>
       <c r="H3" t="n">
-        <v>4.85</v>
+        <v>4.851</v>
       </c>
       <c r="I3" t="n">
-        <v>5.039</v>
+        <v>5.03</v>
       </c>
       <c r="J3" t="n">
-        <v>5.39</v>
+        <v>5.356</v>
       </c>
       <c r="K3" t="n">
-        <v>5.913</v>
+        <v>5.853</v>
       </c>
       <c r="L3" t="n">
-        <v>6.165</v>
+        <v>6.085</v>
       </c>
       <c r="M3" t="n">
-        <v>6.491</v>
+        <v>6.43</v>
       </c>
       <c r="N3" t="n">
-        <v>6.711</v>
+        <v>6.642</v>
       </c>
       <c r="O3" t="n">
-        <v>6.897</v>
+        <v>6.828</v>
       </c>
       <c r="P3" t="n">
-        <v>6.955</v>
+        <v>6.891</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.473</v>
+        <v>7.415</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.7</v>
+        <v>3.691</v>
       </c>
       <c r="G4" t="n">
-        <v>3.989</v>
+        <v>3.981</v>
       </c>
       <c r="H4" t="n">
         <v>4.26</v>
       </c>
       <c r="I4" t="n">
-        <v>4.482</v>
+        <v>4.473</v>
       </c>
       <c r="J4" t="n">
-        <v>4.835</v>
+        <v>4.802</v>
       </c>
       <c r="K4" t="n">
-        <v>5.352</v>
+        <v>5.292</v>
       </c>
       <c r="L4" t="n">
-        <v>5.533</v>
+        <v>5.454</v>
       </c>
       <c r="M4" t="n">
-        <v>5.849</v>
+        <v>5.788</v>
       </c>
       <c r="N4" t="n">
-        <v>6.04</v>
+        <v>5.97</v>
       </c>
       <c r="O4" t="n">
-        <v>6.249</v>
+        <v>6.179</v>
       </c>
       <c r="P4" t="n">
-        <v>6.305</v>
+        <v>6.241</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.826</v>
+        <v>6.768</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.879</v>
+        <v>2.87</v>
       </c>
       <c r="G5" t="n">
-        <v>2.947</v>
+        <v>2.939</v>
       </c>
       <c r="H5" t="n">
-        <v>3.114</v>
+        <v>3.115</v>
       </c>
       <c r="I5" t="n">
-        <v>3.376</v>
+        <v>3.37</v>
       </c>
       <c r="J5" t="n">
-        <v>3.707</v>
+        <v>3.673</v>
       </c>
       <c r="K5" t="n">
-        <v>4.012</v>
+        <v>3.95</v>
       </c>
       <c r="L5" t="n">
-        <v>4.035</v>
+        <v>3.958</v>
       </c>
       <c r="M5" t="n">
-        <v>4.134</v>
+        <v>4.073</v>
       </c>
       <c r="N5" t="n">
-        <v>4.166</v>
+        <v>4.096</v>
       </c>
       <c r="O5" t="n">
-        <v>4.187</v>
+        <v>4.117</v>
       </c>
       <c r="P5" t="n">
-        <v>4.444</v>
+        <v>4.38</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.317</v>
+        <v>5.259</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.918</v>
+        <v>2.909</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>2.992</v>
       </c>
       <c r="H6" t="n">
-        <v>3.183</v>
+        <v>3.184</v>
       </c>
       <c r="I6" t="n">
-        <v>3.457</v>
+        <v>3.45</v>
       </c>
       <c r="J6" t="n">
-        <v>3.793</v>
+        <v>3.761</v>
       </c>
       <c r="K6" t="n">
-        <v>4.121</v>
+        <v>4.059</v>
       </c>
       <c r="L6" t="n">
-        <v>4.152</v>
+        <v>4.072</v>
       </c>
       <c r="M6" t="n">
-        <v>4.29</v>
+        <v>4.229</v>
       </c>
       <c r="N6" t="n">
-        <v>4.333</v>
+        <v>4.264</v>
       </c>
       <c r="O6" t="n">
-        <v>4.453</v>
+        <v>4.384</v>
       </c>
       <c r="P6" t="n">
-        <v>4.876</v>
+        <v>4.812</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.713</v>
+        <v>5.655</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.899</v>
+        <v>2.89</v>
       </c>
       <c r="G7" t="n">
-        <v>2.964</v>
+        <v>2.956</v>
       </c>
       <c r="H7" t="n">
-        <v>3.129</v>
+        <v>3.13</v>
       </c>
       <c r="I7" t="n">
-        <v>3.391</v>
+        <v>3.385</v>
       </c>
       <c r="J7" t="n">
-        <v>3.731</v>
+        <v>3.697</v>
       </c>
       <c r="K7" t="n">
-        <v>4.038</v>
+        <v>3.976</v>
       </c>
       <c r="L7" t="n">
-        <v>4.06</v>
+        <v>3.982</v>
       </c>
       <c r="M7" t="n">
-        <v>4.195</v>
+        <v>4.135</v>
       </c>
       <c r="N7" t="n">
-        <v>4.226</v>
+        <v>4.156</v>
       </c>
       <c r="O7" t="n">
-        <v>4.351</v>
+        <v>4.281</v>
       </c>
       <c r="P7" t="n">
-        <v>4.66</v>
+        <v>4.596</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.481</v>
+        <v>5.423</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.319</v>
+        <v>5.311</v>
       </c>
       <c r="G8" t="n">
-        <v>5.907</v>
+        <v>5.9</v>
       </c>
       <c r="H8" t="n">
-        <v>6.299</v>
+        <v>6.3</v>
       </c>
       <c r="I8" t="n">
-        <v>6.566</v>
+        <v>6.557</v>
       </c>
       <c r="J8" t="n">
-        <v>6.983</v>
+        <v>6.949</v>
       </c>
       <c r="K8" t="n">
-        <v>7.786</v>
+        <v>7.725</v>
       </c>
       <c r="L8" t="n">
-        <v>8.124000000000001</v>
+        <v>8.044</v>
       </c>
       <c r="M8" t="n">
-        <v>8.481</v>
+        <v>8.42</v>
       </c>
       <c r="N8" t="n">
-        <v>8.635999999999999</v>
+        <v>8.566000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>8.907</v>
+        <v>8.837</v>
       </c>
       <c r="P8" t="n">
-        <v>9.066000000000001</v>
+        <v>9.002000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.782999999999999</v>
+        <v>9.724</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.612</v>
+        <v>2.606</v>
       </c>
       <c r="G9" t="n">
-        <v>2.691</v>
+        <v>2.687</v>
       </c>
       <c r="H9" t="n">
-        <v>2.81</v>
+        <v>2.8</v>
       </c>
       <c r="I9" t="n">
-        <v>3.02</v>
+        <v>3.008</v>
       </c>
       <c r="J9" t="n">
-        <v>3.265</v>
+        <v>3.245</v>
       </c>
       <c r="K9" t="n">
-        <v>3.495</v>
+        <v>3.432</v>
       </c>
       <c r="L9" t="n">
-        <v>3.522</v>
+        <v>3.442</v>
       </c>
       <c r="M9" t="n">
-        <v>3.595</v>
+        <v>3.535</v>
       </c>
       <c r="N9" t="n">
-        <v>3.75</v>
+        <v>3.68</v>
       </c>
       <c r="O9" t="n">
-        <v>3.786</v>
+        <v>3.717</v>
       </c>
       <c r="P9" t="n">
-        <v>3.866</v>
+        <v>3.802</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.935</v>
+        <v>3.876</v>
       </c>
       <c r="R9" t="n">
-        <v>3.929</v>
+        <v>3.883</v>
       </c>
       <c r="S9" t="n">
-        <v>3.932</v>
+        <v>3.892</v>
       </c>
       <c r="T9" t="n">
-        <v>3.85</v>
+        <v>3.817</v>
       </c>
       <c r="U9" t="n">
-        <v>3.722</v>
+        <v>3.689</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.626</v>
+        <v>2.62</v>
       </c>
       <c r="G10" t="n">
-        <v>2.723</v>
+        <v>2.72</v>
       </c>
       <c r="H10" t="n">
-        <v>2.824</v>
+        <v>2.813</v>
       </c>
       <c r="I10" t="n">
-        <v>3.032</v>
+        <v>3.021</v>
       </c>
       <c r="J10" t="n">
-        <v>3.292</v>
+        <v>3.267</v>
       </c>
       <c r="K10" t="n">
-        <v>3.528</v>
+        <v>3.465</v>
       </c>
       <c r="L10" t="n">
-        <v>3.574</v>
+        <v>3.49</v>
       </c>
       <c r="M10" t="n">
-        <v>3.693</v>
+        <v>3.632</v>
       </c>
       <c r="N10" t="n">
-        <v>3.767</v>
+        <v>3.697</v>
       </c>
       <c r="O10" t="n">
-        <v>3.995</v>
+        <v>3.925</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.441</v>
+        <v>2.435</v>
       </c>
       <c r="G11" t="n">
-        <v>2.533</v>
+        <v>2.53</v>
       </c>
       <c r="H11" t="n">
-        <v>2.648</v>
+        <v>2.638</v>
       </c>
       <c r="I11" t="n">
-        <v>2.835</v>
+        <v>2.824</v>
       </c>
       <c r="J11" t="n">
-        <v>3.087</v>
+        <v>3.065</v>
       </c>
       <c r="K11" t="n">
-        <v>3.315</v>
+        <v>3.252</v>
       </c>
       <c r="L11" t="n">
-        <v>3.367</v>
+        <v>3.287</v>
       </c>
       <c r="M11" t="n">
-        <v>3.498</v>
+        <v>3.437</v>
       </c>
       <c r="N11" t="n">
-        <v>3.575</v>
+        <v>3.505</v>
       </c>
       <c r="O11" t="n">
-        <v>3.762</v>
+        <v>3.692</v>
       </c>
       <c r="P11" t="n">
-        <v>3.815</v>
+        <v>3.753</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.136</v>
+        <v>4.077</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.173</v>
+        <v>3.17</v>
       </c>
       <c r="G12" t="n">
         <v>3.34</v>
       </c>
       <c r="H12" t="n">
-        <v>3.489</v>
+        <v>3.495</v>
       </c>
       <c r="I12" t="n">
-        <v>3.747</v>
+        <v>3.741</v>
       </c>
       <c r="J12" t="n">
-        <v>4.134</v>
+        <v>4.101</v>
       </c>
       <c r="K12" t="n">
-        <v>4.378</v>
+        <v>4.319</v>
       </c>
       <c r="L12" t="n">
-        <v>4.444</v>
+        <v>4.367</v>
       </c>
       <c r="M12" t="n">
-        <v>4.584</v>
+        <v>4.523</v>
       </c>
       <c r="N12" t="n">
-        <v>4.631</v>
+        <v>4.564</v>
       </c>
       <c r="O12" t="n">
-        <v>4.786</v>
+        <v>4.717</v>
       </c>
       <c r="P12" t="n">
-        <v>4.911</v>
+        <v>4.847</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.262</v>
+        <v>5.204</v>
       </c>
       <c r="R12" t="n">
-        <v>5.429</v>
+        <v>5.382</v>
       </c>
       <c r="S12" t="n">
-        <v>5.642</v>
+        <v>5.602</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.926</v>
+        <v>2.923</v>
       </c>
       <c r="G13" t="n">
         <v>3.03</v>
       </c>
       <c r="H13" t="n">
-        <v>3.156</v>
+        <v>3.162</v>
       </c>
       <c r="I13" t="n">
-        <v>3.395</v>
+        <v>3.389</v>
       </c>
       <c r="J13" t="n">
-        <v>3.771</v>
+        <v>3.738</v>
       </c>
       <c r="K13" t="n">
-        <v>4.011</v>
+        <v>3.952</v>
       </c>
       <c r="L13" t="n">
-        <v>4.084</v>
+        <v>4.006</v>
       </c>
       <c r="M13" t="n">
-        <v>4.212</v>
+        <v>4.151</v>
       </c>
       <c r="N13" t="n">
-        <v>4.26</v>
+        <v>4.192</v>
       </c>
       <c r="O13" t="n">
-        <v>4.414</v>
+        <v>4.346</v>
       </c>
       <c r="P13" t="n">
-        <v>4.503</v>
+        <v>4.439</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.783</v>
+        <v>4.725</v>
       </c>
       <c r="R13" t="n">
-        <v>4.977</v>
+        <v>4.931</v>
       </c>
       <c r="S13" t="n">
-        <v>5.204</v>
+        <v>5.164</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.746</v>
+        <v>2.742</v>
       </c>
       <c r="G14" t="n">
         <v>2.835</v>
       </c>
       <c r="H14" t="n">
-        <v>2.96</v>
+        <v>2.965</v>
       </c>
       <c r="I14" t="n">
-        <v>3.178</v>
+        <v>3.173</v>
       </c>
       <c r="J14" t="n">
-        <v>3.511</v>
+        <v>3.478</v>
       </c>
       <c r="K14" t="n">
-        <v>3.699</v>
+        <v>3.64</v>
       </c>
       <c r="L14" t="n">
-        <v>3.756</v>
+        <v>3.678</v>
       </c>
       <c r="M14" t="n">
-        <v>3.897</v>
+        <v>3.836</v>
       </c>
       <c r="N14" t="n">
-        <v>3.938</v>
+        <v>3.87</v>
       </c>
       <c r="O14" t="n">
-        <v>4.07</v>
+        <v>4.001</v>
       </c>
       <c r="P14" t="n">
-        <v>4.138</v>
+        <v>4.074</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.372</v>
+        <v>4.314</v>
       </c>
       <c r="R14" t="n">
-        <v>4.492</v>
+        <v>4.445</v>
       </c>
       <c r="S14" t="n">
-        <v>4.657</v>
+        <v>4.617</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.723</v>
+        <v>2.72</v>
       </c>
       <c r="G15" t="n">
         <v>2.81</v>
       </c>
       <c r="H15" t="n">
-        <v>2.93</v>
+        <v>2.936</v>
       </c>
       <c r="I15" t="n">
-        <v>3.13</v>
+        <v>3.124</v>
       </c>
       <c r="J15" t="n">
-        <v>3.45</v>
+        <v>3.417</v>
       </c>
       <c r="K15" t="n">
-        <v>3.651</v>
+        <v>3.592</v>
       </c>
       <c r="L15" t="n">
-        <v>3.691</v>
+        <v>3.614</v>
       </c>
       <c r="M15" t="n">
-        <v>3.81</v>
+        <v>3.748</v>
       </c>
       <c r="N15" t="n">
-        <v>3.842</v>
+        <v>3.774</v>
       </c>
       <c r="O15" t="n">
-        <v>4.011</v>
+        <v>3.943</v>
       </c>
       <c r="P15" t="n">
-        <v>4.037</v>
+        <v>3.974</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.275</v>
+        <v>4.217</v>
       </c>
       <c r="R15" t="n">
-        <v>4.389</v>
+        <v>4.342</v>
       </c>
       <c r="S15" t="n">
-        <v>4.552</v>
+        <v>4.512</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.723</v>
+        <v>2.72</v>
       </c>
       <c r="G16" t="n">
         <v>2.81</v>
       </c>
       <c r="H16" t="n">
-        <v>2.93</v>
+        <v>2.936</v>
       </c>
       <c r="I16" t="n">
-        <v>3.13</v>
+        <v>3.124</v>
       </c>
       <c r="J16" t="n">
-        <v>3.45</v>
+        <v>3.417</v>
       </c>
       <c r="K16" t="n">
-        <v>3.651</v>
+        <v>3.592</v>
       </c>
       <c r="L16" t="n">
-        <v>3.691</v>
+        <v>3.614</v>
       </c>
       <c r="M16" t="n">
-        <v>3.81</v>
+        <v>3.748</v>
       </c>
       <c r="N16" t="n">
-        <v>3.845</v>
+        <v>3.777</v>
       </c>
       <c r="O16" t="n">
-        <v>4.018</v>
+        <v>3.95</v>
       </c>
       <c r="P16" t="n">
-        <v>4.061</v>
+        <v>3.997</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.302</v>
+        <v>4.244</v>
       </c>
       <c r="R16" t="n">
-        <v>4.417</v>
+        <v>4.37</v>
       </c>
       <c r="S16" t="n">
-        <v>4.581</v>
+        <v>4.541</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.687</v>
+        <v>2.681</v>
       </c>
       <c r="G17" t="n">
-        <v>2.815</v>
+        <v>2.812</v>
       </c>
       <c r="H17" t="n">
-        <v>2.919</v>
+        <v>2.909</v>
       </c>
       <c r="I17" t="n">
-        <v>3.114</v>
+        <v>3.102</v>
       </c>
       <c r="J17" t="n">
-        <v>3.364</v>
+        <v>3.343</v>
       </c>
       <c r="K17" t="n">
-        <v>3.604</v>
+        <v>3.542</v>
       </c>
       <c r="L17" t="n">
-        <v>3.653</v>
+        <v>3.573</v>
       </c>
       <c r="M17" t="n">
-        <v>3.812</v>
+        <v>3.751</v>
       </c>
       <c r="N17" t="n">
-        <v>3.87</v>
+        <v>3.8</v>
       </c>
       <c r="O17" t="n">
-        <v>4.023</v>
+        <v>3.953</v>
       </c>
       <c r="P17" t="n">
-        <v>4.091</v>
+        <v>4.029</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.688</v>
+        <v>2.682</v>
       </c>
       <c r="G18" t="n">
-        <v>2.816</v>
+        <v>2.813</v>
       </c>
       <c r="H18" t="n">
-        <v>2.919</v>
+        <v>2.909</v>
       </c>
       <c r="I18" t="n">
-        <v>3.114</v>
+        <v>3.103</v>
       </c>
       <c r="J18" t="n">
-        <v>3.364</v>
+        <v>3.343</v>
       </c>
       <c r="K18" t="n">
-        <v>3.605</v>
+        <v>3.542</v>
       </c>
       <c r="L18" t="n">
-        <v>3.653</v>
+        <v>3.573</v>
       </c>
       <c r="M18" t="n">
-        <v>3.812</v>
+        <v>3.751</v>
       </c>
       <c r="N18" t="n">
-        <v>3.87</v>
+        <v>3.8</v>
       </c>
       <c r="O18" t="n">
-        <v>4.021</v>
+        <v>3.95</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.737</v>
+        <v>2.734</v>
       </c>
       <c r="G19" t="n">
         <v>2.826</v>
       </c>
       <c r="H19" t="n">
-        <v>2.949</v>
+        <v>2.955</v>
       </c>
       <c r="I19" t="n">
-        <v>3.165</v>
+        <v>3.16</v>
       </c>
       <c r="J19" t="n">
-        <v>3.495</v>
+        <v>3.462</v>
       </c>
       <c r="K19" t="n">
-        <v>3.695</v>
+        <v>3.636</v>
       </c>
       <c r="L19" t="n">
-        <v>3.753</v>
+        <v>3.675</v>
       </c>
       <c r="M19" t="n">
-        <v>3.887</v>
+        <v>3.826</v>
       </c>
       <c r="N19" t="n">
-        <v>3.927</v>
+        <v>3.86</v>
       </c>
       <c r="O19" t="n">
-        <v>4.054</v>
+        <v>3.985</v>
       </c>
       <c r="P19" t="n">
-        <v>4.097</v>
+        <v>4.033</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.316</v>
+        <v>4.257</v>
       </c>
       <c r="R19" t="n">
-        <v>4.437</v>
+        <v>4.39</v>
       </c>
       <c r="S19" t="n">
-        <v>4.592</v>
+        <v>4.552</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.575</v>
+        <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.649</v>
+        <v>2.646</v>
       </c>
       <c r="H20" t="n">
-        <v>2.705</v>
+        <v>2.703</v>
       </c>
       <c r="I20" t="n">
-        <v>2.85</v>
+        <v>2.843</v>
       </c>
       <c r="J20" t="n">
-        <v>3.27</v>
+        <v>3.24</v>
       </c>
       <c r="K20" t="n">
-        <v>3.508</v>
+        <v>3.449</v>
       </c>
       <c r="L20" t="n">
-        <v>3.545</v>
+        <v>3.483</v>
       </c>
       <c r="M20" t="n">
-        <v>3.635</v>
+        <v>3.573</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.859</v>
+        <v>2.855</v>
       </c>
       <c r="G21" t="n">
-        <v>2.934</v>
+        <v>2.931</v>
       </c>
       <c r="H21" t="n">
-        <v>3.089</v>
+        <v>3.094</v>
       </c>
       <c r="I21" t="n">
-        <v>3.282</v>
+        <v>3.274</v>
       </c>
       <c r="J21" t="n">
-        <v>3.634</v>
+        <v>3.605</v>
       </c>
       <c r="K21" t="n">
-        <v>3.928</v>
+        <v>3.868</v>
       </c>
       <c r="L21" t="n">
-        <v>3.994</v>
+        <v>3.916</v>
       </c>
       <c r="M21" t="n">
-        <v>4.117</v>
+        <v>4.056</v>
       </c>
       <c r="N21" t="n">
-        <v>4.181</v>
+        <v>4.111</v>
       </c>
       <c r="O21" t="n">
-        <v>4.272</v>
+        <v>4.203</v>
       </c>
       <c r="P21" t="n">
-        <v>4.364</v>
+        <v>4.3</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.479</v>
+        <v>4.42</v>
       </c>
       <c r="R21" t="n">
-        <v>4.491</v>
+        <v>4.445</v>
       </c>
       <c r="S21" t="n">
-        <v>4.557</v>
+        <v>4.517</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.806</v>
+        <v>2.803</v>
       </c>
       <c r="G22" t="n">
-        <v>2.88</v>
+        <v>2.878</v>
       </c>
       <c r="H22" t="n">
-        <v>3.021</v>
+        <v>3.027</v>
       </c>
       <c r="I22" t="n">
-        <v>3.199</v>
+        <v>3.191</v>
       </c>
       <c r="J22" t="n">
-        <v>3.52</v>
+        <v>3.491</v>
       </c>
       <c r="K22" t="n">
-        <v>3.809</v>
+        <v>3.749</v>
       </c>
       <c r="L22" t="n">
-        <v>3.862</v>
+        <v>3.784</v>
       </c>
       <c r="M22" t="n">
-        <v>3.986</v>
+        <v>3.925</v>
       </c>
       <c r="N22" t="n">
-        <v>4.053</v>
+        <v>3.984</v>
       </c>
       <c r="O22" t="n">
-        <v>4.14</v>
+        <v>4.07</v>
       </c>
       <c r="P22" t="n">
-        <v>4.226</v>
+        <v>4.162</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.337</v>
+        <v>4.279</v>
       </c>
       <c r="R22" t="n">
-        <v>4.339</v>
+        <v>4.293</v>
       </c>
       <c r="S22" t="n">
-        <v>4.402</v>
+        <v>4.362</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.758</v>
+        <v>2.755</v>
       </c>
       <c r="G23" t="n">
-        <v>2.835</v>
+        <v>2.832</v>
       </c>
       <c r="H23" t="n">
-        <v>2.961</v>
+        <v>2.967</v>
       </c>
       <c r="I23" t="n">
-        <v>3.154</v>
+        <v>3.146</v>
       </c>
       <c r="J23" t="n">
-        <v>3.463</v>
+        <v>3.433</v>
       </c>
       <c r="K23" t="n">
-        <v>3.715</v>
+        <v>3.655</v>
       </c>
       <c r="L23" t="n">
-        <v>3.767</v>
+        <v>3.688</v>
       </c>
       <c r="M23" t="n">
-        <v>3.884</v>
+        <v>3.822</v>
       </c>
       <c r="N23" t="n">
-        <v>3.949</v>
+        <v>3.879</v>
       </c>
       <c r="O23" t="n">
-        <v>4.018</v>
+        <v>3.947</v>
       </c>
       <c r="P23" t="n">
-        <v>4.091</v>
+        <v>4.027</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.143</v>
+        <v>4.085</v>
       </c>
       <c r="R23" t="n">
-        <v>4.123</v>
+        <v>4.077</v>
       </c>
       <c r="S23" t="n">
-        <v>4.157</v>
+        <v>4.117</v>
       </c>
       <c r="T23" t="n">
-        <v>4.066</v>
+        <v>4.032</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.693</v>
+        <v>2.69</v>
       </c>
       <c r="G24" t="n">
-        <v>2.75</v>
+        <v>2.748</v>
       </c>
       <c r="H24" t="n">
-        <v>2.862</v>
+        <v>2.868</v>
       </c>
       <c r="I24" t="n">
-        <v>3.065</v>
+        <v>3.057</v>
       </c>
       <c r="J24" t="n">
-        <v>3.362</v>
+        <v>3.332</v>
       </c>
       <c r="K24" t="n">
-        <v>3.601</v>
+        <v>3.54</v>
       </c>
       <c r="L24" t="n">
-        <v>3.644</v>
+        <v>3.566</v>
       </c>
       <c r="M24" t="n">
-        <v>3.746</v>
+        <v>3.685</v>
       </c>
       <c r="N24" t="n">
-        <v>3.826</v>
+        <v>3.756</v>
       </c>
       <c r="O24" t="n">
-        <v>4.009</v>
+        <v>3.94</v>
       </c>
       <c r="P24" t="n">
-        <v>4.03</v>
+        <v>3.966</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.068</v>
+        <v>4.01</v>
       </c>
       <c r="R24" t="n">
-        <v>4.045</v>
+        <v>3.999</v>
       </c>
       <c r="S24" t="n">
-        <v>4.072</v>
+        <v>4.032</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.752</v>
+        <v>2.748</v>
       </c>
       <c r="G25" t="n">
-        <v>2.834</v>
+        <v>2.832</v>
       </c>
       <c r="H25" t="n">
-        <v>2.964</v>
+        <v>2.97</v>
       </c>
       <c r="I25" t="n">
-        <v>3.161</v>
+        <v>3.153</v>
       </c>
       <c r="J25" t="n">
-        <v>3.479</v>
+        <v>3.448</v>
       </c>
       <c r="K25" t="n">
-        <v>3.747</v>
+        <v>3.687</v>
       </c>
       <c r="L25" t="n">
-        <v>3.796</v>
+        <v>3.718</v>
       </c>
       <c r="M25" t="n">
-        <v>3.914</v>
+        <v>3.853</v>
       </c>
       <c r="N25" t="n">
-        <v>3.975</v>
+        <v>3.906</v>
       </c>
       <c r="O25" t="n">
-        <v>4.047</v>
+        <v>3.977</v>
       </c>
       <c r="P25" t="n">
-        <v>4.113</v>
+        <v>4.049</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.177</v>
+        <v>4.118</v>
       </c>
       <c r="R25" t="n">
-        <v>4.147</v>
+        <v>4.101</v>
       </c>
       <c r="S25" t="n">
-        <v>4.18</v>
+        <v>4.14</v>
       </c>
       <c r="T25" t="n">
-        <v>4.084</v>
+        <v>4.05</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.04</v>
+        <v>3.036</v>
       </c>
       <c r="G26" t="n">
-        <v>3.181</v>
+        <v>3.178</v>
       </c>
       <c r="H26" t="n">
-        <v>3.429</v>
+        <v>3.431</v>
       </c>
       <c r="I26" t="n">
-        <v>3.667</v>
+        <v>3.661</v>
       </c>
       <c r="J26" t="n">
-        <v>4.125</v>
+        <v>4.094</v>
       </c>
       <c r="K26" t="n">
-        <v>4.565</v>
+        <v>4.505</v>
       </c>
       <c r="L26" t="n">
-        <v>4.675</v>
+        <v>4.596</v>
       </c>
       <c r="M26" t="n">
-        <v>4.859</v>
+        <v>4.798</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.124</v>
+        <v>5.054</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.838</v>
+        <v>2.836</v>
       </c>
       <c r="G27" t="n">
         <v>2.917</v>
       </c>
       <c r="H27" t="n">
-        <v>3.063</v>
+        <v>3.067</v>
       </c>
       <c r="I27" t="n">
-        <v>3.277</v>
+        <v>3.271</v>
       </c>
       <c r="J27" t="n">
-        <v>3.628</v>
+        <v>3.597</v>
       </c>
       <c r="K27" t="n">
-        <v>3.878</v>
+        <v>3.819</v>
       </c>
       <c r="L27" t="n">
-        <v>3.938</v>
+        <v>3.859</v>
       </c>
       <c r="M27" t="n">
-        <v>4.067</v>
+        <v>4.005</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.214</v>
+        <v>4.144</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.941</v>
+        <v>2.939</v>
       </c>
       <c r="G28" t="n">
         <v>3.028</v>
       </c>
       <c r="H28" t="n">
-        <v>3.188</v>
+        <v>3.192</v>
       </c>
       <c r="I28" t="n">
-        <v>3.414</v>
+        <v>3.409</v>
       </c>
       <c r="J28" t="n">
-        <v>3.801</v>
+        <v>3.77</v>
       </c>
       <c r="K28" t="n">
-        <v>4.07</v>
+        <v>4.011</v>
       </c>
       <c r="L28" t="n">
-        <v>4.142</v>
+        <v>4.063</v>
       </c>
       <c r="M28" t="n">
-        <v>4.279</v>
+        <v>4.217</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.507</v>
+        <v>4.438</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.794</v>
+        <v>2.789</v>
       </c>
       <c r="G29" t="n">
-        <v>2.873</v>
+        <v>2.871</v>
       </c>
       <c r="H29" t="n">
-        <v>3.003</v>
+        <v>3.007</v>
       </c>
       <c r="I29" t="n">
-        <v>3.209</v>
+        <v>3.204</v>
       </c>
       <c r="J29" t="n">
-        <v>3.541</v>
+        <v>3.509</v>
       </c>
       <c r="K29" t="n">
-        <v>3.774</v>
+        <v>3.715</v>
       </c>
       <c r="L29" t="n">
-        <v>3.823</v>
+        <v>3.744</v>
       </c>
       <c r="M29" t="n">
-        <v>3.93</v>
+        <v>3.867</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.083</v>
+        <v>4.013</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.079</v>
+        <v>3.077</v>
       </c>
       <c r="G30" t="n">
-        <v>3.158</v>
+        <v>3.155</v>
       </c>
       <c r="H30" t="n">
-        <v>3.362</v>
+        <v>3.364</v>
       </c>
       <c r="I30" t="n">
-        <v>3.598</v>
+        <v>3.592</v>
       </c>
       <c r="J30" t="n">
-        <v>3.993</v>
+        <v>3.963</v>
       </c>
       <c r="K30" t="n">
-        <v>4.359</v>
+        <v>4.299</v>
       </c>
       <c r="L30" t="n">
-        <v>4.447</v>
+        <v>4.369</v>
       </c>
       <c r="M30" t="n">
-        <v>4.623</v>
+        <v>4.562</v>
       </c>
       <c r="N30" t="n">
-        <v>4.79</v>
+        <v>4.72</v>
       </c>
       <c r="O30" t="n">
-        <v>5.073</v>
+        <v>5.003</v>
       </c>
       <c r="P30" t="n">
-        <v>5.25</v>
+        <v>5.186</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.009</v>
+        <v>5.951</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.406</v>
+        <v>3.404</v>
       </c>
       <c r="G31" t="n">
-        <v>3.52</v>
+        <v>3.517</v>
       </c>
       <c r="H31" t="n">
-        <v>3.776</v>
+        <v>3.779</v>
       </c>
       <c r="I31" t="n">
-        <v>4.026</v>
+        <v>4.02</v>
       </c>
       <c r="J31" t="n">
-        <v>4.484</v>
+        <v>4.454</v>
       </c>
       <c r="K31" t="n">
-        <v>4.892</v>
+        <v>4.831</v>
       </c>
       <c r="L31" t="n">
-        <v>5.059</v>
+        <v>4.98</v>
       </c>
       <c r="M31" t="n">
-        <v>5.352</v>
+        <v>5.291</v>
       </c>
       <c r="N31" t="n">
-        <v>5.647</v>
+        <v>5.577</v>
       </c>
       <c r="O31" t="n">
-        <v>6.107</v>
+        <v>6.038</v>
       </c>
       <c r="P31" t="n">
-        <v>6.237</v>
+        <v>6.173</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.983</v>
+        <v>6.924</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.178</v>
+        <v>3.176</v>
       </c>
       <c r="G32" t="n">
-        <v>3.275</v>
+        <v>3.272</v>
       </c>
       <c r="H32" t="n">
-        <v>3.506</v>
+        <v>3.508</v>
       </c>
       <c r="I32" t="n">
-        <v>3.757</v>
+        <v>3.751</v>
       </c>
       <c r="J32" t="n">
-        <v>4.171</v>
+        <v>4.141</v>
       </c>
       <c r="K32" t="n">
-        <v>4.545</v>
+        <v>4.484</v>
       </c>
       <c r="L32" t="n">
-        <v>4.651</v>
+        <v>4.573</v>
       </c>
       <c r="M32" t="n">
-        <v>4.895</v>
+        <v>4.834</v>
       </c>
       <c r="N32" t="n">
-        <v>5.151</v>
+        <v>5.081</v>
       </c>
       <c r="O32" t="n">
-        <v>5.519</v>
+        <v>5.449</v>
       </c>
       <c r="P32" t="n">
-        <v>5.709</v>
+        <v>5.645</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.47</v>
+        <v>6.412</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.948</v>
+        <v>2.946</v>
       </c>
       <c r="G33" t="n">
-        <v>3.023</v>
+        <v>3.022</v>
       </c>
       <c r="H33" t="n">
-        <v>3.179</v>
+        <v>3.181</v>
       </c>
       <c r="I33" t="n">
-        <v>3.378</v>
+        <v>3.372</v>
       </c>
       <c r="J33" t="n">
-        <v>3.703</v>
+        <v>3.674</v>
       </c>
       <c r="K33" t="n">
-        <v>4.003</v>
+        <v>3.944</v>
       </c>
       <c r="L33" t="n">
-        <v>4.054</v>
+        <v>3.976</v>
       </c>
       <c r="M33" t="n">
-        <v>4.156</v>
+        <v>4.094</v>
       </c>
       <c r="N33" t="n">
-        <v>4.183</v>
+        <v>4.113</v>
       </c>
       <c r="O33" t="n">
-        <v>4.231</v>
+        <v>4.16</v>
       </c>
       <c r="P33" t="n">
-        <v>4.282</v>
+        <v>4.218</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.726</v>
+        <v>4.668</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.008</v>
+        <v>3.006</v>
       </c>
       <c r="G34" t="n">
-        <v>3.077</v>
+        <v>3.076</v>
       </c>
       <c r="H34" t="n">
-        <v>3.241</v>
+        <v>3.243</v>
       </c>
       <c r="I34" t="n">
-        <v>3.446</v>
+        <v>3.44</v>
       </c>
       <c r="J34" t="n">
-        <v>3.774</v>
+        <v>3.745</v>
       </c>
       <c r="K34" t="n">
-        <v>4.079</v>
+        <v>4.02</v>
       </c>
       <c r="L34" t="n">
-        <v>4.134</v>
+        <v>4.055</v>
       </c>
       <c r="M34" t="n">
-        <v>4.247</v>
+        <v>4.185</v>
       </c>
       <c r="N34" t="n">
-        <v>4.288</v>
+        <v>4.218</v>
       </c>
       <c r="O34" t="n">
-        <v>4.399</v>
+        <v>4.329</v>
       </c>
       <c r="P34" t="n">
-        <v>4.577</v>
+        <v>4.513</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.427</v>
+        <v>5.369</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.982</v>
+        <v>2.98</v>
       </c>
       <c r="G35" t="n">
-        <v>3.05</v>
+        <v>3.049</v>
       </c>
       <c r="H35" t="n">
-        <v>3.209</v>
+        <v>3.211</v>
       </c>
       <c r="I35" t="n">
-        <v>3.413</v>
+        <v>3.407</v>
       </c>
       <c r="J35" t="n">
-        <v>3.743</v>
+        <v>3.714</v>
       </c>
       <c r="K35" t="n">
-        <v>4.034</v>
+        <v>3.974</v>
       </c>
       <c r="L35" t="n">
-        <v>4.088</v>
+        <v>4.01</v>
       </c>
       <c r="M35" t="n">
-        <v>4.193</v>
+        <v>4.132</v>
       </c>
       <c r="N35" t="n">
-        <v>4.224</v>
+        <v>4.154</v>
       </c>
       <c r="O35" t="n">
-        <v>4.297</v>
+        <v>4.226</v>
       </c>
       <c r="P35" t="n">
-        <v>4.379</v>
+        <v>4.315</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.063</v>
+        <v>5.004</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.889</v>
+        <v>2.885</v>
       </c>
       <c r="G36" t="n">
-        <v>2.958</v>
+        <v>2.953</v>
       </c>
       <c r="H36" t="n">
-        <v>3.099</v>
+        <v>3.101</v>
       </c>
       <c r="I36" t="n">
-        <v>3.305</v>
+        <v>3.299</v>
       </c>
       <c r="J36" t="n">
-        <v>3.637</v>
+        <v>3.609</v>
       </c>
       <c r="K36" t="n">
-        <v>3.928</v>
+        <v>3.868</v>
       </c>
       <c r="L36" t="n">
-        <v>3.978</v>
+        <v>3.9</v>
       </c>
       <c r="M36" t="n">
-        <v>4.058</v>
+        <v>3.997</v>
       </c>
       <c r="N36" t="n">
-        <v>4.086</v>
+        <v>4.017</v>
       </c>
       <c r="O36" t="n">
-        <v>4.141</v>
+        <v>4.072</v>
       </c>
       <c r="P36" t="n">
-        <v>4.182</v>
+        <v>4.118</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.443</v>
+        <v>4.385</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.749</v>
+        <v>3.747</v>
       </c>
       <c r="G37" t="n">
-        <v>4.214</v>
+        <v>4.211</v>
       </c>
       <c r="H37" t="n">
-        <v>4.753</v>
+        <v>4.755</v>
       </c>
       <c r="I37" t="n">
-        <v>5.09</v>
+        <v>5.084</v>
       </c>
       <c r="J37" t="n">
-        <v>5.975</v>
+        <v>5.945</v>
       </c>
       <c r="K37" t="n">
-        <v>6.933</v>
+        <v>6.872</v>
       </c>
       <c r="L37" t="n">
-        <v>7.259</v>
+        <v>7.181</v>
       </c>
       <c r="M37" t="n">
-        <v>7.624</v>
+        <v>7.563</v>
       </c>
       <c r="N37" t="n">
-        <v>7.797</v>
+        <v>7.728</v>
       </c>
       <c r="O37" t="n">
-        <v>7.987</v>
+        <v>7.917</v>
       </c>
       <c r="P37" t="n">
-        <v>8.037000000000001</v>
+        <v>7.973</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.471</v>
+        <v>8.413</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.809</v>
+        <v>4.807</v>
       </c>
       <c r="G38" t="n">
-        <v>5.527</v>
+        <v>5.524</v>
       </c>
       <c r="H38" t="n">
-        <v>6.277</v>
+        <v>6.279</v>
       </c>
       <c r="I38" t="n">
-        <v>6.77</v>
+        <v>6.765</v>
       </c>
       <c r="J38" t="n">
-        <v>7.919</v>
+        <v>7.889</v>
       </c>
       <c r="K38" t="n">
-        <v>9.055</v>
+        <v>8.994</v>
       </c>
       <c r="L38" t="n">
-        <v>9.539</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>10.035</v>
+        <v>9.974</v>
       </c>
       <c r="N38" t="n">
-        <v>10.215</v>
+        <v>10.145</v>
       </c>
       <c r="O38" t="n">
-        <v>10.386</v>
+        <v>10.316</v>
       </c>
       <c r="P38" t="n">
-        <v>10.435</v>
+        <v>10.371</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.922</v>
+        <v>10.863</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.13</v>
+        <v>4.128</v>
       </c>
       <c r="G39" t="n">
-        <v>4.725</v>
+        <v>4.722</v>
       </c>
       <c r="H39" t="n">
-        <v>5.342</v>
+        <v>5.343</v>
       </c>
       <c r="I39" t="n">
-        <v>5.775</v>
+        <v>5.769</v>
       </c>
       <c r="J39" t="n">
-        <v>6.791</v>
+        <v>6.761</v>
       </c>
       <c r="K39" t="n">
-        <v>7.887</v>
+        <v>7.827</v>
       </c>
       <c r="L39" t="n">
-        <v>8.295999999999999</v>
+        <v>8.218</v>
       </c>
       <c r="M39" t="n">
-        <v>8.670999999999999</v>
+        <v>8.611000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.843</v>
+        <v>8.773</v>
       </c>
       <c r="O39" t="n">
-        <v>9.036</v>
+        <v>8.967000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>9.089</v>
+        <v>9.025</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.567</v>
+        <v>9.509</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.272</v>
+        <v>3.27</v>
       </c>
       <c r="G40" t="n">
-        <v>3.397</v>
+        <v>3.393</v>
       </c>
       <c r="H40" t="n">
-        <v>3.622</v>
+        <v>3.624</v>
       </c>
       <c r="I40" t="n">
-        <v>3.872</v>
+        <v>3.866</v>
       </c>
       <c r="J40" t="n">
-        <v>4.286</v>
+        <v>4.256</v>
       </c>
       <c r="K40" t="n">
-        <v>4.664</v>
+        <v>4.604</v>
       </c>
       <c r="L40" t="n">
-        <v>4.771</v>
+        <v>4.693</v>
       </c>
       <c r="M40" t="n">
-        <v>4.964</v>
+        <v>4.903</v>
       </c>
       <c r="N40" t="n">
-        <v>5.148</v>
+        <v>5.078</v>
       </c>
       <c r="O40" t="n">
-        <v>5.451</v>
+        <v>5.382</v>
       </c>
       <c r="P40" t="n">
-        <v>5.671</v>
+        <v>5.607</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.46</v>
+        <v>6.402</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.657</v>
+        <v>3.655</v>
       </c>
       <c r="G41" t="n">
-        <v>3.823</v>
+        <v>3.82</v>
       </c>
       <c r="H41" t="n">
-        <v>4.107</v>
+        <v>4.109</v>
       </c>
       <c r="I41" t="n">
-        <v>4.375</v>
+        <v>4.369</v>
       </c>
       <c r="J41" t="n">
-        <v>4.84</v>
+        <v>4.81</v>
       </c>
       <c r="K41" t="n">
-        <v>5.264</v>
+        <v>5.203</v>
       </c>
       <c r="L41" t="n">
-        <v>5.449</v>
+        <v>5.37</v>
       </c>
       <c r="M41" t="n">
-        <v>5.766</v>
+        <v>5.705</v>
       </c>
       <c r="N41" t="n">
-        <v>6.077</v>
+        <v>6.007</v>
       </c>
       <c r="O41" t="n">
-        <v>6.565</v>
+        <v>6.495</v>
       </c>
       <c r="P41" t="n">
-        <v>6.73</v>
+        <v>6.666</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.507</v>
+        <v>7.449</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.393</v>
+        <v>3.391</v>
       </c>
       <c r="G42" t="n">
-        <v>3.546</v>
+        <v>3.543</v>
       </c>
       <c r="H42" t="n">
-        <v>3.798</v>
+        <v>3.8</v>
       </c>
       <c r="I42" t="n">
-        <v>4.061</v>
+        <v>4.055</v>
       </c>
       <c r="J42" t="n">
-        <v>4.488</v>
+        <v>4.458</v>
       </c>
       <c r="K42" t="n">
-        <v>4.885</v>
+        <v>4.825</v>
       </c>
       <c r="L42" t="n">
-        <v>5.007</v>
+        <v>4.929</v>
       </c>
       <c r="M42" t="n">
-        <v>5.271</v>
+        <v>5.21</v>
       </c>
       <c r="N42" t="n">
-        <v>5.562</v>
+        <v>5.493</v>
       </c>
       <c r="O42" t="n">
-        <v>5.943</v>
+        <v>5.873</v>
       </c>
       <c r="P42" t="n">
-        <v>6.172</v>
+        <v>6.108</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.973</v>
+        <v>6.914</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.096</v>
+        <v>3.095</v>
       </c>
       <c r="G43" t="n">
-        <v>3.206</v>
+        <v>3.205</v>
       </c>
       <c r="H43" t="n">
-        <v>3.381</v>
+        <v>3.383</v>
       </c>
       <c r="I43" t="n">
-        <v>3.588</v>
+        <v>3.582</v>
       </c>
       <c r="J43" t="n">
-        <v>3.931</v>
+        <v>3.902</v>
       </c>
       <c r="K43" t="n">
-        <v>4.234</v>
+        <v>4.174</v>
       </c>
       <c r="L43" t="n">
-        <v>4.296</v>
+        <v>4.217</v>
       </c>
       <c r="M43" t="n">
-        <v>4.41</v>
+        <v>4.348</v>
       </c>
       <c r="N43" t="n">
-        <v>4.453</v>
+        <v>4.382</v>
       </c>
       <c r="O43" t="n">
-        <v>4.544</v>
+        <v>4.473</v>
       </c>
       <c r="P43" t="n">
-        <v>4.648</v>
+        <v>4.584</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.336</v>
+        <v>5.278</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.967</v>
+        <v>2.963</v>
       </c>
       <c r="G44" t="n">
-        <v>3.068</v>
+        <v>3.062</v>
       </c>
       <c r="H44" t="n">
-        <v>3.223</v>
+        <v>3.225</v>
       </c>
       <c r="I44" t="n">
-        <v>3.433</v>
+        <v>3.427</v>
       </c>
       <c r="J44" t="n">
-        <v>3.779</v>
+        <v>3.75</v>
       </c>
       <c r="K44" t="n">
-        <v>4.078</v>
+        <v>4.018</v>
       </c>
       <c r="L44" t="n">
-        <v>4.138</v>
+        <v>4.06</v>
       </c>
       <c r="M44" t="n">
-        <v>4.227</v>
+        <v>4.166</v>
       </c>
       <c r="N44" t="n">
-        <v>4.268</v>
+        <v>4.199</v>
       </c>
       <c r="O44" t="n">
-        <v>4.34</v>
+        <v>4.271</v>
       </c>
       <c r="P44" t="n">
-        <v>4.412</v>
+        <v>4.348</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.707</v>
+        <v>4.648</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-08 ~ 2026-05-08
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,10 +552,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.175</v>
+        <v>3.168</v>
       </c>
       <c r="G2" t="n">
-        <v>3.395</v>
+        <v>3.388</v>
       </c>
       <c r="H2" t="n">
         <v>3.613</v>
@@ -564,28 +564,28 @@
         <v>3.798</v>
       </c>
       <c r="J2" t="n">
-        <v>4.111</v>
+        <v>4.121</v>
       </c>
       <c r="K2" t="n">
-        <v>4.537</v>
+        <v>4.54</v>
       </c>
       <c r="L2" t="n">
-        <v>4.7</v>
+        <v>4.717</v>
       </c>
       <c r="M2" t="n">
-        <v>5.013</v>
+        <v>5.029</v>
       </c>
       <c r="N2" t="n">
-        <v>5.282</v>
+        <v>5.3</v>
       </c>
       <c r="O2" t="n">
-        <v>5.518</v>
+        <v>5.536</v>
       </c>
       <c r="P2" t="n">
-        <v>5.711</v>
+        <v>5.738</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.346</v>
+        <v>6.374</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,10 +625,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.199</v>
+        <v>4.192</v>
       </c>
       <c r="G3" t="n">
-        <v>4.6</v>
+        <v>4.593</v>
       </c>
       <c r="H3" t="n">
         <v>4.851</v>
@@ -637,28 +637,28 @@
         <v>5.03</v>
       </c>
       <c r="J3" t="n">
-        <v>5.356</v>
+        <v>5.367</v>
       </c>
       <c r="K3" t="n">
-        <v>5.853</v>
+        <v>5.857</v>
       </c>
       <c r="L3" t="n">
-        <v>6.085</v>
+        <v>6.102</v>
       </c>
       <c r="M3" t="n">
-        <v>6.43</v>
+        <v>6.446</v>
       </c>
       <c r="N3" t="n">
-        <v>6.642</v>
+        <v>6.659</v>
       </c>
       <c r="O3" t="n">
-        <v>6.828</v>
+        <v>6.846</v>
       </c>
       <c r="P3" t="n">
-        <v>6.891</v>
+        <v>6.918</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.415</v>
+        <v>7.442</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.691</v>
+        <v>3.684</v>
       </c>
       <c r="G4" t="n">
-        <v>3.981</v>
+        <v>3.974</v>
       </c>
       <c r="H4" t="n">
         <v>4.26</v>
@@ -710,28 +710,28 @@
         <v>4.473</v>
       </c>
       <c r="J4" t="n">
-        <v>4.802</v>
+        <v>4.812</v>
       </c>
       <c r="K4" t="n">
-        <v>5.292</v>
+        <v>5.295</v>
       </c>
       <c r="L4" t="n">
-        <v>5.454</v>
+        <v>5.471</v>
       </c>
       <c r="M4" t="n">
-        <v>5.788</v>
+        <v>5.804</v>
       </c>
       <c r="N4" t="n">
-        <v>5.97</v>
+        <v>5.987</v>
       </c>
       <c r="O4" t="n">
-        <v>6.179</v>
+        <v>6.197</v>
       </c>
       <c r="P4" t="n">
-        <v>6.241</v>
+        <v>6.268</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.768</v>
+        <v>6.795</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,10 +771,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.87</v>
+        <v>2.863</v>
       </c>
       <c r="G5" t="n">
-        <v>2.939</v>
+        <v>2.932</v>
       </c>
       <c r="H5" t="n">
         <v>3.115</v>
@@ -783,28 +783,28 @@
         <v>3.37</v>
       </c>
       <c r="J5" t="n">
-        <v>3.673</v>
+        <v>3.683</v>
       </c>
       <c r="K5" t="n">
-        <v>3.95</v>
+        <v>3.953</v>
       </c>
       <c r="L5" t="n">
-        <v>3.958</v>
+        <v>3.975</v>
       </c>
       <c r="M5" t="n">
-        <v>4.073</v>
+        <v>4.089</v>
       </c>
       <c r="N5" t="n">
-        <v>4.096</v>
+        <v>4.113</v>
       </c>
       <c r="O5" t="n">
-        <v>4.117</v>
+        <v>4.135</v>
       </c>
       <c r="P5" t="n">
-        <v>4.38</v>
+        <v>4.406</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.259</v>
+        <v>5.286</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,10 +844,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.909</v>
+        <v>2.902</v>
       </c>
       <c r="G6" t="n">
-        <v>2.992</v>
+        <v>2.985</v>
       </c>
       <c r="H6" t="n">
         <v>3.184</v>
@@ -856,28 +856,28 @@
         <v>3.45</v>
       </c>
       <c r="J6" t="n">
-        <v>3.761</v>
+        <v>3.771</v>
       </c>
       <c r="K6" t="n">
-        <v>4.059</v>
+        <v>4.063</v>
       </c>
       <c r="L6" t="n">
-        <v>4.072</v>
+        <v>4.09</v>
       </c>
       <c r="M6" t="n">
-        <v>4.229</v>
+        <v>4.245</v>
       </c>
       <c r="N6" t="n">
-        <v>4.264</v>
+        <v>4.281</v>
       </c>
       <c r="O6" t="n">
-        <v>4.384</v>
+        <v>4.401</v>
       </c>
       <c r="P6" t="n">
-        <v>4.812</v>
+        <v>4.839</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.655</v>
+        <v>5.682</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,10 +917,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.89</v>
+        <v>2.883</v>
       </c>
       <c r="G7" t="n">
-        <v>2.956</v>
+        <v>2.949</v>
       </c>
       <c r="H7" t="n">
         <v>3.13</v>
@@ -929,28 +929,28 @@
         <v>3.385</v>
       </c>
       <c r="J7" t="n">
-        <v>3.697</v>
+        <v>3.707</v>
       </c>
       <c r="K7" t="n">
-        <v>3.976</v>
+        <v>3.98</v>
       </c>
       <c r="L7" t="n">
-        <v>3.982</v>
+        <v>3.999</v>
       </c>
       <c r="M7" t="n">
-        <v>4.135</v>
+        <v>4.15</v>
       </c>
       <c r="N7" t="n">
-        <v>4.156</v>
+        <v>4.173</v>
       </c>
       <c r="O7" t="n">
-        <v>4.281</v>
+        <v>4.299</v>
       </c>
       <c r="P7" t="n">
-        <v>4.596</v>
+        <v>4.622</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.423</v>
+        <v>5.45</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.311</v>
+        <v>5.304</v>
       </c>
       <c r="G8" t="n">
-        <v>5.9</v>
+        <v>5.893</v>
       </c>
       <c r="H8" t="n">
-        <v>6.3</v>
+        <v>6.299</v>
       </c>
       <c r="I8" t="n">
-        <v>6.557</v>
+        <v>6.556</v>
       </c>
       <c r="J8" t="n">
-        <v>6.949</v>
+        <v>6.958</v>
       </c>
       <c r="K8" t="n">
-        <v>7.725</v>
+        <v>7.729</v>
       </c>
       <c r="L8" t="n">
-        <v>8.044</v>
+        <v>8.061</v>
       </c>
       <c r="M8" t="n">
-        <v>8.42</v>
+        <v>8.435</v>
       </c>
       <c r="N8" t="n">
-        <v>8.566000000000001</v>
+        <v>8.583</v>
       </c>
       <c r="O8" t="n">
-        <v>8.837</v>
+        <v>8.855</v>
       </c>
       <c r="P8" t="n">
-        <v>9.002000000000001</v>
+        <v>9.029</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.724</v>
+        <v>9.750999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.606</v>
+        <v>2.603</v>
       </c>
       <c r="G9" t="n">
-        <v>2.687</v>
+        <v>2.689</v>
       </c>
       <c r="H9" t="n">
         <v>2.8</v>
       </c>
       <c r="I9" t="n">
-        <v>3.008</v>
+        <v>3.01</v>
       </c>
       <c r="J9" t="n">
-        <v>3.245</v>
+        <v>3.253</v>
       </c>
       <c r="K9" t="n">
-        <v>3.432</v>
+        <v>3.449</v>
       </c>
       <c r="L9" t="n">
-        <v>3.442</v>
+        <v>3.47</v>
       </c>
       <c r="M9" t="n">
-        <v>3.535</v>
+        <v>3.56</v>
       </c>
       <c r="N9" t="n">
-        <v>3.68</v>
+        <v>3.7</v>
       </c>
       <c r="O9" t="n">
-        <v>3.717</v>
+        <v>3.735</v>
       </c>
       <c r="P9" t="n">
-        <v>3.802</v>
+        <v>3.828</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.876</v>
+        <v>3.903</v>
       </c>
       <c r="R9" t="n">
-        <v>3.883</v>
+        <v>3.905</v>
       </c>
       <c r="S9" t="n">
-        <v>3.892</v>
+        <v>3.905</v>
       </c>
       <c r="T9" t="n">
-        <v>3.817</v>
+        <v>3.835</v>
       </c>
       <c r="U9" t="n">
-        <v>3.689</v>
+        <v>3.706</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.62</v>
+        <v>2.617</v>
       </c>
       <c r="G10" t="n">
-        <v>2.72</v>
+        <v>2.721</v>
       </c>
       <c r="H10" t="n">
-        <v>2.813</v>
+        <v>2.814</v>
       </c>
       <c r="I10" t="n">
-        <v>3.021</v>
+        <v>3.022</v>
       </c>
       <c r="J10" t="n">
-        <v>3.267</v>
+        <v>3.275</v>
       </c>
       <c r="K10" t="n">
-        <v>3.465</v>
+        <v>3.482</v>
       </c>
       <c r="L10" t="n">
-        <v>3.49</v>
+        <v>3.518</v>
       </c>
       <c r="M10" t="n">
-        <v>3.632</v>
+        <v>3.656</v>
       </c>
       <c r="N10" t="n">
-        <v>3.697</v>
+        <v>3.717</v>
       </c>
       <c r="O10" t="n">
-        <v>3.925</v>
+        <v>3.943</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.435</v>
+        <v>2.432</v>
       </c>
       <c r="G11" t="n">
-        <v>2.53</v>
+        <v>2.531</v>
       </c>
       <c r="H11" t="n">
-        <v>2.638</v>
+        <v>2.639</v>
       </c>
       <c r="I11" t="n">
-        <v>2.824</v>
+        <v>2.825</v>
       </c>
       <c r="J11" t="n">
-        <v>3.065</v>
+        <v>3.073</v>
       </c>
       <c r="K11" t="n">
-        <v>3.252</v>
+        <v>3.27</v>
       </c>
       <c r="L11" t="n">
-        <v>3.287</v>
+        <v>3.315</v>
       </c>
       <c r="M11" t="n">
-        <v>3.437</v>
+        <v>3.463</v>
       </c>
       <c r="N11" t="n">
-        <v>3.505</v>
+        <v>3.525</v>
       </c>
       <c r="O11" t="n">
-        <v>3.692</v>
+        <v>3.71</v>
       </c>
       <c r="P11" t="n">
-        <v>3.753</v>
+        <v>3.779</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.077</v>
+        <v>4.105</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1288,40 +1288,40 @@
         <v>3.34</v>
       </c>
       <c r="H12" t="n">
-        <v>3.495</v>
+        <v>3.499</v>
       </c>
       <c r="I12" t="n">
-        <v>3.741</v>
+        <v>3.749</v>
       </c>
       <c r="J12" t="n">
-        <v>4.101</v>
+        <v>4.116</v>
       </c>
       <c r="K12" t="n">
-        <v>4.319</v>
+        <v>4.33</v>
       </c>
       <c r="L12" t="n">
-        <v>4.367</v>
+        <v>4.389</v>
       </c>
       <c r="M12" t="n">
-        <v>4.523</v>
+        <v>4.544</v>
       </c>
       <c r="N12" t="n">
-        <v>4.564</v>
+        <v>4.584</v>
       </c>
       <c r="O12" t="n">
-        <v>4.717</v>
+        <v>4.735</v>
       </c>
       <c r="P12" t="n">
-        <v>4.847</v>
+        <v>4.874</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.204</v>
+        <v>5.231</v>
       </c>
       <c r="R12" t="n">
-        <v>5.382</v>
+        <v>5.404</v>
       </c>
       <c r="S12" t="n">
-        <v>5.602</v>
+        <v>5.615</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1361,40 +1361,40 @@
         <v>3.03</v>
       </c>
       <c r="H13" t="n">
-        <v>3.162</v>
+        <v>3.167</v>
       </c>
       <c r="I13" t="n">
-        <v>3.389</v>
+        <v>3.397</v>
       </c>
       <c r="J13" t="n">
-        <v>3.738</v>
+        <v>3.753</v>
       </c>
       <c r="K13" t="n">
-        <v>3.952</v>
+        <v>3.964</v>
       </c>
       <c r="L13" t="n">
-        <v>4.006</v>
+        <v>4.029</v>
       </c>
       <c r="M13" t="n">
-        <v>4.151</v>
+        <v>4.171</v>
       </c>
       <c r="N13" t="n">
-        <v>4.192</v>
+        <v>4.212</v>
       </c>
       <c r="O13" t="n">
-        <v>4.346</v>
+        <v>4.364</v>
       </c>
       <c r="P13" t="n">
-        <v>4.439</v>
+        <v>4.465</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.725</v>
+        <v>4.752</v>
       </c>
       <c r="R13" t="n">
-        <v>4.931</v>
+        <v>4.953</v>
       </c>
       <c r="S13" t="n">
-        <v>5.164</v>
+        <v>5.177</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1434,40 +1434,40 @@
         <v>2.835</v>
       </c>
       <c r="H14" t="n">
-        <v>2.965</v>
+        <v>2.97</v>
       </c>
       <c r="I14" t="n">
-        <v>3.173</v>
+        <v>3.18</v>
       </c>
       <c r="J14" t="n">
-        <v>3.478</v>
+        <v>3.493</v>
       </c>
       <c r="K14" t="n">
-        <v>3.64</v>
+        <v>3.651</v>
       </c>
       <c r="L14" t="n">
-        <v>3.678</v>
+        <v>3.7</v>
       </c>
       <c r="M14" t="n">
-        <v>3.836</v>
+        <v>3.857</v>
       </c>
       <c r="N14" t="n">
-        <v>3.87</v>
+        <v>3.89</v>
       </c>
       <c r="O14" t="n">
-        <v>4.001</v>
+        <v>4.019</v>
       </c>
       <c r="P14" t="n">
-        <v>4.074</v>
+        <v>4.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.314</v>
+        <v>4.341</v>
       </c>
       <c r="R14" t="n">
-        <v>4.445</v>
+        <v>4.467</v>
       </c>
       <c r="S14" t="n">
-        <v>4.617</v>
+        <v>4.63</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1507,40 +1507,40 @@
         <v>2.81</v>
       </c>
       <c r="H15" t="n">
-        <v>2.936</v>
+        <v>2.941</v>
       </c>
       <c r="I15" t="n">
-        <v>3.124</v>
+        <v>3.132</v>
       </c>
       <c r="J15" t="n">
-        <v>3.417</v>
+        <v>3.432</v>
       </c>
       <c r="K15" t="n">
-        <v>3.592</v>
+        <v>3.604</v>
       </c>
       <c r="L15" t="n">
-        <v>3.614</v>
+        <v>3.636</v>
       </c>
       <c r="M15" t="n">
-        <v>3.748</v>
+        <v>3.769</v>
       </c>
       <c r="N15" t="n">
-        <v>3.774</v>
+        <v>3.794</v>
       </c>
       <c r="O15" t="n">
-        <v>3.943</v>
+        <v>3.961</v>
       </c>
       <c r="P15" t="n">
-        <v>3.974</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.217</v>
+        <v>4.244</v>
       </c>
       <c r="R15" t="n">
-        <v>4.342</v>
+        <v>4.364</v>
       </c>
       <c r="S15" t="n">
-        <v>4.512</v>
+        <v>4.525</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1580,40 +1580,40 @@
         <v>2.81</v>
       </c>
       <c r="H16" t="n">
-        <v>2.936</v>
+        <v>2.941</v>
       </c>
       <c r="I16" t="n">
-        <v>3.124</v>
+        <v>3.132</v>
       </c>
       <c r="J16" t="n">
-        <v>3.417</v>
+        <v>3.432</v>
       </c>
       <c r="K16" t="n">
-        <v>3.592</v>
+        <v>3.604</v>
       </c>
       <c r="L16" t="n">
-        <v>3.614</v>
+        <v>3.636</v>
       </c>
       <c r="M16" t="n">
-        <v>3.748</v>
+        <v>3.769</v>
       </c>
       <c r="N16" t="n">
-        <v>3.777</v>
+        <v>3.797</v>
       </c>
       <c r="O16" t="n">
-        <v>3.95</v>
+        <v>3.968</v>
       </c>
       <c r="P16" t="n">
-        <v>3.997</v>
+        <v>4.024</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.244</v>
+        <v>4.271</v>
       </c>
       <c r="R16" t="n">
-        <v>4.37</v>
+        <v>4.392</v>
       </c>
       <c r="S16" t="n">
-        <v>4.541</v>
+        <v>4.554</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.681</v>
+        <v>2.678</v>
       </c>
       <c r="G17" t="n">
-        <v>2.812</v>
+        <v>2.813</v>
       </c>
       <c r="H17" t="n">
-        <v>2.909</v>
+        <v>2.91</v>
       </c>
       <c r="I17" t="n">
-        <v>3.102</v>
+        <v>3.103</v>
       </c>
       <c r="J17" t="n">
-        <v>3.343</v>
+        <v>3.351</v>
       </c>
       <c r="K17" t="n">
-        <v>3.542</v>
+        <v>3.559</v>
       </c>
       <c r="L17" t="n">
-        <v>3.573</v>
+        <v>3.601</v>
       </c>
       <c r="M17" t="n">
-        <v>3.751</v>
+        <v>3.776</v>
       </c>
       <c r="N17" t="n">
-        <v>3.8</v>
+        <v>3.819</v>
       </c>
       <c r="O17" t="n">
-        <v>3.953</v>
+        <v>3.971</v>
       </c>
       <c r="P17" t="n">
-        <v>4.029</v>
+        <v>4.056</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.682</v>
+        <v>2.679</v>
       </c>
       <c r="G18" t="n">
-        <v>2.813</v>
+        <v>2.814</v>
       </c>
       <c r="H18" t="n">
-        <v>2.909</v>
+        <v>2.91</v>
       </c>
       <c r="I18" t="n">
-        <v>3.103</v>
+        <v>3.104</v>
       </c>
       <c r="J18" t="n">
-        <v>3.343</v>
+        <v>3.351</v>
       </c>
       <c r="K18" t="n">
-        <v>3.542</v>
+        <v>3.56</v>
       </c>
       <c r="L18" t="n">
-        <v>3.573</v>
+        <v>3.601</v>
       </c>
       <c r="M18" t="n">
-        <v>3.751</v>
+        <v>3.776</v>
       </c>
       <c r="N18" t="n">
-        <v>3.8</v>
+        <v>3.82</v>
       </c>
       <c r="O18" t="n">
-        <v>3.95</v>
+        <v>3.969</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1799,40 +1799,40 @@
         <v>2.826</v>
       </c>
       <c r="H19" t="n">
-        <v>2.955</v>
+        <v>2.959</v>
       </c>
       <c r="I19" t="n">
-        <v>3.16</v>
+        <v>3.167</v>
       </c>
       <c r="J19" t="n">
-        <v>3.462</v>
+        <v>3.476</v>
       </c>
       <c r="K19" t="n">
-        <v>3.636</v>
+        <v>3.648</v>
       </c>
       <c r="L19" t="n">
-        <v>3.675</v>
+        <v>3.697</v>
       </c>
       <c r="M19" t="n">
-        <v>3.826</v>
+        <v>3.847</v>
       </c>
       <c r="N19" t="n">
-        <v>3.86</v>
+        <v>3.88</v>
       </c>
       <c r="O19" t="n">
-        <v>3.985</v>
+        <v>4.003</v>
       </c>
       <c r="P19" t="n">
-        <v>4.033</v>
+        <v>4.059</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.257</v>
+        <v>4.283</v>
       </c>
       <c r="R19" t="n">
-        <v>4.39</v>
+        <v>4.412</v>
       </c>
       <c r="S19" t="n">
-        <v>4.552</v>
+        <v>4.565</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.646</v>
+        <v>2.645</v>
       </c>
       <c r="H20" t="n">
-        <v>2.703</v>
+        <v>2.704</v>
       </c>
       <c r="I20" t="n">
-        <v>2.843</v>
+        <v>2.841</v>
       </c>
       <c r="J20" t="n">
-        <v>3.24</v>
+        <v>3.259</v>
       </c>
       <c r="K20" t="n">
-        <v>3.449</v>
+        <v>3.463</v>
       </c>
       <c r="L20" t="n">
-        <v>3.483</v>
+        <v>3.505</v>
       </c>
       <c r="M20" t="n">
-        <v>3.573</v>
+        <v>3.595</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.855</v>
+        <v>2.856</v>
       </c>
       <c r="G21" t="n">
-        <v>2.931</v>
+        <v>2.932</v>
       </c>
       <c r="H21" t="n">
-        <v>3.094</v>
+        <v>3.104</v>
       </c>
       <c r="I21" t="n">
-        <v>3.274</v>
+        <v>3.281</v>
       </c>
       <c r="J21" t="n">
-        <v>3.605</v>
+        <v>3.621</v>
       </c>
       <c r="K21" t="n">
-        <v>3.868</v>
+        <v>3.879</v>
       </c>
       <c r="L21" t="n">
-        <v>3.916</v>
+        <v>3.936</v>
       </c>
       <c r="M21" t="n">
-        <v>4.056</v>
+        <v>4.076</v>
       </c>
       <c r="N21" t="n">
-        <v>4.111</v>
+        <v>4.132</v>
       </c>
       <c r="O21" t="n">
-        <v>4.203</v>
+        <v>4.221</v>
       </c>
       <c r="P21" t="n">
-        <v>4.3</v>
+        <v>4.327</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.42</v>
+        <v>4.447</v>
       </c>
       <c r="R21" t="n">
-        <v>4.445</v>
+        <v>4.465</v>
       </c>
       <c r="S21" t="n">
-        <v>4.517</v>
+        <v>4.53</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.803</v>
+        <v>2.804</v>
       </c>
       <c r="G22" t="n">
-        <v>2.878</v>
+        <v>2.879</v>
       </c>
       <c r="H22" t="n">
-        <v>3.027</v>
+        <v>3.036</v>
       </c>
       <c r="I22" t="n">
-        <v>3.191</v>
+        <v>3.198</v>
       </c>
       <c r="J22" t="n">
-        <v>3.491</v>
+        <v>3.507</v>
       </c>
       <c r="K22" t="n">
-        <v>3.749</v>
+        <v>3.76</v>
       </c>
       <c r="L22" t="n">
-        <v>3.784</v>
+        <v>3.804</v>
       </c>
       <c r="M22" t="n">
-        <v>3.925</v>
+        <v>3.945</v>
       </c>
       <c r="N22" t="n">
-        <v>3.984</v>
+        <v>4.005</v>
       </c>
       <c r="O22" t="n">
-        <v>4.07</v>
+        <v>4.088</v>
       </c>
       <c r="P22" t="n">
-        <v>4.162</v>
+        <v>4.189</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.279</v>
+        <v>4.306</v>
       </c>
       <c r="R22" t="n">
-        <v>4.293</v>
+        <v>4.314</v>
       </c>
       <c r="S22" t="n">
-        <v>4.362</v>
+        <v>4.375</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.755</v>
+        <v>2.756</v>
       </c>
       <c r="G23" t="n">
-        <v>2.832</v>
+        <v>2.834</v>
       </c>
       <c r="H23" t="n">
-        <v>2.967</v>
+        <v>2.976</v>
       </c>
       <c r="I23" t="n">
-        <v>3.146</v>
+        <v>3.153</v>
       </c>
       <c r="J23" t="n">
-        <v>3.433</v>
+        <v>3.449</v>
       </c>
       <c r="K23" t="n">
-        <v>3.655</v>
+        <v>3.666</v>
       </c>
       <c r="L23" t="n">
-        <v>3.688</v>
+        <v>3.707</v>
       </c>
       <c r="M23" t="n">
-        <v>3.822</v>
+        <v>3.842</v>
       </c>
       <c r="N23" t="n">
-        <v>3.879</v>
+        <v>3.9</v>
       </c>
       <c r="O23" t="n">
-        <v>3.947</v>
+        <v>3.965</v>
       </c>
       <c r="P23" t="n">
-        <v>4.027</v>
+        <v>4.054</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.085</v>
+        <v>4.112</v>
       </c>
       <c r="R23" t="n">
-        <v>4.077</v>
+        <v>4.098</v>
       </c>
       <c r="S23" t="n">
-        <v>4.117</v>
+        <v>4.13</v>
       </c>
       <c r="T23" t="n">
-        <v>4.032</v>
+        <v>4.05</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.69</v>
+        <v>2.691</v>
       </c>
       <c r="G24" t="n">
-        <v>2.748</v>
+        <v>2.749</v>
       </c>
       <c r="H24" t="n">
-        <v>2.868</v>
+        <v>2.877</v>
       </c>
       <c r="I24" t="n">
-        <v>3.057</v>
+        <v>3.063</v>
       </c>
       <c r="J24" t="n">
-        <v>3.332</v>
+        <v>3.349</v>
       </c>
       <c r="K24" t="n">
-        <v>3.54</v>
+        <v>3.552</v>
       </c>
       <c r="L24" t="n">
-        <v>3.566</v>
+        <v>3.588</v>
       </c>
       <c r="M24" t="n">
-        <v>3.685</v>
+        <v>3.705</v>
       </c>
       <c r="N24" t="n">
-        <v>3.756</v>
+        <v>3.777</v>
       </c>
       <c r="O24" t="n">
-        <v>3.94</v>
+        <v>3.958</v>
       </c>
       <c r="P24" t="n">
-        <v>3.966</v>
+        <v>3.992</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.01</v>
+        <v>4.037</v>
       </c>
       <c r="R24" t="n">
-        <v>3.999</v>
+        <v>4.02</v>
       </c>
       <c r="S24" t="n">
-        <v>4.032</v>
+        <v>4.045</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.748</v>
+        <v>2.749</v>
       </c>
       <c r="G25" t="n">
         <v>2.832</v>
       </c>
       <c r="H25" t="n">
-        <v>2.97</v>
+        <v>2.979</v>
       </c>
       <c r="I25" t="n">
-        <v>3.153</v>
+        <v>3.16</v>
       </c>
       <c r="J25" t="n">
-        <v>3.448</v>
+        <v>3.465</v>
       </c>
       <c r="K25" t="n">
-        <v>3.687</v>
+        <v>3.698</v>
       </c>
       <c r="L25" t="n">
-        <v>3.718</v>
+        <v>3.737</v>
       </c>
       <c r="M25" t="n">
-        <v>3.853</v>
+        <v>3.873</v>
       </c>
       <c r="N25" t="n">
-        <v>3.906</v>
+        <v>3.927</v>
       </c>
       <c r="O25" t="n">
-        <v>3.977</v>
+        <v>3.995</v>
       </c>
       <c r="P25" t="n">
-        <v>4.049</v>
+        <v>4.075</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.118</v>
+        <v>4.145</v>
       </c>
       <c r="R25" t="n">
-        <v>4.101</v>
+        <v>4.122</v>
       </c>
       <c r="S25" t="n">
-        <v>4.14</v>
+        <v>4.153</v>
       </c>
       <c r="T25" t="n">
-        <v>4.05</v>
+        <v>4.068</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2307,31 +2307,31 @@
         <v>3.036</v>
       </c>
       <c r="G26" t="n">
-        <v>3.178</v>
+        <v>3.176</v>
       </c>
       <c r="H26" t="n">
-        <v>3.431</v>
+        <v>3.432</v>
       </c>
       <c r="I26" t="n">
-        <v>3.661</v>
+        <v>3.666</v>
       </c>
       <c r="J26" t="n">
-        <v>4.094</v>
+        <v>4.111</v>
       </c>
       <c r="K26" t="n">
-        <v>4.505</v>
+        <v>4.515</v>
       </c>
       <c r="L26" t="n">
-        <v>4.596</v>
+        <v>4.621</v>
       </c>
       <c r="M26" t="n">
-        <v>4.798</v>
+        <v>4.82</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.054</v>
+        <v>5.072</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.836</v>
+        <v>2.835</v>
       </c>
       <c r="G27" t="n">
-        <v>2.917</v>
+        <v>2.915</v>
       </c>
       <c r="H27" t="n">
-        <v>3.067</v>
+        <v>3.069</v>
       </c>
       <c r="I27" t="n">
-        <v>3.271</v>
+        <v>3.279</v>
       </c>
       <c r="J27" t="n">
-        <v>3.597</v>
+        <v>3.611</v>
       </c>
       <c r="K27" t="n">
-        <v>3.819</v>
+        <v>3.828</v>
       </c>
       <c r="L27" t="n">
-        <v>3.859</v>
+        <v>3.884</v>
       </c>
       <c r="M27" t="n">
-        <v>4.005</v>
+        <v>4.026</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.144</v>
+        <v>4.161</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.939</v>
+        <v>2.938</v>
       </c>
       <c r="G28" t="n">
-        <v>3.028</v>
+        <v>3.026</v>
       </c>
       <c r="H28" t="n">
-        <v>3.192</v>
+        <v>3.195</v>
       </c>
       <c r="I28" t="n">
-        <v>3.409</v>
+        <v>3.416</v>
       </c>
       <c r="J28" t="n">
-        <v>3.77</v>
+        <v>3.785</v>
       </c>
       <c r="K28" t="n">
-        <v>4.011</v>
+        <v>4.021</v>
       </c>
       <c r="L28" t="n">
-        <v>4.063</v>
+        <v>4.088</v>
       </c>
       <c r="M28" t="n">
-        <v>4.217</v>
+        <v>4.238</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.438</v>
+        <v>4.455</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.789</v>
+        <v>2.786</v>
       </c>
       <c r="G29" t="n">
-        <v>2.871</v>
+        <v>2.869</v>
       </c>
       <c r="H29" t="n">
-        <v>3.007</v>
+        <v>3.01</v>
       </c>
       <c r="I29" t="n">
-        <v>3.204</v>
+        <v>3.211</v>
       </c>
       <c r="J29" t="n">
-        <v>3.509</v>
+        <v>3.524</v>
       </c>
       <c r="K29" t="n">
-        <v>3.715</v>
+        <v>3.724</v>
       </c>
       <c r="L29" t="n">
-        <v>3.744</v>
+        <v>3.769</v>
       </c>
       <c r="M29" t="n">
-        <v>3.867</v>
+        <v>3.888</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.013</v>
+        <v>4.031</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2599,37 +2599,37 @@
         <v>3.077</v>
       </c>
       <c r="G30" t="n">
-        <v>3.155</v>
+        <v>3.153</v>
       </c>
       <c r="H30" t="n">
-        <v>3.364</v>
+        <v>3.367</v>
       </c>
       <c r="I30" t="n">
-        <v>3.592</v>
+        <v>3.597</v>
       </c>
       <c r="J30" t="n">
-        <v>3.963</v>
+        <v>3.982</v>
       </c>
       <c r="K30" t="n">
-        <v>4.299</v>
+        <v>4.311</v>
       </c>
       <c r="L30" t="n">
-        <v>4.369</v>
+        <v>4.396</v>
       </c>
       <c r="M30" t="n">
-        <v>4.562</v>
+        <v>4.587</v>
       </c>
       <c r="N30" t="n">
-        <v>4.72</v>
+        <v>4.739</v>
       </c>
       <c r="O30" t="n">
-        <v>5.003</v>
+        <v>5.021</v>
       </c>
       <c r="P30" t="n">
-        <v>5.186</v>
+        <v>5.212</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.951</v>
+        <v>5.978</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.404</v>
+        <v>3.405</v>
       </c>
       <c r="G31" t="n">
         <v>3.517</v>
       </c>
       <c r="H31" t="n">
-        <v>3.779</v>
+        <v>3.781</v>
       </c>
       <c r="I31" t="n">
-        <v>4.02</v>
+        <v>4.026</v>
       </c>
       <c r="J31" t="n">
-        <v>4.454</v>
+        <v>4.473</v>
       </c>
       <c r="K31" t="n">
-        <v>4.831</v>
+        <v>4.843</v>
       </c>
       <c r="L31" t="n">
-        <v>4.98</v>
+        <v>5.007</v>
       </c>
       <c r="M31" t="n">
-        <v>5.291</v>
+        <v>5.317</v>
       </c>
       <c r="N31" t="n">
-        <v>5.577</v>
+        <v>5.596</v>
       </c>
       <c r="O31" t="n">
-        <v>6.038</v>
+        <v>6.055</v>
       </c>
       <c r="P31" t="n">
-        <v>6.173</v>
+        <v>6.2</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.924</v>
+        <v>6.951</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2745,37 +2745,37 @@
         <v>3.176</v>
       </c>
       <c r="G32" t="n">
-        <v>3.272</v>
+        <v>3.27</v>
       </c>
       <c r="H32" t="n">
-        <v>3.508</v>
+        <v>3.51</v>
       </c>
       <c r="I32" t="n">
-        <v>3.751</v>
+        <v>3.756</v>
       </c>
       <c r="J32" t="n">
-        <v>4.141</v>
+        <v>4.16</v>
       </c>
       <c r="K32" t="n">
-        <v>4.484</v>
+        <v>4.496</v>
       </c>
       <c r="L32" t="n">
-        <v>4.573</v>
+        <v>4.6</v>
       </c>
       <c r="M32" t="n">
-        <v>4.834</v>
+        <v>4.86</v>
       </c>
       <c r="N32" t="n">
-        <v>5.081</v>
+        <v>5.1</v>
       </c>
       <c r="O32" t="n">
-        <v>5.449</v>
+        <v>5.466</v>
       </c>
       <c r="P32" t="n">
-        <v>5.645</v>
+        <v>5.672</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.412</v>
+        <v>6.439</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2818,37 +2818,37 @@
         <v>2.946</v>
       </c>
       <c r="G33" t="n">
-        <v>3.022</v>
+        <v>3.021</v>
       </c>
       <c r="H33" t="n">
-        <v>3.181</v>
+        <v>3.183</v>
       </c>
       <c r="I33" t="n">
-        <v>3.372</v>
+        <v>3.378</v>
       </c>
       <c r="J33" t="n">
-        <v>3.674</v>
+        <v>3.691</v>
       </c>
       <c r="K33" t="n">
-        <v>3.944</v>
+        <v>3.954</v>
       </c>
       <c r="L33" t="n">
-        <v>3.976</v>
+        <v>4.002</v>
       </c>
       <c r="M33" t="n">
-        <v>4.094</v>
+        <v>4.117</v>
       </c>
       <c r="N33" t="n">
-        <v>4.113</v>
+        <v>4.132</v>
       </c>
       <c r="O33" t="n">
-        <v>4.16</v>
+        <v>4.176</v>
       </c>
       <c r="P33" t="n">
-        <v>4.218</v>
+        <v>4.245</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.668</v>
+        <v>4.695</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2891,37 +2891,37 @@
         <v>3.006</v>
       </c>
       <c r="G34" t="n">
-        <v>3.076</v>
+        <v>3.074</v>
       </c>
       <c r="H34" t="n">
-        <v>3.243</v>
+        <v>3.245</v>
       </c>
       <c r="I34" t="n">
-        <v>3.44</v>
+        <v>3.446</v>
       </c>
       <c r="J34" t="n">
-        <v>3.745</v>
+        <v>3.762</v>
       </c>
       <c r="K34" t="n">
-        <v>4.02</v>
+        <v>4.031</v>
       </c>
       <c r="L34" t="n">
-        <v>4.055</v>
+        <v>4.081</v>
       </c>
       <c r="M34" t="n">
-        <v>4.185</v>
+        <v>4.208</v>
       </c>
       <c r="N34" t="n">
-        <v>4.218</v>
+        <v>4.235</v>
       </c>
       <c r="O34" t="n">
-        <v>4.329</v>
+        <v>4.345</v>
       </c>
       <c r="P34" t="n">
-        <v>4.513</v>
+        <v>4.539</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.369</v>
+        <v>5.396</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2964,37 +2964,37 @@
         <v>2.98</v>
       </c>
       <c r="G35" t="n">
-        <v>3.049</v>
+        <v>3.048</v>
       </c>
       <c r="H35" t="n">
-        <v>3.211</v>
+        <v>3.213</v>
       </c>
       <c r="I35" t="n">
-        <v>3.407</v>
+        <v>3.413</v>
       </c>
       <c r="J35" t="n">
-        <v>3.714</v>
+        <v>3.731</v>
       </c>
       <c r="K35" t="n">
-        <v>3.974</v>
+        <v>3.984</v>
       </c>
       <c r="L35" t="n">
-        <v>4.01</v>
+        <v>4.036</v>
       </c>
       <c r="M35" t="n">
-        <v>4.132</v>
+        <v>4.154</v>
       </c>
       <c r="N35" t="n">
-        <v>4.154</v>
+        <v>4.171</v>
       </c>
       <c r="O35" t="n">
-        <v>4.226</v>
+        <v>4.242</v>
       </c>
       <c r="P35" t="n">
-        <v>4.315</v>
+        <v>4.342</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.004</v>
+        <v>5.031</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.885</v>
+        <v>2.882</v>
       </c>
       <c r="G36" t="n">
-        <v>2.953</v>
+        <v>2.952</v>
       </c>
       <c r="H36" t="n">
-        <v>3.101</v>
+        <v>3.103</v>
       </c>
       <c r="I36" t="n">
-        <v>3.299</v>
+        <v>3.304</v>
       </c>
       <c r="J36" t="n">
-        <v>3.609</v>
+        <v>3.626</v>
       </c>
       <c r="K36" t="n">
-        <v>3.868</v>
+        <v>3.878</v>
       </c>
       <c r="L36" t="n">
-        <v>3.9</v>
+        <v>3.926</v>
       </c>
       <c r="M36" t="n">
-        <v>3.997</v>
+        <v>4.02</v>
       </c>
       <c r="N36" t="n">
-        <v>4.017</v>
+        <v>4.035</v>
       </c>
       <c r="O36" t="n">
-        <v>4.072</v>
+        <v>4.088</v>
       </c>
       <c r="P36" t="n">
-        <v>4.118</v>
+        <v>4.144</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.385</v>
+        <v>4.412</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.747</v>
+        <v>3.748</v>
       </c>
       <c r="G37" t="n">
         <v>4.211</v>
       </c>
       <c r="H37" t="n">
-        <v>4.755</v>
+        <v>4.757</v>
       </c>
       <c r="I37" t="n">
-        <v>5.084</v>
+        <v>5.089</v>
       </c>
       <c r="J37" t="n">
-        <v>5.945</v>
+        <v>5.964</v>
       </c>
       <c r="K37" t="n">
-        <v>6.872</v>
+        <v>6.884</v>
       </c>
       <c r="L37" t="n">
-        <v>7.181</v>
+        <v>7.208</v>
       </c>
       <c r="M37" t="n">
-        <v>7.563</v>
+        <v>7.589</v>
       </c>
       <c r="N37" t="n">
-        <v>7.728</v>
+        <v>7.746</v>
       </c>
       <c r="O37" t="n">
-        <v>7.917</v>
+        <v>7.934</v>
       </c>
       <c r="P37" t="n">
-        <v>7.973</v>
+        <v>8</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.413</v>
+        <v>8.44</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3186,34 +3186,34 @@
         <v>5.524</v>
       </c>
       <c r="H38" t="n">
-        <v>6.279</v>
+        <v>6.281</v>
       </c>
       <c r="I38" t="n">
-        <v>6.765</v>
+        <v>6.77</v>
       </c>
       <c r="J38" t="n">
-        <v>7.889</v>
+        <v>7.907</v>
       </c>
       <c r="K38" t="n">
-        <v>8.994</v>
+        <v>9.006</v>
       </c>
       <c r="L38" t="n">
-        <v>9.460000000000001</v>
+        <v>9.487</v>
       </c>
       <c r="M38" t="n">
-        <v>9.974</v>
+        <v>9.999000000000001</v>
       </c>
       <c r="N38" t="n">
-        <v>10.145</v>
+        <v>10.164</v>
       </c>
       <c r="O38" t="n">
-        <v>10.316</v>
+        <v>10.334</v>
       </c>
       <c r="P38" t="n">
-        <v>10.371</v>
+        <v>10.397</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.863</v>
+        <v>10.89</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3259,34 +3259,34 @@
         <v>4.722</v>
       </c>
       <c r="H39" t="n">
-        <v>5.343</v>
+        <v>5.346</v>
       </c>
       <c r="I39" t="n">
-        <v>5.769</v>
+        <v>5.774</v>
       </c>
       <c r="J39" t="n">
-        <v>6.761</v>
+        <v>6.78</v>
       </c>
       <c r="K39" t="n">
-        <v>7.827</v>
+        <v>7.839</v>
       </c>
       <c r="L39" t="n">
-        <v>8.218</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.611000000000001</v>
+        <v>8.635999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.773</v>
+        <v>8.792</v>
       </c>
       <c r="O39" t="n">
-        <v>8.967000000000001</v>
+        <v>8.984</v>
       </c>
       <c r="P39" t="n">
-        <v>9.025</v>
+        <v>9.052</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.509</v>
+        <v>9.536</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3329,37 +3329,37 @@
         <v>3.27</v>
       </c>
       <c r="G40" t="n">
-        <v>3.393</v>
+        <v>3.392</v>
       </c>
       <c r="H40" t="n">
-        <v>3.624</v>
+        <v>3.627</v>
       </c>
       <c r="I40" t="n">
-        <v>3.866</v>
+        <v>3.872</v>
       </c>
       <c r="J40" t="n">
-        <v>4.256</v>
+        <v>4.275</v>
       </c>
       <c r="K40" t="n">
-        <v>4.604</v>
+        <v>4.616</v>
       </c>
       <c r="L40" t="n">
-        <v>4.693</v>
+        <v>4.72</v>
       </c>
       <c r="M40" t="n">
-        <v>4.903</v>
+        <v>4.928</v>
       </c>
       <c r="N40" t="n">
-        <v>5.078</v>
+        <v>5.096</v>
       </c>
       <c r="O40" t="n">
-        <v>5.382</v>
+        <v>5.399</v>
       </c>
       <c r="P40" t="n">
-        <v>5.607</v>
+        <v>5.634</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.402</v>
+        <v>6.429</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3402,37 +3402,37 @@
         <v>3.655</v>
       </c>
       <c r="G41" t="n">
-        <v>3.82</v>
+        <v>3.819</v>
       </c>
       <c r="H41" t="n">
-        <v>4.109</v>
+        <v>4.111</v>
       </c>
       <c r="I41" t="n">
-        <v>4.369</v>
+        <v>4.375</v>
       </c>
       <c r="J41" t="n">
-        <v>4.81</v>
+        <v>4.829</v>
       </c>
       <c r="K41" t="n">
-        <v>5.203</v>
+        <v>5.215</v>
       </c>
       <c r="L41" t="n">
-        <v>5.37</v>
+        <v>5.397</v>
       </c>
       <c r="M41" t="n">
-        <v>5.705</v>
+        <v>5.73</v>
       </c>
       <c r="N41" t="n">
-        <v>6.007</v>
+        <v>6.025</v>
       </c>
       <c r="O41" t="n">
-        <v>6.495</v>
+        <v>6.513</v>
       </c>
       <c r="P41" t="n">
-        <v>6.666</v>
+        <v>6.692</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.449</v>
+        <v>7.476</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3475,37 +3475,37 @@
         <v>3.391</v>
       </c>
       <c r="G42" t="n">
-        <v>3.543</v>
+        <v>3.541</v>
       </c>
       <c r="H42" t="n">
-        <v>3.8</v>
+        <v>3.802</v>
       </c>
       <c r="I42" t="n">
-        <v>4.055</v>
+        <v>4.061</v>
       </c>
       <c r="J42" t="n">
-        <v>4.458</v>
+        <v>4.477</v>
       </c>
       <c r="K42" t="n">
-        <v>4.825</v>
+        <v>4.837</v>
       </c>
       <c r="L42" t="n">
-        <v>4.929</v>
+        <v>4.956</v>
       </c>
       <c r="M42" t="n">
-        <v>5.21</v>
+        <v>5.235</v>
       </c>
       <c r="N42" t="n">
-        <v>5.493</v>
+        <v>5.511</v>
       </c>
       <c r="O42" t="n">
-        <v>5.873</v>
+        <v>5.891</v>
       </c>
       <c r="P42" t="n">
-        <v>6.108</v>
+        <v>6.135</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.914</v>
+        <v>6.942</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.095</v>
+        <v>3.094</v>
       </c>
       <c r="G43" t="n">
-        <v>3.205</v>
+        <v>3.203</v>
       </c>
       <c r="H43" t="n">
-        <v>3.383</v>
+        <v>3.385</v>
       </c>
       <c r="I43" t="n">
-        <v>3.582</v>
+        <v>3.588</v>
       </c>
       <c r="J43" t="n">
-        <v>3.902</v>
+        <v>3.919</v>
       </c>
       <c r="K43" t="n">
-        <v>4.174</v>
+        <v>4.185</v>
       </c>
       <c r="L43" t="n">
-        <v>4.217</v>
+        <v>4.243</v>
       </c>
       <c r="M43" t="n">
-        <v>4.348</v>
+        <v>4.37</v>
       </c>
       <c r="N43" t="n">
-        <v>4.382</v>
+        <v>4.4</v>
       </c>
       <c r="O43" t="n">
-        <v>4.473</v>
+        <v>4.488</v>
       </c>
       <c r="P43" t="n">
-        <v>4.584</v>
+        <v>4.611</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.278</v>
+        <v>5.305</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.963</v>
+        <v>2.96</v>
       </c>
       <c r="G44" t="n">
-        <v>3.062</v>
+        <v>3.061</v>
       </c>
       <c r="H44" t="n">
-        <v>3.225</v>
+        <v>3.227</v>
       </c>
       <c r="I44" t="n">
-        <v>3.427</v>
+        <v>3.433</v>
       </c>
       <c r="J44" t="n">
-        <v>3.75</v>
+        <v>3.767</v>
       </c>
       <c r="K44" t="n">
-        <v>4.018</v>
+        <v>4.029</v>
       </c>
       <c r="L44" t="n">
-        <v>4.06</v>
+        <v>4.086</v>
       </c>
       <c r="M44" t="n">
-        <v>4.166</v>
+        <v>4.188</v>
       </c>
       <c r="N44" t="n">
-        <v>4.199</v>
+        <v>4.217</v>
       </c>
       <c r="O44" t="n">
-        <v>4.271</v>
+        <v>4.287</v>
       </c>
       <c r="P44" t="n">
-        <v>4.348</v>
+        <v>4.374</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.648</v>
+        <v>4.676</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-11 ~ 2026-05-11
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.168</v>
+        <v>3.175</v>
       </c>
       <c r="G2" t="n">
-        <v>3.388</v>
+        <v>3.397</v>
       </c>
       <c r="H2" t="n">
-        <v>3.613</v>
+        <v>3.624</v>
       </c>
       <c r="I2" t="n">
-        <v>3.798</v>
+        <v>3.806</v>
       </c>
       <c r="J2" t="n">
-        <v>4.121</v>
+        <v>4.132</v>
       </c>
       <c r="K2" t="n">
-        <v>4.54</v>
+        <v>4.563</v>
       </c>
       <c r="L2" t="n">
-        <v>4.717</v>
+        <v>4.741</v>
       </c>
       <c r="M2" t="n">
-        <v>5.029</v>
+        <v>5.056</v>
       </c>
       <c r="N2" t="n">
-        <v>5.3</v>
+        <v>5.331</v>
       </c>
       <c r="O2" t="n">
-        <v>5.536</v>
+        <v>5.572</v>
       </c>
       <c r="P2" t="n">
-        <v>5.738</v>
+        <v>5.784</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.374</v>
+        <v>6.419</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.192</v>
+        <v>4.199</v>
       </c>
       <c r="G3" t="n">
-        <v>4.593</v>
+        <v>4.602</v>
       </c>
       <c r="H3" t="n">
-        <v>4.851</v>
+        <v>4.862</v>
       </c>
       <c r="I3" t="n">
-        <v>5.03</v>
+        <v>5.039</v>
       </c>
       <c r="J3" t="n">
-        <v>5.367</v>
+        <v>5.378</v>
       </c>
       <c r="K3" t="n">
-        <v>5.857</v>
+        <v>5.879</v>
       </c>
       <c r="L3" t="n">
-        <v>6.102</v>
+        <v>6.127</v>
       </c>
       <c r="M3" t="n">
-        <v>6.446</v>
+        <v>6.473</v>
       </c>
       <c r="N3" t="n">
-        <v>6.659</v>
+        <v>6.69</v>
       </c>
       <c r="O3" t="n">
-        <v>6.846</v>
+        <v>6.882</v>
       </c>
       <c r="P3" t="n">
-        <v>6.918</v>
+        <v>6.964</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.442</v>
+        <v>7.487</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.684</v>
+        <v>3.691</v>
       </c>
       <c r="G4" t="n">
-        <v>3.974</v>
+        <v>3.983</v>
       </c>
       <c r="H4" t="n">
-        <v>4.26</v>
+        <v>4.271</v>
       </c>
       <c r="I4" t="n">
-        <v>4.473</v>
+        <v>4.482</v>
       </c>
       <c r="J4" t="n">
-        <v>4.812</v>
+        <v>4.824</v>
       </c>
       <c r="K4" t="n">
-        <v>5.295</v>
+        <v>5.318</v>
       </c>
       <c r="L4" t="n">
-        <v>5.471</v>
+        <v>5.495</v>
       </c>
       <c r="M4" t="n">
-        <v>5.804</v>
+        <v>5.831</v>
       </c>
       <c r="N4" t="n">
-        <v>5.987</v>
+        <v>6.018</v>
       </c>
       <c r="O4" t="n">
-        <v>6.197</v>
+        <v>6.233</v>
       </c>
       <c r="P4" t="n">
-        <v>6.268</v>
+        <v>6.314</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.795</v>
+        <v>6.84</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.863</v>
+        <v>2.87</v>
       </c>
       <c r="G5" t="n">
-        <v>2.932</v>
+        <v>2.941</v>
       </c>
       <c r="H5" t="n">
-        <v>3.115</v>
+        <v>3.126</v>
       </c>
       <c r="I5" t="n">
-        <v>3.37</v>
+        <v>3.375</v>
       </c>
       <c r="J5" t="n">
-        <v>3.683</v>
+        <v>3.695</v>
       </c>
       <c r="K5" t="n">
-        <v>3.953</v>
+        <v>3.975</v>
       </c>
       <c r="L5" t="n">
-        <v>3.975</v>
+        <v>3.999</v>
       </c>
       <c r="M5" t="n">
-        <v>4.089</v>
+        <v>4.115</v>
       </c>
       <c r="N5" t="n">
-        <v>4.113</v>
+        <v>4.145</v>
       </c>
       <c r="O5" t="n">
-        <v>4.135</v>
+        <v>4.171</v>
       </c>
       <c r="P5" t="n">
-        <v>4.406</v>
+        <v>4.452</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.286</v>
+        <v>5.331</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.902</v>
+        <v>2.909</v>
       </c>
       <c r="G6" t="n">
-        <v>2.985</v>
+        <v>2.994</v>
       </c>
       <c r="H6" t="n">
-        <v>3.184</v>
+        <v>3.195</v>
       </c>
       <c r="I6" t="n">
-        <v>3.45</v>
+        <v>3.458</v>
       </c>
       <c r="J6" t="n">
-        <v>3.771</v>
+        <v>3.783</v>
       </c>
       <c r="K6" t="n">
-        <v>4.063</v>
+        <v>4.084</v>
       </c>
       <c r="L6" t="n">
-        <v>4.09</v>
+        <v>4.113</v>
       </c>
       <c r="M6" t="n">
-        <v>4.245</v>
+        <v>4.271</v>
       </c>
       <c r="N6" t="n">
-        <v>4.281</v>
+        <v>4.312</v>
       </c>
       <c r="O6" t="n">
-        <v>4.401</v>
+        <v>4.438</v>
       </c>
       <c r="P6" t="n">
-        <v>4.839</v>
+        <v>4.885</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.682</v>
+        <v>5.727</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.883</v>
+        <v>2.89</v>
       </c>
       <c r="G7" t="n">
-        <v>2.949</v>
+        <v>2.958</v>
       </c>
       <c r="H7" t="n">
-        <v>3.13</v>
+        <v>3.141</v>
       </c>
       <c r="I7" t="n">
-        <v>3.385</v>
+        <v>3.393</v>
       </c>
       <c r="J7" t="n">
-        <v>3.707</v>
+        <v>3.719</v>
       </c>
       <c r="K7" t="n">
-        <v>3.98</v>
+        <v>4.001</v>
       </c>
       <c r="L7" t="n">
-        <v>3.999</v>
+        <v>4.022</v>
       </c>
       <c r="M7" t="n">
-        <v>4.15</v>
+        <v>4.176</v>
       </c>
       <c r="N7" t="n">
-        <v>4.173</v>
+        <v>4.204</v>
       </c>
       <c r="O7" t="n">
-        <v>4.299</v>
+        <v>4.335</v>
       </c>
       <c r="P7" t="n">
-        <v>4.622</v>
+        <v>4.668</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.45</v>
+        <v>5.495</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.304</v>
+        <v>5.311</v>
       </c>
       <c r="G8" t="n">
-        <v>5.893</v>
+        <v>5.902</v>
       </c>
       <c r="H8" t="n">
-        <v>6.299</v>
+        <v>6.31</v>
       </c>
       <c r="I8" t="n">
-        <v>6.556</v>
+        <v>6.564</v>
       </c>
       <c r="J8" t="n">
-        <v>6.958</v>
+        <v>6.97</v>
       </c>
       <c r="K8" t="n">
-        <v>7.729</v>
+        <v>7.751</v>
       </c>
       <c r="L8" t="n">
-        <v>8.061</v>
+        <v>8.085000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.435</v>
+        <v>8.462</v>
       </c>
       <c r="N8" t="n">
-        <v>8.583</v>
+        <v>8.615</v>
       </c>
       <c r="O8" t="n">
-        <v>8.855</v>
+        <v>8.891</v>
       </c>
       <c r="P8" t="n">
-        <v>9.029</v>
+        <v>9.074999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.750999999999999</v>
+        <v>9.797000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.603</v>
+        <v>2.604</v>
       </c>
       <c r="G9" t="n">
-        <v>2.689</v>
+        <v>2.699</v>
       </c>
       <c r="H9" t="n">
-        <v>2.8</v>
+        <v>2.811</v>
       </c>
       <c r="I9" t="n">
-        <v>3.01</v>
+        <v>3.05</v>
       </c>
       <c r="J9" t="n">
-        <v>3.253</v>
+        <v>3.278</v>
       </c>
       <c r="K9" t="n">
-        <v>3.449</v>
+        <v>3.483</v>
       </c>
       <c r="L9" t="n">
-        <v>3.47</v>
+        <v>3.503</v>
       </c>
       <c r="M9" t="n">
-        <v>3.56</v>
+        <v>3.592</v>
       </c>
       <c r="N9" t="n">
-        <v>3.7</v>
+        <v>3.735</v>
       </c>
       <c r="O9" t="n">
-        <v>3.735</v>
+        <v>3.772</v>
       </c>
       <c r="P9" t="n">
-        <v>3.828</v>
+        <v>3.875</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.903</v>
+        <v>3.95</v>
       </c>
       <c r="R9" t="n">
-        <v>3.905</v>
+        <v>3.944</v>
       </c>
       <c r="S9" t="n">
-        <v>3.905</v>
+        <v>3.937</v>
       </c>
       <c r="T9" t="n">
-        <v>3.835</v>
+        <v>3.848</v>
       </c>
       <c r="U9" t="n">
-        <v>3.706</v>
+        <v>3.719</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.617</v>
+        <v>2.618</v>
       </c>
       <c r="G10" t="n">
-        <v>2.721</v>
+        <v>2.731</v>
       </c>
       <c r="H10" t="n">
-        <v>2.814</v>
+        <v>2.824</v>
       </c>
       <c r="I10" t="n">
-        <v>3.022</v>
+        <v>3.061</v>
       </c>
       <c r="J10" t="n">
-        <v>3.275</v>
+        <v>3.301</v>
       </c>
       <c r="K10" t="n">
-        <v>3.482</v>
+        <v>3.517</v>
       </c>
       <c r="L10" t="n">
-        <v>3.518</v>
+        <v>3.551</v>
       </c>
       <c r="M10" t="n">
-        <v>3.656</v>
+        <v>3.687</v>
       </c>
       <c r="N10" t="n">
-        <v>3.717</v>
+        <v>3.752</v>
       </c>
       <c r="O10" t="n">
-        <v>3.943</v>
+        <v>3.98</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.432</v>
+        <v>2.433</v>
       </c>
       <c r="G11" t="n">
-        <v>2.531</v>
+        <v>2.541</v>
       </c>
       <c r="H11" t="n">
-        <v>2.639</v>
+        <v>2.649</v>
       </c>
       <c r="I11" t="n">
-        <v>2.825</v>
+        <v>2.864</v>
       </c>
       <c r="J11" t="n">
-        <v>3.073</v>
+        <v>3.099</v>
       </c>
       <c r="K11" t="n">
-        <v>3.27</v>
+        <v>3.304</v>
       </c>
       <c r="L11" t="n">
-        <v>3.315</v>
+        <v>3.348</v>
       </c>
       <c r="M11" t="n">
-        <v>3.463</v>
+        <v>3.494</v>
       </c>
       <c r="N11" t="n">
-        <v>3.525</v>
+        <v>3.56</v>
       </c>
       <c r="O11" t="n">
-        <v>3.71</v>
+        <v>3.747</v>
       </c>
       <c r="P11" t="n">
-        <v>3.779</v>
+        <v>3.825</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.105</v>
+        <v>4.151</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.17</v>
+        <v>3.177</v>
       </c>
       <c r="G12" t="n">
-        <v>3.34</v>
+        <v>3.356</v>
       </c>
       <c r="H12" t="n">
-        <v>3.499</v>
+        <v>3.516</v>
       </c>
       <c r="I12" t="n">
-        <v>3.749</v>
+        <v>3.764</v>
       </c>
       <c r="J12" t="n">
-        <v>4.116</v>
+        <v>4.13</v>
       </c>
       <c r="K12" t="n">
-        <v>4.33</v>
+        <v>4.354</v>
       </c>
       <c r="L12" t="n">
-        <v>4.389</v>
+        <v>4.417</v>
       </c>
       <c r="M12" t="n">
-        <v>4.544</v>
+        <v>4.571</v>
       </c>
       <c r="N12" t="n">
-        <v>4.584</v>
+        <v>4.619</v>
       </c>
       <c r="O12" t="n">
-        <v>4.735</v>
+        <v>4.771</v>
       </c>
       <c r="P12" t="n">
-        <v>4.874</v>
+        <v>4.919</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.231</v>
+        <v>5.274</v>
       </c>
       <c r="R12" t="n">
-        <v>5.404</v>
+        <v>5.443</v>
       </c>
       <c r="S12" t="n">
-        <v>5.615</v>
+        <v>5.647</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.923</v>
+        <v>2.931</v>
       </c>
       <c r="G13" t="n">
-        <v>3.03</v>
+        <v>3.046</v>
       </c>
       <c r="H13" t="n">
-        <v>3.167</v>
+        <v>3.184</v>
       </c>
       <c r="I13" t="n">
-        <v>3.397</v>
+        <v>3.412</v>
       </c>
       <c r="J13" t="n">
-        <v>3.753</v>
+        <v>3.767</v>
       </c>
       <c r="K13" t="n">
-        <v>3.964</v>
+        <v>3.988</v>
       </c>
       <c r="L13" t="n">
-        <v>4.029</v>
+        <v>4.057</v>
       </c>
       <c r="M13" t="n">
-        <v>4.171</v>
+        <v>4.198</v>
       </c>
       <c r="N13" t="n">
-        <v>4.212</v>
+        <v>4.247</v>
       </c>
       <c r="O13" t="n">
-        <v>4.364</v>
+        <v>4.4</v>
       </c>
       <c r="P13" t="n">
-        <v>4.465</v>
+        <v>4.511</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.752</v>
+        <v>4.796</v>
       </c>
       <c r="R13" t="n">
-        <v>4.953</v>
+        <v>4.992</v>
       </c>
       <c r="S13" t="n">
-        <v>5.177</v>
+        <v>5.209</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.742</v>
+        <v>2.75</v>
       </c>
       <c r="G14" t="n">
-        <v>2.835</v>
+        <v>2.851</v>
       </c>
       <c r="H14" t="n">
-        <v>2.97</v>
+        <v>2.987</v>
       </c>
       <c r="I14" t="n">
-        <v>3.18</v>
+        <v>3.196</v>
       </c>
       <c r="J14" t="n">
-        <v>3.493</v>
+        <v>3.507</v>
       </c>
       <c r="K14" t="n">
-        <v>3.651</v>
+        <v>3.676</v>
       </c>
       <c r="L14" t="n">
-        <v>3.7</v>
+        <v>3.729</v>
       </c>
       <c r="M14" t="n">
-        <v>3.857</v>
+        <v>3.884</v>
       </c>
       <c r="N14" t="n">
-        <v>3.89</v>
+        <v>3.925</v>
       </c>
       <c r="O14" t="n">
-        <v>4.019</v>
+        <v>4.055</v>
       </c>
       <c r="P14" t="n">
-        <v>4.1</v>
+        <v>4.146</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.341</v>
+        <v>4.385</v>
       </c>
       <c r="R14" t="n">
-        <v>4.467</v>
+        <v>4.506</v>
       </c>
       <c r="S14" t="n">
-        <v>4.63</v>
+        <v>4.662</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.72</v>
+        <v>2.728</v>
       </c>
       <c r="G15" t="n">
-        <v>2.81</v>
+        <v>2.825</v>
       </c>
       <c r="H15" t="n">
-        <v>2.941</v>
+        <v>2.957</v>
       </c>
       <c r="I15" t="n">
-        <v>3.132</v>
+        <v>3.147</v>
       </c>
       <c r="J15" t="n">
-        <v>3.432</v>
+        <v>3.446</v>
       </c>
       <c r="K15" t="n">
-        <v>3.604</v>
+        <v>3.628</v>
       </c>
       <c r="L15" t="n">
-        <v>3.636</v>
+        <v>3.664</v>
       </c>
       <c r="M15" t="n">
-        <v>3.769</v>
+        <v>3.796</v>
       </c>
       <c r="N15" t="n">
-        <v>3.794</v>
+        <v>3.829</v>
       </c>
       <c r="O15" t="n">
-        <v>3.961</v>
+        <v>3.997</v>
       </c>
       <c r="P15" t="n">
-        <v>4</v>
+        <v>4.046</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.244</v>
+        <v>4.287</v>
       </c>
       <c r="R15" t="n">
-        <v>4.364</v>
+        <v>4.401</v>
       </c>
       <c r="S15" t="n">
-        <v>4.525</v>
+        <v>4.557</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.72</v>
+        <v>2.728</v>
       </c>
       <c r="G16" t="n">
-        <v>2.81</v>
+        <v>2.825</v>
       </c>
       <c r="H16" t="n">
-        <v>2.941</v>
+        <v>2.957</v>
       </c>
       <c r="I16" t="n">
-        <v>3.132</v>
+        <v>3.147</v>
       </c>
       <c r="J16" t="n">
-        <v>3.432</v>
+        <v>3.446</v>
       </c>
       <c r="K16" t="n">
-        <v>3.604</v>
+        <v>3.628</v>
       </c>
       <c r="L16" t="n">
-        <v>3.636</v>
+        <v>3.664</v>
       </c>
       <c r="M16" t="n">
-        <v>3.769</v>
+        <v>3.796</v>
       </c>
       <c r="N16" t="n">
-        <v>3.797</v>
+        <v>3.832</v>
       </c>
       <c r="O16" t="n">
-        <v>3.968</v>
+        <v>4.003</v>
       </c>
       <c r="P16" t="n">
-        <v>4.024</v>
+        <v>4.069</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.271</v>
+        <v>4.314</v>
       </c>
       <c r="R16" t="n">
-        <v>4.392</v>
+        <v>4.43</v>
       </c>
       <c r="S16" t="n">
-        <v>4.554</v>
+        <v>4.586</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.678</v>
+        <v>2.68</v>
       </c>
       <c r="G17" t="n">
-        <v>2.813</v>
+        <v>2.823</v>
       </c>
       <c r="H17" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="I17" t="n">
-        <v>3.103</v>
+        <v>3.142</v>
       </c>
       <c r="J17" t="n">
-        <v>3.351</v>
+        <v>3.377</v>
       </c>
       <c r="K17" t="n">
-        <v>3.559</v>
+        <v>3.593</v>
       </c>
       <c r="L17" t="n">
-        <v>3.601</v>
+        <v>3.634</v>
       </c>
       <c r="M17" t="n">
-        <v>3.776</v>
+        <v>3.808</v>
       </c>
       <c r="N17" t="n">
-        <v>3.819</v>
+        <v>3.854</v>
       </c>
       <c r="O17" t="n">
-        <v>3.971</v>
+        <v>4.008</v>
       </c>
       <c r="P17" t="n">
-        <v>4.056</v>
+        <v>4.102</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.679</v>
+        <v>2.681</v>
       </c>
       <c r="G18" t="n">
-        <v>2.814</v>
+        <v>2.824</v>
       </c>
       <c r="H18" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="I18" t="n">
-        <v>3.104</v>
+        <v>3.142</v>
       </c>
       <c r="J18" t="n">
-        <v>3.351</v>
+        <v>3.377</v>
       </c>
       <c r="K18" t="n">
-        <v>3.56</v>
+        <v>3.594</v>
       </c>
       <c r="L18" t="n">
-        <v>3.601</v>
+        <v>3.634</v>
       </c>
       <c r="M18" t="n">
-        <v>3.776</v>
+        <v>3.808</v>
       </c>
       <c r="N18" t="n">
-        <v>3.82</v>
+        <v>3.855</v>
       </c>
       <c r="O18" t="n">
-        <v>3.969</v>
+        <v>4.006</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.734</v>
+        <v>2.741</v>
       </c>
       <c r="G19" t="n">
-        <v>2.826</v>
+        <v>2.842</v>
       </c>
       <c r="H19" t="n">
-        <v>2.959</v>
+        <v>2.976</v>
       </c>
       <c r="I19" t="n">
-        <v>3.167</v>
+        <v>3.183</v>
       </c>
       <c r="J19" t="n">
-        <v>3.476</v>
+        <v>3.49</v>
       </c>
       <c r="K19" t="n">
-        <v>3.648</v>
+        <v>3.672</v>
       </c>
       <c r="L19" t="n">
-        <v>3.697</v>
+        <v>3.725</v>
       </c>
       <c r="M19" t="n">
-        <v>3.847</v>
+        <v>3.874</v>
       </c>
       <c r="N19" t="n">
-        <v>3.88</v>
+        <v>3.915</v>
       </c>
       <c r="O19" t="n">
-        <v>4.003</v>
+        <v>4.039</v>
       </c>
       <c r="P19" t="n">
-        <v>4.059</v>
+        <v>4.105</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.283</v>
+        <v>4.326</v>
       </c>
       <c r="R19" t="n">
-        <v>4.412</v>
+        <v>4.45</v>
       </c>
       <c r="S19" t="n">
-        <v>4.565</v>
+        <v>4.597</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.573</v>
+        <v>2.578</v>
       </c>
       <c r="G20" t="n">
-        <v>2.645</v>
+        <v>2.654</v>
       </c>
       <c r="H20" t="n">
-        <v>2.704</v>
+        <v>2.715</v>
       </c>
       <c r="I20" t="n">
-        <v>2.841</v>
+        <v>2.851</v>
       </c>
       <c r="J20" t="n">
-        <v>3.259</v>
+        <v>3.276</v>
       </c>
       <c r="K20" t="n">
-        <v>3.463</v>
+        <v>3.495</v>
       </c>
       <c r="L20" t="n">
-        <v>3.505</v>
+        <v>3.538</v>
       </c>
       <c r="M20" t="n">
-        <v>3.595</v>
+        <v>3.629</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.856</v>
+        <v>2.863</v>
       </c>
       <c r="G21" t="n">
-        <v>2.932</v>
+        <v>2.944</v>
       </c>
       <c r="H21" t="n">
-        <v>3.104</v>
+        <v>3.12</v>
       </c>
       <c r="I21" t="n">
-        <v>3.281</v>
+        <v>3.295</v>
       </c>
       <c r="J21" t="n">
-        <v>3.621</v>
+        <v>3.638</v>
       </c>
       <c r="K21" t="n">
-        <v>3.879</v>
+        <v>3.906</v>
       </c>
       <c r="L21" t="n">
-        <v>3.936</v>
+        <v>3.965</v>
       </c>
       <c r="M21" t="n">
-        <v>4.076</v>
+        <v>4.104</v>
       </c>
       <c r="N21" t="n">
-        <v>4.132</v>
+        <v>4.167</v>
       </c>
       <c r="O21" t="n">
-        <v>4.221</v>
+        <v>4.257</v>
       </c>
       <c r="P21" t="n">
-        <v>4.327</v>
+        <v>4.373</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.447</v>
+        <v>4.493</v>
       </c>
       <c r="R21" t="n">
-        <v>4.465</v>
+        <v>4.503</v>
       </c>
       <c r="S21" t="n">
-        <v>4.53</v>
+        <v>4.561</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.804</v>
+        <v>2.81</v>
       </c>
       <c r="G22" t="n">
-        <v>2.879</v>
+        <v>2.89</v>
       </c>
       <c r="H22" t="n">
-        <v>3.036</v>
+        <v>3.052</v>
       </c>
       <c r="I22" t="n">
-        <v>3.198</v>
+        <v>3.212</v>
       </c>
       <c r="J22" t="n">
-        <v>3.507</v>
+        <v>3.524</v>
       </c>
       <c r="K22" t="n">
-        <v>3.76</v>
+        <v>3.787</v>
       </c>
       <c r="L22" t="n">
-        <v>3.804</v>
+        <v>3.834</v>
       </c>
       <c r="M22" t="n">
-        <v>3.945</v>
+        <v>3.973</v>
       </c>
       <c r="N22" t="n">
-        <v>4.005</v>
+        <v>4.04</v>
       </c>
       <c r="O22" t="n">
-        <v>4.088</v>
+        <v>4.124</v>
       </c>
       <c r="P22" t="n">
-        <v>4.189</v>
+        <v>4.235</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.306</v>
+        <v>4.351</v>
       </c>
       <c r="R22" t="n">
-        <v>4.314</v>
+        <v>4.351</v>
       </c>
       <c r="S22" t="n">
-        <v>4.375</v>
+        <v>4.407</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.756</v>
+        <v>2.762</v>
       </c>
       <c r="G23" t="n">
-        <v>2.834</v>
+        <v>2.844</v>
       </c>
       <c r="H23" t="n">
-        <v>2.976</v>
+        <v>2.992</v>
       </c>
       <c r="I23" t="n">
-        <v>3.153</v>
+        <v>3.167</v>
       </c>
       <c r="J23" t="n">
-        <v>3.449</v>
+        <v>3.466</v>
       </c>
       <c r="K23" t="n">
-        <v>3.666</v>
+        <v>3.69</v>
       </c>
       <c r="L23" t="n">
-        <v>3.707</v>
+        <v>3.734</v>
       </c>
       <c r="M23" t="n">
-        <v>3.842</v>
+        <v>3.869</v>
       </c>
       <c r="N23" t="n">
-        <v>3.9</v>
+        <v>3.935</v>
       </c>
       <c r="O23" t="n">
-        <v>3.965</v>
+        <v>4</v>
       </c>
       <c r="P23" t="n">
-        <v>4.054</v>
+        <v>4.1</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.112</v>
+        <v>4.157</v>
       </c>
       <c r="R23" t="n">
-        <v>4.098</v>
+        <v>4.135</v>
       </c>
       <c r="S23" t="n">
-        <v>4.13</v>
+        <v>4.161</v>
       </c>
       <c r="T23" t="n">
-        <v>4.05</v>
+        <v>4.064</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.691</v>
+        <v>2.698</v>
       </c>
       <c r="G24" t="n">
-        <v>2.749</v>
+        <v>2.761</v>
       </c>
       <c r="H24" t="n">
-        <v>2.877</v>
+        <v>2.893</v>
       </c>
       <c r="I24" t="n">
-        <v>3.063</v>
+        <v>3.076</v>
       </c>
       <c r="J24" t="n">
-        <v>3.349</v>
+        <v>3.366</v>
       </c>
       <c r="K24" t="n">
-        <v>3.552</v>
+        <v>3.576</v>
       </c>
       <c r="L24" t="n">
-        <v>3.588</v>
+        <v>3.615</v>
       </c>
       <c r="M24" t="n">
-        <v>3.705</v>
+        <v>3.732</v>
       </c>
       <c r="N24" t="n">
-        <v>3.777</v>
+        <v>3.812</v>
       </c>
       <c r="O24" t="n">
-        <v>3.958</v>
+        <v>3.994</v>
       </c>
       <c r="P24" t="n">
-        <v>3.992</v>
+        <v>4.038</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.037</v>
+        <v>4.082</v>
       </c>
       <c r="R24" t="n">
-        <v>4.02</v>
+        <v>4.057</v>
       </c>
       <c r="S24" t="n">
-        <v>4.045</v>
+        <v>4.076</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.749</v>
+        <v>2.756</v>
       </c>
       <c r="G25" t="n">
-        <v>2.832</v>
+        <v>2.844</v>
       </c>
       <c r="H25" t="n">
-        <v>2.979</v>
+        <v>2.995</v>
       </c>
       <c r="I25" t="n">
-        <v>3.16</v>
+        <v>3.174</v>
       </c>
       <c r="J25" t="n">
-        <v>3.465</v>
+        <v>3.482</v>
       </c>
       <c r="K25" t="n">
-        <v>3.698</v>
+        <v>3.723</v>
       </c>
       <c r="L25" t="n">
-        <v>3.737</v>
+        <v>3.764</v>
       </c>
       <c r="M25" t="n">
-        <v>3.873</v>
+        <v>3.9</v>
       </c>
       <c r="N25" t="n">
-        <v>3.927</v>
+        <v>3.962</v>
       </c>
       <c r="O25" t="n">
-        <v>3.995</v>
+        <v>4.031</v>
       </c>
       <c r="P25" t="n">
-        <v>4.075</v>
+        <v>4.121</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.145</v>
+        <v>4.191</v>
       </c>
       <c r="R25" t="n">
-        <v>4.122</v>
+        <v>4.159</v>
       </c>
       <c r="S25" t="n">
-        <v>4.153</v>
+        <v>4.184</v>
       </c>
       <c r="T25" t="n">
-        <v>4.068</v>
+        <v>4.082</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.036</v>
+        <v>3.04</v>
       </c>
       <c r="G26" t="n">
-        <v>3.176</v>
+        <v>3.183</v>
       </c>
       <c r="H26" t="n">
-        <v>3.432</v>
+        <v>3.442</v>
       </c>
       <c r="I26" t="n">
-        <v>3.666</v>
+        <v>3.676</v>
       </c>
       <c r="J26" t="n">
-        <v>4.111</v>
+        <v>4.126</v>
       </c>
       <c r="K26" t="n">
-        <v>4.515</v>
+        <v>4.542</v>
       </c>
       <c r="L26" t="n">
-        <v>4.621</v>
+        <v>4.65</v>
       </c>
       <c r="M26" t="n">
-        <v>4.82</v>
+        <v>4.849</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.072</v>
+        <v>5.107</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.835</v>
+        <v>2.842</v>
       </c>
       <c r="G27" t="n">
-        <v>2.915</v>
+        <v>2.929</v>
       </c>
       <c r="H27" t="n">
-        <v>3.069</v>
+        <v>3.084</v>
       </c>
       <c r="I27" t="n">
-        <v>3.279</v>
+        <v>3.291</v>
       </c>
       <c r="J27" t="n">
-        <v>3.611</v>
+        <v>3.626</v>
       </c>
       <c r="K27" t="n">
-        <v>3.828</v>
+        <v>3.854</v>
       </c>
       <c r="L27" t="n">
-        <v>3.884</v>
+        <v>3.913</v>
       </c>
       <c r="M27" t="n">
-        <v>4.026</v>
+        <v>4.052</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.161</v>
+        <v>4.196</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.938</v>
+        <v>2.945</v>
       </c>
       <c r="G28" t="n">
-        <v>3.026</v>
+        <v>3.04</v>
       </c>
       <c r="H28" t="n">
-        <v>3.195</v>
+        <v>3.21</v>
       </c>
       <c r="I28" t="n">
-        <v>3.416</v>
+        <v>3.429</v>
       </c>
       <c r="J28" t="n">
-        <v>3.785</v>
+        <v>3.799</v>
       </c>
       <c r="K28" t="n">
-        <v>4.021</v>
+        <v>4.047</v>
       </c>
       <c r="L28" t="n">
-        <v>4.088</v>
+        <v>4.117</v>
       </c>
       <c r="M28" t="n">
-        <v>4.238</v>
+        <v>4.264</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.455</v>
+        <v>4.49</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.786</v>
+        <v>2.794</v>
       </c>
       <c r="G29" t="n">
-        <v>2.869</v>
+        <v>2.882</v>
       </c>
       <c r="H29" t="n">
-        <v>3.01</v>
+        <v>3.025</v>
       </c>
       <c r="I29" t="n">
-        <v>3.211</v>
+        <v>3.224</v>
       </c>
       <c r="J29" t="n">
-        <v>3.524</v>
+        <v>3.538</v>
       </c>
       <c r="K29" t="n">
-        <v>3.724</v>
+        <v>3.75</v>
       </c>
       <c r="L29" t="n">
-        <v>3.769</v>
+        <v>3.798</v>
       </c>
       <c r="M29" t="n">
-        <v>3.888</v>
+        <v>3.914</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.031</v>
+        <v>4.066</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.077</v>
+        <v>3.083</v>
       </c>
       <c r="G30" t="n">
-        <v>3.153</v>
+        <v>3.161</v>
       </c>
       <c r="H30" t="n">
-        <v>3.367</v>
+        <v>3.378</v>
       </c>
       <c r="I30" t="n">
-        <v>3.597</v>
+        <v>3.607</v>
       </c>
       <c r="J30" t="n">
-        <v>3.982</v>
+        <v>3.997</v>
       </c>
       <c r="K30" t="n">
-        <v>4.311</v>
+        <v>4.339</v>
       </c>
       <c r="L30" t="n">
-        <v>4.396</v>
+        <v>4.425</v>
       </c>
       <c r="M30" t="n">
-        <v>4.587</v>
+        <v>4.615</v>
       </c>
       <c r="N30" t="n">
-        <v>4.739</v>
+        <v>4.772</v>
       </c>
       <c r="O30" t="n">
-        <v>5.021</v>
+        <v>5.056</v>
       </c>
       <c r="P30" t="n">
-        <v>5.212</v>
+        <v>5.258</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.978</v>
+        <v>6.022</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.405</v>
+        <v>3.411</v>
       </c>
       <c r="G31" t="n">
-        <v>3.517</v>
+        <v>3.525</v>
       </c>
       <c r="H31" t="n">
-        <v>3.781</v>
+        <v>3.792</v>
       </c>
       <c r="I31" t="n">
-        <v>4.026</v>
+        <v>4.036</v>
       </c>
       <c r="J31" t="n">
-        <v>4.473</v>
+        <v>4.489</v>
       </c>
       <c r="K31" t="n">
-        <v>4.843</v>
+        <v>4.872</v>
       </c>
       <c r="L31" t="n">
-        <v>5.007</v>
+        <v>5.038</v>
       </c>
       <c r="M31" t="n">
-        <v>5.317</v>
+        <v>5.346</v>
       </c>
       <c r="N31" t="n">
-        <v>5.596</v>
+        <v>5.63</v>
       </c>
       <c r="O31" t="n">
-        <v>6.055</v>
+        <v>6.091</v>
       </c>
       <c r="P31" t="n">
-        <v>6.2</v>
+        <v>6.246</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.951</v>
+        <v>6.996</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.176</v>
+        <v>3.182</v>
       </c>
       <c r="G32" t="n">
-        <v>3.27</v>
+        <v>3.278</v>
       </c>
       <c r="H32" t="n">
-        <v>3.51</v>
+        <v>3.521</v>
       </c>
       <c r="I32" t="n">
-        <v>3.756</v>
+        <v>3.766</v>
       </c>
       <c r="J32" t="n">
-        <v>4.16</v>
+        <v>4.175</v>
       </c>
       <c r="K32" t="n">
-        <v>4.496</v>
+        <v>4.524</v>
       </c>
       <c r="L32" t="n">
-        <v>4.6</v>
+        <v>4.63</v>
       </c>
       <c r="M32" t="n">
-        <v>4.86</v>
+        <v>4.888</v>
       </c>
       <c r="N32" t="n">
-        <v>5.1</v>
+        <v>5.133</v>
       </c>
       <c r="O32" t="n">
-        <v>5.466</v>
+        <v>5.501</v>
       </c>
       <c r="P32" t="n">
-        <v>5.672</v>
+        <v>5.718</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.439</v>
+        <v>6.483</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.946</v>
+        <v>2.95</v>
       </c>
       <c r="G33" t="n">
-        <v>3.021</v>
+        <v>3.027</v>
       </c>
       <c r="H33" t="n">
-        <v>3.183</v>
+        <v>3.192</v>
       </c>
       <c r="I33" t="n">
-        <v>3.378</v>
+        <v>3.388</v>
       </c>
       <c r="J33" t="n">
-        <v>3.691</v>
+        <v>3.706</v>
       </c>
       <c r="K33" t="n">
-        <v>3.954</v>
+        <v>3.983</v>
       </c>
       <c r="L33" t="n">
-        <v>4.002</v>
+        <v>4.03</v>
       </c>
       <c r="M33" t="n">
-        <v>4.117</v>
+        <v>4.143</v>
       </c>
       <c r="N33" t="n">
-        <v>4.132</v>
+        <v>4.165</v>
       </c>
       <c r="O33" t="n">
-        <v>4.176</v>
+        <v>4.211</v>
       </c>
       <c r="P33" t="n">
-        <v>4.245</v>
+        <v>4.291</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.695</v>
+        <v>4.739</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.006</v>
+        <v>3.01</v>
       </c>
       <c r="G34" t="n">
-        <v>3.074</v>
+        <v>3.08</v>
       </c>
       <c r="H34" t="n">
-        <v>3.245</v>
+        <v>3.254</v>
       </c>
       <c r="I34" t="n">
-        <v>3.446</v>
+        <v>3.456</v>
       </c>
       <c r="J34" t="n">
-        <v>3.762</v>
+        <v>3.778</v>
       </c>
       <c r="K34" t="n">
-        <v>4.031</v>
+        <v>4.059</v>
       </c>
       <c r="L34" t="n">
-        <v>4.081</v>
+        <v>4.109</v>
       </c>
       <c r="M34" t="n">
-        <v>4.208</v>
+        <v>4.234</v>
       </c>
       <c r="N34" t="n">
-        <v>4.235</v>
+        <v>4.268</v>
       </c>
       <c r="O34" t="n">
-        <v>4.345</v>
+        <v>4.38</v>
       </c>
       <c r="P34" t="n">
-        <v>4.539</v>
+        <v>4.585</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.396</v>
+        <v>5.44</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.98</v>
+        <v>2.984</v>
       </c>
       <c r="G35" t="n">
-        <v>3.048</v>
+        <v>3.054</v>
       </c>
       <c r="H35" t="n">
-        <v>3.213</v>
+        <v>3.222</v>
       </c>
       <c r="I35" t="n">
-        <v>3.413</v>
+        <v>3.422</v>
       </c>
       <c r="J35" t="n">
-        <v>3.731</v>
+        <v>3.746</v>
       </c>
       <c r="K35" t="n">
-        <v>3.984</v>
+        <v>4.013</v>
       </c>
       <c r="L35" t="n">
-        <v>4.036</v>
+        <v>4.064</v>
       </c>
       <c r="M35" t="n">
-        <v>4.154</v>
+        <v>4.181</v>
       </c>
       <c r="N35" t="n">
-        <v>4.171</v>
+        <v>4.204</v>
       </c>
       <c r="O35" t="n">
-        <v>4.242</v>
+        <v>4.277</v>
       </c>
       <c r="P35" t="n">
-        <v>4.342</v>
+        <v>4.388</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.031</v>
+        <v>5.076</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.882</v>
+        <v>2.885</v>
       </c>
       <c r="G36" t="n">
-        <v>2.952</v>
+        <v>2.957</v>
       </c>
       <c r="H36" t="n">
-        <v>3.103</v>
+        <v>3.112</v>
       </c>
       <c r="I36" t="n">
-        <v>3.304</v>
+        <v>3.314</v>
       </c>
       <c r="J36" t="n">
-        <v>3.626</v>
+        <v>3.641</v>
       </c>
       <c r="K36" t="n">
-        <v>3.878</v>
+        <v>3.907</v>
       </c>
       <c r="L36" t="n">
-        <v>3.926</v>
+        <v>3.955</v>
       </c>
       <c r="M36" t="n">
-        <v>4.02</v>
+        <v>4.047</v>
       </c>
       <c r="N36" t="n">
-        <v>4.035</v>
+        <v>4.069</v>
       </c>
       <c r="O36" t="n">
-        <v>4.088</v>
+        <v>4.123</v>
       </c>
       <c r="P36" t="n">
-        <v>4.144</v>
+        <v>4.19</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.412</v>
+        <v>4.456</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.748</v>
+        <v>3.754</v>
       </c>
       <c r="G37" t="n">
-        <v>4.211</v>
+        <v>4.219</v>
       </c>
       <c r="H37" t="n">
-        <v>4.757</v>
+        <v>4.768</v>
       </c>
       <c r="I37" t="n">
-        <v>5.089</v>
+        <v>5.1</v>
       </c>
       <c r="J37" t="n">
-        <v>5.964</v>
+        <v>5.981</v>
       </c>
       <c r="K37" t="n">
-        <v>6.884</v>
+        <v>6.914</v>
       </c>
       <c r="L37" t="n">
-        <v>7.208</v>
+        <v>7.238</v>
       </c>
       <c r="M37" t="n">
-        <v>7.589</v>
+        <v>7.618</v>
       </c>
       <c r="N37" t="n">
-        <v>7.746</v>
+        <v>7.78</v>
       </c>
       <c r="O37" t="n">
-        <v>7.934</v>
+        <v>7.97</v>
       </c>
       <c r="P37" t="n">
-        <v>8</v>
+        <v>8.045999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.44</v>
+        <v>8.484</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.807</v>
+        <v>4.813</v>
       </c>
       <c r="G38" t="n">
-        <v>5.524</v>
+        <v>5.532</v>
       </c>
       <c r="H38" t="n">
-        <v>6.281</v>
+        <v>6.292</v>
       </c>
       <c r="I38" t="n">
-        <v>6.77</v>
+        <v>6.781</v>
       </c>
       <c r="J38" t="n">
-        <v>7.907</v>
+        <v>7.924</v>
       </c>
       <c r="K38" t="n">
-        <v>9.006</v>
+        <v>9.035</v>
       </c>
       <c r="L38" t="n">
-        <v>9.487</v>
+        <v>9.518000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>9.999000000000001</v>
+        <v>10.028</v>
       </c>
       <c r="N38" t="n">
-        <v>10.164</v>
+        <v>10.198</v>
       </c>
       <c r="O38" t="n">
-        <v>10.334</v>
+        <v>10.37</v>
       </c>
       <c r="P38" t="n">
-        <v>10.397</v>
+        <v>10.443</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.89</v>
+        <v>10.934</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.128</v>
+        <v>4.134</v>
       </c>
       <c r="G39" t="n">
-        <v>4.722</v>
+        <v>4.73</v>
       </c>
       <c r="H39" t="n">
-        <v>5.346</v>
+        <v>5.357</v>
       </c>
       <c r="I39" t="n">
-        <v>5.774</v>
+        <v>5.785</v>
       </c>
       <c r="J39" t="n">
-        <v>6.78</v>
+        <v>6.796</v>
       </c>
       <c r="K39" t="n">
-        <v>7.839</v>
+        <v>7.868</v>
       </c>
       <c r="L39" t="n">
-        <v>8.244999999999999</v>
+        <v>8.276</v>
       </c>
       <c r="M39" t="n">
-        <v>8.635999999999999</v>
+        <v>8.664999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.792</v>
+        <v>8.826000000000001</v>
       </c>
       <c r="O39" t="n">
-        <v>8.984</v>
+        <v>9.02</v>
       </c>
       <c r="P39" t="n">
-        <v>9.052</v>
+        <v>9.098000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.536</v>
+        <v>9.58</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.27</v>
+        <v>3.276</v>
       </c>
       <c r="G40" t="n">
-        <v>3.392</v>
+        <v>3.4</v>
       </c>
       <c r="H40" t="n">
-        <v>3.627</v>
+        <v>3.638</v>
       </c>
       <c r="I40" t="n">
-        <v>3.872</v>
+        <v>3.882</v>
       </c>
       <c r="J40" t="n">
-        <v>4.275</v>
+        <v>4.29</v>
       </c>
       <c r="K40" t="n">
-        <v>4.616</v>
+        <v>4.644</v>
       </c>
       <c r="L40" t="n">
-        <v>4.72</v>
+        <v>4.749</v>
       </c>
       <c r="M40" t="n">
-        <v>4.928</v>
+        <v>4.956</v>
       </c>
       <c r="N40" t="n">
-        <v>5.096</v>
+        <v>5.13</v>
       </c>
       <c r="O40" t="n">
-        <v>5.399</v>
+        <v>5.434</v>
       </c>
       <c r="P40" t="n">
-        <v>5.634</v>
+        <v>5.679</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.429</v>
+        <v>6.473</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.655</v>
+        <v>3.661</v>
       </c>
       <c r="G41" t="n">
-        <v>3.819</v>
+        <v>3.827</v>
       </c>
       <c r="H41" t="n">
-        <v>4.111</v>
+        <v>4.122</v>
       </c>
       <c r="I41" t="n">
-        <v>4.375</v>
+        <v>4.385</v>
       </c>
       <c r="J41" t="n">
-        <v>4.829</v>
+        <v>4.845</v>
       </c>
       <c r="K41" t="n">
-        <v>5.215</v>
+        <v>5.244</v>
       </c>
       <c r="L41" t="n">
-        <v>5.397</v>
+        <v>5.428</v>
       </c>
       <c r="M41" t="n">
-        <v>5.73</v>
+        <v>5.759</v>
       </c>
       <c r="N41" t="n">
-        <v>6.025</v>
+        <v>6.059</v>
       </c>
       <c r="O41" t="n">
-        <v>6.513</v>
+        <v>6.548</v>
       </c>
       <c r="P41" t="n">
-        <v>6.692</v>
+        <v>6.738</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.476</v>
+        <v>7.52</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.391</v>
+        <v>3.397</v>
       </c>
       <c r="G42" t="n">
-        <v>3.541</v>
+        <v>3.549</v>
       </c>
       <c r="H42" t="n">
-        <v>3.802</v>
+        <v>3.813</v>
       </c>
       <c r="I42" t="n">
-        <v>4.061</v>
+        <v>4.07</v>
       </c>
       <c r="J42" t="n">
-        <v>4.477</v>
+        <v>4.492</v>
       </c>
       <c r="K42" t="n">
-        <v>4.837</v>
+        <v>4.865</v>
       </c>
       <c r="L42" t="n">
-        <v>4.956</v>
+        <v>4.986</v>
       </c>
       <c r="M42" t="n">
-        <v>5.235</v>
+        <v>5.264</v>
       </c>
       <c r="N42" t="n">
-        <v>5.511</v>
+        <v>5.544</v>
       </c>
       <c r="O42" t="n">
-        <v>5.891</v>
+        <v>5.926</v>
       </c>
       <c r="P42" t="n">
-        <v>6.135</v>
+        <v>6.181</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.942</v>
+        <v>6.986</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.094</v>
+        <v>3.098</v>
       </c>
       <c r="G43" t="n">
-        <v>3.203</v>
+        <v>3.209</v>
       </c>
       <c r="H43" t="n">
-        <v>3.385</v>
+        <v>3.393</v>
       </c>
       <c r="I43" t="n">
-        <v>3.588</v>
+        <v>3.597</v>
       </c>
       <c r="J43" t="n">
-        <v>3.919</v>
+        <v>3.934</v>
       </c>
       <c r="K43" t="n">
-        <v>4.185</v>
+        <v>4.213</v>
       </c>
       <c r="L43" t="n">
-        <v>4.243</v>
+        <v>4.271</v>
       </c>
       <c r="M43" t="n">
-        <v>4.37</v>
+        <v>4.397</v>
       </c>
       <c r="N43" t="n">
-        <v>4.4</v>
+        <v>4.433</v>
       </c>
       <c r="O43" t="n">
-        <v>4.488</v>
+        <v>4.523</v>
       </c>
       <c r="P43" t="n">
-        <v>4.611</v>
+        <v>4.657</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.305</v>
+        <v>5.349</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46150</v>
+        <v>46153</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.96</v>
+        <v>2.963</v>
       </c>
       <c r="G44" t="n">
-        <v>3.061</v>
+        <v>3.066</v>
       </c>
       <c r="H44" t="n">
-        <v>3.227</v>
+        <v>3.236</v>
       </c>
       <c r="I44" t="n">
-        <v>3.433</v>
+        <v>3.442</v>
       </c>
       <c r="J44" t="n">
-        <v>3.767</v>
+        <v>3.783</v>
       </c>
       <c r="K44" t="n">
-        <v>4.029</v>
+        <v>4.057</v>
       </c>
       <c r="L44" t="n">
-        <v>4.086</v>
+        <v>4.116</v>
       </c>
       <c r="M44" t="n">
-        <v>4.188</v>
+        <v>4.216</v>
       </c>
       <c r="N44" t="n">
-        <v>4.217</v>
+        <v>4.251</v>
       </c>
       <c r="O44" t="n">
-        <v>4.287</v>
+        <v>4.322</v>
       </c>
       <c r="P44" t="n">
-        <v>4.374</v>
+        <v>4.42</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.676</v>
+        <v>4.72</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-12 ~ 2026-05-12
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.175</v>
+        <v>3.182</v>
       </c>
       <c r="G2" t="n">
-        <v>3.397</v>
+        <v>3.408</v>
       </c>
       <c r="H2" t="n">
-        <v>3.624</v>
+        <v>3.647</v>
       </c>
       <c r="I2" t="n">
-        <v>3.806</v>
+        <v>3.833</v>
       </c>
       <c r="J2" t="n">
-        <v>4.132</v>
+        <v>4.165</v>
       </c>
       <c r="K2" t="n">
-        <v>4.563</v>
+        <v>4.627</v>
       </c>
       <c r="L2" t="n">
-        <v>4.741</v>
+        <v>4.798</v>
       </c>
       <c r="M2" t="n">
-        <v>5.056</v>
+        <v>5.13</v>
       </c>
       <c r="N2" t="n">
-        <v>5.331</v>
+        <v>5.419</v>
       </c>
       <c r="O2" t="n">
-        <v>5.572</v>
+        <v>5.667</v>
       </c>
       <c r="P2" t="n">
-        <v>5.784</v>
+        <v>5.887</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.419</v>
+        <v>6.527</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.199</v>
+        <v>4.206</v>
       </c>
       <c r="G3" t="n">
-        <v>4.602</v>
+        <v>4.613</v>
       </c>
       <c r="H3" t="n">
-        <v>4.862</v>
+        <v>4.885</v>
       </c>
       <c r="I3" t="n">
-        <v>5.039</v>
+        <v>5.066</v>
       </c>
       <c r="J3" t="n">
-        <v>5.378</v>
+        <v>5.411</v>
       </c>
       <c r="K3" t="n">
-        <v>5.879</v>
+        <v>5.943</v>
       </c>
       <c r="L3" t="n">
-        <v>6.127</v>
+        <v>6.183</v>
       </c>
       <c r="M3" t="n">
-        <v>6.473</v>
+        <v>6.547</v>
       </c>
       <c r="N3" t="n">
-        <v>6.69</v>
+        <v>6.778</v>
       </c>
       <c r="O3" t="n">
-        <v>6.882</v>
+        <v>6.977</v>
       </c>
       <c r="P3" t="n">
-        <v>6.964</v>
+        <v>7.067</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.487</v>
+        <v>7.596</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.691</v>
+        <v>3.698</v>
       </c>
       <c r="G4" t="n">
-        <v>3.983</v>
+        <v>3.994</v>
       </c>
       <c r="H4" t="n">
-        <v>4.271</v>
+        <v>4.294</v>
       </c>
       <c r="I4" t="n">
-        <v>4.482</v>
+        <v>4.509</v>
       </c>
       <c r="J4" t="n">
-        <v>4.824</v>
+        <v>4.857</v>
       </c>
       <c r="K4" t="n">
-        <v>5.318</v>
+        <v>5.382</v>
       </c>
       <c r="L4" t="n">
-        <v>5.495</v>
+        <v>5.552</v>
       </c>
       <c r="M4" t="n">
-        <v>5.831</v>
+        <v>5.905</v>
       </c>
       <c r="N4" t="n">
-        <v>6.018</v>
+        <v>6.106</v>
       </c>
       <c r="O4" t="n">
-        <v>6.233</v>
+        <v>6.328</v>
       </c>
       <c r="P4" t="n">
-        <v>6.314</v>
+        <v>6.417</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.84</v>
+        <v>6.949</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.87</v>
+        <v>2.877</v>
       </c>
       <c r="G5" t="n">
-        <v>2.941</v>
+        <v>2.952</v>
       </c>
       <c r="H5" t="n">
-        <v>3.126</v>
+        <v>3.151</v>
       </c>
       <c r="I5" t="n">
-        <v>3.375</v>
+        <v>3.402</v>
       </c>
       <c r="J5" t="n">
-        <v>3.695</v>
+        <v>3.728</v>
       </c>
       <c r="K5" t="n">
-        <v>3.975</v>
+        <v>4.039</v>
       </c>
       <c r="L5" t="n">
-        <v>3.999</v>
+        <v>4.055</v>
       </c>
       <c r="M5" t="n">
-        <v>4.115</v>
+        <v>4.189</v>
       </c>
       <c r="N5" t="n">
-        <v>4.145</v>
+        <v>4.233</v>
       </c>
       <c r="O5" t="n">
-        <v>4.171</v>
+        <v>4.266</v>
       </c>
       <c r="P5" t="n">
-        <v>4.452</v>
+        <v>4.555</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.331</v>
+        <v>5.439</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.909</v>
+        <v>2.916</v>
       </c>
       <c r="G6" t="n">
-        <v>2.994</v>
+        <v>3.005</v>
       </c>
       <c r="H6" t="n">
-        <v>3.195</v>
+        <v>3.22</v>
       </c>
       <c r="I6" t="n">
-        <v>3.458</v>
+        <v>3.485</v>
       </c>
       <c r="J6" t="n">
-        <v>3.783</v>
+        <v>3.816</v>
       </c>
       <c r="K6" t="n">
-        <v>4.084</v>
+        <v>4.148</v>
       </c>
       <c r="L6" t="n">
-        <v>4.113</v>
+        <v>4.169</v>
       </c>
       <c r="M6" t="n">
-        <v>4.271</v>
+        <v>4.345</v>
       </c>
       <c r="N6" t="n">
-        <v>4.312</v>
+        <v>4.4</v>
       </c>
       <c r="O6" t="n">
-        <v>4.438</v>
+        <v>4.532</v>
       </c>
       <c r="P6" t="n">
-        <v>4.885</v>
+        <v>4.988</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.727</v>
+        <v>5.836</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.89</v>
+        <v>2.897</v>
       </c>
       <c r="G7" t="n">
-        <v>2.958</v>
+        <v>2.969</v>
       </c>
       <c r="H7" t="n">
-        <v>3.141</v>
+        <v>3.166</v>
       </c>
       <c r="I7" t="n">
-        <v>3.393</v>
+        <v>3.42</v>
       </c>
       <c r="J7" t="n">
-        <v>3.719</v>
+        <v>3.752</v>
       </c>
       <c r="K7" t="n">
-        <v>4.001</v>
+        <v>4.065</v>
       </c>
       <c r="L7" t="n">
-        <v>4.022</v>
+        <v>4.079</v>
       </c>
       <c r="M7" t="n">
-        <v>4.176</v>
+        <v>4.25</v>
       </c>
       <c r="N7" t="n">
-        <v>4.204</v>
+        <v>4.292</v>
       </c>
       <c r="O7" t="n">
-        <v>4.335</v>
+        <v>4.43</v>
       </c>
       <c r="P7" t="n">
-        <v>4.668</v>
+        <v>4.771</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.495</v>
+        <v>5.603</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.311</v>
+        <v>5.318</v>
       </c>
       <c r="G8" t="n">
-        <v>5.902</v>
+        <v>5.913</v>
       </c>
       <c r="H8" t="n">
-        <v>6.31</v>
+        <v>6.333</v>
       </c>
       <c r="I8" t="n">
-        <v>6.564</v>
+        <v>6.591</v>
       </c>
       <c r="J8" t="n">
-        <v>6.97</v>
+        <v>7.003</v>
       </c>
       <c r="K8" t="n">
-        <v>7.751</v>
+        <v>7.815</v>
       </c>
       <c r="L8" t="n">
-        <v>8.085000000000001</v>
+        <v>8.141</v>
       </c>
       <c r="M8" t="n">
-        <v>8.462</v>
+        <v>8.536</v>
       </c>
       <c r="N8" t="n">
-        <v>8.615</v>
+        <v>8.702</v>
       </c>
       <c r="O8" t="n">
-        <v>8.891</v>
+        <v>8.986000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.074999999999999</v>
+        <v>9.178000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.797000000000001</v>
+        <v>9.904999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.604</v>
+        <v>2.61</v>
       </c>
       <c r="G9" t="n">
-        <v>2.699</v>
+        <v>2.706</v>
       </c>
       <c r="H9" t="n">
-        <v>2.811</v>
+        <v>2.843</v>
       </c>
       <c r="I9" t="n">
-        <v>3.05</v>
+        <v>3.095</v>
       </c>
       <c r="J9" t="n">
-        <v>3.278</v>
+        <v>3.318</v>
       </c>
       <c r="K9" t="n">
-        <v>3.483</v>
+        <v>3.55</v>
       </c>
       <c r="L9" t="n">
-        <v>3.503</v>
+        <v>3.569</v>
       </c>
       <c r="M9" t="n">
-        <v>3.592</v>
+        <v>3.68</v>
       </c>
       <c r="N9" t="n">
-        <v>3.735</v>
+        <v>3.833</v>
       </c>
       <c r="O9" t="n">
-        <v>3.772</v>
+        <v>3.876</v>
       </c>
       <c r="P9" t="n">
-        <v>3.875</v>
+        <v>3.985</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.95</v>
+        <v>4.065</v>
       </c>
       <c r="R9" t="n">
-        <v>3.944</v>
+        <v>4.07</v>
       </c>
       <c r="S9" t="n">
-        <v>3.937</v>
+        <v>4.07</v>
       </c>
       <c r="T9" t="n">
-        <v>3.848</v>
+        <v>3.975</v>
       </c>
       <c r="U9" t="n">
-        <v>3.719</v>
+        <v>3.845</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.618</v>
+        <v>2.625</v>
       </c>
       <c r="G10" t="n">
-        <v>2.731</v>
+        <v>2.738</v>
       </c>
       <c r="H10" t="n">
-        <v>2.824</v>
+        <v>2.856</v>
       </c>
       <c r="I10" t="n">
-        <v>3.061</v>
+        <v>3.103</v>
       </c>
       <c r="J10" t="n">
-        <v>3.301</v>
+        <v>3.34</v>
       </c>
       <c r="K10" t="n">
-        <v>3.517</v>
+        <v>3.583</v>
       </c>
       <c r="L10" t="n">
-        <v>3.551</v>
+        <v>3.618</v>
       </c>
       <c r="M10" t="n">
-        <v>3.687</v>
+        <v>3.775</v>
       </c>
       <c r="N10" t="n">
-        <v>3.752</v>
+        <v>3.851</v>
       </c>
       <c r="O10" t="n">
-        <v>3.98</v>
+        <v>4.069</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.433</v>
+        <v>2.44</v>
       </c>
       <c r="G11" t="n">
-        <v>2.541</v>
+        <v>2.547</v>
       </c>
       <c r="H11" t="n">
-        <v>2.649</v>
+        <v>2.682</v>
       </c>
       <c r="I11" t="n">
-        <v>2.864</v>
+        <v>2.906</v>
       </c>
       <c r="J11" t="n">
-        <v>3.099</v>
+        <v>3.138</v>
       </c>
       <c r="K11" t="n">
-        <v>3.304</v>
+        <v>3.371</v>
       </c>
       <c r="L11" t="n">
-        <v>3.348</v>
+        <v>3.415</v>
       </c>
       <c r="M11" t="n">
-        <v>3.494</v>
+        <v>3.582</v>
       </c>
       <c r="N11" t="n">
-        <v>3.56</v>
+        <v>3.659</v>
       </c>
       <c r="O11" t="n">
-        <v>3.747</v>
+        <v>3.835</v>
       </c>
       <c r="P11" t="n">
-        <v>3.825</v>
+        <v>3.935</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.151</v>
+        <v>4.266</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.177</v>
+        <v>3.192</v>
       </c>
       <c r="G12" t="n">
-        <v>3.356</v>
+        <v>3.371</v>
       </c>
       <c r="H12" t="n">
-        <v>3.516</v>
+        <v>3.544</v>
       </c>
       <c r="I12" t="n">
-        <v>3.764</v>
+        <v>3.793</v>
       </c>
       <c r="J12" t="n">
-        <v>4.13</v>
+        <v>4.165</v>
       </c>
       <c r="K12" t="n">
-        <v>4.354</v>
+        <v>4.415</v>
       </c>
       <c r="L12" t="n">
-        <v>4.417</v>
+        <v>4.476</v>
       </c>
       <c r="M12" t="n">
-        <v>4.571</v>
+        <v>4.647</v>
       </c>
       <c r="N12" t="n">
-        <v>4.619</v>
+        <v>4.709</v>
       </c>
       <c r="O12" t="n">
-        <v>4.771</v>
+        <v>4.867</v>
       </c>
       <c r="P12" t="n">
-        <v>4.919</v>
+        <v>5.023</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.274</v>
+        <v>5.383</v>
       </c>
       <c r="R12" t="n">
-        <v>5.443</v>
+        <v>5.563</v>
       </c>
       <c r="S12" t="n">
-        <v>5.647</v>
+        <v>5.775</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.931</v>
+        <v>2.946</v>
       </c>
       <c r="G13" t="n">
-        <v>3.046</v>
+        <v>3.061</v>
       </c>
       <c r="H13" t="n">
-        <v>3.184</v>
+        <v>3.211</v>
       </c>
       <c r="I13" t="n">
-        <v>3.412</v>
+        <v>3.441</v>
       </c>
       <c r="J13" t="n">
-        <v>3.767</v>
+        <v>3.802</v>
       </c>
       <c r="K13" t="n">
-        <v>3.988</v>
+        <v>4.049</v>
       </c>
       <c r="L13" t="n">
-        <v>4.057</v>
+        <v>4.115</v>
       </c>
       <c r="M13" t="n">
-        <v>4.198</v>
+        <v>4.274</v>
       </c>
       <c r="N13" t="n">
-        <v>4.247</v>
+        <v>4.337</v>
       </c>
       <c r="O13" t="n">
-        <v>4.4</v>
+        <v>4.495</v>
       </c>
       <c r="P13" t="n">
-        <v>4.511</v>
+        <v>4.615</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.796</v>
+        <v>4.904</v>
       </c>
       <c r="R13" t="n">
-        <v>4.992</v>
+        <v>5.113</v>
       </c>
       <c r="S13" t="n">
-        <v>5.209</v>
+        <v>5.337</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.75</v>
+        <v>2.765</v>
       </c>
       <c r="G14" t="n">
-        <v>2.851</v>
+        <v>2.866</v>
       </c>
       <c r="H14" t="n">
-        <v>2.987</v>
+        <v>3.015</v>
       </c>
       <c r="I14" t="n">
-        <v>3.196</v>
+        <v>3.224</v>
       </c>
       <c r="J14" t="n">
-        <v>3.507</v>
+        <v>3.542</v>
       </c>
       <c r="K14" t="n">
-        <v>3.676</v>
+        <v>3.737</v>
       </c>
       <c r="L14" t="n">
-        <v>3.729</v>
+        <v>3.787</v>
       </c>
       <c r="M14" t="n">
-        <v>3.884</v>
+        <v>3.96</v>
       </c>
       <c r="N14" t="n">
-        <v>3.925</v>
+        <v>4.015</v>
       </c>
       <c r="O14" t="n">
-        <v>4.055</v>
+        <v>4.151</v>
       </c>
       <c r="P14" t="n">
-        <v>4.146</v>
+        <v>4.25</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.385</v>
+        <v>4.494</v>
       </c>
       <c r="R14" t="n">
-        <v>4.506</v>
+        <v>4.627</v>
       </c>
       <c r="S14" t="n">
-        <v>4.662</v>
+        <v>4.79</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.728</v>
+        <v>2.743</v>
       </c>
       <c r="G15" t="n">
-        <v>2.825</v>
+        <v>2.841</v>
       </c>
       <c r="H15" t="n">
-        <v>2.957</v>
+        <v>2.985</v>
       </c>
       <c r="I15" t="n">
-        <v>3.147</v>
+        <v>3.175</v>
       </c>
       <c r="J15" t="n">
-        <v>3.446</v>
+        <v>3.481</v>
       </c>
       <c r="K15" t="n">
-        <v>3.628</v>
+        <v>3.689</v>
       </c>
       <c r="L15" t="n">
-        <v>3.664</v>
+        <v>3.723</v>
       </c>
       <c r="M15" t="n">
-        <v>3.796</v>
+        <v>3.872</v>
       </c>
       <c r="N15" t="n">
-        <v>3.829</v>
+        <v>3.919</v>
       </c>
       <c r="O15" t="n">
-        <v>3.997</v>
+        <v>4.093</v>
       </c>
       <c r="P15" t="n">
-        <v>4.046</v>
+        <v>4.15</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.287</v>
+        <v>4.396</v>
       </c>
       <c r="R15" t="n">
-        <v>4.401</v>
+        <v>4.522</v>
       </c>
       <c r="S15" t="n">
-        <v>4.557</v>
+        <v>4.685</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.728</v>
+        <v>2.743</v>
       </c>
       <c r="G16" t="n">
-        <v>2.825</v>
+        <v>2.841</v>
       </c>
       <c r="H16" t="n">
-        <v>2.957</v>
+        <v>2.985</v>
       </c>
       <c r="I16" t="n">
-        <v>3.147</v>
+        <v>3.175</v>
       </c>
       <c r="J16" t="n">
-        <v>3.446</v>
+        <v>3.481</v>
       </c>
       <c r="K16" t="n">
-        <v>3.628</v>
+        <v>3.689</v>
       </c>
       <c r="L16" t="n">
-        <v>3.664</v>
+        <v>3.723</v>
       </c>
       <c r="M16" t="n">
-        <v>3.796</v>
+        <v>3.872</v>
       </c>
       <c r="N16" t="n">
-        <v>3.832</v>
+        <v>3.922</v>
       </c>
       <c r="O16" t="n">
-        <v>4.003</v>
+        <v>4.099</v>
       </c>
       <c r="P16" t="n">
-        <v>4.069</v>
+        <v>4.173</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.314</v>
+        <v>4.424</v>
       </c>
       <c r="R16" t="n">
-        <v>4.43</v>
+        <v>4.55</v>
       </c>
       <c r="S16" t="n">
-        <v>4.586</v>
+        <v>4.714</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.68</v>
+        <v>2.687</v>
       </c>
       <c r="G17" t="n">
-        <v>2.823</v>
+        <v>2.83</v>
       </c>
       <c r="H17" t="n">
-        <v>2.92</v>
+        <v>2.952</v>
       </c>
       <c r="I17" t="n">
-        <v>3.142</v>
+        <v>3.184</v>
       </c>
       <c r="J17" t="n">
-        <v>3.377</v>
+        <v>3.415</v>
       </c>
       <c r="K17" t="n">
-        <v>3.593</v>
+        <v>3.66</v>
       </c>
       <c r="L17" t="n">
-        <v>3.634</v>
+        <v>3.7</v>
       </c>
       <c r="M17" t="n">
-        <v>3.808</v>
+        <v>3.895</v>
       </c>
       <c r="N17" t="n">
-        <v>3.854</v>
+        <v>3.952</v>
       </c>
       <c r="O17" t="n">
-        <v>4.008</v>
+        <v>4.096</v>
       </c>
       <c r="P17" t="n">
-        <v>4.102</v>
+        <v>4.212</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.681</v>
+        <v>2.687</v>
       </c>
       <c r="G18" t="n">
-        <v>2.824</v>
+        <v>2.831</v>
       </c>
       <c r="H18" t="n">
-        <v>2.92</v>
+        <v>2.953</v>
       </c>
       <c r="I18" t="n">
-        <v>3.142</v>
+        <v>3.185</v>
       </c>
       <c r="J18" t="n">
-        <v>3.377</v>
+        <v>3.415</v>
       </c>
       <c r="K18" t="n">
-        <v>3.594</v>
+        <v>3.661</v>
       </c>
       <c r="L18" t="n">
-        <v>3.634</v>
+        <v>3.7</v>
       </c>
       <c r="M18" t="n">
-        <v>3.808</v>
+        <v>3.895</v>
       </c>
       <c r="N18" t="n">
-        <v>3.855</v>
+        <v>3.953</v>
       </c>
       <c r="O18" t="n">
-        <v>4.006</v>
+        <v>4.094</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.741</v>
+        <v>2.756</v>
       </c>
       <c r="G19" t="n">
-        <v>2.842</v>
+        <v>2.857</v>
       </c>
       <c r="H19" t="n">
-        <v>2.976</v>
+        <v>3.004</v>
       </c>
       <c r="I19" t="n">
-        <v>3.183</v>
+        <v>3.211</v>
       </c>
       <c r="J19" t="n">
-        <v>3.49</v>
+        <v>3.525</v>
       </c>
       <c r="K19" t="n">
-        <v>3.672</v>
+        <v>3.733</v>
       </c>
       <c r="L19" t="n">
-        <v>3.725</v>
+        <v>3.783</v>
       </c>
       <c r="M19" t="n">
-        <v>3.874</v>
+        <v>3.95</v>
       </c>
       <c r="N19" t="n">
-        <v>3.915</v>
+        <v>4.005</v>
       </c>
       <c r="O19" t="n">
-        <v>4.039</v>
+        <v>4.135</v>
       </c>
       <c r="P19" t="n">
-        <v>4.105</v>
+        <v>4.209</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.326</v>
+        <v>4.435</v>
       </c>
       <c r="R19" t="n">
-        <v>4.45</v>
+        <v>4.571</v>
       </c>
       <c r="S19" t="n">
-        <v>4.597</v>
+        <v>4.725</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.578</v>
+        <v>2.589</v>
       </c>
       <c r="G20" t="n">
-        <v>2.654</v>
+        <v>2.669</v>
       </c>
       <c r="H20" t="n">
-        <v>2.715</v>
+        <v>2.734</v>
       </c>
       <c r="I20" t="n">
-        <v>2.851</v>
+        <v>2.87</v>
       </c>
       <c r="J20" t="n">
-        <v>3.276</v>
+        <v>3.315</v>
       </c>
       <c r="K20" t="n">
-        <v>3.495</v>
+        <v>3.569</v>
       </c>
       <c r="L20" t="n">
-        <v>3.538</v>
+        <v>3.614</v>
       </c>
       <c r="M20" t="n">
-        <v>3.629</v>
+        <v>3.72</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.863</v>
+        <v>2.879</v>
       </c>
       <c r="G21" t="n">
-        <v>2.944</v>
+        <v>2.962</v>
       </c>
       <c r="H21" t="n">
-        <v>3.12</v>
+        <v>3.148</v>
       </c>
       <c r="I21" t="n">
-        <v>3.295</v>
+        <v>3.323</v>
       </c>
       <c r="J21" t="n">
-        <v>3.638</v>
+        <v>3.673</v>
       </c>
       <c r="K21" t="n">
-        <v>3.906</v>
+        <v>3.968</v>
       </c>
       <c r="L21" t="n">
-        <v>3.965</v>
+        <v>4.026</v>
       </c>
       <c r="M21" t="n">
-        <v>4.104</v>
+        <v>4.179</v>
       </c>
       <c r="N21" t="n">
-        <v>4.167</v>
+        <v>4.253</v>
       </c>
       <c r="O21" t="n">
-        <v>4.257</v>
+        <v>4.35</v>
       </c>
       <c r="P21" t="n">
-        <v>4.373</v>
+        <v>4.475</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.493</v>
+        <v>4.601</v>
       </c>
       <c r="R21" t="n">
-        <v>4.503</v>
+        <v>4.622</v>
       </c>
       <c r="S21" t="n">
-        <v>4.561</v>
+        <v>4.688</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.81</v>
+        <v>2.826</v>
       </c>
       <c r="G22" t="n">
-        <v>2.89</v>
+        <v>2.908</v>
       </c>
       <c r="H22" t="n">
-        <v>3.052</v>
+        <v>3.08</v>
       </c>
       <c r="I22" t="n">
-        <v>3.212</v>
+        <v>3.242</v>
       </c>
       <c r="J22" t="n">
-        <v>3.524</v>
+        <v>3.559</v>
       </c>
       <c r="K22" t="n">
-        <v>3.787</v>
+        <v>3.85</v>
       </c>
       <c r="L22" t="n">
-        <v>3.834</v>
+        <v>3.893</v>
       </c>
       <c r="M22" t="n">
-        <v>3.973</v>
+        <v>4.048</v>
       </c>
       <c r="N22" t="n">
-        <v>4.04</v>
+        <v>4.125</v>
       </c>
       <c r="O22" t="n">
-        <v>4.124</v>
+        <v>4.217</v>
       </c>
       <c r="P22" t="n">
-        <v>4.235</v>
+        <v>4.337</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.351</v>
+        <v>4.459</v>
       </c>
       <c r="R22" t="n">
-        <v>4.351</v>
+        <v>4.471</v>
       </c>
       <c r="S22" t="n">
-        <v>4.407</v>
+        <v>4.534</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.762</v>
+        <v>2.778</v>
       </c>
       <c r="G23" t="n">
-        <v>2.844</v>
+        <v>2.863</v>
       </c>
       <c r="H23" t="n">
-        <v>2.992</v>
+        <v>3.02</v>
       </c>
       <c r="I23" t="n">
-        <v>3.167</v>
+        <v>3.193</v>
       </c>
       <c r="J23" t="n">
-        <v>3.466</v>
+        <v>3.501</v>
       </c>
       <c r="K23" t="n">
-        <v>3.69</v>
+        <v>3.751</v>
       </c>
       <c r="L23" t="n">
-        <v>3.734</v>
+        <v>3.793</v>
       </c>
       <c r="M23" t="n">
-        <v>3.869</v>
+        <v>3.942</v>
       </c>
       <c r="N23" t="n">
-        <v>3.935</v>
+        <v>4.021</v>
       </c>
       <c r="O23" t="n">
-        <v>4</v>
+        <v>4.093</v>
       </c>
       <c r="P23" t="n">
-        <v>4.1</v>
+        <v>4.202</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.157</v>
+        <v>4.265</v>
       </c>
       <c r="R23" t="n">
-        <v>4.135</v>
+        <v>4.255</v>
       </c>
       <c r="S23" t="n">
-        <v>4.161</v>
+        <v>4.288</v>
       </c>
       <c r="T23" t="n">
-        <v>4.064</v>
+        <v>4.185</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.698</v>
+        <v>2.714</v>
       </c>
       <c r="G24" t="n">
-        <v>2.761</v>
+        <v>2.779</v>
       </c>
       <c r="H24" t="n">
-        <v>2.893</v>
+        <v>2.921</v>
       </c>
       <c r="I24" t="n">
-        <v>3.076</v>
+        <v>3.104</v>
       </c>
       <c r="J24" t="n">
-        <v>3.366</v>
+        <v>3.401</v>
       </c>
       <c r="K24" t="n">
-        <v>3.576</v>
+        <v>3.637</v>
       </c>
       <c r="L24" t="n">
-        <v>3.615</v>
+        <v>3.674</v>
       </c>
       <c r="M24" t="n">
-        <v>3.732</v>
+        <v>3.806</v>
       </c>
       <c r="N24" t="n">
-        <v>3.812</v>
+        <v>3.898</v>
       </c>
       <c r="O24" t="n">
-        <v>3.994</v>
+        <v>4.087</v>
       </c>
       <c r="P24" t="n">
-        <v>4.038</v>
+        <v>4.14</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.082</v>
+        <v>4.19</v>
       </c>
       <c r="R24" t="n">
-        <v>4.057</v>
+        <v>4.176</v>
       </c>
       <c r="S24" t="n">
-        <v>4.076</v>
+        <v>4.203</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.756</v>
+        <v>2.772</v>
       </c>
       <c r="G25" t="n">
-        <v>2.844</v>
+        <v>2.863</v>
       </c>
       <c r="H25" t="n">
-        <v>2.995</v>
+        <v>3.023</v>
       </c>
       <c r="I25" t="n">
-        <v>3.174</v>
+        <v>3.2</v>
       </c>
       <c r="J25" t="n">
-        <v>3.482</v>
+        <v>3.517</v>
       </c>
       <c r="K25" t="n">
-        <v>3.723</v>
+        <v>3.784</v>
       </c>
       <c r="L25" t="n">
-        <v>3.764</v>
+        <v>3.823</v>
       </c>
       <c r="M25" t="n">
-        <v>3.9</v>
+        <v>3.974</v>
       </c>
       <c r="N25" t="n">
-        <v>3.962</v>
+        <v>4.048</v>
       </c>
       <c r="O25" t="n">
-        <v>4.031</v>
+        <v>4.124</v>
       </c>
       <c r="P25" t="n">
-        <v>4.121</v>
+        <v>4.223</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.191</v>
+        <v>4.299</v>
       </c>
       <c r="R25" t="n">
-        <v>4.159</v>
+        <v>4.278</v>
       </c>
       <c r="S25" t="n">
-        <v>4.184</v>
+        <v>4.311</v>
       </c>
       <c r="T25" t="n">
-        <v>4.082</v>
+        <v>4.203</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.04</v>
+        <v>3.05</v>
       </c>
       <c r="G26" t="n">
-        <v>3.183</v>
+        <v>3.198</v>
       </c>
       <c r="H26" t="n">
-        <v>3.442</v>
+        <v>3.465</v>
       </c>
       <c r="I26" t="n">
-        <v>3.676</v>
+        <v>3.702</v>
       </c>
       <c r="J26" t="n">
-        <v>4.126</v>
+        <v>4.161</v>
       </c>
       <c r="K26" t="n">
-        <v>4.542</v>
+        <v>4.611</v>
       </c>
       <c r="L26" t="n">
-        <v>4.65</v>
+        <v>4.71</v>
       </c>
       <c r="M26" t="n">
-        <v>4.849</v>
+        <v>4.927</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.107</v>
+        <v>5.205</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.842</v>
+        <v>2.856</v>
       </c>
       <c r="G27" t="n">
-        <v>2.929</v>
+        <v>2.945</v>
       </c>
       <c r="H27" t="n">
-        <v>3.084</v>
+        <v>3.111</v>
       </c>
       <c r="I27" t="n">
-        <v>3.291</v>
+        <v>3.319</v>
       </c>
       <c r="J27" t="n">
-        <v>3.626</v>
+        <v>3.661</v>
       </c>
       <c r="K27" t="n">
-        <v>3.854</v>
+        <v>3.92</v>
       </c>
       <c r="L27" t="n">
-        <v>3.913</v>
+        <v>3.974</v>
       </c>
       <c r="M27" t="n">
-        <v>4.052</v>
+        <v>4.128</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.196</v>
+        <v>4.293</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.945</v>
+        <v>2.959</v>
       </c>
       <c r="G28" t="n">
-        <v>3.04</v>
+        <v>3.056</v>
       </c>
       <c r="H28" t="n">
-        <v>3.21</v>
+        <v>3.237</v>
       </c>
       <c r="I28" t="n">
-        <v>3.429</v>
+        <v>3.457</v>
       </c>
       <c r="J28" t="n">
-        <v>3.799</v>
+        <v>3.834</v>
       </c>
       <c r="K28" t="n">
-        <v>4.047</v>
+        <v>4.112</v>
       </c>
       <c r="L28" t="n">
-        <v>4.117</v>
+        <v>4.177</v>
       </c>
       <c r="M28" t="n">
-        <v>4.264</v>
+        <v>4.34</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.49</v>
+        <v>4.586</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.794</v>
+        <v>2.806</v>
       </c>
       <c r="G29" t="n">
-        <v>2.882</v>
+        <v>2.896</v>
       </c>
       <c r="H29" t="n">
-        <v>3.025</v>
+        <v>3.052</v>
       </c>
       <c r="I29" t="n">
-        <v>3.224</v>
+        <v>3.249</v>
       </c>
       <c r="J29" t="n">
-        <v>3.538</v>
+        <v>3.573</v>
       </c>
       <c r="K29" t="n">
-        <v>3.75</v>
+        <v>3.815</v>
       </c>
       <c r="L29" t="n">
-        <v>3.798</v>
+        <v>3.859</v>
       </c>
       <c r="M29" t="n">
-        <v>3.914</v>
+        <v>3.991</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.066</v>
+        <v>4.163</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.083</v>
+        <v>3.096</v>
       </c>
       <c r="G30" t="n">
-        <v>3.161</v>
+        <v>3.177</v>
       </c>
       <c r="H30" t="n">
-        <v>3.378</v>
+        <v>3.401</v>
       </c>
       <c r="I30" t="n">
-        <v>3.607</v>
+        <v>3.632</v>
       </c>
       <c r="J30" t="n">
-        <v>3.997</v>
+        <v>4.034</v>
       </c>
       <c r="K30" t="n">
-        <v>4.339</v>
+        <v>4.411</v>
       </c>
       <c r="L30" t="n">
-        <v>4.425</v>
+        <v>4.488</v>
       </c>
       <c r="M30" t="n">
-        <v>4.615</v>
+        <v>4.697</v>
       </c>
       <c r="N30" t="n">
-        <v>4.772</v>
+        <v>4.859</v>
       </c>
       <c r="O30" t="n">
-        <v>5.056</v>
+        <v>5.154</v>
       </c>
       <c r="P30" t="n">
-        <v>5.258</v>
+        <v>5.362</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.022</v>
+        <v>6.129</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.411</v>
+        <v>3.424</v>
       </c>
       <c r="G31" t="n">
-        <v>3.525</v>
+        <v>3.541</v>
       </c>
       <c r="H31" t="n">
-        <v>3.792</v>
+        <v>3.815</v>
       </c>
       <c r="I31" t="n">
-        <v>4.036</v>
+        <v>4.062</v>
       </c>
       <c r="J31" t="n">
-        <v>4.489</v>
+        <v>4.526</v>
       </c>
       <c r="K31" t="n">
-        <v>4.872</v>
+        <v>4.944</v>
       </c>
       <c r="L31" t="n">
-        <v>5.038</v>
+        <v>5.101</v>
       </c>
       <c r="M31" t="n">
-        <v>5.346</v>
+        <v>5.427</v>
       </c>
       <c r="N31" t="n">
-        <v>5.63</v>
+        <v>5.717</v>
       </c>
       <c r="O31" t="n">
-        <v>6.091</v>
+        <v>6.19</v>
       </c>
       <c r="P31" t="n">
-        <v>6.246</v>
+        <v>6.35</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.996</v>
+        <v>7.103</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.182</v>
+        <v>3.195</v>
       </c>
       <c r="G32" t="n">
-        <v>3.278</v>
+        <v>3.295</v>
       </c>
       <c r="H32" t="n">
-        <v>3.521</v>
+        <v>3.544</v>
       </c>
       <c r="I32" t="n">
-        <v>3.766</v>
+        <v>3.791</v>
       </c>
       <c r="J32" t="n">
-        <v>4.175</v>
+        <v>4.212</v>
       </c>
       <c r="K32" t="n">
-        <v>4.524</v>
+        <v>4.596</v>
       </c>
       <c r="L32" t="n">
-        <v>4.63</v>
+        <v>4.692</v>
       </c>
       <c r="M32" t="n">
-        <v>4.888</v>
+        <v>4.969</v>
       </c>
       <c r="N32" t="n">
-        <v>5.133</v>
+        <v>5.219</v>
       </c>
       <c r="O32" t="n">
-        <v>5.501</v>
+        <v>5.6</v>
       </c>
       <c r="P32" t="n">
-        <v>5.718</v>
+        <v>5.822</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.483</v>
+        <v>6.59</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.95</v>
+        <v>2.963</v>
       </c>
       <c r="G33" t="n">
-        <v>3.027</v>
+        <v>3.043</v>
       </c>
       <c r="H33" t="n">
-        <v>3.192</v>
+        <v>3.215</v>
       </c>
       <c r="I33" t="n">
-        <v>3.388</v>
+        <v>3.414</v>
       </c>
       <c r="J33" t="n">
-        <v>3.706</v>
+        <v>3.741</v>
       </c>
       <c r="K33" t="n">
-        <v>3.983</v>
+        <v>4.053</v>
       </c>
       <c r="L33" t="n">
-        <v>4.03</v>
+        <v>4.092</v>
       </c>
       <c r="M33" t="n">
-        <v>4.143</v>
+        <v>4.224</v>
       </c>
       <c r="N33" t="n">
-        <v>4.165</v>
+        <v>4.25</v>
       </c>
       <c r="O33" t="n">
-        <v>4.211</v>
+        <v>4.309</v>
       </c>
       <c r="P33" t="n">
-        <v>4.291</v>
+        <v>4.395</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.739</v>
+        <v>4.846</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.01</v>
+        <v>3.023</v>
       </c>
       <c r="G34" t="n">
-        <v>3.08</v>
+        <v>3.096</v>
       </c>
       <c r="H34" t="n">
-        <v>3.254</v>
+        <v>3.277</v>
       </c>
       <c r="I34" t="n">
-        <v>3.456</v>
+        <v>3.482</v>
       </c>
       <c r="J34" t="n">
-        <v>3.778</v>
+        <v>3.812</v>
       </c>
       <c r="K34" t="n">
-        <v>4.059</v>
+        <v>4.129</v>
       </c>
       <c r="L34" t="n">
-        <v>4.109</v>
+        <v>4.171</v>
       </c>
       <c r="M34" t="n">
-        <v>4.234</v>
+        <v>4.314</v>
       </c>
       <c r="N34" t="n">
-        <v>4.268</v>
+        <v>4.354</v>
       </c>
       <c r="O34" t="n">
-        <v>4.38</v>
+        <v>4.479</v>
       </c>
       <c r="P34" t="n">
-        <v>4.585</v>
+        <v>4.689</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.44</v>
+        <v>5.547</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.984</v>
+        <v>2.997</v>
       </c>
       <c r="G35" t="n">
-        <v>3.054</v>
+        <v>3.07</v>
       </c>
       <c r="H35" t="n">
-        <v>3.222</v>
+        <v>3.245</v>
       </c>
       <c r="I35" t="n">
-        <v>3.422</v>
+        <v>3.449</v>
       </c>
       <c r="J35" t="n">
-        <v>3.746</v>
+        <v>3.781</v>
       </c>
       <c r="K35" t="n">
-        <v>4.013</v>
+        <v>4.083</v>
       </c>
       <c r="L35" t="n">
-        <v>4.064</v>
+        <v>4.126</v>
       </c>
       <c r="M35" t="n">
-        <v>4.181</v>
+        <v>4.261</v>
       </c>
       <c r="N35" t="n">
-        <v>4.204</v>
+        <v>4.29</v>
       </c>
       <c r="O35" t="n">
-        <v>4.277</v>
+        <v>4.376</v>
       </c>
       <c r="P35" t="n">
-        <v>4.388</v>
+        <v>4.492</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.076</v>
+        <v>5.183</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.885</v>
+        <v>2.895</v>
       </c>
       <c r="G36" t="n">
-        <v>2.957</v>
+        <v>2.97</v>
       </c>
       <c r="H36" t="n">
-        <v>3.112</v>
+        <v>3.135</v>
       </c>
       <c r="I36" t="n">
-        <v>3.314</v>
+        <v>3.336</v>
       </c>
       <c r="J36" t="n">
-        <v>3.641</v>
+        <v>3.676</v>
       </c>
       <c r="K36" t="n">
-        <v>3.907</v>
+        <v>3.977</v>
       </c>
       <c r="L36" t="n">
-        <v>3.955</v>
+        <v>4.017</v>
       </c>
       <c r="M36" t="n">
-        <v>4.047</v>
+        <v>4.128</v>
       </c>
       <c r="N36" t="n">
-        <v>4.069</v>
+        <v>4.156</v>
       </c>
       <c r="O36" t="n">
-        <v>4.123</v>
+        <v>4.221</v>
       </c>
       <c r="P36" t="n">
-        <v>4.19</v>
+        <v>4.294</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.456</v>
+        <v>4.563</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.754</v>
+        <v>3.767</v>
       </c>
       <c r="G37" t="n">
-        <v>4.219</v>
+        <v>4.235</v>
       </c>
       <c r="H37" t="n">
-        <v>4.768</v>
+        <v>4.791</v>
       </c>
       <c r="I37" t="n">
-        <v>5.1</v>
+        <v>5.124</v>
       </c>
       <c r="J37" t="n">
-        <v>5.981</v>
+        <v>6.017</v>
       </c>
       <c r="K37" t="n">
-        <v>6.914</v>
+        <v>6.984</v>
       </c>
       <c r="L37" t="n">
-        <v>7.238</v>
+        <v>7.301</v>
       </c>
       <c r="M37" t="n">
-        <v>7.618</v>
+        <v>7.699</v>
       </c>
       <c r="N37" t="n">
-        <v>7.78</v>
+        <v>7.867</v>
       </c>
       <c r="O37" t="n">
-        <v>7.97</v>
+        <v>8.069000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.045999999999999</v>
+        <v>8.15</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.484</v>
+        <v>8.590999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.813</v>
+        <v>4.826</v>
       </c>
       <c r="G38" t="n">
-        <v>5.532</v>
+        <v>5.548</v>
       </c>
       <c r="H38" t="n">
-        <v>6.292</v>
+        <v>6.315</v>
       </c>
       <c r="I38" t="n">
-        <v>6.781</v>
+        <v>6.805</v>
       </c>
       <c r="J38" t="n">
-        <v>7.924</v>
+        <v>7.96</v>
       </c>
       <c r="K38" t="n">
-        <v>9.035</v>
+        <v>9.106</v>
       </c>
       <c r="L38" t="n">
-        <v>9.518000000000001</v>
+        <v>9.581</v>
       </c>
       <c r="M38" t="n">
-        <v>10.028</v>
+        <v>10.111</v>
       </c>
       <c r="N38" t="n">
-        <v>10.198</v>
+        <v>10.286</v>
       </c>
       <c r="O38" t="n">
-        <v>10.37</v>
+        <v>10.469</v>
       </c>
       <c r="P38" t="n">
-        <v>10.443</v>
+        <v>10.547</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.934</v>
+        <v>11.042</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.134</v>
+        <v>4.147</v>
       </c>
       <c r="G39" t="n">
-        <v>4.73</v>
+        <v>4.746</v>
       </c>
       <c r="H39" t="n">
-        <v>5.357</v>
+        <v>5.38</v>
       </c>
       <c r="I39" t="n">
-        <v>5.785</v>
+        <v>5.809</v>
       </c>
       <c r="J39" t="n">
-        <v>6.796</v>
+        <v>6.832</v>
       </c>
       <c r="K39" t="n">
-        <v>7.868</v>
+        <v>7.939</v>
       </c>
       <c r="L39" t="n">
-        <v>8.276</v>
+        <v>8.339</v>
       </c>
       <c r="M39" t="n">
-        <v>8.664999999999999</v>
+        <v>8.747</v>
       </c>
       <c r="N39" t="n">
-        <v>8.826000000000001</v>
+        <v>8.913</v>
       </c>
       <c r="O39" t="n">
-        <v>9.02</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="P39" t="n">
-        <v>9.098000000000001</v>
+        <v>9.202</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.58</v>
+        <v>9.686999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.276</v>
+        <v>3.289</v>
       </c>
       <c r="G40" t="n">
-        <v>3.4</v>
+        <v>3.416</v>
       </c>
       <c r="H40" t="n">
-        <v>3.638</v>
+        <v>3.661</v>
       </c>
       <c r="I40" t="n">
-        <v>3.882</v>
+        <v>3.907</v>
       </c>
       <c r="J40" t="n">
-        <v>4.29</v>
+        <v>4.327</v>
       </c>
       <c r="K40" t="n">
-        <v>4.644</v>
+        <v>4.716</v>
       </c>
       <c r="L40" t="n">
-        <v>4.749</v>
+        <v>4.812</v>
       </c>
       <c r="M40" t="n">
-        <v>4.956</v>
+        <v>5.038</v>
       </c>
       <c r="N40" t="n">
-        <v>5.13</v>
+        <v>5.216</v>
       </c>
       <c r="O40" t="n">
-        <v>5.434</v>
+        <v>5.532</v>
       </c>
       <c r="P40" t="n">
-        <v>5.679</v>
+        <v>5.783</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.473</v>
+        <v>6.58</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.661</v>
+        <v>3.674</v>
       </c>
       <c r="G41" t="n">
-        <v>3.827</v>
+        <v>3.844</v>
       </c>
       <c r="H41" t="n">
-        <v>4.122</v>
+        <v>4.145</v>
       </c>
       <c r="I41" t="n">
-        <v>4.385</v>
+        <v>4.411</v>
       </c>
       <c r="J41" t="n">
-        <v>4.845</v>
+        <v>4.882</v>
       </c>
       <c r="K41" t="n">
-        <v>5.244</v>
+        <v>5.316</v>
       </c>
       <c r="L41" t="n">
-        <v>5.428</v>
+        <v>5.491</v>
       </c>
       <c r="M41" t="n">
-        <v>5.759</v>
+        <v>5.84</v>
       </c>
       <c r="N41" t="n">
-        <v>6.059</v>
+        <v>6.146</v>
       </c>
       <c r="O41" t="n">
-        <v>6.548</v>
+        <v>6.647</v>
       </c>
       <c r="P41" t="n">
-        <v>6.738</v>
+        <v>6.842</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.52</v>
+        <v>7.627</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.397</v>
+        <v>3.41</v>
       </c>
       <c r="G42" t="n">
-        <v>3.549</v>
+        <v>3.565</v>
       </c>
       <c r="H42" t="n">
-        <v>3.813</v>
+        <v>3.836</v>
       </c>
       <c r="I42" t="n">
-        <v>4.07</v>
+        <v>4.096</v>
       </c>
       <c r="J42" t="n">
-        <v>4.492</v>
+        <v>4.529</v>
       </c>
       <c r="K42" t="n">
-        <v>4.865</v>
+        <v>4.937</v>
       </c>
       <c r="L42" t="n">
-        <v>4.986</v>
+        <v>5.048</v>
       </c>
       <c r="M42" t="n">
-        <v>5.264</v>
+        <v>5.345</v>
       </c>
       <c r="N42" t="n">
-        <v>5.544</v>
+        <v>5.631</v>
       </c>
       <c r="O42" t="n">
-        <v>5.926</v>
+        <v>6.024</v>
       </c>
       <c r="P42" t="n">
-        <v>6.181</v>
+        <v>6.285</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.986</v>
+        <v>7.093</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.098</v>
+        <v>3.111</v>
       </c>
       <c r="G43" t="n">
-        <v>3.209</v>
+        <v>3.226</v>
       </c>
       <c r="H43" t="n">
-        <v>3.393</v>
+        <v>3.417</v>
       </c>
       <c r="I43" t="n">
-        <v>3.597</v>
+        <v>3.624</v>
       </c>
       <c r="J43" t="n">
-        <v>3.934</v>
+        <v>3.969</v>
       </c>
       <c r="K43" t="n">
-        <v>4.213</v>
+        <v>4.283</v>
       </c>
       <c r="L43" t="n">
-        <v>4.271</v>
+        <v>4.333</v>
       </c>
       <c r="M43" t="n">
-        <v>4.397</v>
+        <v>4.477</v>
       </c>
       <c r="N43" t="n">
-        <v>4.433</v>
+        <v>4.518</v>
       </c>
       <c r="O43" t="n">
-        <v>4.523</v>
+        <v>4.622</v>
       </c>
       <c r="P43" t="n">
-        <v>4.657</v>
+        <v>4.761</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.349</v>
+        <v>5.456</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.963</v>
+        <v>2.973</v>
       </c>
       <c r="G44" t="n">
-        <v>3.066</v>
+        <v>3.079</v>
       </c>
       <c r="H44" t="n">
-        <v>3.236</v>
+        <v>3.259</v>
       </c>
       <c r="I44" t="n">
-        <v>3.442</v>
+        <v>3.464</v>
       </c>
       <c r="J44" t="n">
-        <v>3.783</v>
+        <v>3.818</v>
       </c>
       <c r="K44" t="n">
-        <v>4.057</v>
+        <v>4.127</v>
       </c>
       <c r="L44" t="n">
-        <v>4.116</v>
+        <v>4.177</v>
       </c>
       <c r="M44" t="n">
-        <v>4.216</v>
+        <v>4.296</v>
       </c>
       <c r="N44" t="n">
-        <v>4.251</v>
+        <v>4.337</v>
       </c>
       <c r="O44" t="n">
-        <v>4.322</v>
+        <v>4.421</v>
       </c>
       <c r="P44" t="n">
-        <v>4.42</v>
+        <v>4.524</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.72</v>
+        <v>4.827</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-13 ~ 2026-05-13
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.182</v>
+        <v>3.177</v>
       </c>
       <c r="G2" t="n">
-        <v>3.408</v>
+        <v>3.402</v>
       </c>
       <c r="H2" t="n">
-        <v>3.647</v>
+        <v>3.645</v>
       </c>
       <c r="I2" t="n">
-        <v>3.833</v>
+        <v>3.823</v>
       </c>
       <c r="J2" t="n">
-        <v>4.165</v>
+        <v>4.142</v>
       </c>
       <c r="K2" t="n">
-        <v>4.627</v>
+        <v>4.586</v>
       </c>
       <c r="L2" t="n">
-        <v>4.798</v>
+        <v>4.756</v>
       </c>
       <c r="M2" t="n">
-        <v>5.13</v>
+        <v>5.089</v>
       </c>
       <c r="N2" t="n">
-        <v>5.419</v>
+        <v>5.392</v>
       </c>
       <c r="O2" t="n">
-        <v>5.667</v>
+        <v>5.649</v>
       </c>
       <c r="P2" t="n">
-        <v>5.887</v>
+        <v>5.872</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.527</v>
+        <v>6.516</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.206</v>
+        <v>4.201</v>
       </c>
       <c r="G3" t="n">
-        <v>4.613</v>
+        <v>4.607</v>
       </c>
       <c r="H3" t="n">
-        <v>4.885</v>
+        <v>4.883</v>
       </c>
       <c r="I3" t="n">
-        <v>5.066</v>
+        <v>5.056</v>
       </c>
       <c r="J3" t="n">
-        <v>5.411</v>
+        <v>5.388</v>
       </c>
       <c r="K3" t="n">
-        <v>5.943</v>
+        <v>5.902</v>
       </c>
       <c r="L3" t="n">
-        <v>6.183</v>
+        <v>6.141</v>
       </c>
       <c r="M3" t="n">
-        <v>6.547</v>
+        <v>6.506</v>
       </c>
       <c r="N3" t="n">
-        <v>6.778</v>
+        <v>6.751</v>
       </c>
       <c r="O3" t="n">
-        <v>6.977</v>
+        <v>6.959</v>
       </c>
       <c r="P3" t="n">
-        <v>7.067</v>
+        <v>7.052</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.596</v>
+        <v>7.585</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.698</v>
+        <v>3.693</v>
       </c>
       <c r="G4" t="n">
-        <v>3.994</v>
+        <v>3.988</v>
       </c>
       <c r="H4" t="n">
-        <v>4.294</v>
+        <v>4.292</v>
       </c>
       <c r="I4" t="n">
-        <v>4.509</v>
+        <v>4.499</v>
       </c>
       <c r="J4" t="n">
-        <v>4.857</v>
+        <v>4.834</v>
       </c>
       <c r="K4" t="n">
-        <v>5.382</v>
+        <v>5.341</v>
       </c>
       <c r="L4" t="n">
-        <v>5.552</v>
+        <v>5.51</v>
       </c>
       <c r="M4" t="n">
-        <v>5.905</v>
+        <v>5.864</v>
       </c>
       <c r="N4" t="n">
-        <v>6.106</v>
+        <v>6.079</v>
       </c>
       <c r="O4" t="n">
-        <v>6.328</v>
+        <v>6.31</v>
       </c>
       <c r="P4" t="n">
-        <v>6.417</v>
+        <v>6.402</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.949</v>
+        <v>6.938</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.877</v>
+        <v>2.872</v>
       </c>
       <c r="G5" t="n">
-        <v>2.952</v>
+        <v>2.946</v>
       </c>
       <c r="H5" t="n">
-        <v>3.151</v>
+        <v>3.149</v>
       </c>
       <c r="I5" t="n">
-        <v>3.402</v>
+        <v>3.392</v>
       </c>
       <c r="J5" t="n">
-        <v>3.728</v>
+        <v>3.702</v>
       </c>
       <c r="K5" t="n">
-        <v>4.039</v>
+        <v>3.996</v>
       </c>
       <c r="L5" t="n">
-        <v>4.055</v>
+        <v>4.011</v>
       </c>
       <c r="M5" t="n">
-        <v>4.189</v>
+        <v>4.147</v>
       </c>
       <c r="N5" t="n">
-        <v>4.233</v>
+        <v>4.206</v>
       </c>
       <c r="O5" t="n">
-        <v>4.266</v>
+        <v>4.248</v>
       </c>
       <c r="P5" t="n">
-        <v>4.555</v>
+        <v>4.54</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.439</v>
+        <v>5.429</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.916</v>
+        <v>2.911</v>
       </c>
       <c r="G6" t="n">
-        <v>3.005</v>
+        <v>2.999</v>
       </c>
       <c r="H6" t="n">
-        <v>3.22</v>
+        <v>3.218</v>
       </c>
       <c r="I6" t="n">
-        <v>3.485</v>
+        <v>3.475</v>
       </c>
       <c r="J6" t="n">
-        <v>3.816</v>
+        <v>3.79</v>
       </c>
       <c r="K6" t="n">
-        <v>4.148</v>
+        <v>4.106</v>
       </c>
       <c r="L6" t="n">
-        <v>4.169</v>
+        <v>4.125</v>
       </c>
       <c r="M6" t="n">
-        <v>4.345</v>
+        <v>4.303</v>
       </c>
       <c r="N6" t="n">
-        <v>4.4</v>
+        <v>4.373</v>
       </c>
       <c r="O6" t="n">
-        <v>4.532</v>
+        <v>4.515</v>
       </c>
       <c r="P6" t="n">
-        <v>4.988</v>
+        <v>4.973</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.836</v>
+        <v>5.825</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.897</v>
+        <v>2.892</v>
       </c>
       <c r="G7" t="n">
-        <v>2.969</v>
+        <v>2.963</v>
       </c>
       <c r="H7" t="n">
-        <v>3.166</v>
+        <v>3.164</v>
       </c>
       <c r="I7" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
       <c r="J7" t="n">
-        <v>3.752</v>
+        <v>3.726</v>
       </c>
       <c r="K7" t="n">
-        <v>4.065</v>
+        <v>4.023</v>
       </c>
       <c r="L7" t="n">
-        <v>4.079</v>
+        <v>4.035</v>
       </c>
       <c r="M7" t="n">
-        <v>4.25</v>
+        <v>4.209</v>
       </c>
       <c r="N7" t="n">
-        <v>4.292</v>
+        <v>4.265</v>
       </c>
       <c r="O7" t="n">
-        <v>4.43</v>
+        <v>4.413</v>
       </c>
       <c r="P7" t="n">
-        <v>4.771</v>
+        <v>4.756</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.603</v>
+        <v>5.592</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.318</v>
+        <v>5.313</v>
       </c>
       <c r="G8" t="n">
-        <v>5.913</v>
+        <v>5.907</v>
       </c>
       <c r="H8" t="n">
-        <v>6.333</v>
+        <v>6.331</v>
       </c>
       <c r="I8" t="n">
-        <v>6.591</v>
+        <v>6.582</v>
       </c>
       <c r="J8" t="n">
-        <v>7.003</v>
+        <v>6.98</v>
       </c>
       <c r="K8" t="n">
-        <v>7.815</v>
+        <v>7.774</v>
       </c>
       <c r="L8" t="n">
-        <v>8.141</v>
+        <v>8.1</v>
       </c>
       <c r="M8" t="n">
-        <v>8.536</v>
+        <v>8.494999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.702</v>
+        <v>8.676</v>
       </c>
       <c r="O8" t="n">
-        <v>8.986000000000001</v>
+        <v>8.968</v>
       </c>
       <c r="P8" t="n">
-        <v>9.178000000000001</v>
+        <v>9.163</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.904999999999999</v>
+        <v>9.894</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.61</v>
+        <v>2.613</v>
       </c>
       <c r="G9" t="n">
-        <v>2.706</v>
+        <v>2.707</v>
       </c>
       <c r="H9" t="n">
-        <v>2.843</v>
+        <v>2.841</v>
       </c>
       <c r="I9" t="n">
-        <v>3.095</v>
+        <v>3.098</v>
       </c>
       <c r="J9" t="n">
-        <v>3.318</v>
+        <v>3.294</v>
       </c>
       <c r="K9" t="n">
-        <v>3.55</v>
+        <v>3.504</v>
       </c>
       <c r="L9" t="n">
-        <v>3.569</v>
+        <v>3.53</v>
       </c>
       <c r="M9" t="n">
-        <v>3.68</v>
+        <v>3.642</v>
       </c>
       <c r="N9" t="n">
-        <v>3.833</v>
+        <v>3.81</v>
       </c>
       <c r="O9" t="n">
-        <v>3.876</v>
+        <v>3.86</v>
       </c>
       <c r="P9" t="n">
-        <v>3.985</v>
+        <v>3.971</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.065</v>
+        <v>4.054</v>
       </c>
       <c r="R9" t="n">
-        <v>4.07</v>
+        <v>4.055</v>
       </c>
       <c r="S9" t="n">
-        <v>4.07</v>
+        <v>4.051</v>
       </c>
       <c r="T9" t="n">
-        <v>3.975</v>
+        <v>3.97</v>
       </c>
       <c r="U9" t="n">
-        <v>3.845</v>
+        <v>3.841</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.625</v>
+        <v>2.627</v>
       </c>
       <c r="G10" t="n">
         <v>2.738</v>
       </c>
       <c r="H10" t="n">
-        <v>2.856</v>
+        <v>2.854</v>
       </c>
       <c r="I10" t="n">
         <v>3.103</v>
       </c>
       <c r="J10" t="n">
-        <v>3.34</v>
+        <v>3.319</v>
       </c>
       <c r="K10" t="n">
-        <v>3.583</v>
+        <v>3.537</v>
       </c>
       <c r="L10" t="n">
-        <v>3.618</v>
+        <v>3.578</v>
       </c>
       <c r="M10" t="n">
-        <v>3.775</v>
+        <v>3.736</v>
       </c>
       <c r="N10" t="n">
-        <v>3.851</v>
+        <v>3.829</v>
       </c>
       <c r="O10" t="n">
-        <v>4.069</v>
+        <v>4.053</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.44</v>
+        <v>2.442</v>
       </c>
       <c r="G11" t="n">
-        <v>2.547</v>
+        <v>2.548</v>
       </c>
       <c r="H11" t="n">
-        <v>2.682</v>
+        <v>2.677</v>
       </c>
       <c r="I11" t="n">
-        <v>2.906</v>
+        <v>2.907</v>
       </c>
       <c r="J11" t="n">
-        <v>3.138</v>
+        <v>3.117</v>
       </c>
       <c r="K11" t="n">
-        <v>3.371</v>
+        <v>3.325</v>
       </c>
       <c r="L11" t="n">
-        <v>3.415</v>
+        <v>3.375</v>
       </c>
       <c r="M11" t="n">
-        <v>3.582</v>
+        <v>3.544</v>
       </c>
       <c r="N11" t="n">
-        <v>3.659</v>
+        <v>3.637</v>
       </c>
       <c r="O11" t="n">
-        <v>3.835</v>
+        <v>3.82</v>
       </c>
       <c r="P11" t="n">
-        <v>3.935</v>
+        <v>3.921</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.266</v>
+        <v>4.256</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.192</v>
+        <v>3.189</v>
       </c>
       <c r="G12" t="n">
-        <v>3.371</v>
+        <v>3.369</v>
       </c>
       <c r="H12" t="n">
-        <v>3.544</v>
+        <v>3.55</v>
       </c>
       <c r="I12" t="n">
-        <v>3.793</v>
+        <v>3.79</v>
       </c>
       <c r="J12" t="n">
-        <v>4.165</v>
+        <v>4.144</v>
       </c>
       <c r="K12" t="n">
-        <v>4.415</v>
+        <v>4.381</v>
       </c>
       <c r="L12" t="n">
-        <v>4.476</v>
+        <v>4.44</v>
       </c>
       <c r="M12" t="n">
-        <v>4.647</v>
+        <v>4.614</v>
       </c>
       <c r="N12" t="n">
-        <v>4.709</v>
+        <v>4.689</v>
       </c>
       <c r="O12" t="n">
-        <v>4.867</v>
+        <v>4.853</v>
       </c>
       <c r="P12" t="n">
-        <v>5.023</v>
+        <v>5.009</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.383</v>
+        <v>5.373</v>
       </c>
       <c r="R12" t="n">
-        <v>5.563</v>
+        <v>5.548</v>
       </c>
       <c r="S12" t="n">
-        <v>5.775</v>
+        <v>5.757</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.946</v>
+        <v>2.943</v>
       </c>
       <c r="G13" t="n">
-        <v>3.061</v>
+        <v>3.059</v>
       </c>
       <c r="H13" t="n">
-        <v>3.211</v>
+        <v>3.218</v>
       </c>
       <c r="I13" t="n">
-        <v>3.441</v>
+        <v>3.437</v>
       </c>
       <c r="J13" t="n">
-        <v>3.802</v>
+        <v>3.781</v>
       </c>
       <c r="K13" t="n">
-        <v>4.049</v>
+        <v>4.014</v>
       </c>
       <c r="L13" t="n">
-        <v>4.115</v>
+        <v>4.079</v>
       </c>
       <c r="M13" t="n">
-        <v>4.274</v>
+        <v>4.241</v>
       </c>
       <c r="N13" t="n">
-        <v>4.337</v>
+        <v>4.318</v>
       </c>
       <c r="O13" t="n">
-        <v>4.495</v>
+        <v>4.481</v>
       </c>
       <c r="P13" t="n">
-        <v>4.615</v>
+        <v>4.601</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.904</v>
+        <v>4.895</v>
       </c>
       <c r="R13" t="n">
-        <v>5.113</v>
+        <v>5.098</v>
       </c>
       <c r="S13" t="n">
-        <v>5.337</v>
+        <v>5.319</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.765</v>
+        <v>2.762</v>
       </c>
       <c r="G14" t="n">
-        <v>2.866</v>
+        <v>2.865</v>
       </c>
       <c r="H14" t="n">
-        <v>3.015</v>
+        <v>3.021</v>
       </c>
       <c r="I14" t="n">
-        <v>3.224</v>
+        <v>3.221</v>
       </c>
       <c r="J14" t="n">
-        <v>3.542</v>
+        <v>3.521</v>
       </c>
       <c r="K14" t="n">
-        <v>3.737</v>
+        <v>3.702</v>
       </c>
       <c r="L14" t="n">
-        <v>3.787</v>
+        <v>3.751</v>
       </c>
       <c r="M14" t="n">
-        <v>3.96</v>
+        <v>3.926</v>
       </c>
       <c r="N14" t="n">
-        <v>4.015</v>
+        <v>3.996</v>
       </c>
       <c r="O14" t="n">
-        <v>4.151</v>
+        <v>4.137</v>
       </c>
       <c r="P14" t="n">
-        <v>4.25</v>
+        <v>4.236</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.494</v>
+        <v>4.484</v>
       </c>
       <c r="R14" t="n">
-        <v>4.627</v>
+        <v>4.612</v>
       </c>
       <c r="S14" t="n">
-        <v>4.79</v>
+        <v>4.772</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.743</v>
+        <v>2.74</v>
       </c>
       <c r="G15" t="n">
-        <v>2.841</v>
+        <v>2.839</v>
       </c>
       <c r="H15" t="n">
-        <v>2.985</v>
+        <v>2.992</v>
       </c>
       <c r="I15" t="n">
-        <v>3.175</v>
+        <v>3.172</v>
       </c>
       <c r="J15" t="n">
-        <v>3.481</v>
+        <v>3.46</v>
       </c>
       <c r="K15" t="n">
-        <v>3.689</v>
+        <v>3.654</v>
       </c>
       <c r="L15" t="n">
-        <v>3.723</v>
+        <v>3.687</v>
       </c>
       <c r="M15" t="n">
-        <v>3.872</v>
+        <v>3.839</v>
       </c>
       <c r="N15" t="n">
-        <v>3.919</v>
+        <v>3.9</v>
       </c>
       <c r="O15" t="n">
-        <v>4.093</v>
+        <v>4.078</v>
       </c>
       <c r="P15" t="n">
-        <v>4.15</v>
+        <v>4.136</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.396</v>
+        <v>4.386</v>
       </c>
       <c r="R15" t="n">
-        <v>4.522</v>
+        <v>4.508</v>
       </c>
       <c r="S15" t="n">
-        <v>4.685</v>
+        <v>4.667</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.743</v>
+        <v>2.74</v>
       </c>
       <c r="G16" t="n">
-        <v>2.841</v>
+        <v>2.839</v>
       </c>
       <c r="H16" t="n">
-        <v>2.985</v>
+        <v>2.992</v>
       </c>
       <c r="I16" t="n">
-        <v>3.175</v>
+        <v>3.172</v>
       </c>
       <c r="J16" t="n">
-        <v>3.481</v>
+        <v>3.46</v>
       </c>
       <c r="K16" t="n">
-        <v>3.689</v>
+        <v>3.654</v>
       </c>
       <c r="L16" t="n">
-        <v>3.723</v>
+        <v>3.687</v>
       </c>
       <c r="M16" t="n">
-        <v>3.872</v>
+        <v>3.839</v>
       </c>
       <c r="N16" t="n">
-        <v>3.922</v>
+        <v>3.903</v>
       </c>
       <c r="O16" t="n">
-        <v>4.099</v>
+        <v>4.085</v>
       </c>
       <c r="P16" t="n">
-        <v>4.173</v>
+        <v>4.159</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.424</v>
+        <v>4.414</v>
       </c>
       <c r="R16" t="n">
-        <v>4.55</v>
+        <v>4.536</v>
       </c>
       <c r="S16" t="n">
-        <v>4.714</v>
+        <v>4.696</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.687</v>
+        <v>2.689</v>
       </c>
       <c r="G17" t="n">
-        <v>2.83</v>
+        <v>2.829</v>
       </c>
       <c r="H17" t="n">
-        <v>2.952</v>
+        <v>2.948</v>
       </c>
       <c r="I17" t="n">
-        <v>3.184</v>
+        <v>3.185</v>
       </c>
       <c r="J17" t="n">
-        <v>3.415</v>
+        <v>3.395</v>
       </c>
       <c r="K17" t="n">
-        <v>3.66</v>
+        <v>3.614</v>
       </c>
       <c r="L17" t="n">
-        <v>3.7</v>
+        <v>3.662</v>
       </c>
       <c r="M17" t="n">
-        <v>3.895</v>
+        <v>3.858</v>
       </c>
       <c r="N17" t="n">
-        <v>3.952</v>
+        <v>3.931</v>
       </c>
       <c r="O17" t="n">
-        <v>4.096</v>
+        <v>4.083</v>
       </c>
       <c r="P17" t="n">
-        <v>4.212</v>
+        <v>4.199</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.687</v>
+        <v>2.69</v>
       </c>
       <c r="G18" t="n">
-        <v>2.831</v>
+        <v>2.83</v>
       </c>
       <c r="H18" t="n">
-        <v>2.953</v>
+        <v>2.948</v>
       </c>
       <c r="I18" t="n">
         <v>3.185</v>
       </c>
       <c r="J18" t="n">
-        <v>3.415</v>
+        <v>3.395</v>
       </c>
       <c r="K18" t="n">
-        <v>3.661</v>
+        <v>3.615</v>
       </c>
       <c r="L18" t="n">
-        <v>3.7</v>
+        <v>3.662</v>
       </c>
       <c r="M18" t="n">
-        <v>3.895</v>
+        <v>3.858</v>
       </c>
       <c r="N18" t="n">
-        <v>3.953</v>
+        <v>3.932</v>
       </c>
       <c r="O18" t="n">
-        <v>4.094</v>
+        <v>4.08</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.756</v>
+        <v>2.753</v>
       </c>
       <c r="G19" t="n">
-        <v>2.857</v>
+        <v>2.855</v>
       </c>
       <c r="H19" t="n">
-        <v>3.004</v>
+        <v>3.01</v>
       </c>
       <c r="I19" t="n">
-        <v>3.211</v>
+        <v>3.208</v>
       </c>
       <c r="J19" t="n">
-        <v>3.525</v>
+        <v>3.504</v>
       </c>
       <c r="K19" t="n">
-        <v>3.733</v>
+        <v>3.698</v>
       </c>
       <c r="L19" t="n">
-        <v>3.783</v>
+        <v>3.748</v>
       </c>
       <c r="M19" t="n">
-        <v>3.95</v>
+        <v>3.917</v>
       </c>
       <c r="N19" t="n">
-        <v>4.005</v>
+        <v>3.985</v>
       </c>
       <c r="O19" t="n">
-        <v>4.135</v>
+        <v>4.12</v>
       </c>
       <c r="P19" t="n">
-        <v>4.209</v>
+        <v>4.195</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.435</v>
+        <v>4.425</v>
       </c>
       <c r="R19" t="n">
-        <v>4.571</v>
+        <v>4.556</v>
       </c>
       <c r="S19" t="n">
-        <v>4.725</v>
+        <v>4.707</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1872,22 +1872,22 @@
         <v>2.669</v>
       </c>
       <c r="H20" t="n">
-        <v>2.734</v>
+        <v>2.735</v>
       </c>
       <c r="I20" t="n">
-        <v>2.87</v>
+        <v>2.858</v>
       </c>
       <c r="J20" t="n">
-        <v>3.315</v>
+        <v>3.29</v>
       </c>
       <c r="K20" t="n">
-        <v>3.569</v>
+        <v>3.53</v>
       </c>
       <c r="L20" t="n">
-        <v>3.614</v>
+        <v>3.573</v>
       </c>
       <c r="M20" t="n">
-        <v>3.72</v>
+        <v>3.681</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.879</v>
+        <v>2.877</v>
       </c>
       <c r="G21" t="n">
-        <v>2.962</v>
+        <v>2.96</v>
       </c>
       <c r="H21" t="n">
-        <v>3.148</v>
+        <v>3.152</v>
       </c>
       <c r="I21" t="n">
-        <v>3.323</v>
+        <v>3.318</v>
       </c>
       <c r="J21" t="n">
-        <v>3.673</v>
+        <v>3.649</v>
       </c>
       <c r="K21" t="n">
-        <v>3.968</v>
+        <v>3.932</v>
       </c>
       <c r="L21" t="n">
-        <v>4.026</v>
+        <v>3.989</v>
       </c>
       <c r="M21" t="n">
-        <v>4.179</v>
+        <v>4.143</v>
       </c>
       <c r="N21" t="n">
-        <v>4.253</v>
+        <v>4.228</v>
       </c>
       <c r="O21" t="n">
-        <v>4.35</v>
+        <v>4.332</v>
       </c>
       <c r="P21" t="n">
-        <v>4.475</v>
+        <v>4.46</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.601</v>
+        <v>4.592</v>
       </c>
       <c r="R21" t="n">
-        <v>4.622</v>
+        <v>4.607</v>
       </c>
       <c r="S21" t="n">
-        <v>4.688</v>
+        <v>4.668</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.826</v>
+        <v>2.824</v>
       </c>
       <c r="G22" t="n">
-        <v>2.908</v>
+        <v>2.905</v>
       </c>
       <c r="H22" t="n">
-        <v>3.08</v>
+        <v>3.084</v>
       </c>
       <c r="I22" t="n">
-        <v>3.242</v>
+        <v>3.237</v>
       </c>
       <c r="J22" t="n">
-        <v>3.559</v>
+        <v>3.535</v>
       </c>
       <c r="K22" t="n">
-        <v>3.85</v>
+        <v>3.814</v>
       </c>
       <c r="L22" t="n">
-        <v>3.893</v>
+        <v>3.856</v>
       </c>
       <c r="M22" t="n">
-        <v>4.048</v>
+        <v>4.013</v>
       </c>
       <c r="N22" t="n">
-        <v>4.125</v>
+        <v>4.1</v>
       </c>
       <c r="O22" t="n">
-        <v>4.217</v>
+        <v>4.2</v>
       </c>
       <c r="P22" t="n">
-        <v>4.337</v>
+        <v>4.322</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.459</v>
+        <v>4.45</v>
       </c>
       <c r="R22" t="n">
-        <v>4.471</v>
+        <v>4.456</v>
       </c>
       <c r="S22" t="n">
-        <v>4.534</v>
+        <v>4.514</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.778</v>
+        <v>2.776</v>
       </c>
       <c r="G23" t="n">
-        <v>2.863</v>
+        <v>2.86</v>
       </c>
       <c r="H23" t="n">
-        <v>3.02</v>
+        <v>3.024</v>
       </c>
       <c r="I23" t="n">
-        <v>3.193</v>
+        <v>3.188</v>
       </c>
       <c r="J23" t="n">
-        <v>3.501</v>
+        <v>3.477</v>
       </c>
       <c r="K23" t="n">
-        <v>3.751</v>
+        <v>3.715</v>
       </c>
       <c r="L23" t="n">
-        <v>3.793</v>
+        <v>3.755</v>
       </c>
       <c r="M23" t="n">
-        <v>3.942</v>
+        <v>3.906</v>
       </c>
       <c r="N23" t="n">
-        <v>4.021</v>
+        <v>3.996</v>
       </c>
       <c r="O23" t="n">
-        <v>4.093</v>
+        <v>4.077</v>
       </c>
       <c r="P23" t="n">
-        <v>4.202</v>
+        <v>4.187</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.265</v>
+        <v>4.256</v>
       </c>
       <c r="R23" t="n">
-        <v>4.255</v>
+        <v>4.24</v>
       </c>
       <c r="S23" t="n">
-        <v>4.288</v>
+        <v>4.268</v>
       </c>
       <c r="T23" t="n">
-        <v>4.185</v>
+        <v>4.179</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.714</v>
+        <v>2.712</v>
       </c>
       <c r="G24" t="n">
-        <v>2.779</v>
+        <v>2.776</v>
       </c>
       <c r="H24" t="n">
-        <v>2.921</v>
+        <v>2.925</v>
       </c>
       <c r="I24" t="n">
-        <v>3.104</v>
+        <v>3.103</v>
       </c>
       <c r="J24" t="n">
-        <v>3.401</v>
+        <v>3.377</v>
       </c>
       <c r="K24" t="n">
+        <v>3.601</v>
+      </c>
+      <c r="L24" t="n">
         <v>3.637</v>
       </c>
-      <c r="L24" t="n">
-        <v>3.674</v>
-      </c>
       <c r="M24" t="n">
-        <v>3.806</v>
+        <v>3.77</v>
       </c>
       <c r="N24" t="n">
-        <v>3.898</v>
+        <v>3.873</v>
       </c>
       <c r="O24" t="n">
-        <v>4.087</v>
+        <v>4.069</v>
       </c>
       <c r="P24" t="n">
-        <v>4.14</v>
+        <v>4.126</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.19</v>
+        <v>4.181</v>
       </c>
       <c r="R24" t="n">
-        <v>4.176</v>
+        <v>4.161</v>
       </c>
       <c r="S24" t="n">
-        <v>4.203</v>
+        <v>4.183</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.772</v>
+        <v>2.77</v>
       </c>
       <c r="G25" t="n">
-        <v>2.863</v>
+        <v>2.86</v>
       </c>
       <c r="H25" t="n">
-        <v>3.023</v>
+        <v>3.027</v>
       </c>
       <c r="I25" t="n">
-        <v>3.2</v>
+        <v>3.196</v>
       </c>
       <c r="J25" t="n">
-        <v>3.517</v>
+        <v>3.493</v>
       </c>
       <c r="K25" t="n">
-        <v>3.784</v>
+        <v>3.747</v>
       </c>
       <c r="L25" t="n">
-        <v>3.823</v>
+        <v>3.786</v>
       </c>
       <c r="M25" t="n">
-        <v>3.974</v>
+        <v>3.938</v>
       </c>
       <c r="N25" t="n">
-        <v>4.048</v>
+        <v>4.022</v>
       </c>
       <c r="O25" t="n">
-        <v>4.124</v>
+        <v>4.106</v>
       </c>
       <c r="P25" t="n">
-        <v>4.223</v>
+        <v>4.209</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.299</v>
+        <v>4.29</v>
       </c>
       <c r="R25" t="n">
-        <v>4.278</v>
+        <v>4.263</v>
       </c>
       <c r="S25" t="n">
-        <v>4.311</v>
+        <v>4.291</v>
       </c>
       <c r="T25" t="n">
-        <v>4.203</v>
+        <v>4.197</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.05</v>
+        <v>3.046</v>
       </c>
       <c r="G26" t="n">
-        <v>3.198</v>
+        <v>3.192</v>
       </c>
       <c r="H26" t="n">
-        <v>3.465</v>
+        <v>3.462</v>
       </c>
       <c r="I26" t="n">
-        <v>3.702</v>
+        <v>3.691</v>
       </c>
       <c r="J26" t="n">
-        <v>4.161</v>
+        <v>4.134</v>
       </c>
       <c r="K26" t="n">
-        <v>4.611</v>
+        <v>4.569</v>
       </c>
       <c r="L26" t="n">
-        <v>4.71</v>
+        <v>4.668</v>
       </c>
       <c r="M26" t="n">
-        <v>4.927</v>
+        <v>4.886</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.205</v>
+        <v>5.187</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.856</v>
+        <v>2.851</v>
       </c>
       <c r="G27" t="n">
-        <v>2.945</v>
+        <v>2.941</v>
       </c>
       <c r="H27" t="n">
-        <v>3.111</v>
+        <v>3.112</v>
       </c>
       <c r="I27" t="n">
-        <v>3.319</v>
+        <v>3.314</v>
       </c>
       <c r="J27" t="n">
-        <v>3.661</v>
+        <v>3.639</v>
       </c>
       <c r="K27" t="n">
-        <v>3.92</v>
+        <v>3.883</v>
       </c>
       <c r="L27" t="n">
-        <v>3.974</v>
+        <v>3.937</v>
       </c>
       <c r="M27" t="n">
-        <v>4.128</v>
+        <v>4.094</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.293</v>
+        <v>4.277</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.959</v>
+        <v>2.954</v>
       </c>
       <c r="G28" t="n">
-        <v>3.056</v>
+        <v>3.052</v>
       </c>
       <c r="H28" t="n">
-        <v>3.237</v>
+        <v>3.238</v>
       </c>
       <c r="I28" t="n">
-        <v>3.457</v>
+        <v>3.452</v>
       </c>
       <c r="J28" t="n">
-        <v>3.834</v>
+        <v>3.813</v>
       </c>
       <c r="K28" t="n">
-        <v>4.112</v>
+        <v>4.075</v>
       </c>
       <c r="L28" t="n">
-        <v>4.177</v>
+        <v>4.14</v>
       </c>
       <c r="M28" t="n">
-        <v>4.34</v>
+        <v>4.306</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.586</v>
+        <v>4.57</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.806</v>
+        <v>2.801</v>
       </c>
       <c r="G29" t="n">
-        <v>2.896</v>
+        <v>2.891</v>
       </c>
       <c r="H29" t="n">
-        <v>3.052</v>
+        <v>3.053</v>
       </c>
       <c r="I29" t="n">
-        <v>3.249</v>
+        <v>3.244</v>
       </c>
       <c r="J29" t="n">
-        <v>3.573</v>
+        <v>3.552</v>
       </c>
       <c r="K29" t="n">
-        <v>3.815</v>
+        <v>3.778</v>
       </c>
       <c r="L29" t="n">
-        <v>3.859</v>
+        <v>3.822</v>
       </c>
       <c r="M29" t="n">
-        <v>3.991</v>
+        <v>3.957</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.163</v>
+        <v>4.147</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.096</v>
+        <v>3.09</v>
       </c>
       <c r="G30" t="n">
-        <v>3.177</v>
+        <v>3.172</v>
       </c>
       <c r="H30" t="n">
-        <v>3.401</v>
+        <v>3.397</v>
       </c>
       <c r="I30" t="n">
-        <v>3.632</v>
+        <v>3.621</v>
       </c>
       <c r="J30" t="n">
-        <v>4.034</v>
+        <v>4.008</v>
       </c>
       <c r="K30" t="n">
-        <v>4.411</v>
+        <v>4.369</v>
       </c>
       <c r="L30" t="n">
-        <v>4.488</v>
+        <v>4.447</v>
       </c>
       <c r="M30" t="n">
-        <v>4.697</v>
+        <v>4.657</v>
       </c>
       <c r="N30" t="n">
-        <v>4.859</v>
+        <v>4.832</v>
       </c>
       <c r="O30" t="n">
-        <v>5.154</v>
+        <v>5.136</v>
       </c>
       <c r="P30" t="n">
-        <v>5.362</v>
+        <v>5.346</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.129</v>
+        <v>6.119</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.424</v>
+        <v>3.419</v>
       </c>
       <c r="G31" t="n">
-        <v>3.541</v>
+        <v>3.537</v>
       </c>
       <c r="H31" t="n">
-        <v>3.815</v>
+        <v>3.812</v>
       </c>
       <c r="I31" t="n">
-        <v>4.062</v>
+        <v>4.05</v>
       </c>
       <c r="J31" t="n">
-        <v>4.526</v>
+        <v>4.5</v>
       </c>
       <c r="K31" t="n">
-        <v>4.944</v>
+        <v>4.902</v>
       </c>
       <c r="L31" t="n">
-        <v>5.101</v>
+        <v>5.06</v>
       </c>
       <c r="M31" t="n">
-        <v>5.427</v>
+        <v>5.387</v>
       </c>
       <c r="N31" t="n">
-        <v>5.717</v>
+        <v>5.691</v>
       </c>
       <c r="O31" t="n">
-        <v>6.19</v>
+        <v>6.172</v>
       </c>
       <c r="P31" t="n">
-        <v>6.35</v>
+        <v>6.335</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.103</v>
+        <v>7.092</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.195</v>
+        <v>3.189</v>
       </c>
       <c r="G32" t="n">
-        <v>3.295</v>
+        <v>3.29</v>
       </c>
       <c r="H32" t="n">
-        <v>3.544</v>
+        <v>3.541</v>
       </c>
       <c r="I32" t="n">
-        <v>3.791</v>
+        <v>3.78</v>
       </c>
       <c r="J32" t="n">
-        <v>4.212</v>
+        <v>4.186</v>
       </c>
       <c r="K32" t="n">
-        <v>4.596</v>
+        <v>4.554</v>
       </c>
       <c r="L32" t="n">
-        <v>4.692</v>
+        <v>4.651</v>
       </c>
       <c r="M32" t="n">
-        <v>4.969</v>
+        <v>4.929</v>
       </c>
       <c r="N32" t="n">
-        <v>5.219</v>
+        <v>5.193</v>
       </c>
       <c r="O32" t="n">
-        <v>5.6</v>
+        <v>5.582</v>
       </c>
       <c r="P32" t="n">
-        <v>5.822</v>
+        <v>5.807</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.59</v>
+        <v>6.58</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.963</v>
+        <v>2.957</v>
       </c>
       <c r="G33" t="n">
-        <v>3.043</v>
+        <v>3.038</v>
       </c>
       <c r="H33" t="n">
-        <v>3.215</v>
+        <v>3.212</v>
       </c>
       <c r="I33" t="n">
-        <v>3.414</v>
+        <v>3.404</v>
       </c>
       <c r="J33" t="n">
-        <v>3.741</v>
+        <v>3.714</v>
       </c>
       <c r="K33" t="n">
-        <v>4.053</v>
+        <v>4.011</v>
       </c>
       <c r="L33" t="n">
-        <v>4.092</v>
+        <v>4.05</v>
       </c>
       <c r="M33" t="n">
-        <v>4.224</v>
+        <v>4.183</v>
       </c>
       <c r="N33" t="n">
-        <v>4.25</v>
+        <v>4.223</v>
       </c>
       <c r="O33" t="n">
-        <v>4.309</v>
+        <v>4.291</v>
       </c>
       <c r="P33" t="n">
-        <v>4.395</v>
+        <v>4.38</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.846</v>
+        <v>4.836</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.023</v>
+        <v>3.017</v>
       </c>
       <c r="G34" t="n">
-        <v>3.096</v>
+        <v>3.091</v>
       </c>
       <c r="H34" t="n">
-        <v>3.277</v>
+        <v>3.274</v>
       </c>
       <c r="I34" t="n">
-        <v>3.482</v>
+        <v>3.472</v>
       </c>
       <c r="J34" t="n">
-        <v>3.812</v>
+        <v>3.786</v>
       </c>
       <c r="K34" t="n">
+        <v>4.087</v>
+      </c>
+      <c r="L34" t="n">
         <v>4.129</v>
       </c>
-      <c r="L34" t="n">
-        <v>4.171</v>
-      </c>
       <c r="M34" t="n">
-        <v>4.314</v>
+        <v>4.273</v>
       </c>
       <c r="N34" t="n">
-        <v>4.354</v>
+        <v>4.327</v>
       </c>
       <c r="O34" t="n">
-        <v>4.479</v>
+        <v>4.46</v>
       </c>
       <c r="P34" t="n">
-        <v>4.689</v>
+        <v>4.674</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.547</v>
+        <v>5.537</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.997</v>
+        <v>2.991</v>
       </c>
       <c r="G35" t="n">
-        <v>3.07</v>
+        <v>3.065</v>
       </c>
       <c r="H35" t="n">
-        <v>3.245</v>
+        <v>3.242</v>
       </c>
       <c r="I35" t="n">
-        <v>3.449</v>
+        <v>3.438</v>
       </c>
       <c r="J35" t="n">
-        <v>3.781</v>
+        <v>3.754</v>
       </c>
       <c r="K35" t="n">
-        <v>4.083</v>
+        <v>4.041</v>
       </c>
       <c r="L35" t="n">
-        <v>4.126</v>
+        <v>4.084</v>
       </c>
       <c r="M35" t="n">
-        <v>4.261</v>
+        <v>4.22</v>
       </c>
       <c r="N35" t="n">
-        <v>4.29</v>
+        <v>4.263</v>
       </c>
       <c r="O35" t="n">
-        <v>4.376</v>
+        <v>4.357</v>
       </c>
       <c r="P35" t="n">
-        <v>4.492</v>
+        <v>4.477</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.183</v>
+        <v>5.173</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.895</v>
+        <v>2.889</v>
       </c>
       <c r="G36" t="n">
-        <v>2.97</v>
+        <v>2.964</v>
       </c>
       <c r="H36" t="n">
-        <v>3.135</v>
+        <v>3.131</v>
       </c>
       <c r="I36" t="n">
-        <v>3.336</v>
+        <v>3.324</v>
       </c>
       <c r="J36" t="n">
-        <v>3.676</v>
+        <v>3.649</v>
       </c>
       <c r="K36" t="n">
-        <v>3.977</v>
+        <v>3.935</v>
       </c>
       <c r="L36" t="n">
-        <v>4.017</v>
+        <v>3.975</v>
       </c>
       <c r="M36" t="n">
-        <v>4.128</v>
+        <v>4.087</v>
       </c>
       <c r="N36" t="n">
-        <v>4.156</v>
+        <v>4.13</v>
       </c>
       <c r="O36" t="n">
-        <v>4.221</v>
+        <v>4.203</v>
       </c>
       <c r="P36" t="n">
-        <v>4.294</v>
+        <v>4.279</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.563</v>
+        <v>4.553</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.767</v>
+        <v>3.762</v>
       </c>
       <c r="G37" t="n">
-        <v>4.235</v>
+        <v>4.231</v>
       </c>
       <c r="H37" t="n">
-        <v>4.791</v>
+        <v>4.788</v>
       </c>
       <c r="I37" t="n">
-        <v>5.124</v>
+        <v>5.113</v>
       </c>
       <c r="J37" t="n">
-        <v>6.017</v>
+        <v>5.991</v>
       </c>
       <c r="K37" t="n">
-        <v>6.984</v>
+        <v>6.943</v>
       </c>
       <c r="L37" t="n">
-        <v>7.301</v>
+        <v>7.26</v>
       </c>
       <c r="M37" t="n">
-        <v>7.699</v>
+        <v>7.659</v>
       </c>
       <c r="N37" t="n">
-        <v>7.867</v>
+        <v>7.842</v>
       </c>
       <c r="O37" t="n">
-        <v>8.069000000000001</v>
+        <v>8.051</v>
       </c>
       <c r="P37" t="n">
-        <v>8.15</v>
+        <v>8.135</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.590999999999999</v>
+        <v>8.581</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.826</v>
+        <v>4.821</v>
       </c>
       <c r="G38" t="n">
-        <v>5.548</v>
+        <v>5.544</v>
       </c>
       <c r="H38" t="n">
-        <v>6.315</v>
+        <v>6.312</v>
       </c>
       <c r="I38" t="n">
-        <v>6.805</v>
+        <v>6.794</v>
       </c>
       <c r="J38" t="n">
-        <v>7.96</v>
+        <v>7.934</v>
       </c>
       <c r="K38" t="n">
-        <v>9.106</v>
+        <v>9.064</v>
       </c>
       <c r="L38" t="n">
-        <v>9.581</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.111</v>
+        <v>10.071</v>
       </c>
       <c r="N38" t="n">
-        <v>10.286</v>
+        <v>10.26</v>
       </c>
       <c r="O38" t="n">
-        <v>10.469</v>
+        <v>10.452</v>
       </c>
       <c r="P38" t="n">
-        <v>10.547</v>
+        <v>10.532</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.042</v>
+        <v>11.032</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.147</v>
+        <v>4.142</v>
       </c>
       <c r="G39" t="n">
-        <v>4.746</v>
+        <v>4.742</v>
       </c>
       <c r="H39" t="n">
-        <v>5.38</v>
+        <v>5.377</v>
       </c>
       <c r="I39" t="n">
-        <v>5.809</v>
+        <v>5.798</v>
       </c>
       <c r="J39" t="n">
-        <v>6.832</v>
+        <v>6.806</v>
       </c>
       <c r="K39" t="n">
-        <v>7.939</v>
+        <v>7.897</v>
       </c>
       <c r="L39" t="n">
-        <v>8.339</v>
+        <v>8.298</v>
       </c>
       <c r="M39" t="n">
-        <v>8.747</v>
+        <v>8.707000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.913</v>
+        <v>8.888</v>
       </c>
       <c r="O39" t="n">
-        <v>9.119999999999999</v>
+        <v>9.102</v>
       </c>
       <c r="P39" t="n">
-        <v>9.202</v>
+        <v>9.186999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.686999999999999</v>
+        <v>9.677</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.289</v>
+        <v>3.283</v>
       </c>
       <c r="G40" t="n">
-        <v>3.416</v>
+        <v>3.411</v>
       </c>
       <c r="H40" t="n">
-        <v>3.661</v>
+        <v>3.658</v>
       </c>
       <c r="I40" t="n">
-        <v>3.907</v>
+        <v>3.896</v>
       </c>
       <c r="J40" t="n">
-        <v>4.327</v>
+        <v>4.301</v>
       </c>
       <c r="K40" t="n">
-        <v>4.716</v>
+        <v>4.674</v>
       </c>
       <c r="L40" t="n">
-        <v>4.812</v>
+        <v>4.771</v>
       </c>
       <c r="M40" t="n">
-        <v>5.038</v>
+        <v>4.998</v>
       </c>
       <c r="N40" t="n">
-        <v>5.216</v>
+        <v>5.19</v>
       </c>
       <c r="O40" t="n">
-        <v>5.532</v>
+        <v>5.514</v>
       </c>
       <c r="P40" t="n">
-        <v>5.783</v>
+        <v>5.768</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.58</v>
+        <v>6.57</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.674</v>
+        <v>3.669</v>
       </c>
       <c r="G41" t="n">
-        <v>3.844</v>
+        <v>3.84</v>
       </c>
       <c r="H41" t="n">
-        <v>4.145</v>
+        <v>4.142</v>
       </c>
       <c r="I41" t="n">
-        <v>4.411</v>
+        <v>4.399</v>
       </c>
       <c r="J41" t="n">
-        <v>4.882</v>
+        <v>4.856</v>
       </c>
       <c r="K41" t="n">
-        <v>5.316</v>
+        <v>5.274</v>
       </c>
       <c r="L41" t="n">
-        <v>5.491</v>
+        <v>5.45</v>
       </c>
       <c r="M41" t="n">
-        <v>5.84</v>
+        <v>5.8</v>
       </c>
       <c r="N41" t="n">
-        <v>6.146</v>
+        <v>6.121</v>
       </c>
       <c r="O41" t="n">
-        <v>6.647</v>
+        <v>6.63</v>
       </c>
       <c r="P41" t="n">
-        <v>6.842</v>
+        <v>6.827</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.627</v>
+        <v>7.617</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.41</v>
+        <v>3.404</v>
       </c>
       <c r="G42" t="n">
-        <v>3.565</v>
+        <v>3.56</v>
       </c>
       <c r="H42" t="n">
-        <v>3.836</v>
+        <v>3.833</v>
       </c>
       <c r="I42" t="n">
-        <v>4.096</v>
+        <v>4.084</v>
       </c>
       <c r="J42" t="n">
-        <v>4.529</v>
+        <v>4.503</v>
       </c>
       <c r="K42" t="n">
-        <v>4.937</v>
+        <v>4.895</v>
       </c>
       <c r="L42" t="n">
-        <v>5.048</v>
+        <v>5.007</v>
       </c>
       <c r="M42" t="n">
-        <v>5.345</v>
+        <v>5.305</v>
       </c>
       <c r="N42" t="n">
-        <v>5.631</v>
+        <v>5.604</v>
       </c>
       <c r="O42" t="n">
-        <v>6.024</v>
+        <v>6.006</v>
       </c>
       <c r="P42" t="n">
-        <v>6.285</v>
+        <v>6.27</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.093</v>
+        <v>7.083</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.111</v>
+        <v>3.105</v>
       </c>
       <c r="G43" t="n">
-        <v>3.226</v>
+        <v>3.221</v>
       </c>
       <c r="H43" t="n">
-        <v>3.417</v>
+        <v>3.414</v>
       </c>
       <c r="I43" t="n">
-        <v>3.624</v>
+        <v>3.613</v>
       </c>
       <c r="J43" t="n">
-        <v>3.969</v>
+        <v>3.942</v>
       </c>
       <c r="K43" t="n">
-        <v>4.283</v>
+        <v>4.241</v>
       </c>
       <c r="L43" t="n">
-        <v>4.333</v>
+        <v>4.291</v>
       </c>
       <c r="M43" t="n">
-        <v>4.477</v>
+        <v>4.436</v>
       </c>
       <c r="N43" t="n">
-        <v>4.518</v>
+        <v>4.491</v>
       </c>
       <c r="O43" t="n">
-        <v>4.622</v>
+        <v>4.604</v>
       </c>
       <c r="P43" t="n">
-        <v>4.761</v>
+        <v>4.746</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.456</v>
+        <v>5.446</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.973</v>
+        <v>2.967</v>
       </c>
       <c r="G44" t="n">
-        <v>3.079</v>
+        <v>3.073</v>
       </c>
       <c r="H44" t="n">
-        <v>3.259</v>
+        <v>3.255</v>
       </c>
       <c r="I44" t="n">
-        <v>3.464</v>
+        <v>3.452</v>
       </c>
       <c r="J44" t="n">
-        <v>3.818</v>
+        <v>3.79</v>
       </c>
       <c r="K44" t="n">
-        <v>4.127</v>
+        <v>4.085</v>
       </c>
       <c r="L44" t="n">
-        <v>4.177</v>
+        <v>4.135</v>
       </c>
       <c r="M44" t="n">
-        <v>4.296</v>
+        <v>4.255</v>
       </c>
       <c r="N44" t="n">
-        <v>4.337</v>
+        <v>4.311</v>
       </c>
       <c r="O44" t="n">
-        <v>4.421</v>
+        <v>4.403</v>
       </c>
       <c r="P44" t="n">
-        <v>4.524</v>
+        <v>4.509</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.827</v>
+        <v>4.817</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-14 ~ 2026-05-14
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.177</v>
+        <v>3.179</v>
       </c>
       <c r="G2" t="n">
-        <v>3.402</v>
+        <v>3.405</v>
       </c>
       <c r="H2" t="n">
-        <v>3.645</v>
+        <v>3.653</v>
       </c>
       <c r="I2" t="n">
-        <v>3.823</v>
+        <v>3.835</v>
       </c>
       <c r="J2" t="n">
-        <v>4.142</v>
+        <v>4.164</v>
       </c>
       <c r="K2" t="n">
-        <v>4.586</v>
+        <v>4.592</v>
       </c>
       <c r="L2" t="n">
-        <v>4.756</v>
+        <v>4.771</v>
       </c>
       <c r="M2" t="n">
-        <v>5.089</v>
+        <v>5.1</v>
       </c>
       <c r="N2" t="n">
-        <v>5.392</v>
+        <v>5.412</v>
       </c>
       <c r="O2" t="n">
-        <v>5.649</v>
+        <v>5.678</v>
       </c>
       <c r="P2" t="n">
-        <v>5.872</v>
+        <v>5.901</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.516</v>
+        <v>6.548</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.201</v>
+        <v>4.203</v>
       </c>
       <c r="G3" t="n">
-        <v>4.607</v>
+        <v>4.61</v>
       </c>
       <c r="H3" t="n">
-        <v>4.883</v>
+        <v>4.891</v>
       </c>
       <c r="I3" t="n">
-        <v>5.056</v>
+        <v>5.068</v>
       </c>
       <c r="J3" t="n">
-        <v>5.388</v>
+        <v>5.41</v>
       </c>
       <c r="K3" t="n">
-        <v>5.902</v>
+        <v>5.908</v>
       </c>
       <c r="L3" t="n">
-        <v>6.141</v>
+        <v>6.157</v>
       </c>
       <c r="M3" t="n">
-        <v>6.506</v>
+        <v>6.517</v>
       </c>
       <c r="N3" t="n">
-        <v>6.751</v>
+        <v>6.771</v>
       </c>
       <c r="O3" t="n">
-        <v>6.959</v>
+        <v>6.988</v>
       </c>
       <c r="P3" t="n">
-        <v>7.052</v>
+        <v>7.082</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.585</v>
+        <v>7.617</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.693</v>
+        <v>3.695</v>
       </c>
       <c r="G4" t="n">
-        <v>3.988</v>
+        <v>3.991</v>
       </c>
       <c r="H4" t="n">
-        <v>4.292</v>
+        <v>4.3</v>
       </c>
       <c r="I4" t="n">
-        <v>4.499</v>
+        <v>4.511</v>
       </c>
       <c r="J4" t="n">
-        <v>4.834</v>
+        <v>4.856</v>
       </c>
       <c r="K4" t="n">
-        <v>5.341</v>
+        <v>5.346</v>
       </c>
       <c r="L4" t="n">
-        <v>5.51</v>
+        <v>5.525</v>
       </c>
       <c r="M4" t="n">
-        <v>5.864</v>
+        <v>5.875</v>
       </c>
       <c r="N4" t="n">
-        <v>6.079</v>
+        <v>6.099</v>
       </c>
       <c r="O4" t="n">
-        <v>6.31</v>
+        <v>6.339</v>
       </c>
       <c r="P4" t="n">
-        <v>6.402</v>
+        <v>6.432</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.938</v>
+        <v>6.97</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.872</v>
+        <v>2.874</v>
       </c>
       <c r="G5" t="n">
-        <v>2.946</v>
+        <v>2.949</v>
       </c>
       <c r="H5" t="n">
-        <v>3.149</v>
+        <v>3.158</v>
       </c>
       <c r="I5" t="n">
-        <v>3.392</v>
+        <v>3.405</v>
       </c>
       <c r="J5" t="n">
-        <v>3.702</v>
+        <v>3.724</v>
       </c>
       <c r="K5" t="n">
-        <v>3.996</v>
+        <v>3.998</v>
       </c>
       <c r="L5" t="n">
-        <v>4.011</v>
+        <v>4.022</v>
       </c>
       <c r="M5" t="n">
-        <v>4.147</v>
+        <v>4.157</v>
       </c>
       <c r="N5" t="n">
-        <v>4.206</v>
+        <v>4.224</v>
       </c>
       <c r="O5" t="n">
-        <v>4.248</v>
+        <v>4.277</v>
       </c>
       <c r="P5" t="n">
-        <v>4.54</v>
+        <v>4.57</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.429</v>
+        <v>5.461</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.911</v>
+        <v>2.913</v>
       </c>
       <c r="G6" t="n">
-        <v>2.999</v>
+        <v>3.002</v>
       </c>
       <c r="H6" t="n">
-        <v>3.218</v>
+        <v>3.227</v>
       </c>
       <c r="I6" t="n">
-        <v>3.475</v>
+        <v>3.488</v>
       </c>
       <c r="J6" t="n">
-        <v>3.79</v>
+        <v>3.812</v>
       </c>
       <c r="K6" t="n">
-        <v>4.106</v>
+        <v>4.108</v>
       </c>
       <c r="L6" t="n">
-        <v>4.125</v>
+        <v>4.137</v>
       </c>
       <c r="M6" t="n">
-        <v>4.303</v>
+        <v>4.313</v>
       </c>
       <c r="N6" t="n">
-        <v>4.373</v>
+        <v>4.392</v>
       </c>
       <c r="O6" t="n">
-        <v>4.515</v>
+        <v>4.544</v>
       </c>
       <c r="P6" t="n">
-        <v>4.973</v>
+        <v>5.003</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.825</v>
+        <v>5.857</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.892</v>
+        <v>2.894</v>
       </c>
       <c r="G7" t="n">
-        <v>2.963</v>
+        <v>2.966</v>
       </c>
       <c r="H7" t="n">
-        <v>3.164</v>
+        <v>3.173</v>
       </c>
       <c r="I7" t="n">
-        <v>3.41</v>
+        <v>3.423</v>
       </c>
       <c r="J7" t="n">
-        <v>3.726</v>
+        <v>3.748</v>
       </c>
       <c r="K7" t="n">
-        <v>4.023</v>
+        <v>4.025</v>
       </c>
       <c r="L7" t="n">
-        <v>4.035</v>
+        <v>4.047</v>
       </c>
       <c r="M7" t="n">
-        <v>4.209</v>
+        <v>4.218</v>
       </c>
       <c r="N7" t="n">
-        <v>4.265</v>
+        <v>4.284</v>
       </c>
       <c r="O7" t="n">
-        <v>4.413</v>
+        <v>4.442</v>
       </c>
       <c r="P7" t="n">
-        <v>4.756</v>
+        <v>4.786</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.592</v>
+        <v>5.624</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.313</v>
+        <v>5.314</v>
       </c>
       <c r="G8" t="n">
-        <v>5.907</v>
+        <v>5.91</v>
       </c>
       <c r="H8" t="n">
-        <v>6.331</v>
+        <v>6.339</v>
       </c>
       <c r="I8" t="n">
-        <v>6.582</v>
+        <v>6.594</v>
       </c>
       <c r="J8" t="n">
-        <v>6.98</v>
+        <v>7.002</v>
       </c>
       <c r="K8" t="n">
-        <v>7.774</v>
+        <v>7.78</v>
       </c>
       <c r="L8" t="n">
-        <v>8.1</v>
+        <v>8.115</v>
       </c>
       <c r="M8" t="n">
-        <v>8.494999999999999</v>
+        <v>8.506</v>
       </c>
       <c r="N8" t="n">
-        <v>8.676</v>
+        <v>8.695</v>
       </c>
       <c r="O8" t="n">
-        <v>8.968</v>
+        <v>8.997</v>
       </c>
       <c r="P8" t="n">
-        <v>9.163</v>
+        <v>9.193</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.894</v>
+        <v>9.926</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.613</v>
+        <v>2.614</v>
       </c>
       <c r="G9" t="n">
-        <v>2.707</v>
+        <v>2.712</v>
       </c>
       <c r="H9" t="n">
-        <v>2.841</v>
+        <v>2.857</v>
       </c>
       <c r="I9" t="n">
-        <v>3.098</v>
+        <v>3.121</v>
       </c>
       <c r="J9" t="n">
-        <v>3.294</v>
+        <v>3.3</v>
       </c>
       <c r="K9" t="n">
-        <v>3.504</v>
+        <v>3.505</v>
       </c>
       <c r="L9" t="n">
-        <v>3.53</v>
+        <v>3.548</v>
       </c>
       <c r="M9" t="n">
-        <v>3.642</v>
+        <v>3.657</v>
       </c>
       <c r="N9" t="n">
-        <v>3.81</v>
+        <v>3.831</v>
       </c>
       <c r="O9" t="n">
-        <v>3.86</v>
+        <v>3.889</v>
       </c>
       <c r="P9" t="n">
-        <v>3.971</v>
+        <v>4</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.054</v>
+        <v>4.086</v>
       </c>
       <c r="R9" t="n">
-        <v>4.055</v>
+        <v>4.09</v>
       </c>
       <c r="S9" t="n">
-        <v>4.051</v>
+        <v>4.09</v>
       </c>
       <c r="T9" t="n">
-        <v>3.97</v>
+        <v>4</v>
       </c>
       <c r="U9" t="n">
-        <v>3.841</v>
+        <v>3.871</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.627</v>
+        <v>2.629</v>
       </c>
       <c r="G10" t="n">
-        <v>2.738</v>
+        <v>2.744</v>
       </c>
       <c r="H10" t="n">
-        <v>2.854</v>
+        <v>2.87</v>
       </c>
       <c r="I10" t="n">
-        <v>3.103</v>
+        <v>3.126</v>
       </c>
       <c r="J10" t="n">
-        <v>3.319</v>
+        <v>3.324</v>
       </c>
       <c r="K10" t="n">
-        <v>3.537</v>
+        <v>3.538</v>
       </c>
       <c r="L10" t="n">
-        <v>3.578</v>
+        <v>3.596</v>
       </c>
       <c r="M10" t="n">
-        <v>3.736</v>
+        <v>3.752</v>
       </c>
       <c r="N10" t="n">
-        <v>3.829</v>
+        <v>3.85</v>
       </c>
       <c r="O10" t="n">
-        <v>4.053</v>
+        <v>4.083</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.442</v>
+        <v>2.444</v>
       </c>
       <c r="G11" t="n">
-        <v>2.548</v>
+        <v>2.554</v>
       </c>
       <c r="H11" t="n">
-        <v>2.677</v>
+        <v>2.693</v>
       </c>
       <c r="I11" t="n">
-        <v>2.907</v>
+        <v>2.93</v>
       </c>
       <c r="J11" t="n">
-        <v>3.117</v>
+        <v>3.122</v>
       </c>
       <c r="K11" t="n">
         <v>3.325</v>
       </c>
       <c r="L11" t="n">
-        <v>3.375</v>
+        <v>3.393</v>
       </c>
       <c r="M11" t="n">
-        <v>3.544</v>
+        <v>3.559</v>
       </c>
       <c r="N11" t="n">
-        <v>3.637</v>
+        <v>3.659</v>
       </c>
       <c r="O11" t="n">
-        <v>3.82</v>
+        <v>3.85</v>
       </c>
       <c r="P11" t="n">
-        <v>3.921</v>
+        <v>3.951</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.256</v>
+        <v>4.288</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.189</v>
+        <v>3.192</v>
       </c>
       <c r="G12" t="n">
-        <v>3.369</v>
+        <v>3.374</v>
       </c>
       <c r="H12" t="n">
-        <v>3.55</v>
+        <v>3.57</v>
       </c>
       <c r="I12" t="n">
-        <v>3.79</v>
+        <v>3.804</v>
       </c>
       <c r="J12" t="n">
-        <v>4.144</v>
+        <v>4.162</v>
       </c>
       <c r="K12" t="n">
-        <v>4.381</v>
+        <v>4.39</v>
       </c>
       <c r="L12" t="n">
-        <v>4.44</v>
+        <v>4.456</v>
       </c>
       <c r="M12" t="n">
-        <v>4.614</v>
+        <v>4.628</v>
       </c>
       <c r="N12" t="n">
-        <v>4.689</v>
+        <v>4.711</v>
       </c>
       <c r="O12" t="n">
-        <v>4.853</v>
+        <v>4.88</v>
       </c>
       <c r="P12" t="n">
-        <v>5.009</v>
+        <v>5.039</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.373</v>
+        <v>5.405</v>
       </c>
       <c r="R12" t="n">
-        <v>5.548</v>
+        <v>5.583</v>
       </c>
       <c r="S12" t="n">
-        <v>5.757</v>
+        <v>5.794</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.943</v>
+        <v>2.945</v>
       </c>
       <c r="G13" t="n">
-        <v>3.059</v>
+        <v>3.064</v>
       </c>
       <c r="H13" t="n">
-        <v>3.218</v>
+        <v>3.238</v>
       </c>
       <c r="I13" t="n">
-        <v>3.437</v>
+        <v>3.451</v>
       </c>
       <c r="J13" t="n">
-        <v>3.781</v>
+        <v>3.799</v>
       </c>
       <c r="K13" t="n">
-        <v>4.014</v>
+        <v>4.023</v>
       </c>
       <c r="L13" t="n">
-        <v>4.079</v>
+        <v>4.095</v>
       </c>
       <c r="M13" t="n">
-        <v>4.241</v>
+        <v>4.256</v>
       </c>
       <c r="N13" t="n">
-        <v>4.318</v>
+        <v>4.339</v>
       </c>
       <c r="O13" t="n">
-        <v>4.481</v>
+        <v>4.509</v>
       </c>
       <c r="P13" t="n">
-        <v>4.601</v>
+        <v>4.63</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.895</v>
+        <v>4.926</v>
       </c>
       <c r="R13" t="n">
-        <v>5.098</v>
+        <v>5.133</v>
       </c>
       <c r="S13" t="n">
-        <v>5.319</v>
+        <v>5.357</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.762</v>
+        <v>2.764</v>
       </c>
       <c r="G14" t="n">
-        <v>2.865</v>
+        <v>2.869</v>
       </c>
       <c r="H14" t="n">
-        <v>3.021</v>
+        <v>3.041</v>
       </c>
       <c r="I14" t="n">
-        <v>3.221</v>
+        <v>3.235</v>
       </c>
       <c r="J14" t="n">
-        <v>3.521</v>
+        <v>3.54</v>
       </c>
       <c r="K14" t="n">
-        <v>3.702</v>
+        <v>3.711</v>
       </c>
       <c r="L14" t="n">
-        <v>3.751</v>
+        <v>3.768</v>
       </c>
       <c r="M14" t="n">
-        <v>3.926</v>
+        <v>3.942</v>
       </c>
       <c r="N14" t="n">
-        <v>3.996</v>
+        <v>4.018</v>
       </c>
       <c r="O14" t="n">
-        <v>4.137</v>
+        <v>4.166</v>
       </c>
       <c r="P14" t="n">
-        <v>4.236</v>
+        <v>4.265</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.484</v>
+        <v>4.515</v>
       </c>
       <c r="R14" t="n">
-        <v>4.612</v>
+        <v>4.647</v>
       </c>
       <c r="S14" t="n">
-        <v>4.772</v>
+        <v>4.809</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.74</v>
+        <v>2.742</v>
       </c>
       <c r="G15" t="n">
-        <v>2.839</v>
+        <v>2.844</v>
       </c>
       <c r="H15" t="n">
-        <v>2.992</v>
+        <v>3.012</v>
       </c>
       <c r="I15" t="n">
-        <v>3.172</v>
+        <v>3.186</v>
       </c>
       <c r="J15" t="n">
-        <v>3.46</v>
+        <v>3.479</v>
       </c>
       <c r="K15" t="n">
-        <v>3.654</v>
+        <v>3.664</v>
       </c>
       <c r="L15" t="n">
-        <v>3.687</v>
+        <v>3.703</v>
       </c>
       <c r="M15" t="n">
-        <v>3.839</v>
+        <v>3.854</v>
       </c>
       <c r="N15" t="n">
-        <v>3.9</v>
+        <v>3.922</v>
       </c>
       <c r="O15" t="n">
-        <v>4.078</v>
+        <v>4.108</v>
       </c>
       <c r="P15" t="n">
-        <v>4.136</v>
+        <v>4.165</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.386</v>
+        <v>4.418</v>
       </c>
       <c r="R15" t="n">
-        <v>4.508</v>
+        <v>4.542</v>
       </c>
       <c r="S15" t="n">
-        <v>4.667</v>
+        <v>4.705</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.74</v>
+        <v>2.742</v>
       </c>
       <c r="G16" t="n">
-        <v>2.839</v>
+        <v>2.844</v>
       </c>
       <c r="H16" t="n">
-        <v>2.992</v>
+        <v>3.012</v>
       </c>
       <c r="I16" t="n">
-        <v>3.172</v>
+        <v>3.186</v>
       </c>
       <c r="J16" t="n">
-        <v>3.46</v>
+        <v>3.479</v>
       </c>
       <c r="K16" t="n">
-        <v>3.654</v>
+        <v>3.664</v>
       </c>
       <c r="L16" t="n">
-        <v>3.687</v>
+        <v>3.703</v>
       </c>
       <c r="M16" t="n">
-        <v>3.839</v>
+        <v>3.854</v>
       </c>
       <c r="N16" t="n">
-        <v>3.903</v>
+        <v>3.925</v>
       </c>
       <c r="O16" t="n">
-        <v>4.085</v>
+        <v>4.114</v>
       </c>
       <c r="P16" t="n">
-        <v>4.159</v>
+        <v>4.189</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.414</v>
+        <v>4.445</v>
       </c>
       <c r="R16" t="n">
-        <v>4.536</v>
+        <v>4.57</v>
       </c>
       <c r="S16" t="n">
-        <v>4.696</v>
+        <v>4.734</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.689</v>
+        <v>2.691</v>
       </c>
       <c r="G17" t="n">
-        <v>2.829</v>
+        <v>2.835</v>
       </c>
       <c r="H17" t="n">
-        <v>2.948</v>
+        <v>2.963</v>
       </c>
       <c r="I17" t="n">
-        <v>3.185</v>
+        <v>3.206</v>
       </c>
       <c r="J17" t="n">
-        <v>3.395</v>
+        <v>3.4</v>
       </c>
       <c r="K17" t="n">
-        <v>3.614</v>
+        <v>3.615</v>
       </c>
       <c r="L17" t="n">
-        <v>3.662</v>
+        <v>3.678</v>
       </c>
       <c r="M17" t="n">
-        <v>3.858</v>
+        <v>3.875</v>
       </c>
       <c r="N17" t="n">
-        <v>3.931</v>
+        <v>3.953</v>
       </c>
       <c r="O17" t="n">
-        <v>4.083</v>
+        <v>4.113</v>
       </c>
       <c r="P17" t="n">
-        <v>4.199</v>
+        <v>4.23</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.69</v>
+        <v>2.692</v>
       </c>
       <c r="G18" t="n">
-        <v>2.83</v>
+        <v>2.836</v>
       </c>
       <c r="H18" t="n">
-        <v>2.948</v>
+        <v>2.963</v>
       </c>
       <c r="I18" t="n">
-        <v>3.185</v>
+        <v>3.207</v>
       </c>
       <c r="J18" t="n">
-        <v>3.395</v>
+        <v>3.4</v>
       </c>
       <c r="K18" t="n">
-        <v>3.615</v>
+        <v>3.616</v>
       </c>
       <c r="L18" t="n">
-        <v>3.662</v>
+        <v>3.678</v>
       </c>
       <c r="M18" t="n">
-        <v>3.858</v>
+        <v>3.875</v>
       </c>
       <c r="N18" t="n">
-        <v>3.932</v>
+        <v>3.953</v>
       </c>
       <c r="O18" t="n">
-        <v>4.08</v>
+        <v>4.11</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.753</v>
+        <v>2.756</v>
       </c>
       <c r="G19" t="n">
-        <v>2.855</v>
+        <v>2.859</v>
       </c>
       <c r="H19" t="n">
-        <v>3.01</v>
+        <v>3.029</v>
       </c>
       <c r="I19" t="n">
-        <v>3.208</v>
+        <v>3.221</v>
       </c>
       <c r="J19" t="n">
-        <v>3.504</v>
+        <v>3.522</v>
       </c>
       <c r="K19" t="n">
-        <v>3.698</v>
+        <v>3.707</v>
       </c>
       <c r="L19" t="n">
-        <v>3.748</v>
+        <v>3.764</v>
       </c>
       <c r="M19" t="n">
-        <v>3.917</v>
+        <v>3.932</v>
       </c>
       <c r="N19" t="n">
-        <v>3.985</v>
+        <v>4.008</v>
       </c>
       <c r="O19" t="n">
-        <v>4.12</v>
+        <v>4.15</v>
       </c>
       <c r="P19" t="n">
-        <v>4.195</v>
+        <v>4.224</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.425</v>
+        <v>4.456</v>
       </c>
       <c r="R19" t="n">
-        <v>4.556</v>
+        <v>4.59</v>
       </c>
       <c r="S19" t="n">
-        <v>4.707</v>
+        <v>4.744</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.589</v>
+        <v>2.59</v>
       </c>
       <c r="G20" t="n">
-        <v>2.669</v>
+        <v>2.67</v>
       </c>
       <c r="H20" t="n">
-        <v>2.735</v>
+        <v>2.738</v>
       </c>
       <c r="I20" t="n">
-        <v>2.858</v>
+        <v>2.86</v>
       </c>
       <c r="J20" t="n">
-        <v>3.29</v>
+        <v>3.31</v>
       </c>
       <c r="K20" t="n">
-        <v>3.53</v>
+        <v>3.54</v>
       </c>
       <c r="L20" t="n">
-        <v>3.573</v>
+        <v>3.583</v>
       </c>
       <c r="M20" t="n">
-        <v>3.681</v>
+        <v>3.694</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.877</v>
+        <v>2.879</v>
       </c>
       <c r="G21" t="n">
-        <v>2.96</v>
+        <v>2.962</v>
       </c>
       <c r="H21" t="n">
-        <v>3.152</v>
+        <v>3.16</v>
       </c>
       <c r="I21" t="n">
-        <v>3.318</v>
+        <v>3.328</v>
       </c>
       <c r="J21" t="n">
-        <v>3.649</v>
+        <v>3.669</v>
       </c>
       <c r="K21" t="n">
-        <v>3.932</v>
+        <v>3.941</v>
       </c>
       <c r="L21" t="n">
-        <v>3.989</v>
+        <v>4.005</v>
       </c>
       <c r="M21" t="n">
-        <v>4.143</v>
+        <v>4.156</v>
       </c>
       <c r="N21" t="n">
-        <v>4.228</v>
+        <v>4.248</v>
       </c>
       <c r="O21" t="n">
-        <v>4.332</v>
+        <v>4.361</v>
       </c>
       <c r="P21" t="n">
-        <v>4.46</v>
+        <v>4.488</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.592</v>
+        <v>4.621</v>
       </c>
       <c r="R21" t="n">
-        <v>4.607</v>
+        <v>4.642</v>
       </c>
       <c r="S21" t="n">
-        <v>4.668</v>
+        <v>4.705</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.824</v>
+        <v>2.826</v>
       </c>
       <c r="G22" t="n">
-        <v>2.905</v>
+        <v>2.908</v>
       </c>
       <c r="H22" t="n">
-        <v>3.084</v>
+        <v>3.091</v>
       </c>
       <c r="I22" t="n">
-        <v>3.237</v>
+        <v>3.247</v>
       </c>
       <c r="J22" t="n">
-        <v>3.535</v>
+        <v>3.555</v>
       </c>
       <c r="K22" t="n">
-        <v>3.814</v>
+        <v>3.823</v>
       </c>
       <c r="L22" t="n">
-        <v>3.856</v>
+        <v>3.872</v>
       </c>
       <c r="M22" t="n">
-        <v>4.013</v>
+        <v>4.026</v>
       </c>
       <c r="N22" t="n">
-        <v>4.1</v>
+        <v>4.121</v>
       </c>
       <c r="O22" t="n">
-        <v>4.2</v>
+        <v>4.229</v>
       </c>
       <c r="P22" t="n">
-        <v>4.322</v>
+        <v>4.35</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.45</v>
+        <v>4.48</v>
       </c>
       <c r="R22" t="n">
-        <v>4.456</v>
+        <v>4.49</v>
       </c>
       <c r="S22" t="n">
-        <v>4.514</v>
+        <v>4.55</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.776</v>
+        <v>2.778</v>
       </c>
       <c r="G23" t="n">
-        <v>2.86</v>
+        <v>2.863</v>
       </c>
       <c r="H23" t="n">
-        <v>3.024</v>
+        <v>3.033</v>
       </c>
       <c r="I23" t="n">
-        <v>3.188</v>
+        <v>3.197</v>
       </c>
       <c r="J23" t="n">
-        <v>3.477</v>
+        <v>3.497</v>
       </c>
       <c r="K23" t="n">
-        <v>3.715</v>
+        <v>3.724</v>
       </c>
       <c r="L23" t="n">
-        <v>3.755</v>
+        <v>3.771</v>
       </c>
       <c r="M23" t="n">
-        <v>3.906</v>
+        <v>3.919</v>
       </c>
       <c r="N23" t="n">
-        <v>3.996</v>
+        <v>4.016</v>
       </c>
       <c r="O23" t="n">
-        <v>4.077</v>
+        <v>4.106</v>
       </c>
       <c r="P23" t="n">
-        <v>4.187</v>
+        <v>4.215</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.256</v>
+        <v>4.286</v>
       </c>
       <c r="R23" t="n">
-        <v>4.24</v>
+        <v>4.274</v>
       </c>
       <c r="S23" t="n">
-        <v>4.268</v>
+        <v>4.304</v>
       </c>
       <c r="T23" t="n">
-        <v>4.179</v>
+        <v>4.208</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.712</v>
+        <v>2.714</v>
       </c>
       <c r="G24" t="n">
-        <v>2.776</v>
+        <v>2.779</v>
       </c>
       <c r="H24" t="n">
-        <v>2.925</v>
+        <v>2.933</v>
       </c>
       <c r="I24" t="n">
-        <v>3.103</v>
+        <v>3.122</v>
       </c>
       <c r="J24" t="n">
-        <v>3.377</v>
+        <v>3.395</v>
       </c>
       <c r="K24" t="n">
-        <v>3.601</v>
+        <v>3.609</v>
       </c>
       <c r="L24" t="n">
-        <v>3.637</v>
+        <v>3.652</v>
       </c>
       <c r="M24" t="n">
-        <v>3.77</v>
+        <v>3.783</v>
       </c>
       <c r="N24" t="n">
-        <v>3.873</v>
+        <v>3.893</v>
       </c>
       <c r="O24" t="n">
-        <v>4.069</v>
+        <v>4.098</v>
       </c>
       <c r="P24" t="n">
-        <v>4.126</v>
+        <v>4.154</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.181</v>
+        <v>4.211</v>
       </c>
       <c r="R24" t="n">
-        <v>4.161</v>
+        <v>4.196</v>
       </c>
       <c r="S24" t="n">
-        <v>4.183</v>
+        <v>4.219</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.77</v>
+        <v>2.772</v>
       </c>
       <c r="G25" t="n">
-        <v>2.86</v>
+        <v>2.863</v>
       </c>
       <c r="H25" t="n">
-        <v>3.027</v>
+        <v>3.036</v>
       </c>
       <c r="I25" t="n">
-        <v>3.196</v>
+        <v>3.204</v>
       </c>
       <c r="J25" t="n">
-        <v>3.493</v>
+        <v>3.513</v>
       </c>
       <c r="K25" t="n">
-        <v>3.747</v>
+        <v>3.756</v>
       </c>
       <c r="L25" t="n">
-        <v>3.786</v>
+        <v>3.801</v>
       </c>
       <c r="M25" t="n">
-        <v>3.938</v>
+        <v>3.95</v>
       </c>
       <c r="N25" t="n">
-        <v>4.022</v>
+        <v>4.043</v>
       </c>
       <c r="O25" t="n">
-        <v>4.106</v>
+        <v>4.135</v>
       </c>
       <c r="P25" t="n">
-        <v>4.209</v>
+        <v>4.237</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.29</v>
+        <v>4.319</v>
       </c>
       <c r="R25" t="n">
-        <v>4.263</v>
+        <v>4.298</v>
       </c>
       <c r="S25" t="n">
-        <v>4.291</v>
+        <v>4.328</v>
       </c>
       <c r="T25" t="n">
-        <v>4.197</v>
+        <v>4.226</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.046</v>
+        <v>3.045</v>
       </c>
       <c r="G26" t="n">
-        <v>3.192</v>
+        <v>3.195</v>
       </c>
       <c r="H26" t="n">
-        <v>3.462</v>
+        <v>3.467</v>
       </c>
       <c r="I26" t="n">
-        <v>3.691</v>
+        <v>3.701</v>
       </c>
       <c r="J26" t="n">
-        <v>4.134</v>
+        <v>4.152</v>
       </c>
       <c r="K26" t="n">
-        <v>4.569</v>
+        <v>4.574</v>
       </c>
       <c r="L26" t="n">
-        <v>4.668</v>
+        <v>4.682</v>
       </c>
       <c r="M26" t="n">
-        <v>4.886</v>
+        <v>4.896</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.187</v>
+        <v>5.213</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.851</v>
+        <v>2.852</v>
       </c>
       <c r="G27" t="n">
-        <v>2.941</v>
+        <v>2.944</v>
       </c>
       <c r="H27" t="n">
-        <v>3.112</v>
+        <v>3.125</v>
       </c>
       <c r="I27" t="n">
-        <v>3.314</v>
+        <v>3.327</v>
       </c>
       <c r="J27" t="n">
-        <v>3.639</v>
+        <v>3.656</v>
       </c>
       <c r="K27" t="n">
-        <v>3.883</v>
+        <v>3.889</v>
       </c>
       <c r="L27" t="n">
-        <v>3.937</v>
+        <v>3.951</v>
       </c>
       <c r="M27" t="n">
-        <v>4.094</v>
+        <v>4.107</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.277</v>
+        <v>4.305</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.954</v>
+        <v>2.955</v>
       </c>
       <c r="G28" t="n">
-        <v>3.052</v>
+        <v>3.055</v>
       </c>
       <c r="H28" t="n">
-        <v>3.238</v>
+        <v>3.251</v>
       </c>
       <c r="I28" t="n">
-        <v>3.452</v>
+        <v>3.465</v>
       </c>
       <c r="J28" t="n">
-        <v>3.813</v>
+        <v>3.828</v>
       </c>
       <c r="K28" t="n">
-        <v>4.075</v>
+        <v>4.081</v>
       </c>
       <c r="L28" t="n">
-        <v>4.14</v>
+        <v>4.154</v>
       </c>
       <c r="M28" t="n">
-        <v>4.306</v>
+        <v>4.319</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.57</v>
+        <v>4.597</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.801</v>
+        <v>2.802</v>
       </c>
       <c r="G29" t="n">
-        <v>2.891</v>
+        <v>2.894</v>
       </c>
       <c r="H29" t="n">
-        <v>3.053</v>
+        <v>3.066</v>
       </c>
       <c r="I29" t="n">
-        <v>3.244</v>
+        <v>3.257</v>
       </c>
       <c r="J29" t="n">
-        <v>3.552</v>
+        <v>3.568</v>
       </c>
       <c r="K29" t="n">
-        <v>3.778</v>
+        <v>3.784</v>
       </c>
       <c r="L29" t="n">
-        <v>3.822</v>
+        <v>3.836</v>
       </c>
       <c r="M29" t="n">
-        <v>3.957</v>
+        <v>3.97</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.147</v>
+        <v>4.175</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.09</v>
+        <v>3.089</v>
       </c>
       <c r="G30" t="n">
-        <v>3.172</v>
+        <v>3.173</v>
       </c>
       <c r="H30" t="n">
-        <v>3.397</v>
+        <v>3.403</v>
       </c>
       <c r="I30" t="n">
-        <v>3.621</v>
+        <v>3.631</v>
       </c>
       <c r="J30" t="n">
-        <v>4.008</v>
+        <v>4.024</v>
       </c>
       <c r="K30" t="n">
-        <v>4.369</v>
+        <v>4.375</v>
       </c>
       <c r="L30" t="n">
-        <v>4.447</v>
+        <v>4.462</v>
       </c>
       <c r="M30" t="n">
-        <v>4.657</v>
+        <v>4.668</v>
       </c>
       <c r="N30" t="n">
-        <v>4.832</v>
+        <v>4.851</v>
       </c>
       <c r="O30" t="n">
-        <v>5.136</v>
+        <v>5.164</v>
       </c>
       <c r="P30" t="n">
-        <v>5.346</v>
+        <v>5.377</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.119</v>
+        <v>6.151</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.419</v>
+        <v>3.418</v>
       </c>
       <c r="G31" t="n">
-        <v>3.537</v>
+        <v>3.538</v>
       </c>
       <c r="H31" t="n">
-        <v>3.812</v>
+        <v>3.817</v>
       </c>
       <c r="I31" t="n">
-        <v>4.05</v>
+        <v>4.06</v>
       </c>
       <c r="J31" t="n">
-        <v>4.5</v>
+        <v>4.516</v>
       </c>
       <c r="K31" t="n">
-        <v>4.902</v>
+        <v>4.908</v>
       </c>
       <c r="L31" t="n">
-        <v>5.06</v>
+        <v>5.075</v>
       </c>
       <c r="M31" t="n">
-        <v>5.387</v>
+        <v>5.398</v>
       </c>
       <c r="N31" t="n">
-        <v>5.691</v>
+        <v>5.711</v>
       </c>
       <c r="O31" t="n">
-        <v>6.172</v>
+        <v>6.2</v>
       </c>
       <c r="P31" t="n">
-        <v>6.335</v>
+        <v>6.365</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.092</v>
+        <v>7.125</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.189</v>
+        <v>3.187</v>
       </c>
       <c r="G32" t="n">
-        <v>3.29</v>
+        <v>3.291</v>
       </c>
       <c r="H32" t="n">
-        <v>3.541</v>
+        <v>3.546</v>
       </c>
       <c r="I32" t="n">
-        <v>3.78</v>
+        <v>3.79</v>
       </c>
       <c r="J32" t="n">
-        <v>4.186</v>
+        <v>4.202</v>
       </c>
       <c r="K32" t="n">
-        <v>4.554</v>
+        <v>4.56</v>
       </c>
       <c r="L32" t="n">
-        <v>4.651</v>
+        <v>4.666</v>
       </c>
       <c r="M32" t="n">
-        <v>4.929</v>
+        <v>4.94</v>
       </c>
       <c r="N32" t="n">
-        <v>5.193</v>
+        <v>5.212</v>
       </c>
       <c r="O32" t="n">
-        <v>5.582</v>
+        <v>5.61</v>
       </c>
       <c r="P32" t="n">
-        <v>5.807</v>
+        <v>5.837</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.58</v>
+        <v>6.612</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.957</v>
+        <v>2.955</v>
       </c>
       <c r="G33" t="n">
-        <v>3.038</v>
+        <v>3.039</v>
       </c>
       <c r="H33" t="n">
-        <v>3.212</v>
+        <v>3.217</v>
       </c>
       <c r="I33" t="n">
-        <v>3.404</v>
+        <v>3.413</v>
       </c>
       <c r="J33" t="n">
-        <v>3.714</v>
+        <v>3.729</v>
       </c>
       <c r="K33" t="n">
-        <v>4.011</v>
+        <v>4.016</v>
       </c>
       <c r="L33" t="n">
-        <v>4.05</v>
+        <v>4.065</v>
       </c>
       <c r="M33" t="n">
-        <v>4.183</v>
+        <v>4.194</v>
       </c>
       <c r="N33" t="n">
-        <v>4.223</v>
+        <v>4.242</v>
       </c>
       <c r="O33" t="n">
-        <v>4.291</v>
+        <v>4.319</v>
       </c>
       <c r="P33" t="n">
-        <v>4.38</v>
+        <v>4.409</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.836</v>
+        <v>4.868</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.017</v>
+        <v>3.015</v>
       </c>
       <c r="G34" t="n">
-        <v>3.091</v>
+        <v>3.092</v>
       </c>
       <c r="H34" t="n">
-        <v>3.274</v>
+        <v>3.279</v>
       </c>
       <c r="I34" t="n">
-        <v>3.472</v>
+        <v>3.481</v>
       </c>
       <c r="J34" t="n">
-        <v>3.786</v>
+        <v>3.8</v>
       </c>
       <c r="K34" t="n">
-        <v>4.087</v>
+        <v>4.092</v>
       </c>
       <c r="L34" t="n">
-        <v>4.129</v>
+        <v>4.144</v>
       </c>
       <c r="M34" t="n">
-        <v>4.273</v>
+        <v>4.284</v>
       </c>
       <c r="N34" t="n">
-        <v>4.327</v>
+        <v>4.346</v>
       </c>
       <c r="O34" t="n">
-        <v>4.46</v>
+        <v>4.488</v>
       </c>
       <c r="P34" t="n">
-        <v>4.674</v>
+        <v>4.703</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.537</v>
+        <v>5.569</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.991</v>
+        <v>2.989</v>
       </c>
       <c r="G35" t="n">
-        <v>3.065</v>
+        <v>3.066</v>
       </c>
       <c r="H35" t="n">
-        <v>3.242</v>
+        <v>3.247</v>
       </c>
       <c r="I35" t="n">
-        <v>3.438</v>
+        <v>3.447</v>
       </c>
       <c r="J35" t="n">
-        <v>3.754</v>
+        <v>3.769</v>
       </c>
       <c r="K35" t="n">
-        <v>4.041</v>
+        <v>4.046</v>
       </c>
       <c r="L35" t="n">
-        <v>4.084</v>
+        <v>4.099</v>
       </c>
       <c r="M35" t="n">
-        <v>4.22</v>
+        <v>4.231</v>
       </c>
       <c r="N35" t="n">
-        <v>4.263</v>
+        <v>4.282</v>
       </c>
       <c r="O35" t="n">
-        <v>4.357</v>
+        <v>4.385</v>
       </c>
       <c r="P35" t="n">
-        <v>4.477</v>
+        <v>4.506</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.173</v>
+        <v>5.205</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.889</v>
+        <v>2.887</v>
       </c>
       <c r="G36" t="n">
-        <v>2.964</v>
+        <v>2.965</v>
       </c>
       <c r="H36" t="n">
-        <v>3.131</v>
+        <v>3.135</v>
       </c>
       <c r="I36" t="n">
-        <v>3.324</v>
+        <v>3.333</v>
       </c>
       <c r="J36" t="n">
-        <v>3.649</v>
+        <v>3.665</v>
       </c>
       <c r="K36" t="n">
-        <v>3.935</v>
+        <v>3.941</v>
       </c>
       <c r="L36" t="n">
-        <v>3.975</v>
+        <v>3.99</v>
       </c>
       <c r="M36" t="n">
-        <v>4.087</v>
+        <v>4.096</v>
       </c>
       <c r="N36" t="n">
-        <v>4.13</v>
+        <v>4.146</v>
       </c>
       <c r="O36" t="n">
-        <v>4.203</v>
+        <v>4.228</v>
       </c>
       <c r="P36" t="n">
-        <v>4.279</v>
+        <v>4.307</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.553</v>
+        <v>4.585</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.762</v>
+        <v>3.761</v>
       </c>
       <c r="G37" t="n">
-        <v>4.231</v>
+        <v>4.232</v>
       </c>
       <c r="H37" t="n">
-        <v>4.788</v>
+        <v>4.793</v>
       </c>
       <c r="I37" t="n">
-        <v>5.113</v>
+        <v>5.122</v>
       </c>
       <c r="J37" t="n">
-        <v>5.991</v>
+        <v>6.007</v>
       </c>
       <c r="K37" t="n">
-        <v>6.943</v>
+        <v>6.949</v>
       </c>
       <c r="L37" t="n">
-        <v>7.26</v>
+        <v>7.275</v>
       </c>
       <c r="M37" t="n">
-        <v>7.659</v>
+        <v>7.67</v>
       </c>
       <c r="N37" t="n">
-        <v>7.842</v>
+        <v>7.861</v>
       </c>
       <c r="O37" t="n">
-        <v>8.051</v>
+        <v>8.079000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.135</v>
+        <v>8.164999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.581</v>
+        <v>8.613</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.821</v>
+        <v>4.82</v>
       </c>
       <c r="G38" t="n">
-        <v>5.544</v>
+        <v>5.545</v>
       </c>
       <c r="H38" t="n">
-        <v>6.312</v>
+        <v>6.317</v>
       </c>
       <c r="I38" t="n">
-        <v>6.794</v>
+        <v>6.803</v>
       </c>
       <c r="J38" t="n">
-        <v>7.934</v>
+        <v>7.95</v>
       </c>
       <c r="K38" t="n">
-        <v>9.064</v>
+        <v>9.07</v>
       </c>
       <c r="L38" t="n">
-        <v>9.539999999999999</v>
+        <v>9.555</v>
       </c>
       <c r="M38" t="n">
-        <v>10.071</v>
+        <v>10.082</v>
       </c>
       <c r="N38" t="n">
-        <v>10.26</v>
+        <v>10.28</v>
       </c>
       <c r="O38" t="n">
-        <v>10.452</v>
+        <v>10.48</v>
       </c>
       <c r="P38" t="n">
-        <v>10.532</v>
+        <v>10.562</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.032</v>
+        <v>11.064</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.142</v>
+        <v>4.141</v>
       </c>
       <c r="G39" t="n">
-        <v>4.742</v>
+        <v>4.743</v>
       </c>
       <c r="H39" t="n">
-        <v>5.377</v>
+        <v>5.382</v>
       </c>
       <c r="I39" t="n">
-        <v>5.798</v>
+        <v>5.807</v>
       </c>
       <c r="J39" t="n">
-        <v>6.806</v>
+        <v>6.822</v>
       </c>
       <c r="K39" t="n">
-        <v>7.897</v>
+        <v>7.903</v>
       </c>
       <c r="L39" t="n">
-        <v>8.298</v>
+        <v>8.313000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.707000000000001</v>
+        <v>8.718</v>
       </c>
       <c r="N39" t="n">
-        <v>8.888</v>
+        <v>8.907</v>
       </c>
       <c r="O39" t="n">
-        <v>9.102</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>9.186999999999999</v>
+        <v>9.217000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.677</v>
+        <v>9.709</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.283</v>
+        <v>3.282</v>
       </c>
       <c r="G40" t="n">
-        <v>3.411</v>
+        <v>3.412</v>
       </c>
       <c r="H40" t="n">
-        <v>3.658</v>
+        <v>3.662</v>
       </c>
       <c r="I40" t="n">
-        <v>3.896</v>
+        <v>3.906</v>
       </c>
       <c r="J40" t="n">
-        <v>4.301</v>
+        <v>4.317</v>
       </c>
       <c r="K40" t="n">
-        <v>4.674</v>
+        <v>4.68</v>
       </c>
       <c r="L40" t="n">
-        <v>4.771</v>
+        <v>4.786</v>
       </c>
       <c r="M40" t="n">
-        <v>4.998</v>
+        <v>5.009</v>
       </c>
       <c r="N40" t="n">
-        <v>5.19</v>
+        <v>5.209</v>
       </c>
       <c r="O40" t="n">
-        <v>5.514</v>
+        <v>5.542</v>
       </c>
       <c r="P40" t="n">
-        <v>5.768</v>
+        <v>5.798</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.57</v>
+        <v>6.602</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.669</v>
+        <v>3.668</v>
       </c>
       <c r="G41" t="n">
-        <v>3.84</v>
+        <v>3.841</v>
       </c>
       <c r="H41" t="n">
-        <v>4.142</v>
+        <v>4.147</v>
       </c>
       <c r="I41" t="n">
-        <v>4.399</v>
+        <v>4.409</v>
       </c>
       <c r="J41" t="n">
-        <v>4.856</v>
+        <v>4.872</v>
       </c>
       <c r="K41" t="n">
-        <v>5.274</v>
+        <v>5.28</v>
       </c>
       <c r="L41" t="n">
-        <v>5.45</v>
+        <v>5.465</v>
       </c>
       <c r="M41" t="n">
-        <v>5.8</v>
+        <v>5.811</v>
       </c>
       <c r="N41" t="n">
-        <v>6.121</v>
+        <v>6.14</v>
       </c>
       <c r="O41" t="n">
-        <v>6.63</v>
+        <v>6.657</v>
       </c>
       <c r="P41" t="n">
-        <v>6.827</v>
+        <v>6.857</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.617</v>
+        <v>7.649</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.404</v>
+        <v>3.403</v>
       </c>
       <c r="G42" t="n">
-        <v>3.56</v>
+        <v>3.561</v>
       </c>
       <c r="H42" t="n">
-        <v>3.833</v>
+        <v>3.838</v>
       </c>
       <c r="I42" t="n">
-        <v>4.084</v>
+        <v>4.094</v>
       </c>
       <c r="J42" t="n">
-        <v>4.503</v>
+        <v>4.519</v>
       </c>
       <c r="K42" t="n">
-        <v>4.895</v>
+        <v>4.901</v>
       </c>
       <c r="L42" t="n">
-        <v>5.007</v>
+        <v>5.022</v>
       </c>
       <c r="M42" t="n">
-        <v>5.305</v>
+        <v>5.316</v>
       </c>
       <c r="N42" t="n">
-        <v>5.604</v>
+        <v>5.624</v>
       </c>
       <c r="O42" t="n">
-        <v>6.006</v>
+        <v>6.034</v>
       </c>
       <c r="P42" t="n">
-        <v>6.27</v>
+        <v>6.3</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.083</v>
+        <v>7.115</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.105</v>
+        <v>3.103</v>
       </c>
       <c r="G43" t="n">
-        <v>3.221</v>
+        <v>3.222</v>
       </c>
       <c r="H43" t="n">
-        <v>3.414</v>
+        <v>3.418</v>
       </c>
       <c r="I43" t="n">
-        <v>3.613</v>
+        <v>3.622</v>
       </c>
       <c r="J43" t="n">
-        <v>3.942</v>
+        <v>3.957</v>
       </c>
       <c r="K43" t="n">
-        <v>4.241</v>
+        <v>4.246</v>
       </c>
       <c r="L43" t="n">
-        <v>4.291</v>
+        <v>4.306</v>
       </c>
       <c r="M43" t="n">
-        <v>4.436</v>
+        <v>4.447</v>
       </c>
       <c r="N43" t="n">
-        <v>4.491</v>
+        <v>4.51</v>
       </c>
       <c r="O43" t="n">
-        <v>4.604</v>
+        <v>4.632</v>
       </c>
       <c r="P43" t="n">
-        <v>4.746</v>
+        <v>4.775</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.446</v>
+        <v>5.478</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.967</v>
+        <v>2.965</v>
       </c>
       <c r="G44" t="n">
-        <v>3.073</v>
+        <v>3.074</v>
       </c>
       <c r="H44" t="n">
-        <v>3.255</v>
+        <v>3.259</v>
       </c>
       <c r="I44" t="n">
-        <v>3.452</v>
+        <v>3.461</v>
       </c>
       <c r="J44" t="n">
-        <v>3.79</v>
+        <v>3.807</v>
       </c>
       <c r="K44" t="n">
-        <v>4.085</v>
+        <v>4.091</v>
       </c>
       <c r="L44" t="n">
-        <v>4.135</v>
+        <v>4.15</v>
       </c>
       <c r="M44" t="n">
-        <v>4.255</v>
+        <v>4.264</v>
       </c>
       <c r="N44" t="n">
-        <v>4.311</v>
+        <v>4.327</v>
       </c>
       <c r="O44" t="n">
-        <v>4.403</v>
+        <v>4.428</v>
       </c>
       <c r="P44" t="n">
-        <v>4.509</v>
+        <v>4.537</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.817</v>
+        <v>4.849</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-15 ~ 2026-05-15
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.179</v>
+        <v>3.209</v>
       </c>
       <c r="G2" t="n">
-        <v>3.405</v>
+        <v>3.439</v>
       </c>
       <c r="H2" t="n">
-        <v>3.653</v>
+        <v>3.692</v>
       </c>
       <c r="I2" t="n">
-        <v>3.835</v>
+        <v>3.88</v>
       </c>
       <c r="J2" t="n">
-        <v>4.164</v>
+        <v>4.243</v>
       </c>
       <c r="K2" t="n">
-        <v>4.592</v>
+        <v>4.68</v>
       </c>
       <c r="L2" t="n">
-        <v>4.771</v>
+        <v>4.879</v>
       </c>
       <c r="M2" t="n">
-        <v>5.1</v>
+        <v>5.205</v>
       </c>
       <c r="N2" t="n">
-        <v>5.412</v>
+        <v>5.519</v>
       </c>
       <c r="O2" t="n">
-        <v>5.678</v>
+        <v>5.791</v>
       </c>
       <c r="P2" t="n">
-        <v>5.901</v>
+        <v>6.039</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.548</v>
+        <v>6.68</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.203</v>
+        <v>4.233</v>
       </c>
       <c r="G3" t="n">
-        <v>4.61</v>
+        <v>4.644</v>
       </c>
       <c r="H3" t="n">
-        <v>4.891</v>
+        <v>4.93</v>
       </c>
       <c r="I3" t="n">
-        <v>5.068</v>
+        <v>5.112</v>
       </c>
       <c r="J3" t="n">
-        <v>5.41</v>
+        <v>5.488</v>
       </c>
       <c r="K3" t="n">
-        <v>5.908</v>
+        <v>5.996</v>
       </c>
       <c r="L3" t="n">
-        <v>6.157</v>
+        <v>6.265</v>
       </c>
       <c r="M3" t="n">
-        <v>6.517</v>
+        <v>6.622</v>
       </c>
       <c r="N3" t="n">
-        <v>6.771</v>
+        <v>6.878</v>
       </c>
       <c r="O3" t="n">
-        <v>6.988</v>
+        <v>7.101</v>
       </c>
       <c r="P3" t="n">
-        <v>7.082</v>
+        <v>7.219</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.617</v>
+        <v>7.749</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.695</v>
+        <v>3.725</v>
       </c>
       <c r="G4" t="n">
-        <v>3.991</v>
+        <v>4.025</v>
       </c>
       <c r="H4" t="n">
-        <v>4.3</v>
+        <v>4.34</v>
       </c>
       <c r="I4" t="n">
-        <v>4.511</v>
+        <v>4.555</v>
       </c>
       <c r="J4" t="n">
-        <v>4.856</v>
+        <v>4.934</v>
       </c>
       <c r="K4" t="n">
-        <v>5.346</v>
+        <v>5.434</v>
       </c>
       <c r="L4" t="n">
-        <v>5.525</v>
+        <v>5.634</v>
       </c>
       <c r="M4" t="n">
-        <v>5.875</v>
+        <v>5.979</v>
       </c>
       <c r="N4" t="n">
-        <v>6.099</v>
+        <v>6.206</v>
       </c>
       <c r="O4" t="n">
-        <v>6.339</v>
+        <v>6.452</v>
       </c>
       <c r="P4" t="n">
-        <v>6.432</v>
+        <v>6.569</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.97</v>
+        <v>7.101</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.874</v>
+        <v>2.904</v>
       </c>
       <c r="G5" t="n">
-        <v>2.949</v>
+        <v>2.983</v>
       </c>
       <c r="H5" t="n">
-        <v>3.158</v>
+        <v>3.199</v>
       </c>
       <c r="I5" t="n">
-        <v>3.405</v>
+        <v>3.45</v>
       </c>
       <c r="J5" t="n">
-        <v>3.724</v>
+        <v>3.801</v>
       </c>
       <c r="K5" t="n">
-        <v>3.998</v>
+        <v>4.086</v>
       </c>
       <c r="L5" t="n">
-        <v>4.022</v>
+        <v>4.131</v>
       </c>
       <c r="M5" t="n">
-        <v>4.157</v>
+        <v>4.262</v>
       </c>
       <c r="N5" t="n">
-        <v>4.224</v>
+        <v>4.332</v>
       </c>
       <c r="O5" t="n">
-        <v>4.277</v>
+        <v>4.39</v>
       </c>
       <c r="P5" t="n">
-        <v>4.57</v>
+        <v>4.707</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.461</v>
+        <v>5.593</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.913</v>
+        <v>2.943</v>
       </c>
       <c r="G6" t="n">
-        <v>3.002</v>
+        <v>3.036</v>
       </c>
       <c r="H6" t="n">
-        <v>3.227</v>
+        <v>3.267</v>
       </c>
       <c r="I6" t="n">
-        <v>3.488</v>
+        <v>3.533</v>
       </c>
       <c r="J6" t="n">
-        <v>3.812</v>
+        <v>3.889</v>
       </c>
       <c r="K6" t="n">
-        <v>4.108</v>
+        <v>4.196</v>
       </c>
       <c r="L6" t="n">
-        <v>4.137</v>
+        <v>4.245</v>
       </c>
       <c r="M6" t="n">
-        <v>4.313</v>
+        <v>4.418</v>
       </c>
       <c r="N6" t="n">
-        <v>4.392</v>
+        <v>4.499</v>
       </c>
       <c r="O6" t="n">
-        <v>4.544</v>
+        <v>4.657</v>
       </c>
       <c r="P6" t="n">
-        <v>5.003</v>
+        <v>5.14</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.857</v>
+        <v>5.989</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.894</v>
+        <v>2.924</v>
       </c>
       <c r="G7" t="n">
-        <v>2.966</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>3.173</v>
+        <v>3.214</v>
       </c>
       <c r="I7" t="n">
-        <v>3.423</v>
+        <v>3.468</v>
       </c>
       <c r="J7" t="n">
-        <v>3.748</v>
+        <v>3.825</v>
       </c>
       <c r="K7" t="n">
-        <v>4.025</v>
+        <v>4.113</v>
       </c>
       <c r="L7" t="n">
-        <v>4.047</v>
+        <v>4.155</v>
       </c>
       <c r="M7" t="n">
-        <v>4.218</v>
+        <v>4.323</v>
       </c>
       <c r="N7" t="n">
-        <v>4.284</v>
+        <v>4.391</v>
       </c>
       <c r="O7" t="n">
-        <v>4.442</v>
+        <v>4.555</v>
       </c>
       <c r="P7" t="n">
-        <v>4.786</v>
+        <v>4.923</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.624</v>
+        <v>5.756</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.314</v>
+        <v>5.345</v>
       </c>
       <c r="G8" t="n">
-        <v>5.91</v>
+        <v>5.944</v>
       </c>
       <c r="H8" t="n">
-        <v>6.339</v>
+        <v>6.378</v>
       </c>
       <c r="I8" t="n">
-        <v>6.594</v>
+        <v>6.639</v>
       </c>
       <c r="J8" t="n">
-        <v>7.002</v>
+        <v>7.08</v>
       </c>
       <c r="K8" t="n">
-        <v>7.78</v>
+        <v>7.868</v>
       </c>
       <c r="L8" t="n">
-        <v>8.115</v>
+        <v>8.223000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.506</v>
+        <v>8.611000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.695</v>
+        <v>8.802</v>
       </c>
       <c r="O8" t="n">
-        <v>8.997</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>9.193</v>
+        <v>9.33</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.926</v>
+        <v>10.058</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.614</v>
+        <v>2.642</v>
       </c>
       <c r="G9" t="n">
-        <v>2.712</v>
+        <v>2.744</v>
       </c>
       <c r="H9" t="n">
-        <v>2.857</v>
+        <v>2.892</v>
       </c>
       <c r="I9" t="n">
-        <v>3.121</v>
+        <v>3.171</v>
       </c>
       <c r="J9" t="n">
-        <v>3.3</v>
+        <v>3.357</v>
       </c>
       <c r="K9" t="n">
-        <v>3.505</v>
+        <v>3.61</v>
       </c>
       <c r="L9" t="n">
-        <v>3.548</v>
+        <v>3.66</v>
       </c>
       <c r="M9" t="n">
-        <v>3.657</v>
+        <v>3.764</v>
       </c>
       <c r="N9" t="n">
-        <v>3.831</v>
+        <v>3.941</v>
       </c>
       <c r="O9" t="n">
-        <v>3.889</v>
+        <v>4.005</v>
       </c>
       <c r="P9" t="n">
-        <v>4</v>
+        <v>4.14</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.086</v>
+        <v>4.22</v>
       </c>
       <c r="R9" t="n">
-        <v>4.09</v>
+        <v>4.218</v>
       </c>
       <c r="S9" t="n">
-        <v>4.09</v>
+        <v>4.211</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>4.135</v>
       </c>
       <c r="U9" t="n">
-        <v>3.871</v>
+        <v>3.967</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.629</v>
+        <v>2.656</v>
       </c>
       <c r="G10" t="n">
-        <v>2.744</v>
+        <v>2.777</v>
       </c>
       <c r="H10" t="n">
-        <v>2.87</v>
+        <v>2.903</v>
       </c>
       <c r="I10" t="n">
-        <v>3.126</v>
+        <v>3.177</v>
       </c>
       <c r="J10" t="n">
-        <v>3.324</v>
+        <v>3.382</v>
       </c>
       <c r="K10" t="n">
-        <v>3.538</v>
+        <v>3.643</v>
       </c>
       <c r="L10" t="n">
-        <v>3.596</v>
+        <v>3.71</v>
       </c>
       <c r="M10" t="n">
-        <v>3.752</v>
+        <v>3.859</v>
       </c>
       <c r="N10" t="n">
-        <v>3.85</v>
+        <v>3.958</v>
       </c>
       <c r="O10" t="n">
-        <v>4.083</v>
+        <v>4.196</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.444</v>
+        <v>2.471</v>
       </c>
       <c r="G11" t="n">
-        <v>2.554</v>
+        <v>2.587</v>
       </c>
       <c r="H11" t="n">
-        <v>2.693</v>
+        <v>2.726</v>
       </c>
       <c r="I11" t="n">
-        <v>2.93</v>
+        <v>2.981</v>
       </c>
       <c r="J11" t="n">
-        <v>3.122</v>
+        <v>3.18</v>
       </c>
       <c r="K11" t="n">
-        <v>3.325</v>
+        <v>3.43</v>
       </c>
       <c r="L11" t="n">
-        <v>3.393</v>
+        <v>3.507</v>
       </c>
       <c r="M11" t="n">
-        <v>3.559</v>
+        <v>3.667</v>
       </c>
       <c r="N11" t="n">
-        <v>3.659</v>
+        <v>3.766</v>
       </c>
       <c r="O11" t="n">
-        <v>3.85</v>
+        <v>3.963</v>
       </c>
       <c r="P11" t="n">
-        <v>3.951</v>
+        <v>4.091</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.288</v>
+        <v>4.421</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.192</v>
+        <v>3.217</v>
       </c>
       <c r="G12" t="n">
-        <v>3.374</v>
+        <v>3.409</v>
       </c>
       <c r="H12" t="n">
-        <v>3.57</v>
+        <v>3.615</v>
       </c>
       <c r="I12" t="n">
-        <v>3.804</v>
+        <v>3.854</v>
       </c>
       <c r="J12" t="n">
-        <v>4.162</v>
+        <v>4.236</v>
       </c>
       <c r="K12" t="n">
-        <v>4.39</v>
+        <v>4.477</v>
       </c>
       <c r="L12" t="n">
-        <v>4.456</v>
+        <v>4.563</v>
       </c>
       <c r="M12" t="n">
-        <v>4.628</v>
+        <v>4.731</v>
       </c>
       <c r="N12" t="n">
-        <v>4.711</v>
+        <v>4.818</v>
       </c>
       <c r="O12" t="n">
-        <v>4.88</v>
+        <v>4.993</v>
       </c>
       <c r="P12" t="n">
-        <v>5.039</v>
+        <v>5.176</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.405</v>
+        <v>5.536</v>
       </c>
       <c r="R12" t="n">
-        <v>5.583</v>
+        <v>5.71</v>
       </c>
       <c r="S12" t="n">
-        <v>5.794</v>
+        <v>5.914</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.945</v>
+        <v>2.97</v>
       </c>
       <c r="G13" t="n">
-        <v>3.064</v>
+        <v>3.099</v>
       </c>
       <c r="H13" t="n">
-        <v>3.238</v>
+        <v>3.283</v>
       </c>
       <c r="I13" t="n">
-        <v>3.451</v>
+        <v>3.502</v>
       </c>
       <c r="J13" t="n">
-        <v>3.799</v>
+        <v>3.873</v>
       </c>
       <c r="K13" t="n">
-        <v>4.023</v>
+        <v>4.11</v>
       </c>
       <c r="L13" t="n">
-        <v>4.095</v>
+        <v>4.203</v>
       </c>
       <c r="M13" t="n">
-        <v>4.256</v>
+        <v>4.359</v>
       </c>
       <c r="N13" t="n">
-        <v>4.339</v>
+        <v>4.446</v>
       </c>
       <c r="O13" t="n">
-        <v>4.509</v>
+        <v>4.622</v>
       </c>
       <c r="P13" t="n">
-        <v>4.63</v>
+        <v>4.767</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.926</v>
+        <v>5.057</v>
       </c>
       <c r="R13" t="n">
-        <v>5.133</v>
+        <v>5.259</v>
       </c>
       <c r="S13" t="n">
-        <v>5.357</v>
+        <v>5.476</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.764</v>
+        <v>2.79</v>
       </c>
       <c r="G14" t="n">
-        <v>2.869</v>
+        <v>2.905</v>
       </c>
       <c r="H14" t="n">
-        <v>3.041</v>
+        <v>3.086</v>
       </c>
       <c r="I14" t="n">
-        <v>3.235</v>
+        <v>3.285</v>
       </c>
       <c r="J14" t="n">
-        <v>3.54</v>
+        <v>3.614</v>
       </c>
       <c r="K14" t="n">
-        <v>3.711</v>
+        <v>3.798</v>
       </c>
       <c r="L14" t="n">
-        <v>3.768</v>
+        <v>3.876</v>
       </c>
       <c r="M14" t="n">
-        <v>3.942</v>
+        <v>4.045</v>
       </c>
       <c r="N14" t="n">
-        <v>4.018</v>
+        <v>4.125</v>
       </c>
       <c r="O14" t="n">
-        <v>4.166</v>
+        <v>4.279</v>
       </c>
       <c r="P14" t="n">
-        <v>4.265</v>
+        <v>4.402</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.515</v>
+        <v>4.646</v>
       </c>
       <c r="R14" t="n">
-        <v>4.647</v>
+        <v>4.773</v>
       </c>
       <c r="S14" t="n">
-        <v>4.809</v>
+        <v>4.929</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.742</v>
+        <v>2.767</v>
       </c>
       <c r="G15" t="n">
-        <v>2.844</v>
+        <v>2.879</v>
       </c>
       <c r="H15" t="n">
-        <v>3.012</v>
+        <v>3.057</v>
       </c>
       <c r="I15" t="n">
-        <v>3.186</v>
+        <v>3.237</v>
       </c>
       <c r="J15" t="n">
-        <v>3.479</v>
+        <v>3.553</v>
       </c>
       <c r="K15" t="n">
-        <v>3.664</v>
+        <v>3.75</v>
       </c>
       <c r="L15" t="n">
-        <v>3.703</v>
+        <v>3.811</v>
       </c>
       <c r="M15" t="n">
-        <v>3.854</v>
+        <v>3.957</v>
       </c>
       <c r="N15" t="n">
-        <v>3.922</v>
+        <v>4.029</v>
       </c>
       <c r="O15" t="n">
-        <v>4.108</v>
+        <v>4.22</v>
       </c>
       <c r="P15" t="n">
-        <v>4.165</v>
+        <v>4.302</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.418</v>
+        <v>4.549</v>
       </c>
       <c r="R15" t="n">
-        <v>4.542</v>
+        <v>4.669</v>
       </c>
       <c r="S15" t="n">
-        <v>4.705</v>
+        <v>4.825</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.742</v>
+        <v>2.767</v>
       </c>
       <c r="G16" t="n">
-        <v>2.844</v>
+        <v>2.879</v>
       </c>
       <c r="H16" t="n">
-        <v>3.012</v>
+        <v>3.057</v>
       </c>
       <c r="I16" t="n">
-        <v>3.186</v>
+        <v>3.237</v>
       </c>
       <c r="J16" t="n">
-        <v>3.479</v>
+        <v>3.553</v>
       </c>
       <c r="K16" t="n">
-        <v>3.664</v>
+        <v>3.75</v>
       </c>
       <c r="L16" t="n">
-        <v>3.703</v>
+        <v>3.811</v>
       </c>
       <c r="M16" t="n">
-        <v>3.854</v>
+        <v>3.957</v>
       </c>
       <c r="N16" t="n">
-        <v>3.925</v>
+        <v>4.032</v>
       </c>
       <c r="O16" t="n">
-        <v>4.114</v>
+        <v>4.227</v>
       </c>
       <c r="P16" t="n">
-        <v>4.189</v>
+        <v>4.325</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.445</v>
+        <v>4.576</v>
       </c>
       <c r="R16" t="n">
-        <v>4.57</v>
+        <v>4.697</v>
       </c>
       <c r="S16" t="n">
-        <v>4.734</v>
+        <v>4.853</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.691</v>
+        <v>2.718</v>
       </c>
       <c r="G17" t="n">
-        <v>2.835</v>
+        <v>2.867</v>
       </c>
       <c r="H17" t="n">
-        <v>2.963</v>
+        <v>2.996</v>
       </c>
       <c r="I17" t="n">
-        <v>3.206</v>
+        <v>3.257</v>
       </c>
       <c r="J17" t="n">
-        <v>3.4</v>
+        <v>3.458</v>
       </c>
       <c r="K17" t="n">
-        <v>3.615</v>
+        <v>3.72</v>
       </c>
       <c r="L17" t="n">
-        <v>3.678</v>
+        <v>3.792</v>
       </c>
       <c r="M17" t="n">
-        <v>3.875</v>
+        <v>3.983</v>
       </c>
       <c r="N17" t="n">
-        <v>3.953</v>
+        <v>4.06</v>
       </c>
       <c r="O17" t="n">
-        <v>4.113</v>
+        <v>4.226</v>
       </c>
       <c r="P17" t="n">
-        <v>4.23</v>
+        <v>4.371</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.692</v>
+        <v>2.719</v>
       </c>
       <c r="G18" t="n">
-        <v>2.836</v>
+        <v>2.868</v>
       </c>
       <c r="H18" t="n">
-        <v>2.963</v>
+        <v>2.996</v>
       </c>
       <c r="I18" t="n">
-        <v>3.207</v>
+        <v>3.258</v>
       </c>
       <c r="J18" t="n">
-        <v>3.4</v>
+        <v>3.458</v>
       </c>
       <c r="K18" t="n">
-        <v>3.616</v>
+        <v>3.721</v>
       </c>
       <c r="L18" t="n">
-        <v>3.678</v>
+        <v>3.792</v>
       </c>
       <c r="M18" t="n">
-        <v>3.875</v>
+        <v>3.983</v>
       </c>
       <c r="N18" t="n">
-        <v>3.953</v>
+        <v>4.061</v>
       </c>
       <c r="O18" t="n">
-        <v>4.11</v>
+        <v>4.224</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.756</v>
+        <v>2.78</v>
       </c>
       <c r="G19" t="n">
-        <v>2.859</v>
+        <v>2.894</v>
       </c>
       <c r="H19" t="n">
-        <v>3.029</v>
+        <v>3.074</v>
       </c>
       <c r="I19" t="n">
-        <v>3.221</v>
+        <v>3.272</v>
       </c>
       <c r="J19" t="n">
-        <v>3.522</v>
+        <v>3.597</v>
       </c>
       <c r="K19" t="n">
-        <v>3.707</v>
+        <v>3.794</v>
       </c>
       <c r="L19" t="n">
-        <v>3.764</v>
+        <v>3.872</v>
       </c>
       <c r="M19" t="n">
-        <v>3.932</v>
+        <v>4.035</v>
       </c>
       <c r="N19" t="n">
-        <v>4.008</v>
+        <v>4.115</v>
       </c>
       <c r="O19" t="n">
-        <v>4.15</v>
+        <v>4.263</v>
       </c>
       <c r="P19" t="n">
-        <v>4.224</v>
+        <v>4.361</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.456</v>
+        <v>4.587</v>
       </c>
       <c r="R19" t="n">
-        <v>4.59</v>
+        <v>4.716</v>
       </c>
       <c r="S19" t="n">
-        <v>4.744</v>
+        <v>4.864</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.59</v>
+        <v>2.61</v>
       </c>
       <c r="G20" t="n">
-        <v>2.67</v>
+        <v>2.692</v>
       </c>
       <c r="H20" t="n">
-        <v>2.738</v>
+        <v>2.763</v>
       </c>
       <c r="I20" t="n">
-        <v>2.86</v>
+        <v>2.888</v>
       </c>
       <c r="J20" t="n">
-        <v>3.31</v>
+        <v>3.376</v>
       </c>
       <c r="K20" t="n">
-        <v>3.54</v>
+        <v>3.627</v>
       </c>
       <c r="L20" t="n">
-        <v>3.583</v>
+        <v>3.679</v>
       </c>
       <c r="M20" t="n">
-        <v>3.694</v>
+        <v>3.795</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.879</v>
+        <v>2.902</v>
       </c>
       <c r="G21" t="n">
-        <v>2.962</v>
+        <v>2.991</v>
       </c>
       <c r="H21" t="n">
-        <v>3.16</v>
+        <v>3.195</v>
       </c>
       <c r="I21" t="n">
-        <v>3.328</v>
+        <v>3.372</v>
       </c>
       <c r="J21" t="n">
-        <v>3.669</v>
+        <v>3.739</v>
       </c>
       <c r="K21" t="n">
-        <v>3.941</v>
+        <v>4.026</v>
       </c>
       <c r="L21" t="n">
-        <v>4.005</v>
+        <v>4.111</v>
       </c>
       <c r="M21" t="n">
-        <v>4.156</v>
+        <v>4.258</v>
       </c>
       <c r="N21" t="n">
-        <v>4.248</v>
+        <v>4.352</v>
       </c>
       <c r="O21" t="n">
-        <v>4.361</v>
+        <v>4.472</v>
       </c>
       <c r="P21" t="n">
-        <v>4.488</v>
+        <v>4.623</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.621</v>
+        <v>4.748</v>
       </c>
       <c r="R21" t="n">
-        <v>4.642</v>
+        <v>4.766</v>
       </c>
       <c r="S21" t="n">
-        <v>4.705</v>
+        <v>4.822</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.826</v>
+        <v>2.849</v>
       </c>
       <c r="G22" t="n">
-        <v>2.908</v>
+        <v>2.937</v>
       </c>
       <c r="H22" t="n">
-        <v>3.091</v>
+        <v>3.127</v>
       </c>
       <c r="I22" t="n">
-        <v>3.247</v>
+        <v>3.291</v>
       </c>
       <c r="J22" t="n">
-        <v>3.555</v>
+        <v>3.625</v>
       </c>
       <c r="K22" t="n">
-        <v>3.823</v>
+        <v>3.908</v>
       </c>
       <c r="L22" t="n">
-        <v>3.872</v>
+        <v>3.978</v>
       </c>
       <c r="M22" t="n">
-        <v>4.026</v>
+        <v>4.127</v>
       </c>
       <c r="N22" t="n">
-        <v>4.121</v>
+        <v>4.225</v>
       </c>
       <c r="O22" t="n">
-        <v>4.229</v>
+        <v>4.34</v>
       </c>
       <c r="P22" t="n">
-        <v>4.35</v>
+        <v>4.485</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.48</v>
+        <v>4.606</v>
       </c>
       <c r="R22" t="n">
-        <v>4.49</v>
+        <v>4.615</v>
       </c>
       <c r="S22" t="n">
-        <v>4.55</v>
+        <v>4.668</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.778</v>
+        <v>2.801</v>
       </c>
       <c r="G23" t="n">
-        <v>2.863</v>
+        <v>2.892</v>
       </c>
       <c r="H23" t="n">
-        <v>3.033</v>
+        <v>3.068</v>
       </c>
       <c r="I23" t="n">
-        <v>3.197</v>
+        <v>3.24</v>
       </c>
       <c r="J23" t="n">
-        <v>3.497</v>
+        <v>3.567</v>
       </c>
       <c r="K23" t="n">
-        <v>3.724</v>
+        <v>3.809</v>
       </c>
       <c r="L23" t="n">
-        <v>3.771</v>
+        <v>3.877</v>
       </c>
       <c r="M23" t="n">
-        <v>3.919</v>
+        <v>4.021</v>
       </c>
       <c r="N23" t="n">
-        <v>4.016</v>
+        <v>4.12</v>
       </c>
       <c r="O23" t="n">
-        <v>4.106</v>
+        <v>4.217</v>
       </c>
       <c r="P23" t="n">
-        <v>4.215</v>
+        <v>4.35</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.286</v>
+        <v>4.412</v>
       </c>
       <c r="R23" t="n">
-        <v>4.274</v>
+        <v>4.398</v>
       </c>
       <c r="S23" t="n">
-        <v>4.304</v>
+        <v>4.422</v>
       </c>
       <c r="T23" t="n">
-        <v>4.208</v>
+        <v>4.34</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.714</v>
+        <v>2.736</v>
       </c>
       <c r="G24" t="n">
-        <v>2.779</v>
+        <v>2.807</v>
       </c>
       <c r="H24" t="n">
-        <v>2.933</v>
+        <v>2.967</v>
       </c>
       <c r="I24" t="n">
-        <v>3.122</v>
+        <v>3.173</v>
       </c>
       <c r="J24" t="n">
-        <v>3.395</v>
+        <v>3.464</v>
       </c>
       <c r="K24" t="n">
-        <v>3.609</v>
+        <v>3.693</v>
       </c>
       <c r="L24" t="n">
-        <v>3.652</v>
+        <v>3.757</v>
       </c>
       <c r="M24" t="n">
-        <v>3.783</v>
+        <v>3.884</v>
       </c>
       <c r="N24" t="n">
-        <v>3.893</v>
+        <v>3.998</v>
       </c>
       <c r="O24" t="n">
-        <v>4.098</v>
+        <v>4.209</v>
       </c>
       <c r="P24" t="n">
-        <v>4.154</v>
+        <v>4.288</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.211</v>
+        <v>4.337</v>
       </c>
       <c r="R24" t="n">
-        <v>4.196</v>
+        <v>4.32</v>
       </c>
       <c r="S24" t="n">
-        <v>4.219</v>
+        <v>4.337</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.772</v>
+        <v>2.795</v>
       </c>
       <c r="G25" t="n">
-        <v>2.863</v>
+        <v>2.892</v>
       </c>
       <c r="H25" t="n">
-        <v>3.036</v>
+        <v>3.071</v>
       </c>
       <c r="I25" t="n">
-        <v>3.204</v>
+        <v>3.248</v>
       </c>
       <c r="J25" t="n">
-        <v>3.513</v>
+        <v>3.582</v>
       </c>
       <c r="K25" t="n">
-        <v>3.756</v>
+        <v>3.841</v>
       </c>
       <c r="L25" t="n">
-        <v>3.801</v>
+        <v>3.908</v>
       </c>
       <c r="M25" t="n">
-        <v>3.95</v>
+        <v>4.052</v>
       </c>
       <c r="N25" t="n">
-        <v>4.043</v>
+        <v>4.147</v>
       </c>
       <c r="O25" t="n">
-        <v>4.135</v>
+        <v>4.246</v>
       </c>
       <c r="P25" t="n">
-        <v>4.237</v>
+        <v>4.372</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.319</v>
+        <v>4.446</v>
       </c>
       <c r="R25" t="n">
-        <v>4.298</v>
+        <v>4.422</v>
       </c>
       <c r="S25" t="n">
-        <v>4.328</v>
+        <v>4.445</v>
       </c>
       <c r="T25" t="n">
-        <v>4.226</v>
+        <v>4.358</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.045</v>
+        <v>3.068</v>
       </c>
       <c r="G26" t="n">
-        <v>3.195</v>
+        <v>3.219</v>
       </c>
       <c r="H26" t="n">
-        <v>3.467</v>
+        <v>3.5</v>
       </c>
       <c r="I26" t="n">
-        <v>3.701</v>
+        <v>3.736</v>
       </c>
       <c r="J26" t="n">
-        <v>4.152</v>
+        <v>4.22</v>
       </c>
       <c r="K26" t="n">
-        <v>4.574</v>
+        <v>4.659</v>
       </c>
       <c r="L26" t="n">
-        <v>4.682</v>
+        <v>4.791</v>
       </c>
       <c r="M26" t="n">
-        <v>4.896</v>
+        <v>4.998</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.213</v>
+        <v>5.324</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.852</v>
+        <v>2.876</v>
       </c>
       <c r="G27" t="n">
-        <v>2.944</v>
+        <v>2.975</v>
       </c>
       <c r="H27" t="n">
-        <v>3.125</v>
+        <v>3.164</v>
       </c>
       <c r="I27" t="n">
-        <v>3.327</v>
+        <v>3.37</v>
       </c>
       <c r="J27" t="n">
-        <v>3.656</v>
+        <v>3.727</v>
       </c>
       <c r="K27" t="n">
-        <v>3.889</v>
+        <v>3.975</v>
       </c>
       <c r="L27" t="n">
-        <v>3.951</v>
+        <v>4.06</v>
       </c>
       <c r="M27" t="n">
-        <v>4.107</v>
+        <v>4.211</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.305</v>
+        <v>4.417</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.955</v>
+        <v>2.979</v>
       </c>
       <c r="G28" t="n">
-        <v>3.055</v>
+        <v>3.086</v>
       </c>
       <c r="H28" t="n">
-        <v>3.251</v>
+        <v>3.289</v>
       </c>
       <c r="I28" t="n">
-        <v>3.465</v>
+        <v>3.508</v>
       </c>
       <c r="J28" t="n">
-        <v>3.828</v>
+        <v>3.9</v>
       </c>
       <c r="K28" t="n">
-        <v>4.081</v>
+        <v>4.168</v>
       </c>
       <c r="L28" t="n">
-        <v>4.154</v>
+        <v>4.263</v>
       </c>
       <c r="M28" t="n">
-        <v>4.319</v>
+        <v>4.423</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.597</v>
+        <v>4.709</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.802</v>
+        <v>2.826</v>
       </c>
       <c r="G29" t="n">
-        <v>2.894</v>
+        <v>2.925</v>
       </c>
       <c r="H29" t="n">
-        <v>3.066</v>
+        <v>3.104</v>
       </c>
       <c r="I29" t="n">
-        <v>3.257</v>
+        <v>3.299</v>
       </c>
       <c r="J29" t="n">
-        <v>3.568</v>
+        <v>3.639</v>
       </c>
       <c r="K29" t="n">
-        <v>3.784</v>
+        <v>3.871</v>
       </c>
       <c r="L29" t="n">
-        <v>3.836</v>
+        <v>3.945</v>
       </c>
       <c r="M29" t="n">
-        <v>3.97</v>
+        <v>4.073</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.175</v>
+        <v>4.287</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.089</v>
+        <v>3.112</v>
       </c>
       <c r="G30" t="n">
-        <v>3.173</v>
+        <v>3.198</v>
       </c>
       <c r="H30" t="n">
-        <v>3.403</v>
+        <v>3.432</v>
       </c>
       <c r="I30" t="n">
-        <v>3.631</v>
+        <v>3.663</v>
       </c>
       <c r="J30" t="n">
-        <v>4.024</v>
+        <v>4.091</v>
       </c>
       <c r="K30" t="n">
-        <v>4.375</v>
+        <v>4.46</v>
       </c>
       <c r="L30" t="n">
-        <v>4.462</v>
+        <v>4.57</v>
       </c>
       <c r="M30" t="n">
-        <v>4.668</v>
+        <v>4.768</v>
       </c>
       <c r="N30" t="n">
-        <v>4.851</v>
+        <v>4.957</v>
       </c>
       <c r="O30" t="n">
-        <v>5.164</v>
+        <v>5.274</v>
       </c>
       <c r="P30" t="n">
-        <v>5.377</v>
+        <v>5.515</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.151</v>
+        <v>6.283</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.418</v>
+        <v>3.441</v>
       </c>
       <c r="G31" t="n">
-        <v>3.538</v>
+        <v>3.563</v>
       </c>
       <c r="H31" t="n">
-        <v>3.817</v>
+        <v>3.846</v>
       </c>
       <c r="I31" t="n">
-        <v>4.06</v>
+        <v>4.093</v>
       </c>
       <c r="J31" t="n">
-        <v>4.516</v>
+        <v>4.582</v>
       </c>
       <c r="K31" t="n">
-        <v>4.908</v>
+        <v>4.993</v>
       </c>
       <c r="L31" t="n">
-        <v>5.075</v>
+        <v>5.183</v>
       </c>
       <c r="M31" t="n">
-        <v>5.398</v>
+        <v>5.499</v>
       </c>
       <c r="N31" t="n">
-        <v>5.711</v>
+        <v>5.816</v>
       </c>
       <c r="O31" t="n">
-        <v>6.2</v>
+        <v>6.31</v>
       </c>
       <c r="P31" t="n">
-        <v>6.365</v>
+        <v>6.503</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.125</v>
+        <v>7.257</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.187</v>
+        <v>3.211</v>
       </c>
       <c r="G32" t="n">
-        <v>3.291</v>
+        <v>3.316</v>
       </c>
       <c r="H32" t="n">
-        <v>3.546</v>
+        <v>3.576</v>
       </c>
       <c r="I32" t="n">
-        <v>3.79</v>
+        <v>3.822</v>
       </c>
       <c r="J32" t="n">
-        <v>4.202</v>
+        <v>4.269</v>
       </c>
       <c r="K32" t="n">
-        <v>4.56</v>
+        <v>4.645</v>
       </c>
       <c r="L32" t="n">
-        <v>4.666</v>
+        <v>4.775</v>
       </c>
       <c r="M32" t="n">
-        <v>4.94</v>
+        <v>5.041</v>
       </c>
       <c r="N32" t="n">
-        <v>5.212</v>
+        <v>5.318</v>
       </c>
       <c r="O32" t="n">
-        <v>5.61</v>
+        <v>5.72</v>
       </c>
       <c r="P32" t="n">
-        <v>5.837</v>
+        <v>5.975</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.612</v>
+        <v>6.744</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.955</v>
+        <v>2.976</v>
       </c>
       <c r="G33" t="n">
-        <v>3.039</v>
+        <v>3.061</v>
       </c>
       <c r="H33" t="n">
-        <v>3.217</v>
+        <v>3.248</v>
       </c>
       <c r="I33" t="n">
-        <v>3.413</v>
+        <v>3.447</v>
       </c>
       <c r="J33" t="n">
-        <v>3.729</v>
+        <v>3.795</v>
       </c>
       <c r="K33" t="n">
-        <v>4.016</v>
+        <v>4.1</v>
       </c>
       <c r="L33" t="n">
-        <v>4.065</v>
+        <v>4.173</v>
       </c>
       <c r="M33" t="n">
-        <v>4.194</v>
+        <v>4.294</v>
       </c>
       <c r="N33" t="n">
-        <v>4.242</v>
+        <v>4.348</v>
       </c>
       <c r="O33" t="n">
-        <v>4.319</v>
+        <v>4.429</v>
       </c>
       <c r="P33" t="n">
-        <v>4.409</v>
+        <v>4.547</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.868</v>
+        <v>5</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.015</v>
+        <v>3.036</v>
       </c>
       <c r="G34" t="n">
-        <v>3.092</v>
+        <v>3.114</v>
       </c>
       <c r="H34" t="n">
-        <v>3.279</v>
+        <v>3.309</v>
       </c>
       <c r="I34" t="n">
-        <v>3.481</v>
+        <v>3.515</v>
       </c>
       <c r="J34" t="n">
-        <v>3.8</v>
+        <v>3.867</v>
       </c>
       <c r="K34" t="n">
-        <v>4.092</v>
+        <v>4.177</v>
       </c>
       <c r="L34" t="n">
-        <v>4.144</v>
+        <v>4.252</v>
       </c>
       <c r="M34" t="n">
-        <v>4.284</v>
+        <v>4.385</v>
       </c>
       <c r="N34" t="n">
-        <v>4.346</v>
+        <v>4.451</v>
       </c>
       <c r="O34" t="n">
-        <v>4.488</v>
+        <v>4.598</v>
       </c>
       <c r="P34" t="n">
-        <v>4.703</v>
+        <v>4.841</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.569</v>
+        <v>5.701</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.989</v>
+        <v>3.01</v>
       </c>
       <c r="G35" t="n">
-        <v>3.066</v>
+        <v>3.088</v>
       </c>
       <c r="H35" t="n">
-        <v>3.247</v>
+        <v>3.277</v>
       </c>
       <c r="I35" t="n">
-        <v>3.447</v>
+        <v>3.482</v>
       </c>
       <c r="J35" t="n">
-        <v>3.769</v>
+        <v>3.835</v>
       </c>
       <c r="K35" t="n">
-        <v>4.046</v>
+        <v>4.131</v>
       </c>
       <c r="L35" t="n">
-        <v>4.099</v>
+        <v>4.207</v>
       </c>
       <c r="M35" t="n">
-        <v>4.231</v>
+        <v>4.332</v>
       </c>
       <c r="N35" t="n">
-        <v>4.282</v>
+        <v>4.387</v>
       </c>
       <c r="O35" t="n">
-        <v>4.385</v>
+        <v>4.495</v>
       </c>
       <c r="P35" t="n">
-        <v>4.506</v>
+        <v>4.644</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.205</v>
+        <v>5.337</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.887</v>
+        <v>2.907</v>
       </c>
       <c r="G36" t="n">
-        <v>2.965</v>
+        <v>2.986</v>
       </c>
       <c r="H36" t="n">
-        <v>3.135</v>
+        <v>3.165</v>
       </c>
       <c r="I36" t="n">
-        <v>3.333</v>
+        <v>3.367</v>
       </c>
       <c r="J36" t="n">
-        <v>3.665</v>
+        <v>3.731</v>
       </c>
       <c r="K36" t="n">
-        <v>3.941</v>
+        <v>4.025</v>
       </c>
       <c r="L36" t="n">
-        <v>3.99</v>
+        <v>4.098</v>
       </c>
       <c r="M36" t="n">
-        <v>4.096</v>
+        <v>4.196</v>
       </c>
       <c r="N36" t="n">
-        <v>4.146</v>
+        <v>4.251</v>
       </c>
       <c r="O36" t="n">
-        <v>4.228</v>
+        <v>4.338</v>
       </c>
       <c r="P36" t="n">
-        <v>4.307</v>
+        <v>4.445</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.585</v>
+        <v>4.717</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.761</v>
+        <v>3.784</v>
       </c>
       <c r="G37" t="n">
-        <v>4.232</v>
+        <v>4.257</v>
       </c>
       <c r="H37" t="n">
-        <v>4.793</v>
+        <v>4.822</v>
       </c>
       <c r="I37" t="n">
-        <v>5.122</v>
+        <v>5.154</v>
       </c>
       <c r="J37" t="n">
-        <v>6.007</v>
+        <v>6.073</v>
       </c>
       <c r="K37" t="n">
-        <v>6.949</v>
+        <v>7.033</v>
       </c>
       <c r="L37" t="n">
-        <v>7.275</v>
+        <v>7.383</v>
       </c>
       <c r="M37" t="n">
-        <v>7.67</v>
+        <v>7.771</v>
       </c>
       <c r="N37" t="n">
-        <v>7.861</v>
+        <v>7.967</v>
       </c>
       <c r="O37" t="n">
-        <v>8.079000000000001</v>
+        <v>8.189</v>
       </c>
       <c r="P37" t="n">
-        <v>8.164999999999999</v>
+        <v>8.303000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.613</v>
+        <v>8.744999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.82</v>
+        <v>4.843</v>
       </c>
       <c r="G38" t="n">
-        <v>5.545</v>
+        <v>5.57</v>
       </c>
       <c r="H38" t="n">
-        <v>6.317</v>
+        <v>6.346</v>
       </c>
       <c r="I38" t="n">
-        <v>6.803</v>
+        <v>6.835</v>
       </c>
       <c r="J38" t="n">
-        <v>7.95</v>
+        <v>8.016</v>
       </c>
       <c r="K38" t="n">
-        <v>9.07</v>
+        <v>9.154999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.555</v>
+        <v>9.664999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.082</v>
+        <v>10.183</v>
       </c>
       <c r="N38" t="n">
-        <v>10.28</v>
+        <v>10.386</v>
       </c>
       <c r="O38" t="n">
-        <v>10.48</v>
+        <v>10.59</v>
       </c>
       <c r="P38" t="n">
-        <v>10.562</v>
+        <v>10.7</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.064</v>
+        <v>11.196</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.141</v>
+        <v>4.164</v>
       </c>
       <c r="G39" t="n">
-        <v>4.743</v>
+        <v>4.768</v>
       </c>
       <c r="H39" t="n">
-        <v>5.382</v>
+        <v>5.411</v>
       </c>
       <c r="I39" t="n">
-        <v>5.807</v>
+        <v>5.839</v>
       </c>
       <c r="J39" t="n">
-        <v>6.822</v>
+        <v>6.889</v>
       </c>
       <c r="K39" t="n">
-        <v>7.903</v>
+        <v>7.988</v>
       </c>
       <c r="L39" t="n">
-        <v>8.313000000000001</v>
+        <v>8.420999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.718</v>
+        <v>8.819000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.907</v>
+        <v>9.013999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.130000000000001</v>
+        <v>9.24</v>
       </c>
       <c r="P39" t="n">
-        <v>9.217000000000001</v>
+        <v>9.355</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.709</v>
+        <v>9.840999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.282</v>
+        <v>3.304</v>
       </c>
       <c r="G40" t="n">
-        <v>3.412</v>
+        <v>3.436</v>
       </c>
       <c r="H40" t="n">
-        <v>3.662</v>
+        <v>3.691</v>
       </c>
       <c r="I40" t="n">
-        <v>3.906</v>
+        <v>3.937</v>
       </c>
       <c r="J40" t="n">
-        <v>4.317</v>
+        <v>4.382</v>
       </c>
       <c r="K40" t="n">
-        <v>4.68</v>
+        <v>4.766</v>
       </c>
       <c r="L40" t="n">
-        <v>4.786</v>
+        <v>4.895</v>
       </c>
       <c r="M40" t="n">
-        <v>5.009</v>
+        <v>5.111</v>
       </c>
       <c r="N40" t="n">
-        <v>5.209</v>
+        <v>5.315</v>
       </c>
       <c r="O40" t="n">
-        <v>5.542</v>
+        <v>5.653</v>
       </c>
       <c r="P40" t="n">
-        <v>5.798</v>
+        <v>5.936</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.602</v>
+        <v>6.734</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.668</v>
+        <v>3.69</v>
       </c>
       <c r="G41" t="n">
-        <v>3.841</v>
+        <v>3.864</v>
       </c>
       <c r="H41" t="n">
-        <v>4.147</v>
+        <v>4.176</v>
       </c>
       <c r="I41" t="n">
-        <v>4.409</v>
+        <v>4.441</v>
       </c>
       <c r="J41" t="n">
-        <v>4.872</v>
+        <v>4.937</v>
       </c>
       <c r="K41" t="n">
-        <v>5.28</v>
+        <v>5.366</v>
       </c>
       <c r="L41" t="n">
-        <v>5.465</v>
+        <v>5.574</v>
       </c>
       <c r="M41" t="n">
-        <v>5.811</v>
+        <v>5.914</v>
       </c>
       <c r="N41" t="n">
-        <v>6.14</v>
+        <v>6.245</v>
       </c>
       <c r="O41" t="n">
-        <v>6.657</v>
+        <v>6.769</v>
       </c>
       <c r="P41" t="n">
-        <v>6.857</v>
+        <v>6.995</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.649</v>
+        <v>7.781</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.403</v>
+        <v>3.425</v>
       </c>
       <c r="G42" t="n">
-        <v>3.561</v>
+        <v>3.585</v>
       </c>
       <c r="H42" t="n">
-        <v>3.838</v>
+        <v>3.867</v>
       </c>
       <c r="I42" t="n">
-        <v>4.094</v>
+        <v>4.125</v>
       </c>
       <c r="J42" t="n">
-        <v>4.519</v>
+        <v>4.585</v>
       </c>
       <c r="K42" t="n">
-        <v>4.901</v>
+        <v>4.987</v>
       </c>
       <c r="L42" t="n">
-        <v>5.022</v>
+        <v>5.131</v>
       </c>
       <c r="M42" t="n">
-        <v>5.316</v>
+        <v>5.418</v>
       </c>
       <c r="N42" t="n">
-        <v>5.624</v>
+        <v>5.729</v>
       </c>
       <c r="O42" t="n">
-        <v>6.034</v>
+        <v>6.145</v>
       </c>
       <c r="P42" t="n">
-        <v>6.3</v>
+        <v>6.438</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.115</v>
+        <v>7.247</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.103</v>
+        <v>3.124</v>
       </c>
       <c r="G43" t="n">
-        <v>3.222</v>
+        <v>3.244</v>
       </c>
       <c r="H43" t="n">
-        <v>3.418</v>
+        <v>3.448</v>
       </c>
       <c r="I43" t="n">
-        <v>3.622</v>
+        <v>3.656</v>
       </c>
       <c r="J43" t="n">
-        <v>3.957</v>
+        <v>4.022</v>
       </c>
       <c r="K43" t="n">
-        <v>4.246</v>
+        <v>4.332</v>
       </c>
       <c r="L43" t="n">
-        <v>4.306</v>
+        <v>4.415</v>
       </c>
       <c r="M43" t="n">
-        <v>4.447</v>
+        <v>4.55</v>
       </c>
       <c r="N43" t="n">
-        <v>4.51</v>
+        <v>4.616</v>
       </c>
       <c r="O43" t="n">
-        <v>4.632</v>
+        <v>4.743</v>
       </c>
       <c r="P43" t="n">
-        <v>4.775</v>
+        <v>4.912</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.478</v>
+        <v>5.61</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.965</v>
+        <v>2.985</v>
       </c>
       <c r="G44" t="n">
-        <v>3.074</v>
+        <v>3.095</v>
       </c>
       <c r="H44" t="n">
-        <v>3.259</v>
+        <v>3.288</v>
       </c>
       <c r="I44" t="n">
-        <v>3.461</v>
+        <v>3.494</v>
       </c>
       <c r="J44" t="n">
-        <v>3.807</v>
+        <v>3.872</v>
       </c>
       <c r="K44" t="n">
-        <v>4.091</v>
+        <v>4.177</v>
       </c>
       <c r="L44" t="n">
-        <v>4.15</v>
+        <v>4.259</v>
       </c>
       <c r="M44" t="n">
-        <v>4.264</v>
+        <v>4.367</v>
       </c>
       <c r="N44" t="n">
-        <v>4.327</v>
+        <v>4.433</v>
       </c>
       <c r="O44" t="n">
-        <v>4.428</v>
+        <v>4.539</v>
       </c>
       <c r="P44" t="n">
-        <v>4.537</v>
+        <v>4.675</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.849</v>
+        <v>4.981</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-18 ~ 2026-05-18
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.209</v>
+        <v>3.215</v>
       </c>
       <c r="G2" t="n">
-        <v>3.439</v>
+        <v>3.445</v>
       </c>
       <c r="H2" t="n">
-        <v>3.692</v>
+        <v>3.695</v>
       </c>
       <c r="I2" t="n">
-        <v>3.88</v>
+        <v>3.864</v>
       </c>
       <c r="J2" t="n">
-        <v>4.243</v>
+        <v>4.244</v>
       </c>
       <c r="K2" t="n">
-        <v>4.68</v>
+        <v>4.679</v>
       </c>
       <c r="L2" t="n">
-        <v>4.879</v>
+        <v>4.874</v>
       </c>
       <c r="M2" t="n">
-        <v>5.205</v>
+        <v>5.196</v>
       </c>
       <c r="N2" t="n">
-        <v>5.519</v>
+        <v>5.51</v>
       </c>
       <c r="O2" t="n">
-        <v>5.791</v>
+        <v>5.778</v>
       </c>
       <c r="P2" t="n">
-        <v>6.039</v>
+        <v>6.046</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.68</v>
+        <v>6.707</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.233</v>
+        <v>4.238</v>
       </c>
       <c r="G3" t="n">
-        <v>4.644</v>
+        <v>4.65</v>
       </c>
       <c r="H3" t="n">
-        <v>4.93</v>
+        <v>4.933</v>
       </c>
       <c r="I3" t="n">
-        <v>5.112</v>
+        <v>5.096</v>
       </c>
       <c r="J3" t="n">
-        <v>5.488</v>
+        <v>5.49</v>
       </c>
       <c r="K3" t="n">
-        <v>5.996</v>
+        <v>5.995</v>
       </c>
       <c r="L3" t="n">
-        <v>6.265</v>
+        <v>6.259</v>
       </c>
       <c r="M3" t="n">
-        <v>6.622</v>
+        <v>6.613</v>
       </c>
       <c r="N3" t="n">
-        <v>6.878</v>
+        <v>6.869</v>
       </c>
       <c r="O3" t="n">
-        <v>7.101</v>
+        <v>7.088</v>
       </c>
       <c r="P3" t="n">
-        <v>7.219</v>
+        <v>7.226</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.749</v>
+        <v>7.776</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.725</v>
+        <v>3.731</v>
       </c>
       <c r="G4" t="n">
-        <v>4.025</v>
+        <v>4.031</v>
       </c>
       <c r="H4" t="n">
-        <v>4.34</v>
+        <v>4.343</v>
       </c>
       <c r="I4" t="n">
-        <v>4.555</v>
+        <v>4.539</v>
       </c>
       <c r="J4" t="n">
-        <v>4.934</v>
+        <v>4.936</v>
       </c>
       <c r="K4" t="n">
-        <v>5.434</v>
+        <v>5.433</v>
       </c>
       <c r="L4" t="n">
-        <v>5.634</v>
+        <v>5.628</v>
       </c>
       <c r="M4" t="n">
-        <v>5.979</v>
+        <v>5.971</v>
       </c>
       <c r="N4" t="n">
-        <v>6.206</v>
+        <v>6.197</v>
       </c>
       <c r="O4" t="n">
-        <v>6.452</v>
+        <v>6.439</v>
       </c>
       <c r="P4" t="n">
-        <v>6.569</v>
+        <v>6.576</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.101</v>
+        <v>7.129</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.904</v>
+        <v>2.909</v>
       </c>
       <c r="G5" t="n">
-        <v>2.983</v>
+        <v>2.988</v>
       </c>
       <c r="H5" t="n">
-        <v>3.199</v>
+        <v>3.201</v>
       </c>
       <c r="I5" t="n">
-        <v>3.45</v>
+        <v>3.434</v>
       </c>
       <c r="J5" t="n">
-        <v>3.801</v>
+        <v>3.802</v>
       </c>
       <c r="K5" t="n">
-        <v>4.086</v>
+        <v>4.08</v>
       </c>
       <c r="L5" t="n">
-        <v>4.131</v>
+        <v>4.121</v>
       </c>
       <c r="M5" t="n">
-        <v>4.262</v>
+        <v>4.254</v>
       </c>
       <c r="N5" t="n">
-        <v>4.332</v>
+        <v>4.322</v>
       </c>
       <c r="O5" t="n">
-        <v>4.39</v>
+        <v>4.377</v>
       </c>
       <c r="P5" t="n">
-        <v>4.707</v>
+        <v>4.715</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.593</v>
+        <v>5.62</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.943</v>
+        <v>2.949</v>
       </c>
       <c r="G6" t="n">
-        <v>3.036</v>
+        <v>3.042</v>
       </c>
       <c r="H6" t="n">
-        <v>3.267</v>
+        <v>3.27</v>
       </c>
       <c r="I6" t="n">
-        <v>3.533</v>
+        <v>3.517</v>
       </c>
       <c r="J6" t="n">
-        <v>3.889</v>
+        <v>3.891</v>
       </c>
       <c r="K6" t="n">
-        <v>4.196</v>
+        <v>4.194</v>
       </c>
       <c r="L6" t="n">
-        <v>4.245</v>
+        <v>4.239</v>
       </c>
       <c r="M6" t="n">
-        <v>4.418</v>
+        <v>4.409</v>
       </c>
       <c r="N6" t="n">
-        <v>4.499</v>
+        <v>4.49</v>
       </c>
       <c r="O6" t="n">
-        <v>4.657</v>
+        <v>4.644</v>
       </c>
       <c r="P6" t="n">
-        <v>5.14</v>
+        <v>5.147</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.989</v>
+        <v>6.016</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.924</v>
+        <v>2.929</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>3.005</v>
       </c>
       <c r="H7" t="n">
-        <v>3.214</v>
+        <v>3.217</v>
       </c>
       <c r="I7" t="n">
-        <v>3.468</v>
+        <v>3.452</v>
       </c>
       <c r="J7" t="n">
-        <v>3.825</v>
+        <v>3.826</v>
       </c>
       <c r="K7" t="n">
-        <v>4.113</v>
+        <v>4.108</v>
       </c>
       <c r="L7" t="n">
-        <v>4.155</v>
+        <v>4.147</v>
       </c>
       <c r="M7" t="n">
-        <v>4.323</v>
+        <v>4.315</v>
       </c>
       <c r="N7" t="n">
-        <v>4.391</v>
+        <v>4.382</v>
       </c>
       <c r="O7" t="n">
-        <v>4.555</v>
+        <v>4.542</v>
       </c>
       <c r="P7" t="n">
-        <v>4.923</v>
+        <v>4.931</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.756</v>
+        <v>5.783</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.345</v>
+        <v>5.35</v>
       </c>
       <c r="G8" t="n">
-        <v>5.944</v>
+        <v>5.95</v>
       </c>
       <c r="H8" t="n">
-        <v>6.378</v>
+        <v>6.381</v>
       </c>
       <c r="I8" t="n">
-        <v>6.639</v>
+        <v>6.623</v>
       </c>
       <c r="J8" t="n">
-        <v>7.08</v>
+        <v>7.082</v>
       </c>
       <c r="K8" t="n">
-        <v>7.868</v>
+        <v>7.867</v>
       </c>
       <c r="L8" t="n">
-        <v>8.223000000000001</v>
+        <v>8.218</v>
       </c>
       <c r="M8" t="n">
-        <v>8.611000000000001</v>
+        <v>8.603</v>
       </c>
       <c r="N8" t="n">
-        <v>8.802</v>
+        <v>8.792999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.109999999999999</v>
+        <v>9.097</v>
       </c>
       <c r="P8" t="n">
-        <v>9.33</v>
+        <v>9.337</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.058</v>
+        <v>10.085</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.642</v>
+        <v>2.638</v>
       </c>
       <c r="G9" t="n">
-        <v>2.744</v>
+        <v>2.74</v>
       </c>
       <c r="H9" t="n">
-        <v>2.892</v>
+        <v>2.889</v>
       </c>
       <c r="I9" t="n">
-        <v>3.171</v>
+        <v>3.165</v>
       </c>
       <c r="J9" t="n">
-        <v>3.357</v>
+        <v>3.35</v>
       </c>
       <c r="K9" t="n">
-        <v>3.61</v>
+        <v>3.6</v>
       </c>
       <c r="L9" t="n">
-        <v>3.66</v>
+        <v>3.651</v>
       </c>
       <c r="M9" t="n">
-        <v>3.764</v>
+        <v>3.757</v>
       </c>
       <c r="N9" t="n">
-        <v>3.941</v>
+        <v>3.932</v>
       </c>
       <c r="O9" t="n">
-        <v>4.005</v>
+        <v>3.992</v>
       </c>
       <c r="P9" t="n">
-        <v>4.14</v>
+        <v>4.147</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.22</v>
+        <v>4.247</v>
       </c>
       <c r="R9" t="n">
-        <v>4.218</v>
+        <v>4.263</v>
       </c>
       <c r="S9" t="n">
-        <v>4.211</v>
+        <v>4.27</v>
       </c>
       <c r="T9" t="n">
-        <v>4.135</v>
+        <v>4.197</v>
       </c>
       <c r="U9" t="n">
-        <v>3.967</v>
+        <v>4.048</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.656</v>
+        <v>2.652</v>
       </c>
       <c r="G10" t="n">
-        <v>2.777</v>
+        <v>2.773</v>
       </c>
       <c r="H10" t="n">
-        <v>2.903</v>
+        <v>2.901</v>
       </c>
       <c r="I10" t="n">
-        <v>3.177</v>
+        <v>3.168</v>
       </c>
       <c r="J10" t="n">
-        <v>3.382</v>
+        <v>3.375</v>
       </c>
       <c r="K10" t="n">
-        <v>3.643</v>
+        <v>3.633</v>
       </c>
       <c r="L10" t="n">
-        <v>3.71</v>
+        <v>3.701</v>
       </c>
       <c r="M10" t="n">
-        <v>3.859</v>
+        <v>3.852</v>
       </c>
       <c r="N10" t="n">
-        <v>3.958</v>
+        <v>3.949</v>
       </c>
       <c r="O10" t="n">
-        <v>4.196</v>
+        <v>4.185</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.471</v>
+        <v>2.467</v>
       </c>
       <c r="G11" t="n">
-        <v>2.587</v>
+        <v>2.583</v>
       </c>
       <c r="H11" t="n">
-        <v>2.726</v>
+        <v>2.724</v>
       </c>
       <c r="I11" t="n">
-        <v>2.981</v>
+        <v>2.972</v>
       </c>
       <c r="J11" t="n">
-        <v>3.18</v>
+        <v>3.173</v>
       </c>
       <c r="K11" t="n">
-        <v>3.43</v>
+        <v>3.42</v>
       </c>
       <c r="L11" t="n">
-        <v>3.507</v>
+        <v>3.498</v>
       </c>
       <c r="M11" t="n">
-        <v>3.667</v>
+        <v>3.659</v>
       </c>
       <c r="N11" t="n">
-        <v>3.766</v>
+        <v>3.758</v>
       </c>
       <c r="O11" t="n">
-        <v>3.963</v>
+        <v>3.952</v>
       </c>
       <c r="P11" t="n">
-        <v>4.091</v>
+        <v>4.098</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.421</v>
+        <v>4.448</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1285,43 +1285,43 @@
         <v>3.217</v>
       </c>
       <c r="G12" t="n">
-        <v>3.409</v>
+        <v>3.41</v>
       </c>
       <c r="H12" t="n">
-        <v>3.615</v>
+        <v>3.614</v>
       </c>
       <c r="I12" t="n">
-        <v>3.854</v>
+        <v>3.839</v>
       </c>
       <c r="J12" t="n">
-        <v>4.236</v>
+        <v>4.234</v>
       </c>
       <c r="K12" t="n">
-        <v>4.477</v>
+        <v>4.476</v>
       </c>
       <c r="L12" t="n">
-        <v>4.563</v>
+        <v>4.556</v>
       </c>
       <c r="M12" t="n">
-        <v>4.731</v>
+        <v>4.724</v>
       </c>
       <c r="N12" t="n">
-        <v>4.818</v>
+        <v>4.808</v>
       </c>
       <c r="O12" t="n">
-        <v>4.993</v>
+        <v>4.979</v>
       </c>
       <c r="P12" t="n">
-        <v>5.176</v>
+        <v>5.183</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.536</v>
+        <v>5.562</v>
       </c>
       <c r="R12" t="n">
-        <v>5.71</v>
+        <v>5.755</v>
       </c>
       <c r="S12" t="n">
-        <v>5.914</v>
+        <v>5.973</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.97</v>
+        <v>2.971</v>
       </c>
       <c r="G13" t="n">
-        <v>3.099</v>
+        <v>3.1</v>
       </c>
       <c r="H13" t="n">
-        <v>3.283</v>
+        <v>3.282</v>
       </c>
       <c r="I13" t="n">
-        <v>3.502</v>
+        <v>3.487</v>
       </c>
       <c r="J13" t="n">
-        <v>3.873</v>
+        <v>3.87</v>
       </c>
       <c r="K13" t="n">
-        <v>4.11</v>
+        <v>4.109</v>
       </c>
       <c r="L13" t="n">
-        <v>4.203</v>
+        <v>4.195</v>
       </c>
       <c r="M13" t="n">
-        <v>4.359</v>
+        <v>4.351</v>
       </c>
       <c r="N13" t="n">
-        <v>4.446</v>
+        <v>4.436</v>
       </c>
       <c r="O13" t="n">
-        <v>4.622</v>
+        <v>4.608</v>
       </c>
       <c r="P13" t="n">
-        <v>4.767</v>
+        <v>4.775</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.057</v>
+        <v>5.083</v>
       </c>
       <c r="R13" t="n">
-        <v>5.259</v>
+        <v>5.304</v>
       </c>
       <c r="S13" t="n">
-        <v>5.476</v>
+        <v>5.536</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1431,43 +1431,43 @@
         <v>2.79</v>
       </c>
       <c r="G14" t="n">
-        <v>2.905</v>
+        <v>2.906</v>
       </c>
       <c r="H14" t="n">
-        <v>3.086</v>
+        <v>3.085</v>
       </c>
       <c r="I14" t="n">
-        <v>3.285</v>
+        <v>3.27</v>
       </c>
       <c r="J14" t="n">
-        <v>3.614</v>
+        <v>3.612</v>
       </c>
       <c r="K14" t="n">
-        <v>3.798</v>
+        <v>3.797</v>
       </c>
       <c r="L14" t="n">
-        <v>3.876</v>
+        <v>3.868</v>
       </c>
       <c r="M14" t="n">
-        <v>4.045</v>
+        <v>4.037</v>
       </c>
       <c r="N14" t="n">
-        <v>4.125</v>
+        <v>4.115</v>
       </c>
       <c r="O14" t="n">
-        <v>4.279</v>
+        <v>4.265</v>
       </c>
       <c r="P14" t="n">
-        <v>4.402</v>
+        <v>4.41</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.646</v>
+        <v>4.672</v>
       </c>
       <c r="R14" t="n">
-        <v>4.773</v>
+        <v>4.819</v>
       </c>
       <c r="S14" t="n">
-        <v>4.929</v>
+        <v>4.988</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.767</v>
+        <v>2.768</v>
       </c>
       <c r="G15" t="n">
-        <v>2.879</v>
+        <v>2.88</v>
       </c>
       <c r="H15" t="n">
-        <v>3.057</v>
+        <v>3.056</v>
       </c>
       <c r="I15" t="n">
-        <v>3.237</v>
+        <v>3.222</v>
       </c>
       <c r="J15" t="n">
-        <v>3.553</v>
+        <v>3.551</v>
       </c>
       <c r="K15" t="n">
-        <v>3.75</v>
+        <v>3.749</v>
       </c>
       <c r="L15" t="n">
-        <v>3.811</v>
+        <v>3.804</v>
       </c>
       <c r="M15" t="n">
-        <v>3.957</v>
+        <v>3.95</v>
       </c>
       <c r="N15" t="n">
-        <v>4.029</v>
+        <v>4.019</v>
       </c>
       <c r="O15" t="n">
-        <v>4.22</v>
+        <v>4.206</v>
       </c>
       <c r="P15" t="n">
-        <v>4.302</v>
+        <v>4.309</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.549</v>
+        <v>4.575</v>
       </c>
       <c r="R15" t="n">
-        <v>4.669</v>
+        <v>4.714</v>
       </c>
       <c r="S15" t="n">
-        <v>4.825</v>
+        <v>4.884</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.767</v>
+        <v>2.768</v>
       </c>
       <c r="G16" t="n">
-        <v>2.879</v>
+        <v>2.88</v>
       </c>
       <c r="H16" t="n">
-        <v>3.057</v>
+        <v>3.056</v>
       </c>
       <c r="I16" t="n">
-        <v>3.237</v>
+        <v>3.222</v>
       </c>
       <c r="J16" t="n">
-        <v>3.553</v>
+        <v>3.551</v>
       </c>
       <c r="K16" t="n">
-        <v>3.75</v>
+        <v>3.749</v>
       </c>
       <c r="L16" t="n">
-        <v>3.811</v>
+        <v>3.804</v>
       </c>
       <c r="M16" t="n">
-        <v>3.957</v>
+        <v>3.95</v>
       </c>
       <c r="N16" t="n">
-        <v>4.032</v>
+        <v>4.022</v>
       </c>
       <c r="O16" t="n">
-        <v>4.227</v>
+        <v>4.213</v>
       </c>
       <c r="P16" t="n">
-        <v>4.325</v>
+        <v>4.332</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.576</v>
+        <v>4.602</v>
       </c>
       <c r="R16" t="n">
-        <v>4.697</v>
+        <v>4.742</v>
       </c>
       <c r="S16" t="n">
-        <v>4.853</v>
+        <v>4.912</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.718</v>
+        <v>2.714</v>
       </c>
       <c r="G17" t="n">
-        <v>2.867</v>
+        <v>2.863</v>
       </c>
       <c r="H17" t="n">
-        <v>2.996</v>
+        <v>2.994</v>
       </c>
       <c r="I17" t="n">
-        <v>3.257</v>
+        <v>3.249</v>
       </c>
       <c r="J17" t="n">
-        <v>3.458</v>
+        <v>3.45</v>
       </c>
       <c r="K17" t="n">
-        <v>3.72</v>
+        <v>3.711</v>
       </c>
       <c r="L17" t="n">
-        <v>3.792</v>
+        <v>3.785</v>
       </c>
       <c r="M17" t="n">
-        <v>3.983</v>
+        <v>3.975</v>
       </c>
       <c r="N17" t="n">
-        <v>4.06</v>
+        <v>4.051</v>
       </c>
       <c r="O17" t="n">
-        <v>4.226</v>
+        <v>4.215</v>
       </c>
       <c r="P17" t="n">
-        <v>4.371</v>
+        <v>4.379</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.719</v>
+        <v>2.715</v>
       </c>
       <c r="G18" t="n">
-        <v>2.868</v>
+        <v>2.864</v>
       </c>
       <c r="H18" t="n">
-        <v>2.996</v>
+        <v>2.994</v>
       </c>
       <c r="I18" t="n">
-        <v>3.258</v>
+        <v>3.249</v>
       </c>
       <c r="J18" t="n">
-        <v>3.458</v>
+        <v>3.45</v>
       </c>
       <c r="K18" t="n">
-        <v>3.721</v>
+        <v>3.712</v>
       </c>
       <c r="L18" t="n">
-        <v>3.792</v>
+        <v>3.785</v>
       </c>
       <c r="M18" t="n">
-        <v>3.983</v>
+        <v>3.975</v>
       </c>
       <c r="N18" t="n">
-        <v>4.061</v>
+        <v>4.052</v>
       </c>
       <c r="O18" t="n">
-        <v>4.224</v>
+        <v>4.212</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.78</v>
+        <v>2.781</v>
       </c>
       <c r="G19" t="n">
-        <v>2.894</v>
+        <v>2.895</v>
       </c>
       <c r="H19" t="n">
-        <v>3.074</v>
+        <v>3.073</v>
       </c>
       <c r="I19" t="n">
-        <v>3.272</v>
+        <v>3.255</v>
       </c>
       <c r="J19" t="n">
-        <v>3.597</v>
+        <v>3.594</v>
       </c>
       <c r="K19" t="n">
-        <v>3.794</v>
+        <v>3.793</v>
       </c>
       <c r="L19" t="n">
-        <v>3.872</v>
+        <v>3.864</v>
       </c>
       <c r="M19" t="n">
-        <v>4.035</v>
+        <v>4.027</v>
       </c>
       <c r="N19" t="n">
-        <v>4.115</v>
+        <v>4.105</v>
       </c>
       <c r="O19" t="n">
-        <v>4.263</v>
+        <v>4.249</v>
       </c>
       <c r="P19" t="n">
-        <v>4.361</v>
+        <v>4.369</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.587</v>
+        <v>4.612</v>
       </c>
       <c r="R19" t="n">
-        <v>4.716</v>
+        <v>4.761</v>
       </c>
       <c r="S19" t="n">
-        <v>4.864</v>
+        <v>4.923</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.61</v>
+        <v>2.609</v>
       </c>
       <c r="G20" t="n">
-        <v>2.692</v>
+        <v>2.691</v>
       </c>
       <c r="H20" t="n">
-        <v>2.763</v>
+        <v>2.76</v>
       </c>
       <c r="I20" t="n">
-        <v>2.888</v>
+        <v>2.863</v>
       </c>
       <c r="J20" t="n">
-        <v>3.376</v>
+        <v>3.375</v>
       </c>
       <c r="K20" t="n">
-        <v>3.627</v>
+        <v>3.622</v>
       </c>
       <c r="L20" t="n">
-        <v>3.679</v>
+        <v>3.673</v>
       </c>
       <c r="M20" t="n">
-        <v>3.795</v>
+        <v>3.787</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.902</v>
+        <v>2.904</v>
       </c>
       <c r="G21" t="n">
-        <v>2.991</v>
+        <v>2.992</v>
       </c>
       <c r="H21" t="n">
-        <v>3.195</v>
+        <v>3.194</v>
       </c>
       <c r="I21" t="n">
-        <v>3.372</v>
+        <v>3.359</v>
       </c>
       <c r="J21" t="n">
         <v>3.739</v>
       </c>
       <c r="K21" t="n">
-        <v>4.026</v>
+        <v>4.02</v>
       </c>
       <c r="L21" t="n">
-        <v>4.111</v>
+        <v>4.1</v>
       </c>
       <c r="M21" t="n">
-        <v>4.258</v>
+        <v>4.247</v>
       </c>
       <c r="N21" t="n">
-        <v>4.352</v>
+        <v>4.341</v>
       </c>
       <c r="O21" t="n">
-        <v>4.472</v>
+        <v>4.459</v>
       </c>
       <c r="P21" t="n">
-        <v>4.623</v>
+        <v>4.629</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.748</v>
+        <v>4.773</v>
       </c>
       <c r="R21" t="n">
-        <v>4.766</v>
+        <v>4.812</v>
       </c>
       <c r="S21" t="n">
-        <v>4.822</v>
+        <v>4.881</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.849</v>
+        <v>2.851</v>
       </c>
       <c r="G22" t="n">
-        <v>2.937</v>
+        <v>2.938</v>
       </c>
       <c r="H22" t="n">
-        <v>3.127</v>
+        <v>3.125</v>
       </c>
       <c r="I22" t="n">
-        <v>3.291</v>
+        <v>3.277</v>
       </c>
       <c r="J22" t="n">
         <v>3.625</v>
       </c>
       <c r="K22" t="n">
-        <v>3.908</v>
+        <v>3.902</v>
       </c>
       <c r="L22" t="n">
-        <v>3.978</v>
+        <v>3.967</v>
       </c>
       <c r="M22" t="n">
-        <v>4.127</v>
+        <v>4.117</v>
       </c>
       <c r="N22" t="n">
-        <v>4.225</v>
+        <v>4.215</v>
       </c>
       <c r="O22" t="n">
-        <v>4.34</v>
+        <v>4.33</v>
       </c>
       <c r="P22" t="n">
-        <v>4.485</v>
+        <v>4.492</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.606</v>
+        <v>4.631</v>
       </c>
       <c r="R22" t="n">
-        <v>4.615</v>
+        <v>4.66</v>
       </c>
       <c r="S22" t="n">
-        <v>4.668</v>
+        <v>4.726</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2088,46 +2088,46 @@
         <v>2.801</v>
       </c>
       <c r="G23" t="n">
-        <v>2.892</v>
+        <v>2.893</v>
       </c>
       <c r="H23" t="n">
-        <v>3.068</v>
+        <v>3.067</v>
       </c>
       <c r="I23" t="n">
-        <v>3.24</v>
+        <v>3.227</v>
       </c>
       <c r="J23" t="n">
-        <v>3.567</v>
+        <v>3.566</v>
       </c>
       <c r="K23" t="n">
-        <v>3.809</v>
+        <v>3.803</v>
       </c>
       <c r="L23" t="n">
-        <v>3.877</v>
+        <v>3.867</v>
       </c>
       <c r="M23" t="n">
-        <v>4.021</v>
+        <v>4.011</v>
       </c>
       <c r="N23" t="n">
-        <v>4.12</v>
+        <v>4.109</v>
       </c>
       <c r="O23" t="n">
-        <v>4.217</v>
+        <v>4.203</v>
       </c>
       <c r="P23" t="n">
-        <v>4.35</v>
+        <v>4.355</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.412</v>
+        <v>4.438</v>
       </c>
       <c r="R23" t="n">
-        <v>4.398</v>
+        <v>4.444</v>
       </c>
       <c r="S23" t="n">
-        <v>4.422</v>
+        <v>4.48</v>
       </c>
       <c r="T23" t="n">
-        <v>4.34</v>
+        <v>4.401</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.736</v>
+        <v>2.739</v>
       </c>
       <c r="G24" t="n">
-        <v>2.807</v>
+        <v>2.808</v>
       </c>
       <c r="H24" t="n">
-        <v>2.967</v>
+        <v>2.966</v>
       </c>
       <c r="I24" t="n">
-        <v>3.173</v>
+        <v>3.166</v>
       </c>
       <c r="J24" t="n">
-        <v>3.464</v>
+        <v>3.463</v>
       </c>
       <c r="K24" t="n">
-        <v>3.693</v>
+        <v>3.687</v>
       </c>
       <c r="L24" t="n">
-        <v>3.757</v>
+        <v>3.747</v>
       </c>
       <c r="M24" t="n">
-        <v>3.884</v>
+        <v>3.874</v>
       </c>
       <c r="N24" t="n">
-        <v>3.998</v>
+        <v>3.986</v>
       </c>
       <c r="O24" t="n">
-        <v>4.209</v>
+        <v>4.195</v>
       </c>
       <c r="P24" t="n">
-        <v>4.288</v>
+        <v>4.293</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.337</v>
+        <v>4.362</v>
       </c>
       <c r="R24" t="n">
-        <v>4.32</v>
+        <v>4.366</v>
       </c>
       <c r="S24" t="n">
-        <v>4.337</v>
+        <v>4.395</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2234,46 +2234,46 @@
         <v>2.795</v>
       </c>
       <c r="G25" t="n">
-        <v>2.892</v>
+        <v>2.893</v>
       </c>
       <c r="H25" t="n">
-        <v>3.071</v>
+        <v>3.07</v>
       </c>
       <c r="I25" t="n">
-        <v>3.248</v>
+        <v>3.234</v>
       </c>
       <c r="J25" t="n">
-        <v>3.582</v>
+        <v>3.581</v>
       </c>
       <c r="K25" t="n">
-        <v>3.841</v>
+        <v>3.835</v>
       </c>
       <c r="L25" t="n">
-        <v>3.908</v>
+        <v>3.897</v>
       </c>
       <c r="M25" t="n">
-        <v>4.052</v>
+        <v>4.042</v>
       </c>
       <c r="N25" t="n">
-        <v>4.147</v>
+        <v>4.136</v>
       </c>
       <c r="O25" t="n">
-        <v>4.246</v>
+        <v>4.232</v>
       </c>
       <c r="P25" t="n">
-        <v>4.372</v>
+        <v>4.377</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.446</v>
+        <v>4.471</v>
       </c>
       <c r="R25" t="n">
-        <v>4.422</v>
+        <v>4.468</v>
       </c>
       <c r="S25" t="n">
-        <v>4.445</v>
+        <v>4.504</v>
       </c>
       <c r="T25" t="n">
-        <v>4.358</v>
+        <v>4.419</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.068</v>
+        <v>3.065</v>
       </c>
       <c r="G26" t="n">
-        <v>3.219</v>
+        <v>3.217</v>
       </c>
       <c r="H26" t="n">
-        <v>3.5</v>
+        <v>3.499</v>
       </c>
       <c r="I26" t="n">
-        <v>3.736</v>
+        <v>3.717</v>
       </c>
       <c r="J26" t="n">
-        <v>4.22</v>
+        <v>4.217</v>
       </c>
       <c r="K26" t="n">
-        <v>4.659</v>
+        <v>4.653</v>
       </c>
       <c r="L26" t="n">
-        <v>4.791</v>
+        <v>4.78</v>
       </c>
       <c r="M26" t="n">
-        <v>4.998</v>
+        <v>4.988</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.324</v>
+        <v>5.309</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.876</v>
+        <v>2.875</v>
       </c>
       <c r="G27" t="n">
-        <v>2.975</v>
+        <v>2.974</v>
       </c>
       <c r="H27" t="n">
-        <v>3.164</v>
+        <v>3.163</v>
       </c>
       <c r="I27" t="n">
-        <v>3.37</v>
+        <v>3.351</v>
       </c>
       <c r="J27" t="n">
-        <v>3.727</v>
+        <v>3.723</v>
       </c>
       <c r="K27" t="n">
-        <v>3.975</v>
+        <v>3.971</v>
       </c>
       <c r="L27" t="n">
-        <v>4.06</v>
+        <v>4.049</v>
       </c>
       <c r="M27" t="n">
-        <v>4.211</v>
+        <v>4.203</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.417</v>
+        <v>4.403</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.979</v>
+        <v>2.978</v>
       </c>
       <c r="G28" t="n">
-        <v>3.086</v>
+        <v>3.085</v>
       </c>
       <c r="H28" t="n">
         <v>3.289</v>
       </c>
       <c r="I28" t="n">
-        <v>3.508</v>
+        <v>3.489</v>
       </c>
       <c r="J28" t="n">
-        <v>3.9</v>
+        <v>3.896</v>
       </c>
       <c r="K28" t="n">
-        <v>4.168</v>
+        <v>4.164</v>
       </c>
       <c r="L28" t="n">
-        <v>4.263</v>
+        <v>4.252</v>
       </c>
       <c r="M28" t="n">
-        <v>4.423</v>
+        <v>4.415</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.709</v>
+        <v>4.695</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.826</v>
+        <v>2.825</v>
       </c>
       <c r="G29" t="n">
         <v>2.925</v>
@@ -2532,25 +2532,25 @@
         <v>3.104</v>
       </c>
       <c r="I29" t="n">
-        <v>3.299</v>
+        <v>3.281</v>
       </c>
       <c r="J29" t="n">
-        <v>3.639</v>
+        <v>3.636</v>
       </c>
       <c r="K29" t="n">
-        <v>3.871</v>
+        <v>3.867</v>
       </c>
       <c r="L29" t="n">
-        <v>3.945</v>
+        <v>3.934</v>
       </c>
       <c r="M29" t="n">
-        <v>4.073</v>
+        <v>4.065</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.287</v>
+        <v>4.273</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.112</v>
+        <v>3.109</v>
       </c>
       <c r="G30" t="n">
-        <v>3.198</v>
+        <v>3.196</v>
       </c>
       <c r="H30" t="n">
-        <v>3.432</v>
+        <v>3.431</v>
       </c>
       <c r="I30" t="n">
-        <v>3.663</v>
+        <v>3.643</v>
       </c>
       <c r="J30" t="n">
-        <v>4.091</v>
+        <v>4.087</v>
       </c>
       <c r="K30" t="n">
-        <v>4.46</v>
+        <v>4.454</v>
       </c>
       <c r="L30" t="n">
-        <v>4.57</v>
+        <v>4.56</v>
       </c>
       <c r="M30" t="n">
-        <v>4.768</v>
+        <v>4.758</v>
       </c>
       <c r="N30" t="n">
-        <v>4.957</v>
+        <v>4.946</v>
       </c>
       <c r="O30" t="n">
-        <v>5.274</v>
+        <v>5.259</v>
       </c>
       <c r="P30" t="n">
-        <v>5.515</v>
+        <v>5.522</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.283</v>
+        <v>6.31</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.441</v>
+        <v>3.438</v>
       </c>
       <c r="G31" t="n">
-        <v>3.563</v>
+        <v>3.561</v>
       </c>
       <c r="H31" t="n">
-        <v>3.846</v>
+        <v>3.845</v>
       </c>
       <c r="I31" t="n">
-        <v>4.093</v>
+        <v>4.072</v>
       </c>
       <c r="J31" t="n">
-        <v>4.582</v>
+        <v>4.579</v>
       </c>
       <c r="K31" t="n">
-        <v>4.993</v>
+        <v>4.987</v>
       </c>
       <c r="L31" t="n">
-        <v>5.183</v>
+        <v>5.172</v>
       </c>
       <c r="M31" t="n">
-        <v>5.499</v>
+        <v>5.489</v>
       </c>
       <c r="N31" t="n">
-        <v>5.816</v>
+        <v>5.805</v>
       </c>
       <c r="O31" t="n">
-        <v>6.31</v>
+        <v>6.295</v>
       </c>
       <c r="P31" t="n">
-        <v>6.503</v>
+        <v>6.51</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.257</v>
+        <v>7.284</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.211</v>
+        <v>3.207</v>
       </c>
       <c r="G32" t="n">
-        <v>3.316</v>
+        <v>3.314</v>
       </c>
       <c r="H32" t="n">
-        <v>3.576</v>
+        <v>3.574</v>
       </c>
       <c r="I32" t="n">
-        <v>3.822</v>
+        <v>3.802</v>
       </c>
       <c r="J32" t="n">
-        <v>4.269</v>
+        <v>4.265</v>
       </c>
       <c r="K32" t="n">
-        <v>4.645</v>
+        <v>4.639</v>
       </c>
       <c r="L32" t="n">
-        <v>4.775</v>
+        <v>4.764</v>
       </c>
       <c r="M32" t="n">
-        <v>5.041</v>
+        <v>5.031</v>
       </c>
       <c r="N32" t="n">
-        <v>5.318</v>
+        <v>5.306</v>
       </c>
       <c r="O32" t="n">
-        <v>5.72</v>
+        <v>5.705</v>
       </c>
       <c r="P32" t="n">
-        <v>5.975</v>
+        <v>5.982</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.744</v>
+        <v>6.771</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.976</v>
+        <v>2.973</v>
       </c>
       <c r="G33" t="n">
-        <v>3.061</v>
+        <v>3.059</v>
       </c>
       <c r="H33" t="n">
-        <v>3.248</v>
+        <v>3.247</v>
       </c>
       <c r="I33" t="n">
-        <v>3.447</v>
+        <v>3.426</v>
       </c>
       <c r="J33" t="n">
-        <v>3.795</v>
+        <v>3.793</v>
       </c>
       <c r="K33" t="n">
-        <v>4.1</v>
+        <v>4.094</v>
       </c>
       <c r="L33" t="n">
-        <v>4.173</v>
+        <v>4.162</v>
       </c>
       <c r="M33" t="n">
-        <v>4.294</v>
+        <v>4.284</v>
       </c>
       <c r="N33" t="n">
-        <v>4.348</v>
+        <v>4.336</v>
       </c>
       <c r="O33" t="n">
-        <v>4.429</v>
+        <v>4.414</v>
       </c>
       <c r="P33" t="n">
-        <v>4.547</v>
+        <v>4.554</v>
       </c>
       <c r="Q33" t="n">
-        <v>5</v>
+        <v>5.027</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.036</v>
+        <v>3.033</v>
       </c>
       <c r="G34" t="n">
-        <v>3.114</v>
+        <v>3.112</v>
       </c>
       <c r="H34" t="n">
         <v>3.309</v>
       </c>
       <c r="I34" t="n">
-        <v>3.515</v>
+        <v>3.495</v>
       </c>
       <c r="J34" t="n">
-        <v>3.867</v>
+        <v>3.864</v>
       </c>
       <c r="K34" t="n">
-        <v>4.177</v>
+        <v>4.171</v>
       </c>
       <c r="L34" t="n">
-        <v>4.252</v>
+        <v>4.242</v>
       </c>
       <c r="M34" t="n">
-        <v>4.385</v>
+        <v>4.375</v>
       </c>
       <c r="N34" t="n">
-        <v>4.451</v>
+        <v>4.439</v>
       </c>
       <c r="O34" t="n">
-        <v>4.598</v>
+        <v>4.583</v>
       </c>
       <c r="P34" t="n">
-        <v>4.841</v>
+        <v>4.849</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.701</v>
+        <v>5.728</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.01</v>
+        <v>3.007</v>
       </c>
       <c r="G35" t="n">
-        <v>3.088</v>
+        <v>3.086</v>
       </c>
       <c r="H35" t="n">
-        <v>3.277</v>
+        <v>3.276</v>
       </c>
       <c r="I35" t="n">
-        <v>3.482</v>
+        <v>3.461</v>
       </c>
       <c r="J35" t="n">
-        <v>3.835</v>
+        <v>3.832</v>
       </c>
       <c r="K35" t="n">
-        <v>4.131</v>
+        <v>4.125</v>
       </c>
       <c r="L35" t="n">
-        <v>4.207</v>
+        <v>4.196</v>
       </c>
       <c r="M35" t="n">
-        <v>4.332</v>
+        <v>4.321</v>
       </c>
       <c r="N35" t="n">
-        <v>4.387</v>
+        <v>4.375</v>
       </c>
       <c r="O35" t="n">
-        <v>4.495</v>
+        <v>4.48</v>
       </c>
       <c r="P35" t="n">
-        <v>4.644</v>
+        <v>4.651</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.337</v>
+        <v>5.364</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.907</v>
+        <v>2.903</v>
       </c>
       <c r="G36" t="n">
-        <v>2.986</v>
+        <v>2.983</v>
       </c>
       <c r="H36" t="n">
-        <v>3.165</v>
+        <v>3.164</v>
       </c>
       <c r="I36" t="n">
-        <v>3.367</v>
+        <v>3.346</v>
       </c>
       <c r="J36" t="n">
-        <v>3.731</v>
+        <v>3.728</v>
       </c>
       <c r="K36" t="n">
-        <v>4.025</v>
+        <v>4.019</v>
       </c>
       <c r="L36" t="n">
-        <v>4.098</v>
+        <v>4.088</v>
       </c>
       <c r="M36" t="n">
-        <v>4.196</v>
+        <v>4.186</v>
       </c>
       <c r="N36" t="n">
-        <v>4.251</v>
+        <v>4.239</v>
       </c>
       <c r="O36" t="n">
-        <v>4.338</v>
+        <v>4.323</v>
       </c>
       <c r="P36" t="n">
-        <v>4.445</v>
+        <v>4.453</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.717</v>
+        <v>4.744</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.784</v>
+        <v>3.782</v>
       </c>
       <c r="G37" t="n">
-        <v>4.257</v>
+        <v>4.256</v>
       </c>
       <c r="H37" t="n">
-        <v>4.822</v>
+        <v>4.821</v>
       </c>
       <c r="I37" t="n">
-        <v>5.154</v>
+        <v>5.134</v>
       </c>
       <c r="J37" t="n">
-        <v>6.073</v>
+        <v>6.07</v>
       </c>
       <c r="K37" t="n">
-        <v>7.033</v>
+        <v>7.027</v>
       </c>
       <c r="L37" t="n">
-        <v>7.383</v>
+        <v>7.372</v>
       </c>
       <c r="M37" t="n">
-        <v>7.771</v>
+        <v>7.761</v>
       </c>
       <c r="N37" t="n">
-        <v>7.967</v>
+        <v>7.956</v>
       </c>
       <c r="O37" t="n">
-        <v>8.189</v>
+        <v>8.173999999999999</v>
       </c>
       <c r="P37" t="n">
-        <v>8.303000000000001</v>
+        <v>8.31</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.744999999999999</v>
+        <v>8.772</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.843</v>
+        <v>4.841</v>
       </c>
       <c r="G38" t="n">
-        <v>5.57</v>
+        <v>5.569</v>
       </c>
       <c r="H38" t="n">
-        <v>6.346</v>
+        <v>6.345</v>
       </c>
       <c r="I38" t="n">
-        <v>6.835</v>
+        <v>6.815</v>
       </c>
       <c r="J38" t="n">
-        <v>8.016</v>
+        <v>8.013</v>
       </c>
       <c r="K38" t="n">
-        <v>9.154999999999999</v>
+        <v>9.148999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.664999999999999</v>
+        <v>9.654999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.183</v>
+        <v>10.173</v>
       </c>
       <c r="N38" t="n">
-        <v>10.386</v>
+        <v>10.375</v>
       </c>
       <c r="O38" t="n">
-        <v>10.59</v>
+        <v>10.575</v>
       </c>
       <c r="P38" t="n">
-        <v>10.7</v>
+        <v>10.708</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.196</v>
+        <v>11.223</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.164</v>
+        <v>4.162</v>
       </c>
       <c r="G39" t="n">
-        <v>4.768</v>
+        <v>4.767</v>
       </c>
       <c r="H39" t="n">
-        <v>5.411</v>
+        <v>5.41</v>
       </c>
       <c r="I39" t="n">
-        <v>5.839</v>
+        <v>5.819</v>
       </c>
       <c r="J39" t="n">
-        <v>6.889</v>
+        <v>6.885</v>
       </c>
       <c r="K39" t="n">
-        <v>7.988</v>
+        <v>7.982</v>
       </c>
       <c r="L39" t="n">
-        <v>8.420999999999999</v>
+        <v>8.41</v>
       </c>
       <c r="M39" t="n">
-        <v>8.819000000000001</v>
+        <v>8.808999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>9.013999999999999</v>
+        <v>9.002000000000001</v>
       </c>
       <c r="O39" t="n">
-        <v>9.24</v>
+        <v>9.225</v>
       </c>
       <c r="P39" t="n">
-        <v>9.355</v>
+        <v>9.362</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.840999999999999</v>
+        <v>9.868</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.304</v>
+        <v>3.3</v>
       </c>
       <c r="G40" t="n">
-        <v>3.436</v>
+        <v>3.434</v>
       </c>
       <c r="H40" t="n">
-        <v>3.691</v>
+        <v>3.69</v>
       </c>
       <c r="I40" t="n">
-        <v>3.937</v>
+        <v>3.917</v>
       </c>
       <c r="J40" t="n">
-        <v>4.382</v>
+        <v>4.379</v>
       </c>
       <c r="K40" t="n">
-        <v>4.766</v>
+        <v>4.76</v>
       </c>
       <c r="L40" t="n">
-        <v>4.895</v>
+        <v>4.884</v>
       </c>
       <c r="M40" t="n">
-        <v>5.111</v>
+        <v>5.101</v>
       </c>
       <c r="N40" t="n">
-        <v>5.315</v>
+        <v>5.303</v>
       </c>
       <c r="O40" t="n">
-        <v>5.653</v>
+        <v>5.638</v>
       </c>
       <c r="P40" t="n">
-        <v>5.936</v>
+        <v>5.943</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.734</v>
+        <v>6.761</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.69</v>
+        <v>3.687</v>
       </c>
       <c r="G41" t="n">
-        <v>3.864</v>
+        <v>3.863</v>
       </c>
       <c r="H41" t="n">
-        <v>4.176</v>
+        <v>4.174</v>
       </c>
       <c r="I41" t="n">
-        <v>4.441</v>
+        <v>4.42</v>
       </c>
       <c r="J41" t="n">
-        <v>4.937</v>
+        <v>4.934</v>
       </c>
       <c r="K41" t="n">
-        <v>5.366</v>
+        <v>5.36</v>
       </c>
       <c r="L41" t="n">
-        <v>5.574</v>
+        <v>5.563</v>
       </c>
       <c r="M41" t="n">
-        <v>5.914</v>
+        <v>5.904</v>
       </c>
       <c r="N41" t="n">
-        <v>6.245</v>
+        <v>6.234</v>
       </c>
       <c r="O41" t="n">
-        <v>6.769</v>
+        <v>6.754</v>
       </c>
       <c r="P41" t="n">
-        <v>6.995</v>
+        <v>7.003</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.781</v>
+        <v>7.808</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.425</v>
+        <v>3.422</v>
       </c>
       <c r="G42" t="n">
-        <v>3.585</v>
+        <v>3.583</v>
       </c>
       <c r="H42" t="n">
-        <v>3.867</v>
+        <v>3.865</v>
       </c>
       <c r="I42" t="n">
-        <v>4.125</v>
+        <v>4.105</v>
       </c>
       <c r="J42" t="n">
-        <v>4.585</v>
+        <v>4.581</v>
       </c>
       <c r="K42" t="n">
-        <v>4.987</v>
+        <v>4.981</v>
       </c>
       <c r="L42" t="n">
-        <v>5.131</v>
+        <v>5.12</v>
       </c>
       <c r="M42" t="n">
-        <v>5.418</v>
+        <v>5.408</v>
       </c>
       <c r="N42" t="n">
-        <v>5.729</v>
+        <v>5.718</v>
       </c>
       <c r="O42" t="n">
-        <v>6.145</v>
+        <v>6.13</v>
       </c>
       <c r="P42" t="n">
-        <v>6.438</v>
+        <v>6.445</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.247</v>
+        <v>7.274</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.124</v>
+        <v>3.121</v>
       </c>
       <c r="G43" t="n">
-        <v>3.244</v>
+        <v>3.242</v>
       </c>
       <c r="H43" t="n">
         <v>3.448</v>
       </c>
       <c r="I43" t="n">
-        <v>3.656</v>
+        <v>3.635</v>
       </c>
       <c r="J43" t="n">
-        <v>4.022</v>
+        <v>4.02</v>
       </c>
       <c r="K43" t="n">
-        <v>4.332</v>
+        <v>4.326</v>
       </c>
       <c r="L43" t="n">
-        <v>4.415</v>
+        <v>4.404</v>
       </c>
       <c r="M43" t="n">
-        <v>4.55</v>
+        <v>4.539</v>
       </c>
       <c r="N43" t="n">
-        <v>4.616</v>
+        <v>4.604</v>
       </c>
       <c r="O43" t="n">
-        <v>4.743</v>
+        <v>4.727</v>
       </c>
       <c r="P43" t="n">
-        <v>4.912</v>
+        <v>4.92</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.61</v>
+        <v>5.637</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46157</v>
+        <v>46160</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.985</v>
+        <v>2.981</v>
       </c>
       <c r="G44" t="n">
-        <v>3.095</v>
+        <v>3.092</v>
       </c>
       <c r="H44" t="n">
-        <v>3.288</v>
+        <v>3.287</v>
       </c>
       <c r="I44" t="n">
-        <v>3.494</v>
+        <v>3.473</v>
       </c>
       <c r="J44" t="n">
-        <v>3.872</v>
+        <v>3.869</v>
       </c>
       <c r="K44" t="n">
-        <v>4.177</v>
+        <v>4.171</v>
       </c>
       <c r="L44" t="n">
-        <v>4.259</v>
+        <v>4.248</v>
       </c>
       <c r="M44" t="n">
-        <v>4.367</v>
+        <v>4.356</v>
       </c>
       <c r="N44" t="n">
-        <v>4.433</v>
+        <v>4.421</v>
       </c>
       <c r="O44" t="n">
-        <v>4.539</v>
+        <v>4.523</v>
       </c>
       <c r="P44" t="n">
-        <v>4.675</v>
+        <v>4.683</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.981</v>
+        <v>5.008</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-19 ~ 2026-05-19
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.215</v>
+        <v>3.22</v>
       </c>
       <c r="G2" t="n">
-        <v>3.445</v>
+        <v>3.455</v>
       </c>
       <c r="H2" t="n">
-        <v>3.695</v>
+        <v>3.706</v>
       </c>
       <c r="I2" t="n">
-        <v>3.864</v>
+        <v>3.879</v>
       </c>
       <c r="J2" t="n">
-        <v>4.244</v>
+        <v>4.255</v>
       </c>
       <c r="K2" t="n">
-        <v>4.679</v>
+        <v>4.69</v>
       </c>
       <c r="L2" t="n">
-        <v>4.874</v>
+        <v>4.876</v>
       </c>
       <c r="M2" t="n">
-        <v>5.196</v>
+        <v>5.195</v>
       </c>
       <c r="N2" t="n">
-        <v>5.51</v>
+        <v>5.495</v>
       </c>
       <c r="O2" t="n">
-        <v>5.778</v>
+        <v>5.751</v>
       </c>
       <c r="P2" t="n">
-        <v>6.046</v>
+        <v>6.017</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.707</v>
+        <v>6.665</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.238</v>
+        <v>4.243</v>
       </c>
       <c r="G3" t="n">
-        <v>4.65</v>
+        <v>4.66</v>
       </c>
       <c r="H3" t="n">
-        <v>4.933</v>
+        <v>4.944</v>
       </c>
       <c r="I3" t="n">
-        <v>5.096</v>
+        <v>5.112</v>
       </c>
       <c r="J3" t="n">
-        <v>5.49</v>
+        <v>5.501</v>
       </c>
       <c r="K3" t="n">
-        <v>5.995</v>
+        <v>6.007</v>
       </c>
       <c r="L3" t="n">
-        <v>6.259</v>
+        <v>6.262</v>
       </c>
       <c r="M3" t="n">
-        <v>6.613</v>
+        <v>6.612</v>
       </c>
       <c r="N3" t="n">
-        <v>6.869</v>
+        <v>6.854</v>
       </c>
       <c r="O3" t="n">
-        <v>7.088</v>
+        <v>7.061</v>
       </c>
       <c r="P3" t="n">
-        <v>7.226</v>
+        <v>7.197</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.776</v>
+        <v>7.734</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.731</v>
+        <v>3.735</v>
       </c>
       <c r="G4" t="n">
-        <v>4.031</v>
+        <v>4.041</v>
       </c>
       <c r="H4" t="n">
-        <v>4.343</v>
+        <v>4.354</v>
       </c>
       <c r="I4" t="n">
-        <v>4.539</v>
+        <v>4.555</v>
       </c>
       <c r="J4" t="n">
-        <v>4.936</v>
+        <v>4.947</v>
       </c>
       <c r="K4" t="n">
-        <v>5.433</v>
+        <v>5.445</v>
       </c>
       <c r="L4" t="n">
-        <v>5.628</v>
+        <v>5.631</v>
       </c>
       <c r="M4" t="n">
-        <v>5.971</v>
+        <v>5.97</v>
       </c>
       <c r="N4" t="n">
-        <v>6.197</v>
+        <v>6.182</v>
       </c>
       <c r="O4" t="n">
-        <v>6.439</v>
+        <v>6.412</v>
       </c>
       <c r="P4" t="n">
-        <v>6.576</v>
+        <v>6.547</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.129</v>
+        <v>7.087</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.909</v>
+        <v>2.913</v>
       </c>
       <c r="G5" t="n">
-        <v>2.988</v>
+        <v>2.996</v>
       </c>
       <c r="H5" t="n">
-        <v>3.201</v>
+        <v>3.213</v>
       </c>
       <c r="I5" t="n">
-        <v>3.434</v>
+        <v>3.451</v>
       </c>
       <c r="J5" t="n">
-        <v>3.802</v>
+        <v>3.813</v>
       </c>
       <c r="K5" t="n">
-        <v>4.08</v>
+        <v>4.091</v>
       </c>
       <c r="L5" t="n">
-        <v>4.121</v>
+        <v>4.124</v>
       </c>
       <c r="M5" t="n">
-        <v>4.254</v>
+        <v>4.253</v>
       </c>
       <c r="N5" t="n">
-        <v>4.322</v>
+        <v>4.307</v>
       </c>
       <c r="O5" t="n">
-        <v>4.377</v>
+        <v>4.35</v>
       </c>
       <c r="P5" t="n">
-        <v>4.715</v>
+        <v>4.686</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.62</v>
+        <v>5.578</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.949</v>
+        <v>2.954</v>
       </c>
       <c r="G6" t="n">
-        <v>3.042</v>
+        <v>3.052</v>
       </c>
       <c r="H6" t="n">
-        <v>3.27</v>
+        <v>3.282</v>
       </c>
       <c r="I6" t="n">
-        <v>3.517</v>
+        <v>3.534</v>
       </c>
       <c r="J6" t="n">
-        <v>3.891</v>
+        <v>3.902</v>
       </c>
       <c r="K6" t="n">
-        <v>4.194</v>
+        <v>4.206</v>
       </c>
       <c r="L6" t="n">
-        <v>4.239</v>
+        <v>4.241</v>
       </c>
       <c r="M6" t="n">
-        <v>4.409</v>
+        <v>4.408</v>
       </c>
       <c r="N6" t="n">
-        <v>4.49</v>
+        <v>4.475</v>
       </c>
       <c r="O6" t="n">
-        <v>4.644</v>
+        <v>4.617</v>
       </c>
       <c r="P6" t="n">
-        <v>5.147</v>
+        <v>5.118</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.016</v>
+        <v>5.974</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.929</v>
+        <v>2.934</v>
       </c>
       <c r="G7" t="n">
-        <v>3.005</v>
+        <v>3.015</v>
       </c>
       <c r="H7" t="n">
-        <v>3.217</v>
+        <v>3.229</v>
       </c>
       <c r="I7" t="n">
-        <v>3.452</v>
+        <v>3.469</v>
       </c>
       <c r="J7" t="n">
-        <v>3.826</v>
+        <v>3.837</v>
       </c>
       <c r="K7" t="n">
-        <v>4.108</v>
+        <v>4.119</v>
       </c>
       <c r="L7" t="n">
-        <v>4.147</v>
+        <v>4.15</v>
       </c>
       <c r="M7" t="n">
-        <v>4.315</v>
+        <v>4.314</v>
       </c>
       <c r="N7" t="n">
-        <v>4.382</v>
+        <v>4.367</v>
       </c>
       <c r="O7" t="n">
-        <v>4.542</v>
+        <v>4.515</v>
       </c>
       <c r="P7" t="n">
-        <v>4.931</v>
+        <v>4.901</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.783</v>
+        <v>5.741</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.35</v>
+        <v>5.355</v>
       </c>
       <c r="G8" t="n">
-        <v>5.95</v>
+        <v>5.96</v>
       </c>
       <c r="H8" t="n">
-        <v>6.381</v>
+        <v>6.392</v>
       </c>
       <c r="I8" t="n">
-        <v>6.623</v>
+        <v>6.638</v>
       </c>
       <c r="J8" t="n">
-        <v>7.082</v>
+        <v>7.093</v>
       </c>
       <c r="K8" t="n">
-        <v>7.867</v>
+        <v>7.879</v>
       </c>
       <c r="L8" t="n">
-        <v>8.218</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.603</v>
+        <v>8.602</v>
       </c>
       <c r="N8" t="n">
-        <v>8.792999999999999</v>
+        <v>8.778</v>
       </c>
       <c r="O8" t="n">
-        <v>9.097</v>
+        <v>9.07</v>
       </c>
       <c r="P8" t="n">
-        <v>9.337</v>
+        <v>9.308</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.085</v>
+        <v>10.043</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,46 +1063,46 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.638</v>
+        <v>2.637</v>
       </c>
       <c r="G9" t="n">
         <v>2.74</v>
       </c>
       <c r="H9" t="n">
-        <v>2.889</v>
+        <v>2.914</v>
       </c>
       <c r="I9" t="n">
-        <v>3.165</v>
+        <v>3.17</v>
       </c>
       <c r="J9" t="n">
-        <v>3.35</v>
+        <v>3.349</v>
       </c>
       <c r="K9" t="n">
         <v>3.6</v>
       </c>
       <c r="L9" t="n">
-        <v>3.651</v>
+        <v>3.648</v>
       </c>
       <c r="M9" t="n">
-        <v>3.757</v>
+        <v>3.75</v>
       </c>
       <c r="N9" t="n">
-        <v>3.932</v>
+        <v>3.917</v>
       </c>
       <c r="O9" t="n">
-        <v>3.992</v>
+        <v>3.965</v>
       </c>
       <c r="P9" t="n">
-        <v>4.147</v>
+        <v>4.118</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.247</v>
+        <v>4.205</v>
       </c>
       <c r="R9" t="n">
-        <v>4.263</v>
+        <v>4.235</v>
       </c>
       <c r="S9" t="n">
-        <v>4.27</v>
+        <v>4.255</v>
       </c>
       <c r="T9" t="n">
         <v>4.197</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.652</v>
+        <v>2.651</v>
       </c>
       <c r="G10" t="n">
         <v>2.773</v>
       </c>
       <c r="H10" t="n">
-        <v>2.901</v>
+        <v>2.924</v>
       </c>
       <c r="I10" t="n">
-        <v>3.168</v>
+        <v>3.173</v>
       </c>
       <c r="J10" t="n">
-        <v>3.375</v>
+        <v>3.374</v>
       </c>
       <c r="K10" t="n">
         <v>3.633</v>
       </c>
       <c r="L10" t="n">
-        <v>3.701</v>
+        <v>3.697</v>
       </c>
       <c r="M10" t="n">
-        <v>3.852</v>
+        <v>3.844</v>
       </c>
       <c r="N10" t="n">
-        <v>3.949</v>
+        <v>3.934</v>
       </c>
       <c r="O10" t="n">
-        <v>4.185</v>
+        <v>4.172</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.467</v>
+        <v>2.466</v>
       </c>
       <c r="G11" t="n">
         <v>2.583</v>
       </c>
       <c r="H11" t="n">
-        <v>2.724</v>
+        <v>2.747</v>
       </c>
       <c r="I11" t="n">
-        <v>2.972</v>
+        <v>2.977</v>
       </c>
       <c r="J11" t="n">
-        <v>3.173</v>
+        <v>3.172</v>
       </c>
       <c r="K11" t="n">
         <v>3.42</v>
       </c>
       <c r="L11" t="n">
-        <v>3.498</v>
+        <v>3.495</v>
       </c>
       <c r="M11" t="n">
-        <v>3.659</v>
+        <v>3.652</v>
       </c>
       <c r="N11" t="n">
-        <v>3.758</v>
+        <v>3.742</v>
       </c>
       <c r="O11" t="n">
-        <v>3.952</v>
+        <v>3.938</v>
       </c>
       <c r="P11" t="n">
-        <v>4.098</v>
+        <v>4.07</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.448</v>
+        <v>4.406</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.217</v>
+        <v>3.218</v>
       </c>
       <c r="G12" t="n">
-        <v>3.41</v>
+        <v>3.418</v>
       </c>
       <c r="H12" t="n">
-        <v>3.614</v>
+        <v>3.627</v>
       </c>
       <c r="I12" t="n">
-        <v>3.839</v>
+        <v>3.854</v>
       </c>
       <c r="J12" t="n">
-        <v>4.234</v>
+        <v>4.243</v>
       </c>
       <c r="K12" t="n">
-        <v>4.476</v>
+        <v>4.483</v>
       </c>
       <c r="L12" t="n">
         <v>4.556</v>
       </c>
       <c r="M12" t="n">
-        <v>4.724</v>
+        <v>4.721</v>
       </c>
       <c r="N12" t="n">
-        <v>4.808</v>
+        <v>4.794</v>
       </c>
       <c r="O12" t="n">
-        <v>4.979</v>
+        <v>4.953</v>
       </c>
       <c r="P12" t="n">
-        <v>5.183</v>
+        <v>5.154</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.562</v>
+        <v>5.52</v>
       </c>
       <c r="R12" t="n">
-        <v>5.755</v>
+        <v>5.726</v>
       </c>
       <c r="S12" t="n">
-        <v>5.973</v>
+        <v>5.958</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.971</v>
+        <v>2.972</v>
       </c>
       <c r="G13" t="n">
-        <v>3.1</v>
+        <v>3.109</v>
       </c>
       <c r="H13" t="n">
-        <v>3.282</v>
+        <v>3.294</v>
       </c>
       <c r="I13" t="n">
-        <v>3.487</v>
+        <v>3.502</v>
       </c>
       <c r="J13" t="n">
-        <v>3.87</v>
+        <v>3.879</v>
       </c>
       <c r="K13" t="n">
-        <v>4.109</v>
+        <v>4.117</v>
       </c>
       <c r="L13" t="n">
         <v>4.195</v>
       </c>
       <c r="M13" t="n">
-        <v>4.351</v>
+        <v>4.348</v>
       </c>
       <c r="N13" t="n">
-        <v>4.436</v>
+        <v>4.422</v>
       </c>
       <c r="O13" t="n">
-        <v>4.608</v>
+        <v>4.582</v>
       </c>
       <c r="P13" t="n">
-        <v>4.775</v>
+        <v>4.745</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.083</v>
+        <v>5.041</v>
       </c>
       <c r="R13" t="n">
-        <v>5.304</v>
+        <v>5.276</v>
       </c>
       <c r="S13" t="n">
-        <v>5.536</v>
+        <v>5.52</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.79</v>
+        <v>2.791</v>
       </c>
       <c r="G14" t="n">
-        <v>2.906</v>
+        <v>2.914</v>
       </c>
       <c r="H14" t="n">
-        <v>3.085</v>
+        <v>3.097</v>
       </c>
       <c r="I14" t="n">
-        <v>3.27</v>
+        <v>3.285</v>
       </c>
       <c r="J14" t="n">
-        <v>3.612</v>
+        <v>3.621</v>
       </c>
       <c r="K14" t="n">
-        <v>3.797</v>
+        <v>3.805</v>
       </c>
       <c r="L14" t="n">
         <v>3.868</v>
       </c>
       <c r="M14" t="n">
-        <v>4.037</v>
+        <v>4.034</v>
       </c>
       <c r="N14" t="n">
-        <v>4.115</v>
+        <v>4.101</v>
       </c>
       <c r="O14" t="n">
-        <v>4.265</v>
+        <v>4.24</v>
       </c>
       <c r="P14" t="n">
-        <v>4.41</v>
+        <v>4.38</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.672</v>
+        <v>4.63</v>
       </c>
       <c r="R14" t="n">
-        <v>4.819</v>
+        <v>4.79</v>
       </c>
       <c r="S14" t="n">
-        <v>4.988</v>
+        <v>4.973</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.768</v>
+        <v>2.769</v>
       </c>
       <c r="G15" t="n">
-        <v>2.88</v>
+        <v>2.888</v>
       </c>
       <c r="H15" t="n">
-        <v>3.056</v>
+        <v>3.068</v>
       </c>
       <c r="I15" t="n">
-        <v>3.222</v>
+        <v>3.237</v>
       </c>
       <c r="J15" t="n">
-        <v>3.551</v>
+        <v>3.56</v>
       </c>
       <c r="K15" t="n">
-        <v>3.749</v>
+        <v>3.757</v>
       </c>
       <c r="L15" t="n">
         <v>3.804</v>
       </c>
       <c r="M15" t="n">
-        <v>3.95</v>
+        <v>3.947</v>
       </c>
       <c r="N15" t="n">
-        <v>4.019</v>
+        <v>4.005</v>
       </c>
       <c r="O15" t="n">
-        <v>4.206</v>
+        <v>4.181</v>
       </c>
       <c r="P15" t="n">
-        <v>4.309</v>
+        <v>4.279</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.575</v>
+        <v>4.533</v>
       </c>
       <c r="R15" t="n">
-        <v>4.714</v>
+        <v>4.685</v>
       </c>
       <c r="S15" t="n">
-        <v>4.884</v>
+        <v>4.868</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.768</v>
+        <v>2.769</v>
       </c>
       <c r="G16" t="n">
-        <v>2.88</v>
+        <v>2.888</v>
       </c>
       <c r="H16" t="n">
-        <v>3.056</v>
+        <v>3.068</v>
       </c>
       <c r="I16" t="n">
-        <v>3.222</v>
+        <v>3.237</v>
       </c>
       <c r="J16" t="n">
-        <v>3.551</v>
+        <v>3.56</v>
       </c>
       <c r="K16" t="n">
-        <v>3.749</v>
+        <v>3.757</v>
       </c>
       <c r="L16" t="n">
         <v>3.804</v>
       </c>
       <c r="M16" t="n">
-        <v>3.95</v>
+        <v>3.947</v>
       </c>
       <c r="N16" t="n">
-        <v>4.022</v>
+        <v>4.008</v>
       </c>
       <c r="O16" t="n">
-        <v>4.213</v>
+        <v>4.188</v>
       </c>
       <c r="P16" t="n">
-        <v>4.332</v>
+        <v>4.303</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.602</v>
+        <v>4.56</v>
       </c>
       <c r="R16" t="n">
-        <v>4.742</v>
+        <v>4.713</v>
       </c>
       <c r="S16" t="n">
-        <v>4.912</v>
+        <v>4.897</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,16 +1647,16 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.714</v>
+        <v>2.713</v>
       </c>
       <c r="G17" t="n">
         <v>2.863</v>
       </c>
       <c r="H17" t="n">
-        <v>2.994</v>
+        <v>3.016</v>
       </c>
       <c r="I17" t="n">
-        <v>3.249</v>
+        <v>3.253</v>
       </c>
       <c r="J17" t="n">
         <v>3.45</v>
@@ -1665,19 +1665,19 @@
         <v>3.711</v>
       </c>
       <c r="L17" t="n">
-        <v>3.785</v>
+        <v>3.781</v>
       </c>
       <c r="M17" t="n">
-        <v>3.975</v>
+        <v>3.967</v>
       </c>
       <c r="N17" t="n">
-        <v>4.051</v>
+        <v>4.037</v>
       </c>
       <c r="O17" t="n">
-        <v>4.215</v>
+        <v>4.201</v>
       </c>
       <c r="P17" t="n">
-        <v>4.379</v>
+        <v>4.35</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,16 +1720,16 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.715</v>
+        <v>2.714</v>
       </c>
       <c r="G18" t="n">
         <v>2.864</v>
       </c>
       <c r="H18" t="n">
-        <v>2.994</v>
+        <v>3.017</v>
       </c>
       <c r="I18" t="n">
-        <v>3.249</v>
+        <v>3.254</v>
       </c>
       <c r="J18" t="n">
         <v>3.45</v>
@@ -1738,16 +1738,16 @@
         <v>3.712</v>
       </c>
       <c r="L18" t="n">
-        <v>3.785</v>
+        <v>3.781</v>
       </c>
       <c r="M18" t="n">
-        <v>3.975</v>
+        <v>3.967</v>
       </c>
       <c r="N18" t="n">
-        <v>4.052</v>
+        <v>4.037</v>
       </c>
       <c r="O18" t="n">
-        <v>4.212</v>
+        <v>4.199</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1796,43 +1796,43 @@
         <v>2.781</v>
       </c>
       <c r="G19" t="n">
-        <v>2.895</v>
+        <v>2.903</v>
       </c>
       <c r="H19" t="n">
-        <v>3.073</v>
+        <v>3.085</v>
       </c>
       <c r="I19" t="n">
-        <v>3.255</v>
+        <v>3.269</v>
       </c>
       <c r="J19" t="n">
-        <v>3.594</v>
+        <v>3.603</v>
       </c>
       <c r="K19" t="n">
-        <v>3.793</v>
+        <v>3.801</v>
       </c>
       <c r="L19" t="n">
         <v>3.864</v>
       </c>
       <c r="M19" t="n">
-        <v>4.027</v>
+        <v>4.024</v>
       </c>
       <c r="N19" t="n">
-        <v>4.105</v>
+        <v>4.091</v>
       </c>
       <c r="O19" t="n">
-        <v>4.249</v>
+        <v>4.224</v>
       </c>
       <c r="P19" t="n">
-        <v>4.369</v>
+        <v>4.34</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.612</v>
+        <v>4.571</v>
       </c>
       <c r="R19" t="n">
-        <v>4.761</v>
+        <v>4.733</v>
       </c>
       <c r="S19" t="n">
-        <v>4.923</v>
+        <v>4.908</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.609</v>
+        <v>2.607</v>
       </c>
       <c r="G20" t="n">
         <v>2.691</v>
       </c>
       <c r="H20" t="n">
-        <v>2.76</v>
+        <v>2.762</v>
       </c>
       <c r="I20" t="n">
-        <v>2.863</v>
+        <v>2.869</v>
       </c>
       <c r="J20" t="n">
-        <v>3.375</v>
+        <v>3.376</v>
       </c>
       <c r="K20" t="n">
-        <v>3.622</v>
+        <v>3.625</v>
       </c>
       <c r="L20" t="n">
         <v>3.673</v>
       </c>
       <c r="M20" t="n">
-        <v>3.787</v>
+        <v>3.79</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.904</v>
+        <v>2.906</v>
       </c>
       <c r="G21" t="n">
-        <v>2.992</v>
+        <v>3.002</v>
       </c>
       <c r="H21" t="n">
-        <v>3.194</v>
+        <v>3.204</v>
       </c>
       <c r="I21" t="n">
-        <v>3.359</v>
+        <v>3.375</v>
       </c>
       <c r="J21" t="n">
-        <v>3.739</v>
+        <v>3.747</v>
       </c>
       <c r="K21" t="n">
-        <v>4.02</v>
+        <v>4.029</v>
       </c>
       <c r="L21" t="n">
-        <v>4.1</v>
+        <v>4.099</v>
       </c>
       <c r="M21" t="n">
-        <v>4.247</v>
+        <v>4.245</v>
       </c>
       <c r="N21" t="n">
-        <v>4.341</v>
+        <v>4.33</v>
       </c>
       <c r="O21" t="n">
-        <v>4.459</v>
+        <v>4.437</v>
       </c>
       <c r="P21" t="n">
-        <v>4.629</v>
+        <v>4.6</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.773</v>
+        <v>4.733</v>
       </c>
       <c r="R21" t="n">
-        <v>4.812</v>
+        <v>4.782</v>
       </c>
       <c r="S21" t="n">
-        <v>4.881</v>
+        <v>4.865</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.851</v>
+        <v>2.852</v>
       </c>
       <c r="G22" t="n">
-        <v>2.938</v>
+        <v>2.948</v>
       </c>
       <c r="H22" t="n">
-        <v>3.125</v>
+        <v>3.136</v>
       </c>
       <c r="I22" t="n">
-        <v>3.277</v>
+        <v>3.293</v>
       </c>
       <c r="J22" t="n">
-        <v>3.625</v>
+        <v>3.632</v>
       </c>
       <c r="K22" t="n">
-        <v>3.902</v>
+        <v>3.911</v>
       </c>
       <c r="L22" t="n">
-        <v>3.967</v>
+        <v>3.966</v>
       </c>
       <c r="M22" t="n">
-        <v>4.117</v>
+        <v>4.115</v>
       </c>
       <c r="N22" t="n">
-        <v>4.215</v>
+        <v>4.203</v>
       </c>
       <c r="O22" t="n">
-        <v>4.33</v>
+        <v>4.307</v>
       </c>
       <c r="P22" t="n">
-        <v>4.492</v>
+        <v>4.464</v>
       </c>
       <c r="Q22" t="n">
+        <v>4.592</v>
+      </c>
+      <c r="R22" t="n">
         <v>4.631</v>
       </c>
-      <c r="R22" t="n">
-        <v>4.66</v>
-      </c>
       <c r="S22" t="n">
-        <v>4.726</v>
+        <v>4.71</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,46 +2085,46 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.801</v>
+        <v>2.803</v>
       </c>
       <c r="G23" t="n">
-        <v>2.893</v>
+        <v>2.903</v>
       </c>
       <c r="H23" t="n">
-        <v>3.067</v>
+        <v>3.078</v>
       </c>
       <c r="I23" t="n">
-        <v>3.227</v>
+        <v>3.243</v>
       </c>
       <c r="J23" t="n">
-        <v>3.566</v>
+        <v>3.573</v>
       </c>
       <c r="K23" t="n">
-        <v>3.803</v>
+        <v>3.812</v>
       </c>
       <c r="L23" t="n">
-        <v>3.867</v>
+        <v>3.865</v>
       </c>
       <c r="M23" t="n">
-        <v>4.011</v>
+        <v>4.008</v>
       </c>
       <c r="N23" t="n">
-        <v>4.109</v>
+        <v>4.098</v>
       </c>
       <c r="O23" t="n">
-        <v>4.203</v>
+        <v>4.18</v>
       </c>
       <c r="P23" t="n">
-        <v>4.355</v>
+        <v>4.327</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.438</v>
+        <v>4.398</v>
       </c>
       <c r="R23" t="n">
-        <v>4.444</v>
+        <v>4.415</v>
       </c>
       <c r="S23" t="n">
-        <v>4.48</v>
+        <v>4.465</v>
       </c>
       <c r="T23" t="n">
         <v>4.401</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.739</v>
+        <v>2.74</v>
       </c>
       <c r="G24" t="n">
-        <v>2.808</v>
+        <v>2.817</v>
       </c>
       <c r="H24" t="n">
-        <v>2.966</v>
+        <v>2.976</v>
       </c>
       <c r="I24" t="n">
-        <v>3.166</v>
+        <v>3.182</v>
       </c>
       <c r="J24" t="n">
-        <v>3.463</v>
+        <v>3.469</v>
       </c>
       <c r="K24" t="n">
-        <v>3.687</v>
+        <v>3.695</v>
       </c>
       <c r="L24" t="n">
-        <v>3.747</v>
+        <v>3.744</v>
       </c>
       <c r="M24" t="n">
-        <v>3.874</v>
+        <v>3.869</v>
       </c>
       <c r="N24" t="n">
-        <v>3.986</v>
+        <v>3.973</v>
       </c>
       <c r="O24" t="n">
-        <v>4.195</v>
+        <v>4.171</v>
       </c>
       <c r="P24" t="n">
-        <v>4.293</v>
+        <v>4.264</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.362</v>
+        <v>4.323</v>
       </c>
       <c r="R24" t="n">
-        <v>4.366</v>
+        <v>4.337</v>
       </c>
       <c r="S24" t="n">
-        <v>4.395</v>
+        <v>4.38</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,46 +2231,46 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.795</v>
+        <v>2.797</v>
       </c>
       <c r="G25" t="n">
-        <v>2.893</v>
+        <v>2.903</v>
       </c>
       <c r="H25" t="n">
-        <v>3.07</v>
+        <v>3.081</v>
       </c>
       <c r="I25" t="n">
-        <v>3.234</v>
+        <v>3.25</v>
       </c>
       <c r="J25" t="n">
-        <v>3.581</v>
+        <v>3.588</v>
       </c>
       <c r="K25" t="n">
-        <v>3.835</v>
+        <v>3.844</v>
       </c>
       <c r="L25" t="n">
-        <v>3.897</v>
+        <v>3.896</v>
       </c>
       <c r="M25" t="n">
-        <v>4.042</v>
+        <v>4.039</v>
       </c>
       <c r="N25" t="n">
-        <v>4.136</v>
+        <v>4.125</v>
       </c>
       <c r="O25" t="n">
-        <v>4.232</v>
+        <v>4.209</v>
       </c>
       <c r="P25" t="n">
-        <v>4.377</v>
+        <v>4.349</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.471</v>
+        <v>4.431</v>
       </c>
       <c r="R25" t="n">
-        <v>4.468</v>
+        <v>4.438</v>
       </c>
       <c r="S25" t="n">
-        <v>4.504</v>
+        <v>4.488</v>
       </c>
       <c r="T25" t="n">
         <v>4.419</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.065</v>
+        <v>3.068</v>
       </c>
       <c r="G26" t="n">
-        <v>3.217</v>
+        <v>3.225</v>
       </c>
       <c r="H26" t="n">
-        <v>3.499</v>
+        <v>3.51</v>
       </c>
       <c r="I26" t="n">
-        <v>3.717</v>
+        <v>3.731</v>
       </c>
       <c r="J26" t="n">
-        <v>4.217</v>
+        <v>4.224</v>
       </c>
       <c r="K26" t="n">
-        <v>4.653</v>
+        <v>4.661</v>
       </c>
       <c r="L26" t="n">
-        <v>4.78</v>
+        <v>4.781</v>
       </c>
       <c r="M26" t="n">
-        <v>4.988</v>
+        <v>4.982</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.309</v>
+        <v>5.282</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.875</v>
+        <v>2.877</v>
       </c>
       <c r="G27" t="n">
-        <v>2.974</v>
+        <v>2.983</v>
       </c>
       <c r="H27" t="n">
-        <v>3.163</v>
+        <v>3.176</v>
       </c>
       <c r="I27" t="n">
-        <v>3.351</v>
+        <v>3.367</v>
       </c>
       <c r="J27" t="n">
-        <v>3.723</v>
+        <v>3.731</v>
       </c>
       <c r="K27" t="n">
-        <v>3.971</v>
+        <v>3.979</v>
       </c>
       <c r="L27" t="n">
         <v>4.049</v>
       </c>
       <c r="M27" t="n">
-        <v>4.203</v>
+        <v>4.197</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.403</v>
+        <v>4.377</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.978</v>
+        <v>2.98</v>
       </c>
       <c r="G28" t="n">
-        <v>3.085</v>
+        <v>3.094</v>
       </c>
       <c r="H28" t="n">
-        <v>3.289</v>
+        <v>3.301</v>
       </c>
       <c r="I28" t="n">
-        <v>3.489</v>
+        <v>3.505</v>
       </c>
       <c r="J28" t="n">
-        <v>3.896</v>
+        <v>3.904</v>
       </c>
       <c r="K28" t="n">
-        <v>4.164</v>
+        <v>4.171</v>
       </c>
       <c r="L28" t="n">
         <v>4.252</v>
       </c>
       <c r="M28" t="n">
-        <v>4.415</v>
+        <v>4.409</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.695</v>
+        <v>4.669</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.825</v>
+        <v>2.827</v>
       </c>
       <c r="G29" t="n">
-        <v>2.925</v>
+        <v>2.934</v>
       </c>
       <c r="H29" t="n">
-        <v>3.104</v>
+        <v>3.116</v>
       </c>
       <c r="I29" t="n">
-        <v>3.281</v>
+        <v>3.296</v>
       </c>
       <c r="J29" t="n">
-        <v>3.636</v>
+        <v>3.643</v>
       </c>
       <c r="K29" t="n">
-        <v>3.867</v>
+        <v>3.875</v>
       </c>
       <c r="L29" t="n">
-        <v>3.934</v>
+        <v>3.935</v>
       </c>
       <c r="M29" t="n">
-        <v>4.065</v>
+        <v>4.06</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.273</v>
+        <v>4.247</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.109</v>
+        <v>3.112</v>
       </c>
       <c r="G30" t="n">
-        <v>3.196</v>
+        <v>3.205</v>
       </c>
       <c r="H30" t="n">
-        <v>3.431</v>
+        <v>3.443</v>
       </c>
       <c r="I30" t="n">
-        <v>3.643</v>
+        <v>3.656</v>
       </c>
       <c r="J30" t="n">
-        <v>4.087</v>
+        <v>4.093</v>
       </c>
       <c r="K30" t="n">
-        <v>4.454</v>
+        <v>4.461</v>
       </c>
       <c r="L30" t="n">
         <v>4.56</v>
       </c>
       <c r="M30" t="n">
-        <v>4.758</v>
+        <v>4.751</v>
       </c>
       <c r="N30" t="n">
-        <v>4.946</v>
+        <v>4.931</v>
       </c>
       <c r="O30" t="n">
-        <v>5.259</v>
+        <v>5.232</v>
       </c>
       <c r="P30" t="n">
-        <v>5.522</v>
+        <v>5.493</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.31</v>
+        <v>6.267</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.438</v>
+        <v>3.441</v>
       </c>
       <c r="G31" t="n">
-        <v>3.561</v>
+        <v>3.57</v>
       </c>
       <c r="H31" t="n">
-        <v>3.845</v>
+        <v>3.857</v>
       </c>
       <c r="I31" t="n">
-        <v>4.072</v>
+        <v>4.085</v>
       </c>
       <c r="J31" t="n">
-        <v>4.579</v>
+        <v>4.585</v>
       </c>
       <c r="K31" t="n">
-        <v>4.987</v>
+        <v>4.993</v>
       </c>
       <c r="L31" t="n">
         <v>5.172</v>
       </c>
       <c r="M31" t="n">
-        <v>5.489</v>
+        <v>5.482</v>
       </c>
       <c r="N31" t="n">
-        <v>5.805</v>
+        <v>5.79</v>
       </c>
       <c r="O31" t="n">
-        <v>6.295</v>
+        <v>6.268</v>
       </c>
       <c r="P31" t="n">
-        <v>6.51</v>
+        <v>6.481</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.284</v>
+        <v>7.241</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.207</v>
+        <v>3.211</v>
       </c>
       <c r="G32" t="n">
-        <v>3.314</v>
+        <v>3.323</v>
       </c>
       <c r="H32" t="n">
-        <v>3.574</v>
+        <v>3.586</v>
       </c>
       <c r="I32" t="n">
-        <v>3.802</v>
+        <v>3.815</v>
       </c>
       <c r="J32" t="n">
-        <v>4.265</v>
+        <v>4.271</v>
       </c>
       <c r="K32" t="n">
-        <v>4.639</v>
+        <v>4.646</v>
       </c>
       <c r="L32" t="n">
         <v>4.764</v>
       </c>
       <c r="M32" t="n">
-        <v>5.031</v>
+        <v>5.024</v>
       </c>
       <c r="N32" t="n">
-        <v>5.306</v>
+        <v>5.291</v>
       </c>
       <c r="O32" t="n">
-        <v>5.705</v>
+        <v>5.678</v>
       </c>
       <c r="P32" t="n">
-        <v>5.982</v>
+        <v>5.953</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.771</v>
+        <v>6.728</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.973</v>
+        <v>2.976</v>
       </c>
       <c r="G33" t="n">
-        <v>3.059</v>
+        <v>3.069</v>
       </c>
       <c r="H33" t="n">
-        <v>3.247</v>
+        <v>3.26</v>
       </c>
       <c r="I33" t="n">
-        <v>3.426</v>
+        <v>3.439</v>
       </c>
       <c r="J33" t="n">
-        <v>3.793</v>
+        <v>3.799</v>
       </c>
       <c r="K33" t="n">
-        <v>4.094</v>
+        <v>4.102</v>
       </c>
       <c r="L33" t="n">
         <v>4.162</v>
       </c>
       <c r="M33" t="n">
-        <v>4.284</v>
+        <v>4.277</v>
       </c>
       <c r="N33" t="n">
-        <v>4.336</v>
+        <v>4.321</v>
       </c>
       <c r="O33" t="n">
-        <v>4.414</v>
+        <v>4.386</v>
       </c>
       <c r="P33" t="n">
-        <v>4.554</v>
+        <v>4.525</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.027</v>
+        <v>4.984</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.033</v>
+        <v>3.036</v>
       </c>
       <c r="G34" t="n">
-        <v>3.112</v>
+        <v>3.122</v>
       </c>
       <c r="H34" t="n">
-        <v>3.309</v>
+        <v>3.322</v>
       </c>
       <c r="I34" t="n">
-        <v>3.495</v>
+        <v>3.507</v>
       </c>
       <c r="J34" t="n">
-        <v>3.864</v>
+        <v>3.87</v>
       </c>
       <c r="K34" t="n">
-        <v>4.171</v>
+        <v>4.179</v>
       </c>
       <c r="L34" t="n">
         <v>4.242</v>
       </c>
       <c r="M34" t="n">
-        <v>4.375</v>
+        <v>4.368</v>
       </c>
       <c r="N34" t="n">
-        <v>4.439</v>
+        <v>4.424</v>
       </c>
       <c r="O34" t="n">
-        <v>4.583</v>
+        <v>4.555</v>
       </c>
       <c r="P34" t="n">
-        <v>4.849</v>
+        <v>4.82</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.728</v>
+        <v>5.685</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.007</v>
+        <v>3.01</v>
       </c>
       <c r="G35" t="n">
-        <v>3.086</v>
+        <v>3.096</v>
       </c>
       <c r="H35" t="n">
-        <v>3.276</v>
+        <v>3.29</v>
       </c>
       <c r="I35" t="n">
-        <v>3.461</v>
+        <v>3.474</v>
       </c>
       <c r="J35" t="n">
-        <v>3.832</v>
+        <v>3.839</v>
       </c>
       <c r="K35" t="n">
-        <v>4.125</v>
+        <v>4.132</v>
       </c>
       <c r="L35" t="n">
         <v>4.196</v>
       </c>
       <c r="M35" t="n">
-        <v>4.321</v>
+        <v>4.314</v>
       </c>
       <c r="N35" t="n">
-        <v>4.375</v>
+        <v>4.361</v>
       </c>
       <c r="O35" t="n">
-        <v>4.48</v>
+        <v>4.452</v>
       </c>
       <c r="P35" t="n">
-        <v>4.651</v>
+        <v>4.622</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.364</v>
+        <v>5.321</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.903</v>
+        <v>2.906</v>
       </c>
       <c r="G36" t="n">
-        <v>2.983</v>
+        <v>2.992</v>
       </c>
       <c r="H36" t="n">
-        <v>3.164</v>
+        <v>3.175</v>
       </c>
       <c r="I36" t="n">
-        <v>3.346</v>
+        <v>3.358</v>
       </c>
       <c r="J36" t="n">
-        <v>3.728</v>
+        <v>3.734</v>
       </c>
       <c r="K36" t="n">
-        <v>4.019</v>
+        <v>4.026</v>
       </c>
       <c r="L36" t="n">
         <v>4.088</v>
       </c>
       <c r="M36" t="n">
-        <v>4.186</v>
+        <v>4.179</v>
       </c>
       <c r="N36" t="n">
-        <v>4.239</v>
+        <v>4.224</v>
       </c>
       <c r="O36" t="n">
-        <v>4.323</v>
+        <v>4.295</v>
       </c>
       <c r="P36" t="n">
-        <v>4.453</v>
+        <v>4.423</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.744</v>
+        <v>4.701</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.782</v>
+        <v>3.785</v>
       </c>
       <c r="G37" t="n">
-        <v>4.256</v>
+        <v>4.265</v>
       </c>
       <c r="H37" t="n">
-        <v>4.821</v>
+        <v>4.833</v>
       </c>
       <c r="I37" t="n">
-        <v>5.134</v>
+        <v>5.147</v>
       </c>
       <c r="J37" t="n">
-        <v>6.07</v>
+        <v>6.076</v>
       </c>
       <c r="K37" t="n">
-        <v>7.027</v>
+        <v>7.034</v>
       </c>
       <c r="L37" t="n">
         <v>7.372</v>
       </c>
       <c r="M37" t="n">
-        <v>7.761</v>
+        <v>7.754</v>
       </c>
       <c r="N37" t="n">
-        <v>7.956</v>
+        <v>7.941</v>
       </c>
       <c r="O37" t="n">
-        <v>8.173999999999999</v>
+        <v>8.147</v>
       </c>
       <c r="P37" t="n">
-        <v>8.31</v>
+        <v>8.281000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.772</v>
+        <v>8.728999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.841</v>
+        <v>4.844</v>
       </c>
       <c r="G38" t="n">
-        <v>5.569</v>
+        <v>5.578</v>
       </c>
       <c r="H38" t="n">
-        <v>6.345</v>
+        <v>6.357</v>
       </c>
       <c r="I38" t="n">
-        <v>6.815</v>
+        <v>6.828</v>
       </c>
       <c r="J38" t="n">
-        <v>8.013</v>
+        <v>8.019</v>
       </c>
       <c r="K38" t="n">
-        <v>9.148999999999999</v>
+        <v>9.156000000000001</v>
       </c>
       <c r="L38" t="n">
         <v>9.654999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.173</v>
+        <v>10.166</v>
       </c>
       <c r="N38" t="n">
-        <v>10.375</v>
+        <v>10.36</v>
       </c>
       <c r="O38" t="n">
-        <v>10.575</v>
+        <v>10.547</v>
       </c>
       <c r="P38" t="n">
-        <v>10.708</v>
+        <v>10.678</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.223</v>
+        <v>11.18</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.162</v>
+        <v>4.165</v>
       </c>
       <c r="G39" t="n">
-        <v>4.767</v>
+        <v>4.776</v>
       </c>
       <c r="H39" t="n">
-        <v>5.41</v>
+        <v>5.422</v>
       </c>
       <c r="I39" t="n">
-        <v>5.819</v>
+        <v>5.832</v>
       </c>
       <c r="J39" t="n">
-        <v>6.885</v>
+        <v>6.891</v>
       </c>
       <c r="K39" t="n">
-        <v>7.982</v>
+        <v>7.988</v>
       </c>
       <c r="L39" t="n">
         <v>8.41</v>
       </c>
       <c r="M39" t="n">
-        <v>8.808999999999999</v>
+        <v>8.802</v>
       </c>
       <c r="N39" t="n">
-        <v>9.002000000000001</v>
+        <v>8.987</v>
       </c>
       <c r="O39" t="n">
-        <v>9.225</v>
+        <v>9.198</v>
       </c>
       <c r="P39" t="n">
-        <v>9.362</v>
+        <v>9.333</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.868</v>
+        <v>9.824999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.3</v>
+        <v>3.304</v>
       </c>
       <c r="G40" t="n">
-        <v>3.434</v>
+        <v>3.443</v>
       </c>
       <c r="H40" t="n">
-        <v>3.69</v>
+        <v>3.702</v>
       </c>
       <c r="I40" t="n">
-        <v>3.917</v>
+        <v>3.929</v>
       </c>
       <c r="J40" t="n">
-        <v>4.379</v>
+        <v>4.385</v>
       </c>
       <c r="K40" t="n">
-        <v>4.76</v>
+        <v>4.767</v>
       </c>
       <c r="L40" t="n">
         <v>4.884</v>
       </c>
       <c r="M40" t="n">
-        <v>5.101</v>
+        <v>5.094</v>
       </c>
       <c r="N40" t="n">
-        <v>5.303</v>
+        <v>5.288</v>
       </c>
       <c r="O40" t="n">
-        <v>5.638</v>
+        <v>5.611</v>
       </c>
       <c r="P40" t="n">
-        <v>5.943</v>
+        <v>5.914</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.761</v>
+        <v>6.718</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.687</v>
+        <v>3.69</v>
       </c>
       <c r="G41" t="n">
-        <v>3.863</v>
+        <v>3.872</v>
       </c>
       <c r="H41" t="n">
-        <v>4.174</v>
+        <v>4.186</v>
       </c>
       <c r="I41" t="n">
-        <v>4.42</v>
+        <v>4.433</v>
       </c>
       <c r="J41" t="n">
-        <v>4.934</v>
+        <v>4.94</v>
       </c>
       <c r="K41" t="n">
-        <v>5.36</v>
+        <v>5.367</v>
       </c>
       <c r="L41" t="n">
         <v>5.563</v>
       </c>
       <c r="M41" t="n">
-        <v>5.904</v>
+        <v>5.897</v>
       </c>
       <c r="N41" t="n">
-        <v>6.234</v>
+        <v>6.219</v>
       </c>
       <c r="O41" t="n">
-        <v>6.754</v>
+        <v>6.726</v>
       </c>
       <c r="P41" t="n">
-        <v>7.003</v>
+        <v>6.973</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.808</v>
+        <v>7.765</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.422</v>
+        <v>3.425</v>
       </c>
       <c r="G42" t="n">
-        <v>3.583</v>
+        <v>3.592</v>
       </c>
       <c r="H42" t="n">
-        <v>3.865</v>
+        <v>3.877</v>
       </c>
       <c r="I42" t="n">
-        <v>4.105</v>
+        <v>4.118</v>
       </c>
       <c r="J42" t="n">
-        <v>4.581</v>
+        <v>4.587</v>
       </c>
       <c r="K42" t="n">
-        <v>4.981</v>
+        <v>4.988</v>
       </c>
       <c r="L42" t="n">
         <v>5.12</v>
       </c>
       <c r="M42" t="n">
-        <v>5.408</v>
+        <v>5.401</v>
       </c>
       <c r="N42" t="n">
-        <v>5.718</v>
+        <v>5.703</v>
       </c>
       <c r="O42" t="n">
-        <v>6.13</v>
+        <v>6.103</v>
       </c>
       <c r="P42" t="n">
-        <v>6.445</v>
+        <v>6.416</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.274</v>
+        <v>7.231</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.121</v>
+        <v>3.124</v>
       </c>
       <c r="G43" t="n">
-        <v>3.242</v>
+        <v>3.252</v>
       </c>
       <c r="H43" t="n">
-        <v>3.448</v>
+        <v>3.461</v>
       </c>
       <c r="I43" t="n">
-        <v>3.635</v>
+        <v>3.648</v>
       </c>
       <c r="J43" t="n">
-        <v>4.02</v>
+        <v>4.026</v>
       </c>
       <c r="K43" t="n">
-        <v>4.326</v>
+        <v>4.334</v>
       </c>
       <c r="L43" t="n">
         <v>4.404</v>
       </c>
       <c r="M43" t="n">
-        <v>4.539</v>
+        <v>4.532</v>
       </c>
       <c r="N43" t="n">
-        <v>4.604</v>
+        <v>4.589</v>
       </c>
       <c r="O43" t="n">
-        <v>4.727</v>
+        <v>4.7</v>
       </c>
       <c r="P43" t="n">
-        <v>4.92</v>
+        <v>4.891</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.637</v>
+        <v>5.594</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.981</v>
+        <v>2.984</v>
       </c>
       <c r="G44" t="n">
-        <v>3.092</v>
+        <v>3.101</v>
       </c>
       <c r="H44" t="n">
-        <v>3.287</v>
+        <v>3.298</v>
       </c>
       <c r="I44" t="n">
-        <v>3.473</v>
+        <v>3.485</v>
       </c>
       <c r="J44" t="n">
-        <v>3.869</v>
+        <v>3.875</v>
       </c>
       <c r="K44" t="n">
-        <v>4.171</v>
+        <v>4.178</v>
       </c>
       <c r="L44" t="n">
         <v>4.248</v>
       </c>
       <c r="M44" t="n">
-        <v>4.356</v>
+        <v>4.349</v>
       </c>
       <c r="N44" t="n">
-        <v>4.421</v>
+        <v>4.406</v>
       </c>
       <c r="O44" t="n">
-        <v>4.523</v>
+        <v>4.496</v>
       </c>
       <c r="P44" t="n">
-        <v>4.683</v>
+        <v>4.653</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.008</v>
+        <v>4.965</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-20 ~ 2026-05-20
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.22</v>
+        <v>3.229</v>
       </c>
       <c r="G2" t="n">
-        <v>3.455</v>
+        <v>3.466</v>
       </c>
       <c r="H2" t="n">
-        <v>3.706</v>
+        <v>3.719</v>
       </c>
       <c r="I2" t="n">
-        <v>3.879</v>
+        <v>3.898</v>
       </c>
       <c r="J2" t="n">
-        <v>4.255</v>
+        <v>4.271</v>
       </c>
       <c r="K2" t="n">
-        <v>4.69</v>
+        <v>4.704</v>
       </c>
       <c r="L2" t="n">
-        <v>4.876</v>
+        <v>4.886</v>
       </c>
       <c r="M2" t="n">
-        <v>5.195</v>
+        <v>5.203</v>
       </c>
       <c r="N2" t="n">
-        <v>5.495</v>
+        <v>5.509</v>
       </c>
       <c r="O2" t="n">
-        <v>5.751</v>
+        <v>5.76</v>
       </c>
       <c r="P2" t="n">
         <v>6.017</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.665</v>
+        <v>6.655</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.243</v>
+        <v>4.252</v>
       </c>
       <c r="G3" t="n">
-        <v>4.66</v>
+        <v>4.671</v>
       </c>
       <c r="H3" t="n">
-        <v>4.944</v>
+        <v>4.957</v>
       </c>
       <c r="I3" t="n">
-        <v>5.112</v>
+        <v>5.131</v>
       </c>
       <c r="J3" t="n">
-        <v>5.501</v>
+        <v>5.516</v>
       </c>
       <c r="K3" t="n">
-        <v>6.007</v>
+        <v>6.02</v>
       </c>
       <c r="L3" t="n">
-        <v>6.262</v>
+        <v>6.271</v>
       </c>
       <c r="M3" t="n">
-        <v>6.612</v>
+        <v>6.62</v>
       </c>
       <c r="N3" t="n">
-        <v>6.854</v>
+        <v>6.868</v>
       </c>
       <c r="O3" t="n">
-        <v>7.061</v>
+        <v>7.07</v>
       </c>
       <c r="P3" t="n">
-        <v>7.197</v>
+        <v>7.198</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.734</v>
+        <v>7.724</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.735</v>
+        <v>3.745</v>
       </c>
       <c r="G4" t="n">
-        <v>4.041</v>
+        <v>4.052</v>
       </c>
       <c r="H4" t="n">
-        <v>4.354</v>
+        <v>4.367</v>
       </c>
       <c r="I4" t="n">
-        <v>4.555</v>
+        <v>4.574</v>
       </c>
       <c r="J4" t="n">
-        <v>4.947</v>
+        <v>4.962</v>
       </c>
       <c r="K4" t="n">
-        <v>5.445</v>
+        <v>5.459</v>
       </c>
       <c r="L4" t="n">
-        <v>5.631</v>
+        <v>5.64</v>
       </c>
       <c r="M4" t="n">
-        <v>5.97</v>
+        <v>5.978</v>
       </c>
       <c r="N4" t="n">
-        <v>6.182</v>
+        <v>6.197</v>
       </c>
       <c r="O4" t="n">
-        <v>6.412</v>
+        <v>6.421</v>
       </c>
       <c r="P4" t="n">
-        <v>6.547</v>
+        <v>6.548</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.087</v>
+        <v>7.077</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.913</v>
+        <v>2.922</v>
       </c>
       <c r="G5" t="n">
-        <v>2.996</v>
+        <v>3.007</v>
       </c>
       <c r="H5" t="n">
-        <v>3.213</v>
+        <v>3.226</v>
       </c>
       <c r="I5" t="n">
-        <v>3.451</v>
+        <v>3.47</v>
       </c>
       <c r="J5" t="n">
-        <v>3.813</v>
+        <v>3.828</v>
       </c>
       <c r="K5" t="n">
-        <v>4.091</v>
+        <v>4.104</v>
       </c>
       <c r="L5" t="n">
-        <v>4.124</v>
+        <v>4.133</v>
       </c>
       <c r="M5" t="n">
-        <v>4.253</v>
+        <v>4.26</v>
       </c>
       <c r="N5" t="n">
-        <v>4.307</v>
+        <v>4.322</v>
       </c>
       <c r="O5" t="n">
-        <v>4.35</v>
+        <v>4.359</v>
       </c>
       <c r="P5" t="n">
         <v>4.686</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.578</v>
+        <v>5.568</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.954</v>
+        <v>2.963</v>
       </c>
       <c r="G6" t="n">
-        <v>3.052</v>
+        <v>3.062</v>
       </c>
       <c r="H6" t="n">
-        <v>3.282</v>
+        <v>3.295</v>
       </c>
       <c r="I6" t="n">
-        <v>3.534</v>
+        <v>3.553</v>
       </c>
       <c r="J6" t="n">
-        <v>3.902</v>
+        <v>3.917</v>
       </c>
       <c r="K6" t="n">
-        <v>4.206</v>
+        <v>4.219</v>
       </c>
       <c r="L6" t="n">
-        <v>4.241</v>
+        <v>4.251</v>
       </c>
       <c r="M6" t="n">
-        <v>4.408</v>
+        <v>4.416</v>
       </c>
       <c r="N6" t="n">
-        <v>4.475</v>
+        <v>4.489</v>
       </c>
       <c r="O6" t="n">
-        <v>4.617</v>
+        <v>4.626</v>
       </c>
       <c r="P6" t="n">
         <v>5.118</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.974</v>
+        <v>5.964</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.934</v>
+        <v>2.943</v>
       </c>
       <c r="G7" t="n">
-        <v>3.015</v>
+        <v>3.026</v>
       </c>
       <c r="H7" t="n">
-        <v>3.229</v>
+        <v>3.242</v>
       </c>
       <c r="I7" t="n">
-        <v>3.469</v>
+        <v>3.488</v>
       </c>
       <c r="J7" t="n">
-        <v>3.837</v>
+        <v>3.851</v>
       </c>
       <c r="K7" t="n">
-        <v>4.119</v>
+        <v>4.132</v>
       </c>
       <c r="L7" t="n">
-        <v>4.15</v>
+        <v>4.159</v>
       </c>
       <c r="M7" t="n">
-        <v>4.314</v>
+        <v>4.321</v>
       </c>
       <c r="N7" t="n">
-        <v>4.367</v>
+        <v>4.382</v>
       </c>
       <c r="O7" t="n">
-        <v>4.515</v>
+        <v>4.524</v>
       </c>
       <c r="P7" t="n">
-        <v>4.901</v>
+        <v>4.902</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.741</v>
+        <v>5.731</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.355</v>
+        <v>5.364</v>
       </c>
       <c r="G8" t="n">
-        <v>5.96</v>
+        <v>5.971</v>
       </c>
       <c r="H8" t="n">
-        <v>6.392</v>
+        <v>6.405</v>
       </c>
       <c r="I8" t="n">
-        <v>6.638</v>
+        <v>6.657</v>
       </c>
       <c r="J8" t="n">
-        <v>7.093</v>
+        <v>7.108</v>
       </c>
       <c r="K8" t="n">
-        <v>7.879</v>
+        <v>7.893</v>
       </c>
       <c r="L8" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="M8" t="n">
-        <v>8.602</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.778</v>
+        <v>8.792999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.07</v>
+        <v>9.079000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.308</v>
+        <v>9.308999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.043</v>
+        <v>10.033</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1072,48 +1072,48 @@
         <v>2.914</v>
       </c>
       <c r="I9" t="n">
-        <v>3.17</v>
+        <v>3.172</v>
       </c>
       <c r="J9" t="n">
-        <v>3.349</v>
+        <v>3.355</v>
       </c>
       <c r="K9" t="n">
-        <v>3.6</v>
+        <v>3.61</v>
       </c>
       <c r="L9" t="n">
-        <v>3.648</v>
+        <v>3.656</v>
       </c>
       <c r="M9" t="n">
-        <v>3.75</v>
+        <v>3.757</v>
       </c>
       <c r="N9" t="n">
-        <v>3.917</v>
+        <v>3.931</v>
       </c>
       <c r="O9" t="n">
-        <v>3.965</v>
+        <v>3.975</v>
       </c>
       <c r="P9" t="n">
-        <v>4.118</v>
+        <v>4.119</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.205</v>
+        <v>4.195</v>
       </c>
       <c r="R9" t="n">
-        <v>4.235</v>
+        <v>4.217</v>
       </c>
       <c r="S9" t="n">
-        <v>4.255</v>
+        <v>4.23</v>
       </c>
       <c r="T9" t="n">
-        <v>4.197</v>
+        <v>4.185</v>
       </c>
       <c r="U9" t="n">
-        <v>4.048</v>
+        <v>4.035</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1145,25 +1145,25 @@
         <v>2.924</v>
       </c>
       <c r="I10" t="n">
-        <v>3.173</v>
+        <v>3.176</v>
       </c>
       <c r="J10" t="n">
-        <v>3.374</v>
+        <v>3.381</v>
       </c>
       <c r="K10" t="n">
-        <v>3.633</v>
+        <v>3.643</v>
       </c>
       <c r="L10" t="n">
-        <v>3.697</v>
+        <v>3.707</v>
       </c>
       <c r="M10" t="n">
-        <v>3.844</v>
+        <v>3.851</v>
       </c>
       <c r="N10" t="n">
-        <v>3.934</v>
+        <v>3.949</v>
       </c>
       <c r="O10" t="n">
-        <v>4.172</v>
+        <v>4.181</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1218,31 +1218,31 @@
         <v>2.747</v>
       </c>
       <c r="I11" t="n">
-        <v>2.977</v>
+        <v>2.98</v>
       </c>
       <c r="J11" t="n">
-        <v>3.172</v>
+        <v>3.179</v>
       </c>
       <c r="K11" t="n">
-        <v>3.42</v>
+        <v>3.43</v>
       </c>
       <c r="L11" t="n">
-        <v>3.495</v>
+        <v>3.504</v>
       </c>
       <c r="M11" t="n">
-        <v>3.652</v>
+        <v>3.659</v>
       </c>
       <c r="N11" t="n">
-        <v>3.742</v>
+        <v>3.757</v>
       </c>
       <c r="O11" t="n">
-        <v>3.938</v>
+        <v>3.948</v>
       </c>
       <c r="P11" t="n">
         <v>4.07</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.406</v>
+        <v>4.396</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.218</v>
+        <v>3.225</v>
       </c>
       <c r="G12" t="n">
-        <v>3.418</v>
+        <v>3.43</v>
       </c>
       <c r="H12" t="n">
-        <v>3.627</v>
+        <v>3.647</v>
       </c>
       <c r="I12" t="n">
-        <v>3.854</v>
+        <v>3.874</v>
       </c>
       <c r="J12" t="n">
-        <v>4.243</v>
+        <v>4.255</v>
       </c>
       <c r="K12" t="n">
-        <v>4.483</v>
+        <v>4.495</v>
       </c>
       <c r="L12" t="n">
-        <v>4.556</v>
+        <v>4.566</v>
       </c>
       <c r="M12" t="n">
-        <v>4.721</v>
+        <v>4.729</v>
       </c>
       <c r="N12" t="n">
-        <v>4.794</v>
+        <v>4.809</v>
       </c>
       <c r="O12" t="n">
-        <v>4.953</v>
+        <v>4.963</v>
       </c>
       <c r="P12" t="n">
         <v>5.154</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.52</v>
+        <v>5.51</v>
       </c>
       <c r="R12" t="n">
-        <v>5.726</v>
+        <v>5.708</v>
       </c>
       <c r="S12" t="n">
-        <v>5.958</v>
+        <v>5.933</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.972</v>
+        <v>2.979</v>
       </c>
       <c r="G13" t="n">
-        <v>3.109</v>
+        <v>3.12</v>
       </c>
       <c r="H13" t="n">
-        <v>3.294</v>
+        <v>3.314</v>
       </c>
       <c r="I13" t="n">
-        <v>3.502</v>
+        <v>3.522</v>
       </c>
       <c r="J13" t="n">
-        <v>3.879</v>
+        <v>3.892</v>
       </c>
       <c r="K13" t="n">
-        <v>4.117</v>
+        <v>4.129</v>
       </c>
       <c r="L13" t="n">
-        <v>4.195</v>
+        <v>4.206</v>
       </c>
       <c r="M13" t="n">
-        <v>4.348</v>
+        <v>4.356</v>
       </c>
       <c r="N13" t="n">
-        <v>4.422</v>
+        <v>4.437</v>
       </c>
       <c r="O13" t="n">
-        <v>4.582</v>
+        <v>4.592</v>
       </c>
       <c r="P13" t="n">
-        <v>4.745</v>
+        <v>4.746</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.041</v>
+        <v>5.031</v>
       </c>
       <c r="R13" t="n">
-        <v>5.276</v>
+        <v>5.258</v>
       </c>
       <c r="S13" t="n">
-        <v>5.52</v>
+        <v>5.495</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.791</v>
+        <v>2.798</v>
       </c>
       <c r="G14" t="n">
-        <v>2.914</v>
+        <v>2.926</v>
       </c>
       <c r="H14" t="n">
-        <v>3.097</v>
+        <v>3.117</v>
       </c>
       <c r="I14" t="n">
-        <v>3.285</v>
+        <v>3.306</v>
       </c>
       <c r="J14" t="n">
-        <v>3.621</v>
+        <v>3.633</v>
       </c>
       <c r="K14" t="n">
-        <v>3.805</v>
+        <v>3.817</v>
       </c>
       <c r="L14" t="n">
-        <v>3.868</v>
+        <v>3.879</v>
       </c>
       <c r="M14" t="n">
-        <v>4.034</v>
+        <v>4.042</v>
       </c>
       <c r="N14" t="n">
-        <v>4.101</v>
+        <v>4.117</v>
       </c>
       <c r="O14" t="n">
-        <v>4.24</v>
+        <v>4.25</v>
       </c>
       <c r="P14" t="n">
-        <v>4.38</v>
+        <v>4.381</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.63</v>
+        <v>4.62</v>
       </c>
       <c r="R14" t="n">
-        <v>4.79</v>
+        <v>4.772</v>
       </c>
       <c r="S14" t="n">
-        <v>4.973</v>
+        <v>4.948</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.769</v>
+        <v>2.775</v>
       </c>
       <c r="G15" t="n">
-        <v>2.888</v>
+        <v>2.9</v>
       </c>
       <c r="H15" t="n">
-        <v>3.068</v>
+        <v>3.088</v>
       </c>
       <c r="I15" t="n">
-        <v>3.237</v>
+        <v>3.258</v>
       </c>
       <c r="J15" t="n">
-        <v>3.56</v>
+        <v>3.572</v>
       </c>
       <c r="K15" t="n">
-        <v>3.757</v>
+        <v>3.769</v>
       </c>
       <c r="L15" t="n">
-        <v>3.804</v>
+        <v>3.814</v>
       </c>
       <c r="M15" t="n">
-        <v>3.947</v>
+        <v>3.954</v>
       </c>
       <c r="N15" t="n">
-        <v>4.005</v>
+        <v>4.02</v>
       </c>
       <c r="O15" t="n">
-        <v>4.181</v>
+        <v>4.191</v>
       </c>
       <c r="P15" t="n">
-        <v>4.279</v>
+        <v>4.28</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.533</v>
+        <v>4.523</v>
       </c>
       <c r="R15" t="n">
-        <v>4.685</v>
+        <v>4.667</v>
       </c>
       <c r="S15" t="n">
-        <v>4.868</v>
+        <v>4.843</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.769</v>
+        <v>2.775</v>
       </c>
       <c r="G16" t="n">
-        <v>2.888</v>
+        <v>2.9</v>
       </c>
       <c r="H16" t="n">
-        <v>3.068</v>
+        <v>3.088</v>
       </c>
       <c r="I16" t="n">
-        <v>3.237</v>
+        <v>3.258</v>
       </c>
       <c r="J16" t="n">
-        <v>3.56</v>
+        <v>3.572</v>
       </c>
       <c r="K16" t="n">
-        <v>3.757</v>
+        <v>3.769</v>
       </c>
       <c r="L16" t="n">
-        <v>3.804</v>
+        <v>3.814</v>
       </c>
       <c r="M16" t="n">
-        <v>3.947</v>
+        <v>3.954</v>
       </c>
       <c r="N16" t="n">
-        <v>4.008</v>
+        <v>4.023</v>
       </c>
       <c r="O16" t="n">
-        <v>4.188</v>
+        <v>4.198</v>
       </c>
       <c r="P16" t="n">
         <v>4.303</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.56</v>
+        <v>4.55</v>
       </c>
       <c r="R16" t="n">
-        <v>4.713</v>
+        <v>4.695</v>
       </c>
       <c r="S16" t="n">
-        <v>4.897</v>
+        <v>4.872</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1656,28 +1656,28 @@
         <v>3.016</v>
       </c>
       <c r="I17" t="n">
-        <v>3.253</v>
+        <v>3.256</v>
       </c>
       <c r="J17" t="n">
-        <v>3.45</v>
+        <v>3.456</v>
       </c>
       <c r="K17" t="n">
-        <v>3.711</v>
+        <v>3.721</v>
       </c>
       <c r="L17" t="n">
-        <v>3.781</v>
+        <v>3.791</v>
       </c>
       <c r="M17" t="n">
-        <v>3.967</v>
+        <v>3.975</v>
       </c>
       <c r="N17" t="n">
-        <v>4.037</v>
+        <v>4.052</v>
       </c>
       <c r="O17" t="n">
-        <v>4.201</v>
+        <v>4.211</v>
       </c>
       <c r="P17" t="n">
-        <v>4.35</v>
+        <v>4.351</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1729,25 +1729,25 @@
         <v>3.017</v>
       </c>
       <c r="I18" t="n">
-        <v>3.254</v>
+        <v>3.257</v>
       </c>
       <c r="J18" t="n">
-        <v>3.45</v>
+        <v>3.456</v>
       </c>
       <c r="K18" t="n">
-        <v>3.712</v>
+        <v>3.722</v>
       </c>
       <c r="L18" t="n">
-        <v>3.781</v>
+        <v>3.791</v>
       </c>
       <c r="M18" t="n">
-        <v>3.967</v>
+        <v>3.975</v>
       </c>
       <c r="N18" t="n">
-        <v>4.037</v>
+        <v>4.053</v>
       </c>
       <c r="O18" t="n">
-        <v>4.199</v>
+        <v>4.209</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.781</v>
+        <v>2.787</v>
       </c>
       <c r="G19" t="n">
-        <v>2.903</v>
+        <v>2.914</v>
       </c>
       <c r="H19" t="n">
-        <v>3.085</v>
+        <v>3.105</v>
       </c>
       <c r="I19" t="n">
-        <v>3.269</v>
+        <v>3.29</v>
       </c>
       <c r="J19" t="n">
-        <v>3.603</v>
+        <v>3.616</v>
       </c>
       <c r="K19" t="n">
-        <v>3.801</v>
+        <v>3.813</v>
       </c>
       <c r="L19" t="n">
-        <v>3.864</v>
+        <v>3.875</v>
       </c>
       <c r="M19" t="n">
-        <v>4.024</v>
+        <v>4.032</v>
       </c>
       <c r="N19" t="n">
-        <v>4.091</v>
+        <v>4.106</v>
       </c>
       <c r="O19" t="n">
-        <v>4.224</v>
+        <v>4.234</v>
       </c>
       <c r="P19" t="n">
         <v>4.34</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.571</v>
+        <v>4.56</v>
       </c>
       <c r="R19" t="n">
-        <v>4.733</v>
+        <v>4.714</v>
       </c>
       <c r="S19" t="n">
-        <v>4.908</v>
+        <v>4.883</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.607</v>
+        <v>2.61</v>
       </c>
       <c r="G20" t="n">
-        <v>2.691</v>
+        <v>2.693</v>
       </c>
       <c r="H20" t="n">
-        <v>2.762</v>
+        <v>2.768</v>
       </c>
       <c r="I20" t="n">
-        <v>2.869</v>
+        <v>2.881</v>
       </c>
       <c r="J20" t="n">
-        <v>3.376</v>
+        <v>3.386</v>
       </c>
       <c r="K20" t="n">
-        <v>3.625</v>
+        <v>3.635</v>
       </c>
       <c r="L20" t="n">
-        <v>3.673</v>
+        <v>3.68</v>
       </c>
       <c r="M20" t="n">
-        <v>3.79</v>
+        <v>3.8</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.906</v>
+        <v>2.91</v>
       </c>
       <c r="G21" t="n">
-        <v>3.002</v>
+        <v>3.012</v>
       </c>
       <c r="H21" t="n">
-        <v>3.204</v>
+        <v>3.221</v>
       </c>
       <c r="I21" t="n">
-        <v>3.375</v>
+        <v>3.397</v>
       </c>
       <c r="J21" t="n">
-        <v>3.747</v>
+        <v>3.76</v>
       </c>
       <c r="K21" t="n">
-        <v>4.029</v>
+        <v>4.044</v>
       </c>
       <c r="L21" t="n">
-        <v>4.099</v>
+        <v>4.11</v>
       </c>
       <c r="M21" t="n">
-        <v>4.245</v>
+        <v>4.257</v>
       </c>
       <c r="N21" t="n">
-        <v>4.33</v>
+        <v>4.346</v>
       </c>
       <c r="O21" t="n">
-        <v>4.437</v>
+        <v>4.448</v>
       </c>
       <c r="P21" t="n">
-        <v>4.6</v>
+        <v>4.602</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.733</v>
+        <v>4.723</v>
       </c>
       <c r="R21" t="n">
-        <v>4.782</v>
+        <v>4.763</v>
       </c>
       <c r="S21" t="n">
-        <v>4.865</v>
+        <v>4.839</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.852</v>
+        <v>2.856</v>
       </c>
       <c r="G22" t="n">
-        <v>2.948</v>
+        <v>2.958</v>
       </c>
       <c r="H22" t="n">
-        <v>3.136</v>
+        <v>3.152</v>
       </c>
       <c r="I22" t="n">
-        <v>3.293</v>
+        <v>3.315</v>
       </c>
       <c r="J22" t="n">
-        <v>3.632</v>
+        <v>3.645</v>
       </c>
       <c r="K22" t="n">
-        <v>3.911</v>
+        <v>3.925</v>
       </c>
       <c r="L22" t="n">
-        <v>3.966</v>
+        <v>3.977</v>
       </c>
       <c r="M22" t="n">
-        <v>4.115</v>
+        <v>4.127</v>
       </c>
       <c r="N22" t="n">
-        <v>4.203</v>
+        <v>4.219</v>
       </c>
       <c r="O22" t="n">
-        <v>4.307</v>
+        <v>4.319</v>
       </c>
       <c r="P22" t="n">
-        <v>4.464</v>
+        <v>4.465</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.592</v>
+        <v>4.581</v>
       </c>
       <c r="R22" t="n">
-        <v>4.631</v>
+        <v>4.612</v>
       </c>
       <c r="S22" t="n">
-        <v>4.71</v>
+        <v>4.684</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.803</v>
+        <v>2.807</v>
       </c>
       <c r="G23" t="n">
-        <v>2.903</v>
+        <v>2.913</v>
       </c>
       <c r="H23" t="n">
-        <v>3.078</v>
+        <v>3.094</v>
       </c>
       <c r="I23" t="n">
-        <v>3.243</v>
+        <v>3.264</v>
       </c>
       <c r="J23" t="n">
-        <v>3.573</v>
+        <v>3.586</v>
       </c>
       <c r="K23" t="n">
-        <v>3.812</v>
+        <v>3.826</v>
       </c>
       <c r="L23" t="n">
-        <v>3.865</v>
+        <v>3.876</v>
       </c>
       <c r="M23" t="n">
-        <v>4.008</v>
+        <v>4.02</v>
       </c>
       <c r="N23" t="n">
-        <v>4.098</v>
+        <v>4.114</v>
       </c>
       <c r="O23" t="n">
-        <v>4.18</v>
+        <v>4.192</v>
       </c>
       <c r="P23" t="n">
-        <v>4.327</v>
+        <v>4.329</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.398</v>
+        <v>4.388</v>
       </c>
       <c r="R23" t="n">
-        <v>4.415</v>
+        <v>4.395</v>
       </c>
       <c r="S23" t="n">
-        <v>4.465</v>
+        <v>4.439</v>
       </c>
       <c r="T23" t="n">
-        <v>4.401</v>
+        <v>4.389</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.74</v>
+        <v>2.744</v>
       </c>
       <c r="G24" t="n">
-        <v>2.817</v>
+        <v>2.827</v>
       </c>
       <c r="H24" t="n">
-        <v>2.976</v>
+        <v>2.992</v>
       </c>
       <c r="I24" t="n">
-        <v>3.182</v>
+        <v>3.204</v>
       </c>
       <c r="J24" t="n">
-        <v>3.469</v>
+        <v>3.482</v>
       </c>
       <c r="K24" t="n">
-        <v>3.695</v>
+        <v>3.709</v>
       </c>
       <c r="L24" t="n">
-        <v>3.744</v>
+        <v>3.755</v>
       </c>
       <c r="M24" t="n">
-        <v>3.869</v>
+        <v>3.88</v>
       </c>
       <c r="N24" t="n">
-        <v>3.973</v>
+        <v>3.989</v>
       </c>
       <c r="O24" t="n">
-        <v>4.171</v>
+        <v>4.182</v>
       </c>
       <c r="P24" t="n">
-        <v>4.264</v>
+        <v>4.266</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.323</v>
+        <v>4.312</v>
       </c>
       <c r="R24" t="n">
-        <v>4.337</v>
+        <v>4.317</v>
       </c>
       <c r="S24" t="n">
-        <v>4.38</v>
+        <v>4.354</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.797</v>
+        <v>2.801</v>
       </c>
       <c r="G25" t="n">
-        <v>2.903</v>
+        <v>2.913</v>
       </c>
       <c r="H25" t="n">
-        <v>3.081</v>
+        <v>3.097</v>
       </c>
       <c r="I25" t="n">
-        <v>3.25</v>
+        <v>3.272</v>
       </c>
       <c r="J25" t="n">
-        <v>3.588</v>
+        <v>3.601</v>
       </c>
       <c r="K25" t="n">
-        <v>3.844</v>
+        <v>3.859</v>
       </c>
       <c r="L25" t="n">
-        <v>3.896</v>
+        <v>3.906</v>
       </c>
       <c r="M25" t="n">
-        <v>4.039</v>
+        <v>4.051</v>
       </c>
       <c r="N25" t="n">
-        <v>4.125</v>
+        <v>4.14</v>
       </c>
       <c r="O25" t="n">
-        <v>4.209</v>
+        <v>4.221</v>
       </c>
       <c r="P25" t="n">
-        <v>4.349</v>
+        <v>4.35</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.431</v>
+        <v>4.421</v>
       </c>
       <c r="R25" t="n">
-        <v>4.438</v>
+        <v>4.419</v>
       </c>
       <c r="S25" t="n">
-        <v>4.488</v>
+        <v>4.462</v>
       </c>
       <c r="T25" t="n">
-        <v>4.419</v>
+        <v>4.407</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.068</v>
+        <v>3.071</v>
       </c>
       <c r="G26" t="n">
-        <v>3.225</v>
+        <v>3.23</v>
       </c>
       <c r="H26" t="n">
-        <v>3.51</v>
+        <v>3.524</v>
       </c>
       <c r="I26" t="n">
-        <v>3.731</v>
+        <v>3.747</v>
       </c>
       <c r="J26" t="n">
-        <v>4.224</v>
+        <v>4.238</v>
       </c>
       <c r="K26" t="n">
-        <v>4.661</v>
+        <v>4.674</v>
       </c>
       <c r="L26" t="n">
-        <v>4.781</v>
+        <v>4.79</v>
       </c>
       <c r="M26" t="n">
-        <v>4.982</v>
+        <v>4.989</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.282</v>
+        <v>5.292</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.877</v>
+        <v>2.883</v>
       </c>
       <c r="G27" t="n">
-        <v>2.983</v>
+        <v>2.992</v>
       </c>
       <c r="H27" t="n">
-        <v>3.176</v>
+        <v>3.195</v>
       </c>
       <c r="I27" t="n">
-        <v>3.367</v>
+        <v>3.386</v>
       </c>
       <c r="J27" t="n">
-        <v>3.731</v>
+        <v>3.744</v>
       </c>
       <c r="K27" t="n">
-        <v>3.979</v>
+        <v>3.992</v>
       </c>
       <c r="L27" t="n">
-        <v>4.049</v>
+        <v>4.06</v>
       </c>
       <c r="M27" t="n">
-        <v>4.197</v>
+        <v>4.205</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.377</v>
+        <v>4.387</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.98</v>
+        <v>2.986</v>
       </c>
       <c r="G28" t="n">
-        <v>3.094</v>
+        <v>3.103</v>
       </c>
       <c r="H28" t="n">
-        <v>3.301</v>
+        <v>3.32</v>
       </c>
       <c r="I28" t="n">
-        <v>3.505</v>
+        <v>3.523</v>
       </c>
       <c r="J28" t="n">
-        <v>3.904</v>
+        <v>3.917</v>
       </c>
       <c r="K28" t="n">
-        <v>4.171</v>
+        <v>4.184</v>
       </c>
       <c r="L28" t="n">
-        <v>4.252</v>
+        <v>4.263</v>
       </c>
       <c r="M28" t="n">
-        <v>4.409</v>
+        <v>4.417</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.669</v>
+        <v>4.679</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.827</v>
+        <v>2.832</v>
       </c>
       <c r="G29" t="n">
-        <v>2.934</v>
+        <v>2.943</v>
       </c>
       <c r="H29" t="n">
-        <v>3.116</v>
+        <v>3.135</v>
       </c>
       <c r="I29" t="n">
-        <v>3.296</v>
+        <v>3.315</v>
       </c>
       <c r="J29" t="n">
-        <v>3.643</v>
+        <v>3.656</v>
       </c>
       <c r="K29" t="n">
-        <v>3.875</v>
+        <v>3.887</v>
       </c>
       <c r="L29" t="n">
-        <v>3.935</v>
+        <v>3.945</v>
       </c>
       <c r="M29" t="n">
-        <v>4.06</v>
+        <v>4.067</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.247</v>
+        <v>4.257</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.112</v>
+        <v>3.114</v>
       </c>
       <c r="G30" t="n">
-        <v>3.205</v>
+        <v>3.208</v>
       </c>
       <c r="H30" t="n">
-        <v>3.443</v>
+        <v>3.456</v>
       </c>
       <c r="I30" t="n">
-        <v>3.656</v>
+        <v>3.67</v>
       </c>
       <c r="J30" t="n">
-        <v>4.093</v>
+        <v>4.106</v>
       </c>
       <c r="K30" t="n">
-        <v>4.461</v>
+        <v>4.473</v>
       </c>
       <c r="L30" t="n">
-        <v>4.56</v>
+        <v>4.57</v>
       </c>
       <c r="M30" t="n">
-        <v>4.751</v>
+        <v>4.759</v>
       </c>
       <c r="N30" t="n">
-        <v>4.931</v>
+        <v>4.946</v>
       </c>
       <c r="O30" t="n">
-        <v>5.232</v>
+        <v>5.242</v>
       </c>
       <c r="P30" t="n">
         <v>5.493</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.267</v>
+        <v>6.256</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.441</v>
+        <v>3.443</v>
       </c>
       <c r="G31" t="n">
-        <v>3.57</v>
+        <v>3.573</v>
       </c>
       <c r="H31" t="n">
-        <v>3.857</v>
+        <v>3.871</v>
       </c>
       <c r="I31" t="n">
-        <v>4.085</v>
+        <v>4.1</v>
       </c>
       <c r="J31" t="n">
-        <v>4.585</v>
+        <v>4.598</v>
       </c>
       <c r="K31" t="n">
-        <v>4.993</v>
+        <v>5.005</v>
       </c>
       <c r="L31" t="n">
-        <v>5.172</v>
+        <v>5.183</v>
       </c>
       <c r="M31" t="n">
-        <v>5.482</v>
+        <v>5.489</v>
       </c>
       <c r="N31" t="n">
-        <v>5.79</v>
+        <v>5.805</v>
       </c>
       <c r="O31" t="n">
-        <v>6.268</v>
+        <v>6.278</v>
       </c>
       <c r="P31" t="n">
-        <v>6.481</v>
+        <v>6.482</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.241</v>
+        <v>7.229</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.211</v>
+        <v>3.213</v>
       </c>
       <c r="G32" t="n">
-        <v>3.323</v>
+        <v>3.326</v>
       </c>
       <c r="H32" t="n">
-        <v>3.586</v>
+        <v>3.6</v>
       </c>
       <c r="I32" t="n">
-        <v>3.815</v>
+        <v>3.829</v>
       </c>
       <c r="J32" t="n">
-        <v>4.271</v>
+        <v>4.284</v>
       </c>
       <c r="K32" t="n">
-        <v>4.646</v>
+        <v>4.658</v>
       </c>
       <c r="L32" t="n">
-        <v>4.764</v>
+        <v>4.774</v>
       </c>
       <c r="M32" t="n">
-        <v>5.024</v>
+        <v>5.031</v>
       </c>
       <c r="N32" t="n">
-        <v>5.291</v>
+        <v>5.307</v>
       </c>
       <c r="O32" t="n">
-        <v>5.678</v>
+        <v>5.688</v>
       </c>
       <c r="P32" t="n">
         <v>5.953</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.728</v>
+        <v>6.717</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.976</v>
+        <v>2.978</v>
       </c>
       <c r="G33" t="n">
-        <v>3.069</v>
+        <v>3.072</v>
       </c>
       <c r="H33" t="n">
-        <v>3.26</v>
+        <v>3.274</v>
       </c>
       <c r="I33" t="n">
-        <v>3.439</v>
+        <v>3.454</v>
       </c>
       <c r="J33" t="n">
-        <v>3.799</v>
+        <v>3.813</v>
       </c>
       <c r="K33" t="n">
-        <v>4.102</v>
+        <v>4.115</v>
       </c>
       <c r="L33" t="n">
-        <v>4.162</v>
+        <v>4.173</v>
       </c>
       <c r="M33" t="n">
-        <v>4.277</v>
+        <v>4.284</v>
       </c>
       <c r="N33" t="n">
-        <v>4.321</v>
+        <v>4.336</v>
       </c>
       <c r="O33" t="n">
-        <v>4.386</v>
+        <v>4.396</v>
       </c>
       <c r="P33" t="n">
-        <v>4.525</v>
+        <v>4.526</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.984</v>
+        <v>4.973</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.036</v>
+        <v>3.038</v>
       </c>
       <c r="G34" t="n">
-        <v>3.122</v>
+        <v>3.125</v>
       </c>
       <c r="H34" t="n">
-        <v>3.322</v>
+        <v>3.336</v>
       </c>
       <c r="I34" t="n">
-        <v>3.507</v>
+        <v>3.522</v>
       </c>
       <c r="J34" t="n">
-        <v>3.87</v>
+        <v>3.884</v>
       </c>
       <c r="K34" t="n">
-        <v>4.179</v>
+        <v>4.192</v>
       </c>
       <c r="L34" t="n">
-        <v>4.242</v>
+        <v>4.252</v>
       </c>
       <c r="M34" t="n">
-        <v>4.368</v>
+        <v>4.375</v>
       </c>
       <c r="N34" t="n">
-        <v>4.424</v>
+        <v>4.44</v>
       </c>
       <c r="O34" t="n">
-        <v>4.555</v>
+        <v>4.565</v>
       </c>
       <c r="P34" t="n">
         <v>4.82</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.685</v>
+        <v>5.674</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.01</v>
+        <v>3.012</v>
       </c>
       <c r="G35" t="n">
-        <v>3.096</v>
+        <v>3.099</v>
       </c>
       <c r="H35" t="n">
-        <v>3.29</v>
+        <v>3.304</v>
       </c>
       <c r="I35" t="n">
-        <v>3.474</v>
+        <v>3.489</v>
       </c>
       <c r="J35" t="n">
-        <v>3.839</v>
+        <v>3.853</v>
       </c>
       <c r="K35" t="n">
-        <v>4.132</v>
+        <v>4.145</v>
       </c>
       <c r="L35" t="n">
-        <v>4.196</v>
+        <v>4.207</v>
       </c>
       <c r="M35" t="n">
-        <v>4.314</v>
+        <v>4.321</v>
       </c>
       <c r="N35" t="n">
-        <v>4.361</v>
+        <v>4.376</v>
       </c>
       <c r="O35" t="n">
-        <v>4.452</v>
+        <v>4.462</v>
       </c>
       <c r="P35" t="n">
-        <v>4.622</v>
+        <v>4.623</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.321</v>
+        <v>5.31</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.906</v>
+        <v>2.908</v>
       </c>
       <c r="G36" t="n">
-        <v>2.992</v>
+        <v>2.995</v>
       </c>
       <c r="H36" t="n">
-        <v>3.175</v>
+        <v>3.189</v>
       </c>
       <c r="I36" t="n">
-        <v>3.358</v>
+        <v>3.373</v>
       </c>
       <c r="J36" t="n">
-        <v>3.734</v>
+        <v>3.748</v>
       </c>
       <c r="K36" t="n">
-        <v>4.026</v>
+        <v>4.039</v>
       </c>
       <c r="L36" t="n">
-        <v>4.088</v>
+        <v>4.098</v>
       </c>
       <c r="M36" t="n">
-        <v>4.179</v>
+        <v>4.185</v>
       </c>
       <c r="N36" t="n">
-        <v>4.224</v>
+        <v>4.239</v>
       </c>
       <c r="O36" t="n">
-        <v>4.295</v>
+        <v>4.305</v>
       </c>
       <c r="P36" t="n">
-        <v>4.423</v>
+        <v>4.424</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.701</v>
+        <v>4.69</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.785</v>
+        <v>3.787</v>
       </c>
       <c r="G37" t="n">
-        <v>4.265</v>
+        <v>4.269</v>
       </c>
       <c r="H37" t="n">
-        <v>4.833</v>
+        <v>4.847</v>
       </c>
       <c r="I37" t="n">
-        <v>5.147</v>
+        <v>5.162</v>
       </c>
       <c r="J37" t="n">
-        <v>6.076</v>
+        <v>6.089</v>
       </c>
       <c r="K37" t="n">
-        <v>7.034</v>
+        <v>7.046</v>
       </c>
       <c r="L37" t="n">
-        <v>7.372</v>
+        <v>7.382</v>
       </c>
       <c r="M37" t="n">
-        <v>7.754</v>
+        <v>7.761</v>
       </c>
       <c r="N37" t="n">
-        <v>7.941</v>
+        <v>7.956</v>
       </c>
       <c r="O37" t="n">
-        <v>8.147</v>
+        <v>8.157</v>
       </c>
       <c r="P37" t="n">
         <v>8.281000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.728999999999999</v>
+        <v>8.718</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.844</v>
+        <v>4.846</v>
       </c>
       <c r="G38" t="n">
-        <v>5.578</v>
+        <v>5.582</v>
       </c>
       <c r="H38" t="n">
-        <v>6.357</v>
+        <v>6.371</v>
       </c>
       <c r="I38" t="n">
-        <v>6.828</v>
+        <v>6.843</v>
       </c>
       <c r="J38" t="n">
-        <v>8.019</v>
+        <v>8.032</v>
       </c>
       <c r="K38" t="n">
-        <v>9.156000000000001</v>
+        <v>9.167999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.654999999999999</v>
+        <v>9.664999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.166</v>
+        <v>10.173</v>
       </c>
       <c r="N38" t="n">
-        <v>10.36</v>
+        <v>10.375</v>
       </c>
       <c r="O38" t="n">
-        <v>10.547</v>
+        <v>10.558</v>
       </c>
       <c r="P38" t="n">
-        <v>10.678</v>
+        <v>10.679</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.18</v>
+        <v>11.169</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.165</v>
+        <v>4.167</v>
       </c>
       <c r="G39" t="n">
-        <v>4.776</v>
+        <v>4.78</v>
       </c>
       <c r="H39" t="n">
-        <v>5.422</v>
+        <v>5.436</v>
       </c>
       <c r="I39" t="n">
-        <v>5.832</v>
+        <v>5.846</v>
       </c>
       <c r="J39" t="n">
-        <v>6.891</v>
+        <v>6.904</v>
       </c>
       <c r="K39" t="n">
-        <v>7.988</v>
+        <v>8</v>
       </c>
       <c r="L39" t="n">
-        <v>8.41</v>
+        <v>8.42</v>
       </c>
       <c r="M39" t="n">
-        <v>8.802</v>
+        <v>8.81</v>
       </c>
       <c r="N39" t="n">
-        <v>8.987</v>
+        <v>9.003</v>
       </c>
       <c r="O39" t="n">
-        <v>9.198</v>
+        <v>9.208</v>
       </c>
       <c r="P39" t="n">
-        <v>9.333</v>
+        <v>9.334</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.824999999999999</v>
+        <v>9.814</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.304</v>
+        <v>3.306</v>
       </c>
       <c r="G40" t="n">
-        <v>3.443</v>
+        <v>3.446</v>
       </c>
       <c r="H40" t="n">
-        <v>3.702</v>
+        <v>3.715</v>
       </c>
       <c r="I40" t="n">
-        <v>3.929</v>
+        <v>3.944</v>
       </c>
       <c r="J40" t="n">
-        <v>4.385</v>
+        <v>4.398</v>
       </c>
       <c r="K40" t="n">
-        <v>4.767</v>
+        <v>4.779</v>
       </c>
       <c r="L40" t="n">
-        <v>4.884</v>
+        <v>4.895</v>
       </c>
       <c r="M40" t="n">
-        <v>5.094</v>
+        <v>5.102</v>
       </c>
       <c r="N40" t="n">
-        <v>5.288</v>
+        <v>5.304</v>
       </c>
       <c r="O40" t="n">
-        <v>5.611</v>
+        <v>5.621</v>
       </c>
       <c r="P40" t="n">
-        <v>5.914</v>
+        <v>5.915</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.718</v>
+        <v>6.707</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.69</v>
+        <v>3.692</v>
       </c>
       <c r="G41" t="n">
-        <v>3.872</v>
+        <v>3.875</v>
       </c>
       <c r="H41" t="n">
-        <v>4.186</v>
+        <v>4.2</v>
       </c>
       <c r="I41" t="n">
-        <v>4.433</v>
+        <v>4.447</v>
       </c>
       <c r="J41" t="n">
-        <v>4.94</v>
+        <v>4.953</v>
       </c>
       <c r="K41" t="n">
-        <v>5.367</v>
+        <v>5.379</v>
       </c>
       <c r="L41" t="n">
-        <v>5.563</v>
+        <v>5.573</v>
       </c>
       <c r="M41" t="n">
-        <v>5.897</v>
+        <v>5.904</v>
       </c>
       <c r="N41" t="n">
-        <v>6.219</v>
+        <v>6.235</v>
       </c>
       <c r="O41" t="n">
-        <v>6.726</v>
+        <v>6.737</v>
       </c>
       <c r="P41" t="n">
-        <v>6.973</v>
+        <v>6.974</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.765</v>
+        <v>7.754</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.425</v>
+        <v>3.427</v>
       </c>
       <c r="G42" t="n">
-        <v>3.592</v>
+        <v>3.595</v>
       </c>
       <c r="H42" t="n">
-        <v>3.877</v>
+        <v>3.891</v>
       </c>
       <c r="I42" t="n">
-        <v>4.118</v>
+        <v>4.132</v>
       </c>
       <c r="J42" t="n">
-        <v>4.587</v>
+        <v>4.6</v>
       </c>
       <c r="K42" t="n">
-        <v>4.988</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
-        <v>5.12</v>
+        <v>5.131</v>
       </c>
       <c r="M42" t="n">
-        <v>5.401</v>
+        <v>5.409</v>
       </c>
       <c r="N42" t="n">
-        <v>5.703</v>
+        <v>5.718</v>
       </c>
       <c r="O42" t="n">
-        <v>6.103</v>
+        <v>6.113</v>
       </c>
       <c r="P42" t="n">
-        <v>6.416</v>
+        <v>6.417</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.231</v>
+        <v>7.22</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.124</v>
+        <v>3.126</v>
       </c>
       <c r="G43" t="n">
-        <v>3.252</v>
+        <v>3.255</v>
       </c>
       <c r="H43" t="n">
-        <v>3.461</v>
+        <v>3.475</v>
       </c>
       <c r="I43" t="n">
-        <v>3.648</v>
+        <v>3.663</v>
       </c>
       <c r="J43" t="n">
-        <v>4.026</v>
+        <v>4.04</v>
       </c>
       <c r="K43" t="n">
-        <v>4.334</v>
+        <v>4.347</v>
       </c>
       <c r="L43" t="n">
-        <v>4.404</v>
+        <v>4.415</v>
       </c>
       <c r="M43" t="n">
-        <v>4.532</v>
+        <v>4.539</v>
       </c>
       <c r="N43" t="n">
-        <v>4.589</v>
+        <v>4.604</v>
       </c>
       <c r="O43" t="n">
-        <v>4.7</v>
+        <v>4.71</v>
       </c>
       <c r="P43" t="n">
         <v>4.891</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.594</v>
+        <v>5.583</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.984</v>
+        <v>2.986</v>
       </c>
       <c r="G44" t="n">
-        <v>3.101</v>
+        <v>3.104</v>
       </c>
       <c r="H44" t="n">
-        <v>3.298</v>
+        <v>3.312</v>
       </c>
       <c r="I44" t="n">
-        <v>3.485</v>
+        <v>3.5</v>
       </c>
       <c r="J44" t="n">
-        <v>3.875</v>
+        <v>3.889</v>
       </c>
       <c r="K44" t="n">
-        <v>4.178</v>
+        <v>4.191</v>
       </c>
       <c r="L44" t="n">
-        <v>4.248</v>
+        <v>4.258</v>
       </c>
       <c r="M44" t="n">
-        <v>4.349</v>
+        <v>4.356</v>
       </c>
       <c r="N44" t="n">
-        <v>4.406</v>
+        <v>4.421</v>
       </c>
       <c r="O44" t="n">
-        <v>4.496</v>
+        <v>4.505</v>
       </c>
       <c r="P44" t="n">
-        <v>4.653</v>
+        <v>4.654</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.965</v>
+        <v>4.954</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-21 ~ 2026-05-21
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.229</v>
+        <v>3.241</v>
       </c>
       <c r="G2" t="n">
-        <v>3.466</v>
+        <v>3.489</v>
       </c>
       <c r="H2" t="n">
-        <v>3.719</v>
+        <v>3.744</v>
       </c>
       <c r="I2" t="n">
-        <v>3.898</v>
+        <v>3.924</v>
       </c>
       <c r="J2" t="n">
-        <v>4.271</v>
+        <v>4.275</v>
       </c>
       <c r="K2" t="n">
-        <v>4.704</v>
+        <v>4.705</v>
       </c>
       <c r="L2" t="n">
-        <v>4.886</v>
+        <v>4.881</v>
       </c>
       <c r="M2" t="n">
-        <v>5.203</v>
+        <v>5.199</v>
       </c>
       <c r="N2" t="n">
-        <v>5.509</v>
+        <v>5.507</v>
       </c>
       <c r="O2" t="n">
-        <v>5.76</v>
+        <v>5.774</v>
       </c>
       <c r="P2" t="n">
-        <v>6.017</v>
+        <v>6.016</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.655</v>
+        <v>6.642</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.252</v>
+        <v>4.264</v>
       </c>
       <c r="G3" t="n">
-        <v>4.671</v>
+        <v>4.694</v>
       </c>
       <c r="H3" t="n">
-        <v>4.957</v>
+        <v>4.981</v>
       </c>
       <c r="I3" t="n">
-        <v>5.131</v>
+        <v>5.157</v>
       </c>
       <c r="J3" t="n">
-        <v>5.516</v>
+        <v>5.521</v>
       </c>
       <c r="K3" t="n">
-        <v>6.02</v>
+        <v>6.022</v>
       </c>
       <c r="L3" t="n">
-        <v>6.271</v>
+        <v>6.267</v>
       </c>
       <c r="M3" t="n">
-        <v>6.62</v>
+        <v>6.616</v>
       </c>
       <c r="N3" t="n">
-        <v>6.868</v>
+        <v>6.866</v>
       </c>
       <c r="O3" t="n">
-        <v>7.07</v>
+        <v>7.084</v>
       </c>
       <c r="P3" t="n">
-        <v>7.198</v>
+        <v>7.196</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.724</v>
+        <v>7.711</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.745</v>
+        <v>3.757</v>
       </c>
       <c r="G4" t="n">
-        <v>4.052</v>
+        <v>4.075</v>
       </c>
       <c r="H4" t="n">
-        <v>4.367</v>
+        <v>4.391</v>
       </c>
       <c r="I4" t="n">
-        <v>4.574</v>
+        <v>4.6</v>
       </c>
       <c r="J4" t="n">
-        <v>4.962</v>
+        <v>4.966</v>
       </c>
       <c r="K4" t="n">
-        <v>5.459</v>
+        <v>5.46</v>
       </c>
       <c r="L4" t="n">
-        <v>5.64</v>
+        <v>5.636</v>
       </c>
       <c r="M4" t="n">
-        <v>5.978</v>
+        <v>5.974</v>
       </c>
       <c r="N4" t="n">
-        <v>6.197</v>
+        <v>6.194</v>
       </c>
       <c r="O4" t="n">
-        <v>6.421</v>
+        <v>6.435</v>
       </c>
       <c r="P4" t="n">
-        <v>6.548</v>
+        <v>6.546</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.077</v>
+        <v>7.064</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.922</v>
+        <v>2.934</v>
       </c>
       <c r="G5" t="n">
-        <v>3.007</v>
+        <v>3.03</v>
       </c>
       <c r="H5" t="n">
-        <v>3.226</v>
+        <v>3.25</v>
       </c>
       <c r="I5" t="n">
-        <v>3.47</v>
+        <v>3.496</v>
       </c>
       <c r="J5" t="n">
-        <v>3.828</v>
+        <v>3.832</v>
       </c>
       <c r="K5" t="n">
-        <v>4.104</v>
+        <v>4.106</v>
       </c>
       <c r="L5" t="n">
-        <v>4.133</v>
+        <v>4.129</v>
       </c>
       <c r="M5" t="n">
-        <v>4.26</v>
+        <v>4.257</v>
       </c>
       <c r="N5" t="n">
-        <v>4.322</v>
+        <v>4.319</v>
       </c>
       <c r="O5" t="n">
-        <v>4.359</v>
+        <v>4.373</v>
       </c>
       <c r="P5" t="n">
-        <v>4.686</v>
+        <v>4.684</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.568</v>
+        <v>5.555</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.963</v>
+        <v>2.975</v>
       </c>
       <c r="G6" t="n">
-        <v>3.062</v>
+        <v>3.086</v>
       </c>
       <c r="H6" t="n">
-        <v>3.295</v>
+        <v>3.319</v>
       </c>
       <c r="I6" t="n">
-        <v>3.553</v>
+        <v>3.579</v>
       </c>
       <c r="J6" t="n">
-        <v>3.917</v>
+        <v>3.922</v>
       </c>
       <c r="K6" t="n">
-        <v>4.219</v>
+        <v>4.221</v>
       </c>
       <c r="L6" t="n">
-        <v>4.251</v>
+        <v>4.246</v>
       </c>
       <c r="M6" t="n">
-        <v>4.416</v>
+        <v>4.412</v>
       </c>
       <c r="N6" t="n">
-        <v>4.489</v>
+        <v>4.487</v>
       </c>
       <c r="O6" t="n">
-        <v>4.626</v>
+        <v>4.64</v>
       </c>
       <c r="P6" t="n">
-        <v>5.118</v>
+        <v>5.117</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.964</v>
+        <v>5.951</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.943</v>
+        <v>2.955</v>
       </c>
       <c r="G7" t="n">
-        <v>3.026</v>
+        <v>3.049</v>
       </c>
       <c r="H7" t="n">
-        <v>3.242</v>
+        <v>3.266</v>
       </c>
       <c r="I7" t="n">
-        <v>3.488</v>
+        <v>3.514</v>
       </c>
       <c r="J7" t="n">
-        <v>3.851</v>
+        <v>3.856</v>
       </c>
       <c r="K7" t="n">
-        <v>4.132</v>
+        <v>4.134</v>
       </c>
       <c r="L7" t="n">
-        <v>4.159</v>
+        <v>4.154</v>
       </c>
       <c r="M7" t="n">
-        <v>4.321</v>
+        <v>4.318</v>
       </c>
       <c r="N7" t="n">
-        <v>4.382</v>
+        <v>4.379</v>
       </c>
       <c r="O7" t="n">
-        <v>4.524</v>
+        <v>4.538</v>
       </c>
       <c r="P7" t="n">
-        <v>4.902</v>
+        <v>4.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.731</v>
+        <v>5.718</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.364</v>
+        <v>5.376</v>
       </c>
       <c r="G8" t="n">
-        <v>5.971</v>
+        <v>5.994</v>
       </c>
       <c r="H8" t="n">
-        <v>6.405</v>
+        <v>6.43</v>
       </c>
       <c r="I8" t="n">
-        <v>6.657</v>
+        <v>6.683</v>
       </c>
       <c r="J8" t="n">
-        <v>7.108</v>
+        <v>7.113</v>
       </c>
       <c r="K8" t="n">
-        <v>7.893</v>
+        <v>7.894</v>
       </c>
       <c r="L8" t="n">
-        <v>8.23</v>
+        <v>8.225</v>
       </c>
       <c r="M8" t="n">
-        <v>8.609999999999999</v>
+        <v>8.606</v>
       </c>
       <c r="N8" t="n">
-        <v>8.792999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.079000000000001</v>
+        <v>9.093</v>
       </c>
       <c r="P8" t="n">
-        <v>9.308999999999999</v>
+        <v>9.307</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.033</v>
+        <v>10.02</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1069,51 +1069,51 @@
         <v>2.74</v>
       </c>
       <c r="H9" t="n">
-        <v>2.914</v>
+        <v>2.913</v>
       </c>
       <c r="I9" t="n">
         <v>3.172</v>
       </c>
       <c r="J9" t="n">
-        <v>3.355</v>
+        <v>3.358</v>
       </c>
       <c r="K9" t="n">
-        <v>3.61</v>
+        <v>3.604</v>
       </c>
       <c r="L9" t="n">
-        <v>3.656</v>
+        <v>3.65</v>
       </c>
       <c r="M9" t="n">
-        <v>3.757</v>
+        <v>3.755</v>
       </c>
       <c r="N9" t="n">
-        <v>3.931</v>
+        <v>3.93</v>
       </c>
       <c r="O9" t="n">
-        <v>3.975</v>
+        <v>3.99</v>
       </c>
       <c r="P9" t="n">
-        <v>4.119</v>
+        <v>4.117</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.195</v>
+        <v>4.182</v>
       </c>
       <c r="R9" t="n">
-        <v>4.217</v>
+        <v>4.21</v>
       </c>
       <c r="S9" t="n">
         <v>4.23</v>
       </c>
       <c r="T9" t="n">
-        <v>4.185</v>
+        <v>4.183</v>
       </c>
       <c r="U9" t="n">
-        <v>4.035</v>
+        <v>4.033</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.651</v>
+        <v>2.657</v>
       </c>
       <c r="G10" t="n">
         <v>2.773</v>
@@ -1145,25 +1145,25 @@
         <v>2.924</v>
       </c>
       <c r="I10" t="n">
-        <v>3.176</v>
+        <v>3.177</v>
       </c>
       <c r="J10" t="n">
-        <v>3.381</v>
+        <v>3.386</v>
       </c>
       <c r="K10" t="n">
-        <v>3.643</v>
+        <v>3.637</v>
       </c>
       <c r="L10" t="n">
-        <v>3.707</v>
+        <v>3.701</v>
       </c>
       <c r="M10" t="n">
-        <v>3.851</v>
+        <v>3.849</v>
       </c>
       <c r="N10" t="n">
         <v>3.949</v>
       </c>
       <c r="O10" t="n">
-        <v>4.181</v>
+        <v>4.192</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.466</v>
+        <v>2.467</v>
       </c>
       <c r="G11" t="n">
         <v>2.583</v>
@@ -1218,31 +1218,31 @@
         <v>2.747</v>
       </c>
       <c r="I11" t="n">
-        <v>2.98</v>
+        <v>2.981</v>
       </c>
       <c r="J11" t="n">
-        <v>3.179</v>
+        <v>3.182</v>
       </c>
       <c r="K11" t="n">
-        <v>3.43</v>
+        <v>3.424</v>
       </c>
       <c r="L11" t="n">
-        <v>3.504</v>
+        <v>3.499</v>
       </c>
       <c r="M11" t="n">
-        <v>3.659</v>
+        <v>3.657</v>
       </c>
       <c r="N11" t="n">
         <v>3.757</v>
       </c>
       <c r="O11" t="n">
-        <v>3.948</v>
+        <v>3.959</v>
       </c>
       <c r="P11" t="n">
-        <v>4.07</v>
+        <v>4.069</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.396</v>
+        <v>4.383</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,43 +1282,43 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.225</v>
+        <v>3.238</v>
       </c>
       <c r="G12" t="n">
-        <v>3.43</v>
+        <v>3.446</v>
       </c>
       <c r="H12" t="n">
-        <v>3.647</v>
+        <v>3.665</v>
       </c>
       <c r="I12" t="n">
-        <v>3.874</v>
+        <v>3.895</v>
       </c>
       <c r="J12" t="n">
-        <v>4.255</v>
+        <v>4.258</v>
       </c>
       <c r="K12" t="n">
-        <v>4.495</v>
+        <v>4.494</v>
       </c>
       <c r="L12" t="n">
-        <v>4.566</v>
+        <v>4.562</v>
       </c>
       <c r="M12" t="n">
-        <v>4.729</v>
+        <v>4.726</v>
       </c>
       <c r="N12" t="n">
-        <v>4.809</v>
+        <v>4.807</v>
       </c>
       <c r="O12" t="n">
-        <v>4.963</v>
+        <v>4.977</v>
       </c>
       <c r="P12" t="n">
-        <v>5.154</v>
+        <v>5.153</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.51</v>
+        <v>5.497</v>
       </c>
       <c r="R12" t="n">
-        <v>5.708</v>
+        <v>5.701</v>
       </c>
       <c r="S12" t="n">
         <v>5.933</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,43 +1355,43 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.979</v>
+        <v>2.992</v>
       </c>
       <c r="G13" t="n">
-        <v>3.12</v>
+        <v>3.136</v>
       </c>
       <c r="H13" t="n">
-        <v>3.314</v>
+        <v>3.333</v>
       </c>
       <c r="I13" t="n">
-        <v>3.522</v>
+        <v>3.543</v>
       </c>
       <c r="J13" t="n">
-        <v>3.892</v>
+        <v>3.895</v>
       </c>
       <c r="K13" t="n">
-        <v>4.129</v>
+        <v>4.128</v>
       </c>
       <c r="L13" t="n">
-        <v>4.206</v>
+        <v>4.202</v>
       </c>
       <c r="M13" t="n">
-        <v>4.356</v>
+        <v>4.354</v>
       </c>
       <c r="N13" t="n">
-        <v>4.437</v>
+        <v>4.436</v>
       </c>
       <c r="O13" t="n">
-        <v>4.592</v>
+        <v>4.606</v>
       </c>
       <c r="P13" t="n">
-        <v>4.746</v>
+        <v>4.744</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.031</v>
+        <v>5.018</v>
       </c>
       <c r="R13" t="n">
-        <v>5.258</v>
+        <v>5.25</v>
       </c>
       <c r="S13" t="n">
         <v>5.495</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,43 +1428,43 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.798</v>
+        <v>2.811</v>
       </c>
       <c r="G14" t="n">
-        <v>2.926</v>
+        <v>2.942</v>
       </c>
       <c r="H14" t="n">
-        <v>3.117</v>
+        <v>3.136</v>
       </c>
       <c r="I14" t="n">
-        <v>3.306</v>
+        <v>3.327</v>
       </c>
       <c r="J14" t="n">
-        <v>3.633</v>
+        <v>3.636</v>
       </c>
       <c r="K14" t="n">
-        <v>3.817</v>
+        <v>3.816</v>
       </c>
       <c r="L14" t="n">
-        <v>3.879</v>
+        <v>3.875</v>
       </c>
       <c r="M14" t="n">
-        <v>4.042</v>
+        <v>4.04</v>
       </c>
       <c r="N14" t="n">
-        <v>4.117</v>
+        <v>4.115</v>
       </c>
       <c r="O14" t="n">
-        <v>4.25</v>
+        <v>4.264</v>
       </c>
       <c r="P14" t="n">
-        <v>4.381</v>
+        <v>4.379</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.62</v>
+        <v>4.607</v>
       </c>
       <c r="R14" t="n">
-        <v>4.772</v>
+        <v>4.765</v>
       </c>
       <c r="S14" t="n">
         <v>4.948</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,43 +1501,43 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.775</v>
+        <v>2.788</v>
       </c>
       <c r="G15" t="n">
-        <v>2.9</v>
+        <v>2.916</v>
       </c>
       <c r="H15" t="n">
-        <v>3.088</v>
+        <v>3.107</v>
       </c>
       <c r="I15" t="n">
-        <v>3.258</v>
+        <v>3.279</v>
       </c>
       <c r="J15" t="n">
-        <v>3.572</v>
+        <v>3.575</v>
       </c>
       <c r="K15" t="n">
-        <v>3.769</v>
+        <v>3.768</v>
       </c>
       <c r="L15" t="n">
-        <v>3.814</v>
+        <v>3.81</v>
       </c>
       <c r="M15" t="n">
-        <v>3.954</v>
+        <v>3.952</v>
       </c>
       <c r="N15" t="n">
-        <v>4.02</v>
+        <v>4.019</v>
       </c>
       <c r="O15" t="n">
-        <v>4.191</v>
+        <v>4.206</v>
       </c>
       <c r="P15" t="n">
-        <v>4.28</v>
+        <v>4.278</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.523</v>
+        <v>4.51</v>
       </c>
       <c r="R15" t="n">
-        <v>4.667</v>
+        <v>4.66</v>
       </c>
       <c r="S15" t="n">
         <v>4.843</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,43 +1574,43 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.775</v>
+        <v>2.788</v>
       </c>
       <c r="G16" t="n">
-        <v>2.9</v>
+        <v>2.916</v>
       </c>
       <c r="H16" t="n">
-        <v>3.088</v>
+        <v>3.107</v>
       </c>
       <c r="I16" t="n">
-        <v>3.258</v>
+        <v>3.279</v>
       </c>
       <c r="J16" t="n">
-        <v>3.572</v>
+        <v>3.575</v>
       </c>
       <c r="K16" t="n">
-        <v>3.769</v>
+        <v>3.768</v>
       </c>
       <c r="L16" t="n">
-        <v>3.814</v>
+        <v>3.81</v>
       </c>
       <c r="M16" t="n">
-        <v>3.954</v>
+        <v>3.952</v>
       </c>
       <c r="N16" t="n">
-        <v>4.023</v>
+        <v>4.022</v>
       </c>
       <c r="O16" t="n">
-        <v>4.198</v>
+        <v>4.213</v>
       </c>
       <c r="P16" t="n">
-        <v>4.303</v>
+        <v>4.302</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.55</v>
+        <v>4.537</v>
       </c>
       <c r="R16" t="n">
-        <v>4.695</v>
+        <v>4.688</v>
       </c>
       <c r="S16" t="n">
         <v>4.872</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1656,28 +1656,28 @@
         <v>3.016</v>
       </c>
       <c r="I17" t="n">
-        <v>3.256</v>
+        <v>3.257</v>
       </c>
       <c r="J17" t="n">
-        <v>3.456</v>
+        <v>3.459</v>
       </c>
       <c r="K17" t="n">
-        <v>3.721</v>
+        <v>3.715</v>
       </c>
       <c r="L17" t="n">
-        <v>3.791</v>
+        <v>3.785</v>
       </c>
       <c r="M17" t="n">
-        <v>3.975</v>
+        <v>3.972</v>
       </c>
       <c r="N17" t="n">
-        <v>4.052</v>
+        <v>4.053</v>
       </c>
       <c r="O17" t="n">
-        <v>4.211</v>
+        <v>4.221</v>
       </c>
       <c r="P17" t="n">
-        <v>4.351</v>
+        <v>4.349</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1729,25 +1729,25 @@
         <v>3.017</v>
       </c>
       <c r="I18" t="n">
-        <v>3.257</v>
+        <v>3.258</v>
       </c>
       <c r="J18" t="n">
-        <v>3.456</v>
+        <v>3.459</v>
       </c>
       <c r="K18" t="n">
-        <v>3.722</v>
+        <v>3.716</v>
       </c>
       <c r="L18" t="n">
-        <v>3.791</v>
+        <v>3.785</v>
       </c>
       <c r="M18" t="n">
-        <v>3.975</v>
+        <v>3.972</v>
       </c>
       <c r="N18" t="n">
         <v>4.053</v>
       </c>
       <c r="O18" t="n">
-        <v>4.209</v>
+        <v>4.219</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,43 +1793,43 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.787</v>
+        <v>2.8</v>
       </c>
       <c r="G19" t="n">
-        <v>2.914</v>
+        <v>2.929</v>
       </c>
       <c r="H19" t="n">
-        <v>3.105</v>
+        <v>3.122</v>
       </c>
       <c r="I19" t="n">
-        <v>3.29</v>
+        <v>3.31</v>
       </c>
       <c r="J19" t="n">
-        <v>3.616</v>
+        <v>3.618</v>
       </c>
       <c r="K19" t="n">
-        <v>3.813</v>
+        <v>3.812</v>
       </c>
       <c r="L19" t="n">
-        <v>3.875</v>
+        <v>3.871</v>
       </c>
       <c r="M19" t="n">
-        <v>4.032</v>
+        <v>4.029</v>
       </c>
       <c r="N19" t="n">
-        <v>4.106</v>
+        <v>4.105</v>
       </c>
       <c r="O19" t="n">
-        <v>4.234</v>
+        <v>4.249</v>
       </c>
       <c r="P19" t="n">
-        <v>4.34</v>
+        <v>4.338</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.56</v>
+        <v>4.547</v>
       </c>
       <c r="R19" t="n">
-        <v>4.714</v>
+        <v>4.707</v>
       </c>
       <c r="S19" t="n">
         <v>4.883</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.61</v>
+        <v>2.621</v>
       </c>
       <c r="G20" t="n">
-        <v>2.693</v>
+        <v>2.704</v>
       </c>
       <c r="H20" t="n">
-        <v>2.768</v>
+        <v>2.781</v>
       </c>
       <c r="I20" t="n">
-        <v>2.881</v>
+        <v>2.901</v>
       </c>
       <c r="J20" t="n">
-        <v>3.386</v>
+        <v>3.385</v>
       </c>
       <c r="K20" t="n">
-        <v>3.635</v>
+        <v>3.634</v>
       </c>
       <c r="L20" t="n">
-        <v>3.68</v>
+        <v>3.677</v>
       </c>
       <c r="M20" t="n">
-        <v>3.8</v>
+        <v>3.796</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,43 +1939,43 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.91</v>
+        <v>2.918</v>
       </c>
       <c r="G21" t="n">
-        <v>3.012</v>
+        <v>3.027</v>
       </c>
       <c r="H21" t="n">
-        <v>3.221</v>
+        <v>3.242</v>
       </c>
       <c r="I21" t="n">
-        <v>3.397</v>
+        <v>3.424</v>
       </c>
       <c r="J21" t="n">
-        <v>3.76</v>
+        <v>3.761</v>
       </c>
       <c r="K21" t="n">
         <v>4.044</v>
       </c>
       <c r="L21" t="n">
-        <v>4.11</v>
+        <v>4.104</v>
       </c>
       <c r="M21" t="n">
-        <v>4.257</v>
+        <v>4.256</v>
       </c>
       <c r="N21" t="n">
-        <v>4.346</v>
+        <v>4.344</v>
       </c>
       <c r="O21" t="n">
-        <v>4.448</v>
+        <v>4.462</v>
       </c>
       <c r="P21" t="n">
-        <v>4.602</v>
+        <v>4.601</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.723</v>
+        <v>4.71</v>
       </c>
       <c r="R21" t="n">
-        <v>4.763</v>
+        <v>4.756</v>
       </c>
       <c r="S21" t="n">
         <v>4.839</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,43 +2012,43 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.856</v>
+        <v>2.864</v>
       </c>
       <c r="G22" t="n">
-        <v>2.958</v>
+        <v>2.973</v>
       </c>
       <c r="H22" t="n">
-        <v>3.152</v>
+        <v>3.173</v>
       </c>
       <c r="I22" t="n">
-        <v>3.315</v>
+        <v>3.342</v>
       </c>
       <c r="J22" t="n">
-        <v>3.645</v>
+        <v>3.646</v>
       </c>
       <c r="K22" t="n">
         <v>3.925</v>
       </c>
       <c r="L22" t="n">
-        <v>3.977</v>
+        <v>3.971</v>
       </c>
       <c r="M22" t="n">
-        <v>4.127</v>
+        <v>4.126</v>
       </c>
       <c r="N22" t="n">
-        <v>4.219</v>
+        <v>4.218</v>
       </c>
       <c r="O22" t="n">
-        <v>4.319</v>
+        <v>4.332</v>
       </c>
       <c r="P22" t="n">
         <v>4.465</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.581</v>
+        <v>4.568</v>
       </c>
       <c r="R22" t="n">
-        <v>4.612</v>
+        <v>4.604</v>
       </c>
       <c r="S22" t="n">
         <v>4.684</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.807</v>
+        <v>2.815</v>
       </c>
       <c r="G23" t="n">
-        <v>2.913</v>
+        <v>2.928</v>
       </c>
       <c r="H23" t="n">
-        <v>3.094</v>
+        <v>3.114</v>
       </c>
       <c r="I23" t="n">
-        <v>3.264</v>
+        <v>3.291</v>
       </c>
       <c r="J23" t="n">
-        <v>3.586</v>
+        <v>3.587</v>
       </c>
       <c r="K23" t="n">
-        <v>3.826</v>
+        <v>3.825</v>
       </c>
       <c r="L23" t="n">
-        <v>3.876</v>
+        <v>3.871</v>
       </c>
       <c r="M23" t="n">
-        <v>4.02</v>
+        <v>4.019</v>
       </c>
       <c r="N23" t="n">
-        <v>4.114</v>
+        <v>4.112</v>
       </c>
       <c r="O23" t="n">
-        <v>4.192</v>
+        <v>4.205</v>
       </c>
       <c r="P23" t="n">
-        <v>4.329</v>
+        <v>4.328</v>
       </c>
       <c r="Q23" t="n">
+        <v>4.375</v>
+      </c>
+      <c r="R23" t="n">
         <v>4.388</v>
-      </c>
-      <c r="R23" t="n">
-        <v>4.395</v>
       </c>
       <c r="S23" t="n">
         <v>4.439</v>
       </c>
       <c r="T23" t="n">
-        <v>4.389</v>
+        <v>4.387</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,43 +2158,43 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.744</v>
+        <v>2.752</v>
       </c>
       <c r="G24" t="n">
-        <v>2.827</v>
+        <v>2.842</v>
       </c>
       <c r="H24" t="n">
-        <v>2.992</v>
+        <v>3.013</v>
       </c>
       <c r="I24" t="n">
-        <v>3.204</v>
+        <v>3.231</v>
       </c>
       <c r="J24" t="n">
-        <v>3.482</v>
+        <v>3.483</v>
       </c>
       <c r="K24" t="n">
-        <v>3.709</v>
+        <v>3.708</v>
       </c>
       <c r="L24" t="n">
-        <v>3.755</v>
+        <v>3.75</v>
       </c>
       <c r="M24" t="n">
         <v>3.88</v>
       </c>
       <c r="N24" t="n">
-        <v>3.989</v>
+        <v>3.988</v>
       </c>
       <c r="O24" t="n">
-        <v>4.182</v>
+        <v>4.196</v>
       </c>
       <c r="P24" t="n">
-        <v>4.266</v>
+        <v>4.265</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.312</v>
+        <v>4.299</v>
       </c>
       <c r="R24" t="n">
-        <v>4.317</v>
+        <v>4.31</v>
       </c>
       <c r="S24" t="n">
         <v>4.354</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.801</v>
+        <v>2.809</v>
       </c>
       <c r="G25" t="n">
-        <v>2.913</v>
+        <v>2.928</v>
       </c>
       <c r="H25" t="n">
-        <v>3.097</v>
+        <v>3.118</v>
       </c>
       <c r="I25" t="n">
-        <v>3.272</v>
+        <v>3.299</v>
       </c>
       <c r="J25" t="n">
-        <v>3.601</v>
+        <v>3.603</v>
       </c>
       <c r="K25" t="n">
-        <v>3.859</v>
+        <v>3.858</v>
       </c>
       <c r="L25" t="n">
-        <v>3.906</v>
+        <v>3.901</v>
       </c>
       <c r="M25" t="n">
         <v>4.051</v>
       </c>
       <c r="N25" t="n">
-        <v>4.14</v>
+        <v>4.139</v>
       </c>
       <c r="O25" t="n">
-        <v>4.221</v>
+        <v>4.234</v>
       </c>
       <c r="P25" t="n">
         <v>4.35</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.421</v>
+        <v>4.408</v>
       </c>
       <c r="R25" t="n">
-        <v>4.419</v>
+        <v>4.412</v>
       </c>
       <c r="S25" t="n">
         <v>4.462</v>
       </c>
       <c r="T25" t="n">
-        <v>4.407</v>
+        <v>4.405</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.071</v>
+        <v>3.083</v>
       </c>
       <c r="G26" t="n">
-        <v>3.23</v>
+        <v>3.249</v>
       </c>
       <c r="H26" t="n">
-        <v>3.524</v>
+        <v>3.548</v>
       </c>
       <c r="I26" t="n">
-        <v>3.747</v>
+        <v>3.772</v>
       </c>
       <c r="J26" t="n">
-        <v>4.238</v>
+        <v>4.237</v>
       </c>
       <c r="K26" t="n">
-        <v>4.674</v>
+        <v>4.673</v>
       </c>
       <c r="L26" t="n">
-        <v>4.79</v>
+        <v>4.785</v>
       </c>
       <c r="M26" t="n">
-        <v>4.989</v>
+        <v>4.986</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.292</v>
+        <v>5.306</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.883</v>
+        <v>2.896</v>
       </c>
       <c r="G27" t="n">
-        <v>2.992</v>
+        <v>3.01</v>
       </c>
       <c r="H27" t="n">
-        <v>3.195</v>
+        <v>3.217</v>
       </c>
       <c r="I27" t="n">
-        <v>3.386</v>
+        <v>3.411</v>
       </c>
       <c r="J27" t="n">
-        <v>3.744</v>
+        <v>3.745</v>
       </c>
       <c r="K27" t="n">
         <v>3.992</v>
       </c>
       <c r="L27" t="n">
-        <v>4.06</v>
+        <v>4.056</v>
       </c>
       <c r="M27" t="n">
-        <v>4.205</v>
+        <v>4.203</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.387</v>
+        <v>4.401</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.986</v>
+        <v>2.999</v>
       </c>
       <c r="G28" t="n">
-        <v>3.103</v>
+        <v>3.121</v>
       </c>
       <c r="H28" t="n">
-        <v>3.32</v>
+        <v>3.343</v>
       </c>
       <c r="I28" t="n">
-        <v>3.523</v>
+        <v>3.548</v>
       </c>
       <c r="J28" t="n">
-        <v>3.917</v>
+        <v>3.918</v>
       </c>
       <c r="K28" t="n">
         <v>4.184</v>
       </c>
       <c r="L28" t="n">
-        <v>4.263</v>
+        <v>4.259</v>
       </c>
       <c r="M28" t="n">
-        <v>4.417</v>
+        <v>4.415</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.679</v>
+        <v>4.693</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.832</v>
+        <v>2.846</v>
       </c>
       <c r="G29" t="n">
-        <v>2.943</v>
+        <v>2.961</v>
       </c>
       <c r="H29" t="n">
-        <v>3.135</v>
+        <v>3.158</v>
       </c>
       <c r="I29" t="n">
-        <v>3.315</v>
+        <v>3.341</v>
       </c>
       <c r="J29" t="n">
-        <v>3.656</v>
+        <v>3.658</v>
       </c>
       <c r="K29" t="n">
         <v>3.887</v>
       </c>
       <c r="L29" t="n">
-        <v>3.945</v>
+        <v>3.941</v>
       </c>
       <c r="M29" t="n">
-        <v>4.067</v>
+        <v>4.066</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.257</v>
+        <v>4.271</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.114</v>
+        <v>3.126</v>
       </c>
       <c r="G30" t="n">
-        <v>3.208</v>
+        <v>3.226</v>
       </c>
       <c r="H30" t="n">
-        <v>3.456</v>
+        <v>3.479</v>
       </c>
       <c r="I30" t="n">
-        <v>3.67</v>
+        <v>3.695</v>
       </c>
       <c r="J30" t="n">
-        <v>4.106</v>
+        <v>4.105</v>
       </c>
       <c r="K30" t="n">
-        <v>4.473</v>
+        <v>4.472</v>
       </c>
       <c r="L30" t="n">
-        <v>4.57</v>
+        <v>4.565</v>
       </c>
       <c r="M30" t="n">
-        <v>4.759</v>
+        <v>4.756</v>
       </c>
       <c r="N30" t="n">
-        <v>4.946</v>
+        <v>4.945</v>
       </c>
       <c r="O30" t="n">
-        <v>5.242</v>
+        <v>5.257</v>
       </c>
       <c r="P30" t="n">
-        <v>5.493</v>
+        <v>5.492</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.256</v>
+        <v>6.243</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.443</v>
+        <v>3.455</v>
       </c>
       <c r="G31" t="n">
-        <v>3.573</v>
+        <v>3.591</v>
       </c>
       <c r="H31" t="n">
-        <v>3.871</v>
+        <v>3.893</v>
       </c>
       <c r="I31" t="n">
-        <v>4.1</v>
+        <v>4.125</v>
       </c>
       <c r="J31" t="n">
-        <v>4.598</v>
+        <v>4.596</v>
       </c>
       <c r="K31" t="n">
         <v>5.005</v>
       </c>
       <c r="L31" t="n">
-        <v>5.183</v>
+        <v>5.178</v>
       </c>
       <c r="M31" t="n">
-        <v>5.489</v>
+        <v>5.487</v>
       </c>
       <c r="N31" t="n">
-        <v>5.805</v>
+        <v>5.804</v>
       </c>
       <c r="O31" t="n">
-        <v>6.278</v>
+        <v>6.293</v>
       </c>
       <c r="P31" t="n">
-        <v>6.482</v>
+        <v>6.48</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.229</v>
+        <v>7.217</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.213</v>
+        <v>3.225</v>
       </c>
       <c r="G32" t="n">
-        <v>3.326</v>
+        <v>3.344</v>
       </c>
       <c r="H32" t="n">
-        <v>3.6</v>
+        <v>3.623</v>
       </c>
       <c r="I32" t="n">
-        <v>3.829</v>
+        <v>3.854</v>
       </c>
       <c r="J32" t="n">
-        <v>4.284</v>
+        <v>4.283</v>
       </c>
       <c r="K32" t="n">
-        <v>4.658</v>
+        <v>4.657</v>
       </c>
       <c r="L32" t="n">
-        <v>4.774</v>
+        <v>4.769</v>
       </c>
       <c r="M32" t="n">
-        <v>5.031</v>
+        <v>5.029</v>
       </c>
       <c r="N32" t="n">
-        <v>5.307</v>
+        <v>5.305</v>
       </c>
       <c r="O32" t="n">
-        <v>5.688</v>
+        <v>5.703</v>
       </c>
       <c r="P32" t="n">
-        <v>5.953</v>
+        <v>5.952</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.717</v>
+        <v>6.704</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.978</v>
+        <v>2.99</v>
       </c>
       <c r="G33" t="n">
-        <v>3.072</v>
+        <v>3.09</v>
       </c>
       <c r="H33" t="n">
-        <v>3.274</v>
+        <v>3.298</v>
       </c>
       <c r="I33" t="n">
-        <v>3.454</v>
+        <v>3.479</v>
       </c>
       <c r="J33" t="n">
-        <v>3.813</v>
+        <v>3.812</v>
       </c>
       <c r="K33" t="n">
         <v>4.115</v>
       </c>
       <c r="L33" t="n">
-        <v>4.173</v>
+        <v>4.168</v>
       </c>
       <c r="M33" t="n">
-        <v>4.284</v>
+        <v>4.282</v>
       </c>
       <c r="N33" t="n">
-        <v>4.336</v>
+        <v>4.334</v>
       </c>
       <c r="O33" t="n">
-        <v>4.396</v>
+        <v>4.411</v>
       </c>
       <c r="P33" t="n">
-        <v>4.526</v>
+        <v>4.524</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.973</v>
+        <v>4.96</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.038</v>
+        <v>3.05</v>
       </c>
       <c r="G34" t="n">
-        <v>3.125</v>
+        <v>3.143</v>
       </c>
       <c r="H34" t="n">
-        <v>3.336</v>
+        <v>3.36</v>
       </c>
       <c r="I34" t="n">
-        <v>3.522</v>
+        <v>3.547</v>
       </c>
       <c r="J34" t="n">
-        <v>3.884</v>
+        <v>3.883</v>
       </c>
       <c r="K34" t="n">
         <v>4.192</v>
       </c>
       <c r="L34" t="n">
-        <v>4.252</v>
+        <v>4.247</v>
       </c>
       <c r="M34" t="n">
-        <v>4.375</v>
+        <v>4.372</v>
       </c>
       <c r="N34" t="n">
-        <v>4.44</v>
+        <v>4.438</v>
       </c>
       <c r="O34" t="n">
-        <v>4.565</v>
+        <v>4.58</v>
       </c>
       <c r="P34" t="n">
-        <v>4.82</v>
+        <v>4.818</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.674</v>
+        <v>5.661</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.012</v>
+        <v>3.024</v>
       </c>
       <c r="G35" t="n">
-        <v>3.099</v>
+        <v>3.117</v>
       </c>
       <c r="H35" t="n">
-        <v>3.304</v>
+        <v>3.328</v>
       </c>
       <c r="I35" t="n">
-        <v>3.489</v>
+        <v>3.514</v>
       </c>
       <c r="J35" t="n">
-        <v>3.853</v>
+        <v>3.851</v>
       </c>
       <c r="K35" t="n">
-        <v>4.145</v>
+        <v>4.146</v>
       </c>
       <c r="L35" t="n">
-        <v>4.207</v>
+        <v>4.202</v>
       </c>
       <c r="M35" t="n">
-        <v>4.321</v>
+        <v>4.319</v>
       </c>
       <c r="N35" t="n">
-        <v>4.376</v>
+        <v>4.375</v>
       </c>
       <c r="O35" t="n">
-        <v>4.462</v>
+        <v>4.477</v>
       </c>
       <c r="P35" t="n">
-        <v>4.623</v>
+        <v>4.621</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.31</v>
+        <v>5.297</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.908</v>
+        <v>2.92</v>
       </c>
       <c r="G36" t="n">
-        <v>2.995</v>
+        <v>3.012</v>
       </c>
       <c r="H36" t="n">
-        <v>3.189</v>
+        <v>3.211</v>
       </c>
       <c r="I36" t="n">
-        <v>3.373</v>
+        <v>3.398</v>
       </c>
       <c r="J36" t="n">
-        <v>3.748</v>
+        <v>3.746</v>
       </c>
       <c r="K36" t="n">
         <v>4.039</v>
       </c>
       <c r="L36" t="n">
-        <v>4.098</v>
+        <v>4.093</v>
       </c>
       <c r="M36" t="n">
-        <v>4.185</v>
+        <v>4.183</v>
       </c>
       <c r="N36" t="n">
-        <v>4.239</v>
+        <v>4.237</v>
       </c>
       <c r="O36" t="n">
-        <v>4.305</v>
+        <v>4.32</v>
       </c>
       <c r="P36" t="n">
-        <v>4.424</v>
+        <v>4.422</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.69</v>
+        <v>4.677</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.787</v>
+        <v>3.799</v>
       </c>
       <c r="G37" t="n">
-        <v>4.269</v>
+        <v>4.286</v>
       </c>
       <c r="H37" t="n">
-        <v>4.847</v>
+        <v>4.87</v>
       </c>
       <c r="I37" t="n">
-        <v>5.162</v>
+        <v>5.187</v>
       </c>
       <c r="J37" t="n">
-        <v>6.089</v>
+        <v>6.087</v>
       </c>
       <c r="K37" t="n">
-        <v>7.046</v>
+        <v>7.045</v>
       </c>
       <c r="L37" t="n">
-        <v>7.382</v>
+        <v>7.378</v>
       </c>
       <c r="M37" t="n">
-        <v>7.761</v>
+        <v>7.759</v>
       </c>
       <c r="N37" t="n">
-        <v>7.956</v>
+        <v>7.955</v>
       </c>
       <c r="O37" t="n">
-        <v>8.157</v>
+        <v>8.172000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.281000000000001</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.718</v>
+        <v>8.705</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.846</v>
+        <v>4.858</v>
       </c>
       <c r="G38" t="n">
-        <v>5.582</v>
+        <v>5.599</v>
       </c>
       <c r="H38" t="n">
-        <v>6.371</v>
+        <v>6.394</v>
       </c>
       <c r="I38" t="n">
-        <v>6.843</v>
+        <v>6.868</v>
       </c>
       <c r="J38" t="n">
-        <v>8.032</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="K38" t="n">
-        <v>9.167999999999999</v>
+        <v>9.167</v>
       </c>
       <c r="L38" t="n">
-        <v>9.664999999999999</v>
+        <v>9.66</v>
       </c>
       <c r="M38" t="n">
-        <v>10.173</v>
+        <v>10.171</v>
       </c>
       <c r="N38" t="n">
-        <v>10.375</v>
+        <v>10.374</v>
       </c>
       <c r="O38" t="n">
-        <v>10.558</v>
+        <v>10.573</v>
       </c>
       <c r="P38" t="n">
-        <v>10.679</v>
+        <v>10.677</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.169</v>
+        <v>11.156</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.167</v>
+        <v>4.179</v>
       </c>
       <c r="G39" t="n">
-        <v>4.78</v>
+        <v>4.797</v>
       </c>
       <c r="H39" t="n">
-        <v>5.436</v>
+        <v>5.459</v>
       </c>
       <c r="I39" t="n">
-        <v>5.846</v>
+        <v>5.872</v>
       </c>
       <c r="J39" t="n">
-        <v>6.904</v>
+        <v>6.903</v>
       </c>
       <c r="K39" t="n">
         <v>8</v>
       </c>
       <c r="L39" t="n">
-        <v>8.42</v>
+        <v>8.416</v>
       </c>
       <c r="M39" t="n">
-        <v>8.81</v>
+        <v>8.807</v>
       </c>
       <c r="N39" t="n">
-        <v>9.003</v>
+        <v>9.000999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.208</v>
+        <v>9.223000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>9.334</v>
+        <v>9.332000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.814</v>
+        <v>9.801</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.306</v>
+        <v>3.318</v>
       </c>
       <c r="G40" t="n">
-        <v>3.446</v>
+        <v>3.464</v>
       </c>
       <c r="H40" t="n">
-        <v>3.715</v>
+        <v>3.738</v>
       </c>
       <c r="I40" t="n">
-        <v>3.944</v>
+        <v>3.969</v>
       </c>
       <c r="J40" t="n">
-        <v>4.398</v>
+        <v>4.396</v>
       </c>
       <c r="K40" t="n">
-        <v>4.779</v>
+        <v>4.778</v>
       </c>
       <c r="L40" t="n">
-        <v>4.895</v>
+        <v>4.89</v>
       </c>
       <c r="M40" t="n">
-        <v>5.102</v>
+        <v>5.099</v>
       </c>
       <c r="N40" t="n">
-        <v>5.304</v>
+        <v>5.302</v>
       </c>
       <c r="O40" t="n">
-        <v>5.621</v>
+        <v>5.636</v>
       </c>
       <c r="P40" t="n">
-        <v>5.915</v>
+        <v>5.913</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.707</v>
+        <v>6.694</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.692</v>
+        <v>3.704</v>
       </c>
       <c r="G41" t="n">
-        <v>3.875</v>
+        <v>3.893</v>
       </c>
       <c r="H41" t="n">
-        <v>4.2</v>
+        <v>4.223</v>
       </c>
       <c r="I41" t="n">
-        <v>4.447</v>
+        <v>4.473</v>
       </c>
       <c r="J41" t="n">
-        <v>4.953</v>
+        <v>4.951</v>
       </c>
       <c r="K41" t="n">
         <v>5.379</v>
       </c>
       <c r="L41" t="n">
-        <v>5.573</v>
+        <v>5.568</v>
       </c>
       <c r="M41" t="n">
-        <v>5.904</v>
+        <v>5.902</v>
       </c>
       <c r="N41" t="n">
-        <v>6.235</v>
+        <v>6.233</v>
       </c>
       <c r="O41" t="n">
-        <v>6.737</v>
+        <v>6.752</v>
       </c>
       <c r="P41" t="n">
-        <v>6.974</v>
+        <v>6.972</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.754</v>
+        <v>7.741</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.427</v>
+        <v>3.439</v>
       </c>
       <c r="G42" t="n">
-        <v>3.595</v>
+        <v>3.613</v>
       </c>
       <c r="H42" t="n">
-        <v>3.891</v>
+        <v>3.914</v>
       </c>
       <c r="I42" t="n">
-        <v>4.132</v>
+        <v>4.157</v>
       </c>
       <c r="J42" t="n">
-        <v>4.6</v>
+        <v>4.599</v>
       </c>
       <c r="K42" t="n">
-        <v>5</v>
+        <v>4.999</v>
       </c>
       <c r="L42" t="n">
-        <v>5.131</v>
+        <v>5.126</v>
       </c>
       <c r="M42" t="n">
-        <v>5.409</v>
+        <v>5.406</v>
       </c>
       <c r="N42" t="n">
-        <v>5.718</v>
+        <v>5.717</v>
       </c>
       <c r="O42" t="n">
-        <v>6.113</v>
+        <v>6.128</v>
       </c>
       <c r="P42" t="n">
-        <v>6.417</v>
+        <v>6.415</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.22</v>
+        <v>7.207</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.126</v>
+        <v>3.138</v>
       </c>
       <c r="G43" t="n">
-        <v>3.255</v>
+        <v>3.273</v>
       </c>
       <c r="H43" t="n">
-        <v>3.475</v>
+        <v>3.499</v>
       </c>
       <c r="I43" t="n">
-        <v>3.663</v>
+        <v>3.688</v>
       </c>
       <c r="J43" t="n">
-        <v>4.04</v>
+        <v>4.039</v>
       </c>
       <c r="K43" t="n">
         <v>4.347</v>
       </c>
       <c r="L43" t="n">
-        <v>4.415</v>
+        <v>4.41</v>
       </c>
       <c r="M43" t="n">
-        <v>4.539</v>
+        <v>4.537</v>
       </c>
       <c r="N43" t="n">
-        <v>4.604</v>
+        <v>4.603</v>
       </c>
       <c r="O43" t="n">
-        <v>4.71</v>
+        <v>4.725</v>
       </c>
       <c r="P43" t="n">
-        <v>4.891</v>
+        <v>4.89</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.583</v>
+        <v>5.57</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.986</v>
+        <v>2.998</v>
       </c>
       <c r="G44" t="n">
-        <v>3.104</v>
+        <v>3.121</v>
       </c>
       <c r="H44" t="n">
-        <v>3.312</v>
+        <v>3.335</v>
       </c>
       <c r="I44" t="n">
-        <v>3.5</v>
+        <v>3.525</v>
       </c>
       <c r="J44" t="n">
-        <v>3.889</v>
+        <v>3.887</v>
       </c>
       <c r="K44" t="n">
         <v>4.191</v>
       </c>
       <c r="L44" t="n">
-        <v>4.258</v>
+        <v>4.254</v>
       </c>
       <c r="M44" t="n">
-        <v>4.356</v>
+        <v>4.353</v>
       </c>
       <c r="N44" t="n">
-        <v>4.421</v>
+        <v>4.419</v>
       </c>
       <c r="O44" t="n">
-        <v>4.505</v>
+        <v>4.52</v>
       </c>
       <c r="P44" t="n">
-        <v>4.654</v>
+        <v>4.652</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.954</v>
+        <v>4.941</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-22 ~ 2026-05-22
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.241</v>
+        <v>3.245</v>
       </c>
       <c r="G2" t="n">
-        <v>3.489</v>
+        <v>3.507</v>
       </c>
       <c r="H2" t="n">
-        <v>3.744</v>
+        <v>3.774</v>
       </c>
       <c r="I2" t="n">
-        <v>3.924</v>
+        <v>3.963</v>
       </c>
       <c r="J2" t="n">
-        <v>4.275</v>
+        <v>4.262</v>
       </c>
       <c r="K2" t="n">
-        <v>4.705</v>
+        <v>4.683</v>
       </c>
       <c r="L2" t="n">
-        <v>4.881</v>
+        <v>4.849</v>
       </c>
       <c r="M2" t="n">
-        <v>5.199</v>
+        <v>5.171</v>
       </c>
       <c r="N2" t="n">
-        <v>5.507</v>
+        <v>5.468</v>
       </c>
       <c r="O2" t="n">
-        <v>5.774</v>
+        <v>5.74</v>
       </c>
       <c r="P2" t="n">
-        <v>6.016</v>
+        <v>5.973</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.642</v>
+        <v>6.587</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.264</v>
+        <v>4.268</v>
       </c>
       <c r="G3" t="n">
-        <v>4.694</v>
+        <v>4.712</v>
       </c>
       <c r="H3" t="n">
-        <v>4.981</v>
+        <v>5.011</v>
       </c>
       <c r="I3" t="n">
-        <v>5.157</v>
+        <v>5.196</v>
       </c>
       <c r="J3" t="n">
-        <v>5.521</v>
+        <v>5.508</v>
       </c>
       <c r="K3" t="n">
-        <v>6.022</v>
+        <v>6</v>
       </c>
       <c r="L3" t="n">
-        <v>6.267</v>
+        <v>6.234</v>
       </c>
       <c r="M3" t="n">
-        <v>6.616</v>
+        <v>6.588</v>
       </c>
       <c r="N3" t="n">
-        <v>6.866</v>
+        <v>6.828</v>
       </c>
       <c r="O3" t="n">
-        <v>7.084</v>
+        <v>7.05</v>
       </c>
       <c r="P3" t="n">
-        <v>7.196</v>
+        <v>7.153</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.711</v>
+        <v>7.655</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.757</v>
+        <v>3.761</v>
       </c>
       <c r="G4" t="n">
-        <v>4.075</v>
+        <v>4.093</v>
       </c>
       <c r="H4" t="n">
-        <v>4.391</v>
+        <v>4.421</v>
       </c>
       <c r="I4" t="n">
-        <v>4.6</v>
+        <v>4.639</v>
       </c>
       <c r="J4" t="n">
-        <v>4.966</v>
+        <v>4.953</v>
       </c>
       <c r="K4" t="n">
-        <v>5.46</v>
+        <v>5.438</v>
       </c>
       <c r="L4" t="n">
-        <v>5.636</v>
+        <v>5.603</v>
       </c>
       <c r="M4" t="n">
-        <v>5.974</v>
+        <v>5.946</v>
       </c>
       <c r="N4" t="n">
-        <v>6.194</v>
+        <v>6.156</v>
       </c>
       <c r="O4" t="n">
-        <v>6.435</v>
+        <v>6.401</v>
       </c>
       <c r="P4" t="n">
-        <v>6.546</v>
+        <v>6.503</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.064</v>
+        <v>7.008</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.934</v>
+        <v>2.942</v>
       </c>
       <c r="G5" t="n">
-        <v>3.03</v>
+        <v>3.048</v>
       </c>
       <c r="H5" t="n">
-        <v>3.25</v>
+        <v>3.28</v>
       </c>
       <c r="I5" t="n">
-        <v>3.496</v>
+        <v>3.535</v>
       </c>
       <c r="J5" t="n">
-        <v>3.832</v>
+        <v>3.819</v>
       </c>
       <c r="K5" t="n">
-        <v>4.106</v>
+        <v>4.084</v>
       </c>
       <c r="L5" t="n">
-        <v>4.129</v>
+        <v>4.095</v>
       </c>
       <c r="M5" t="n">
-        <v>4.257</v>
+        <v>4.229</v>
       </c>
       <c r="N5" t="n">
-        <v>4.319</v>
+        <v>4.281</v>
       </c>
       <c r="O5" t="n">
-        <v>4.373</v>
+        <v>4.339</v>
       </c>
       <c r="P5" t="n">
-        <v>4.684</v>
+        <v>4.642</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.555</v>
+        <v>5.499</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.975</v>
+        <v>2.983</v>
       </c>
       <c r="G6" t="n">
-        <v>3.086</v>
+        <v>3.104</v>
       </c>
       <c r="H6" t="n">
-        <v>3.319</v>
+        <v>3.349</v>
       </c>
       <c r="I6" t="n">
-        <v>3.579</v>
+        <v>3.618</v>
       </c>
       <c r="J6" t="n">
-        <v>3.922</v>
+        <v>3.909</v>
       </c>
       <c r="K6" t="n">
-        <v>4.221</v>
+        <v>4.199</v>
       </c>
       <c r="L6" t="n">
-        <v>4.246</v>
+        <v>4.213</v>
       </c>
       <c r="M6" t="n">
-        <v>4.412</v>
+        <v>4.384</v>
       </c>
       <c r="N6" t="n">
-        <v>4.487</v>
+        <v>4.449</v>
       </c>
       <c r="O6" t="n">
-        <v>4.64</v>
+        <v>4.606</v>
       </c>
       <c r="P6" t="n">
-        <v>5.117</v>
+        <v>5.074</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.951</v>
+        <v>5.895</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.955</v>
+        <v>2.963</v>
       </c>
       <c r="G7" t="n">
-        <v>3.049</v>
+        <v>3.067</v>
       </c>
       <c r="H7" t="n">
-        <v>3.266</v>
+        <v>3.296</v>
       </c>
       <c r="I7" t="n">
-        <v>3.514</v>
+        <v>3.553</v>
       </c>
       <c r="J7" t="n">
-        <v>3.856</v>
+        <v>3.843</v>
       </c>
       <c r="K7" t="n">
-        <v>4.134</v>
+        <v>4.112</v>
       </c>
       <c r="L7" t="n">
-        <v>4.154</v>
+        <v>4.121</v>
       </c>
       <c r="M7" t="n">
-        <v>4.318</v>
+        <v>4.29</v>
       </c>
       <c r="N7" t="n">
-        <v>4.379</v>
+        <v>4.341</v>
       </c>
       <c r="O7" t="n">
-        <v>4.538</v>
+        <v>4.504</v>
       </c>
       <c r="P7" t="n">
-        <v>4.9</v>
+        <v>4.858</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.718</v>
+        <v>5.663</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.376</v>
+        <v>5.38</v>
       </c>
       <c r="G8" t="n">
-        <v>5.994</v>
+        <v>6.012</v>
       </c>
       <c r="H8" t="n">
-        <v>6.43</v>
+        <v>6.46</v>
       </c>
       <c r="I8" t="n">
-        <v>6.683</v>
+        <v>6.722</v>
       </c>
       <c r="J8" t="n">
-        <v>7.113</v>
+        <v>7.1</v>
       </c>
       <c r="K8" t="n">
-        <v>7.894</v>
+        <v>7.872</v>
       </c>
       <c r="L8" t="n">
-        <v>8.225</v>
+        <v>8.192</v>
       </c>
       <c r="M8" t="n">
-        <v>8.606</v>
+        <v>8.577999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.789999999999999</v>
+        <v>8.752000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.093</v>
+        <v>9.058999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>9.307</v>
+        <v>9.263999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.02</v>
+        <v>9.964</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.637</v>
+        <v>2.636</v>
       </c>
       <c r="G9" t="n">
-        <v>2.74</v>
+        <v>2.731</v>
       </c>
       <c r="H9" t="n">
-        <v>2.913</v>
+        <v>2.911</v>
       </c>
       <c r="I9" t="n">
-        <v>3.172</v>
+        <v>3.17</v>
       </c>
       <c r="J9" t="n">
-        <v>3.358</v>
+        <v>3.357</v>
       </c>
       <c r="K9" t="n">
-        <v>3.604</v>
+        <v>3.587</v>
       </c>
       <c r="L9" t="n">
-        <v>3.65</v>
+        <v>3.615</v>
       </c>
       <c r="M9" t="n">
-        <v>3.755</v>
+        <v>3.725</v>
       </c>
       <c r="N9" t="n">
-        <v>3.93</v>
+        <v>3.891</v>
       </c>
       <c r="O9" t="n">
-        <v>3.99</v>
+        <v>3.957</v>
       </c>
       <c r="P9" t="n">
-        <v>4.117</v>
+        <v>4.075</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.182</v>
+        <v>4.126</v>
       </c>
       <c r="R9" t="n">
-        <v>4.21</v>
+        <v>4.169</v>
       </c>
       <c r="S9" t="n">
-        <v>4.23</v>
+        <v>4.205</v>
       </c>
       <c r="T9" t="n">
-        <v>4.183</v>
+        <v>4.15</v>
       </c>
       <c r="U9" t="n">
-        <v>4.033</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.657</v>
+        <v>2.656</v>
       </c>
       <c r="G10" t="n">
-        <v>2.773</v>
+        <v>2.766</v>
       </c>
       <c r="H10" t="n">
-        <v>2.924</v>
+        <v>2.921</v>
       </c>
       <c r="I10" t="n">
-        <v>3.177</v>
+        <v>3.174</v>
       </c>
       <c r="J10" t="n">
-        <v>3.386</v>
+        <v>3.383</v>
       </c>
       <c r="K10" t="n">
-        <v>3.637</v>
+        <v>3.621</v>
       </c>
       <c r="L10" t="n">
-        <v>3.701</v>
+        <v>3.666</v>
       </c>
       <c r="M10" t="n">
-        <v>3.849</v>
+        <v>3.819</v>
       </c>
       <c r="N10" t="n">
-        <v>3.949</v>
+        <v>3.911</v>
       </c>
       <c r="O10" t="n">
-        <v>4.192</v>
+        <v>4.173</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.467</v>
+        <v>2.466</v>
       </c>
       <c r="G11" t="n">
-        <v>2.583</v>
+        <v>2.574</v>
       </c>
       <c r="H11" t="n">
-        <v>2.747</v>
+        <v>2.744</v>
       </c>
       <c r="I11" t="n">
-        <v>2.981</v>
+        <v>2.978</v>
       </c>
       <c r="J11" t="n">
-        <v>3.182</v>
+        <v>3.18</v>
       </c>
       <c r="K11" t="n">
-        <v>3.424</v>
+        <v>3.408</v>
       </c>
       <c r="L11" t="n">
-        <v>3.499</v>
+        <v>3.464</v>
       </c>
       <c r="M11" t="n">
-        <v>3.657</v>
+        <v>3.627</v>
       </c>
       <c r="N11" t="n">
-        <v>3.757</v>
+        <v>3.719</v>
       </c>
       <c r="O11" t="n">
-        <v>3.959</v>
+        <v>3.94</v>
       </c>
       <c r="P11" t="n">
-        <v>4.069</v>
+        <v>4.026</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.383</v>
+        <v>4.327</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.238</v>
+        <v>3.25</v>
       </c>
       <c r="G12" t="n">
-        <v>3.446</v>
+        <v>3.467</v>
       </c>
       <c r="H12" t="n">
-        <v>3.665</v>
+        <v>3.693</v>
       </c>
       <c r="I12" t="n">
-        <v>3.895</v>
+        <v>3.93</v>
       </c>
       <c r="J12" t="n">
-        <v>4.258</v>
+        <v>4.254</v>
       </c>
       <c r="K12" t="n">
-        <v>4.494</v>
+        <v>4.474</v>
       </c>
       <c r="L12" t="n">
-        <v>4.562</v>
+        <v>4.532</v>
       </c>
       <c r="M12" t="n">
-        <v>4.726</v>
+        <v>4.702</v>
       </c>
       <c r="N12" t="n">
-        <v>4.807</v>
+        <v>4.773</v>
       </c>
       <c r="O12" t="n">
-        <v>4.977</v>
+        <v>4.948</v>
       </c>
       <c r="P12" t="n">
-        <v>5.153</v>
+        <v>5.11</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.497</v>
+        <v>5.441</v>
       </c>
       <c r="R12" t="n">
-        <v>5.701</v>
+        <v>5.66</v>
       </c>
       <c r="S12" t="n">
-        <v>5.933</v>
+        <v>5.907</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.992</v>
+        <v>3.003</v>
       </c>
       <c r="G13" t="n">
-        <v>3.136</v>
+        <v>3.158</v>
       </c>
       <c r="H13" t="n">
-        <v>3.333</v>
+        <v>3.361</v>
       </c>
       <c r="I13" t="n">
-        <v>3.543</v>
+        <v>3.578</v>
       </c>
       <c r="J13" t="n">
-        <v>3.895</v>
+        <v>3.891</v>
       </c>
       <c r="K13" t="n">
-        <v>4.128</v>
+        <v>4.108</v>
       </c>
       <c r="L13" t="n">
-        <v>4.202</v>
+        <v>4.171</v>
       </c>
       <c r="M13" t="n">
-        <v>4.354</v>
+        <v>4.33</v>
       </c>
       <c r="N13" t="n">
-        <v>4.436</v>
+        <v>4.401</v>
       </c>
       <c r="O13" t="n">
-        <v>4.606</v>
+        <v>4.576</v>
       </c>
       <c r="P13" t="n">
-        <v>4.744</v>
+        <v>4.702</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.018</v>
+        <v>4.962</v>
       </c>
       <c r="R13" t="n">
-        <v>5.25</v>
+        <v>5.21</v>
       </c>
       <c r="S13" t="n">
-        <v>5.495</v>
+        <v>5.47</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.811</v>
+        <v>2.822</v>
       </c>
       <c r="G14" t="n">
-        <v>2.942</v>
+        <v>2.963</v>
       </c>
       <c r="H14" t="n">
-        <v>3.136</v>
+        <v>3.164</v>
       </c>
       <c r="I14" t="n">
-        <v>3.327</v>
+        <v>3.362</v>
       </c>
       <c r="J14" t="n">
-        <v>3.636</v>
+        <v>3.632</v>
       </c>
       <c r="K14" t="n">
-        <v>3.816</v>
+        <v>3.796</v>
       </c>
       <c r="L14" t="n">
-        <v>3.875</v>
+        <v>3.844</v>
       </c>
       <c r="M14" t="n">
-        <v>4.04</v>
+        <v>4.016</v>
       </c>
       <c r="N14" t="n">
-        <v>4.115</v>
+        <v>4.081</v>
       </c>
       <c r="O14" t="n">
-        <v>4.264</v>
+        <v>4.235</v>
       </c>
       <c r="P14" t="n">
-        <v>4.379</v>
+        <v>4.337</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.607</v>
+        <v>4.551</v>
       </c>
       <c r="R14" t="n">
-        <v>4.765</v>
+        <v>4.724</v>
       </c>
       <c r="S14" t="n">
-        <v>4.948</v>
+        <v>4.923</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.788</v>
+        <v>2.8</v>
       </c>
       <c r="G15" t="n">
-        <v>2.916</v>
+        <v>2.937</v>
       </c>
       <c r="H15" t="n">
-        <v>3.107</v>
+        <v>3.135</v>
       </c>
       <c r="I15" t="n">
-        <v>3.279</v>
+        <v>3.314</v>
       </c>
       <c r="J15" t="n">
-        <v>3.575</v>
+        <v>3.571</v>
       </c>
       <c r="K15" t="n">
-        <v>3.768</v>
+        <v>3.748</v>
       </c>
       <c r="L15" t="n">
-        <v>3.81</v>
+        <v>3.781</v>
       </c>
       <c r="M15" t="n">
-        <v>3.952</v>
+        <v>3.928</v>
       </c>
       <c r="N15" t="n">
-        <v>4.019</v>
+        <v>3.985</v>
       </c>
       <c r="O15" t="n">
-        <v>4.206</v>
+        <v>4.177</v>
       </c>
       <c r="P15" t="n">
-        <v>4.278</v>
+        <v>4.236</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.51</v>
+        <v>4.454</v>
       </c>
       <c r="R15" t="n">
-        <v>4.66</v>
+        <v>4.619</v>
       </c>
       <c r="S15" t="n">
-        <v>4.843</v>
+        <v>4.818</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.788</v>
+        <v>2.8</v>
       </c>
       <c r="G16" t="n">
-        <v>2.916</v>
+        <v>2.937</v>
       </c>
       <c r="H16" t="n">
-        <v>3.107</v>
+        <v>3.135</v>
       </c>
       <c r="I16" t="n">
-        <v>3.279</v>
+        <v>3.314</v>
       </c>
       <c r="J16" t="n">
-        <v>3.575</v>
+        <v>3.571</v>
       </c>
       <c r="K16" t="n">
-        <v>3.768</v>
+        <v>3.748</v>
       </c>
       <c r="L16" t="n">
-        <v>3.81</v>
+        <v>3.781</v>
       </c>
       <c r="M16" t="n">
-        <v>3.952</v>
+        <v>3.928</v>
       </c>
       <c r="N16" t="n">
-        <v>4.022</v>
+        <v>3.988</v>
       </c>
       <c r="O16" t="n">
-        <v>4.213</v>
+        <v>4.184</v>
       </c>
       <c r="P16" t="n">
-        <v>4.302</v>
+        <v>4.259</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.537</v>
+        <v>4.481</v>
       </c>
       <c r="R16" t="n">
-        <v>4.688</v>
+        <v>4.647</v>
       </c>
       <c r="S16" t="n">
-        <v>4.872</v>
+        <v>4.847</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.713</v>
+        <v>2.712</v>
       </c>
       <c r="G17" t="n">
-        <v>2.863</v>
+        <v>2.854</v>
       </c>
       <c r="H17" t="n">
-        <v>3.016</v>
+        <v>3.013</v>
       </c>
       <c r="I17" t="n">
-        <v>3.257</v>
+        <v>3.254</v>
       </c>
       <c r="J17" t="n">
-        <v>3.459</v>
+        <v>3.457</v>
       </c>
       <c r="K17" t="n">
-        <v>3.715</v>
+        <v>3.699</v>
       </c>
       <c r="L17" t="n">
-        <v>3.785</v>
+        <v>3.75</v>
       </c>
       <c r="M17" t="n">
-        <v>3.972</v>
+        <v>3.942</v>
       </c>
       <c r="N17" t="n">
-        <v>4.053</v>
+        <v>4.014</v>
       </c>
       <c r="O17" t="n">
-        <v>4.221</v>
+        <v>4.199</v>
       </c>
       <c r="P17" t="n">
-        <v>4.349</v>
+        <v>4.307</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.714</v>
+        <v>2.713</v>
       </c>
       <c r="G18" t="n">
-        <v>2.864</v>
+        <v>2.855</v>
       </c>
       <c r="H18" t="n">
-        <v>3.017</v>
+        <v>3.014</v>
       </c>
       <c r="I18" t="n">
-        <v>3.258</v>
+        <v>3.255</v>
       </c>
       <c r="J18" t="n">
-        <v>3.459</v>
+        <v>3.457</v>
       </c>
       <c r="K18" t="n">
-        <v>3.716</v>
+        <v>3.7</v>
       </c>
       <c r="L18" t="n">
-        <v>3.785</v>
+        <v>3.75</v>
       </c>
       <c r="M18" t="n">
-        <v>3.972</v>
+        <v>3.942</v>
       </c>
       <c r="N18" t="n">
-        <v>4.053</v>
+        <v>4.014</v>
       </c>
       <c r="O18" t="n">
-        <v>4.219</v>
+        <v>4.198</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.8</v>
+        <v>2.812</v>
       </c>
       <c r="G19" t="n">
-        <v>2.929</v>
+        <v>2.95</v>
       </c>
       <c r="H19" t="n">
-        <v>3.122</v>
+        <v>3.149</v>
       </c>
       <c r="I19" t="n">
-        <v>3.31</v>
+        <v>3.345</v>
       </c>
       <c r="J19" t="n">
-        <v>3.618</v>
+        <v>3.612</v>
       </c>
       <c r="K19" t="n">
-        <v>3.812</v>
+        <v>3.791</v>
       </c>
       <c r="L19" t="n">
-        <v>3.871</v>
+        <v>3.841</v>
       </c>
       <c r="M19" t="n">
-        <v>4.029</v>
+        <v>4.006</v>
       </c>
       <c r="N19" t="n">
-        <v>4.105</v>
+        <v>4.071</v>
       </c>
       <c r="O19" t="n">
-        <v>4.249</v>
+        <v>4.219</v>
       </c>
       <c r="P19" t="n">
-        <v>4.338</v>
+        <v>4.295</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.547</v>
+        <v>4.491</v>
       </c>
       <c r="R19" t="n">
-        <v>4.707</v>
+        <v>4.667</v>
       </c>
       <c r="S19" t="n">
-        <v>4.883</v>
+        <v>4.858</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.621</v>
+        <v>2.623</v>
       </c>
       <c r="G20" t="n">
-        <v>2.704</v>
+        <v>2.714</v>
       </c>
       <c r="H20" t="n">
-        <v>2.781</v>
+        <v>2.8</v>
       </c>
       <c r="I20" t="n">
-        <v>2.901</v>
+        <v>2.939</v>
       </c>
       <c r="J20" t="n">
-        <v>3.385</v>
+        <v>3.369</v>
       </c>
       <c r="K20" t="n">
-        <v>3.634</v>
+        <v>3.61</v>
       </c>
       <c r="L20" t="n">
-        <v>3.677</v>
+        <v>3.646</v>
       </c>
       <c r="M20" t="n">
-        <v>3.796</v>
+        <v>3.764</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.918</v>
+        <v>2.923</v>
       </c>
       <c r="G21" t="n">
-        <v>3.027</v>
+        <v>3.044</v>
       </c>
       <c r="H21" t="n">
-        <v>3.242</v>
+        <v>3.268</v>
       </c>
       <c r="I21" t="n">
-        <v>3.424</v>
+        <v>3.462</v>
       </c>
       <c r="J21" t="n">
-        <v>3.761</v>
+        <v>3.752</v>
       </c>
       <c r="K21" t="n">
-        <v>4.044</v>
+        <v>4.025</v>
       </c>
       <c r="L21" t="n">
-        <v>4.104</v>
+        <v>4.075</v>
       </c>
       <c r="M21" t="n">
-        <v>4.256</v>
+        <v>4.232</v>
       </c>
       <c r="N21" t="n">
-        <v>4.344</v>
+        <v>4.31</v>
       </c>
       <c r="O21" t="n">
-        <v>4.462</v>
+        <v>4.432</v>
       </c>
       <c r="P21" t="n">
-        <v>4.601</v>
+        <v>4.559</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.71</v>
+        <v>4.654</v>
       </c>
       <c r="R21" t="n">
-        <v>4.756</v>
+        <v>4.714</v>
       </c>
       <c r="S21" t="n">
-        <v>4.839</v>
+        <v>4.813</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.864</v>
+        <v>2.87</v>
       </c>
       <c r="G22" t="n">
-        <v>2.973</v>
+        <v>2.99</v>
       </c>
       <c r="H22" t="n">
-        <v>3.173</v>
+        <v>3.2</v>
       </c>
       <c r="I22" t="n">
-        <v>3.342</v>
+        <v>3.38</v>
       </c>
       <c r="J22" t="n">
-        <v>3.646</v>
+        <v>3.637</v>
       </c>
       <c r="K22" t="n">
-        <v>3.925</v>
+        <v>3.907</v>
       </c>
       <c r="L22" t="n">
-        <v>3.971</v>
+        <v>3.942</v>
       </c>
       <c r="M22" t="n">
-        <v>4.126</v>
+        <v>4.102</v>
       </c>
       <c r="N22" t="n">
-        <v>4.218</v>
+        <v>4.184</v>
       </c>
       <c r="O22" t="n">
-        <v>4.332</v>
+        <v>4.302</v>
       </c>
       <c r="P22" t="n">
-        <v>4.465</v>
+        <v>4.422</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.568</v>
+        <v>4.513</v>
       </c>
       <c r="R22" t="n">
-        <v>4.604</v>
+        <v>4.563</v>
       </c>
       <c r="S22" t="n">
-        <v>4.684</v>
+        <v>4.658</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.815</v>
+        <v>2.82</v>
       </c>
       <c r="G23" t="n">
-        <v>2.928</v>
+        <v>2.945</v>
       </c>
       <c r="H23" t="n">
-        <v>3.114</v>
+        <v>3.141</v>
       </c>
       <c r="I23" t="n">
-        <v>3.291</v>
+        <v>3.329</v>
       </c>
       <c r="J23" t="n">
-        <v>3.587</v>
+        <v>3.578</v>
       </c>
       <c r="K23" t="n">
-        <v>3.825</v>
+        <v>3.806</v>
       </c>
       <c r="L23" t="n">
-        <v>3.871</v>
+        <v>3.842</v>
       </c>
       <c r="M23" t="n">
-        <v>4.019</v>
+        <v>3.995</v>
       </c>
       <c r="N23" t="n">
-        <v>4.112</v>
+        <v>4.078</v>
       </c>
       <c r="O23" t="n">
-        <v>4.205</v>
+        <v>4.175</v>
       </c>
       <c r="P23" t="n">
-        <v>4.328</v>
+        <v>4.286</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.375</v>
+        <v>4.319</v>
       </c>
       <c r="R23" t="n">
-        <v>4.388</v>
+        <v>4.348</v>
       </c>
       <c r="S23" t="n">
-        <v>4.439</v>
+        <v>4.414</v>
       </c>
       <c r="T23" t="n">
-        <v>4.387</v>
+        <v>4.354</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.752</v>
+        <v>2.758</v>
       </c>
       <c r="G24" t="n">
-        <v>2.842</v>
+        <v>2.859</v>
       </c>
       <c r="H24" t="n">
-        <v>3.013</v>
+        <v>3.039</v>
       </c>
       <c r="I24" t="n">
-        <v>3.231</v>
+        <v>3.269</v>
       </c>
       <c r="J24" t="n">
-        <v>3.483</v>
+        <v>3.474</v>
       </c>
       <c r="K24" t="n">
-        <v>3.708</v>
+        <v>3.689</v>
       </c>
       <c r="L24" t="n">
-        <v>3.75</v>
+        <v>3.721</v>
       </c>
       <c r="M24" t="n">
-        <v>3.88</v>
+        <v>3.856</v>
       </c>
       <c r="N24" t="n">
-        <v>3.988</v>
+        <v>3.954</v>
       </c>
       <c r="O24" t="n">
-        <v>4.196</v>
+        <v>4.171</v>
       </c>
       <c r="P24" t="n">
-        <v>4.265</v>
+        <v>4.224</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.299</v>
+        <v>4.244</v>
       </c>
       <c r="R24" t="n">
-        <v>4.31</v>
+        <v>4.27</v>
       </c>
       <c r="S24" t="n">
-        <v>4.354</v>
+        <v>4.329</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.809</v>
+        <v>2.814</v>
       </c>
       <c r="G25" t="n">
-        <v>2.928</v>
+        <v>2.945</v>
       </c>
       <c r="H25" t="n">
-        <v>3.118</v>
+        <v>3.144</v>
       </c>
       <c r="I25" t="n">
-        <v>3.299</v>
+        <v>3.337</v>
       </c>
       <c r="J25" t="n">
-        <v>3.603</v>
+        <v>3.594</v>
       </c>
       <c r="K25" t="n">
-        <v>3.858</v>
+        <v>3.839</v>
       </c>
       <c r="L25" t="n">
-        <v>3.901</v>
+        <v>3.872</v>
       </c>
       <c r="M25" t="n">
-        <v>4.051</v>
+        <v>4.027</v>
       </c>
       <c r="N25" t="n">
-        <v>4.139</v>
+        <v>4.105</v>
       </c>
       <c r="O25" t="n">
-        <v>4.234</v>
+        <v>4.204</v>
       </c>
       <c r="P25" t="n">
-        <v>4.35</v>
+        <v>4.308</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.408</v>
+        <v>4.352</v>
       </c>
       <c r="R25" t="n">
-        <v>4.412</v>
+        <v>4.371</v>
       </c>
       <c r="S25" t="n">
-        <v>4.462</v>
+        <v>4.437</v>
       </c>
       <c r="T25" t="n">
-        <v>4.405</v>
+        <v>4.372</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.083</v>
+        <v>3.087</v>
       </c>
       <c r="G26" t="n">
-        <v>3.249</v>
+        <v>3.262</v>
       </c>
       <c r="H26" t="n">
-        <v>3.548</v>
+        <v>3.575</v>
       </c>
       <c r="I26" t="n">
-        <v>3.772</v>
+        <v>3.811</v>
       </c>
       <c r="J26" t="n">
-        <v>4.237</v>
+        <v>4.223</v>
       </c>
       <c r="K26" t="n">
-        <v>4.673</v>
+        <v>4.65</v>
       </c>
       <c r="L26" t="n">
-        <v>4.785</v>
+        <v>4.752</v>
       </c>
       <c r="M26" t="n">
-        <v>4.986</v>
+        <v>4.956</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.306</v>
+        <v>5.274</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.896</v>
+        <v>2.904</v>
       </c>
       <c r="G27" t="n">
-        <v>3.01</v>
+        <v>3.028</v>
       </c>
       <c r="H27" t="n">
-        <v>3.217</v>
+        <v>3.245</v>
       </c>
       <c r="I27" t="n">
-        <v>3.411</v>
+        <v>3.448</v>
       </c>
       <c r="J27" t="n">
-        <v>3.745</v>
+        <v>3.736</v>
       </c>
       <c r="K27" t="n">
-        <v>3.992</v>
+        <v>3.97</v>
       </c>
       <c r="L27" t="n">
-        <v>4.056</v>
+        <v>4.024</v>
       </c>
       <c r="M27" t="n">
-        <v>4.203</v>
+        <v>4.176</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.401</v>
+        <v>4.369</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.999</v>
+        <v>3.007</v>
       </c>
       <c r="G28" t="n">
-        <v>3.121</v>
+        <v>3.139</v>
       </c>
       <c r="H28" t="n">
-        <v>3.343</v>
+        <v>3.371</v>
       </c>
       <c r="I28" t="n">
-        <v>3.548</v>
+        <v>3.585</v>
       </c>
       <c r="J28" t="n">
-        <v>3.918</v>
+        <v>3.909</v>
       </c>
       <c r="K28" t="n">
-        <v>4.184</v>
+        <v>4.162</v>
       </c>
       <c r="L28" t="n">
-        <v>4.259</v>
+        <v>4.227</v>
       </c>
       <c r="M28" t="n">
-        <v>4.415</v>
+        <v>4.388</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.693</v>
+        <v>4.661</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.846</v>
+        <v>2.854</v>
       </c>
       <c r="G29" t="n">
-        <v>2.961</v>
+        <v>2.978</v>
       </c>
       <c r="H29" t="n">
-        <v>3.158</v>
+        <v>3.186</v>
       </c>
       <c r="I29" t="n">
-        <v>3.341</v>
+        <v>3.378</v>
       </c>
       <c r="J29" t="n">
-        <v>3.658</v>
+        <v>3.648</v>
       </c>
       <c r="K29" t="n">
-        <v>3.887</v>
+        <v>3.865</v>
       </c>
       <c r="L29" t="n">
-        <v>3.941</v>
+        <v>3.91</v>
       </c>
       <c r="M29" t="n">
-        <v>4.066</v>
+        <v>4.038</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.271</v>
+        <v>4.24</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.126</v>
+        <v>3.129</v>
       </c>
       <c r="G30" t="n">
-        <v>3.226</v>
+        <v>3.238</v>
       </c>
       <c r="H30" t="n">
-        <v>3.479</v>
+        <v>3.505</v>
       </c>
       <c r="I30" t="n">
-        <v>3.695</v>
+        <v>3.733</v>
       </c>
       <c r="J30" t="n">
-        <v>4.105</v>
+        <v>4.089</v>
       </c>
       <c r="K30" t="n">
-        <v>4.472</v>
+        <v>4.447</v>
       </c>
       <c r="L30" t="n">
-        <v>4.565</v>
+        <v>4.531</v>
       </c>
       <c r="M30" t="n">
-        <v>4.756</v>
+        <v>4.726</v>
       </c>
       <c r="N30" t="n">
-        <v>4.945</v>
+        <v>4.906</v>
       </c>
       <c r="O30" t="n">
-        <v>5.257</v>
+        <v>5.225</v>
       </c>
       <c r="P30" t="n">
-        <v>5.492</v>
+        <v>5.449</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.243</v>
+        <v>6.187</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.455</v>
+        <v>3.458</v>
       </c>
       <c r="G31" t="n">
-        <v>3.591</v>
+        <v>3.603</v>
       </c>
       <c r="H31" t="n">
-        <v>3.893</v>
+        <v>3.92</v>
       </c>
       <c r="I31" t="n">
-        <v>4.125</v>
+        <v>4.163</v>
       </c>
       <c r="J31" t="n">
-        <v>4.596</v>
+        <v>4.58</v>
       </c>
       <c r="K31" t="n">
-        <v>5.005</v>
+        <v>4.98</v>
       </c>
       <c r="L31" t="n">
-        <v>5.178</v>
+        <v>5.143</v>
       </c>
       <c r="M31" t="n">
-        <v>5.487</v>
+        <v>5.456</v>
       </c>
       <c r="N31" t="n">
-        <v>5.804</v>
+        <v>5.765</v>
       </c>
       <c r="O31" t="n">
-        <v>6.293</v>
+        <v>6.261</v>
       </c>
       <c r="P31" t="n">
-        <v>6.48</v>
+        <v>6.438</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.217</v>
+        <v>7.161</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.225</v>
+        <v>3.228</v>
       </c>
       <c r="G32" t="n">
-        <v>3.344</v>
+        <v>3.356</v>
       </c>
       <c r="H32" t="n">
-        <v>3.623</v>
+        <v>3.649</v>
       </c>
       <c r="I32" t="n">
-        <v>3.854</v>
+        <v>3.892</v>
       </c>
       <c r="J32" t="n">
-        <v>4.283</v>
+        <v>4.267</v>
       </c>
       <c r="K32" t="n">
-        <v>4.657</v>
+        <v>4.632</v>
       </c>
       <c r="L32" t="n">
-        <v>4.769</v>
+        <v>4.735</v>
       </c>
       <c r="M32" t="n">
-        <v>5.029</v>
+        <v>4.998</v>
       </c>
       <c r="N32" t="n">
-        <v>5.305</v>
+        <v>5.266</v>
       </c>
       <c r="O32" t="n">
-        <v>5.703</v>
+        <v>5.67</v>
       </c>
       <c r="P32" t="n">
-        <v>5.952</v>
+        <v>5.909</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.704</v>
+        <v>6.648</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.99</v>
+        <v>2.993</v>
       </c>
       <c r="G33" t="n">
-        <v>3.09</v>
+        <v>3.102</v>
       </c>
       <c r="H33" t="n">
-        <v>3.298</v>
+        <v>3.324</v>
       </c>
       <c r="I33" t="n">
-        <v>3.479</v>
+        <v>3.516</v>
       </c>
       <c r="J33" t="n">
-        <v>3.812</v>
+        <v>3.796</v>
       </c>
       <c r="K33" t="n">
-        <v>4.115</v>
+        <v>4.089</v>
       </c>
       <c r="L33" t="n">
-        <v>4.168</v>
+        <v>4.133</v>
       </c>
       <c r="M33" t="n">
-        <v>4.282</v>
+        <v>4.251</v>
       </c>
       <c r="N33" t="n">
-        <v>4.334</v>
+        <v>4.295</v>
       </c>
       <c r="O33" t="n">
-        <v>4.411</v>
+        <v>4.379</v>
       </c>
       <c r="P33" t="n">
-        <v>4.524</v>
+        <v>4.482</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.96</v>
+        <v>4.904</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.05</v>
+        <v>3.053</v>
       </c>
       <c r="G34" t="n">
-        <v>3.143</v>
+        <v>3.155</v>
       </c>
       <c r="H34" t="n">
-        <v>3.36</v>
+        <v>3.386</v>
       </c>
       <c r="I34" t="n">
-        <v>3.547</v>
+        <v>3.584</v>
       </c>
       <c r="J34" t="n">
-        <v>3.883</v>
+        <v>3.867</v>
       </c>
       <c r="K34" t="n">
-        <v>4.192</v>
+        <v>4.166</v>
       </c>
       <c r="L34" t="n">
-        <v>4.247</v>
+        <v>4.212</v>
       </c>
       <c r="M34" t="n">
-        <v>4.372</v>
+        <v>4.342</v>
       </c>
       <c r="N34" t="n">
-        <v>4.438</v>
+        <v>4.399</v>
       </c>
       <c r="O34" t="n">
-        <v>4.58</v>
+        <v>4.548</v>
       </c>
       <c r="P34" t="n">
-        <v>4.818</v>
+        <v>4.776</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.661</v>
+        <v>5.605</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.024</v>
+        <v>3.027</v>
       </c>
       <c r="G35" t="n">
-        <v>3.117</v>
+        <v>3.129</v>
       </c>
       <c r="H35" t="n">
-        <v>3.328</v>
+        <v>3.354</v>
       </c>
       <c r="I35" t="n">
-        <v>3.514</v>
+        <v>3.551</v>
       </c>
       <c r="J35" t="n">
-        <v>3.851</v>
+        <v>3.836</v>
       </c>
       <c r="K35" t="n">
-        <v>4.146</v>
+        <v>4.12</v>
       </c>
       <c r="L35" t="n">
-        <v>4.202</v>
+        <v>4.167</v>
       </c>
       <c r="M35" t="n">
-        <v>4.319</v>
+        <v>4.288</v>
       </c>
       <c r="N35" t="n">
-        <v>4.375</v>
+        <v>4.336</v>
       </c>
       <c r="O35" t="n">
-        <v>4.477</v>
+        <v>4.445</v>
       </c>
       <c r="P35" t="n">
-        <v>4.621</v>
+        <v>4.579</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.297</v>
+        <v>5.241</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.92</v>
+        <v>2.923</v>
       </c>
       <c r="G36" t="n">
-        <v>3.012</v>
+        <v>3.024</v>
       </c>
       <c r="H36" t="n">
-        <v>3.211</v>
+        <v>3.238</v>
       </c>
       <c r="I36" t="n">
-        <v>3.398</v>
+        <v>3.435</v>
       </c>
       <c r="J36" t="n">
-        <v>3.746</v>
+        <v>3.731</v>
       </c>
       <c r="K36" t="n">
-        <v>4.039</v>
+        <v>4.015</v>
       </c>
       <c r="L36" t="n">
-        <v>4.093</v>
+        <v>4.059</v>
       </c>
       <c r="M36" t="n">
-        <v>4.183</v>
+        <v>4.152</v>
       </c>
       <c r="N36" t="n">
-        <v>4.237</v>
+        <v>4.198</v>
       </c>
       <c r="O36" t="n">
-        <v>4.32</v>
+        <v>4.287</v>
       </c>
       <c r="P36" t="n">
-        <v>4.422</v>
+        <v>4.38</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.677</v>
+        <v>4.621</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.799</v>
+        <v>3.802</v>
       </c>
       <c r="G37" t="n">
-        <v>4.286</v>
+        <v>4.298</v>
       </c>
       <c r="H37" t="n">
-        <v>4.87</v>
+        <v>4.896</v>
       </c>
       <c r="I37" t="n">
-        <v>5.187</v>
+        <v>5.225</v>
       </c>
       <c r="J37" t="n">
-        <v>6.087</v>
+        <v>6.071</v>
       </c>
       <c r="K37" t="n">
-        <v>7.045</v>
+        <v>7.021</v>
       </c>
       <c r="L37" t="n">
-        <v>7.378</v>
+        <v>7.343</v>
       </c>
       <c r="M37" t="n">
-        <v>7.759</v>
+        <v>7.728</v>
       </c>
       <c r="N37" t="n">
-        <v>7.955</v>
+        <v>7.916</v>
       </c>
       <c r="O37" t="n">
-        <v>8.172000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.279999999999999</v>
+        <v>8.237</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.705</v>
+        <v>8.648999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.858</v>
+        <v>4.861</v>
       </c>
       <c r="G38" t="n">
-        <v>5.599</v>
+        <v>5.611</v>
       </c>
       <c r="H38" t="n">
-        <v>6.394</v>
+        <v>6.42</v>
       </c>
       <c r="I38" t="n">
-        <v>6.868</v>
+        <v>6.906</v>
       </c>
       <c r="J38" t="n">
-        <v>8.029999999999999</v>
+        <v>8.013999999999999</v>
       </c>
       <c r="K38" t="n">
-        <v>9.167</v>
+        <v>9.141999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.66</v>
+        <v>9.625999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.171</v>
+        <v>10.14</v>
       </c>
       <c r="N38" t="n">
-        <v>10.374</v>
+        <v>10.334</v>
       </c>
       <c r="O38" t="n">
-        <v>10.573</v>
+        <v>10.54</v>
       </c>
       <c r="P38" t="n">
-        <v>10.677</v>
+        <v>10.635</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.156</v>
+        <v>11.1</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.179</v>
+        <v>4.182</v>
       </c>
       <c r="G39" t="n">
-        <v>4.797</v>
+        <v>4.809</v>
       </c>
       <c r="H39" t="n">
-        <v>5.459</v>
+        <v>5.485</v>
       </c>
       <c r="I39" t="n">
-        <v>5.872</v>
+        <v>5.909</v>
       </c>
       <c r="J39" t="n">
-        <v>6.903</v>
+        <v>6.887</v>
       </c>
       <c r="K39" t="n">
-        <v>8</v>
+        <v>7.975</v>
       </c>
       <c r="L39" t="n">
-        <v>8.416</v>
+        <v>8.381</v>
       </c>
       <c r="M39" t="n">
-        <v>8.807</v>
+        <v>8.776999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>9.000999999999999</v>
+        <v>8.962</v>
       </c>
       <c r="O39" t="n">
-        <v>9.223000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="P39" t="n">
-        <v>9.332000000000001</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.801</v>
+        <v>9.744999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.318</v>
+        <v>3.321</v>
       </c>
       <c r="G40" t="n">
-        <v>3.464</v>
+        <v>3.476</v>
       </c>
       <c r="H40" t="n">
-        <v>3.738</v>
+        <v>3.764</v>
       </c>
       <c r="I40" t="n">
-        <v>3.969</v>
+        <v>4.007</v>
       </c>
       <c r="J40" t="n">
-        <v>4.396</v>
+        <v>4.38</v>
       </c>
       <c r="K40" t="n">
-        <v>4.778</v>
+        <v>4.753</v>
       </c>
       <c r="L40" t="n">
-        <v>4.89</v>
+        <v>4.855</v>
       </c>
       <c r="M40" t="n">
-        <v>5.099</v>
+        <v>5.068</v>
       </c>
       <c r="N40" t="n">
-        <v>5.302</v>
+        <v>5.263</v>
       </c>
       <c r="O40" t="n">
-        <v>5.636</v>
+        <v>5.604</v>
       </c>
       <c r="P40" t="n">
-        <v>5.913</v>
+        <v>5.871</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.694</v>
+        <v>6.639</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.704</v>
+        <v>3.707</v>
       </c>
       <c r="G41" t="n">
-        <v>3.893</v>
+        <v>3.905</v>
       </c>
       <c r="H41" t="n">
-        <v>4.223</v>
+        <v>4.249</v>
       </c>
       <c r="I41" t="n">
-        <v>4.473</v>
+        <v>4.511</v>
       </c>
       <c r="J41" t="n">
-        <v>4.951</v>
+        <v>4.935</v>
       </c>
       <c r="K41" t="n">
-        <v>5.379</v>
+        <v>5.354</v>
       </c>
       <c r="L41" t="n">
-        <v>5.568</v>
+        <v>5.534</v>
       </c>
       <c r="M41" t="n">
-        <v>5.902</v>
+        <v>5.871</v>
       </c>
       <c r="N41" t="n">
-        <v>6.233</v>
+        <v>6.194</v>
       </c>
       <c r="O41" t="n">
-        <v>6.752</v>
+        <v>6.719</v>
       </c>
       <c r="P41" t="n">
-        <v>6.972</v>
+        <v>6.93</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.741</v>
+        <v>7.686</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.439</v>
+        <v>3.442</v>
       </c>
       <c r="G42" t="n">
-        <v>3.613</v>
+        <v>3.625</v>
       </c>
       <c r="H42" t="n">
-        <v>3.914</v>
+        <v>3.94</v>
       </c>
       <c r="I42" t="n">
-        <v>4.157</v>
+        <v>4.195</v>
       </c>
       <c r="J42" t="n">
-        <v>4.599</v>
+        <v>4.583</v>
       </c>
       <c r="K42" t="n">
-        <v>4.999</v>
+        <v>4.974</v>
       </c>
       <c r="L42" t="n">
-        <v>5.126</v>
+        <v>5.092</v>
       </c>
       <c r="M42" t="n">
-        <v>5.406</v>
+        <v>5.375</v>
       </c>
       <c r="N42" t="n">
-        <v>5.717</v>
+        <v>5.678</v>
       </c>
       <c r="O42" t="n">
-        <v>6.128</v>
+        <v>6.096</v>
       </c>
       <c r="P42" t="n">
-        <v>6.415</v>
+        <v>6.373</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.207</v>
+        <v>7.151</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.138</v>
+        <v>3.141</v>
       </c>
       <c r="G43" t="n">
-        <v>3.273</v>
+        <v>3.285</v>
       </c>
       <c r="H43" t="n">
-        <v>3.499</v>
+        <v>3.525</v>
       </c>
       <c r="I43" t="n">
-        <v>3.688</v>
+        <v>3.725</v>
       </c>
       <c r="J43" t="n">
-        <v>4.039</v>
+        <v>4.023</v>
       </c>
       <c r="K43" t="n">
-        <v>4.347</v>
+        <v>4.321</v>
       </c>
       <c r="L43" t="n">
-        <v>4.41</v>
+        <v>4.374</v>
       </c>
       <c r="M43" t="n">
-        <v>4.537</v>
+        <v>4.506</v>
       </c>
       <c r="N43" t="n">
-        <v>4.603</v>
+        <v>4.564</v>
       </c>
       <c r="O43" t="n">
-        <v>4.725</v>
+        <v>4.692</v>
       </c>
       <c r="P43" t="n">
-        <v>4.89</v>
+        <v>4.847</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.57</v>
+        <v>5.514</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.998</v>
+        <v>3.001</v>
       </c>
       <c r="G44" t="n">
-        <v>3.121</v>
+        <v>3.133</v>
       </c>
       <c r="H44" t="n">
-        <v>3.335</v>
+        <v>3.361</v>
       </c>
       <c r="I44" t="n">
-        <v>3.525</v>
+        <v>3.562</v>
       </c>
       <c r="J44" t="n">
-        <v>3.887</v>
+        <v>3.872</v>
       </c>
       <c r="K44" t="n">
-        <v>4.191</v>
+        <v>4.167</v>
       </c>
       <c r="L44" t="n">
-        <v>4.254</v>
+        <v>4.22</v>
       </c>
       <c r="M44" t="n">
-        <v>4.353</v>
+        <v>4.322</v>
       </c>
       <c r="N44" t="n">
-        <v>4.419</v>
+        <v>4.38</v>
       </c>
       <c r="O44" t="n">
-        <v>4.52</v>
+        <v>4.488</v>
       </c>
       <c r="P44" t="n">
-        <v>4.652</v>
+        <v>4.61</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.941</v>
+        <v>4.885</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-27 ~ 2026-05-27
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.254</v>
+        <v>3.262</v>
       </c>
       <c r="G2" t="n">
-        <v>3.517</v>
+        <v>3.529</v>
       </c>
       <c r="H2" t="n">
-        <v>3.79</v>
+        <v>3.809</v>
       </c>
       <c r="I2" t="n">
-        <v>3.982</v>
+        <v>4.018</v>
       </c>
       <c r="J2" t="n">
-        <v>4.243</v>
+        <v>4.265</v>
       </c>
       <c r="K2" t="n">
-        <v>4.638</v>
+        <v>4.68</v>
       </c>
       <c r="L2" t="n">
-        <v>4.802</v>
+        <v>4.851</v>
       </c>
       <c r="M2" t="n">
-        <v>5.118</v>
+        <v>5.168</v>
       </c>
       <c r="N2" t="n">
-        <v>5.404</v>
+        <v>5.458</v>
       </c>
       <c r="O2" t="n">
-        <v>5.685</v>
+        <v>5.74</v>
       </c>
       <c r="P2" t="n">
-        <v>5.923</v>
+        <v>5.966</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.535</v>
+        <v>6.567</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.277</v>
+        <v>4.283</v>
       </c>
       <c r="G3" t="n">
-        <v>4.722</v>
+        <v>4.732</v>
       </c>
       <c r="H3" t="n">
-        <v>5.028</v>
+        <v>5.044</v>
       </c>
       <c r="I3" t="n">
-        <v>5.215</v>
+        <v>5.247</v>
       </c>
       <c r="J3" t="n">
-        <v>5.488</v>
+        <v>5.51</v>
       </c>
       <c r="K3" t="n">
-        <v>5.954</v>
+        <v>5.996</v>
       </c>
       <c r="L3" t="n">
-        <v>6.188</v>
+        <v>6.237</v>
       </c>
       <c r="M3" t="n">
-        <v>6.535</v>
+        <v>6.584</v>
       </c>
       <c r="N3" t="n">
-        <v>6.764</v>
+        <v>6.818</v>
       </c>
       <c r="O3" t="n">
-        <v>6.995</v>
+        <v>7.05</v>
       </c>
       <c r="P3" t="n">
-        <v>7.103</v>
+        <v>7.147</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.604</v>
+        <v>7.636</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.77</v>
+        <v>3.776</v>
       </c>
       <c r="G4" t="n">
-        <v>4.103</v>
+        <v>4.113</v>
       </c>
       <c r="H4" t="n">
-        <v>4.438</v>
+        <v>4.454</v>
       </c>
       <c r="I4" t="n">
-        <v>4.657</v>
+        <v>4.689</v>
       </c>
       <c r="J4" t="n">
-        <v>4.934</v>
+        <v>4.956</v>
       </c>
       <c r="K4" t="n">
-        <v>5.393</v>
+        <v>5.435</v>
       </c>
       <c r="L4" t="n">
-        <v>5.557</v>
+        <v>5.606</v>
       </c>
       <c r="M4" t="n">
-        <v>5.893</v>
+        <v>5.942</v>
       </c>
       <c r="N4" t="n">
-        <v>6.092</v>
+        <v>6.146</v>
       </c>
       <c r="O4" t="n">
-        <v>6.346</v>
+        <v>6.401</v>
       </c>
       <c r="P4" t="n">
-        <v>6.453</v>
+        <v>6.497</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.956</v>
+        <v>6.989</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.951</v>
+        <v>2.959</v>
       </c>
       <c r="G5" t="n">
-        <v>3.058</v>
+        <v>3.07</v>
       </c>
       <c r="H5" t="n">
-        <v>3.297</v>
+        <v>3.315</v>
       </c>
       <c r="I5" t="n">
-        <v>3.554</v>
+        <v>3.59</v>
       </c>
       <c r="J5" t="n">
-        <v>3.797</v>
+        <v>3.821</v>
       </c>
       <c r="K5" t="n">
-        <v>4.038</v>
+        <v>4.081</v>
       </c>
       <c r="L5" t="n">
-        <v>4.049</v>
+        <v>4.098</v>
       </c>
       <c r="M5" t="n">
-        <v>4.175</v>
+        <v>4.226</v>
       </c>
       <c r="N5" t="n">
-        <v>4.217</v>
+        <v>4.271</v>
       </c>
       <c r="O5" t="n">
-        <v>4.284</v>
+        <v>4.339</v>
       </c>
       <c r="P5" t="n">
-        <v>4.592</v>
+        <v>4.635</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.448</v>
+        <v>5.479</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.992</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>3.114</v>
+        <v>3.126</v>
       </c>
       <c r="H6" t="n">
-        <v>3.366</v>
+        <v>3.384</v>
       </c>
       <c r="I6" t="n">
-        <v>3.637</v>
+        <v>3.673</v>
       </c>
       <c r="J6" t="n">
-        <v>3.89</v>
+        <v>3.913</v>
       </c>
       <c r="K6" t="n">
-        <v>4.154</v>
+        <v>4.197</v>
       </c>
       <c r="L6" t="n">
-        <v>4.168</v>
+        <v>4.217</v>
       </c>
       <c r="M6" t="n">
-        <v>4.332</v>
+        <v>4.383</v>
       </c>
       <c r="N6" t="n">
-        <v>4.385</v>
+        <v>4.438</v>
       </c>
       <c r="O6" t="n">
-        <v>4.551</v>
+        <v>4.606</v>
       </c>
       <c r="P6" t="n">
-        <v>5.024</v>
+        <v>5.067</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.843</v>
+        <v>5.876</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.972</v>
+        <v>2.98</v>
       </c>
       <c r="G7" t="n">
-        <v>3.077</v>
+        <v>3.089</v>
       </c>
       <c r="H7" t="n">
-        <v>3.313</v>
+        <v>3.331</v>
       </c>
       <c r="I7" t="n">
-        <v>3.572</v>
+        <v>3.608</v>
       </c>
       <c r="J7" t="n">
-        <v>3.821</v>
+        <v>3.844</v>
       </c>
       <c r="K7" t="n">
-        <v>4.066</v>
+        <v>4.108</v>
       </c>
       <c r="L7" t="n">
-        <v>4.074</v>
+        <v>4.124</v>
       </c>
       <c r="M7" t="n">
-        <v>4.236</v>
+        <v>4.286</v>
       </c>
       <c r="N7" t="n">
-        <v>4.277</v>
+        <v>4.33</v>
       </c>
       <c r="O7" t="n">
-        <v>4.449</v>
+        <v>4.504</v>
       </c>
       <c r="P7" t="n">
-        <v>4.808</v>
+        <v>4.851</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.611</v>
+        <v>5.643</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.389</v>
+        <v>5.395</v>
       </c>
       <c r="G8" t="n">
-        <v>6.022</v>
+        <v>6.032</v>
       </c>
       <c r="H8" t="n">
-        <v>6.477</v>
+        <v>6.493</v>
       </c>
       <c r="I8" t="n">
-        <v>6.741</v>
+        <v>6.773</v>
       </c>
       <c r="J8" t="n">
-        <v>7.08</v>
+        <v>7.103</v>
       </c>
       <c r="K8" t="n">
-        <v>7.827</v>
+        <v>7.87</v>
       </c>
       <c r="L8" t="n">
-        <v>8.146000000000001</v>
+        <v>8.195</v>
       </c>
       <c r="M8" t="n">
-        <v>8.523999999999999</v>
+        <v>8.574999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.688000000000001</v>
+        <v>8.742000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.004</v>
+        <v>9.058999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>9.214</v>
+        <v>9.257999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.913</v>
+        <v>9.945</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1072,48 +1072,48 @@
         <v>2.914</v>
       </c>
       <c r="I9" t="n">
-        <v>3.152</v>
+        <v>3.157</v>
       </c>
       <c r="J9" t="n">
-        <v>3.345</v>
+        <v>3.36</v>
       </c>
       <c r="K9" t="n">
-        <v>3.527</v>
+        <v>3.565</v>
       </c>
       <c r="L9" t="n">
-        <v>3.56</v>
+        <v>3.612</v>
       </c>
       <c r="M9" t="n">
-        <v>3.664</v>
+        <v>3.717</v>
       </c>
       <c r="N9" t="n">
-        <v>3.826</v>
+        <v>3.88</v>
       </c>
       <c r="O9" t="n">
-        <v>3.902</v>
+        <v>3.957</v>
       </c>
       <c r="P9" t="n">
-        <v>4.025</v>
+        <v>4.068</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.075</v>
+        <v>4.107</v>
       </c>
       <c r="R9" t="n">
-        <v>4.115</v>
+        <v>4.136</v>
       </c>
       <c r="S9" t="n">
-        <v>4.15</v>
+        <v>4.16</v>
       </c>
       <c r="T9" t="n">
         <v>4.105</v>
       </c>
       <c r="U9" t="n">
-        <v>3.954</v>
+        <v>3.97</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1142,28 +1142,28 @@
         <v>2.767</v>
       </c>
       <c r="H10" t="n">
-        <v>2.925</v>
+        <v>2.926</v>
       </c>
       <c r="I10" t="n">
-        <v>3.157</v>
+        <v>3.162</v>
       </c>
       <c r="J10" t="n">
-        <v>3.372</v>
+        <v>3.388</v>
       </c>
       <c r="K10" t="n">
-        <v>3.56</v>
+        <v>3.598</v>
       </c>
       <c r="L10" t="n">
-        <v>3.611</v>
+        <v>3.663</v>
       </c>
       <c r="M10" t="n">
-        <v>3.758</v>
+        <v>3.811</v>
       </c>
       <c r="N10" t="n">
-        <v>3.847</v>
+        <v>3.901</v>
       </c>
       <c r="O10" t="n">
-        <v>4.121</v>
+        <v>4.178</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1218,31 +1218,31 @@
         <v>2.748</v>
       </c>
       <c r="I11" t="n">
-        <v>2.961</v>
+        <v>2.966</v>
       </c>
       <c r="J11" t="n">
-        <v>3.168</v>
+        <v>3.184</v>
       </c>
       <c r="K11" t="n">
-        <v>3.347</v>
+        <v>3.385</v>
       </c>
       <c r="L11" t="n">
-        <v>3.409</v>
+        <v>3.461</v>
       </c>
       <c r="M11" t="n">
-        <v>3.566</v>
+        <v>3.619</v>
       </c>
       <c r="N11" t="n">
-        <v>3.655</v>
+        <v>3.708</v>
       </c>
       <c r="O11" t="n">
-        <v>3.888</v>
+        <v>3.945</v>
       </c>
       <c r="P11" t="n">
-        <v>3.976</v>
+        <v>4.019</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.276</v>
+        <v>4.308</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.257</v>
+        <v>3.263</v>
       </c>
       <c r="G12" t="n">
-        <v>3.476</v>
+        <v>3.488</v>
       </c>
       <c r="H12" t="n">
-        <v>3.709</v>
+        <v>3.724</v>
       </c>
       <c r="I12" t="n">
-        <v>3.946</v>
+        <v>3.979</v>
       </c>
       <c r="J12" t="n">
-        <v>4.229</v>
+        <v>4.254</v>
       </c>
       <c r="K12" t="n">
-        <v>4.427</v>
+        <v>4.469</v>
       </c>
       <c r="L12" t="n">
-        <v>4.48</v>
+        <v>4.529</v>
       </c>
       <c r="M12" t="n">
-        <v>4.644</v>
+        <v>4.694</v>
       </c>
       <c r="N12" t="n">
-        <v>4.713</v>
+        <v>4.766</v>
       </c>
       <c r="O12" t="n">
-        <v>4.895</v>
+        <v>4.951</v>
       </c>
       <c r="P12" t="n">
-        <v>5.06</v>
+        <v>5.104</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.389</v>
+        <v>5.421</v>
       </c>
       <c r="R12" t="n">
-        <v>5.606</v>
+        <v>5.627</v>
       </c>
       <c r="S12" t="n">
-        <v>5.853</v>
+        <v>5.863</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.011</v>
+        <v>3.017</v>
       </c>
       <c r="G13" t="n">
-        <v>3.166</v>
+        <v>3.178</v>
       </c>
       <c r="H13" t="n">
-        <v>3.376</v>
+        <v>3.391</v>
       </c>
       <c r="I13" t="n">
-        <v>3.594</v>
+        <v>3.627</v>
       </c>
       <c r="J13" t="n">
-        <v>3.866</v>
+        <v>3.891</v>
       </c>
       <c r="K13" t="n">
-        <v>4.061</v>
+        <v>4.102</v>
       </c>
       <c r="L13" t="n">
-        <v>4.119</v>
+        <v>4.168</v>
       </c>
       <c r="M13" t="n">
-        <v>4.271</v>
+        <v>4.322</v>
       </c>
       <c r="N13" t="n">
-        <v>4.341</v>
+        <v>4.394</v>
       </c>
       <c r="O13" t="n">
-        <v>4.524</v>
+        <v>4.58</v>
       </c>
       <c r="P13" t="n">
-        <v>4.651</v>
+        <v>4.695</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.91</v>
+        <v>4.942</v>
       </c>
       <c r="R13" t="n">
-        <v>5.156</v>
+        <v>5.176</v>
       </c>
       <c r="S13" t="n">
-        <v>5.415</v>
+        <v>5.425</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.83</v>
+        <v>2.836</v>
       </c>
       <c r="G14" t="n">
-        <v>2.972</v>
+        <v>2.984</v>
       </c>
       <c r="H14" t="n">
-        <v>3.179</v>
+        <v>3.194</v>
       </c>
       <c r="I14" t="n">
-        <v>3.378</v>
+        <v>3.411</v>
       </c>
       <c r="J14" t="n">
-        <v>3.607</v>
+        <v>3.632</v>
       </c>
       <c r="K14" t="n">
-        <v>3.749</v>
+        <v>3.79</v>
       </c>
       <c r="L14" t="n">
-        <v>3.792</v>
+        <v>3.841</v>
       </c>
       <c r="M14" t="n">
-        <v>3.957</v>
+        <v>4.008</v>
       </c>
       <c r="N14" t="n">
-        <v>4.02</v>
+        <v>4.073</v>
       </c>
       <c r="O14" t="n">
-        <v>4.182</v>
+        <v>4.238</v>
       </c>
       <c r="P14" t="n">
-        <v>4.286</v>
+        <v>4.331</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.5</v>
+        <v>4.532</v>
       </c>
       <c r="R14" t="n">
-        <v>4.67</v>
+        <v>4.69</v>
       </c>
       <c r="S14" t="n">
-        <v>4.868</v>
+        <v>4.878</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.807</v>
+        <v>2.813</v>
       </c>
       <c r="G15" t="n">
-        <v>2.946</v>
+        <v>2.958</v>
       </c>
       <c r="H15" t="n">
-        <v>3.15</v>
+        <v>3.165</v>
       </c>
       <c r="I15" t="n">
-        <v>3.329</v>
+        <v>3.363</v>
       </c>
       <c r="J15" t="n">
-        <v>3.546</v>
+        <v>3.571</v>
       </c>
       <c r="K15" t="n">
-        <v>3.701</v>
+        <v>3.742</v>
       </c>
       <c r="L15" t="n">
-        <v>3.729</v>
+        <v>3.777</v>
       </c>
       <c r="M15" t="n">
-        <v>3.87</v>
+        <v>3.92</v>
       </c>
       <c r="N15" t="n">
-        <v>3.924</v>
+        <v>3.977</v>
       </c>
       <c r="O15" t="n">
-        <v>4.125</v>
+        <v>4.181</v>
       </c>
       <c r="P15" t="n">
-        <v>4.185</v>
+        <v>4.229</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.402</v>
+        <v>4.434</v>
       </c>
       <c r="R15" t="n">
-        <v>4.565</v>
+        <v>4.586</v>
       </c>
       <c r="S15" t="n">
-        <v>4.763</v>
+        <v>4.773</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.807</v>
+        <v>2.813</v>
       </c>
       <c r="G16" t="n">
-        <v>2.946</v>
+        <v>2.958</v>
       </c>
       <c r="H16" t="n">
-        <v>3.15</v>
+        <v>3.165</v>
       </c>
       <c r="I16" t="n">
-        <v>3.329</v>
+        <v>3.363</v>
       </c>
       <c r="J16" t="n">
-        <v>3.546</v>
+        <v>3.571</v>
       </c>
       <c r="K16" t="n">
-        <v>3.701</v>
+        <v>3.742</v>
       </c>
       <c r="L16" t="n">
-        <v>3.729</v>
+        <v>3.777</v>
       </c>
       <c r="M16" t="n">
-        <v>3.87</v>
+        <v>3.92</v>
       </c>
       <c r="N16" t="n">
-        <v>3.927</v>
+        <v>3.98</v>
       </c>
       <c r="O16" t="n">
-        <v>4.132</v>
+        <v>4.188</v>
       </c>
       <c r="P16" t="n">
-        <v>4.209</v>
+        <v>4.253</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.429</v>
+        <v>4.461</v>
       </c>
       <c r="R16" t="n">
-        <v>4.593</v>
+        <v>4.614</v>
       </c>
       <c r="S16" t="n">
-        <v>4.792</v>
+        <v>4.802</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.712</v>
       </c>
       <c r="G17" t="n">
-        <v>2.854</v>
+        <v>2.855</v>
       </c>
       <c r="H17" t="n">
-        <v>3.017</v>
+        <v>3.018</v>
       </c>
       <c r="I17" t="n">
-        <v>3.237</v>
+        <v>3.243</v>
       </c>
       <c r="J17" t="n">
-        <v>3.446</v>
+        <v>3.462</v>
       </c>
       <c r="K17" t="n">
-        <v>3.639</v>
+        <v>3.676</v>
       </c>
       <c r="L17" t="n">
-        <v>3.695</v>
+        <v>3.747</v>
       </c>
       <c r="M17" t="n">
-        <v>3.882</v>
+        <v>3.934</v>
       </c>
       <c r="N17" t="n">
-        <v>3.95</v>
+        <v>4.004</v>
       </c>
       <c r="O17" t="n">
-        <v>4.145</v>
+        <v>4.201</v>
       </c>
       <c r="P17" t="n">
-        <v>4.257</v>
+        <v>4.3</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.713</v>
       </c>
       <c r="G18" t="n">
-        <v>2.855</v>
+        <v>2.856</v>
       </c>
       <c r="H18" t="n">
-        <v>3.017</v>
+        <v>3.018</v>
       </c>
       <c r="I18" t="n">
-        <v>3.238</v>
+        <v>3.244</v>
       </c>
       <c r="J18" t="n">
-        <v>3.446</v>
+        <v>3.462</v>
       </c>
       <c r="K18" t="n">
-        <v>3.64</v>
+        <v>3.677</v>
       </c>
       <c r="L18" t="n">
-        <v>3.695</v>
+        <v>3.747</v>
       </c>
       <c r="M18" t="n">
-        <v>3.882</v>
+        <v>3.934</v>
       </c>
       <c r="N18" t="n">
-        <v>3.951</v>
+        <v>4.005</v>
       </c>
       <c r="O18" t="n">
-        <v>4.144</v>
+        <v>4.2</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.819</v>
+        <v>2.825</v>
       </c>
       <c r="G19" t="n">
-        <v>2.959</v>
+        <v>2.971</v>
       </c>
       <c r="H19" t="n">
-        <v>3.165</v>
+        <v>3.18</v>
       </c>
       <c r="I19" t="n">
-        <v>3.361</v>
+        <v>3.394</v>
       </c>
       <c r="J19" t="n">
-        <v>3.587</v>
+        <v>3.612</v>
       </c>
       <c r="K19" t="n">
-        <v>3.744</v>
+        <v>3.785</v>
       </c>
       <c r="L19" t="n">
-        <v>3.789</v>
+        <v>3.837</v>
       </c>
       <c r="M19" t="n">
-        <v>3.946</v>
+        <v>3.997</v>
       </c>
       <c r="N19" t="n">
-        <v>4.01</v>
+        <v>4.063</v>
       </c>
       <c r="O19" t="n">
-        <v>4.167</v>
+        <v>4.223</v>
       </c>
       <c r="P19" t="n">
-        <v>4.245</v>
+        <v>4.289</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.439</v>
+        <v>4.471</v>
       </c>
       <c r="R19" t="n">
-        <v>4.612</v>
+        <v>4.632</v>
       </c>
       <c r="S19" t="n">
-        <v>4.803</v>
+        <v>4.813</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.626</v>
       </c>
       <c r="G20" t="n">
-        <v>2.712</v>
+        <v>2.713</v>
       </c>
       <c r="H20" t="n">
-        <v>2.804</v>
+        <v>2.811</v>
       </c>
       <c r="I20" t="n">
-        <v>2.947</v>
+        <v>2.982</v>
       </c>
       <c r="J20" t="n">
-        <v>3.341</v>
+        <v>3.361</v>
       </c>
       <c r="K20" t="n">
-        <v>3.555</v>
+        <v>3.6</v>
       </c>
       <c r="L20" t="n">
-        <v>3.587</v>
+        <v>3.635</v>
       </c>
       <c r="M20" t="n">
-        <v>3.704</v>
+        <v>3.756</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.926</v>
+        <v>2.93</v>
       </c>
       <c r="G21" t="n">
-        <v>3.047</v>
+        <v>3.056</v>
       </c>
       <c r="H21" t="n">
-        <v>3.283</v>
+        <v>3.299</v>
       </c>
       <c r="I21" t="n">
-        <v>3.484</v>
+        <v>3.523</v>
       </c>
       <c r="J21" t="n">
-        <v>3.733</v>
+        <v>3.759</v>
       </c>
       <c r="K21" t="n">
-        <v>3.978</v>
+        <v>4.021</v>
       </c>
       <c r="L21" t="n">
-        <v>4.024</v>
+        <v>4.075</v>
       </c>
       <c r="M21" t="n">
-        <v>4.177</v>
+        <v>4.229</v>
       </c>
       <c r="N21" t="n">
-        <v>4.25</v>
+        <v>4.304</v>
       </c>
       <c r="O21" t="n">
-        <v>4.378</v>
+        <v>4.432</v>
       </c>
       <c r="P21" t="n">
-        <v>4.509</v>
+        <v>4.553</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.602</v>
+        <v>4.633</v>
       </c>
       <c r="R21" t="n">
-        <v>4.661</v>
+        <v>4.681</v>
       </c>
       <c r="S21" t="n">
-        <v>4.757</v>
+        <v>4.766</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.872</v>
+        <v>2.876</v>
       </c>
       <c r="G22" t="n">
-        <v>2.993</v>
+        <v>3.002</v>
       </c>
       <c r="H22" t="n">
-        <v>3.215</v>
+        <v>3.231</v>
       </c>
       <c r="I22" t="n">
-        <v>3.402</v>
+        <v>3.441</v>
       </c>
       <c r="J22" t="n">
-        <v>3.618</v>
+        <v>3.644</v>
       </c>
       <c r="K22" t="n">
-        <v>3.86</v>
+        <v>3.903</v>
       </c>
       <c r="L22" t="n">
-        <v>3.891</v>
+        <v>3.942</v>
       </c>
       <c r="M22" t="n">
-        <v>4.047</v>
+        <v>4.099</v>
       </c>
       <c r="N22" t="n">
-        <v>4.124</v>
+        <v>4.178</v>
       </c>
       <c r="O22" t="n">
-        <v>4.248</v>
+        <v>4.302</v>
       </c>
       <c r="P22" t="n">
-        <v>4.372</v>
+        <v>4.416</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.461</v>
+        <v>4.492</v>
       </c>
       <c r="R22" t="n">
-        <v>4.509</v>
+        <v>4.53</v>
       </c>
       <c r="S22" t="n">
-        <v>4.602</v>
+        <v>4.612</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.823</v>
+        <v>2.826</v>
       </c>
       <c r="G23" t="n">
-        <v>2.948</v>
+        <v>2.957</v>
       </c>
       <c r="H23" t="n">
-        <v>3.156</v>
+        <v>3.172</v>
       </c>
       <c r="I23" t="n">
-        <v>3.351</v>
+        <v>3.389</v>
       </c>
       <c r="J23" t="n">
-        <v>3.559</v>
+        <v>3.585</v>
       </c>
       <c r="K23" t="n">
-        <v>3.759</v>
+        <v>3.802</v>
       </c>
       <c r="L23" t="n">
-        <v>3.789</v>
+        <v>3.839</v>
       </c>
       <c r="M23" t="n">
-        <v>3.939</v>
+        <v>3.99</v>
       </c>
       <c r="N23" t="n">
-        <v>4.019</v>
+        <v>4.072</v>
       </c>
       <c r="O23" t="n">
-        <v>4.121</v>
+        <v>4.177</v>
       </c>
       <c r="P23" t="n">
-        <v>4.236</v>
+        <v>4.278</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.267</v>
+        <v>4.298</v>
       </c>
       <c r="R23" t="n">
-        <v>4.294</v>
+        <v>4.314</v>
       </c>
       <c r="S23" t="n">
-        <v>4.359</v>
+        <v>4.368</v>
       </c>
       <c r="T23" t="n">
-        <v>4.309</v>
+        <v>4.31</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.76</v>
+        <v>2.764</v>
       </c>
       <c r="G24" t="n">
-        <v>2.862</v>
+        <v>2.869</v>
       </c>
       <c r="H24" t="n">
-        <v>3.054</v>
+        <v>3.069</v>
       </c>
       <c r="I24" t="n">
-        <v>3.291</v>
+        <v>3.327</v>
       </c>
       <c r="J24" t="n">
-        <v>3.455</v>
+        <v>3.479</v>
       </c>
       <c r="K24" t="n">
-        <v>3.642</v>
+        <v>3.686</v>
       </c>
       <c r="L24" t="n">
-        <v>3.669</v>
+        <v>3.72</v>
       </c>
       <c r="M24" t="n">
-        <v>3.801</v>
+        <v>3.852</v>
       </c>
       <c r="N24" t="n">
-        <v>3.894</v>
+        <v>3.948</v>
       </c>
       <c r="O24" t="n">
-        <v>4.119</v>
+        <v>4.176</v>
       </c>
       <c r="P24" t="n">
-        <v>4.173</v>
+        <v>4.215</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.192</v>
+        <v>4.223</v>
       </c>
       <c r="R24" t="n">
-        <v>4.216</v>
+        <v>4.236</v>
       </c>
       <c r="S24" t="n">
-        <v>4.274</v>
+        <v>4.283</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.817</v>
+        <v>2.821</v>
       </c>
       <c r="G25" t="n">
-        <v>2.948</v>
+        <v>2.957</v>
       </c>
       <c r="H25" t="n">
-        <v>3.159</v>
+        <v>3.176</v>
       </c>
       <c r="I25" t="n">
-        <v>3.359</v>
+        <v>3.398</v>
       </c>
       <c r="J25" t="n">
-        <v>3.575</v>
+        <v>3.6</v>
       </c>
       <c r="K25" t="n">
-        <v>3.792</v>
+        <v>3.835</v>
       </c>
       <c r="L25" t="n">
-        <v>3.821</v>
+        <v>3.87</v>
       </c>
       <c r="M25" t="n">
-        <v>3.972</v>
+        <v>4.023</v>
       </c>
       <c r="N25" t="n">
-        <v>4.045</v>
+        <v>4.099</v>
       </c>
       <c r="O25" t="n">
-        <v>4.15</v>
+        <v>4.206</v>
       </c>
       <c r="P25" t="n">
-        <v>4.257</v>
+        <v>4.3</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.3</v>
+        <v>4.331</v>
       </c>
       <c r="R25" t="n">
-        <v>4.318</v>
+        <v>4.338</v>
       </c>
       <c r="S25" t="n">
-        <v>4.382</v>
+        <v>4.391</v>
       </c>
       <c r="T25" t="n">
-        <v>4.327</v>
+        <v>4.328</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.092</v>
+        <v>3.098</v>
       </c>
       <c r="G26" t="n">
-        <v>3.269</v>
+        <v>3.279</v>
       </c>
       <c r="H26" t="n">
-        <v>3.588</v>
+        <v>3.604</v>
       </c>
       <c r="I26" t="n">
-        <v>3.828</v>
+        <v>3.864</v>
       </c>
       <c r="J26" t="n">
-        <v>4.2</v>
+        <v>4.221</v>
       </c>
       <c r="K26" t="n">
-        <v>4.598</v>
+        <v>4.642</v>
       </c>
       <c r="L26" t="n">
-        <v>4.7</v>
+        <v>4.751</v>
       </c>
       <c r="M26" t="n">
-        <v>4.897</v>
+        <v>4.949</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.219</v>
+        <v>5.274</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.91</v>
+        <v>2.915</v>
       </c>
       <c r="G27" t="n">
-        <v>3.036</v>
+        <v>3.048</v>
       </c>
       <c r="H27" t="n">
-        <v>3.259</v>
+        <v>3.275</v>
       </c>
       <c r="I27" t="n">
-        <v>3.465</v>
+        <v>3.499</v>
       </c>
       <c r="J27" t="n">
-        <v>3.713</v>
+        <v>3.739</v>
       </c>
       <c r="K27" t="n">
-        <v>3.92</v>
+        <v>3.963</v>
       </c>
       <c r="L27" t="n">
-        <v>3.973</v>
+        <v>4.022</v>
       </c>
       <c r="M27" t="n">
-        <v>4.117</v>
+        <v>4.168</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.315</v>
+        <v>4.37</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.013</v>
+        <v>3.018</v>
       </c>
       <c r="G28" t="n">
-        <v>3.147</v>
+        <v>3.159</v>
       </c>
       <c r="H28" t="n">
-        <v>3.385</v>
+        <v>3.401</v>
       </c>
       <c r="I28" t="n">
-        <v>3.602</v>
+        <v>3.636</v>
       </c>
       <c r="J28" t="n">
-        <v>3.886</v>
+        <v>3.912</v>
       </c>
       <c r="K28" t="n">
-        <v>4.112</v>
+        <v>4.156</v>
       </c>
       <c r="L28" t="n">
-        <v>4.176</v>
+        <v>4.225</v>
       </c>
       <c r="M28" t="n">
-        <v>4.329</v>
+        <v>4.38</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.607</v>
+        <v>4.662</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.86</v>
+        <v>2.865</v>
       </c>
       <c r="G29" t="n">
-        <v>2.986</v>
+        <v>2.996</v>
       </c>
       <c r="H29" t="n">
-        <v>3.2</v>
+        <v>3.214</v>
       </c>
       <c r="I29" t="n">
-        <v>3.395</v>
+        <v>3.427</v>
       </c>
       <c r="J29" t="n">
-        <v>3.625</v>
+        <v>3.651</v>
       </c>
       <c r="K29" t="n">
-        <v>3.816</v>
+        <v>3.859</v>
       </c>
       <c r="L29" t="n">
-        <v>3.859</v>
+        <v>3.907</v>
       </c>
       <c r="M29" t="n">
-        <v>3.98</v>
+        <v>4.031</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.186</v>
+        <v>4.241</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.133</v>
+        <v>3.14</v>
       </c>
       <c r="G30" t="n">
-        <v>3.244</v>
+        <v>3.256</v>
       </c>
       <c r="H30" t="n">
-        <v>3.517</v>
+        <v>3.537</v>
       </c>
       <c r="I30" t="n">
-        <v>3.749</v>
+        <v>3.788</v>
       </c>
       <c r="J30" t="n">
-        <v>4.064</v>
+        <v>4.087</v>
       </c>
       <c r="K30" t="n">
-        <v>4.394</v>
+        <v>4.44</v>
       </c>
       <c r="L30" t="n">
-        <v>4.478</v>
+        <v>4.53</v>
       </c>
       <c r="M30" t="n">
-        <v>4.666</v>
+        <v>4.717</v>
       </c>
       <c r="N30" t="n">
-        <v>4.843</v>
+        <v>4.896</v>
       </c>
       <c r="O30" t="n">
-        <v>5.17</v>
+        <v>5.225</v>
       </c>
       <c r="P30" t="n">
-        <v>5.399</v>
+        <v>5.443</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.135</v>
+        <v>6.167</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.462</v>
+        <v>3.469</v>
       </c>
       <c r="G31" t="n">
-        <v>3.609</v>
+        <v>3.621</v>
       </c>
       <c r="H31" t="n">
-        <v>3.932</v>
+        <v>3.951</v>
       </c>
       <c r="I31" t="n">
-        <v>4.179</v>
+        <v>4.218</v>
       </c>
       <c r="J31" t="n">
-        <v>4.555</v>
+        <v>4.578</v>
       </c>
       <c r="K31" t="n">
-        <v>4.927</v>
+        <v>4.973</v>
       </c>
       <c r="L31" t="n">
-        <v>5.09</v>
+        <v>5.142</v>
       </c>
       <c r="M31" t="n">
-        <v>5.397</v>
+        <v>5.448</v>
       </c>
       <c r="N31" t="n">
-        <v>5.702</v>
+        <v>5.755</v>
       </c>
       <c r="O31" t="n">
-        <v>6.206</v>
+        <v>6.261</v>
       </c>
       <c r="P31" t="n">
-        <v>6.388</v>
+        <v>6.431</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.109</v>
+        <v>7.141</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.232</v>
+        <v>3.239</v>
       </c>
       <c r="G32" t="n">
-        <v>3.362</v>
+        <v>3.374</v>
       </c>
       <c r="H32" t="n">
-        <v>3.661</v>
+        <v>3.681</v>
       </c>
       <c r="I32" t="n">
-        <v>3.908</v>
+        <v>3.947</v>
       </c>
       <c r="J32" t="n">
-        <v>4.242</v>
+        <v>4.265</v>
       </c>
       <c r="K32" t="n">
-        <v>4.579</v>
+        <v>4.625</v>
       </c>
       <c r="L32" t="n">
-        <v>4.682</v>
+        <v>4.734</v>
       </c>
       <c r="M32" t="n">
-        <v>4.939</v>
+        <v>4.99</v>
       </c>
       <c r="N32" t="n">
-        <v>5.203</v>
+        <v>5.257</v>
       </c>
       <c r="O32" t="n">
-        <v>5.615</v>
+        <v>5.67</v>
       </c>
       <c r="P32" t="n">
-        <v>5.859</v>
+        <v>5.903</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.596</v>
+        <v>6.628</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.997</v>
+        <v>3.004</v>
       </c>
       <c r="G33" t="n">
-        <v>3.109</v>
+        <v>3.121</v>
       </c>
       <c r="H33" t="n">
-        <v>3.336</v>
+        <v>3.354</v>
       </c>
       <c r="I33" t="n">
-        <v>3.533</v>
+        <v>3.572</v>
       </c>
       <c r="J33" t="n">
-        <v>3.771</v>
+        <v>3.793</v>
       </c>
       <c r="K33" t="n">
-        <v>4.036</v>
+        <v>4.082</v>
       </c>
       <c r="L33" t="n">
-        <v>4.08</v>
+        <v>4.131</v>
       </c>
       <c r="M33" t="n">
-        <v>4.191</v>
+        <v>4.243</v>
       </c>
       <c r="N33" t="n">
-        <v>4.232</v>
+        <v>4.286</v>
       </c>
       <c r="O33" t="n">
-        <v>4.324</v>
+        <v>4.379</v>
       </c>
       <c r="P33" t="n">
-        <v>4.432</v>
+        <v>4.475</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.852</v>
+        <v>4.884</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.057</v>
+        <v>3.064</v>
       </c>
       <c r="G34" t="n">
-        <v>3.162</v>
+        <v>3.174</v>
       </c>
       <c r="H34" t="n">
-        <v>3.398</v>
+        <v>3.416</v>
       </c>
       <c r="I34" t="n">
-        <v>3.601</v>
+        <v>3.64</v>
       </c>
       <c r="J34" t="n">
-        <v>3.842</v>
+        <v>3.865</v>
       </c>
       <c r="K34" t="n">
-        <v>4.113</v>
+        <v>4.159</v>
       </c>
       <c r="L34" t="n">
-        <v>4.159</v>
+        <v>4.21</v>
       </c>
       <c r="M34" t="n">
-        <v>4.282</v>
+        <v>4.333</v>
       </c>
       <c r="N34" t="n">
-        <v>4.336</v>
+        <v>4.39</v>
       </c>
       <c r="O34" t="n">
-        <v>4.493</v>
+        <v>4.548</v>
       </c>
       <c r="P34" t="n">
-        <v>4.726</v>
+        <v>4.77</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.553</v>
+        <v>5.585</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.031</v>
+        <v>3.038</v>
       </c>
       <c r="G35" t="n">
-        <v>3.136</v>
+        <v>3.148</v>
       </c>
       <c r="H35" t="n">
-        <v>3.365</v>
+        <v>3.384</v>
       </c>
       <c r="I35" t="n">
-        <v>3.568</v>
+        <v>3.607</v>
       </c>
       <c r="J35" t="n">
-        <v>3.811</v>
+        <v>3.834</v>
       </c>
       <c r="K35" t="n">
-        <v>4.067</v>
+        <v>4.113</v>
       </c>
       <c r="L35" t="n">
-        <v>4.114</v>
+        <v>4.165</v>
       </c>
       <c r="M35" t="n">
-        <v>4.229</v>
+        <v>4.28</v>
       </c>
       <c r="N35" t="n">
-        <v>4.273</v>
+        <v>4.326</v>
       </c>
       <c r="O35" t="n">
-        <v>4.39</v>
+        <v>4.445</v>
       </c>
       <c r="P35" t="n">
-        <v>4.529</v>
+        <v>4.572</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.189</v>
+        <v>5.221</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.926</v>
+        <v>2.933</v>
       </c>
       <c r="G36" t="n">
-        <v>3.03</v>
+        <v>3.039</v>
       </c>
       <c r="H36" t="n">
-        <v>3.25</v>
+        <v>3.265</v>
       </c>
       <c r="I36" t="n">
-        <v>3.451</v>
+        <v>3.488</v>
       </c>
       <c r="J36" t="n">
-        <v>3.709</v>
+        <v>3.732</v>
       </c>
       <c r="K36" t="n">
-        <v>3.962</v>
+        <v>4.008</v>
       </c>
       <c r="L36" t="n">
-        <v>4.006</v>
+        <v>4.058</v>
       </c>
       <c r="M36" t="n">
-        <v>4.092</v>
+        <v>4.144</v>
       </c>
       <c r="N36" t="n">
-        <v>4.135</v>
+        <v>4.189</v>
       </c>
       <c r="O36" t="n">
-        <v>4.232</v>
+        <v>4.287</v>
       </c>
       <c r="P36" t="n">
-        <v>4.33</v>
+        <v>4.373</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.569</v>
+        <v>4.601</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.806</v>
+        <v>3.812</v>
       </c>
       <c r="G37" t="n">
-        <v>4.304</v>
+        <v>4.314</v>
       </c>
       <c r="H37" t="n">
-        <v>4.908</v>
+        <v>4.924</v>
       </c>
       <c r="I37" t="n">
-        <v>5.241</v>
+        <v>5.278</v>
       </c>
       <c r="J37" t="n">
-        <v>6.046</v>
+        <v>6.068</v>
       </c>
       <c r="K37" t="n">
-        <v>6.968</v>
+        <v>7.013</v>
       </c>
       <c r="L37" t="n">
-        <v>7.29</v>
+        <v>7.342</v>
       </c>
       <c r="M37" t="n">
-        <v>7.669</v>
+        <v>7.72</v>
       </c>
       <c r="N37" t="n">
-        <v>7.853</v>
+        <v>7.906</v>
       </c>
       <c r="O37" t="n">
-        <v>8.085000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.186999999999999</v>
+        <v>8.231</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.597</v>
+        <v>8.629</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.865</v>
+        <v>4.872</v>
       </c>
       <c r="G38" t="n">
-        <v>5.617</v>
+        <v>5.629</v>
       </c>
       <c r="H38" t="n">
-        <v>6.432</v>
+        <v>6.45</v>
       </c>
       <c r="I38" t="n">
-        <v>6.922</v>
+        <v>6.961</v>
       </c>
       <c r="J38" t="n">
-        <v>7.989</v>
+        <v>8.012</v>
       </c>
       <c r="K38" t="n">
-        <v>9.089</v>
+        <v>9.135</v>
       </c>
       <c r="L38" t="n">
-        <v>9.573</v>
+        <v>9.625</v>
       </c>
       <c r="M38" t="n">
-        <v>10.08</v>
+        <v>10.132</v>
       </c>
       <c r="N38" t="n">
-        <v>10.272</v>
+        <v>10.325</v>
       </c>
       <c r="O38" t="n">
-        <v>10.485</v>
+        <v>10.54</v>
       </c>
       <c r="P38" t="n">
-        <v>10.585</v>
+        <v>10.629</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.048</v>
+        <v>11.08</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.186</v>
+        <v>4.193</v>
       </c>
       <c r="G39" t="n">
-        <v>4.815</v>
+        <v>4.827</v>
       </c>
       <c r="H39" t="n">
-        <v>5.497</v>
+        <v>5.515</v>
       </c>
       <c r="I39" t="n">
-        <v>5.926</v>
+        <v>5.965</v>
       </c>
       <c r="J39" t="n">
-        <v>6.862</v>
+        <v>6.885</v>
       </c>
       <c r="K39" t="n">
-        <v>7.922</v>
+        <v>7.968</v>
       </c>
       <c r="L39" t="n">
-        <v>8.327999999999999</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.717000000000001</v>
+        <v>8.768000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.898999999999999</v>
+        <v>8.952999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.135999999999999</v>
+        <v>9.19</v>
       </c>
       <c r="P39" t="n">
-        <v>9.24</v>
+        <v>9.282999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.693</v>
+        <v>9.725</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.325</v>
+        <v>3.332</v>
       </c>
       <c r="G40" t="n">
-        <v>3.482</v>
+        <v>3.494</v>
       </c>
       <c r="H40" t="n">
-        <v>3.776</v>
+        <v>3.796</v>
       </c>
       <c r="I40" t="n">
-        <v>4.023</v>
+        <v>4.062</v>
       </c>
       <c r="J40" t="n">
-        <v>4.355</v>
+        <v>4.378</v>
       </c>
       <c r="K40" t="n">
-        <v>4.7</v>
+        <v>4.746</v>
       </c>
       <c r="L40" t="n">
-        <v>4.802</v>
+        <v>4.854</v>
       </c>
       <c r="M40" t="n">
-        <v>5.009</v>
+        <v>5.06</v>
       </c>
       <c r="N40" t="n">
-        <v>5.2</v>
+        <v>5.254</v>
       </c>
       <c r="O40" t="n">
-        <v>5.549</v>
+        <v>5.604</v>
       </c>
       <c r="P40" t="n">
-        <v>5.821</v>
+        <v>5.864</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.586</v>
+        <v>6.618</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.711</v>
+        <v>3.718</v>
       </c>
       <c r="G41" t="n">
-        <v>3.911</v>
+        <v>3.923</v>
       </c>
       <c r="H41" t="n">
-        <v>4.261</v>
+        <v>4.281</v>
       </c>
       <c r="I41" t="n">
-        <v>4.526</v>
+        <v>4.566</v>
       </c>
       <c r="J41" t="n">
-        <v>4.91</v>
+        <v>4.933</v>
       </c>
       <c r="K41" t="n">
-        <v>5.301</v>
+        <v>5.346</v>
       </c>
       <c r="L41" t="n">
-        <v>5.481</v>
+        <v>5.533</v>
       </c>
       <c r="M41" t="n">
-        <v>5.811</v>
+        <v>5.863</v>
       </c>
       <c r="N41" t="n">
-        <v>6.131</v>
+        <v>6.185</v>
       </c>
       <c r="O41" t="n">
-        <v>6.664</v>
+        <v>6.719</v>
       </c>
       <c r="P41" t="n">
-        <v>6.88</v>
+        <v>6.923</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.633</v>
+        <v>7.665</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.446</v>
+        <v>3.453</v>
       </c>
       <c r="G42" t="n">
-        <v>3.631</v>
+        <v>3.643</v>
       </c>
       <c r="H42" t="n">
-        <v>3.952</v>
+        <v>3.972</v>
       </c>
       <c r="I42" t="n">
-        <v>4.211</v>
+        <v>4.25</v>
       </c>
       <c r="J42" t="n">
-        <v>4.558</v>
+        <v>4.581</v>
       </c>
       <c r="K42" t="n">
-        <v>4.921</v>
+        <v>4.967</v>
       </c>
       <c r="L42" t="n">
-        <v>5.039</v>
+        <v>5.09</v>
       </c>
       <c r="M42" t="n">
-        <v>5.316</v>
+        <v>5.367</v>
       </c>
       <c r="N42" t="n">
-        <v>5.615</v>
+        <v>5.669</v>
       </c>
       <c r="O42" t="n">
-        <v>6.041</v>
+        <v>6.096</v>
       </c>
       <c r="P42" t="n">
-        <v>6.323</v>
+        <v>6.366</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.099</v>
+        <v>7.131</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.145</v>
+        <v>3.152</v>
       </c>
       <c r="G43" t="n">
-        <v>3.292</v>
+        <v>3.304</v>
       </c>
       <c r="H43" t="n">
-        <v>3.537</v>
+        <v>3.555</v>
       </c>
       <c r="I43" t="n">
-        <v>3.742</v>
+        <v>3.781</v>
       </c>
       <c r="J43" t="n">
-        <v>3.998</v>
+        <v>4.021</v>
       </c>
       <c r="K43" t="n">
-        <v>4.268</v>
+        <v>4.314</v>
       </c>
       <c r="L43" t="n">
-        <v>4.321</v>
+        <v>4.373</v>
       </c>
       <c r="M43" t="n">
-        <v>4.447</v>
+        <v>4.498</v>
       </c>
       <c r="N43" t="n">
-        <v>4.501</v>
+        <v>4.555</v>
       </c>
       <c r="O43" t="n">
-        <v>4.637</v>
+        <v>4.692</v>
       </c>
       <c r="P43" t="n">
-        <v>4.797</v>
+        <v>4.841</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.462</v>
+        <v>5.494</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.004</v>
+        <v>3.011</v>
       </c>
       <c r="G44" t="n">
-        <v>3.139</v>
+        <v>3.148</v>
       </c>
       <c r="H44" t="n">
-        <v>3.373</v>
+        <v>3.389</v>
       </c>
       <c r="I44" t="n">
-        <v>3.578</v>
+        <v>3.615</v>
       </c>
       <c r="J44" t="n">
-        <v>3.85</v>
+        <v>3.873</v>
       </c>
       <c r="K44" t="n">
-        <v>4.114</v>
+        <v>4.16</v>
       </c>
       <c r="L44" t="n">
-        <v>4.167</v>
+        <v>4.219</v>
       </c>
       <c r="M44" t="n">
-        <v>4.263</v>
+        <v>4.314</v>
       </c>
       <c r="N44" t="n">
-        <v>4.317</v>
+        <v>4.371</v>
       </c>
       <c r="O44" t="n">
-        <v>4.433</v>
+        <v>4.488</v>
       </c>
       <c r="P44" t="n">
-        <v>4.56</v>
+        <v>4.603</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.833</v>
+        <v>4.865</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-28 ~ 2026-05-28
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.262</v>
+        <v>3.279</v>
       </c>
       <c r="G2" t="n">
-        <v>3.529</v>
+        <v>3.55</v>
       </c>
       <c r="H2" t="n">
-        <v>3.809</v>
+        <v>3.839</v>
       </c>
       <c r="I2" t="n">
-        <v>4.018</v>
+        <v>4.058</v>
       </c>
       <c r="J2" t="n">
-        <v>4.265</v>
+        <v>4.317</v>
       </c>
       <c r="K2" t="n">
-        <v>4.68</v>
+        <v>4.731</v>
       </c>
       <c r="L2" t="n">
-        <v>4.851</v>
+        <v>4.907</v>
       </c>
       <c r="M2" t="n">
-        <v>5.168</v>
+        <v>5.219</v>
       </c>
       <c r="N2" t="n">
-        <v>5.458</v>
+        <v>5.5</v>
       </c>
       <c r="O2" t="n">
-        <v>5.74</v>
+        <v>5.773</v>
       </c>
       <c r="P2" t="n">
-        <v>5.966</v>
+        <v>6.002</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.567</v>
+        <v>6.606</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.283</v>
+        <v>4.3</v>
       </c>
       <c r="G3" t="n">
-        <v>4.732</v>
+        <v>4.753</v>
       </c>
       <c r="H3" t="n">
-        <v>5.044</v>
+        <v>5.074</v>
       </c>
       <c r="I3" t="n">
-        <v>5.247</v>
+        <v>5.287</v>
       </c>
       <c r="J3" t="n">
-        <v>5.51</v>
+        <v>5.563</v>
       </c>
       <c r="K3" t="n">
-        <v>5.996</v>
+        <v>6.047</v>
       </c>
       <c r="L3" t="n">
-        <v>6.237</v>
+        <v>6.293</v>
       </c>
       <c r="M3" t="n">
-        <v>6.584</v>
+        <v>6.635</v>
       </c>
       <c r="N3" t="n">
-        <v>6.818</v>
+        <v>6.859</v>
       </c>
       <c r="O3" t="n">
-        <v>7.05</v>
+        <v>7.083</v>
       </c>
       <c r="P3" t="n">
-        <v>7.147</v>
+        <v>7.182</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.636</v>
+        <v>7.674</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.776</v>
+        <v>3.793</v>
       </c>
       <c r="G4" t="n">
-        <v>4.113</v>
+        <v>4.134</v>
       </c>
       <c r="H4" t="n">
-        <v>4.454</v>
+        <v>4.484</v>
       </c>
       <c r="I4" t="n">
-        <v>4.689</v>
+        <v>4.729</v>
       </c>
       <c r="J4" t="n">
-        <v>4.956</v>
+        <v>5.009</v>
       </c>
       <c r="K4" t="n">
-        <v>5.435</v>
+        <v>5.486</v>
       </c>
       <c r="L4" t="n">
-        <v>5.606</v>
+        <v>5.662</v>
       </c>
       <c r="M4" t="n">
-        <v>5.942</v>
+        <v>5.993</v>
       </c>
       <c r="N4" t="n">
-        <v>6.146</v>
+        <v>6.187</v>
       </c>
       <c r="O4" t="n">
-        <v>6.401</v>
+        <v>6.434</v>
       </c>
       <c r="P4" t="n">
-        <v>6.497</v>
+        <v>6.532</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.989</v>
+        <v>7.027</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.959</v>
+        <v>2.976</v>
       </c>
       <c r="G5" t="n">
-        <v>3.07</v>
+        <v>3.091</v>
       </c>
       <c r="H5" t="n">
-        <v>3.315</v>
+        <v>3.345</v>
       </c>
       <c r="I5" t="n">
-        <v>3.59</v>
+        <v>3.631</v>
       </c>
       <c r="J5" t="n">
-        <v>3.821</v>
+        <v>3.873</v>
       </c>
       <c r="K5" t="n">
-        <v>4.081</v>
+        <v>4.132</v>
       </c>
       <c r="L5" t="n">
-        <v>4.098</v>
+        <v>4.154</v>
       </c>
       <c r="M5" t="n">
-        <v>4.226</v>
+        <v>4.277</v>
       </c>
       <c r="N5" t="n">
-        <v>4.271</v>
+        <v>4.312</v>
       </c>
       <c r="O5" t="n">
-        <v>4.339</v>
+        <v>4.372</v>
       </c>
       <c r="P5" t="n">
-        <v>4.635</v>
+        <v>4.671</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.479</v>
+        <v>5.518</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>3.017</v>
       </c>
       <c r="G6" t="n">
-        <v>3.126</v>
+        <v>3.147</v>
       </c>
       <c r="H6" t="n">
-        <v>3.384</v>
+        <v>3.414</v>
       </c>
       <c r="I6" t="n">
-        <v>3.673</v>
+        <v>3.715</v>
       </c>
       <c r="J6" t="n">
-        <v>3.913</v>
+        <v>3.965</v>
       </c>
       <c r="K6" t="n">
-        <v>4.197</v>
+        <v>4.248</v>
       </c>
       <c r="L6" t="n">
-        <v>4.217</v>
+        <v>4.273</v>
       </c>
       <c r="M6" t="n">
-        <v>4.383</v>
+        <v>4.434</v>
       </c>
       <c r="N6" t="n">
-        <v>4.438</v>
+        <v>4.479</v>
       </c>
       <c r="O6" t="n">
-        <v>4.606</v>
+        <v>4.639</v>
       </c>
       <c r="P6" t="n">
-        <v>5.067</v>
+        <v>5.103</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.876</v>
+        <v>5.914</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.98</v>
+        <v>2.997</v>
       </c>
       <c r="G7" t="n">
-        <v>3.089</v>
+        <v>3.11</v>
       </c>
       <c r="H7" t="n">
-        <v>3.331</v>
+        <v>3.361</v>
       </c>
       <c r="I7" t="n">
-        <v>3.608</v>
+        <v>3.65</v>
       </c>
       <c r="J7" t="n">
-        <v>3.844</v>
+        <v>3.896</v>
       </c>
       <c r="K7" t="n">
-        <v>4.108</v>
+        <v>4.159</v>
       </c>
       <c r="L7" t="n">
-        <v>4.124</v>
+        <v>4.18</v>
       </c>
       <c r="M7" t="n">
-        <v>4.286</v>
+        <v>4.337</v>
       </c>
       <c r="N7" t="n">
-        <v>4.33</v>
+        <v>4.371</v>
       </c>
       <c r="O7" t="n">
-        <v>4.504</v>
+        <v>4.536</v>
       </c>
       <c r="P7" t="n">
-        <v>4.851</v>
+        <v>4.887</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.643</v>
+        <v>5.682</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.395</v>
+        <v>5.412</v>
       </c>
       <c r="G8" t="n">
-        <v>6.032</v>
+        <v>6.053</v>
       </c>
       <c r="H8" t="n">
-        <v>6.493</v>
+        <v>6.523</v>
       </c>
       <c r="I8" t="n">
-        <v>6.773</v>
+        <v>6.813</v>
       </c>
       <c r="J8" t="n">
-        <v>7.103</v>
+        <v>7.156</v>
       </c>
       <c r="K8" t="n">
-        <v>7.87</v>
+        <v>7.921</v>
       </c>
       <c r="L8" t="n">
-        <v>8.195</v>
+        <v>8.250999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.574999999999999</v>
+        <v>8.625999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.742000000000001</v>
+        <v>8.782999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.058999999999999</v>
+        <v>9.092000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.257999999999999</v>
+        <v>9.292999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.945</v>
+        <v>9.983000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.636</v>
+        <v>2.637</v>
       </c>
       <c r="G9" t="n">
-        <v>2.731</v>
+        <v>2.737</v>
       </c>
       <c r="H9" t="n">
-        <v>2.914</v>
+        <v>2.938</v>
       </c>
       <c r="I9" t="n">
-        <v>3.157</v>
+        <v>3.182</v>
       </c>
       <c r="J9" t="n">
-        <v>3.36</v>
+        <v>3.391</v>
       </c>
       <c r="K9" t="n">
-        <v>3.565</v>
+        <v>3.613</v>
       </c>
       <c r="L9" t="n">
-        <v>3.612</v>
+        <v>3.667</v>
       </c>
       <c r="M9" t="n">
-        <v>3.717</v>
+        <v>3.767</v>
       </c>
       <c r="N9" t="n">
-        <v>3.88</v>
+        <v>3.921</v>
       </c>
       <c r="O9" t="n">
-        <v>3.957</v>
+        <v>3.99</v>
       </c>
       <c r="P9" t="n">
-        <v>4.068</v>
+        <v>4.103</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.107</v>
+        <v>4.145</v>
       </c>
       <c r="R9" t="n">
-        <v>4.136</v>
+        <v>4.168</v>
       </c>
       <c r="S9" t="n">
-        <v>4.16</v>
+        <v>4.185</v>
       </c>
       <c r="T9" t="n">
-        <v>4.105</v>
+        <v>4.114</v>
       </c>
       <c r="U9" t="n">
-        <v>3.97</v>
+        <v>3.993</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.656</v>
+        <v>2.657</v>
       </c>
       <c r="G10" t="n">
-        <v>2.767</v>
+        <v>2.774</v>
       </c>
       <c r="H10" t="n">
-        <v>2.926</v>
+        <v>2.95</v>
       </c>
       <c r="I10" t="n">
-        <v>3.162</v>
+        <v>3.187</v>
       </c>
       <c r="J10" t="n">
-        <v>3.388</v>
+        <v>3.418</v>
       </c>
       <c r="K10" t="n">
-        <v>3.598</v>
+        <v>3.646</v>
       </c>
       <c r="L10" t="n">
-        <v>3.663</v>
+        <v>3.718</v>
       </c>
       <c r="M10" t="n">
-        <v>3.811</v>
+        <v>3.861</v>
       </c>
       <c r="N10" t="n">
-        <v>3.901</v>
+        <v>3.942</v>
       </c>
       <c r="O10" t="n">
-        <v>4.178</v>
+        <v>4.228</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.466</v>
+        <v>2.467</v>
       </c>
       <c r="G11" t="n">
-        <v>2.575</v>
+        <v>2.581</v>
       </c>
       <c r="H11" t="n">
-        <v>2.748</v>
+        <v>2.773</v>
       </c>
       <c r="I11" t="n">
-        <v>2.966</v>
+        <v>2.991</v>
       </c>
       <c r="J11" t="n">
-        <v>3.184</v>
+        <v>3.215</v>
       </c>
       <c r="K11" t="n">
-        <v>3.385</v>
+        <v>3.433</v>
       </c>
       <c r="L11" t="n">
-        <v>3.461</v>
+        <v>3.515</v>
       </c>
       <c r="M11" t="n">
-        <v>3.619</v>
+        <v>3.669</v>
       </c>
       <c r="N11" t="n">
-        <v>3.708</v>
+        <v>3.749</v>
       </c>
       <c r="O11" t="n">
-        <v>3.945</v>
+        <v>3.994</v>
       </c>
       <c r="P11" t="n">
-        <v>4.019</v>
+        <v>4.054</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.308</v>
+        <v>4.346</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.263</v>
+        <v>3.276</v>
       </c>
       <c r="G12" t="n">
-        <v>3.488</v>
+        <v>3.505</v>
       </c>
       <c r="H12" t="n">
-        <v>3.724</v>
+        <v>3.753</v>
       </c>
       <c r="I12" t="n">
-        <v>3.979</v>
+        <v>4.021</v>
       </c>
       <c r="J12" t="n">
-        <v>4.254</v>
+        <v>4.3</v>
       </c>
       <c r="K12" t="n">
-        <v>4.469</v>
+        <v>4.521</v>
       </c>
       <c r="L12" t="n">
-        <v>4.529</v>
+        <v>4.584</v>
       </c>
       <c r="M12" t="n">
-        <v>4.694</v>
+        <v>4.744</v>
       </c>
       <c r="N12" t="n">
-        <v>4.766</v>
+        <v>4.81</v>
       </c>
       <c r="O12" t="n">
-        <v>4.951</v>
+        <v>4.993</v>
       </c>
       <c r="P12" t="n">
-        <v>5.104</v>
+        <v>5.139</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.421</v>
+        <v>5.46</v>
       </c>
       <c r="R12" t="n">
-        <v>5.627</v>
+        <v>5.659</v>
       </c>
       <c r="S12" t="n">
-        <v>5.863</v>
+        <v>5.888</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.017</v>
+        <v>3.03</v>
       </c>
       <c r="G13" t="n">
-        <v>3.178</v>
+        <v>3.195</v>
       </c>
       <c r="H13" t="n">
-        <v>3.391</v>
+        <v>3.42</v>
       </c>
       <c r="I13" t="n">
-        <v>3.627</v>
+        <v>3.668</v>
       </c>
       <c r="J13" t="n">
-        <v>3.891</v>
+        <v>3.937</v>
       </c>
       <c r="K13" t="n">
-        <v>4.102</v>
+        <v>4.154</v>
       </c>
       <c r="L13" t="n">
-        <v>4.168</v>
+        <v>4.223</v>
       </c>
       <c r="M13" t="n">
-        <v>4.322</v>
+        <v>4.371</v>
       </c>
       <c r="N13" t="n">
-        <v>4.394</v>
+        <v>4.438</v>
       </c>
       <c r="O13" t="n">
-        <v>4.58</v>
+        <v>4.621</v>
       </c>
       <c r="P13" t="n">
-        <v>4.695</v>
+        <v>4.731</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.942</v>
+        <v>4.981</v>
       </c>
       <c r="R13" t="n">
-        <v>5.176</v>
+        <v>5.209</v>
       </c>
       <c r="S13" t="n">
-        <v>5.425</v>
+        <v>5.45</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.836</v>
+        <v>2.849</v>
       </c>
       <c r="G14" t="n">
-        <v>2.984</v>
+        <v>3.001</v>
       </c>
       <c r="H14" t="n">
-        <v>3.194</v>
+        <v>3.223</v>
       </c>
       <c r="I14" t="n">
-        <v>3.411</v>
+        <v>3.453</v>
       </c>
       <c r="J14" t="n">
-        <v>3.632</v>
+        <v>3.678</v>
       </c>
       <c r="K14" t="n">
-        <v>3.79</v>
+        <v>3.842</v>
       </c>
       <c r="L14" t="n">
-        <v>3.841</v>
+        <v>3.896</v>
       </c>
       <c r="M14" t="n">
-        <v>4.008</v>
+        <v>4.058</v>
       </c>
       <c r="N14" t="n">
-        <v>4.073</v>
+        <v>4.117</v>
       </c>
       <c r="O14" t="n">
-        <v>4.238</v>
+        <v>4.279</v>
       </c>
       <c r="P14" t="n">
-        <v>4.331</v>
+        <v>4.367</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.532</v>
+        <v>4.57</v>
       </c>
       <c r="R14" t="n">
-        <v>4.69</v>
+        <v>4.723</v>
       </c>
       <c r="S14" t="n">
-        <v>4.878</v>
+        <v>4.903</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.813</v>
+        <v>2.826</v>
       </c>
       <c r="G15" t="n">
-        <v>2.958</v>
+        <v>2.975</v>
       </c>
       <c r="H15" t="n">
-        <v>3.165</v>
+        <v>3.194</v>
       </c>
       <c r="I15" t="n">
-        <v>3.363</v>
+        <v>3.405</v>
       </c>
       <c r="J15" t="n">
-        <v>3.571</v>
+        <v>3.617</v>
       </c>
       <c r="K15" t="n">
-        <v>3.742</v>
+        <v>3.794</v>
       </c>
       <c r="L15" t="n">
-        <v>3.777</v>
+        <v>3.832</v>
       </c>
       <c r="M15" t="n">
-        <v>3.92</v>
+        <v>3.97</v>
       </c>
       <c r="N15" t="n">
-        <v>3.977</v>
+        <v>4.021</v>
       </c>
       <c r="O15" t="n">
-        <v>4.181</v>
+        <v>4.224</v>
       </c>
       <c r="P15" t="n">
-        <v>4.229</v>
+        <v>4.264</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.434</v>
+        <v>4.472</v>
       </c>
       <c r="R15" t="n">
-        <v>4.586</v>
+        <v>4.618</v>
       </c>
       <c r="S15" t="n">
-        <v>4.773</v>
+        <v>4.798</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.813</v>
+        <v>2.826</v>
       </c>
       <c r="G16" t="n">
-        <v>2.958</v>
+        <v>2.975</v>
       </c>
       <c r="H16" t="n">
-        <v>3.165</v>
+        <v>3.194</v>
       </c>
       <c r="I16" t="n">
-        <v>3.363</v>
+        <v>3.405</v>
       </c>
       <c r="J16" t="n">
-        <v>3.571</v>
+        <v>3.617</v>
       </c>
       <c r="K16" t="n">
-        <v>3.742</v>
+        <v>3.794</v>
       </c>
       <c r="L16" t="n">
-        <v>3.777</v>
+        <v>3.832</v>
       </c>
       <c r="M16" t="n">
-        <v>3.92</v>
+        <v>3.97</v>
       </c>
       <c r="N16" t="n">
-        <v>3.98</v>
+        <v>4.024</v>
       </c>
       <c r="O16" t="n">
-        <v>4.188</v>
+        <v>4.23</v>
       </c>
       <c r="P16" t="n">
-        <v>4.253</v>
+        <v>4.287</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.461</v>
+        <v>4.499</v>
       </c>
       <c r="R16" t="n">
-        <v>4.614</v>
+        <v>4.646</v>
       </c>
       <c r="S16" t="n">
-        <v>4.802</v>
+        <v>4.827</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.712</v>
+        <v>2.713</v>
       </c>
       <c r="G17" t="n">
-        <v>2.855</v>
+        <v>2.86</v>
       </c>
       <c r="H17" t="n">
-        <v>3.018</v>
+        <v>3.042</v>
       </c>
       <c r="I17" t="n">
-        <v>3.243</v>
+        <v>3.269</v>
       </c>
       <c r="J17" t="n">
-        <v>3.462</v>
+        <v>3.493</v>
       </c>
       <c r="K17" t="n">
-        <v>3.676</v>
+        <v>3.725</v>
       </c>
       <c r="L17" t="n">
-        <v>3.747</v>
+        <v>3.802</v>
       </c>
       <c r="M17" t="n">
-        <v>3.934</v>
+        <v>3.985</v>
       </c>
       <c r="N17" t="n">
-        <v>4.004</v>
+        <v>4.045</v>
       </c>
       <c r="O17" t="n">
-        <v>4.201</v>
+        <v>4.25</v>
       </c>
       <c r="P17" t="n">
-        <v>4.3</v>
+        <v>4.335</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.713</v>
+        <v>2.714</v>
       </c>
       <c r="G18" t="n">
-        <v>2.856</v>
+        <v>2.861</v>
       </c>
       <c r="H18" t="n">
-        <v>3.018</v>
+        <v>3.043</v>
       </c>
       <c r="I18" t="n">
-        <v>3.244</v>
+        <v>3.269</v>
       </c>
       <c r="J18" t="n">
-        <v>3.462</v>
+        <v>3.493</v>
       </c>
       <c r="K18" t="n">
-        <v>3.677</v>
+        <v>3.726</v>
       </c>
       <c r="L18" t="n">
-        <v>3.747</v>
+        <v>3.802</v>
       </c>
       <c r="M18" t="n">
-        <v>3.934</v>
+        <v>3.985</v>
       </c>
       <c r="N18" t="n">
-        <v>4.005</v>
+        <v>4.046</v>
       </c>
       <c r="O18" t="n">
-        <v>4.2</v>
+        <v>4.249</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.825</v>
+        <v>2.838</v>
       </c>
       <c r="G19" t="n">
-        <v>2.971</v>
+        <v>2.988</v>
       </c>
       <c r="H19" t="n">
-        <v>3.18</v>
+        <v>3.209</v>
       </c>
       <c r="I19" t="n">
-        <v>3.394</v>
+        <v>3.436</v>
       </c>
       <c r="J19" t="n">
-        <v>3.612</v>
+        <v>3.658</v>
       </c>
       <c r="K19" t="n">
-        <v>3.785</v>
+        <v>3.837</v>
       </c>
       <c r="L19" t="n">
-        <v>3.837</v>
+        <v>3.892</v>
       </c>
       <c r="M19" t="n">
-        <v>3.997</v>
+        <v>4.047</v>
       </c>
       <c r="N19" t="n">
-        <v>4.063</v>
+        <v>4.107</v>
       </c>
       <c r="O19" t="n">
-        <v>4.223</v>
+        <v>4.265</v>
       </c>
       <c r="P19" t="n">
-        <v>4.289</v>
+        <v>4.324</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.471</v>
+        <v>4.509</v>
       </c>
       <c r="R19" t="n">
-        <v>4.632</v>
+        <v>4.665</v>
       </c>
       <c r="S19" t="n">
-        <v>4.813</v>
+        <v>4.838</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.626</v>
+        <v>2.636</v>
       </c>
       <c r="G20" t="n">
-        <v>2.713</v>
+        <v>2.725</v>
       </c>
       <c r="H20" t="n">
-        <v>2.811</v>
+        <v>2.833</v>
       </c>
       <c r="I20" t="n">
-        <v>2.982</v>
+        <v>3.016</v>
       </c>
       <c r="J20" t="n">
-        <v>3.361</v>
+        <v>3.404</v>
       </c>
       <c r="K20" t="n">
-        <v>3.6</v>
+        <v>3.65</v>
       </c>
       <c r="L20" t="n">
-        <v>3.635</v>
+        <v>3.685</v>
       </c>
       <c r="M20" t="n">
-        <v>3.756</v>
+        <v>3.806</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.93</v>
+        <v>2.939</v>
       </c>
       <c r="G21" t="n">
-        <v>3.056</v>
+        <v>3.072</v>
       </c>
       <c r="H21" t="n">
-        <v>3.299</v>
+        <v>3.326</v>
       </c>
       <c r="I21" t="n">
-        <v>3.523</v>
+        <v>3.562</v>
       </c>
       <c r="J21" t="n">
-        <v>3.759</v>
+        <v>3.808</v>
       </c>
       <c r="K21" t="n">
-        <v>4.021</v>
+        <v>4.074</v>
       </c>
       <c r="L21" t="n">
-        <v>4.075</v>
+        <v>4.13</v>
       </c>
       <c r="M21" t="n">
-        <v>4.229</v>
+        <v>4.281</v>
       </c>
       <c r="N21" t="n">
-        <v>4.304</v>
+        <v>4.348</v>
       </c>
       <c r="O21" t="n">
-        <v>4.432</v>
+        <v>4.475</v>
       </c>
       <c r="P21" t="n">
-        <v>4.553</v>
+        <v>4.589</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.633</v>
+        <v>4.672</v>
       </c>
       <c r="R21" t="n">
-        <v>4.681</v>
+        <v>4.714</v>
       </c>
       <c r="S21" t="n">
-        <v>4.766</v>
+        <v>4.791</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.876</v>
+        <v>2.885</v>
       </c>
       <c r="G22" t="n">
-        <v>3.002</v>
+        <v>3.018</v>
       </c>
       <c r="H22" t="n">
-        <v>3.231</v>
+        <v>3.258</v>
       </c>
       <c r="I22" t="n">
-        <v>3.441</v>
+        <v>3.48</v>
       </c>
       <c r="J22" t="n">
-        <v>3.644</v>
+        <v>3.693</v>
       </c>
       <c r="K22" t="n">
-        <v>3.903</v>
+        <v>3.955</v>
       </c>
       <c r="L22" t="n">
-        <v>3.942</v>
+        <v>3.997</v>
       </c>
       <c r="M22" t="n">
-        <v>4.099</v>
+        <v>4.151</v>
       </c>
       <c r="N22" t="n">
-        <v>4.178</v>
+        <v>4.221</v>
       </c>
       <c r="O22" t="n">
-        <v>4.302</v>
+        <v>4.346</v>
       </c>
       <c r="P22" t="n">
-        <v>4.416</v>
+        <v>4.452</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.492</v>
+        <v>4.53</v>
       </c>
       <c r="R22" t="n">
-        <v>4.53</v>
+        <v>4.563</v>
       </c>
       <c r="S22" t="n">
-        <v>4.612</v>
+        <v>4.637</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.826</v>
+        <v>2.835</v>
       </c>
       <c r="G23" t="n">
-        <v>2.957</v>
+        <v>2.973</v>
       </c>
       <c r="H23" t="n">
-        <v>3.172</v>
+        <v>3.199</v>
       </c>
       <c r="I23" t="n">
-        <v>3.389</v>
+        <v>3.429</v>
       </c>
       <c r="J23" t="n">
-        <v>3.585</v>
+        <v>3.633</v>
       </c>
       <c r="K23" t="n">
-        <v>3.802</v>
+        <v>3.854</v>
       </c>
       <c r="L23" t="n">
-        <v>3.839</v>
+        <v>3.893</v>
       </c>
       <c r="M23" t="n">
-        <v>3.99</v>
+        <v>4.042</v>
       </c>
       <c r="N23" t="n">
-        <v>4.072</v>
+        <v>4.116</v>
       </c>
       <c r="O23" t="n">
-        <v>4.177</v>
+        <v>4.221</v>
       </c>
       <c r="P23" t="n">
-        <v>4.278</v>
+        <v>4.315</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.298</v>
+        <v>4.336</v>
       </c>
       <c r="R23" t="n">
-        <v>4.314</v>
+        <v>4.348</v>
       </c>
       <c r="S23" t="n">
-        <v>4.368</v>
+        <v>4.393</v>
       </c>
       <c r="T23" t="n">
-        <v>4.31</v>
+        <v>4.32</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.764</v>
+        <v>2.773</v>
       </c>
       <c r="G24" t="n">
-        <v>2.869</v>
+        <v>2.885</v>
       </c>
       <c r="H24" t="n">
-        <v>3.069</v>
+        <v>3.095</v>
       </c>
       <c r="I24" t="n">
-        <v>3.327</v>
+        <v>3.366</v>
       </c>
       <c r="J24" t="n">
-        <v>3.479</v>
+        <v>3.527</v>
       </c>
       <c r="K24" t="n">
-        <v>3.686</v>
+        <v>3.738</v>
       </c>
       <c r="L24" t="n">
-        <v>3.72</v>
+        <v>3.775</v>
       </c>
       <c r="M24" t="n">
-        <v>3.852</v>
+        <v>3.905</v>
       </c>
       <c r="N24" t="n">
-        <v>3.948</v>
+        <v>3.991</v>
       </c>
       <c r="O24" t="n">
-        <v>4.176</v>
+        <v>4.223</v>
       </c>
       <c r="P24" t="n">
-        <v>4.215</v>
+        <v>4.251</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.223</v>
+        <v>4.262</v>
       </c>
       <c r="R24" t="n">
-        <v>4.236</v>
+        <v>4.269</v>
       </c>
       <c r="S24" t="n">
-        <v>4.283</v>
+        <v>4.308</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.821</v>
+        <v>2.83</v>
       </c>
       <c r="G25" t="n">
-        <v>2.957</v>
+        <v>2.973</v>
       </c>
       <c r="H25" t="n">
-        <v>3.176</v>
+        <v>3.202</v>
       </c>
       <c r="I25" t="n">
-        <v>3.398</v>
+        <v>3.437</v>
       </c>
       <c r="J25" t="n">
-        <v>3.6</v>
+        <v>3.648</v>
       </c>
       <c r="K25" t="n">
-        <v>3.835</v>
+        <v>3.886</v>
       </c>
       <c r="L25" t="n">
-        <v>3.87</v>
+        <v>3.925</v>
       </c>
       <c r="M25" t="n">
-        <v>4.023</v>
+        <v>4.075</v>
       </c>
       <c r="N25" t="n">
-        <v>4.099</v>
+        <v>4.142</v>
       </c>
       <c r="O25" t="n">
-        <v>4.206</v>
+        <v>4.25</v>
       </c>
       <c r="P25" t="n">
-        <v>4.3</v>
+        <v>4.336</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.331</v>
+        <v>4.37</v>
       </c>
       <c r="R25" t="n">
+        <v>4.371</v>
+      </c>
+      <c r="S25" t="n">
+        <v>4.416</v>
+      </c>
+      <c r="T25" t="n">
         <v>4.338</v>
-      </c>
-      <c r="S25" t="n">
-        <v>4.391</v>
-      </c>
-      <c r="T25" t="n">
-        <v>4.328</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.098</v>
+        <v>3.113</v>
       </c>
       <c r="G26" t="n">
-        <v>3.279</v>
+        <v>3.299</v>
       </c>
       <c r="H26" t="n">
-        <v>3.604</v>
+        <v>3.636</v>
       </c>
       <c r="I26" t="n">
-        <v>3.864</v>
+        <v>3.905</v>
       </c>
       <c r="J26" t="n">
-        <v>4.221</v>
+        <v>4.273</v>
       </c>
       <c r="K26" t="n">
-        <v>4.642</v>
+        <v>4.695</v>
       </c>
       <c r="L26" t="n">
-        <v>4.751</v>
+        <v>4.806</v>
       </c>
       <c r="M26" t="n">
-        <v>4.949</v>
+        <v>4.999</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.274</v>
+        <v>5.307</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.915</v>
+        <v>2.929</v>
       </c>
       <c r="G27" t="n">
-        <v>3.048</v>
+        <v>3.065</v>
       </c>
       <c r="H27" t="n">
-        <v>3.275</v>
+        <v>3.305</v>
       </c>
       <c r="I27" t="n">
-        <v>3.499</v>
+        <v>3.541</v>
       </c>
       <c r="J27" t="n">
-        <v>3.739</v>
+        <v>3.786</v>
       </c>
       <c r="K27" t="n">
-        <v>3.963</v>
+        <v>4.016</v>
       </c>
       <c r="L27" t="n">
-        <v>4.022</v>
+        <v>4.077</v>
       </c>
       <c r="M27" t="n">
-        <v>4.168</v>
+        <v>4.218</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.37</v>
+        <v>4.408</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.018</v>
+        <v>3.032</v>
       </c>
       <c r="G28" t="n">
-        <v>3.159</v>
+        <v>3.176</v>
       </c>
       <c r="H28" t="n">
-        <v>3.401</v>
+        <v>3.431</v>
       </c>
       <c r="I28" t="n">
-        <v>3.636</v>
+        <v>3.678</v>
       </c>
       <c r="J28" t="n">
-        <v>3.912</v>
+        <v>3.959</v>
       </c>
       <c r="K28" t="n">
-        <v>4.156</v>
+        <v>4.209</v>
       </c>
       <c r="L28" t="n">
-        <v>4.225</v>
+        <v>4.279</v>
       </c>
       <c r="M28" t="n">
-        <v>4.38</v>
+        <v>4.429</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.662</v>
+        <v>4.7</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.865</v>
+        <v>2.879</v>
       </c>
       <c r="G29" t="n">
-        <v>2.996</v>
+        <v>3.013</v>
       </c>
       <c r="H29" t="n">
-        <v>3.214</v>
+        <v>3.244</v>
       </c>
       <c r="I29" t="n">
-        <v>3.427</v>
+        <v>3.469</v>
       </c>
       <c r="J29" t="n">
-        <v>3.651</v>
+        <v>3.698</v>
       </c>
       <c r="K29" t="n">
-        <v>3.859</v>
+        <v>3.912</v>
       </c>
       <c r="L29" t="n">
-        <v>3.907</v>
+        <v>3.962</v>
       </c>
       <c r="M29" t="n">
-        <v>4.031</v>
+        <v>4.081</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.241</v>
+        <v>4.28</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.14</v>
+        <v>3.155</v>
       </c>
       <c r="G30" t="n">
-        <v>3.256</v>
+        <v>3.276</v>
       </c>
       <c r="H30" t="n">
-        <v>3.537</v>
+        <v>3.57</v>
       </c>
       <c r="I30" t="n">
-        <v>3.788</v>
+        <v>3.828</v>
       </c>
       <c r="J30" t="n">
-        <v>4.087</v>
+        <v>4.137</v>
       </c>
       <c r="K30" t="n">
-        <v>4.44</v>
+        <v>4.493</v>
       </c>
       <c r="L30" t="n">
-        <v>4.53</v>
+        <v>4.584</v>
       </c>
       <c r="M30" t="n">
-        <v>4.717</v>
+        <v>4.767</v>
       </c>
       <c r="N30" t="n">
-        <v>4.896</v>
+        <v>4.938</v>
       </c>
       <c r="O30" t="n">
-        <v>5.225</v>
+        <v>5.258</v>
       </c>
       <c r="P30" t="n">
-        <v>5.443</v>
+        <v>5.478</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.167</v>
+        <v>6.203</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.469</v>
+        <v>3.484</v>
       </c>
       <c r="G31" t="n">
-        <v>3.621</v>
+        <v>3.641</v>
       </c>
       <c r="H31" t="n">
-        <v>3.951</v>
+        <v>3.985</v>
       </c>
       <c r="I31" t="n">
-        <v>4.218</v>
+        <v>4.258</v>
       </c>
       <c r="J31" t="n">
-        <v>4.578</v>
+        <v>4.628</v>
       </c>
       <c r="K31" t="n">
-        <v>4.973</v>
+        <v>5.026</v>
       </c>
       <c r="L31" t="n">
-        <v>5.142</v>
+        <v>5.197</v>
       </c>
       <c r="M31" t="n">
-        <v>5.448</v>
+        <v>5.498</v>
       </c>
       <c r="N31" t="n">
-        <v>5.755</v>
+        <v>5.797</v>
       </c>
       <c r="O31" t="n">
-        <v>6.261</v>
+        <v>6.294</v>
       </c>
       <c r="P31" t="n">
-        <v>6.431</v>
+        <v>6.467</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.141</v>
+        <v>7.176</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.239</v>
+        <v>3.254</v>
       </c>
       <c r="G32" t="n">
-        <v>3.374</v>
+        <v>3.394</v>
       </c>
       <c r="H32" t="n">
-        <v>3.681</v>
+        <v>3.714</v>
       </c>
       <c r="I32" t="n">
-        <v>3.947</v>
+        <v>3.987</v>
       </c>
       <c r="J32" t="n">
-        <v>4.265</v>
+        <v>4.315</v>
       </c>
       <c r="K32" t="n">
-        <v>4.625</v>
+        <v>4.678</v>
       </c>
       <c r="L32" t="n">
-        <v>4.734</v>
+        <v>4.789</v>
       </c>
       <c r="M32" t="n">
-        <v>4.99</v>
+        <v>5.04</v>
       </c>
       <c r="N32" t="n">
-        <v>5.257</v>
+        <v>5.298</v>
       </c>
       <c r="O32" t="n">
-        <v>5.67</v>
+        <v>5.703</v>
       </c>
       <c r="P32" t="n">
-        <v>5.903</v>
+        <v>5.938</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.628</v>
+        <v>6.664</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.004</v>
+        <v>3.021</v>
       </c>
       <c r="G33" t="n">
-        <v>3.121</v>
+        <v>3.142</v>
       </c>
       <c r="H33" t="n">
-        <v>3.354</v>
+        <v>3.388</v>
       </c>
       <c r="I33" t="n">
-        <v>3.572</v>
+        <v>3.612</v>
       </c>
       <c r="J33" t="n">
-        <v>3.793</v>
+        <v>3.844</v>
       </c>
       <c r="K33" t="n">
-        <v>4.082</v>
+        <v>4.135</v>
       </c>
       <c r="L33" t="n">
-        <v>4.131</v>
+        <v>4.186</v>
       </c>
       <c r="M33" t="n">
-        <v>4.243</v>
+        <v>4.293</v>
       </c>
       <c r="N33" t="n">
-        <v>4.286</v>
+        <v>4.327</v>
       </c>
       <c r="O33" t="n">
-        <v>4.379</v>
+        <v>4.412</v>
       </c>
       <c r="P33" t="n">
-        <v>4.475</v>
+        <v>4.511</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.884</v>
+        <v>4.919</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.064</v>
+        <v>3.081</v>
       </c>
       <c r="G34" t="n">
-        <v>3.174</v>
+        <v>3.195</v>
       </c>
       <c r="H34" t="n">
-        <v>3.416</v>
+        <v>3.45</v>
       </c>
       <c r="I34" t="n">
-        <v>3.64</v>
+        <v>3.68</v>
       </c>
       <c r="J34" t="n">
-        <v>3.865</v>
+        <v>3.915</v>
       </c>
       <c r="K34" t="n">
-        <v>4.159</v>
+        <v>4.212</v>
       </c>
       <c r="L34" t="n">
-        <v>4.21</v>
+        <v>4.265</v>
       </c>
       <c r="M34" t="n">
-        <v>4.333</v>
+        <v>4.383</v>
       </c>
       <c r="N34" t="n">
-        <v>4.39</v>
+        <v>4.431</v>
       </c>
       <c r="O34" t="n">
-        <v>4.548</v>
+        <v>4.581</v>
       </c>
       <c r="P34" t="n">
-        <v>4.77</v>
+        <v>4.805</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.585</v>
+        <v>5.62</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.038</v>
+        <v>3.055</v>
       </c>
       <c r="G35" t="n">
-        <v>3.148</v>
+        <v>3.169</v>
       </c>
       <c r="H35" t="n">
-        <v>3.384</v>
+        <v>3.418</v>
       </c>
       <c r="I35" t="n">
-        <v>3.607</v>
+        <v>3.647</v>
       </c>
       <c r="J35" t="n">
-        <v>3.834</v>
+        <v>3.883</v>
       </c>
       <c r="K35" t="n">
-        <v>4.113</v>
+        <v>4.165</v>
       </c>
       <c r="L35" t="n">
-        <v>4.165</v>
+        <v>4.22</v>
       </c>
       <c r="M35" t="n">
-        <v>4.28</v>
+        <v>4.33</v>
       </c>
       <c r="N35" t="n">
-        <v>4.326</v>
+        <v>4.368</v>
       </c>
       <c r="O35" t="n">
-        <v>4.445</v>
+        <v>4.478</v>
       </c>
       <c r="P35" t="n">
-        <v>4.572</v>
+        <v>4.608</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.221</v>
+        <v>5.256</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.933</v>
+        <v>2.948</v>
       </c>
       <c r="G36" t="n">
-        <v>3.039</v>
+        <v>3.059</v>
       </c>
       <c r="H36" t="n">
-        <v>3.265</v>
+        <v>3.299</v>
       </c>
       <c r="I36" t="n">
-        <v>3.488</v>
+        <v>3.528</v>
       </c>
       <c r="J36" t="n">
-        <v>3.732</v>
+        <v>3.782</v>
       </c>
       <c r="K36" t="n">
-        <v>4.008</v>
+        <v>4.061</v>
       </c>
       <c r="L36" t="n">
-        <v>4.058</v>
+        <v>4.113</v>
       </c>
       <c r="M36" t="n">
-        <v>4.144</v>
+        <v>4.194</v>
       </c>
       <c r="N36" t="n">
-        <v>4.189</v>
+        <v>4.23</v>
       </c>
       <c r="O36" t="n">
-        <v>4.287</v>
+        <v>4.32</v>
       </c>
       <c r="P36" t="n">
-        <v>4.373</v>
+        <v>4.409</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.601</v>
+        <v>4.636</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.812</v>
+        <v>3.827</v>
       </c>
       <c r="G37" t="n">
-        <v>4.314</v>
+        <v>4.334</v>
       </c>
       <c r="H37" t="n">
-        <v>4.924</v>
+        <v>4.957</v>
       </c>
       <c r="I37" t="n">
-        <v>5.278</v>
+        <v>5.319</v>
       </c>
       <c r="J37" t="n">
-        <v>6.068</v>
+        <v>6.119</v>
       </c>
       <c r="K37" t="n">
-        <v>7.013</v>
+        <v>7.066</v>
       </c>
       <c r="L37" t="n">
-        <v>7.342</v>
+        <v>7.397</v>
       </c>
       <c r="M37" t="n">
-        <v>7.72</v>
+        <v>7.77</v>
       </c>
       <c r="N37" t="n">
-        <v>7.906</v>
+        <v>7.948</v>
       </c>
       <c r="O37" t="n">
-        <v>8.140000000000001</v>
+        <v>8.173</v>
       </c>
       <c r="P37" t="n">
-        <v>8.231</v>
+        <v>8.266</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.629</v>
+        <v>8.666</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.872</v>
+        <v>4.888</v>
       </c>
       <c r="G38" t="n">
-        <v>5.629</v>
+        <v>5.649</v>
       </c>
       <c r="H38" t="n">
-        <v>6.45</v>
+        <v>6.483</v>
       </c>
       <c r="I38" t="n">
-        <v>6.961</v>
+        <v>7.002</v>
       </c>
       <c r="J38" t="n">
-        <v>8.012</v>
+        <v>8.063000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.135</v>
+        <v>9.188000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.625</v>
+        <v>9.679</v>
       </c>
       <c r="M38" t="n">
-        <v>10.132</v>
+        <v>10.181</v>
       </c>
       <c r="N38" t="n">
-        <v>10.325</v>
+        <v>10.367</v>
       </c>
       <c r="O38" t="n">
-        <v>10.54</v>
+        <v>10.573</v>
       </c>
       <c r="P38" t="n">
-        <v>10.629</v>
+        <v>10.664</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.08</v>
+        <v>11.117</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.193</v>
+        <v>4.209</v>
       </c>
       <c r="G39" t="n">
-        <v>4.827</v>
+        <v>4.847</v>
       </c>
       <c r="H39" t="n">
-        <v>5.515</v>
+        <v>5.548</v>
       </c>
       <c r="I39" t="n">
-        <v>5.965</v>
+        <v>6.006</v>
       </c>
       <c r="J39" t="n">
-        <v>6.885</v>
+        <v>6.936</v>
       </c>
       <c r="K39" t="n">
-        <v>7.968</v>
+        <v>8.021000000000001</v>
       </c>
       <c r="L39" t="n">
-        <v>8.380000000000001</v>
+        <v>8.435</v>
       </c>
       <c r="M39" t="n">
-        <v>8.768000000000001</v>
+        <v>8.818</v>
       </c>
       <c r="N39" t="n">
-        <v>8.952999999999999</v>
+        <v>8.994</v>
       </c>
       <c r="O39" t="n">
-        <v>9.19</v>
+        <v>9.224</v>
       </c>
       <c r="P39" t="n">
-        <v>9.282999999999999</v>
+        <v>9.318</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.725</v>
+        <v>9.762</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.332</v>
+        <v>3.347</v>
       </c>
       <c r="G40" t="n">
-        <v>3.494</v>
+        <v>3.514</v>
       </c>
       <c r="H40" t="n">
-        <v>3.796</v>
+        <v>3.829</v>
       </c>
       <c r="I40" t="n">
-        <v>4.062</v>
+        <v>4.102</v>
       </c>
       <c r="J40" t="n">
-        <v>4.378</v>
+        <v>4.428</v>
       </c>
       <c r="K40" t="n">
-        <v>4.746</v>
+        <v>4.799</v>
       </c>
       <c r="L40" t="n">
-        <v>4.854</v>
+        <v>4.909</v>
       </c>
       <c r="M40" t="n">
-        <v>5.06</v>
+        <v>5.11</v>
       </c>
       <c r="N40" t="n">
-        <v>5.254</v>
+        <v>5.295</v>
       </c>
       <c r="O40" t="n">
-        <v>5.604</v>
+        <v>5.637</v>
       </c>
       <c r="P40" t="n">
-        <v>5.864</v>
+        <v>5.899</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.618</v>
+        <v>6.654</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.718</v>
+        <v>3.733</v>
       </c>
       <c r="G41" t="n">
-        <v>3.923</v>
+        <v>3.943</v>
       </c>
       <c r="H41" t="n">
-        <v>4.281</v>
+        <v>4.314</v>
       </c>
       <c r="I41" t="n">
-        <v>4.566</v>
+        <v>4.606</v>
       </c>
       <c r="J41" t="n">
-        <v>4.933</v>
+        <v>4.983</v>
       </c>
       <c r="K41" t="n">
-        <v>5.346</v>
+        <v>5.4</v>
       </c>
       <c r="L41" t="n">
-        <v>5.533</v>
+        <v>5.588</v>
       </c>
       <c r="M41" t="n">
-        <v>5.863</v>
+        <v>5.913</v>
       </c>
       <c r="N41" t="n">
-        <v>6.185</v>
+        <v>6.226</v>
       </c>
       <c r="O41" t="n">
-        <v>6.719</v>
+        <v>6.752</v>
       </c>
       <c r="P41" t="n">
-        <v>6.923</v>
+        <v>6.959</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.665</v>
+        <v>7.701</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.453</v>
+        <v>3.468</v>
       </c>
       <c r="G42" t="n">
-        <v>3.643</v>
+        <v>3.663</v>
       </c>
       <c r="H42" t="n">
-        <v>3.972</v>
+        <v>4.005</v>
       </c>
       <c r="I42" t="n">
-        <v>4.25</v>
+        <v>4.29</v>
       </c>
       <c r="J42" t="n">
-        <v>4.581</v>
+        <v>4.631</v>
       </c>
       <c r="K42" t="n">
-        <v>4.967</v>
+        <v>5.02</v>
       </c>
       <c r="L42" t="n">
-        <v>5.09</v>
+        <v>5.145</v>
       </c>
       <c r="M42" t="n">
-        <v>5.367</v>
+        <v>5.417</v>
       </c>
       <c r="N42" t="n">
-        <v>5.669</v>
+        <v>5.71</v>
       </c>
       <c r="O42" t="n">
-        <v>6.096</v>
+        <v>6.129</v>
       </c>
       <c r="P42" t="n">
-        <v>6.366</v>
+        <v>6.401</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.131</v>
+        <v>7.166</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.152</v>
+        <v>3.169</v>
       </c>
       <c r="G43" t="n">
-        <v>3.304</v>
+        <v>3.325</v>
       </c>
       <c r="H43" t="n">
-        <v>3.555</v>
+        <v>3.589</v>
       </c>
       <c r="I43" t="n">
-        <v>3.781</v>
+        <v>3.821</v>
       </c>
       <c r="J43" t="n">
-        <v>4.021</v>
+        <v>4.071</v>
       </c>
       <c r="K43" t="n">
-        <v>4.314</v>
+        <v>4.367</v>
       </c>
       <c r="L43" t="n">
-        <v>4.373</v>
+        <v>4.428</v>
       </c>
       <c r="M43" t="n">
-        <v>4.498</v>
+        <v>4.548</v>
       </c>
       <c r="N43" t="n">
-        <v>4.555</v>
+        <v>4.596</v>
       </c>
       <c r="O43" t="n">
-        <v>4.692</v>
+        <v>4.725</v>
       </c>
       <c r="P43" t="n">
-        <v>4.841</v>
+        <v>4.876</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.494</v>
+        <v>5.529</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.011</v>
+        <v>3.026</v>
       </c>
       <c r="G44" t="n">
-        <v>3.148</v>
+        <v>3.168</v>
       </c>
       <c r="H44" t="n">
-        <v>3.389</v>
+        <v>3.422</v>
       </c>
       <c r="I44" t="n">
-        <v>3.615</v>
+        <v>3.655</v>
       </c>
       <c r="J44" t="n">
-        <v>3.873</v>
+        <v>3.923</v>
       </c>
       <c r="K44" t="n">
-        <v>4.16</v>
+        <v>4.212</v>
       </c>
       <c r="L44" t="n">
-        <v>4.219</v>
+        <v>4.273</v>
       </c>
       <c r="M44" t="n">
-        <v>4.314</v>
+        <v>4.364</v>
       </c>
       <c r="N44" t="n">
-        <v>4.371</v>
+        <v>4.412</v>
       </c>
       <c r="O44" t="n">
-        <v>4.488</v>
+        <v>4.521</v>
       </c>
       <c r="P44" t="n">
-        <v>4.603</v>
+        <v>4.639</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.865</v>
+        <v>4.9</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-05-29 ~ 2026-05-29
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -555,37 +555,37 @@
         <v>3.279</v>
       </c>
       <c r="G2" t="n">
-        <v>3.55</v>
+        <v>3.553</v>
       </c>
       <c r="H2" t="n">
-        <v>3.839</v>
+        <v>3.841</v>
       </c>
       <c r="I2" t="n">
-        <v>4.058</v>
+        <v>4.055</v>
       </c>
       <c r="J2" t="n">
-        <v>4.317</v>
+        <v>4.313</v>
       </c>
       <c r="K2" t="n">
-        <v>4.731</v>
+        <v>4.72</v>
       </c>
       <c r="L2" t="n">
-        <v>4.907</v>
+        <v>4.885</v>
       </c>
       <c r="M2" t="n">
-        <v>5.219</v>
+        <v>5.174</v>
       </c>
       <c r="N2" t="n">
-        <v>5.5</v>
+        <v>5.451</v>
       </c>
       <c r="O2" t="n">
-        <v>5.773</v>
+        <v>5.698</v>
       </c>
       <c r="P2" t="n">
-        <v>6.002</v>
+        <v>5.919</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.606</v>
+        <v>6.525</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -628,37 +628,37 @@
         <v>4.3</v>
       </c>
       <c r="G3" t="n">
-        <v>4.753</v>
+        <v>4.756</v>
       </c>
       <c r="H3" t="n">
-        <v>5.074</v>
+        <v>5.077</v>
       </c>
       <c r="I3" t="n">
-        <v>5.287</v>
+        <v>5.284</v>
       </c>
       <c r="J3" t="n">
-        <v>5.563</v>
+        <v>5.559</v>
       </c>
       <c r="K3" t="n">
-        <v>6.047</v>
+        <v>6.036</v>
       </c>
       <c r="L3" t="n">
-        <v>6.293</v>
+        <v>6.271</v>
       </c>
       <c r="M3" t="n">
-        <v>6.635</v>
+        <v>6.591</v>
       </c>
       <c r="N3" t="n">
-        <v>6.859</v>
+        <v>6.811</v>
       </c>
       <c r="O3" t="n">
-        <v>7.083</v>
+        <v>7.008</v>
       </c>
       <c r="P3" t="n">
-        <v>7.182</v>
+        <v>7.098</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.674</v>
+        <v>7.592</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -701,37 +701,37 @@
         <v>3.793</v>
       </c>
       <c r="G4" t="n">
-        <v>4.134</v>
+        <v>4.137</v>
       </c>
       <c r="H4" t="n">
-        <v>4.484</v>
+        <v>4.487</v>
       </c>
       <c r="I4" t="n">
-        <v>4.729</v>
+        <v>4.726</v>
       </c>
       <c r="J4" t="n">
-        <v>5.009</v>
+        <v>5.005</v>
       </c>
       <c r="K4" t="n">
-        <v>5.486</v>
+        <v>5.474</v>
       </c>
       <c r="L4" t="n">
-        <v>5.662</v>
+        <v>5.639</v>
       </c>
       <c r="M4" t="n">
-        <v>5.993</v>
+        <v>5.949</v>
       </c>
       <c r="N4" t="n">
-        <v>6.187</v>
+        <v>6.139</v>
       </c>
       <c r="O4" t="n">
-        <v>6.434</v>
+        <v>6.359</v>
       </c>
       <c r="P4" t="n">
-        <v>6.532</v>
+        <v>6.45</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.027</v>
+        <v>6.947</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -774,37 +774,37 @@
         <v>2.976</v>
       </c>
       <c r="G5" t="n">
-        <v>3.091</v>
+        <v>3.094</v>
       </c>
       <c r="H5" t="n">
-        <v>3.345</v>
+        <v>3.348</v>
       </c>
       <c r="I5" t="n">
-        <v>3.631</v>
+        <v>3.627</v>
       </c>
       <c r="J5" t="n">
-        <v>3.873</v>
+        <v>3.87</v>
       </c>
       <c r="K5" t="n">
+        <v>4.123</v>
+      </c>
+      <c r="L5" t="n">
         <v>4.132</v>
       </c>
-      <c r="L5" t="n">
-        <v>4.154</v>
-      </c>
       <c r="M5" t="n">
-        <v>4.277</v>
+        <v>4.233</v>
       </c>
       <c r="N5" t="n">
-        <v>4.312</v>
+        <v>4.264</v>
       </c>
       <c r="O5" t="n">
-        <v>4.372</v>
+        <v>4.297</v>
       </c>
       <c r="P5" t="n">
-        <v>4.671</v>
+        <v>4.588</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.518</v>
+        <v>5.438</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -847,37 +847,37 @@
         <v>3.017</v>
       </c>
       <c r="G6" t="n">
-        <v>3.147</v>
+        <v>3.15</v>
       </c>
       <c r="H6" t="n">
-        <v>3.414</v>
+        <v>3.417</v>
       </c>
       <c r="I6" t="n">
-        <v>3.715</v>
+        <v>3.711</v>
       </c>
       <c r="J6" t="n">
-        <v>3.965</v>
+        <v>3.961</v>
       </c>
       <c r="K6" t="n">
-        <v>4.248</v>
+        <v>4.237</v>
       </c>
       <c r="L6" t="n">
-        <v>4.273</v>
+        <v>4.251</v>
       </c>
       <c r="M6" t="n">
-        <v>4.434</v>
+        <v>4.389</v>
       </c>
       <c r="N6" t="n">
-        <v>4.479</v>
+        <v>4.431</v>
       </c>
       <c r="O6" t="n">
-        <v>4.639</v>
+        <v>4.564</v>
       </c>
       <c r="P6" t="n">
-        <v>5.103</v>
+        <v>5.02</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.914</v>
+        <v>5.834</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -920,37 +920,37 @@
         <v>2.997</v>
       </c>
       <c r="G7" t="n">
-        <v>3.11</v>
+        <v>3.113</v>
       </c>
       <c r="H7" t="n">
-        <v>3.361</v>
+        <v>3.364</v>
       </c>
       <c r="I7" t="n">
-        <v>3.65</v>
+        <v>3.646</v>
       </c>
       <c r="J7" t="n">
-        <v>3.896</v>
+        <v>3.893</v>
       </c>
       <c r="K7" t="n">
-        <v>4.159</v>
+        <v>4.15</v>
       </c>
       <c r="L7" t="n">
-        <v>4.18</v>
+        <v>4.158</v>
       </c>
       <c r="M7" t="n">
-        <v>4.337</v>
+        <v>4.293</v>
       </c>
       <c r="N7" t="n">
-        <v>4.371</v>
+        <v>4.323</v>
       </c>
       <c r="O7" t="n">
-        <v>4.536</v>
+        <v>4.461</v>
       </c>
       <c r="P7" t="n">
-        <v>4.887</v>
+        <v>4.804</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.682</v>
+        <v>5.601</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -993,37 +993,37 @@
         <v>5.412</v>
       </c>
       <c r="G8" t="n">
-        <v>6.053</v>
+        <v>6.056</v>
       </c>
       <c r="H8" t="n">
-        <v>6.523</v>
+        <v>6.525</v>
       </c>
       <c r="I8" t="n">
-        <v>6.813</v>
+        <v>6.81</v>
       </c>
       <c r="J8" t="n">
-        <v>7.156</v>
+        <v>7.152</v>
       </c>
       <c r="K8" t="n">
-        <v>7.921</v>
+        <v>7.909</v>
       </c>
       <c r="L8" t="n">
-        <v>8.250999999999999</v>
+        <v>8.228999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.625999999999999</v>
+        <v>8.581</v>
       </c>
       <c r="N8" t="n">
-        <v>8.782999999999999</v>
+        <v>8.734999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.092000000000001</v>
+        <v>9.016999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>9.292999999999999</v>
+        <v>9.211</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.983000000000001</v>
+        <v>9.903</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.637</v>
+        <v>2.635</v>
       </c>
       <c r="G9" t="n">
-        <v>2.737</v>
+        <v>2.735</v>
       </c>
       <c r="H9" t="n">
-        <v>2.938</v>
+        <v>2.939</v>
       </c>
       <c r="I9" t="n">
-        <v>3.182</v>
+        <v>3.177</v>
       </c>
       <c r="J9" t="n">
-        <v>3.391</v>
+        <v>3.383</v>
       </c>
       <c r="K9" t="n">
-        <v>3.613</v>
+        <v>3.627</v>
       </c>
       <c r="L9" t="n">
-        <v>3.667</v>
+        <v>3.644</v>
       </c>
       <c r="M9" t="n">
-        <v>3.767</v>
+        <v>3.722</v>
       </c>
       <c r="N9" t="n">
-        <v>3.921</v>
+        <v>3.873</v>
       </c>
       <c r="O9" t="n">
-        <v>3.99</v>
+        <v>3.915</v>
       </c>
       <c r="P9" t="n">
-        <v>4.103</v>
+        <v>4.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.145</v>
+        <v>4.065</v>
       </c>
       <c r="R9" t="n">
-        <v>4.168</v>
+        <v>4.074</v>
       </c>
       <c r="S9" t="n">
-        <v>4.185</v>
+        <v>4.078</v>
       </c>
       <c r="T9" t="n">
-        <v>4.114</v>
+        <v>3.996</v>
       </c>
       <c r="U9" t="n">
-        <v>3.993</v>
+        <v>3.894</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.657</v>
+        <v>2.656</v>
       </c>
       <c r="G10" t="n">
-        <v>2.774</v>
+        <v>2.773</v>
       </c>
       <c r="H10" t="n">
-        <v>2.95</v>
+        <v>2.952</v>
       </c>
       <c r="I10" t="n">
-        <v>3.187</v>
+        <v>3.182</v>
       </c>
       <c r="J10" t="n">
-        <v>3.418</v>
+        <v>3.41</v>
       </c>
       <c r="K10" t="n">
-        <v>3.646</v>
+        <v>3.655</v>
       </c>
       <c r="L10" t="n">
-        <v>3.718</v>
+        <v>3.696</v>
       </c>
       <c r="M10" t="n">
-        <v>3.861</v>
+        <v>3.817</v>
       </c>
       <c r="N10" t="n">
-        <v>3.942</v>
+        <v>3.893</v>
       </c>
       <c r="O10" t="n">
-        <v>4.228</v>
+        <v>4.154</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.467</v>
+        <v>2.466</v>
       </c>
       <c r="G11" t="n">
-        <v>2.581</v>
+        <v>2.58</v>
       </c>
       <c r="H11" t="n">
-        <v>2.773</v>
+        <v>2.775</v>
       </c>
       <c r="I11" t="n">
-        <v>2.991</v>
+        <v>2.986</v>
       </c>
       <c r="J11" t="n">
-        <v>3.215</v>
+        <v>3.207</v>
       </c>
       <c r="K11" t="n">
-        <v>3.433</v>
+        <v>3.442</v>
       </c>
       <c r="L11" t="n">
-        <v>3.515</v>
+        <v>3.493</v>
       </c>
       <c r="M11" t="n">
-        <v>3.669</v>
+        <v>3.625</v>
       </c>
       <c r="N11" t="n">
-        <v>3.749</v>
+        <v>3.7</v>
       </c>
       <c r="O11" t="n">
-        <v>3.994</v>
+        <v>3.92</v>
       </c>
       <c r="P11" t="n">
-        <v>4.054</v>
+        <v>3.971</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.346</v>
+        <v>4.266</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.276</v>
+        <v>3.277</v>
       </c>
       <c r="G12" t="n">
-        <v>3.505</v>
+        <v>3.512</v>
       </c>
       <c r="H12" t="n">
-        <v>3.753</v>
+        <v>3.76</v>
       </c>
       <c r="I12" t="n">
-        <v>4.021</v>
+        <v>4.02</v>
       </c>
       <c r="J12" t="n">
         <v>4.3</v>
       </c>
       <c r="K12" t="n">
-        <v>4.521</v>
+        <v>4.514</v>
       </c>
       <c r="L12" t="n">
-        <v>4.584</v>
+        <v>4.56</v>
       </c>
       <c r="M12" t="n">
-        <v>4.744</v>
+        <v>4.698</v>
       </c>
       <c r="N12" t="n">
-        <v>4.81</v>
+        <v>4.763</v>
       </c>
       <c r="O12" t="n">
-        <v>4.993</v>
+        <v>4.92</v>
       </c>
       <c r="P12" t="n">
-        <v>5.139</v>
+        <v>5.056</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.46</v>
+        <v>5.379</v>
       </c>
       <c r="R12" t="n">
-        <v>5.659</v>
+        <v>5.565</v>
       </c>
       <c r="S12" t="n">
-        <v>5.888</v>
+        <v>5.781</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.03</v>
+        <v>3.031</v>
       </c>
       <c r="G13" t="n">
-        <v>3.195</v>
+        <v>3.202</v>
       </c>
       <c r="H13" t="n">
-        <v>3.42</v>
+        <v>3.427</v>
       </c>
       <c r="I13" t="n">
         <v>3.668</v>
       </c>
       <c r="J13" t="n">
-        <v>3.937</v>
+        <v>3.936</v>
       </c>
       <c r="K13" t="n">
-        <v>4.154</v>
+        <v>4.148</v>
       </c>
       <c r="L13" t="n">
-        <v>4.223</v>
+        <v>4.199</v>
       </c>
       <c r="M13" t="n">
-        <v>4.371</v>
+        <v>4.326</v>
       </c>
       <c r="N13" t="n">
-        <v>4.438</v>
+        <v>4.391</v>
       </c>
       <c r="O13" t="n">
-        <v>4.621</v>
+        <v>4.548</v>
       </c>
       <c r="P13" t="n">
-        <v>4.731</v>
+        <v>4.647</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.981</v>
+        <v>4.9</v>
       </c>
       <c r="R13" t="n">
-        <v>5.209</v>
+        <v>5.114</v>
       </c>
       <c r="S13" t="n">
-        <v>5.45</v>
+        <v>5.344</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,13 +1428,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.849</v>
+        <v>2.85</v>
       </c>
       <c r="G14" t="n">
-        <v>3.001</v>
+        <v>3.008</v>
       </c>
       <c r="H14" t="n">
-        <v>3.223</v>
+        <v>3.23</v>
       </c>
       <c r="I14" t="n">
         <v>3.453</v>
@@ -1443,31 +1443,31 @@
         <v>3.678</v>
       </c>
       <c r="K14" t="n">
-        <v>3.842</v>
+        <v>3.836</v>
       </c>
       <c r="L14" t="n">
-        <v>3.896</v>
+        <v>3.872</v>
       </c>
       <c r="M14" t="n">
-        <v>4.058</v>
+        <v>4.012</v>
       </c>
       <c r="N14" t="n">
-        <v>4.117</v>
+        <v>4.07</v>
       </c>
       <c r="O14" t="n">
-        <v>4.279</v>
+        <v>4.207</v>
       </c>
       <c r="P14" t="n">
-        <v>4.367</v>
+        <v>4.283</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.57</v>
+        <v>4.49</v>
       </c>
       <c r="R14" t="n">
-        <v>4.723</v>
+        <v>4.629</v>
       </c>
       <c r="S14" t="n">
-        <v>4.903</v>
+        <v>4.796</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.826</v>
+        <v>2.827</v>
       </c>
       <c r="G15" t="n">
-        <v>2.975</v>
+        <v>2.982</v>
       </c>
       <c r="H15" t="n">
-        <v>3.194</v>
+        <v>3.201</v>
       </c>
       <c r="I15" t="n">
-        <v>3.405</v>
+        <v>3.404</v>
       </c>
       <c r="J15" t="n">
         <v>3.617</v>
       </c>
       <c r="K15" t="n">
-        <v>3.794</v>
+        <v>3.788</v>
       </c>
       <c r="L15" t="n">
-        <v>3.832</v>
+        <v>3.809</v>
       </c>
       <c r="M15" t="n">
-        <v>3.97</v>
+        <v>3.925</v>
       </c>
       <c r="N15" t="n">
-        <v>4.021</v>
+        <v>3.974</v>
       </c>
       <c r="O15" t="n">
-        <v>4.224</v>
+        <v>4.151</v>
       </c>
       <c r="P15" t="n">
-        <v>4.264</v>
+        <v>4.181</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.472</v>
+        <v>4.392</v>
       </c>
       <c r="R15" t="n">
-        <v>4.618</v>
+        <v>4.523</v>
       </c>
       <c r="S15" t="n">
-        <v>4.798</v>
+        <v>4.691</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.826</v>
+        <v>2.827</v>
       </c>
       <c r="G16" t="n">
-        <v>2.975</v>
+        <v>2.982</v>
       </c>
       <c r="H16" t="n">
-        <v>3.194</v>
+        <v>3.201</v>
       </c>
       <c r="I16" t="n">
-        <v>3.405</v>
+        <v>3.404</v>
       </c>
       <c r="J16" t="n">
         <v>3.617</v>
       </c>
       <c r="K16" t="n">
-        <v>3.794</v>
+        <v>3.788</v>
       </c>
       <c r="L16" t="n">
-        <v>3.832</v>
+        <v>3.809</v>
       </c>
       <c r="M16" t="n">
-        <v>3.97</v>
+        <v>3.925</v>
       </c>
       <c r="N16" t="n">
-        <v>4.024</v>
+        <v>3.977</v>
       </c>
       <c r="O16" t="n">
-        <v>4.23</v>
+        <v>4.157</v>
       </c>
       <c r="P16" t="n">
-        <v>4.287</v>
+        <v>4.204</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.499</v>
+        <v>4.419</v>
       </c>
       <c r="R16" t="n">
-        <v>4.646</v>
+        <v>4.551</v>
       </c>
       <c r="S16" t="n">
-        <v>4.827</v>
+        <v>4.72</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.713</v>
+        <v>2.711</v>
       </c>
       <c r="G17" t="n">
-        <v>2.86</v>
+        <v>2.859</v>
       </c>
       <c r="H17" t="n">
-        <v>3.042</v>
+        <v>3.044</v>
       </c>
       <c r="I17" t="n">
-        <v>3.269</v>
+        <v>3.264</v>
       </c>
       <c r="J17" t="n">
-        <v>3.493</v>
+        <v>3.484</v>
       </c>
       <c r="K17" t="n">
-        <v>3.725</v>
+        <v>3.734</v>
       </c>
       <c r="L17" t="n">
-        <v>3.802</v>
+        <v>3.779</v>
       </c>
       <c r="M17" t="n">
-        <v>3.985</v>
+        <v>3.94</v>
       </c>
       <c r="N17" t="n">
-        <v>4.045</v>
+        <v>3.996</v>
       </c>
       <c r="O17" t="n">
-        <v>4.25</v>
+        <v>4.176</v>
       </c>
       <c r="P17" t="n">
-        <v>4.335</v>
+        <v>4.252</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.714</v>
+        <v>2.712</v>
       </c>
       <c r="G18" t="n">
-        <v>2.861</v>
+        <v>2.86</v>
       </c>
       <c r="H18" t="n">
-        <v>3.043</v>
+        <v>3.044</v>
       </c>
       <c r="I18" t="n">
-        <v>3.269</v>
+        <v>3.264</v>
       </c>
       <c r="J18" t="n">
-        <v>3.493</v>
+        <v>3.484</v>
       </c>
       <c r="K18" t="n">
-        <v>3.726</v>
+        <v>3.735</v>
       </c>
       <c r="L18" t="n">
-        <v>3.802</v>
+        <v>3.779</v>
       </c>
       <c r="M18" t="n">
-        <v>3.985</v>
+        <v>3.94</v>
       </c>
       <c r="N18" t="n">
-        <v>4.046</v>
+        <v>3.997</v>
       </c>
       <c r="O18" t="n">
-        <v>4.249</v>
+        <v>4.175</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.838</v>
+        <v>2.839</v>
       </c>
       <c r="G19" t="n">
-        <v>2.988</v>
+        <v>2.995</v>
       </c>
       <c r="H19" t="n">
-        <v>3.209</v>
+        <v>3.216</v>
       </c>
       <c r="I19" t="n">
         <v>3.436</v>
       </c>
       <c r="J19" t="n">
-        <v>3.658</v>
+        <v>3.657</v>
       </c>
       <c r="K19" t="n">
-        <v>3.837</v>
+        <v>3.831</v>
       </c>
       <c r="L19" t="n">
-        <v>3.892</v>
+        <v>3.869</v>
       </c>
       <c r="M19" t="n">
-        <v>4.047</v>
+        <v>4.002</v>
       </c>
       <c r="N19" t="n">
-        <v>4.107</v>
+        <v>4.06</v>
       </c>
       <c r="O19" t="n">
-        <v>4.265</v>
+        <v>4.192</v>
       </c>
       <c r="P19" t="n">
-        <v>4.324</v>
+        <v>4.241</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.509</v>
+        <v>4.429</v>
       </c>
       <c r="R19" t="n">
-        <v>4.665</v>
+        <v>4.57</v>
       </c>
       <c r="S19" t="n">
-        <v>4.838</v>
+        <v>4.731</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.636</v>
+        <v>2.634</v>
       </c>
       <c r="G20" t="n">
-        <v>2.725</v>
+        <v>2.723</v>
       </c>
       <c r="H20" t="n">
-        <v>2.833</v>
+        <v>2.831</v>
       </c>
       <c r="I20" t="n">
-        <v>3.016</v>
+        <v>3.008</v>
       </c>
       <c r="J20" t="n">
-        <v>3.404</v>
+        <v>3.397</v>
       </c>
       <c r="K20" t="n">
-        <v>3.65</v>
+        <v>3.645</v>
       </c>
       <c r="L20" t="n">
-        <v>3.685</v>
+        <v>3.659</v>
       </c>
       <c r="M20" t="n">
-        <v>3.806</v>
+        <v>3.761</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.939</v>
+        <v>2.937</v>
       </c>
       <c r="G21" t="n">
-        <v>3.072</v>
+        <v>3.077</v>
       </c>
       <c r="H21" t="n">
-        <v>3.326</v>
+        <v>3.329</v>
       </c>
       <c r="I21" t="n">
-        <v>3.562</v>
+        <v>3.56</v>
       </c>
       <c r="J21" t="n">
-        <v>3.808</v>
+        <v>3.805</v>
       </c>
       <c r="K21" t="n">
-        <v>4.074</v>
+        <v>4.066</v>
       </c>
       <c r="L21" t="n">
-        <v>4.13</v>
+        <v>4.107</v>
       </c>
       <c r="M21" t="n">
-        <v>4.281</v>
+        <v>4.237</v>
       </c>
       <c r="N21" t="n">
-        <v>4.348</v>
+        <v>4.302</v>
       </c>
       <c r="O21" t="n">
-        <v>4.475</v>
+        <v>4.401</v>
       </c>
       <c r="P21" t="n">
-        <v>4.589</v>
+        <v>4.506</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.672</v>
+        <v>4.592</v>
       </c>
       <c r="R21" t="n">
-        <v>4.714</v>
+        <v>4.622</v>
       </c>
       <c r="S21" t="n">
-        <v>4.791</v>
+        <v>4.685</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.885</v>
+        <v>2.883</v>
       </c>
       <c r="G22" t="n">
-        <v>3.018</v>
+        <v>3.023</v>
       </c>
       <c r="H22" t="n">
-        <v>3.258</v>
+        <v>3.261</v>
       </c>
       <c r="I22" t="n">
-        <v>3.48</v>
+        <v>3.478</v>
       </c>
       <c r="J22" t="n">
-        <v>3.693</v>
+        <v>3.69</v>
       </c>
       <c r="K22" t="n">
-        <v>3.955</v>
+        <v>3.947</v>
       </c>
       <c r="L22" t="n">
-        <v>3.997</v>
+        <v>3.974</v>
       </c>
       <c r="M22" t="n">
-        <v>4.151</v>
+        <v>4.107</v>
       </c>
       <c r="N22" t="n">
-        <v>4.221</v>
+        <v>4.176</v>
       </c>
       <c r="O22" t="n">
-        <v>4.346</v>
+        <v>4.273</v>
       </c>
       <c r="P22" t="n">
-        <v>4.452</v>
+        <v>4.369</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.53</v>
+        <v>4.45</v>
       </c>
       <c r="R22" t="n">
-        <v>4.563</v>
+        <v>4.471</v>
       </c>
       <c r="S22" t="n">
-        <v>4.637</v>
+        <v>4.531</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.835</v>
+        <v>2.833</v>
       </c>
       <c r="G23" t="n">
-        <v>2.973</v>
+        <v>2.977</v>
       </c>
       <c r="H23" t="n">
-        <v>3.199</v>
+        <v>3.203</v>
       </c>
       <c r="I23" t="n">
-        <v>3.429</v>
+        <v>3.427</v>
       </c>
       <c r="J23" t="n">
-        <v>3.633</v>
+        <v>3.63</v>
       </c>
       <c r="K23" t="n">
-        <v>3.854</v>
+        <v>3.846</v>
       </c>
       <c r="L23" t="n">
-        <v>3.893</v>
+        <v>3.871</v>
       </c>
       <c r="M23" t="n">
-        <v>4.042</v>
+        <v>3.997</v>
       </c>
       <c r="N23" t="n">
-        <v>4.116</v>
+        <v>4.07</v>
       </c>
       <c r="O23" t="n">
-        <v>4.221</v>
+        <v>4.148</v>
       </c>
       <c r="P23" t="n">
-        <v>4.315</v>
+        <v>4.232</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.336</v>
+        <v>4.256</v>
       </c>
       <c r="R23" t="n">
-        <v>4.348</v>
+        <v>4.256</v>
       </c>
       <c r="S23" t="n">
-        <v>4.393</v>
+        <v>4.287</v>
       </c>
       <c r="T23" t="n">
-        <v>4.32</v>
+        <v>4.203</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.773</v>
+        <v>2.771</v>
       </c>
       <c r="G24" t="n">
-        <v>2.885</v>
+        <v>2.889</v>
       </c>
       <c r="H24" t="n">
-        <v>3.095</v>
+        <v>3.097</v>
       </c>
       <c r="I24" t="n">
-        <v>3.366</v>
+        <v>3.364</v>
       </c>
       <c r="J24" t="n">
-        <v>3.527</v>
+        <v>3.524</v>
       </c>
       <c r="K24" t="n">
-        <v>3.738</v>
+        <v>3.73</v>
       </c>
       <c r="L24" t="n">
-        <v>3.775</v>
+        <v>3.752</v>
       </c>
       <c r="M24" t="n">
-        <v>3.905</v>
+        <v>3.86</v>
       </c>
       <c r="N24" t="n">
-        <v>3.991</v>
+        <v>3.946</v>
       </c>
       <c r="O24" t="n">
-        <v>4.223</v>
+        <v>4.151</v>
       </c>
       <c r="P24" t="n">
-        <v>4.251</v>
+        <v>4.168</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.262</v>
+        <v>4.182</v>
       </c>
       <c r="R24" t="n">
-        <v>4.269</v>
+        <v>4.178</v>
       </c>
       <c r="S24" t="n">
-        <v>4.308</v>
+        <v>4.202</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.83</v>
+        <v>2.828</v>
       </c>
       <c r="G25" t="n">
-        <v>2.973</v>
+        <v>2.977</v>
       </c>
       <c r="H25" t="n">
-        <v>3.202</v>
+        <v>3.206</v>
       </c>
       <c r="I25" t="n">
-        <v>3.437</v>
+        <v>3.435</v>
       </c>
       <c r="J25" t="n">
-        <v>3.648</v>
+        <v>3.645</v>
       </c>
       <c r="K25" t="n">
-        <v>3.886</v>
+        <v>3.878</v>
       </c>
       <c r="L25" t="n">
-        <v>3.925</v>
+        <v>3.902</v>
       </c>
       <c r="M25" t="n">
-        <v>4.075</v>
+        <v>4.03</v>
       </c>
       <c r="N25" t="n">
-        <v>4.142</v>
+        <v>4.097</v>
       </c>
       <c r="O25" t="n">
-        <v>4.25</v>
+        <v>4.177</v>
       </c>
       <c r="P25" t="n">
-        <v>4.336</v>
+        <v>4.254</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.37</v>
+        <v>4.289</v>
       </c>
       <c r="R25" t="n">
-        <v>4.371</v>
+        <v>4.279</v>
       </c>
       <c r="S25" t="n">
-        <v>4.416</v>
+        <v>4.31</v>
       </c>
       <c r="T25" t="n">
-        <v>4.338</v>
+        <v>4.221</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.113</v>
+        <v>3.114</v>
       </c>
       <c r="G26" t="n">
-        <v>3.299</v>
+        <v>3.3</v>
       </c>
       <c r="H26" t="n">
-        <v>3.636</v>
+        <v>3.637</v>
       </c>
       <c r="I26" t="n">
-        <v>3.905</v>
+        <v>3.901</v>
       </c>
       <c r="J26" t="n">
-        <v>4.273</v>
+        <v>4.268</v>
       </c>
       <c r="K26" t="n">
-        <v>4.695</v>
+        <v>4.69</v>
       </c>
       <c r="L26" t="n">
-        <v>4.806</v>
+        <v>4.784</v>
       </c>
       <c r="M26" t="n">
-        <v>4.999</v>
+        <v>4.955</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.307</v>
+        <v>5.233</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.929</v>
+        <v>2.931</v>
       </c>
       <c r="G27" t="n">
-        <v>3.065</v>
+        <v>3.07</v>
       </c>
       <c r="H27" t="n">
-        <v>3.305</v>
+        <v>3.31</v>
       </c>
       <c r="I27" t="n">
-        <v>3.541</v>
+        <v>3.54</v>
       </c>
       <c r="J27" t="n">
-        <v>3.786</v>
+        <v>3.784</v>
       </c>
       <c r="K27" t="n">
-        <v>4.016</v>
+        <v>4.011</v>
       </c>
       <c r="L27" t="n">
-        <v>4.077</v>
+        <v>4.054</v>
       </c>
       <c r="M27" t="n">
-        <v>4.218</v>
+        <v>4.173</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.408</v>
+        <v>4.335</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.032</v>
+        <v>3.034</v>
       </c>
       <c r="G28" t="n">
-        <v>3.176</v>
+        <v>3.181</v>
       </c>
       <c r="H28" t="n">
-        <v>3.431</v>
+        <v>3.436</v>
       </c>
       <c r="I28" t="n">
-        <v>3.678</v>
+        <v>3.677</v>
       </c>
       <c r="J28" t="n">
-        <v>3.959</v>
+        <v>3.957</v>
       </c>
       <c r="K28" t="n">
-        <v>4.209</v>
+        <v>4.204</v>
       </c>
       <c r="L28" t="n">
-        <v>4.279</v>
+        <v>4.257</v>
       </c>
       <c r="M28" t="n">
-        <v>4.429</v>
+        <v>4.385</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.7</v>
+        <v>4.627</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.879</v>
+        <v>2.881</v>
       </c>
       <c r="G29" t="n">
-        <v>3.013</v>
+        <v>3.018</v>
       </c>
       <c r="H29" t="n">
-        <v>3.244</v>
+        <v>3.249</v>
       </c>
       <c r="I29" t="n">
-        <v>3.469</v>
+        <v>3.467</v>
       </c>
       <c r="J29" t="n">
-        <v>3.698</v>
+        <v>3.697</v>
       </c>
       <c r="K29" t="n">
-        <v>3.912</v>
+        <v>3.907</v>
       </c>
       <c r="L29" t="n">
-        <v>3.962</v>
+        <v>3.94</v>
       </c>
       <c r="M29" t="n">
-        <v>4.081</v>
+        <v>4.036</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.28</v>
+        <v>4.207</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2599,37 +2599,37 @@
         <v>3.155</v>
       </c>
       <c r="G30" t="n">
-        <v>3.276</v>
+        <v>3.277</v>
       </c>
       <c r="H30" t="n">
-        <v>3.57</v>
+        <v>3.573</v>
       </c>
       <c r="I30" t="n">
-        <v>3.828</v>
+        <v>3.826</v>
       </c>
       <c r="J30" t="n">
-        <v>4.137</v>
+        <v>4.132</v>
       </c>
       <c r="K30" t="n">
-        <v>4.493</v>
+        <v>4.489</v>
       </c>
       <c r="L30" t="n">
-        <v>4.584</v>
+        <v>4.563</v>
       </c>
       <c r="M30" t="n">
-        <v>4.767</v>
+        <v>4.723</v>
       </c>
       <c r="N30" t="n">
-        <v>4.938</v>
+        <v>4.89</v>
       </c>
       <c r="O30" t="n">
-        <v>5.258</v>
+        <v>5.184</v>
       </c>
       <c r="P30" t="n">
-        <v>5.478</v>
+        <v>5.396</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.203</v>
+        <v>6.123</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2672,37 +2672,37 @@
         <v>3.484</v>
       </c>
       <c r="G31" t="n">
-        <v>3.641</v>
+        <v>3.642</v>
       </c>
       <c r="H31" t="n">
-        <v>3.985</v>
+        <v>3.987</v>
       </c>
       <c r="I31" t="n">
-        <v>4.258</v>
+        <v>4.256</v>
       </c>
       <c r="J31" t="n">
-        <v>4.628</v>
+        <v>4.623</v>
       </c>
       <c r="K31" t="n">
-        <v>5.026</v>
+        <v>5.022</v>
       </c>
       <c r="L31" t="n">
-        <v>5.197</v>
+        <v>5.175</v>
       </c>
       <c r="M31" t="n">
-        <v>5.498</v>
+        <v>5.453</v>
       </c>
       <c r="N31" t="n">
-        <v>5.797</v>
+        <v>5.749</v>
       </c>
       <c r="O31" t="n">
-        <v>6.294</v>
+        <v>6.22</v>
       </c>
       <c r="P31" t="n">
-        <v>6.467</v>
+        <v>6.384</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.176</v>
+        <v>7.096</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2745,37 +2745,37 @@
         <v>3.254</v>
       </c>
       <c r="G32" t="n">
-        <v>3.394</v>
+        <v>3.395</v>
       </c>
       <c r="H32" t="n">
-        <v>3.714</v>
+        <v>3.717</v>
       </c>
       <c r="I32" t="n">
-        <v>3.987</v>
+        <v>3.985</v>
       </c>
       <c r="J32" t="n">
-        <v>4.315</v>
+        <v>4.31</v>
       </c>
       <c r="K32" t="n">
-        <v>4.678</v>
+        <v>4.674</v>
       </c>
       <c r="L32" t="n">
-        <v>4.789</v>
+        <v>4.767</v>
       </c>
       <c r="M32" t="n">
-        <v>5.04</v>
+        <v>4.995</v>
       </c>
       <c r="N32" t="n">
-        <v>5.298</v>
+        <v>5.251</v>
       </c>
       <c r="O32" t="n">
-        <v>5.703</v>
+        <v>5.629</v>
       </c>
       <c r="P32" t="n">
-        <v>5.938</v>
+        <v>5.856</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.664</v>
+        <v>6.584</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.021</v>
+        <v>3.02</v>
       </c>
       <c r="G33" t="n">
         <v>3.142</v>
       </c>
       <c r="H33" t="n">
-        <v>3.388</v>
+        <v>3.391</v>
       </c>
       <c r="I33" t="n">
-        <v>3.612</v>
+        <v>3.611</v>
       </c>
       <c r="J33" t="n">
-        <v>3.844</v>
+        <v>3.84</v>
       </c>
       <c r="K33" t="n">
-        <v>4.135</v>
+        <v>4.132</v>
       </c>
       <c r="L33" t="n">
-        <v>4.186</v>
+        <v>4.165</v>
       </c>
       <c r="M33" t="n">
-        <v>4.293</v>
+        <v>4.249</v>
       </c>
       <c r="N33" t="n">
-        <v>4.327</v>
+        <v>4.28</v>
       </c>
       <c r="O33" t="n">
-        <v>4.412</v>
+        <v>4.338</v>
       </c>
       <c r="P33" t="n">
-        <v>4.511</v>
+        <v>4.428</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.919</v>
+        <v>4.84</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.081</v>
+        <v>3.08</v>
       </c>
       <c r="G34" t="n">
         <v>3.195</v>
       </c>
       <c r="H34" t="n">
-        <v>3.45</v>
+        <v>3.453</v>
       </c>
       <c r="I34" t="n">
-        <v>3.68</v>
+        <v>3.679</v>
       </c>
       <c r="J34" t="n">
-        <v>3.915</v>
+        <v>3.912</v>
       </c>
       <c r="K34" t="n">
-        <v>4.212</v>
+        <v>4.209</v>
       </c>
       <c r="L34" t="n">
-        <v>4.265</v>
+        <v>4.244</v>
       </c>
       <c r="M34" t="n">
-        <v>4.383</v>
+        <v>4.34</v>
       </c>
       <c r="N34" t="n">
-        <v>4.431</v>
+        <v>4.384</v>
       </c>
       <c r="O34" t="n">
-        <v>4.581</v>
+        <v>4.507</v>
       </c>
       <c r="P34" t="n">
-        <v>4.805</v>
+        <v>4.723</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.62</v>
+        <v>5.541</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.055</v>
+        <v>3.054</v>
       </c>
       <c r="G35" t="n">
         <v>3.169</v>
       </c>
       <c r="H35" t="n">
-        <v>3.418</v>
+        <v>3.421</v>
       </c>
       <c r="I35" t="n">
-        <v>3.647</v>
+        <v>3.646</v>
       </c>
       <c r="J35" t="n">
-        <v>3.883</v>
+        <v>3.881</v>
       </c>
       <c r="K35" t="n">
-        <v>4.165</v>
+        <v>4.162</v>
       </c>
       <c r="L35" t="n">
-        <v>4.22</v>
+        <v>4.199</v>
       </c>
       <c r="M35" t="n">
-        <v>4.33</v>
+        <v>4.286</v>
       </c>
       <c r="N35" t="n">
-        <v>4.368</v>
+        <v>4.32</v>
       </c>
       <c r="O35" t="n">
-        <v>4.478</v>
+        <v>4.404</v>
       </c>
       <c r="P35" t="n">
-        <v>4.608</v>
+        <v>4.525</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.256</v>
+        <v>5.177</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.948</v>
+        <v>2.949</v>
       </c>
       <c r="G36" t="n">
-        <v>3.059</v>
+        <v>3.06</v>
       </c>
       <c r="H36" t="n">
-        <v>3.299</v>
+        <v>3.3</v>
       </c>
       <c r="I36" t="n">
-        <v>3.528</v>
+        <v>3.526</v>
       </c>
       <c r="J36" t="n">
-        <v>3.782</v>
+        <v>3.777</v>
       </c>
       <c r="K36" t="n">
-        <v>4.061</v>
+        <v>4.057</v>
       </c>
       <c r="L36" t="n">
-        <v>4.113</v>
+        <v>4.091</v>
       </c>
       <c r="M36" t="n">
-        <v>4.194</v>
+        <v>4.151</v>
       </c>
       <c r="N36" t="n">
-        <v>4.23</v>
+        <v>4.183</v>
       </c>
       <c r="O36" t="n">
-        <v>4.32</v>
+        <v>4.246</v>
       </c>
       <c r="P36" t="n">
-        <v>4.409</v>
+        <v>4.326</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.636</v>
+        <v>4.557</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3110,37 +3110,37 @@
         <v>3.827</v>
       </c>
       <c r="G37" t="n">
-        <v>4.334</v>
+        <v>4.335</v>
       </c>
       <c r="H37" t="n">
-        <v>4.957</v>
+        <v>4.96</v>
       </c>
       <c r="I37" t="n">
-        <v>5.319</v>
+        <v>5.317</v>
       </c>
       <c r="J37" t="n">
-        <v>6.119</v>
+        <v>6.114</v>
       </c>
       <c r="K37" t="n">
-        <v>7.066</v>
+        <v>7.062</v>
       </c>
       <c r="L37" t="n">
-        <v>7.397</v>
+        <v>7.375</v>
       </c>
       <c r="M37" t="n">
-        <v>7.77</v>
+        <v>7.725</v>
       </c>
       <c r="N37" t="n">
-        <v>7.948</v>
+        <v>7.901</v>
       </c>
       <c r="O37" t="n">
-        <v>8.173</v>
+        <v>8.099</v>
       </c>
       <c r="P37" t="n">
-        <v>8.266</v>
+        <v>8.183999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.666</v>
+        <v>8.587</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3183,37 +3183,37 @@
         <v>4.888</v>
       </c>
       <c r="G38" t="n">
-        <v>5.649</v>
+        <v>5.65</v>
       </c>
       <c r="H38" t="n">
-        <v>6.483</v>
+        <v>6.486</v>
       </c>
       <c r="I38" t="n">
-        <v>7.002</v>
+        <v>7</v>
       </c>
       <c r="J38" t="n">
-        <v>8.063000000000001</v>
+        <v>8.058</v>
       </c>
       <c r="K38" t="n">
-        <v>9.188000000000001</v>
+        <v>9.183999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.679</v>
+        <v>9.657999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.181</v>
+        <v>10.137</v>
       </c>
       <c r="N38" t="n">
-        <v>10.367</v>
+        <v>10.319</v>
       </c>
       <c r="O38" t="n">
-        <v>10.573</v>
+        <v>10.499</v>
       </c>
       <c r="P38" t="n">
-        <v>10.664</v>
+        <v>10.582</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.117</v>
+        <v>11.038</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3256,37 +3256,37 @@
         <v>4.209</v>
       </c>
       <c r="G39" t="n">
-        <v>4.847</v>
+        <v>4.848</v>
       </c>
       <c r="H39" t="n">
-        <v>5.548</v>
+        <v>5.551</v>
       </c>
       <c r="I39" t="n">
-        <v>6.006</v>
+        <v>6.004</v>
       </c>
       <c r="J39" t="n">
-        <v>6.936</v>
+        <v>6.931</v>
       </c>
       <c r="K39" t="n">
-        <v>8.021000000000001</v>
+        <v>8.016999999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>8.435</v>
+        <v>8.413</v>
       </c>
       <c r="M39" t="n">
-        <v>8.818</v>
+        <v>8.773999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.994</v>
+        <v>8.946999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.224</v>
+        <v>9.15</v>
       </c>
       <c r="P39" t="n">
-        <v>9.318</v>
+        <v>9.236000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.762</v>
+        <v>9.683</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3329,37 +3329,37 @@
         <v>3.347</v>
       </c>
       <c r="G40" t="n">
-        <v>3.514</v>
+        <v>3.515</v>
       </c>
       <c r="H40" t="n">
-        <v>3.829</v>
+        <v>3.832</v>
       </c>
       <c r="I40" t="n">
-        <v>4.102</v>
+        <v>4.1</v>
       </c>
       <c r="J40" t="n">
-        <v>4.428</v>
+        <v>4.423</v>
       </c>
       <c r="K40" t="n">
-        <v>4.799</v>
+        <v>4.795</v>
       </c>
       <c r="L40" t="n">
-        <v>4.909</v>
+        <v>4.887</v>
       </c>
       <c r="M40" t="n">
-        <v>5.11</v>
+        <v>5.066</v>
       </c>
       <c r="N40" t="n">
-        <v>5.295</v>
+        <v>5.248</v>
       </c>
       <c r="O40" t="n">
-        <v>5.637</v>
+        <v>5.563</v>
       </c>
       <c r="P40" t="n">
-        <v>5.899</v>
+        <v>5.817</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.654</v>
+        <v>6.574</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3402,37 +3402,37 @@
         <v>3.733</v>
       </c>
       <c r="G41" t="n">
-        <v>3.943</v>
+        <v>3.944</v>
       </c>
       <c r="H41" t="n">
-        <v>4.314</v>
+        <v>4.317</v>
       </c>
       <c r="I41" t="n">
-        <v>4.606</v>
+        <v>4.604</v>
       </c>
       <c r="J41" t="n">
-        <v>4.983</v>
+        <v>4.978</v>
       </c>
       <c r="K41" t="n">
-        <v>5.4</v>
+        <v>5.395</v>
       </c>
       <c r="L41" t="n">
-        <v>5.588</v>
+        <v>5.566</v>
       </c>
       <c r="M41" t="n">
-        <v>5.913</v>
+        <v>5.868</v>
       </c>
       <c r="N41" t="n">
-        <v>6.226</v>
+        <v>6.179</v>
       </c>
       <c r="O41" t="n">
-        <v>6.752</v>
+        <v>6.678</v>
       </c>
       <c r="P41" t="n">
-        <v>6.959</v>
+        <v>6.877</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.701</v>
+        <v>7.621</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3475,37 +3475,37 @@
         <v>3.468</v>
       </c>
       <c r="G42" t="n">
-        <v>3.663</v>
+        <v>3.664</v>
       </c>
       <c r="H42" t="n">
-        <v>4.005</v>
+        <v>4.008</v>
       </c>
       <c r="I42" t="n">
-        <v>4.29</v>
+        <v>4.288</v>
       </c>
       <c r="J42" t="n">
-        <v>4.631</v>
+        <v>4.625</v>
       </c>
       <c r="K42" t="n">
-        <v>5.02</v>
+        <v>5.016</v>
       </c>
       <c r="L42" t="n">
-        <v>5.145</v>
+        <v>5.124</v>
       </c>
       <c r="M42" t="n">
-        <v>5.417</v>
+        <v>5.373</v>
       </c>
       <c r="N42" t="n">
-        <v>5.71</v>
+        <v>5.663</v>
       </c>
       <c r="O42" t="n">
-        <v>6.129</v>
+        <v>6.055</v>
       </c>
       <c r="P42" t="n">
-        <v>6.401</v>
+        <v>6.319</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.166</v>
+        <v>7.087</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.169</v>
+        <v>3.168</v>
       </c>
       <c r="G43" t="n">
         <v>3.325</v>
       </c>
       <c r="H43" t="n">
-        <v>3.589</v>
+        <v>3.592</v>
       </c>
       <c r="I43" t="n">
-        <v>3.821</v>
+        <v>3.82</v>
       </c>
       <c r="J43" t="n">
-        <v>4.071</v>
+        <v>4.068</v>
       </c>
       <c r="K43" t="n">
-        <v>4.367</v>
+        <v>4.364</v>
       </c>
       <c r="L43" t="n">
-        <v>4.428</v>
+        <v>4.407</v>
       </c>
       <c r="M43" t="n">
-        <v>4.548</v>
+        <v>4.504</v>
       </c>
       <c r="N43" t="n">
-        <v>4.596</v>
+        <v>4.549</v>
       </c>
       <c r="O43" t="n">
-        <v>4.725</v>
+        <v>4.651</v>
       </c>
       <c r="P43" t="n">
-        <v>4.876</v>
+        <v>4.794</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.529</v>
+        <v>5.45</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.026</v>
+        <v>3.027</v>
       </c>
       <c r="G44" t="n">
-        <v>3.168</v>
+        <v>3.169</v>
       </c>
       <c r="H44" t="n">
-        <v>3.422</v>
+        <v>3.424</v>
       </c>
       <c r="I44" t="n">
-        <v>3.655</v>
+        <v>3.653</v>
       </c>
       <c r="J44" t="n">
-        <v>3.923</v>
+        <v>3.918</v>
       </c>
       <c r="K44" t="n">
-        <v>4.212</v>
+        <v>4.209</v>
       </c>
       <c r="L44" t="n">
-        <v>4.273</v>
+        <v>4.252</v>
       </c>
       <c r="M44" t="n">
-        <v>4.364</v>
+        <v>4.322</v>
       </c>
       <c r="N44" t="n">
-        <v>4.412</v>
+        <v>4.365</v>
       </c>
       <c r="O44" t="n">
-        <v>4.521</v>
+        <v>4.447</v>
       </c>
       <c r="P44" t="n">
-        <v>4.639</v>
+        <v>4.556</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.9</v>
+        <v>4.821</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-01 ~ 2026-06-01
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.279</v>
+        <v>3.294</v>
       </c>
       <c r="G2" t="n">
-        <v>3.553</v>
+        <v>3.574</v>
       </c>
       <c r="H2" t="n">
-        <v>3.841</v>
+        <v>3.862</v>
       </c>
       <c r="I2" t="n">
-        <v>4.055</v>
+        <v>4.079</v>
       </c>
       <c r="J2" t="n">
-        <v>4.313</v>
+        <v>4.37</v>
       </c>
       <c r="K2" t="n">
-        <v>4.72</v>
+        <v>4.774</v>
       </c>
       <c r="L2" t="n">
-        <v>4.885</v>
+        <v>4.951</v>
       </c>
       <c r="M2" t="n">
-        <v>5.174</v>
+        <v>5.242</v>
       </c>
       <c r="N2" t="n">
-        <v>5.451</v>
+        <v>5.522</v>
       </c>
       <c r="O2" t="n">
-        <v>5.698</v>
+        <v>5.778</v>
       </c>
       <c r="P2" t="n">
-        <v>5.919</v>
+        <v>6.013</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.525</v>
+        <v>6.639</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.3</v>
+        <v>4.315</v>
       </c>
       <c r="G3" t="n">
-        <v>4.756</v>
+        <v>4.777</v>
       </c>
       <c r="H3" t="n">
-        <v>5.077</v>
+        <v>5.098</v>
       </c>
       <c r="I3" t="n">
-        <v>5.284</v>
+        <v>5.307</v>
       </c>
       <c r="J3" t="n">
-        <v>5.559</v>
+        <v>5.616</v>
       </c>
       <c r="K3" t="n">
-        <v>6.036</v>
+        <v>6.09</v>
       </c>
       <c r="L3" t="n">
-        <v>6.271</v>
+        <v>6.336</v>
       </c>
       <c r="M3" t="n">
-        <v>6.591</v>
+        <v>6.658</v>
       </c>
       <c r="N3" t="n">
-        <v>6.811</v>
+        <v>6.881</v>
       </c>
       <c r="O3" t="n">
-        <v>7.008</v>
+        <v>7.088</v>
       </c>
       <c r="P3" t="n">
-        <v>7.098</v>
+        <v>7.191</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.592</v>
+        <v>7.705</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.793</v>
+        <v>3.808</v>
       </c>
       <c r="G4" t="n">
-        <v>4.137</v>
+        <v>4.157</v>
       </c>
       <c r="H4" t="n">
-        <v>4.487</v>
+        <v>4.508</v>
       </c>
       <c r="I4" t="n">
-        <v>4.726</v>
+        <v>4.75</v>
       </c>
       <c r="J4" t="n">
-        <v>5.005</v>
+        <v>5.059</v>
       </c>
       <c r="K4" t="n">
-        <v>5.474</v>
+        <v>5.529</v>
       </c>
       <c r="L4" t="n">
-        <v>5.639</v>
+        <v>5.705</v>
       </c>
       <c r="M4" t="n">
-        <v>5.949</v>
+        <v>6.016</v>
       </c>
       <c r="N4" t="n">
-        <v>6.139</v>
+        <v>6.21</v>
       </c>
       <c r="O4" t="n">
-        <v>6.359</v>
+        <v>6.44</v>
       </c>
       <c r="P4" t="n">
-        <v>6.45</v>
+        <v>6.543</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.947</v>
+        <v>7.06</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.976</v>
+        <v>2.991</v>
       </c>
       <c r="G5" t="n">
-        <v>3.094</v>
+        <v>3.115</v>
       </c>
       <c r="H5" t="n">
-        <v>3.348</v>
+        <v>3.369</v>
       </c>
       <c r="I5" t="n">
-        <v>3.627</v>
+        <v>3.651</v>
       </c>
       <c r="J5" t="n">
-        <v>3.87</v>
+        <v>3.928</v>
       </c>
       <c r="K5" t="n">
-        <v>4.123</v>
+        <v>4.179</v>
       </c>
       <c r="L5" t="n">
-        <v>4.132</v>
+        <v>4.198</v>
       </c>
       <c r="M5" t="n">
-        <v>4.233</v>
+        <v>4.301</v>
       </c>
       <c r="N5" t="n">
-        <v>4.264</v>
+        <v>4.334</v>
       </c>
       <c r="O5" t="n">
-        <v>4.297</v>
+        <v>4.378</v>
       </c>
       <c r="P5" t="n">
-        <v>4.588</v>
+        <v>4.682</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.438</v>
+        <v>5.551</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.017</v>
+        <v>3.032</v>
       </c>
       <c r="G6" t="n">
-        <v>3.15</v>
+        <v>3.17</v>
       </c>
       <c r="H6" t="n">
-        <v>3.417</v>
+        <v>3.438</v>
       </c>
       <c r="I6" t="n">
-        <v>3.711</v>
+        <v>3.733</v>
       </c>
       <c r="J6" t="n">
-        <v>3.961</v>
+        <v>4.017</v>
       </c>
       <c r="K6" t="n">
-        <v>4.237</v>
+        <v>4.291</v>
       </c>
       <c r="L6" t="n">
-        <v>4.251</v>
+        <v>4.316</v>
       </c>
       <c r="M6" t="n">
-        <v>4.389</v>
+        <v>4.456</v>
       </c>
       <c r="N6" t="n">
-        <v>4.431</v>
+        <v>4.502</v>
       </c>
       <c r="O6" t="n">
-        <v>4.564</v>
+        <v>4.644</v>
       </c>
       <c r="P6" t="n">
-        <v>5.02</v>
+        <v>5.114</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.834</v>
+        <v>5.947</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.997</v>
+        <v>3.012</v>
       </c>
       <c r="G7" t="n">
-        <v>3.113</v>
+        <v>3.133</v>
       </c>
       <c r="H7" t="n">
-        <v>3.364</v>
+        <v>3.385</v>
       </c>
       <c r="I7" t="n">
-        <v>3.646</v>
+        <v>3.67</v>
       </c>
       <c r="J7" t="n">
-        <v>3.893</v>
+        <v>3.951</v>
       </c>
       <c r="K7" t="n">
-        <v>4.15</v>
+        <v>4.206</v>
       </c>
       <c r="L7" t="n">
-        <v>4.158</v>
+        <v>4.225</v>
       </c>
       <c r="M7" t="n">
-        <v>4.293</v>
+        <v>4.361</v>
       </c>
       <c r="N7" t="n">
-        <v>4.323</v>
+        <v>4.394</v>
       </c>
       <c r="O7" t="n">
-        <v>4.461</v>
+        <v>4.541</v>
       </c>
       <c r="P7" t="n">
-        <v>4.804</v>
+        <v>4.898</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.601</v>
+        <v>5.715</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.412</v>
+        <v>5.427</v>
       </c>
       <c r="G8" t="n">
-        <v>6.056</v>
+        <v>6.076</v>
       </c>
       <c r="H8" t="n">
-        <v>6.525</v>
+        <v>6.546</v>
       </c>
       <c r="I8" t="n">
-        <v>6.81</v>
+        <v>6.834</v>
       </c>
       <c r="J8" t="n">
-        <v>7.152</v>
+        <v>7.208</v>
       </c>
       <c r="K8" t="n">
-        <v>7.909</v>
+        <v>7.964</v>
       </c>
       <c r="L8" t="n">
-        <v>8.228999999999999</v>
+        <v>8.294</v>
       </c>
       <c r="M8" t="n">
-        <v>8.581</v>
+        <v>8.648999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.734999999999999</v>
+        <v>8.805999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.016999999999999</v>
+        <v>9.098000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.211</v>
+        <v>9.304</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.903</v>
+        <v>10.016</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.635</v>
+        <v>2.636</v>
       </c>
       <c r="G9" t="n">
-        <v>2.735</v>
+        <v>2.737</v>
       </c>
       <c r="H9" t="n">
-        <v>2.939</v>
+        <v>2.945</v>
       </c>
       <c r="I9" t="n">
-        <v>3.177</v>
+        <v>3.187</v>
       </c>
       <c r="J9" t="n">
-        <v>3.383</v>
+        <v>3.43</v>
       </c>
       <c r="K9" t="n">
-        <v>3.627</v>
+        <v>3.685</v>
       </c>
       <c r="L9" t="n">
-        <v>3.644</v>
+        <v>3.71</v>
       </c>
       <c r="M9" t="n">
-        <v>3.722</v>
+        <v>3.79</v>
       </c>
       <c r="N9" t="n">
-        <v>3.873</v>
+        <v>3.944</v>
       </c>
       <c r="O9" t="n">
-        <v>3.915</v>
+        <v>3.995</v>
       </c>
       <c r="P9" t="n">
-        <v>4.02</v>
+        <v>4.113</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.065</v>
+        <v>4.178</v>
       </c>
       <c r="R9" t="n">
-        <v>4.074</v>
+        <v>4.192</v>
       </c>
       <c r="S9" t="n">
-        <v>4.078</v>
+        <v>4.2</v>
       </c>
       <c r="T9" t="n">
-        <v>3.996</v>
+        <v>4.132</v>
       </c>
       <c r="U9" t="n">
-        <v>3.894</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.656</v>
+        <v>2.658</v>
       </c>
       <c r="G10" t="n">
-        <v>2.773</v>
+        <v>2.775</v>
       </c>
       <c r="H10" t="n">
-        <v>2.952</v>
+        <v>2.958</v>
       </c>
       <c r="I10" t="n">
-        <v>3.182</v>
+        <v>3.193</v>
       </c>
       <c r="J10" t="n">
-        <v>3.41</v>
+        <v>3.457</v>
       </c>
       <c r="K10" t="n">
-        <v>3.655</v>
+        <v>3.715</v>
       </c>
       <c r="L10" t="n">
-        <v>3.696</v>
+        <v>3.762</v>
       </c>
       <c r="M10" t="n">
-        <v>3.817</v>
+        <v>3.884</v>
       </c>
       <c r="N10" t="n">
-        <v>3.893</v>
+        <v>3.964</v>
       </c>
       <c r="O10" t="n">
-        <v>4.154</v>
+        <v>4.233</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.466</v>
+        <v>2.468</v>
       </c>
       <c r="G11" t="n">
-        <v>2.58</v>
+        <v>2.582</v>
       </c>
       <c r="H11" t="n">
-        <v>2.775</v>
+        <v>2.781</v>
       </c>
       <c r="I11" t="n">
-        <v>2.986</v>
+        <v>2.997</v>
       </c>
       <c r="J11" t="n">
-        <v>3.207</v>
+        <v>3.253</v>
       </c>
       <c r="K11" t="n">
-        <v>3.442</v>
+        <v>3.502</v>
       </c>
       <c r="L11" t="n">
-        <v>3.493</v>
+        <v>3.56</v>
       </c>
       <c r="M11" t="n">
-        <v>3.625</v>
+        <v>3.692</v>
       </c>
       <c r="N11" t="n">
-        <v>3.7</v>
+        <v>3.772</v>
       </c>
       <c r="O11" t="n">
-        <v>3.92</v>
+        <v>3.999</v>
       </c>
       <c r="P11" t="n">
-        <v>3.971</v>
+        <v>4.064</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.266</v>
+        <v>4.379</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.277</v>
+        <v>3.283</v>
       </c>
       <c r="G12" t="n">
-        <v>3.512</v>
+        <v>3.528</v>
       </c>
       <c r="H12" t="n">
-        <v>3.76</v>
+        <v>3.781</v>
       </c>
       <c r="I12" t="n">
-        <v>4.02</v>
+        <v>4.045</v>
       </c>
       <c r="J12" t="n">
-        <v>4.3</v>
+        <v>4.354</v>
       </c>
       <c r="K12" t="n">
-        <v>4.514</v>
+        <v>4.568</v>
       </c>
       <c r="L12" t="n">
-        <v>4.56</v>
+        <v>4.627</v>
       </c>
       <c r="M12" t="n">
-        <v>4.698</v>
+        <v>4.766</v>
       </c>
       <c r="N12" t="n">
-        <v>4.763</v>
+        <v>4.834</v>
       </c>
       <c r="O12" t="n">
-        <v>4.92</v>
+        <v>5</v>
       </c>
       <c r="P12" t="n">
-        <v>5.056</v>
+        <v>5.15</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.379</v>
+        <v>5.492</v>
       </c>
       <c r="R12" t="n">
-        <v>5.565</v>
+        <v>5.683</v>
       </c>
       <c r="S12" t="n">
-        <v>5.781</v>
+        <v>5.903</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.031</v>
+        <v>3.037</v>
       </c>
       <c r="G13" t="n">
-        <v>3.202</v>
+        <v>3.218</v>
       </c>
       <c r="H13" t="n">
-        <v>3.427</v>
+        <v>3.448</v>
       </c>
       <c r="I13" t="n">
-        <v>3.668</v>
+        <v>3.692</v>
       </c>
       <c r="J13" t="n">
-        <v>3.936</v>
+        <v>3.99</v>
       </c>
       <c r="K13" t="n">
-        <v>4.148</v>
+        <v>4.201</v>
       </c>
       <c r="L13" t="n">
-        <v>4.199</v>
+        <v>4.266</v>
       </c>
       <c r="M13" t="n">
-        <v>4.326</v>
+        <v>4.394</v>
       </c>
       <c r="N13" t="n">
-        <v>4.391</v>
+        <v>4.462</v>
       </c>
       <c r="O13" t="n">
-        <v>4.548</v>
+        <v>4.629</v>
       </c>
       <c r="P13" t="n">
-        <v>4.647</v>
+        <v>4.741</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.9</v>
+        <v>5.014</v>
       </c>
       <c r="R13" t="n">
-        <v>5.114</v>
+        <v>5.232</v>
       </c>
       <c r="S13" t="n">
-        <v>5.344</v>
+        <v>5.465</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.85</v>
+        <v>2.856</v>
       </c>
       <c r="G14" t="n">
-        <v>3.008</v>
+        <v>3.023</v>
       </c>
       <c r="H14" t="n">
-        <v>3.23</v>
+        <v>3.251</v>
       </c>
       <c r="I14" t="n">
-        <v>3.453</v>
+        <v>3.477</v>
       </c>
       <c r="J14" t="n">
-        <v>3.678</v>
+        <v>3.732</v>
       </c>
       <c r="K14" t="n">
-        <v>3.836</v>
+        <v>3.889</v>
       </c>
       <c r="L14" t="n">
-        <v>3.872</v>
+        <v>3.939</v>
       </c>
       <c r="M14" t="n">
-        <v>4.012</v>
+        <v>4.08</v>
       </c>
       <c r="N14" t="n">
-        <v>4.07</v>
+        <v>4.142</v>
       </c>
       <c r="O14" t="n">
-        <v>4.207</v>
+        <v>4.287</v>
       </c>
       <c r="P14" t="n">
-        <v>4.283</v>
+        <v>4.377</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.49</v>
+        <v>4.603</v>
       </c>
       <c r="R14" t="n">
-        <v>4.629</v>
+        <v>4.747</v>
       </c>
       <c r="S14" t="n">
-        <v>4.796</v>
+        <v>4.918</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.827</v>
+        <v>2.834</v>
       </c>
       <c r="G15" t="n">
-        <v>2.982</v>
+        <v>2.998</v>
       </c>
       <c r="H15" t="n">
-        <v>3.201</v>
+        <v>3.222</v>
       </c>
       <c r="I15" t="n">
-        <v>3.404</v>
+        <v>3.428</v>
       </c>
       <c r="J15" t="n">
-        <v>3.617</v>
+        <v>3.671</v>
       </c>
       <c r="K15" t="n">
-        <v>3.788</v>
+        <v>3.841</v>
       </c>
       <c r="L15" t="n">
-        <v>3.809</v>
+        <v>3.875</v>
       </c>
       <c r="M15" t="n">
-        <v>3.925</v>
+        <v>3.993</v>
       </c>
       <c r="N15" t="n">
-        <v>3.974</v>
+        <v>4.045</v>
       </c>
       <c r="O15" t="n">
-        <v>4.151</v>
+        <v>4.232</v>
       </c>
       <c r="P15" t="n">
-        <v>4.181</v>
+        <v>4.275</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.392</v>
+        <v>4.505</v>
       </c>
       <c r="R15" t="n">
-        <v>4.523</v>
+        <v>4.641</v>
       </c>
       <c r="S15" t="n">
-        <v>4.691</v>
+        <v>4.813</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.827</v>
+        <v>2.834</v>
       </c>
       <c r="G16" t="n">
-        <v>2.982</v>
+        <v>2.998</v>
       </c>
       <c r="H16" t="n">
-        <v>3.201</v>
+        <v>3.222</v>
       </c>
       <c r="I16" t="n">
-        <v>3.404</v>
+        <v>3.428</v>
       </c>
       <c r="J16" t="n">
-        <v>3.617</v>
+        <v>3.671</v>
       </c>
       <c r="K16" t="n">
-        <v>3.788</v>
+        <v>3.841</v>
       </c>
       <c r="L16" t="n">
-        <v>3.809</v>
+        <v>3.875</v>
       </c>
       <c r="M16" t="n">
-        <v>3.925</v>
+        <v>3.993</v>
       </c>
       <c r="N16" t="n">
-        <v>3.977</v>
+        <v>4.048</v>
       </c>
       <c r="O16" t="n">
-        <v>4.157</v>
+        <v>4.238</v>
       </c>
       <c r="P16" t="n">
-        <v>4.204</v>
+        <v>4.298</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.419</v>
+        <v>4.532</v>
       </c>
       <c r="R16" t="n">
-        <v>4.551</v>
+        <v>4.669</v>
       </c>
       <c r="S16" t="n">
-        <v>4.72</v>
+        <v>4.842</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.711</v>
+        <v>2.713</v>
       </c>
       <c r="G17" t="n">
-        <v>2.859</v>
+        <v>2.861</v>
       </c>
       <c r="H17" t="n">
-        <v>3.044</v>
+        <v>3.05</v>
       </c>
       <c r="I17" t="n">
-        <v>3.264</v>
+        <v>3.275</v>
       </c>
       <c r="J17" t="n">
-        <v>3.484</v>
+        <v>3.531</v>
       </c>
       <c r="K17" t="n">
-        <v>3.734</v>
+        <v>3.793</v>
       </c>
       <c r="L17" t="n">
-        <v>3.779</v>
+        <v>3.846</v>
       </c>
       <c r="M17" t="n">
-        <v>3.94</v>
+        <v>4.008</v>
       </c>
       <c r="N17" t="n">
-        <v>3.996</v>
+        <v>4.067</v>
       </c>
       <c r="O17" t="n">
-        <v>4.176</v>
+        <v>4.254</v>
       </c>
       <c r="P17" t="n">
-        <v>4.252</v>
+        <v>4.345</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.712</v>
+        <v>2.714</v>
       </c>
       <c r="G18" t="n">
-        <v>2.86</v>
+        <v>2.862</v>
       </c>
       <c r="H18" t="n">
-        <v>3.044</v>
+        <v>3.05</v>
       </c>
       <c r="I18" t="n">
-        <v>3.264</v>
+        <v>3.276</v>
       </c>
       <c r="J18" t="n">
-        <v>3.484</v>
+        <v>3.531</v>
       </c>
       <c r="K18" t="n">
-        <v>3.735</v>
+        <v>3.794</v>
       </c>
       <c r="L18" t="n">
-        <v>3.779</v>
+        <v>3.846</v>
       </c>
       <c r="M18" t="n">
-        <v>3.94</v>
+        <v>4.008</v>
       </c>
       <c r="N18" t="n">
-        <v>3.997</v>
+        <v>4.068</v>
       </c>
       <c r="O18" t="n">
-        <v>4.175</v>
+        <v>4.253</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.839</v>
+        <v>2.845</v>
       </c>
       <c r="G19" t="n">
-        <v>2.995</v>
+        <v>3.011</v>
       </c>
       <c r="H19" t="n">
-        <v>3.216</v>
+        <v>3.237</v>
       </c>
       <c r="I19" t="n">
-        <v>3.436</v>
+        <v>3.46</v>
       </c>
       <c r="J19" t="n">
-        <v>3.657</v>
+        <v>3.711</v>
       </c>
       <c r="K19" t="n">
-        <v>3.831</v>
+        <v>3.884</v>
       </c>
       <c r="L19" t="n">
-        <v>3.869</v>
+        <v>3.936</v>
       </c>
       <c r="M19" t="n">
-        <v>4.002</v>
+        <v>4.07</v>
       </c>
       <c r="N19" t="n">
-        <v>4.06</v>
+        <v>4.131</v>
       </c>
       <c r="O19" t="n">
-        <v>4.192</v>
+        <v>4.273</v>
       </c>
       <c r="P19" t="n">
-        <v>4.241</v>
+        <v>4.335</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.429</v>
+        <v>4.542</v>
       </c>
       <c r="R19" t="n">
-        <v>4.57</v>
+        <v>4.688</v>
       </c>
       <c r="S19" t="n">
-        <v>4.731</v>
+        <v>4.853</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.634</v>
+        <v>2.639</v>
       </c>
       <c r="G20" t="n">
-        <v>2.723</v>
+        <v>2.733</v>
       </c>
       <c r="H20" t="n">
-        <v>2.831</v>
+        <v>2.842</v>
       </c>
       <c r="I20" t="n">
-        <v>3.008</v>
+        <v>3.021</v>
       </c>
       <c r="J20" t="n">
-        <v>3.397</v>
+        <v>3.453</v>
       </c>
       <c r="K20" t="n">
-        <v>3.645</v>
+        <v>3.7</v>
       </c>
       <c r="L20" t="n">
-        <v>3.659</v>
+        <v>3.722</v>
       </c>
       <c r="M20" t="n">
-        <v>3.761</v>
+        <v>3.828</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.937</v>
+        <v>2.943</v>
       </c>
       <c r="G21" t="n">
-        <v>3.077</v>
+        <v>3.096</v>
       </c>
       <c r="H21" t="n">
-        <v>3.329</v>
+        <v>3.351</v>
       </c>
       <c r="I21" t="n">
-        <v>3.56</v>
+        <v>3.583</v>
       </c>
       <c r="J21" t="n">
-        <v>3.805</v>
+        <v>3.859</v>
       </c>
       <c r="K21" t="n">
-        <v>4.066</v>
+        <v>4.121</v>
       </c>
       <c r="L21" t="n">
-        <v>4.107</v>
+        <v>4.173</v>
       </c>
       <c r="M21" t="n">
-        <v>4.237</v>
+        <v>4.305</v>
       </c>
       <c r="N21" t="n">
-        <v>4.302</v>
+        <v>4.375</v>
       </c>
       <c r="O21" t="n">
-        <v>4.401</v>
+        <v>4.482</v>
       </c>
       <c r="P21" t="n">
-        <v>4.506</v>
+        <v>4.599</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.592</v>
+        <v>4.703</v>
       </c>
       <c r="R21" t="n">
-        <v>4.622</v>
+        <v>4.74</v>
       </c>
       <c r="S21" t="n">
-        <v>4.685</v>
+        <v>4.806</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.883</v>
+        <v>2.889</v>
       </c>
       <c r="G22" t="n">
-        <v>3.023</v>
+        <v>3.041</v>
       </c>
       <c r="H22" t="n">
-        <v>3.261</v>
+        <v>3.283</v>
       </c>
       <c r="I22" t="n">
-        <v>3.478</v>
+        <v>3.501</v>
       </c>
       <c r="J22" t="n">
-        <v>3.69</v>
+        <v>3.744</v>
       </c>
       <c r="K22" t="n">
-        <v>3.947</v>
+        <v>4.002</v>
       </c>
       <c r="L22" t="n">
-        <v>3.974</v>
+        <v>4.04</v>
       </c>
       <c r="M22" t="n">
-        <v>4.107</v>
+        <v>4.175</v>
       </c>
       <c r="N22" t="n">
-        <v>4.176</v>
+        <v>4.248</v>
       </c>
       <c r="O22" t="n">
-        <v>4.273</v>
+        <v>4.353</v>
       </c>
       <c r="P22" t="n">
-        <v>4.369</v>
+        <v>4.462</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.45</v>
+        <v>4.561</v>
       </c>
       <c r="R22" t="n">
-        <v>4.471</v>
+        <v>4.589</v>
       </c>
       <c r="S22" t="n">
-        <v>4.531</v>
+        <v>4.651</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.833</v>
+        <v>2.84</v>
       </c>
       <c r="G23" t="n">
-        <v>2.977</v>
+        <v>2.995</v>
       </c>
       <c r="H23" t="n">
-        <v>3.203</v>
+        <v>3.224</v>
       </c>
       <c r="I23" t="n">
-        <v>3.427</v>
+        <v>3.45</v>
       </c>
       <c r="J23" t="n">
-        <v>3.63</v>
+        <v>3.684</v>
       </c>
       <c r="K23" t="n">
-        <v>3.846</v>
+        <v>3.901</v>
       </c>
       <c r="L23" t="n">
-        <v>3.871</v>
+        <v>3.938</v>
       </c>
       <c r="M23" t="n">
-        <v>3.997</v>
+        <v>4.065</v>
       </c>
       <c r="N23" t="n">
-        <v>4.07</v>
+        <v>4.143</v>
       </c>
       <c r="O23" t="n">
-        <v>4.148</v>
+        <v>4.228</v>
       </c>
       <c r="P23" t="n">
-        <v>4.232</v>
+        <v>4.325</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.256</v>
+        <v>4.367</v>
       </c>
       <c r="R23" t="n">
-        <v>4.256</v>
+        <v>4.374</v>
       </c>
       <c r="S23" t="n">
-        <v>4.287</v>
+        <v>4.407</v>
       </c>
       <c r="T23" t="n">
-        <v>4.203</v>
+        <v>4.338</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.771</v>
+        <v>2.777</v>
       </c>
       <c r="G24" t="n">
-        <v>2.889</v>
+        <v>2.907</v>
       </c>
       <c r="H24" t="n">
-        <v>3.097</v>
+        <v>3.118</v>
       </c>
       <c r="I24" t="n">
-        <v>3.364</v>
+        <v>3.387</v>
       </c>
       <c r="J24" t="n">
-        <v>3.524</v>
+        <v>3.578</v>
       </c>
       <c r="K24" t="n">
-        <v>3.73</v>
+        <v>3.785</v>
       </c>
       <c r="L24" t="n">
-        <v>3.752</v>
+        <v>3.819</v>
       </c>
       <c r="M24" t="n">
-        <v>3.86</v>
+        <v>3.928</v>
       </c>
       <c r="N24" t="n">
-        <v>3.946</v>
+        <v>4.018</v>
       </c>
       <c r="O24" t="n">
-        <v>4.151</v>
+        <v>4.231</v>
       </c>
       <c r="P24" t="n">
-        <v>4.168</v>
+        <v>4.261</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.182</v>
+        <v>4.293</v>
       </c>
       <c r="R24" t="n">
-        <v>4.178</v>
+        <v>4.296</v>
       </c>
       <c r="S24" t="n">
-        <v>4.202</v>
+        <v>4.323</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.828</v>
+        <v>2.834</v>
       </c>
       <c r="G25" t="n">
-        <v>2.977</v>
+        <v>2.995</v>
       </c>
       <c r="H25" t="n">
-        <v>3.206</v>
+        <v>3.227</v>
       </c>
       <c r="I25" t="n">
-        <v>3.435</v>
+        <v>3.458</v>
       </c>
       <c r="J25" t="n">
-        <v>3.645</v>
+        <v>3.699</v>
       </c>
       <c r="K25" t="n">
-        <v>3.878</v>
+        <v>3.933</v>
       </c>
       <c r="L25" t="n">
-        <v>3.902</v>
+        <v>3.969</v>
       </c>
       <c r="M25" t="n">
-        <v>4.03</v>
+        <v>4.098</v>
       </c>
       <c r="N25" t="n">
-        <v>4.097</v>
+        <v>4.17</v>
       </c>
       <c r="O25" t="n">
-        <v>4.177</v>
+        <v>4.258</v>
       </c>
       <c r="P25" t="n">
-        <v>4.254</v>
+        <v>4.347</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.289</v>
+        <v>4.4</v>
       </c>
       <c r="R25" t="n">
-        <v>4.279</v>
+        <v>4.397</v>
       </c>
       <c r="S25" t="n">
-        <v>4.31</v>
+        <v>4.431</v>
       </c>
       <c r="T25" t="n">
-        <v>4.221</v>
+        <v>4.356</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.114</v>
+        <v>3.121</v>
       </c>
       <c r="G26" t="n">
-        <v>3.3</v>
+        <v>3.314</v>
       </c>
       <c r="H26" t="n">
-        <v>3.637</v>
+        <v>3.651</v>
       </c>
       <c r="I26" t="n">
-        <v>3.901</v>
+        <v>3.917</v>
       </c>
       <c r="J26" t="n">
-        <v>4.268</v>
+        <v>4.325</v>
       </c>
       <c r="K26" t="n">
-        <v>4.69</v>
+        <v>4.745</v>
       </c>
       <c r="L26" t="n">
-        <v>4.784</v>
+        <v>4.849</v>
       </c>
       <c r="M26" t="n">
-        <v>4.955</v>
+        <v>5.022</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.233</v>
+        <v>5.313</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.931</v>
+        <v>2.937</v>
       </c>
       <c r="G27" t="n">
-        <v>3.07</v>
+        <v>3.085</v>
       </c>
       <c r="H27" t="n">
-        <v>3.31</v>
+        <v>3.328</v>
       </c>
       <c r="I27" t="n">
-        <v>3.54</v>
+        <v>3.559</v>
       </c>
       <c r="J27" t="n">
-        <v>3.784</v>
+        <v>3.839</v>
       </c>
       <c r="K27" t="n">
-        <v>4.011</v>
+        <v>4.064</v>
       </c>
       <c r="L27" t="n">
-        <v>4.054</v>
+        <v>4.12</v>
       </c>
       <c r="M27" t="n">
-        <v>4.173</v>
+        <v>4.241</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.335</v>
+        <v>4.416</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.034</v>
+        <v>3.04</v>
       </c>
       <c r="G28" t="n">
-        <v>3.181</v>
+        <v>3.196</v>
       </c>
       <c r="H28" t="n">
-        <v>3.436</v>
+        <v>3.453</v>
       </c>
       <c r="I28" t="n">
-        <v>3.677</v>
+        <v>3.696</v>
       </c>
       <c r="J28" t="n">
-        <v>3.957</v>
+        <v>4.012</v>
       </c>
       <c r="K28" t="n">
-        <v>4.204</v>
+        <v>4.257</v>
       </c>
       <c r="L28" t="n">
-        <v>4.257</v>
+        <v>4.322</v>
       </c>
       <c r="M28" t="n">
-        <v>4.385</v>
+        <v>4.453</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.627</v>
+        <v>4.708</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.881</v>
+        <v>2.887</v>
       </c>
       <c r="G29" t="n">
-        <v>3.018</v>
+        <v>3.033</v>
       </c>
       <c r="H29" t="n">
-        <v>3.249</v>
+        <v>3.266</v>
       </c>
       <c r="I29" t="n">
-        <v>3.467</v>
+        <v>3.487</v>
       </c>
       <c r="J29" t="n">
-        <v>3.697</v>
+        <v>3.752</v>
       </c>
       <c r="K29" t="n">
-        <v>3.907</v>
+        <v>3.96</v>
       </c>
       <c r="L29" t="n">
-        <v>3.94</v>
+        <v>4.005</v>
       </c>
       <c r="M29" t="n">
-        <v>4.036</v>
+        <v>4.104</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.207</v>
+        <v>4.288</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.155</v>
+        <v>3.162</v>
       </c>
       <c r="G30" t="n">
-        <v>3.277</v>
+        <v>3.292</v>
       </c>
       <c r="H30" t="n">
-        <v>3.573</v>
+        <v>3.588</v>
       </c>
       <c r="I30" t="n">
-        <v>3.826</v>
+        <v>3.843</v>
       </c>
       <c r="J30" t="n">
-        <v>4.132</v>
+        <v>4.187</v>
       </c>
       <c r="K30" t="n">
-        <v>4.489</v>
+        <v>4.544</v>
       </c>
       <c r="L30" t="n">
-        <v>4.563</v>
+        <v>4.627</v>
       </c>
       <c r="M30" t="n">
-        <v>4.723</v>
+        <v>4.789</v>
       </c>
       <c r="N30" t="n">
-        <v>4.89</v>
+        <v>4.96</v>
       </c>
       <c r="O30" t="n">
-        <v>5.184</v>
+        <v>5.264</v>
       </c>
       <c r="P30" t="n">
-        <v>5.396</v>
+        <v>5.489</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.123</v>
+        <v>6.236</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.484</v>
+        <v>3.491</v>
       </c>
       <c r="G31" t="n">
-        <v>3.642</v>
+        <v>3.657</v>
       </c>
       <c r="H31" t="n">
-        <v>3.987</v>
+        <v>4.003</v>
       </c>
       <c r="I31" t="n">
-        <v>4.256</v>
+        <v>4.272</v>
       </c>
       <c r="J31" t="n">
-        <v>4.623</v>
+        <v>4.678</v>
       </c>
       <c r="K31" t="n">
-        <v>5.022</v>
+        <v>5.076</v>
       </c>
       <c r="L31" t="n">
-        <v>5.175</v>
+        <v>5.24</v>
       </c>
       <c r="M31" t="n">
-        <v>5.453</v>
+        <v>5.52</v>
       </c>
       <c r="N31" t="n">
-        <v>5.749</v>
+        <v>5.819</v>
       </c>
       <c r="O31" t="n">
-        <v>6.22</v>
+        <v>6.3</v>
       </c>
       <c r="P31" t="n">
-        <v>6.384</v>
+        <v>6.478</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.096</v>
+        <v>7.21</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.254</v>
+        <v>3.261</v>
       </c>
       <c r="G32" t="n">
-        <v>3.395</v>
+        <v>3.409</v>
       </c>
       <c r="H32" t="n">
-        <v>3.717</v>
+        <v>3.731</v>
       </c>
       <c r="I32" t="n">
-        <v>3.985</v>
+        <v>4.002</v>
       </c>
       <c r="J32" t="n">
-        <v>4.31</v>
+        <v>4.365</v>
       </c>
       <c r="K32" t="n">
-        <v>4.674</v>
+        <v>4.729</v>
       </c>
       <c r="L32" t="n">
-        <v>4.767</v>
+        <v>4.831</v>
       </c>
       <c r="M32" t="n">
-        <v>4.995</v>
+        <v>5.062</v>
       </c>
       <c r="N32" t="n">
-        <v>5.251</v>
+        <v>5.321</v>
       </c>
       <c r="O32" t="n">
-        <v>5.629</v>
+        <v>5.71</v>
       </c>
       <c r="P32" t="n">
-        <v>5.856</v>
+        <v>5.949</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.584</v>
+        <v>6.698</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.02</v>
+        <v>3.027</v>
       </c>
       <c r="G33" t="n">
-        <v>3.142</v>
+        <v>3.157</v>
       </c>
       <c r="H33" t="n">
-        <v>3.391</v>
+        <v>3.405</v>
       </c>
       <c r="I33" t="n">
-        <v>3.611</v>
+        <v>3.628</v>
       </c>
       <c r="J33" t="n">
-        <v>3.84</v>
+        <v>3.896</v>
       </c>
       <c r="K33" t="n">
-        <v>4.132</v>
+        <v>4.186</v>
       </c>
       <c r="L33" t="n">
-        <v>4.165</v>
+        <v>4.23</v>
       </c>
       <c r="M33" t="n">
-        <v>4.249</v>
+        <v>4.316</v>
       </c>
       <c r="N33" t="n">
-        <v>4.28</v>
+        <v>4.35</v>
       </c>
       <c r="O33" t="n">
-        <v>4.338</v>
+        <v>4.418</v>
       </c>
       <c r="P33" t="n">
-        <v>4.428</v>
+        <v>4.522</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.84</v>
+        <v>4.953</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.08</v>
+        <v>3.087</v>
       </c>
       <c r="G34" t="n">
-        <v>3.195</v>
+        <v>3.21</v>
       </c>
       <c r="H34" t="n">
-        <v>3.453</v>
+        <v>3.467</v>
       </c>
       <c r="I34" t="n">
-        <v>3.679</v>
+        <v>3.696</v>
       </c>
       <c r="J34" t="n">
-        <v>3.912</v>
+        <v>3.968</v>
       </c>
       <c r="K34" t="n">
-        <v>4.209</v>
+        <v>4.262</v>
       </c>
       <c r="L34" t="n">
-        <v>4.244</v>
+        <v>4.309</v>
       </c>
       <c r="M34" t="n">
-        <v>4.34</v>
+        <v>4.406</v>
       </c>
       <c r="N34" t="n">
-        <v>4.384</v>
+        <v>4.454</v>
       </c>
       <c r="O34" t="n">
-        <v>4.507</v>
+        <v>4.587</v>
       </c>
       <c r="P34" t="n">
-        <v>4.723</v>
+        <v>4.816</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.541</v>
+        <v>5.654</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.054</v>
+        <v>3.061</v>
       </c>
       <c r="G35" t="n">
-        <v>3.169</v>
+        <v>3.184</v>
       </c>
       <c r="H35" t="n">
-        <v>3.421</v>
+        <v>3.436</v>
       </c>
       <c r="I35" t="n">
-        <v>3.646</v>
+        <v>3.662</v>
       </c>
       <c r="J35" t="n">
-        <v>3.881</v>
+        <v>3.936</v>
       </c>
       <c r="K35" t="n">
-        <v>4.162</v>
+        <v>4.216</v>
       </c>
       <c r="L35" t="n">
-        <v>4.199</v>
+        <v>4.264</v>
       </c>
       <c r="M35" t="n">
-        <v>4.286</v>
+        <v>4.353</v>
       </c>
       <c r="N35" t="n">
-        <v>4.32</v>
+        <v>4.39</v>
       </c>
       <c r="O35" t="n">
-        <v>4.404</v>
+        <v>4.484</v>
       </c>
       <c r="P35" t="n">
-        <v>4.525</v>
+        <v>4.619</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.177</v>
+        <v>5.29</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.949</v>
+        <v>2.954</v>
       </c>
       <c r="G36" t="n">
-        <v>3.06</v>
+        <v>3.073</v>
       </c>
       <c r="H36" t="n">
-        <v>3.3</v>
+        <v>3.313</v>
       </c>
       <c r="I36" t="n">
-        <v>3.526</v>
+        <v>3.54</v>
       </c>
       <c r="J36" t="n">
-        <v>3.777</v>
+        <v>3.833</v>
       </c>
       <c r="K36" t="n">
-        <v>4.057</v>
+        <v>4.111</v>
       </c>
       <c r="L36" t="n">
-        <v>4.091</v>
+        <v>4.156</v>
       </c>
       <c r="M36" t="n">
-        <v>4.151</v>
+        <v>4.218</v>
       </c>
       <c r="N36" t="n">
-        <v>4.183</v>
+        <v>4.253</v>
       </c>
       <c r="O36" t="n">
-        <v>4.246</v>
+        <v>4.327</v>
       </c>
       <c r="P36" t="n">
-        <v>4.326</v>
+        <v>4.42</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.557</v>
+        <v>4.67</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.827</v>
+        <v>3.834</v>
       </c>
       <c r="G37" t="n">
-        <v>4.335</v>
+        <v>4.351</v>
       </c>
       <c r="H37" t="n">
-        <v>4.96</v>
+        <v>4.976</v>
       </c>
       <c r="I37" t="n">
-        <v>5.317</v>
+        <v>5.334</v>
       </c>
       <c r="J37" t="n">
-        <v>6.114</v>
+        <v>6.17</v>
       </c>
       <c r="K37" t="n">
-        <v>7.062</v>
+        <v>7.116</v>
       </c>
       <c r="L37" t="n">
-        <v>7.375</v>
+        <v>7.44</v>
       </c>
       <c r="M37" t="n">
-        <v>7.725</v>
+        <v>7.792</v>
       </c>
       <c r="N37" t="n">
-        <v>7.901</v>
+        <v>7.972</v>
       </c>
       <c r="O37" t="n">
-        <v>8.099</v>
+        <v>8.179</v>
       </c>
       <c r="P37" t="n">
-        <v>8.183999999999999</v>
+        <v>8.279</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.587</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.888</v>
+        <v>4.895</v>
       </c>
       <c r="G38" t="n">
-        <v>5.65</v>
+        <v>5.665</v>
       </c>
       <c r="H38" t="n">
-        <v>6.486</v>
+        <v>6.503</v>
       </c>
       <c r="I38" t="n">
-        <v>7</v>
+        <v>7.017</v>
       </c>
       <c r="J38" t="n">
-        <v>8.058</v>
+        <v>8.114000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.183999999999999</v>
+        <v>9.239000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.657999999999999</v>
+        <v>9.723000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>10.137</v>
+        <v>10.204</v>
       </c>
       <c r="N38" t="n">
-        <v>10.319</v>
+        <v>10.391</v>
       </c>
       <c r="O38" t="n">
-        <v>10.499</v>
+        <v>10.58</v>
       </c>
       <c r="P38" t="n">
-        <v>10.582</v>
+        <v>10.677</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.038</v>
+        <v>11.151</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.209</v>
+        <v>4.216</v>
       </c>
       <c r="G39" t="n">
-        <v>4.848</v>
+        <v>4.864</v>
       </c>
       <c r="H39" t="n">
-        <v>5.551</v>
+        <v>5.567</v>
       </c>
       <c r="I39" t="n">
-        <v>6.004</v>
+        <v>6.021</v>
       </c>
       <c r="J39" t="n">
-        <v>6.931</v>
+        <v>6.986</v>
       </c>
       <c r="K39" t="n">
-        <v>8.016999999999999</v>
+        <v>8.071</v>
       </c>
       <c r="L39" t="n">
-        <v>8.413</v>
+        <v>8.478</v>
       </c>
       <c r="M39" t="n">
-        <v>8.773999999999999</v>
+        <v>8.84</v>
       </c>
       <c r="N39" t="n">
-        <v>8.946999999999999</v>
+        <v>9.019</v>
       </c>
       <c r="O39" t="n">
-        <v>9.15</v>
+        <v>9.23</v>
       </c>
       <c r="P39" t="n">
-        <v>9.236000000000001</v>
+        <v>9.331</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.683</v>
+        <v>9.795999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.347</v>
+        <v>3.354</v>
       </c>
       <c r="G40" t="n">
-        <v>3.515</v>
+        <v>3.53</v>
       </c>
       <c r="H40" t="n">
-        <v>3.832</v>
+        <v>3.847</v>
       </c>
       <c r="I40" t="n">
-        <v>4.1</v>
+        <v>4.116</v>
       </c>
       <c r="J40" t="n">
-        <v>4.423</v>
+        <v>4.479</v>
       </c>
       <c r="K40" t="n">
-        <v>4.795</v>
+        <v>4.85</v>
       </c>
       <c r="L40" t="n">
-        <v>4.887</v>
+        <v>4.952</v>
       </c>
       <c r="M40" t="n">
-        <v>5.066</v>
+        <v>5.132</v>
       </c>
       <c r="N40" t="n">
-        <v>5.248</v>
+        <v>5.318</v>
       </c>
       <c r="O40" t="n">
-        <v>5.563</v>
+        <v>5.643</v>
       </c>
       <c r="P40" t="n">
-        <v>5.817</v>
+        <v>5.91</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.574</v>
+        <v>6.688</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.733</v>
+        <v>3.74</v>
       </c>
       <c r="G41" t="n">
-        <v>3.944</v>
+        <v>3.959</v>
       </c>
       <c r="H41" t="n">
-        <v>4.317</v>
+        <v>4.332</v>
       </c>
       <c r="I41" t="n">
-        <v>4.604</v>
+        <v>4.62</v>
       </c>
       <c r="J41" t="n">
-        <v>4.978</v>
+        <v>5.034</v>
       </c>
       <c r="K41" t="n">
-        <v>5.395</v>
+        <v>5.45</v>
       </c>
       <c r="L41" t="n">
-        <v>5.566</v>
+        <v>5.63</v>
       </c>
       <c r="M41" t="n">
-        <v>5.868</v>
+        <v>5.935</v>
       </c>
       <c r="N41" t="n">
-        <v>6.179</v>
+        <v>6.249</v>
       </c>
       <c r="O41" t="n">
-        <v>6.678</v>
+        <v>6.759</v>
       </c>
       <c r="P41" t="n">
-        <v>6.877</v>
+        <v>6.97</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.621</v>
+        <v>7.734</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.468</v>
+        <v>3.475</v>
       </c>
       <c r="G42" t="n">
-        <v>3.664</v>
+        <v>3.679</v>
       </c>
       <c r="H42" t="n">
-        <v>4.008</v>
+        <v>4.022</v>
       </c>
       <c r="I42" t="n">
-        <v>4.288</v>
+        <v>4.305</v>
       </c>
       <c r="J42" t="n">
-        <v>4.625</v>
+        <v>4.681</v>
       </c>
       <c r="K42" t="n">
-        <v>5.016</v>
+        <v>5.071</v>
       </c>
       <c r="L42" t="n">
-        <v>5.124</v>
+        <v>5.188</v>
       </c>
       <c r="M42" t="n">
-        <v>5.373</v>
+        <v>5.439</v>
       </c>
       <c r="N42" t="n">
-        <v>5.663</v>
+        <v>5.732</v>
       </c>
       <c r="O42" t="n">
-        <v>6.055</v>
+        <v>6.135</v>
       </c>
       <c r="P42" t="n">
-        <v>6.319</v>
+        <v>6.412</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.087</v>
+        <v>7.2</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.168</v>
+        <v>3.175</v>
       </c>
       <c r="G43" t="n">
-        <v>3.325</v>
+        <v>3.339</v>
       </c>
       <c r="H43" t="n">
-        <v>3.592</v>
+        <v>3.607</v>
       </c>
       <c r="I43" t="n">
-        <v>3.82</v>
+        <v>3.836</v>
       </c>
       <c r="J43" t="n">
-        <v>4.068</v>
+        <v>4.123</v>
       </c>
       <c r="K43" t="n">
-        <v>4.364</v>
+        <v>4.418</v>
       </c>
       <c r="L43" t="n">
-        <v>4.407</v>
+        <v>4.472</v>
       </c>
       <c r="M43" t="n">
-        <v>4.504</v>
+        <v>4.571</v>
       </c>
       <c r="N43" t="n">
-        <v>4.549</v>
+        <v>4.619</v>
       </c>
       <c r="O43" t="n">
-        <v>4.651</v>
+        <v>4.732</v>
       </c>
       <c r="P43" t="n">
-        <v>4.794</v>
+        <v>4.887</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.45</v>
+        <v>5.563</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46171</v>
+        <v>46174</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.027</v>
+        <v>3.032</v>
       </c>
       <c r="G44" t="n">
-        <v>3.169</v>
+        <v>3.182</v>
       </c>
       <c r="H44" t="n">
-        <v>3.424</v>
+        <v>3.436</v>
       </c>
       <c r="I44" t="n">
-        <v>3.653</v>
+        <v>3.667</v>
       </c>
       <c r="J44" t="n">
-        <v>3.918</v>
+        <v>3.973</v>
       </c>
       <c r="K44" t="n">
-        <v>4.209</v>
+        <v>4.263</v>
       </c>
       <c r="L44" t="n">
-        <v>4.252</v>
+        <v>4.317</v>
       </c>
       <c r="M44" t="n">
-        <v>4.322</v>
+        <v>4.388</v>
       </c>
       <c r="N44" t="n">
-        <v>4.365</v>
+        <v>4.435</v>
       </c>
       <c r="O44" t="n">
-        <v>4.447</v>
+        <v>4.527</v>
       </c>
       <c r="P44" t="n">
-        <v>4.556</v>
+        <v>4.65</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.821</v>
+        <v>4.934</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-02 ~ 2026-06-02
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.294</v>
+        <v>3.3</v>
       </c>
       <c r="G2" t="n">
-        <v>3.574</v>
+        <v>3.582</v>
       </c>
       <c r="H2" t="n">
-        <v>3.862</v>
+        <v>3.871</v>
       </c>
       <c r="I2" t="n">
-        <v>4.079</v>
+        <v>4.077</v>
       </c>
       <c r="J2" t="n">
-        <v>4.37</v>
+        <v>4.381</v>
       </c>
       <c r="K2" t="n">
-        <v>4.774</v>
+        <v>4.799</v>
       </c>
       <c r="L2" t="n">
-        <v>4.951</v>
+        <v>4.955</v>
       </c>
       <c r="M2" t="n">
-        <v>5.242</v>
+        <v>5.223</v>
       </c>
       <c r="N2" t="n">
-        <v>5.522</v>
+        <v>5.5</v>
       </c>
       <c r="O2" t="n">
-        <v>5.778</v>
+        <v>5.753</v>
       </c>
       <c r="P2" t="n">
-        <v>6.013</v>
+        <v>5.978</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.639</v>
+        <v>6.596</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.315</v>
+        <v>4.322</v>
       </c>
       <c r="G3" t="n">
-        <v>4.777</v>
+        <v>4.785</v>
       </c>
       <c r="H3" t="n">
-        <v>5.098</v>
+        <v>5.106</v>
       </c>
       <c r="I3" t="n">
-        <v>5.307</v>
+        <v>5.306</v>
       </c>
       <c r="J3" t="n">
-        <v>5.616</v>
+        <v>5.626</v>
       </c>
       <c r="K3" t="n">
-        <v>6.09</v>
+        <v>6.115</v>
       </c>
       <c r="L3" t="n">
-        <v>6.336</v>
+        <v>6.341</v>
       </c>
       <c r="M3" t="n">
-        <v>6.658</v>
+        <v>6.639</v>
       </c>
       <c r="N3" t="n">
-        <v>6.881</v>
+        <v>6.86</v>
       </c>
       <c r="O3" t="n">
-        <v>7.088</v>
+        <v>7.063</v>
       </c>
       <c r="P3" t="n">
-        <v>7.191</v>
+        <v>7.156</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.705</v>
+        <v>7.663</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.808</v>
+        <v>3.814</v>
       </c>
       <c r="G4" t="n">
-        <v>4.157</v>
+        <v>4.166</v>
       </c>
       <c r="H4" t="n">
-        <v>4.508</v>
+        <v>4.516</v>
       </c>
       <c r="I4" t="n">
-        <v>4.75</v>
+        <v>4.748</v>
       </c>
       <c r="J4" t="n">
-        <v>5.059</v>
+        <v>5.07</v>
       </c>
       <c r="K4" t="n">
-        <v>5.529</v>
+        <v>5.554</v>
       </c>
       <c r="L4" t="n">
-        <v>5.705</v>
+        <v>5.71</v>
       </c>
       <c r="M4" t="n">
-        <v>6.016</v>
+        <v>5.997</v>
       </c>
       <c r="N4" t="n">
-        <v>6.21</v>
+        <v>6.188</v>
       </c>
       <c r="O4" t="n">
-        <v>6.44</v>
+        <v>6.415</v>
       </c>
       <c r="P4" t="n">
-        <v>6.543</v>
+        <v>6.509</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.06</v>
+        <v>7.018</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.991</v>
+        <v>2.998</v>
       </c>
       <c r="G5" t="n">
-        <v>3.115</v>
+        <v>3.123</v>
       </c>
       <c r="H5" t="n">
-        <v>3.369</v>
+        <v>3.377</v>
       </c>
       <c r="I5" t="n">
-        <v>3.651</v>
+        <v>3.649</v>
       </c>
       <c r="J5" t="n">
-        <v>3.928</v>
+        <v>3.938</v>
       </c>
       <c r="K5" t="n">
-        <v>4.179</v>
+        <v>4.204</v>
       </c>
       <c r="L5" t="n">
-        <v>4.198</v>
+        <v>4.204</v>
       </c>
       <c r="M5" t="n">
-        <v>4.301</v>
+        <v>4.282</v>
       </c>
       <c r="N5" t="n">
-        <v>4.334</v>
+        <v>4.313</v>
       </c>
       <c r="O5" t="n">
-        <v>4.378</v>
+        <v>4.353</v>
       </c>
       <c r="P5" t="n">
-        <v>4.682</v>
+        <v>4.647</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.551</v>
+        <v>5.509</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.032</v>
+        <v>3.038</v>
       </c>
       <c r="G6" t="n">
-        <v>3.17</v>
+        <v>3.178</v>
       </c>
       <c r="H6" t="n">
-        <v>3.438</v>
+        <v>3.446</v>
       </c>
       <c r="I6" t="n">
-        <v>3.733</v>
+        <v>3.731</v>
       </c>
       <c r="J6" t="n">
-        <v>4.017</v>
+        <v>4.028</v>
       </c>
       <c r="K6" t="n">
-        <v>4.291</v>
+        <v>4.316</v>
       </c>
       <c r="L6" t="n">
-        <v>4.316</v>
+        <v>4.321</v>
       </c>
       <c r="M6" t="n">
-        <v>4.456</v>
+        <v>4.437</v>
       </c>
       <c r="N6" t="n">
-        <v>4.502</v>
+        <v>4.48</v>
       </c>
       <c r="O6" t="n">
-        <v>4.644</v>
+        <v>4.619</v>
       </c>
       <c r="P6" t="n">
-        <v>5.114</v>
+        <v>5.079</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.947</v>
+        <v>5.905</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.012</v>
+        <v>3.018</v>
       </c>
       <c r="G7" t="n">
-        <v>3.133</v>
+        <v>3.142</v>
       </c>
       <c r="H7" t="n">
-        <v>3.385</v>
+        <v>3.393</v>
       </c>
       <c r="I7" t="n">
-        <v>3.67</v>
+        <v>3.668</v>
       </c>
       <c r="J7" t="n">
-        <v>3.951</v>
+        <v>3.962</v>
       </c>
       <c r="K7" t="n">
-        <v>4.206</v>
+        <v>4.231</v>
       </c>
       <c r="L7" t="n">
-        <v>4.225</v>
+        <v>4.23</v>
       </c>
       <c r="M7" t="n">
-        <v>4.361</v>
+        <v>4.342</v>
       </c>
       <c r="N7" t="n">
-        <v>4.394</v>
+        <v>4.372</v>
       </c>
       <c r="O7" t="n">
-        <v>4.541</v>
+        <v>4.516</v>
       </c>
       <c r="P7" t="n">
-        <v>4.898</v>
+        <v>4.863</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.715</v>
+        <v>5.673</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.427</v>
+        <v>5.434</v>
       </c>
       <c r="G8" t="n">
-        <v>6.076</v>
+        <v>6.085</v>
       </c>
       <c r="H8" t="n">
-        <v>6.546</v>
+        <v>6.555</v>
       </c>
       <c r="I8" t="n">
-        <v>6.834</v>
+        <v>6.832</v>
       </c>
       <c r="J8" t="n">
-        <v>7.208</v>
+        <v>7.219</v>
       </c>
       <c r="K8" t="n">
-        <v>7.964</v>
+        <v>7.989</v>
       </c>
       <c r="L8" t="n">
-        <v>8.294</v>
+        <v>8.298999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.648999999999999</v>
+        <v>8.629</v>
       </c>
       <c r="N8" t="n">
-        <v>8.805999999999999</v>
+        <v>8.784000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.098000000000001</v>
+        <v>9.073</v>
       </c>
       <c r="P8" t="n">
-        <v>9.304</v>
+        <v>9.27</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.016</v>
+        <v>9.974</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,19 +1063,19 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.636</v>
+        <v>2.635</v>
       </c>
       <c r="G9" t="n">
         <v>2.737</v>
       </c>
       <c r="H9" t="n">
-        <v>2.945</v>
+        <v>2.942</v>
       </c>
       <c r="I9" t="n">
         <v>3.187</v>
       </c>
       <c r="J9" t="n">
-        <v>3.43</v>
+        <v>3.429</v>
       </c>
       <c r="K9" t="n">
         <v>3.685</v>
@@ -1084,36 +1084,36 @@
         <v>3.71</v>
       </c>
       <c r="M9" t="n">
-        <v>3.79</v>
+        <v>3.77</v>
       </c>
       <c r="N9" t="n">
-        <v>3.944</v>
+        <v>3.921</v>
       </c>
       <c r="O9" t="n">
-        <v>3.995</v>
+        <v>3.97</v>
       </c>
       <c r="P9" t="n">
-        <v>4.113</v>
+        <v>4.08</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.178</v>
+        <v>4.136</v>
       </c>
       <c r="R9" t="n">
-        <v>4.192</v>
+        <v>4.155</v>
       </c>
       <c r="S9" t="n">
-        <v>4.2</v>
+        <v>4.168</v>
       </c>
       <c r="T9" t="n">
-        <v>4.132</v>
+        <v>4.125</v>
       </c>
       <c r="U9" t="n">
-        <v>4.03</v>
+        <v>4.038</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.658</v>
+        <v>2.659</v>
       </c>
       <c r="G10" t="n">
-        <v>2.775</v>
+        <v>2.777</v>
       </c>
       <c r="H10" t="n">
-        <v>2.958</v>
+        <v>2.957</v>
       </c>
       <c r="I10" t="n">
-        <v>3.193</v>
+        <v>3.195</v>
       </c>
       <c r="J10" t="n">
         <v>3.457</v>
       </c>
       <c r="K10" t="n">
-        <v>3.715</v>
+        <v>3.717</v>
       </c>
       <c r="L10" t="n">
         <v>3.762</v>
       </c>
       <c r="M10" t="n">
-        <v>3.884</v>
+        <v>3.864</v>
       </c>
       <c r="N10" t="n">
-        <v>3.964</v>
+        <v>3.942</v>
       </c>
       <c r="O10" t="n">
-        <v>4.233</v>
+        <v>4.205</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.468</v>
+        <v>2.469</v>
       </c>
       <c r="G11" t="n">
-        <v>2.582</v>
+        <v>2.584</v>
       </c>
       <c r="H11" t="n">
         <v>2.781</v>
       </c>
       <c r="I11" t="n">
-        <v>2.997</v>
+        <v>2.999</v>
       </c>
       <c r="J11" t="n">
-        <v>3.253</v>
+        <v>3.254</v>
       </c>
       <c r="K11" t="n">
-        <v>3.502</v>
+        <v>3.504</v>
       </c>
       <c r="L11" t="n">
         <v>3.56</v>
       </c>
       <c r="M11" t="n">
-        <v>3.692</v>
+        <v>3.672</v>
       </c>
       <c r="N11" t="n">
-        <v>3.772</v>
+        <v>3.75</v>
       </c>
       <c r="O11" t="n">
-        <v>3.999</v>
+        <v>3.972</v>
       </c>
       <c r="P11" t="n">
-        <v>4.064</v>
+        <v>4.03</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.379</v>
+        <v>4.336</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.283</v>
+        <v>3.292</v>
       </c>
       <c r="G12" t="n">
-        <v>3.528</v>
+        <v>3.537</v>
       </c>
       <c r="H12" t="n">
-        <v>3.781</v>
+        <v>3.79</v>
       </c>
       <c r="I12" t="n">
-        <v>4.045</v>
+        <v>4.051</v>
       </c>
       <c r="J12" t="n">
-        <v>4.354</v>
+        <v>4.367</v>
       </c>
       <c r="K12" t="n">
-        <v>4.568</v>
+        <v>4.592</v>
       </c>
       <c r="L12" t="n">
         <v>4.627</v>
       </c>
       <c r="M12" t="n">
-        <v>4.766</v>
+        <v>4.748</v>
       </c>
       <c r="N12" t="n">
-        <v>4.834</v>
+        <v>4.812</v>
       </c>
       <c r="O12" t="n">
-        <v>5</v>
+        <v>4.977</v>
       </c>
       <c r="P12" t="n">
-        <v>5.15</v>
+        <v>5.118</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.492</v>
+        <v>5.45</v>
       </c>
       <c r="R12" t="n">
-        <v>5.683</v>
+        <v>5.646</v>
       </c>
       <c r="S12" t="n">
-        <v>5.903</v>
+        <v>5.871</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.037</v>
+        <v>3.045</v>
       </c>
       <c r="G13" t="n">
-        <v>3.218</v>
+        <v>3.227</v>
       </c>
       <c r="H13" t="n">
-        <v>3.448</v>
+        <v>3.457</v>
       </c>
       <c r="I13" t="n">
-        <v>3.692</v>
+        <v>3.699</v>
       </c>
       <c r="J13" t="n">
-        <v>3.99</v>
+        <v>4.003</v>
       </c>
       <c r="K13" t="n">
-        <v>4.201</v>
+        <v>4.225</v>
       </c>
       <c r="L13" t="n">
-        <v>4.266</v>
+        <v>4.267</v>
       </c>
       <c r="M13" t="n">
-        <v>4.394</v>
+        <v>4.376</v>
       </c>
       <c r="N13" t="n">
-        <v>4.462</v>
+        <v>4.44</v>
       </c>
       <c r="O13" t="n">
-        <v>4.629</v>
+        <v>4.606</v>
       </c>
       <c r="P13" t="n">
-        <v>4.741</v>
+        <v>4.709</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.014</v>
+        <v>4.971</v>
       </c>
       <c r="R13" t="n">
-        <v>5.232</v>
+        <v>5.196</v>
       </c>
       <c r="S13" t="n">
-        <v>5.465</v>
+        <v>5.434</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.856</v>
+        <v>2.863</v>
       </c>
       <c r="G14" t="n">
-        <v>3.023</v>
+        <v>3.032</v>
       </c>
       <c r="H14" t="n">
-        <v>3.251</v>
+        <v>3.261</v>
       </c>
       <c r="I14" t="n">
-        <v>3.477</v>
+        <v>3.484</v>
       </c>
       <c r="J14" t="n">
-        <v>3.732</v>
+        <v>3.745</v>
       </c>
       <c r="K14" t="n">
-        <v>3.889</v>
+        <v>3.913</v>
       </c>
       <c r="L14" t="n">
-        <v>3.939</v>
+        <v>3.94</v>
       </c>
       <c r="M14" t="n">
-        <v>4.08</v>
+        <v>4.062</v>
       </c>
       <c r="N14" t="n">
-        <v>4.142</v>
+        <v>4.12</v>
       </c>
       <c r="O14" t="n">
-        <v>4.287</v>
+        <v>4.264</v>
       </c>
       <c r="P14" t="n">
-        <v>4.377</v>
+        <v>4.345</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.603</v>
+        <v>4.561</v>
       </c>
       <c r="R14" t="n">
-        <v>4.747</v>
+        <v>4.71</v>
       </c>
       <c r="S14" t="n">
-        <v>4.918</v>
+        <v>4.886</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.834</v>
+        <v>2.84</v>
       </c>
       <c r="G15" t="n">
-        <v>2.998</v>
+        <v>3.007</v>
       </c>
       <c r="H15" t="n">
-        <v>3.222</v>
+        <v>3.232</v>
       </c>
       <c r="I15" t="n">
-        <v>3.428</v>
+        <v>3.435</v>
       </c>
       <c r="J15" t="n">
-        <v>3.671</v>
+        <v>3.684</v>
       </c>
       <c r="K15" t="n">
-        <v>3.841</v>
+        <v>3.865</v>
       </c>
       <c r="L15" t="n">
-        <v>3.875</v>
+        <v>3.876</v>
       </c>
       <c r="M15" t="n">
-        <v>3.993</v>
+        <v>3.975</v>
       </c>
       <c r="N15" t="n">
-        <v>4.045</v>
+        <v>4.023</v>
       </c>
       <c r="O15" t="n">
-        <v>4.232</v>
+        <v>4.208</v>
       </c>
       <c r="P15" t="n">
-        <v>4.275</v>
+        <v>4.242</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.505</v>
+        <v>4.463</v>
       </c>
       <c r="R15" t="n">
-        <v>4.641</v>
+        <v>4.604</v>
       </c>
       <c r="S15" t="n">
-        <v>4.813</v>
+        <v>4.782</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.834</v>
+        <v>2.84</v>
       </c>
       <c r="G16" t="n">
-        <v>2.998</v>
+        <v>3.007</v>
       </c>
       <c r="H16" t="n">
-        <v>3.222</v>
+        <v>3.232</v>
       </c>
       <c r="I16" t="n">
-        <v>3.428</v>
+        <v>3.435</v>
       </c>
       <c r="J16" t="n">
-        <v>3.671</v>
+        <v>3.684</v>
       </c>
       <c r="K16" t="n">
-        <v>3.841</v>
+        <v>3.865</v>
       </c>
       <c r="L16" t="n">
-        <v>3.875</v>
+        <v>3.876</v>
       </c>
       <c r="M16" t="n">
-        <v>3.993</v>
+        <v>3.975</v>
       </c>
       <c r="N16" t="n">
-        <v>4.048</v>
+        <v>4.026</v>
       </c>
       <c r="O16" t="n">
-        <v>4.238</v>
+        <v>4.214</v>
       </c>
       <c r="P16" t="n">
-        <v>4.298</v>
+        <v>4.266</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.532</v>
+        <v>4.49</v>
       </c>
       <c r="R16" t="n">
-        <v>4.669</v>
+        <v>4.633</v>
       </c>
       <c r="S16" t="n">
-        <v>4.842</v>
+        <v>4.81</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.713</v>
+        <v>2.714</v>
       </c>
       <c r="G17" t="n">
-        <v>2.861</v>
+        <v>2.863</v>
       </c>
       <c r="H17" t="n">
         <v>3.05</v>
       </c>
       <c r="I17" t="n">
-        <v>3.275</v>
+        <v>3.277</v>
       </c>
       <c r="J17" t="n">
         <v>3.531</v>
       </c>
       <c r="K17" t="n">
-        <v>3.793</v>
+        <v>3.795</v>
       </c>
       <c r="L17" t="n">
         <v>3.846</v>
       </c>
       <c r="M17" t="n">
-        <v>4.008</v>
+        <v>3.987</v>
       </c>
       <c r="N17" t="n">
-        <v>4.067</v>
+        <v>4.045</v>
       </c>
       <c r="O17" t="n">
-        <v>4.254</v>
+        <v>4.226</v>
       </c>
       <c r="P17" t="n">
-        <v>4.345</v>
+        <v>4.311</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.714</v>
+        <v>2.715</v>
       </c>
       <c r="G18" t="n">
-        <v>2.862</v>
+        <v>2.864</v>
       </c>
       <c r="H18" t="n">
         <v>3.05</v>
       </c>
       <c r="I18" t="n">
-        <v>3.276</v>
+        <v>3.278</v>
       </c>
       <c r="J18" t="n">
         <v>3.531</v>
       </c>
       <c r="K18" t="n">
-        <v>3.794</v>
+        <v>3.796</v>
       </c>
       <c r="L18" t="n">
         <v>3.846</v>
       </c>
       <c r="M18" t="n">
-        <v>4.008</v>
+        <v>3.987</v>
       </c>
       <c r="N18" t="n">
-        <v>4.068</v>
+        <v>4.045</v>
       </c>
       <c r="O18" t="n">
-        <v>4.253</v>
+        <v>4.225</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.845</v>
+        <v>2.852</v>
       </c>
       <c r="G19" t="n">
-        <v>3.011</v>
+        <v>3.02</v>
       </c>
       <c r="H19" t="n">
-        <v>3.237</v>
+        <v>3.246</v>
       </c>
       <c r="I19" t="n">
-        <v>3.46</v>
+        <v>3.467</v>
       </c>
       <c r="J19" t="n">
-        <v>3.711</v>
+        <v>3.724</v>
       </c>
       <c r="K19" t="n">
-        <v>3.884</v>
+        <v>3.908</v>
       </c>
       <c r="L19" t="n">
-        <v>3.936</v>
+        <v>3.937</v>
       </c>
       <c r="M19" t="n">
-        <v>4.07</v>
+        <v>4.052</v>
       </c>
       <c r="N19" t="n">
-        <v>4.131</v>
+        <v>4.109</v>
       </c>
       <c r="O19" t="n">
-        <v>4.273</v>
+        <v>4.25</v>
       </c>
       <c r="P19" t="n">
-        <v>4.335</v>
+        <v>4.303</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.542</v>
+        <v>4.5</v>
       </c>
       <c r="R19" t="n">
-        <v>4.688</v>
+        <v>4.652</v>
       </c>
       <c r="S19" t="n">
-        <v>4.853</v>
+        <v>4.822</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.639</v>
       </c>
       <c r="G20" t="n">
-        <v>2.733</v>
+        <v>2.734</v>
       </c>
       <c r="H20" t="n">
-        <v>2.842</v>
+        <v>2.843</v>
       </c>
       <c r="I20" t="n">
-        <v>3.021</v>
+        <v>3.018</v>
       </c>
       <c r="J20" t="n">
-        <v>3.453</v>
+        <v>3.46</v>
       </c>
       <c r="K20" t="n">
-        <v>3.7</v>
+        <v>3.725</v>
       </c>
       <c r="L20" t="n">
-        <v>3.722</v>
+        <v>3.723</v>
       </c>
       <c r="M20" t="n">
-        <v>3.828</v>
+        <v>3.809</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.943</v>
+        <v>2.947</v>
       </c>
       <c r="G21" t="n">
-        <v>3.096</v>
+        <v>3.104</v>
       </c>
       <c r="H21" t="n">
-        <v>3.351</v>
+        <v>3.36</v>
       </c>
       <c r="I21" t="n">
-        <v>3.583</v>
+        <v>3.585</v>
       </c>
       <c r="J21" t="n">
-        <v>3.859</v>
+        <v>3.868</v>
       </c>
       <c r="K21" t="n">
-        <v>4.121</v>
+        <v>4.148</v>
       </c>
       <c r="L21" t="n">
-        <v>4.173</v>
+        <v>4.176</v>
       </c>
       <c r="M21" t="n">
-        <v>4.305</v>
+        <v>4.287</v>
       </c>
       <c r="N21" t="n">
-        <v>4.375</v>
+        <v>4.354</v>
       </c>
       <c r="O21" t="n">
-        <v>4.482</v>
+        <v>4.457</v>
       </c>
       <c r="P21" t="n">
-        <v>4.599</v>
+        <v>4.565</v>
       </c>
       <c r="Q21" t="n">
+        <v>4.661</v>
+      </c>
+      <c r="R21" t="n">
         <v>4.703</v>
       </c>
-      <c r="R21" t="n">
-        <v>4.74</v>
-      </c>
       <c r="S21" t="n">
-        <v>4.806</v>
+        <v>4.774</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.889</v>
+        <v>2.893</v>
       </c>
       <c r="G22" t="n">
-        <v>3.041</v>
+        <v>3.05</v>
       </c>
       <c r="H22" t="n">
-        <v>3.283</v>
+        <v>3.291</v>
       </c>
       <c r="I22" t="n">
-        <v>3.501</v>
+        <v>3.503</v>
       </c>
       <c r="J22" t="n">
-        <v>3.744</v>
+        <v>3.753</v>
       </c>
       <c r="K22" t="n">
-        <v>4.002</v>
+        <v>4.029</v>
       </c>
       <c r="L22" t="n">
-        <v>4.04</v>
+        <v>4.043</v>
       </c>
       <c r="M22" t="n">
-        <v>4.175</v>
+        <v>4.157</v>
       </c>
       <c r="N22" t="n">
-        <v>4.248</v>
+        <v>4.228</v>
       </c>
       <c r="O22" t="n">
-        <v>4.353</v>
+        <v>4.328</v>
       </c>
       <c r="P22" t="n">
-        <v>4.462</v>
+        <v>4.429</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.561</v>
+        <v>4.52</v>
       </c>
       <c r="R22" t="n">
-        <v>4.589</v>
+        <v>4.551</v>
       </c>
       <c r="S22" t="n">
-        <v>4.651</v>
+        <v>4.62</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.84</v>
+        <v>2.844</v>
       </c>
       <c r="G23" t="n">
-        <v>2.995</v>
+        <v>3.004</v>
       </c>
       <c r="H23" t="n">
-        <v>3.224</v>
+        <v>3.232</v>
       </c>
       <c r="I23" t="n">
-        <v>3.45</v>
+        <v>3.451</v>
       </c>
       <c r="J23" t="n">
-        <v>3.684</v>
+        <v>3.693</v>
       </c>
       <c r="K23" t="n">
-        <v>3.901</v>
+        <v>3.929</v>
       </c>
       <c r="L23" t="n">
-        <v>3.938</v>
+        <v>3.941</v>
       </c>
       <c r="M23" t="n">
-        <v>4.065</v>
+        <v>4.049</v>
       </c>
       <c r="N23" t="n">
-        <v>4.143</v>
+        <v>4.122</v>
       </c>
       <c r="O23" t="n">
-        <v>4.228</v>
+        <v>4.204</v>
       </c>
       <c r="P23" t="n">
-        <v>4.325</v>
+        <v>4.292</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.367</v>
+        <v>4.326</v>
       </c>
       <c r="R23" t="n">
-        <v>4.374</v>
+        <v>4.337</v>
       </c>
       <c r="S23" t="n">
-        <v>4.407</v>
+        <v>4.376</v>
       </c>
       <c r="T23" t="n">
-        <v>4.338</v>
+        <v>4.332</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.777</v>
+        <v>2.781</v>
       </c>
       <c r="G24" t="n">
-        <v>2.907</v>
+        <v>2.915</v>
       </c>
       <c r="H24" t="n">
-        <v>3.118</v>
+        <v>3.126</v>
       </c>
       <c r="I24" t="n">
-        <v>3.387</v>
+        <v>3.389</v>
       </c>
       <c r="J24" t="n">
-        <v>3.578</v>
+        <v>3.586</v>
       </c>
       <c r="K24" t="n">
-        <v>3.785</v>
+        <v>3.812</v>
       </c>
       <c r="L24" t="n">
-        <v>3.819</v>
+        <v>3.822</v>
       </c>
       <c r="M24" t="n">
-        <v>3.928</v>
+        <v>3.91</v>
       </c>
       <c r="N24" t="n">
-        <v>4.018</v>
+        <v>3.997</v>
       </c>
       <c r="O24" t="n">
-        <v>4.231</v>
+        <v>4.205</v>
       </c>
       <c r="P24" t="n">
-        <v>4.261</v>
+        <v>4.228</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.293</v>
+        <v>4.251</v>
       </c>
       <c r="R24" t="n">
-        <v>4.296</v>
+        <v>4.259</v>
       </c>
       <c r="S24" t="n">
-        <v>4.323</v>
+        <v>4.291</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.834</v>
+        <v>2.838</v>
       </c>
       <c r="G25" t="n">
-        <v>2.995</v>
+        <v>3.004</v>
       </c>
       <c r="H25" t="n">
-        <v>3.227</v>
+        <v>3.236</v>
       </c>
       <c r="I25" t="n">
-        <v>3.458</v>
+        <v>3.46</v>
       </c>
       <c r="J25" t="n">
-        <v>3.699</v>
+        <v>3.708</v>
       </c>
       <c r="K25" t="n">
-        <v>3.933</v>
+        <v>3.96</v>
       </c>
       <c r="L25" t="n">
-        <v>3.969</v>
+        <v>3.972</v>
       </c>
       <c r="M25" t="n">
-        <v>4.098</v>
+        <v>4.08</v>
       </c>
       <c r="N25" t="n">
-        <v>4.17</v>
+        <v>4.149</v>
       </c>
       <c r="O25" t="n">
-        <v>4.258</v>
+        <v>4.233</v>
       </c>
       <c r="P25" t="n">
-        <v>4.347</v>
+        <v>4.313</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.4</v>
+        <v>4.359</v>
       </c>
       <c r="R25" t="n">
-        <v>4.397</v>
+        <v>4.361</v>
       </c>
       <c r="S25" t="n">
-        <v>4.431</v>
+        <v>4.399</v>
       </c>
       <c r="T25" t="n">
-        <v>4.356</v>
+        <v>4.35</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.121</v>
+        <v>3.126</v>
       </c>
       <c r="G26" t="n">
-        <v>3.314</v>
+        <v>3.32</v>
       </c>
       <c r="H26" t="n">
-        <v>3.651</v>
+        <v>3.658</v>
       </c>
       <c r="I26" t="n">
-        <v>3.917</v>
+        <v>3.92</v>
       </c>
       <c r="J26" t="n">
-        <v>4.325</v>
+        <v>4.334</v>
       </c>
       <c r="K26" t="n">
-        <v>4.745</v>
+        <v>4.769</v>
       </c>
       <c r="L26" t="n">
-        <v>4.849</v>
+        <v>4.85</v>
       </c>
       <c r="M26" t="n">
-        <v>5.022</v>
+        <v>5.003</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.313</v>
+        <v>5.288</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.937</v>
+        <v>2.944</v>
       </c>
       <c r="G27" t="n">
-        <v>3.085</v>
+        <v>3.093</v>
       </c>
       <c r="H27" t="n">
-        <v>3.328</v>
+        <v>3.336</v>
       </c>
       <c r="I27" t="n">
-        <v>3.559</v>
+        <v>3.564</v>
       </c>
       <c r="J27" t="n">
-        <v>3.839</v>
+        <v>3.851</v>
       </c>
       <c r="K27" t="n">
-        <v>4.064</v>
+        <v>4.087</v>
       </c>
       <c r="L27" t="n">
-        <v>4.12</v>
+        <v>4.119</v>
       </c>
       <c r="M27" t="n">
-        <v>4.241</v>
+        <v>4.222</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.416</v>
+        <v>4.391</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.04</v>
+        <v>3.047</v>
       </c>
       <c r="G28" t="n">
-        <v>3.196</v>
+        <v>3.204</v>
       </c>
       <c r="H28" t="n">
-        <v>3.453</v>
+        <v>3.461</v>
       </c>
       <c r="I28" t="n">
-        <v>3.696</v>
+        <v>3.7</v>
       </c>
       <c r="J28" t="n">
-        <v>4.012</v>
+        <v>4.024</v>
       </c>
       <c r="K28" t="n">
-        <v>4.257</v>
+        <v>4.279</v>
       </c>
       <c r="L28" t="n">
         <v>4.322</v>
       </c>
       <c r="M28" t="n">
-        <v>4.453</v>
+        <v>4.434</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.708</v>
+        <v>4.683</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.887</v>
+        <v>2.893</v>
       </c>
       <c r="G29" t="n">
-        <v>3.033</v>
+        <v>3.04</v>
       </c>
       <c r="H29" t="n">
-        <v>3.266</v>
+        <v>3.275</v>
       </c>
       <c r="I29" t="n">
-        <v>3.487</v>
+        <v>3.491</v>
       </c>
       <c r="J29" t="n">
-        <v>3.752</v>
+        <v>3.763</v>
       </c>
       <c r="K29" t="n">
-        <v>3.96</v>
+        <v>3.983</v>
       </c>
       <c r="L29" t="n">
         <v>4.005</v>
       </c>
       <c r="M29" t="n">
-        <v>4.104</v>
+        <v>4.085</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.288</v>
+        <v>4.263</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.162</v>
+        <v>3.167</v>
       </c>
       <c r="G30" t="n">
-        <v>3.292</v>
+        <v>3.298</v>
       </c>
       <c r="H30" t="n">
-        <v>3.588</v>
+        <v>3.595</v>
       </c>
       <c r="I30" t="n">
-        <v>3.843</v>
+        <v>3.847</v>
       </c>
       <c r="J30" t="n">
-        <v>4.187</v>
+        <v>4.195</v>
       </c>
       <c r="K30" t="n">
-        <v>4.544</v>
+        <v>4.567</v>
       </c>
       <c r="L30" t="n">
         <v>4.627</v>
       </c>
       <c r="M30" t="n">
-        <v>4.789</v>
+        <v>4.769</v>
       </c>
       <c r="N30" t="n">
-        <v>4.96</v>
+        <v>4.938</v>
       </c>
       <c r="O30" t="n">
-        <v>5.264</v>
+        <v>5.239</v>
       </c>
       <c r="P30" t="n">
-        <v>5.489</v>
+        <v>5.455</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.236</v>
+        <v>6.194</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.491</v>
+        <v>3.496</v>
       </c>
       <c r="G31" t="n">
-        <v>3.657</v>
+        <v>3.663</v>
       </c>
       <c r="H31" t="n">
-        <v>4.003</v>
+        <v>4.01</v>
       </c>
       <c r="I31" t="n">
-        <v>4.272</v>
+        <v>4.276</v>
       </c>
       <c r="J31" t="n">
-        <v>4.678</v>
+        <v>4.686</v>
       </c>
       <c r="K31" t="n">
-        <v>5.076</v>
+        <v>5.099</v>
       </c>
       <c r="L31" t="n">
-        <v>5.24</v>
+        <v>5.239</v>
       </c>
       <c r="M31" t="n">
-        <v>5.52</v>
+        <v>5.5</v>
       </c>
       <c r="N31" t="n">
-        <v>5.819</v>
+        <v>5.797</v>
       </c>
       <c r="O31" t="n">
-        <v>6.3</v>
+        <v>6.275</v>
       </c>
       <c r="P31" t="n">
-        <v>6.478</v>
+        <v>6.444</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.21</v>
+        <v>7.168</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.261</v>
+        <v>3.265</v>
       </c>
       <c r="G32" t="n">
-        <v>3.409</v>
+        <v>3.415</v>
       </c>
       <c r="H32" t="n">
-        <v>3.731</v>
+        <v>3.738</v>
       </c>
       <c r="I32" t="n">
-        <v>4.002</v>
+        <v>4.006</v>
       </c>
       <c r="J32" t="n">
-        <v>4.365</v>
+        <v>4.373</v>
       </c>
       <c r="K32" t="n">
-        <v>4.729</v>
+        <v>4.752</v>
       </c>
       <c r="L32" t="n">
         <v>4.831</v>
       </c>
       <c r="M32" t="n">
-        <v>5.062</v>
+        <v>5.042</v>
       </c>
       <c r="N32" t="n">
-        <v>5.321</v>
+        <v>5.299</v>
       </c>
       <c r="O32" t="n">
-        <v>5.71</v>
+        <v>5.684</v>
       </c>
       <c r="P32" t="n">
-        <v>5.949</v>
+        <v>5.915</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.698</v>
+        <v>6.656</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.027</v>
+        <v>3.032</v>
       </c>
       <c r="G33" t="n">
-        <v>3.157</v>
+        <v>3.163</v>
       </c>
       <c r="H33" t="n">
-        <v>3.405</v>
+        <v>3.412</v>
       </c>
       <c r="I33" t="n">
-        <v>3.628</v>
+        <v>3.632</v>
       </c>
       <c r="J33" t="n">
-        <v>3.896</v>
+        <v>3.905</v>
       </c>
       <c r="K33" t="n">
-        <v>4.186</v>
+        <v>4.21</v>
       </c>
       <c r="L33" t="n">
         <v>4.23</v>
       </c>
       <c r="M33" t="n">
-        <v>4.316</v>
+        <v>4.296</v>
       </c>
       <c r="N33" t="n">
-        <v>4.35</v>
+        <v>4.328</v>
       </c>
       <c r="O33" t="n">
-        <v>4.418</v>
+        <v>4.393</v>
       </c>
       <c r="P33" t="n">
-        <v>4.522</v>
+        <v>4.488</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.953</v>
+        <v>4.911</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.087</v>
+        <v>3.092</v>
       </c>
       <c r="G34" t="n">
-        <v>3.21</v>
+        <v>3.216</v>
       </c>
       <c r="H34" t="n">
-        <v>3.467</v>
+        <v>3.474</v>
       </c>
       <c r="I34" t="n">
-        <v>3.696</v>
+        <v>3.7</v>
       </c>
       <c r="J34" t="n">
-        <v>3.968</v>
+        <v>3.976</v>
       </c>
       <c r="K34" t="n">
-        <v>4.262</v>
+        <v>4.286</v>
       </c>
       <c r="L34" t="n">
         <v>4.309</v>
       </c>
       <c r="M34" t="n">
-        <v>4.406</v>
+        <v>4.386</v>
       </c>
       <c r="N34" t="n">
-        <v>4.454</v>
+        <v>4.432</v>
       </c>
       <c r="O34" t="n">
-        <v>4.587</v>
+        <v>4.562</v>
       </c>
       <c r="P34" t="n">
-        <v>4.816</v>
+        <v>4.782</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.654</v>
+        <v>5.612</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.061</v>
+        <v>3.066</v>
       </c>
       <c r="G35" t="n">
-        <v>3.184</v>
+        <v>3.19</v>
       </c>
       <c r="H35" t="n">
-        <v>3.436</v>
+        <v>3.443</v>
       </c>
       <c r="I35" t="n">
-        <v>3.662</v>
+        <v>3.666</v>
       </c>
       <c r="J35" t="n">
-        <v>3.936</v>
+        <v>3.945</v>
       </c>
       <c r="K35" t="n">
-        <v>4.216</v>
+        <v>4.24</v>
       </c>
       <c r="L35" t="n">
         <v>4.264</v>
       </c>
       <c r="M35" t="n">
-        <v>4.353</v>
+        <v>4.333</v>
       </c>
       <c r="N35" t="n">
-        <v>4.39</v>
+        <v>4.368</v>
       </c>
       <c r="O35" t="n">
-        <v>4.484</v>
+        <v>4.459</v>
       </c>
       <c r="P35" t="n">
-        <v>4.619</v>
+        <v>4.585</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.29</v>
+        <v>5.248</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.954</v>
+        <v>2.957</v>
       </c>
       <c r="G36" t="n">
-        <v>3.073</v>
+        <v>3.077</v>
       </c>
       <c r="H36" t="n">
-        <v>3.313</v>
+        <v>3.32</v>
       </c>
       <c r="I36" t="n">
-        <v>3.54</v>
+        <v>3.543</v>
       </c>
       <c r="J36" t="n">
-        <v>3.833</v>
+        <v>3.841</v>
       </c>
       <c r="K36" t="n">
-        <v>4.111</v>
+        <v>4.135</v>
       </c>
       <c r="L36" t="n">
         <v>4.156</v>
       </c>
       <c r="M36" t="n">
-        <v>4.218</v>
+        <v>4.199</v>
       </c>
       <c r="N36" t="n">
-        <v>4.253</v>
+        <v>4.232</v>
       </c>
       <c r="O36" t="n">
-        <v>4.327</v>
+        <v>4.301</v>
       </c>
       <c r="P36" t="n">
-        <v>4.42</v>
+        <v>4.386</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.67</v>
+        <v>4.628</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.834</v>
+        <v>3.839</v>
       </c>
       <c r="G37" t="n">
-        <v>4.351</v>
+        <v>4.357</v>
       </c>
       <c r="H37" t="n">
-        <v>4.976</v>
+        <v>4.983</v>
       </c>
       <c r="I37" t="n">
-        <v>5.334</v>
+        <v>5.337</v>
       </c>
       <c r="J37" t="n">
-        <v>6.17</v>
+        <v>6.177</v>
       </c>
       <c r="K37" t="n">
-        <v>7.116</v>
+        <v>7.139</v>
       </c>
       <c r="L37" t="n">
         <v>7.44</v>
       </c>
       <c r="M37" t="n">
-        <v>7.792</v>
+        <v>7.772</v>
       </c>
       <c r="N37" t="n">
-        <v>7.972</v>
+        <v>7.952</v>
       </c>
       <c r="O37" t="n">
-        <v>8.179</v>
+        <v>8.154</v>
       </c>
       <c r="P37" t="n">
-        <v>8.279</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.699999999999999</v>
+        <v>8.657999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.895</v>
+        <v>4.9</v>
       </c>
       <c r="G38" t="n">
-        <v>5.665</v>
+        <v>5.672</v>
       </c>
       <c r="H38" t="n">
-        <v>6.503</v>
+        <v>6.51</v>
       </c>
       <c r="I38" t="n">
-        <v>7.017</v>
+        <v>7.021</v>
       </c>
       <c r="J38" t="n">
-        <v>8.114000000000001</v>
+        <v>8.121</v>
       </c>
       <c r="K38" t="n">
-        <v>9.239000000000001</v>
+        <v>9.262</v>
       </c>
       <c r="L38" t="n">
-        <v>9.723000000000001</v>
+        <v>9.722</v>
       </c>
       <c r="M38" t="n">
-        <v>10.204</v>
+        <v>10.184</v>
       </c>
       <c r="N38" t="n">
-        <v>10.391</v>
+        <v>10.371</v>
       </c>
       <c r="O38" t="n">
-        <v>10.58</v>
+        <v>10.554</v>
       </c>
       <c r="P38" t="n">
-        <v>10.677</v>
+        <v>10.643</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.151</v>
+        <v>11.109</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.216</v>
+        <v>4.221</v>
       </c>
       <c r="G39" t="n">
-        <v>4.864</v>
+        <v>4.87</v>
       </c>
       <c r="H39" t="n">
-        <v>5.567</v>
+        <v>5.574</v>
       </c>
       <c r="I39" t="n">
-        <v>6.021</v>
+        <v>6.025</v>
       </c>
       <c r="J39" t="n">
-        <v>6.986</v>
+        <v>6.994</v>
       </c>
       <c r="K39" t="n">
-        <v>8.071</v>
+        <v>8.093999999999999</v>
       </c>
       <c r="L39" t="n">
         <v>8.478</v>
       </c>
       <c r="M39" t="n">
-        <v>8.84</v>
+        <v>8.82</v>
       </c>
       <c r="N39" t="n">
-        <v>9.019</v>
+        <v>8.999000000000001</v>
       </c>
       <c r="O39" t="n">
-        <v>9.23</v>
+        <v>9.205</v>
       </c>
       <c r="P39" t="n">
-        <v>9.331</v>
+        <v>9.298</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.795999999999999</v>
+        <v>9.754</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.354</v>
+        <v>3.359</v>
       </c>
       <c r="G40" t="n">
-        <v>3.53</v>
+        <v>3.536</v>
       </c>
       <c r="H40" t="n">
-        <v>3.847</v>
+        <v>3.854</v>
       </c>
       <c r="I40" t="n">
-        <v>4.116</v>
+        <v>4.12</v>
       </c>
       <c r="J40" t="n">
-        <v>4.479</v>
+        <v>4.486</v>
       </c>
       <c r="K40" t="n">
-        <v>4.85</v>
+        <v>4.873</v>
       </c>
       <c r="L40" t="n">
-        <v>4.952</v>
+        <v>4.951</v>
       </c>
       <c r="M40" t="n">
-        <v>5.132</v>
+        <v>5.112</v>
       </c>
       <c r="N40" t="n">
-        <v>5.318</v>
+        <v>5.296</v>
       </c>
       <c r="O40" t="n">
-        <v>5.643</v>
+        <v>5.618</v>
       </c>
       <c r="P40" t="n">
-        <v>5.91</v>
+        <v>5.877</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.688</v>
+        <v>6.646</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.74</v>
+        <v>3.745</v>
       </c>
       <c r="G41" t="n">
-        <v>3.959</v>
+        <v>3.965</v>
       </c>
       <c r="H41" t="n">
-        <v>4.332</v>
+        <v>4.339</v>
       </c>
       <c r="I41" t="n">
-        <v>4.62</v>
+        <v>4.624</v>
       </c>
       <c r="J41" t="n">
-        <v>5.034</v>
+        <v>5.041</v>
       </c>
       <c r="K41" t="n">
-        <v>5.45</v>
+        <v>5.473</v>
       </c>
       <c r="L41" t="n">
         <v>5.63</v>
       </c>
       <c r="M41" t="n">
-        <v>5.935</v>
+        <v>5.915</v>
       </c>
       <c r="N41" t="n">
-        <v>6.249</v>
+        <v>6.227</v>
       </c>
       <c r="O41" t="n">
-        <v>6.759</v>
+        <v>6.733</v>
       </c>
       <c r="P41" t="n">
-        <v>6.97</v>
+        <v>6.936</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.734</v>
+        <v>7.693</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.475</v>
+        <v>3.48</v>
       </c>
       <c r="G42" t="n">
-        <v>3.679</v>
+        <v>3.685</v>
       </c>
       <c r="H42" t="n">
-        <v>4.022</v>
+        <v>4.029</v>
       </c>
       <c r="I42" t="n">
-        <v>4.305</v>
+        <v>4.309</v>
       </c>
       <c r="J42" t="n">
-        <v>4.681</v>
+        <v>4.689</v>
       </c>
       <c r="K42" t="n">
-        <v>5.071</v>
+        <v>5.094</v>
       </c>
       <c r="L42" t="n">
         <v>5.188</v>
       </c>
       <c r="M42" t="n">
-        <v>5.439</v>
+        <v>5.419</v>
       </c>
       <c r="N42" t="n">
-        <v>5.732</v>
+        <v>5.71</v>
       </c>
       <c r="O42" t="n">
-        <v>6.135</v>
+        <v>6.11</v>
       </c>
       <c r="P42" t="n">
-        <v>6.412</v>
+        <v>6.379</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.2</v>
+        <v>7.158</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.175</v>
+        <v>3.18</v>
       </c>
       <c r="G43" t="n">
-        <v>3.339</v>
+        <v>3.345</v>
       </c>
       <c r="H43" t="n">
-        <v>3.607</v>
+        <v>3.614</v>
       </c>
       <c r="I43" t="n">
-        <v>3.836</v>
+        <v>3.84</v>
       </c>
       <c r="J43" t="n">
-        <v>4.123</v>
+        <v>4.132</v>
       </c>
       <c r="K43" t="n">
-        <v>4.418</v>
+        <v>4.442</v>
       </c>
       <c r="L43" t="n">
-        <v>4.472</v>
+        <v>4.471</v>
       </c>
       <c r="M43" t="n">
-        <v>4.571</v>
+        <v>4.551</v>
       </c>
       <c r="N43" t="n">
-        <v>4.619</v>
+        <v>4.596</v>
       </c>
       <c r="O43" t="n">
-        <v>4.732</v>
+        <v>4.706</v>
       </c>
       <c r="P43" t="n">
-        <v>4.887</v>
+        <v>4.853</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.563</v>
+        <v>5.521</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.032</v>
+        <v>3.035</v>
       </c>
       <c r="G44" t="n">
-        <v>3.182</v>
+        <v>3.186</v>
       </c>
       <c r="H44" t="n">
-        <v>3.436</v>
+        <v>3.443</v>
       </c>
       <c r="I44" t="n">
-        <v>3.667</v>
+        <v>3.67</v>
       </c>
       <c r="J44" t="n">
-        <v>3.973</v>
+        <v>3.982</v>
       </c>
       <c r="K44" t="n">
-        <v>4.263</v>
+        <v>4.287</v>
       </c>
       <c r="L44" t="n">
-        <v>4.317</v>
+        <v>4.316</v>
       </c>
       <c r="M44" t="n">
-        <v>4.388</v>
+        <v>4.369</v>
       </c>
       <c r="N44" t="n">
-        <v>4.435</v>
+        <v>4.414</v>
       </c>
       <c r="O44" t="n">
-        <v>4.527</v>
+        <v>4.502</v>
       </c>
       <c r="P44" t="n">
-        <v>4.65</v>
+        <v>4.616</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.934</v>
+        <v>4.892</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-05 ~ 2026-06-05
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.317</v>
+        <v>3.323</v>
       </c>
       <c r="G2" t="n">
-        <v>3.617</v>
+        <v>3.628</v>
       </c>
       <c r="H2" t="n">
-        <v>3.913</v>
+        <v>3.928</v>
       </c>
       <c r="I2" t="n">
-        <v>4.149</v>
+        <v>4.16</v>
       </c>
       <c r="J2" t="n">
-        <v>4.449</v>
+        <v>4.457</v>
       </c>
       <c r="K2" t="n">
-        <v>4.877</v>
+        <v>4.891</v>
       </c>
       <c r="L2" t="n">
-        <v>5.044</v>
+        <v>5.056</v>
       </c>
       <c r="M2" t="n">
-        <v>5.312</v>
+        <v>5.33</v>
       </c>
       <c r="N2" t="n">
-        <v>5.59</v>
+        <v>5.615</v>
       </c>
       <c r="O2" t="n">
-        <v>5.857</v>
+        <v>5.901</v>
       </c>
       <c r="P2" t="n">
-        <v>6.071</v>
+        <v>6.095</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.688</v>
+        <v>6.712</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.339</v>
+        <v>4.345</v>
       </c>
       <c r="G3" t="n">
-        <v>4.82</v>
+        <v>4.831</v>
       </c>
       <c r="H3" t="n">
-        <v>5.148</v>
+        <v>5.163</v>
       </c>
       <c r="I3" t="n">
-        <v>5.377</v>
+        <v>5.388</v>
       </c>
       <c r="J3" t="n">
-        <v>5.694</v>
+        <v>5.703</v>
       </c>
       <c r="K3" t="n">
-        <v>6.193</v>
+        <v>6.207</v>
       </c>
       <c r="L3" t="n">
-        <v>6.43</v>
+        <v>6.442</v>
       </c>
       <c r="M3" t="n">
-        <v>6.728</v>
+        <v>6.746</v>
       </c>
       <c r="N3" t="n">
-        <v>6.949</v>
+        <v>6.974</v>
       </c>
       <c r="O3" t="n">
-        <v>7.167</v>
+        <v>7.211</v>
       </c>
       <c r="P3" t="n">
-        <v>7.25</v>
+        <v>7.273</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.754</v>
+        <v>7.778</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.831</v>
+        <v>3.837</v>
       </c>
       <c r="G4" t="n">
-        <v>4.201</v>
+        <v>4.212</v>
       </c>
       <c r="H4" t="n">
-        <v>4.558</v>
+        <v>4.573</v>
       </c>
       <c r="I4" t="n">
-        <v>4.82</v>
+        <v>4.831</v>
       </c>
       <c r="J4" t="n">
-        <v>5.138</v>
+        <v>5.146</v>
       </c>
       <c r="K4" t="n">
-        <v>5.632</v>
+        <v>5.646</v>
       </c>
       <c r="L4" t="n">
-        <v>5.799</v>
+        <v>5.811</v>
       </c>
       <c r="M4" t="n">
-        <v>6.086</v>
+        <v>6.104</v>
       </c>
       <c r="N4" t="n">
-        <v>6.277</v>
+        <v>6.302</v>
       </c>
       <c r="O4" t="n">
-        <v>6.519</v>
+        <v>6.563</v>
       </c>
       <c r="P4" t="n">
-        <v>6.602</v>
+        <v>6.625</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.109</v>
+        <v>7.133</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.015</v>
+        <v>3.021</v>
       </c>
       <c r="G5" t="n">
-        <v>3.158</v>
+        <v>3.171</v>
       </c>
       <c r="H5" t="n">
-        <v>3.419</v>
+        <v>3.435</v>
       </c>
       <c r="I5" t="n">
-        <v>3.721</v>
+        <v>3.732</v>
       </c>
       <c r="J5" t="n">
-        <v>4.006</v>
+        <v>4.016</v>
       </c>
       <c r="K5" t="n">
-        <v>4.281</v>
+        <v>4.296</v>
       </c>
       <c r="L5" t="n">
-        <v>4.293</v>
+        <v>4.305</v>
       </c>
       <c r="M5" t="n">
-        <v>4.371</v>
+        <v>4.389</v>
       </c>
       <c r="N5" t="n">
-        <v>4.402</v>
+        <v>4.427</v>
       </c>
       <c r="O5" t="n">
-        <v>4.457</v>
+        <v>4.501</v>
       </c>
       <c r="P5" t="n">
-        <v>4.74</v>
+        <v>4.763</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.6</v>
+        <v>5.624</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.055</v>
+        <v>3.062</v>
       </c>
       <c r="G6" t="n">
-        <v>3.213</v>
+        <v>3.226</v>
       </c>
       <c r="H6" t="n">
-        <v>3.488</v>
+        <v>3.504</v>
       </c>
       <c r="I6" t="n">
-        <v>3.803</v>
+        <v>3.815</v>
       </c>
       <c r="J6" t="n">
-        <v>4.096</v>
+        <v>4.106</v>
       </c>
       <c r="K6" t="n">
-        <v>4.393</v>
+        <v>4.408</v>
       </c>
       <c r="L6" t="n">
-        <v>4.41</v>
+        <v>4.423</v>
       </c>
       <c r="M6" t="n">
-        <v>4.526</v>
+        <v>4.544</v>
       </c>
       <c r="N6" t="n">
-        <v>4.569</v>
+        <v>4.594</v>
       </c>
       <c r="O6" t="n">
-        <v>4.723</v>
+        <v>4.767</v>
       </c>
       <c r="P6" t="n">
-        <v>5.172</v>
+        <v>5.196</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.996</v>
+        <v>6.02</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.036</v>
+        <v>3.042</v>
       </c>
       <c r="G7" t="n">
-        <v>3.176</v>
+        <v>3.19</v>
       </c>
       <c r="H7" t="n">
-        <v>3.435</v>
+        <v>3.451</v>
       </c>
       <c r="I7" t="n">
-        <v>3.74</v>
+        <v>3.752</v>
       </c>
       <c r="J7" t="n">
-        <v>4.03</v>
+        <v>4.04</v>
       </c>
       <c r="K7" t="n">
-        <v>4.308</v>
+        <v>4.323</v>
       </c>
       <c r="L7" t="n">
-        <v>4.319</v>
+        <v>4.331</v>
       </c>
       <c r="M7" t="n">
-        <v>4.431</v>
+        <v>4.449</v>
       </c>
       <c r="N7" t="n">
-        <v>4.462</v>
+        <v>4.486</v>
       </c>
       <c r="O7" t="n">
-        <v>4.62</v>
+        <v>4.664</v>
       </c>
       <c r="P7" t="n">
-        <v>4.956</v>
+        <v>4.979</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.764</v>
+        <v>5.788</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.451</v>
+        <v>5.457</v>
       </c>
       <c r="G8" t="n">
-        <v>6.119</v>
+        <v>6.13</v>
       </c>
       <c r="H8" t="n">
-        <v>6.597</v>
+        <v>6.612</v>
       </c>
       <c r="I8" t="n">
-        <v>6.904</v>
+        <v>6.915</v>
       </c>
       <c r="J8" t="n">
-        <v>7.287</v>
+        <v>7.295</v>
       </c>
       <c r="K8" t="n">
-        <v>8.066000000000001</v>
+        <v>8.081</v>
       </c>
       <c r="L8" t="n">
-        <v>8.388</v>
+        <v>8.4</v>
       </c>
       <c r="M8" t="n">
-        <v>8.718999999999999</v>
+        <v>8.737</v>
       </c>
       <c r="N8" t="n">
-        <v>8.872999999999999</v>
+        <v>8.898</v>
       </c>
       <c r="O8" t="n">
-        <v>9.177</v>
+        <v>9.221</v>
       </c>
       <c r="P8" t="n">
-        <v>9.363</v>
+        <v>9.385999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.065</v>
+        <v>10.09</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.635</v>
+        <v>2.634</v>
       </c>
       <c r="G9" t="n">
-        <v>2.751</v>
+        <v>2.745</v>
       </c>
       <c r="H9" t="n">
-        <v>2.967</v>
+        <v>2.969</v>
       </c>
       <c r="I9" t="n">
-        <v>3.234</v>
+        <v>3.239</v>
       </c>
       <c r="J9" t="n">
-        <v>3.5</v>
+        <v>3.502</v>
       </c>
       <c r="K9" t="n">
-        <v>3.77</v>
+        <v>3.785</v>
       </c>
       <c r="L9" t="n">
-        <v>3.8</v>
+        <v>3.812</v>
       </c>
       <c r="M9" t="n">
-        <v>3.86</v>
+        <v>3.88</v>
       </c>
       <c r="N9" t="n">
-        <v>4.012</v>
+        <v>4.038</v>
       </c>
       <c r="O9" t="n">
-        <v>4.075</v>
+        <v>4.12</v>
       </c>
       <c r="P9" t="n">
-        <v>4.173</v>
+        <v>4.198</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.227</v>
+        <v>4.252</v>
       </c>
       <c r="R9" t="n">
-        <v>4.245</v>
+        <v>4.291</v>
       </c>
       <c r="S9" t="n">
-        <v>4.26</v>
+        <v>4.326</v>
       </c>
       <c r="T9" t="n">
-        <v>4.207</v>
+        <v>4.265</v>
       </c>
       <c r="U9" t="n">
-        <v>4.12</v>
+        <v>4.192</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.667</v>
+        <v>2.668</v>
       </c>
       <c r="G10" t="n">
-        <v>2.796</v>
+        <v>2.795</v>
       </c>
       <c r="H10" t="n">
-        <v>2.984</v>
+        <v>2.987</v>
       </c>
       <c r="I10" t="n">
-        <v>3.244</v>
+        <v>3.25</v>
       </c>
       <c r="J10" t="n">
-        <v>3.532</v>
+        <v>3.534</v>
       </c>
       <c r="K10" t="n">
-        <v>3.803</v>
+        <v>3.818</v>
       </c>
       <c r="L10" t="n">
-        <v>3.852</v>
+        <v>3.865</v>
       </c>
       <c r="M10" t="n">
-        <v>3.954</v>
+        <v>3.974</v>
       </c>
       <c r="N10" t="n">
-        <v>4.032</v>
+        <v>4.061</v>
       </c>
       <c r="O10" t="n">
-        <v>4.302</v>
+        <v>4.337</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.471</v>
+        <v>2.472</v>
       </c>
       <c r="G11" t="n">
-        <v>2.6</v>
+        <v>2.595</v>
       </c>
       <c r="H11" t="n">
-        <v>2.807</v>
+        <v>2.81</v>
       </c>
       <c r="I11" t="n">
-        <v>3.048</v>
+        <v>3.054</v>
       </c>
       <c r="J11" t="n">
-        <v>3.326</v>
+        <v>3.328</v>
       </c>
       <c r="K11" t="n">
-        <v>3.589</v>
+        <v>3.605</v>
       </c>
       <c r="L11" t="n">
-        <v>3.65</v>
+        <v>3.662</v>
       </c>
       <c r="M11" t="n">
-        <v>3.762</v>
+        <v>3.782</v>
       </c>
       <c r="N11" t="n">
-        <v>3.84</v>
+        <v>3.869</v>
       </c>
       <c r="O11" t="n">
-        <v>4.069</v>
+        <v>4.104</v>
       </c>
       <c r="P11" t="n">
-        <v>4.124</v>
+        <v>4.149</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.427</v>
+        <v>4.452</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.298</v>
+        <v>3.3</v>
       </c>
       <c r="G12" t="n">
-        <v>3.557</v>
+        <v>3.565</v>
       </c>
       <c r="H12" t="n">
-        <v>3.822</v>
+        <v>3.837</v>
       </c>
       <c r="I12" t="n">
-        <v>4.117</v>
+        <v>4.133</v>
       </c>
       <c r="J12" t="n">
-        <v>4.43</v>
+        <v>4.448</v>
       </c>
       <c r="K12" t="n">
-        <v>4.665</v>
+        <v>4.683</v>
       </c>
       <c r="L12" t="n">
-        <v>4.712</v>
+        <v>4.726</v>
       </c>
       <c r="M12" t="n">
-        <v>4.838</v>
+        <v>4.858</v>
       </c>
       <c r="N12" t="n">
-        <v>4.902</v>
+        <v>4.93</v>
       </c>
       <c r="O12" t="n">
-        <v>5.082</v>
+        <v>5.126</v>
       </c>
       <c r="P12" t="n">
-        <v>5.212</v>
+        <v>5.237</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.542</v>
+        <v>5.567</v>
       </c>
       <c r="R12" t="n">
-        <v>5.736</v>
+        <v>5.782</v>
       </c>
       <c r="S12" t="n">
-        <v>5.962</v>
+        <v>6.029</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.052</v>
+        <v>3.054</v>
       </c>
       <c r="G13" t="n">
-        <v>3.247</v>
+        <v>3.255</v>
       </c>
       <c r="H13" t="n">
-        <v>3.489</v>
+        <v>3.505</v>
       </c>
       <c r="I13" t="n">
-        <v>3.765</v>
+        <v>3.781</v>
       </c>
       <c r="J13" t="n">
-        <v>4.067</v>
+        <v>4.085</v>
       </c>
       <c r="K13" t="n">
-        <v>4.298</v>
+        <v>4.316</v>
       </c>
       <c r="L13" t="n">
-        <v>4.352</v>
+        <v>4.365</v>
       </c>
       <c r="M13" t="n">
-        <v>4.466</v>
+        <v>4.486</v>
       </c>
       <c r="N13" t="n">
-        <v>4.531</v>
+        <v>4.558</v>
       </c>
       <c r="O13" t="n">
-        <v>4.711</v>
+        <v>4.755</v>
       </c>
       <c r="P13" t="n">
-        <v>4.803</v>
+        <v>4.828</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.063</v>
+        <v>5.088</v>
       </c>
       <c r="R13" t="n">
-        <v>5.286</v>
+        <v>5.332</v>
       </c>
       <c r="S13" t="n">
-        <v>5.525</v>
+        <v>5.592</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.869</v>
+        <v>2.871</v>
       </c>
       <c r="G14" t="n">
-        <v>3.053</v>
+        <v>3.061</v>
       </c>
       <c r="H14" t="n">
-        <v>3.292</v>
+        <v>3.308</v>
       </c>
       <c r="I14" t="n">
-        <v>3.55</v>
+        <v>3.565</v>
       </c>
       <c r="J14" t="n">
-        <v>3.808</v>
+        <v>3.827</v>
       </c>
       <c r="K14" t="n">
-        <v>3.986</v>
+        <v>4.004</v>
       </c>
       <c r="L14" t="n">
-        <v>4.025</v>
+        <v>4.038</v>
       </c>
       <c r="M14" t="n">
-        <v>4.152</v>
+        <v>4.172</v>
       </c>
       <c r="N14" t="n">
-        <v>4.21</v>
+        <v>4.238</v>
       </c>
       <c r="O14" t="n">
-        <v>4.369</v>
+        <v>4.413</v>
       </c>
       <c r="P14" t="n">
-        <v>4.439</v>
+        <v>4.464</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.652</v>
+        <v>4.677</v>
       </c>
       <c r="R14" t="n">
-        <v>4.8</v>
+        <v>4.846</v>
       </c>
       <c r="S14" t="n">
-        <v>4.978</v>
+        <v>5.044</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.847</v>
+        <v>2.849</v>
       </c>
       <c r="G15" t="n">
-        <v>3.027</v>
+        <v>3.035</v>
       </c>
       <c r="H15" t="n">
-        <v>3.263</v>
+        <v>3.279</v>
       </c>
       <c r="I15" t="n">
-        <v>3.5</v>
+        <v>3.515</v>
       </c>
       <c r="J15" t="n">
-        <v>3.747</v>
+        <v>3.765</v>
       </c>
       <c r="K15" t="n">
-        <v>3.939</v>
+        <v>3.956</v>
       </c>
       <c r="L15" t="n">
-        <v>3.961</v>
+        <v>3.974</v>
       </c>
       <c r="M15" t="n">
-        <v>4.065</v>
+        <v>4.085</v>
       </c>
       <c r="N15" t="n">
-        <v>4.114</v>
+        <v>4.141</v>
       </c>
       <c r="O15" t="n">
-        <v>4.313</v>
+        <v>4.356</v>
       </c>
       <c r="P15" t="n">
-        <v>4.336</v>
+        <v>4.36</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.554</v>
+        <v>4.579</v>
       </c>
       <c r="R15" t="n">
-        <v>4.695</v>
+        <v>4.741</v>
       </c>
       <c r="S15" t="n">
-        <v>4.873</v>
+        <v>4.939</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.847</v>
+        <v>2.849</v>
       </c>
       <c r="G16" t="n">
-        <v>3.027</v>
+        <v>3.035</v>
       </c>
       <c r="H16" t="n">
-        <v>3.263</v>
+        <v>3.279</v>
       </c>
       <c r="I16" t="n">
-        <v>3.5</v>
+        <v>3.515</v>
       </c>
       <c r="J16" t="n">
-        <v>3.747</v>
+        <v>3.765</v>
       </c>
       <c r="K16" t="n">
-        <v>3.939</v>
+        <v>3.956</v>
       </c>
       <c r="L16" t="n">
-        <v>3.961</v>
+        <v>3.974</v>
       </c>
       <c r="M16" t="n">
-        <v>4.065</v>
+        <v>4.085</v>
       </c>
       <c r="N16" t="n">
-        <v>4.117</v>
+        <v>4.144</v>
       </c>
       <c r="O16" t="n">
-        <v>4.319</v>
+        <v>4.362</v>
       </c>
       <c r="P16" t="n">
-        <v>4.359</v>
+        <v>4.384</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.581</v>
+        <v>4.606</v>
       </c>
       <c r="R16" t="n">
-        <v>4.723</v>
+        <v>4.769</v>
       </c>
       <c r="S16" t="n">
-        <v>4.902</v>
+        <v>4.968</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.716</v>
+        <v>2.717</v>
       </c>
       <c r="G17" t="n">
-        <v>2.878</v>
+        <v>2.873</v>
       </c>
       <c r="H17" t="n">
-        <v>3.076</v>
+        <v>3.079</v>
       </c>
       <c r="I17" t="n">
-        <v>3.326</v>
+        <v>3.331</v>
       </c>
       <c r="J17" t="n">
-        <v>3.603</v>
+        <v>3.605</v>
       </c>
       <c r="K17" t="n">
-        <v>3.88</v>
+        <v>3.896</v>
       </c>
       <c r="L17" t="n">
-        <v>3.936</v>
+        <v>3.948</v>
       </c>
       <c r="M17" t="n">
-        <v>4.077</v>
+        <v>4.097</v>
       </c>
       <c r="N17" t="n">
-        <v>4.135</v>
+        <v>4.165</v>
       </c>
       <c r="O17" t="n">
-        <v>4.323</v>
+        <v>4.358</v>
       </c>
       <c r="P17" t="n">
-        <v>4.405</v>
+        <v>4.429</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.717</v>
+        <v>2.718</v>
       </c>
       <c r="G18" t="n">
-        <v>2.879</v>
+        <v>2.874</v>
       </c>
       <c r="H18" t="n">
-        <v>3.077</v>
+        <v>3.079</v>
       </c>
       <c r="I18" t="n">
-        <v>3.326</v>
+        <v>3.332</v>
       </c>
       <c r="J18" t="n">
-        <v>3.603</v>
+        <v>3.605</v>
       </c>
       <c r="K18" t="n">
-        <v>3.881</v>
+        <v>3.897</v>
       </c>
       <c r="L18" t="n">
-        <v>3.936</v>
+        <v>3.948</v>
       </c>
       <c r="M18" t="n">
-        <v>4.077</v>
+        <v>4.097</v>
       </c>
       <c r="N18" t="n">
-        <v>4.136</v>
+        <v>4.166</v>
       </c>
       <c r="O18" t="n">
-        <v>4.321</v>
+        <v>4.356</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.859</v>
+        <v>2.86</v>
       </c>
       <c r="G19" t="n">
-        <v>3.04</v>
+        <v>3.048</v>
       </c>
       <c r="H19" t="n">
-        <v>3.278</v>
+        <v>3.293</v>
       </c>
       <c r="I19" t="n">
-        <v>3.533</v>
+        <v>3.548</v>
       </c>
       <c r="J19" t="n">
-        <v>3.787</v>
+        <v>3.806</v>
       </c>
       <c r="K19" t="n">
-        <v>3.982</v>
+        <v>3.999</v>
       </c>
       <c r="L19" t="n">
-        <v>4.022</v>
+        <v>4.035</v>
       </c>
       <c r="M19" t="n">
-        <v>4.142</v>
+        <v>4.163</v>
       </c>
       <c r="N19" t="n">
-        <v>4.199</v>
+        <v>4.227</v>
       </c>
       <c r="O19" t="n">
-        <v>4.355</v>
+        <v>4.399</v>
       </c>
       <c r="P19" t="n">
-        <v>4.397</v>
+        <v>4.422</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.592</v>
+        <v>4.617</v>
       </c>
       <c r="R19" t="n">
-        <v>4.742</v>
+        <v>4.788</v>
       </c>
       <c r="S19" t="n">
-        <v>4.913</v>
+        <v>4.979</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.647</v>
       </c>
       <c r="G20" t="n">
-        <v>2.754</v>
+        <v>2.755</v>
       </c>
       <c r="H20" t="n">
-        <v>2.872</v>
+        <v>2.877</v>
       </c>
       <c r="I20" t="n">
-        <v>3.082</v>
+        <v>3.086</v>
       </c>
       <c r="J20" t="n">
-        <v>3.526</v>
+        <v>3.533</v>
       </c>
       <c r="K20" t="n">
-        <v>3.802</v>
+        <v>3.819</v>
       </c>
       <c r="L20" t="n">
-        <v>3.809</v>
+        <v>3.827</v>
       </c>
       <c r="M20" t="n">
-        <v>3.903</v>
+        <v>3.922</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.957</v>
+        <v>2.96</v>
       </c>
       <c r="G21" t="n">
-        <v>3.126</v>
+        <v>3.138</v>
       </c>
       <c r="H21" t="n">
-        <v>3.394</v>
+        <v>3.408</v>
       </c>
       <c r="I21" t="n">
-        <v>3.65</v>
+        <v>3.662</v>
       </c>
       <c r="J21" t="n">
-        <v>3.935</v>
+        <v>3.95</v>
       </c>
       <c r="K21" t="n">
-        <v>4.226</v>
+        <v>4.244</v>
       </c>
       <c r="L21" t="n">
-        <v>4.265</v>
+        <v>4.279</v>
       </c>
       <c r="M21" t="n">
-        <v>4.377</v>
+        <v>4.399</v>
       </c>
       <c r="N21" t="n">
-        <v>4.445</v>
+        <v>4.472</v>
       </c>
       <c r="O21" t="n">
-        <v>4.56</v>
+        <v>4.605</v>
       </c>
       <c r="P21" t="n">
-        <v>4.658</v>
+        <v>4.682</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.749</v>
+        <v>4.773</v>
       </c>
       <c r="R21" t="n">
-        <v>4.793</v>
+        <v>4.839</v>
       </c>
       <c r="S21" t="n">
-        <v>4.865</v>
+        <v>4.932</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.903</v>
+        <v>2.906</v>
       </c>
       <c r="G22" t="n">
-        <v>3.072</v>
+        <v>3.082</v>
       </c>
       <c r="H22" t="n">
-        <v>3.326</v>
+        <v>3.339</v>
       </c>
       <c r="I22" t="n">
-        <v>3.569</v>
+        <v>3.58</v>
       </c>
       <c r="J22" t="n">
-        <v>3.82</v>
+        <v>3.836</v>
       </c>
       <c r="K22" t="n">
-        <v>4.108</v>
+        <v>4.125</v>
       </c>
       <c r="L22" t="n">
-        <v>4.132</v>
+        <v>4.146</v>
       </c>
       <c r="M22" t="n">
-        <v>4.248</v>
+        <v>4.27</v>
       </c>
       <c r="N22" t="n">
-        <v>4.318</v>
+        <v>4.346</v>
       </c>
       <c r="O22" t="n">
-        <v>4.431</v>
+        <v>4.476</v>
       </c>
       <c r="P22" t="n">
-        <v>4.522</v>
+        <v>4.545</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.608</v>
+        <v>4.632</v>
       </c>
       <c r="R22" t="n">
-        <v>4.641</v>
+        <v>4.687</v>
       </c>
       <c r="S22" t="n">
-        <v>4.711</v>
+        <v>4.777</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.854</v>
+        <v>2.857</v>
       </c>
       <c r="G23" t="n">
-        <v>3.026</v>
+        <v>3.037</v>
       </c>
       <c r="H23" t="n">
-        <v>3.267</v>
+        <v>3.281</v>
       </c>
       <c r="I23" t="n">
-        <v>3.517</v>
+        <v>3.528</v>
       </c>
       <c r="J23" t="n">
-        <v>3.76</v>
+        <v>3.776</v>
       </c>
       <c r="K23" t="n">
-        <v>4.008</v>
+        <v>4.025</v>
       </c>
       <c r="L23" t="n">
-        <v>4.029</v>
+        <v>4.044</v>
       </c>
       <c r="M23" t="n">
-        <v>4.14</v>
+        <v>4.161</v>
       </c>
       <c r="N23" t="n">
-        <v>4.213</v>
+        <v>4.24</v>
       </c>
       <c r="O23" t="n">
-        <v>4.308</v>
+        <v>4.352</v>
       </c>
       <c r="P23" t="n">
-        <v>4.385</v>
+        <v>4.408</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.414</v>
+        <v>4.438</v>
       </c>
       <c r="R23" t="n">
-        <v>4.427</v>
+        <v>4.473</v>
       </c>
       <c r="S23" t="n">
-        <v>4.467</v>
+        <v>4.533</v>
       </c>
       <c r="T23" t="n">
-        <v>4.413</v>
+        <v>4.471</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.791</v>
+        <v>2.794</v>
       </c>
       <c r="G24" t="n">
-        <v>2.937</v>
+        <v>2.948</v>
       </c>
       <c r="H24" t="n">
-        <v>3.161</v>
+        <v>3.174</v>
       </c>
       <c r="I24" t="n">
-        <v>3.454</v>
+        <v>3.466</v>
       </c>
       <c r="J24" t="n">
-        <v>3.654</v>
+        <v>3.669</v>
       </c>
       <c r="K24" t="n">
-        <v>3.891</v>
+        <v>3.908</v>
       </c>
       <c r="L24" t="n">
-        <v>3.91</v>
+        <v>3.925</v>
       </c>
       <c r="M24" t="n">
-        <v>4</v>
+        <v>4.021</v>
       </c>
       <c r="N24" t="n">
-        <v>4.087</v>
+        <v>4.114</v>
       </c>
       <c r="O24" t="n">
-        <v>4.309</v>
+        <v>4.351</v>
       </c>
       <c r="P24" t="n">
-        <v>4.32</v>
+        <v>4.347</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.339</v>
+        <v>4.363</v>
       </c>
       <c r="R24" t="n">
-        <v>4.349</v>
+        <v>4.395</v>
       </c>
       <c r="S24" t="n">
-        <v>4.382</v>
+        <v>4.448</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.848</v>
+        <v>2.851</v>
       </c>
       <c r="G25" t="n">
-        <v>3.026</v>
+        <v>3.037</v>
       </c>
       <c r="H25" t="n">
-        <v>3.27</v>
+        <v>3.284</v>
       </c>
       <c r="I25" t="n">
-        <v>3.526</v>
+        <v>3.537</v>
       </c>
       <c r="J25" t="n">
-        <v>3.775</v>
+        <v>3.791</v>
       </c>
       <c r="K25" t="n">
-        <v>4.039</v>
+        <v>4.057</v>
       </c>
       <c r="L25" t="n">
-        <v>4.06</v>
+        <v>4.075</v>
       </c>
       <c r="M25" t="n">
-        <v>4.171</v>
+        <v>4.192</v>
       </c>
       <c r="N25" t="n">
-        <v>4.239</v>
+        <v>4.267</v>
       </c>
       <c r="O25" t="n">
-        <v>4.337</v>
+        <v>4.381</v>
       </c>
       <c r="P25" t="n">
-        <v>4.406</v>
+        <v>4.429</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.447</v>
+        <v>4.471</v>
       </c>
       <c r="R25" t="n">
-        <v>4.451</v>
+        <v>4.497</v>
       </c>
       <c r="S25" t="n">
-        <v>4.49</v>
+        <v>4.557</v>
       </c>
       <c r="T25" t="n">
-        <v>4.431</v>
+        <v>4.489</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.142</v>
+        <v>3.147</v>
       </c>
       <c r="G26" t="n">
-        <v>3.351</v>
+        <v>3.36</v>
       </c>
       <c r="H26" t="n">
-        <v>3.699</v>
+        <v>3.711</v>
       </c>
       <c r="I26" t="n">
-        <v>3.989</v>
+        <v>3.998</v>
       </c>
       <c r="J26" t="n">
-        <v>4.403</v>
+        <v>4.41</v>
       </c>
       <c r="K26" t="n">
-        <v>4.846</v>
+        <v>4.863</v>
       </c>
       <c r="L26" t="n">
-        <v>4.939</v>
+        <v>4.951</v>
       </c>
       <c r="M26" t="n">
-        <v>5.093</v>
+        <v>5.112</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.392</v>
+        <v>5.437</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.955</v>
+        <v>2.958</v>
       </c>
       <c r="G27" t="n">
-        <v>3.119</v>
+        <v>3.126</v>
       </c>
       <c r="H27" t="n">
-        <v>3.373</v>
+        <v>3.385</v>
       </c>
       <c r="I27" t="n">
-        <v>3.63</v>
+        <v>3.643</v>
       </c>
       <c r="J27" t="n">
-        <v>3.915</v>
+        <v>3.93</v>
       </c>
       <c r="K27" t="n">
-        <v>4.161</v>
+        <v>4.179</v>
       </c>
       <c r="L27" t="n">
-        <v>4.206</v>
+        <v>4.219</v>
       </c>
       <c r="M27" t="n">
-        <v>4.312</v>
+        <v>4.332</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.496</v>
+        <v>4.54</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.058</v>
+        <v>3.061</v>
       </c>
       <c r="G28" t="n">
-        <v>3.23</v>
+        <v>3.237</v>
       </c>
       <c r="H28" t="n">
-        <v>3.498</v>
+        <v>3.51</v>
       </c>
       <c r="I28" t="n">
-        <v>3.767</v>
+        <v>3.78</v>
       </c>
       <c r="J28" t="n">
-        <v>4.088</v>
+        <v>4.103</v>
       </c>
       <c r="K28" t="n">
-        <v>4.353</v>
+        <v>4.371</v>
       </c>
       <c r="L28" t="n">
-        <v>4.409</v>
+        <v>4.422</v>
       </c>
       <c r="M28" t="n">
-        <v>4.524</v>
+        <v>4.544</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.788</v>
+        <v>4.833</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.904</v>
+        <v>2.907</v>
       </c>
       <c r="G29" t="n">
-        <v>3.066</v>
+        <v>3.074</v>
       </c>
       <c r="H29" t="n">
-        <v>3.311</v>
+        <v>3.324</v>
       </c>
       <c r="I29" t="n">
-        <v>3.557</v>
+        <v>3.57</v>
       </c>
       <c r="J29" t="n">
-        <v>3.828</v>
+        <v>3.842</v>
       </c>
       <c r="K29" t="n">
-        <v>4.057</v>
+        <v>4.074</v>
       </c>
       <c r="L29" t="n">
-        <v>4.092</v>
+        <v>4.104</v>
       </c>
       <c r="M29" t="n">
-        <v>4.175</v>
+        <v>4.195</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.368</v>
+        <v>4.412</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.183</v>
+        <v>3.188</v>
       </c>
       <c r="G30" t="n">
-        <v>3.327</v>
+        <v>3.335</v>
       </c>
       <c r="H30" t="n">
-        <v>3.634</v>
+        <v>3.645</v>
       </c>
       <c r="I30" t="n">
-        <v>3.917</v>
+        <v>3.925</v>
       </c>
       <c r="J30" t="n">
-        <v>4.266</v>
+        <v>4.274</v>
       </c>
       <c r="K30" t="n">
-        <v>4.644</v>
+        <v>4.663</v>
       </c>
       <c r="L30" t="n">
-        <v>4.717</v>
+        <v>4.729</v>
       </c>
       <c r="M30" t="n">
-        <v>4.859</v>
+        <v>4.879</v>
       </c>
       <c r="N30" t="n">
-        <v>5.028</v>
+        <v>5.055</v>
       </c>
       <c r="O30" t="n">
-        <v>5.344</v>
+        <v>5.389</v>
       </c>
       <c r="P30" t="n">
-        <v>5.549</v>
+        <v>5.575</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.286</v>
+        <v>6.311</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.512</v>
+        <v>3.517</v>
       </c>
       <c r="G31" t="n">
-        <v>3.692</v>
+        <v>3.7</v>
       </c>
       <c r="H31" t="n">
-        <v>4.05</v>
+        <v>4.061</v>
       </c>
       <c r="I31" t="n">
-        <v>4.346</v>
+        <v>4.354</v>
       </c>
       <c r="J31" t="n">
-        <v>4.757</v>
+        <v>4.765</v>
       </c>
       <c r="K31" t="n">
-        <v>5.177</v>
+        <v>5.195</v>
       </c>
       <c r="L31" t="n">
-        <v>5.329</v>
+        <v>5.342</v>
       </c>
       <c r="M31" t="n">
-        <v>5.59</v>
+        <v>5.61</v>
       </c>
       <c r="N31" t="n">
-        <v>5.887</v>
+        <v>5.914</v>
       </c>
       <c r="O31" t="n">
-        <v>6.38</v>
+        <v>6.425</v>
       </c>
       <c r="P31" t="n">
-        <v>6.538</v>
+        <v>6.563</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.259</v>
+        <v>7.284</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.282</v>
+        <v>3.287</v>
       </c>
       <c r="G32" t="n">
-        <v>3.444</v>
+        <v>3.452</v>
       </c>
       <c r="H32" t="n">
-        <v>3.778</v>
+        <v>3.789</v>
       </c>
       <c r="I32" t="n">
-        <v>4.076</v>
+        <v>4.084</v>
       </c>
       <c r="J32" t="n">
-        <v>4.444</v>
+        <v>4.452</v>
       </c>
       <c r="K32" t="n">
-        <v>4.829</v>
+        <v>4.848</v>
       </c>
       <c r="L32" t="n">
-        <v>4.921</v>
+        <v>4.934</v>
       </c>
       <c r="M32" t="n">
-        <v>5.132</v>
+        <v>5.152</v>
       </c>
       <c r="N32" t="n">
-        <v>5.389</v>
+        <v>5.416</v>
       </c>
       <c r="O32" t="n">
-        <v>5.789</v>
+        <v>5.834</v>
       </c>
       <c r="P32" t="n">
-        <v>6.009</v>
+        <v>6.035</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.747</v>
+        <v>6.772</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.048</v>
+        <v>3.053</v>
       </c>
       <c r="G33" t="n">
-        <v>3.192</v>
+        <v>3.2</v>
       </c>
       <c r="H33" t="n">
-        <v>3.452</v>
+        <v>3.463</v>
       </c>
       <c r="I33" t="n">
-        <v>3.702</v>
+        <v>3.71</v>
       </c>
       <c r="J33" t="n">
-        <v>3.973</v>
+        <v>3.981</v>
       </c>
       <c r="K33" t="n">
-        <v>4.286</v>
+        <v>4.305</v>
       </c>
       <c r="L33" t="n">
-        <v>4.32</v>
+        <v>4.333</v>
       </c>
       <c r="M33" t="n">
-        <v>4.386</v>
+        <v>4.406</v>
       </c>
       <c r="N33" t="n">
-        <v>4.418</v>
+        <v>4.445</v>
       </c>
       <c r="O33" t="n">
-        <v>4.498</v>
+        <v>4.543</v>
       </c>
       <c r="P33" t="n">
-        <v>4.582</v>
+        <v>4.607</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.003</v>
+        <v>5.028</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.108</v>
+        <v>3.113</v>
       </c>
       <c r="G34" t="n">
-        <v>3.245</v>
+        <v>3.253</v>
       </c>
       <c r="H34" t="n">
-        <v>3.514</v>
+        <v>3.525</v>
       </c>
       <c r="I34" t="n">
-        <v>3.77</v>
+        <v>3.778</v>
       </c>
       <c r="J34" t="n">
-        <v>4.045</v>
+        <v>4.053</v>
       </c>
       <c r="K34" t="n">
-        <v>4.363</v>
+        <v>4.381</v>
       </c>
       <c r="L34" t="n">
-        <v>4.4</v>
+        <v>4.412</v>
       </c>
       <c r="M34" t="n">
-        <v>4.476</v>
+        <v>4.496</v>
       </c>
       <c r="N34" t="n">
-        <v>4.522</v>
+        <v>4.549</v>
       </c>
       <c r="O34" t="n">
-        <v>4.667</v>
+        <v>4.712</v>
       </c>
       <c r="P34" t="n">
-        <v>4.876</v>
+        <v>4.901</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.704</v>
+        <v>5.729</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.082</v>
+        <v>3.087</v>
       </c>
       <c r="G35" t="n">
-        <v>3.219</v>
+        <v>3.226</v>
       </c>
       <c r="H35" t="n">
-        <v>3.482</v>
+        <v>3.493</v>
       </c>
       <c r="I35" t="n">
-        <v>3.737</v>
+        <v>3.744</v>
       </c>
       <c r="J35" t="n">
-        <v>4.013</v>
+        <v>4.021</v>
       </c>
       <c r="K35" t="n">
-        <v>4.317</v>
+        <v>4.335</v>
       </c>
       <c r="L35" t="n">
-        <v>4.354</v>
+        <v>4.367</v>
       </c>
       <c r="M35" t="n">
-        <v>4.423</v>
+        <v>4.443</v>
       </c>
       <c r="N35" t="n">
-        <v>4.458</v>
+        <v>4.485</v>
       </c>
       <c r="O35" t="n">
-        <v>4.564</v>
+        <v>4.609</v>
       </c>
       <c r="P35" t="n">
-        <v>4.679</v>
+        <v>4.704</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.339</v>
+        <v>5.364</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.973</v>
+        <v>2.977</v>
       </c>
       <c r="G36" t="n">
-        <v>3.106</v>
+        <v>3.114</v>
       </c>
       <c r="H36" t="n">
-        <v>3.36</v>
+        <v>3.372</v>
       </c>
       <c r="I36" t="n">
-        <v>3.614</v>
+        <v>3.622</v>
       </c>
       <c r="J36" t="n">
-        <v>3.91</v>
+        <v>3.918</v>
       </c>
       <c r="K36" t="n">
-        <v>4.212</v>
+        <v>4.23</v>
       </c>
       <c r="L36" t="n">
-        <v>4.246</v>
+        <v>4.258</v>
       </c>
       <c r="M36" t="n">
-        <v>4.289</v>
+        <v>4.309</v>
       </c>
       <c r="N36" t="n">
-        <v>4.322</v>
+        <v>4.349</v>
       </c>
       <c r="O36" t="n">
-        <v>4.406</v>
+        <v>4.451</v>
       </c>
       <c r="P36" t="n">
-        <v>4.48</v>
+        <v>4.505</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.72</v>
+        <v>4.745</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.855</v>
+        <v>3.86</v>
       </c>
       <c r="G37" t="n">
-        <v>4.386</v>
+        <v>4.394</v>
       </c>
       <c r="H37" t="n">
-        <v>5.022</v>
+        <v>5.033</v>
       </c>
       <c r="I37" t="n">
-        <v>5.407</v>
+        <v>5.415</v>
       </c>
       <c r="J37" t="n">
-        <v>6.247</v>
+        <v>6.254</v>
       </c>
       <c r="K37" t="n">
-        <v>7.217</v>
+        <v>7.235</v>
       </c>
       <c r="L37" t="n">
-        <v>7.53</v>
+        <v>7.542</v>
       </c>
       <c r="M37" t="n">
-        <v>7.862</v>
+        <v>7.882</v>
       </c>
       <c r="N37" t="n">
-        <v>8.042999999999999</v>
+        <v>8.069000000000001</v>
       </c>
       <c r="O37" t="n">
-        <v>8.259</v>
+        <v>8.304</v>
       </c>
       <c r="P37" t="n">
-        <v>8.339</v>
+        <v>8.365</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.75</v>
+        <v>8.775</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.916</v>
+        <v>4.922</v>
       </c>
       <c r="G38" t="n">
-        <v>5.701</v>
+        <v>5.709</v>
       </c>
       <c r="H38" t="n">
-        <v>6.549</v>
+        <v>6.56</v>
       </c>
       <c r="I38" t="n">
-        <v>7.092</v>
+        <v>7.099</v>
       </c>
       <c r="J38" t="n">
-        <v>8.191000000000001</v>
+        <v>8.198</v>
       </c>
       <c r="K38" t="n">
-        <v>9.339</v>
+        <v>9.358000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.811999999999999</v>
+        <v>9.824999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.274</v>
+        <v>10.294</v>
       </c>
       <c r="N38" t="n">
-        <v>10.461</v>
+        <v>10.488</v>
       </c>
       <c r="O38" t="n">
-        <v>10.659</v>
+        <v>10.704</v>
       </c>
       <c r="P38" t="n">
-        <v>10.737</v>
+        <v>10.762</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.2</v>
+        <v>11.225</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.237</v>
+        <v>4.242</v>
       </c>
       <c r="G39" t="n">
-        <v>4.898</v>
+        <v>4.907</v>
       </c>
       <c r="H39" t="n">
-        <v>5.614</v>
+        <v>5.625</v>
       </c>
       <c r="I39" t="n">
-        <v>6.096</v>
+        <v>6.103</v>
       </c>
       <c r="J39" t="n">
-        <v>7.063</v>
+        <v>7.071</v>
       </c>
       <c r="K39" t="n">
-        <v>8.172000000000001</v>
+        <v>8.19</v>
       </c>
       <c r="L39" t="n">
-        <v>8.568</v>
+        <v>8.58</v>
       </c>
       <c r="M39" t="n">
-        <v>8.91</v>
+        <v>8.93</v>
       </c>
       <c r="N39" t="n">
-        <v>9.089</v>
+        <v>9.116</v>
       </c>
       <c r="O39" t="n">
-        <v>9.308999999999999</v>
+        <v>9.355</v>
       </c>
       <c r="P39" t="n">
-        <v>9.391999999999999</v>
+        <v>9.417</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.846</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.375</v>
+        <v>3.38</v>
       </c>
       <c r="G40" t="n">
-        <v>3.565</v>
+        <v>3.573</v>
       </c>
       <c r="H40" t="n">
-        <v>3.893</v>
+        <v>3.904</v>
       </c>
       <c r="I40" t="n">
-        <v>4.191</v>
+        <v>4.198</v>
       </c>
       <c r="J40" t="n">
-        <v>4.558</v>
+        <v>4.565</v>
       </c>
       <c r="K40" t="n">
-        <v>4.95</v>
+        <v>4.969</v>
       </c>
       <c r="L40" t="n">
-        <v>5.041</v>
+        <v>5.054</v>
       </c>
       <c r="M40" t="n">
-        <v>5.202</v>
+        <v>5.222</v>
       </c>
       <c r="N40" t="n">
-        <v>5.386</v>
+        <v>5.413</v>
       </c>
       <c r="O40" t="n">
-        <v>5.723</v>
+        <v>5.768</v>
       </c>
       <c r="P40" t="n">
-        <v>5.971</v>
+        <v>5.996</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.737</v>
+        <v>6.762</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.761</v>
+        <v>3.766</v>
       </c>
       <c r="G41" t="n">
-        <v>3.994</v>
+        <v>4.002</v>
       </c>
       <c r="H41" t="n">
-        <v>4.379</v>
+        <v>4.39</v>
       </c>
       <c r="I41" t="n">
-        <v>4.695</v>
+        <v>4.702</v>
       </c>
       <c r="J41" t="n">
-        <v>5.113</v>
+        <v>5.12</v>
       </c>
       <c r="K41" t="n">
-        <v>5.551</v>
+        <v>5.569</v>
       </c>
       <c r="L41" t="n">
-        <v>5.72</v>
+        <v>5.733</v>
       </c>
       <c r="M41" t="n">
-        <v>6.005</v>
+        <v>6.025</v>
       </c>
       <c r="N41" t="n">
-        <v>6.317</v>
+        <v>6.344</v>
       </c>
       <c r="O41" t="n">
-        <v>6.838</v>
+        <v>6.883</v>
       </c>
       <c r="P41" t="n">
-        <v>7.03</v>
+        <v>7.055</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.784</v>
+        <v>7.809</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.496</v>
+        <v>3.501</v>
       </c>
       <c r="G42" t="n">
-        <v>3.714</v>
+        <v>3.722</v>
       </c>
       <c r="H42" t="n">
-        <v>4.069</v>
+        <v>4.08</v>
       </c>
       <c r="I42" t="n">
-        <v>4.379</v>
+        <v>4.387</v>
       </c>
       <c r="J42" t="n">
-        <v>4.76</v>
+        <v>4.768</v>
       </c>
       <c r="K42" t="n">
-        <v>5.171</v>
+        <v>5.19</v>
       </c>
       <c r="L42" t="n">
-        <v>5.278</v>
+        <v>5.29</v>
       </c>
       <c r="M42" t="n">
-        <v>5.509</v>
+        <v>5.529</v>
       </c>
       <c r="N42" t="n">
-        <v>5.801</v>
+        <v>5.827</v>
       </c>
       <c r="O42" t="n">
-        <v>6.215</v>
+        <v>6.26</v>
       </c>
       <c r="P42" t="n">
-        <v>6.473</v>
+        <v>6.498</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.249</v>
+        <v>7.274</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.196</v>
+        <v>3.201</v>
       </c>
       <c r="G43" t="n">
-        <v>3.374</v>
+        <v>3.382</v>
       </c>
       <c r="H43" t="n">
-        <v>3.653</v>
+        <v>3.664</v>
       </c>
       <c r="I43" t="n">
-        <v>3.911</v>
+        <v>3.918</v>
       </c>
       <c r="J43" t="n">
-        <v>4.201</v>
+        <v>4.208</v>
       </c>
       <c r="K43" t="n">
-        <v>4.518</v>
+        <v>4.537</v>
       </c>
       <c r="L43" t="n">
-        <v>4.562</v>
+        <v>4.575</v>
       </c>
       <c r="M43" t="n">
-        <v>4.641</v>
+        <v>4.661</v>
       </c>
       <c r="N43" t="n">
-        <v>4.687</v>
+        <v>4.714</v>
       </c>
       <c r="O43" t="n">
-        <v>4.811</v>
+        <v>4.856</v>
       </c>
       <c r="P43" t="n">
-        <v>4.947</v>
+        <v>4.973</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.613</v>
+        <v>5.638</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.051</v>
+        <v>3.055</v>
       </c>
       <c r="G44" t="n">
-        <v>3.215</v>
+        <v>3.223</v>
       </c>
       <c r="H44" t="n">
-        <v>3.484</v>
+        <v>3.495</v>
       </c>
       <c r="I44" t="n">
-        <v>3.741</v>
+        <v>3.749</v>
       </c>
       <c r="J44" t="n">
-        <v>4.051</v>
+        <v>4.058</v>
       </c>
       <c r="K44" t="n">
-        <v>4.364</v>
+        <v>4.382</v>
       </c>
       <c r="L44" t="n">
-        <v>4.406</v>
+        <v>4.419</v>
       </c>
       <c r="M44" t="n">
-        <v>4.459</v>
+        <v>4.479</v>
       </c>
       <c r="N44" t="n">
-        <v>4.504</v>
+        <v>4.531</v>
       </c>
       <c r="O44" t="n">
-        <v>4.607</v>
+        <v>4.652</v>
       </c>
       <c r="P44" t="n">
-        <v>4.71</v>
+        <v>4.735</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.983</v>
+        <v>5.008</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-08 ~ 2026-06-08
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.323</v>
+        <v>3.35</v>
       </c>
       <c r="G2" t="n">
-        <v>3.628</v>
+        <v>3.661</v>
       </c>
       <c r="H2" t="n">
-        <v>3.928</v>
+        <v>3.965</v>
       </c>
       <c r="I2" t="n">
-        <v>4.16</v>
+        <v>4.201</v>
       </c>
       <c r="J2" t="n">
-        <v>4.457</v>
+        <v>4.516</v>
       </c>
       <c r="K2" t="n">
-        <v>4.891</v>
+        <v>4.959</v>
       </c>
       <c r="L2" t="n">
-        <v>5.056</v>
+        <v>5.115</v>
       </c>
       <c r="M2" t="n">
-        <v>5.33</v>
+        <v>5.382</v>
       </c>
       <c r="N2" t="n">
-        <v>5.615</v>
+        <v>5.669</v>
       </c>
       <c r="O2" t="n">
-        <v>5.901</v>
+        <v>5.962</v>
       </c>
       <c r="P2" t="n">
-        <v>6.095</v>
+        <v>6.178</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.712</v>
+        <v>6.805</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.345</v>
+        <v>4.372</v>
       </c>
       <c r="G3" t="n">
-        <v>4.831</v>
+        <v>4.864</v>
       </c>
       <c r="H3" t="n">
-        <v>5.163</v>
+        <v>5.2</v>
       </c>
       <c r="I3" t="n">
-        <v>5.388</v>
+        <v>5.429</v>
       </c>
       <c r="J3" t="n">
-        <v>5.703</v>
+        <v>5.761</v>
       </c>
       <c r="K3" t="n">
-        <v>6.207</v>
+        <v>6.275</v>
       </c>
       <c r="L3" t="n">
-        <v>6.442</v>
+        <v>6.5</v>
       </c>
       <c r="M3" t="n">
-        <v>6.746</v>
+        <v>6.798</v>
       </c>
       <c r="N3" t="n">
-        <v>6.974</v>
+        <v>7.028</v>
       </c>
       <c r="O3" t="n">
-        <v>7.211</v>
+        <v>7.272</v>
       </c>
       <c r="P3" t="n">
-        <v>7.273</v>
+        <v>7.356</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.778</v>
+        <v>7.872</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.837</v>
+        <v>3.864</v>
       </c>
       <c r="G4" t="n">
-        <v>4.212</v>
+        <v>4.245</v>
       </c>
       <c r="H4" t="n">
-        <v>4.573</v>
+        <v>4.61</v>
       </c>
       <c r="I4" t="n">
-        <v>4.831</v>
+        <v>4.872</v>
       </c>
       <c r="J4" t="n">
-        <v>5.146</v>
+        <v>5.205</v>
       </c>
       <c r="K4" t="n">
-        <v>5.646</v>
+        <v>5.714</v>
       </c>
       <c r="L4" t="n">
-        <v>5.811</v>
+        <v>5.869</v>
       </c>
       <c r="M4" t="n">
-        <v>6.104</v>
+        <v>6.156</v>
       </c>
       <c r="N4" t="n">
-        <v>6.302</v>
+        <v>6.357</v>
       </c>
       <c r="O4" t="n">
-        <v>6.563</v>
+        <v>6.624</v>
       </c>
       <c r="P4" t="n">
-        <v>6.625</v>
+        <v>6.708</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.133</v>
+        <v>7.226</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.021</v>
+        <v>3.048</v>
       </c>
       <c r="G5" t="n">
-        <v>3.171</v>
+        <v>3.204</v>
       </c>
       <c r="H5" t="n">
-        <v>3.435</v>
+        <v>3.472</v>
       </c>
       <c r="I5" t="n">
-        <v>3.732</v>
+        <v>3.773</v>
       </c>
       <c r="J5" t="n">
-        <v>4.016</v>
+        <v>4.074</v>
       </c>
       <c r="K5" t="n">
-        <v>4.296</v>
+        <v>4.364</v>
       </c>
       <c r="L5" t="n">
-        <v>4.305</v>
+        <v>4.363</v>
       </c>
       <c r="M5" t="n">
-        <v>4.389</v>
+        <v>4.441</v>
       </c>
       <c r="N5" t="n">
-        <v>4.427</v>
+        <v>4.481</v>
       </c>
       <c r="O5" t="n">
-        <v>4.501</v>
+        <v>4.562</v>
       </c>
       <c r="P5" t="n">
-        <v>4.763</v>
+        <v>4.846</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.624</v>
+        <v>5.718</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.062</v>
+        <v>3.089</v>
       </c>
       <c r="G6" t="n">
-        <v>3.226</v>
+        <v>3.259</v>
       </c>
       <c r="H6" t="n">
-        <v>3.504</v>
+        <v>3.541</v>
       </c>
       <c r="I6" t="n">
-        <v>3.815</v>
+        <v>3.855</v>
       </c>
       <c r="J6" t="n">
-        <v>4.106</v>
+        <v>4.164</v>
       </c>
       <c r="K6" t="n">
-        <v>4.408</v>
+        <v>4.476</v>
       </c>
       <c r="L6" t="n">
-        <v>4.423</v>
+        <v>4.481</v>
       </c>
       <c r="M6" t="n">
-        <v>4.544</v>
+        <v>4.596</v>
       </c>
       <c r="N6" t="n">
-        <v>4.594</v>
+        <v>4.649</v>
       </c>
       <c r="O6" t="n">
-        <v>4.767</v>
+        <v>4.828</v>
       </c>
       <c r="P6" t="n">
-        <v>5.196</v>
+        <v>5.279</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.02</v>
+        <v>6.114</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.042</v>
+        <v>3.069</v>
       </c>
       <c r="G7" t="n">
-        <v>3.19</v>
+        <v>3.223</v>
       </c>
       <c r="H7" t="n">
-        <v>3.451</v>
+        <v>3.488</v>
       </c>
       <c r="I7" t="n">
-        <v>3.752</v>
+        <v>3.792</v>
       </c>
       <c r="J7" t="n">
-        <v>4.04</v>
+        <v>4.098</v>
       </c>
       <c r="K7" t="n">
-        <v>4.323</v>
+        <v>4.391</v>
       </c>
       <c r="L7" t="n">
-        <v>4.331</v>
+        <v>4.39</v>
       </c>
       <c r="M7" t="n">
-        <v>4.449</v>
+        <v>4.501</v>
       </c>
       <c r="N7" t="n">
-        <v>4.486</v>
+        <v>4.541</v>
       </c>
       <c r="O7" t="n">
-        <v>4.664</v>
+        <v>4.725</v>
       </c>
       <c r="P7" t="n">
-        <v>4.979</v>
+        <v>5.063</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.788</v>
+        <v>5.881</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.457</v>
+        <v>5.484</v>
       </c>
       <c r="G8" t="n">
-        <v>6.13</v>
+        <v>6.163</v>
       </c>
       <c r="H8" t="n">
-        <v>6.612</v>
+        <v>6.649</v>
       </c>
       <c r="I8" t="n">
-        <v>6.915</v>
+        <v>6.956</v>
       </c>
       <c r="J8" t="n">
-        <v>7.295</v>
+        <v>7.354</v>
       </c>
       <c r="K8" t="n">
-        <v>8.081</v>
+        <v>8.148999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>8.4</v>
+        <v>8.458</v>
       </c>
       <c r="M8" t="n">
-        <v>8.737</v>
+        <v>8.789</v>
       </c>
       <c r="N8" t="n">
-        <v>8.898</v>
+        <v>8.952999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.221</v>
+        <v>9.282</v>
       </c>
       <c r="P8" t="n">
-        <v>9.385999999999999</v>
+        <v>9.468999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.09</v>
+        <v>10.183</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.634</v>
+        <v>2.646</v>
       </c>
       <c r="G9" t="n">
-        <v>2.745</v>
+        <v>2.763</v>
       </c>
       <c r="H9" t="n">
-        <v>2.969</v>
+        <v>2.999</v>
       </c>
       <c r="I9" t="n">
-        <v>3.239</v>
+        <v>3.282</v>
       </c>
       <c r="J9" t="n">
-        <v>3.502</v>
+        <v>3.545</v>
       </c>
       <c r="K9" t="n">
-        <v>3.785</v>
+        <v>3.829</v>
       </c>
       <c r="L9" t="n">
-        <v>3.812</v>
+        <v>3.86</v>
       </c>
       <c r="M9" t="n">
-        <v>3.88</v>
+        <v>3.93</v>
       </c>
       <c r="N9" t="n">
-        <v>4.038</v>
+        <v>4.091</v>
       </c>
       <c r="O9" t="n">
-        <v>4.12</v>
+        <v>4.18</v>
       </c>
       <c r="P9" t="n">
-        <v>4.198</v>
+        <v>4.281</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.252</v>
+        <v>4.345</v>
       </c>
       <c r="R9" t="n">
-        <v>4.291</v>
+        <v>4.376</v>
       </c>
       <c r="S9" t="n">
-        <v>4.326</v>
+        <v>4.397</v>
       </c>
       <c r="T9" t="n">
-        <v>4.265</v>
+        <v>4.33</v>
       </c>
       <c r="U9" t="n">
-        <v>4.192</v>
+        <v>4.267</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.668</v>
+        <v>2.682</v>
       </c>
       <c r="G10" t="n">
-        <v>2.795</v>
+        <v>2.815</v>
       </c>
       <c r="H10" t="n">
-        <v>2.987</v>
+        <v>3.02</v>
       </c>
       <c r="I10" t="n">
-        <v>3.25</v>
+        <v>3.293</v>
       </c>
       <c r="J10" t="n">
-        <v>3.534</v>
+        <v>3.581</v>
       </c>
       <c r="K10" t="n">
-        <v>3.818</v>
+        <v>3.864</v>
       </c>
       <c r="L10" t="n">
-        <v>3.865</v>
+        <v>3.913</v>
       </c>
       <c r="M10" t="n">
-        <v>3.974</v>
+        <v>4.024</v>
       </c>
       <c r="N10" t="n">
-        <v>4.061</v>
+        <v>4.115</v>
       </c>
       <c r="O10" t="n">
-        <v>4.337</v>
+        <v>4.4</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.472</v>
+        <v>2.486</v>
       </c>
       <c r="G11" t="n">
-        <v>2.595</v>
+        <v>2.615</v>
       </c>
       <c r="H11" t="n">
-        <v>2.81</v>
+        <v>2.843</v>
       </c>
       <c r="I11" t="n">
-        <v>3.054</v>
+        <v>3.098</v>
       </c>
       <c r="J11" t="n">
-        <v>3.328</v>
+        <v>3.373</v>
       </c>
       <c r="K11" t="n">
-        <v>3.605</v>
+        <v>3.651</v>
       </c>
       <c r="L11" t="n">
-        <v>3.662</v>
+        <v>3.711</v>
       </c>
       <c r="M11" t="n">
-        <v>3.782</v>
+        <v>3.832</v>
       </c>
       <c r="N11" t="n">
-        <v>3.869</v>
+        <v>3.922</v>
       </c>
       <c r="O11" t="n">
-        <v>4.104</v>
+        <v>4.166</v>
       </c>
       <c r="P11" t="n">
-        <v>4.149</v>
+        <v>4.232</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.452</v>
+        <v>4.545</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.3</v>
+        <v>3.318</v>
       </c>
       <c r="G12" t="n">
-        <v>3.565</v>
+        <v>3.587</v>
       </c>
       <c r="H12" t="n">
-        <v>3.837</v>
+        <v>3.881</v>
       </c>
       <c r="I12" t="n">
-        <v>4.133</v>
+        <v>4.187</v>
       </c>
       <c r="J12" t="n">
-        <v>4.448</v>
+        <v>4.512</v>
       </c>
       <c r="K12" t="n">
-        <v>4.683</v>
+        <v>4.752</v>
       </c>
       <c r="L12" t="n">
-        <v>4.726</v>
+        <v>4.78</v>
       </c>
       <c r="M12" t="n">
-        <v>4.858</v>
+        <v>4.91</v>
       </c>
       <c r="N12" t="n">
-        <v>4.93</v>
+        <v>4.984</v>
       </c>
       <c r="O12" t="n">
-        <v>5.126</v>
+        <v>5.186</v>
       </c>
       <c r="P12" t="n">
-        <v>5.237</v>
+        <v>5.32</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.567</v>
+        <v>5.66</v>
       </c>
       <c r="R12" t="n">
-        <v>5.782</v>
+        <v>5.867</v>
       </c>
       <c r="S12" t="n">
-        <v>6.029</v>
+        <v>6.1</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.054</v>
+        <v>3.072</v>
       </c>
       <c r="G13" t="n">
-        <v>3.255</v>
+        <v>3.277</v>
       </c>
       <c r="H13" t="n">
-        <v>3.505</v>
+        <v>3.549</v>
       </c>
       <c r="I13" t="n">
-        <v>3.781</v>
+        <v>3.835</v>
       </c>
       <c r="J13" t="n">
-        <v>4.085</v>
+        <v>4.149</v>
       </c>
       <c r="K13" t="n">
-        <v>4.316</v>
+        <v>4.385</v>
       </c>
       <c r="L13" t="n">
-        <v>4.365</v>
+        <v>4.419</v>
       </c>
       <c r="M13" t="n">
-        <v>4.486</v>
+        <v>4.538</v>
       </c>
       <c r="N13" t="n">
-        <v>4.558</v>
+        <v>4.612</v>
       </c>
       <c r="O13" t="n">
-        <v>4.755</v>
+        <v>4.814</v>
       </c>
       <c r="P13" t="n">
-        <v>4.828</v>
+        <v>4.911</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.088</v>
+        <v>5.181</v>
       </c>
       <c r="R13" t="n">
-        <v>5.332</v>
+        <v>5.416</v>
       </c>
       <c r="S13" t="n">
-        <v>5.592</v>
+        <v>5.663</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.871</v>
+        <v>2.889</v>
       </c>
       <c r="G14" t="n">
-        <v>3.061</v>
+        <v>3.082</v>
       </c>
       <c r="H14" t="n">
-        <v>3.308</v>
+        <v>3.352</v>
       </c>
       <c r="I14" t="n">
-        <v>3.565</v>
+        <v>3.619</v>
       </c>
       <c r="J14" t="n">
-        <v>3.827</v>
+        <v>3.89</v>
       </c>
       <c r="K14" t="n">
-        <v>4.004</v>
+        <v>4.073</v>
       </c>
       <c r="L14" t="n">
-        <v>4.038</v>
+        <v>4.092</v>
       </c>
       <c r="M14" t="n">
-        <v>4.172</v>
+        <v>4.224</v>
       </c>
       <c r="N14" t="n">
-        <v>4.238</v>
+        <v>4.291</v>
       </c>
       <c r="O14" t="n">
-        <v>4.413</v>
+        <v>4.473</v>
       </c>
       <c r="P14" t="n">
-        <v>4.464</v>
+        <v>4.547</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.677</v>
+        <v>4.771</v>
       </c>
       <c r="R14" t="n">
-        <v>4.846</v>
+        <v>4.93</v>
       </c>
       <c r="S14" t="n">
-        <v>5.044</v>
+        <v>5.115</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.849</v>
+        <v>2.867</v>
       </c>
       <c r="G15" t="n">
-        <v>3.035</v>
+        <v>3.057</v>
       </c>
       <c r="H15" t="n">
-        <v>3.279</v>
+        <v>3.323</v>
       </c>
       <c r="I15" t="n">
-        <v>3.515</v>
+        <v>3.57</v>
       </c>
       <c r="J15" t="n">
-        <v>3.765</v>
+        <v>3.828</v>
       </c>
       <c r="K15" t="n">
-        <v>3.956</v>
+        <v>4.025</v>
       </c>
       <c r="L15" t="n">
-        <v>3.974</v>
+        <v>4.028</v>
       </c>
       <c r="M15" t="n">
-        <v>4.085</v>
+        <v>4.137</v>
       </c>
       <c r="N15" t="n">
-        <v>4.141</v>
+        <v>4.195</v>
       </c>
       <c r="O15" t="n">
-        <v>4.356</v>
+        <v>4.415</v>
       </c>
       <c r="P15" t="n">
-        <v>4.36</v>
+        <v>4.444</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.579</v>
+        <v>4.673</v>
       </c>
       <c r="R15" t="n">
-        <v>4.741</v>
+        <v>4.825</v>
       </c>
       <c r="S15" t="n">
-        <v>4.939</v>
+        <v>5.01</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.849</v>
+        <v>2.867</v>
       </c>
       <c r="G16" t="n">
-        <v>3.035</v>
+        <v>3.057</v>
       </c>
       <c r="H16" t="n">
-        <v>3.279</v>
+        <v>3.323</v>
       </c>
       <c r="I16" t="n">
-        <v>3.515</v>
+        <v>3.57</v>
       </c>
       <c r="J16" t="n">
-        <v>3.765</v>
+        <v>3.828</v>
       </c>
       <c r="K16" t="n">
-        <v>3.956</v>
+        <v>4.025</v>
       </c>
       <c r="L16" t="n">
-        <v>3.974</v>
+        <v>4.028</v>
       </c>
       <c r="M16" t="n">
-        <v>4.085</v>
+        <v>4.137</v>
       </c>
       <c r="N16" t="n">
-        <v>4.144</v>
+        <v>4.198</v>
       </c>
       <c r="O16" t="n">
-        <v>4.362</v>
+        <v>4.422</v>
       </c>
       <c r="P16" t="n">
-        <v>4.384</v>
+        <v>4.467</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.606</v>
+        <v>4.7</v>
       </c>
       <c r="R16" t="n">
-        <v>4.769</v>
+        <v>4.853</v>
       </c>
       <c r="S16" t="n">
-        <v>4.968</v>
+        <v>5.039</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.717</v>
+        <v>2.731</v>
       </c>
       <c r="G17" t="n">
-        <v>2.873</v>
+        <v>2.893</v>
       </c>
       <c r="H17" t="n">
-        <v>3.079</v>
+        <v>3.112</v>
       </c>
       <c r="I17" t="n">
-        <v>3.331</v>
+        <v>3.375</v>
       </c>
       <c r="J17" t="n">
-        <v>3.605</v>
+        <v>3.651</v>
       </c>
       <c r="K17" t="n">
-        <v>3.896</v>
+        <v>3.942</v>
       </c>
       <c r="L17" t="n">
-        <v>3.948</v>
+        <v>3.997</v>
       </c>
       <c r="M17" t="n">
-        <v>4.097</v>
+        <v>4.147</v>
       </c>
       <c r="N17" t="n">
-        <v>4.165</v>
+        <v>4.218</v>
       </c>
       <c r="O17" t="n">
-        <v>4.358</v>
+        <v>4.42</v>
       </c>
       <c r="P17" t="n">
-        <v>4.429</v>
+        <v>4.513</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.718</v>
+        <v>2.732</v>
       </c>
       <c r="G18" t="n">
-        <v>2.874</v>
+        <v>2.894</v>
       </c>
       <c r="H18" t="n">
-        <v>3.079</v>
+        <v>3.113</v>
       </c>
       <c r="I18" t="n">
-        <v>3.332</v>
+        <v>3.376</v>
       </c>
       <c r="J18" t="n">
-        <v>3.605</v>
+        <v>3.651</v>
       </c>
       <c r="K18" t="n">
-        <v>3.897</v>
+        <v>3.943</v>
       </c>
       <c r="L18" t="n">
-        <v>3.948</v>
+        <v>3.997</v>
       </c>
       <c r="M18" t="n">
-        <v>4.097</v>
+        <v>4.147</v>
       </c>
       <c r="N18" t="n">
-        <v>4.166</v>
+        <v>4.218</v>
       </c>
       <c r="O18" t="n">
-        <v>4.356</v>
+        <v>4.418</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.86</v>
+        <v>2.878</v>
       </c>
       <c r="G19" t="n">
-        <v>3.048</v>
+        <v>3.071</v>
       </c>
       <c r="H19" t="n">
-        <v>3.293</v>
+        <v>3.338</v>
       </c>
       <c r="I19" t="n">
-        <v>3.548</v>
+        <v>3.602</v>
       </c>
       <c r="J19" t="n">
-        <v>3.806</v>
+        <v>3.87</v>
       </c>
       <c r="K19" t="n">
-        <v>3.999</v>
+        <v>4.068</v>
       </c>
       <c r="L19" t="n">
-        <v>4.035</v>
+        <v>4.089</v>
       </c>
       <c r="M19" t="n">
-        <v>4.163</v>
+        <v>4.215</v>
       </c>
       <c r="N19" t="n">
-        <v>4.227</v>
+        <v>4.281</v>
       </c>
       <c r="O19" t="n">
-        <v>4.399</v>
+        <v>4.459</v>
       </c>
       <c r="P19" t="n">
-        <v>4.422</v>
+        <v>4.505</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.617</v>
+        <v>4.71</v>
       </c>
       <c r="R19" t="n">
-        <v>4.788</v>
+        <v>4.872</v>
       </c>
       <c r="S19" t="n">
-        <v>4.979</v>
+        <v>5.05</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.647</v>
+        <v>2.659</v>
       </c>
       <c r="G20" t="n">
-        <v>2.755</v>
+        <v>2.771</v>
       </c>
       <c r="H20" t="n">
-        <v>2.877</v>
+        <v>2.9</v>
       </c>
       <c r="I20" t="n">
-        <v>3.086</v>
+        <v>3.114</v>
       </c>
       <c r="J20" t="n">
-        <v>3.533</v>
+        <v>3.581</v>
       </c>
       <c r="K20" t="n">
-        <v>3.819</v>
+        <v>3.887</v>
       </c>
       <c r="L20" t="n">
-        <v>3.827</v>
+        <v>3.881</v>
       </c>
       <c r="M20" t="n">
-        <v>3.922</v>
+        <v>3.974</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.96</v>
+        <v>2.98</v>
       </c>
       <c r="G21" t="n">
-        <v>3.138</v>
+        <v>3.187</v>
       </c>
       <c r="H21" t="n">
-        <v>3.408</v>
+        <v>3.465</v>
       </c>
       <c r="I21" t="n">
-        <v>3.662</v>
+        <v>3.723</v>
       </c>
       <c r="J21" t="n">
-        <v>3.95</v>
+        <v>4.018</v>
       </c>
       <c r="K21" t="n">
-        <v>4.244</v>
+        <v>4.311</v>
       </c>
       <c r="L21" t="n">
-        <v>4.279</v>
+        <v>4.334</v>
       </c>
       <c r="M21" t="n">
-        <v>4.399</v>
+        <v>4.452</v>
       </c>
       <c r="N21" t="n">
-        <v>4.472</v>
+        <v>4.526</v>
       </c>
       <c r="O21" t="n">
-        <v>4.605</v>
+        <v>4.665</v>
       </c>
       <c r="P21" t="n">
-        <v>4.682</v>
+        <v>4.765</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.773</v>
+        <v>4.867</v>
       </c>
       <c r="R21" t="n">
-        <v>4.839</v>
+        <v>4.923</v>
       </c>
       <c r="S21" t="n">
-        <v>4.932</v>
+        <v>5.003</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.906</v>
+        <v>2.926</v>
       </c>
       <c r="G22" t="n">
-        <v>3.082</v>
+        <v>3.132</v>
       </c>
       <c r="H22" t="n">
-        <v>3.339</v>
+        <v>3.397</v>
       </c>
       <c r="I22" t="n">
-        <v>3.58</v>
+        <v>3.642</v>
       </c>
       <c r="J22" t="n">
-        <v>3.836</v>
+        <v>3.903</v>
       </c>
       <c r="K22" t="n">
-        <v>4.125</v>
+        <v>4.193</v>
       </c>
       <c r="L22" t="n">
-        <v>4.146</v>
+        <v>4.201</v>
       </c>
       <c r="M22" t="n">
-        <v>4.27</v>
+        <v>4.324</v>
       </c>
       <c r="N22" t="n">
-        <v>4.346</v>
+        <v>4.4</v>
       </c>
       <c r="O22" t="n">
-        <v>4.476</v>
+        <v>4.536</v>
       </c>
       <c r="P22" t="n">
-        <v>4.545</v>
+        <v>4.628</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.632</v>
+        <v>4.725</v>
       </c>
       <c r="R22" t="n">
-        <v>4.687</v>
+        <v>4.772</v>
       </c>
       <c r="S22" t="n">
-        <v>4.777</v>
+        <v>4.848</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.857</v>
+        <v>2.876</v>
       </c>
       <c r="G23" t="n">
-        <v>3.037</v>
+        <v>3.086</v>
       </c>
       <c r="H23" t="n">
-        <v>3.281</v>
+        <v>3.338</v>
       </c>
       <c r="I23" t="n">
-        <v>3.528</v>
+        <v>3.59</v>
       </c>
       <c r="J23" t="n">
-        <v>3.776</v>
+        <v>3.843</v>
       </c>
       <c r="K23" t="n">
-        <v>4.025</v>
+        <v>4.092</v>
       </c>
       <c r="L23" t="n">
-        <v>4.044</v>
+        <v>4.099</v>
       </c>
       <c r="M23" t="n">
-        <v>4.161</v>
+        <v>4.215</v>
       </c>
       <c r="N23" t="n">
-        <v>4.24</v>
+        <v>4.294</v>
       </c>
       <c r="O23" t="n">
-        <v>4.352</v>
+        <v>4.412</v>
       </c>
       <c r="P23" t="n">
-        <v>4.408</v>
+        <v>4.491</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.438</v>
+        <v>4.531</v>
       </c>
       <c r="R23" t="n">
-        <v>4.473</v>
+        <v>4.558</v>
       </c>
       <c r="S23" t="n">
-        <v>4.533</v>
+        <v>4.604</v>
       </c>
       <c r="T23" t="n">
-        <v>4.471</v>
+        <v>4.536</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.794</v>
+        <v>2.814</v>
       </c>
       <c r="G24" t="n">
-        <v>2.948</v>
+        <v>2.997</v>
       </c>
       <c r="H24" t="n">
-        <v>3.174</v>
+        <v>3.231</v>
       </c>
       <c r="I24" t="n">
-        <v>3.466</v>
+        <v>3.528</v>
       </c>
       <c r="J24" t="n">
-        <v>3.669</v>
+        <v>3.736</v>
       </c>
       <c r="K24" t="n">
-        <v>3.908</v>
+        <v>3.975</v>
       </c>
       <c r="L24" t="n">
-        <v>3.925</v>
+        <v>3.98</v>
       </c>
       <c r="M24" t="n">
-        <v>4.021</v>
+        <v>4.074</v>
       </c>
       <c r="N24" t="n">
-        <v>4.114</v>
+        <v>4.168</v>
       </c>
       <c r="O24" t="n">
-        <v>4.351</v>
+        <v>4.412</v>
       </c>
       <c r="P24" t="n">
-        <v>4.347</v>
+        <v>4.43</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.363</v>
+        <v>4.457</v>
       </c>
       <c r="R24" t="n">
-        <v>4.395</v>
+        <v>4.479</v>
       </c>
       <c r="S24" t="n">
-        <v>4.448</v>
+        <v>4.519</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.851</v>
+        <v>2.871</v>
       </c>
       <c r="G25" t="n">
-        <v>3.037</v>
+        <v>3.086</v>
       </c>
       <c r="H25" t="n">
-        <v>3.284</v>
+        <v>3.341</v>
       </c>
       <c r="I25" t="n">
-        <v>3.537</v>
+        <v>3.599</v>
       </c>
       <c r="J25" t="n">
-        <v>3.791</v>
+        <v>3.858</v>
       </c>
       <c r="K25" t="n">
-        <v>4.057</v>
+        <v>4.124</v>
       </c>
       <c r="L25" t="n">
-        <v>4.075</v>
+        <v>4.129</v>
       </c>
       <c r="M25" t="n">
-        <v>4.192</v>
+        <v>4.246</v>
       </c>
       <c r="N25" t="n">
-        <v>4.267</v>
+        <v>4.321</v>
       </c>
       <c r="O25" t="n">
-        <v>4.381</v>
+        <v>4.441</v>
       </c>
       <c r="P25" t="n">
-        <v>4.429</v>
+        <v>4.513</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.471</v>
+        <v>4.564</v>
       </c>
       <c r="R25" t="n">
-        <v>4.497</v>
+        <v>4.581</v>
       </c>
       <c r="S25" t="n">
-        <v>4.557</v>
+        <v>4.628</v>
       </c>
       <c r="T25" t="n">
-        <v>4.489</v>
+        <v>4.554</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.147</v>
+        <v>3.171</v>
       </c>
       <c r="G26" t="n">
-        <v>3.36</v>
+        <v>3.387</v>
       </c>
       <c r="H26" t="n">
-        <v>3.711</v>
+        <v>3.743</v>
       </c>
       <c r="I26" t="n">
-        <v>3.998</v>
+        <v>4.037</v>
       </c>
       <c r="J26" t="n">
-        <v>4.41</v>
+        <v>4.464</v>
       </c>
       <c r="K26" t="n">
-        <v>4.863</v>
+        <v>4.933</v>
       </c>
       <c r="L26" t="n">
-        <v>4.951</v>
+        <v>5.008</v>
       </c>
       <c r="M26" t="n">
-        <v>5.112</v>
+        <v>5.164</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.437</v>
+        <v>5.498</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.958</v>
+        <v>2.978</v>
       </c>
       <c r="G27" t="n">
-        <v>3.126</v>
+        <v>3.148</v>
       </c>
       <c r="H27" t="n">
-        <v>3.385</v>
+        <v>3.423</v>
       </c>
       <c r="I27" t="n">
-        <v>3.643</v>
+        <v>3.69</v>
       </c>
       <c r="J27" t="n">
-        <v>3.93</v>
+        <v>3.989</v>
       </c>
       <c r="K27" t="n">
-        <v>4.179</v>
+        <v>4.25</v>
       </c>
       <c r="L27" t="n">
-        <v>4.219</v>
+        <v>4.274</v>
       </c>
       <c r="M27" t="n">
-        <v>4.332</v>
+        <v>4.384</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.54</v>
+        <v>4.601</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.061</v>
+        <v>3.081</v>
       </c>
       <c r="G28" t="n">
-        <v>3.237</v>
+        <v>3.259</v>
       </c>
       <c r="H28" t="n">
-        <v>3.51</v>
+        <v>3.548</v>
       </c>
       <c r="I28" t="n">
-        <v>3.78</v>
+        <v>3.827</v>
       </c>
       <c r="J28" t="n">
-        <v>4.103</v>
+        <v>4.162</v>
       </c>
       <c r="K28" t="n">
-        <v>4.371</v>
+        <v>4.442</v>
       </c>
       <c r="L28" t="n">
-        <v>4.422</v>
+        <v>4.477</v>
       </c>
       <c r="M28" t="n">
-        <v>4.544</v>
+        <v>4.596</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.833</v>
+        <v>4.894</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.907</v>
+        <v>2.927</v>
       </c>
       <c r="G29" t="n">
-        <v>3.074</v>
+        <v>3.096</v>
       </c>
       <c r="H29" t="n">
-        <v>3.324</v>
+        <v>3.362</v>
       </c>
       <c r="I29" t="n">
-        <v>3.57</v>
+        <v>3.617</v>
       </c>
       <c r="J29" t="n">
-        <v>3.842</v>
+        <v>3.901</v>
       </c>
       <c r="K29" t="n">
-        <v>4.074</v>
+        <v>4.145</v>
       </c>
       <c r="L29" t="n">
-        <v>4.104</v>
+        <v>4.159</v>
       </c>
       <c r="M29" t="n">
-        <v>4.195</v>
+        <v>4.247</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.412</v>
+        <v>4.473</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.188</v>
+        <v>3.212</v>
       </c>
       <c r="G30" t="n">
-        <v>3.335</v>
+        <v>3.361</v>
       </c>
       <c r="H30" t="n">
-        <v>3.645</v>
+        <v>3.676</v>
       </c>
       <c r="I30" t="n">
-        <v>3.925</v>
+        <v>3.963</v>
       </c>
       <c r="J30" t="n">
-        <v>4.274</v>
+        <v>4.327</v>
       </c>
       <c r="K30" t="n">
-        <v>4.663</v>
+        <v>4.733</v>
       </c>
       <c r="L30" t="n">
-        <v>4.729</v>
+        <v>4.784</v>
       </c>
       <c r="M30" t="n">
-        <v>4.879</v>
+        <v>4.931</v>
       </c>
       <c r="N30" t="n">
-        <v>5.055</v>
+        <v>5.109</v>
       </c>
       <c r="O30" t="n">
-        <v>5.389</v>
+        <v>5.45</v>
       </c>
       <c r="P30" t="n">
-        <v>5.575</v>
+        <v>5.658</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.311</v>
+        <v>6.404</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.517</v>
+        <v>3.541</v>
       </c>
       <c r="G31" t="n">
-        <v>3.7</v>
+        <v>3.726</v>
       </c>
       <c r="H31" t="n">
-        <v>4.061</v>
+        <v>4.092</v>
       </c>
       <c r="I31" t="n">
-        <v>4.354</v>
+        <v>4.392</v>
       </c>
       <c r="J31" t="n">
-        <v>4.765</v>
+        <v>4.818</v>
       </c>
       <c r="K31" t="n">
-        <v>5.195</v>
+        <v>5.266</v>
       </c>
       <c r="L31" t="n">
-        <v>5.342</v>
+        <v>5.397</v>
       </c>
       <c r="M31" t="n">
-        <v>5.61</v>
+        <v>5.662</v>
       </c>
       <c r="N31" t="n">
-        <v>5.914</v>
+        <v>5.968</v>
       </c>
       <c r="O31" t="n">
-        <v>6.425</v>
+        <v>6.486</v>
       </c>
       <c r="P31" t="n">
-        <v>6.563</v>
+        <v>6.646</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.284</v>
+        <v>7.378</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.287</v>
+        <v>3.311</v>
       </c>
       <c r="G32" t="n">
-        <v>3.452</v>
+        <v>3.478</v>
       </c>
       <c r="H32" t="n">
-        <v>3.789</v>
+        <v>3.82</v>
       </c>
       <c r="I32" t="n">
-        <v>4.084</v>
+        <v>4.122</v>
       </c>
       <c r="J32" t="n">
-        <v>4.452</v>
+        <v>4.505</v>
       </c>
       <c r="K32" t="n">
-        <v>4.848</v>
+        <v>4.918</v>
       </c>
       <c r="L32" t="n">
-        <v>4.934</v>
+        <v>4.989</v>
       </c>
       <c r="M32" t="n">
-        <v>5.152</v>
+        <v>5.204</v>
       </c>
       <c r="N32" t="n">
-        <v>5.416</v>
+        <v>5.47</v>
       </c>
       <c r="O32" t="n">
-        <v>5.834</v>
+        <v>5.895</v>
       </c>
       <c r="P32" t="n">
-        <v>6.035</v>
+        <v>6.118</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.772</v>
+        <v>6.865</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.053</v>
+        <v>3.077</v>
       </c>
       <c r="G33" t="n">
-        <v>3.2</v>
+        <v>3.226</v>
       </c>
       <c r="H33" t="n">
-        <v>3.463</v>
+        <v>3.494</v>
       </c>
       <c r="I33" t="n">
-        <v>3.71</v>
+        <v>3.748</v>
       </c>
       <c r="J33" t="n">
-        <v>3.981</v>
+        <v>4.034</v>
       </c>
       <c r="K33" t="n">
-        <v>4.305</v>
+        <v>4.374</v>
       </c>
       <c r="L33" t="n">
-        <v>4.333</v>
+        <v>4.39</v>
       </c>
       <c r="M33" t="n">
-        <v>4.406</v>
+        <v>4.458</v>
       </c>
       <c r="N33" t="n">
-        <v>4.445</v>
+        <v>4.498</v>
       </c>
       <c r="O33" t="n">
-        <v>4.543</v>
+        <v>4.604</v>
       </c>
       <c r="P33" t="n">
-        <v>4.607</v>
+        <v>4.69</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.028</v>
+        <v>5.121</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.113</v>
+        <v>3.137</v>
       </c>
       <c r="G34" t="n">
-        <v>3.253</v>
+        <v>3.279</v>
       </c>
       <c r="H34" t="n">
-        <v>3.525</v>
+        <v>3.556</v>
       </c>
       <c r="I34" t="n">
-        <v>3.778</v>
+        <v>3.816</v>
       </c>
       <c r="J34" t="n">
-        <v>4.053</v>
+        <v>4.106</v>
       </c>
       <c r="K34" t="n">
-        <v>4.381</v>
+        <v>4.45</v>
       </c>
       <c r="L34" t="n">
-        <v>4.412</v>
+        <v>4.469</v>
       </c>
       <c r="M34" t="n">
-        <v>4.496</v>
+        <v>4.548</v>
       </c>
       <c r="N34" t="n">
-        <v>4.549</v>
+        <v>4.603</v>
       </c>
       <c r="O34" t="n">
-        <v>4.712</v>
+        <v>4.773</v>
       </c>
       <c r="P34" t="n">
-        <v>4.901</v>
+        <v>4.985</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.729</v>
+        <v>5.822</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.087</v>
+        <v>3.111</v>
       </c>
       <c r="G35" t="n">
-        <v>3.226</v>
+        <v>3.253</v>
       </c>
       <c r="H35" t="n">
-        <v>3.493</v>
+        <v>3.524</v>
       </c>
       <c r="I35" t="n">
-        <v>3.744</v>
+        <v>3.782</v>
       </c>
       <c r="J35" t="n">
-        <v>4.021</v>
+        <v>4.074</v>
       </c>
       <c r="K35" t="n">
-        <v>4.335</v>
+        <v>4.404</v>
       </c>
       <c r="L35" t="n">
-        <v>4.367</v>
+        <v>4.424</v>
       </c>
       <c r="M35" t="n">
-        <v>4.443</v>
+        <v>4.495</v>
       </c>
       <c r="N35" t="n">
-        <v>4.485</v>
+        <v>4.539</v>
       </c>
       <c r="O35" t="n">
-        <v>4.609</v>
+        <v>4.67</v>
       </c>
       <c r="P35" t="n">
-        <v>4.704</v>
+        <v>4.787</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.364</v>
+        <v>5.458</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.977</v>
+        <v>3.001</v>
       </c>
       <c r="G36" t="n">
-        <v>3.114</v>
+        <v>3.139</v>
       </c>
       <c r="H36" t="n">
-        <v>3.372</v>
+        <v>3.403</v>
       </c>
       <c r="I36" t="n">
-        <v>3.622</v>
+        <v>3.66</v>
       </c>
       <c r="J36" t="n">
-        <v>3.918</v>
+        <v>3.971</v>
       </c>
       <c r="K36" t="n">
-        <v>4.23</v>
+        <v>4.3</v>
       </c>
       <c r="L36" t="n">
-        <v>4.258</v>
+        <v>4.313</v>
       </c>
       <c r="M36" t="n">
-        <v>4.309</v>
+        <v>4.361</v>
       </c>
       <c r="N36" t="n">
-        <v>4.349</v>
+        <v>4.403</v>
       </c>
       <c r="O36" t="n">
-        <v>4.451</v>
+        <v>4.512</v>
       </c>
       <c r="P36" t="n">
-        <v>4.505</v>
+        <v>4.588</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.745</v>
+        <v>4.838</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.86</v>
+        <v>3.884</v>
       </c>
       <c r="G37" t="n">
-        <v>4.394</v>
+        <v>4.42</v>
       </c>
       <c r="H37" t="n">
-        <v>5.033</v>
+        <v>5.064</v>
       </c>
       <c r="I37" t="n">
-        <v>5.415</v>
+        <v>5.453</v>
       </c>
       <c r="J37" t="n">
-        <v>6.254</v>
+        <v>6.308</v>
       </c>
       <c r="K37" t="n">
-        <v>7.235</v>
+        <v>7.305</v>
       </c>
       <c r="L37" t="n">
-        <v>7.542</v>
+        <v>7.598</v>
       </c>
       <c r="M37" t="n">
-        <v>7.882</v>
+        <v>7.934</v>
       </c>
       <c r="N37" t="n">
-        <v>8.069000000000001</v>
+        <v>8.122999999999999</v>
       </c>
       <c r="O37" t="n">
-        <v>8.304</v>
+        <v>8.365</v>
       </c>
       <c r="P37" t="n">
-        <v>8.365</v>
+        <v>8.448</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.775</v>
+        <v>8.868</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.922</v>
+        <v>4.946</v>
       </c>
       <c r="G38" t="n">
-        <v>5.709</v>
+        <v>5.735</v>
       </c>
       <c r="H38" t="n">
-        <v>6.56</v>
+        <v>6.591</v>
       </c>
       <c r="I38" t="n">
-        <v>7.099</v>
+        <v>7.137</v>
       </c>
       <c r="J38" t="n">
-        <v>8.198</v>
+        <v>8.252000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.358000000000001</v>
+        <v>9.428000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.824999999999999</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>10.294</v>
+        <v>10.346</v>
       </c>
       <c r="N38" t="n">
-        <v>10.488</v>
+        <v>10.542</v>
       </c>
       <c r="O38" t="n">
-        <v>10.704</v>
+        <v>10.765</v>
       </c>
       <c r="P38" t="n">
-        <v>10.762</v>
+        <v>10.846</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.225</v>
+        <v>11.318</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.242</v>
+        <v>4.266</v>
       </c>
       <c r="G39" t="n">
-        <v>4.907</v>
+        <v>4.933</v>
       </c>
       <c r="H39" t="n">
-        <v>5.625</v>
+        <v>5.656</v>
       </c>
       <c r="I39" t="n">
-        <v>6.103</v>
+        <v>6.141</v>
       </c>
       <c r="J39" t="n">
-        <v>7.071</v>
+        <v>7.124</v>
       </c>
       <c r="K39" t="n">
-        <v>8.19</v>
+        <v>8.260999999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>8.58</v>
+        <v>8.635999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.93</v>
+        <v>8.981999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>9.116</v>
+        <v>9.17</v>
       </c>
       <c r="O39" t="n">
-        <v>9.355</v>
+        <v>9.416</v>
       </c>
       <c r="P39" t="n">
-        <v>9.417</v>
+        <v>9.5</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.869999999999999</v>
+        <v>9.964</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.38</v>
+        <v>3.404</v>
       </c>
       <c r="G40" t="n">
-        <v>3.573</v>
+        <v>3.599</v>
       </c>
       <c r="H40" t="n">
-        <v>3.904</v>
+        <v>3.935</v>
       </c>
       <c r="I40" t="n">
-        <v>4.198</v>
+        <v>4.236</v>
       </c>
       <c r="J40" t="n">
-        <v>4.565</v>
+        <v>4.619</v>
       </c>
       <c r="K40" t="n">
-        <v>4.969</v>
+        <v>5.039</v>
       </c>
       <c r="L40" t="n">
-        <v>5.054</v>
+        <v>5.109</v>
       </c>
       <c r="M40" t="n">
-        <v>5.222</v>
+        <v>5.274</v>
       </c>
       <c r="N40" t="n">
-        <v>5.413</v>
+        <v>5.467</v>
       </c>
       <c r="O40" t="n">
-        <v>5.768</v>
+        <v>5.829</v>
       </c>
       <c r="P40" t="n">
-        <v>5.996</v>
+        <v>6.079</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.762</v>
+        <v>6.855</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.766</v>
+        <v>3.79</v>
       </c>
       <c r="G41" t="n">
-        <v>4.002</v>
+        <v>4.028</v>
       </c>
       <c r="H41" t="n">
-        <v>4.39</v>
+        <v>4.421</v>
       </c>
       <c r="I41" t="n">
-        <v>4.702</v>
+        <v>4.74</v>
       </c>
       <c r="J41" t="n">
-        <v>5.12</v>
+        <v>5.174</v>
       </c>
       <c r="K41" t="n">
-        <v>5.569</v>
+        <v>5.639</v>
       </c>
       <c r="L41" t="n">
-        <v>5.733</v>
+        <v>5.788</v>
       </c>
       <c r="M41" t="n">
-        <v>6.025</v>
+        <v>6.077</v>
       </c>
       <c r="N41" t="n">
-        <v>6.344</v>
+        <v>6.397</v>
       </c>
       <c r="O41" t="n">
-        <v>6.883</v>
+        <v>6.944</v>
       </c>
       <c r="P41" t="n">
-        <v>7.055</v>
+        <v>7.139</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.809</v>
+        <v>7.902</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.501</v>
+        <v>3.525</v>
       </c>
       <c r="G42" t="n">
-        <v>3.722</v>
+        <v>3.748</v>
       </c>
       <c r="H42" t="n">
-        <v>4.08</v>
+        <v>4.111</v>
       </c>
       <c r="I42" t="n">
-        <v>4.387</v>
+        <v>4.425</v>
       </c>
       <c r="J42" t="n">
-        <v>4.768</v>
+        <v>4.821</v>
       </c>
       <c r="K42" t="n">
-        <v>5.19</v>
+        <v>5.26</v>
       </c>
       <c r="L42" t="n">
-        <v>5.29</v>
+        <v>5.345</v>
       </c>
       <c r="M42" t="n">
-        <v>5.529</v>
+        <v>5.581</v>
       </c>
       <c r="N42" t="n">
-        <v>5.827</v>
+        <v>5.881</v>
       </c>
       <c r="O42" t="n">
-        <v>6.26</v>
+        <v>6.321</v>
       </c>
       <c r="P42" t="n">
-        <v>6.498</v>
+        <v>6.581</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.274</v>
+        <v>7.368</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.201</v>
+        <v>3.225</v>
       </c>
       <c r="G43" t="n">
-        <v>3.382</v>
+        <v>3.408</v>
       </c>
       <c r="H43" t="n">
-        <v>3.664</v>
+        <v>3.695</v>
       </c>
       <c r="I43" t="n">
-        <v>3.918</v>
+        <v>3.956</v>
       </c>
       <c r="J43" t="n">
-        <v>4.208</v>
+        <v>4.262</v>
       </c>
       <c r="K43" t="n">
-        <v>4.537</v>
+        <v>4.606</v>
       </c>
       <c r="L43" t="n">
-        <v>4.575</v>
+        <v>4.631</v>
       </c>
       <c r="M43" t="n">
-        <v>4.661</v>
+        <v>4.713</v>
       </c>
       <c r="N43" t="n">
-        <v>4.714</v>
+        <v>4.767</v>
       </c>
       <c r="O43" t="n">
-        <v>4.856</v>
+        <v>4.917</v>
       </c>
       <c r="P43" t="n">
-        <v>4.973</v>
+        <v>5.056</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.638</v>
+        <v>5.731</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.055</v>
+        <v>3.079</v>
       </c>
       <c r="G44" t="n">
-        <v>3.223</v>
+        <v>3.249</v>
       </c>
       <c r="H44" t="n">
-        <v>3.495</v>
+        <v>3.526</v>
       </c>
       <c r="I44" t="n">
-        <v>3.749</v>
+        <v>3.787</v>
       </c>
       <c r="J44" t="n">
-        <v>4.058</v>
+        <v>4.112</v>
       </c>
       <c r="K44" t="n">
-        <v>4.382</v>
+        <v>4.452</v>
       </c>
       <c r="L44" t="n">
-        <v>4.419</v>
+        <v>4.474</v>
       </c>
       <c r="M44" t="n">
-        <v>4.479</v>
+        <v>4.531</v>
       </c>
       <c r="N44" t="n">
-        <v>4.531</v>
+        <v>4.584</v>
       </c>
       <c r="O44" t="n">
-        <v>4.652</v>
+        <v>4.713</v>
       </c>
       <c r="P44" t="n">
-        <v>4.735</v>
+        <v>4.818</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.008</v>
+        <v>5.102</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-09 ~ 2026-06-09
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.35</v>
+        <v>3.376</v>
       </c>
       <c r="G2" t="n">
-        <v>3.661</v>
+        <v>3.688</v>
       </c>
       <c r="H2" t="n">
-        <v>3.965</v>
+        <v>3.988</v>
       </c>
       <c r="I2" t="n">
-        <v>4.201</v>
+        <v>4.196</v>
       </c>
       <c r="J2" t="n">
-        <v>4.516</v>
+        <v>4.505</v>
       </c>
       <c r="K2" t="n">
-        <v>4.959</v>
+        <v>4.897</v>
       </c>
       <c r="L2" t="n">
-        <v>5.115</v>
+        <v>5.067</v>
       </c>
       <c r="M2" t="n">
-        <v>5.382</v>
+        <v>5.324</v>
       </c>
       <c r="N2" t="n">
-        <v>5.669</v>
+        <v>5.59</v>
       </c>
       <c r="O2" t="n">
-        <v>5.962</v>
+        <v>5.884</v>
       </c>
       <c r="P2" t="n">
-        <v>6.178</v>
+        <v>6.095</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.805</v>
+        <v>6.732</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.372</v>
+        <v>4.398</v>
       </c>
       <c r="G3" t="n">
-        <v>4.864</v>
+        <v>4.891</v>
       </c>
       <c r="H3" t="n">
-        <v>5.2</v>
+        <v>5.223</v>
       </c>
       <c r="I3" t="n">
-        <v>5.429</v>
+        <v>5.425</v>
       </c>
       <c r="J3" t="n">
-        <v>5.761</v>
+        <v>5.751</v>
       </c>
       <c r="K3" t="n">
-        <v>6.275</v>
+        <v>6.213</v>
       </c>
       <c r="L3" t="n">
-        <v>6.5</v>
+        <v>6.453</v>
       </c>
       <c r="M3" t="n">
-        <v>6.798</v>
+        <v>6.74</v>
       </c>
       <c r="N3" t="n">
-        <v>7.028</v>
+        <v>6.949</v>
       </c>
       <c r="O3" t="n">
-        <v>7.272</v>
+        <v>7.194</v>
       </c>
       <c r="P3" t="n">
-        <v>7.356</v>
+        <v>7.273</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.872</v>
+        <v>7.798</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.864</v>
+        <v>3.89</v>
       </c>
       <c r="G4" t="n">
-        <v>4.245</v>
+        <v>4.272</v>
       </c>
       <c r="H4" t="n">
-        <v>4.61</v>
+        <v>4.633</v>
       </c>
       <c r="I4" t="n">
-        <v>4.872</v>
+        <v>4.867</v>
       </c>
       <c r="J4" t="n">
-        <v>5.205</v>
+        <v>5.194</v>
       </c>
       <c r="K4" t="n">
-        <v>5.714</v>
+        <v>5.652</v>
       </c>
       <c r="L4" t="n">
-        <v>5.869</v>
+        <v>5.822</v>
       </c>
       <c r="M4" t="n">
-        <v>6.156</v>
+        <v>6.098</v>
       </c>
       <c r="N4" t="n">
-        <v>6.357</v>
+        <v>6.277</v>
       </c>
       <c r="O4" t="n">
-        <v>6.624</v>
+        <v>6.545</v>
       </c>
       <c r="P4" t="n">
-        <v>6.708</v>
+        <v>6.626</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.226</v>
+        <v>7.153</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.048</v>
+        <v>3.074</v>
       </c>
       <c r="G5" t="n">
-        <v>3.204</v>
+        <v>3.231</v>
       </c>
       <c r="H5" t="n">
-        <v>3.472</v>
+        <v>3.495</v>
       </c>
       <c r="I5" t="n">
-        <v>3.773</v>
+        <v>3.768</v>
       </c>
       <c r="J5" t="n">
-        <v>4.074</v>
+        <v>4.064</v>
       </c>
       <c r="K5" t="n">
-        <v>4.364</v>
+        <v>4.302</v>
       </c>
       <c r="L5" t="n">
-        <v>4.363</v>
+        <v>4.316</v>
       </c>
       <c r="M5" t="n">
-        <v>4.441</v>
+        <v>4.383</v>
       </c>
       <c r="N5" t="n">
-        <v>4.481</v>
+        <v>4.402</v>
       </c>
       <c r="O5" t="n">
-        <v>4.562</v>
+        <v>4.484</v>
       </c>
       <c r="P5" t="n">
-        <v>4.846</v>
+        <v>4.764</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.718</v>
+        <v>5.644</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.089</v>
+        <v>3.115</v>
       </c>
       <c r="G6" t="n">
-        <v>3.259</v>
+        <v>3.286</v>
       </c>
       <c r="H6" t="n">
-        <v>3.541</v>
+        <v>3.564</v>
       </c>
       <c r="I6" t="n">
-        <v>3.855</v>
+        <v>3.851</v>
       </c>
       <c r="J6" t="n">
-        <v>4.164</v>
+        <v>4.154</v>
       </c>
       <c r="K6" t="n">
-        <v>4.476</v>
+        <v>4.414</v>
       </c>
       <c r="L6" t="n">
-        <v>4.481</v>
+        <v>4.434</v>
       </c>
       <c r="M6" t="n">
-        <v>4.596</v>
+        <v>4.538</v>
       </c>
       <c r="N6" t="n">
-        <v>4.649</v>
+        <v>4.57</v>
       </c>
       <c r="O6" t="n">
-        <v>4.828</v>
+        <v>4.75</v>
       </c>
       <c r="P6" t="n">
-        <v>5.279</v>
+        <v>5.196</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.114</v>
+        <v>6.04</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.069</v>
+        <v>3.095</v>
       </c>
       <c r="G7" t="n">
-        <v>3.223</v>
+        <v>3.25</v>
       </c>
       <c r="H7" t="n">
-        <v>3.488</v>
+        <v>3.511</v>
       </c>
       <c r="I7" t="n">
-        <v>3.792</v>
+        <v>3.788</v>
       </c>
       <c r="J7" t="n">
-        <v>4.098</v>
+        <v>4.088</v>
       </c>
       <c r="K7" t="n">
-        <v>4.391</v>
+        <v>4.329</v>
       </c>
       <c r="L7" t="n">
-        <v>4.39</v>
+        <v>4.343</v>
       </c>
       <c r="M7" t="n">
-        <v>4.501</v>
+        <v>4.443</v>
       </c>
       <c r="N7" t="n">
-        <v>4.541</v>
+        <v>4.462</v>
       </c>
       <c r="O7" t="n">
-        <v>4.725</v>
+        <v>4.647</v>
       </c>
       <c r="P7" t="n">
-        <v>5.063</v>
+        <v>4.98</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.881</v>
+        <v>5.808</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.484</v>
+        <v>5.51</v>
       </c>
       <c r="G8" t="n">
-        <v>6.163</v>
+        <v>6.19</v>
       </c>
       <c r="H8" t="n">
-        <v>6.649</v>
+        <v>6.672</v>
       </c>
       <c r="I8" t="n">
-        <v>6.956</v>
+        <v>6.951</v>
       </c>
       <c r="J8" t="n">
-        <v>7.354</v>
+        <v>7.343</v>
       </c>
       <c r="K8" t="n">
-        <v>8.148999999999999</v>
+        <v>8.087</v>
       </c>
       <c r="L8" t="n">
-        <v>8.458</v>
+        <v>8.411</v>
       </c>
       <c r="M8" t="n">
-        <v>8.789</v>
+        <v>8.731</v>
       </c>
       <c r="N8" t="n">
-        <v>8.952999999999999</v>
+        <v>8.874000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.282</v>
+        <v>9.204000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.468999999999999</v>
+        <v>9.387</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.183</v>
+        <v>10.11</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.646</v>
+        <v>2.652</v>
       </c>
       <c r="G9" t="n">
-        <v>2.763</v>
+        <v>2.769</v>
       </c>
       <c r="H9" t="n">
-        <v>2.999</v>
+        <v>3.007</v>
       </c>
       <c r="I9" t="n">
-        <v>3.282</v>
+        <v>3.286</v>
       </c>
       <c r="J9" t="n">
-        <v>3.545</v>
+        <v>3.522</v>
       </c>
       <c r="K9" t="n">
-        <v>3.829</v>
+        <v>3.759</v>
       </c>
       <c r="L9" t="n">
+        <v>3.795</v>
+      </c>
+      <c r="M9" t="n">
         <v>3.86</v>
       </c>
-      <c r="M9" t="n">
-        <v>3.93</v>
-      </c>
       <c r="N9" t="n">
-        <v>4.091</v>
+        <v>4.004</v>
       </c>
       <c r="O9" t="n">
-        <v>4.18</v>
+        <v>4.1</v>
       </c>
       <c r="P9" t="n">
-        <v>4.281</v>
+        <v>4.198</v>
       </c>
       <c r="Q9" t="n">
+        <v>4.272</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.313</v>
+      </c>
+      <c r="S9" t="n">
         <v>4.345</v>
       </c>
-      <c r="R9" t="n">
-        <v>4.376</v>
-      </c>
-      <c r="S9" t="n">
-        <v>4.397</v>
-      </c>
       <c r="T9" t="n">
-        <v>4.33</v>
+        <v>4.285</v>
       </c>
       <c r="U9" t="n">
-        <v>4.267</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.682</v>
+        <v>2.686</v>
       </c>
       <c r="G10" t="n">
-        <v>2.815</v>
+        <v>2.818</v>
       </c>
       <c r="H10" t="n">
-        <v>3.02</v>
+        <v>3.03</v>
       </c>
       <c r="I10" t="n">
-        <v>3.293</v>
+        <v>3.3</v>
       </c>
       <c r="J10" t="n">
-        <v>3.581</v>
+        <v>3.56</v>
       </c>
       <c r="K10" t="n">
-        <v>3.864</v>
+        <v>3.795</v>
       </c>
       <c r="L10" t="n">
-        <v>3.913</v>
+        <v>3.848</v>
       </c>
       <c r="M10" t="n">
-        <v>4.024</v>
+        <v>3.954</v>
       </c>
       <c r="N10" t="n">
-        <v>4.115</v>
+        <v>4.029</v>
       </c>
       <c r="O10" t="n">
-        <v>4.4</v>
+        <v>4.32</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.486</v>
+        <v>2.49</v>
       </c>
       <c r="G11" t="n">
-        <v>2.615</v>
+        <v>2.618</v>
       </c>
       <c r="H11" t="n">
-        <v>2.843</v>
+        <v>2.853</v>
       </c>
       <c r="I11" t="n">
-        <v>3.098</v>
+        <v>3.104</v>
       </c>
       <c r="J11" t="n">
-        <v>3.373</v>
+        <v>3.352</v>
       </c>
       <c r="K11" t="n">
-        <v>3.651</v>
+        <v>3.581</v>
       </c>
       <c r="L11" t="n">
-        <v>3.711</v>
+        <v>3.645</v>
       </c>
       <c r="M11" t="n">
-        <v>3.832</v>
+        <v>3.762</v>
       </c>
       <c r="N11" t="n">
-        <v>3.922</v>
+        <v>3.836</v>
       </c>
       <c r="O11" t="n">
-        <v>4.166</v>
+        <v>4.086</v>
       </c>
       <c r="P11" t="n">
-        <v>4.232</v>
+        <v>4.148</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.545</v>
+        <v>4.471</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.318</v>
+        <v>3.322</v>
       </c>
       <c r="G12" t="n">
-        <v>3.587</v>
+        <v>3.598</v>
       </c>
       <c r="H12" t="n">
-        <v>3.881</v>
+        <v>3.897</v>
       </c>
       <c r="I12" t="n">
-        <v>4.187</v>
+        <v>4.184</v>
       </c>
       <c r="J12" t="n">
-        <v>4.512</v>
+        <v>4.508</v>
       </c>
       <c r="K12" t="n">
-        <v>4.752</v>
+        <v>4.69</v>
       </c>
       <c r="L12" t="n">
-        <v>4.78</v>
+        <v>4.733</v>
       </c>
       <c r="M12" t="n">
-        <v>4.91</v>
+        <v>4.857</v>
       </c>
       <c r="N12" t="n">
-        <v>4.984</v>
+        <v>4.909</v>
       </c>
       <c r="O12" t="n">
-        <v>5.186</v>
+        <v>5.107</v>
       </c>
       <c r="P12" t="n">
-        <v>5.32</v>
+        <v>5.237</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.66</v>
+        <v>5.587</v>
       </c>
       <c r="R12" t="n">
-        <v>5.867</v>
+        <v>5.804</v>
       </c>
       <c r="S12" t="n">
-        <v>6.1</v>
+        <v>6.048</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.072</v>
+        <v>3.076</v>
       </c>
       <c r="G13" t="n">
-        <v>3.277</v>
+        <v>3.288</v>
       </c>
       <c r="H13" t="n">
-        <v>3.549</v>
+        <v>3.564</v>
       </c>
       <c r="I13" t="n">
-        <v>3.835</v>
+        <v>3.832</v>
       </c>
       <c r="J13" t="n">
-        <v>4.149</v>
+        <v>4.145</v>
       </c>
       <c r="K13" t="n">
-        <v>4.385</v>
+        <v>4.323</v>
       </c>
       <c r="L13" t="n">
-        <v>4.419</v>
+        <v>4.372</v>
       </c>
       <c r="M13" t="n">
+        <v>4.485</v>
+      </c>
+      <c r="N13" t="n">
         <v>4.538</v>
       </c>
-      <c r="N13" t="n">
-        <v>4.612</v>
-      </c>
       <c r="O13" t="n">
-        <v>4.814</v>
+        <v>4.735</v>
       </c>
       <c r="P13" t="n">
-        <v>4.911</v>
+        <v>4.828</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.181</v>
+        <v>5.108</v>
       </c>
       <c r="R13" t="n">
-        <v>5.416</v>
+        <v>5.354</v>
       </c>
       <c r="S13" t="n">
-        <v>5.663</v>
+        <v>5.611</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.889</v>
+        <v>2.893</v>
       </c>
       <c r="G14" t="n">
-        <v>3.082</v>
+        <v>3.094</v>
       </c>
       <c r="H14" t="n">
-        <v>3.352</v>
+        <v>3.367</v>
       </c>
       <c r="I14" t="n">
-        <v>3.619</v>
+        <v>3.616</v>
       </c>
       <c r="J14" t="n">
-        <v>3.89</v>
+        <v>3.886</v>
       </c>
       <c r="K14" t="n">
-        <v>4.073</v>
+        <v>4.011</v>
       </c>
       <c r="L14" t="n">
-        <v>4.092</v>
+        <v>4.045</v>
       </c>
       <c r="M14" t="n">
-        <v>4.224</v>
+        <v>4.171</v>
       </c>
       <c r="N14" t="n">
-        <v>4.291</v>
+        <v>4.217</v>
       </c>
       <c r="O14" t="n">
-        <v>4.473</v>
+        <v>4.394</v>
       </c>
       <c r="P14" t="n">
-        <v>4.547</v>
+        <v>4.464</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.771</v>
+        <v>4.697</v>
       </c>
       <c r="R14" t="n">
-        <v>4.93</v>
+        <v>4.868</v>
       </c>
       <c r="S14" t="n">
-        <v>5.115</v>
+        <v>5.064</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.867</v>
+        <v>2.871</v>
       </c>
       <c r="G15" t="n">
-        <v>3.057</v>
+        <v>3.068</v>
       </c>
       <c r="H15" t="n">
-        <v>3.323</v>
+        <v>3.338</v>
       </c>
       <c r="I15" t="n">
-        <v>3.57</v>
+        <v>3.567</v>
       </c>
       <c r="J15" t="n">
-        <v>3.828</v>
+        <v>3.825</v>
       </c>
       <c r="K15" t="n">
-        <v>4.025</v>
+        <v>3.963</v>
       </c>
       <c r="L15" t="n">
-        <v>4.028</v>
+        <v>3.982</v>
       </c>
       <c r="M15" t="n">
-        <v>4.137</v>
+        <v>4.084</v>
       </c>
       <c r="N15" t="n">
-        <v>4.195</v>
+        <v>4.121</v>
       </c>
       <c r="O15" t="n">
-        <v>4.415</v>
+        <v>4.336</v>
       </c>
       <c r="P15" t="n">
-        <v>4.444</v>
+        <v>4.36</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.673</v>
+        <v>4.599</v>
       </c>
       <c r="R15" t="n">
-        <v>4.825</v>
+        <v>4.763</v>
       </c>
       <c r="S15" t="n">
-        <v>5.01</v>
+        <v>4.959</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.867</v>
+        <v>2.871</v>
       </c>
       <c r="G16" t="n">
-        <v>3.057</v>
+        <v>3.068</v>
       </c>
       <c r="H16" t="n">
-        <v>3.323</v>
+        <v>3.338</v>
       </c>
       <c r="I16" t="n">
-        <v>3.57</v>
+        <v>3.567</v>
       </c>
       <c r="J16" t="n">
-        <v>3.828</v>
+        <v>3.825</v>
       </c>
       <c r="K16" t="n">
-        <v>4.025</v>
+        <v>3.963</v>
       </c>
       <c r="L16" t="n">
-        <v>4.028</v>
+        <v>3.982</v>
       </c>
       <c r="M16" t="n">
-        <v>4.137</v>
+        <v>4.084</v>
       </c>
       <c r="N16" t="n">
-        <v>4.198</v>
+        <v>4.124</v>
       </c>
       <c r="O16" t="n">
-        <v>4.422</v>
+        <v>4.343</v>
       </c>
       <c r="P16" t="n">
-        <v>4.467</v>
+        <v>4.384</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.7</v>
+        <v>4.626</v>
       </c>
       <c r="R16" t="n">
-        <v>4.853</v>
+        <v>4.79</v>
       </c>
       <c r="S16" t="n">
-        <v>5.039</v>
+        <v>4.988</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.731</v>
+        <v>2.735</v>
       </c>
       <c r="G17" t="n">
-        <v>2.893</v>
+        <v>2.897</v>
       </c>
       <c r="H17" t="n">
-        <v>3.112</v>
+        <v>3.122</v>
       </c>
       <c r="I17" t="n">
-        <v>3.375</v>
+        <v>3.381</v>
       </c>
       <c r="J17" t="n">
-        <v>3.651</v>
+        <v>3.63</v>
       </c>
       <c r="K17" t="n">
-        <v>3.942</v>
+        <v>3.873</v>
       </c>
       <c r="L17" t="n">
-        <v>3.997</v>
+        <v>3.932</v>
       </c>
       <c r="M17" t="n">
-        <v>4.147</v>
+        <v>4.077</v>
       </c>
       <c r="N17" t="n">
-        <v>4.218</v>
+        <v>4.132</v>
       </c>
       <c r="O17" t="n">
-        <v>4.42</v>
+        <v>4.34</v>
       </c>
       <c r="P17" t="n">
-        <v>4.513</v>
+        <v>4.429</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.732</v>
+        <v>2.736</v>
       </c>
       <c r="G18" t="n">
-        <v>2.894</v>
+        <v>2.898</v>
       </c>
       <c r="H18" t="n">
-        <v>3.113</v>
+        <v>3.123</v>
       </c>
       <c r="I18" t="n">
-        <v>3.376</v>
+        <v>3.382</v>
       </c>
       <c r="J18" t="n">
-        <v>3.651</v>
+        <v>3.63</v>
       </c>
       <c r="K18" t="n">
-        <v>3.943</v>
+        <v>3.874</v>
       </c>
       <c r="L18" t="n">
-        <v>3.997</v>
+        <v>3.932</v>
       </c>
       <c r="M18" t="n">
-        <v>4.147</v>
+        <v>4.077</v>
       </c>
       <c r="N18" t="n">
-        <v>4.218</v>
+        <v>4.132</v>
       </c>
       <c r="O18" t="n">
-        <v>4.418</v>
+        <v>4.338</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.878</v>
+        <v>2.882</v>
       </c>
       <c r="G19" t="n">
-        <v>3.071</v>
+        <v>3.082</v>
       </c>
       <c r="H19" t="n">
-        <v>3.338</v>
+        <v>3.354</v>
       </c>
       <c r="I19" t="n">
-        <v>3.602</v>
+        <v>3.599</v>
       </c>
       <c r="J19" t="n">
-        <v>3.87</v>
+        <v>3.866</v>
       </c>
       <c r="K19" t="n">
-        <v>4.068</v>
+        <v>4.006</v>
       </c>
       <c r="L19" t="n">
-        <v>4.089</v>
+        <v>4.043</v>
       </c>
       <c r="M19" t="n">
-        <v>4.215</v>
+        <v>4.162</v>
       </c>
       <c r="N19" t="n">
-        <v>4.281</v>
+        <v>4.206</v>
       </c>
       <c r="O19" t="n">
-        <v>4.459</v>
+        <v>4.379</v>
       </c>
       <c r="P19" t="n">
-        <v>4.505</v>
+        <v>4.422</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.71</v>
+        <v>4.637</v>
       </c>
       <c r="R19" t="n">
-        <v>4.872</v>
+        <v>4.81</v>
       </c>
       <c r="S19" t="n">
-        <v>5.05</v>
+        <v>4.999</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.659</v>
+        <v>2.66</v>
       </c>
       <c r="G20" t="n">
-        <v>2.771</v>
+        <v>2.772</v>
       </c>
       <c r="H20" t="n">
-        <v>2.9</v>
+        <v>2.897</v>
       </c>
       <c r="I20" t="n">
-        <v>3.114</v>
+        <v>3.08</v>
       </c>
       <c r="J20" t="n">
-        <v>3.581</v>
+        <v>3.543</v>
       </c>
       <c r="K20" t="n">
-        <v>3.887</v>
+        <v>3.804</v>
       </c>
       <c r="L20" t="n">
-        <v>3.881</v>
+        <v>3.809</v>
       </c>
       <c r="M20" t="n">
-        <v>3.974</v>
+        <v>3.905</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.98</v>
+        <v>2.987</v>
       </c>
       <c r="G21" t="n">
-        <v>3.187</v>
+        <v>3.204</v>
       </c>
       <c r="H21" t="n">
-        <v>3.465</v>
+        <v>3.485</v>
       </c>
       <c r="I21" t="n">
-        <v>3.723</v>
+        <v>3.73</v>
       </c>
       <c r="J21" t="n">
         <v>4.018</v>
       </c>
       <c r="K21" t="n">
-        <v>4.311</v>
+        <v>4.251</v>
       </c>
       <c r="L21" t="n">
-        <v>4.334</v>
+        <v>4.285</v>
       </c>
       <c r="M21" t="n">
-        <v>4.452</v>
+        <v>4.397</v>
       </c>
       <c r="N21" t="n">
-        <v>4.526</v>
+        <v>4.443</v>
       </c>
       <c r="O21" t="n">
-        <v>4.665</v>
+        <v>4.585</v>
       </c>
       <c r="P21" t="n">
-        <v>4.765</v>
+        <v>4.682</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.867</v>
+        <v>4.792</v>
       </c>
       <c r="R21" t="n">
-        <v>4.923</v>
+        <v>4.861</v>
       </c>
       <c r="S21" t="n">
-        <v>5.003</v>
+        <v>4.951</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.926</v>
+        <v>2.933</v>
       </c>
       <c r="G22" t="n">
-        <v>3.132</v>
+        <v>3.149</v>
       </c>
       <c r="H22" t="n">
-        <v>3.397</v>
+        <v>3.417</v>
       </c>
       <c r="I22" t="n">
-        <v>3.642</v>
+        <v>3.649</v>
       </c>
       <c r="J22" t="n">
         <v>3.903</v>
       </c>
       <c r="K22" t="n">
-        <v>4.193</v>
+        <v>4.133</v>
       </c>
       <c r="L22" t="n">
-        <v>4.201</v>
+        <v>4.152</v>
       </c>
       <c r="M22" t="n">
-        <v>4.324</v>
+        <v>4.269</v>
       </c>
       <c r="N22" t="n">
-        <v>4.4</v>
+        <v>4.317</v>
       </c>
       <c r="O22" t="n">
-        <v>4.536</v>
+        <v>4.456</v>
       </c>
       <c r="P22" t="n">
-        <v>4.628</v>
+        <v>4.545</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.725</v>
+        <v>4.651</v>
       </c>
       <c r="R22" t="n">
-        <v>4.772</v>
+        <v>4.709</v>
       </c>
       <c r="S22" t="n">
-        <v>4.848</v>
+        <v>4.797</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.876</v>
+        <v>2.881</v>
       </c>
       <c r="G23" t="n">
-        <v>3.086</v>
+        <v>3.103</v>
       </c>
       <c r="H23" t="n">
-        <v>3.338</v>
+        <v>3.358</v>
       </c>
       <c r="I23" t="n">
-        <v>3.59</v>
+        <v>3.597</v>
       </c>
       <c r="J23" t="n">
         <v>3.843</v>
       </c>
       <c r="K23" t="n">
-        <v>4.092</v>
+        <v>4.032</v>
       </c>
       <c r="L23" t="n">
-        <v>4.099</v>
+        <v>4.05</v>
       </c>
       <c r="M23" t="n">
-        <v>4.215</v>
+        <v>4.16</v>
       </c>
       <c r="N23" t="n">
-        <v>4.294</v>
+        <v>4.211</v>
       </c>
       <c r="O23" t="n">
-        <v>4.412</v>
+        <v>4.332</v>
       </c>
       <c r="P23" t="n">
+        <v>4.408</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>4.457</v>
+      </c>
+      <c r="R23" t="n">
+        <v>4.495</v>
+      </c>
+      <c r="S23" t="n">
+        <v>4.553</v>
+      </c>
+      <c r="T23" t="n">
         <v>4.491</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>4.531</v>
-      </c>
-      <c r="R23" t="n">
-        <v>4.558</v>
-      </c>
-      <c r="S23" t="n">
-        <v>4.604</v>
-      </c>
-      <c r="T23" t="n">
-        <v>4.536</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.814</v>
+        <v>2.819</v>
       </c>
       <c r="G24" t="n">
-        <v>2.997</v>
+        <v>3.014</v>
       </c>
       <c r="H24" t="n">
-        <v>3.231</v>
+        <v>3.251</v>
       </c>
       <c r="I24" t="n">
-        <v>3.528</v>
+        <v>3.535</v>
       </c>
       <c r="J24" t="n">
         <v>3.736</v>
       </c>
       <c r="K24" t="n">
-        <v>3.975</v>
+        <v>3.915</v>
       </c>
       <c r="L24" t="n">
-        <v>3.98</v>
+        <v>3.931</v>
       </c>
       <c r="M24" t="n">
-        <v>4.074</v>
+        <v>4.019</v>
       </c>
       <c r="N24" t="n">
-        <v>4.168</v>
+        <v>4.085</v>
       </c>
       <c r="O24" t="n">
-        <v>4.412</v>
+        <v>4.332</v>
       </c>
       <c r="P24" t="n">
-        <v>4.43</v>
+        <v>4.348</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.457</v>
+        <v>4.382</v>
       </c>
       <c r="R24" t="n">
-        <v>4.479</v>
+        <v>4.417</v>
       </c>
       <c r="S24" t="n">
-        <v>4.519</v>
+        <v>4.468</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.871</v>
+        <v>2.876</v>
       </c>
       <c r="G25" t="n">
-        <v>3.086</v>
+        <v>3.103</v>
       </c>
       <c r="H25" t="n">
-        <v>3.341</v>
+        <v>3.361</v>
       </c>
       <c r="I25" t="n">
-        <v>3.599</v>
+        <v>3.606</v>
       </c>
       <c r="J25" t="n">
         <v>3.858</v>
       </c>
       <c r="K25" t="n">
-        <v>4.124</v>
+        <v>4.064</v>
       </c>
       <c r="L25" t="n">
-        <v>4.129</v>
+        <v>4.081</v>
       </c>
       <c r="M25" t="n">
-        <v>4.246</v>
+        <v>4.191</v>
       </c>
       <c r="N25" t="n">
-        <v>4.321</v>
+        <v>4.238</v>
       </c>
       <c r="O25" t="n">
-        <v>4.441</v>
+        <v>4.361</v>
       </c>
       <c r="P25" t="n">
-        <v>4.513</v>
+        <v>4.43</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.564</v>
+        <v>4.49</v>
       </c>
       <c r="R25" t="n">
-        <v>4.581</v>
+        <v>4.519</v>
       </c>
       <c r="S25" t="n">
-        <v>4.628</v>
+        <v>4.576</v>
       </c>
       <c r="T25" t="n">
-        <v>4.554</v>
+        <v>4.509</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.171</v>
+        <v>3.192</v>
       </c>
       <c r="G26" t="n">
-        <v>3.387</v>
+        <v>3.41</v>
       </c>
       <c r="H26" t="n">
-        <v>3.743</v>
+        <v>3.762</v>
       </c>
       <c r="I26" t="n">
-        <v>4.037</v>
+        <v>4.024</v>
       </c>
       <c r="J26" t="n">
-        <v>4.464</v>
+        <v>4.442</v>
       </c>
       <c r="K26" t="n">
-        <v>4.933</v>
+        <v>4.868</v>
       </c>
       <c r="L26" t="n">
-        <v>5.008</v>
+        <v>4.954</v>
       </c>
       <c r="M26" t="n">
-        <v>5.164</v>
+        <v>5.106</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.498</v>
+        <v>5.419</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.978</v>
+        <v>2.989</v>
       </c>
       <c r="G27" t="n">
-        <v>3.148</v>
+        <v>3.166</v>
       </c>
       <c r="H27" t="n">
-        <v>3.423</v>
+        <v>3.442</v>
       </c>
       <c r="I27" t="n">
-        <v>3.69</v>
+        <v>3.684</v>
       </c>
       <c r="J27" t="n">
-        <v>3.989</v>
+        <v>3.98</v>
       </c>
       <c r="K27" t="n">
-        <v>4.25</v>
+        <v>4.187</v>
       </c>
       <c r="L27" t="n">
-        <v>4.274</v>
+        <v>4.224</v>
       </c>
       <c r="M27" t="n">
-        <v>4.384</v>
+        <v>4.329</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.601</v>
+        <v>4.522</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.081</v>
+        <v>3.092</v>
       </c>
       <c r="G28" t="n">
-        <v>3.259</v>
+        <v>3.277</v>
       </c>
       <c r="H28" t="n">
-        <v>3.548</v>
+        <v>3.568</v>
       </c>
       <c r="I28" t="n">
-        <v>3.827</v>
+        <v>3.821</v>
       </c>
       <c r="J28" t="n">
-        <v>4.162</v>
+        <v>4.153</v>
       </c>
       <c r="K28" t="n">
-        <v>4.442</v>
+        <v>4.379</v>
       </c>
       <c r="L28" t="n">
-        <v>4.477</v>
+        <v>4.427</v>
       </c>
       <c r="M28" t="n">
-        <v>4.596</v>
+        <v>4.541</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.894</v>
+        <v>4.814</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.927</v>
+        <v>2.938</v>
       </c>
       <c r="G29" t="n">
-        <v>3.096</v>
+        <v>3.112</v>
       </c>
       <c r="H29" t="n">
-        <v>3.362</v>
+        <v>3.379</v>
       </c>
       <c r="I29" t="n">
-        <v>3.617</v>
+        <v>3.609</v>
       </c>
       <c r="J29" t="n">
-        <v>3.901</v>
+        <v>3.892</v>
       </c>
       <c r="K29" t="n">
-        <v>4.145</v>
+        <v>4.082</v>
       </c>
       <c r="L29" t="n">
-        <v>4.159</v>
+        <v>4.109</v>
       </c>
       <c r="M29" t="n">
-        <v>4.247</v>
+        <v>4.192</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.473</v>
+        <v>4.393</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.212</v>
+        <v>3.232</v>
       </c>
       <c r="G30" t="n">
-        <v>3.361</v>
+        <v>3.383</v>
       </c>
       <c r="H30" t="n">
-        <v>3.676</v>
+        <v>3.694</v>
       </c>
       <c r="I30" t="n">
-        <v>3.963</v>
+        <v>3.949</v>
       </c>
       <c r="J30" t="n">
-        <v>4.327</v>
+        <v>4.304</v>
       </c>
       <c r="K30" t="n">
-        <v>4.733</v>
+        <v>4.67</v>
       </c>
       <c r="L30" t="n">
-        <v>4.784</v>
+        <v>4.732</v>
       </c>
       <c r="M30" t="n">
-        <v>4.931</v>
+        <v>4.872</v>
       </c>
       <c r="N30" t="n">
-        <v>5.109</v>
+        <v>5.028</v>
       </c>
       <c r="O30" t="n">
-        <v>5.45</v>
+        <v>5.37</v>
       </c>
       <c r="P30" t="n">
-        <v>5.658</v>
+        <v>5.574</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.404</v>
+        <v>6.331</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.541</v>
+        <v>3.561</v>
       </c>
       <c r="G31" t="n">
-        <v>3.726</v>
+        <v>3.748</v>
       </c>
       <c r="H31" t="n">
-        <v>4.092</v>
+        <v>4.11</v>
       </c>
       <c r="I31" t="n">
-        <v>4.392</v>
+        <v>4.378</v>
       </c>
       <c r="J31" t="n">
-        <v>4.818</v>
+        <v>4.795</v>
       </c>
       <c r="K31" t="n">
-        <v>5.266</v>
+        <v>5.203</v>
       </c>
       <c r="L31" t="n">
-        <v>5.397</v>
+        <v>5.344</v>
       </c>
       <c r="M31" t="n">
-        <v>5.662</v>
+        <v>5.603</v>
       </c>
       <c r="N31" t="n">
-        <v>5.968</v>
+        <v>5.887</v>
       </c>
       <c r="O31" t="n">
-        <v>6.486</v>
+        <v>6.406</v>
       </c>
       <c r="P31" t="n">
-        <v>6.646</v>
+        <v>6.563</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.378</v>
+        <v>7.304</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.311</v>
+        <v>3.331</v>
       </c>
       <c r="G32" t="n">
-        <v>3.478</v>
+        <v>3.5</v>
       </c>
       <c r="H32" t="n">
-        <v>3.82</v>
+        <v>3.838</v>
       </c>
       <c r="I32" t="n">
-        <v>4.122</v>
+        <v>4.108</v>
       </c>
       <c r="J32" t="n">
-        <v>4.505</v>
+        <v>4.482</v>
       </c>
       <c r="K32" t="n">
-        <v>4.918</v>
+        <v>4.855</v>
       </c>
       <c r="L32" t="n">
-        <v>4.989</v>
+        <v>4.936</v>
       </c>
       <c r="M32" t="n">
-        <v>5.204</v>
+        <v>5.145</v>
       </c>
       <c r="N32" t="n">
-        <v>5.47</v>
+        <v>5.389</v>
       </c>
       <c r="O32" t="n">
-        <v>5.895</v>
+        <v>5.815</v>
       </c>
       <c r="P32" t="n">
-        <v>6.118</v>
+        <v>6.034</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.865</v>
+        <v>6.792</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.077</v>
+        <v>3.097</v>
       </c>
       <c r="G33" t="n">
-        <v>3.226</v>
+        <v>3.248</v>
       </c>
       <c r="H33" t="n">
-        <v>3.494</v>
+        <v>3.512</v>
       </c>
       <c r="I33" t="n">
-        <v>3.748</v>
+        <v>3.734</v>
       </c>
       <c r="J33" t="n">
-        <v>4.034</v>
+        <v>4.011</v>
       </c>
       <c r="K33" t="n">
-        <v>4.374</v>
+        <v>4.31</v>
       </c>
       <c r="L33" t="n">
-        <v>4.39</v>
+        <v>4.337</v>
       </c>
       <c r="M33" t="n">
-        <v>4.458</v>
+        <v>4.401</v>
       </c>
       <c r="N33" t="n">
-        <v>4.498</v>
+        <v>4.417</v>
       </c>
       <c r="O33" t="n">
-        <v>4.604</v>
+        <v>4.524</v>
       </c>
       <c r="P33" t="n">
-        <v>4.69</v>
+        <v>4.607</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.121</v>
+        <v>5.048</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.137</v>
+        <v>3.157</v>
       </c>
       <c r="G34" t="n">
-        <v>3.279</v>
+        <v>3.301</v>
       </c>
       <c r="H34" t="n">
-        <v>3.556</v>
+        <v>3.574</v>
       </c>
       <c r="I34" t="n">
-        <v>3.816</v>
+        <v>3.802</v>
       </c>
       <c r="J34" t="n">
-        <v>4.106</v>
+        <v>4.083</v>
       </c>
       <c r="K34" t="n">
-        <v>4.45</v>
+        <v>4.386</v>
       </c>
       <c r="L34" t="n">
-        <v>4.469</v>
+        <v>4.416</v>
       </c>
       <c r="M34" t="n">
-        <v>4.548</v>
+        <v>4.491</v>
       </c>
       <c r="N34" t="n">
-        <v>4.603</v>
+        <v>4.522</v>
       </c>
       <c r="O34" t="n">
-        <v>4.773</v>
+        <v>4.693</v>
       </c>
       <c r="P34" t="n">
-        <v>4.985</v>
+        <v>4.901</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.822</v>
+        <v>5.749</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.111</v>
+        <v>3.131</v>
       </c>
       <c r="G35" t="n">
-        <v>3.253</v>
+        <v>3.275</v>
       </c>
       <c r="H35" t="n">
-        <v>3.524</v>
+        <v>3.542</v>
       </c>
       <c r="I35" t="n">
-        <v>3.782</v>
+        <v>3.768</v>
       </c>
       <c r="J35" t="n">
-        <v>4.074</v>
+        <v>4.051</v>
       </c>
       <c r="K35" t="n">
-        <v>4.404</v>
+        <v>4.34</v>
       </c>
       <c r="L35" t="n">
-        <v>4.424</v>
+        <v>4.371</v>
       </c>
       <c r="M35" t="n">
-        <v>4.495</v>
+        <v>4.438</v>
       </c>
       <c r="N35" t="n">
-        <v>4.539</v>
+        <v>4.458</v>
       </c>
       <c r="O35" t="n">
-        <v>4.67</v>
+        <v>4.59</v>
       </c>
       <c r="P35" t="n">
-        <v>4.787</v>
+        <v>4.704</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.458</v>
+        <v>5.384</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.001</v>
+        <v>3.021</v>
       </c>
       <c r="G36" t="n">
-        <v>3.139</v>
+        <v>3.159</v>
       </c>
       <c r="H36" t="n">
-        <v>3.403</v>
+        <v>3.418</v>
       </c>
       <c r="I36" t="n">
-        <v>3.66</v>
+        <v>3.644</v>
       </c>
       <c r="J36" t="n">
-        <v>3.971</v>
+        <v>3.946</v>
       </c>
       <c r="K36" t="n">
-        <v>4.3</v>
+        <v>4.234</v>
       </c>
       <c r="L36" t="n">
-        <v>4.313</v>
+        <v>4.258</v>
       </c>
       <c r="M36" t="n">
-        <v>4.361</v>
+        <v>4.302</v>
       </c>
       <c r="N36" t="n">
-        <v>4.403</v>
+        <v>4.322</v>
       </c>
       <c r="O36" t="n">
-        <v>4.512</v>
+        <v>4.432</v>
       </c>
       <c r="P36" t="n">
-        <v>4.588</v>
+        <v>4.505</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.838</v>
+        <v>4.765</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.884</v>
+        <v>3.904</v>
       </c>
       <c r="G37" t="n">
-        <v>4.42</v>
+        <v>4.442</v>
       </c>
       <c r="H37" t="n">
-        <v>5.064</v>
+        <v>5.082</v>
       </c>
       <c r="I37" t="n">
-        <v>5.453</v>
+        <v>5.439</v>
       </c>
       <c r="J37" t="n">
-        <v>6.308</v>
+        <v>6.285</v>
       </c>
       <c r="K37" t="n">
-        <v>7.305</v>
+        <v>7.242</v>
       </c>
       <c r="L37" t="n">
-        <v>7.598</v>
+        <v>7.545</v>
       </c>
       <c r="M37" t="n">
-        <v>7.934</v>
+        <v>7.875</v>
       </c>
       <c r="N37" t="n">
-        <v>8.122999999999999</v>
+        <v>8.042</v>
       </c>
       <c r="O37" t="n">
-        <v>8.365</v>
+        <v>8.285</v>
       </c>
       <c r="P37" t="n">
-        <v>8.448</v>
+        <v>8.364000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.868</v>
+        <v>8.795</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.946</v>
+        <v>4.966</v>
       </c>
       <c r="G38" t="n">
-        <v>5.735</v>
+        <v>5.757</v>
       </c>
       <c r="H38" t="n">
-        <v>6.591</v>
+        <v>6.609</v>
       </c>
       <c r="I38" t="n">
-        <v>7.137</v>
+        <v>7.123</v>
       </c>
       <c r="J38" t="n">
-        <v>8.252000000000001</v>
+        <v>8.228999999999999</v>
       </c>
       <c r="K38" t="n">
-        <v>9.428000000000001</v>
+        <v>9.365</v>
       </c>
       <c r="L38" t="n">
-        <v>9.880000000000001</v>
+        <v>9.827999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.346</v>
+        <v>10.287</v>
       </c>
       <c r="N38" t="n">
-        <v>10.542</v>
+        <v>10.461</v>
       </c>
       <c r="O38" t="n">
-        <v>10.765</v>
+        <v>10.685</v>
       </c>
       <c r="P38" t="n">
-        <v>10.846</v>
+        <v>10.762</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.318</v>
+        <v>11.245</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.266</v>
+        <v>4.286</v>
       </c>
       <c r="G39" t="n">
-        <v>4.933</v>
+        <v>4.955</v>
       </c>
       <c r="H39" t="n">
-        <v>5.656</v>
+        <v>5.674</v>
       </c>
       <c r="I39" t="n">
-        <v>6.141</v>
+        <v>6.127</v>
       </c>
       <c r="J39" t="n">
-        <v>7.124</v>
+        <v>7.101</v>
       </c>
       <c r="K39" t="n">
-        <v>8.260999999999999</v>
+        <v>8.198</v>
       </c>
       <c r="L39" t="n">
-        <v>8.635999999999999</v>
+        <v>8.583</v>
       </c>
       <c r="M39" t="n">
-        <v>8.981999999999999</v>
+        <v>8.923</v>
       </c>
       <c r="N39" t="n">
-        <v>9.17</v>
+        <v>9.089</v>
       </c>
       <c r="O39" t="n">
-        <v>9.416</v>
+        <v>9.336</v>
       </c>
       <c r="P39" t="n">
-        <v>9.5</v>
+        <v>9.417</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.964</v>
+        <v>9.891</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.404</v>
+        <v>3.424</v>
       </c>
       <c r="G40" t="n">
-        <v>3.599</v>
+        <v>3.621</v>
       </c>
       <c r="H40" t="n">
-        <v>3.935</v>
+        <v>3.953</v>
       </c>
       <c r="I40" t="n">
-        <v>4.236</v>
+        <v>4.222</v>
       </c>
       <c r="J40" t="n">
-        <v>4.619</v>
+        <v>4.596</v>
       </c>
       <c r="K40" t="n">
-        <v>5.039</v>
+        <v>4.976</v>
       </c>
       <c r="L40" t="n">
-        <v>5.109</v>
+        <v>5.056</v>
       </c>
       <c r="M40" t="n">
-        <v>5.274</v>
+        <v>5.215</v>
       </c>
       <c r="N40" t="n">
-        <v>5.467</v>
+        <v>5.386</v>
       </c>
       <c r="O40" t="n">
-        <v>5.829</v>
+        <v>5.749</v>
       </c>
       <c r="P40" t="n">
-        <v>6.079</v>
+        <v>5.996</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.855</v>
+        <v>6.782</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.79</v>
+        <v>3.81</v>
       </c>
       <c r="G41" t="n">
-        <v>4.028</v>
+        <v>4.05</v>
       </c>
       <c r="H41" t="n">
-        <v>4.421</v>
+        <v>4.439</v>
       </c>
       <c r="I41" t="n">
-        <v>4.74</v>
+        <v>4.726</v>
       </c>
       <c r="J41" t="n">
-        <v>5.174</v>
+        <v>5.151</v>
       </c>
       <c r="K41" t="n">
-        <v>5.639</v>
+        <v>5.576</v>
       </c>
       <c r="L41" t="n">
-        <v>5.788</v>
+        <v>5.735</v>
       </c>
       <c r="M41" t="n">
-        <v>6.077</v>
+        <v>6.018</v>
       </c>
       <c r="N41" t="n">
-        <v>6.397</v>
+        <v>6.317</v>
       </c>
       <c r="O41" t="n">
-        <v>6.944</v>
+        <v>6.864</v>
       </c>
       <c r="P41" t="n">
-        <v>7.139</v>
+        <v>7.055</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.902</v>
+        <v>7.829</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.525</v>
+        <v>3.545</v>
       </c>
       <c r="G42" t="n">
-        <v>3.748</v>
+        <v>3.77</v>
       </c>
       <c r="H42" t="n">
-        <v>4.111</v>
+        <v>4.129</v>
       </c>
       <c r="I42" t="n">
-        <v>4.425</v>
+        <v>4.411</v>
       </c>
       <c r="J42" t="n">
-        <v>4.821</v>
+        <v>4.798</v>
       </c>
       <c r="K42" t="n">
-        <v>5.26</v>
+        <v>5.197</v>
       </c>
       <c r="L42" t="n">
-        <v>5.345</v>
+        <v>5.293</v>
       </c>
       <c r="M42" t="n">
-        <v>5.581</v>
+        <v>5.522</v>
       </c>
       <c r="N42" t="n">
-        <v>5.881</v>
+        <v>5.8</v>
       </c>
       <c r="O42" t="n">
-        <v>6.321</v>
+        <v>6.241</v>
       </c>
       <c r="P42" t="n">
-        <v>6.581</v>
+        <v>6.498</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.368</v>
+        <v>7.294</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.225</v>
+        <v>3.245</v>
       </c>
       <c r="G43" t="n">
-        <v>3.408</v>
+        <v>3.43</v>
       </c>
       <c r="H43" t="n">
-        <v>3.695</v>
+        <v>3.713</v>
       </c>
       <c r="I43" t="n">
-        <v>3.956</v>
+        <v>3.942</v>
       </c>
       <c r="J43" t="n">
-        <v>4.262</v>
+        <v>4.239</v>
       </c>
       <c r="K43" t="n">
-        <v>4.606</v>
+        <v>4.542</v>
       </c>
       <c r="L43" t="n">
-        <v>4.631</v>
+        <v>4.579</v>
       </c>
       <c r="M43" t="n">
-        <v>4.713</v>
+        <v>4.656</v>
       </c>
       <c r="N43" t="n">
-        <v>4.767</v>
+        <v>4.686</v>
       </c>
       <c r="O43" t="n">
-        <v>4.917</v>
+        <v>4.837</v>
       </c>
       <c r="P43" t="n">
-        <v>5.056</v>
+        <v>4.972</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.731</v>
+        <v>5.658</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.079</v>
+        <v>3.099</v>
       </c>
       <c r="G44" t="n">
-        <v>3.249</v>
+        <v>3.269</v>
       </c>
       <c r="H44" t="n">
-        <v>3.526</v>
+        <v>3.542</v>
       </c>
       <c r="I44" t="n">
-        <v>3.787</v>
+        <v>3.771</v>
       </c>
       <c r="J44" t="n">
-        <v>4.112</v>
+        <v>4.087</v>
       </c>
       <c r="K44" t="n">
-        <v>4.452</v>
+        <v>4.386</v>
       </c>
       <c r="L44" t="n">
-        <v>4.474</v>
+        <v>4.419</v>
       </c>
       <c r="M44" t="n">
-        <v>4.531</v>
+        <v>4.472</v>
       </c>
       <c r="N44" t="n">
-        <v>4.584</v>
+        <v>4.503</v>
       </c>
       <c r="O44" t="n">
-        <v>4.713</v>
+        <v>4.633</v>
       </c>
       <c r="P44" t="n">
-        <v>4.818</v>
+        <v>4.735</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.102</v>
+        <v>5.028</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-10 ~ 2026-06-10
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.376</v>
+        <v>3.401</v>
       </c>
       <c r="G2" t="n">
-        <v>3.688</v>
+        <v>3.713</v>
       </c>
       <c r="H2" t="n">
-        <v>3.988</v>
+        <v>4.007</v>
       </c>
       <c r="I2" t="n">
-        <v>4.196</v>
+        <v>4.195</v>
       </c>
       <c r="J2" t="n">
-        <v>4.505</v>
+        <v>4.511</v>
       </c>
       <c r="K2" t="n">
-        <v>4.897</v>
+        <v>4.895</v>
       </c>
       <c r="L2" t="n">
-        <v>5.067</v>
+        <v>5.06</v>
       </c>
       <c r="M2" t="n">
-        <v>5.324</v>
+        <v>5.312</v>
       </c>
       <c r="N2" t="n">
-        <v>5.59</v>
+        <v>5.577</v>
       </c>
       <c r="O2" t="n">
-        <v>5.884</v>
+        <v>5.859</v>
       </c>
       <c r="P2" t="n">
-        <v>6.095</v>
+        <v>6.076</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.732</v>
+        <v>6.722</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.398</v>
+        <v>4.423</v>
       </c>
       <c r="G3" t="n">
-        <v>4.891</v>
+        <v>4.915</v>
       </c>
       <c r="H3" t="n">
-        <v>5.223</v>
+        <v>5.243</v>
       </c>
       <c r="I3" t="n">
-        <v>5.425</v>
+        <v>5.423</v>
       </c>
       <c r="J3" t="n">
-        <v>5.751</v>
+        <v>5.756</v>
       </c>
       <c r="K3" t="n">
-        <v>6.213</v>
+        <v>6.211</v>
       </c>
       <c r="L3" t="n">
-        <v>6.453</v>
+        <v>6.445</v>
       </c>
       <c r="M3" t="n">
-        <v>6.74</v>
+        <v>6.729</v>
       </c>
       <c r="N3" t="n">
-        <v>6.949</v>
+        <v>6.936</v>
       </c>
       <c r="O3" t="n">
-        <v>7.194</v>
+        <v>7.169</v>
       </c>
       <c r="P3" t="n">
-        <v>7.273</v>
+        <v>7.255</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.798</v>
+        <v>7.788</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.89</v>
+        <v>3.915</v>
       </c>
       <c r="G4" t="n">
-        <v>4.272</v>
+        <v>4.297</v>
       </c>
       <c r="H4" t="n">
-        <v>4.633</v>
+        <v>4.652</v>
       </c>
       <c r="I4" t="n">
-        <v>4.867</v>
+        <v>4.866</v>
       </c>
       <c r="J4" t="n">
-        <v>5.194</v>
+        <v>5.2</v>
       </c>
       <c r="K4" t="n">
-        <v>5.652</v>
+        <v>5.65</v>
       </c>
       <c r="L4" t="n">
-        <v>5.822</v>
+        <v>5.814</v>
       </c>
       <c r="M4" t="n">
-        <v>6.098</v>
+        <v>6.086</v>
       </c>
       <c r="N4" t="n">
-        <v>6.277</v>
+        <v>6.264</v>
       </c>
       <c r="O4" t="n">
-        <v>6.545</v>
+        <v>6.52</v>
       </c>
       <c r="P4" t="n">
-        <v>6.626</v>
+        <v>6.607</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.153</v>
+        <v>7.143</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.074</v>
+        <v>3.099</v>
       </c>
       <c r="G5" t="n">
-        <v>3.231</v>
+        <v>3.256</v>
       </c>
       <c r="H5" t="n">
-        <v>3.495</v>
+        <v>3.514</v>
       </c>
       <c r="I5" t="n">
-        <v>3.768</v>
+        <v>3.767</v>
       </c>
       <c r="J5" t="n">
-        <v>4.064</v>
+        <v>4.068</v>
       </c>
       <c r="K5" t="n">
-        <v>4.302</v>
+        <v>4.299</v>
       </c>
       <c r="L5" t="n">
-        <v>4.316</v>
+        <v>4.307</v>
       </c>
       <c r="M5" t="n">
-        <v>4.383</v>
+        <v>4.37</v>
       </c>
       <c r="N5" t="n">
-        <v>4.402</v>
+        <v>4.389</v>
       </c>
       <c r="O5" t="n">
-        <v>4.484</v>
+        <v>4.459</v>
       </c>
       <c r="P5" t="n">
-        <v>4.764</v>
+        <v>4.745</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.644</v>
+        <v>5.634</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.115</v>
+        <v>3.14</v>
       </c>
       <c r="G6" t="n">
-        <v>3.286</v>
+        <v>3.311</v>
       </c>
       <c r="H6" t="n">
-        <v>3.564</v>
+        <v>3.584</v>
       </c>
       <c r="I6" t="n">
-        <v>3.851</v>
+        <v>3.85</v>
       </c>
       <c r="J6" t="n">
-        <v>4.154</v>
+        <v>4.159</v>
       </c>
       <c r="K6" t="n">
-        <v>4.414</v>
+        <v>4.412</v>
       </c>
       <c r="L6" t="n">
-        <v>4.434</v>
+        <v>4.426</v>
       </c>
       <c r="M6" t="n">
-        <v>4.538</v>
+        <v>4.526</v>
       </c>
       <c r="N6" t="n">
-        <v>4.57</v>
+        <v>4.556</v>
       </c>
       <c r="O6" t="n">
-        <v>4.75</v>
+        <v>4.725</v>
       </c>
       <c r="P6" t="n">
-        <v>5.196</v>
+        <v>5.177</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.04</v>
+        <v>6.03</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.095</v>
+        <v>3.12</v>
       </c>
       <c r="G7" t="n">
-        <v>3.25</v>
+        <v>3.275</v>
       </c>
       <c r="H7" t="n">
-        <v>3.511</v>
+        <v>3.53</v>
       </c>
       <c r="I7" t="n">
-        <v>3.788</v>
+        <v>3.787</v>
       </c>
       <c r="J7" t="n">
-        <v>4.088</v>
+        <v>4.092</v>
       </c>
       <c r="K7" t="n">
-        <v>4.329</v>
+        <v>4.326</v>
       </c>
       <c r="L7" t="n">
-        <v>4.343</v>
+        <v>4.334</v>
       </c>
       <c r="M7" t="n">
-        <v>4.443</v>
+        <v>4.43</v>
       </c>
       <c r="N7" t="n">
-        <v>4.462</v>
+        <v>4.448</v>
       </c>
       <c r="O7" t="n">
-        <v>4.647</v>
+        <v>4.622</v>
       </c>
       <c r="P7" t="n">
-        <v>4.98</v>
+        <v>4.961</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.808</v>
+        <v>5.798</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.51</v>
+        <v>5.534</v>
       </c>
       <c r="G8" t="n">
-        <v>6.19</v>
+        <v>6.215</v>
       </c>
       <c r="H8" t="n">
-        <v>6.672</v>
+        <v>6.691</v>
       </c>
       <c r="I8" t="n">
-        <v>6.951</v>
+        <v>6.95</v>
       </c>
       <c r="J8" t="n">
-        <v>7.343</v>
+        <v>7.349</v>
       </c>
       <c r="K8" t="n">
-        <v>8.087</v>
+        <v>8.085000000000001</v>
       </c>
       <c r="L8" t="n">
-        <v>8.411</v>
+        <v>8.403</v>
       </c>
       <c r="M8" t="n">
-        <v>8.731</v>
+        <v>8.718999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.874000000000001</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.204000000000001</v>
+        <v>9.179</v>
       </c>
       <c r="P8" t="n">
-        <v>9.387</v>
+        <v>9.368</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.11</v>
+        <v>10.099</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.652</v>
+        <v>2.752</v>
       </c>
       <c r="G9" t="n">
-        <v>2.769</v>
+        <v>2.988</v>
       </c>
       <c r="H9" t="n">
-        <v>3.007</v>
+        <v>3.254</v>
       </c>
       <c r="I9" t="n">
-        <v>3.286</v>
+        <v>3.403</v>
       </c>
       <c r="J9" t="n">
-        <v>3.522</v>
+        <v>3.598</v>
       </c>
       <c r="K9" t="n">
-        <v>3.759</v>
+        <v>3.733</v>
       </c>
       <c r="L9" t="n">
-        <v>3.795</v>
+        <v>3.829</v>
       </c>
       <c r="M9" t="n">
-        <v>3.86</v>
+        <v>3.877</v>
       </c>
       <c r="N9" t="n">
-        <v>4.004</v>
+        <v>3.985</v>
       </c>
       <c r="O9" t="n">
-        <v>4.1</v>
+        <v>4.07</v>
       </c>
       <c r="P9" t="n">
-        <v>4.198</v>
+        <v>4.191</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.272</v>
+        <v>4.265</v>
       </c>
       <c r="R9" t="n">
-        <v>4.313</v>
+        <v>4.315</v>
       </c>
       <c r="S9" t="n">
-        <v>4.345</v>
+        <v>4.36</v>
       </c>
       <c r="T9" t="n">
-        <v>4.285</v>
+        <v>4.31</v>
       </c>
       <c r="U9" t="n">
-        <v>4.22</v>
+        <v>4.259</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.686</v>
+        <v>2.761</v>
       </c>
       <c r="G10" t="n">
-        <v>2.818</v>
+        <v>3.001</v>
       </c>
       <c r="H10" t="n">
-        <v>3.03</v>
+        <v>3.259</v>
       </c>
       <c r="I10" t="n">
-        <v>3.3</v>
+        <v>3.406</v>
       </c>
       <c r="J10" t="n">
-        <v>3.56</v>
+        <v>3.613</v>
       </c>
       <c r="K10" t="n">
-        <v>3.795</v>
+        <v>3.768</v>
       </c>
       <c r="L10" t="n">
-        <v>3.848</v>
+        <v>3.844</v>
       </c>
       <c r="M10" t="n">
-        <v>3.954</v>
+        <v>3.943</v>
       </c>
       <c r="N10" t="n">
-        <v>4.029</v>
+        <v>4.009</v>
       </c>
       <c r="O10" t="n">
-        <v>4.32</v>
+        <v>4.29</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.49</v>
+        <v>2.565</v>
       </c>
       <c r="G11" t="n">
-        <v>2.618</v>
+        <v>2.805</v>
       </c>
       <c r="H11" t="n">
-        <v>2.853</v>
+        <v>3.084</v>
       </c>
       <c r="I11" t="n">
-        <v>3.104</v>
+        <v>3.21</v>
       </c>
       <c r="J11" t="n">
-        <v>3.352</v>
+        <v>3.405</v>
       </c>
       <c r="K11" t="n">
-        <v>3.581</v>
+        <v>3.555</v>
       </c>
       <c r="L11" t="n">
-        <v>3.645</v>
+        <v>3.641</v>
       </c>
       <c r="M11" t="n">
-        <v>3.762</v>
+        <v>3.751</v>
       </c>
       <c r="N11" t="n">
-        <v>3.836</v>
+        <v>3.816</v>
       </c>
       <c r="O11" t="n">
-        <v>4.086</v>
+        <v>4.056</v>
       </c>
       <c r="P11" t="n">
-        <v>4.148</v>
+        <v>4.137</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.471</v>
+        <v>4.463</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.322</v>
+        <v>3.345</v>
       </c>
       <c r="G12" t="n">
-        <v>3.598</v>
+        <v>3.622</v>
       </c>
       <c r="H12" t="n">
-        <v>3.897</v>
+        <v>3.917</v>
       </c>
       <c r="I12" t="n">
-        <v>4.184</v>
+        <v>4.18</v>
       </c>
       <c r="J12" t="n">
-        <v>4.508</v>
+        <v>4.509</v>
       </c>
       <c r="K12" t="n">
-        <v>4.69</v>
+        <v>4.688</v>
       </c>
       <c r="L12" t="n">
-        <v>4.733</v>
+        <v>4.718</v>
       </c>
       <c r="M12" t="n">
-        <v>4.857</v>
+        <v>4.845</v>
       </c>
       <c r="N12" t="n">
-        <v>4.909</v>
+        <v>4.901</v>
       </c>
       <c r="O12" t="n">
-        <v>5.107</v>
+        <v>5.079</v>
       </c>
       <c r="P12" t="n">
-        <v>5.237</v>
+        <v>5.218</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.587</v>
+        <v>5.577</v>
       </c>
       <c r="R12" t="n">
-        <v>5.804</v>
+        <v>5.806</v>
       </c>
       <c r="S12" t="n">
-        <v>6.048</v>
+        <v>6.064</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.076</v>
+        <v>3.099</v>
       </c>
       <c r="G13" t="n">
-        <v>3.288</v>
+        <v>3.312</v>
       </c>
       <c r="H13" t="n">
-        <v>3.564</v>
+        <v>3.584</v>
       </c>
       <c r="I13" t="n">
-        <v>3.832</v>
+        <v>3.828</v>
       </c>
       <c r="J13" t="n">
-        <v>4.145</v>
+        <v>4.146</v>
       </c>
       <c r="K13" t="n">
-        <v>4.323</v>
+        <v>4.321</v>
       </c>
       <c r="L13" t="n">
-        <v>4.372</v>
+        <v>4.358</v>
       </c>
       <c r="M13" t="n">
-        <v>4.485</v>
+        <v>4.473</v>
       </c>
       <c r="N13" t="n">
-        <v>4.538</v>
+        <v>4.529</v>
       </c>
       <c r="O13" t="n">
-        <v>4.735</v>
+        <v>4.707</v>
       </c>
       <c r="P13" t="n">
-        <v>4.828</v>
+        <v>4.809</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.108</v>
+        <v>5.098</v>
       </c>
       <c r="R13" t="n">
-        <v>5.354</v>
+        <v>5.355</v>
       </c>
       <c r="S13" t="n">
-        <v>5.611</v>
+        <v>5.626</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.893</v>
+        <v>2.916</v>
       </c>
       <c r="G14" t="n">
-        <v>3.094</v>
+        <v>3.118</v>
       </c>
       <c r="H14" t="n">
-        <v>3.367</v>
+        <v>3.387</v>
       </c>
       <c r="I14" t="n">
-        <v>3.616</v>
+        <v>3.612</v>
       </c>
       <c r="J14" t="n">
-        <v>3.886</v>
+        <v>3.888</v>
       </c>
       <c r="K14" t="n">
-        <v>4.011</v>
+        <v>4.009</v>
       </c>
       <c r="L14" t="n">
-        <v>4.045</v>
+        <v>4.031</v>
       </c>
       <c r="M14" t="n">
-        <v>4.171</v>
+        <v>4.159</v>
       </c>
       <c r="N14" t="n">
-        <v>4.217</v>
+        <v>4.208</v>
       </c>
       <c r="O14" t="n">
-        <v>4.394</v>
+        <v>4.366</v>
       </c>
       <c r="P14" t="n">
-        <v>4.464</v>
+        <v>4.445</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.697</v>
+        <v>4.687</v>
       </c>
       <c r="R14" t="n">
-        <v>4.868</v>
+        <v>4.87</v>
       </c>
       <c r="S14" t="n">
-        <v>5.064</v>
+        <v>5.079</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.871</v>
+        <v>2.894</v>
       </c>
       <c r="G15" t="n">
-        <v>3.068</v>
+        <v>3.092</v>
       </c>
       <c r="H15" t="n">
-        <v>3.338</v>
+        <v>3.358</v>
       </c>
       <c r="I15" t="n">
-        <v>3.567</v>
+        <v>3.563</v>
       </c>
       <c r="J15" t="n">
         <v>3.825</v>
       </c>
       <c r="K15" t="n">
-        <v>3.963</v>
+        <v>3.961</v>
       </c>
       <c r="L15" t="n">
-        <v>3.982</v>
+        <v>3.967</v>
       </c>
       <c r="M15" t="n">
-        <v>4.084</v>
+        <v>4.072</v>
       </c>
       <c r="N15" t="n">
-        <v>4.121</v>
+        <v>4.111</v>
       </c>
       <c r="O15" t="n">
-        <v>4.336</v>
+        <v>4.308</v>
       </c>
       <c r="P15" t="n">
-        <v>4.36</v>
+        <v>4.341</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.599</v>
+        <v>4.589</v>
       </c>
       <c r="R15" t="n">
-        <v>4.763</v>
+        <v>4.764</v>
       </c>
       <c r="S15" t="n">
-        <v>4.959</v>
+        <v>4.974</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.871</v>
+        <v>2.894</v>
       </c>
       <c r="G16" t="n">
-        <v>3.068</v>
+        <v>3.092</v>
       </c>
       <c r="H16" t="n">
-        <v>3.338</v>
+        <v>3.358</v>
       </c>
       <c r="I16" t="n">
-        <v>3.567</v>
+        <v>3.563</v>
       </c>
       <c r="J16" t="n">
         <v>3.825</v>
       </c>
       <c r="K16" t="n">
-        <v>3.963</v>
+        <v>3.961</v>
       </c>
       <c r="L16" t="n">
-        <v>3.982</v>
+        <v>3.967</v>
       </c>
       <c r="M16" t="n">
-        <v>4.084</v>
+        <v>4.072</v>
       </c>
       <c r="N16" t="n">
-        <v>4.124</v>
+        <v>4.114</v>
       </c>
       <c r="O16" t="n">
-        <v>4.343</v>
+        <v>4.315</v>
       </c>
       <c r="P16" t="n">
-        <v>4.384</v>
+        <v>4.365</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.626</v>
+        <v>4.616</v>
       </c>
       <c r="R16" t="n">
-        <v>4.79</v>
+        <v>4.792</v>
       </c>
       <c r="S16" t="n">
-        <v>4.988</v>
+        <v>5.003</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.735</v>
+        <v>2.796</v>
       </c>
       <c r="G17" t="n">
-        <v>2.897</v>
+        <v>3.059</v>
       </c>
       <c r="H17" t="n">
-        <v>3.122</v>
+        <v>3.32</v>
       </c>
       <c r="I17" t="n">
-        <v>3.381</v>
+        <v>3.464</v>
       </c>
       <c r="J17" t="n">
-        <v>3.63</v>
+        <v>3.677</v>
       </c>
       <c r="K17" t="n">
-        <v>3.873</v>
+        <v>3.847</v>
       </c>
       <c r="L17" t="n">
-        <v>3.932</v>
+        <v>3.927</v>
       </c>
       <c r="M17" t="n">
-        <v>4.077</v>
+        <v>4.066</v>
       </c>
       <c r="N17" t="n">
-        <v>4.132</v>
+        <v>4.112</v>
       </c>
       <c r="O17" t="n">
-        <v>4.34</v>
+        <v>4.309</v>
       </c>
       <c r="P17" t="n">
-        <v>4.429</v>
+        <v>4.418</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.736</v>
+        <v>2.796</v>
       </c>
       <c r="G18" t="n">
-        <v>2.898</v>
+        <v>3.06</v>
       </c>
       <c r="H18" t="n">
-        <v>3.123</v>
+        <v>3.32</v>
       </c>
       <c r="I18" t="n">
-        <v>3.382</v>
+        <v>3.465</v>
       </c>
       <c r="J18" t="n">
-        <v>3.63</v>
+        <v>3.677</v>
       </c>
       <c r="K18" t="n">
-        <v>3.874</v>
+        <v>3.848</v>
       </c>
       <c r="L18" t="n">
-        <v>3.932</v>
+        <v>3.927</v>
       </c>
       <c r="M18" t="n">
-        <v>4.077</v>
+        <v>4.066</v>
       </c>
       <c r="N18" t="n">
-        <v>4.132</v>
+        <v>4.113</v>
       </c>
       <c r="O18" t="n">
-        <v>4.338</v>
+        <v>4.307</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.882</v>
+        <v>2.905</v>
       </c>
       <c r="G19" t="n">
-        <v>3.082</v>
+        <v>3.106</v>
       </c>
       <c r="H19" t="n">
-        <v>3.354</v>
+        <v>3.374</v>
       </c>
       <c r="I19" t="n">
-        <v>3.599</v>
+        <v>3.596</v>
       </c>
       <c r="J19" t="n">
-        <v>3.866</v>
+        <v>3.867</v>
       </c>
       <c r="K19" t="n">
-        <v>4.006</v>
+        <v>4.004</v>
       </c>
       <c r="L19" t="n">
-        <v>4.043</v>
+        <v>4.028</v>
       </c>
       <c r="M19" t="n">
-        <v>4.162</v>
+        <v>4.15</v>
       </c>
       <c r="N19" t="n">
-        <v>4.206</v>
+        <v>4.197</v>
       </c>
       <c r="O19" t="n">
-        <v>4.379</v>
+        <v>4.351</v>
       </c>
       <c r="P19" t="n">
-        <v>4.422</v>
+        <v>4.403</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.637</v>
+        <v>4.627</v>
       </c>
       <c r="R19" t="n">
-        <v>4.81</v>
+        <v>4.811</v>
       </c>
       <c r="S19" t="n">
-        <v>4.999</v>
+        <v>5.014</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.66</v>
       </c>
       <c r="G20" t="n">
-        <v>2.772</v>
+        <v>2.771</v>
       </c>
       <c r="H20" t="n">
-        <v>2.897</v>
+        <v>2.891</v>
       </c>
       <c r="I20" t="n">
-        <v>3.08</v>
+        <v>3.053</v>
       </c>
       <c r="J20" t="n">
-        <v>3.543</v>
+        <v>3.532</v>
       </c>
       <c r="K20" t="n">
-        <v>3.804</v>
+        <v>3.785</v>
       </c>
       <c r="L20" t="n">
-        <v>3.809</v>
+        <v>3.786</v>
       </c>
       <c r="M20" t="n">
-        <v>3.905</v>
+        <v>3.88</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.987</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>3.204</v>
+        <v>3.22</v>
       </c>
       <c r="H21" t="n">
-        <v>3.485</v>
+        <v>3.501</v>
       </c>
       <c r="I21" t="n">
-        <v>3.73</v>
+        <v>3.725</v>
       </c>
       <c r="J21" t="n">
-        <v>4.018</v>
+        <v>4.022</v>
       </c>
       <c r="K21" t="n">
-        <v>4.251</v>
+        <v>4.247</v>
       </c>
       <c r="L21" t="n">
-        <v>4.285</v>
+        <v>4.275</v>
       </c>
       <c r="M21" t="n">
-        <v>4.397</v>
+        <v>4.387</v>
       </c>
       <c r="N21" t="n">
-        <v>4.443</v>
+        <v>4.43</v>
       </c>
       <c r="O21" t="n">
-        <v>4.585</v>
+        <v>4.557</v>
       </c>
       <c r="P21" t="n">
-        <v>4.682</v>
+        <v>4.663</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.792</v>
+        <v>4.783</v>
       </c>
       <c r="R21" t="n">
-        <v>4.861</v>
+        <v>4.862</v>
       </c>
       <c r="S21" t="n">
-        <v>4.951</v>
+        <v>4.966</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.933</v>
+        <v>2.946</v>
       </c>
       <c r="G22" t="n">
-        <v>3.149</v>
+        <v>3.165</v>
       </c>
       <c r="H22" t="n">
-        <v>3.417</v>
+        <v>3.433</v>
       </c>
       <c r="I22" t="n">
-        <v>3.649</v>
+        <v>3.643</v>
       </c>
       <c r="J22" t="n">
-        <v>3.903</v>
+        <v>3.907</v>
       </c>
       <c r="K22" t="n">
-        <v>4.133</v>
+        <v>4.129</v>
       </c>
       <c r="L22" t="n">
-        <v>4.152</v>
+        <v>4.142</v>
       </c>
       <c r="M22" t="n">
-        <v>4.269</v>
+        <v>4.258</v>
       </c>
       <c r="N22" t="n">
-        <v>4.317</v>
+        <v>4.304</v>
       </c>
       <c r="O22" t="n">
-        <v>4.456</v>
+        <v>4.428</v>
       </c>
       <c r="P22" t="n">
-        <v>4.545</v>
+        <v>4.526</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.651</v>
+        <v>4.642</v>
       </c>
       <c r="R22" t="n">
-        <v>4.709</v>
+        <v>4.711</v>
       </c>
       <c r="S22" t="n">
-        <v>4.797</v>
+        <v>4.812</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.881</v>
+        <v>2.895</v>
       </c>
       <c r="G23" t="n">
-        <v>3.103</v>
+        <v>3.119</v>
       </c>
       <c r="H23" t="n">
-        <v>3.358</v>
+        <v>3.374</v>
       </c>
       <c r="I23" t="n">
-        <v>3.597</v>
+        <v>3.592</v>
       </c>
       <c r="J23" t="n">
-        <v>3.843</v>
+        <v>3.847</v>
       </c>
       <c r="K23" t="n">
-        <v>4.032</v>
+        <v>4.029</v>
       </c>
       <c r="L23" t="n">
-        <v>4.05</v>
+        <v>4.04</v>
       </c>
       <c r="M23" t="n">
-        <v>4.16</v>
+        <v>4.149</v>
       </c>
       <c r="N23" t="n">
-        <v>4.211</v>
+        <v>4.198</v>
       </c>
       <c r="O23" t="n">
-        <v>4.332</v>
+        <v>4.304</v>
       </c>
       <c r="P23" t="n">
-        <v>4.408</v>
+        <v>4.389</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.457</v>
+        <v>4.447</v>
       </c>
       <c r="R23" t="n">
-        <v>4.495</v>
+        <v>4.497</v>
       </c>
       <c r="S23" t="n">
-        <v>4.553</v>
+        <v>4.568</v>
       </c>
       <c r="T23" t="n">
-        <v>4.491</v>
+        <v>4.516</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.819</v>
+        <v>2.832</v>
       </c>
       <c r="G24" t="n">
-        <v>3.014</v>
+        <v>3.032</v>
       </c>
       <c r="H24" t="n">
-        <v>3.251</v>
+        <v>3.271</v>
       </c>
       <c r="I24" t="n">
-        <v>3.535</v>
+        <v>3.53</v>
       </c>
       <c r="J24" t="n">
-        <v>3.736</v>
+        <v>3.741</v>
       </c>
       <c r="K24" t="n">
-        <v>3.915</v>
+        <v>3.912</v>
       </c>
       <c r="L24" t="n">
-        <v>3.931</v>
+        <v>3.921</v>
       </c>
       <c r="M24" t="n">
-        <v>4.019</v>
+        <v>4.009</v>
       </c>
       <c r="N24" t="n">
-        <v>4.085</v>
+        <v>4.072</v>
       </c>
       <c r="O24" t="n">
-        <v>4.332</v>
+        <v>4.304</v>
       </c>
       <c r="P24" t="n">
-        <v>4.348</v>
+        <v>4.329</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.382</v>
+        <v>4.373</v>
       </c>
       <c r="R24" t="n">
-        <v>4.417</v>
+        <v>4.419</v>
       </c>
       <c r="S24" t="n">
-        <v>4.468</v>
+        <v>4.483</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.876</v>
+        <v>2.889</v>
       </c>
       <c r="G25" t="n">
-        <v>3.103</v>
+        <v>3.119</v>
       </c>
       <c r="H25" t="n">
-        <v>3.361</v>
+        <v>3.377</v>
       </c>
       <c r="I25" t="n">
-        <v>3.606</v>
+        <v>3.601</v>
       </c>
       <c r="J25" t="n">
-        <v>3.858</v>
+        <v>3.862</v>
       </c>
       <c r="K25" t="n">
-        <v>4.064</v>
+        <v>4.06</v>
       </c>
       <c r="L25" t="n">
-        <v>4.081</v>
+        <v>4.07</v>
       </c>
       <c r="M25" t="n">
-        <v>4.191</v>
+        <v>4.18</v>
       </c>
       <c r="N25" t="n">
-        <v>4.238</v>
+        <v>4.225</v>
       </c>
       <c r="O25" t="n">
-        <v>4.361</v>
+        <v>4.333</v>
       </c>
       <c r="P25" t="n">
-        <v>4.43</v>
+        <v>4.411</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.49</v>
+        <v>4.481</v>
       </c>
       <c r="R25" t="n">
-        <v>4.519</v>
+        <v>4.52</v>
       </c>
       <c r="S25" t="n">
-        <v>4.576</v>
+        <v>4.591</v>
       </c>
       <c r="T25" t="n">
-        <v>4.509</v>
+        <v>4.534</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.192</v>
+        <v>3.208</v>
       </c>
       <c r="G26" t="n">
-        <v>3.41</v>
+        <v>3.426</v>
       </c>
       <c r="H26" t="n">
-        <v>3.762</v>
+        <v>3.775</v>
       </c>
       <c r="I26" t="n">
-        <v>4.024</v>
+        <v>4.018</v>
       </c>
       <c r="J26" t="n">
-        <v>4.442</v>
+        <v>4.445</v>
       </c>
       <c r="K26" t="n">
-        <v>4.868</v>
+        <v>4.864</v>
       </c>
       <c r="L26" t="n">
-        <v>4.954</v>
+        <v>4.942</v>
       </c>
       <c r="M26" t="n">
-        <v>5.106</v>
+        <v>5.092</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.419</v>
+        <v>5.392</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.989</v>
+        <v>3.007</v>
       </c>
       <c r="G27" t="n">
-        <v>3.166</v>
+        <v>3.185</v>
       </c>
       <c r="H27" t="n">
-        <v>3.442</v>
+        <v>3.458</v>
       </c>
       <c r="I27" t="n">
-        <v>3.684</v>
+        <v>3.678</v>
       </c>
       <c r="J27" t="n">
-        <v>3.98</v>
+        <v>3.981</v>
       </c>
       <c r="K27" t="n">
-        <v>4.187</v>
+        <v>4.186</v>
       </c>
       <c r="L27" t="n">
-        <v>4.224</v>
+        <v>4.209</v>
       </c>
       <c r="M27" t="n">
-        <v>4.329</v>
+        <v>4.316</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.522</v>
+        <v>4.494</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.092</v>
+        <v>3.11</v>
       </c>
       <c r="G28" t="n">
-        <v>3.277</v>
+        <v>3.296</v>
       </c>
       <c r="H28" t="n">
-        <v>3.568</v>
+        <v>3.584</v>
       </c>
       <c r="I28" t="n">
-        <v>3.821</v>
+        <v>3.815</v>
       </c>
       <c r="J28" t="n">
-        <v>4.153</v>
+        <v>4.154</v>
       </c>
       <c r="K28" t="n">
-        <v>4.379</v>
+        <v>4.378</v>
       </c>
       <c r="L28" t="n">
-        <v>4.427</v>
+        <v>4.412</v>
       </c>
       <c r="M28" t="n">
-        <v>4.541</v>
+        <v>4.528</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.814</v>
+        <v>4.786</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.938</v>
+        <v>2.956</v>
       </c>
       <c r="G29" t="n">
-        <v>3.112</v>
+        <v>3.131</v>
       </c>
       <c r="H29" t="n">
-        <v>3.379</v>
+        <v>3.395</v>
       </c>
       <c r="I29" t="n">
-        <v>3.609</v>
+        <v>3.603</v>
       </c>
       <c r="J29" t="n">
-        <v>3.892</v>
+        <v>3.893</v>
       </c>
       <c r="K29" t="n">
-        <v>4.082</v>
+        <v>4.081</v>
       </c>
       <c r="L29" t="n">
-        <v>4.109</v>
+        <v>4.095</v>
       </c>
       <c r="M29" t="n">
-        <v>4.192</v>
+        <v>4.179</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.393</v>
+        <v>4.365</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.232</v>
+        <v>3.244</v>
       </c>
       <c r="G30" t="n">
-        <v>3.383</v>
+        <v>3.396</v>
       </c>
       <c r="H30" t="n">
-        <v>3.694</v>
+        <v>3.705</v>
       </c>
       <c r="I30" t="n">
-        <v>3.949</v>
+        <v>3.94</v>
       </c>
       <c r="J30" t="n">
-        <v>4.304</v>
+        <v>4.306</v>
       </c>
       <c r="K30" t="n">
-        <v>4.67</v>
+        <v>4.662</v>
       </c>
       <c r="L30" t="n">
-        <v>4.732</v>
+        <v>4.716</v>
       </c>
       <c r="M30" t="n">
-        <v>4.872</v>
+        <v>4.856</v>
       </c>
       <c r="N30" t="n">
-        <v>5.028</v>
+        <v>5.014</v>
       </c>
       <c r="O30" t="n">
-        <v>5.37</v>
+        <v>5.342</v>
       </c>
       <c r="P30" t="n">
-        <v>5.574</v>
+        <v>5.555</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.331</v>
+        <v>6.322</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.561</v>
+        <v>3.573</v>
       </c>
       <c r="G31" t="n">
-        <v>3.748</v>
+        <v>3.761</v>
       </c>
       <c r="H31" t="n">
-        <v>4.11</v>
+        <v>4.121</v>
       </c>
       <c r="I31" t="n">
-        <v>4.378</v>
+        <v>4.369</v>
       </c>
       <c r="J31" t="n">
-        <v>4.795</v>
+        <v>4.797</v>
       </c>
       <c r="K31" t="n">
-        <v>5.203</v>
+        <v>5.195</v>
       </c>
       <c r="L31" t="n">
-        <v>5.344</v>
+        <v>5.329</v>
       </c>
       <c r="M31" t="n">
-        <v>5.603</v>
+        <v>5.587</v>
       </c>
       <c r="N31" t="n">
-        <v>5.887</v>
+        <v>5.873</v>
       </c>
       <c r="O31" t="n">
-        <v>6.406</v>
+        <v>6.378</v>
       </c>
       <c r="P31" t="n">
-        <v>6.563</v>
+        <v>6.544</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.304</v>
+        <v>7.295</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.331</v>
+        <v>3.343</v>
       </c>
       <c r="G32" t="n">
-        <v>3.5</v>
+        <v>3.513</v>
       </c>
       <c r="H32" t="n">
-        <v>3.838</v>
+        <v>3.849</v>
       </c>
       <c r="I32" t="n">
-        <v>4.108</v>
+        <v>4.099</v>
       </c>
       <c r="J32" t="n">
-        <v>4.482</v>
+        <v>4.484</v>
       </c>
       <c r="K32" t="n">
-        <v>4.855</v>
+        <v>4.847</v>
       </c>
       <c r="L32" t="n">
-        <v>4.936</v>
+        <v>4.92</v>
       </c>
       <c r="M32" t="n">
-        <v>5.145</v>
+        <v>5.129</v>
       </c>
       <c r="N32" t="n">
-        <v>5.389</v>
+        <v>5.374</v>
       </c>
       <c r="O32" t="n">
-        <v>5.815</v>
+        <v>5.787</v>
       </c>
       <c r="P32" t="n">
-        <v>6.034</v>
+        <v>6.015</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.792</v>
+        <v>6.783</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.097</v>
+        <v>3.109</v>
       </c>
       <c r="G33" t="n">
-        <v>3.248</v>
+        <v>3.261</v>
       </c>
       <c r="H33" t="n">
-        <v>3.512</v>
+        <v>3.523</v>
       </c>
       <c r="I33" t="n">
-        <v>3.734</v>
+        <v>3.726</v>
       </c>
       <c r="J33" t="n">
-        <v>4.011</v>
+        <v>4.013</v>
       </c>
       <c r="K33" t="n">
-        <v>4.31</v>
+        <v>4.305</v>
       </c>
       <c r="L33" t="n">
-        <v>4.337</v>
+        <v>4.322</v>
       </c>
       <c r="M33" t="n">
-        <v>4.401</v>
+        <v>4.385</v>
       </c>
       <c r="N33" t="n">
-        <v>4.417</v>
+        <v>4.403</v>
       </c>
       <c r="O33" t="n">
-        <v>4.524</v>
+        <v>4.496</v>
       </c>
       <c r="P33" t="n">
-        <v>4.607</v>
+        <v>4.588</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.048</v>
+        <v>5.038</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.157</v>
+        <v>3.169</v>
       </c>
       <c r="G34" t="n">
-        <v>3.301</v>
+        <v>3.314</v>
       </c>
       <c r="H34" t="n">
-        <v>3.574</v>
+        <v>3.585</v>
       </c>
       <c r="I34" t="n">
-        <v>3.802</v>
+        <v>3.794</v>
       </c>
       <c r="J34" t="n">
-        <v>4.083</v>
+        <v>4.085</v>
       </c>
       <c r="K34" t="n">
-        <v>4.386</v>
+        <v>4.381</v>
       </c>
       <c r="L34" t="n">
-        <v>4.416</v>
+        <v>4.4</v>
       </c>
       <c r="M34" t="n">
-        <v>4.491</v>
+        <v>4.476</v>
       </c>
       <c r="N34" t="n">
-        <v>4.522</v>
+        <v>4.507</v>
       </c>
       <c r="O34" t="n">
-        <v>4.693</v>
+        <v>4.665</v>
       </c>
       <c r="P34" t="n">
-        <v>4.901</v>
+        <v>4.882</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.749</v>
+        <v>5.739</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.131</v>
+        <v>3.143</v>
       </c>
       <c r="G35" t="n">
-        <v>3.275</v>
+        <v>3.288</v>
       </c>
       <c r="H35" t="n">
-        <v>3.542</v>
+        <v>3.553</v>
       </c>
       <c r="I35" t="n">
-        <v>3.768</v>
+        <v>3.76</v>
       </c>
       <c r="J35" t="n">
-        <v>4.051</v>
+        <v>4.053</v>
       </c>
       <c r="K35" t="n">
-        <v>4.34</v>
+        <v>4.335</v>
       </c>
       <c r="L35" t="n">
-        <v>4.371</v>
+        <v>4.356</v>
       </c>
       <c r="M35" t="n">
-        <v>4.438</v>
+        <v>4.423</v>
       </c>
       <c r="N35" t="n">
-        <v>4.458</v>
+        <v>4.444</v>
       </c>
       <c r="O35" t="n">
-        <v>4.59</v>
+        <v>4.562</v>
       </c>
       <c r="P35" t="n">
-        <v>4.704</v>
+        <v>4.685</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.384</v>
+        <v>5.375</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.021</v>
+        <v>3.033</v>
       </c>
       <c r="G36" t="n">
-        <v>3.159</v>
+        <v>3.173</v>
       </c>
       <c r="H36" t="n">
-        <v>3.418</v>
+        <v>3.429</v>
       </c>
       <c r="I36" t="n">
-        <v>3.644</v>
+        <v>3.635</v>
       </c>
       <c r="J36" t="n">
-        <v>3.946</v>
+        <v>3.948</v>
       </c>
       <c r="K36" t="n">
-        <v>4.234</v>
+        <v>4.23</v>
       </c>
       <c r="L36" t="n">
-        <v>4.258</v>
+        <v>4.246</v>
       </c>
       <c r="M36" t="n">
-        <v>4.302</v>
+        <v>4.288</v>
       </c>
       <c r="N36" t="n">
-        <v>4.322</v>
+        <v>4.307</v>
       </c>
       <c r="O36" t="n">
-        <v>4.432</v>
+        <v>4.404</v>
       </c>
       <c r="P36" t="n">
-        <v>4.505</v>
+        <v>4.486</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.765</v>
+        <v>4.755</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.904</v>
+        <v>3.916</v>
       </c>
       <c r="G37" t="n">
-        <v>4.442</v>
+        <v>4.455</v>
       </c>
       <c r="H37" t="n">
-        <v>5.082</v>
+        <v>5.093</v>
       </c>
       <c r="I37" t="n">
-        <v>5.439</v>
+        <v>5.43</v>
       </c>
       <c r="J37" t="n">
-        <v>6.285</v>
+        <v>6.286</v>
       </c>
       <c r="K37" t="n">
-        <v>7.242</v>
+        <v>7.234</v>
       </c>
       <c r="L37" t="n">
-        <v>7.545</v>
+        <v>7.529</v>
       </c>
       <c r="M37" t="n">
-        <v>7.875</v>
+        <v>7.859</v>
       </c>
       <c r="N37" t="n">
-        <v>8.042</v>
+        <v>8.029</v>
       </c>
       <c r="O37" t="n">
-        <v>8.285</v>
+        <v>8.257</v>
       </c>
       <c r="P37" t="n">
-        <v>8.364000000000001</v>
+        <v>8.345000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.795</v>
+        <v>8.785</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.966</v>
+        <v>4.978</v>
       </c>
       <c r="G38" t="n">
-        <v>5.757</v>
+        <v>5.77</v>
       </c>
       <c r="H38" t="n">
-        <v>6.609</v>
+        <v>6.62</v>
       </c>
       <c r="I38" t="n">
-        <v>7.123</v>
+        <v>7.114</v>
       </c>
       <c r="J38" t="n">
-        <v>8.228999999999999</v>
+        <v>8.23</v>
       </c>
       <c r="K38" t="n">
-        <v>9.365</v>
+        <v>9.358000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.827999999999999</v>
+        <v>9.811999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.287</v>
+        <v>10.27</v>
       </c>
       <c r="N38" t="n">
-        <v>10.461</v>
+        <v>10.448</v>
       </c>
       <c r="O38" t="n">
-        <v>10.685</v>
+        <v>10.657</v>
       </c>
       <c r="P38" t="n">
-        <v>10.762</v>
+        <v>10.743</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.245</v>
+        <v>11.236</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.286</v>
+        <v>4.298</v>
       </c>
       <c r="G39" t="n">
-        <v>4.955</v>
+        <v>4.968</v>
       </c>
       <c r="H39" t="n">
-        <v>5.674</v>
+        <v>5.685</v>
       </c>
       <c r="I39" t="n">
-        <v>6.127</v>
+        <v>6.118</v>
       </c>
       <c r="J39" t="n">
-        <v>7.101</v>
+        <v>7.103</v>
       </c>
       <c r="K39" t="n">
-        <v>8.198</v>
+        <v>8.19</v>
       </c>
       <c r="L39" t="n">
-        <v>8.583</v>
+        <v>8.568</v>
       </c>
       <c r="M39" t="n">
-        <v>8.923</v>
+        <v>8.907</v>
       </c>
       <c r="N39" t="n">
-        <v>9.089</v>
+        <v>9.074999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.336</v>
+        <v>9.308</v>
       </c>
       <c r="P39" t="n">
-        <v>9.417</v>
+        <v>9.398</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.891</v>
+        <v>9.881</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.424</v>
+        <v>3.436</v>
       </c>
       <c r="G40" t="n">
-        <v>3.621</v>
+        <v>3.634</v>
       </c>
       <c r="H40" t="n">
-        <v>3.953</v>
+        <v>3.964</v>
       </c>
       <c r="I40" t="n">
-        <v>4.222</v>
+        <v>4.213</v>
       </c>
       <c r="J40" t="n">
-        <v>4.596</v>
+        <v>4.597</v>
       </c>
       <c r="K40" t="n">
-        <v>4.976</v>
+        <v>4.968</v>
       </c>
       <c r="L40" t="n">
-        <v>5.056</v>
+        <v>5.041</v>
       </c>
       <c r="M40" t="n">
-        <v>5.215</v>
+        <v>5.199</v>
       </c>
       <c r="N40" t="n">
-        <v>5.386</v>
+        <v>5.371</v>
       </c>
       <c r="O40" t="n">
-        <v>5.749</v>
+        <v>5.721</v>
       </c>
       <c r="P40" t="n">
-        <v>5.996</v>
+        <v>5.977</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.782</v>
+        <v>6.773</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.81</v>
+        <v>3.822</v>
       </c>
       <c r="G41" t="n">
-        <v>4.05</v>
+        <v>4.063</v>
       </c>
       <c r="H41" t="n">
-        <v>4.439</v>
+        <v>4.45</v>
       </c>
       <c r="I41" t="n">
-        <v>4.726</v>
+        <v>4.717</v>
       </c>
       <c r="J41" t="n">
-        <v>5.151</v>
+        <v>5.152</v>
       </c>
       <c r="K41" t="n">
-        <v>5.576</v>
+        <v>5.568</v>
       </c>
       <c r="L41" t="n">
-        <v>5.735</v>
+        <v>5.719</v>
       </c>
       <c r="M41" t="n">
-        <v>6.018</v>
+        <v>6.002</v>
       </c>
       <c r="N41" t="n">
-        <v>6.317</v>
+        <v>6.302</v>
       </c>
       <c r="O41" t="n">
-        <v>6.864</v>
+        <v>6.836</v>
       </c>
       <c r="P41" t="n">
-        <v>7.055</v>
+        <v>7.036</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.829</v>
+        <v>7.82</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.545</v>
+        <v>3.557</v>
       </c>
       <c r="G42" t="n">
-        <v>3.77</v>
+        <v>3.783</v>
       </c>
       <c r="H42" t="n">
-        <v>4.129</v>
+        <v>4.14</v>
       </c>
       <c r="I42" t="n">
-        <v>4.411</v>
+        <v>4.402</v>
       </c>
       <c r="J42" t="n">
-        <v>4.798</v>
+        <v>4.8</v>
       </c>
       <c r="K42" t="n">
-        <v>5.197</v>
+        <v>5.189</v>
       </c>
       <c r="L42" t="n">
-        <v>5.293</v>
+        <v>5.277</v>
       </c>
       <c r="M42" t="n">
-        <v>5.522</v>
+        <v>5.506</v>
       </c>
       <c r="N42" t="n">
-        <v>5.8</v>
+        <v>5.786</v>
       </c>
       <c r="O42" t="n">
-        <v>6.241</v>
+        <v>6.213</v>
       </c>
       <c r="P42" t="n">
-        <v>6.498</v>
+        <v>6.479</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.294</v>
+        <v>7.285</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.245</v>
+        <v>3.257</v>
       </c>
       <c r="G43" t="n">
-        <v>3.43</v>
+        <v>3.443</v>
       </c>
       <c r="H43" t="n">
-        <v>3.713</v>
+        <v>3.724</v>
       </c>
       <c r="I43" t="n">
-        <v>3.942</v>
+        <v>3.934</v>
       </c>
       <c r="J43" t="n">
-        <v>4.239</v>
+        <v>4.24</v>
       </c>
       <c r="K43" t="n">
-        <v>4.542</v>
+        <v>4.537</v>
       </c>
       <c r="L43" t="n">
-        <v>4.579</v>
+        <v>4.564</v>
       </c>
       <c r="M43" t="n">
-        <v>4.656</v>
+        <v>4.641</v>
       </c>
       <c r="N43" t="n">
-        <v>4.686</v>
+        <v>4.672</v>
       </c>
       <c r="O43" t="n">
-        <v>4.837</v>
+        <v>4.809</v>
       </c>
       <c r="P43" t="n">
-        <v>4.972</v>
+        <v>4.953</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.658</v>
+        <v>5.649</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.099</v>
+        <v>3.111</v>
       </c>
       <c r="G44" t="n">
-        <v>3.269</v>
+        <v>3.282</v>
       </c>
       <c r="H44" t="n">
-        <v>3.542</v>
+        <v>3.553</v>
       </c>
       <c r="I44" t="n">
-        <v>3.771</v>
+        <v>3.762</v>
       </c>
       <c r="J44" t="n">
-        <v>4.087</v>
+        <v>4.088</v>
       </c>
       <c r="K44" t="n">
-        <v>4.386</v>
+        <v>4.381</v>
       </c>
       <c r="L44" t="n">
-        <v>4.419</v>
+        <v>4.407</v>
       </c>
       <c r="M44" t="n">
-        <v>4.472</v>
+        <v>4.459</v>
       </c>
       <c r="N44" t="n">
-        <v>4.503</v>
+        <v>4.489</v>
       </c>
       <c r="O44" t="n">
-        <v>4.633</v>
+        <v>4.605</v>
       </c>
       <c r="P44" t="n">
-        <v>4.735</v>
+        <v>4.716</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.028</v>
+        <v>5.019</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-11 ~ 2026-06-11
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.401</v>
+        <v>3.423</v>
       </c>
       <c r="G2" t="n">
-        <v>3.713</v>
+        <v>3.735</v>
       </c>
       <c r="H2" t="n">
-        <v>4.007</v>
+        <v>4.026</v>
       </c>
       <c r="I2" t="n">
-        <v>4.195</v>
+        <v>4.198</v>
       </c>
       <c r="J2" t="n">
-        <v>4.511</v>
+        <v>4.536</v>
       </c>
       <c r="K2" t="n">
-        <v>4.895</v>
+        <v>4.92</v>
       </c>
       <c r="L2" t="n">
-        <v>5.06</v>
+        <v>5.096</v>
       </c>
       <c r="M2" t="n">
-        <v>5.312</v>
+        <v>5.345</v>
       </c>
       <c r="N2" t="n">
-        <v>5.577</v>
+        <v>5.606</v>
       </c>
       <c r="O2" t="n">
-        <v>5.859</v>
+        <v>5.87</v>
       </c>
       <c r="P2" t="n">
-        <v>6.076</v>
+        <v>6.107</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.722</v>
+        <v>6.772</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.423</v>
+        <v>4.445</v>
       </c>
       <c r="G3" t="n">
-        <v>4.915</v>
+        <v>4.938</v>
       </c>
       <c r="H3" t="n">
-        <v>5.243</v>
+        <v>5.262</v>
       </c>
       <c r="I3" t="n">
-        <v>5.423</v>
+        <v>5.427</v>
       </c>
       <c r="J3" t="n">
-        <v>5.756</v>
+        <v>5.781</v>
       </c>
       <c r="K3" t="n">
-        <v>6.211</v>
+        <v>6.237</v>
       </c>
       <c r="L3" t="n">
-        <v>6.445</v>
+        <v>6.482</v>
       </c>
       <c r="M3" t="n">
-        <v>6.729</v>
+        <v>6.762</v>
       </c>
       <c r="N3" t="n">
-        <v>6.936</v>
+        <v>6.965</v>
       </c>
       <c r="O3" t="n">
-        <v>7.169</v>
+        <v>7.18</v>
       </c>
       <c r="P3" t="n">
-        <v>7.255</v>
+        <v>7.285</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.788</v>
+        <v>7.838</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.915</v>
+        <v>3.937</v>
       </c>
       <c r="G4" t="n">
-        <v>4.297</v>
+        <v>4.319</v>
       </c>
       <c r="H4" t="n">
-        <v>4.652</v>
+        <v>4.671</v>
       </c>
       <c r="I4" t="n">
-        <v>4.866</v>
+        <v>4.869</v>
       </c>
       <c r="J4" t="n">
-        <v>5.2</v>
+        <v>5.225</v>
       </c>
       <c r="K4" t="n">
-        <v>5.65</v>
+        <v>5.675</v>
       </c>
       <c r="L4" t="n">
-        <v>5.814</v>
+        <v>5.851</v>
       </c>
       <c r="M4" t="n">
-        <v>6.086</v>
+        <v>6.12</v>
       </c>
       <c r="N4" t="n">
-        <v>6.264</v>
+        <v>6.293</v>
       </c>
       <c r="O4" t="n">
-        <v>6.52</v>
+        <v>6.531</v>
       </c>
       <c r="P4" t="n">
-        <v>6.607</v>
+        <v>6.638</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.143</v>
+        <v>7.193</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.099</v>
+        <v>3.121</v>
       </c>
       <c r="G5" t="n">
-        <v>3.256</v>
+        <v>3.278</v>
       </c>
       <c r="H5" t="n">
-        <v>3.514</v>
+        <v>3.533</v>
       </c>
       <c r="I5" t="n">
-        <v>3.767</v>
+        <v>3.77</v>
       </c>
       <c r="J5" t="n">
-        <v>4.068</v>
+        <v>4.093</v>
       </c>
       <c r="K5" t="n">
-        <v>4.299</v>
+        <v>4.324</v>
       </c>
       <c r="L5" t="n">
-        <v>4.307</v>
+        <v>4.344</v>
       </c>
       <c r="M5" t="n">
-        <v>4.37</v>
+        <v>4.403</v>
       </c>
       <c r="N5" t="n">
-        <v>4.389</v>
+        <v>4.418</v>
       </c>
       <c r="O5" t="n">
-        <v>4.459</v>
+        <v>4.469</v>
       </c>
       <c r="P5" t="n">
-        <v>4.745</v>
+        <v>4.776</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.634</v>
+        <v>5.684</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.14</v>
+        <v>3.162</v>
       </c>
       <c r="G6" t="n">
-        <v>3.311</v>
+        <v>3.333</v>
       </c>
       <c r="H6" t="n">
-        <v>3.584</v>
+        <v>3.603</v>
       </c>
       <c r="I6" t="n">
-        <v>3.85</v>
+        <v>3.853</v>
       </c>
       <c r="J6" t="n">
-        <v>4.159</v>
+        <v>4.184</v>
       </c>
       <c r="K6" t="n">
-        <v>4.412</v>
+        <v>4.437</v>
       </c>
       <c r="L6" t="n">
-        <v>4.426</v>
+        <v>4.463</v>
       </c>
       <c r="M6" t="n">
-        <v>4.526</v>
+        <v>4.559</v>
       </c>
       <c r="N6" t="n">
-        <v>4.556</v>
+        <v>4.585</v>
       </c>
       <c r="O6" t="n">
-        <v>4.725</v>
+        <v>4.736</v>
       </c>
       <c r="P6" t="n">
-        <v>5.177</v>
+        <v>5.208</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.03</v>
+        <v>6.08</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.12</v>
+        <v>3.142</v>
       </c>
       <c r="G7" t="n">
-        <v>3.275</v>
+        <v>3.297</v>
       </c>
       <c r="H7" t="n">
-        <v>3.53</v>
+        <v>3.549</v>
       </c>
       <c r="I7" t="n">
-        <v>3.787</v>
+        <v>3.79</v>
       </c>
       <c r="J7" t="n">
-        <v>4.092</v>
+        <v>4.117</v>
       </c>
       <c r="K7" t="n">
-        <v>4.326</v>
+        <v>4.351</v>
       </c>
       <c r="L7" t="n">
-        <v>4.334</v>
+        <v>4.371</v>
       </c>
       <c r="M7" t="n">
-        <v>4.43</v>
+        <v>4.463</v>
       </c>
       <c r="N7" t="n">
-        <v>4.448</v>
+        <v>4.477</v>
       </c>
       <c r="O7" t="n">
-        <v>4.622</v>
+        <v>4.633</v>
       </c>
       <c r="P7" t="n">
-        <v>4.961</v>
+        <v>4.992</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.798</v>
+        <v>5.848</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.534</v>
+        <v>5.557</v>
       </c>
       <c r="G8" t="n">
-        <v>6.215</v>
+        <v>6.237</v>
       </c>
       <c r="H8" t="n">
-        <v>6.691</v>
+        <v>6.71</v>
       </c>
       <c r="I8" t="n">
-        <v>6.95</v>
+        <v>6.953</v>
       </c>
       <c r="J8" t="n">
-        <v>7.349</v>
+        <v>7.374</v>
       </c>
       <c r="K8" t="n">
-        <v>8.085000000000001</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>8.403</v>
+        <v>8.44</v>
       </c>
       <c r="M8" t="n">
-        <v>8.718999999999999</v>
+        <v>8.752000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.859999999999999</v>
+        <v>8.888999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.179</v>
+        <v>9.189</v>
       </c>
       <c r="P8" t="n">
-        <v>9.368</v>
+        <v>9.398999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.099</v>
+        <v>10.149</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.752</v>
+        <v>2.755</v>
       </c>
       <c r="G9" t="n">
-        <v>2.988</v>
+        <v>2.99</v>
       </c>
       <c r="H9" t="n">
-        <v>3.254</v>
+        <v>3.232</v>
       </c>
       <c r="I9" t="n">
-        <v>3.403</v>
+        <v>3.393</v>
       </c>
       <c r="J9" t="n">
-        <v>3.598</v>
+        <v>3.615</v>
       </c>
       <c r="K9" t="n">
-        <v>3.733</v>
+        <v>3.744</v>
       </c>
       <c r="L9" t="n">
-        <v>3.829</v>
+        <v>3.858</v>
       </c>
       <c r="M9" t="n">
-        <v>3.877</v>
+        <v>3.906</v>
       </c>
       <c r="N9" t="n">
-        <v>3.985</v>
+        <v>4.011</v>
       </c>
       <c r="O9" t="n">
-        <v>4.07</v>
+        <v>4.08</v>
       </c>
       <c r="P9" t="n">
-        <v>4.191</v>
+        <v>4.222</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.265</v>
+        <v>4.315</v>
       </c>
       <c r="R9" t="n">
-        <v>4.315</v>
+        <v>4.361</v>
       </c>
       <c r="S9" t="n">
+        <v>4.405</v>
+      </c>
+      <c r="T9" t="n">
         <v>4.36</v>
       </c>
-      <c r="T9" t="n">
-        <v>4.31</v>
-      </c>
       <c r="U9" t="n">
-        <v>4.259</v>
+        <v>4.323</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.761</v>
+        <v>2.762</v>
       </c>
       <c r="G10" t="n">
-        <v>3.001</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>3.259</v>
+        <v>3.235</v>
       </c>
       <c r="I10" t="n">
-        <v>3.406</v>
+        <v>3.396</v>
       </c>
       <c r="J10" t="n">
-        <v>3.613</v>
+        <v>3.631</v>
       </c>
       <c r="K10" t="n">
-        <v>3.768</v>
+        <v>3.78</v>
       </c>
       <c r="L10" t="n">
-        <v>3.844</v>
+        <v>3.871</v>
       </c>
       <c r="M10" t="n">
-        <v>3.943</v>
+        <v>3.97</v>
       </c>
       <c r="N10" t="n">
-        <v>4.009</v>
+        <v>4.036</v>
       </c>
       <c r="O10" t="n">
-        <v>4.29</v>
+        <v>4.31</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.565</v>
+        <v>2.566</v>
       </c>
       <c r="G11" t="n">
         <v>2.805</v>
       </c>
       <c r="H11" t="n">
-        <v>3.084</v>
+        <v>3.06</v>
       </c>
       <c r="I11" t="n">
-        <v>3.21</v>
+        <v>3.2</v>
       </c>
       <c r="J11" t="n">
-        <v>3.405</v>
+        <v>3.424</v>
       </c>
       <c r="K11" t="n">
-        <v>3.555</v>
+        <v>3.565</v>
       </c>
       <c r="L11" t="n">
-        <v>3.641</v>
+        <v>3.668</v>
       </c>
       <c r="M11" t="n">
-        <v>3.751</v>
+        <v>3.778</v>
       </c>
       <c r="N11" t="n">
-        <v>3.816</v>
+        <v>3.843</v>
       </c>
       <c r="O11" t="n">
-        <v>4.056</v>
+        <v>4.076</v>
       </c>
       <c r="P11" t="n">
-        <v>4.137</v>
+        <v>4.168</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.463</v>
+        <v>4.513</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.345</v>
+        <v>3.365</v>
       </c>
       <c r="G12" t="n">
-        <v>3.622</v>
+        <v>3.641</v>
       </c>
       <c r="H12" t="n">
-        <v>3.917</v>
+        <v>3.937</v>
       </c>
       <c r="I12" t="n">
-        <v>4.18</v>
+        <v>4.179</v>
       </c>
       <c r="J12" t="n">
-        <v>4.509</v>
+        <v>4.531</v>
       </c>
       <c r="K12" t="n">
-        <v>4.688</v>
+        <v>4.707</v>
       </c>
       <c r="L12" t="n">
-        <v>4.718</v>
+        <v>4.749</v>
       </c>
       <c r="M12" t="n">
-        <v>4.845</v>
+        <v>4.875</v>
       </c>
       <c r="N12" t="n">
-        <v>4.901</v>
+        <v>4.929</v>
       </c>
       <c r="O12" t="n">
-        <v>5.079</v>
+        <v>5.09</v>
       </c>
       <c r="P12" t="n">
-        <v>5.218</v>
+        <v>5.248</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.577</v>
+        <v>5.627</v>
       </c>
       <c r="R12" t="n">
-        <v>5.806</v>
+        <v>5.852</v>
       </c>
       <c r="S12" t="n">
-        <v>6.064</v>
+        <v>6.109</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.099</v>
+        <v>3.118</v>
       </c>
       <c r="G13" t="n">
-        <v>3.312</v>
+        <v>3.331</v>
       </c>
       <c r="H13" t="n">
-        <v>3.584</v>
+        <v>3.604</v>
       </c>
       <c r="I13" t="n">
-        <v>3.828</v>
+        <v>3.826</v>
       </c>
       <c r="J13" t="n">
-        <v>4.146</v>
+        <v>4.168</v>
       </c>
       <c r="K13" t="n">
-        <v>4.321</v>
+        <v>4.34</v>
       </c>
       <c r="L13" t="n">
-        <v>4.358</v>
+        <v>4.388</v>
       </c>
       <c r="M13" t="n">
-        <v>4.473</v>
+        <v>4.503</v>
       </c>
       <c r="N13" t="n">
-        <v>4.529</v>
+        <v>4.557</v>
       </c>
       <c r="O13" t="n">
-        <v>4.707</v>
+        <v>4.718</v>
       </c>
       <c r="P13" t="n">
-        <v>4.809</v>
+        <v>4.84</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.098</v>
+        <v>5.148</v>
       </c>
       <c r="R13" t="n">
-        <v>5.355</v>
+        <v>5.401</v>
       </c>
       <c r="S13" t="n">
-        <v>5.626</v>
+        <v>5.671</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.916</v>
+        <v>2.936</v>
       </c>
       <c r="G14" t="n">
-        <v>3.118</v>
+        <v>3.137</v>
       </c>
       <c r="H14" t="n">
-        <v>3.387</v>
+        <v>3.407</v>
       </c>
       <c r="I14" t="n">
-        <v>3.612</v>
+        <v>3.611</v>
       </c>
       <c r="J14" t="n">
-        <v>3.888</v>
+        <v>3.909</v>
       </c>
       <c r="K14" t="n">
-        <v>4.009</v>
+        <v>4.029</v>
       </c>
       <c r="L14" t="n">
-        <v>4.031</v>
+        <v>4.061</v>
       </c>
       <c r="M14" t="n">
-        <v>4.159</v>
+        <v>4.189</v>
       </c>
       <c r="N14" t="n">
-        <v>4.208</v>
+        <v>4.236</v>
       </c>
       <c r="O14" t="n">
-        <v>4.366</v>
+        <v>4.377</v>
       </c>
       <c r="P14" t="n">
-        <v>4.445</v>
+        <v>4.476</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.687</v>
+        <v>4.737</v>
       </c>
       <c r="R14" t="n">
-        <v>4.87</v>
+        <v>4.916</v>
       </c>
       <c r="S14" t="n">
-        <v>5.079</v>
+        <v>5.124</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.894</v>
+        <v>2.913</v>
       </c>
       <c r="G15" t="n">
-        <v>3.092</v>
+        <v>3.111</v>
       </c>
       <c r="H15" t="n">
-        <v>3.358</v>
+        <v>3.378</v>
       </c>
       <c r="I15" t="n">
-        <v>3.563</v>
+        <v>3.562</v>
       </c>
       <c r="J15" t="n">
-        <v>3.825</v>
+        <v>3.847</v>
       </c>
       <c r="K15" t="n">
-        <v>3.961</v>
+        <v>3.981</v>
       </c>
       <c r="L15" t="n">
-        <v>3.967</v>
+        <v>3.997</v>
       </c>
       <c r="M15" t="n">
-        <v>4.072</v>
+        <v>4.102</v>
       </c>
       <c r="N15" t="n">
-        <v>4.111</v>
+        <v>4.139</v>
       </c>
       <c r="O15" t="n">
-        <v>4.308</v>
+        <v>4.32</v>
       </c>
       <c r="P15" t="n">
-        <v>4.341</v>
+        <v>4.372</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.589</v>
+        <v>4.639</v>
       </c>
       <c r="R15" t="n">
-        <v>4.764</v>
+        <v>4.81</v>
       </c>
       <c r="S15" t="n">
-        <v>4.974</v>
+        <v>5.019</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.894</v>
+        <v>2.913</v>
       </c>
       <c r="G16" t="n">
-        <v>3.092</v>
+        <v>3.111</v>
       </c>
       <c r="H16" t="n">
-        <v>3.358</v>
+        <v>3.378</v>
       </c>
       <c r="I16" t="n">
-        <v>3.563</v>
+        <v>3.562</v>
       </c>
       <c r="J16" t="n">
-        <v>3.825</v>
+        <v>3.847</v>
       </c>
       <c r="K16" t="n">
-        <v>3.961</v>
+        <v>3.981</v>
       </c>
       <c r="L16" t="n">
-        <v>3.967</v>
+        <v>3.997</v>
       </c>
       <c r="M16" t="n">
-        <v>4.072</v>
+        <v>4.102</v>
       </c>
       <c r="N16" t="n">
-        <v>4.114</v>
+        <v>4.142</v>
       </c>
       <c r="O16" t="n">
-        <v>4.315</v>
+        <v>4.327</v>
       </c>
       <c r="P16" t="n">
-        <v>4.365</v>
+        <v>4.395</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.616</v>
+        <v>4.666</v>
       </c>
       <c r="R16" t="n">
-        <v>4.792</v>
+        <v>4.838</v>
       </c>
       <c r="S16" t="n">
-        <v>5.003</v>
+        <v>5.048</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.796</v>
+        <v>2.795</v>
       </c>
       <c r="G17" t="n">
-        <v>3.059</v>
+        <v>3.054</v>
       </c>
       <c r="H17" t="n">
-        <v>3.32</v>
+        <v>3.292</v>
       </c>
       <c r="I17" t="n">
-        <v>3.464</v>
+        <v>3.453</v>
       </c>
       <c r="J17" t="n">
-        <v>3.677</v>
+        <v>3.696</v>
       </c>
       <c r="K17" t="n">
-        <v>3.847</v>
+        <v>3.856</v>
       </c>
       <c r="L17" t="n">
-        <v>3.927</v>
+        <v>3.955</v>
       </c>
       <c r="M17" t="n">
-        <v>4.066</v>
+        <v>4.094</v>
       </c>
       <c r="N17" t="n">
-        <v>4.112</v>
+        <v>4.141</v>
       </c>
       <c r="O17" t="n">
-        <v>4.309</v>
+        <v>4.33</v>
       </c>
       <c r="P17" t="n">
-        <v>4.418</v>
+        <v>4.45</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.796</v>
       </c>
       <c r="G18" t="n">
-        <v>3.06</v>
+        <v>3.055</v>
       </c>
       <c r="H18" t="n">
-        <v>3.32</v>
+        <v>3.292</v>
       </c>
       <c r="I18" t="n">
-        <v>3.465</v>
+        <v>3.453</v>
       </c>
       <c r="J18" t="n">
-        <v>3.677</v>
+        <v>3.696</v>
       </c>
       <c r="K18" t="n">
-        <v>3.848</v>
+        <v>3.857</v>
       </c>
       <c r="L18" t="n">
-        <v>3.927</v>
+        <v>3.955</v>
       </c>
       <c r="M18" t="n">
-        <v>4.066</v>
+        <v>4.094</v>
       </c>
       <c r="N18" t="n">
-        <v>4.113</v>
+        <v>4.142</v>
       </c>
       <c r="O18" t="n">
-        <v>4.307</v>
+        <v>4.328</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.905</v>
+        <v>2.924</v>
       </c>
       <c r="G19" t="n">
-        <v>3.106</v>
+        <v>3.124</v>
       </c>
       <c r="H19" t="n">
-        <v>3.374</v>
+        <v>3.395</v>
       </c>
       <c r="I19" t="n">
-        <v>3.596</v>
+        <v>3.595</v>
       </c>
       <c r="J19" t="n">
-        <v>3.867</v>
+        <v>3.888</v>
       </c>
       <c r="K19" t="n">
-        <v>4.004</v>
+        <v>4.024</v>
       </c>
       <c r="L19" t="n">
-        <v>4.028</v>
+        <v>4.058</v>
       </c>
       <c r="M19" t="n">
-        <v>4.15</v>
+        <v>4.18</v>
       </c>
       <c r="N19" t="n">
-        <v>4.197</v>
+        <v>4.228</v>
       </c>
       <c r="O19" t="n">
-        <v>4.351</v>
+        <v>4.363</v>
       </c>
       <c r="P19" t="n">
-        <v>4.403</v>
+        <v>4.434</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.627</v>
+        <v>4.677</v>
       </c>
       <c r="R19" t="n">
-        <v>4.811</v>
+        <v>4.857</v>
       </c>
       <c r="S19" t="n">
-        <v>5.014</v>
+        <v>5.059</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.66</v>
+        <v>2.662</v>
       </c>
       <c r="G20" t="n">
-        <v>2.771</v>
+        <v>2.772</v>
       </c>
       <c r="H20" t="n">
-        <v>2.891</v>
+        <v>2.888</v>
       </c>
       <c r="I20" t="n">
-        <v>3.053</v>
+        <v>3.037</v>
       </c>
       <c r="J20" t="n">
-        <v>3.532</v>
+        <v>3.541</v>
       </c>
       <c r="K20" t="n">
-        <v>3.785</v>
+        <v>3.802</v>
       </c>
       <c r="L20" t="n">
-        <v>3.786</v>
+        <v>3.81</v>
       </c>
       <c r="M20" t="n">
-        <v>3.88</v>
+        <v>3.906</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>3.009</v>
       </c>
       <c r="G21" t="n">
-        <v>3.22</v>
+        <v>3.234</v>
       </c>
       <c r="H21" t="n">
-        <v>3.501</v>
+        <v>3.514</v>
       </c>
       <c r="I21" t="n">
-        <v>3.725</v>
+        <v>3.727</v>
       </c>
       <c r="J21" t="n">
-        <v>4.022</v>
+        <v>4.047</v>
       </c>
       <c r="K21" t="n">
-        <v>4.247</v>
+        <v>4.272</v>
       </c>
       <c r="L21" t="n">
-        <v>4.275</v>
+        <v>4.307</v>
       </c>
       <c r="M21" t="n">
-        <v>4.387</v>
+        <v>4.419</v>
       </c>
       <c r="N21" t="n">
-        <v>4.43</v>
+        <v>4.46</v>
       </c>
       <c r="O21" t="n">
-        <v>4.557</v>
+        <v>4.568</v>
       </c>
       <c r="P21" t="n">
-        <v>4.663</v>
+        <v>4.694</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.783</v>
+        <v>4.833</v>
       </c>
       <c r="R21" t="n">
-        <v>4.862</v>
+        <v>4.908</v>
       </c>
       <c r="S21" t="n">
-        <v>4.966</v>
+        <v>5.011</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.946</v>
+        <v>2.955</v>
       </c>
       <c r="G22" t="n">
-        <v>3.165</v>
+        <v>3.179</v>
       </c>
       <c r="H22" t="n">
-        <v>3.433</v>
+        <v>3.446</v>
       </c>
       <c r="I22" t="n">
-        <v>3.643</v>
+        <v>3.646</v>
       </c>
       <c r="J22" t="n">
-        <v>3.907</v>
+        <v>3.932</v>
       </c>
       <c r="K22" t="n">
-        <v>4.129</v>
+        <v>4.153</v>
       </c>
       <c r="L22" t="n">
-        <v>4.142</v>
+        <v>4.174</v>
       </c>
       <c r="M22" t="n">
-        <v>4.258</v>
+        <v>4.29</v>
       </c>
       <c r="N22" t="n">
-        <v>4.304</v>
+        <v>4.334</v>
       </c>
       <c r="O22" t="n">
-        <v>4.428</v>
+        <v>4.439</v>
       </c>
       <c r="P22" t="n">
-        <v>4.526</v>
+        <v>4.557</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.642</v>
+        <v>4.692</v>
       </c>
       <c r="R22" t="n">
-        <v>4.711</v>
+        <v>4.757</v>
       </c>
       <c r="S22" t="n">
-        <v>4.812</v>
+        <v>4.857</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.895</v>
+        <v>2.903</v>
       </c>
       <c r="G23" t="n">
-        <v>3.119</v>
+        <v>3.133</v>
       </c>
       <c r="H23" t="n">
-        <v>3.374</v>
+        <v>3.387</v>
       </c>
       <c r="I23" t="n">
-        <v>3.592</v>
+        <v>3.594</v>
       </c>
       <c r="J23" t="n">
-        <v>3.847</v>
+        <v>3.872</v>
       </c>
       <c r="K23" t="n">
-        <v>4.029</v>
+        <v>4.053</v>
       </c>
       <c r="L23" t="n">
-        <v>4.04</v>
+        <v>4.072</v>
       </c>
       <c r="M23" t="n">
-        <v>4.149</v>
+        <v>4.182</v>
       </c>
       <c r="N23" t="n">
-        <v>4.198</v>
+        <v>4.228</v>
       </c>
       <c r="O23" t="n">
-        <v>4.304</v>
+        <v>4.315</v>
       </c>
       <c r="P23" t="n">
-        <v>4.389</v>
+        <v>4.42</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.447</v>
+        <v>4.497</v>
       </c>
       <c r="R23" t="n">
-        <v>4.497</v>
+        <v>4.542</v>
       </c>
       <c r="S23" t="n">
-        <v>4.568</v>
+        <v>4.613</v>
       </c>
       <c r="T23" t="n">
-        <v>4.516</v>
+        <v>4.566</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.832</v>
+        <v>2.839</v>
       </c>
       <c r="G24" t="n">
-        <v>3.032</v>
+        <v>3.044</v>
       </c>
       <c r="H24" t="n">
-        <v>3.271</v>
+        <v>3.284</v>
       </c>
       <c r="I24" t="n">
-        <v>3.53</v>
+        <v>3.532</v>
       </c>
       <c r="J24" t="n">
-        <v>3.741</v>
+        <v>3.766</v>
       </c>
       <c r="K24" t="n">
-        <v>3.912</v>
+        <v>3.936</v>
       </c>
       <c r="L24" t="n">
-        <v>3.921</v>
+        <v>3.953</v>
       </c>
       <c r="M24" t="n">
-        <v>4.009</v>
+        <v>4.04</v>
       </c>
       <c r="N24" t="n">
-        <v>4.072</v>
+        <v>4.102</v>
       </c>
       <c r="O24" t="n">
-        <v>4.304</v>
+        <v>4.315</v>
       </c>
       <c r="P24" t="n">
-        <v>4.329</v>
+        <v>4.36</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.373</v>
+        <v>4.423</v>
       </c>
       <c r="R24" t="n">
-        <v>4.419</v>
+        <v>4.464</v>
       </c>
       <c r="S24" t="n">
-        <v>4.483</v>
+        <v>4.528</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.889</v>
+        <v>2.898</v>
       </c>
       <c r="G25" t="n">
-        <v>3.119</v>
+        <v>3.133</v>
       </c>
       <c r="H25" t="n">
-        <v>3.377</v>
+        <v>3.39</v>
       </c>
       <c r="I25" t="n">
-        <v>3.601</v>
+        <v>3.603</v>
       </c>
       <c r="J25" t="n">
-        <v>3.862</v>
+        <v>3.887</v>
       </c>
       <c r="K25" t="n">
-        <v>4.06</v>
+        <v>4.085</v>
       </c>
       <c r="L25" t="n">
-        <v>4.07</v>
+        <v>4.103</v>
       </c>
       <c r="M25" t="n">
-        <v>4.18</v>
+        <v>4.213</v>
       </c>
       <c r="N25" t="n">
-        <v>4.225</v>
+        <v>4.255</v>
       </c>
       <c r="O25" t="n">
-        <v>4.333</v>
+        <v>4.343</v>
       </c>
       <c r="P25" t="n">
-        <v>4.411</v>
+        <v>4.442</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.481</v>
+        <v>4.531</v>
       </c>
       <c r="R25" t="n">
-        <v>4.52</v>
+        <v>4.566</v>
       </c>
       <c r="S25" t="n">
-        <v>4.591</v>
+        <v>4.636</v>
       </c>
       <c r="T25" t="n">
-        <v>4.534</v>
+        <v>4.584</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.208</v>
+        <v>3.22</v>
       </c>
       <c r="G26" t="n">
-        <v>3.426</v>
+        <v>3.438</v>
       </c>
       <c r="H26" t="n">
-        <v>3.775</v>
+        <v>3.786</v>
       </c>
       <c r="I26" t="n">
-        <v>4.018</v>
+        <v>4.016</v>
       </c>
       <c r="J26" t="n">
-        <v>4.445</v>
+        <v>4.464</v>
       </c>
       <c r="K26" t="n">
-        <v>4.864</v>
+        <v>4.887</v>
       </c>
       <c r="L26" t="n">
-        <v>4.942</v>
+        <v>4.975</v>
       </c>
       <c r="M26" t="n">
-        <v>5.092</v>
+        <v>5.124</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.392</v>
+        <v>5.403</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.007</v>
+        <v>3.022</v>
       </c>
       <c r="G27" t="n">
-        <v>3.185</v>
+        <v>3.2</v>
       </c>
       <c r="H27" t="n">
-        <v>3.458</v>
+        <v>3.475</v>
       </c>
       <c r="I27" t="n">
-        <v>3.678</v>
+        <v>3.676</v>
       </c>
       <c r="J27" t="n">
-        <v>3.981</v>
+        <v>4.001</v>
       </c>
       <c r="K27" t="n">
-        <v>4.186</v>
+        <v>4.205</v>
       </c>
       <c r="L27" t="n">
-        <v>4.209</v>
+        <v>4.241</v>
       </c>
       <c r="M27" t="n">
-        <v>4.316</v>
+        <v>4.347</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.494</v>
+        <v>4.506</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.11</v>
+        <v>3.125</v>
       </c>
       <c r="G28" t="n">
-        <v>3.296</v>
+        <v>3.311</v>
       </c>
       <c r="H28" t="n">
-        <v>3.584</v>
+        <v>3.601</v>
       </c>
       <c r="I28" t="n">
-        <v>3.815</v>
+        <v>3.813</v>
       </c>
       <c r="J28" t="n">
-        <v>4.154</v>
+        <v>4.174</v>
       </c>
       <c r="K28" t="n">
-        <v>4.378</v>
+        <v>4.398</v>
       </c>
       <c r="L28" t="n">
-        <v>4.412</v>
+        <v>4.444</v>
       </c>
       <c r="M28" t="n">
-        <v>4.528</v>
+        <v>4.559</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.786</v>
+        <v>4.798</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.956</v>
+        <v>2.971</v>
       </c>
       <c r="G29" t="n">
-        <v>3.131</v>
+        <v>3.146</v>
       </c>
       <c r="H29" t="n">
-        <v>3.395</v>
+        <v>3.412</v>
       </c>
       <c r="I29" t="n">
-        <v>3.603</v>
+        <v>3.601</v>
       </c>
       <c r="J29" t="n">
-        <v>3.893</v>
+        <v>3.914</v>
       </c>
       <c r="K29" t="n">
-        <v>4.081</v>
+        <v>4.101</v>
       </c>
       <c r="L29" t="n">
-        <v>4.095</v>
+        <v>4.126</v>
       </c>
       <c r="M29" t="n">
-        <v>4.179</v>
+        <v>4.21</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.365</v>
+        <v>4.378</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.244</v>
+        <v>3.255</v>
       </c>
       <c r="G30" t="n">
-        <v>3.396</v>
+        <v>3.407</v>
       </c>
       <c r="H30" t="n">
-        <v>3.705</v>
+        <v>3.715</v>
       </c>
       <c r="I30" t="n">
-        <v>3.94</v>
+        <v>3.935</v>
       </c>
       <c r="J30" t="n">
-        <v>4.306</v>
+        <v>4.325</v>
       </c>
       <c r="K30" t="n">
-        <v>4.662</v>
+        <v>4.686</v>
       </c>
       <c r="L30" t="n">
-        <v>4.716</v>
+        <v>4.749</v>
       </c>
       <c r="M30" t="n">
-        <v>4.856</v>
+        <v>4.887</v>
       </c>
       <c r="N30" t="n">
-        <v>5.014</v>
+        <v>5.044</v>
       </c>
       <c r="O30" t="n">
-        <v>5.342</v>
+        <v>5.353</v>
       </c>
       <c r="P30" t="n">
-        <v>5.555</v>
+        <v>5.586</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.322</v>
+        <v>6.372</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.573</v>
+        <v>3.584</v>
       </c>
       <c r="G31" t="n">
-        <v>3.761</v>
+        <v>3.772</v>
       </c>
       <c r="H31" t="n">
-        <v>4.121</v>
+        <v>4.131</v>
       </c>
       <c r="I31" t="n">
-        <v>4.369</v>
+        <v>4.364</v>
       </c>
       <c r="J31" t="n">
-        <v>4.797</v>
+        <v>4.816</v>
       </c>
       <c r="K31" t="n">
-        <v>5.195</v>
+        <v>5.218</v>
       </c>
       <c r="L31" t="n">
-        <v>5.329</v>
+        <v>5.362</v>
       </c>
       <c r="M31" t="n">
-        <v>5.587</v>
+        <v>5.617</v>
       </c>
       <c r="N31" t="n">
-        <v>5.873</v>
+        <v>5.903</v>
       </c>
       <c r="O31" t="n">
-        <v>6.378</v>
+        <v>6.389</v>
       </c>
       <c r="P31" t="n">
-        <v>6.544</v>
+        <v>6.575</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.295</v>
+        <v>7.345</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.343</v>
+        <v>3.354</v>
       </c>
       <c r="G32" t="n">
-        <v>3.513</v>
+        <v>3.524</v>
       </c>
       <c r="H32" t="n">
-        <v>3.849</v>
+        <v>3.859</v>
       </c>
       <c r="I32" t="n">
-        <v>4.099</v>
+        <v>4.093</v>
       </c>
       <c r="J32" t="n">
-        <v>4.484</v>
+        <v>4.503</v>
       </c>
       <c r="K32" t="n">
-        <v>4.847</v>
+        <v>4.871</v>
       </c>
       <c r="L32" t="n">
-        <v>4.92</v>
+        <v>4.953</v>
       </c>
       <c r="M32" t="n">
-        <v>5.129</v>
+        <v>5.159</v>
       </c>
       <c r="N32" t="n">
-        <v>5.374</v>
+        <v>5.404</v>
       </c>
       <c r="O32" t="n">
-        <v>5.787</v>
+        <v>5.798</v>
       </c>
       <c r="P32" t="n">
-        <v>6.015</v>
+        <v>6.046</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.783</v>
+        <v>6.833</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.109</v>
+        <v>3.12</v>
       </c>
       <c r="G33" t="n">
-        <v>3.261</v>
+        <v>3.272</v>
       </c>
       <c r="H33" t="n">
-        <v>3.523</v>
+        <v>3.533</v>
       </c>
       <c r="I33" t="n">
-        <v>3.726</v>
+        <v>3.721</v>
       </c>
       <c r="J33" t="n">
-        <v>4.013</v>
+        <v>4.031</v>
       </c>
       <c r="K33" t="n">
-        <v>4.305</v>
+        <v>4.328</v>
       </c>
       <c r="L33" t="n">
-        <v>4.322</v>
+        <v>4.355</v>
       </c>
       <c r="M33" t="n">
-        <v>4.385</v>
+        <v>4.416</v>
       </c>
       <c r="N33" t="n">
-        <v>4.403</v>
+        <v>4.433</v>
       </c>
       <c r="O33" t="n">
-        <v>4.496</v>
+        <v>4.507</v>
       </c>
       <c r="P33" t="n">
-        <v>4.588</v>
+        <v>4.619</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.038</v>
+        <v>5.088</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.169</v>
+        <v>3.18</v>
       </c>
       <c r="G34" t="n">
-        <v>3.314</v>
+        <v>3.325</v>
       </c>
       <c r="H34" t="n">
-        <v>3.585</v>
+        <v>3.595</v>
       </c>
       <c r="I34" t="n">
-        <v>3.794</v>
+        <v>3.789</v>
       </c>
       <c r="J34" t="n">
-        <v>4.085</v>
+        <v>4.103</v>
       </c>
       <c r="K34" t="n">
-        <v>4.381</v>
+        <v>4.404</v>
       </c>
       <c r="L34" t="n">
-        <v>4.4</v>
+        <v>4.433</v>
       </c>
       <c r="M34" t="n">
-        <v>4.476</v>
+        <v>4.507</v>
       </c>
       <c r="N34" t="n">
-        <v>4.507</v>
+        <v>4.537</v>
       </c>
       <c r="O34" t="n">
-        <v>4.665</v>
+        <v>4.676</v>
       </c>
       <c r="P34" t="n">
-        <v>4.882</v>
+        <v>4.913</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.739</v>
+        <v>5.789</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.143</v>
+        <v>3.154</v>
       </c>
       <c r="G35" t="n">
-        <v>3.288</v>
+        <v>3.299</v>
       </c>
       <c r="H35" t="n">
-        <v>3.553</v>
+        <v>3.563</v>
       </c>
       <c r="I35" t="n">
-        <v>3.76</v>
+        <v>3.755</v>
       </c>
       <c r="J35" t="n">
-        <v>4.053</v>
+        <v>4.071</v>
       </c>
       <c r="K35" t="n">
-        <v>4.335</v>
+        <v>4.358</v>
       </c>
       <c r="L35" t="n">
-        <v>4.356</v>
+        <v>4.389</v>
       </c>
       <c r="M35" t="n">
-        <v>4.423</v>
+        <v>4.453</v>
       </c>
       <c r="N35" t="n">
-        <v>4.444</v>
+        <v>4.474</v>
       </c>
       <c r="O35" t="n">
-        <v>4.562</v>
+        <v>4.573</v>
       </c>
       <c r="P35" t="n">
-        <v>4.685</v>
+        <v>4.715</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.375</v>
+        <v>5.425</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.033</v>
+        <v>3.043</v>
       </c>
       <c r="G36" t="n">
-        <v>3.173</v>
+        <v>3.183</v>
       </c>
       <c r="H36" t="n">
-        <v>3.429</v>
+        <v>3.44</v>
       </c>
       <c r="I36" t="n">
-        <v>3.635</v>
+        <v>3.632</v>
       </c>
       <c r="J36" t="n">
-        <v>3.948</v>
+        <v>3.968</v>
       </c>
       <c r="K36" t="n">
-        <v>4.23</v>
+        <v>4.254</v>
       </c>
       <c r="L36" t="n">
-        <v>4.246</v>
+        <v>4.279</v>
       </c>
       <c r="M36" t="n">
-        <v>4.288</v>
+        <v>4.319</v>
       </c>
       <c r="N36" t="n">
-        <v>4.307</v>
+        <v>4.337</v>
       </c>
       <c r="O36" t="n">
-        <v>4.404</v>
+        <v>4.415</v>
       </c>
       <c r="P36" t="n">
-        <v>4.486</v>
+        <v>4.517</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.755</v>
+        <v>4.805</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.916</v>
+        <v>3.927</v>
       </c>
       <c r="G37" t="n">
-        <v>4.455</v>
+        <v>4.465</v>
       </c>
       <c r="H37" t="n">
-        <v>5.093</v>
+        <v>5.103</v>
       </c>
       <c r="I37" t="n">
-        <v>5.43</v>
+        <v>5.425</v>
       </c>
       <c r="J37" t="n">
-        <v>6.286</v>
+        <v>6.305</v>
       </c>
       <c r="K37" t="n">
-        <v>7.234</v>
+        <v>7.258</v>
       </c>
       <c r="L37" t="n">
-        <v>7.529</v>
+        <v>7.562</v>
       </c>
       <c r="M37" t="n">
-        <v>7.859</v>
+        <v>7.889</v>
       </c>
       <c r="N37" t="n">
-        <v>8.029</v>
+        <v>8.058999999999999</v>
       </c>
       <c r="O37" t="n">
-        <v>8.257</v>
+        <v>8.268000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.345000000000001</v>
+        <v>8.375999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.785</v>
+        <v>8.835000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.978</v>
+        <v>4.989</v>
       </c>
       <c r="G38" t="n">
-        <v>5.77</v>
+        <v>5.781</v>
       </c>
       <c r="H38" t="n">
-        <v>6.62</v>
+        <v>6.63</v>
       </c>
       <c r="I38" t="n">
-        <v>7.114</v>
+        <v>7.109</v>
       </c>
       <c r="J38" t="n">
-        <v>8.23</v>
+        <v>8.249000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.358000000000001</v>
+        <v>9.382</v>
       </c>
       <c r="L38" t="n">
-        <v>9.811999999999999</v>
+        <v>9.845000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>10.27</v>
+        <v>10.301</v>
       </c>
       <c r="N38" t="n">
-        <v>10.448</v>
+        <v>10.478</v>
       </c>
       <c r="O38" t="n">
-        <v>10.657</v>
+        <v>10.668</v>
       </c>
       <c r="P38" t="n">
-        <v>10.743</v>
+        <v>10.774</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.236</v>
+        <v>11.286</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.298</v>
+        <v>4.309</v>
       </c>
       <c r="G39" t="n">
-        <v>4.968</v>
+        <v>4.979</v>
       </c>
       <c r="H39" t="n">
-        <v>5.685</v>
+        <v>5.695</v>
       </c>
       <c r="I39" t="n">
-        <v>6.118</v>
+        <v>6.113</v>
       </c>
       <c r="J39" t="n">
-        <v>7.103</v>
+        <v>7.122</v>
       </c>
       <c r="K39" t="n">
-        <v>8.19</v>
+        <v>8.214</v>
       </c>
       <c r="L39" t="n">
-        <v>8.568</v>
+        <v>8.601000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.907</v>
+        <v>8.936999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>9.074999999999999</v>
+        <v>9.105</v>
       </c>
       <c r="O39" t="n">
-        <v>9.308</v>
+        <v>9.318</v>
       </c>
       <c r="P39" t="n">
-        <v>9.398</v>
+        <v>9.428000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.881</v>
+        <v>9.930999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.436</v>
+        <v>3.447</v>
       </c>
       <c r="G40" t="n">
-        <v>3.634</v>
+        <v>3.645</v>
       </c>
       <c r="H40" t="n">
-        <v>3.964</v>
+        <v>3.974</v>
       </c>
       <c r="I40" t="n">
-        <v>4.213</v>
+        <v>4.208</v>
       </c>
       <c r="J40" t="n">
-        <v>4.597</v>
+        <v>4.616</v>
       </c>
       <c r="K40" t="n">
-        <v>4.968</v>
+        <v>4.992</v>
       </c>
       <c r="L40" t="n">
-        <v>5.041</v>
+        <v>5.074</v>
       </c>
       <c r="M40" t="n">
-        <v>5.199</v>
+        <v>5.229</v>
       </c>
       <c r="N40" t="n">
-        <v>5.371</v>
+        <v>5.401</v>
       </c>
       <c r="O40" t="n">
-        <v>5.721</v>
+        <v>5.732</v>
       </c>
       <c r="P40" t="n">
-        <v>5.977</v>
+        <v>6.007</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.773</v>
+        <v>6.823</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.822</v>
+        <v>3.833</v>
       </c>
       <c r="G41" t="n">
-        <v>4.063</v>
+        <v>4.074</v>
       </c>
       <c r="H41" t="n">
-        <v>4.45</v>
+        <v>4.46</v>
       </c>
       <c r="I41" t="n">
-        <v>4.717</v>
+        <v>4.712</v>
       </c>
       <c r="J41" t="n">
-        <v>5.152</v>
+        <v>5.171</v>
       </c>
       <c r="K41" t="n">
-        <v>5.568</v>
+        <v>5.592</v>
       </c>
       <c r="L41" t="n">
-        <v>5.719</v>
+        <v>5.752</v>
       </c>
       <c r="M41" t="n">
-        <v>6.002</v>
+        <v>6.032</v>
       </c>
       <c r="N41" t="n">
-        <v>6.302</v>
+        <v>6.332</v>
       </c>
       <c r="O41" t="n">
-        <v>6.836</v>
+        <v>6.847</v>
       </c>
       <c r="P41" t="n">
-        <v>7.036</v>
+        <v>7.067</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.82</v>
+        <v>7.87</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.557</v>
+        <v>3.568</v>
       </c>
       <c r="G42" t="n">
-        <v>3.783</v>
+        <v>3.794</v>
       </c>
       <c r="H42" t="n">
-        <v>4.14</v>
+        <v>4.15</v>
       </c>
       <c r="I42" t="n">
-        <v>4.402</v>
+        <v>4.397</v>
       </c>
       <c r="J42" t="n">
-        <v>4.8</v>
+        <v>4.819</v>
       </c>
       <c r="K42" t="n">
-        <v>5.189</v>
+        <v>5.213</v>
       </c>
       <c r="L42" t="n">
-        <v>5.277</v>
+        <v>5.31</v>
       </c>
       <c r="M42" t="n">
-        <v>5.506</v>
+        <v>5.537</v>
       </c>
       <c r="N42" t="n">
-        <v>5.786</v>
+        <v>5.816</v>
       </c>
       <c r="O42" t="n">
-        <v>6.213</v>
+        <v>6.224</v>
       </c>
       <c r="P42" t="n">
-        <v>6.479</v>
+        <v>6.51</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.285</v>
+        <v>7.335</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.257</v>
+        <v>3.268</v>
       </c>
       <c r="G43" t="n">
-        <v>3.443</v>
+        <v>3.454</v>
       </c>
       <c r="H43" t="n">
-        <v>3.724</v>
+        <v>3.734</v>
       </c>
       <c r="I43" t="n">
-        <v>3.934</v>
+        <v>3.929</v>
       </c>
       <c r="J43" t="n">
-        <v>4.24</v>
+        <v>4.258</v>
       </c>
       <c r="K43" t="n">
-        <v>4.537</v>
+        <v>4.559</v>
       </c>
       <c r="L43" t="n">
-        <v>4.564</v>
+        <v>4.597</v>
       </c>
       <c r="M43" t="n">
-        <v>4.641</v>
+        <v>4.671</v>
       </c>
       <c r="N43" t="n">
-        <v>4.672</v>
+        <v>4.702</v>
       </c>
       <c r="O43" t="n">
-        <v>4.809</v>
+        <v>4.82</v>
       </c>
       <c r="P43" t="n">
-        <v>4.953</v>
+        <v>4.984</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.649</v>
+        <v>5.699</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.111</v>
+        <v>3.121</v>
       </c>
       <c r="G44" t="n">
-        <v>3.282</v>
+        <v>3.292</v>
       </c>
       <c r="H44" t="n">
-        <v>3.553</v>
+        <v>3.563</v>
       </c>
       <c r="I44" t="n">
-        <v>3.762</v>
+        <v>3.759</v>
       </c>
       <c r="J44" t="n">
-        <v>4.088</v>
+        <v>4.108</v>
       </c>
       <c r="K44" t="n">
-        <v>4.381</v>
+        <v>4.404</v>
       </c>
       <c r="L44" t="n">
-        <v>4.407</v>
+        <v>4.44</v>
       </c>
       <c r="M44" t="n">
-        <v>4.459</v>
+        <v>4.489</v>
       </c>
       <c r="N44" t="n">
-        <v>4.489</v>
+        <v>4.519</v>
       </c>
       <c r="O44" t="n">
-        <v>4.605</v>
+        <v>4.616</v>
       </c>
       <c r="P44" t="n">
-        <v>4.716</v>
+        <v>4.747</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.019</v>
+        <v>5.069</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-12 ~ 2026-06-12
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.423</v>
+        <v>3.438</v>
       </c>
       <c r="G2" t="n">
-        <v>3.735</v>
+        <v>3.75</v>
       </c>
       <c r="H2" t="n">
-        <v>4.026</v>
+        <v>4.029</v>
       </c>
       <c r="I2" t="n">
-        <v>4.198</v>
+        <v>4.172</v>
       </c>
       <c r="J2" t="n">
-        <v>4.536</v>
+        <v>4.486</v>
       </c>
       <c r="K2" t="n">
-        <v>4.92</v>
+        <v>4.853</v>
       </c>
       <c r="L2" t="n">
-        <v>5.096</v>
+        <v>5.028</v>
       </c>
       <c r="M2" t="n">
-        <v>5.345</v>
+        <v>5.253</v>
       </c>
       <c r="N2" t="n">
-        <v>5.606</v>
+        <v>5.516</v>
       </c>
       <c r="O2" t="n">
-        <v>5.87</v>
+        <v>5.762</v>
       </c>
       <c r="P2" t="n">
-        <v>6.107</v>
+        <v>5.999</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.772</v>
+        <v>6.662</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.445</v>
+        <v>4.46</v>
       </c>
       <c r="G3" t="n">
-        <v>4.938</v>
+        <v>4.953</v>
       </c>
       <c r="H3" t="n">
-        <v>5.262</v>
+        <v>5.265</v>
       </c>
       <c r="I3" t="n">
-        <v>5.427</v>
+        <v>5.401</v>
       </c>
       <c r="J3" t="n">
-        <v>5.781</v>
+        <v>5.732</v>
       </c>
       <c r="K3" t="n">
-        <v>6.237</v>
+        <v>6.169</v>
       </c>
       <c r="L3" t="n">
-        <v>6.482</v>
+        <v>6.413</v>
       </c>
       <c r="M3" t="n">
-        <v>6.762</v>
+        <v>6.67</v>
       </c>
       <c r="N3" t="n">
-        <v>6.965</v>
+        <v>6.875</v>
       </c>
       <c r="O3" t="n">
-        <v>7.18</v>
+        <v>7.073</v>
       </c>
       <c r="P3" t="n">
-        <v>7.285</v>
+        <v>7.178</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.838</v>
+        <v>7.728</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.937</v>
+        <v>3.952</v>
       </c>
       <c r="G4" t="n">
-        <v>4.319</v>
+        <v>4.334</v>
       </c>
       <c r="H4" t="n">
-        <v>4.671</v>
+        <v>4.674</v>
       </c>
       <c r="I4" t="n">
-        <v>4.869</v>
+        <v>4.843</v>
       </c>
       <c r="J4" t="n">
-        <v>5.225</v>
+        <v>5.175</v>
       </c>
       <c r="K4" t="n">
-        <v>5.675</v>
+        <v>5.607</v>
       </c>
       <c r="L4" t="n">
-        <v>5.851</v>
+        <v>5.782</v>
       </c>
       <c r="M4" t="n">
-        <v>6.12</v>
+        <v>6.028</v>
       </c>
       <c r="N4" t="n">
-        <v>6.293</v>
+        <v>6.204</v>
       </c>
       <c r="O4" t="n">
-        <v>6.531</v>
+        <v>6.424</v>
       </c>
       <c r="P4" t="n">
-        <v>6.638</v>
+        <v>6.53</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.193</v>
+        <v>7.083</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.121</v>
+        <v>3.136</v>
       </c>
       <c r="G5" t="n">
-        <v>3.278</v>
+        <v>3.293</v>
       </c>
       <c r="H5" t="n">
-        <v>3.533</v>
+        <v>3.536</v>
       </c>
       <c r="I5" t="n">
-        <v>3.77</v>
+        <v>3.744</v>
       </c>
       <c r="J5" t="n">
-        <v>4.093</v>
+        <v>4.044</v>
       </c>
       <c r="K5" t="n">
-        <v>4.324</v>
+        <v>4.256</v>
       </c>
       <c r="L5" t="n">
-        <v>4.344</v>
+        <v>4.275</v>
       </c>
       <c r="M5" t="n">
-        <v>4.403</v>
+        <v>4.311</v>
       </c>
       <c r="N5" t="n">
-        <v>4.418</v>
+        <v>4.328</v>
       </c>
       <c r="O5" t="n">
-        <v>4.469</v>
+        <v>4.362</v>
       </c>
       <c r="P5" t="n">
-        <v>4.776</v>
+        <v>4.668</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.684</v>
+        <v>5.574</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.162</v>
+        <v>3.177</v>
       </c>
       <c r="G6" t="n">
-        <v>3.333</v>
+        <v>3.348</v>
       </c>
       <c r="H6" t="n">
-        <v>3.603</v>
+        <v>3.606</v>
       </c>
       <c r="I6" t="n">
-        <v>3.853</v>
+        <v>3.827</v>
       </c>
       <c r="J6" t="n">
-        <v>4.184</v>
+        <v>4.135</v>
       </c>
       <c r="K6" t="n">
-        <v>4.437</v>
+        <v>4.369</v>
       </c>
       <c r="L6" t="n">
-        <v>4.463</v>
+        <v>4.394</v>
       </c>
       <c r="M6" t="n">
-        <v>4.559</v>
+        <v>4.467</v>
       </c>
       <c r="N6" t="n">
-        <v>4.585</v>
+        <v>4.496</v>
       </c>
       <c r="O6" t="n">
-        <v>4.736</v>
+        <v>4.628</v>
       </c>
       <c r="P6" t="n">
-        <v>5.208</v>
+        <v>5.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.08</v>
+        <v>5.97</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.142</v>
+        <v>3.157</v>
       </c>
       <c r="G7" t="n">
-        <v>3.297</v>
+        <v>3.312</v>
       </c>
       <c r="H7" t="n">
-        <v>3.549</v>
+        <v>3.552</v>
       </c>
       <c r="I7" t="n">
-        <v>3.79</v>
+        <v>3.764</v>
       </c>
       <c r="J7" t="n">
-        <v>4.117</v>
+        <v>4.067</v>
       </c>
       <c r="K7" t="n">
-        <v>4.351</v>
+        <v>4.283</v>
       </c>
       <c r="L7" t="n">
+        <v>4.302</v>
+      </c>
+      <c r="M7" t="n">
         <v>4.371</v>
       </c>
-      <c r="M7" t="n">
-        <v>4.463</v>
-      </c>
       <c r="N7" t="n">
-        <v>4.477</v>
+        <v>4.388</v>
       </c>
       <c r="O7" t="n">
-        <v>4.633</v>
+        <v>4.526</v>
       </c>
       <c r="P7" t="n">
-        <v>4.992</v>
+        <v>4.884</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.848</v>
+        <v>5.738</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.557</v>
+        <v>5.572</v>
       </c>
       <c r="G8" t="n">
-        <v>6.237</v>
+        <v>6.252</v>
       </c>
       <c r="H8" t="n">
-        <v>6.71</v>
+        <v>6.713</v>
       </c>
       <c r="I8" t="n">
-        <v>6.953</v>
+        <v>6.927</v>
       </c>
       <c r="J8" t="n">
-        <v>7.374</v>
+        <v>7.325</v>
       </c>
       <c r="K8" t="n">
-        <v>8.109999999999999</v>
+        <v>8.042</v>
       </c>
       <c r="L8" t="n">
-        <v>8.44</v>
+        <v>8.371</v>
       </c>
       <c r="M8" t="n">
-        <v>8.752000000000001</v>
+        <v>8.66</v>
       </c>
       <c r="N8" t="n">
-        <v>8.888999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.189</v>
+        <v>9.082000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.398999999999999</v>
+        <v>9.291</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.149</v>
+        <v>10.039</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.755</v>
+        <v>2.752</v>
       </c>
       <c r="G9" t="n">
-        <v>2.99</v>
+        <v>2.984</v>
       </c>
       <c r="H9" t="n">
-        <v>3.232</v>
+        <v>3.214</v>
       </c>
       <c r="I9" t="n">
-        <v>3.393</v>
+        <v>3.382</v>
       </c>
       <c r="J9" t="n">
-        <v>3.615</v>
+        <v>3.536</v>
       </c>
       <c r="K9" t="n">
-        <v>3.744</v>
+        <v>3.647</v>
       </c>
       <c r="L9" t="n">
-        <v>3.858</v>
+        <v>3.764</v>
       </c>
       <c r="M9" t="n">
-        <v>3.906</v>
+        <v>3.79</v>
       </c>
       <c r="N9" t="n">
-        <v>4.011</v>
+        <v>3.905</v>
       </c>
       <c r="O9" t="n">
-        <v>4.08</v>
+        <v>3.955</v>
       </c>
       <c r="P9" t="n">
-        <v>4.222</v>
+        <v>4.101</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.315</v>
+        <v>4.195</v>
       </c>
       <c r="R9" t="n">
-        <v>4.361</v>
+        <v>4.244</v>
       </c>
       <c r="S9" t="n">
-        <v>4.405</v>
+        <v>4.293</v>
       </c>
       <c r="T9" t="n">
-        <v>4.36</v>
+        <v>4.22</v>
       </c>
       <c r="U9" t="n">
-        <v>4.323</v>
+        <v>4.133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.762</v>
+        <v>2.759</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>2.994</v>
       </c>
       <c r="H10" t="n">
-        <v>3.235</v>
+        <v>3.217</v>
       </c>
       <c r="I10" t="n">
-        <v>3.396</v>
+        <v>3.385</v>
       </c>
       <c r="J10" t="n">
-        <v>3.631</v>
+        <v>3.552</v>
       </c>
       <c r="K10" t="n">
-        <v>3.78</v>
+        <v>3.684</v>
       </c>
       <c r="L10" t="n">
-        <v>3.871</v>
+        <v>3.776</v>
       </c>
       <c r="M10" t="n">
-        <v>3.97</v>
+        <v>3.852</v>
       </c>
       <c r="N10" t="n">
-        <v>4.036</v>
+        <v>3.93</v>
       </c>
       <c r="O10" t="n">
-        <v>4.31</v>
+        <v>4.2</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.566</v>
+        <v>2.563</v>
       </c>
       <c r="G11" t="n">
-        <v>2.805</v>
+        <v>2.797</v>
       </c>
       <c r="H11" t="n">
-        <v>3.06</v>
+        <v>3.041</v>
       </c>
       <c r="I11" t="n">
-        <v>3.2</v>
+        <v>3.19</v>
       </c>
       <c r="J11" t="n">
-        <v>3.424</v>
+        <v>3.346</v>
       </c>
       <c r="K11" t="n">
-        <v>3.565</v>
+        <v>3.469</v>
       </c>
       <c r="L11" t="n">
-        <v>3.668</v>
+        <v>3.573</v>
       </c>
       <c r="M11" t="n">
-        <v>3.778</v>
+        <v>3.66</v>
       </c>
       <c r="N11" t="n">
-        <v>3.843</v>
+        <v>3.736</v>
       </c>
       <c r="O11" t="n">
-        <v>4.076</v>
+        <v>3.966</v>
       </c>
       <c r="P11" t="n">
-        <v>4.168</v>
+        <v>4.047</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.513</v>
+        <v>4.393</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.365</v>
+        <v>3.372</v>
       </c>
       <c r="G12" t="n">
-        <v>3.641</v>
+        <v>3.651</v>
       </c>
       <c r="H12" t="n">
-        <v>3.937</v>
+        <v>3.934</v>
       </c>
       <c r="I12" t="n">
-        <v>4.179</v>
+        <v>4.153</v>
       </c>
       <c r="J12" t="n">
-        <v>4.531</v>
+        <v>4.479</v>
       </c>
       <c r="K12" t="n">
-        <v>4.707</v>
+        <v>4.638</v>
       </c>
       <c r="L12" t="n">
-        <v>4.749</v>
+        <v>4.676</v>
       </c>
       <c r="M12" t="n">
-        <v>4.875</v>
+        <v>4.779</v>
       </c>
       <c r="N12" t="n">
-        <v>4.929</v>
+        <v>4.84</v>
       </c>
       <c r="O12" t="n">
-        <v>5.09</v>
+        <v>4.982</v>
       </c>
       <c r="P12" t="n">
-        <v>5.248</v>
+        <v>5.139</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.627</v>
+        <v>5.516</v>
       </c>
       <c r="R12" t="n">
-        <v>5.852</v>
+        <v>5.74</v>
       </c>
       <c r="S12" t="n">
-        <v>6.109</v>
+        <v>6.002</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.118</v>
+        <v>3.125</v>
       </c>
       <c r="G13" t="n">
-        <v>3.331</v>
+        <v>3.341</v>
       </c>
       <c r="H13" t="n">
-        <v>3.604</v>
+        <v>3.601</v>
       </c>
       <c r="I13" t="n">
-        <v>3.826</v>
+        <v>3.8</v>
       </c>
       <c r="J13" t="n">
-        <v>4.168</v>
+        <v>4.116</v>
       </c>
       <c r="K13" t="n">
-        <v>4.34</v>
+        <v>4.271</v>
       </c>
       <c r="L13" t="n">
-        <v>4.388</v>
+        <v>4.316</v>
       </c>
       <c r="M13" t="n">
-        <v>4.503</v>
+        <v>4.406</v>
       </c>
       <c r="N13" t="n">
-        <v>4.557</v>
+        <v>4.468</v>
       </c>
       <c r="O13" t="n">
-        <v>4.718</v>
+        <v>4.61</v>
       </c>
       <c r="P13" t="n">
-        <v>4.84</v>
+        <v>4.73</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.148</v>
+        <v>5.037</v>
       </c>
       <c r="R13" t="n">
-        <v>5.401</v>
+        <v>5.29</v>
       </c>
       <c r="S13" t="n">
-        <v>5.671</v>
+        <v>5.564</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.936</v>
+        <v>2.943</v>
       </c>
       <c r="G14" t="n">
-        <v>3.137</v>
+        <v>3.144</v>
       </c>
       <c r="H14" t="n">
-        <v>3.407</v>
+        <v>3.404</v>
       </c>
       <c r="I14" t="n">
-        <v>3.611</v>
+        <v>3.585</v>
       </c>
       <c r="J14" t="n">
-        <v>3.909</v>
+        <v>3.857</v>
       </c>
       <c r="K14" t="n">
-        <v>4.029</v>
+        <v>3.96</v>
       </c>
       <c r="L14" t="n">
-        <v>4.061</v>
+        <v>3.989</v>
       </c>
       <c r="M14" t="n">
-        <v>4.189</v>
+        <v>4.093</v>
       </c>
       <c r="N14" t="n">
-        <v>4.236</v>
+        <v>4.147</v>
       </c>
       <c r="O14" t="n">
-        <v>4.377</v>
+        <v>4.269</v>
       </c>
       <c r="P14" t="n">
-        <v>4.476</v>
+        <v>4.366</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.737</v>
+        <v>4.626</v>
       </c>
       <c r="R14" t="n">
-        <v>4.916</v>
+        <v>4.804</v>
       </c>
       <c r="S14" t="n">
-        <v>5.124</v>
+        <v>5.017</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.913</v>
+        <v>2.92</v>
       </c>
       <c r="G15" t="n">
-        <v>3.111</v>
+        <v>3.118</v>
       </c>
       <c r="H15" t="n">
-        <v>3.378</v>
+        <v>3.375</v>
       </c>
       <c r="I15" t="n">
-        <v>3.562</v>
+        <v>3.536</v>
       </c>
       <c r="J15" t="n">
-        <v>3.847</v>
+        <v>3.796</v>
       </c>
       <c r="K15" t="n">
-        <v>3.981</v>
+        <v>3.913</v>
       </c>
       <c r="L15" t="n">
-        <v>3.997</v>
+        <v>3.925</v>
       </c>
       <c r="M15" t="n">
-        <v>4.102</v>
+        <v>4.006</v>
       </c>
       <c r="N15" t="n">
-        <v>4.139</v>
+        <v>4.05</v>
       </c>
       <c r="O15" t="n">
-        <v>4.32</v>
+        <v>4.212</v>
       </c>
       <c r="P15" t="n">
-        <v>4.372</v>
+        <v>4.262</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.639</v>
+        <v>4.528</v>
       </c>
       <c r="R15" t="n">
-        <v>4.81</v>
+        <v>4.698</v>
       </c>
       <c r="S15" t="n">
-        <v>5.019</v>
+        <v>4.912</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.913</v>
+        <v>2.92</v>
       </c>
       <c r="G16" t="n">
-        <v>3.111</v>
+        <v>3.118</v>
       </c>
       <c r="H16" t="n">
-        <v>3.378</v>
+        <v>3.375</v>
       </c>
       <c r="I16" t="n">
-        <v>3.562</v>
+        <v>3.536</v>
       </c>
       <c r="J16" t="n">
-        <v>3.847</v>
+        <v>3.796</v>
       </c>
       <c r="K16" t="n">
-        <v>3.981</v>
+        <v>3.913</v>
       </c>
       <c r="L16" t="n">
-        <v>3.997</v>
+        <v>3.925</v>
       </c>
       <c r="M16" t="n">
-        <v>4.102</v>
+        <v>4.006</v>
       </c>
       <c r="N16" t="n">
-        <v>4.142</v>
+        <v>4.053</v>
       </c>
       <c r="O16" t="n">
-        <v>4.327</v>
+        <v>4.218</v>
       </c>
       <c r="P16" t="n">
-        <v>4.395</v>
+        <v>4.286</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.666</v>
+        <v>4.555</v>
       </c>
       <c r="R16" t="n">
-        <v>4.838</v>
+        <v>4.726</v>
       </c>
       <c r="S16" t="n">
-        <v>5.048</v>
+        <v>4.941</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.795</v>
+        <v>2.79</v>
       </c>
       <c r="G17" t="n">
-        <v>3.054</v>
+        <v>3.046</v>
       </c>
       <c r="H17" t="n">
-        <v>3.292</v>
+        <v>3.272</v>
       </c>
       <c r="I17" t="n">
-        <v>3.453</v>
+        <v>3.44</v>
       </c>
       <c r="J17" t="n">
-        <v>3.696</v>
+        <v>3.619</v>
       </c>
       <c r="K17" t="n">
-        <v>3.856</v>
+        <v>3.759</v>
       </c>
       <c r="L17" t="n">
-        <v>3.955</v>
+        <v>3.86</v>
       </c>
       <c r="M17" t="n">
-        <v>4.094</v>
+        <v>3.977</v>
       </c>
       <c r="N17" t="n">
-        <v>4.141</v>
+        <v>4.035</v>
       </c>
       <c r="O17" t="n">
-        <v>4.33</v>
+        <v>4.22</v>
       </c>
       <c r="P17" t="n">
-        <v>4.45</v>
+        <v>4.329</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.796</v>
+        <v>2.791</v>
       </c>
       <c r="G18" t="n">
-        <v>3.055</v>
+        <v>3.047</v>
       </c>
       <c r="H18" t="n">
-        <v>3.292</v>
+        <v>3.272</v>
       </c>
       <c r="I18" t="n">
-        <v>3.453</v>
+        <v>3.44</v>
       </c>
       <c r="J18" t="n">
-        <v>3.696</v>
+        <v>3.619</v>
       </c>
       <c r="K18" t="n">
-        <v>3.857</v>
+        <v>3.76</v>
       </c>
       <c r="L18" t="n">
-        <v>3.955</v>
+        <v>3.86</v>
       </c>
       <c r="M18" t="n">
-        <v>4.094</v>
+        <v>3.977</v>
       </c>
       <c r="N18" t="n">
-        <v>4.142</v>
+        <v>4.036</v>
       </c>
       <c r="O18" t="n">
-        <v>4.328</v>
+        <v>4.218</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.924</v>
+        <v>2.931</v>
       </c>
       <c r="G19" t="n">
-        <v>3.124</v>
+        <v>3.131</v>
       </c>
       <c r="H19" t="n">
-        <v>3.395</v>
+        <v>3.392</v>
       </c>
       <c r="I19" t="n">
-        <v>3.595</v>
+        <v>3.569</v>
       </c>
       <c r="J19" t="n">
-        <v>3.888</v>
+        <v>3.837</v>
       </c>
       <c r="K19" t="n">
-        <v>4.024</v>
+        <v>3.956</v>
       </c>
       <c r="L19" t="n">
-        <v>4.058</v>
+        <v>3.986</v>
       </c>
       <c r="M19" t="n">
-        <v>4.18</v>
+        <v>4.084</v>
       </c>
       <c r="N19" t="n">
-        <v>4.228</v>
+        <v>4.139</v>
       </c>
       <c r="O19" t="n">
-        <v>4.363</v>
+        <v>4.255</v>
       </c>
       <c r="P19" t="n">
-        <v>4.434</v>
+        <v>4.324</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.677</v>
+        <v>4.566</v>
       </c>
       <c r="R19" t="n">
-        <v>4.857</v>
+        <v>4.745</v>
       </c>
       <c r="S19" t="n">
-        <v>5.059</v>
+        <v>4.952</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.662</v>
+        <v>2.66</v>
       </c>
       <c r="G20" t="n">
-        <v>2.772</v>
+        <v>2.768</v>
       </c>
       <c r="H20" t="n">
-        <v>2.888</v>
+        <v>2.873</v>
       </c>
       <c r="I20" t="n">
-        <v>3.037</v>
+        <v>2.991</v>
       </c>
       <c r="J20" t="n">
-        <v>3.541</v>
+        <v>3.465</v>
       </c>
       <c r="K20" t="n">
-        <v>3.802</v>
+        <v>3.707</v>
       </c>
       <c r="L20" t="n">
-        <v>3.81</v>
+        <v>3.708</v>
       </c>
       <c r="M20" t="n">
-        <v>3.906</v>
+        <v>3.795</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.009</v>
+        <v>3.011</v>
       </c>
       <c r="G21" t="n">
-        <v>3.234</v>
+        <v>3.238</v>
       </c>
       <c r="H21" t="n">
-        <v>3.514</v>
+        <v>3.512</v>
       </c>
       <c r="I21" t="n">
-        <v>3.727</v>
+        <v>3.704</v>
       </c>
       <c r="J21" t="n">
-        <v>4.047</v>
+        <v>4.003</v>
       </c>
       <c r="K21" t="n">
-        <v>4.272</v>
+        <v>4.202</v>
       </c>
       <c r="L21" t="n">
-        <v>4.307</v>
+        <v>4.24</v>
       </c>
       <c r="M21" t="n">
-        <v>4.419</v>
+        <v>4.329</v>
       </c>
       <c r="N21" t="n">
+        <v>4.374</v>
+      </c>
+      <c r="O21" t="n">
         <v>4.46</v>
       </c>
-      <c r="O21" t="n">
-        <v>4.568</v>
-      </c>
       <c r="P21" t="n">
-        <v>4.694</v>
+        <v>4.581</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.833</v>
+        <v>4.719</v>
       </c>
       <c r="R21" t="n">
-        <v>4.908</v>
+        <v>4.797</v>
       </c>
       <c r="S21" t="n">
-        <v>5.011</v>
+        <v>4.905</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.955</v>
+        <v>2.957</v>
       </c>
       <c r="G22" t="n">
-        <v>3.179</v>
+        <v>3.183</v>
       </c>
       <c r="H22" t="n">
-        <v>3.446</v>
+        <v>3.444</v>
       </c>
       <c r="I22" t="n">
-        <v>3.646</v>
+        <v>3.623</v>
       </c>
       <c r="J22" t="n">
-        <v>3.932</v>
+        <v>3.888</v>
       </c>
       <c r="K22" t="n">
-        <v>4.153</v>
+        <v>4.084</v>
       </c>
       <c r="L22" t="n">
-        <v>4.174</v>
+        <v>4.107</v>
       </c>
       <c r="M22" t="n">
-        <v>4.29</v>
+        <v>4.2</v>
       </c>
       <c r="N22" t="n">
-        <v>4.334</v>
+        <v>4.248</v>
       </c>
       <c r="O22" t="n">
-        <v>4.439</v>
+        <v>4.331</v>
       </c>
       <c r="P22" t="n">
-        <v>4.557</v>
+        <v>4.444</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.692</v>
+        <v>4.578</v>
       </c>
       <c r="R22" t="n">
-        <v>4.757</v>
+        <v>4.646</v>
       </c>
       <c r="S22" t="n">
-        <v>4.857</v>
+        <v>4.751</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.903</v>
+        <v>2.905</v>
       </c>
       <c r="G23" t="n">
-        <v>3.133</v>
+        <v>3.137</v>
       </c>
       <c r="H23" t="n">
-        <v>3.387</v>
+        <v>3.385</v>
       </c>
       <c r="I23" t="n">
-        <v>3.594</v>
+        <v>3.571</v>
       </c>
       <c r="J23" t="n">
-        <v>3.872</v>
+        <v>3.828</v>
       </c>
       <c r="K23" t="n">
-        <v>4.053</v>
+        <v>3.984</v>
       </c>
       <c r="L23" t="n">
-        <v>4.072</v>
+        <v>4.005</v>
       </c>
       <c r="M23" t="n">
-        <v>4.182</v>
+        <v>4.092</v>
       </c>
       <c r="N23" t="n">
-        <v>4.228</v>
+        <v>4.142</v>
       </c>
       <c r="O23" t="n">
-        <v>4.315</v>
+        <v>4.207</v>
       </c>
       <c r="P23" t="n">
-        <v>4.42</v>
+        <v>4.307</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.497</v>
+        <v>4.383</v>
       </c>
       <c r="R23" t="n">
-        <v>4.542</v>
+        <v>4.431</v>
       </c>
       <c r="S23" t="n">
-        <v>4.613</v>
+        <v>4.507</v>
       </c>
       <c r="T23" t="n">
-        <v>4.566</v>
+        <v>4.433</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.839</v>
+        <v>2.841</v>
       </c>
       <c r="G24" t="n">
-        <v>3.044</v>
+        <v>3.048</v>
       </c>
       <c r="H24" t="n">
-        <v>3.284</v>
+        <v>3.282</v>
       </c>
       <c r="I24" t="n">
-        <v>3.532</v>
+        <v>3.509</v>
       </c>
       <c r="J24" t="n">
-        <v>3.766</v>
+        <v>3.721</v>
       </c>
       <c r="K24" t="n">
-        <v>3.936</v>
+        <v>3.867</v>
       </c>
       <c r="L24" t="n">
-        <v>3.953</v>
+        <v>3.886</v>
       </c>
       <c r="M24" t="n">
-        <v>4.04</v>
+        <v>3.95</v>
       </c>
       <c r="N24" t="n">
-        <v>4.102</v>
+        <v>4.016</v>
       </c>
       <c r="O24" t="n">
-        <v>4.315</v>
+        <v>4.205</v>
       </c>
       <c r="P24" t="n">
-        <v>4.36</v>
+        <v>4.246</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.423</v>
+        <v>4.309</v>
       </c>
       <c r="R24" t="n">
-        <v>4.464</v>
+        <v>4.353</v>
       </c>
       <c r="S24" t="n">
-        <v>4.528</v>
+        <v>4.422</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.898</v>
+        <v>2.9</v>
       </c>
       <c r="G25" t="n">
-        <v>3.133</v>
+        <v>3.137</v>
       </c>
       <c r="H25" t="n">
-        <v>3.39</v>
+        <v>3.388</v>
       </c>
       <c r="I25" t="n">
-        <v>3.603</v>
+        <v>3.579</v>
       </c>
       <c r="J25" t="n">
-        <v>3.887</v>
+        <v>3.843</v>
       </c>
       <c r="K25" t="n">
-        <v>4.085</v>
+        <v>4.015</v>
       </c>
       <c r="L25" t="n">
-        <v>4.103</v>
+        <v>4.035</v>
       </c>
       <c r="M25" t="n">
-        <v>4.213</v>
+        <v>4.123</v>
       </c>
       <c r="N25" t="n">
-        <v>4.255</v>
+        <v>4.169</v>
       </c>
       <c r="O25" t="n">
-        <v>4.343</v>
+        <v>4.235</v>
       </c>
       <c r="P25" t="n">
-        <v>4.442</v>
+        <v>4.328</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.531</v>
+        <v>4.417</v>
       </c>
       <c r="R25" t="n">
-        <v>4.566</v>
+        <v>4.455</v>
       </c>
       <c r="S25" t="n">
-        <v>4.636</v>
+        <v>4.53</v>
       </c>
       <c r="T25" t="n">
-        <v>4.584</v>
+        <v>4.451</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.22</v>
+        <v>3.224</v>
       </c>
       <c r="G26" t="n">
-        <v>3.438</v>
+        <v>3.44</v>
       </c>
       <c r="H26" t="n">
-        <v>3.786</v>
+        <v>3.777</v>
       </c>
       <c r="I26" t="n">
-        <v>4.016</v>
+        <v>3.983</v>
       </c>
       <c r="J26" t="n">
-        <v>4.464</v>
+        <v>4.409</v>
       </c>
       <c r="K26" t="n">
-        <v>4.887</v>
+        <v>4.816</v>
       </c>
       <c r="L26" t="n">
-        <v>4.975</v>
+        <v>4.9</v>
       </c>
       <c r="M26" t="n">
-        <v>5.124</v>
+        <v>5.025</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.403</v>
+        <v>5.293</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.022</v>
+        <v>3.027</v>
       </c>
       <c r="G27" t="n">
-        <v>3.2</v>
+        <v>3.205</v>
       </c>
       <c r="H27" t="n">
-        <v>3.475</v>
+        <v>3.468</v>
       </c>
       <c r="I27" t="n">
-        <v>3.676</v>
+        <v>3.649</v>
       </c>
       <c r="J27" t="n">
-        <v>4.001</v>
+        <v>3.947</v>
       </c>
       <c r="K27" t="n">
-        <v>4.205</v>
+        <v>4.137</v>
       </c>
       <c r="L27" t="n">
-        <v>4.241</v>
+        <v>4.166</v>
       </c>
       <c r="M27" t="n">
-        <v>4.347</v>
+        <v>4.249</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.506</v>
+        <v>4.398</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.125</v>
+        <v>3.13</v>
       </c>
       <c r="G28" t="n">
-        <v>3.311</v>
+        <v>3.316</v>
       </c>
       <c r="H28" t="n">
-        <v>3.601</v>
+        <v>3.594</v>
       </c>
       <c r="I28" t="n">
-        <v>3.813</v>
+        <v>3.786</v>
       </c>
       <c r="J28" t="n">
-        <v>4.174</v>
+        <v>4.12</v>
       </c>
       <c r="K28" t="n">
-        <v>4.398</v>
+        <v>4.329</v>
       </c>
       <c r="L28" t="n">
-        <v>4.444</v>
+        <v>4.369</v>
       </c>
       <c r="M28" t="n">
-        <v>4.559</v>
+        <v>4.461</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.798</v>
+        <v>4.69</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.971</v>
+        <v>2.976</v>
       </c>
       <c r="G29" t="n">
-        <v>3.146</v>
+        <v>3.151</v>
       </c>
       <c r="H29" t="n">
-        <v>3.412</v>
+        <v>3.405</v>
       </c>
       <c r="I29" t="n">
-        <v>3.601</v>
+        <v>3.574</v>
       </c>
       <c r="J29" t="n">
-        <v>3.914</v>
+        <v>3.859</v>
       </c>
       <c r="K29" t="n">
-        <v>4.101</v>
+        <v>4.032</v>
       </c>
       <c r="L29" t="n">
-        <v>4.126</v>
+        <v>4.052</v>
       </c>
       <c r="M29" t="n">
-        <v>4.21</v>
+        <v>4.112</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.378</v>
+        <v>4.27</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.255</v>
+        <v>3.257</v>
       </c>
       <c r="G30" t="n">
         <v>3.407</v>
       </c>
       <c r="H30" t="n">
-        <v>3.715</v>
+        <v>3.704</v>
       </c>
       <c r="I30" t="n">
-        <v>3.935</v>
+        <v>3.901</v>
       </c>
       <c r="J30" t="n">
-        <v>4.325</v>
+        <v>4.267</v>
       </c>
       <c r="K30" t="n">
-        <v>4.686</v>
+        <v>4.612</v>
       </c>
       <c r="L30" t="n">
-        <v>4.749</v>
+        <v>4.671</v>
       </c>
       <c r="M30" t="n">
-        <v>4.887</v>
+        <v>4.786</v>
       </c>
       <c r="N30" t="n">
-        <v>5.044</v>
+        <v>4.952</v>
       </c>
       <c r="O30" t="n">
-        <v>5.353</v>
+        <v>5.241</v>
       </c>
       <c r="P30" t="n">
-        <v>5.586</v>
+        <v>5.475</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.372</v>
+        <v>6.262</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.584</v>
+        <v>3.586</v>
       </c>
       <c r="G31" t="n">
-        <v>3.772</v>
+        <v>3.773</v>
       </c>
       <c r="H31" t="n">
-        <v>4.131</v>
+        <v>4.12</v>
       </c>
       <c r="I31" t="n">
-        <v>4.364</v>
+        <v>4.331</v>
       </c>
       <c r="J31" t="n">
-        <v>4.816</v>
+        <v>4.759</v>
       </c>
       <c r="K31" t="n">
-        <v>5.218</v>
+        <v>5.145</v>
       </c>
       <c r="L31" t="n">
-        <v>5.362</v>
+        <v>5.284</v>
       </c>
       <c r="M31" t="n">
-        <v>5.617</v>
+        <v>5.516</v>
       </c>
       <c r="N31" t="n">
-        <v>5.903</v>
+        <v>5.811</v>
       </c>
       <c r="O31" t="n">
-        <v>6.389</v>
+        <v>6.277</v>
       </c>
       <c r="P31" t="n">
-        <v>6.575</v>
+        <v>6.463</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.345</v>
+        <v>7.235</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.354</v>
+        <v>3.356</v>
       </c>
       <c r="G32" t="n">
-        <v>3.524</v>
+        <v>3.525</v>
       </c>
       <c r="H32" t="n">
-        <v>3.859</v>
+        <v>3.848</v>
       </c>
       <c r="I32" t="n">
-        <v>4.093</v>
+        <v>4.061</v>
       </c>
       <c r="J32" t="n">
-        <v>4.503</v>
+        <v>4.445</v>
       </c>
       <c r="K32" t="n">
-        <v>4.871</v>
+        <v>4.797</v>
       </c>
       <c r="L32" t="n">
-        <v>4.953</v>
+        <v>4.875</v>
       </c>
       <c r="M32" t="n">
-        <v>5.159</v>
+        <v>5.058</v>
       </c>
       <c r="N32" t="n">
-        <v>5.404</v>
+        <v>5.312</v>
       </c>
       <c r="O32" t="n">
-        <v>5.798</v>
+        <v>5.686</v>
       </c>
       <c r="P32" t="n">
-        <v>6.046</v>
+        <v>5.935</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.833</v>
+        <v>6.723</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.12</v>
+        <v>3.122</v>
       </c>
       <c r="G33" t="n">
         <v>3.272</v>
       </c>
       <c r="H33" t="n">
-        <v>3.533</v>
+        <v>3.522</v>
       </c>
       <c r="I33" t="n">
-        <v>3.721</v>
+        <v>3.688</v>
       </c>
       <c r="J33" t="n">
-        <v>4.031</v>
+        <v>3.974</v>
       </c>
       <c r="K33" t="n">
-        <v>4.328</v>
+        <v>4.254</v>
       </c>
       <c r="L33" t="n">
-        <v>4.355</v>
+        <v>4.277</v>
       </c>
       <c r="M33" t="n">
-        <v>4.416</v>
+        <v>4.315</v>
       </c>
       <c r="N33" t="n">
-        <v>4.433</v>
+        <v>4.341</v>
       </c>
       <c r="O33" t="n">
+        <v>4.395</v>
+      </c>
+      <c r="P33" t="n">
         <v>4.507</v>
       </c>
-      <c r="P33" t="n">
-        <v>4.619</v>
-      </c>
       <c r="Q33" t="n">
-        <v>5.088</v>
+        <v>4.978</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.18</v>
+        <v>3.182</v>
       </c>
       <c r="G34" t="n">
         <v>3.325</v>
       </c>
       <c r="H34" t="n">
-        <v>3.595</v>
+        <v>3.584</v>
       </c>
       <c r="I34" t="n">
-        <v>3.789</v>
+        <v>3.756</v>
       </c>
       <c r="J34" t="n">
-        <v>4.103</v>
+        <v>4.045</v>
       </c>
       <c r="K34" t="n">
-        <v>4.404</v>
+        <v>4.33</v>
       </c>
       <c r="L34" t="n">
-        <v>4.433</v>
+        <v>4.355</v>
       </c>
       <c r="M34" t="n">
-        <v>4.507</v>
+        <v>4.406</v>
       </c>
       <c r="N34" t="n">
-        <v>4.537</v>
+        <v>4.445</v>
       </c>
       <c r="O34" t="n">
-        <v>4.676</v>
+        <v>4.564</v>
       </c>
       <c r="P34" t="n">
-        <v>4.913</v>
+        <v>4.802</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.789</v>
+        <v>5.679</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.154</v>
+        <v>3.156</v>
       </c>
       <c r="G35" t="n">
         <v>3.299</v>
       </c>
       <c r="H35" t="n">
-        <v>3.563</v>
+        <v>3.552</v>
       </c>
       <c r="I35" t="n">
-        <v>3.755</v>
+        <v>3.722</v>
       </c>
       <c r="J35" t="n">
-        <v>4.071</v>
+        <v>4.014</v>
       </c>
       <c r="K35" t="n">
-        <v>4.358</v>
+        <v>4.284</v>
       </c>
       <c r="L35" t="n">
-        <v>4.389</v>
+        <v>4.311</v>
       </c>
       <c r="M35" t="n">
-        <v>4.453</v>
+        <v>4.352</v>
       </c>
       <c r="N35" t="n">
-        <v>4.474</v>
+        <v>4.382</v>
       </c>
       <c r="O35" t="n">
-        <v>4.573</v>
+        <v>4.461</v>
       </c>
       <c r="P35" t="n">
-        <v>4.715</v>
+        <v>4.604</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.425</v>
+        <v>5.315</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.043</v>
+        <v>3.045</v>
       </c>
       <c r="G36" t="n">
-        <v>3.183</v>
+        <v>3.182</v>
       </c>
       <c r="H36" t="n">
-        <v>3.44</v>
+        <v>3.428</v>
       </c>
       <c r="I36" t="n">
-        <v>3.632</v>
+        <v>3.598</v>
       </c>
       <c r="J36" t="n">
-        <v>3.968</v>
+        <v>3.91</v>
       </c>
       <c r="K36" t="n">
-        <v>4.254</v>
+        <v>4.18</v>
       </c>
       <c r="L36" t="n">
-        <v>4.279</v>
+        <v>4.201</v>
       </c>
       <c r="M36" t="n">
-        <v>4.319</v>
+        <v>4.218</v>
       </c>
       <c r="N36" t="n">
-        <v>4.337</v>
+        <v>4.245</v>
       </c>
       <c r="O36" t="n">
-        <v>4.415</v>
+        <v>4.303</v>
       </c>
       <c r="P36" t="n">
-        <v>4.517</v>
+        <v>4.406</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.805</v>
+        <v>4.695</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.927</v>
+        <v>3.929</v>
       </c>
       <c r="G37" t="n">
-        <v>4.465</v>
+        <v>4.466</v>
       </c>
       <c r="H37" t="n">
-        <v>5.103</v>
+        <v>5.092</v>
       </c>
       <c r="I37" t="n">
-        <v>5.425</v>
+        <v>5.392</v>
       </c>
       <c r="J37" t="n">
-        <v>6.305</v>
+        <v>6.248</v>
       </c>
       <c r="K37" t="n">
-        <v>7.258</v>
+        <v>7.185</v>
       </c>
       <c r="L37" t="n">
-        <v>7.562</v>
+        <v>7.484</v>
       </c>
       <c r="M37" t="n">
-        <v>7.889</v>
+        <v>7.788</v>
       </c>
       <c r="N37" t="n">
-        <v>8.058999999999999</v>
+        <v>7.967</v>
       </c>
       <c r="O37" t="n">
-        <v>8.268000000000001</v>
+        <v>8.156000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>8.375999999999999</v>
+        <v>8.265000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.835000000000001</v>
+        <v>8.725</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.989</v>
+        <v>4.991</v>
       </c>
       <c r="G38" t="n">
         <v>5.781</v>
       </c>
       <c r="H38" t="n">
-        <v>6.63</v>
+        <v>6.619</v>
       </c>
       <c r="I38" t="n">
-        <v>7.109</v>
+        <v>7.076</v>
       </c>
       <c r="J38" t="n">
-        <v>8.249000000000001</v>
+        <v>8.192</v>
       </c>
       <c r="K38" t="n">
-        <v>9.382</v>
+        <v>9.308</v>
       </c>
       <c r="L38" t="n">
-        <v>9.845000000000001</v>
+        <v>9.766999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.301</v>
+        <v>10.2</v>
       </c>
       <c r="N38" t="n">
-        <v>10.478</v>
+        <v>10.386</v>
       </c>
       <c r="O38" t="n">
-        <v>10.668</v>
+        <v>10.556</v>
       </c>
       <c r="P38" t="n">
-        <v>10.774</v>
+        <v>10.663</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.286</v>
+        <v>11.176</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.309</v>
+        <v>4.311</v>
       </c>
       <c r="G39" t="n">
         <v>4.979</v>
       </c>
       <c r="H39" t="n">
-        <v>5.695</v>
+        <v>5.684</v>
       </c>
       <c r="I39" t="n">
-        <v>6.113</v>
+        <v>6.08</v>
       </c>
       <c r="J39" t="n">
-        <v>7.122</v>
+        <v>7.064</v>
       </c>
       <c r="K39" t="n">
-        <v>8.214</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="L39" t="n">
-        <v>8.601000000000001</v>
+        <v>8.522</v>
       </c>
       <c r="M39" t="n">
-        <v>8.936999999999999</v>
+        <v>8.836</v>
       </c>
       <c r="N39" t="n">
-        <v>9.105</v>
+        <v>9.013</v>
       </c>
       <c r="O39" t="n">
-        <v>9.318</v>
+        <v>9.206</v>
       </c>
       <c r="P39" t="n">
-        <v>9.428000000000001</v>
+        <v>9.317</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.930999999999999</v>
+        <v>9.821</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.447</v>
+        <v>3.449</v>
       </c>
       <c r="G40" t="n">
         <v>3.645</v>
       </c>
       <c r="H40" t="n">
-        <v>3.974</v>
+        <v>3.963</v>
       </c>
       <c r="I40" t="n">
-        <v>4.208</v>
+        <v>4.175</v>
       </c>
       <c r="J40" t="n">
-        <v>4.616</v>
+        <v>4.559</v>
       </c>
       <c r="K40" t="n">
-        <v>4.992</v>
+        <v>4.918</v>
       </c>
       <c r="L40" t="n">
-        <v>5.074</v>
+        <v>4.996</v>
       </c>
       <c r="M40" t="n">
-        <v>5.229</v>
+        <v>5.128</v>
       </c>
       <c r="N40" t="n">
-        <v>5.401</v>
+        <v>5.309</v>
       </c>
       <c r="O40" t="n">
-        <v>5.732</v>
+        <v>5.62</v>
       </c>
       <c r="P40" t="n">
-        <v>6.007</v>
+        <v>5.896</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.823</v>
+        <v>6.713</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.833</v>
+        <v>3.835</v>
       </c>
       <c r="G41" t="n">
         <v>4.074</v>
       </c>
       <c r="H41" t="n">
-        <v>4.46</v>
+        <v>4.449</v>
       </c>
       <c r="I41" t="n">
-        <v>4.712</v>
+        <v>4.679</v>
       </c>
       <c r="J41" t="n">
-        <v>5.171</v>
+        <v>5.114</v>
       </c>
       <c r="K41" t="n">
-        <v>5.592</v>
+        <v>5.519</v>
       </c>
       <c r="L41" t="n">
-        <v>5.752</v>
+        <v>5.674</v>
       </c>
       <c r="M41" t="n">
-        <v>6.032</v>
+        <v>5.931</v>
       </c>
       <c r="N41" t="n">
-        <v>6.332</v>
+        <v>6.24</v>
       </c>
       <c r="O41" t="n">
-        <v>6.847</v>
+        <v>6.735</v>
       </c>
       <c r="P41" t="n">
-        <v>7.067</v>
+        <v>6.956</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.87</v>
+        <v>7.76</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.568</v>
+        <v>3.57</v>
       </c>
       <c r="G42" t="n">
         <v>3.794</v>
       </c>
       <c r="H42" t="n">
-        <v>4.15</v>
+        <v>4.139</v>
       </c>
       <c r="I42" t="n">
-        <v>4.397</v>
+        <v>4.364</v>
       </c>
       <c r="J42" t="n">
-        <v>4.819</v>
+        <v>4.761</v>
       </c>
       <c r="K42" t="n">
-        <v>5.213</v>
+        <v>5.139</v>
       </c>
       <c r="L42" t="n">
-        <v>5.31</v>
+        <v>5.232</v>
       </c>
       <c r="M42" t="n">
-        <v>5.537</v>
+        <v>5.435</v>
       </c>
       <c r="N42" t="n">
-        <v>5.816</v>
+        <v>5.724</v>
       </c>
       <c r="O42" t="n">
-        <v>6.224</v>
+        <v>6.112</v>
       </c>
       <c r="P42" t="n">
-        <v>6.51</v>
+        <v>6.398</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.335</v>
+        <v>7.225</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.268</v>
+        <v>3.27</v>
       </c>
       <c r="G43" t="n">
         <v>3.454</v>
       </c>
       <c r="H43" t="n">
-        <v>3.734</v>
+        <v>3.723</v>
       </c>
       <c r="I43" t="n">
-        <v>3.929</v>
+        <v>3.896</v>
       </c>
       <c r="J43" t="n">
-        <v>4.258</v>
+        <v>4.201</v>
       </c>
       <c r="K43" t="n">
-        <v>4.559</v>
+        <v>4.486</v>
       </c>
       <c r="L43" t="n">
-        <v>4.597</v>
+        <v>4.519</v>
       </c>
       <c r="M43" t="n">
-        <v>4.671</v>
+        <v>4.57</v>
       </c>
       <c r="N43" t="n">
-        <v>4.702</v>
+        <v>4.61</v>
       </c>
       <c r="O43" t="n">
-        <v>4.82</v>
+        <v>4.708</v>
       </c>
       <c r="P43" t="n">
-        <v>4.984</v>
+        <v>4.873</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.699</v>
+        <v>5.589</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.121</v>
+        <v>3.123</v>
       </c>
       <c r="G44" t="n">
-        <v>3.292</v>
+        <v>3.291</v>
       </c>
       <c r="H44" t="n">
-        <v>3.563</v>
+        <v>3.551</v>
       </c>
       <c r="I44" t="n">
-        <v>3.759</v>
+        <v>3.725</v>
       </c>
       <c r="J44" t="n">
-        <v>4.108</v>
+        <v>4.051</v>
       </c>
       <c r="K44" t="n">
-        <v>4.404</v>
+        <v>4.331</v>
       </c>
       <c r="L44" t="n">
-        <v>4.44</v>
+        <v>4.362</v>
       </c>
       <c r="M44" t="n">
-        <v>4.489</v>
+        <v>4.388</v>
       </c>
       <c r="N44" t="n">
-        <v>4.519</v>
+        <v>4.427</v>
       </c>
       <c r="O44" t="n">
-        <v>4.616</v>
+        <v>4.504</v>
       </c>
       <c r="P44" t="n">
-        <v>4.747</v>
+        <v>4.636</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.069</v>
+        <v>4.959</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-15 ~ 2026-06-15
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.438</v>
+        <v>3.449</v>
       </c>
       <c r="G2" t="n">
-        <v>3.75</v>
+        <v>3.755</v>
       </c>
       <c r="H2" t="n">
-        <v>4.029</v>
+        <v>4.021</v>
       </c>
       <c r="I2" t="n">
-        <v>4.172</v>
+        <v>4.151</v>
       </c>
       <c r="J2" t="n">
-        <v>4.486</v>
+        <v>4.463</v>
       </c>
       <c r="K2" t="n">
-        <v>4.853</v>
+        <v>4.82</v>
       </c>
       <c r="L2" t="n">
-        <v>5.028</v>
+        <v>4.978</v>
       </c>
       <c r="M2" t="n">
-        <v>5.253</v>
+        <v>5.208</v>
       </c>
       <c r="N2" t="n">
-        <v>5.516</v>
+        <v>5.472</v>
       </c>
       <c r="O2" t="n">
-        <v>5.762</v>
+        <v>5.728</v>
       </c>
       <c r="P2" t="n">
-        <v>5.999</v>
+        <v>5.952</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.662</v>
+        <v>6.587</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.46</v>
+        <v>4.471</v>
       </c>
       <c r="G3" t="n">
-        <v>4.953</v>
+        <v>4.958</v>
       </c>
       <c r="H3" t="n">
-        <v>5.265</v>
+        <v>5.257</v>
       </c>
       <c r="I3" t="n">
-        <v>5.401</v>
+        <v>5.38</v>
       </c>
       <c r="J3" t="n">
-        <v>5.732</v>
+        <v>5.708</v>
       </c>
       <c r="K3" t="n">
-        <v>6.169</v>
+        <v>6.136</v>
       </c>
       <c r="L3" t="n">
-        <v>6.413</v>
+        <v>6.364</v>
       </c>
       <c r="M3" t="n">
-        <v>6.67</v>
+        <v>6.625</v>
       </c>
       <c r="N3" t="n">
-        <v>6.875</v>
+        <v>6.831</v>
       </c>
       <c r="O3" t="n">
-        <v>7.073</v>
+        <v>7.038</v>
       </c>
       <c r="P3" t="n">
-        <v>7.178</v>
+        <v>7.13</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.728</v>
+        <v>7.653</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.952</v>
+        <v>3.963</v>
       </c>
       <c r="G4" t="n">
-        <v>4.334</v>
+        <v>4.339</v>
       </c>
       <c r="H4" t="n">
-        <v>4.674</v>
+        <v>4.666</v>
       </c>
       <c r="I4" t="n">
-        <v>4.843</v>
+        <v>4.823</v>
       </c>
       <c r="J4" t="n">
-        <v>5.175</v>
+        <v>5.152</v>
       </c>
       <c r="K4" t="n">
-        <v>5.607</v>
+        <v>5.574</v>
       </c>
       <c r="L4" t="n">
-        <v>5.782</v>
+        <v>5.733</v>
       </c>
       <c r="M4" t="n">
-        <v>6.028</v>
+        <v>5.983</v>
       </c>
       <c r="N4" t="n">
-        <v>6.204</v>
+        <v>6.16</v>
       </c>
       <c r="O4" t="n">
-        <v>6.424</v>
+        <v>6.389</v>
       </c>
       <c r="P4" t="n">
-        <v>6.53</v>
+        <v>6.483</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.083</v>
+        <v>7.008</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.136</v>
+        <v>3.147</v>
       </c>
       <c r="G5" t="n">
-        <v>3.293</v>
+        <v>3.298</v>
       </c>
       <c r="H5" t="n">
-        <v>3.536</v>
+        <v>3.528</v>
       </c>
       <c r="I5" t="n">
-        <v>3.744</v>
+        <v>3.724</v>
       </c>
       <c r="J5" t="n">
-        <v>4.044</v>
+        <v>4.022</v>
       </c>
       <c r="K5" t="n">
-        <v>4.256</v>
+        <v>4.223</v>
       </c>
       <c r="L5" t="n">
-        <v>4.275</v>
+        <v>4.227</v>
       </c>
       <c r="M5" t="n">
-        <v>4.311</v>
+        <v>4.266</v>
       </c>
       <c r="N5" t="n">
-        <v>4.328</v>
+        <v>4.285</v>
       </c>
       <c r="O5" t="n">
-        <v>4.362</v>
+        <v>4.327</v>
       </c>
       <c r="P5" t="n">
-        <v>4.668</v>
+        <v>4.621</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.574</v>
+        <v>5.499</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.177</v>
+        <v>3.188</v>
       </c>
       <c r="G6" t="n">
-        <v>3.348</v>
+        <v>3.353</v>
       </c>
       <c r="H6" t="n">
-        <v>3.606</v>
+        <v>3.598</v>
       </c>
       <c r="I6" t="n">
-        <v>3.827</v>
+        <v>3.806</v>
       </c>
       <c r="J6" t="n">
-        <v>4.135</v>
+        <v>4.113</v>
       </c>
       <c r="K6" t="n">
-        <v>4.369</v>
+        <v>4.336</v>
       </c>
       <c r="L6" t="n">
-        <v>4.394</v>
+        <v>4.345</v>
       </c>
       <c r="M6" t="n">
-        <v>4.467</v>
+        <v>4.422</v>
       </c>
       <c r="N6" t="n">
-        <v>4.496</v>
+        <v>4.452</v>
       </c>
       <c r="O6" t="n">
-        <v>4.628</v>
+        <v>4.593</v>
       </c>
       <c r="P6" t="n">
-        <v>5.1</v>
+        <v>5.053</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.97</v>
+        <v>5.895</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.157</v>
+        <v>3.168</v>
       </c>
       <c r="G7" t="n">
-        <v>3.312</v>
+        <v>3.317</v>
       </c>
       <c r="H7" t="n">
-        <v>3.552</v>
+        <v>3.544</v>
       </c>
       <c r="I7" t="n">
-        <v>3.764</v>
+        <v>3.743</v>
       </c>
       <c r="J7" t="n">
-        <v>4.067</v>
+        <v>4.046</v>
       </c>
       <c r="K7" t="n">
-        <v>4.283</v>
+        <v>4.25</v>
       </c>
       <c r="L7" t="n">
-        <v>4.302</v>
+        <v>4.253</v>
       </c>
       <c r="M7" t="n">
-        <v>4.371</v>
+        <v>4.326</v>
       </c>
       <c r="N7" t="n">
-        <v>4.388</v>
+        <v>4.344</v>
       </c>
       <c r="O7" t="n">
-        <v>4.526</v>
+        <v>4.491</v>
       </c>
       <c r="P7" t="n">
-        <v>4.884</v>
+        <v>4.837</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.738</v>
+        <v>5.663</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.572</v>
+        <v>5.583</v>
       </c>
       <c r="G8" t="n">
-        <v>6.252</v>
+        <v>6.257</v>
       </c>
       <c r="H8" t="n">
-        <v>6.713</v>
+        <v>6.705</v>
       </c>
       <c r="I8" t="n">
-        <v>6.927</v>
+        <v>6.906</v>
       </c>
       <c r="J8" t="n">
-        <v>7.325</v>
+        <v>7.303</v>
       </c>
       <c r="K8" t="n">
-        <v>8.042</v>
+        <v>8.009</v>
       </c>
       <c r="L8" t="n">
-        <v>8.371</v>
+        <v>8.321999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.66</v>
+        <v>8.615</v>
       </c>
       <c r="N8" t="n">
-        <v>8.800000000000001</v>
+        <v>8.756</v>
       </c>
       <c r="O8" t="n">
-        <v>9.082000000000001</v>
+        <v>9.047000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.291</v>
+        <v>9.244</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.039</v>
+        <v>9.964</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.752</v>
+        <v>2.747</v>
       </c>
       <c r="G9" t="n">
-        <v>2.984</v>
+        <v>2.974</v>
       </c>
       <c r="H9" t="n">
-        <v>3.214</v>
+        <v>3.188</v>
       </c>
       <c r="I9" t="n">
-        <v>3.382</v>
+        <v>3.336</v>
       </c>
       <c r="J9" t="n">
-        <v>3.536</v>
+        <v>3.506</v>
       </c>
       <c r="K9" t="n">
-        <v>3.647</v>
+        <v>3.602</v>
       </c>
       <c r="L9" t="n">
-        <v>3.764</v>
+        <v>3.707</v>
       </c>
       <c r="M9" t="n">
-        <v>3.79</v>
+        <v>3.74</v>
       </c>
       <c r="N9" t="n">
-        <v>3.905</v>
+        <v>3.856</v>
       </c>
       <c r="O9" t="n">
-        <v>3.955</v>
+        <v>3.92</v>
       </c>
       <c r="P9" t="n">
-        <v>4.101</v>
+        <v>4.052</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.195</v>
+        <v>4.12</v>
       </c>
       <c r="R9" t="n">
-        <v>4.244</v>
+        <v>4.2</v>
       </c>
       <c r="S9" t="n">
-        <v>4.293</v>
+        <v>4.245</v>
       </c>
       <c r="T9" t="n">
-        <v>4.22</v>
+        <v>4.185</v>
       </c>
       <c r="U9" t="n">
-        <v>4.133</v>
+        <v>4.08</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.759</v>
+        <v>2.756</v>
       </c>
       <c r="G10" t="n">
-        <v>2.994</v>
+        <v>2.984</v>
       </c>
       <c r="H10" t="n">
-        <v>3.217</v>
+        <v>3.191</v>
       </c>
       <c r="I10" t="n">
-        <v>3.385</v>
+        <v>3.339</v>
       </c>
       <c r="J10" t="n">
-        <v>3.552</v>
+        <v>3.522</v>
       </c>
       <c r="K10" t="n">
-        <v>3.684</v>
+        <v>3.64</v>
       </c>
       <c r="L10" t="n">
-        <v>3.776</v>
+        <v>3.719</v>
       </c>
       <c r="M10" t="n">
-        <v>3.852</v>
+        <v>3.802</v>
       </c>
       <c r="N10" t="n">
-        <v>3.93</v>
+        <v>3.881</v>
       </c>
       <c r="O10" t="n">
-        <v>4.2</v>
+        <v>4.16</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.563</v>
+        <v>2.56</v>
       </c>
       <c r="G11" t="n">
-        <v>2.797</v>
+        <v>2.787</v>
       </c>
       <c r="H11" t="n">
-        <v>3.041</v>
+        <v>3.014</v>
       </c>
       <c r="I11" t="n">
-        <v>3.19</v>
+        <v>3.143</v>
       </c>
       <c r="J11" t="n">
-        <v>3.346</v>
+        <v>3.316</v>
       </c>
       <c r="K11" t="n">
-        <v>3.469</v>
+        <v>3.423</v>
       </c>
       <c r="L11" t="n">
-        <v>3.573</v>
+        <v>3.516</v>
       </c>
       <c r="M11" t="n">
-        <v>3.66</v>
+        <v>3.61</v>
       </c>
       <c r="N11" t="n">
-        <v>3.736</v>
+        <v>3.688</v>
       </c>
       <c r="O11" t="n">
-        <v>3.966</v>
+        <v>3.926</v>
       </c>
       <c r="P11" t="n">
-        <v>4.047</v>
+        <v>3.996</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.393</v>
+        <v>4.318</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.372</v>
+        <v>3.377</v>
       </c>
       <c r="G12" t="n">
         <v>3.651</v>
       </c>
       <c r="H12" t="n">
-        <v>3.934</v>
+        <v>3.922</v>
       </c>
       <c r="I12" t="n">
-        <v>4.153</v>
+        <v>4.129</v>
       </c>
       <c r="J12" t="n">
-        <v>4.479</v>
+        <v>4.454</v>
       </c>
       <c r="K12" t="n">
-        <v>4.638</v>
+        <v>4.604</v>
       </c>
       <c r="L12" t="n">
-        <v>4.676</v>
+        <v>4.631</v>
       </c>
       <c r="M12" t="n">
-        <v>4.779</v>
+        <v>4.734</v>
       </c>
       <c r="N12" t="n">
-        <v>4.84</v>
+        <v>4.795</v>
       </c>
       <c r="O12" t="n">
-        <v>4.982</v>
+        <v>4.946</v>
       </c>
       <c r="P12" t="n">
-        <v>5.139</v>
+        <v>5.09</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.516</v>
+        <v>5.441</v>
       </c>
       <c r="R12" t="n">
-        <v>5.74</v>
+        <v>5.696</v>
       </c>
       <c r="S12" t="n">
-        <v>6.002</v>
+        <v>5.954</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.125</v>
+        <v>3.13</v>
       </c>
       <c r="G13" t="n">
         <v>3.341</v>
       </c>
       <c r="H13" t="n">
-        <v>3.601</v>
+        <v>3.59</v>
       </c>
       <c r="I13" t="n">
-        <v>3.8</v>
+        <v>3.777</v>
       </c>
       <c r="J13" t="n">
-        <v>4.116</v>
+        <v>4.091</v>
       </c>
       <c r="K13" t="n">
-        <v>4.271</v>
+        <v>4.237</v>
       </c>
       <c r="L13" t="n">
-        <v>4.316</v>
+        <v>4.27</v>
       </c>
       <c r="M13" t="n">
-        <v>4.406</v>
+        <v>4.361</v>
       </c>
       <c r="N13" t="n">
-        <v>4.468</v>
+        <v>4.423</v>
       </c>
       <c r="O13" t="n">
-        <v>4.61</v>
+        <v>4.574</v>
       </c>
       <c r="P13" t="n">
-        <v>4.73</v>
+        <v>4.682</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.037</v>
+        <v>4.962</v>
       </c>
       <c r="R13" t="n">
-        <v>5.29</v>
+        <v>5.245</v>
       </c>
       <c r="S13" t="n">
-        <v>5.564</v>
+        <v>5.516</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.943</v>
+        <v>2.948</v>
       </c>
       <c r="G14" t="n">
         <v>3.144</v>
       </c>
       <c r="H14" t="n">
-        <v>3.404</v>
+        <v>3.393</v>
       </c>
       <c r="I14" t="n">
-        <v>3.585</v>
+        <v>3.561</v>
       </c>
       <c r="J14" t="n">
-        <v>3.857</v>
+        <v>3.832</v>
       </c>
       <c r="K14" t="n">
-        <v>3.96</v>
+        <v>3.926</v>
       </c>
       <c r="L14" t="n">
-        <v>3.989</v>
+        <v>3.943</v>
       </c>
       <c r="M14" t="n">
-        <v>4.093</v>
+        <v>4.047</v>
       </c>
       <c r="N14" t="n">
-        <v>4.147</v>
+        <v>4.103</v>
       </c>
       <c r="O14" t="n">
-        <v>4.269</v>
+        <v>4.233</v>
       </c>
       <c r="P14" t="n">
-        <v>4.366</v>
+        <v>4.318</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.626</v>
+        <v>4.551</v>
       </c>
       <c r="R14" t="n">
-        <v>4.804</v>
+        <v>4.76</v>
       </c>
       <c r="S14" t="n">
-        <v>5.017</v>
+        <v>4.968</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.92</v>
+        <v>2.925</v>
       </c>
       <c r="G15" t="n">
         <v>3.118</v>
       </c>
       <c r="H15" t="n">
-        <v>3.375</v>
+        <v>3.364</v>
       </c>
       <c r="I15" t="n">
-        <v>3.536</v>
+        <v>3.512</v>
       </c>
       <c r="J15" t="n">
-        <v>3.796</v>
+        <v>3.771</v>
       </c>
       <c r="K15" t="n">
-        <v>3.913</v>
+        <v>3.879</v>
       </c>
       <c r="L15" t="n">
-        <v>3.925</v>
+        <v>3.88</v>
       </c>
       <c r="M15" t="n">
-        <v>4.006</v>
+        <v>3.96</v>
       </c>
       <c r="N15" t="n">
-        <v>4.05</v>
+        <v>4.005</v>
       </c>
       <c r="O15" t="n">
-        <v>4.212</v>
+        <v>4.176</v>
       </c>
       <c r="P15" t="n">
-        <v>4.262</v>
+        <v>4.214</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.528</v>
+        <v>4.453</v>
       </c>
       <c r="R15" t="n">
-        <v>4.698</v>
+        <v>4.654</v>
       </c>
       <c r="S15" t="n">
-        <v>4.912</v>
+        <v>4.864</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.92</v>
+        <v>2.925</v>
       </c>
       <c r="G16" t="n">
         <v>3.118</v>
       </c>
       <c r="H16" t="n">
-        <v>3.375</v>
+        <v>3.364</v>
       </c>
       <c r="I16" t="n">
-        <v>3.536</v>
+        <v>3.512</v>
       </c>
       <c r="J16" t="n">
-        <v>3.796</v>
+        <v>3.771</v>
       </c>
       <c r="K16" t="n">
-        <v>3.913</v>
+        <v>3.879</v>
       </c>
       <c r="L16" t="n">
-        <v>3.925</v>
+        <v>3.88</v>
       </c>
       <c r="M16" t="n">
-        <v>4.006</v>
+        <v>3.96</v>
       </c>
       <c r="N16" t="n">
-        <v>4.053</v>
+        <v>4.008</v>
       </c>
       <c r="O16" t="n">
-        <v>4.218</v>
+        <v>4.183</v>
       </c>
       <c r="P16" t="n">
-        <v>4.286</v>
+        <v>4.237</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.555</v>
+        <v>4.48</v>
       </c>
       <c r="R16" t="n">
-        <v>4.726</v>
+        <v>4.682</v>
       </c>
       <c r="S16" t="n">
-        <v>4.941</v>
+        <v>4.893</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.79</v>
+        <v>2.787</v>
       </c>
       <c r="G17" t="n">
-        <v>3.046</v>
+        <v>3.036</v>
       </c>
       <c r="H17" t="n">
-        <v>3.272</v>
+        <v>3.246</v>
       </c>
       <c r="I17" t="n">
-        <v>3.44</v>
+        <v>3.393</v>
       </c>
       <c r="J17" t="n">
-        <v>3.619</v>
+        <v>3.592</v>
       </c>
       <c r="K17" t="n">
-        <v>3.759</v>
+        <v>3.717</v>
       </c>
       <c r="L17" t="n">
-        <v>3.86</v>
+        <v>3.804</v>
       </c>
       <c r="M17" t="n">
-        <v>3.977</v>
+        <v>3.929</v>
       </c>
       <c r="N17" t="n">
-        <v>4.035</v>
+        <v>3.99</v>
       </c>
       <c r="O17" t="n">
-        <v>4.22</v>
+        <v>4.18</v>
       </c>
       <c r="P17" t="n">
-        <v>4.329</v>
+        <v>4.281</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.791</v>
+        <v>2.788</v>
       </c>
       <c r="G18" t="n">
-        <v>3.047</v>
+        <v>3.037</v>
       </c>
       <c r="H18" t="n">
-        <v>3.272</v>
+        <v>3.246</v>
       </c>
       <c r="I18" t="n">
-        <v>3.44</v>
+        <v>3.394</v>
       </c>
       <c r="J18" t="n">
-        <v>3.619</v>
+        <v>3.592</v>
       </c>
       <c r="K18" t="n">
-        <v>3.76</v>
+        <v>3.718</v>
       </c>
       <c r="L18" t="n">
-        <v>3.86</v>
+        <v>3.804</v>
       </c>
       <c r="M18" t="n">
-        <v>3.977</v>
+        <v>3.929</v>
       </c>
       <c r="N18" t="n">
-        <v>4.036</v>
+        <v>3.991</v>
       </c>
       <c r="O18" t="n">
-        <v>4.218</v>
+        <v>4.178</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.931</v>
+        <v>2.936</v>
       </c>
       <c r="G19" t="n">
-        <v>3.131</v>
+        <v>3.132</v>
       </c>
       <c r="H19" t="n">
-        <v>3.392</v>
+        <v>3.381</v>
       </c>
       <c r="I19" t="n">
-        <v>3.569</v>
+        <v>3.546</v>
       </c>
       <c r="J19" t="n">
-        <v>3.837</v>
+        <v>3.812</v>
       </c>
       <c r="K19" t="n">
-        <v>3.956</v>
+        <v>3.921</v>
       </c>
       <c r="L19" t="n">
-        <v>3.986</v>
+        <v>3.941</v>
       </c>
       <c r="M19" t="n">
-        <v>4.084</v>
+        <v>4.038</v>
       </c>
       <c r="N19" t="n">
-        <v>4.139</v>
+        <v>4.095</v>
       </c>
       <c r="O19" t="n">
-        <v>4.255</v>
+        <v>4.219</v>
       </c>
       <c r="P19" t="n">
-        <v>4.324</v>
+        <v>4.276</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.566</v>
+        <v>4.491</v>
       </c>
       <c r="R19" t="n">
-        <v>4.745</v>
+        <v>4.7</v>
       </c>
       <c r="S19" t="n">
-        <v>4.952</v>
+        <v>4.904</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.66</v>
+        <v>2.664</v>
       </c>
       <c r="G20" t="n">
-        <v>2.768</v>
+        <v>2.759</v>
       </c>
       <c r="H20" t="n">
-        <v>2.873</v>
+        <v>2.852</v>
       </c>
       <c r="I20" t="n">
-        <v>2.991</v>
+        <v>2.956</v>
       </c>
       <c r="J20" t="n">
-        <v>3.465</v>
+        <v>3.427</v>
       </c>
       <c r="K20" t="n">
-        <v>3.707</v>
+        <v>3.66</v>
       </c>
       <c r="L20" t="n">
-        <v>3.708</v>
+        <v>3.658</v>
       </c>
       <c r="M20" t="n">
-        <v>3.795</v>
+        <v>3.745</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.011</v>
+        <v>3.014</v>
       </c>
       <c r="G21" t="n">
-        <v>3.238</v>
+        <v>3.235</v>
       </c>
       <c r="H21" t="n">
-        <v>3.512</v>
+        <v>3.503</v>
       </c>
       <c r="I21" t="n">
-        <v>3.704</v>
+        <v>3.683</v>
       </c>
       <c r="J21" t="n">
-        <v>4.003</v>
+        <v>3.979</v>
       </c>
       <c r="K21" t="n">
-        <v>4.202</v>
+        <v>4.164</v>
       </c>
       <c r="L21" t="n">
-        <v>4.24</v>
+        <v>4.197</v>
       </c>
       <c r="M21" t="n">
+        <v>4.285</v>
+      </c>
+      <c r="N21" t="n">
         <v>4.329</v>
       </c>
-      <c r="N21" t="n">
-        <v>4.374</v>
-      </c>
       <c r="O21" t="n">
-        <v>4.46</v>
+        <v>4.426</v>
       </c>
       <c r="P21" t="n">
-        <v>4.581</v>
+        <v>4.536</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.719</v>
+        <v>4.643</v>
       </c>
       <c r="R21" t="n">
-        <v>4.797</v>
+        <v>4.753</v>
       </c>
       <c r="S21" t="n">
-        <v>4.905</v>
+        <v>4.857</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.957</v>
+        <v>2.96</v>
       </c>
       <c r="G22" t="n">
-        <v>3.183</v>
+        <v>3.18</v>
       </c>
       <c r="H22" t="n">
-        <v>3.444</v>
+        <v>3.435</v>
       </c>
       <c r="I22" t="n">
-        <v>3.623</v>
+        <v>3.601</v>
       </c>
       <c r="J22" t="n">
-        <v>3.888</v>
+        <v>3.864</v>
       </c>
       <c r="K22" t="n">
-        <v>4.084</v>
+        <v>4.046</v>
       </c>
       <c r="L22" t="n">
-        <v>4.107</v>
+        <v>4.064</v>
       </c>
       <c r="M22" t="n">
-        <v>4.2</v>
+        <v>4.156</v>
       </c>
       <c r="N22" t="n">
-        <v>4.248</v>
+        <v>4.203</v>
       </c>
       <c r="O22" t="n">
-        <v>4.331</v>
+        <v>4.297</v>
       </c>
       <c r="P22" t="n">
-        <v>4.444</v>
+        <v>4.399</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.578</v>
+        <v>4.502</v>
       </c>
       <c r="R22" t="n">
-        <v>4.646</v>
+        <v>4.602</v>
       </c>
       <c r="S22" t="n">
-        <v>4.751</v>
+        <v>4.702</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.905</v>
+        <v>2.908</v>
       </c>
       <c r="G23" t="n">
-        <v>3.137</v>
+        <v>3.134</v>
       </c>
       <c r="H23" t="n">
-        <v>3.385</v>
+        <v>3.376</v>
       </c>
       <c r="I23" t="n">
-        <v>3.571</v>
+        <v>3.549</v>
       </c>
       <c r="J23" t="n">
-        <v>3.828</v>
+        <v>3.804</v>
       </c>
       <c r="K23" t="n">
-        <v>3.984</v>
+        <v>3.946</v>
       </c>
       <c r="L23" t="n">
-        <v>4.005</v>
+        <v>3.961</v>
       </c>
       <c r="M23" t="n">
-        <v>4.092</v>
+        <v>4.047</v>
       </c>
       <c r="N23" t="n">
-        <v>4.142</v>
+        <v>4.097</v>
       </c>
       <c r="O23" t="n">
-        <v>4.207</v>
+        <v>4.173</v>
       </c>
       <c r="P23" t="n">
+        <v>4.262</v>
+      </c>
+      <c r="Q23" t="n">
         <v>4.307</v>
       </c>
-      <c r="Q23" t="n">
-        <v>4.383</v>
-      </c>
       <c r="R23" t="n">
-        <v>4.431</v>
+        <v>4.388</v>
       </c>
       <c r="S23" t="n">
-        <v>4.507</v>
+        <v>4.459</v>
       </c>
       <c r="T23" t="n">
-        <v>4.433</v>
+        <v>4.397</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.841</v>
+        <v>2.844</v>
       </c>
       <c r="G24" t="n">
-        <v>3.048</v>
+        <v>3.044</v>
       </c>
       <c r="H24" t="n">
-        <v>3.282</v>
+        <v>3.274</v>
       </c>
       <c r="I24" t="n">
-        <v>3.509</v>
+        <v>3.487</v>
       </c>
       <c r="J24" t="n">
-        <v>3.721</v>
+        <v>3.698</v>
       </c>
       <c r="K24" t="n">
-        <v>3.867</v>
+        <v>3.828</v>
       </c>
       <c r="L24" t="n">
-        <v>3.886</v>
+        <v>3.843</v>
       </c>
       <c r="M24" t="n">
-        <v>3.95</v>
+        <v>3.906</v>
       </c>
       <c r="N24" t="n">
-        <v>4.016</v>
+        <v>3.972</v>
       </c>
       <c r="O24" t="n">
-        <v>4.205</v>
+        <v>4.171</v>
       </c>
       <c r="P24" t="n">
-        <v>4.246</v>
+        <v>4.201</v>
       </c>
       <c r="Q24" t="n">
+        <v>4.234</v>
+      </c>
+      <c r="R24" t="n">
         <v>4.309</v>
       </c>
-      <c r="R24" t="n">
-        <v>4.353</v>
-      </c>
       <c r="S24" t="n">
-        <v>4.422</v>
+        <v>4.374</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.9</v>
+        <v>2.903</v>
       </c>
       <c r="G25" t="n">
-        <v>3.137</v>
+        <v>3.134</v>
       </c>
       <c r="H25" t="n">
-        <v>3.388</v>
+        <v>3.38</v>
       </c>
       <c r="I25" t="n">
-        <v>3.579</v>
+        <v>3.558</v>
       </c>
       <c r="J25" t="n">
-        <v>3.843</v>
+        <v>3.82</v>
       </c>
       <c r="K25" t="n">
-        <v>4.015</v>
+        <v>3.977</v>
       </c>
       <c r="L25" t="n">
-        <v>4.035</v>
+        <v>3.992</v>
       </c>
       <c r="M25" t="n">
-        <v>4.123</v>
+        <v>4.078</v>
       </c>
       <c r="N25" t="n">
-        <v>4.169</v>
+        <v>4.124</v>
       </c>
       <c r="O25" t="n">
-        <v>4.235</v>
+        <v>4.202</v>
       </c>
       <c r="P25" t="n">
-        <v>4.328</v>
+        <v>4.284</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.417</v>
+        <v>4.341</v>
       </c>
       <c r="R25" t="n">
-        <v>4.455</v>
+        <v>4.411</v>
       </c>
       <c r="S25" t="n">
-        <v>4.53</v>
+        <v>4.482</v>
       </c>
       <c r="T25" t="n">
-        <v>4.451</v>
+        <v>4.415</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.224</v>
+        <v>3.23</v>
       </c>
       <c r="G26" t="n">
-        <v>3.44</v>
+        <v>3.438</v>
       </c>
       <c r="H26" t="n">
-        <v>3.777</v>
+        <v>3.767</v>
       </c>
       <c r="I26" t="n">
-        <v>3.983</v>
+        <v>3.962</v>
       </c>
       <c r="J26" t="n">
-        <v>4.409</v>
+        <v>4.387</v>
       </c>
       <c r="K26" t="n">
-        <v>4.816</v>
+        <v>4.778</v>
       </c>
       <c r="L26" t="n">
-        <v>4.9</v>
+        <v>4.851</v>
       </c>
       <c r="M26" t="n">
-        <v>5.025</v>
+        <v>4.981</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.293</v>
+        <v>5.26</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.027</v>
+        <v>3.03</v>
       </c>
       <c r="G27" t="n">
-        <v>3.205</v>
+        <v>3.202</v>
       </c>
       <c r="H27" t="n">
-        <v>3.468</v>
+        <v>3.456</v>
       </c>
       <c r="I27" t="n">
-        <v>3.649</v>
+        <v>3.626</v>
       </c>
       <c r="J27" t="n">
-        <v>3.947</v>
+        <v>3.923</v>
       </c>
       <c r="K27" t="n">
-        <v>4.137</v>
+        <v>4.101</v>
       </c>
       <c r="L27" t="n">
-        <v>4.166</v>
+        <v>4.118</v>
       </c>
       <c r="M27" t="n">
-        <v>4.249</v>
+        <v>4.203</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.398</v>
+        <v>4.362</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.13</v>
+        <v>3.133</v>
       </c>
       <c r="G28" t="n">
-        <v>3.316</v>
+        <v>3.313</v>
       </c>
       <c r="H28" t="n">
-        <v>3.594</v>
+        <v>3.582</v>
       </c>
       <c r="I28" t="n">
-        <v>3.786</v>
+        <v>3.763</v>
       </c>
       <c r="J28" t="n">
-        <v>4.12</v>
+        <v>4.096</v>
       </c>
       <c r="K28" t="n">
-        <v>4.329</v>
+        <v>4.293</v>
       </c>
       <c r="L28" t="n">
-        <v>4.369</v>
+        <v>4.321</v>
       </c>
       <c r="M28" t="n">
-        <v>4.461</v>
+        <v>4.415</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.69</v>
+        <v>4.654</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.976</v>
+        <v>2.979</v>
       </c>
       <c r="G29" t="n">
-        <v>3.151</v>
+        <v>3.148</v>
       </c>
       <c r="H29" t="n">
-        <v>3.405</v>
+        <v>3.393</v>
       </c>
       <c r="I29" t="n">
-        <v>3.574</v>
+        <v>3.551</v>
       </c>
       <c r="J29" t="n">
-        <v>3.859</v>
+        <v>3.835</v>
       </c>
       <c r="K29" t="n">
-        <v>4.032</v>
+        <v>3.997</v>
       </c>
       <c r="L29" t="n">
-        <v>4.052</v>
+        <v>4.004</v>
       </c>
       <c r="M29" t="n">
-        <v>4.112</v>
+        <v>4.066</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.27</v>
+        <v>4.234</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.257</v>
+        <v>3.263</v>
       </c>
       <c r="G30" t="n">
-        <v>3.407</v>
+        <v>3.405</v>
       </c>
       <c r="H30" t="n">
-        <v>3.704</v>
+        <v>3.694</v>
       </c>
       <c r="I30" t="n">
-        <v>3.901</v>
+        <v>3.88</v>
       </c>
       <c r="J30" t="n">
-        <v>4.267</v>
+        <v>4.244</v>
       </c>
       <c r="K30" t="n">
-        <v>4.612</v>
+        <v>4.573</v>
       </c>
       <c r="L30" t="n">
-        <v>4.671</v>
+        <v>4.623</v>
       </c>
       <c r="M30" t="n">
-        <v>4.786</v>
+        <v>4.743</v>
       </c>
       <c r="N30" t="n">
-        <v>4.952</v>
+        <v>4.909</v>
       </c>
       <c r="O30" t="n">
-        <v>5.241</v>
+        <v>5.208</v>
       </c>
       <c r="P30" t="n">
-        <v>5.475</v>
+        <v>5.43</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.262</v>
+        <v>6.187</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.586</v>
+        <v>3.592</v>
       </c>
       <c r="G31" t="n">
-        <v>3.773</v>
+        <v>3.771</v>
       </c>
       <c r="H31" t="n">
-        <v>4.12</v>
+        <v>4.11</v>
       </c>
       <c r="I31" t="n">
-        <v>4.331</v>
+        <v>4.309</v>
       </c>
       <c r="J31" t="n">
-        <v>4.759</v>
+        <v>4.737</v>
       </c>
       <c r="K31" t="n">
-        <v>5.145</v>
+        <v>5.108</v>
       </c>
       <c r="L31" t="n">
-        <v>5.284</v>
+        <v>5.235</v>
       </c>
       <c r="M31" t="n">
-        <v>5.516</v>
+        <v>5.473</v>
       </c>
       <c r="N31" t="n">
-        <v>5.811</v>
+        <v>5.768</v>
       </c>
       <c r="O31" t="n">
-        <v>6.277</v>
+        <v>6.244</v>
       </c>
       <c r="P31" t="n">
-        <v>6.463</v>
+        <v>6.418</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.235</v>
+        <v>7.16</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.356</v>
+        <v>3.361</v>
       </c>
       <c r="G32" t="n">
-        <v>3.525</v>
+        <v>3.523</v>
       </c>
       <c r="H32" t="n">
-        <v>3.848</v>
+        <v>3.838</v>
       </c>
       <c r="I32" t="n">
-        <v>4.061</v>
+        <v>4.039</v>
       </c>
       <c r="J32" t="n">
-        <v>4.445</v>
+        <v>4.424</v>
       </c>
       <c r="K32" t="n">
-        <v>4.797</v>
+        <v>4.758</v>
       </c>
       <c r="L32" t="n">
-        <v>4.875</v>
+        <v>4.827</v>
       </c>
       <c r="M32" t="n">
-        <v>5.058</v>
+        <v>5.015</v>
       </c>
       <c r="N32" t="n">
-        <v>5.312</v>
+        <v>5.27</v>
       </c>
       <c r="O32" t="n">
-        <v>5.686</v>
+        <v>5.653</v>
       </c>
       <c r="P32" t="n">
-        <v>5.935</v>
+        <v>5.89</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.723</v>
+        <v>6.648</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.122</v>
+        <v>3.128</v>
       </c>
       <c r="G33" t="n">
-        <v>3.272</v>
+        <v>3.27</v>
       </c>
       <c r="H33" t="n">
-        <v>3.522</v>
+        <v>3.512</v>
       </c>
       <c r="I33" t="n">
-        <v>3.688</v>
+        <v>3.666</v>
       </c>
       <c r="J33" t="n">
-        <v>3.974</v>
+        <v>3.95</v>
       </c>
       <c r="K33" t="n">
-        <v>4.254</v>
+        <v>4.215</v>
       </c>
       <c r="L33" t="n">
-        <v>4.277</v>
+        <v>4.229</v>
       </c>
       <c r="M33" t="n">
-        <v>4.315</v>
+        <v>4.272</v>
       </c>
       <c r="N33" t="n">
-        <v>4.341</v>
+        <v>4.298</v>
       </c>
       <c r="O33" t="n">
-        <v>4.395</v>
+        <v>4.364</v>
       </c>
       <c r="P33" t="n">
-        <v>4.507</v>
+        <v>4.462</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.978</v>
+        <v>4.903</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.182</v>
+        <v>3.188</v>
       </c>
       <c r="G34" t="n">
-        <v>3.325</v>
+        <v>3.323</v>
       </c>
       <c r="H34" t="n">
-        <v>3.584</v>
+        <v>3.574</v>
       </c>
       <c r="I34" t="n">
-        <v>3.756</v>
+        <v>3.734</v>
       </c>
       <c r="J34" t="n">
-        <v>4.045</v>
+        <v>4.022</v>
       </c>
       <c r="K34" t="n">
-        <v>4.33</v>
+        <v>4.291</v>
       </c>
       <c r="L34" t="n">
-        <v>4.355</v>
+        <v>4.307</v>
       </c>
       <c r="M34" t="n">
-        <v>4.406</v>
+        <v>4.363</v>
       </c>
       <c r="N34" t="n">
-        <v>4.445</v>
+        <v>4.403</v>
       </c>
       <c r="O34" t="n">
-        <v>4.564</v>
+        <v>4.533</v>
       </c>
       <c r="P34" t="n">
-        <v>4.802</v>
+        <v>4.757</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.679</v>
+        <v>5.604</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.156</v>
+        <v>3.162</v>
       </c>
       <c r="G35" t="n">
-        <v>3.299</v>
+        <v>3.297</v>
       </c>
       <c r="H35" t="n">
-        <v>3.552</v>
+        <v>3.542</v>
       </c>
       <c r="I35" t="n">
-        <v>3.722</v>
+        <v>3.701</v>
       </c>
       <c r="J35" t="n">
-        <v>4.014</v>
+        <v>3.99</v>
       </c>
       <c r="K35" t="n">
-        <v>4.284</v>
+        <v>4.245</v>
       </c>
       <c r="L35" t="n">
-        <v>4.311</v>
+        <v>4.263</v>
       </c>
       <c r="M35" t="n">
-        <v>4.352</v>
+        <v>4.309</v>
       </c>
       <c r="N35" t="n">
-        <v>4.382</v>
+        <v>4.339</v>
       </c>
       <c r="O35" t="n">
-        <v>4.461</v>
+        <v>4.43</v>
       </c>
       <c r="P35" t="n">
-        <v>4.604</v>
+        <v>4.559</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.315</v>
+        <v>5.24</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.045</v>
+        <v>3.051</v>
       </c>
       <c r="G36" t="n">
-        <v>3.182</v>
+        <v>3.18</v>
       </c>
       <c r="H36" t="n">
-        <v>3.428</v>
+        <v>3.418</v>
       </c>
       <c r="I36" t="n">
-        <v>3.598</v>
+        <v>3.576</v>
       </c>
       <c r="J36" t="n">
-        <v>3.91</v>
+        <v>3.887</v>
       </c>
       <c r="K36" t="n">
-        <v>4.18</v>
+        <v>4.14</v>
       </c>
       <c r="L36" t="n">
-        <v>4.201</v>
+        <v>4.153</v>
       </c>
       <c r="M36" t="n">
-        <v>4.218</v>
+        <v>4.175</v>
       </c>
       <c r="N36" t="n">
-        <v>4.245</v>
+        <v>4.203</v>
       </c>
       <c r="O36" t="n">
-        <v>4.303</v>
+        <v>4.272</v>
       </c>
       <c r="P36" t="n">
-        <v>4.406</v>
+        <v>4.36</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.695</v>
+        <v>4.62</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.929</v>
+        <v>3.935</v>
       </c>
       <c r="G37" t="n">
-        <v>4.466</v>
+        <v>4.464</v>
       </c>
       <c r="H37" t="n">
-        <v>5.092</v>
+        <v>5.082</v>
       </c>
       <c r="I37" t="n">
-        <v>5.392</v>
+        <v>5.37</v>
       </c>
       <c r="J37" t="n">
-        <v>6.248</v>
+        <v>6.226</v>
       </c>
       <c r="K37" t="n">
-        <v>7.185</v>
+        <v>7.148</v>
       </c>
       <c r="L37" t="n">
-        <v>7.484</v>
+        <v>7.436</v>
       </c>
       <c r="M37" t="n">
-        <v>7.788</v>
+        <v>7.745</v>
       </c>
       <c r="N37" t="n">
-        <v>7.967</v>
+        <v>7.924</v>
       </c>
       <c r="O37" t="n">
-        <v>8.156000000000001</v>
+        <v>8.122999999999999</v>
       </c>
       <c r="P37" t="n">
-        <v>8.265000000000001</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.725</v>
+        <v>8.65</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.991</v>
+        <v>4.997</v>
       </c>
       <c r="G38" t="n">
-        <v>5.781</v>
+        <v>5.779</v>
       </c>
       <c r="H38" t="n">
-        <v>6.619</v>
+        <v>6.609</v>
       </c>
       <c r="I38" t="n">
-        <v>7.076</v>
+        <v>7.054</v>
       </c>
       <c r="J38" t="n">
-        <v>8.192</v>
+        <v>8.17</v>
       </c>
       <c r="K38" t="n">
-        <v>9.308</v>
+        <v>9.271000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.766999999999999</v>
+        <v>9.718999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.2</v>
+        <v>10.157</v>
       </c>
       <c r="N38" t="n">
-        <v>10.386</v>
+        <v>10.343</v>
       </c>
       <c r="O38" t="n">
-        <v>10.556</v>
+        <v>10.523</v>
       </c>
       <c r="P38" t="n">
-        <v>10.663</v>
+        <v>10.618</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.176</v>
+        <v>11.101</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.311</v>
+        <v>4.317</v>
       </c>
       <c r="G39" t="n">
-        <v>4.979</v>
+        <v>4.977</v>
       </c>
       <c r="H39" t="n">
-        <v>5.684</v>
+        <v>5.674</v>
       </c>
       <c r="I39" t="n">
-        <v>6.08</v>
+        <v>6.058</v>
       </c>
       <c r="J39" t="n">
-        <v>7.064</v>
+        <v>7.043</v>
       </c>
       <c r="K39" t="n">
-        <v>8.140000000000001</v>
+        <v>8.103</v>
       </c>
       <c r="L39" t="n">
-        <v>8.522</v>
+        <v>8.474</v>
       </c>
       <c r="M39" t="n">
-        <v>8.836</v>
+        <v>8.792999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>9.013</v>
+        <v>8.971</v>
       </c>
       <c r="O39" t="n">
-        <v>9.206</v>
+        <v>9.173999999999999</v>
       </c>
       <c r="P39" t="n">
-        <v>9.317</v>
+        <v>9.272</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.821</v>
+        <v>9.746</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.449</v>
+        <v>3.454</v>
       </c>
       <c r="G40" t="n">
-        <v>3.645</v>
+        <v>3.643</v>
       </c>
       <c r="H40" t="n">
-        <v>3.963</v>
+        <v>3.953</v>
       </c>
       <c r="I40" t="n">
-        <v>4.175</v>
+        <v>4.154</v>
       </c>
       <c r="J40" t="n">
-        <v>4.559</v>
+        <v>4.536</v>
       </c>
       <c r="K40" t="n">
-        <v>4.918</v>
+        <v>4.879</v>
       </c>
       <c r="L40" t="n">
-        <v>4.996</v>
+        <v>4.948</v>
       </c>
       <c r="M40" t="n">
-        <v>5.128</v>
+        <v>5.085</v>
       </c>
       <c r="N40" t="n">
-        <v>5.309</v>
+        <v>5.267</v>
       </c>
       <c r="O40" t="n">
-        <v>5.62</v>
+        <v>5.587</v>
       </c>
       <c r="P40" t="n">
-        <v>5.896</v>
+        <v>5.851</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.713</v>
+        <v>6.638</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.835</v>
+        <v>3.841</v>
       </c>
       <c r="G41" t="n">
-        <v>4.074</v>
+        <v>4.072</v>
       </c>
       <c r="H41" t="n">
-        <v>4.449</v>
+        <v>4.439</v>
       </c>
       <c r="I41" t="n">
-        <v>4.679</v>
+        <v>4.657</v>
       </c>
       <c r="J41" t="n">
-        <v>5.114</v>
+        <v>5.092</v>
       </c>
       <c r="K41" t="n">
-        <v>5.519</v>
+        <v>5.482</v>
       </c>
       <c r="L41" t="n">
-        <v>5.674</v>
+        <v>5.626</v>
       </c>
       <c r="M41" t="n">
-        <v>5.931</v>
+        <v>5.888</v>
       </c>
       <c r="N41" t="n">
-        <v>6.24</v>
+        <v>6.197</v>
       </c>
       <c r="O41" t="n">
-        <v>6.735</v>
+        <v>6.702</v>
       </c>
       <c r="P41" t="n">
-        <v>6.956</v>
+        <v>6.911</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.76</v>
+        <v>7.685</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.57</v>
+        <v>3.576</v>
       </c>
       <c r="G42" t="n">
-        <v>3.794</v>
+        <v>3.792</v>
       </c>
       <c r="H42" t="n">
-        <v>4.139</v>
+        <v>4.129</v>
       </c>
       <c r="I42" t="n">
-        <v>4.364</v>
+        <v>4.342</v>
       </c>
       <c r="J42" t="n">
-        <v>4.761</v>
+        <v>4.74</v>
       </c>
       <c r="K42" t="n">
-        <v>5.139</v>
+        <v>5.1</v>
       </c>
       <c r="L42" t="n">
-        <v>5.232</v>
+        <v>5.184</v>
       </c>
       <c r="M42" t="n">
-        <v>5.435</v>
+        <v>5.392</v>
       </c>
       <c r="N42" t="n">
-        <v>5.724</v>
+        <v>5.681</v>
       </c>
       <c r="O42" t="n">
-        <v>6.112</v>
+        <v>6.079</v>
       </c>
       <c r="P42" t="n">
-        <v>6.398</v>
+        <v>6.353</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.225</v>
+        <v>7.15</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.27</v>
+        <v>3.276</v>
       </c>
       <c r="G43" t="n">
-        <v>3.454</v>
+        <v>3.453</v>
       </c>
       <c r="H43" t="n">
-        <v>3.723</v>
+        <v>3.713</v>
       </c>
       <c r="I43" t="n">
-        <v>3.896</v>
+        <v>3.875</v>
       </c>
       <c r="J43" t="n">
-        <v>4.201</v>
+        <v>4.177</v>
       </c>
       <c r="K43" t="n">
-        <v>4.486</v>
+        <v>4.447</v>
       </c>
       <c r="L43" t="n">
-        <v>4.519</v>
+        <v>4.471</v>
       </c>
       <c r="M43" t="n">
-        <v>4.57</v>
+        <v>4.527</v>
       </c>
       <c r="N43" t="n">
-        <v>4.61</v>
+        <v>4.567</v>
       </c>
       <c r="O43" t="n">
-        <v>4.708</v>
+        <v>4.677</v>
       </c>
       <c r="P43" t="n">
-        <v>4.873</v>
+        <v>4.828</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.589</v>
+        <v>5.514</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.123</v>
+        <v>3.129</v>
       </c>
       <c r="G44" t="n">
-        <v>3.291</v>
+        <v>3.289</v>
       </c>
       <c r="H44" t="n">
-        <v>3.551</v>
+        <v>3.541</v>
       </c>
       <c r="I44" t="n">
-        <v>3.725</v>
+        <v>3.703</v>
       </c>
       <c r="J44" t="n">
-        <v>4.051</v>
+        <v>4.028</v>
       </c>
       <c r="K44" t="n">
-        <v>4.331</v>
+        <v>4.291</v>
       </c>
       <c r="L44" t="n">
-        <v>4.362</v>
+        <v>4.314</v>
       </c>
       <c r="M44" t="n">
-        <v>4.388</v>
+        <v>4.345</v>
       </c>
       <c r="N44" t="n">
-        <v>4.427</v>
+        <v>4.384</v>
       </c>
       <c r="O44" t="n">
-        <v>4.504</v>
+        <v>4.473</v>
       </c>
       <c r="P44" t="n">
-        <v>4.636</v>
+        <v>4.59</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.959</v>
+        <v>4.884</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-16 ~ 2026-06-16
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.449</v>
+        <v>3.461</v>
       </c>
       <c r="G2" t="n">
-        <v>3.755</v>
+        <v>3.77</v>
       </c>
       <c r="H2" t="n">
-        <v>4.021</v>
+        <v>4.034</v>
       </c>
       <c r="I2" t="n">
-        <v>4.151</v>
+        <v>4.157</v>
       </c>
       <c r="J2" t="n">
-        <v>4.463</v>
+        <v>4.456</v>
       </c>
       <c r="K2" t="n">
-        <v>4.82</v>
+        <v>4.803</v>
       </c>
       <c r="L2" t="n">
-        <v>4.978</v>
+        <v>4.96</v>
       </c>
       <c r="M2" t="n">
-        <v>5.208</v>
+        <v>5.193</v>
       </c>
       <c r="N2" t="n">
-        <v>5.472</v>
+        <v>5.459</v>
       </c>
       <c r="O2" t="n">
-        <v>5.728</v>
+        <v>5.712</v>
       </c>
       <c r="P2" t="n">
-        <v>5.952</v>
+        <v>5.94</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.587</v>
+        <v>6.577</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.471</v>
+        <v>4.482</v>
       </c>
       <c r="G3" t="n">
-        <v>4.958</v>
+        <v>4.971</v>
       </c>
       <c r="H3" t="n">
-        <v>5.257</v>
+        <v>5.269</v>
       </c>
       <c r="I3" t="n">
-        <v>5.38</v>
+        <v>5.386</v>
       </c>
       <c r="J3" t="n">
-        <v>5.708</v>
+        <v>5.702</v>
       </c>
       <c r="K3" t="n">
-        <v>6.136</v>
+        <v>6.119</v>
       </c>
       <c r="L3" t="n">
-        <v>6.364</v>
+        <v>6.346</v>
       </c>
       <c r="M3" t="n">
-        <v>6.625</v>
+        <v>6.609</v>
       </c>
       <c r="N3" t="n">
-        <v>6.831</v>
+        <v>6.819</v>
       </c>
       <c r="O3" t="n">
-        <v>7.038</v>
+        <v>7.022</v>
       </c>
       <c r="P3" t="n">
-        <v>7.13</v>
+        <v>7.118</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.653</v>
+        <v>7.643</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.963</v>
+        <v>3.974</v>
       </c>
       <c r="G4" t="n">
-        <v>4.339</v>
+        <v>4.353</v>
       </c>
       <c r="H4" t="n">
-        <v>4.666</v>
+        <v>4.678</v>
       </c>
       <c r="I4" t="n">
-        <v>4.823</v>
+        <v>4.829</v>
       </c>
       <c r="J4" t="n">
-        <v>5.152</v>
+        <v>5.145</v>
       </c>
       <c r="K4" t="n">
-        <v>5.574</v>
+        <v>5.557</v>
       </c>
       <c r="L4" t="n">
-        <v>5.733</v>
+        <v>5.715</v>
       </c>
       <c r="M4" t="n">
-        <v>5.983</v>
+        <v>5.967</v>
       </c>
       <c r="N4" t="n">
-        <v>6.16</v>
+        <v>6.147</v>
       </c>
       <c r="O4" t="n">
-        <v>6.389</v>
+        <v>6.374</v>
       </c>
       <c r="P4" t="n">
-        <v>6.483</v>
+        <v>6.47</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.008</v>
+        <v>6.998</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.147</v>
+        <v>3.159</v>
       </c>
       <c r="G5" t="n">
-        <v>3.298</v>
+        <v>3.313</v>
       </c>
       <c r="H5" t="n">
-        <v>3.528</v>
+        <v>3.541</v>
       </c>
       <c r="I5" t="n">
-        <v>3.724</v>
+        <v>3.73</v>
       </c>
       <c r="J5" t="n">
-        <v>4.022</v>
+        <v>4.016</v>
       </c>
       <c r="K5" t="n">
-        <v>4.223</v>
+        <v>4.206</v>
       </c>
       <c r="L5" t="n">
-        <v>4.227</v>
+        <v>4.209</v>
       </c>
       <c r="M5" t="n">
-        <v>4.266</v>
+        <v>4.251</v>
       </c>
       <c r="N5" t="n">
-        <v>4.285</v>
+        <v>4.272</v>
       </c>
       <c r="O5" t="n">
-        <v>4.327</v>
+        <v>4.312</v>
       </c>
       <c r="P5" t="n">
-        <v>4.621</v>
+        <v>4.609</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.499</v>
+        <v>5.489</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.188</v>
+        <v>3.2</v>
       </c>
       <c r="G6" t="n">
-        <v>3.353</v>
+        <v>3.368</v>
       </c>
       <c r="H6" t="n">
-        <v>3.598</v>
+        <v>3.61</v>
       </c>
       <c r="I6" t="n">
-        <v>3.806</v>
+        <v>3.812</v>
       </c>
       <c r="J6" t="n">
-        <v>4.113</v>
+        <v>4.107</v>
       </c>
       <c r="K6" t="n">
-        <v>4.336</v>
+        <v>4.319</v>
       </c>
       <c r="L6" t="n">
-        <v>4.345</v>
+        <v>4.327</v>
       </c>
       <c r="M6" t="n">
-        <v>4.422</v>
+        <v>4.407</v>
       </c>
       <c r="N6" t="n">
-        <v>4.452</v>
+        <v>4.439</v>
       </c>
       <c r="O6" t="n">
-        <v>4.593</v>
+        <v>4.578</v>
       </c>
       <c r="P6" t="n">
-        <v>5.053</v>
+        <v>5.041</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.895</v>
+        <v>5.885</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.168</v>
+        <v>3.18</v>
       </c>
       <c r="G7" t="n">
-        <v>3.317</v>
+        <v>3.332</v>
       </c>
       <c r="H7" t="n">
-        <v>3.544</v>
+        <v>3.557</v>
       </c>
       <c r="I7" t="n">
-        <v>3.743</v>
+        <v>3.749</v>
       </c>
       <c r="J7" t="n">
-        <v>4.046</v>
+        <v>4.04</v>
       </c>
       <c r="K7" t="n">
-        <v>4.25</v>
+        <v>4.233</v>
       </c>
       <c r="L7" t="n">
-        <v>4.253</v>
+        <v>4.235</v>
       </c>
       <c r="M7" t="n">
-        <v>4.326</v>
+        <v>4.311</v>
       </c>
       <c r="N7" t="n">
-        <v>4.344</v>
+        <v>4.331</v>
       </c>
       <c r="O7" t="n">
-        <v>4.491</v>
+        <v>4.475</v>
       </c>
       <c r="P7" t="n">
-        <v>4.837</v>
+        <v>4.825</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.663</v>
+        <v>5.653</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.583</v>
+        <v>5.593</v>
       </c>
       <c r="G8" t="n">
-        <v>6.257</v>
+        <v>6.271</v>
       </c>
       <c r="H8" t="n">
-        <v>6.705</v>
+        <v>6.717</v>
       </c>
       <c r="I8" t="n">
-        <v>6.906</v>
+        <v>6.912</v>
       </c>
       <c r="J8" t="n">
-        <v>7.303</v>
+        <v>7.297</v>
       </c>
       <c r="K8" t="n">
-        <v>8.009</v>
+        <v>7.992</v>
       </c>
       <c r="L8" t="n">
-        <v>8.321999999999999</v>
+        <v>8.304</v>
       </c>
       <c r="M8" t="n">
-        <v>8.615</v>
+        <v>8.6</v>
       </c>
       <c r="N8" t="n">
-        <v>8.756</v>
+        <v>8.743</v>
       </c>
       <c r="O8" t="n">
-        <v>9.047000000000001</v>
+        <v>9.032</v>
       </c>
       <c r="P8" t="n">
-        <v>9.244</v>
+        <v>9.231999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.964</v>
+        <v>9.954000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.747</v>
+        <v>2.745</v>
       </c>
       <c r="G9" t="n">
-        <v>2.974</v>
+        <v>2.972</v>
       </c>
       <c r="H9" t="n">
-        <v>3.188</v>
+        <v>3.181</v>
       </c>
       <c r="I9" t="n">
-        <v>3.336</v>
+        <v>3.294</v>
       </c>
       <c r="J9" t="n">
-        <v>3.506</v>
+        <v>3.487</v>
       </c>
       <c r="K9" t="n">
-        <v>3.602</v>
+        <v>3.573</v>
       </c>
       <c r="L9" t="n">
-        <v>3.707</v>
+        <v>3.677</v>
       </c>
       <c r="M9" t="n">
-        <v>3.74</v>
+        <v>3.715</v>
       </c>
       <c r="N9" t="n">
-        <v>3.856</v>
+        <v>3.84</v>
       </c>
       <c r="O9" t="n">
-        <v>3.92</v>
+        <v>3.905</v>
       </c>
       <c r="P9" t="n">
-        <v>4.052</v>
+        <v>4.041</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.12</v>
+        <v>4.11</v>
       </c>
       <c r="R9" t="n">
         <v>4.2</v>
       </c>
       <c r="S9" t="n">
-        <v>4.245</v>
+        <v>4.258</v>
       </c>
       <c r="T9" t="n">
-        <v>4.185</v>
+        <v>4.212</v>
       </c>
       <c r="U9" t="n">
-        <v>4.08</v>
+        <v>4.096</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.756</v>
+        <v>2.753</v>
       </c>
       <c r="G10" t="n">
-        <v>2.984</v>
+        <v>2.981</v>
       </c>
       <c r="H10" t="n">
-        <v>3.191</v>
+        <v>3.184</v>
       </c>
       <c r="I10" t="n">
-        <v>3.339</v>
+        <v>3.297</v>
       </c>
       <c r="J10" t="n">
-        <v>3.522</v>
+        <v>3.502</v>
       </c>
       <c r="K10" t="n">
-        <v>3.64</v>
+        <v>3.612</v>
       </c>
       <c r="L10" t="n">
-        <v>3.719</v>
+        <v>3.69</v>
       </c>
       <c r="M10" t="n">
-        <v>3.802</v>
+        <v>3.777</v>
       </c>
       <c r="N10" t="n">
-        <v>3.881</v>
+        <v>3.865</v>
       </c>
       <c r="O10" t="n">
-        <v>4.16</v>
+        <v>4.145</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.56</v>
+        <v>2.558</v>
       </c>
       <c r="G11" t="n">
-        <v>2.787</v>
+        <v>2.785</v>
       </c>
       <c r="H11" t="n">
-        <v>3.014</v>
+        <v>3.007</v>
       </c>
       <c r="I11" t="n">
-        <v>3.143</v>
+        <v>3.102</v>
       </c>
       <c r="J11" t="n">
-        <v>3.316</v>
+        <v>3.297</v>
       </c>
       <c r="K11" t="n">
-        <v>3.423</v>
+        <v>3.395</v>
       </c>
       <c r="L11" t="n">
-        <v>3.516</v>
+        <v>3.487</v>
       </c>
       <c r="M11" t="n">
-        <v>3.61</v>
+        <v>3.585</v>
       </c>
       <c r="N11" t="n">
-        <v>3.688</v>
+        <v>3.671</v>
       </c>
       <c r="O11" t="n">
-        <v>3.926</v>
+        <v>3.911</v>
       </c>
       <c r="P11" t="n">
-        <v>3.996</v>
+        <v>3.984</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.318</v>
+        <v>4.308</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.377</v>
+        <v>3.381</v>
       </c>
       <c r="G12" t="n">
-        <v>3.651</v>
+        <v>3.663</v>
       </c>
       <c r="H12" t="n">
-        <v>3.922</v>
+        <v>3.933</v>
       </c>
       <c r="I12" t="n">
-        <v>4.129</v>
+        <v>4.133</v>
       </c>
       <c r="J12" t="n">
-        <v>4.454</v>
+        <v>4.447</v>
       </c>
       <c r="K12" t="n">
-        <v>4.604</v>
+        <v>4.588</v>
       </c>
       <c r="L12" t="n">
-        <v>4.631</v>
+        <v>4.611</v>
       </c>
       <c r="M12" t="n">
-        <v>4.734</v>
+        <v>4.715</v>
       </c>
       <c r="N12" t="n">
-        <v>4.795</v>
+        <v>4.783</v>
       </c>
       <c r="O12" t="n">
-        <v>4.946</v>
+        <v>4.931</v>
       </c>
       <c r="P12" t="n">
-        <v>5.09</v>
+        <v>5.078</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.441</v>
+        <v>5.43</v>
       </c>
       <c r="R12" t="n">
         <v>5.696</v>
       </c>
       <c r="S12" t="n">
-        <v>5.954</v>
+        <v>5.967</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.13</v>
+        <v>3.134</v>
       </c>
       <c r="G13" t="n">
-        <v>3.341</v>
+        <v>3.353</v>
       </c>
       <c r="H13" t="n">
-        <v>3.59</v>
+        <v>3.601</v>
       </c>
       <c r="I13" t="n">
-        <v>3.777</v>
+        <v>3.78</v>
       </c>
       <c r="J13" t="n">
-        <v>4.091</v>
+        <v>4.084</v>
       </c>
       <c r="K13" t="n">
-        <v>4.237</v>
+        <v>4.221</v>
       </c>
       <c r="L13" t="n">
-        <v>4.27</v>
+        <v>4.25</v>
       </c>
       <c r="M13" t="n">
-        <v>4.361</v>
+        <v>4.343</v>
       </c>
       <c r="N13" t="n">
-        <v>4.423</v>
+        <v>4.411</v>
       </c>
       <c r="O13" t="n">
-        <v>4.574</v>
+        <v>4.56</v>
       </c>
       <c r="P13" t="n">
-        <v>4.682</v>
+        <v>4.67</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.962</v>
+        <v>4.951</v>
       </c>
       <c r="R13" t="n">
         <v>5.245</v>
       </c>
       <c r="S13" t="n">
-        <v>5.516</v>
+        <v>5.529</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.948</v>
+        <v>2.952</v>
       </c>
       <c r="G14" t="n">
-        <v>3.144</v>
+        <v>3.154</v>
       </c>
       <c r="H14" t="n">
-        <v>3.393</v>
+        <v>3.402</v>
       </c>
       <c r="I14" t="n">
-        <v>3.561</v>
+        <v>3.565</v>
       </c>
       <c r="J14" t="n">
-        <v>3.832</v>
+        <v>3.825</v>
       </c>
       <c r="K14" t="n">
-        <v>3.926</v>
+        <v>3.91</v>
       </c>
       <c r="L14" t="n">
-        <v>3.943</v>
+        <v>3.923</v>
       </c>
       <c r="M14" t="n">
-        <v>4.047</v>
+        <v>4.029</v>
       </c>
       <c r="N14" t="n">
-        <v>4.103</v>
+        <v>4.09</v>
       </c>
       <c r="O14" t="n">
-        <v>4.233</v>
+        <v>4.218</v>
       </c>
       <c r="P14" t="n">
-        <v>4.318</v>
+        <v>4.306</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.551</v>
+        <v>4.54</v>
       </c>
       <c r="R14" t="n">
         <v>4.76</v>
       </c>
       <c r="S14" t="n">
-        <v>4.968</v>
+        <v>4.982</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.925</v>
+        <v>2.929</v>
       </c>
       <c r="G15" t="n">
-        <v>3.118</v>
+        <v>3.129</v>
       </c>
       <c r="H15" t="n">
-        <v>3.364</v>
+        <v>3.373</v>
       </c>
       <c r="I15" t="n">
-        <v>3.512</v>
+        <v>3.515</v>
       </c>
       <c r="J15" t="n">
-        <v>3.771</v>
+        <v>3.763</v>
       </c>
       <c r="K15" t="n">
-        <v>3.879</v>
+        <v>3.863</v>
       </c>
       <c r="L15" t="n">
-        <v>3.88</v>
+        <v>3.859</v>
       </c>
       <c r="M15" t="n">
-        <v>3.96</v>
+        <v>3.942</v>
       </c>
       <c r="N15" t="n">
-        <v>4.005</v>
+        <v>3.993</v>
       </c>
       <c r="O15" t="n">
-        <v>4.176</v>
+        <v>4.162</v>
       </c>
       <c r="P15" t="n">
-        <v>4.214</v>
+        <v>4.202</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.453</v>
+        <v>4.442</v>
       </c>
       <c r="R15" t="n">
         <v>4.654</v>
       </c>
       <c r="S15" t="n">
-        <v>4.864</v>
+        <v>4.877</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.925</v>
+        <v>2.929</v>
       </c>
       <c r="G16" t="n">
-        <v>3.118</v>
+        <v>3.129</v>
       </c>
       <c r="H16" t="n">
-        <v>3.364</v>
+        <v>3.373</v>
       </c>
       <c r="I16" t="n">
-        <v>3.512</v>
+        <v>3.515</v>
       </c>
       <c r="J16" t="n">
-        <v>3.771</v>
+        <v>3.763</v>
       </c>
       <c r="K16" t="n">
-        <v>3.879</v>
+        <v>3.863</v>
       </c>
       <c r="L16" t="n">
-        <v>3.88</v>
+        <v>3.859</v>
       </c>
       <c r="M16" t="n">
-        <v>3.96</v>
+        <v>3.942</v>
       </c>
       <c r="N16" t="n">
-        <v>4.008</v>
+        <v>3.996</v>
       </c>
       <c r="O16" t="n">
-        <v>4.183</v>
+        <v>4.168</v>
       </c>
       <c r="P16" t="n">
-        <v>4.237</v>
+        <v>4.225</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.48</v>
+        <v>4.469</v>
       </c>
       <c r="R16" t="n">
         <v>4.682</v>
       </c>
       <c r="S16" t="n">
-        <v>4.893</v>
+        <v>4.906</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.787</v>
+        <v>2.784</v>
       </c>
       <c r="G17" t="n">
-        <v>3.036</v>
+        <v>3.032</v>
       </c>
       <c r="H17" t="n">
-        <v>3.246</v>
+        <v>3.237</v>
       </c>
       <c r="I17" t="n">
-        <v>3.393</v>
+        <v>3.354</v>
       </c>
       <c r="J17" t="n">
-        <v>3.592</v>
+        <v>3.574</v>
       </c>
       <c r="K17" t="n">
-        <v>3.717</v>
+        <v>3.691</v>
       </c>
       <c r="L17" t="n">
-        <v>3.804</v>
+        <v>3.775</v>
       </c>
       <c r="M17" t="n">
-        <v>3.929</v>
+        <v>3.904</v>
       </c>
       <c r="N17" t="n">
-        <v>3.99</v>
+        <v>3.976</v>
       </c>
       <c r="O17" t="n">
-        <v>4.18</v>
+        <v>4.166</v>
       </c>
       <c r="P17" t="n">
-        <v>4.281</v>
+        <v>4.271</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.788</v>
+        <v>2.785</v>
       </c>
       <c r="G18" t="n">
-        <v>3.037</v>
+        <v>3.033</v>
       </c>
       <c r="H18" t="n">
-        <v>3.246</v>
+        <v>3.237</v>
       </c>
       <c r="I18" t="n">
-        <v>3.394</v>
+        <v>3.354</v>
       </c>
       <c r="J18" t="n">
-        <v>3.592</v>
+        <v>3.574</v>
       </c>
       <c r="K18" t="n">
-        <v>3.718</v>
+        <v>3.692</v>
       </c>
       <c r="L18" t="n">
-        <v>3.804</v>
+        <v>3.775</v>
       </c>
       <c r="M18" t="n">
-        <v>3.929</v>
+        <v>3.904</v>
       </c>
       <c r="N18" t="n">
-        <v>3.991</v>
+        <v>3.977</v>
       </c>
       <c r="O18" t="n">
-        <v>4.178</v>
+        <v>4.164</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.936</v>
+        <v>2.94</v>
       </c>
       <c r="G19" t="n">
-        <v>3.132</v>
+        <v>3.142</v>
       </c>
       <c r="H19" t="n">
-        <v>3.381</v>
+        <v>3.389</v>
       </c>
       <c r="I19" t="n">
-        <v>3.546</v>
+        <v>3.549</v>
       </c>
       <c r="J19" t="n">
-        <v>3.812</v>
+        <v>3.805</v>
       </c>
       <c r="K19" t="n">
-        <v>3.921</v>
+        <v>3.906</v>
       </c>
       <c r="L19" t="n">
-        <v>3.941</v>
+        <v>3.92</v>
       </c>
       <c r="M19" t="n">
-        <v>4.038</v>
+        <v>4.02</v>
       </c>
       <c r="N19" t="n">
-        <v>4.095</v>
+        <v>4.083</v>
       </c>
       <c r="O19" t="n">
-        <v>4.219</v>
+        <v>4.205</v>
       </c>
       <c r="P19" t="n">
-        <v>4.276</v>
+        <v>4.263</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.491</v>
+        <v>4.48</v>
       </c>
       <c r="R19" t="n">
         <v>4.7</v>
       </c>
       <c r="S19" t="n">
-        <v>4.904</v>
+        <v>4.917</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.664</v>
+        <v>2.666</v>
       </c>
       <c r="G20" t="n">
-        <v>2.759</v>
+        <v>2.76</v>
       </c>
       <c r="H20" t="n">
-        <v>2.852</v>
+        <v>2.85</v>
       </c>
       <c r="I20" t="n">
-        <v>2.956</v>
+        <v>2.949</v>
       </c>
       <c r="J20" t="n">
-        <v>3.427</v>
+        <v>3.404</v>
       </c>
       <c r="K20" t="n">
-        <v>3.66</v>
+        <v>3.63</v>
       </c>
       <c r="L20" t="n">
-        <v>3.658</v>
+        <v>3.634</v>
       </c>
       <c r="M20" t="n">
-        <v>3.745</v>
+        <v>3.74</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.014</v>
+        <v>3.02</v>
       </c>
       <c r="G21" t="n">
-        <v>3.235</v>
+        <v>3.245</v>
       </c>
       <c r="H21" t="n">
-        <v>3.503</v>
+        <v>3.513</v>
       </c>
       <c r="I21" t="n">
-        <v>3.683</v>
+        <v>3.685</v>
       </c>
       <c r="J21" t="n">
-        <v>3.979</v>
+        <v>3.974</v>
       </c>
       <c r="K21" t="n">
-        <v>4.164</v>
+        <v>4.147</v>
       </c>
       <c r="L21" t="n">
-        <v>4.197</v>
+        <v>4.181</v>
       </c>
       <c r="M21" t="n">
-        <v>4.285</v>
+        <v>4.267</v>
       </c>
       <c r="N21" t="n">
-        <v>4.329</v>
+        <v>4.319</v>
       </c>
       <c r="O21" t="n">
-        <v>4.426</v>
+        <v>4.414</v>
       </c>
       <c r="P21" t="n">
-        <v>4.536</v>
+        <v>4.526</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.643</v>
+        <v>4.634</v>
       </c>
       <c r="R21" t="n">
         <v>4.753</v>
       </c>
       <c r="S21" t="n">
-        <v>4.857</v>
+        <v>4.87</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.96</v>
+        <v>2.966</v>
       </c>
       <c r="G22" t="n">
-        <v>3.18</v>
+        <v>3.19</v>
       </c>
       <c r="H22" t="n">
-        <v>3.435</v>
+        <v>3.445</v>
       </c>
       <c r="I22" t="n">
-        <v>3.601</v>
+        <v>3.604</v>
       </c>
       <c r="J22" t="n">
-        <v>3.864</v>
+        <v>3.859</v>
       </c>
       <c r="K22" t="n">
-        <v>4.046</v>
+        <v>4.028</v>
       </c>
       <c r="L22" t="n">
-        <v>4.064</v>
+        <v>4.048</v>
       </c>
       <c r="M22" t="n">
-        <v>4.156</v>
+        <v>4.139</v>
       </c>
       <c r="N22" t="n">
-        <v>4.203</v>
+        <v>4.193</v>
       </c>
       <c r="O22" t="n">
-        <v>4.297</v>
+        <v>4.285</v>
       </c>
       <c r="P22" t="n">
-        <v>4.399</v>
+        <v>4.39</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.502</v>
+        <v>4.493</v>
       </c>
       <c r="R22" t="n">
         <v>4.602</v>
       </c>
       <c r="S22" t="n">
-        <v>4.702</v>
+        <v>4.715</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.908</v>
+        <v>2.913</v>
       </c>
       <c r="G23" t="n">
-        <v>3.134</v>
+        <v>3.143</v>
       </c>
       <c r="H23" t="n">
-        <v>3.376</v>
+        <v>3.385</v>
       </c>
       <c r="I23" t="n">
-        <v>3.549</v>
+        <v>3.551</v>
       </c>
       <c r="J23" t="n">
-        <v>3.804</v>
+        <v>3.798</v>
       </c>
       <c r="K23" t="n">
-        <v>3.946</v>
+        <v>3.927</v>
       </c>
       <c r="L23" t="n">
-        <v>3.961</v>
+        <v>3.945</v>
       </c>
       <c r="M23" t="n">
-        <v>4.047</v>
+        <v>4.029</v>
       </c>
       <c r="N23" t="n">
-        <v>4.097</v>
+        <v>4.086</v>
       </c>
       <c r="O23" t="n">
-        <v>4.173</v>
+        <v>4.159</v>
       </c>
       <c r="P23" t="n">
-        <v>4.262</v>
+        <v>4.252</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.307</v>
+        <v>4.298</v>
       </c>
       <c r="R23" t="n">
         <v>4.388</v>
       </c>
       <c r="S23" t="n">
-        <v>4.459</v>
+        <v>4.472</v>
       </c>
       <c r="T23" t="n">
-        <v>4.397</v>
+        <v>4.425</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.844</v>
+        <v>2.849</v>
       </c>
       <c r="G24" t="n">
-        <v>3.044</v>
+        <v>3.053</v>
       </c>
       <c r="H24" t="n">
-        <v>3.274</v>
+        <v>3.283</v>
       </c>
       <c r="I24" t="n">
-        <v>3.487</v>
+        <v>3.489</v>
       </c>
       <c r="J24" t="n">
-        <v>3.698</v>
+        <v>3.691</v>
       </c>
       <c r="K24" t="n">
-        <v>3.828</v>
+        <v>3.81</v>
       </c>
       <c r="L24" t="n">
-        <v>3.843</v>
+        <v>3.826</v>
       </c>
       <c r="M24" t="n">
-        <v>3.906</v>
+        <v>3.887</v>
       </c>
       <c r="N24" t="n">
-        <v>3.972</v>
+        <v>3.961</v>
       </c>
       <c r="O24" t="n">
-        <v>4.171</v>
+        <v>4.158</v>
       </c>
       <c r="P24" t="n">
-        <v>4.201</v>
+        <v>4.19</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.234</v>
+        <v>4.225</v>
       </c>
       <c r="R24" t="n">
         <v>4.309</v>
       </c>
       <c r="S24" t="n">
-        <v>4.374</v>
+        <v>4.387</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.903</v>
+        <v>2.908</v>
       </c>
       <c r="G25" t="n">
-        <v>3.134</v>
+        <v>3.143</v>
       </c>
       <c r="H25" t="n">
-        <v>3.38</v>
+        <v>3.389</v>
       </c>
       <c r="I25" t="n">
-        <v>3.558</v>
+        <v>3.56</v>
       </c>
       <c r="J25" t="n">
-        <v>3.82</v>
+        <v>3.813</v>
       </c>
       <c r="K25" t="n">
-        <v>3.977</v>
+        <v>3.958</v>
       </c>
       <c r="L25" t="n">
-        <v>3.992</v>
+        <v>3.975</v>
       </c>
       <c r="M25" t="n">
-        <v>4.078</v>
+        <v>4.06</v>
       </c>
       <c r="N25" t="n">
-        <v>4.124</v>
+        <v>4.113</v>
       </c>
       <c r="O25" t="n">
-        <v>4.202</v>
+        <v>4.188</v>
       </c>
       <c r="P25" t="n">
-        <v>4.284</v>
+        <v>4.273</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.341</v>
+        <v>4.332</v>
       </c>
       <c r="R25" t="n">
         <v>4.411</v>
       </c>
       <c r="S25" t="n">
-        <v>4.482</v>
+        <v>4.495</v>
       </c>
       <c r="T25" t="n">
-        <v>4.415</v>
+        <v>4.443</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.23</v>
+        <v>3.237</v>
       </c>
       <c r="G26" t="n">
-        <v>3.438</v>
+        <v>3.449</v>
       </c>
       <c r="H26" t="n">
-        <v>3.767</v>
+        <v>3.778</v>
       </c>
       <c r="I26" t="n">
-        <v>3.962</v>
+        <v>3.966</v>
       </c>
       <c r="J26" t="n">
-        <v>4.387</v>
+        <v>4.377</v>
       </c>
       <c r="K26" t="n">
-        <v>4.778</v>
+        <v>4.759</v>
       </c>
       <c r="L26" t="n">
-        <v>4.851</v>
+        <v>4.831</v>
       </c>
       <c r="M26" t="n">
-        <v>4.981</v>
+        <v>4.962</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.26</v>
+        <v>5.246</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.03</v>
+        <v>3.036</v>
       </c>
       <c r="G27" t="n">
-        <v>3.202</v>
+        <v>3.213</v>
       </c>
       <c r="H27" t="n">
-        <v>3.456</v>
+        <v>3.466</v>
       </c>
       <c r="I27" t="n">
-        <v>3.626</v>
+        <v>3.631</v>
       </c>
       <c r="J27" t="n">
-        <v>3.923</v>
+        <v>3.915</v>
       </c>
       <c r="K27" t="n">
-        <v>4.101</v>
+        <v>4.083</v>
       </c>
       <c r="L27" t="n">
-        <v>4.118</v>
+        <v>4.097</v>
       </c>
       <c r="M27" t="n">
-        <v>4.203</v>
+        <v>4.183</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.362</v>
+        <v>4.348</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.133</v>
+        <v>3.139</v>
       </c>
       <c r="G28" t="n">
-        <v>3.313</v>
+        <v>3.325</v>
       </c>
       <c r="H28" t="n">
-        <v>3.582</v>
+        <v>3.593</v>
       </c>
       <c r="I28" t="n">
-        <v>3.763</v>
+        <v>3.768</v>
       </c>
       <c r="J28" t="n">
-        <v>4.096</v>
+        <v>4.088</v>
       </c>
       <c r="K28" t="n">
-        <v>4.293</v>
+        <v>4.275</v>
       </c>
       <c r="L28" t="n">
-        <v>4.321</v>
+        <v>4.3</v>
       </c>
       <c r="M28" t="n">
-        <v>4.415</v>
+        <v>4.395</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.654</v>
+        <v>4.64</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.979</v>
+        <v>2.984</v>
       </c>
       <c r="G29" t="n">
-        <v>3.148</v>
+        <v>3.157</v>
       </c>
       <c r="H29" t="n">
-        <v>3.393</v>
+        <v>3.402</v>
       </c>
       <c r="I29" t="n">
-        <v>3.551</v>
+        <v>3.556</v>
       </c>
       <c r="J29" t="n">
-        <v>3.835</v>
+        <v>3.827</v>
       </c>
       <c r="K29" t="n">
-        <v>3.997</v>
+        <v>3.979</v>
       </c>
       <c r="L29" t="n">
-        <v>4.004</v>
+        <v>3.982</v>
       </c>
       <c r="M29" t="n">
-        <v>4.066</v>
+        <v>4.046</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.234</v>
+        <v>4.22</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.263</v>
+        <v>3.271</v>
       </c>
       <c r="G30" t="n">
-        <v>3.405</v>
+        <v>3.415</v>
       </c>
       <c r="H30" t="n">
-        <v>3.694</v>
+        <v>3.703</v>
       </c>
       <c r="I30" t="n">
-        <v>3.88</v>
+        <v>3.883</v>
       </c>
       <c r="J30" t="n">
-        <v>4.244</v>
+        <v>4.232</v>
       </c>
       <c r="K30" t="n">
-        <v>4.573</v>
+        <v>4.553</v>
       </c>
       <c r="L30" t="n">
-        <v>4.623</v>
+        <v>4.602</v>
       </c>
       <c r="M30" t="n">
-        <v>4.743</v>
+        <v>4.721</v>
       </c>
       <c r="N30" t="n">
-        <v>4.909</v>
+        <v>4.897</v>
       </c>
       <c r="O30" t="n">
-        <v>5.208</v>
+        <v>5.195</v>
       </c>
       <c r="P30" t="n">
-        <v>5.43</v>
+        <v>5.419</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.187</v>
+        <v>6.175</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.592</v>
+        <v>3.6</v>
       </c>
       <c r="G31" t="n">
-        <v>3.771</v>
+        <v>3.781</v>
       </c>
       <c r="H31" t="n">
-        <v>4.11</v>
+        <v>4.119</v>
       </c>
       <c r="I31" t="n">
-        <v>4.309</v>
+        <v>4.312</v>
       </c>
       <c r="J31" t="n">
-        <v>4.737</v>
+        <v>4.726</v>
       </c>
       <c r="K31" t="n">
-        <v>5.108</v>
+        <v>5.088</v>
       </c>
       <c r="L31" t="n">
-        <v>5.235</v>
+        <v>5.215</v>
       </c>
       <c r="M31" t="n">
-        <v>5.473</v>
+        <v>5.452</v>
       </c>
       <c r="N31" t="n">
-        <v>5.768</v>
+        <v>5.756</v>
       </c>
       <c r="O31" t="n">
-        <v>6.244</v>
+        <v>6.231</v>
       </c>
       <c r="P31" t="n">
-        <v>6.418</v>
+        <v>6.407</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.16</v>
+        <v>7.148</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.361</v>
+        <v>3.37</v>
       </c>
       <c r="G32" t="n">
-        <v>3.523</v>
+        <v>3.533</v>
       </c>
       <c r="H32" t="n">
-        <v>3.838</v>
+        <v>3.847</v>
       </c>
       <c r="I32" t="n">
-        <v>4.039</v>
+        <v>4.042</v>
       </c>
       <c r="J32" t="n">
-        <v>4.424</v>
+        <v>4.412</v>
       </c>
       <c r="K32" t="n">
-        <v>4.758</v>
+        <v>4.738</v>
       </c>
       <c r="L32" t="n">
-        <v>4.827</v>
+        <v>4.806</v>
       </c>
       <c r="M32" t="n">
-        <v>5.015</v>
+        <v>4.994</v>
       </c>
       <c r="N32" t="n">
-        <v>5.27</v>
+        <v>5.258</v>
       </c>
       <c r="O32" t="n">
-        <v>5.653</v>
+        <v>5.64</v>
       </c>
       <c r="P32" t="n">
-        <v>5.89</v>
+        <v>5.879</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.648</v>
+        <v>6.636</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.128</v>
+        <v>3.136</v>
       </c>
       <c r="G33" t="n">
-        <v>3.27</v>
+        <v>3.278</v>
       </c>
       <c r="H33" t="n">
-        <v>3.512</v>
+        <v>3.52</v>
       </c>
       <c r="I33" t="n">
-        <v>3.666</v>
+        <v>3.669</v>
       </c>
       <c r="J33" t="n">
-        <v>3.95</v>
+        <v>3.939</v>
       </c>
       <c r="K33" t="n">
-        <v>4.215</v>
+        <v>4.194</v>
       </c>
       <c r="L33" t="n">
-        <v>4.229</v>
+        <v>4.208</v>
       </c>
       <c r="M33" t="n">
-        <v>4.272</v>
+        <v>4.251</v>
       </c>
       <c r="N33" t="n">
-        <v>4.298</v>
+        <v>4.286</v>
       </c>
       <c r="O33" t="n">
-        <v>4.364</v>
+        <v>4.351</v>
       </c>
       <c r="P33" t="n">
-        <v>4.462</v>
+        <v>4.451</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.903</v>
+        <v>4.892</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.188</v>
+        <v>3.196</v>
       </c>
       <c r="G34" t="n">
-        <v>3.323</v>
+        <v>3.332</v>
       </c>
       <c r="H34" t="n">
-        <v>3.574</v>
+        <v>3.583</v>
       </c>
       <c r="I34" t="n">
-        <v>3.734</v>
+        <v>3.737</v>
       </c>
       <c r="J34" t="n">
-        <v>4.022</v>
+        <v>4.01</v>
       </c>
       <c r="K34" t="n">
-        <v>4.291</v>
+        <v>4.27</v>
       </c>
       <c r="L34" t="n">
-        <v>4.307</v>
+        <v>4.286</v>
       </c>
       <c r="M34" t="n">
-        <v>4.363</v>
+        <v>4.342</v>
       </c>
       <c r="N34" t="n">
-        <v>4.403</v>
+        <v>4.391</v>
       </c>
       <c r="O34" t="n">
-        <v>4.533</v>
+        <v>4.52</v>
       </c>
       <c r="P34" t="n">
-        <v>4.757</v>
+        <v>4.746</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.604</v>
+        <v>5.593</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.162</v>
+        <v>3.17</v>
       </c>
       <c r="G35" t="n">
-        <v>3.297</v>
+        <v>3.306</v>
       </c>
       <c r="H35" t="n">
-        <v>3.542</v>
+        <v>3.551</v>
       </c>
       <c r="I35" t="n">
-        <v>3.701</v>
+        <v>3.704</v>
       </c>
       <c r="J35" t="n">
-        <v>3.99</v>
+        <v>3.979</v>
       </c>
       <c r="K35" t="n">
-        <v>4.245</v>
+        <v>4.224</v>
       </c>
       <c r="L35" t="n">
-        <v>4.263</v>
+        <v>4.242</v>
       </c>
       <c r="M35" t="n">
-        <v>4.309</v>
+        <v>4.288</v>
       </c>
       <c r="N35" t="n">
-        <v>4.339</v>
+        <v>4.327</v>
       </c>
       <c r="O35" t="n">
-        <v>4.43</v>
+        <v>4.417</v>
       </c>
       <c r="P35" t="n">
-        <v>4.559</v>
+        <v>4.548</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.24</v>
+        <v>5.228</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.051</v>
+        <v>3.056</v>
       </c>
       <c r="G36" t="n">
-        <v>3.18</v>
+        <v>3.186</v>
       </c>
       <c r="H36" t="n">
-        <v>3.418</v>
+        <v>3.425</v>
       </c>
       <c r="I36" t="n">
-        <v>3.576</v>
+        <v>3.579</v>
       </c>
       <c r="J36" t="n">
-        <v>3.887</v>
+        <v>3.875</v>
       </c>
       <c r="K36" t="n">
-        <v>4.14</v>
+        <v>4.12</v>
       </c>
       <c r="L36" t="n">
-        <v>4.153</v>
+        <v>4.132</v>
       </c>
       <c r="M36" t="n">
-        <v>4.175</v>
+        <v>4.154</v>
       </c>
       <c r="N36" t="n">
-        <v>4.203</v>
+        <v>4.191</v>
       </c>
       <c r="O36" t="n">
-        <v>4.272</v>
+        <v>4.258</v>
       </c>
       <c r="P36" t="n">
-        <v>4.36</v>
+        <v>4.349</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.62</v>
+        <v>4.609</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.935</v>
+        <v>3.943</v>
       </c>
       <c r="G37" t="n">
-        <v>4.464</v>
+        <v>4.474</v>
       </c>
       <c r="H37" t="n">
-        <v>5.082</v>
+        <v>5.091</v>
       </c>
       <c r="I37" t="n">
-        <v>5.37</v>
+        <v>5.373</v>
       </c>
       <c r="J37" t="n">
-        <v>6.226</v>
+        <v>6.215</v>
       </c>
       <c r="K37" t="n">
-        <v>7.148</v>
+        <v>7.129</v>
       </c>
       <c r="L37" t="n">
-        <v>7.436</v>
+        <v>7.415</v>
       </c>
       <c r="M37" t="n">
-        <v>7.745</v>
+        <v>7.724</v>
       </c>
       <c r="N37" t="n">
-        <v>7.924</v>
+        <v>7.912</v>
       </c>
       <c r="O37" t="n">
-        <v>8.122999999999999</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="P37" t="n">
-        <v>8.220000000000001</v>
+        <v>8.209</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.65</v>
+        <v>8.638999999999999</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.997</v>
+        <v>5.005</v>
       </c>
       <c r="G38" t="n">
-        <v>5.779</v>
+        <v>5.789</v>
       </c>
       <c r="H38" t="n">
-        <v>6.609</v>
+        <v>6.618</v>
       </c>
       <c r="I38" t="n">
-        <v>7.054</v>
+        <v>7.057</v>
       </c>
       <c r="J38" t="n">
-        <v>8.17</v>
+        <v>8.159000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.271000000000001</v>
+        <v>9.252000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.718999999999999</v>
+        <v>9.698</v>
       </c>
       <c r="M38" t="n">
-        <v>10.157</v>
+        <v>10.136</v>
       </c>
       <c r="N38" t="n">
-        <v>10.343</v>
+        <v>10.331</v>
       </c>
       <c r="O38" t="n">
-        <v>10.523</v>
+        <v>10.51</v>
       </c>
       <c r="P38" t="n">
-        <v>10.618</v>
+        <v>10.607</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.101</v>
+        <v>11.089</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.317</v>
+        <v>4.325</v>
       </c>
       <c r="G39" t="n">
-        <v>4.977</v>
+        <v>4.987</v>
       </c>
       <c r="H39" t="n">
-        <v>5.674</v>
+        <v>5.683</v>
       </c>
       <c r="I39" t="n">
-        <v>6.058</v>
+        <v>6.061</v>
       </c>
       <c r="J39" t="n">
-        <v>7.043</v>
+        <v>7.031</v>
       </c>
       <c r="K39" t="n">
-        <v>8.103</v>
+        <v>8.084</v>
       </c>
       <c r="L39" t="n">
-        <v>8.474</v>
+        <v>8.454000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.792999999999999</v>
+        <v>8.772</v>
       </c>
       <c r="N39" t="n">
-        <v>8.971</v>
+        <v>8.959</v>
       </c>
       <c r="O39" t="n">
-        <v>9.173999999999999</v>
+        <v>9.161</v>
       </c>
       <c r="P39" t="n">
-        <v>9.272</v>
+        <v>9.260999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.746</v>
+        <v>9.734999999999999</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.454</v>
+        <v>3.463</v>
       </c>
       <c r="G40" t="n">
-        <v>3.643</v>
+        <v>3.653</v>
       </c>
       <c r="H40" t="n">
-        <v>3.953</v>
+        <v>3.962</v>
       </c>
       <c r="I40" t="n">
-        <v>4.154</v>
+        <v>4.157</v>
       </c>
       <c r="J40" t="n">
-        <v>4.536</v>
+        <v>4.524</v>
       </c>
       <c r="K40" t="n">
-        <v>4.879</v>
+        <v>4.859</v>
       </c>
       <c r="L40" t="n">
-        <v>4.948</v>
+        <v>4.928</v>
       </c>
       <c r="M40" t="n">
-        <v>5.085</v>
+        <v>5.064</v>
       </c>
       <c r="N40" t="n">
-        <v>5.267</v>
+        <v>5.255</v>
       </c>
       <c r="O40" t="n">
-        <v>5.587</v>
+        <v>5.574</v>
       </c>
       <c r="P40" t="n">
-        <v>5.851</v>
+        <v>5.84</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.638</v>
+        <v>6.626</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.841</v>
+        <v>3.849</v>
       </c>
       <c r="G41" t="n">
-        <v>4.072</v>
+        <v>4.082</v>
       </c>
       <c r="H41" t="n">
-        <v>4.439</v>
+        <v>4.448</v>
       </c>
       <c r="I41" t="n">
-        <v>4.657</v>
+        <v>4.66</v>
       </c>
       <c r="J41" t="n">
-        <v>5.092</v>
+        <v>5.081</v>
       </c>
       <c r="K41" t="n">
-        <v>5.482</v>
+        <v>5.462</v>
       </c>
       <c r="L41" t="n">
-        <v>5.626</v>
+        <v>5.605</v>
       </c>
       <c r="M41" t="n">
-        <v>5.888</v>
+        <v>5.867</v>
       </c>
       <c r="N41" t="n">
-        <v>6.197</v>
+        <v>6.186</v>
       </c>
       <c r="O41" t="n">
-        <v>6.702</v>
+        <v>6.689</v>
       </c>
       <c r="P41" t="n">
-        <v>6.911</v>
+        <v>6.9</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.685</v>
+        <v>7.673</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.576</v>
+        <v>3.584</v>
       </c>
       <c r="G42" t="n">
-        <v>3.792</v>
+        <v>3.802</v>
       </c>
       <c r="H42" t="n">
-        <v>4.129</v>
+        <v>4.138</v>
       </c>
       <c r="I42" t="n">
-        <v>4.342</v>
+        <v>4.345</v>
       </c>
       <c r="J42" t="n">
-        <v>4.74</v>
+        <v>4.728</v>
       </c>
       <c r="K42" t="n">
-        <v>5.1</v>
+        <v>5.08</v>
       </c>
       <c r="L42" t="n">
-        <v>5.184</v>
+        <v>5.163</v>
       </c>
       <c r="M42" t="n">
-        <v>5.392</v>
+        <v>5.371</v>
       </c>
       <c r="N42" t="n">
-        <v>5.681</v>
+        <v>5.669</v>
       </c>
       <c r="O42" t="n">
-        <v>6.079</v>
+        <v>6.066</v>
       </c>
       <c r="P42" t="n">
-        <v>6.353</v>
+        <v>6.342</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.15</v>
+        <v>7.139</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.276</v>
+        <v>3.284</v>
       </c>
       <c r="G43" t="n">
-        <v>3.453</v>
+        <v>3.461</v>
       </c>
       <c r="H43" t="n">
-        <v>3.713</v>
+        <v>3.722</v>
       </c>
       <c r="I43" t="n">
-        <v>3.875</v>
+        <v>3.878</v>
       </c>
       <c r="J43" t="n">
-        <v>4.177</v>
+        <v>4.166</v>
       </c>
       <c r="K43" t="n">
-        <v>4.447</v>
+        <v>4.426</v>
       </c>
       <c r="L43" t="n">
-        <v>4.471</v>
+        <v>4.451</v>
       </c>
       <c r="M43" t="n">
-        <v>4.527</v>
+        <v>4.506</v>
       </c>
       <c r="N43" t="n">
-        <v>4.567</v>
+        <v>4.555</v>
       </c>
       <c r="O43" t="n">
-        <v>4.677</v>
+        <v>4.664</v>
       </c>
       <c r="P43" t="n">
-        <v>4.828</v>
+        <v>4.817</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.514</v>
+        <v>5.502</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.129</v>
+        <v>3.134</v>
       </c>
       <c r="G44" t="n">
-        <v>3.289</v>
+        <v>3.295</v>
       </c>
       <c r="H44" t="n">
-        <v>3.541</v>
+        <v>3.548</v>
       </c>
       <c r="I44" t="n">
-        <v>3.703</v>
+        <v>3.706</v>
       </c>
       <c r="J44" t="n">
-        <v>4.028</v>
+        <v>4.016</v>
       </c>
       <c r="K44" t="n">
-        <v>4.291</v>
+        <v>4.271</v>
       </c>
       <c r="L44" t="n">
-        <v>4.314</v>
+        <v>4.294</v>
       </c>
       <c r="M44" t="n">
-        <v>4.345</v>
+        <v>4.324</v>
       </c>
       <c r="N44" t="n">
-        <v>4.384</v>
+        <v>4.372</v>
       </c>
       <c r="O44" t="n">
-        <v>4.473</v>
+        <v>4.459</v>
       </c>
       <c r="P44" t="n">
-        <v>4.59</v>
+        <v>4.579</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.884</v>
+        <v>4.873</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-17 ~ 2026-06-17
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.461</v>
+        <v>3.469</v>
       </c>
       <c r="G2" t="n">
-        <v>3.77</v>
+        <v>3.779</v>
       </c>
       <c r="H2" t="n">
-        <v>4.034</v>
+        <v>4.043</v>
       </c>
       <c r="I2" t="n">
-        <v>4.157</v>
+        <v>4.17</v>
       </c>
       <c r="J2" t="n">
-        <v>4.456</v>
+        <v>4.459</v>
       </c>
       <c r="K2" t="n">
-        <v>4.803</v>
+        <v>4.793</v>
       </c>
       <c r="L2" t="n">
-        <v>4.96</v>
+        <v>4.945</v>
       </c>
       <c r="M2" t="n">
-        <v>5.193</v>
+        <v>5.188</v>
       </c>
       <c r="N2" t="n">
-        <v>5.459</v>
+        <v>5.453</v>
       </c>
       <c r="O2" t="n">
-        <v>5.712</v>
+        <v>5.699</v>
       </c>
       <c r="P2" t="n">
-        <v>5.94</v>
+        <v>5.907</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.577</v>
+        <v>6.528</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.482</v>
+        <v>4.49</v>
       </c>
       <c r="G3" t="n">
-        <v>4.971</v>
+        <v>4.981</v>
       </c>
       <c r="H3" t="n">
-        <v>5.269</v>
+        <v>5.278</v>
       </c>
       <c r="I3" t="n">
-        <v>5.386</v>
+        <v>5.399</v>
       </c>
       <c r="J3" t="n">
-        <v>5.702</v>
+        <v>5.704</v>
       </c>
       <c r="K3" t="n">
-        <v>6.119</v>
+        <v>6.109</v>
       </c>
       <c r="L3" t="n">
-        <v>6.346</v>
+        <v>6.331</v>
       </c>
       <c r="M3" t="n">
-        <v>6.609</v>
+        <v>6.604</v>
       </c>
       <c r="N3" t="n">
-        <v>6.819</v>
+        <v>6.812</v>
       </c>
       <c r="O3" t="n">
-        <v>7.022</v>
+        <v>7.009</v>
       </c>
       <c r="P3" t="n">
-        <v>7.118</v>
+        <v>7.085</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.643</v>
+        <v>7.594</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.974</v>
+        <v>3.982</v>
       </c>
       <c r="G4" t="n">
-        <v>4.353</v>
+        <v>4.362</v>
       </c>
       <c r="H4" t="n">
-        <v>4.678</v>
+        <v>4.687</v>
       </c>
       <c r="I4" t="n">
-        <v>4.829</v>
+        <v>4.842</v>
       </c>
       <c r="J4" t="n">
-        <v>5.145</v>
+        <v>5.148</v>
       </c>
       <c r="K4" t="n">
-        <v>5.557</v>
+        <v>5.548</v>
       </c>
       <c r="L4" t="n">
-        <v>5.715</v>
+        <v>5.699</v>
       </c>
       <c r="M4" t="n">
-        <v>5.967</v>
+        <v>5.962</v>
       </c>
       <c r="N4" t="n">
-        <v>6.147</v>
+        <v>6.14</v>
       </c>
       <c r="O4" t="n">
-        <v>6.374</v>
+        <v>6.361</v>
       </c>
       <c r="P4" t="n">
-        <v>6.47</v>
+        <v>6.437</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.998</v>
+        <v>6.949</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.159</v>
+        <v>3.167</v>
       </c>
       <c r="G5" t="n">
-        <v>3.313</v>
+        <v>3.322</v>
       </c>
       <c r="H5" t="n">
-        <v>3.541</v>
+        <v>3.55</v>
       </c>
       <c r="I5" t="n">
-        <v>3.73</v>
+        <v>3.743</v>
       </c>
       <c r="J5" t="n">
-        <v>4.016</v>
+        <v>4.018</v>
       </c>
       <c r="K5" t="n">
-        <v>4.206</v>
+        <v>4.196</v>
       </c>
       <c r="L5" t="n">
-        <v>4.209</v>
+        <v>4.194</v>
       </c>
       <c r="M5" t="n">
-        <v>4.251</v>
+        <v>4.246</v>
       </c>
       <c r="N5" t="n">
-        <v>4.272</v>
+        <v>4.265</v>
       </c>
       <c r="O5" t="n">
-        <v>4.312</v>
+        <v>4.299</v>
       </c>
       <c r="P5" t="n">
-        <v>4.609</v>
+        <v>4.575</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.489</v>
+        <v>5.44</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.2</v>
+        <v>3.208</v>
       </c>
       <c r="G6" t="n">
-        <v>3.368</v>
+        <v>3.377</v>
       </c>
       <c r="H6" t="n">
-        <v>3.61</v>
+        <v>3.62</v>
       </c>
       <c r="I6" t="n">
-        <v>3.812</v>
+        <v>3.825</v>
       </c>
       <c r="J6" t="n">
-        <v>4.107</v>
+        <v>4.109</v>
       </c>
       <c r="K6" t="n">
-        <v>4.319</v>
+        <v>4.308</v>
       </c>
       <c r="L6" t="n">
-        <v>4.327</v>
+        <v>4.312</v>
       </c>
       <c r="M6" t="n">
-        <v>4.407</v>
+        <v>4.401</v>
       </c>
       <c r="N6" t="n">
-        <v>4.439</v>
+        <v>4.432</v>
       </c>
       <c r="O6" t="n">
-        <v>4.578</v>
+        <v>4.565</v>
       </c>
       <c r="P6" t="n">
-        <v>5.041</v>
+        <v>5.008</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.885</v>
+        <v>5.836</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.18</v>
+        <v>3.188</v>
       </c>
       <c r="G7" t="n">
-        <v>3.332</v>
+        <v>3.341</v>
       </c>
       <c r="H7" t="n">
-        <v>3.557</v>
+        <v>3.566</v>
       </c>
       <c r="I7" t="n">
-        <v>3.749</v>
+        <v>3.762</v>
       </c>
       <c r="J7" t="n">
-        <v>4.04</v>
+        <v>4.042</v>
       </c>
       <c r="K7" t="n">
-        <v>4.233</v>
+        <v>4.223</v>
       </c>
       <c r="L7" t="n">
-        <v>4.235</v>
+        <v>4.22</v>
       </c>
       <c r="M7" t="n">
-        <v>4.311</v>
+        <v>4.305</v>
       </c>
       <c r="N7" t="n">
-        <v>4.331</v>
+        <v>4.324</v>
       </c>
       <c r="O7" t="n">
-        <v>4.475</v>
+        <v>4.462</v>
       </c>
       <c r="P7" t="n">
-        <v>4.825</v>
+        <v>4.791</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.653</v>
+        <v>5.604</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.593</v>
+        <v>5.602</v>
       </c>
       <c r="G8" t="n">
-        <v>6.271</v>
+        <v>6.28</v>
       </c>
       <c r="H8" t="n">
-        <v>6.717</v>
+        <v>6.726</v>
       </c>
       <c r="I8" t="n">
-        <v>6.912</v>
+        <v>6.926</v>
       </c>
       <c r="J8" t="n">
-        <v>7.297</v>
+        <v>7.299</v>
       </c>
       <c r="K8" t="n">
-        <v>7.992</v>
+        <v>7.983</v>
       </c>
       <c r="L8" t="n">
-        <v>8.304</v>
+        <v>8.289</v>
       </c>
       <c r="M8" t="n">
-        <v>8.6</v>
+        <v>8.593999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.743</v>
+        <v>8.736000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.032</v>
+        <v>9.019</v>
       </c>
       <c r="P8" t="n">
-        <v>9.231999999999999</v>
+        <v>9.198</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.954000000000001</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.745</v>
+        <v>2.739</v>
       </c>
       <c r="G9" t="n">
-        <v>2.972</v>
+        <v>2.962</v>
       </c>
       <c r="H9" t="n">
-        <v>3.181</v>
+        <v>3.173</v>
       </c>
       <c r="I9" t="n">
-        <v>3.294</v>
+        <v>3.27</v>
       </c>
       <c r="J9" t="n">
-        <v>3.487</v>
+        <v>3.473</v>
       </c>
       <c r="K9" t="n">
-        <v>3.573</v>
+        <v>3.561</v>
       </c>
       <c r="L9" t="n">
-        <v>3.677</v>
+        <v>3.65</v>
       </c>
       <c r="M9" t="n">
-        <v>3.715</v>
+        <v>3.7</v>
       </c>
       <c r="N9" t="n">
-        <v>3.84</v>
+        <v>3.825</v>
       </c>
       <c r="O9" t="n">
-        <v>3.905</v>
+        <v>3.889</v>
       </c>
       <c r="P9" t="n">
-        <v>4.041</v>
+        <v>4.008</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.11</v>
+        <v>4.062</v>
       </c>
       <c r="R9" t="n">
-        <v>4.2</v>
+        <v>4.143</v>
       </c>
       <c r="S9" t="n">
-        <v>4.258</v>
+        <v>4.195</v>
       </c>
       <c r="T9" t="n">
-        <v>4.212</v>
+        <v>4.155</v>
       </c>
       <c r="U9" t="n">
-        <v>4.096</v>
+        <v>4.039</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.753</v>
+        <v>2.747</v>
       </c>
       <c r="G10" t="n">
-        <v>2.981</v>
+        <v>2.971</v>
       </c>
       <c r="H10" t="n">
-        <v>3.184</v>
+        <v>3.176</v>
       </c>
       <c r="I10" t="n">
-        <v>3.297</v>
+        <v>3.273</v>
       </c>
       <c r="J10" t="n">
-        <v>3.502</v>
+        <v>3.489</v>
       </c>
       <c r="K10" t="n">
-        <v>3.612</v>
+        <v>3.601</v>
       </c>
       <c r="L10" t="n">
-        <v>3.69</v>
+        <v>3.662</v>
       </c>
       <c r="M10" t="n">
-        <v>3.777</v>
+        <v>3.762</v>
       </c>
       <c r="N10" t="n">
-        <v>3.865</v>
+        <v>3.851</v>
       </c>
       <c r="O10" t="n">
-        <v>4.145</v>
+        <v>4.13</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.558</v>
+        <v>2.552</v>
       </c>
       <c r="G11" t="n">
-        <v>2.785</v>
+        <v>2.774</v>
       </c>
       <c r="H11" t="n">
-        <v>3.007</v>
+        <v>2.998</v>
       </c>
       <c r="I11" t="n">
-        <v>3.102</v>
+        <v>3.077</v>
       </c>
       <c r="J11" t="n">
-        <v>3.297</v>
+        <v>3.284</v>
       </c>
       <c r="K11" t="n">
-        <v>3.395</v>
+        <v>3.383</v>
       </c>
       <c r="L11" t="n">
-        <v>3.487</v>
+        <v>3.459</v>
       </c>
       <c r="M11" t="n">
-        <v>3.585</v>
+        <v>3.57</v>
       </c>
       <c r="N11" t="n">
-        <v>3.671</v>
+        <v>3.658</v>
       </c>
       <c r="O11" t="n">
-        <v>3.911</v>
+        <v>3.896</v>
       </c>
       <c r="P11" t="n">
-        <v>3.984</v>
+        <v>3.952</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.308</v>
+        <v>4.26</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.381</v>
+        <v>3.388</v>
       </c>
       <c r="G12" t="n">
-        <v>3.663</v>
+        <v>3.674</v>
       </c>
       <c r="H12" t="n">
-        <v>3.933</v>
+        <v>3.941</v>
       </c>
       <c r="I12" t="n">
-        <v>4.133</v>
+        <v>4.14</v>
       </c>
       <c r="J12" t="n">
-        <v>4.447</v>
+        <v>4.446</v>
       </c>
       <c r="K12" t="n">
-        <v>4.588</v>
+        <v>4.578</v>
       </c>
       <c r="L12" t="n">
-        <v>4.611</v>
+        <v>4.596</v>
       </c>
       <c r="M12" t="n">
-        <v>4.715</v>
+        <v>4.708</v>
       </c>
       <c r="N12" t="n">
-        <v>4.783</v>
+        <v>4.775</v>
       </c>
       <c r="O12" t="n">
-        <v>4.931</v>
+        <v>4.92</v>
       </c>
       <c r="P12" t="n">
-        <v>5.078</v>
+        <v>5.048</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.43</v>
+        <v>5.382</v>
       </c>
       <c r="R12" t="n">
-        <v>5.696</v>
+        <v>5.64</v>
       </c>
       <c r="S12" t="n">
-        <v>5.967</v>
+        <v>5.904</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.134</v>
+        <v>3.142</v>
       </c>
       <c r="G13" t="n">
-        <v>3.353</v>
+        <v>3.364</v>
       </c>
       <c r="H13" t="n">
-        <v>3.601</v>
+        <v>3.608</v>
       </c>
       <c r="I13" t="n">
-        <v>3.78</v>
+        <v>3.788</v>
       </c>
       <c r="J13" t="n">
-        <v>4.084</v>
+        <v>4.083</v>
       </c>
       <c r="K13" t="n">
-        <v>4.221</v>
+        <v>4.211</v>
       </c>
       <c r="L13" t="n">
-        <v>4.25</v>
+        <v>4.235</v>
       </c>
       <c r="M13" t="n">
-        <v>4.343</v>
+        <v>4.335</v>
       </c>
       <c r="N13" t="n">
-        <v>4.411</v>
+        <v>4.403</v>
       </c>
       <c r="O13" t="n">
-        <v>4.56</v>
+        <v>4.549</v>
       </c>
       <c r="P13" t="n">
-        <v>4.67</v>
+        <v>4.639</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.951</v>
+        <v>4.903</v>
       </c>
       <c r="R13" t="n">
-        <v>5.245</v>
+        <v>5.189</v>
       </c>
       <c r="S13" t="n">
-        <v>5.529</v>
+        <v>5.466</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.952</v>
+        <v>2.959</v>
       </c>
       <c r="G14" t="n">
-        <v>3.154</v>
+        <v>3.165</v>
       </c>
       <c r="H14" t="n">
-        <v>3.402</v>
+        <v>3.409</v>
       </c>
       <c r="I14" t="n">
-        <v>3.565</v>
+        <v>3.572</v>
       </c>
       <c r="J14" t="n">
-        <v>3.825</v>
+        <v>3.824</v>
       </c>
       <c r="K14" t="n">
-        <v>3.91</v>
+        <v>3.9</v>
       </c>
       <c r="L14" t="n">
-        <v>3.923</v>
+        <v>3.908</v>
       </c>
       <c r="M14" t="n">
-        <v>4.029</v>
+        <v>4.022</v>
       </c>
       <c r="N14" t="n">
-        <v>4.09</v>
+        <v>4.082</v>
       </c>
       <c r="O14" t="n">
-        <v>4.218</v>
+        <v>4.207</v>
       </c>
       <c r="P14" t="n">
-        <v>4.306</v>
+        <v>4.275</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.54</v>
+        <v>4.492</v>
       </c>
       <c r="R14" t="n">
-        <v>4.76</v>
+        <v>4.703</v>
       </c>
       <c r="S14" t="n">
-        <v>4.982</v>
+        <v>4.919</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.929</v>
+        <v>2.937</v>
       </c>
       <c r="G15" t="n">
-        <v>3.129</v>
+        <v>3.139</v>
       </c>
       <c r="H15" t="n">
-        <v>3.373</v>
+        <v>3.38</v>
       </c>
       <c r="I15" t="n">
-        <v>3.515</v>
+        <v>3.523</v>
       </c>
       <c r="J15" t="n">
-        <v>3.763</v>
+        <v>3.762</v>
       </c>
       <c r="K15" t="n">
-        <v>3.863</v>
+        <v>3.853</v>
       </c>
       <c r="L15" t="n">
-        <v>3.859</v>
+        <v>3.844</v>
       </c>
       <c r="M15" t="n">
-        <v>3.942</v>
+        <v>3.934</v>
       </c>
       <c r="N15" t="n">
-        <v>3.993</v>
+        <v>3.985</v>
       </c>
       <c r="O15" t="n">
-        <v>4.162</v>
+        <v>4.15</v>
       </c>
       <c r="P15" t="n">
-        <v>4.202</v>
+        <v>4.171</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.442</v>
+        <v>4.394</v>
       </c>
       <c r="R15" t="n">
-        <v>4.654</v>
+        <v>4.598</v>
       </c>
       <c r="S15" t="n">
-        <v>4.877</v>
+        <v>4.814</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.929</v>
+        <v>2.937</v>
       </c>
       <c r="G16" t="n">
-        <v>3.129</v>
+        <v>3.139</v>
       </c>
       <c r="H16" t="n">
-        <v>3.373</v>
+        <v>3.38</v>
       </c>
       <c r="I16" t="n">
-        <v>3.515</v>
+        <v>3.523</v>
       </c>
       <c r="J16" t="n">
-        <v>3.763</v>
+        <v>3.762</v>
       </c>
       <c r="K16" t="n">
-        <v>3.863</v>
+        <v>3.853</v>
       </c>
       <c r="L16" t="n">
-        <v>3.859</v>
+        <v>3.844</v>
       </c>
       <c r="M16" t="n">
-        <v>3.942</v>
+        <v>3.934</v>
       </c>
       <c r="N16" t="n">
-        <v>3.996</v>
+        <v>3.988</v>
       </c>
       <c r="O16" t="n">
-        <v>4.168</v>
+        <v>4.157</v>
       </c>
       <c r="P16" t="n">
-        <v>4.225</v>
+        <v>4.194</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.469</v>
+        <v>4.421</v>
       </c>
       <c r="R16" t="n">
-        <v>4.682</v>
+        <v>4.626</v>
       </c>
       <c r="S16" t="n">
-        <v>4.906</v>
+        <v>4.843</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.784</v>
+        <v>2.777</v>
       </c>
       <c r="G17" t="n">
-        <v>3.032</v>
+        <v>3.02</v>
       </c>
       <c r="H17" t="n">
-        <v>3.237</v>
+        <v>3.227</v>
       </c>
       <c r="I17" t="n">
-        <v>3.354</v>
+        <v>3.329</v>
       </c>
       <c r="J17" t="n">
-        <v>3.574</v>
+        <v>3.56</v>
       </c>
       <c r="K17" t="n">
-        <v>3.691</v>
+        <v>3.682</v>
       </c>
       <c r="L17" t="n">
-        <v>3.775</v>
+        <v>3.748</v>
       </c>
       <c r="M17" t="n">
-        <v>3.904</v>
+        <v>3.889</v>
       </c>
       <c r="N17" t="n">
-        <v>3.976</v>
+        <v>3.963</v>
       </c>
       <c r="O17" t="n">
-        <v>4.166</v>
+        <v>4.151</v>
       </c>
       <c r="P17" t="n">
-        <v>4.271</v>
+        <v>4.238</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.785</v>
+        <v>2.779</v>
       </c>
       <c r="G18" t="n">
-        <v>3.033</v>
+        <v>3.021</v>
       </c>
       <c r="H18" t="n">
-        <v>3.237</v>
+        <v>3.227</v>
       </c>
       <c r="I18" t="n">
-        <v>3.354</v>
+        <v>3.33</v>
       </c>
       <c r="J18" t="n">
-        <v>3.574</v>
+        <v>3.56</v>
       </c>
       <c r="K18" t="n">
-        <v>3.692</v>
+        <v>3.682</v>
       </c>
       <c r="L18" t="n">
-        <v>3.775</v>
+        <v>3.748</v>
       </c>
       <c r="M18" t="n">
-        <v>3.904</v>
+        <v>3.889</v>
       </c>
       <c r="N18" t="n">
-        <v>3.977</v>
+        <v>3.964</v>
       </c>
       <c r="O18" t="n">
-        <v>4.164</v>
+        <v>4.15</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.94</v>
+        <v>2.948</v>
       </c>
       <c r="G19" t="n">
-        <v>3.142</v>
+        <v>3.153</v>
       </c>
       <c r="H19" t="n">
-        <v>3.389</v>
+        <v>3.396</v>
       </c>
       <c r="I19" t="n">
-        <v>3.549</v>
+        <v>3.557</v>
       </c>
       <c r="J19" t="n">
-        <v>3.805</v>
+        <v>3.803</v>
       </c>
       <c r="K19" t="n">
-        <v>3.906</v>
+        <v>3.896</v>
       </c>
       <c r="L19" t="n">
-        <v>3.92</v>
+        <v>3.905</v>
       </c>
       <c r="M19" t="n">
-        <v>4.02</v>
+        <v>4.013</v>
       </c>
       <c r="N19" t="n">
-        <v>4.083</v>
+        <v>4.075</v>
       </c>
       <c r="O19" t="n">
-        <v>4.205</v>
+        <v>4.194</v>
       </c>
       <c r="P19" t="n">
-        <v>4.263</v>
+        <v>4.233</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.48</v>
+        <v>4.432</v>
       </c>
       <c r="R19" t="n">
-        <v>4.7</v>
+        <v>4.644</v>
       </c>
       <c r="S19" t="n">
-        <v>4.917</v>
+        <v>4.854</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1872,22 +1872,22 @@
         <v>2.76</v>
       </c>
       <c r="H20" t="n">
-        <v>2.85</v>
+        <v>2.849</v>
       </c>
       <c r="I20" t="n">
         <v>2.949</v>
       </c>
       <c r="J20" t="n">
-        <v>3.404</v>
+        <v>3.389</v>
       </c>
       <c r="K20" t="n">
-        <v>3.63</v>
+        <v>3.61</v>
       </c>
       <c r="L20" t="n">
-        <v>3.634</v>
+        <v>3.614</v>
       </c>
       <c r="M20" t="n">
-        <v>3.74</v>
+        <v>3.724</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.02</v>
+        <v>3.022</v>
       </c>
       <c r="G21" t="n">
-        <v>3.245</v>
+        <v>3.253</v>
       </c>
       <c r="H21" t="n">
-        <v>3.513</v>
+        <v>3.519</v>
       </c>
       <c r="I21" t="n">
-        <v>3.685</v>
+        <v>3.691</v>
       </c>
       <c r="J21" t="n">
-        <v>3.974</v>
+        <v>3.973</v>
       </c>
       <c r="K21" t="n">
-        <v>4.147</v>
+        <v>4.137</v>
       </c>
       <c r="L21" t="n">
-        <v>4.181</v>
+        <v>4.163</v>
       </c>
       <c r="M21" t="n">
-        <v>4.267</v>
+        <v>4.258</v>
       </c>
       <c r="N21" t="n">
-        <v>4.319</v>
+        <v>4.313</v>
       </c>
       <c r="O21" t="n">
-        <v>4.414</v>
+        <v>4.403</v>
       </c>
       <c r="P21" t="n">
-        <v>4.526</v>
+        <v>4.496</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.634</v>
+        <v>4.587</v>
       </c>
       <c r="R21" t="n">
-        <v>4.753</v>
+        <v>4.697</v>
       </c>
       <c r="S21" t="n">
-        <v>4.87</v>
+        <v>4.807</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.966</v>
+        <v>2.968</v>
       </c>
       <c r="G22" t="n">
-        <v>3.19</v>
+        <v>3.198</v>
       </c>
       <c r="H22" t="n">
-        <v>3.445</v>
+        <v>3.451</v>
       </c>
       <c r="I22" t="n">
-        <v>3.604</v>
+        <v>3.609</v>
       </c>
       <c r="J22" t="n">
-        <v>3.859</v>
+        <v>3.858</v>
       </c>
       <c r="K22" t="n">
-        <v>4.028</v>
+        <v>4.018</v>
       </c>
       <c r="L22" t="n">
-        <v>4.048</v>
+        <v>4.03</v>
       </c>
       <c r="M22" t="n">
-        <v>4.139</v>
+        <v>4.129</v>
       </c>
       <c r="N22" t="n">
-        <v>4.193</v>
+        <v>4.186</v>
       </c>
       <c r="O22" t="n">
-        <v>4.285</v>
+        <v>4.274</v>
       </c>
       <c r="P22" t="n">
-        <v>4.39</v>
+        <v>4.359</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.493</v>
+        <v>4.446</v>
       </c>
       <c r="R22" t="n">
-        <v>4.602</v>
+        <v>4.546</v>
       </c>
       <c r="S22" t="n">
-        <v>4.715</v>
+        <v>4.652</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.913</v>
+        <v>2.915</v>
       </c>
       <c r="G23" t="n">
-        <v>3.143</v>
+        <v>3.151</v>
       </c>
       <c r="H23" t="n">
-        <v>3.385</v>
+        <v>3.391</v>
       </c>
       <c r="I23" t="n">
-        <v>3.551</v>
+        <v>3.556</v>
       </c>
       <c r="J23" t="n">
-        <v>3.798</v>
+        <v>3.797</v>
       </c>
       <c r="K23" t="n">
-        <v>3.927</v>
+        <v>3.917</v>
       </c>
       <c r="L23" t="n">
-        <v>3.945</v>
+        <v>3.931</v>
       </c>
       <c r="M23" t="n">
-        <v>4.029</v>
+        <v>4.022</v>
       </c>
       <c r="N23" t="n">
-        <v>4.086</v>
+        <v>4.078</v>
       </c>
       <c r="O23" t="n">
-        <v>4.159</v>
+        <v>4.148</v>
       </c>
       <c r="P23" t="n">
-        <v>4.252</v>
+        <v>4.221</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.298</v>
+        <v>4.251</v>
       </c>
       <c r="R23" t="n">
-        <v>4.388</v>
+        <v>4.331</v>
       </c>
       <c r="S23" t="n">
-        <v>4.472</v>
+        <v>4.409</v>
       </c>
       <c r="T23" t="n">
-        <v>4.425</v>
+        <v>4.368</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.849</v>
+        <v>2.851</v>
       </c>
       <c r="G24" t="n">
-        <v>3.053</v>
+        <v>3.061</v>
       </c>
       <c r="H24" t="n">
-        <v>3.283</v>
+        <v>3.289</v>
       </c>
       <c r="I24" t="n">
-        <v>3.489</v>
+        <v>3.494</v>
       </c>
       <c r="J24" t="n">
-        <v>3.691</v>
+        <v>3.69</v>
       </c>
       <c r="K24" t="n">
-        <v>3.81</v>
+        <v>3.8</v>
       </c>
       <c r="L24" t="n">
-        <v>3.826</v>
+        <v>3.813</v>
       </c>
       <c r="M24" t="n">
-        <v>3.887</v>
+        <v>3.882</v>
       </c>
       <c r="N24" t="n">
-        <v>3.961</v>
+        <v>3.953</v>
       </c>
       <c r="O24" t="n">
-        <v>4.158</v>
+        <v>4.145</v>
       </c>
       <c r="P24" t="n">
-        <v>4.19</v>
+        <v>4.159</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.225</v>
+        <v>4.178</v>
       </c>
       <c r="R24" t="n">
-        <v>4.309</v>
+        <v>4.253</v>
       </c>
       <c r="S24" t="n">
-        <v>4.387</v>
+        <v>4.324</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.908</v>
+        <v>2.91</v>
       </c>
       <c r="G25" t="n">
-        <v>3.143</v>
+        <v>3.151</v>
       </c>
       <c r="H25" t="n">
-        <v>3.389</v>
+        <v>3.394</v>
       </c>
       <c r="I25" t="n">
-        <v>3.56</v>
+        <v>3.565</v>
       </c>
       <c r="J25" t="n">
         <v>3.813</v>
       </c>
       <c r="K25" t="n">
-        <v>3.958</v>
+        <v>3.949</v>
       </c>
       <c r="L25" t="n">
-        <v>3.975</v>
+        <v>3.961</v>
       </c>
       <c r="M25" t="n">
-        <v>4.06</v>
+        <v>4.054</v>
       </c>
       <c r="N25" t="n">
-        <v>4.113</v>
+        <v>4.106</v>
       </c>
       <c r="O25" t="n">
-        <v>4.188</v>
+        <v>4.177</v>
       </c>
       <c r="P25" t="n">
-        <v>4.273</v>
+        <v>4.242</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.332</v>
+        <v>4.285</v>
       </c>
       <c r="R25" t="n">
-        <v>4.411</v>
+        <v>4.355</v>
       </c>
       <c r="S25" t="n">
-        <v>4.495</v>
+        <v>4.432</v>
       </c>
       <c r="T25" t="n">
-        <v>4.443</v>
+        <v>4.386</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.237</v>
+        <v>3.244</v>
       </c>
       <c r="G26" t="n">
-        <v>3.449</v>
+        <v>3.457</v>
       </c>
       <c r="H26" t="n">
-        <v>3.778</v>
+        <v>3.787</v>
       </c>
       <c r="I26" t="n">
-        <v>3.966</v>
+        <v>3.978</v>
       </c>
       <c r="J26" t="n">
-        <v>4.377</v>
+        <v>4.379</v>
       </c>
       <c r="K26" t="n">
-        <v>4.759</v>
+        <v>4.748</v>
       </c>
       <c r="L26" t="n">
-        <v>4.831</v>
+        <v>4.815</v>
       </c>
       <c r="M26" t="n">
-        <v>4.962</v>
+        <v>4.954</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.246</v>
+        <v>5.232</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.036</v>
+        <v>3.043</v>
       </c>
       <c r="G27" t="n">
-        <v>3.213</v>
+        <v>3.223</v>
       </c>
       <c r="H27" t="n">
-        <v>3.466</v>
+        <v>3.474</v>
       </c>
       <c r="I27" t="n">
-        <v>3.631</v>
+        <v>3.64</v>
       </c>
       <c r="J27" t="n">
-        <v>3.915</v>
+        <v>3.914</v>
       </c>
       <c r="K27" t="n">
-        <v>4.083</v>
+        <v>4.073</v>
       </c>
       <c r="L27" t="n">
-        <v>4.097</v>
+        <v>4.081</v>
       </c>
       <c r="M27" t="n">
-        <v>4.183</v>
+        <v>4.177</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.348</v>
+        <v>4.335</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.139</v>
+        <v>3.146</v>
       </c>
       <c r="G28" t="n">
-        <v>3.325</v>
+        <v>3.335</v>
       </c>
       <c r="H28" t="n">
-        <v>3.593</v>
+        <v>3.601</v>
       </c>
       <c r="I28" t="n">
-        <v>3.768</v>
+        <v>3.777</v>
       </c>
       <c r="J28" t="n">
-        <v>4.088</v>
+        <v>4.087</v>
       </c>
       <c r="K28" t="n">
-        <v>4.275</v>
+        <v>4.265</v>
       </c>
       <c r="L28" t="n">
-        <v>4.3</v>
+        <v>4.284</v>
       </c>
       <c r="M28" t="n">
-        <v>4.395</v>
+        <v>4.388</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.64</v>
+        <v>4.627</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.984</v>
+        <v>2.991</v>
       </c>
       <c r="G29" t="n">
-        <v>3.157</v>
+        <v>3.167</v>
       </c>
       <c r="H29" t="n">
-        <v>3.402</v>
+        <v>3.41</v>
       </c>
       <c r="I29" t="n">
-        <v>3.556</v>
+        <v>3.565</v>
       </c>
       <c r="J29" t="n">
-        <v>3.827</v>
+        <v>3.826</v>
       </c>
       <c r="K29" t="n">
-        <v>3.979</v>
+        <v>3.969</v>
       </c>
       <c r="L29" t="n">
-        <v>3.982</v>
+        <v>3.967</v>
       </c>
       <c r="M29" t="n">
-        <v>4.046</v>
+        <v>4.04</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.22</v>
+        <v>4.206</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.271</v>
+        <v>3.277</v>
       </c>
       <c r="G30" t="n">
-        <v>3.415</v>
+        <v>3.422</v>
       </c>
       <c r="H30" t="n">
-        <v>3.703</v>
+        <v>3.711</v>
       </c>
       <c r="I30" t="n">
-        <v>3.883</v>
+        <v>3.894</v>
       </c>
       <c r="J30" t="n">
         <v>4.232</v>
       </c>
       <c r="K30" t="n">
-        <v>4.553</v>
+        <v>4.542</v>
       </c>
       <c r="L30" t="n">
-        <v>4.602</v>
+        <v>4.586</v>
       </c>
       <c r="M30" t="n">
-        <v>4.721</v>
+        <v>4.714</v>
       </c>
       <c r="N30" t="n">
-        <v>4.897</v>
+        <v>4.886</v>
       </c>
       <c r="O30" t="n">
-        <v>5.195</v>
+        <v>5.181</v>
       </c>
       <c r="P30" t="n">
-        <v>5.419</v>
+        <v>5.386</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.175</v>
+        <v>6.127</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.6</v>
+        <v>3.606</v>
       </c>
       <c r="G31" t="n">
-        <v>3.781</v>
+        <v>3.788</v>
       </c>
       <c r="H31" t="n">
-        <v>4.119</v>
+        <v>4.127</v>
       </c>
       <c r="I31" t="n">
-        <v>4.312</v>
+        <v>4.324</v>
       </c>
       <c r="J31" t="n">
-        <v>4.726</v>
+        <v>4.727</v>
       </c>
       <c r="K31" t="n">
-        <v>5.088</v>
+        <v>5.078</v>
       </c>
       <c r="L31" t="n">
-        <v>5.215</v>
+        <v>5.199</v>
       </c>
       <c r="M31" t="n">
-        <v>5.452</v>
+        <v>5.444</v>
       </c>
       <c r="N31" t="n">
-        <v>5.756</v>
+        <v>5.745</v>
       </c>
       <c r="O31" t="n">
-        <v>6.231</v>
+        <v>6.217</v>
       </c>
       <c r="P31" t="n">
-        <v>6.407</v>
+        <v>6.374</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.148</v>
+        <v>7.1</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.37</v>
+        <v>3.376</v>
       </c>
       <c r="G32" t="n">
-        <v>3.533</v>
+        <v>3.54</v>
       </c>
       <c r="H32" t="n">
-        <v>3.847</v>
+        <v>3.855</v>
       </c>
       <c r="I32" t="n">
-        <v>4.042</v>
+        <v>4.053</v>
       </c>
       <c r="J32" t="n">
-        <v>4.412</v>
+        <v>4.413</v>
       </c>
       <c r="K32" t="n">
-        <v>4.738</v>
+        <v>4.727</v>
       </c>
       <c r="L32" t="n">
-        <v>4.806</v>
+        <v>4.79</v>
       </c>
       <c r="M32" t="n">
-        <v>4.994</v>
+        <v>4.986</v>
       </c>
       <c r="N32" t="n">
-        <v>5.258</v>
+        <v>5.247</v>
       </c>
       <c r="O32" t="n">
-        <v>5.64</v>
+        <v>5.626</v>
       </c>
       <c r="P32" t="n">
-        <v>5.879</v>
+        <v>5.846</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.636</v>
+        <v>6.588</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.136</v>
+        <v>3.142</v>
       </c>
       <c r="G33" t="n">
-        <v>3.278</v>
+        <v>3.286</v>
       </c>
       <c r="H33" t="n">
-        <v>3.52</v>
+        <v>3.528</v>
       </c>
       <c r="I33" t="n">
-        <v>3.669</v>
+        <v>3.68</v>
       </c>
       <c r="J33" t="n">
         <v>3.939</v>
       </c>
       <c r="K33" t="n">
-        <v>4.194</v>
+        <v>4.183</v>
       </c>
       <c r="L33" t="n">
-        <v>4.208</v>
+        <v>4.191</v>
       </c>
       <c r="M33" t="n">
-        <v>4.251</v>
+        <v>4.242</v>
       </c>
       <c r="N33" t="n">
-        <v>4.286</v>
+        <v>4.274</v>
       </c>
       <c r="O33" t="n">
-        <v>4.351</v>
+        <v>4.337</v>
       </c>
       <c r="P33" t="n">
-        <v>4.451</v>
+        <v>4.418</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.892</v>
+        <v>4.843</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.196</v>
+        <v>3.202</v>
       </c>
       <c r="G34" t="n">
-        <v>3.332</v>
+        <v>3.34</v>
       </c>
       <c r="H34" t="n">
-        <v>3.583</v>
+        <v>3.591</v>
       </c>
       <c r="I34" t="n">
-        <v>3.737</v>
+        <v>3.748</v>
       </c>
       <c r="J34" t="n">
         <v>4.01</v>
       </c>
       <c r="K34" t="n">
+        <v>4.259</v>
+      </c>
+      <c r="L34" t="n">
         <v>4.27</v>
       </c>
-      <c r="L34" t="n">
-        <v>4.286</v>
-      </c>
       <c r="M34" t="n">
-        <v>4.342</v>
+        <v>4.333</v>
       </c>
       <c r="N34" t="n">
-        <v>4.391</v>
+        <v>4.379</v>
       </c>
       <c r="O34" t="n">
-        <v>4.52</v>
+        <v>4.506</v>
       </c>
       <c r="P34" t="n">
-        <v>4.746</v>
+        <v>4.712</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.593</v>
+        <v>5.544</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.17</v>
+        <v>3.176</v>
       </c>
       <c r="G35" t="n">
-        <v>3.306</v>
+        <v>3.314</v>
       </c>
       <c r="H35" t="n">
-        <v>3.551</v>
+        <v>3.559</v>
       </c>
       <c r="I35" t="n">
-        <v>3.704</v>
+        <v>3.715</v>
       </c>
       <c r="J35" t="n">
         <v>3.979</v>
       </c>
       <c r="K35" t="n">
-        <v>4.224</v>
+        <v>4.213</v>
       </c>
       <c r="L35" t="n">
-        <v>4.242</v>
+        <v>4.225</v>
       </c>
       <c r="M35" t="n">
-        <v>4.288</v>
+        <v>4.279</v>
       </c>
       <c r="N35" t="n">
-        <v>4.327</v>
+        <v>4.315</v>
       </c>
       <c r="O35" t="n">
-        <v>4.417</v>
+        <v>4.403</v>
       </c>
       <c r="P35" t="n">
-        <v>4.548</v>
+        <v>4.515</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.228</v>
+        <v>5.18</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.056</v>
+        <v>3.062</v>
       </c>
       <c r="G36" t="n">
-        <v>3.186</v>
+        <v>3.193</v>
       </c>
       <c r="H36" t="n">
-        <v>3.425</v>
+        <v>3.432</v>
       </c>
       <c r="I36" t="n">
-        <v>3.579</v>
+        <v>3.591</v>
       </c>
       <c r="J36" t="n">
         <v>3.875</v>
       </c>
       <c r="K36" t="n">
-        <v>4.12</v>
+        <v>4.108</v>
       </c>
       <c r="L36" t="n">
-        <v>4.132</v>
+        <v>4.115</v>
       </c>
       <c r="M36" t="n">
-        <v>4.154</v>
+        <v>4.145</v>
       </c>
       <c r="N36" t="n">
-        <v>4.191</v>
+        <v>4.179</v>
       </c>
       <c r="O36" t="n">
-        <v>4.258</v>
+        <v>4.244</v>
       </c>
       <c r="P36" t="n">
-        <v>4.349</v>
+        <v>4.316</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.609</v>
+        <v>4.56</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.943</v>
+        <v>3.95</v>
       </c>
       <c r="G37" t="n">
-        <v>4.474</v>
+        <v>4.482</v>
       </c>
       <c r="H37" t="n">
-        <v>5.091</v>
+        <v>5.1</v>
       </c>
       <c r="I37" t="n">
-        <v>5.373</v>
+        <v>5.385</v>
       </c>
       <c r="J37" t="n">
-        <v>6.215</v>
+        <v>6.216</v>
       </c>
       <c r="K37" t="n">
-        <v>7.129</v>
+        <v>7.119</v>
       </c>
       <c r="L37" t="n">
-        <v>7.415</v>
+        <v>7.399</v>
       </c>
       <c r="M37" t="n">
-        <v>7.724</v>
+        <v>7.716</v>
       </c>
       <c r="N37" t="n">
-        <v>7.912</v>
+        <v>7.901</v>
       </c>
       <c r="O37" t="n">
-        <v>8.109999999999999</v>
+        <v>8.096</v>
       </c>
       <c r="P37" t="n">
-        <v>8.209</v>
+        <v>8.176</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.638999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.005</v>
+        <v>5.012</v>
       </c>
       <c r="G38" t="n">
-        <v>5.789</v>
+        <v>5.797</v>
       </c>
       <c r="H38" t="n">
-        <v>6.618</v>
+        <v>6.627</v>
       </c>
       <c r="I38" t="n">
-        <v>7.057</v>
+        <v>7.069</v>
       </c>
       <c r="J38" t="n">
-        <v>8.159000000000001</v>
+        <v>8.16</v>
       </c>
       <c r="K38" t="n">
-        <v>9.252000000000001</v>
+        <v>9.242000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.698</v>
+        <v>9.682</v>
       </c>
       <c r="M38" t="n">
-        <v>10.136</v>
+        <v>10.128</v>
       </c>
       <c r="N38" t="n">
-        <v>10.331</v>
+        <v>10.32</v>
       </c>
       <c r="O38" t="n">
-        <v>10.51</v>
+        <v>10.496</v>
       </c>
       <c r="P38" t="n">
-        <v>10.607</v>
+        <v>10.573</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.089</v>
+        <v>11.041</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.325</v>
+        <v>4.332</v>
       </c>
       <c r="G39" t="n">
-        <v>4.987</v>
+        <v>4.995</v>
       </c>
       <c r="H39" t="n">
-        <v>5.683</v>
+        <v>5.692</v>
       </c>
       <c r="I39" t="n">
-        <v>6.061</v>
+        <v>6.073</v>
       </c>
       <c r="J39" t="n">
-        <v>7.031</v>
+        <v>7.032</v>
       </c>
       <c r="K39" t="n">
-        <v>8.084</v>
+        <v>8.074</v>
       </c>
       <c r="L39" t="n">
-        <v>8.454000000000001</v>
+        <v>8.436999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.772</v>
+        <v>8.763999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.959</v>
+        <v>8.948</v>
       </c>
       <c r="O39" t="n">
-        <v>9.161</v>
+        <v>9.147</v>
       </c>
       <c r="P39" t="n">
-        <v>9.260999999999999</v>
+        <v>9.228</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.734999999999999</v>
+        <v>9.686</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.463</v>
+        <v>3.469</v>
       </c>
       <c r="G40" t="n">
-        <v>3.653</v>
+        <v>3.66</v>
       </c>
       <c r="H40" t="n">
-        <v>3.962</v>
+        <v>3.97</v>
       </c>
       <c r="I40" t="n">
-        <v>4.157</v>
+        <v>4.168</v>
       </c>
       <c r="J40" t="n">
         <v>4.524</v>
       </c>
       <c r="K40" t="n">
-        <v>4.859</v>
+        <v>4.848</v>
       </c>
       <c r="L40" t="n">
-        <v>4.928</v>
+        <v>4.912</v>
       </c>
       <c r="M40" t="n">
-        <v>5.064</v>
+        <v>5.056</v>
       </c>
       <c r="N40" t="n">
-        <v>5.255</v>
+        <v>5.244</v>
       </c>
       <c r="O40" t="n">
-        <v>5.574</v>
+        <v>5.56</v>
       </c>
       <c r="P40" t="n">
-        <v>5.84</v>
+        <v>5.807</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.626</v>
+        <v>6.578</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.849</v>
+        <v>3.855</v>
       </c>
       <c r="G41" t="n">
-        <v>4.082</v>
+        <v>4.089</v>
       </c>
       <c r="H41" t="n">
-        <v>4.448</v>
+        <v>4.456</v>
       </c>
       <c r="I41" t="n">
-        <v>4.66</v>
+        <v>4.672</v>
       </c>
       <c r="J41" t="n">
-        <v>5.081</v>
+        <v>5.082</v>
       </c>
       <c r="K41" t="n">
-        <v>5.462</v>
+        <v>5.452</v>
       </c>
       <c r="L41" t="n">
-        <v>5.605</v>
+        <v>5.589</v>
       </c>
       <c r="M41" t="n">
-        <v>5.867</v>
+        <v>5.859</v>
       </c>
       <c r="N41" t="n">
-        <v>6.186</v>
+        <v>6.175</v>
       </c>
       <c r="O41" t="n">
-        <v>6.689</v>
+        <v>6.675</v>
       </c>
       <c r="P41" t="n">
-        <v>6.9</v>
+        <v>6.866</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.673</v>
+        <v>7.625</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.584</v>
+        <v>3.59</v>
       </c>
       <c r="G42" t="n">
-        <v>3.802</v>
+        <v>3.809</v>
       </c>
       <c r="H42" t="n">
-        <v>4.138</v>
+        <v>4.146</v>
       </c>
       <c r="I42" t="n">
-        <v>4.345</v>
+        <v>4.356</v>
       </c>
       <c r="J42" t="n">
-        <v>4.728</v>
+        <v>4.729</v>
       </c>
       <c r="K42" t="n">
-        <v>5.08</v>
+        <v>5.069</v>
       </c>
       <c r="L42" t="n">
-        <v>5.163</v>
+        <v>5.147</v>
       </c>
       <c r="M42" t="n">
-        <v>5.371</v>
+        <v>5.363</v>
       </c>
       <c r="N42" t="n">
-        <v>5.669</v>
+        <v>5.658</v>
       </c>
       <c r="O42" t="n">
-        <v>6.066</v>
+        <v>6.052</v>
       </c>
       <c r="P42" t="n">
-        <v>6.342</v>
+        <v>6.309</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.139</v>
+        <v>7.09</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.284</v>
+        <v>3.29</v>
       </c>
       <c r="G43" t="n">
-        <v>3.461</v>
+        <v>3.47</v>
       </c>
       <c r="H43" t="n">
-        <v>3.722</v>
+        <v>3.73</v>
       </c>
       <c r="I43" t="n">
-        <v>3.878</v>
+        <v>3.889</v>
       </c>
       <c r="J43" t="n">
         <v>4.166</v>
       </c>
       <c r="K43" t="n">
-        <v>4.426</v>
+        <v>4.415</v>
       </c>
       <c r="L43" t="n">
-        <v>4.451</v>
+        <v>4.434</v>
       </c>
       <c r="M43" t="n">
-        <v>4.506</v>
+        <v>4.497</v>
       </c>
       <c r="N43" t="n">
-        <v>4.555</v>
+        <v>4.543</v>
       </c>
       <c r="O43" t="n">
-        <v>4.664</v>
+        <v>4.65</v>
       </c>
       <c r="P43" t="n">
-        <v>4.817</v>
+        <v>4.784</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.502</v>
+        <v>5.454</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.134</v>
+        <v>3.14</v>
       </c>
       <c r="G44" t="n">
-        <v>3.295</v>
+        <v>3.302</v>
       </c>
       <c r="H44" t="n">
-        <v>3.548</v>
+        <v>3.555</v>
       </c>
       <c r="I44" t="n">
-        <v>3.706</v>
+        <v>3.718</v>
       </c>
       <c r="J44" t="n">
         <v>4.016</v>
       </c>
       <c r="K44" t="n">
-        <v>4.271</v>
+        <v>4.259</v>
       </c>
       <c r="L44" t="n">
-        <v>4.294</v>
+        <v>4.277</v>
       </c>
       <c r="M44" t="n">
-        <v>4.324</v>
+        <v>4.315</v>
       </c>
       <c r="N44" t="n">
-        <v>4.372</v>
+        <v>4.36</v>
       </c>
       <c r="O44" t="n">
-        <v>4.459</v>
+        <v>4.445</v>
       </c>
       <c r="P44" t="n">
-        <v>4.579</v>
+        <v>4.546</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.873</v>
+        <v>4.824</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-18 ~ 2026-06-18
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.469</v>
+        <v>3.484</v>
       </c>
       <c r="G2" t="n">
-        <v>3.779</v>
+        <v>3.794</v>
       </c>
       <c r="H2" t="n">
-        <v>4.043</v>
+        <v>4.06</v>
       </c>
       <c r="I2" t="n">
-        <v>4.17</v>
+        <v>4.196</v>
       </c>
       <c r="J2" t="n">
-        <v>4.459</v>
+        <v>4.488</v>
       </c>
       <c r="K2" t="n">
-        <v>4.793</v>
+        <v>4.837</v>
       </c>
       <c r="L2" t="n">
-        <v>4.945</v>
+        <v>4.994</v>
       </c>
       <c r="M2" t="n">
-        <v>5.188</v>
+        <v>5.242</v>
       </c>
       <c r="N2" t="n">
-        <v>5.453</v>
+        <v>5.518</v>
       </c>
       <c r="O2" t="n">
-        <v>5.699</v>
+        <v>5.761</v>
       </c>
       <c r="P2" t="n">
-        <v>5.907</v>
+        <v>5.962</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.528</v>
+        <v>6.584</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.49</v>
+        <v>4.504</v>
       </c>
       <c r="G3" t="n">
-        <v>4.981</v>
+        <v>4.996</v>
       </c>
       <c r="H3" t="n">
-        <v>5.278</v>
+        <v>5.295</v>
       </c>
       <c r="I3" t="n">
-        <v>5.399</v>
+        <v>5.424</v>
       </c>
       <c r="J3" t="n">
-        <v>5.704</v>
+        <v>5.734</v>
       </c>
       <c r="K3" t="n">
-        <v>6.109</v>
+        <v>6.153</v>
       </c>
       <c r="L3" t="n">
-        <v>6.331</v>
+        <v>6.38</v>
       </c>
       <c r="M3" t="n">
-        <v>6.604</v>
+        <v>6.658</v>
       </c>
       <c r="N3" t="n">
-        <v>6.812</v>
+        <v>6.877</v>
       </c>
       <c r="O3" t="n">
-        <v>7.009</v>
+        <v>7.071</v>
       </c>
       <c r="P3" t="n">
-        <v>7.085</v>
+        <v>7.14</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.594</v>
+        <v>7.65</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.982</v>
+        <v>3.996</v>
       </c>
       <c r="G4" t="n">
-        <v>4.362</v>
+        <v>4.377</v>
       </c>
       <c r="H4" t="n">
-        <v>4.687</v>
+        <v>4.704</v>
       </c>
       <c r="I4" t="n">
-        <v>4.842</v>
+        <v>4.867</v>
       </c>
       <c r="J4" t="n">
-        <v>5.148</v>
+        <v>5.177</v>
       </c>
       <c r="K4" t="n">
-        <v>5.548</v>
+        <v>5.591</v>
       </c>
       <c r="L4" t="n">
-        <v>5.699</v>
+        <v>5.749</v>
       </c>
       <c r="M4" t="n">
-        <v>5.962</v>
+        <v>6.016</v>
       </c>
       <c r="N4" t="n">
-        <v>6.14</v>
+        <v>6.205</v>
       </c>
       <c r="O4" t="n">
-        <v>6.361</v>
+        <v>6.422</v>
       </c>
       <c r="P4" t="n">
-        <v>6.437</v>
+        <v>6.492</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.949</v>
+        <v>7.005</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.167</v>
+        <v>3.182</v>
       </c>
       <c r="G5" t="n">
-        <v>3.322</v>
+        <v>3.337</v>
       </c>
       <c r="H5" t="n">
-        <v>3.55</v>
+        <v>3.567</v>
       </c>
       <c r="I5" t="n">
-        <v>3.743</v>
+        <v>3.768</v>
       </c>
       <c r="J5" t="n">
-        <v>4.018</v>
+        <v>4.048</v>
       </c>
       <c r="K5" t="n">
-        <v>4.196</v>
+        <v>4.239</v>
       </c>
       <c r="L5" t="n">
-        <v>4.194</v>
+        <v>4.243</v>
       </c>
       <c r="M5" t="n">
-        <v>4.246</v>
+        <v>4.3</v>
       </c>
       <c r="N5" t="n">
-        <v>4.265</v>
+        <v>4.33</v>
       </c>
       <c r="O5" t="n">
-        <v>4.299</v>
+        <v>4.36</v>
       </c>
       <c r="P5" t="n">
-        <v>4.575</v>
+        <v>4.631</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.44</v>
+        <v>5.496</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.208</v>
+        <v>3.222</v>
       </c>
       <c r="G6" t="n">
-        <v>3.377</v>
+        <v>3.392</v>
       </c>
       <c r="H6" t="n">
-        <v>3.62</v>
+        <v>3.636</v>
       </c>
       <c r="I6" t="n">
-        <v>3.825</v>
+        <v>3.85</v>
       </c>
       <c r="J6" t="n">
-        <v>4.109</v>
+        <v>4.139</v>
       </c>
       <c r="K6" t="n">
-        <v>4.308</v>
+        <v>4.351</v>
       </c>
       <c r="L6" t="n">
-        <v>4.312</v>
+        <v>4.361</v>
       </c>
       <c r="M6" t="n">
-        <v>4.401</v>
+        <v>4.456</v>
       </c>
       <c r="N6" t="n">
-        <v>4.432</v>
+        <v>4.497</v>
       </c>
       <c r="O6" t="n">
-        <v>4.565</v>
+        <v>4.627</v>
       </c>
       <c r="P6" t="n">
-        <v>5.008</v>
+        <v>5.063</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.836</v>
+        <v>5.892</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.188</v>
+        <v>3.203</v>
       </c>
       <c r="G7" t="n">
-        <v>3.341</v>
+        <v>3.356</v>
       </c>
       <c r="H7" t="n">
-        <v>3.566</v>
+        <v>3.583</v>
       </c>
       <c r="I7" t="n">
-        <v>3.762</v>
+        <v>3.787</v>
       </c>
       <c r="J7" t="n">
-        <v>4.042</v>
+        <v>4.072</v>
       </c>
       <c r="K7" t="n">
-        <v>4.223</v>
+        <v>4.267</v>
       </c>
       <c r="L7" t="n">
-        <v>4.22</v>
+        <v>4.269</v>
       </c>
       <c r="M7" t="n">
-        <v>4.305</v>
+        <v>4.359</v>
       </c>
       <c r="N7" t="n">
-        <v>4.324</v>
+        <v>4.389</v>
       </c>
       <c r="O7" t="n">
-        <v>4.462</v>
+        <v>4.524</v>
       </c>
       <c r="P7" t="n">
-        <v>4.791</v>
+        <v>4.847</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.604</v>
+        <v>5.66</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.602</v>
+        <v>5.617</v>
       </c>
       <c r="G8" t="n">
-        <v>6.28</v>
+        <v>6.295</v>
       </c>
       <c r="H8" t="n">
-        <v>6.726</v>
+        <v>6.743</v>
       </c>
       <c r="I8" t="n">
-        <v>6.926</v>
+        <v>6.951</v>
       </c>
       <c r="J8" t="n">
-        <v>7.299</v>
+        <v>7.33</v>
       </c>
       <c r="K8" t="n">
-        <v>7.983</v>
+        <v>8.026</v>
       </c>
       <c r="L8" t="n">
-        <v>8.289</v>
+        <v>8.337999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.593999999999999</v>
+        <v>8.648</v>
       </c>
       <c r="N8" t="n">
-        <v>8.736000000000001</v>
+        <v>8.801</v>
       </c>
       <c r="O8" t="n">
-        <v>9.019</v>
+        <v>9.08</v>
       </c>
       <c r="P8" t="n">
-        <v>9.198</v>
+        <v>9.253</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.906000000000001</v>
+        <v>9.962</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.739</v>
+        <v>2.742</v>
       </c>
       <c r="G9" t="n">
-        <v>2.962</v>
+        <v>2.981</v>
       </c>
       <c r="H9" t="n">
-        <v>3.173</v>
+        <v>3.19</v>
       </c>
       <c r="I9" t="n">
-        <v>3.27</v>
+        <v>3.268</v>
       </c>
       <c r="J9" t="n">
-        <v>3.473</v>
+        <v>3.489</v>
       </c>
       <c r="K9" t="n">
-        <v>3.561</v>
+        <v>3.604</v>
       </c>
       <c r="L9" t="n">
-        <v>3.65</v>
+        <v>3.694</v>
       </c>
       <c r="M9" t="n">
-        <v>3.7</v>
+        <v>3.752</v>
       </c>
       <c r="N9" t="n">
-        <v>3.825</v>
+        <v>3.889</v>
       </c>
       <c r="O9" t="n">
-        <v>3.889</v>
+        <v>3.951</v>
       </c>
       <c r="P9" t="n">
-        <v>4.008</v>
+        <v>4.067</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.062</v>
+        <v>4.118</v>
       </c>
       <c r="R9" t="n">
-        <v>4.143</v>
+        <v>4.192</v>
       </c>
       <c r="S9" t="n">
-        <v>4.195</v>
+        <v>4.235</v>
       </c>
       <c r="T9" t="n">
-        <v>4.155</v>
+        <v>4.207</v>
       </c>
       <c r="U9" t="n">
-        <v>4.039</v>
+        <v>4.092</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.747</v>
+        <v>2.75</v>
       </c>
       <c r="G10" t="n">
-        <v>2.971</v>
+        <v>2.988</v>
       </c>
       <c r="H10" t="n">
-        <v>3.176</v>
+        <v>3.193</v>
       </c>
       <c r="I10" t="n">
-        <v>3.273</v>
+        <v>3.271</v>
       </c>
       <c r="J10" t="n">
-        <v>3.489</v>
+        <v>3.505</v>
       </c>
       <c r="K10" t="n">
-        <v>3.601</v>
+        <v>3.645</v>
       </c>
       <c r="L10" t="n">
-        <v>3.662</v>
+        <v>3.707</v>
       </c>
       <c r="M10" t="n">
-        <v>3.762</v>
+        <v>3.812</v>
       </c>
       <c r="N10" t="n">
-        <v>3.851</v>
+        <v>3.917</v>
       </c>
       <c r="O10" t="n">
-        <v>4.13</v>
+        <v>4.18</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.552</v>
+        <v>2.555</v>
       </c>
       <c r="G11" t="n">
-        <v>2.774</v>
+        <v>2.791</v>
       </c>
       <c r="H11" t="n">
-        <v>2.998</v>
+        <v>3.015</v>
       </c>
       <c r="I11" t="n">
-        <v>3.077</v>
+        <v>3.075</v>
       </c>
       <c r="J11" t="n">
-        <v>3.284</v>
+        <v>3.3</v>
       </c>
       <c r="K11" t="n">
-        <v>3.383</v>
+        <v>3.428</v>
       </c>
       <c r="L11" t="n">
-        <v>3.459</v>
+        <v>3.504</v>
       </c>
       <c r="M11" t="n">
-        <v>3.57</v>
+        <v>3.62</v>
       </c>
       <c r="N11" t="n">
-        <v>3.658</v>
+        <v>3.724</v>
       </c>
       <c r="O11" t="n">
-        <v>3.896</v>
+        <v>3.946</v>
       </c>
       <c r="P11" t="n">
-        <v>3.952</v>
+        <v>4.011</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.26</v>
+        <v>4.317</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.388</v>
+        <v>3.401</v>
       </c>
       <c r="G12" t="n">
-        <v>3.674</v>
+        <v>3.687</v>
       </c>
       <c r="H12" t="n">
-        <v>3.941</v>
+        <v>3.956</v>
       </c>
       <c r="I12" t="n">
-        <v>4.14</v>
+        <v>4.16</v>
       </c>
       <c r="J12" t="n">
-        <v>4.446</v>
+        <v>4.471</v>
       </c>
       <c r="K12" t="n">
-        <v>4.578</v>
+        <v>4.619</v>
       </c>
       <c r="L12" t="n">
-        <v>4.596</v>
+        <v>4.646</v>
       </c>
       <c r="M12" t="n">
-        <v>4.708</v>
+        <v>4.764</v>
       </c>
       <c r="N12" t="n">
-        <v>4.775</v>
+        <v>4.842</v>
       </c>
       <c r="O12" t="n">
-        <v>4.92</v>
+        <v>4.985</v>
       </c>
       <c r="P12" t="n">
-        <v>5.048</v>
+        <v>5.108</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.382</v>
+        <v>5.437</v>
       </c>
       <c r="R12" t="n">
-        <v>5.64</v>
+        <v>5.688</v>
       </c>
       <c r="S12" t="n">
-        <v>5.904</v>
+        <v>5.944</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.142</v>
+        <v>3.154</v>
       </c>
       <c r="G13" t="n">
-        <v>3.364</v>
+        <v>3.377</v>
       </c>
       <c r="H13" t="n">
-        <v>3.608</v>
+        <v>3.623</v>
       </c>
       <c r="I13" t="n">
-        <v>3.788</v>
+        <v>3.808</v>
       </c>
       <c r="J13" t="n">
-        <v>4.083</v>
+        <v>4.108</v>
       </c>
       <c r="K13" t="n">
-        <v>4.211</v>
+        <v>4.252</v>
       </c>
       <c r="L13" t="n">
-        <v>4.235</v>
+        <v>4.285</v>
       </c>
       <c r="M13" t="n">
-        <v>4.335</v>
+        <v>4.391</v>
       </c>
       <c r="N13" t="n">
-        <v>4.403</v>
+        <v>4.471</v>
       </c>
       <c r="O13" t="n">
-        <v>4.549</v>
+        <v>4.614</v>
       </c>
       <c r="P13" t="n">
-        <v>4.639</v>
+        <v>4.699</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.903</v>
+        <v>4.959</v>
       </c>
       <c r="R13" t="n">
-        <v>5.189</v>
+        <v>5.238</v>
       </c>
       <c r="S13" t="n">
-        <v>5.466</v>
+        <v>5.506</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.959</v>
+        <v>2.972</v>
       </c>
       <c r="G14" t="n">
-        <v>3.165</v>
+        <v>3.178</v>
       </c>
       <c r="H14" t="n">
-        <v>3.409</v>
+        <v>3.424</v>
       </c>
       <c r="I14" t="n">
-        <v>3.572</v>
+        <v>3.592</v>
       </c>
       <c r="J14" t="n">
-        <v>3.824</v>
+        <v>3.849</v>
       </c>
       <c r="K14" t="n">
-        <v>3.9</v>
+        <v>3.941</v>
       </c>
       <c r="L14" t="n">
-        <v>3.908</v>
+        <v>3.958</v>
       </c>
       <c r="M14" t="n">
-        <v>4.022</v>
+        <v>4.078</v>
       </c>
       <c r="N14" t="n">
-        <v>4.082</v>
+        <v>4.15</v>
       </c>
       <c r="O14" t="n">
-        <v>4.207</v>
+        <v>4.272</v>
       </c>
       <c r="P14" t="n">
-        <v>4.275</v>
+        <v>4.335</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.492</v>
+        <v>4.548</v>
       </c>
       <c r="R14" t="n">
-        <v>4.703</v>
+        <v>4.752</v>
       </c>
       <c r="S14" t="n">
-        <v>4.919</v>
+        <v>4.959</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.937</v>
+        <v>2.949</v>
       </c>
       <c r="G15" t="n">
-        <v>3.139</v>
+        <v>3.153</v>
       </c>
       <c r="H15" t="n">
-        <v>3.38</v>
+        <v>3.395</v>
       </c>
       <c r="I15" t="n">
-        <v>3.523</v>
+        <v>3.543</v>
       </c>
       <c r="J15" t="n">
-        <v>3.762</v>
+        <v>3.787</v>
       </c>
       <c r="K15" t="n">
-        <v>3.853</v>
+        <v>3.893</v>
       </c>
       <c r="L15" t="n">
-        <v>3.844</v>
+        <v>3.894</v>
       </c>
       <c r="M15" t="n">
-        <v>3.934</v>
+        <v>3.99</v>
       </c>
       <c r="N15" t="n">
-        <v>3.985</v>
+        <v>4.053</v>
       </c>
       <c r="O15" t="n">
-        <v>4.15</v>
+        <v>4.215</v>
       </c>
       <c r="P15" t="n">
-        <v>4.171</v>
+        <v>4.231</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.394</v>
+        <v>4.45</v>
       </c>
       <c r="R15" t="n">
-        <v>4.598</v>
+        <v>4.647</v>
       </c>
       <c r="S15" t="n">
-        <v>4.814</v>
+        <v>4.854</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.937</v>
+        <v>2.949</v>
       </c>
       <c r="G16" t="n">
-        <v>3.139</v>
+        <v>3.153</v>
       </c>
       <c r="H16" t="n">
-        <v>3.38</v>
+        <v>3.395</v>
       </c>
       <c r="I16" t="n">
-        <v>3.523</v>
+        <v>3.543</v>
       </c>
       <c r="J16" t="n">
-        <v>3.762</v>
+        <v>3.787</v>
       </c>
       <c r="K16" t="n">
-        <v>3.853</v>
+        <v>3.893</v>
       </c>
       <c r="L16" t="n">
-        <v>3.844</v>
+        <v>3.894</v>
       </c>
       <c r="M16" t="n">
-        <v>3.934</v>
+        <v>3.99</v>
       </c>
       <c r="N16" t="n">
-        <v>3.988</v>
+        <v>4.056</v>
       </c>
       <c r="O16" t="n">
-        <v>4.157</v>
+        <v>4.222</v>
       </c>
       <c r="P16" t="n">
-        <v>4.194</v>
+        <v>4.255</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.421</v>
+        <v>4.477</v>
       </c>
       <c r="R16" t="n">
-        <v>4.626</v>
+        <v>4.675</v>
       </c>
       <c r="S16" t="n">
-        <v>4.843</v>
+        <v>4.883</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.777</v>
+        <v>2.78</v>
       </c>
       <c r="G17" t="n">
-        <v>3.02</v>
+        <v>3.037</v>
       </c>
       <c r="H17" t="n">
-        <v>3.227</v>
+        <v>3.244</v>
       </c>
       <c r="I17" t="n">
-        <v>3.329</v>
+        <v>3.328</v>
       </c>
       <c r="J17" t="n">
-        <v>3.56</v>
+        <v>3.575</v>
       </c>
       <c r="K17" t="n">
-        <v>3.682</v>
+        <v>3.723</v>
       </c>
       <c r="L17" t="n">
-        <v>3.748</v>
+        <v>3.792</v>
       </c>
       <c r="M17" t="n">
-        <v>3.889</v>
+        <v>3.94</v>
       </c>
       <c r="N17" t="n">
-        <v>3.963</v>
+        <v>4.031</v>
       </c>
       <c r="O17" t="n">
-        <v>4.151</v>
+        <v>4.2</v>
       </c>
       <c r="P17" t="n">
-        <v>4.238</v>
+        <v>4.297</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.779</v>
+        <v>2.782</v>
       </c>
       <c r="G18" t="n">
-        <v>3.021</v>
+        <v>3.038</v>
       </c>
       <c r="H18" t="n">
-        <v>3.227</v>
+        <v>3.244</v>
       </c>
       <c r="I18" t="n">
-        <v>3.33</v>
+        <v>3.328</v>
       </c>
       <c r="J18" t="n">
-        <v>3.56</v>
+        <v>3.575</v>
       </c>
       <c r="K18" t="n">
-        <v>3.682</v>
+        <v>3.724</v>
       </c>
       <c r="L18" t="n">
-        <v>3.748</v>
+        <v>3.792</v>
       </c>
       <c r="M18" t="n">
-        <v>3.889</v>
+        <v>3.94</v>
       </c>
       <c r="N18" t="n">
-        <v>3.964</v>
+        <v>4.032</v>
       </c>
       <c r="O18" t="n">
-        <v>4.15</v>
+        <v>4.199</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.948</v>
+        <v>2.96</v>
       </c>
       <c r="G19" t="n">
-        <v>3.153</v>
+        <v>3.166</v>
       </c>
       <c r="H19" t="n">
-        <v>3.396</v>
+        <v>3.411</v>
       </c>
       <c r="I19" t="n">
-        <v>3.557</v>
+        <v>3.577</v>
       </c>
       <c r="J19" t="n">
-        <v>3.803</v>
+        <v>3.828</v>
       </c>
       <c r="K19" t="n">
-        <v>3.896</v>
+        <v>3.937</v>
       </c>
       <c r="L19" t="n">
-        <v>3.905</v>
+        <v>3.955</v>
       </c>
       <c r="M19" t="n">
-        <v>4.013</v>
+        <v>4.069</v>
       </c>
       <c r="N19" t="n">
-        <v>4.075</v>
+        <v>4.142</v>
       </c>
       <c r="O19" t="n">
-        <v>4.194</v>
+        <v>4.259</v>
       </c>
       <c r="P19" t="n">
-        <v>4.233</v>
+        <v>4.293</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.432</v>
+        <v>4.488</v>
       </c>
       <c r="R19" t="n">
-        <v>4.644</v>
+        <v>4.693</v>
       </c>
       <c r="S19" t="n">
-        <v>4.854</v>
+        <v>4.894</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.666</v>
+        <v>2.671</v>
       </c>
       <c r="G20" t="n">
-        <v>2.76</v>
+        <v>2.767</v>
       </c>
       <c r="H20" t="n">
-        <v>2.849</v>
+        <v>2.856</v>
       </c>
       <c r="I20" t="n">
-        <v>2.949</v>
+        <v>2.964</v>
       </c>
       <c r="J20" t="n">
-        <v>3.389</v>
+        <v>3.412</v>
       </c>
       <c r="K20" t="n">
-        <v>3.61</v>
+        <v>3.65</v>
       </c>
       <c r="L20" t="n">
-        <v>3.614</v>
+        <v>3.652</v>
       </c>
       <c r="M20" t="n">
-        <v>3.724</v>
+        <v>3.764</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.022</v>
+        <v>3.032</v>
       </c>
       <c r="G21" t="n">
-        <v>3.253</v>
+        <v>3.267</v>
       </c>
       <c r="H21" t="n">
-        <v>3.519</v>
+        <v>3.535</v>
       </c>
       <c r="I21" t="n">
-        <v>3.691</v>
+        <v>3.71</v>
       </c>
       <c r="J21" t="n">
-        <v>3.973</v>
+        <v>4.002</v>
       </c>
       <c r="K21" t="n">
-        <v>4.137</v>
+        <v>4.179</v>
       </c>
       <c r="L21" t="n">
-        <v>4.163</v>
+        <v>4.208</v>
       </c>
       <c r="M21" t="n">
-        <v>4.258</v>
+        <v>4.312</v>
       </c>
       <c r="N21" t="n">
-        <v>4.313</v>
+        <v>4.378</v>
       </c>
       <c r="O21" t="n">
-        <v>4.403</v>
+        <v>4.463</v>
       </c>
       <c r="P21" t="n">
-        <v>4.496</v>
+        <v>4.553</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.587</v>
+        <v>4.641</v>
       </c>
       <c r="R21" t="n">
-        <v>4.697</v>
+        <v>4.745</v>
       </c>
       <c r="S21" t="n">
-        <v>4.807</v>
+        <v>4.846</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.968</v>
+        <v>2.979</v>
       </c>
       <c r="G22" t="n">
-        <v>3.198</v>
+        <v>3.211</v>
       </c>
       <c r="H22" t="n">
-        <v>3.451</v>
+        <v>3.467</v>
       </c>
       <c r="I22" t="n">
-        <v>3.609</v>
+        <v>3.628</v>
       </c>
       <c r="J22" t="n">
-        <v>3.858</v>
+        <v>3.887</v>
       </c>
       <c r="K22" t="n">
-        <v>4.018</v>
+        <v>4.061</v>
       </c>
       <c r="L22" t="n">
-        <v>4.03</v>
+        <v>4.077</v>
       </c>
       <c r="M22" t="n">
-        <v>4.129</v>
+        <v>4.185</v>
       </c>
       <c r="N22" t="n">
-        <v>4.186</v>
+        <v>4.254</v>
       </c>
       <c r="O22" t="n">
-        <v>4.274</v>
+        <v>4.334</v>
       </c>
       <c r="P22" t="n">
-        <v>4.359</v>
+        <v>4.416</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.446</v>
+        <v>4.5</v>
       </c>
       <c r="R22" t="n">
-        <v>4.546</v>
+        <v>4.593</v>
       </c>
       <c r="S22" t="n">
-        <v>4.652</v>
+        <v>4.691</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.915</v>
+        <v>2.926</v>
       </c>
       <c r="G23" t="n">
-        <v>3.151</v>
+        <v>3.165</v>
       </c>
       <c r="H23" t="n">
-        <v>3.391</v>
+        <v>3.407</v>
       </c>
       <c r="I23" t="n">
-        <v>3.556</v>
+        <v>3.575</v>
       </c>
       <c r="J23" t="n">
-        <v>3.797</v>
+        <v>3.824</v>
       </c>
       <c r="K23" t="n">
-        <v>3.917</v>
+        <v>3.958</v>
       </c>
       <c r="L23" t="n">
-        <v>3.931</v>
+        <v>3.976</v>
       </c>
       <c r="M23" t="n">
-        <v>4.022</v>
+        <v>4.077</v>
       </c>
       <c r="N23" t="n">
-        <v>4.078</v>
+        <v>4.143</v>
       </c>
       <c r="O23" t="n">
-        <v>4.148</v>
+        <v>4.208</v>
       </c>
       <c r="P23" t="n">
-        <v>4.221</v>
+        <v>4.278</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.251</v>
+        <v>4.306</v>
       </c>
       <c r="R23" t="n">
-        <v>4.331</v>
+        <v>4.379</v>
       </c>
       <c r="S23" t="n">
-        <v>4.409</v>
+        <v>4.448</v>
       </c>
       <c r="T23" t="n">
-        <v>4.368</v>
+        <v>4.419</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.851</v>
+        <v>2.861</v>
       </c>
       <c r="G24" t="n">
-        <v>3.061</v>
+        <v>3.075</v>
       </c>
       <c r="H24" t="n">
-        <v>3.289</v>
+        <v>3.302</v>
       </c>
       <c r="I24" t="n">
-        <v>3.494</v>
+        <v>3.513</v>
       </c>
       <c r="J24" t="n">
-        <v>3.69</v>
+        <v>3.719</v>
       </c>
       <c r="K24" t="n">
-        <v>3.8</v>
+        <v>3.842</v>
       </c>
       <c r="L24" t="n">
-        <v>3.813</v>
+        <v>3.858</v>
       </c>
       <c r="M24" t="n">
-        <v>3.882</v>
+        <v>3.936</v>
       </c>
       <c r="N24" t="n">
-        <v>3.953</v>
+        <v>4.018</v>
       </c>
       <c r="O24" t="n">
-        <v>4.145</v>
+        <v>4.205</v>
       </c>
       <c r="P24" t="n">
-        <v>4.159</v>
+        <v>4.216</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.178</v>
+        <v>4.232</v>
       </c>
       <c r="R24" t="n">
-        <v>4.253</v>
+        <v>4.301</v>
       </c>
       <c r="S24" t="n">
-        <v>4.324</v>
+        <v>4.363</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.91</v>
+        <v>2.92</v>
       </c>
       <c r="G25" t="n">
-        <v>3.151</v>
+        <v>3.165</v>
       </c>
       <c r="H25" t="n">
-        <v>3.394</v>
+        <v>3.41</v>
       </c>
       <c r="I25" t="n">
-        <v>3.565</v>
+        <v>3.584</v>
       </c>
       <c r="J25" t="n">
-        <v>3.813</v>
+        <v>3.841</v>
       </c>
       <c r="K25" t="n">
-        <v>3.949</v>
+        <v>3.99</v>
       </c>
       <c r="L25" t="n">
-        <v>3.961</v>
+        <v>4.006</v>
       </c>
       <c r="M25" t="n">
-        <v>4.054</v>
+        <v>4.109</v>
       </c>
       <c r="N25" t="n">
-        <v>4.106</v>
+        <v>4.171</v>
       </c>
       <c r="O25" t="n">
-        <v>4.177</v>
+        <v>4.237</v>
       </c>
       <c r="P25" t="n">
-        <v>4.242</v>
+        <v>4.3</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.285</v>
+        <v>4.339</v>
       </c>
       <c r="R25" t="n">
-        <v>4.355</v>
+        <v>4.403</v>
       </c>
       <c r="S25" t="n">
-        <v>4.432</v>
+        <v>4.471</v>
       </c>
       <c r="T25" t="n">
-        <v>4.386</v>
+        <v>4.437</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.244</v>
+        <v>3.257</v>
       </c>
       <c r="G26" t="n">
-        <v>3.457</v>
+        <v>3.473</v>
       </c>
       <c r="H26" t="n">
-        <v>3.787</v>
+        <v>3.805</v>
       </c>
       <c r="I26" t="n">
-        <v>3.978</v>
+        <v>4.003</v>
       </c>
       <c r="J26" t="n">
-        <v>4.379</v>
+        <v>4.408</v>
       </c>
       <c r="K26" t="n">
-        <v>4.748</v>
+        <v>4.792</v>
       </c>
       <c r="L26" t="n">
-        <v>4.815</v>
+        <v>4.863</v>
       </c>
       <c r="M26" t="n">
-        <v>4.954</v>
+        <v>5.007</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.232</v>
+        <v>5.294</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.043</v>
+        <v>3.056</v>
       </c>
       <c r="G27" t="n">
-        <v>3.223</v>
+        <v>3.238</v>
       </c>
       <c r="H27" t="n">
-        <v>3.474</v>
+        <v>3.492</v>
       </c>
       <c r="I27" t="n">
-        <v>3.64</v>
+        <v>3.662</v>
       </c>
       <c r="J27" t="n">
-        <v>3.914</v>
+        <v>3.94</v>
       </c>
       <c r="K27" t="n">
-        <v>4.073</v>
+        <v>4.114</v>
       </c>
       <c r="L27" t="n">
-        <v>4.081</v>
+        <v>4.13</v>
       </c>
       <c r="M27" t="n">
-        <v>4.177</v>
+        <v>4.232</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.335</v>
+        <v>4.4</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.146</v>
+        <v>3.159</v>
       </c>
       <c r="G28" t="n">
-        <v>3.335</v>
+        <v>3.35</v>
       </c>
       <c r="H28" t="n">
-        <v>3.601</v>
+        <v>3.619</v>
       </c>
       <c r="I28" t="n">
-        <v>3.777</v>
+        <v>3.799</v>
       </c>
       <c r="J28" t="n">
-        <v>4.087</v>
+        <v>4.113</v>
       </c>
       <c r="K28" t="n">
-        <v>4.265</v>
+        <v>4.306</v>
       </c>
       <c r="L28" t="n">
-        <v>4.284</v>
+        <v>4.333</v>
       </c>
       <c r="M28" t="n">
-        <v>4.388</v>
+        <v>4.443</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.627</v>
+        <v>4.692</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.991</v>
+        <v>3.004</v>
       </c>
       <c r="G29" t="n">
-        <v>3.167</v>
+        <v>3.182</v>
       </c>
       <c r="H29" t="n">
-        <v>3.41</v>
+        <v>3.428</v>
       </c>
       <c r="I29" t="n">
-        <v>3.565</v>
+        <v>3.586</v>
       </c>
       <c r="J29" t="n">
-        <v>3.826</v>
+        <v>3.852</v>
       </c>
       <c r="K29" t="n">
-        <v>3.969</v>
+        <v>4.01</v>
       </c>
       <c r="L29" t="n">
-        <v>3.967</v>
+        <v>4.016</v>
       </c>
       <c r="M29" t="n">
-        <v>4.04</v>
+        <v>4.095</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.206</v>
+        <v>4.271</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.277</v>
+        <v>3.288</v>
       </c>
       <c r="G30" t="n">
-        <v>3.422</v>
+        <v>3.438</v>
       </c>
       <c r="H30" t="n">
-        <v>3.711</v>
+        <v>3.729</v>
       </c>
       <c r="I30" t="n">
-        <v>3.894</v>
+        <v>3.918</v>
       </c>
       <c r="J30" t="n">
-        <v>4.232</v>
+        <v>4.262</v>
       </c>
       <c r="K30" t="n">
-        <v>4.542</v>
+        <v>4.587</v>
       </c>
       <c r="L30" t="n">
-        <v>4.586</v>
+        <v>4.634</v>
       </c>
       <c r="M30" t="n">
-        <v>4.714</v>
+        <v>4.767</v>
       </c>
       <c r="N30" t="n">
-        <v>4.886</v>
+        <v>4.952</v>
       </c>
       <c r="O30" t="n">
-        <v>5.181</v>
+        <v>5.243</v>
       </c>
       <c r="P30" t="n">
-        <v>5.386</v>
+        <v>5.444</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.127</v>
+        <v>6.183</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.606</v>
+        <v>3.617</v>
       </c>
       <c r="G31" t="n">
-        <v>3.788</v>
+        <v>3.804</v>
       </c>
       <c r="H31" t="n">
-        <v>4.127</v>
+        <v>4.145</v>
       </c>
       <c r="I31" t="n">
-        <v>4.324</v>
+        <v>4.348</v>
       </c>
       <c r="J31" t="n">
-        <v>4.727</v>
+        <v>4.756</v>
       </c>
       <c r="K31" t="n">
-        <v>5.078</v>
+        <v>5.123</v>
       </c>
       <c r="L31" t="n">
-        <v>5.199</v>
+        <v>5.247</v>
       </c>
       <c r="M31" t="n">
-        <v>5.444</v>
+        <v>5.497</v>
       </c>
       <c r="N31" t="n">
-        <v>5.745</v>
+        <v>5.811</v>
       </c>
       <c r="O31" t="n">
-        <v>6.217</v>
+        <v>6.279</v>
       </c>
       <c r="P31" t="n">
-        <v>6.374</v>
+        <v>6.433</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.1</v>
+        <v>7.156</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.376</v>
+        <v>3.386</v>
       </c>
       <c r="G32" t="n">
-        <v>3.54</v>
+        <v>3.556</v>
       </c>
       <c r="H32" t="n">
-        <v>3.855</v>
+        <v>3.873</v>
       </c>
       <c r="I32" t="n">
-        <v>4.053</v>
+        <v>4.077</v>
       </c>
       <c r="J32" t="n">
-        <v>4.413</v>
+        <v>4.443</v>
       </c>
       <c r="K32" t="n">
-        <v>4.727</v>
+        <v>4.772</v>
       </c>
       <c r="L32" t="n">
-        <v>4.79</v>
+        <v>4.838</v>
       </c>
       <c r="M32" t="n">
-        <v>4.986</v>
+        <v>5.039</v>
       </c>
       <c r="N32" t="n">
-        <v>5.247</v>
+        <v>5.313</v>
       </c>
       <c r="O32" t="n">
-        <v>5.626</v>
+        <v>5.688</v>
       </c>
       <c r="P32" t="n">
-        <v>5.846</v>
+        <v>5.904</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.588</v>
+        <v>6.644</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.142</v>
+        <v>3.154</v>
       </c>
       <c r="G33" t="n">
-        <v>3.286</v>
+        <v>3.303</v>
       </c>
       <c r="H33" t="n">
-        <v>3.528</v>
+        <v>3.546</v>
       </c>
       <c r="I33" t="n">
-        <v>3.68</v>
+        <v>3.704</v>
       </c>
       <c r="J33" t="n">
-        <v>3.939</v>
+        <v>3.968</v>
       </c>
       <c r="K33" t="n">
-        <v>4.183</v>
+        <v>4.228</v>
       </c>
       <c r="L33" t="n">
-        <v>4.191</v>
+        <v>4.24</v>
       </c>
       <c r="M33" t="n">
-        <v>4.242</v>
+        <v>4.295</v>
       </c>
       <c r="N33" t="n">
-        <v>4.274</v>
+        <v>4.34</v>
       </c>
       <c r="O33" t="n">
-        <v>4.337</v>
+        <v>4.399</v>
       </c>
       <c r="P33" t="n">
-        <v>4.418</v>
+        <v>4.477</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.843</v>
+        <v>4.9</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.202</v>
+        <v>3.214</v>
       </c>
       <c r="G34" t="n">
-        <v>3.34</v>
+        <v>3.357</v>
       </c>
       <c r="H34" t="n">
-        <v>3.591</v>
+        <v>3.609</v>
       </c>
       <c r="I34" t="n">
-        <v>3.748</v>
+        <v>3.772</v>
       </c>
       <c r="J34" t="n">
-        <v>4.01</v>
+        <v>4.04</v>
       </c>
       <c r="K34" t="n">
-        <v>4.259</v>
+        <v>4.304</v>
       </c>
       <c r="L34" t="n">
-        <v>4.27</v>
+        <v>4.319</v>
       </c>
       <c r="M34" t="n">
-        <v>4.333</v>
+        <v>4.386</v>
       </c>
       <c r="N34" t="n">
-        <v>4.379</v>
+        <v>4.445</v>
       </c>
       <c r="O34" t="n">
-        <v>4.506</v>
+        <v>4.568</v>
       </c>
       <c r="P34" t="n">
-        <v>4.712</v>
+        <v>4.771</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.544</v>
+        <v>5.601</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.176</v>
+        <v>3.188</v>
       </c>
       <c r="G35" t="n">
-        <v>3.314</v>
+        <v>3.331</v>
       </c>
       <c r="H35" t="n">
-        <v>3.559</v>
+        <v>3.577</v>
       </c>
       <c r="I35" t="n">
-        <v>3.715</v>
+        <v>3.739</v>
       </c>
       <c r="J35" t="n">
-        <v>3.979</v>
+        <v>4.008</v>
       </c>
       <c r="K35" t="n">
-        <v>4.213</v>
+        <v>4.258</v>
       </c>
       <c r="L35" t="n">
-        <v>4.225</v>
+        <v>4.274</v>
       </c>
       <c r="M35" t="n">
-        <v>4.279</v>
+        <v>4.332</v>
       </c>
       <c r="N35" t="n">
-        <v>4.315</v>
+        <v>4.382</v>
       </c>
       <c r="O35" t="n">
-        <v>4.403</v>
+        <v>4.465</v>
       </c>
       <c r="P35" t="n">
-        <v>4.515</v>
+        <v>4.574</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.18</v>
+        <v>5.236</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.062</v>
+        <v>3.073</v>
       </c>
       <c r="G36" t="n">
-        <v>3.193</v>
+        <v>3.207</v>
       </c>
       <c r="H36" t="n">
-        <v>3.432</v>
+        <v>3.45</v>
       </c>
       <c r="I36" t="n">
-        <v>3.591</v>
+        <v>3.615</v>
       </c>
       <c r="J36" t="n">
-        <v>3.875</v>
+        <v>3.905</v>
       </c>
       <c r="K36" t="n">
-        <v>4.108</v>
+        <v>4.153</v>
       </c>
       <c r="L36" t="n">
-        <v>4.115</v>
+        <v>4.164</v>
       </c>
       <c r="M36" t="n">
-        <v>4.145</v>
+        <v>4.198</v>
       </c>
       <c r="N36" t="n">
-        <v>4.179</v>
+        <v>4.245</v>
       </c>
       <c r="O36" t="n">
-        <v>4.244</v>
+        <v>4.306</v>
       </c>
       <c r="P36" t="n">
-        <v>4.316</v>
+        <v>4.375</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.56</v>
+        <v>4.617</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.95</v>
+        <v>3.962</v>
       </c>
       <c r="G37" t="n">
-        <v>4.482</v>
+        <v>4.499</v>
       </c>
       <c r="H37" t="n">
-        <v>5.1</v>
+        <v>5.118</v>
       </c>
       <c r="I37" t="n">
-        <v>5.385</v>
+        <v>5.409</v>
       </c>
       <c r="J37" t="n">
-        <v>6.216</v>
+        <v>6.245</v>
       </c>
       <c r="K37" t="n">
-        <v>7.119</v>
+        <v>7.165</v>
       </c>
       <c r="L37" t="n">
-        <v>7.399</v>
+        <v>7.447</v>
       </c>
       <c r="M37" t="n">
-        <v>7.716</v>
+        <v>7.769</v>
       </c>
       <c r="N37" t="n">
-        <v>7.901</v>
+        <v>7.967</v>
       </c>
       <c r="O37" t="n">
-        <v>8.096</v>
+        <v>8.157999999999999</v>
       </c>
       <c r="P37" t="n">
-        <v>8.176</v>
+        <v>8.234</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.59</v>
+        <v>8.647</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.012</v>
+        <v>5.024</v>
       </c>
       <c r="G38" t="n">
-        <v>5.797</v>
+        <v>5.814</v>
       </c>
       <c r="H38" t="n">
-        <v>6.627</v>
+        <v>6.645</v>
       </c>
       <c r="I38" t="n">
-        <v>7.069</v>
+        <v>7.093</v>
       </c>
       <c r="J38" t="n">
-        <v>8.16</v>
+        <v>8.189</v>
       </c>
       <c r="K38" t="n">
-        <v>9.242000000000001</v>
+        <v>9.288</v>
       </c>
       <c r="L38" t="n">
-        <v>9.682</v>
+        <v>9.73</v>
       </c>
       <c r="M38" t="n">
-        <v>10.128</v>
+        <v>10.181</v>
       </c>
       <c r="N38" t="n">
-        <v>10.32</v>
+        <v>10.386</v>
       </c>
       <c r="O38" t="n">
-        <v>10.496</v>
+        <v>10.558</v>
       </c>
       <c r="P38" t="n">
-        <v>10.573</v>
+        <v>10.632</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.041</v>
+        <v>11.097</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.332</v>
+        <v>4.344</v>
       </c>
       <c r="G39" t="n">
-        <v>4.995</v>
+        <v>5.012</v>
       </c>
       <c r="H39" t="n">
-        <v>5.692</v>
+        <v>5.71</v>
       </c>
       <c r="I39" t="n">
-        <v>6.073</v>
+        <v>6.097</v>
       </c>
       <c r="J39" t="n">
-        <v>7.032</v>
+        <v>7.062</v>
       </c>
       <c r="K39" t="n">
-        <v>8.074</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>8.436999999999999</v>
+        <v>8.484999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.763999999999999</v>
+        <v>8.817</v>
       </c>
       <c r="N39" t="n">
-        <v>8.948</v>
+        <v>9.013999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.147</v>
+        <v>9.209</v>
       </c>
       <c r="P39" t="n">
-        <v>9.228</v>
+        <v>9.287000000000001</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.686</v>
+        <v>9.743</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.469</v>
+        <v>3.48</v>
       </c>
       <c r="G40" t="n">
-        <v>3.66</v>
+        <v>3.676</v>
       </c>
       <c r="H40" t="n">
-        <v>3.97</v>
+        <v>3.988</v>
       </c>
       <c r="I40" t="n">
-        <v>4.168</v>
+        <v>4.192</v>
       </c>
       <c r="J40" t="n">
-        <v>4.524</v>
+        <v>4.553</v>
       </c>
       <c r="K40" t="n">
-        <v>4.848</v>
+        <v>4.893</v>
       </c>
       <c r="L40" t="n">
-        <v>4.912</v>
+        <v>4.96</v>
       </c>
       <c r="M40" t="n">
-        <v>5.056</v>
+        <v>5.109</v>
       </c>
       <c r="N40" t="n">
-        <v>5.244</v>
+        <v>5.31</v>
       </c>
       <c r="O40" t="n">
-        <v>5.56</v>
+        <v>5.622</v>
       </c>
       <c r="P40" t="n">
-        <v>5.807</v>
+        <v>5.866</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.578</v>
+        <v>6.634</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.855</v>
+        <v>3.866</v>
       </c>
       <c r="G41" t="n">
-        <v>4.089</v>
+        <v>4.105</v>
       </c>
       <c r="H41" t="n">
-        <v>4.456</v>
+        <v>4.474</v>
       </c>
       <c r="I41" t="n">
-        <v>4.672</v>
+        <v>4.696</v>
       </c>
       <c r="J41" t="n">
-        <v>5.082</v>
+        <v>5.111</v>
       </c>
       <c r="K41" t="n">
-        <v>5.452</v>
+        <v>5.497</v>
       </c>
       <c r="L41" t="n">
-        <v>5.589</v>
+        <v>5.637</v>
       </c>
       <c r="M41" t="n">
-        <v>5.859</v>
+        <v>5.912</v>
       </c>
       <c r="N41" t="n">
-        <v>6.175</v>
+        <v>6.241</v>
       </c>
       <c r="O41" t="n">
-        <v>6.675</v>
+        <v>6.737</v>
       </c>
       <c r="P41" t="n">
-        <v>6.866</v>
+        <v>6.925</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.625</v>
+        <v>7.681</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.59</v>
+        <v>3.601</v>
       </c>
       <c r="G42" t="n">
-        <v>3.809</v>
+        <v>3.825</v>
       </c>
       <c r="H42" t="n">
-        <v>4.146</v>
+        <v>4.164</v>
       </c>
       <c r="I42" t="n">
-        <v>4.356</v>
+        <v>4.38</v>
       </c>
       <c r="J42" t="n">
-        <v>4.729</v>
+        <v>4.758</v>
       </c>
       <c r="K42" t="n">
-        <v>5.069</v>
+        <v>5.114</v>
       </c>
       <c r="L42" t="n">
-        <v>5.147</v>
+        <v>5.195</v>
       </c>
       <c r="M42" t="n">
-        <v>5.363</v>
+        <v>5.416</v>
       </c>
       <c r="N42" t="n">
-        <v>5.658</v>
+        <v>5.724</v>
       </c>
       <c r="O42" t="n">
-        <v>6.052</v>
+        <v>6.114</v>
       </c>
       <c r="P42" t="n">
-        <v>6.309</v>
+        <v>6.368</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.09</v>
+        <v>7.146</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.29</v>
+        <v>3.302</v>
       </c>
       <c r="G43" t="n">
-        <v>3.47</v>
+        <v>3.486</v>
       </c>
       <c r="H43" t="n">
-        <v>3.73</v>
+        <v>3.748</v>
       </c>
       <c r="I43" t="n">
-        <v>3.889</v>
+        <v>3.913</v>
       </c>
       <c r="J43" t="n">
-        <v>4.166</v>
+        <v>4.195</v>
       </c>
       <c r="K43" t="n">
-        <v>4.415</v>
+        <v>4.46</v>
       </c>
       <c r="L43" t="n">
-        <v>4.434</v>
+        <v>4.483</v>
       </c>
       <c r="M43" t="n">
-        <v>4.497</v>
+        <v>4.55</v>
       </c>
       <c r="N43" t="n">
-        <v>4.543</v>
+        <v>4.61</v>
       </c>
       <c r="O43" t="n">
-        <v>4.65</v>
+        <v>4.712</v>
       </c>
       <c r="P43" t="n">
-        <v>4.784</v>
+        <v>4.842</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.454</v>
+        <v>5.51</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.14</v>
+        <v>3.151</v>
       </c>
       <c r="G44" t="n">
-        <v>3.302</v>
+        <v>3.316</v>
       </c>
       <c r="H44" t="n">
-        <v>3.555</v>
+        <v>3.573</v>
       </c>
       <c r="I44" t="n">
-        <v>3.718</v>
+        <v>3.742</v>
       </c>
       <c r="J44" t="n">
-        <v>4.016</v>
+        <v>4.045</v>
       </c>
       <c r="K44" t="n">
-        <v>4.259</v>
+        <v>4.304</v>
       </c>
       <c r="L44" t="n">
-        <v>4.277</v>
+        <v>4.326</v>
       </c>
       <c r="M44" t="n">
-        <v>4.315</v>
+        <v>4.368</v>
       </c>
       <c r="N44" t="n">
-        <v>4.36</v>
+        <v>4.426</v>
       </c>
       <c r="O44" t="n">
-        <v>4.445</v>
+        <v>4.507</v>
       </c>
       <c r="P44" t="n">
-        <v>4.546</v>
+        <v>4.605</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.824</v>
+        <v>4.88</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-19 ~ 2026-06-19
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.484</v>
+        <v>3.5</v>
       </c>
       <c r="G2" t="n">
-        <v>3.794</v>
+        <v>3.819</v>
       </c>
       <c r="H2" t="n">
-        <v>4.06</v>
+        <v>4.088</v>
       </c>
       <c r="I2" t="n">
-        <v>4.196</v>
+        <v>4.233</v>
       </c>
       <c r="J2" t="n">
-        <v>4.488</v>
+        <v>4.524</v>
       </c>
       <c r="K2" t="n">
-        <v>4.837</v>
+        <v>4.875</v>
       </c>
       <c r="L2" t="n">
-        <v>4.994</v>
+        <v>5.036</v>
       </c>
       <c r="M2" t="n">
-        <v>5.242</v>
+        <v>5.279</v>
       </c>
       <c r="N2" t="n">
-        <v>5.518</v>
+        <v>5.555</v>
       </c>
       <c r="O2" t="n">
-        <v>5.761</v>
+        <v>5.811</v>
       </c>
       <c r="P2" t="n">
-        <v>5.962</v>
+        <v>6.011</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.584</v>
+        <v>6.631</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.504</v>
+        <v>4.52</v>
       </c>
       <c r="G3" t="n">
-        <v>4.996</v>
+        <v>5.021</v>
       </c>
       <c r="H3" t="n">
-        <v>5.295</v>
+        <v>5.323</v>
       </c>
       <c r="I3" t="n">
-        <v>5.424</v>
+        <v>5.461</v>
       </c>
       <c r="J3" t="n">
-        <v>5.734</v>
+        <v>5.77</v>
       </c>
       <c r="K3" t="n">
-        <v>6.153</v>
+        <v>6.192</v>
       </c>
       <c r="L3" t="n">
-        <v>6.38</v>
+        <v>6.422</v>
       </c>
       <c r="M3" t="n">
-        <v>6.658</v>
+        <v>6.695</v>
       </c>
       <c r="N3" t="n">
-        <v>6.877</v>
+        <v>6.914</v>
       </c>
       <c r="O3" t="n">
-        <v>7.071</v>
+        <v>7.121</v>
       </c>
       <c r="P3" t="n">
-        <v>7.14</v>
+        <v>7.19</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.65</v>
+        <v>7.698</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.996</v>
+        <v>4.012</v>
       </c>
       <c r="G4" t="n">
-        <v>4.377</v>
+        <v>4.402</v>
       </c>
       <c r="H4" t="n">
-        <v>4.704</v>
+        <v>4.732</v>
       </c>
       <c r="I4" t="n">
-        <v>4.867</v>
+        <v>4.904</v>
       </c>
       <c r="J4" t="n">
-        <v>5.177</v>
+        <v>5.213</v>
       </c>
       <c r="K4" t="n">
-        <v>5.591</v>
+        <v>5.63</v>
       </c>
       <c r="L4" t="n">
-        <v>5.749</v>
+        <v>5.79</v>
       </c>
       <c r="M4" t="n">
-        <v>6.016</v>
+        <v>6.053</v>
       </c>
       <c r="N4" t="n">
-        <v>6.205</v>
+        <v>6.242</v>
       </c>
       <c r="O4" t="n">
-        <v>6.422</v>
+        <v>6.473</v>
       </c>
       <c r="P4" t="n">
-        <v>6.492</v>
+        <v>6.542</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.005</v>
+        <v>7.053</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.182</v>
+        <v>3.198</v>
       </c>
       <c r="G5" t="n">
-        <v>3.337</v>
+        <v>3.361</v>
       </c>
       <c r="H5" t="n">
-        <v>3.567</v>
+        <v>3.594</v>
       </c>
       <c r="I5" t="n">
-        <v>3.768</v>
+        <v>3.805</v>
       </c>
       <c r="J5" t="n">
-        <v>4.048</v>
+        <v>4.085</v>
       </c>
       <c r="K5" t="n">
-        <v>4.239</v>
+        <v>4.279</v>
       </c>
       <c r="L5" t="n">
-        <v>4.243</v>
+        <v>4.285</v>
       </c>
       <c r="M5" t="n">
-        <v>4.3</v>
+        <v>4.337</v>
       </c>
       <c r="N5" t="n">
-        <v>4.33</v>
+        <v>4.367</v>
       </c>
       <c r="O5" t="n">
-        <v>4.36</v>
+        <v>4.411</v>
       </c>
       <c r="P5" t="n">
-        <v>4.631</v>
+        <v>4.68</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.496</v>
+        <v>5.544</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.222</v>
+        <v>3.238</v>
       </c>
       <c r="G6" t="n">
-        <v>3.392</v>
+        <v>3.417</v>
       </c>
       <c r="H6" t="n">
-        <v>3.636</v>
+        <v>3.665</v>
       </c>
       <c r="I6" t="n">
-        <v>3.85</v>
+        <v>3.888</v>
       </c>
       <c r="J6" t="n">
-        <v>4.139</v>
+        <v>4.174</v>
       </c>
       <c r="K6" t="n">
-        <v>4.351</v>
+        <v>4.391</v>
       </c>
       <c r="L6" t="n">
-        <v>4.361</v>
+        <v>4.402</v>
       </c>
       <c r="M6" t="n">
-        <v>4.456</v>
+        <v>4.493</v>
       </c>
       <c r="N6" t="n">
-        <v>4.497</v>
+        <v>4.534</v>
       </c>
       <c r="O6" t="n">
-        <v>4.627</v>
+        <v>4.677</v>
       </c>
       <c r="P6" t="n">
-        <v>5.063</v>
+        <v>5.112</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.892</v>
+        <v>5.94</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.203</v>
+        <v>3.219</v>
       </c>
       <c r="G7" t="n">
-        <v>3.356</v>
+        <v>3.38</v>
       </c>
       <c r="H7" t="n">
-        <v>3.583</v>
+        <v>3.61</v>
       </c>
       <c r="I7" t="n">
-        <v>3.787</v>
+        <v>3.824</v>
       </c>
       <c r="J7" t="n">
-        <v>4.072</v>
+        <v>4.109</v>
       </c>
       <c r="K7" t="n">
-        <v>4.267</v>
+        <v>4.307</v>
       </c>
       <c r="L7" t="n">
-        <v>4.269</v>
+        <v>4.311</v>
       </c>
       <c r="M7" t="n">
-        <v>4.359</v>
+        <v>4.396</v>
       </c>
       <c r="N7" t="n">
-        <v>4.389</v>
+        <v>4.426</v>
       </c>
       <c r="O7" t="n">
-        <v>4.524</v>
+        <v>4.574</v>
       </c>
       <c r="P7" t="n">
-        <v>4.847</v>
+        <v>4.896</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.66</v>
+        <v>5.707</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.617</v>
+        <v>5.633</v>
       </c>
       <c r="G8" t="n">
-        <v>6.295</v>
+        <v>6.32</v>
       </c>
       <c r="H8" t="n">
-        <v>6.743</v>
+        <v>6.771</v>
       </c>
       <c r="I8" t="n">
-        <v>6.951</v>
+        <v>6.988</v>
       </c>
       <c r="J8" t="n">
-        <v>7.33</v>
+        <v>7.365</v>
       </c>
       <c r="K8" t="n">
-        <v>8.026</v>
+        <v>8.065</v>
       </c>
       <c r="L8" t="n">
-        <v>8.337999999999999</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.648</v>
+        <v>8.685</v>
       </c>
       <c r="N8" t="n">
-        <v>8.801</v>
+        <v>8.837999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>9.08</v>
+        <v>9.131</v>
       </c>
       <c r="P8" t="n">
-        <v>9.253</v>
+        <v>9.303000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.962</v>
+        <v>10.014</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.742</v>
+        <v>2.745</v>
       </c>
       <c r="G9" t="n">
-        <v>2.981</v>
+        <v>2.989</v>
       </c>
       <c r="H9" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="I9" t="n">
-        <v>3.268</v>
+        <v>3.285</v>
       </c>
       <c r="J9" t="n">
-        <v>3.489</v>
+        <v>3.511</v>
       </c>
       <c r="K9" t="n">
-        <v>3.604</v>
+        <v>3.634</v>
       </c>
       <c r="L9" t="n">
-        <v>3.694</v>
+        <v>3.726</v>
       </c>
       <c r="M9" t="n">
-        <v>3.752</v>
+        <v>3.782</v>
       </c>
       <c r="N9" t="n">
-        <v>3.889</v>
+        <v>3.92</v>
       </c>
       <c r="O9" t="n">
-        <v>3.951</v>
+        <v>4.002</v>
       </c>
       <c r="P9" t="n">
-        <v>4.067</v>
+        <v>4.117</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.118</v>
+        <v>4.17</v>
       </c>
       <c r="R9" t="n">
-        <v>4.192</v>
+        <v>4.232</v>
       </c>
       <c r="S9" t="n">
-        <v>4.235</v>
+        <v>4.265</v>
       </c>
       <c r="T9" t="n">
-        <v>4.207</v>
+        <v>4.265</v>
       </c>
       <c r="U9" t="n">
-        <v>4.092</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.75</v>
+        <v>2.754</v>
       </c>
       <c r="G10" t="n">
-        <v>2.988</v>
+        <v>2.997</v>
       </c>
       <c r="H10" t="n">
-        <v>3.193</v>
+        <v>3.204</v>
       </c>
       <c r="I10" t="n">
-        <v>3.271</v>
+        <v>3.288</v>
       </c>
       <c r="J10" t="n">
-        <v>3.505</v>
+        <v>3.526</v>
       </c>
       <c r="K10" t="n">
-        <v>3.645</v>
+        <v>3.675</v>
       </c>
       <c r="L10" t="n">
-        <v>3.707</v>
+        <v>3.739</v>
       </c>
       <c r="M10" t="n">
-        <v>3.812</v>
+        <v>3.843</v>
       </c>
       <c r="N10" t="n">
-        <v>3.917</v>
+        <v>3.948</v>
       </c>
       <c r="O10" t="n">
-        <v>4.18</v>
+        <v>4.23</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.555</v>
+        <v>2.559</v>
       </c>
       <c r="G11" t="n">
-        <v>2.791</v>
+        <v>2.798</v>
       </c>
       <c r="H11" t="n">
-        <v>3.015</v>
+        <v>3.026</v>
       </c>
       <c r="I11" t="n">
-        <v>3.075</v>
+        <v>3.092</v>
       </c>
       <c r="J11" t="n">
-        <v>3.3</v>
+        <v>3.322</v>
       </c>
       <c r="K11" t="n">
-        <v>3.428</v>
+        <v>3.457</v>
       </c>
       <c r="L11" t="n">
-        <v>3.504</v>
+        <v>3.536</v>
       </c>
       <c r="M11" t="n">
-        <v>3.62</v>
+        <v>3.651</v>
       </c>
       <c r="N11" t="n">
-        <v>3.724</v>
+        <v>3.755</v>
       </c>
       <c r="O11" t="n">
-        <v>3.946</v>
+        <v>3.996</v>
       </c>
       <c r="P11" t="n">
-        <v>4.011</v>
+        <v>4.061</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.317</v>
+        <v>4.368</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.401</v>
+        <v>3.41</v>
       </c>
       <c r="G12" t="n">
-        <v>3.687</v>
+        <v>3.704</v>
       </c>
       <c r="H12" t="n">
-        <v>3.956</v>
+        <v>3.975</v>
       </c>
       <c r="I12" t="n">
-        <v>4.16</v>
+        <v>4.195</v>
       </c>
       <c r="J12" t="n">
-        <v>4.471</v>
+        <v>4.504</v>
       </c>
       <c r="K12" t="n">
-        <v>4.619</v>
+        <v>4.653</v>
       </c>
       <c r="L12" t="n">
-        <v>4.646</v>
+        <v>4.685</v>
       </c>
       <c r="M12" t="n">
-        <v>4.764</v>
+        <v>4.804</v>
       </c>
       <c r="N12" t="n">
-        <v>4.842</v>
+        <v>4.881</v>
       </c>
       <c r="O12" t="n">
-        <v>4.985</v>
+        <v>5.036</v>
       </c>
       <c r="P12" t="n">
-        <v>5.108</v>
+        <v>5.159</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.437</v>
+        <v>5.487</v>
       </c>
       <c r="R12" t="n">
-        <v>5.688</v>
+        <v>5.727</v>
       </c>
       <c r="S12" t="n">
-        <v>5.944</v>
+        <v>5.972</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.154</v>
+        <v>3.164</v>
       </c>
       <c r="G13" t="n">
-        <v>3.377</v>
+        <v>3.394</v>
       </c>
       <c r="H13" t="n">
-        <v>3.623</v>
+        <v>3.642</v>
       </c>
       <c r="I13" t="n">
-        <v>3.808</v>
+        <v>3.843</v>
       </c>
       <c r="J13" t="n">
-        <v>4.108</v>
+        <v>4.14</v>
       </c>
       <c r="K13" t="n">
-        <v>4.252</v>
+        <v>4.286</v>
       </c>
       <c r="L13" t="n">
-        <v>4.285</v>
+        <v>4.324</v>
       </c>
       <c r="M13" t="n">
-        <v>4.391</v>
+        <v>4.432</v>
       </c>
       <c r="N13" t="n">
-        <v>4.471</v>
+        <v>4.509</v>
       </c>
       <c r="O13" t="n">
-        <v>4.614</v>
+        <v>4.664</v>
       </c>
       <c r="P13" t="n">
-        <v>4.699</v>
+        <v>4.75</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.959</v>
+        <v>5.008</v>
       </c>
       <c r="R13" t="n">
-        <v>5.238</v>
+        <v>5.277</v>
       </c>
       <c r="S13" t="n">
-        <v>5.506</v>
+        <v>5.535</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.972</v>
+        <v>2.981</v>
       </c>
       <c r="G14" t="n">
-        <v>3.178</v>
+        <v>3.195</v>
       </c>
       <c r="H14" t="n">
-        <v>3.424</v>
+        <v>3.443</v>
       </c>
       <c r="I14" t="n">
-        <v>3.592</v>
+        <v>3.627</v>
       </c>
       <c r="J14" t="n">
-        <v>3.849</v>
+        <v>3.882</v>
       </c>
       <c r="K14" t="n">
-        <v>3.941</v>
+        <v>3.975</v>
       </c>
       <c r="L14" t="n">
-        <v>3.958</v>
+        <v>3.997</v>
       </c>
       <c r="M14" t="n">
-        <v>4.078</v>
+        <v>4.118</v>
       </c>
       <c r="N14" t="n">
-        <v>4.15</v>
+        <v>4.188</v>
       </c>
       <c r="O14" t="n">
-        <v>4.272</v>
+        <v>4.323</v>
       </c>
       <c r="P14" t="n">
-        <v>4.335</v>
+        <v>4.386</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.548</v>
+        <v>4.598</v>
       </c>
       <c r="R14" t="n">
-        <v>4.752</v>
+        <v>4.791</v>
       </c>
       <c r="S14" t="n">
-        <v>4.959</v>
+        <v>4.987</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.949</v>
+        <v>2.959</v>
       </c>
       <c r="G15" t="n">
-        <v>3.153</v>
+        <v>3.17</v>
       </c>
       <c r="H15" t="n">
-        <v>3.395</v>
+        <v>3.414</v>
       </c>
       <c r="I15" t="n">
-        <v>3.543</v>
+        <v>3.578</v>
       </c>
       <c r="J15" t="n">
-        <v>3.787</v>
+        <v>3.82</v>
       </c>
       <c r="K15" t="n">
-        <v>3.893</v>
+        <v>3.928</v>
       </c>
       <c r="L15" t="n">
-        <v>3.894</v>
+        <v>3.933</v>
       </c>
       <c r="M15" t="n">
-        <v>3.99</v>
+        <v>4.031</v>
       </c>
       <c r="N15" t="n">
-        <v>4.053</v>
+        <v>4.091</v>
       </c>
       <c r="O15" t="n">
-        <v>4.215</v>
+        <v>4.266</v>
       </c>
       <c r="P15" t="n">
-        <v>4.231</v>
+        <v>4.282</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.45</v>
+        <v>4.5</v>
       </c>
       <c r="R15" t="n">
-        <v>4.647</v>
+        <v>4.686</v>
       </c>
       <c r="S15" t="n">
-        <v>4.854</v>
+        <v>4.882</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.949</v>
+        <v>2.959</v>
       </c>
       <c r="G16" t="n">
-        <v>3.153</v>
+        <v>3.17</v>
       </c>
       <c r="H16" t="n">
-        <v>3.395</v>
+        <v>3.414</v>
       </c>
       <c r="I16" t="n">
-        <v>3.543</v>
+        <v>3.578</v>
       </c>
       <c r="J16" t="n">
-        <v>3.787</v>
+        <v>3.82</v>
       </c>
       <c r="K16" t="n">
-        <v>3.893</v>
+        <v>3.928</v>
       </c>
       <c r="L16" t="n">
-        <v>3.894</v>
+        <v>3.933</v>
       </c>
       <c r="M16" t="n">
-        <v>3.99</v>
+        <v>4.031</v>
       </c>
       <c r="N16" t="n">
-        <v>4.056</v>
+        <v>4.094</v>
       </c>
       <c r="O16" t="n">
-        <v>4.222</v>
+        <v>4.272</v>
       </c>
       <c r="P16" t="n">
-        <v>4.255</v>
+        <v>4.306</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.477</v>
+        <v>4.527</v>
       </c>
       <c r="R16" t="n">
-        <v>4.675</v>
+        <v>4.714</v>
       </c>
       <c r="S16" t="n">
-        <v>4.883</v>
+        <v>4.911</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.78</v>
+        <v>2.785</v>
       </c>
       <c r="G17" t="n">
-        <v>3.037</v>
+        <v>3.046</v>
       </c>
       <c r="H17" t="n">
-        <v>3.244</v>
+        <v>3.254</v>
       </c>
       <c r="I17" t="n">
-        <v>3.328</v>
+        <v>3.345</v>
       </c>
       <c r="J17" t="n">
-        <v>3.575</v>
+        <v>3.598</v>
       </c>
       <c r="K17" t="n">
-        <v>3.723</v>
+        <v>3.754</v>
       </c>
       <c r="L17" t="n">
-        <v>3.792</v>
+        <v>3.824</v>
       </c>
       <c r="M17" t="n">
-        <v>3.94</v>
+        <v>3.97</v>
       </c>
       <c r="N17" t="n">
-        <v>4.031</v>
+        <v>4.061</v>
       </c>
       <c r="O17" t="n">
-        <v>4.2</v>
+        <v>4.251</v>
       </c>
       <c r="P17" t="n">
-        <v>4.297</v>
+        <v>4.347</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.782</v>
+        <v>2.786</v>
       </c>
       <c r="G18" t="n">
-        <v>3.038</v>
+        <v>3.047</v>
       </c>
       <c r="H18" t="n">
-        <v>3.244</v>
+        <v>3.254</v>
       </c>
       <c r="I18" t="n">
-        <v>3.328</v>
+        <v>3.345</v>
       </c>
       <c r="J18" t="n">
-        <v>3.575</v>
+        <v>3.598</v>
       </c>
       <c r="K18" t="n">
-        <v>3.724</v>
+        <v>3.753</v>
       </c>
       <c r="L18" t="n">
-        <v>3.792</v>
+        <v>3.824</v>
       </c>
       <c r="M18" t="n">
-        <v>3.94</v>
+        <v>3.97</v>
       </c>
       <c r="N18" t="n">
-        <v>4.032</v>
+        <v>4.062</v>
       </c>
       <c r="O18" t="n">
-        <v>4.199</v>
+        <v>4.25</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.96</v>
+        <v>2.969</v>
       </c>
       <c r="G19" t="n">
-        <v>3.166</v>
+        <v>3.183</v>
       </c>
       <c r="H19" t="n">
-        <v>3.411</v>
+        <v>3.43</v>
       </c>
       <c r="I19" t="n">
-        <v>3.577</v>
+        <v>3.611</v>
       </c>
       <c r="J19" t="n">
-        <v>3.828</v>
+        <v>3.861</v>
       </c>
       <c r="K19" t="n">
-        <v>3.937</v>
+        <v>3.971</v>
       </c>
       <c r="L19" t="n">
-        <v>3.955</v>
+        <v>3.994</v>
       </c>
       <c r="M19" t="n">
-        <v>4.069</v>
+        <v>4.109</v>
       </c>
       <c r="N19" t="n">
-        <v>4.142</v>
+        <v>4.181</v>
       </c>
       <c r="O19" t="n">
-        <v>4.259</v>
+        <v>4.31</v>
       </c>
       <c r="P19" t="n">
-        <v>4.293</v>
+        <v>4.344</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.488</v>
+        <v>4.538</v>
       </c>
       <c r="R19" t="n">
-        <v>4.693</v>
+        <v>4.732</v>
       </c>
       <c r="S19" t="n">
-        <v>4.894</v>
+        <v>4.922</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.671</v>
+        <v>2.68</v>
       </c>
       <c r="G20" t="n">
-        <v>2.767</v>
+        <v>2.778</v>
       </c>
       <c r="H20" t="n">
-        <v>2.856</v>
+        <v>2.87</v>
       </c>
       <c r="I20" t="n">
-        <v>2.964</v>
+        <v>2.999</v>
       </c>
       <c r="J20" t="n">
-        <v>3.412</v>
+        <v>3.44</v>
       </c>
       <c r="K20" t="n">
-        <v>3.65</v>
+        <v>3.68</v>
       </c>
       <c r="L20" t="n">
-        <v>3.652</v>
+        <v>3.682</v>
       </c>
       <c r="M20" t="n">
-        <v>3.764</v>
+        <v>3.795</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.032</v>
+        <v>3.04</v>
       </c>
       <c r="G21" t="n">
-        <v>3.267</v>
+        <v>3.281</v>
       </c>
       <c r="H21" t="n">
-        <v>3.535</v>
+        <v>3.551</v>
       </c>
       <c r="I21" t="n">
-        <v>3.71</v>
+        <v>3.744</v>
       </c>
       <c r="J21" t="n">
-        <v>4.002</v>
+        <v>4.034</v>
       </c>
       <c r="K21" t="n">
-        <v>4.179</v>
+        <v>4.213</v>
       </c>
       <c r="L21" t="n">
-        <v>4.208</v>
+        <v>4.244</v>
       </c>
       <c r="M21" t="n">
-        <v>4.312</v>
+        <v>4.348</v>
       </c>
       <c r="N21" t="n">
-        <v>4.378</v>
+        <v>4.417</v>
       </c>
       <c r="O21" t="n">
-        <v>4.463</v>
+        <v>4.512</v>
       </c>
       <c r="P21" t="n">
-        <v>4.553</v>
+        <v>4.603</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.641</v>
+        <v>4.693</v>
       </c>
       <c r="R21" t="n">
-        <v>4.745</v>
+        <v>4.785</v>
       </c>
       <c r="S21" t="n">
-        <v>4.846</v>
+        <v>4.876</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.979</v>
+        <v>2.987</v>
       </c>
       <c r="G22" t="n">
-        <v>3.211</v>
+        <v>3.225</v>
       </c>
       <c r="H22" t="n">
-        <v>3.467</v>
+        <v>3.483</v>
       </c>
       <c r="I22" t="n">
-        <v>3.628</v>
+        <v>3.662</v>
       </c>
       <c r="J22" t="n">
-        <v>3.887</v>
+        <v>3.92</v>
       </c>
       <c r="K22" t="n">
-        <v>4.061</v>
+        <v>4.095</v>
       </c>
       <c r="L22" t="n">
-        <v>4.077</v>
+        <v>4.113</v>
       </c>
       <c r="M22" t="n">
-        <v>4.185</v>
+        <v>4.221</v>
       </c>
       <c r="N22" t="n">
-        <v>4.254</v>
+        <v>4.292</v>
       </c>
       <c r="O22" t="n">
-        <v>4.334</v>
+        <v>4.383</v>
       </c>
       <c r="P22" t="n">
-        <v>4.416</v>
+        <v>4.466</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.5</v>
+        <v>4.552</v>
       </c>
       <c r="R22" t="n">
-        <v>4.593</v>
+        <v>4.633</v>
       </c>
       <c r="S22" t="n">
-        <v>4.691</v>
+        <v>4.721</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.926</v>
+        <v>2.934</v>
       </c>
       <c r="G23" t="n">
-        <v>3.165</v>
+        <v>3.179</v>
       </c>
       <c r="H23" t="n">
-        <v>3.407</v>
+        <v>3.423</v>
       </c>
       <c r="I23" t="n">
-        <v>3.575</v>
+        <v>3.607</v>
       </c>
       <c r="J23" t="n">
-        <v>3.824</v>
+        <v>3.855</v>
       </c>
       <c r="K23" t="n">
-        <v>3.958</v>
+        <v>3.992</v>
       </c>
       <c r="L23" t="n">
-        <v>3.976</v>
+        <v>4.012</v>
       </c>
       <c r="M23" t="n">
-        <v>4.077</v>
+        <v>4.112</v>
       </c>
       <c r="N23" t="n">
-        <v>4.143</v>
+        <v>4.181</v>
       </c>
       <c r="O23" t="n">
-        <v>4.208</v>
+        <v>4.258</v>
       </c>
       <c r="P23" t="n">
-        <v>4.278</v>
+        <v>4.328</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.306</v>
+        <v>4.357</v>
       </c>
       <c r="R23" t="n">
-        <v>4.379</v>
+        <v>4.419</v>
       </c>
       <c r="S23" t="n">
-        <v>4.448</v>
+        <v>4.478</v>
       </c>
       <c r="T23" t="n">
-        <v>4.419</v>
+        <v>4.477</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.861</v>
+        <v>2.869</v>
       </c>
       <c r="G24" t="n">
-        <v>3.075</v>
+        <v>3.089</v>
       </c>
       <c r="H24" t="n">
-        <v>3.302</v>
+        <v>3.318</v>
       </c>
       <c r="I24" t="n">
-        <v>3.513</v>
+        <v>3.545</v>
       </c>
       <c r="J24" t="n">
-        <v>3.719</v>
+        <v>3.751</v>
       </c>
       <c r="K24" t="n">
-        <v>3.842</v>
+        <v>3.876</v>
       </c>
       <c r="L24" t="n">
-        <v>3.858</v>
+        <v>3.894</v>
       </c>
       <c r="M24" t="n">
-        <v>3.936</v>
+        <v>3.972</v>
       </c>
       <c r="N24" t="n">
-        <v>4.018</v>
+        <v>4.056</v>
       </c>
       <c r="O24" t="n">
-        <v>4.205</v>
+        <v>4.254</v>
       </c>
       <c r="P24" t="n">
-        <v>4.216</v>
+        <v>4.266</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.232</v>
+        <v>4.284</v>
       </c>
       <c r="R24" t="n">
-        <v>4.301</v>
+        <v>4.341</v>
       </c>
       <c r="S24" t="n">
-        <v>4.363</v>
+        <v>4.393</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.92</v>
+        <v>2.928</v>
       </c>
       <c r="G25" t="n">
-        <v>3.165</v>
+        <v>3.179</v>
       </c>
       <c r="H25" t="n">
-        <v>3.41</v>
+        <v>3.426</v>
       </c>
       <c r="I25" t="n">
-        <v>3.584</v>
+        <v>3.616</v>
       </c>
       <c r="J25" t="n">
-        <v>3.841</v>
+        <v>3.873</v>
       </c>
       <c r="K25" t="n">
-        <v>3.99</v>
+        <v>4.025</v>
       </c>
       <c r="L25" t="n">
-        <v>4.006</v>
+        <v>4.043</v>
       </c>
       <c r="M25" t="n">
-        <v>4.109</v>
+        <v>4.144</v>
       </c>
       <c r="N25" t="n">
-        <v>4.171</v>
+        <v>4.209</v>
       </c>
       <c r="O25" t="n">
-        <v>4.237</v>
+        <v>4.287</v>
       </c>
       <c r="P25" t="n">
-        <v>4.3</v>
+        <v>4.35</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.339</v>
+        <v>4.391</v>
       </c>
       <c r="R25" t="n">
-        <v>4.403</v>
+        <v>4.443</v>
       </c>
       <c r="S25" t="n">
-        <v>4.471</v>
+        <v>4.501</v>
       </c>
       <c r="T25" t="n">
-        <v>4.437</v>
+        <v>4.495</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.257</v>
+        <v>3.277</v>
       </c>
       <c r="G26" t="n">
-        <v>3.473</v>
+        <v>3.497</v>
       </c>
       <c r="H26" t="n">
-        <v>3.805</v>
+        <v>3.835</v>
       </c>
       <c r="I26" t="n">
-        <v>4.003</v>
+        <v>4.042</v>
       </c>
       <c r="J26" t="n">
-        <v>4.408</v>
+        <v>4.443</v>
       </c>
       <c r="K26" t="n">
-        <v>4.792</v>
+        <v>4.828</v>
       </c>
       <c r="L26" t="n">
-        <v>4.863</v>
+        <v>4.9</v>
       </c>
       <c r="M26" t="n">
-        <v>5.007</v>
+        <v>5.041</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.294</v>
+        <v>5.343</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.056</v>
+        <v>3.071</v>
       </c>
       <c r="G27" t="n">
-        <v>3.238</v>
+        <v>3.259</v>
       </c>
       <c r="H27" t="n">
-        <v>3.492</v>
+        <v>3.518</v>
       </c>
       <c r="I27" t="n">
-        <v>3.662</v>
+        <v>3.7</v>
       </c>
       <c r="J27" t="n">
-        <v>3.94</v>
+        <v>3.974</v>
       </c>
       <c r="K27" t="n">
-        <v>4.114</v>
+        <v>4.149</v>
       </c>
       <c r="L27" t="n">
-        <v>4.13</v>
+        <v>4.17</v>
       </c>
       <c r="M27" t="n">
-        <v>4.232</v>
+        <v>4.27</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.4</v>
+        <v>4.45</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.159</v>
+        <v>3.174</v>
       </c>
       <c r="G28" t="n">
-        <v>3.35</v>
+        <v>3.371</v>
       </c>
       <c r="H28" t="n">
-        <v>3.619</v>
+        <v>3.645</v>
       </c>
       <c r="I28" t="n">
-        <v>3.799</v>
+        <v>3.837</v>
       </c>
       <c r="J28" t="n">
-        <v>4.113</v>
+        <v>4.146</v>
       </c>
       <c r="K28" t="n">
-        <v>4.306</v>
+        <v>4.341</v>
       </c>
       <c r="L28" t="n">
-        <v>4.333</v>
+        <v>4.373</v>
       </c>
       <c r="M28" t="n">
-        <v>4.443</v>
+        <v>4.482</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.692</v>
+        <v>4.742</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3.004</v>
+        <v>3.019</v>
       </c>
       <c r="G29" t="n">
-        <v>3.182</v>
+        <v>3.203</v>
       </c>
       <c r="H29" t="n">
-        <v>3.428</v>
+        <v>3.454</v>
       </c>
       <c r="I29" t="n">
-        <v>3.586</v>
+        <v>3.624</v>
       </c>
       <c r="J29" t="n">
-        <v>3.852</v>
+        <v>3.885</v>
       </c>
       <c r="K29" t="n">
-        <v>4.01</v>
+        <v>4.045</v>
       </c>
       <c r="L29" t="n">
-        <v>4.016</v>
+        <v>4.056</v>
       </c>
       <c r="M29" t="n">
-        <v>4.095</v>
+        <v>4.133</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.271</v>
+        <v>4.322</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.288</v>
+        <v>3.308</v>
       </c>
       <c r="G30" t="n">
-        <v>3.438</v>
+        <v>3.464</v>
       </c>
       <c r="H30" t="n">
-        <v>3.729</v>
+        <v>3.759</v>
       </c>
       <c r="I30" t="n">
-        <v>3.918</v>
+        <v>3.957</v>
       </c>
       <c r="J30" t="n">
-        <v>4.262</v>
+        <v>4.294</v>
       </c>
       <c r="K30" t="n">
-        <v>4.587</v>
+        <v>4.62</v>
       </c>
       <c r="L30" t="n">
-        <v>4.634</v>
+        <v>4.67</v>
       </c>
       <c r="M30" t="n">
-        <v>4.767</v>
+        <v>4.8</v>
       </c>
       <c r="N30" t="n">
-        <v>4.952</v>
+        <v>4.984</v>
       </c>
       <c r="O30" t="n">
-        <v>5.243</v>
+        <v>5.293</v>
       </c>
       <c r="P30" t="n">
-        <v>5.444</v>
+        <v>5.494</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.183</v>
+        <v>6.232</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.617</v>
+        <v>3.637</v>
       </c>
       <c r="G31" t="n">
-        <v>3.804</v>
+        <v>3.83</v>
       </c>
       <c r="H31" t="n">
-        <v>4.145</v>
+        <v>4.175</v>
       </c>
       <c r="I31" t="n">
-        <v>4.348</v>
+        <v>4.388</v>
       </c>
       <c r="J31" t="n">
-        <v>4.756</v>
+        <v>4.788</v>
       </c>
       <c r="K31" t="n">
-        <v>5.123</v>
+        <v>5.156</v>
       </c>
       <c r="L31" t="n">
-        <v>5.247</v>
+        <v>5.282</v>
       </c>
       <c r="M31" t="n">
-        <v>5.497</v>
+        <v>5.53</v>
       </c>
       <c r="N31" t="n">
-        <v>5.811</v>
+        <v>5.843</v>
       </c>
       <c r="O31" t="n">
-        <v>6.279</v>
+        <v>6.329</v>
       </c>
       <c r="P31" t="n">
-        <v>6.433</v>
+        <v>6.483</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.156</v>
+        <v>7.205</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.386</v>
+        <v>3.407</v>
       </c>
       <c r="G32" t="n">
-        <v>3.556</v>
+        <v>3.582</v>
       </c>
       <c r="H32" t="n">
-        <v>3.873</v>
+        <v>3.903</v>
       </c>
       <c r="I32" t="n">
-        <v>4.077</v>
+        <v>4.116</v>
       </c>
       <c r="J32" t="n">
-        <v>4.443</v>
+        <v>4.475</v>
       </c>
       <c r="K32" t="n">
-        <v>4.772</v>
+        <v>4.805</v>
       </c>
       <c r="L32" t="n">
-        <v>4.838</v>
+        <v>4.874</v>
       </c>
       <c r="M32" t="n">
-        <v>5.039</v>
+        <v>5.072</v>
       </c>
       <c r="N32" t="n">
-        <v>5.313</v>
+        <v>5.345</v>
       </c>
       <c r="O32" t="n">
-        <v>5.688</v>
+        <v>5.738</v>
       </c>
       <c r="P32" t="n">
-        <v>5.904</v>
+        <v>5.954</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.644</v>
+        <v>6.693</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.154</v>
+        <v>3.174</v>
       </c>
       <c r="G33" t="n">
-        <v>3.303</v>
+        <v>3.329</v>
       </c>
       <c r="H33" t="n">
-        <v>3.546</v>
+        <v>3.576</v>
       </c>
       <c r="I33" t="n">
-        <v>3.704</v>
+        <v>3.744</v>
       </c>
       <c r="J33" t="n">
-        <v>3.968</v>
+        <v>4</v>
       </c>
       <c r="K33" t="n">
-        <v>4.228</v>
+        <v>4.261</v>
       </c>
       <c r="L33" t="n">
-        <v>4.24</v>
+        <v>4.276</v>
       </c>
       <c r="M33" t="n">
-        <v>4.295</v>
+        <v>4.328</v>
       </c>
       <c r="N33" t="n">
-        <v>4.34</v>
+        <v>4.372</v>
       </c>
       <c r="O33" t="n">
-        <v>4.399</v>
+        <v>4.449</v>
       </c>
       <c r="P33" t="n">
-        <v>4.477</v>
+        <v>4.527</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.9</v>
+        <v>4.949</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.214</v>
+        <v>3.234</v>
       </c>
       <c r="G34" t="n">
-        <v>3.357</v>
+        <v>3.383</v>
       </c>
       <c r="H34" t="n">
-        <v>3.609</v>
+        <v>3.639</v>
       </c>
       <c r="I34" t="n">
-        <v>3.772</v>
+        <v>3.813</v>
       </c>
       <c r="J34" t="n">
-        <v>4.04</v>
+        <v>4.072</v>
       </c>
       <c r="K34" t="n">
-        <v>4.304</v>
+        <v>4.339</v>
       </c>
       <c r="L34" t="n">
-        <v>4.319</v>
+        <v>4.354</v>
       </c>
       <c r="M34" t="n">
-        <v>4.386</v>
+        <v>4.419</v>
       </c>
       <c r="N34" t="n">
-        <v>4.445</v>
+        <v>4.477</v>
       </c>
       <c r="O34" t="n">
-        <v>4.568</v>
+        <v>4.618</v>
       </c>
       <c r="P34" t="n">
-        <v>4.771</v>
+        <v>4.821</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.601</v>
+        <v>5.65</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.188</v>
+        <v>3.208</v>
       </c>
       <c r="G35" t="n">
-        <v>3.331</v>
+        <v>3.357</v>
       </c>
       <c r="H35" t="n">
-        <v>3.577</v>
+        <v>3.607</v>
       </c>
       <c r="I35" t="n">
-        <v>3.739</v>
+        <v>3.779</v>
       </c>
       <c r="J35" t="n">
-        <v>4.008</v>
+        <v>4.04</v>
       </c>
       <c r="K35" t="n">
-        <v>4.258</v>
+        <v>4.291</v>
       </c>
       <c r="L35" t="n">
-        <v>4.274</v>
+        <v>4.31</v>
       </c>
       <c r="M35" t="n">
-        <v>4.332</v>
+        <v>4.365</v>
       </c>
       <c r="N35" t="n">
-        <v>4.382</v>
+        <v>4.414</v>
       </c>
       <c r="O35" t="n">
-        <v>4.465</v>
+        <v>4.515</v>
       </c>
       <c r="P35" t="n">
-        <v>4.574</v>
+        <v>4.624</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.236</v>
+        <v>5.285</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.073</v>
+        <v>3.093</v>
       </c>
       <c r="G36" t="n">
-        <v>3.207</v>
+        <v>3.232</v>
       </c>
       <c r="H36" t="n">
-        <v>3.45</v>
+        <v>3.479</v>
       </c>
       <c r="I36" t="n">
-        <v>3.615</v>
+        <v>3.655</v>
       </c>
       <c r="J36" t="n">
-        <v>3.905</v>
+        <v>3.938</v>
       </c>
       <c r="K36" t="n">
-        <v>4.153</v>
+        <v>4.188</v>
       </c>
       <c r="L36" t="n">
-        <v>4.164</v>
+        <v>4.2</v>
       </c>
       <c r="M36" t="n">
-        <v>4.198</v>
+        <v>4.231</v>
       </c>
       <c r="N36" t="n">
-        <v>4.245</v>
+        <v>4.277</v>
       </c>
       <c r="O36" t="n">
-        <v>4.306</v>
+        <v>4.356</v>
       </c>
       <c r="P36" t="n">
-        <v>4.375</v>
+        <v>4.425</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.617</v>
+        <v>4.666</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.962</v>
+        <v>3.982</v>
       </c>
       <c r="G37" t="n">
-        <v>4.499</v>
+        <v>4.524</v>
       </c>
       <c r="H37" t="n">
-        <v>5.118</v>
+        <v>5.148</v>
       </c>
       <c r="I37" t="n">
-        <v>5.409</v>
+        <v>5.449</v>
       </c>
       <c r="J37" t="n">
-        <v>6.245</v>
+        <v>6.278</v>
       </c>
       <c r="K37" t="n">
-        <v>7.165</v>
+        <v>7.198</v>
       </c>
       <c r="L37" t="n">
-        <v>7.447</v>
+        <v>7.483</v>
       </c>
       <c r="M37" t="n">
-        <v>7.769</v>
+        <v>7.802</v>
       </c>
       <c r="N37" t="n">
-        <v>7.967</v>
+        <v>7.999</v>
       </c>
       <c r="O37" t="n">
-        <v>8.157999999999999</v>
+        <v>8.208</v>
       </c>
       <c r="P37" t="n">
-        <v>8.234</v>
+        <v>8.284000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.647</v>
+        <v>8.698</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.024</v>
+        <v>5.044</v>
       </c>
       <c r="G38" t="n">
-        <v>5.814</v>
+        <v>5.839</v>
       </c>
       <c r="H38" t="n">
-        <v>6.645</v>
+        <v>6.675</v>
       </c>
       <c r="I38" t="n">
-        <v>7.093</v>
+        <v>7.133</v>
       </c>
       <c r="J38" t="n">
-        <v>8.189</v>
+        <v>8.222</v>
       </c>
       <c r="K38" t="n">
-        <v>9.288</v>
+        <v>9.321</v>
       </c>
       <c r="L38" t="n">
-        <v>9.73</v>
+        <v>9.765000000000001</v>
       </c>
       <c r="M38" t="n">
-        <v>10.181</v>
+        <v>10.214</v>
       </c>
       <c r="N38" t="n">
-        <v>10.386</v>
+        <v>10.418</v>
       </c>
       <c r="O38" t="n">
-        <v>10.558</v>
+        <v>10.608</v>
       </c>
       <c r="P38" t="n">
-        <v>10.632</v>
+        <v>10.682</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.097</v>
+        <v>11.148</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.344</v>
+        <v>4.364</v>
       </c>
       <c r="G39" t="n">
-        <v>5.012</v>
+        <v>5.037</v>
       </c>
       <c r="H39" t="n">
-        <v>5.71</v>
+        <v>5.74</v>
       </c>
       <c r="I39" t="n">
-        <v>6.097</v>
+        <v>6.137</v>
       </c>
       <c r="J39" t="n">
-        <v>7.062</v>
+        <v>7.094</v>
       </c>
       <c r="K39" t="n">
-        <v>8.119999999999999</v>
+        <v>8.153</v>
       </c>
       <c r="L39" t="n">
-        <v>8.484999999999999</v>
+        <v>8.521000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.817</v>
+        <v>8.85</v>
       </c>
       <c r="N39" t="n">
-        <v>9.013999999999999</v>
+        <v>9.045999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.209</v>
+        <v>9.259</v>
       </c>
       <c r="P39" t="n">
-        <v>9.287000000000001</v>
+        <v>9.337</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.743</v>
+        <v>9.794</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.48</v>
+        <v>3.5</v>
       </c>
       <c r="G40" t="n">
-        <v>3.676</v>
+        <v>3.702</v>
       </c>
       <c r="H40" t="n">
-        <v>3.988</v>
+        <v>4.018</v>
       </c>
       <c r="I40" t="n">
-        <v>4.192</v>
+        <v>4.231</v>
       </c>
       <c r="J40" t="n">
-        <v>4.553</v>
+        <v>4.586</v>
       </c>
       <c r="K40" t="n">
-        <v>4.893</v>
+        <v>4.926</v>
       </c>
       <c r="L40" t="n">
-        <v>4.96</v>
+        <v>4.995</v>
       </c>
       <c r="M40" t="n">
-        <v>5.109</v>
+        <v>5.142</v>
       </c>
       <c r="N40" t="n">
-        <v>5.31</v>
+        <v>5.342</v>
       </c>
       <c r="O40" t="n">
-        <v>5.622</v>
+        <v>5.672</v>
       </c>
       <c r="P40" t="n">
-        <v>5.866</v>
+        <v>5.915</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.634</v>
+        <v>6.683</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.866</v>
+        <v>3.886</v>
       </c>
       <c r="G41" t="n">
-        <v>4.105</v>
+        <v>4.131</v>
       </c>
       <c r="H41" t="n">
-        <v>4.474</v>
+        <v>4.504</v>
       </c>
       <c r="I41" t="n">
-        <v>4.696</v>
+        <v>4.736</v>
       </c>
       <c r="J41" t="n">
-        <v>5.111</v>
+        <v>5.144</v>
       </c>
       <c r="K41" t="n">
-        <v>5.497</v>
+        <v>5.529</v>
       </c>
       <c r="L41" t="n">
-        <v>5.637</v>
+        <v>5.673</v>
       </c>
       <c r="M41" t="n">
-        <v>5.912</v>
+        <v>5.945</v>
       </c>
       <c r="N41" t="n">
-        <v>6.241</v>
+        <v>6.273</v>
       </c>
       <c r="O41" t="n">
-        <v>6.737</v>
+        <v>6.787</v>
       </c>
       <c r="P41" t="n">
-        <v>6.925</v>
+        <v>6.975</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.681</v>
+        <v>7.73</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.601</v>
+        <v>3.621</v>
       </c>
       <c r="G42" t="n">
-        <v>3.825</v>
+        <v>3.851</v>
       </c>
       <c r="H42" t="n">
-        <v>4.164</v>
+        <v>4.194</v>
       </c>
       <c r="I42" t="n">
-        <v>4.38</v>
+        <v>4.42</v>
       </c>
       <c r="J42" t="n">
-        <v>4.758</v>
+        <v>4.791</v>
       </c>
       <c r="K42" t="n">
-        <v>5.114</v>
+        <v>5.147</v>
       </c>
       <c r="L42" t="n">
-        <v>5.195</v>
+        <v>5.23</v>
       </c>
       <c r="M42" t="n">
-        <v>5.416</v>
+        <v>5.449</v>
       </c>
       <c r="N42" t="n">
-        <v>5.724</v>
+        <v>5.756</v>
       </c>
       <c r="O42" t="n">
-        <v>6.114</v>
+        <v>6.164</v>
       </c>
       <c r="P42" t="n">
-        <v>6.368</v>
+        <v>6.418</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.146</v>
+        <v>7.196</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.302</v>
+        <v>3.324</v>
       </c>
       <c r="G43" t="n">
-        <v>3.486</v>
+        <v>3.514</v>
       </c>
       <c r="H43" t="n">
-        <v>3.748</v>
+        <v>3.778</v>
       </c>
       <c r="I43" t="n">
-        <v>3.913</v>
+        <v>3.953</v>
       </c>
       <c r="J43" t="n">
-        <v>4.195</v>
+        <v>4.228</v>
       </c>
       <c r="K43" t="n">
-        <v>4.46</v>
+        <v>4.493</v>
       </c>
       <c r="L43" t="n">
-        <v>4.483</v>
+        <v>4.519</v>
       </c>
       <c r="M43" t="n">
-        <v>4.55</v>
+        <v>4.583</v>
       </c>
       <c r="N43" t="n">
-        <v>4.61</v>
+        <v>4.642</v>
       </c>
       <c r="O43" t="n">
-        <v>4.712</v>
+        <v>4.762</v>
       </c>
       <c r="P43" t="n">
-        <v>4.842</v>
+        <v>4.892</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.51</v>
+        <v>5.559</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.151</v>
+        <v>3.173</v>
       </c>
       <c r="G44" t="n">
-        <v>3.316</v>
+        <v>3.343</v>
       </c>
       <c r="H44" t="n">
-        <v>3.573</v>
+        <v>3.603</v>
       </c>
       <c r="I44" t="n">
-        <v>3.742</v>
+        <v>3.782</v>
       </c>
       <c r="J44" t="n">
-        <v>4.045</v>
+        <v>4.079</v>
       </c>
       <c r="K44" t="n">
-        <v>4.304</v>
+        <v>4.339</v>
       </c>
       <c r="L44" t="n">
-        <v>4.326</v>
+        <v>4.362</v>
       </c>
       <c r="M44" t="n">
-        <v>4.368</v>
+        <v>4.401</v>
       </c>
       <c r="N44" t="n">
-        <v>4.426</v>
+        <v>4.458</v>
       </c>
       <c r="O44" t="n">
-        <v>4.507</v>
+        <v>4.557</v>
       </c>
       <c r="P44" t="n">
-        <v>4.605</v>
+        <v>4.655</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.88</v>
+        <v>4.93</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-22 ~ 2026-06-22
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.5</v>
+        <v>3.51</v>
       </c>
       <c r="G2" t="n">
-        <v>3.819</v>
+        <v>3.83</v>
       </c>
       <c r="H2" t="n">
-        <v>4.088</v>
+        <v>4.105</v>
       </c>
       <c r="I2" t="n">
-        <v>4.233</v>
+        <v>4.261</v>
       </c>
       <c r="J2" t="n">
-        <v>4.524</v>
+        <v>4.57</v>
       </c>
       <c r="K2" t="n">
-        <v>4.875</v>
+        <v>4.901</v>
       </c>
       <c r="L2" t="n">
-        <v>5.036</v>
+        <v>5.058</v>
       </c>
       <c r="M2" t="n">
-        <v>5.279</v>
+        <v>5.305</v>
       </c>
       <c r="N2" t="n">
-        <v>5.555</v>
+        <v>5.587</v>
       </c>
       <c r="O2" t="n">
-        <v>5.811</v>
+        <v>5.85</v>
       </c>
       <c r="P2" t="n">
-        <v>6.011</v>
+        <v>6.039</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.631</v>
+        <v>6.653</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.52</v>
+        <v>4.53</v>
       </c>
       <c r="G3" t="n">
-        <v>5.021</v>
+        <v>5.032</v>
       </c>
       <c r="H3" t="n">
-        <v>5.323</v>
+        <v>5.34</v>
       </c>
       <c r="I3" t="n">
-        <v>5.461</v>
+        <v>5.489</v>
       </c>
       <c r="J3" t="n">
-        <v>5.77</v>
+        <v>5.815</v>
       </c>
       <c r="K3" t="n">
-        <v>6.192</v>
+        <v>6.217</v>
       </c>
       <c r="L3" t="n">
-        <v>6.422</v>
+        <v>6.444</v>
       </c>
       <c r="M3" t="n">
-        <v>6.695</v>
+        <v>6.721</v>
       </c>
       <c r="N3" t="n">
-        <v>6.914</v>
+        <v>6.946</v>
       </c>
       <c r="O3" t="n">
-        <v>7.121</v>
+        <v>7.16</v>
       </c>
       <c r="P3" t="n">
-        <v>7.19</v>
+        <v>7.217</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.698</v>
+        <v>7.719</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4.012</v>
+        <v>4.022</v>
       </c>
       <c r="G4" t="n">
-        <v>4.402</v>
+        <v>4.413</v>
       </c>
       <c r="H4" t="n">
-        <v>4.732</v>
+        <v>4.749</v>
       </c>
       <c r="I4" t="n">
-        <v>4.904</v>
+        <v>4.932</v>
       </c>
       <c r="J4" t="n">
-        <v>5.213</v>
+        <v>5.259</v>
       </c>
       <c r="K4" t="n">
-        <v>5.63</v>
+        <v>5.655</v>
       </c>
       <c r="L4" t="n">
-        <v>5.79</v>
+        <v>5.813</v>
       </c>
       <c r="M4" t="n">
-        <v>6.053</v>
+        <v>6.079</v>
       </c>
       <c r="N4" t="n">
-        <v>6.242</v>
+        <v>6.274</v>
       </c>
       <c r="O4" t="n">
-        <v>6.473</v>
+        <v>6.511</v>
       </c>
       <c r="P4" t="n">
-        <v>6.542</v>
+        <v>6.569</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.053</v>
+        <v>7.074</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.198</v>
+        <v>3.206</v>
       </c>
       <c r="G5" t="n">
-        <v>3.361</v>
+        <v>3.37</v>
       </c>
       <c r="H5" t="n">
-        <v>3.594</v>
+        <v>3.61</v>
       </c>
       <c r="I5" t="n">
-        <v>3.805</v>
+        <v>3.833</v>
       </c>
       <c r="J5" t="n">
-        <v>4.085</v>
+        <v>4.13</v>
       </c>
       <c r="K5" t="n">
-        <v>4.279</v>
+        <v>4.303</v>
       </c>
       <c r="L5" t="n">
-        <v>4.285</v>
+        <v>4.307</v>
       </c>
       <c r="M5" t="n">
-        <v>4.337</v>
+        <v>4.363</v>
       </c>
       <c r="N5" t="n">
-        <v>4.367</v>
+        <v>4.399</v>
       </c>
       <c r="O5" t="n">
-        <v>4.411</v>
+        <v>4.449</v>
       </c>
       <c r="P5" t="n">
-        <v>4.68</v>
+        <v>4.708</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.544</v>
+        <v>5.561</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.238</v>
+        <v>3.248</v>
       </c>
       <c r="G6" t="n">
-        <v>3.417</v>
+        <v>3.428</v>
       </c>
       <c r="H6" t="n">
-        <v>3.665</v>
+        <v>3.682</v>
       </c>
       <c r="I6" t="n">
-        <v>3.888</v>
+        <v>3.915</v>
       </c>
       <c r="J6" t="n">
-        <v>4.174</v>
+        <v>4.221</v>
       </c>
       <c r="K6" t="n">
-        <v>4.391</v>
+        <v>4.417</v>
       </c>
       <c r="L6" t="n">
-        <v>4.402</v>
+        <v>4.424</v>
       </c>
       <c r="M6" t="n">
-        <v>4.493</v>
+        <v>4.519</v>
       </c>
       <c r="N6" t="n">
-        <v>4.534</v>
+        <v>4.567</v>
       </c>
       <c r="O6" t="n">
-        <v>4.677</v>
+        <v>4.715</v>
       </c>
       <c r="P6" t="n">
-        <v>5.112</v>
+        <v>5.14</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.94</v>
+        <v>5.957</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.219</v>
+        <v>3.227</v>
       </c>
       <c r="G7" t="n">
-        <v>3.38</v>
+        <v>3.389</v>
       </c>
       <c r="H7" t="n">
-        <v>3.61</v>
+        <v>3.626</v>
       </c>
       <c r="I7" t="n">
-        <v>3.824</v>
+        <v>3.852</v>
       </c>
       <c r="J7" t="n">
-        <v>4.109</v>
+        <v>4.154</v>
       </c>
       <c r="K7" t="n">
-        <v>4.307</v>
+        <v>4.332</v>
       </c>
       <c r="L7" t="n">
-        <v>4.311</v>
+        <v>4.334</v>
       </c>
       <c r="M7" t="n">
-        <v>4.396</v>
+        <v>4.423</v>
       </c>
       <c r="N7" t="n">
-        <v>4.426</v>
+        <v>4.459</v>
       </c>
       <c r="O7" t="n">
-        <v>4.574</v>
+        <v>4.613</v>
       </c>
       <c r="P7" t="n">
-        <v>4.896</v>
+        <v>4.924</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.707</v>
+        <v>5.725</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.633</v>
+        <v>5.643</v>
       </c>
       <c r="G8" t="n">
-        <v>6.32</v>
+        <v>6.331</v>
       </c>
       <c r="H8" t="n">
-        <v>6.771</v>
+        <v>6.788</v>
       </c>
       <c r="I8" t="n">
-        <v>6.988</v>
+        <v>7.016</v>
       </c>
       <c r="J8" t="n">
-        <v>7.365</v>
+        <v>7.411</v>
       </c>
       <c r="K8" t="n">
-        <v>8.065</v>
+        <v>8.09</v>
       </c>
       <c r="L8" t="n">
-        <v>8.380000000000001</v>
+        <v>8.401999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.685</v>
+        <v>8.711</v>
       </c>
       <c r="N8" t="n">
-        <v>8.837999999999999</v>
+        <v>8.871</v>
       </c>
       <c r="O8" t="n">
-        <v>9.131</v>
+        <v>9.17</v>
       </c>
       <c r="P8" t="n">
-        <v>9.303000000000001</v>
+        <v>9.331</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.014</v>
+        <v>10.035</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.745</v>
+        <v>2.748</v>
       </c>
       <c r="G9" t="n">
-        <v>2.989</v>
+        <v>2.99</v>
       </c>
       <c r="H9" t="n">
-        <v>3.2</v>
+        <v>3.214</v>
       </c>
       <c r="I9" t="n">
-        <v>3.285</v>
+        <v>3.297</v>
       </c>
       <c r="J9" t="n">
-        <v>3.511</v>
+        <v>3.526</v>
       </c>
       <c r="K9" t="n">
-        <v>3.634</v>
+        <v>3.668</v>
       </c>
       <c r="L9" t="n">
-        <v>3.726</v>
+        <v>3.738</v>
       </c>
       <c r="M9" t="n">
-        <v>3.782</v>
+        <v>3.805</v>
       </c>
       <c r="N9" t="n">
-        <v>3.92</v>
+        <v>3.95</v>
       </c>
       <c r="O9" t="n">
-        <v>4.002</v>
+        <v>4.04</v>
       </c>
       <c r="P9" t="n">
-        <v>4.117</v>
+        <v>4.145</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.17</v>
+        <v>4.192</v>
       </c>
       <c r="R9" t="n">
-        <v>4.232</v>
+        <v>4.255</v>
       </c>
       <c r="S9" t="n">
-        <v>4.265</v>
+        <v>4.29</v>
       </c>
       <c r="T9" t="n">
-        <v>4.265</v>
+        <v>4.305</v>
       </c>
       <c r="U9" t="n">
-        <v>4.15</v>
+        <v>4.187</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.754</v>
+        <v>2.757</v>
       </c>
       <c r="G10" t="n">
-        <v>2.997</v>
+        <v>2.998</v>
       </c>
       <c r="H10" t="n">
-        <v>3.204</v>
+        <v>3.217</v>
       </c>
       <c r="I10" t="n">
-        <v>3.288</v>
+        <v>3.299</v>
       </c>
       <c r="J10" t="n">
-        <v>3.526</v>
+        <v>3.542</v>
       </c>
       <c r="K10" t="n">
-        <v>3.675</v>
+        <v>3.708</v>
       </c>
       <c r="L10" t="n">
-        <v>3.739</v>
+        <v>3.751</v>
       </c>
       <c r="M10" t="n">
-        <v>3.843</v>
+        <v>3.867</v>
       </c>
       <c r="N10" t="n">
-        <v>3.948</v>
+        <v>3.98</v>
       </c>
       <c r="O10" t="n">
-        <v>4.23</v>
+        <v>4.267</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.559</v>
+        <v>2.562</v>
       </c>
       <c r="G11" t="n">
-        <v>2.798</v>
+        <v>2.799</v>
       </c>
       <c r="H11" t="n">
-        <v>3.026</v>
+        <v>3.039</v>
       </c>
       <c r="I11" t="n">
-        <v>3.092</v>
+        <v>3.103</v>
       </c>
       <c r="J11" t="n">
-        <v>3.322</v>
+        <v>3.337</v>
       </c>
       <c r="K11" t="n">
-        <v>3.457</v>
+        <v>3.49</v>
       </c>
       <c r="L11" t="n">
-        <v>3.536</v>
+        <v>3.548</v>
       </c>
       <c r="M11" t="n">
-        <v>3.651</v>
+        <v>3.675</v>
       </c>
       <c r="N11" t="n">
-        <v>3.755</v>
+        <v>3.787</v>
       </c>
       <c r="O11" t="n">
-        <v>3.996</v>
+        <v>4.034</v>
       </c>
       <c r="P11" t="n">
-        <v>4.061</v>
+        <v>4.089</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.368</v>
+        <v>4.39</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.41</v>
+        <v>3.42</v>
       </c>
       <c r="G12" t="n">
-        <v>3.704</v>
+        <v>3.721</v>
       </c>
       <c r="H12" t="n">
-        <v>3.975</v>
+        <v>3.993</v>
       </c>
       <c r="I12" t="n">
-        <v>4.195</v>
+        <v>4.221</v>
       </c>
       <c r="J12" t="n">
-        <v>4.504</v>
+        <v>4.546</v>
       </c>
       <c r="K12" t="n">
-        <v>4.653</v>
+        <v>4.679</v>
       </c>
       <c r="L12" t="n">
-        <v>4.685</v>
+        <v>4.704</v>
       </c>
       <c r="M12" t="n">
-        <v>4.804</v>
+        <v>4.834</v>
       </c>
       <c r="N12" t="n">
-        <v>4.881</v>
+        <v>4.915</v>
       </c>
       <c r="O12" t="n">
-        <v>5.036</v>
+        <v>5.075</v>
       </c>
       <c r="P12" t="n">
-        <v>5.159</v>
+        <v>5.188</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.487</v>
+        <v>5.508</v>
       </c>
       <c r="R12" t="n">
-        <v>5.727</v>
+        <v>5.75</v>
       </c>
       <c r="S12" t="n">
-        <v>5.972</v>
+        <v>5.997</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.164</v>
+        <v>3.174</v>
       </c>
       <c r="G13" t="n">
-        <v>3.394</v>
+        <v>3.411</v>
       </c>
       <c r="H13" t="n">
-        <v>3.642</v>
+        <v>3.66</v>
       </c>
       <c r="I13" t="n">
-        <v>3.843</v>
+        <v>3.869</v>
       </c>
       <c r="J13" t="n">
-        <v>4.14</v>
+        <v>4.183</v>
       </c>
       <c r="K13" t="n">
-        <v>4.286</v>
+        <v>4.312</v>
       </c>
       <c r="L13" t="n">
-        <v>4.324</v>
+        <v>4.343</v>
       </c>
       <c r="M13" t="n">
-        <v>4.432</v>
+        <v>4.461</v>
       </c>
       <c r="N13" t="n">
-        <v>4.509</v>
+        <v>4.543</v>
       </c>
       <c r="O13" t="n">
-        <v>4.664</v>
+        <v>4.704</v>
       </c>
       <c r="P13" t="n">
-        <v>4.75</v>
+        <v>4.779</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.008</v>
+        <v>5.03</v>
       </c>
       <c r="R13" t="n">
-        <v>5.277</v>
+        <v>5.3</v>
       </c>
       <c r="S13" t="n">
-        <v>5.535</v>
+        <v>5.56</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.981</v>
+        <v>2.991</v>
       </c>
       <c r="G14" t="n">
-        <v>3.195</v>
+        <v>3.212</v>
       </c>
       <c r="H14" t="n">
-        <v>3.443</v>
+        <v>3.461</v>
       </c>
       <c r="I14" t="n">
-        <v>3.627</v>
+        <v>3.653</v>
       </c>
       <c r="J14" t="n">
-        <v>3.882</v>
+        <v>3.924</v>
       </c>
       <c r="K14" t="n">
-        <v>3.975</v>
+        <v>4.001</v>
       </c>
       <c r="L14" t="n">
-        <v>3.997</v>
+        <v>4.016</v>
       </c>
       <c r="M14" t="n">
-        <v>4.118</v>
+        <v>4.148</v>
       </c>
       <c r="N14" t="n">
-        <v>4.188</v>
+        <v>4.223</v>
       </c>
       <c r="O14" t="n">
-        <v>4.323</v>
+        <v>4.362</v>
       </c>
       <c r="P14" t="n">
-        <v>4.386</v>
+        <v>4.415</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.598</v>
+        <v>4.619</v>
       </c>
       <c r="R14" t="n">
-        <v>4.791</v>
+        <v>4.814</v>
       </c>
       <c r="S14" t="n">
-        <v>4.987</v>
+        <v>5.012</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.959</v>
+        <v>2.969</v>
       </c>
       <c r="G15" t="n">
-        <v>3.17</v>
+        <v>3.187</v>
       </c>
       <c r="H15" t="n">
-        <v>3.414</v>
+        <v>3.432</v>
       </c>
       <c r="I15" t="n">
-        <v>3.578</v>
+        <v>3.604</v>
       </c>
       <c r="J15" t="n">
-        <v>3.82</v>
+        <v>3.862</v>
       </c>
       <c r="K15" t="n">
-        <v>3.928</v>
+        <v>3.953</v>
       </c>
       <c r="L15" t="n">
-        <v>3.933</v>
+        <v>3.953</v>
       </c>
       <c r="M15" t="n">
-        <v>4.031</v>
+        <v>4.06</v>
       </c>
       <c r="N15" t="n">
-        <v>4.091</v>
+        <v>4.126</v>
       </c>
       <c r="O15" t="n">
-        <v>4.266</v>
+        <v>4.305</v>
       </c>
       <c r="P15" t="n">
-        <v>4.282</v>
+        <v>4.312</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.5</v>
+        <v>4.521</v>
       </c>
       <c r="R15" t="n">
-        <v>4.686</v>
+        <v>4.709</v>
       </c>
       <c r="S15" t="n">
-        <v>4.882</v>
+        <v>4.907</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.959</v>
+        <v>2.969</v>
       </c>
       <c r="G16" t="n">
-        <v>3.17</v>
+        <v>3.187</v>
       </c>
       <c r="H16" t="n">
-        <v>3.414</v>
+        <v>3.432</v>
       </c>
       <c r="I16" t="n">
-        <v>3.578</v>
+        <v>3.604</v>
       </c>
       <c r="J16" t="n">
-        <v>3.82</v>
+        <v>3.862</v>
       </c>
       <c r="K16" t="n">
-        <v>3.928</v>
+        <v>3.953</v>
       </c>
       <c r="L16" t="n">
-        <v>3.933</v>
+        <v>3.953</v>
       </c>
       <c r="M16" t="n">
-        <v>4.031</v>
+        <v>4.06</v>
       </c>
       <c r="N16" t="n">
-        <v>4.094</v>
+        <v>4.129</v>
       </c>
       <c r="O16" t="n">
-        <v>4.272</v>
+        <v>4.312</v>
       </c>
       <c r="P16" t="n">
-        <v>4.306</v>
+        <v>4.335</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.527</v>
+        <v>4.548</v>
       </c>
       <c r="R16" t="n">
-        <v>4.714</v>
+        <v>4.737</v>
       </c>
       <c r="S16" t="n">
-        <v>4.911</v>
+        <v>4.936</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.785</v>
+        <v>2.788</v>
       </c>
       <c r="G17" t="n">
-        <v>3.046</v>
+        <v>3.047</v>
       </c>
       <c r="H17" t="n">
-        <v>3.254</v>
+        <v>3.266</v>
       </c>
       <c r="I17" t="n">
-        <v>3.345</v>
+        <v>3.356</v>
       </c>
       <c r="J17" t="n">
-        <v>3.598</v>
+        <v>3.613</v>
       </c>
       <c r="K17" t="n">
-        <v>3.754</v>
+        <v>3.788</v>
       </c>
       <c r="L17" t="n">
-        <v>3.824</v>
+        <v>3.835</v>
       </c>
       <c r="M17" t="n">
-        <v>3.97</v>
+        <v>3.994</v>
       </c>
       <c r="N17" t="n">
-        <v>4.061</v>
+        <v>4.093</v>
       </c>
       <c r="O17" t="n">
-        <v>4.251</v>
+        <v>4.288</v>
       </c>
       <c r="P17" t="n">
-        <v>4.347</v>
+        <v>4.371</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.786</v>
+        <v>2.789</v>
       </c>
       <c r="G18" t="n">
-        <v>3.047</v>
+        <v>3.048</v>
       </c>
       <c r="H18" t="n">
-        <v>3.254</v>
+        <v>3.266</v>
       </c>
       <c r="I18" t="n">
-        <v>3.345</v>
+        <v>3.356</v>
       </c>
       <c r="J18" t="n">
-        <v>3.598</v>
+        <v>3.613</v>
       </c>
       <c r="K18" t="n">
-        <v>3.753</v>
+        <v>3.788</v>
       </c>
       <c r="L18" t="n">
-        <v>3.824</v>
+        <v>3.835</v>
       </c>
       <c r="M18" t="n">
-        <v>3.97</v>
+        <v>3.994</v>
       </c>
       <c r="N18" t="n">
-        <v>4.062</v>
+        <v>4.094</v>
       </c>
       <c r="O18" t="n">
-        <v>4.25</v>
+        <v>4.287</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.969</v>
+        <v>2.979</v>
       </c>
       <c r="G19" t="n">
-        <v>3.183</v>
+        <v>3.2</v>
       </c>
       <c r="H19" t="n">
-        <v>3.43</v>
+        <v>3.448</v>
       </c>
       <c r="I19" t="n">
-        <v>3.611</v>
+        <v>3.637</v>
       </c>
       <c r="J19" t="n">
-        <v>3.861</v>
+        <v>3.904</v>
       </c>
       <c r="K19" t="n">
-        <v>3.971</v>
+        <v>3.996</v>
       </c>
       <c r="L19" t="n">
-        <v>3.994</v>
+        <v>4.014</v>
       </c>
       <c r="M19" t="n">
-        <v>4.109</v>
+        <v>4.137</v>
       </c>
       <c r="N19" t="n">
-        <v>4.181</v>
+        <v>4.215</v>
       </c>
       <c r="O19" t="n">
-        <v>4.31</v>
+        <v>4.349</v>
       </c>
       <c r="P19" t="n">
-        <v>4.344</v>
+        <v>4.373</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.538</v>
+        <v>4.559</v>
       </c>
       <c r="R19" t="n">
-        <v>4.732</v>
+        <v>4.755</v>
       </c>
       <c r="S19" t="n">
-        <v>4.922</v>
+        <v>4.947</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.68</v>
+        <v>2.686</v>
       </c>
       <c r="G20" t="n">
-        <v>2.778</v>
+        <v>2.785</v>
       </c>
       <c r="H20" t="n">
-        <v>2.87</v>
+        <v>2.881</v>
       </c>
       <c r="I20" t="n">
-        <v>2.999</v>
+        <v>3.024</v>
       </c>
       <c r="J20" t="n">
-        <v>3.44</v>
+        <v>3.48</v>
       </c>
       <c r="K20" t="n">
-        <v>3.68</v>
+        <v>3.698</v>
       </c>
       <c r="L20" t="n">
-        <v>3.682</v>
+        <v>3.701</v>
       </c>
       <c r="M20" t="n">
-        <v>3.795</v>
+        <v>3.818</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.04</v>
+        <v>3.048</v>
       </c>
       <c r="G21" t="n">
-        <v>3.281</v>
+        <v>3.293</v>
       </c>
       <c r="H21" t="n">
-        <v>3.551</v>
+        <v>3.566</v>
       </c>
       <c r="I21" t="n">
-        <v>3.744</v>
+        <v>3.77</v>
       </c>
       <c r="J21" t="n">
-        <v>4.034</v>
+        <v>4.077</v>
       </c>
       <c r="K21" t="n">
-        <v>4.213</v>
+        <v>4.236</v>
       </c>
       <c r="L21" t="n">
-        <v>4.244</v>
+        <v>4.268</v>
       </c>
       <c r="M21" t="n">
-        <v>4.348</v>
+        <v>4.377</v>
       </c>
       <c r="N21" t="n">
-        <v>4.417</v>
+        <v>4.453</v>
       </c>
       <c r="O21" t="n">
-        <v>4.512</v>
+        <v>4.55</v>
       </c>
       <c r="P21" t="n">
-        <v>4.603</v>
+        <v>4.631</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.693</v>
+        <v>4.715</v>
       </c>
       <c r="R21" t="n">
-        <v>4.785</v>
+        <v>4.807</v>
       </c>
       <c r="S21" t="n">
-        <v>4.876</v>
+        <v>4.9</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.987</v>
+        <v>2.994</v>
       </c>
       <c r="G22" t="n">
-        <v>3.225</v>
+        <v>3.237</v>
       </c>
       <c r="H22" t="n">
-        <v>3.483</v>
+        <v>3.498</v>
       </c>
       <c r="I22" t="n">
-        <v>3.662</v>
+        <v>3.688</v>
       </c>
       <c r="J22" t="n">
-        <v>3.92</v>
+        <v>3.963</v>
       </c>
       <c r="K22" t="n">
-        <v>4.095</v>
+        <v>4.119</v>
       </c>
       <c r="L22" t="n">
-        <v>4.113</v>
+        <v>4.137</v>
       </c>
       <c r="M22" t="n">
-        <v>4.221</v>
+        <v>4.25</v>
       </c>
       <c r="N22" t="n">
-        <v>4.292</v>
+        <v>4.328</v>
       </c>
       <c r="O22" t="n">
-        <v>4.383</v>
+        <v>4.422</v>
       </c>
       <c r="P22" t="n">
-        <v>4.466</v>
+        <v>4.494</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.552</v>
+        <v>4.574</v>
       </c>
       <c r="R22" t="n">
-        <v>4.633</v>
+        <v>4.656</v>
       </c>
       <c r="S22" t="n">
-        <v>4.721</v>
+        <v>4.745</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.934</v>
+        <v>2.941</v>
       </c>
       <c r="G23" t="n">
-        <v>3.179</v>
+        <v>3.191</v>
       </c>
       <c r="H23" t="n">
-        <v>3.423</v>
+        <v>3.438</v>
       </c>
       <c r="I23" t="n">
-        <v>3.607</v>
+        <v>3.633</v>
       </c>
       <c r="J23" t="n">
-        <v>3.855</v>
+        <v>3.897</v>
       </c>
       <c r="K23" t="n">
-        <v>3.992</v>
+        <v>4.016</v>
       </c>
       <c r="L23" t="n">
-        <v>4.012</v>
+        <v>4.036</v>
       </c>
       <c r="M23" t="n">
-        <v>4.112</v>
+        <v>4.141</v>
       </c>
       <c r="N23" t="n">
-        <v>4.181</v>
+        <v>4.216</v>
       </c>
       <c r="O23" t="n">
-        <v>4.258</v>
+        <v>4.296</v>
       </c>
       <c r="P23" t="n">
-        <v>4.328</v>
+        <v>4.356</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.357</v>
+        <v>4.379</v>
       </c>
       <c r="R23" t="n">
-        <v>4.419</v>
+        <v>4.441</v>
       </c>
       <c r="S23" t="n">
-        <v>4.478</v>
+        <v>4.502</v>
       </c>
       <c r="T23" t="n">
-        <v>4.477</v>
+        <v>4.516</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.869</v>
+        <v>2.877</v>
       </c>
       <c r="G24" t="n">
-        <v>3.089</v>
+        <v>3.101</v>
       </c>
       <c r="H24" t="n">
-        <v>3.318</v>
+        <v>3.332</v>
       </c>
       <c r="I24" t="n">
-        <v>3.545</v>
+        <v>3.571</v>
       </c>
       <c r="J24" t="n">
-        <v>3.751</v>
+        <v>3.793</v>
       </c>
       <c r="K24" t="n">
-        <v>3.876</v>
+        <v>3.9</v>
       </c>
       <c r="L24" t="n">
-        <v>3.894</v>
+        <v>3.918</v>
       </c>
       <c r="M24" t="n">
-        <v>3.972</v>
+        <v>4.001</v>
       </c>
       <c r="N24" t="n">
-        <v>4.056</v>
+        <v>4.091</v>
       </c>
       <c r="O24" t="n">
-        <v>4.254</v>
+        <v>4.292</v>
       </c>
       <c r="P24" t="n">
-        <v>4.266</v>
+        <v>4.295</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.284</v>
+        <v>4.306</v>
       </c>
       <c r="R24" t="n">
-        <v>4.341</v>
+        <v>4.363</v>
       </c>
       <c r="S24" t="n">
-        <v>4.393</v>
+        <v>4.417</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.928</v>
+        <v>2.936</v>
       </c>
       <c r="G25" t="n">
-        <v>3.179</v>
+        <v>3.191</v>
       </c>
       <c r="H25" t="n">
-        <v>3.426</v>
+        <v>3.441</v>
       </c>
       <c r="I25" t="n">
-        <v>3.616</v>
+        <v>3.642</v>
       </c>
       <c r="J25" t="n">
-        <v>3.873</v>
+        <v>3.915</v>
       </c>
       <c r="K25" t="n">
-        <v>4.025</v>
+        <v>4.048</v>
       </c>
       <c r="L25" t="n">
-        <v>4.043</v>
+        <v>4.067</v>
       </c>
       <c r="M25" t="n">
-        <v>4.144</v>
+        <v>4.173</v>
       </c>
       <c r="N25" t="n">
-        <v>4.209</v>
+        <v>4.244</v>
       </c>
       <c r="O25" t="n">
-        <v>4.287</v>
+        <v>4.325</v>
       </c>
       <c r="P25" t="n">
-        <v>4.35</v>
+        <v>4.378</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.391</v>
+        <v>4.413</v>
       </c>
       <c r="R25" t="n">
-        <v>4.443</v>
+        <v>4.465</v>
       </c>
       <c r="S25" t="n">
-        <v>4.501</v>
+        <v>4.525</v>
       </c>
       <c r="T25" t="n">
-        <v>4.495</v>
+        <v>4.534</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.277</v>
+        <v>3.284</v>
       </c>
       <c r="G26" t="n">
-        <v>3.497</v>
+        <v>3.507</v>
       </c>
       <c r="H26" t="n">
-        <v>3.835</v>
+        <v>3.854</v>
       </c>
       <c r="I26" t="n">
-        <v>4.042</v>
+        <v>4.068</v>
       </c>
       <c r="J26" t="n">
-        <v>4.443</v>
+        <v>4.488</v>
       </c>
       <c r="K26" t="n">
-        <v>4.828</v>
+        <v>4.852</v>
       </c>
       <c r="L26" t="n">
-        <v>4.9</v>
+        <v>4.918</v>
       </c>
       <c r="M26" t="n">
-        <v>5.041</v>
+        <v>5.067</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.343</v>
+        <v>5.381</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.071</v>
+        <v>3.079</v>
       </c>
       <c r="G27" t="n">
-        <v>3.259</v>
+        <v>3.272</v>
       </c>
       <c r="H27" t="n">
-        <v>3.518</v>
+        <v>3.535</v>
       </c>
       <c r="I27" t="n">
-        <v>3.7</v>
+        <v>3.725</v>
       </c>
       <c r="J27" t="n">
-        <v>3.974</v>
+        <v>4.017</v>
       </c>
       <c r="K27" t="n">
-        <v>4.149</v>
+        <v>4.173</v>
       </c>
       <c r="L27" t="n">
-        <v>4.17</v>
+        <v>4.188</v>
       </c>
       <c r="M27" t="n">
-        <v>4.27</v>
+        <v>4.298</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.45</v>
+        <v>4.49</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.174</v>
+        <v>3.182</v>
       </c>
       <c r="G28" t="n">
-        <v>3.371</v>
+        <v>3.384</v>
       </c>
       <c r="H28" t="n">
-        <v>3.645</v>
+        <v>3.662</v>
       </c>
       <c r="I28" t="n">
-        <v>3.837</v>
+        <v>3.862</v>
       </c>
       <c r="J28" t="n">
-        <v>4.146</v>
+        <v>4.19</v>
       </c>
       <c r="K28" t="n">
-        <v>4.341</v>
+        <v>4.365</v>
       </c>
       <c r="L28" t="n">
-        <v>4.373</v>
+        <v>4.391</v>
       </c>
       <c r="M28" t="n">
-        <v>4.482</v>
+        <v>4.51</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.742</v>
+        <v>4.782</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3.019</v>
+        <v>3.027</v>
       </c>
       <c r="G29" t="n">
-        <v>3.203</v>
+        <v>3.216</v>
       </c>
       <c r="H29" t="n">
-        <v>3.454</v>
+        <v>3.471</v>
       </c>
       <c r="I29" t="n">
-        <v>3.624</v>
+        <v>3.649</v>
       </c>
       <c r="J29" t="n">
-        <v>3.885</v>
+        <v>3.928</v>
       </c>
       <c r="K29" t="n">
-        <v>4.045</v>
+        <v>4.069</v>
       </c>
       <c r="L29" t="n">
-        <v>4.056</v>
+        <v>4.074</v>
       </c>
       <c r="M29" t="n">
-        <v>4.133</v>
+        <v>4.161</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.322</v>
+        <v>4.362</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.308</v>
+        <v>3.318</v>
       </c>
       <c r="G30" t="n">
-        <v>3.464</v>
+        <v>3.476</v>
       </c>
       <c r="H30" t="n">
-        <v>3.759</v>
+        <v>3.779</v>
       </c>
       <c r="I30" t="n">
-        <v>3.957</v>
+        <v>3.983</v>
       </c>
       <c r="J30" t="n">
-        <v>4.294</v>
+        <v>4.34</v>
       </c>
       <c r="K30" t="n">
-        <v>4.62</v>
+        <v>4.644</v>
       </c>
       <c r="L30" t="n">
-        <v>4.67</v>
+        <v>4.686</v>
       </c>
       <c r="M30" t="n">
-        <v>4.8</v>
+        <v>4.826</v>
       </c>
       <c r="N30" t="n">
-        <v>4.984</v>
+        <v>5.015</v>
       </c>
       <c r="O30" t="n">
-        <v>5.293</v>
+        <v>5.33</v>
       </c>
       <c r="P30" t="n">
-        <v>5.494</v>
+        <v>5.523</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.232</v>
+        <v>6.254</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.637</v>
+        <v>3.647</v>
       </c>
       <c r="G31" t="n">
-        <v>3.83</v>
+        <v>3.842</v>
       </c>
       <c r="H31" t="n">
-        <v>4.175</v>
+        <v>4.195</v>
       </c>
       <c r="I31" t="n">
-        <v>4.388</v>
+        <v>4.414</v>
       </c>
       <c r="J31" t="n">
-        <v>4.788</v>
+        <v>4.835</v>
       </c>
       <c r="K31" t="n">
-        <v>5.156</v>
+        <v>5.18</v>
       </c>
       <c r="L31" t="n">
-        <v>5.282</v>
+        <v>5.299</v>
       </c>
       <c r="M31" t="n">
-        <v>5.53</v>
+        <v>5.556</v>
       </c>
       <c r="N31" t="n">
-        <v>5.843</v>
+        <v>5.874</v>
       </c>
       <c r="O31" t="n">
-        <v>6.329</v>
+        <v>6.366</v>
       </c>
       <c r="P31" t="n">
-        <v>6.483</v>
+        <v>6.511</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.205</v>
+        <v>7.227</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.407</v>
+        <v>3.417</v>
       </c>
       <c r="G32" t="n">
-        <v>3.582</v>
+        <v>3.594</v>
       </c>
       <c r="H32" t="n">
-        <v>3.903</v>
+        <v>3.923</v>
       </c>
       <c r="I32" t="n">
-        <v>4.116</v>
+        <v>4.142</v>
       </c>
       <c r="J32" t="n">
-        <v>4.475</v>
+        <v>4.521</v>
       </c>
       <c r="K32" t="n">
-        <v>4.805</v>
+        <v>4.829</v>
       </c>
       <c r="L32" t="n">
-        <v>4.874</v>
+        <v>4.89</v>
       </c>
       <c r="M32" t="n">
-        <v>5.072</v>
+        <v>5.098</v>
       </c>
       <c r="N32" t="n">
-        <v>5.345</v>
+        <v>5.376</v>
       </c>
       <c r="O32" t="n">
-        <v>5.738</v>
+        <v>5.776</v>
       </c>
       <c r="P32" t="n">
-        <v>5.954</v>
+        <v>5.983</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.693</v>
+        <v>6.715</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.174</v>
+        <v>3.186</v>
       </c>
       <c r="G33" t="n">
-        <v>3.329</v>
+        <v>3.342</v>
       </c>
       <c r="H33" t="n">
-        <v>3.576</v>
+        <v>3.597</v>
       </c>
       <c r="I33" t="n">
-        <v>3.744</v>
+        <v>3.772</v>
       </c>
       <c r="J33" t="n">
-        <v>4</v>
+        <v>4.048</v>
       </c>
       <c r="K33" t="n">
-        <v>4.261</v>
+        <v>4.286</v>
       </c>
       <c r="L33" t="n">
-        <v>4.276</v>
+        <v>4.295</v>
       </c>
       <c r="M33" t="n">
-        <v>4.328</v>
+        <v>4.354</v>
       </c>
       <c r="N33" t="n">
-        <v>4.372</v>
+        <v>4.404</v>
       </c>
       <c r="O33" t="n">
-        <v>4.449</v>
+        <v>4.488</v>
       </c>
       <c r="P33" t="n">
-        <v>4.527</v>
+        <v>4.556</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.949</v>
+        <v>4.971</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.234</v>
+        <v>3.246</v>
       </c>
       <c r="G34" t="n">
-        <v>3.383</v>
+        <v>3.396</v>
       </c>
       <c r="H34" t="n">
-        <v>3.639</v>
+        <v>3.66</v>
       </c>
       <c r="I34" t="n">
-        <v>3.813</v>
+        <v>3.84</v>
       </c>
       <c r="J34" t="n">
-        <v>4.072</v>
+        <v>4.119</v>
       </c>
       <c r="K34" t="n">
-        <v>4.339</v>
+        <v>4.364</v>
       </c>
       <c r="L34" t="n">
-        <v>4.354</v>
+        <v>4.373</v>
       </c>
       <c r="M34" t="n">
-        <v>4.419</v>
+        <v>4.445</v>
       </c>
       <c r="N34" t="n">
-        <v>4.477</v>
+        <v>4.509</v>
       </c>
       <c r="O34" t="n">
-        <v>4.618</v>
+        <v>4.657</v>
       </c>
       <c r="P34" t="n">
-        <v>4.821</v>
+        <v>4.85</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.65</v>
+        <v>5.672</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.208</v>
+        <v>3.22</v>
       </c>
       <c r="G35" t="n">
-        <v>3.357</v>
+        <v>3.37</v>
       </c>
       <c r="H35" t="n">
-        <v>3.607</v>
+        <v>3.628</v>
       </c>
       <c r="I35" t="n">
-        <v>3.779</v>
+        <v>3.807</v>
       </c>
       <c r="J35" t="n">
-        <v>4.04</v>
+        <v>4.088</v>
       </c>
       <c r="K35" t="n">
-        <v>4.291</v>
+        <v>4.316</v>
       </c>
       <c r="L35" t="n">
-        <v>4.31</v>
+        <v>4.329</v>
       </c>
       <c r="M35" t="n">
-        <v>4.365</v>
+        <v>4.391</v>
       </c>
       <c r="N35" t="n">
-        <v>4.414</v>
+        <v>4.446</v>
       </c>
       <c r="O35" t="n">
-        <v>4.515</v>
+        <v>4.554</v>
       </c>
       <c r="P35" t="n">
-        <v>4.624</v>
+        <v>4.653</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.285</v>
+        <v>5.307</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.093</v>
+        <v>3.104</v>
       </c>
       <c r="G36" t="n">
-        <v>3.232</v>
+        <v>3.244</v>
       </c>
       <c r="H36" t="n">
-        <v>3.479</v>
+        <v>3.501</v>
       </c>
       <c r="I36" t="n">
-        <v>3.655</v>
+        <v>3.683</v>
       </c>
       <c r="J36" t="n">
-        <v>3.938</v>
+        <v>3.985</v>
       </c>
       <c r="K36" t="n">
-        <v>4.188</v>
+        <v>4.213</v>
       </c>
       <c r="L36" t="n">
-        <v>4.2</v>
+        <v>4.219</v>
       </c>
       <c r="M36" t="n">
-        <v>4.231</v>
+        <v>4.257</v>
       </c>
       <c r="N36" t="n">
-        <v>4.277</v>
+        <v>4.309</v>
       </c>
       <c r="O36" t="n">
-        <v>4.356</v>
+        <v>4.395</v>
       </c>
       <c r="P36" t="n">
-        <v>4.425</v>
+        <v>4.454</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.666</v>
+        <v>4.688</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.982</v>
+        <v>3.992</v>
       </c>
       <c r="G37" t="n">
-        <v>4.524</v>
+        <v>4.536</v>
       </c>
       <c r="H37" t="n">
-        <v>5.148</v>
+        <v>5.168</v>
       </c>
       <c r="I37" t="n">
-        <v>5.449</v>
+        <v>5.475</v>
       </c>
       <c r="J37" t="n">
-        <v>6.278</v>
+        <v>6.324</v>
       </c>
       <c r="K37" t="n">
-        <v>7.198</v>
+        <v>7.221</v>
       </c>
       <c r="L37" t="n">
-        <v>7.483</v>
+        <v>7.499</v>
       </c>
       <c r="M37" t="n">
-        <v>7.802</v>
+        <v>7.828</v>
       </c>
       <c r="N37" t="n">
-        <v>7.999</v>
+        <v>8.032</v>
       </c>
       <c r="O37" t="n">
-        <v>8.208</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="P37" t="n">
-        <v>8.284000000000001</v>
+        <v>8.311999999999999</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.698</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.044</v>
+        <v>5.054</v>
       </c>
       <c r="G38" t="n">
-        <v>5.839</v>
+        <v>5.851</v>
       </c>
       <c r="H38" t="n">
-        <v>6.675</v>
+        <v>6.695</v>
       </c>
       <c r="I38" t="n">
-        <v>7.133</v>
+        <v>7.159</v>
       </c>
       <c r="J38" t="n">
-        <v>8.222</v>
+        <v>8.268000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.321</v>
+        <v>9.345000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.765000000000001</v>
+        <v>9.782</v>
       </c>
       <c r="M38" t="n">
-        <v>10.214</v>
+        <v>10.24</v>
       </c>
       <c r="N38" t="n">
-        <v>10.418</v>
+        <v>10.45</v>
       </c>
       <c r="O38" t="n">
-        <v>10.608</v>
+        <v>10.646</v>
       </c>
       <c r="P38" t="n">
-        <v>10.682</v>
+        <v>10.71</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.148</v>
+        <v>11.17</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.364</v>
+        <v>4.374</v>
       </c>
       <c r="G39" t="n">
-        <v>5.037</v>
+        <v>5.049</v>
       </c>
       <c r="H39" t="n">
-        <v>5.74</v>
+        <v>5.76</v>
       </c>
       <c r="I39" t="n">
-        <v>6.137</v>
+        <v>6.163</v>
       </c>
       <c r="J39" t="n">
-        <v>7.094</v>
+        <v>7.14</v>
       </c>
       <c r="K39" t="n">
-        <v>8.153</v>
+        <v>8.177</v>
       </c>
       <c r="L39" t="n">
-        <v>8.521000000000001</v>
+        <v>8.537000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.85</v>
+        <v>8.875999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>9.045999999999999</v>
+        <v>9.077999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>9.259</v>
+        <v>9.295999999999999</v>
       </c>
       <c r="P39" t="n">
-        <v>9.337</v>
+        <v>9.365</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.794</v>
+        <v>9.816000000000001</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.5</v>
+        <v>3.51</v>
       </c>
       <c r="G40" t="n">
-        <v>3.702</v>
+        <v>3.714</v>
       </c>
       <c r="H40" t="n">
-        <v>4.018</v>
+        <v>4.038</v>
       </c>
       <c r="I40" t="n">
-        <v>4.231</v>
+        <v>4.257</v>
       </c>
       <c r="J40" t="n">
-        <v>4.586</v>
+        <v>4.632</v>
       </c>
       <c r="K40" t="n">
-        <v>4.926</v>
+        <v>4.95</v>
       </c>
       <c r="L40" t="n">
-        <v>4.995</v>
+        <v>5.012</v>
       </c>
       <c r="M40" t="n">
-        <v>5.142</v>
+        <v>5.168</v>
       </c>
       <c r="N40" t="n">
-        <v>5.342</v>
+        <v>5.373</v>
       </c>
       <c r="O40" t="n">
-        <v>5.672</v>
+        <v>5.709</v>
       </c>
       <c r="P40" t="n">
-        <v>5.915</v>
+        <v>5.944</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.683</v>
+        <v>6.705</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.886</v>
+        <v>3.896</v>
       </c>
       <c r="G41" t="n">
-        <v>4.131</v>
+        <v>4.143</v>
       </c>
       <c r="H41" t="n">
-        <v>4.504</v>
+        <v>4.524</v>
       </c>
       <c r="I41" t="n">
-        <v>4.736</v>
+        <v>4.762</v>
       </c>
       <c r="J41" t="n">
-        <v>5.144</v>
+        <v>5.19</v>
       </c>
       <c r="K41" t="n">
-        <v>5.529</v>
+        <v>5.554</v>
       </c>
       <c r="L41" t="n">
-        <v>5.673</v>
+        <v>5.689</v>
       </c>
       <c r="M41" t="n">
-        <v>5.945</v>
+        <v>5.971</v>
       </c>
       <c r="N41" t="n">
-        <v>6.273</v>
+        <v>6.304</v>
       </c>
       <c r="O41" t="n">
-        <v>6.787</v>
+        <v>6.825</v>
       </c>
       <c r="P41" t="n">
-        <v>6.975</v>
+        <v>7.003</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.73</v>
+        <v>7.752</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.621</v>
+        <v>3.631</v>
       </c>
       <c r="G42" t="n">
-        <v>3.851</v>
+        <v>3.863</v>
       </c>
       <c r="H42" t="n">
-        <v>4.194</v>
+        <v>4.214</v>
       </c>
       <c r="I42" t="n">
-        <v>4.42</v>
+        <v>4.446</v>
       </c>
       <c r="J42" t="n">
-        <v>4.791</v>
+        <v>4.837</v>
       </c>
       <c r="K42" t="n">
-        <v>5.147</v>
+        <v>5.171</v>
       </c>
       <c r="L42" t="n">
-        <v>5.23</v>
+        <v>5.247</v>
       </c>
       <c r="M42" t="n">
-        <v>5.449</v>
+        <v>5.475</v>
       </c>
       <c r="N42" t="n">
-        <v>5.756</v>
+        <v>5.787</v>
       </c>
       <c r="O42" t="n">
-        <v>6.164</v>
+        <v>6.201</v>
       </c>
       <c r="P42" t="n">
-        <v>6.418</v>
+        <v>6.446</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.196</v>
+        <v>7.218</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.324</v>
+        <v>3.336</v>
       </c>
       <c r="G43" t="n">
-        <v>3.514</v>
+        <v>3.526</v>
       </c>
       <c r="H43" t="n">
-        <v>3.778</v>
+        <v>3.799</v>
       </c>
       <c r="I43" t="n">
-        <v>3.953</v>
+        <v>3.981</v>
       </c>
       <c r="J43" t="n">
-        <v>4.228</v>
+        <v>4.275</v>
       </c>
       <c r="K43" t="n">
-        <v>4.493</v>
+        <v>4.518</v>
       </c>
       <c r="L43" t="n">
-        <v>4.519</v>
+        <v>4.538</v>
       </c>
       <c r="M43" t="n">
-        <v>4.583</v>
+        <v>4.609</v>
       </c>
       <c r="N43" t="n">
-        <v>4.642</v>
+        <v>4.674</v>
       </c>
       <c r="O43" t="n">
-        <v>4.762</v>
+        <v>4.801</v>
       </c>
       <c r="P43" t="n">
-        <v>4.892</v>
+        <v>4.922</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.559</v>
+        <v>5.581</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46192</v>
+        <v>46195</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.173</v>
+        <v>3.184</v>
       </c>
       <c r="G44" t="n">
-        <v>3.343</v>
+        <v>3.355</v>
       </c>
       <c r="H44" t="n">
-        <v>3.603</v>
+        <v>3.624</v>
       </c>
       <c r="I44" t="n">
-        <v>3.782</v>
+        <v>3.81</v>
       </c>
       <c r="J44" t="n">
-        <v>4.079</v>
+        <v>4.126</v>
       </c>
       <c r="K44" t="n">
-        <v>4.339</v>
+        <v>4.364</v>
       </c>
       <c r="L44" t="n">
-        <v>4.362</v>
+        <v>4.381</v>
       </c>
       <c r="M44" t="n">
-        <v>4.401</v>
+        <v>4.428</v>
       </c>
       <c r="N44" t="n">
-        <v>4.458</v>
+        <v>4.49</v>
       </c>
       <c r="O44" t="n">
-        <v>4.557</v>
+        <v>4.596</v>
       </c>
       <c r="P44" t="n">
-        <v>4.655</v>
+        <v>4.684</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.93</v>
+        <v>4.952</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-06-23 ~ 2026-06-23
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.51</v>
+        <v>3.517</v>
       </c>
       <c r="G2" t="n">
-        <v>3.83</v>
+        <v>3.836</v>
       </c>
       <c r="H2" t="n">
-        <v>4.105</v>
+        <v>4.111</v>
       </c>
       <c r="I2" t="n">
-        <v>4.261</v>
+        <v>4.263</v>
       </c>
       <c r="J2" t="n">
-        <v>4.57</v>
+        <v>4.566</v>
       </c>
       <c r="K2" t="n">
-        <v>4.901</v>
+        <v>4.889</v>
       </c>
       <c r="L2" t="n">
-        <v>5.058</v>
+        <v>5.023</v>
       </c>
       <c r="M2" t="n">
-        <v>5